<commit_message>
chore: auto-refresh NSE data and pipeline outputs (2026-03-25)
</commit_message>
<xml_diff>
--- a/working-sector/output/auto_components_comprehensive_report.xlsx
+++ b/working-sector/output/auto_components_comprehensive_report.xlsx
@@ -447,7 +447,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
     </row>
@@ -779,48 +779,48 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1923.9</v>
+        <v>1736.5</v>
       </c>
       <c r="D2" t="n">
-        <v>0.2092394720301698</v>
+        <v>-0.0521288209606987</v>
       </c>
       <c r="E2" t="n">
-        <v>0.3775597880567092</v>
+        <v>0.2350640113798008</v>
       </c>
       <c r="F2" t="n">
-        <v>0.6694724054147865</v>
+        <v>0.5304953287502205</v>
       </c>
       <c r="G2" t="n">
-        <v>0.5345076577139405</v>
+        <v>0.5510679700881947</v>
       </c>
       <c r="H2" t="n">
-        <v>0.6733406116836733</v>
+        <v>0.5853350604923128</v>
       </c>
       <c r="I2" t="n">
-        <v>74.69975980784629</v>
+        <v>37.49420670477369</v>
       </c>
       <c r="J2" t="n">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="K2" t="n">
         <v>54.83</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M2" t="n">
         <v>54.83</v>
       </c>
       <c r="N2" t="n">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="O2" t="n">
         <v>97.87234042553192</v>
       </c>
       <c r="P2" t="n">
-        <v>69.50646808510639</v>
+        <v>61.50646808510639</v>
       </c>
       <c r="Q2" t="b">
         <v>0</v>
@@ -844,54 +844,54 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1121.3</v>
+        <v>1087.6</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.0693061088977423</v>
+        <v>-0.0906354515050168</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.1323222162036679</v>
+        <v>-0.1452373467463062</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0485318870394613</v>
+        <v>-0.1691367456073339</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.0864328606613846</v>
+        <v>-0.1485641042693597</v>
       </c>
       <c r="H3" t="n">
-        <v>0.0524000933083481</v>
+        <v>-0.1142970138652417</v>
       </c>
       <c r="I3" t="n">
-        <v>25.05083367222446</v>
+        <v>46.095141185449</v>
       </c>
       <c r="J3" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="K3" t="n">
         <v>49.36</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M3" t="n">
         <v>49.36</v>
       </c>
       <c r="N3" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="O3" t="n">
-        <v>51.06382978723404</v>
+        <v>27.65957446808511</v>
       </c>
       <c r="P3" t="n">
-        <v>37.95676595744681</v>
+        <v>41.27591489361702</v>
       </c>
       <c r="Q3" t="b">
         <v>0</v>
       </c>
       <c r="R3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S3" t="b">
         <v>0</v>
@@ -909,25 +909,25 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>33335</v>
+        <v>30390</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.0919368019613184</v>
+        <v>-0.1400679117147708</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.1001484680793629</v>
+        <v>-0.1768689057421452</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.1366226366226366</v>
+        <v>-0.2644318044293839</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.2715873843234826</v>
+        <v>-0.2438591630914097</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.1327544303537497</v>
+        <v>-0.2095920726872917</v>
       </c>
       <c r="I4" t="n">
-        <v>32.36173393124065</v>
+        <v>33.62168396770474</v>
       </c>
       <c r="J4" t="n">
         <v>30</v>
@@ -937,7 +937,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M4" t="n">
@@ -947,10 +947,10 @@
         <v>30</v>
       </c>
       <c r="O4" t="n">
-        <v>19.14893617021277</v>
+        <v>10.63829787234042</v>
       </c>
       <c r="P4" t="n">
-        <v>37.22178723404255</v>
+        <v>35.51965957446808</v>
       </c>
       <c r="Q4" t="b">
         <v>0</v>
@@ -974,48 +974,48 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>315.95</v>
+        <v>307.15</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.0748169838945828</v>
+        <v>-0.0923463356973995</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.1718217562254259</v>
+        <v>-0.1920294620544521</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.1606004250797024</v>
+        <v>-0.2620134550696781</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.2955651727805484</v>
+        <v>-0.2414408137317039</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.1567322188108155</v>
+        <v>-0.2071737233275858</v>
       </c>
       <c r="I5" t="n">
-        <v>32.66832917705733</v>
+        <v>43.0862831858407</v>
       </c>
       <c r="J5" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K5" t="n">
         <v>51.12</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M5" t="n">
         <v>51.12</v>
       </c>
       <c r="N5" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O5" t="n">
-        <v>14.8936170212766</v>
+        <v>12.76595744680851</v>
       </c>
       <c r="P5" t="n">
-        <v>35.42672340425532</v>
+        <v>39.0011914893617</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
@@ -1039,48 +1039,48 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>122.77</v>
+        <v>113.13</v>
       </c>
       <c r="D6" t="n">
-        <v>0.0012232914695806</v>
+        <v>-0.1352239718697446</v>
       </c>
       <c r="E6" t="n">
-        <v>0.1267437591776798</v>
+        <v>-0.033489961554891</v>
       </c>
       <c r="F6" t="n">
-        <v>0.3600310180569404</v>
+        <v>0.1726961749766766</v>
       </c>
       <c r="G6" t="n">
-        <v>0.2250662703560944</v>
+        <v>0.1932688163146508</v>
       </c>
       <c r="H6" t="n">
-        <v>0.3638992243258272</v>
+        <v>0.2275359067187689</v>
       </c>
       <c r="I6" t="n">
-        <v>36.94247923715782</v>
+        <v>35.66312133709572</v>
       </c>
       <c r="J6" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="K6" t="n">
         <v>51.57</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M6" t="n">
         <v>51.57</v>
       </c>
       <c r="N6" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="O6" t="n">
-        <v>82.97872340425532</v>
+        <v>85.1063829787234</v>
       </c>
       <c r="P6" t="n">
-        <v>57.22374468085107</v>
+        <v>49.64927659574468</v>
       </c>
       <c r="Q6" t="b">
         <v>0</v>
@@ -1104,25 +1104,25 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2722.9</v>
+        <v>2682.4</v>
       </c>
       <c r="D7" t="n">
-        <v>0.0324182907408812</v>
+        <v>0.0562293274531422</v>
       </c>
       <c r="E7" t="n">
-        <v>-0.1018570439027607</v>
+        <v>0.0058874264071699</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.098884733759142</v>
+        <v>-0.1198031173092698</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.233849481459988</v>
+        <v>-0.0992304759712956</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.0950165274902552</v>
+        <v>-0.0649633855671776</v>
       </c>
       <c r="I7" t="n">
-        <v>67.22469666717861</v>
+        <v>44.36388353914127</v>
       </c>
       <c r="J7" t="n">
         <v>80</v>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M7" t="n">
@@ -1142,10 +1142,10 @@
         <v>80</v>
       </c>
       <c r="O7" t="n">
-        <v>29.78723404255319</v>
+        <v>38.29787234042553</v>
       </c>
       <c r="P7" t="n">
-        <v>57.44944680851064</v>
+        <v>59.15157446808512</v>
       </c>
       <c r="Q7" t="b">
         <v>0</v>
@@ -1169,48 +1169,48 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>514.95</v>
+        <v>511.45</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.033592943605142</v>
+        <v>-0.045891241488667</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0540374577832361</v>
+        <v>0.0377396773866287</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1696763202725724</v>
+        <v>0.1494549949432519</v>
       </c>
       <c r="G8" t="n">
-        <v>0.0347115725717264</v>
+        <v>0.1700276362812262</v>
       </c>
       <c r="H8" t="n">
-        <v>0.1735445265414592</v>
+        <v>0.2042947266853442</v>
       </c>
       <c r="I8" t="n">
-        <v>43.58341559723593</v>
+        <v>50.15782828282829</v>
       </c>
       <c r="J8" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K8" t="n">
         <v>49.66</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M8" t="n">
         <v>49.66</v>
       </c>
       <c r="N8" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O8" t="n">
-        <v>70.21276595744681</v>
+        <v>82.97872340425532</v>
       </c>
       <c r="P8" t="n">
-        <v>57.90655319148937</v>
+        <v>68.45974468085107</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
@@ -1234,48 +1234,48 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>439.75</v>
+        <v>419.65</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.142202282258851</v>
+        <v>-0.07464167585446529</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.1588561591430757</v>
+        <v>-0.1952248537731327</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.0154483376245382</v>
+        <v>-0.1397088970889709</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.1504130853253842</v>
+        <v>-0.1191362557509967</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.0115801313556513</v>
+        <v>-0.0848691653468787</v>
       </c>
       <c r="I9" t="n">
-        <v>23.87434554973822</v>
+        <v>40.15936254980078</v>
       </c>
       <c r="J9" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="K9" t="n">
         <v>53.44</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M9" t="n">
         <v>53.44</v>
       </c>
       <c r="N9" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="O9" t="n">
-        <v>40.42553191489361</v>
+        <v>31.91489361702128</v>
       </c>
       <c r="P9" t="n">
-        <v>37.46110638297873</v>
+        <v>43.75897872340426</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -1299,25 +1299,25 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>138780</v>
+        <v>129970</v>
       </c>
       <c r="D10" t="n">
-        <v>0.008282476024411499</v>
+        <v>-0.1083287596048299</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.1058565814058372</v>
+        <v>-0.1516872266823314</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.0124879923150816</v>
+        <v>-0.1554082594144978</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.1474527400159276</v>
+        <v>-0.1348356180765236</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.008619786046194801</v>
+        <v>-0.1005685276724056</v>
       </c>
       <c r="I10" t="n">
-        <v>32.46089515254762</v>
+        <v>33.76129339039468</v>
       </c>
       <c r="J10" t="n">
         <v>30</v>
@@ -1327,7 +1327,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M10" t="n">
@@ -1337,10 +1337,10 @@
         <v>30</v>
       </c>
       <c r="O10" t="n">
-        <v>42.5531914893617</v>
+        <v>29.78723404255319</v>
       </c>
       <c r="P10" t="n">
-        <v>40.27463829787234</v>
+        <v>37.72144680851064</v>
       </c>
       <c r="Q10" t="b">
         <v>0</v>
@@ -1376,10 +1376,10 @@
         <v>-0.0042030657656173</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.1391678134664633</v>
+        <v>0.0163695755723568</v>
       </c>
       <c r="H11" t="n">
-        <v>-0.0003348594967305</v>
+        <v>0.0506366659764748</v>
       </c>
       <c r="I11" t="n">
         <v>27.6054590570719</v>
@@ -1392,7 +1392,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M11" t="n">
@@ -1402,16 +1402,16 @@
         <v>20</v>
       </c>
       <c r="O11" t="n">
-        <v>46.80851063829788</v>
+        <v>63.82978723404256</v>
       </c>
       <c r="P11" t="n">
-        <v>21.36170212765958</v>
+        <v>24.76595744680852</v>
       </c>
       <c r="Q11" t="b">
         <v>0</v>
       </c>
       <c r="R11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S11" t="b">
         <v>0</v>
@@ -1429,48 +1429,48 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>391.85</v>
+        <v>444.15</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.1468539081210537</v>
+        <v>0.0255137381667049</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.1829649708090075</v>
+        <v>-0.0730460189919649</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.1688408102661999</v>
+        <v>-0.1285195722554694</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.3038055579670459</v>
+        <v>-0.1079469309174951</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.164972603997313</v>
+        <v>-0.0736798405133771</v>
       </c>
       <c r="I12" t="n">
-        <v>24.08242112041213</v>
+        <v>69.83381502890172</v>
       </c>
       <c r="J12" t="n">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="K12" t="n">
         <v>71.28</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M12" t="n">
         <v>71.28</v>
       </c>
       <c r="N12" t="n">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="O12" t="n">
-        <v>12.76595744680851</v>
+        <v>34.04255319148936</v>
       </c>
       <c r="P12" t="n">
-        <v>39.0651914893617</v>
+        <v>67.32051063829788</v>
       </c>
       <c r="Q12" t="b">
         <v>1</v>
@@ -1494,54 +1494,54 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1987</v>
+        <v>1650.4</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.0579813208173328</v>
+        <v>-0.1813085966565801</v>
       </c>
       <c r="E13" t="n">
-        <v>0.2024933430162188</v>
+        <v>-0.0945797673908271</v>
       </c>
       <c r="F13" t="n">
-        <v>0.2149932738168032</v>
+        <v>-0.0678865921156669</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0800285261159572</v>
+        <v>-0.0473139507776927</v>
       </c>
       <c r="H13" t="n">
-        <v>0.21886148008569</v>
+        <v>-0.0130468603735747</v>
       </c>
       <c r="I13" t="n">
-        <v>45.62982005141387</v>
+        <v>19.06348649596633</v>
       </c>
       <c r="J13" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="K13" t="n">
         <v>58.77</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M13" t="n">
         <v>58.77</v>
       </c>
       <c r="N13" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="O13" t="n">
-        <v>78.72340425531915</v>
+        <v>53.19148936170212</v>
       </c>
       <c r="P13" t="n">
-        <v>63.25268085106384</v>
+        <v>42.14629787234043</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
       </c>
       <c r="R13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S13" t="b">
         <v>0</v>
@@ -1559,54 +1559,54 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>581.9</v>
+        <v>560.75</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.09656885576773799</v>
+        <v>-0.1464342796255423</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.2519123224272033</v>
+        <v>-0.25008358408559</v>
       </c>
       <c r="F14" t="n">
-        <v>0.0775925925925926</v>
+        <v>-0.0585914547133383</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.0573721551082533</v>
+        <v>-0.0380188133753641</v>
       </c>
       <c r="H14" t="n">
-        <v>0.0814607988614795</v>
+        <v>-0.0037517229712461</v>
       </c>
       <c r="I14" t="n">
-        <v>20.58823529411769</v>
+        <v>44.04982772329711</v>
       </c>
       <c r="J14" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="K14" t="n">
         <v>54.64</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M14" t="n">
         <v>54.64</v>
       </c>
       <c r="N14" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="O14" t="n">
-        <v>55.31914893617022</v>
+        <v>57.44680851063831</v>
       </c>
       <c r="P14" t="n">
-        <v>40.91982978723404</v>
+        <v>49.34536170212766</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
       </c>
       <c r="R14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S14" t="b">
         <v>0</v>
@@ -1624,48 +1624,48 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>101.15</v>
+        <v>95.70999999999999</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.1271895763223746</v>
+        <v>-0.1321969353522533</v>
       </c>
       <c r="E15" t="n">
-        <v>0.1275220153829006</v>
+        <v>-0.0096233443708609</v>
       </c>
       <c r="F15" t="n">
-        <v>0.1401036970243463</v>
+        <v>0.0413447938200413</v>
       </c>
       <c r="G15" t="n">
-        <v>0.0051389493235003</v>
+        <v>0.0619174351580155</v>
       </c>
       <c r="H15" t="n">
-        <v>0.1439719032932331</v>
+        <v>0.0961845255621335</v>
       </c>
       <c r="I15" t="n">
-        <v>36.4294710327456</v>
+        <v>41.2743823146944</v>
       </c>
       <c r="J15" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K15" t="n">
         <v>51.91</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M15" t="n">
         <v>51.91</v>
       </c>
       <c r="N15" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O15" t="n">
-        <v>65.95744680851064</v>
+        <v>70.21276595744681</v>
       </c>
       <c r="P15" t="n">
-        <v>45.95548936170212</v>
+        <v>50.80655319148936</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
@@ -1689,54 +1689,54 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>176.48</v>
+        <v>158.74</v>
       </c>
       <c r="D16" t="n">
-        <v>0.1158320687910976</v>
+        <v>-0.2123257083312657</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.0170983013088277</v>
+        <v>-0.0942082738944364</v>
       </c>
       <c r="F16" t="n">
-        <v>0.618637072365404</v>
+        <v>-0.07741485528304071</v>
       </c>
       <c r="G16" t="n">
-        <v>0.483672324664558</v>
+        <v>-0.0568422139450665</v>
       </c>
       <c r="H16" t="n">
-        <v>0.6225052786342908</v>
+        <v>-0.0225751235409484</v>
       </c>
       <c r="I16" t="n">
-        <v>55.20238191035647</v>
+        <v>35.63903520931521</v>
       </c>
       <c r="J16" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="K16" t="n">
         <v>52.61</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M16" t="n">
         <v>52.61</v>
       </c>
       <c r="N16" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="O16" t="n">
-        <v>93.61702127659576</v>
+        <v>51.06382978723404</v>
       </c>
       <c r="P16" t="n">
-        <v>63.76740425531915</v>
+        <v>43.2567659574468</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>
       </c>
       <c r="R16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S16" t="b">
         <v>0</v>
@@ -1754,48 +1754,48 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>7458</v>
+        <v>7049</v>
       </c>
       <c r="D17" t="n">
-        <v>-0.0497547302032235</v>
+        <v>-0.1198651517043326</v>
       </c>
       <c r="E17" t="n">
-        <v>0.1119725659758461</v>
+        <v>-0.0075325589581133</v>
       </c>
       <c r="F17" t="n">
-        <v>0.083854090975149</v>
+        <v>0.0117697717812543</v>
       </c>
       <c r="G17" t="n">
-        <v>-0.0511106567256969</v>
+        <v>0.0323424131192285</v>
       </c>
       <c r="H17" t="n">
-        <v>0.08772229724403589</v>
+        <v>0.0666095035233466</v>
       </c>
       <c r="I17" t="n">
-        <v>41.21840570317563</v>
+        <v>38.97757122651041</v>
       </c>
       <c r="J17" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K17" t="n">
         <v>54.65</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M17" t="n">
         <v>54.65</v>
       </c>
       <c r="N17" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O17" t="n">
-        <v>57.44680851063831</v>
+        <v>65.95744680851064</v>
       </c>
       <c r="P17" t="n">
-        <v>49.34936170212766</v>
+        <v>47.05148936170213</v>
       </c>
       <c r="Q17" t="b">
         <v>0</v>
@@ -1819,48 +1819,48 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>721.05</v>
+        <v>697.65</v>
       </c>
       <c r="D18" t="n">
-        <v>0.152942117045091</v>
+        <v>-0.0896457232335095</v>
       </c>
       <c r="E18" t="n">
-        <v>0.1205998912114381</v>
+        <v>0.1612983770287139</v>
       </c>
       <c r="F18" t="n">
-        <v>0.1096491228070175</v>
+        <v>0.0669062547790182</v>
       </c>
       <c r="G18" t="n">
-        <v>-0.0253156248938284</v>
+        <v>0.0874788961169924</v>
       </c>
       <c r="H18" t="n">
-        <v>0.1135173290759044</v>
+        <v>0.1217459865211104</v>
       </c>
       <c r="I18" t="n">
-        <v>46.48203592814371</v>
+        <v>49.20332525112573</v>
       </c>
       <c r="J18" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K18" t="n">
         <v>49.92</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M18" t="n">
         <v>49.92</v>
       </c>
       <c r="N18" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O18" t="n">
-        <v>63.82978723404256</v>
+        <v>72.3404255319149</v>
       </c>
       <c r="P18" t="n">
-        <v>64.73395744680852</v>
+        <v>58.43608510638298</v>
       </c>
       <c r="Q18" t="b">
         <v>0</v>
@@ -1884,48 +1884,48 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2451.8</v>
+        <v>2333.1</v>
       </c>
       <c r="D19" t="n">
-        <v>0.0021253985122211</v>
+        <v>-0.0867778299671208</v>
       </c>
       <c r="E19" t="n">
-        <v>-0.0624450307827615</v>
+        <v>-0.1225648740127868</v>
       </c>
       <c r="F19" t="n">
-        <v>-0.0231872509960158</v>
+        <v>-0.1985779060181368</v>
       </c>
       <c r="G19" t="n">
-        <v>-0.1581519986968618</v>
+        <v>-0.1780052646801626</v>
       </c>
       <c r="H19" t="n">
-        <v>-0.0193190447271289</v>
+        <v>-0.1437381742760446</v>
       </c>
       <c r="I19" t="n">
-        <v>47.42038216560513</v>
+        <v>35.89414595028067</v>
       </c>
       <c r="J19" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K19" t="n">
         <v>51.27</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M19" t="n">
         <v>51.27</v>
       </c>
       <c r="N19" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O19" t="n">
-        <v>38.29787234042553</v>
+        <v>21.27659574468085</v>
       </c>
       <c r="P19" t="n">
-        <v>44.16757446808511</v>
+        <v>36.76331914893618</v>
       </c>
       <c r="Q19" t="b">
         <v>0</v>
@@ -1949,48 +1949,48 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2094.7</v>
+        <v>2083.6</v>
       </c>
       <c r="D20" t="n">
-        <v>-0.1003307133960401</v>
+        <v>-0.0729667200569496</v>
       </c>
       <c r="E20" t="n">
-        <v>-0.09527922947350249</v>
+        <v>-0.07535280021301149</v>
       </c>
       <c r="F20" t="n">
-        <v>0.1576765778711173</v>
+        <v>-0.0492790655229056</v>
       </c>
       <c r="G20" t="n">
-        <v>0.0227118301702713</v>
+        <v>-0.0287064241849314</v>
       </c>
       <c r="H20" t="n">
-        <v>0.1615447841400041</v>
+        <v>0.0055606662191866</v>
       </c>
       <c r="I20" t="n">
-        <v>26.98985343855693</v>
+        <v>46.00603897886356</v>
       </c>
       <c r="J20" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="K20" t="n">
         <v>49.06</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M20" t="n">
         <v>49.06</v>
       </c>
       <c r="N20" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="O20" t="n">
-        <v>68.08510638297872</v>
+        <v>59.57446808510638</v>
       </c>
       <c r="P20" t="n">
-        <v>41.24102127659575</v>
+        <v>47.53889361702128</v>
       </c>
       <c r="Q20" t="b">
         <v>0</v>
@@ -2014,48 +2014,48 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>916.25</v>
+        <v>881.25</v>
       </c>
       <c r="D21" t="n">
-        <v>-0.0543399731654453</v>
+        <v>-0.09355070973050809</v>
       </c>
       <c r="E21" t="n">
-        <v>-0.0671451842801873</v>
+        <v>-0.081265638031693</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.1401557807807807</v>
+        <v>-0.3033596837944664</v>
       </c>
       <c r="G21" t="n">
-        <v>-0.2751205284816267</v>
+        <v>-0.2827870424564922</v>
       </c>
       <c r="H21" t="n">
-        <v>-0.1362875745118938</v>
+        <v>-0.2485199520523742</v>
       </c>
       <c r="I21" t="n">
-        <v>35.76557345235786</v>
+        <v>41.35438182354677</v>
       </c>
       <c r="J21" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K21" t="n">
         <v>48.43</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M21" t="n">
         <v>48.43</v>
       </c>
       <c r="N21" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O21" t="n">
-        <v>17.02127659574468</v>
+        <v>8.51063829787234</v>
       </c>
       <c r="P21" t="n">
-        <v>34.77625531914894</v>
+        <v>37.07412765957447</v>
       </c>
       <c r="Q21" t="b">
         <v>0</v>
@@ -2079,48 +2079,48 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>426.25</v>
+        <v>396.15</v>
       </c>
       <c r="D22" t="n">
-        <v>0.0248857898533301</v>
+        <v>-0.0439242186557259</v>
       </c>
       <c r="E22" t="n">
-        <v>0.3633455941148249</v>
+        <v>0.2727710843373494</v>
       </c>
       <c r="F22" t="n">
-        <v>0.4046795188663701</v>
+        <v>0.2610218048702848</v>
       </c>
       <c r="G22" t="n">
-        <v>0.2697147711655241</v>
+        <v>0.281594446208259</v>
       </c>
       <c r="H22" t="n">
-        <v>0.4085477251352569</v>
+        <v>0.315861536612377</v>
       </c>
       <c r="I22" t="n">
-        <v>47.02058504875406</v>
+        <v>39.38129996524157</v>
       </c>
       <c r="J22" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="K22" t="n">
         <v>54.47</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M22" t="n">
         <v>54.47</v>
       </c>
       <c r="N22" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="O22" t="n">
-        <v>85.1063829787234</v>
+        <v>91.48936170212764</v>
       </c>
       <c r="P22" t="n">
-        <v>62.80927659574468</v>
+        <v>52.08587234042552</v>
       </c>
       <c r="Q22" t="b">
         <v>0</v>
@@ -2144,25 +2144,25 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>362.05</v>
+        <v>335.15</v>
       </c>
       <c r="D23" t="n">
-        <v>-0.0888385554297219</v>
+        <v>-0.0921034809697954</v>
       </c>
       <c r="E23" t="n">
-        <v>-0.0819069354634208</v>
+        <v>-0.1009924892703864</v>
       </c>
       <c r="F23" t="n">
-        <v>-0.115980954706385</v>
+        <v>-0.1699071207430341</v>
       </c>
       <c r="G23" t="n">
-        <v>-0.250945702407231</v>
+        <v>-0.1493344794050599</v>
       </c>
       <c r="H23" t="n">
-        <v>-0.1121127484374981</v>
+        <v>-0.1150673890009419</v>
       </c>
       <c r="I23" t="n">
-        <v>34.79968578161827</v>
+        <v>31.39534883720927</v>
       </c>
       <c r="J23" t="n">
         <v>30</v>
@@ -2172,7 +2172,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M23" t="n">
@@ -2209,48 +2209,48 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>132.57</v>
+        <v>121.47</v>
       </c>
       <c r="D24" t="n">
-        <v>0.017968210089841</v>
+        <v>-0.1223900007224911</v>
       </c>
       <c r="E24" t="n">
-        <v>0.2102428336680664</v>
+        <v>-0.005159705159705</v>
       </c>
       <c r="F24" t="n">
-        <v>0.457293613279103</v>
+        <v>0.1259733036707453</v>
       </c>
       <c r="G24" t="n">
-        <v>0.322328865578257</v>
+        <v>0.1465459450087195</v>
       </c>
       <c r="H24" t="n">
-        <v>0.4611618195479898</v>
+        <v>0.1808130354128375</v>
       </c>
       <c r="I24" t="n">
-        <v>47.25532330533308</v>
+        <v>36.21378621378621</v>
       </c>
       <c r="J24" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="K24" t="n">
         <v>48.3</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M24" t="n">
         <v>48.3</v>
       </c>
       <c r="N24" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="O24" t="n">
-        <v>87.2340425531915</v>
+        <v>78.72340425531915</v>
       </c>
       <c r="P24" t="n">
-        <v>60.7668085106383</v>
+        <v>47.06468085106384</v>
       </c>
       <c r="Q24" t="b">
         <v>0</v>
@@ -2274,48 +2274,48 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>521.9</v>
+        <v>572.65</v>
       </c>
       <c r="D25" t="n">
-        <v>-0.1270385548214435</v>
+        <v>0.0089859924235751</v>
       </c>
       <c r="E25" t="n">
-        <v>-0.1726379201014584</v>
+        <v>-0.0294890263536987</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.1319028609447772</v>
+        <v>-0.0634557200098128</v>
       </c>
       <c r="G25" t="n">
-        <v>-0.2668676086456232</v>
+        <v>-0.0428830786718386</v>
       </c>
       <c r="H25" t="n">
-        <v>-0.1280346546758903</v>
+        <v>-0.0086159882677205</v>
       </c>
       <c r="I25" t="n">
-        <v>22.33890214797134</v>
+        <v>60.2561852956659</v>
       </c>
       <c r="J25" t="n">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="K25" t="n">
         <v>56.91</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M25" t="n">
         <v>56.91</v>
       </c>
       <c r="N25" t="n">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="O25" t="n">
-        <v>21.27659574468085</v>
+        <v>55.31914893617022</v>
       </c>
       <c r="P25" t="n">
-        <v>35.01931914893617</v>
+        <v>65.82782978723404</v>
       </c>
       <c r="Q25" t="b">
         <v>0</v>
@@ -2339,25 +2339,25 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>131.86</v>
+        <v>125.84</v>
       </c>
       <c r="D26" t="n">
-        <v>-0.0895532693502727</v>
+        <v>-0.0838005096468874</v>
       </c>
       <c r="E26" t="n">
-        <v>-0.166972013393139</v>
+        <v>-0.1233716475095786</v>
       </c>
       <c r="F26" t="n">
-        <v>0.0535314797059764</v>
+        <v>-0.0829993441667272</v>
       </c>
       <c r="G26" t="n">
-        <v>-0.0814332679948695</v>
+        <v>-0.062426702828753</v>
       </c>
       <c r="H26" t="n">
-        <v>0.0573996859748633</v>
+        <v>-0.028159612424635</v>
       </c>
       <c r="I26" t="n">
-        <v>42.57309941520469</v>
+        <v>41.5401600883246</v>
       </c>
       <c r="J26" t="n">
         <v>40</v>
@@ -2367,7 +2367,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M26" t="n">
@@ -2377,16 +2377,16 @@
         <v>40</v>
       </c>
       <c r="O26" t="n">
-        <v>53.19148936170212</v>
+        <v>48.93617021276596</v>
       </c>
       <c r="P26" t="n">
-        <v>47.25429787234042</v>
+        <v>46.4032340425532</v>
       </c>
       <c r="Q26" t="b">
         <v>0</v>
       </c>
       <c r="R26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S26" t="b">
         <v>0</v>
@@ -2404,48 +2404,48 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>5576.5</v>
+        <v>5148.5</v>
       </c>
       <c r="D27" t="n">
-        <v>0.0538599640933572</v>
+        <v>-0.1565781498288092</v>
       </c>
       <c r="E27" t="n">
-        <v>0.0908219553225617</v>
+        <v>-0.09189522885616019</v>
       </c>
       <c r="F27" t="n">
-        <v>0.6683120923831749</v>
+        <v>0.2336759878273788</v>
       </c>
       <c r="G27" t="n">
-        <v>0.5333473446823289</v>
+        <v>0.254248629165353</v>
       </c>
       <c r="H27" t="n">
-        <v>0.6721802986520617</v>
+        <v>0.2885157195694711</v>
       </c>
       <c r="I27" t="n">
-        <v>33.83625351503353</v>
+        <v>38.56340288924559</v>
       </c>
       <c r="J27" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="K27" t="n">
         <v>57.69</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M27" t="n">
         <v>57.69</v>
       </c>
       <c r="N27" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="O27" t="n">
-        <v>95.74468085106383</v>
+        <v>89.36170212765957</v>
       </c>
       <c r="P27" t="n">
-        <v>62.22493617021277</v>
+        <v>52.94834042553191</v>
       </c>
       <c r="Q27" t="b">
         <v>0</v>
@@ -2469,48 +2469,48 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1531.9</v>
+        <v>1623.3</v>
       </c>
       <c r="D28" t="n">
-        <v>0.0025523560209423</v>
+        <v>-0.0232264275828871</v>
       </c>
       <c r="E28" t="n">
-        <v>0.1208751006073023</v>
+        <v>0.06459863588667369</v>
       </c>
       <c r="F28" t="n">
-        <v>0.4965806955842127</v>
+        <v>0.4412678682411435</v>
       </c>
       <c r="G28" t="n">
-        <v>0.3616159478833667</v>
+        <v>0.4618405095791177</v>
       </c>
       <c r="H28" t="n">
-        <v>0.5004489018530995</v>
+        <v>0.4961075999832357</v>
       </c>
       <c r="I28" t="n">
-        <v>42.36420670298829</v>
+        <v>57.3173835581573</v>
       </c>
       <c r="J28" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="K28" t="n">
         <v>54.51</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M28" t="n">
         <v>54.51</v>
       </c>
       <c r="N28" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="O28" t="n">
-        <v>91.48936170212764</v>
+        <v>93.61702127659576</v>
       </c>
       <c r="P28" t="n">
-        <v>56.10187234042553</v>
+        <v>72.52740425531915</v>
       </c>
       <c r="Q28" t="b">
         <v>0</v>
@@ -2534,48 +2534,48 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>520.95</v>
+        <v>543.95</v>
       </c>
       <c r="D29" t="n">
-        <v>-0.1048969072164948</v>
+        <v>-0.0612649926654585</v>
       </c>
       <c r="E29" t="n">
-        <v>-0.1248215035699285</v>
+        <v>-0.071995223065768</v>
       </c>
       <c r="F29" t="n">
-        <v>0.1052296594887027</v>
+        <v>0.0716115051221435</v>
       </c>
       <c r="G29" t="n">
-        <v>-0.0297350882121432</v>
+        <v>0.0921841464601177</v>
       </c>
       <c r="H29" t="n">
-        <v>0.1090978657575896</v>
+        <v>0.1264512368642357</v>
       </c>
       <c r="I29" t="n">
-        <v>16.60164716081491</v>
+        <v>54.80591497227357</v>
       </c>
       <c r="J29" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="K29" t="n">
         <v>49.42</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M29" t="n">
         <v>49.42</v>
       </c>
       <c r="N29" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="O29" t="n">
-        <v>61.70212765957447</v>
+        <v>74.46808510638297</v>
       </c>
       <c r="P29" t="n">
-        <v>40.1084255319149</v>
+        <v>58.6616170212766</v>
       </c>
       <c r="Q29" t="b">
         <v>0</v>
@@ -2599,25 +2599,25 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>117.49</v>
+        <v>111.94</v>
       </c>
       <c r="D30" t="n">
-        <v>-0.0227083679920147</v>
+        <v>-0.0594067725401227</v>
       </c>
       <c r="E30" t="n">
-        <v>0.0174937213128951</v>
+        <v>0.0506851886615355</v>
       </c>
       <c r="F30" t="n">
-        <v>-0.1167493609983462</v>
+        <v>-0.1103163249085995</v>
       </c>
       <c r="G30" t="n">
-        <v>-0.2517141086991922</v>
+        <v>-0.0897436835706253</v>
       </c>
       <c r="H30" t="n">
-        <v>-0.1128811547294593</v>
+        <v>-0.0554765931665073</v>
       </c>
       <c r="I30" t="n">
-        <v>48.87186036611323</v>
+        <v>41.92680301399354</v>
       </c>
       <c r="J30" t="n">
         <v>40</v>
@@ -2627,7 +2627,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M30" t="n">
@@ -2637,10 +2637,10 @@
         <v>40</v>
       </c>
       <c r="O30" t="n">
-        <v>23.40425531914894</v>
+        <v>44.68085106382978</v>
       </c>
       <c r="P30" t="n">
-        <v>41.63285106382978</v>
+        <v>45.88817021276596</v>
       </c>
       <c r="Q30" t="b">
         <v>0</v>
@@ -2664,25 +2664,25 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>41.27</v>
+        <v>37.98</v>
       </c>
       <c r="D31" t="n">
-        <v>-0.0901675485008817</v>
+        <v>-0.1459410838767709</v>
       </c>
       <c r="E31" t="n">
-        <v>-0.1476662536142089</v>
+        <v>-0.1671052631578948</v>
       </c>
       <c r="F31" t="n">
-        <v>0.0900686740623351</v>
+        <v>-0.1167441860465117</v>
       </c>
       <c r="G31" t="n">
-        <v>-0.0448960736385108</v>
+        <v>-0.0961715447085375</v>
       </c>
       <c r="H31" t="n">
-        <v>0.0939368803312219</v>
+        <v>-0.0619044543044194</v>
       </c>
       <c r="I31" t="n">
-        <v>37.97468354430387</v>
+        <v>30.71120689655172</v>
       </c>
       <c r="J31" t="n">
         <v>30</v>
@@ -2692,7 +2692,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M31" t="n">
@@ -2702,16 +2702,16 @@
         <v>30</v>
       </c>
       <c r="O31" t="n">
-        <v>59.57446808510638</v>
+        <v>40.42553191489361</v>
       </c>
       <c r="P31" t="n">
-        <v>43.51089361702128</v>
+        <v>39.68110638297873</v>
       </c>
       <c r="Q31" t="b">
         <v>0</v>
       </c>
       <c r="R31" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S31" t="b">
         <v>0</v>
@@ -2729,25 +2729,25 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>717</v>
+        <v>686.55</v>
       </c>
       <c r="D32" t="n">
-        <v>-0.020759355367386</v>
+        <v>-0.1282458256618627</v>
       </c>
       <c r="E32" t="n">
-        <v>-0.1648223645894001</v>
+        <v>-0.1817531732316309</v>
       </c>
       <c r="F32" t="n">
-        <v>-0.2543289480526233</v>
+        <v>-0.3496732026143792</v>
       </c>
       <c r="G32" t="n">
-        <v>-0.3892936957534693</v>
+        <v>-0.3291005612764049</v>
       </c>
       <c r="H32" t="n">
-        <v>-0.2504607417837364</v>
+        <v>-0.2948334708722869</v>
       </c>
       <c r="I32" t="n">
-        <v>45.50706033376123</v>
+        <v>47.40046838407492</v>
       </c>
       <c r="J32" t="n">
         <v>40</v>
@@ -2757,7 +2757,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M32" t="n">
@@ -2767,10 +2767,10 @@
         <v>40</v>
       </c>
       <c r="O32" t="n">
-        <v>4.25531914893617</v>
+        <v>2.127659574468085</v>
       </c>
       <c r="P32" t="n">
-        <v>35.99506382978724</v>
+        <v>35.56953191489362</v>
       </c>
       <c r="Q32" t="b">
         <v>0</v>
@@ -2794,48 +2794,48 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>565.8</v>
+        <v>543.95</v>
       </c>
       <c r="D33" t="n">
-        <v>-0.0249870756505256</v>
+        <v>-0.1378189887462354</v>
       </c>
       <c r="E33" t="n">
-        <v>-0.1044634377967711</v>
+        <v>-0.0963535177340311</v>
       </c>
       <c r="F33" t="n">
-        <v>0.3165794066317626</v>
+        <v>0.1429922252574071</v>
       </c>
       <c r="G33" t="n">
-        <v>0.1816146589309166</v>
+        <v>0.1635648665953814</v>
       </c>
       <c r="H33" t="n">
-        <v>0.3204476129006495</v>
+        <v>0.1978319569994994</v>
       </c>
       <c r="I33" t="n">
-        <v>27.457514161946</v>
+        <v>44.98910675381264</v>
       </c>
       <c r="J33" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="K33" t="n">
         <v>49.98</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M33" t="n">
         <v>49.98</v>
       </c>
       <c r="N33" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="O33" t="n">
         <v>80.85106382978722</v>
       </c>
       <c r="P33" t="n">
-        <v>44.16221276595745</v>
+        <v>52.16221276595745</v>
       </c>
       <c r="Q33" t="b">
         <v>0</v>
@@ -2871,10 +2871,10 @@
         <v>-0.2401052253975846</v>
       </c>
       <c r="G34" t="n">
-        <v>-0.3750699730984306</v>
+        <v>-0.2195325840596104</v>
       </c>
       <c r="H34" t="n">
-        <v>-0.2362370191286977</v>
+        <v>-0.1852654936554923</v>
       </c>
       <c r="I34" t="n">
         <v>63.3225806451613</v>
@@ -2887,7 +2887,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M34" t="n">
@@ -2897,10 +2897,10 @@
         <v>80</v>
       </c>
       <c r="O34" t="n">
-        <v>6.382978723404255</v>
+        <v>17.02127659574468</v>
       </c>
       <c r="P34" t="n">
-        <v>53.62859574468086</v>
+        <v>55.75625531914894</v>
       </c>
       <c r="Q34" t="b">
         <v>0</v>
@@ -2924,48 +2924,48 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>113.3</v>
+        <v>109.14</v>
       </c>
       <c r="D35" t="n">
-        <v>-0.1335270724992352</v>
+        <v>-0.1325013909864081</v>
       </c>
       <c r="E35" t="n">
-        <v>0.0055915505458417</v>
+        <v>-0.0156038603770182</v>
       </c>
       <c r="F35" t="n">
-        <v>0.494525788154597</v>
+        <v>0.1063355296502788</v>
       </c>
       <c r="G35" t="n">
-        <v>0.359561040453751</v>
+        <v>0.126908170988253</v>
       </c>
       <c r="H35" t="n">
-        <v>0.4983939944234838</v>
+        <v>0.161175261392371</v>
       </c>
       <c r="I35" t="n">
-        <v>39.08828923238146</v>
+        <v>42.75874906924796</v>
       </c>
       <c r="J35" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K35" t="n">
         <v>49.07</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M35" t="n">
         <v>49.07</v>
       </c>
       <c r="N35" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O35" t="n">
-        <v>89.36170212765957</v>
+        <v>76.59574468085107</v>
       </c>
       <c r="P35" t="n">
-        <v>49.50034042553192</v>
+        <v>50.94714893617022</v>
       </c>
       <c r="Q35" t="b">
         <v>0</v>
@@ -2989,25 +2989,25 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>498.1</v>
+        <v>465</v>
       </c>
       <c r="D36" t="n">
-        <v>-0.0935395814376706</v>
+        <v>-0.0433083016150601</v>
       </c>
       <c r="E36" t="n">
-        <v>-0.09854311826983971</v>
+        <v>-0.1528511568591728</v>
       </c>
       <c r="F36" t="n">
-        <v>0.1943412060903968</v>
+        <v>0.028533510285335</v>
       </c>
       <c r="G36" t="n">
-        <v>0.0593764583895508</v>
+        <v>0.0491061516233092</v>
       </c>
       <c r="H36" t="n">
-        <v>0.1982094123592837</v>
+        <v>0.0833732420274272</v>
       </c>
       <c r="I36" t="n">
-        <v>36.03682595352917</v>
+        <v>33.50762527233114</v>
       </c>
       <c r="J36" t="n">
         <v>30</v>
@@ -3017,7 +3017,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M36" t="n">
@@ -3027,10 +3027,10 @@
         <v>30</v>
       </c>
       <c r="O36" t="n">
-        <v>72.3404255319149</v>
+        <v>68.08510638297872</v>
       </c>
       <c r="P36" t="n">
-        <v>45.58808510638298</v>
+        <v>44.73702127659575</v>
       </c>
       <c r="Q36" t="b">
         <v>0</v>
@@ -3054,48 +3054,48 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2197.7</v>
+        <v>2183</v>
       </c>
       <c r="D37" t="n">
-        <v>0.1565016050097352</v>
+        <v>-0.06329113924050631</v>
       </c>
       <c r="E37" t="n">
-        <v>0.4207123925269893</v>
+        <v>0.3173616559048942</v>
       </c>
       <c r="F37" t="n">
-        <v>0.723821476194211</v>
+        <v>0.6919857386451713</v>
       </c>
       <c r="G37" t="n">
-        <v>0.588856728493365</v>
+        <v>0.7125583799831455</v>
       </c>
       <c r="H37" t="n">
-        <v>0.7276896824630978</v>
+        <v>0.7468254703872635</v>
       </c>
       <c r="I37" t="n">
-        <v>46.03960396039601</v>
+        <v>47.6534296028881</v>
       </c>
       <c r="J37" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K37" t="n">
         <v>48.59</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M37" t="n">
         <v>48.59</v>
       </c>
       <c r="N37" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O37" t="n">
         <v>100</v>
       </c>
       <c r="P37" t="n">
-        <v>63.43600000000001</v>
+        <v>71.43600000000001</v>
       </c>
       <c r="Q37" t="b">
         <v>0</v>
@@ -3119,48 +3119,48 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>830.85</v>
+        <v>795.15</v>
       </c>
       <c r="D38" t="n">
-        <v>-0.0958210904342148</v>
+        <v>-0.182659197204091</v>
       </c>
       <c r="E38" t="n">
-        <v>-0.1528853996737357</v>
+        <v>-0.1828271928472329</v>
       </c>
       <c r="F38" t="n">
-        <v>-0.2015664039976935</v>
+        <v>-0.2431467732724157</v>
       </c>
       <c r="G38" t="n">
-        <v>-0.3365311516985395</v>
+        <v>-0.2225741319344415</v>
       </c>
       <c r="H38" t="n">
-        <v>-0.1976981977288067</v>
+        <v>-0.1883070415303235</v>
       </c>
       <c r="I38" t="n">
-        <v>29.82805429864254</v>
+        <v>41.92412357931806</v>
       </c>
       <c r="J38" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="K38" t="n">
         <v>49.87</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M38" t="n">
         <v>49.87</v>
       </c>
       <c r="N38" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="O38" t="n">
-        <v>10.63829787234042</v>
+        <v>14.8936170212766</v>
       </c>
       <c r="P38" t="n">
-        <v>30.07565957446808</v>
+        <v>38.92672340425532</v>
       </c>
       <c r="Q38" t="b">
         <v>0</v>
@@ -3184,48 +3184,48 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>2928.7</v>
+        <v>3102.1</v>
       </c>
       <c r="D39" t="n">
-        <v>-0.058204971540663</v>
+        <v>0.008747398543184201</v>
       </c>
       <c r="E39" t="n">
-        <v>0.07400344713777519</v>
+        <v>0.0930970083512456</v>
       </c>
       <c r="F39" t="n">
-        <v>0.2043837644446271</v>
+        <v>0.2254483684917436</v>
       </c>
       <c r="G39" t="n">
-        <v>0.06941901674378111</v>
+        <v>0.2460210098297178</v>
       </c>
       <c r="H39" t="n">
-        <v>0.2082519707135139</v>
+        <v>0.2802881002338359</v>
       </c>
       <c r="I39" t="n">
-        <v>39.47118644067795</v>
+        <v>53.98535417546823</v>
       </c>
       <c r="J39" t="n">
-        <v>30</v>
+        <v>80</v>
       </c>
       <c r="K39" t="n">
         <v>48.69</v>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M39" t="n">
         <v>48.69</v>
       </c>
       <c r="N39" t="n">
-        <v>30</v>
+        <v>80</v>
       </c>
       <c r="O39" t="n">
-        <v>74.46808510638297</v>
+        <v>87.2340425531915</v>
       </c>
       <c r="P39" t="n">
-        <v>46.3696170212766</v>
+        <v>68.9228085106383</v>
       </c>
       <c r="Q39" t="b">
         <v>0</v>
@@ -3249,48 +3249,48 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>195.74</v>
+        <v>185.82</v>
       </c>
       <c r="D40" t="n">
-        <v>-0.09892740413386721</v>
+        <v>-0.1464792614027835</v>
       </c>
       <c r="E40" t="n">
-        <v>-0.0484200291686921</v>
+        <v>-0.0304706250652196</v>
       </c>
       <c r="F40" t="n">
-        <v>-0.0883092687470888</v>
+        <v>-0.1755257786848877</v>
       </c>
       <c r="G40" t="n">
-        <v>-0.2232740164479348</v>
+        <v>-0.1549531373469135</v>
       </c>
       <c r="H40" t="n">
-        <v>-0.084441062478202</v>
+        <v>-0.1206860469427955</v>
       </c>
       <c r="I40" t="n">
-        <v>22.19707879037237</v>
+        <v>40.83181542197934</v>
       </c>
       <c r="J40" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="K40" t="n">
         <v>45.44</v>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M40" t="n">
         <v>45.44</v>
       </c>
       <c r="N40" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="O40" t="n">
-        <v>31.91489361702128</v>
+        <v>23.40425531914894</v>
       </c>
       <c r="P40" t="n">
-        <v>32.55897872340425</v>
+        <v>38.85685106382979</v>
       </c>
       <c r="Q40" t="b">
         <v>0</v>
@@ -3314,25 +3314,25 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>848.4</v>
+        <v>799</v>
       </c>
       <c r="D41" t="n">
-        <v>-0.1073232323232323</v>
+        <v>-0.138776610078146</v>
       </c>
       <c r="E41" t="n">
-        <v>-0.1384615384615385</v>
+        <v>-0.1522096662952942</v>
       </c>
       <c r="F41" t="n">
-        <v>-0.1003658342611738</v>
+        <v>-0.2199550912818509</v>
       </c>
       <c r="G41" t="n">
-        <v>-0.2353305819620198</v>
+        <v>-0.1993824499438767</v>
       </c>
       <c r="H41" t="n">
-        <v>-0.09649762799228701</v>
+        <v>-0.1651153595397587</v>
       </c>
       <c r="I41" t="n">
-        <v>26.14439324116745</v>
+        <v>27.5675675675676</v>
       </c>
       <c r="J41" t="n">
         <v>20</v>
@@ -3342,7 +3342,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M41" t="n">
@@ -3352,10 +3352,10 @@
         <v>20</v>
       </c>
       <c r="O41" t="n">
-        <v>27.65957446808511</v>
+        <v>19.14893617021277</v>
       </c>
       <c r="P41" t="n">
-        <v>32.75191489361702</v>
+        <v>31.04978723404255</v>
       </c>
       <c r="Q41" t="b">
         <v>0</v>
@@ -3379,48 +3379,48 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>594.75</v>
+        <v>525.55</v>
       </c>
       <c r="D42" t="n">
-        <v>0.0123404255319148</v>
+        <v>-0.2231911905993644</v>
       </c>
       <c r="E42" t="n">
-        <v>-0.2108405758641278</v>
+        <v>-0.2653760134190662</v>
       </c>
       <c r="F42" t="n">
-        <v>-0.2394501278772378</v>
+        <v>-0.3267358442223931</v>
       </c>
       <c r="G42" t="n">
-        <v>-0.3744148755780838</v>
+        <v>-0.3061632028844189</v>
       </c>
       <c r="H42" t="n">
-        <v>-0.235581921608351</v>
+        <v>-0.2718961124803009</v>
       </c>
       <c r="I42" t="n">
-        <v>40.33149171270718</v>
+        <v>38.38383838383837</v>
       </c>
       <c r="J42" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K42" t="n">
         <v>47.66</v>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M42" t="n">
         <v>47.66</v>
       </c>
       <c r="N42" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O42" t="n">
-        <v>8.51063829787234</v>
+        <v>4.25531914893617</v>
       </c>
       <c r="P42" t="n">
-        <v>36.76612765957447</v>
+        <v>31.91506382978724</v>
       </c>
       <c r="Q42" t="b">
         <v>0</v>
@@ -3444,25 +3444,25 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>425.35</v>
+        <v>410.45</v>
       </c>
       <c r="D43" t="n">
-        <v>-0.10168954593453</v>
+        <v>-0.0178272313950705</v>
       </c>
       <c r="E43" t="n">
-        <v>-0.0951925122314401</v>
+        <v>-0.1063575005443066</v>
       </c>
       <c r="F43" t="n">
-        <v>-0.0346118928733545</v>
+        <v>-0.1105211832267851</v>
       </c>
       <c r="G43" t="n">
-        <v>-0.1695766405742005</v>
+        <v>-0.08994854188881091</v>
       </c>
       <c r="H43" t="n">
-        <v>-0.0307436866044676</v>
+        <v>-0.0556814514846929</v>
       </c>
       <c r="I43" t="n">
-        <v>45.54455445544556</v>
+        <v>40.36970781156825</v>
       </c>
       <c r="J43" t="n">
         <v>40</v>
@@ -3472,7 +3472,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M43" t="n">
@@ -3482,10 +3482,10 @@
         <v>40</v>
       </c>
       <c r="O43" t="n">
-        <v>36.17021276595745</v>
+        <v>42.5531914893617</v>
       </c>
       <c r="P43" t="n">
-        <v>43.82604255319149</v>
+        <v>45.10263829787234</v>
       </c>
       <c r="Q43" t="b">
         <v>0</v>
@@ -3509,48 +3509,48 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>240.95</v>
+        <v>238.9</v>
       </c>
       <c r="D44" t="n">
-        <v>-0.0987469609126614</v>
+        <v>-0.1361417465196167</v>
       </c>
       <c r="E44" t="n">
-        <v>-0.1448092280390417</v>
+        <v>-0.1623422159887797</v>
       </c>
       <c r="F44" t="n">
-        <v>-0.061903834923107</v>
+        <v>-0.0979799886728337</v>
       </c>
       <c r="G44" t="n">
-        <v>-0.196868582623953</v>
+        <v>-0.0774073473348595</v>
       </c>
       <c r="H44" t="n">
-        <v>-0.0580356286542201</v>
+        <v>-0.0431402569307415</v>
       </c>
       <c r="I44" t="n">
-        <v>19.35714285714286</v>
+        <v>46.77242888402625</v>
       </c>
       <c r="J44" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="K44" t="n">
         <v>47.2</v>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M44" t="n">
         <v>47.2</v>
       </c>
       <c r="N44" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="O44" t="n">
-        <v>34.04255319148936</v>
+        <v>46.80851063829788</v>
       </c>
       <c r="P44" t="n">
-        <v>33.68851063829788</v>
+        <v>44.24170212765958</v>
       </c>
       <c r="Q44" t="b">
         <v>0</v>
@@ -3574,48 +3574,48 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>100.25</v>
+        <v>92.33</v>
       </c>
       <c r="D45" t="n">
-        <v>-0.1127533410036285</v>
+        <v>-0.1465939550790276</v>
       </c>
       <c r="E45" t="n">
-        <v>-0.1929640959587828</v>
+        <v>-0.1683480453972257</v>
       </c>
       <c r="F45" t="n">
-        <v>-0.299147091722595</v>
+        <v>-0.316074074074074</v>
       </c>
       <c r="G45" t="n">
-        <v>-0.434111839423441</v>
+        <v>-0.2955014327360998</v>
       </c>
       <c r="H45" t="n">
-        <v>-0.2952788854537082</v>
+        <v>-0.2612343423319818</v>
       </c>
       <c r="I45" t="n">
-        <v>19.27570093457948</v>
+        <v>31.15942028985505</v>
       </c>
       <c r="J45" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="K45" t="n">
         <v>59.6</v>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M45" t="n">
         <v>59.6</v>
       </c>
       <c r="N45" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="O45" t="n">
-        <v>2.127659574468085</v>
+        <v>6.382978723404255</v>
       </c>
       <c r="P45" t="n">
-        <v>32.26553191489362</v>
+        <v>37.11659574468086</v>
       </c>
       <c r="Q45" t="b">
         <v>0</v>
@@ -3639,48 +3639,48 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>514.65</v>
+        <v>493.4</v>
       </c>
       <c r="D46" t="n">
-        <v>-0.1616712819677471</v>
+        <v>-0.1059164628069222</v>
       </c>
       <c r="E46" t="n">
-        <v>-0.1933385579937304</v>
+        <v>-0.2267669644256387</v>
       </c>
       <c r="F46" t="n">
-        <v>-0.0096218608678918</v>
+        <v>-0.1265710745264648</v>
       </c>
       <c r="G46" t="n">
-        <v>-0.1445866085687378</v>
+        <v>-0.1059984331884906</v>
       </c>
       <c r="H46" t="n">
-        <v>-0.005753654599005</v>
+        <v>-0.0717313427843726</v>
       </c>
       <c r="I46" t="n">
-        <v>28.31991951710265</v>
+        <v>45.43721056932715</v>
       </c>
       <c r="J46" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="K46" t="n">
         <v>49.61</v>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M46" t="n">
         <v>49.61</v>
       </c>
       <c r="N46" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="O46" t="n">
-        <v>44.68085106382978</v>
+        <v>36.17021276595745</v>
       </c>
       <c r="P46" t="n">
-        <v>36.78017021276596</v>
+        <v>43.07804255319149</v>
       </c>
       <c r="Q46" t="b">
         <v>0</v>
@@ -3704,48 +3704,48 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>880.25</v>
+        <v>1089.55</v>
       </c>
       <c r="D47" t="n">
-        <v>0.0270096838175242</v>
+        <v>0.21276714158504</v>
       </c>
       <c r="E47" t="n">
-        <v>-0.0143329040927159</v>
+        <v>0.3153256473712802</v>
       </c>
       <c r="F47" t="n">
-        <v>0.2068138195777351</v>
+        <v>0.4779571351058056</v>
       </c>
       <c r="G47" t="n">
-        <v>0.0718490718768891</v>
+        <v>0.4985297764437798</v>
       </c>
       <c r="H47" t="n">
-        <v>0.210682025846622</v>
+        <v>0.5327968668478978</v>
       </c>
       <c r="I47" t="n">
-        <v>53.79574003276898</v>
+        <v>76.0805057411947</v>
       </c>
       <c r="J47" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K47" t="n">
         <v>46.83</v>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M47" t="n">
         <v>46.83</v>
       </c>
       <c r="N47" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O47" t="n">
-        <v>76.59574468085107</v>
+        <v>95.74468085106383</v>
       </c>
       <c r="P47" t="n">
-        <v>58.05114893617021</v>
+        <v>65.88093617021276</v>
       </c>
       <c r="Q47" t="b">
         <v>0</v>
@@ -3769,48 +3769,48 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>14376</v>
+        <v>13592</v>
       </c>
       <c r="D48" t="n">
-        <v>-0.0620473673908787</v>
+        <v>-0.1284386021160628</v>
       </c>
       <c r="E48" t="n">
-        <v>0.1381521653075765</v>
+        <v>-0.081187047928074</v>
       </c>
       <c r="F48" t="n">
-        <v>0.0445397079125191</v>
+        <v>-0.0421423537702607</v>
       </c>
       <c r="G48" t="n">
-        <v>-0.09042503978832681</v>
+        <v>-0.0215697124322865</v>
       </c>
       <c r="H48" t="n">
-        <v>0.048407914181406</v>
+        <v>0.0126973779718314</v>
       </c>
       <c r="I48" t="n">
-        <v>26.40127388535032</v>
+        <v>37.02397743300423</v>
       </c>
       <c r="J48" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="K48" t="n">
         <v>50.29</v>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M48" t="n">
         <v>50.29</v>
       </c>
       <c r="N48" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="O48" t="n">
-        <v>48.93617021276596</v>
+        <v>61.70212765957447</v>
       </c>
       <c r="P48" t="n">
-        <v>37.9032340425532</v>
+        <v>44.4564255319149</v>
       </c>
       <c r="Q48" t="b">
         <v>0</v>
@@ -3936,57 +3936,57 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>LUMAXTECH</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Forgings</t>
+          <t>Lighting</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1923.9</v>
+        <v>1623.3</v>
       </c>
       <c r="D2" t="n">
-        <v>0.2092394720301698</v>
+        <v>-0.0232264275828871</v>
       </c>
       <c r="E2" t="n">
-        <v>0.3775597880567092</v>
+        <v>0.06459863588667369</v>
       </c>
       <c r="F2" t="n">
-        <v>0.6694724054147865</v>
+        <v>0.4412678682411435</v>
       </c>
       <c r="G2" t="n">
-        <v>0.5345076577139405</v>
+        <v>0.4618405095791177</v>
       </c>
       <c r="H2" t="n">
-        <v>0.6733406116836733</v>
+        <v>0.4961075999832357</v>
       </c>
       <c r="I2" t="n">
-        <v>74.69975980784629</v>
+        <v>57.3173835581573</v>
       </c>
       <c r="J2" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K2" t="n">
-        <v>54.83</v>
+        <v>54.51</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M2" t="n">
-        <v>54.83</v>
+        <v>54.51</v>
       </c>
       <c r="N2" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O2" t="n">
-        <v>97.87234042553192</v>
+        <v>93.61702127659576</v>
       </c>
       <c r="P2" t="n">
-        <v>69.50646808510639</v>
+        <v>72.52740425531915</v>
       </c>
       <c r="Q2" t="b">
         <v>0</v>
@@ -4001,57 +4001,57 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DIVGIITTS</t>
+          <t>SANSERA</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Transmission</t>
+          <t>Forgings</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>721.05</v>
+        <v>2183</v>
       </c>
       <c r="D3" t="n">
-        <v>0.152942117045091</v>
+        <v>-0.06329113924050631</v>
       </c>
       <c r="E3" t="n">
-        <v>0.1205998912114381</v>
+        <v>0.3173616559048942</v>
       </c>
       <c r="F3" t="n">
-        <v>0.1096491228070175</v>
+        <v>0.6919857386451713</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.0253156248938284</v>
+        <v>0.7125583799831455</v>
       </c>
       <c r="H3" t="n">
-        <v>0.1135173290759044</v>
+        <v>0.7468254703872635</v>
       </c>
       <c r="I3" t="n">
-        <v>46.48203592814371</v>
+        <v>47.6534296028881</v>
       </c>
       <c r="J3" t="n">
         <v>80</v>
       </c>
       <c r="K3" t="n">
-        <v>49.92</v>
+        <v>48.59</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M3" t="n">
-        <v>49.92</v>
+        <v>48.59</v>
       </c>
       <c r="N3" t="n">
         <v>80</v>
       </c>
       <c r="O3" t="n">
-        <v>63.82978723404256</v>
+        <v>100</v>
       </c>
       <c r="P3" t="n">
-        <v>64.73395744680852</v>
+        <v>71.43600000000001</v>
       </c>
       <c r="Q3" t="b">
         <v>0</v>
@@ -4066,57 +4066,57 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BHARATSE</t>
+          <t>SHRIPISTON</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Seating</t>
+          <t>Engine/Parts</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>176.48</v>
+        <v>3102.1</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1158320687910976</v>
+        <v>0.008747398543184201</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.0170983013088277</v>
+        <v>0.0930970083512456</v>
       </c>
       <c r="F4" t="n">
-        <v>0.618637072365404</v>
+        <v>0.2254483684917436</v>
       </c>
       <c r="G4" t="n">
-        <v>0.483672324664558</v>
+        <v>0.2460210098297178</v>
       </c>
       <c r="H4" t="n">
-        <v>0.6225052786342908</v>
+        <v>0.2802881002338359</v>
       </c>
       <c r="I4" t="n">
-        <v>55.20238191035647</v>
+        <v>53.98535417546823</v>
       </c>
       <c r="J4" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K4" t="n">
-        <v>52.61</v>
+        <v>48.69</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M4" t="n">
-        <v>52.61</v>
+        <v>48.69</v>
       </c>
       <c r="N4" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O4" t="n">
-        <v>93.61702127659576</v>
+        <v>87.2340425531915</v>
       </c>
       <c r="P4" t="n">
-        <v>63.76740425531915</v>
+        <v>68.9228085106383</v>
       </c>
       <c r="Q4" t="b">
         <v>0</v>
@@ -4131,57 +4131,57 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SANSERA</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Forgings</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>2197.7</v>
+        <v>511.45</v>
       </c>
       <c r="D5" t="n">
-        <v>0.1565016050097352</v>
+        <v>-0.045891241488667</v>
       </c>
       <c r="E5" t="n">
-        <v>0.4207123925269893</v>
+        <v>0.0377396773866287</v>
       </c>
       <c r="F5" t="n">
-        <v>0.723821476194211</v>
+        <v>0.1494549949432519</v>
       </c>
       <c r="G5" t="n">
-        <v>0.588856728493365</v>
+        <v>0.1700276362812262</v>
       </c>
       <c r="H5" t="n">
-        <v>0.7276896824630978</v>
+        <v>0.2042947266853442</v>
       </c>
       <c r="I5" t="n">
-        <v>46.03960396039601</v>
+        <v>50.15782828282829</v>
       </c>
       <c r="J5" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K5" t="n">
-        <v>48.59</v>
+        <v>49.66</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M5" t="n">
-        <v>48.59</v>
+        <v>49.66</v>
       </c>
       <c r="N5" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O5" t="n">
-        <v>100</v>
+        <v>82.97872340425532</v>
       </c>
       <c r="P5" t="n">
-        <v>63.43600000000001</v>
+        <v>68.45974468085107</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
@@ -4196,63 +4196,63 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AUTOAXLES</t>
+          <t>ASKAUTOLTD</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Axles</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1987</v>
+        <v>444.15</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.0579813208173328</v>
+        <v>0.0255137381667049</v>
       </c>
       <c r="E6" t="n">
-        <v>0.2024933430162188</v>
+        <v>-0.0730460189919649</v>
       </c>
       <c r="F6" t="n">
-        <v>0.2149932738168032</v>
+        <v>-0.1285195722554694</v>
       </c>
       <c r="G6" t="n">
-        <v>0.0800285261159572</v>
+        <v>-0.1079469309174951</v>
       </c>
       <c r="H6" t="n">
-        <v>0.21886148008569</v>
+        <v>-0.0736798405133771</v>
       </c>
       <c r="I6" t="n">
-        <v>45.62982005141387</v>
+        <v>69.83381502890172</v>
       </c>
       <c r="J6" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K6" t="n">
-        <v>58.77</v>
+        <v>71.28</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M6" t="n">
-        <v>58.77</v>
+        <v>71.28</v>
       </c>
       <c r="N6" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O6" t="n">
-        <v>78.72340425531915</v>
+        <v>34.04255319148936</v>
       </c>
       <c r="P6" t="n">
-        <v>63.25268085106384</v>
+        <v>67.32051063829788</v>
       </c>
       <c r="Q6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S6" t="b">
         <v>0</v>
@@ -4261,57 +4261,57 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>GNA</t>
+          <t>WHEELS</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Axles</t>
+          <t>Wheels</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>426.25</v>
+        <v>1089.55</v>
       </c>
       <c r="D7" t="n">
-        <v>0.0248857898533301</v>
+        <v>0.21276714158504</v>
       </c>
       <c r="E7" t="n">
-        <v>0.3633455941148249</v>
+        <v>0.3153256473712802</v>
       </c>
       <c r="F7" t="n">
-        <v>0.4046795188663701</v>
+        <v>0.4779571351058056</v>
       </c>
       <c r="G7" t="n">
-        <v>0.2697147711655241</v>
+        <v>0.4985297764437798</v>
       </c>
       <c r="H7" t="n">
-        <v>0.4085477251352569</v>
+        <v>0.5327968668478978</v>
       </c>
       <c r="I7" t="n">
-        <v>47.02058504875406</v>
+        <v>76.0805057411947</v>
       </c>
       <c r="J7" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K7" t="n">
-        <v>54.47</v>
+        <v>46.83</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M7" t="n">
-        <v>54.47</v>
+        <v>46.83</v>
       </c>
       <c r="N7" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O7" t="n">
-        <v>85.1063829787234</v>
+        <v>95.74468085106383</v>
       </c>
       <c r="P7" t="n">
-        <v>62.80927659574468</v>
+        <v>65.88093617021276</v>
       </c>
       <c r="Q7" t="b">
         <v>0</v>
@@ -4326,63 +4326,63 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>LUMAXIND</t>
+          <t>JBMA</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Lighting</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>5576.5</v>
+        <v>572.65</v>
       </c>
       <c r="D8" t="n">
-        <v>0.0538599640933572</v>
+        <v>0.0089859924235751</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0908219553225617</v>
+        <v>-0.0294890263536987</v>
       </c>
       <c r="F8" t="n">
-        <v>0.6683120923831749</v>
+        <v>-0.0634557200098128</v>
       </c>
       <c r="G8" t="n">
-        <v>0.5333473446823289</v>
+        <v>-0.0428830786718386</v>
       </c>
       <c r="H8" t="n">
-        <v>0.6721802986520617</v>
+        <v>-0.0086159882677205</v>
       </c>
       <c r="I8" t="n">
-        <v>33.83625351503353</v>
+        <v>60.2561852956659</v>
       </c>
       <c r="J8" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="K8" t="n">
-        <v>57.69</v>
+        <v>56.91</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M8" t="n">
-        <v>57.69</v>
+        <v>56.91</v>
       </c>
       <c r="N8" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="O8" t="n">
-        <v>95.74468085106383</v>
+        <v>55.31914893617022</v>
       </c>
       <c r="P8" t="n">
-        <v>62.22493617021277</v>
+        <v>65.82782978723404</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
       </c>
       <c r="R8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S8" t="b">
         <v>0</v>
@@ -4391,57 +4391,57 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>JAMNAAUTO</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Suspension</t>
+          <t>Forgings</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>132.57</v>
+        <v>1736.5</v>
       </c>
       <c r="D9" t="n">
-        <v>0.017968210089841</v>
+        <v>-0.0521288209606987</v>
       </c>
       <c r="E9" t="n">
-        <v>0.2102428336680664</v>
+        <v>0.2350640113798008</v>
       </c>
       <c r="F9" t="n">
-        <v>0.457293613279103</v>
+        <v>0.5304953287502205</v>
       </c>
       <c r="G9" t="n">
-        <v>0.322328865578257</v>
+        <v>0.5510679700881947</v>
       </c>
       <c r="H9" t="n">
-        <v>0.4611618195479898</v>
+        <v>0.5853350604923128</v>
       </c>
       <c r="I9" t="n">
-        <v>47.25532330533308</v>
+        <v>37.49420670477369</v>
       </c>
       <c r="J9" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="K9" t="n">
-        <v>48.3</v>
+        <v>54.83</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M9" t="n">
-        <v>48.3</v>
+        <v>54.83</v>
       </c>
       <c r="N9" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="O9" t="n">
-        <v>87.2340425531915</v>
+        <v>97.87234042553192</v>
       </c>
       <c r="P9" t="n">
-        <v>60.7668085106383</v>
+        <v>61.50646808510639</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -4456,63 +4456,63 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>WHEELS</t>
+          <t>TIINDIA</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Wheels</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>880.25</v>
+        <v>2682.4</v>
       </c>
       <c r="D10" t="n">
-        <v>0.0270096838175242</v>
+        <v>0.0562293274531422</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.0143329040927159</v>
+        <v>0.0058874264071699</v>
       </c>
       <c r="F10" t="n">
-        <v>0.2068138195777351</v>
+        <v>-0.1198031173092698</v>
       </c>
       <c r="G10" t="n">
-        <v>0.0718490718768891</v>
+        <v>-0.0992304759712956</v>
       </c>
       <c r="H10" t="n">
-        <v>0.210682025846622</v>
+        <v>-0.0649633855671776</v>
       </c>
       <c r="I10" t="n">
-        <v>53.79574003276898</v>
+        <v>44.36388353914127</v>
       </c>
       <c r="J10" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K10" t="n">
-        <v>46.83</v>
+        <v>48.73</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M10" t="n">
-        <v>46.83</v>
+        <v>48.73</v>
       </c>
       <c r="N10" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O10" t="n">
-        <v>76.59574468085107</v>
+        <v>38.29787234042553</v>
       </c>
       <c r="P10" t="n">
-        <v>58.05114893617021</v>
+        <v>59.15157446808512</v>
       </c>
       <c r="Q10" t="b">
         <v>0</v>
       </c>
       <c r="R10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S10" t="b">
         <v>0</v>
@@ -4521,7 +4521,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>MINDACORP</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -4530,48 +4530,48 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>514.95</v>
+        <v>543.95</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.033592943605142</v>
+        <v>-0.0612649926654585</v>
       </c>
       <c r="E11" t="n">
-        <v>0.0540374577832361</v>
+        <v>-0.071995223065768</v>
       </c>
       <c r="F11" t="n">
-        <v>0.1696763202725724</v>
+        <v>0.0716115051221435</v>
       </c>
       <c r="G11" t="n">
-        <v>0.0347115725717264</v>
+        <v>0.0921841464601177</v>
       </c>
       <c r="H11" t="n">
-        <v>0.1735445265414592</v>
+        <v>0.1264512368642357</v>
       </c>
       <c r="I11" t="n">
-        <v>43.58341559723593</v>
+        <v>54.80591497227357</v>
       </c>
       <c r="J11" t="n">
         <v>60</v>
       </c>
       <c r="K11" t="n">
-        <v>49.66</v>
+        <v>49.42</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M11" t="n">
-        <v>49.66</v>
+        <v>49.42</v>
       </c>
       <c r="N11" t="n">
         <v>60</v>
       </c>
       <c r="O11" t="n">
-        <v>70.21276595744681</v>
+        <v>74.46808510638297</v>
       </c>
       <c r="P11" t="n">
-        <v>57.90655319148937</v>
+        <v>58.6616170212766</v>
       </c>
       <c r="Q11" t="b">
         <v>0</v>
@@ -4586,63 +4586,63 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TIINDIA</t>
+          <t>DIVGIITTS</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Transmission</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>2722.9</v>
+        <v>697.65</v>
       </c>
       <c r="D12" t="n">
-        <v>0.0324182907408812</v>
+        <v>-0.0896457232335095</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.1018570439027607</v>
+        <v>0.1612983770287139</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.098884733759142</v>
+        <v>0.0669062547790182</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.233849481459988</v>
+        <v>0.0874788961169924</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.0950165274902552</v>
+        <v>0.1217459865211104</v>
       </c>
       <c r="I12" t="n">
-        <v>67.22469666717861</v>
+        <v>49.20332525112573</v>
       </c>
       <c r="J12" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K12" t="n">
-        <v>48.73</v>
+        <v>49.92</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M12" t="n">
-        <v>48.73</v>
+        <v>49.92</v>
       </c>
       <c r="N12" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O12" t="n">
-        <v>29.78723404255319</v>
+        <v>72.3404255319149</v>
       </c>
       <c r="P12" t="n">
-        <v>57.44944680851064</v>
+        <v>58.43608510638298</v>
       </c>
       <c r="Q12" t="b">
         <v>0</v>
       </c>
       <c r="R12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S12" t="b">
         <v>0</v>
@@ -4651,63 +4651,63 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MOTHERSON</t>
+          <t>RANEENGINE</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Engine/Parts</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>122.77</v>
+        <v>317.75</v>
       </c>
       <c r="D13" t="n">
-        <v>0.0012232914695806</v>
+        <v>0.1790352504638219</v>
       </c>
       <c r="E13" t="n">
-        <v>0.1267437591776798</v>
+        <v>-0.156154561147258</v>
       </c>
       <c r="F13" t="n">
-        <v>0.3600310180569404</v>
+        <v>-0.2401052253975846</v>
       </c>
       <c r="G13" t="n">
-        <v>0.2250662703560944</v>
+        <v>-0.2195325840596104</v>
       </c>
       <c r="H13" t="n">
-        <v>0.3638992243258272</v>
+        <v>-0.1852654936554923</v>
       </c>
       <c r="I13" t="n">
-        <v>36.94247923715782</v>
+        <v>63.3225806451613</v>
       </c>
       <c r="J13" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="K13" t="n">
-        <v>51.57</v>
+        <v>50.88</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M13" t="n">
-        <v>51.57</v>
+        <v>50.88</v>
       </c>
       <c r="N13" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="O13" t="n">
-        <v>82.97872340425532</v>
+        <v>17.02127659574468</v>
       </c>
       <c r="P13" t="n">
-        <v>57.22374468085107</v>
+        <v>55.75625531914894</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
       </c>
       <c r="R13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S13" t="b">
         <v>0</v>
@@ -4716,7 +4716,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>LUMAXTECH</t>
+          <t>LUMAXIND</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -4725,48 +4725,48 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1531.9</v>
+        <v>5148.5</v>
       </c>
       <c r="D14" t="n">
-        <v>0.0025523560209423</v>
+        <v>-0.1565781498288092</v>
       </c>
       <c r="E14" t="n">
-        <v>0.1208751006073023</v>
+        <v>-0.09189522885616019</v>
       </c>
       <c r="F14" t="n">
-        <v>0.4965806955842127</v>
+        <v>0.2336759878273788</v>
       </c>
       <c r="G14" t="n">
-        <v>0.3616159478833667</v>
+        <v>0.254248629165353</v>
       </c>
       <c r="H14" t="n">
-        <v>0.5004489018530995</v>
+        <v>0.2885157195694711</v>
       </c>
       <c r="I14" t="n">
-        <v>42.36420670298829</v>
+        <v>38.56340288924559</v>
       </c>
       <c r="J14" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K14" t="n">
-        <v>54.51</v>
+        <v>57.69</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M14" t="n">
-        <v>54.51</v>
+        <v>57.69</v>
       </c>
       <c r="N14" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O14" t="n">
-        <v>91.48936170212764</v>
+        <v>89.36170212765957</v>
       </c>
       <c r="P14" t="n">
-        <v>56.10187234042553</v>
+        <v>52.94834042553191</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
@@ -4781,63 +4781,63 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>RANEENGINE</t>
+          <t>PRICOLLTD</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Engine/Parts</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>317.75</v>
+        <v>543.95</v>
       </c>
       <c r="D15" t="n">
-        <v>0.1790352504638219</v>
+        <v>-0.1378189887462354</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.156154561147258</v>
+        <v>-0.0963535177340311</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.2401052253975846</v>
+        <v>0.1429922252574071</v>
       </c>
       <c r="G15" t="n">
-        <v>-0.3750699730984306</v>
+        <v>0.1635648665953814</v>
       </c>
       <c r="H15" t="n">
-        <v>-0.2362370191286977</v>
+        <v>0.1978319569994994</v>
       </c>
       <c r="I15" t="n">
-        <v>63.3225806451613</v>
+        <v>44.98910675381264</v>
       </c>
       <c r="J15" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="K15" t="n">
-        <v>50.88</v>
+        <v>49.98</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M15" t="n">
-        <v>50.88</v>
+        <v>49.98</v>
       </c>
       <c r="N15" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="O15" t="n">
-        <v>6.382978723404255</v>
+        <v>80.85106382978722</v>
       </c>
       <c r="P15" t="n">
-        <v>53.62859574468086</v>
+        <v>52.16221276595745</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
       </c>
       <c r="R15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S15" t="b">
         <v>0</v>
@@ -4846,57 +4846,57 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>RICOAUTO</t>
+          <t>GNA</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Castings</t>
+          <t>Axles</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>113.3</v>
+        <v>396.15</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.1335270724992352</v>
+        <v>-0.0439242186557259</v>
       </c>
       <c r="E16" t="n">
-        <v>0.0055915505458417</v>
+        <v>0.2727710843373494</v>
       </c>
       <c r="F16" t="n">
-        <v>0.494525788154597</v>
+        <v>0.2610218048702848</v>
       </c>
       <c r="G16" t="n">
-        <v>0.359561040453751</v>
+        <v>0.281594446208259</v>
       </c>
       <c r="H16" t="n">
-        <v>0.4983939944234838</v>
+        <v>0.315861536612377</v>
       </c>
       <c r="I16" t="n">
-        <v>39.08828923238146</v>
+        <v>39.38129996524157</v>
       </c>
       <c r="J16" t="n">
         <v>30</v>
       </c>
       <c r="K16" t="n">
-        <v>49.07</v>
+        <v>54.47</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M16" t="n">
-        <v>49.07</v>
+        <v>54.47</v>
       </c>
       <c r="N16" t="n">
         <v>30</v>
       </c>
       <c r="O16" t="n">
-        <v>89.36170212765957</v>
+        <v>91.48936170212764</v>
       </c>
       <c r="P16" t="n">
-        <v>49.50034042553192</v>
+        <v>52.08587234042552</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>
@@ -4919,7 +4919,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5368,6 +5368,25 @@
       </c>
       <c r="E26" t="n">
         <v>0.1735265188095714</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2025-02-11</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>6</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0.06729471111296829</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0.0542595245326515</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.0130351865803167</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: pipeline outputs refreshed with Mar 25 data (local run)
Data as of 2026-03-25 — new top pick LUMAXTECH (composite 72.5, tech score 80,
RS +49.6% vs Nifty500); SANSERA #2 at 71.4; ASKAUTOLTD enters shortlist
with highest fund score (71.3) in universe.

https://claude.ai/code/session_01D6UEzdFERzfpopPdoSiiyt
</commit_message>
<xml_diff>
--- a/working-sector/output/auto_components_comprehensive_report.xlsx
+++ b/working-sector/output/auto_components_comprehensive_report.xlsx
@@ -447,7 +447,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
     </row>
@@ -779,48 +779,48 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1923.9</v>
+        <v>1736.5</v>
       </c>
       <c r="D2" t="n">
-        <v>0.2092394720301698</v>
+        <v>-0.0521288209606987</v>
       </c>
       <c r="E2" t="n">
-        <v>0.3775597880567092</v>
+        <v>0.2350640113798008</v>
       </c>
       <c r="F2" t="n">
-        <v>0.6694724054147865</v>
+        <v>0.5304953287502205</v>
       </c>
       <c r="G2" t="n">
-        <v>0.5345076577139405</v>
+        <v>0.5510679700881947</v>
       </c>
       <c r="H2" t="n">
-        <v>0.6733406116836733</v>
+        <v>0.5853350604923128</v>
       </c>
       <c r="I2" t="n">
-        <v>74.69975980784629</v>
+        <v>37.49420670477369</v>
       </c>
       <c r="J2" t="n">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="K2" t="n">
         <v>54.83</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M2" t="n">
         <v>54.83</v>
       </c>
       <c r="N2" t="n">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="O2" t="n">
         <v>97.87234042553192</v>
       </c>
       <c r="P2" t="n">
-        <v>69.50646808510639</v>
+        <v>61.50646808510639</v>
       </c>
       <c r="Q2" t="b">
         <v>0</v>
@@ -844,54 +844,54 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1121.3</v>
+        <v>1087.6</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.0693061088977423</v>
+        <v>-0.0906354515050168</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.1323222162036679</v>
+        <v>-0.1452373467463062</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0485318870394613</v>
+        <v>-0.1691367456073339</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.0864328606613846</v>
+        <v>-0.1485641042693597</v>
       </c>
       <c r="H3" t="n">
-        <v>0.0524000933083481</v>
+        <v>-0.1142970138652417</v>
       </c>
       <c r="I3" t="n">
-        <v>25.05083367222446</v>
+        <v>46.095141185449</v>
       </c>
       <c r="J3" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="K3" t="n">
         <v>49.36</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M3" t="n">
         <v>49.36</v>
       </c>
       <c r="N3" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="O3" t="n">
-        <v>51.06382978723404</v>
+        <v>27.65957446808511</v>
       </c>
       <c r="P3" t="n">
-        <v>37.95676595744681</v>
+        <v>41.27591489361702</v>
       </c>
       <c r="Q3" t="b">
         <v>0</v>
       </c>
       <c r="R3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S3" t="b">
         <v>0</v>
@@ -909,25 +909,25 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>33335</v>
+        <v>30390</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.0919368019613184</v>
+        <v>-0.1400679117147708</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.1001484680793629</v>
+        <v>-0.1768689057421452</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.1366226366226366</v>
+        <v>-0.2644318044293839</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.2715873843234826</v>
+        <v>-0.2438591630914097</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.1327544303537497</v>
+        <v>-0.2095920726872917</v>
       </c>
       <c r="I4" t="n">
-        <v>32.36173393124065</v>
+        <v>33.62168396770474</v>
       </c>
       <c r="J4" t="n">
         <v>30</v>
@@ -937,7 +937,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M4" t="n">
@@ -947,10 +947,10 @@
         <v>30</v>
       </c>
       <c r="O4" t="n">
-        <v>19.14893617021277</v>
+        <v>10.63829787234042</v>
       </c>
       <c r="P4" t="n">
-        <v>37.22178723404255</v>
+        <v>35.51965957446808</v>
       </c>
       <c r="Q4" t="b">
         <v>0</v>
@@ -974,48 +974,48 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>315.95</v>
+        <v>307.15</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.0748169838945828</v>
+        <v>-0.0923463356973995</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.1718217562254259</v>
+        <v>-0.1920294620544521</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.1606004250797024</v>
+        <v>-0.2620134550696781</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.2955651727805484</v>
+        <v>-0.2414408137317039</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.1567322188108155</v>
+        <v>-0.2071737233275858</v>
       </c>
       <c r="I5" t="n">
-        <v>32.66832917705733</v>
+        <v>43.0862831858407</v>
       </c>
       <c r="J5" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K5" t="n">
         <v>51.12</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M5" t="n">
         <v>51.12</v>
       </c>
       <c r="N5" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O5" t="n">
-        <v>14.8936170212766</v>
+        <v>12.76595744680851</v>
       </c>
       <c r="P5" t="n">
-        <v>35.42672340425532</v>
+        <v>39.0011914893617</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
@@ -1039,48 +1039,48 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>122.77</v>
+        <v>113.13</v>
       </c>
       <c r="D6" t="n">
-        <v>0.0012232914695806</v>
+        <v>-0.1352239718697446</v>
       </c>
       <c r="E6" t="n">
-        <v>0.1267437591776798</v>
+        <v>-0.033489961554891</v>
       </c>
       <c r="F6" t="n">
-        <v>0.3600310180569404</v>
+        <v>0.1726961749766766</v>
       </c>
       <c r="G6" t="n">
-        <v>0.2250662703560944</v>
+        <v>0.1932688163146508</v>
       </c>
       <c r="H6" t="n">
-        <v>0.3638992243258272</v>
+        <v>0.2275359067187689</v>
       </c>
       <c r="I6" t="n">
-        <v>36.94247923715782</v>
+        <v>35.66312133709572</v>
       </c>
       <c r="J6" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="K6" t="n">
         <v>51.57</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M6" t="n">
         <v>51.57</v>
       </c>
       <c r="N6" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="O6" t="n">
-        <v>82.97872340425532</v>
+        <v>85.1063829787234</v>
       </c>
       <c r="P6" t="n">
-        <v>57.22374468085107</v>
+        <v>49.64927659574468</v>
       </c>
       <c r="Q6" t="b">
         <v>0</v>
@@ -1104,25 +1104,25 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2722.9</v>
+        <v>2682.4</v>
       </c>
       <c r="D7" t="n">
-        <v>0.0324182907408812</v>
+        <v>0.0562293274531422</v>
       </c>
       <c r="E7" t="n">
-        <v>-0.1018570439027607</v>
+        <v>0.0058874264071699</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.098884733759142</v>
+        <v>-0.1198031173092698</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.233849481459988</v>
+        <v>-0.0992304759712956</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.0950165274902552</v>
+        <v>-0.0649633855671776</v>
       </c>
       <c r="I7" t="n">
-        <v>67.22469666717861</v>
+        <v>44.36388353914127</v>
       </c>
       <c r="J7" t="n">
         <v>80</v>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M7" t="n">
@@ -1142,10 +1142,10 @@
         <v>80</v>
       </c>
       <c r="O7" t="n">
-        <v>29.78723404255319</v>
+        <v>38.29787234042553</v>
       </c>
       <c r="P7" t="n">
-        <v>57.44944680851064</v>
+        <v>59.15157446808512</v>
       </c>
       <c r="Q7" t="b">
         <v>0</v>
@@ -1169,48 +1169,48 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>514.95</v>
+        <v>511.45</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.033592943605142</v>
+        <v>-0.045891241488667</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0540374577832361</v>
+        <v>0.0377396773866287</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1696763202725724</v>
+        <v>0.1494549949432519</v>
       </c>
       <c r="G8" t="n">
-        <v>0.0347115725717264</v>
+        <v>0.1700276362812262</v>
       </c>
       <c r="H8" t="n">
-        <v>0.1735445265414592</v>
+        <v>0.2042947266853442</v>
       </c>
       <c r="I8" t="n">
-        <v>43.58341559723593</v>
+        <v>50.15782828282829</v>
       </c>
       <c r="J8" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K8" t="n">
         <v>49.66</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M8" t="n">
         <v>49.66</v>
       </c>
       <c r="N8" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O8" t="n">
-        <v>70.21276595744681</v>
+        <v>82.97872340425532</v>
       </c>
       <c r="P8" t="n">
-        <v>57.90655319148937</v>
+        <v>68.45974468085107</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
@@ -1234,48 +1234,48 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>439.75</v>
+        <v>419.65</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.142202282258851</v>
+        <v>-0.07464167585446529</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.1588561591430757</v>
+        <v>-0.1952248537731327</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.0154483376245382</v>
+        <v>-0.1397088970889709</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.1504130853253842</v>
+        <v>-0.1191362557509967</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.0115801313556513</v>
+        <v>-0.0848691653468787</v>
       </c>
       <c r="I9" t="n">
-        <v>23.87434554973822</v>
+        <v>40.15936254980078</v>
       </c>
       <c r="J9" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="K9" t="n">
         <v>53.44</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M9" t="n">
         <v>53.44</v>
       </c>
       <c r="N9" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="O9" t="n">
-        <v>40.42553191489361</v>
+        <v>31.91489361702128</v>
       </c>
       <c r="P9" t="n">
-        <v>37.46110638297873</v>
+        <v>43.75897872340426</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -1299,25 +1299,25 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>138780</v>
+        <v>129970</v>
       </c>
       <c r="D10" t="n">
-        <v>0.008282476024411499</v>
+        <v>-0.1083287596048299</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.1058565814058372</v>
+        <v>-0.1516872266823314</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.0124879923150816</v>
+        <v>-0.1554082594144978</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.1474527400159276</v>
+        <v>-0.1348356180765236</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.008619786046194801</v>
+        <v>-0.1005685276724056</v>
       </c>
       <c r="I10" t="n">
-        <v>32.46089515254762</v>
+        <v>33.76129339039468</v>
       </c>
       <c r="J10" t="n">
         <v>30</v>
@@ -1327,7 +1327,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M10" t="n">
@@ -1337,10 +1337,10 @@
         <v>30</v>
       </c>
       <c r="O10" t="n">
-        <v>42.5531914893617</v>
+        <v>29.78723404255319</v>
       </c>
       <c r="P10" t="n">
-        <v>40.27463829787234</v>
+        <v>37.72144680851064</v>
       </c>
       <c r="Q10" t="b">
         <v>0</v>
@@ -1376,10 +1376,10 @@
         <v>-0.0042030657656173</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.1391678134664633</v>
+        <v>0.0163695755723568</v>
       </c>
       <c r="H11" t="n">
-        <v>-0.0003348594967305</v>
+        <v>0.0506366659764748</v>
       </c>
       <c r="I11" t="n">
         <v>27.6054590570719</v>
@@ -1392,7 +1392,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M11" t="n">
@@ -1402,16 +1402,16 @@
         <v>20</v>
       </c>
       <c r="O11" t="n">
-        <v>46.80851063829788</v>
+        <v>63.82978723404256</v>
       </c>
       <c r="P11" t="n">
-        <v>21.36170212765958</v>
+        <v>24.76595744680852</v>
       </c>
       <c r="Q11" t="b">
         <v>0</v>
       </c>
       <c r="R11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S11" t="b">
         <v>0</v>
@@ -1429,48 +1429,48 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>391.85</v>
+        <v>444.15</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.1468539081210537</v>
+        <v>0.0255137381667049</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.1829649708090075</v>
+        <v>-0.0730460189919649</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.1688408102661999</v>
+        <v>-0.1285195722554694</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.3038055579670459</v>
+        <v>-0.1079469309174951</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.164972603997313</v>
+        <v>-0.0736798405133771</v>
       </c>
       <c r="I12" t="n">
-        <v>24.08242112041213</v>
+        <v>69.83381502890172</v>
       </c>
       <c r="J12" t="n">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="K12" t="n">
         <v>71.28</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M12" t="n">
         <v>71.28</v>
       </c>
       <c r="N12" t="n">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="O12" t="n">
-        <v>12.76595744680851</v>
+        <v>34.04255319148936</v>
       </c>
       <c r="P12" t="n">
-        <v>39.0651914893617</v>
+        <v>67.32051063829788</v>
       </c>
       <c r="Q12" t="b">
         <v>1</v>
@@ -1494,54 +1494,54 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1987</v>
+        <v>1650.4</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.0579813208173328</v>
+        <v>-0.1813085966565801</v>
       </c>
       <c r="E13" t="n">
-        <v>0.2024933430162188</v>
+        <v>-0.0945797673908271</v>
       </c>
       <c r="F13" t="n">
-        <v>0.2149932738168032</v>
+        <v>-0.0678865921156669</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0800285261159572</v>
+        <v>-0.0473139507776927</v>
       </c>
       <c r="H13" t="n">
-        <v>0.21886148008569</v>
+        <v>-0.0130468603735747</v>
       </c>
       <c r="I13" t="n">
-        <v>45.62982005141387</v>
+        <v>19.06348649596633</v>
       </c>
       <c r="J13" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="K13" t="n">
         <v>58.77</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M13" t="n">
         <v>58.77</v>
       </c>
       <c r="N13" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="O13" t="n">
-        <v>78.72340425531915</v>
+        <v>53.19148936170212</v>
       </c>
       <c r="P13" t="n">
-        <v>63.25268085106384</v>
+        <v>42.14629787234043</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
       </c>
       <c r="R13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S13" t="b">
         <v>0</v>
@@ -1559,54 +1559,54 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>581.9</v>
+        <v>560.75</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.09656885576773799</v>
+        <v>-0.1464342796255423</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.2519123224272033</v>
+        <v>-0.25008358408559</v>
       </c>
       <c r="F14" t="n">
-        <v>0.0775925925925926</v>
+        <v>-0.0585914547133383</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.0573721551082533</v>
+        <v>-0.0380188133753641</v>
       </c>
       <c r="H14" t="n">
-        <v>0.0814607988614795</v>
+        <v>-0.0037517229712461</v>
       </c>
       <c r="I14" t="n">
-        <v>20.58823529411769</v>
+        <v>44.04982772329711</v>
       </c>
       <c r="J14" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="K14" t="n">
         <v>54.64</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M14" t="n">
         <v>54.64</v>
       </c>
       <c r="N14" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="O14" t="n">
-        <v>55.31914893617022</v>
+        <v>57.44680851063831</v>
       </c>
       <c r="P14" t="n">
-        <v>40.91982978723404</v>
+        <v>49.34536170212766</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
       </c>
       <c r="R14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S14" t="b">
         <v>0</v>
@@ -1624,48 +1624,48 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>101.15</v>
+        <v>95.70999999999999</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.1271895763223746</v>
+        <v>-0.1321969353522533</v>
       </c>
       <c r="E15" t="n">
-        <v>0.1275220153829006</v>
+        <v>-0.0096233443708609</v>
       </c>
       <c r="F15" t="n">
-        <v>0.1401036970243463</v>
+        <v>0.0413447938200413</v>
       </c>
       <c r="G15" t="n">
-        <v>0.0051389493235003</v>
+        <v>0.0619174351580155</v>
       </c>
       <c r="H15" t="n">
-        <v>0.1439719032932331</v>
+        <v>0.0961845255621335</v>
       </c>
       <c r="I15" t="n">
-        <v>36.4294710327456</v>
+        <v>41.2743823146944</v>
       </c>
       <c r="J15" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K15" t="n">
         <v>51.91</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M15" t="n">
         <v>51.91</v>
       </c>
       <c r="N15" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O15" t="n">
-        <v>65.95744680851064</v>
+        <v>70.21276595744681</v>
       </c>
       <c r="P15" t="n">
-        <v>45.95548936170212</v>
+        <v>50.80655319148936</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
@@ -1689,54 +1689,54 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>176.48</v>
+        <v>158.74</v>
       </c>
       <c r="D16" t="n">
-        <v>0.1158320687910976</v>
+        <v>-0.2123257083312657</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.0170983013088277</v>
+        <v>-0.0942082738944364</v>
       </c>
       <c r="F16" t="n">
-        <v>0.618637072365404</v>
+        <v>-0.07741485528304071</v>
       </c>
       <c r="G16" t="n">
-        <v>0.483672324664558</v>
+        <v>-0.0568422139450665</v>
       </c>
       <c r="H16" t="n">
-        <v>0.6225052786342908</v>
+        <v>-0.0225751235409484</v>
       </c>
       <c r="I16" t="n">
-        <v>55.20238191035647</v>
+        <v>35.63903520931521</v>
       </c>
       <c r="J16" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="K16" t="n">
         <v>52.61</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M16" t="n">
         <v>52.61</v>
       </c>
       <c r="N16" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="O16" t="n">
-        <v>93.61702127659576</v>
+        <v>51.06382978723404</v>
       </c>
       <c r="P16" t="n">
-        <v>63.76740425531915</v>
+        <v>43.2567659574468</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>
       </c>
       <c r="R16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S16" t="b">
         <v>0</v>
@@ -1754,48 +1754,48 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>7458</v>
+        <v>7049</v>
       </c>
       <c r="D17" t="n">
-        <v>-0.0497547302032235</v>
+        <v>-0.1198651517043326</v>
       </c>
       <c r="E17" t="n">
-        <v>0.1119725659758461</v>
+        <v>-0.0075325589581133</v>
       </c>
       <c r="F17" t="n">
-        <v>0.083854090975149</v>
+        <v>0.0117697717812543</v>
       </c>
       <c r="G17" t="n">
-        <v>-0.0511106567256969</v>
+        <v>0.0323424131192285</v>
       </c>
       <c r="H17" t="n">
-        <v>0.08772229724403589</v>
+        <v>0.0666095035233466</v>
       </c>
       <c r="I17" t="n">
-        <v>41.21840570317563</v>
+        <v>38.97757122651041</v>
       </c>
       <c r="J17" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K17" t="n">
         <v>54.65</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M17" t="n">
         <v>54.65</v>
       </c>
       <c r="N17" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O17" t="n">
-        <v>57.44680851063831</v>
+        <v>65.95744680851064</v>
       </c>
       <c r="P17" t="n">
-        <v>49.34936170212766</v>
+        <v>47.05148936170213</v>
       </c>
       <c r="Q17" t="b">
         <v>0</v>
@@ -1819,48 +1819,48 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>721.05</v>
+        <v>697.65</v>
       </c>
       <c r="D18" t="n">
-        <v>0.152942117045091</v>
+        <v>-0.0896457232335095</v>
       </c>
       <c r="E18" t="n">
-        <v>0.1205998912114381</v>
+        <v>0.1612983770287139</v>
       </c>
       <c r="F18" t="n">
-        <v>0.1096491228070175</v>
+        <v>0.0669062547790182</v>
       </c>
       <c r="G18" t="n">
-        <v>-0.0253156248938284</v>
+        <v>0.0874788961169924</v>
       </c>
       <c r="H18" t="n">
-        <v>0.1135173290759044</v>
+        <v>0.1217459865211104</v>
       </c>
       <c r="I18" t="n">
-        <v>46.48203592814371</v>
+        <v>49.20332525112573</v>
       </c>
       <c r="J18" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K18" t="n">
         <v>49.92</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M18" t="n">
         <v>49.92</v>
       </c>
       <c r="N18" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O18" t="n">
-        <v>63.82978723404256</v>
+        <v>72.3404255319149</v>
       </c>
       <c r="P18" t="n">
-        <v>64.73395744680852</v>
+        <v>58.43608510638298</v>
       </c>
       <c r="Q18" t="b">
         <v>0</v>
@@ -1884,48 +1884,48 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2451.8</v>
+        <v>2333.1</v>
       </c>
       <c r="D19" t="n">
-        <v>0.0021253985122211</v>
+        <v>-0.0867778299671208</v>
       </c>
       <c r="E19" t="n">
-        <v>-0.0624450307827615</v>
+        <v>-0.1225648740127868</v>
       </c>
       <c r="F19" t="n">
-        <v>-0.0231872509960158</v>
+        <v>-0.1985779060181368</v>
       </c>
       <c r="G19" t="n">
-        <v>-0.1581519986968618</v>
+        <v>-0.1780052646801626</v>
       </c>
       <c r="H19" t="n">
-        <v>-0.0193190447271289</v>
+        <v>-0.1437381742760446</v>
       </c>
       <c r="I19" t="n">
-        <v>47.42038216560513</v>
+        <v>35.89414595028067</v>
       </c>
       <c r="J19" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K19" t="n">
         <v>51.27</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M19" t="n">
         <v>51.27</v>
       </c>
       <c r="N19" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O19" t="n">
-        <v>38.29787234042553</v>
+        <v>21.27659574468085</v>
       </c>
       <c r="P19" t="n">
-        <v>44.16757446808511</v>
+        <v>36.76331914893618</v>
       </c>
       <c r="Q19" t="b">
         <v>0</v>
@@ -1949,48 +1949,48 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2094.7</v>
+        <v>2083.6</v>
       </c>
       <c r="D20" t="n">
-        <v>-0.1003307133960401</v>
+        <v>-0.0729667200569496</v>
       </c>
       <c r="E20" t="n">
-        <v>-0.09527922947350249</v>
+        <v>-0.07535280021301149</v>
       </c>
       <c r="F20" t="n">
-        <v>0.1576765778711173</v>
+        <v>-0.0492790655229056</v>
       </c>
       <c r="G20" t="n">
-        <v>0.0227118301702713</v>
+        <v>-0.0287064241849314</v>
       </c>
       <c r="H20" t="n">
-        <v>0.1615447841400041</v>
+        <v>0.0055606662191866</v>
       </c>
       <c r="I20" t="n">
-        <v>26.98985343855693</v>
+        <v>46.00603897886356</v>
       </c>
       <c r="J20" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="K20" t="n">
         <v>49.06</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M20" t="n">
         <v>49.06</v>
       </c>
       <c r="N20" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="O20" t="n">
-        <v>68.08510638297872</v>
+        <v>59.57446808510638</v>
       </c>
       <c r="P20" t="n">
-        <v>41.24102127659575</v>
+        <v>47.53889361702128</v>
       </c>
       <c r="Q20" t="b">
         <v>0</v>
@@ -2014,48 +2014,48 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>916.25</v>
+        <v>881.25</v>
       </c>
       <c r="D21" t="n">
-        <v>-0.0543399731654453</v>
+        <v>-0.09355070973050809</v>
       </c>
       <c r="E21" t="n">
-        <v>-0.0671451842801873</v>
+        <v>-0.081265638031693</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.1401557807807807</v>
+        <v>-0.3033596837944664</v>
       </c>
       <c r="G21" t="n">
-        <v>-0.2751205284816267</v>
+        <v>-0.2827870424564922</v>
       </c>
       <c r="H21" t="n">
-        <v>-0.1362875745118938</v>
+        <v>-0.2485199520523742</v>
       </c>
       <c r="I21" t="n">
-        <v>35.76557345235786</v>
+        <v>41.35438182354677</v>
       </c>
       <c r="J21" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K21" t="n">
         <v>48.43</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M21" t="n">
         <v>48.43</v>
       </c>
       <c r="N21" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O21" t="n">
-        <v>17.02127659574468</v>
+        <v>8.51063829787234</v>
       </c>
       <c r="P21" t="n">
-        <v>34.77625531914894</v>
+        <v>37.07412765957447</v>
       </c>
       <c r="Q21" t="b">
         <v>0</v>
@@ -2079,48 +2079,48 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>426.25</v>
+        <v>396.15</v>
       </c>
       <c r="D22" t="n">
-        <v>0.0248857898533301</v>
+        <v>-0.0439242186557259</v>
       </c>
       <c r="E22" t="n">
-        <v>0.3633455941148249</v>
+        <v>0.2727710843373494</v>
       </c>
       <c r="F22" t="n">
-        <v>0.4046795188663701</v>
+        <v>0.2610218048702848</v>
       </c>
       <c r="G22" t="n">
-        <v>0.2697147711655241</v>
+        <v>0.281594446208259</v>
       </c>
       <c r="H22" t="n">
-        <v>0.4085477251352569</v>
+        <v>0.315861536612377</v>
       </c>
       <c r="I22" t="n">
-        <v>47.02058504875406</v>
+        <v>39.38129996524157</v>
       </c>
       <c r="J22" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="K22" t="n">
         <v>54.47</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M22" t="n">
         <v>54.47</v>
       </c>
       <c r="N22" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="O22" t="n">
-        <v>85.1063829787234</v>
+        <v>91.48936170212764</v>
       </c>
       <c r="P22" t="n">
-        <v>62.80927659574468</v>
+        <v>52.08587234042552</v>
       </c>
       <c r="Q22" t="b">
         <v>0</v>
@@ -2144,25 +2144,25 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>362.05</v>
+        <v>335.15</v>
       </c>
       <c r="D23" t="n">
-        <v>-0.0888385554297219</v>
+        <v>-0.0921034809697954</v>
       </c>
       <c r="E23" t="n">
-        <v>-0.0819069354634208</v>
+        <v>-0.1009924892703864</v>
       </c>
       <c r="F23" t="n">
-        <v>-0.115980954706385</v>
+        <v>-0.1699071207430341</v>
       </c>
       <c r="G23" t="n">
-        <v>-0.250945702407231</v>
+        <v>-0.1493344794050599</v>
       </c>
       <c r="H23" t="n">
-        <v>-0.1121127484374981</v>
+        <v>-0.1150673890009419</v>
       </c>
       <c r="I23" t="n">
-        <v>34.79968578161827</v>
+        <v>31.39534883720927</v>
       </c>
       <c r="J23" t="n">
         <v>30</v>
@@ -2172,7 +2172,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M23" t="n">
@@ -2209,48 +2209,48 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>132.57</v>
+        <v>121.47</v>
       </c>
       <c r="D24" t="n">
-        <v>0.017968210089841</v>
+        <v>-0.1223900007224911</v>
       </c>
       <c r="E24" t="n">
-        <v>0.2102428336680664</v>
+        <v>-0.005159705159705</v>
       </c>
       <c r="F24" t="n">
-        <v>0.457293613279103</v>
+        <v>0.1259733036707453</v>
       </c>
       <c r="G24" t="n">
-        <v>0.322328865578257</v>
+        <v>0.1465459450087195</v>
       </c>
       <c r="H24" t="n">
-        <v>0.4611618195479898</v>
+        <v>0.1808130354128375</v>
       </c>
       <c r="I24" t="n">
-        <v>47.25532330533308</v>
+        <v>36.21378621378621</v>
       </c>
       <c r="J24" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="K24" t="n">
         <v>48.3</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M24" t="n">
         <v>48.3</v>
       </c>
       <c r="N24" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="O24" t="n">
-        <v>87.2340425531915</v>
+        <v>78.72340425531915</v>
       </c>
       <c r="P24" t="n">
-        <v>60.7668085106383</v>
+        <v>47.06468085106384</v>
       </c>
       <c r="Q24" t="b">
         <v>0</v>
@@ -2274,48 +2274,48 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>521.9</v>
+        <v>572.65</v>
       </c>
       <c r="D25" t="n">
-        <v>-0.1270385548214435</v>
+        <v>0.0089859924235751</v>
       </c>
       <c r="E25" t="n">
-        <v>-0.1726379201014584</v>
+        <v>-0.0294890263536987</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.1319028609447772</v>
+        <v>-0.0634557200098128</v>
       </c>
       <c r="G25" t="n">
-        <v>-0.2668676086456232</v>
+        <v>-0.0428830786718386</v>
       </c>
       <c r="H25" t="n">
-        <v>-0.1280346546758903</v>
+        <v>-0.0086159882677205</v>
       </c>
       <c r="I25" t="n">
-        <v>22.33890214797134</v>
+        <v>60.2561852956659</v>
       </c>
       <c r="J25" t="n">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="K25" t="n">
         <v>56.91</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M25" t="n">
         <v>56.91</v>
       </c>
       <c r="N25" t="n">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="O25" t="n">
-        <v>21.27659574468085</v>
+        <v>55.31914893617022</v>
       </c>
       <c r="P25" t="n">
-        <v>35.01931914893617</v>
+        <v>65.82782978723404</v>
       </c>
       <c r="Q25" t="b">
         <v>0</v>
@@ -2339,25 +2339,25 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>131.86</v>
+        <v>125.84</v>
       </c>
       <c r="D26" t="n">
-        <v>-0.0895532693502727</v>
+        <v>-0.0838005096468874</v>
       </c>
       <c r="E26" t="n">
-        <v>-0.166972013393139</v>
+        <v>-0.1233716475095786</v>
       </c>
       <c r="F26" t="n">
-        <v>0.0535314797059764</v>
+        <v>-0.0829993441667272</v>
       </c>
       <c r="G26" t="n">
-        <v>-0.0814332679948695</v>
+        <v>-0.062426702828753</v>
       </c>
       <c r="H26" t="n">
-        <v>0.0573996859748633</v>
+        <v>-0.028159612424635</v>
       </c>
       <c r="I26" t="n">
-        <v>42.57309941520469</v>
+        <v>41.5401600883246</v>
       </c>
       <c r="J26" t="n">
         <v>40</v>
@@ -2367,7 +2367,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M26" t="n">
@@ -2377,16 +2377,16 @@
         <v>40</v>
       </c>
       <c r="O26" t="n">
-        <v>53.19148936170212</v>
+        <v>48.93617021276596</v>
       </c>
       <c r="P26" t="n">
-        <v>47.25429787234042</v>
+        <v>46.4032340425532</v>
       </c>
       <c r="Q26" t="b">
         <v>0</v>
       </c>
       <c r="R26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S26" t="b">
         <v>0</v>
@@ -2404,48 +2404,48 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>5576.5</v>
+        <v>5148.5</v>
       </c>
       <c r="D27" t="n">
-        <v>0.0538599640933572</v>
+        <v>-0.1565781498288092</v>
       </c>
       <c r="E27" t="n">
-        <v>0.0908219553225617</v>
+        <v>-0.09189522885616019</v>
       </c>
       <c r="F27" t="n">
-        <v>0.6683120923831749</v>
+        <v>0.2336759878273788</v>
       </c>
       <c r="G27" t="n">
-        <v>0.5333473446823289</v>
+        <v>0.254248629165353</v>
       </c>
       <c r="H27" t="n">
-        <v>0.6721802986520617</v>
+        <v>0.2885157195694711</v>
       </c>
       <c r="I27" t="n">
-        <v>33.83625351503353</v>
+        <v>38.56340288924559</v>
       </c>
       <c r="J27" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="K27" t="n">
         <v>57.69</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M27" t="n">
         <v>57.69</v>
       </c>
       <c r="N27" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="O27" t="n">
-        <v>95.74468085106383</v>
+        <v>89.36170212765957</v>
       </c>
       <c r="P27" t="n">
-        <v>62.22493617021277</v>
+        <v>52.94834042553191</v>
       </c>
       <c r="Q27" t="b">
         <v>0</v>
@@ -2469,48 +2469,48 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1531.9</v>
+        <v>1623.3</v>
       </c>
       <c r="D28" t="n">
-        <v>0.0025523560209423</v>
+        <v>-0.0232264275828871</v>
       </c>
       <c r="E28" t="n">
-        <v>0.1208751006073023</v>
+        <v>0.06459863588667369</v>
       </c>
       <c r="F28" t="n">
-        <v>0.4965806955842127</v>
+        <v>0.4412678682411435</v>
       </c>
       <c r="G28" t="n">
-        <v>0.3616159478833667</v>
+        <v>0.4618405095791177</v>
       </c>
       <c r="H28" t="n">
-        <v>0.5004489018530995</v>
+        <v>0.4961075999832357</v>
       </c>
       <c r="I28" t="n">
-        <v>42.36420670298829</v>
+        <v>57.3173835581573</v>
       </c>
       <c r="J28" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="K28" t="n">
         <v>54.51</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M28" t="n">
         <v>54.51</v>
       </c>
       <c r="N28" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="O28" t="n">
-        <v>91.48936170212764</v>
+        <v>93.61702127659576</v>
       </c>
       <c r="P28" t="n">
-        <v>56.10187234042553</v>
+        <v>72.52740425531915</v>
       </c>
       <c r="Q28" t="b">
         <v>0</v>
@@ -2534,48 +2534,48 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>520.95</v>
+        <v>543.95</v>
       </c>
       <c r="D29" t="n">
-        <v>-0.1048969072164948</v>
+        <v>-0.0612649926654585</v>
       </c>
       <c r="E29" t="n">
-        <v>-0.1248215035699285</v>
+        <v>-0.071995223065768</v>
       </c>
       <c r="F29" t="n">
-        <v>0.1052296594887027</v>
+        <v>0.0716115051221435</v>
       </c>
       <c r="G29" t="n">
-        <v>-0.0297350882121432</v>
+        <v>0.0921841464601177</v>
       </c>
       <c r="H29" t="n">
-        <v>0.1090978657575896</v>
+        <v>0.1264512368642357</v>
       </c>
       <c r="I29" t="n">
-        <v>16.60164716081491</v>
+        <v>54.80591497227357</v>
       </c>
       <c r="J29" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="K29" t="n">
         <v>49.42</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M29" t="n">
         <v>49.42</v>
       </c>
       <c r="N29" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="O29" t="n">
-        <v>61.70212765957447</v>
+        <v>74.46808510638297</v>
       </c>
       <c r="P29" t="n">
-        <v>40.1084255319149</v>
+        <v>58.6616170212766</v>
       </c>
       <c r="Q29" t="b">
         <v>0</v>
@@ -2599,25 +2599,25 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>117.49</v>
+        <v>111.94</v>
       </c>
       <c r="D30" t="n">
-        <v>-0.0227083679920147</v>
+        <v>-0.0594067725401227</v>
       </c>
       <c r="E30" t="n">
-        <v>0.0174937213128951</v>
+        <v>0.0506851886615355</v>
       </c>
       <c r="F30" t="n">
-        <v>-0.1167493609983462</v>
+        <v>-0.1103163249085995</v>
       </c>
       <c r="G30" t="n">
-        <v>-0.2517141086991922</v>
+        <v>-0.0897436835706253</v>
       </c>
       <c r="H30" t="n">
-        <v>-0.1128811547294593</v>
+        <v>-0.0554765931665073</v>
       </c>
       <c r="I30" t="n">
-        <v>48.87186036611323</v>
+        <v>41.92680301399354</v>
       </c>
       <c r="J30" t="n">
         <v>40</v>
@@ -2627,7 +2627,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M30" t="n">
@@ -2637,10 +2637,10 @@
         <v>40</v>
       </c>
       <c r="O30" t="n">
-        <v>23.40425531914894</v>
+        <v>44.68085106382978</v>
       </c>
       <c r="P30" t="n">
-        <v>41.63285106382978</v>
+        <v>45.88817021276596</v>
       </c>
       <c r="Q30" t="b">
         <v>0</v>
@@ -2664,25 +2664,25 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>41.27</v>
+        <v>37.98</v>
       </c>
       <c r="D31" t="n">
-        <v>-0.0901675485008817</v>
+        <v>-0.1459410838767709</v>
       </c>
       <c r="E31" t="n">
-        <v>-0.1476662536142089</v>
+        <v>-0.1671052631578948</v>
       </c>
       <c r="F31" t="n">
-        <v>0.0900686740623351</v>
+        <v>-0.1167441860465117</v>
       </c>
       <c r="G31" t="n">
-        <v>-0.0448960736385108</v>
+        <v>-0.0961715447085375</v>
       </c>
       <c r="H31" t="n">
-        <v>0.0939368803312219</v>
+        <v>-0.0619044543044194</v>
       </c>
       <c r="I31" t="n">
-        <v>37.97468354430387</v>
+        <v>30.71120689655172</v>
       </c>
       <c r="J31" t="n">
         <v>30</v>
@@ -2692,7 +2692,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M31" t="n">
@@ -2702,16 +2702,16 @@
         <v>30</v>
       </c>
       <c r="O31" t="n">
-        <v>59.57446808510638</v>
+        <v>40.42553191489361</v>
       </c>
       <c r="P31" t="n">
-        <v>43.51089361702128</v>
+        <v>39.68110638297873</v>
       </c>
       <c r="Q31" t="b">
         <v>0</v>
       </c>
       <c r="R31" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S31" t="b">
         <v>0</v>
@@ -2729,25 +2729,25 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>717</v>
+        <v>686.55</v>
       </c>
       <c r="D32" t="n">
-        <v>-0.020759355367386</v>
+        <v>-0.1282458256618627</v>
       </c>
       <c r="E32" t="n">
-        <v>-0.1648223645894001</v>
+        <v>-0.1817531732316309</v>
       </c>
       <c r="F32" t="n">
-        <v>-0.2543289480526233</v>
+        <v>-0.3496732026143792</v>
       </c>
       <c r="G32" t="n">
-        <v>-0.3892936957534693</v>
+        <v>-0.3291005612764049</v>
       </c>
       <c r="H32" t="n">
-        <v>-0.2504607417837364</v>
+        <v>-0.2948334708722869</v>
       </c>
       <c r="I32" t="n">
-        <v>45.50706033376123</v>
+        <v>47.40046838407492</v>
       </c>
       <c r="J32" t="n">
         <v>40</v>
@@ -2757,7 +2757,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M32" t="n">
@@ -2767,10 +2767,10 @@
         <v>40</v>
       </c>
       <c r="O32" t="n">
-        <v>4.25531914893617</v>
+        <v>2.127659574468085</v>
       </c>
       <c r="P32" t="n">
-        <v>35.99506382978724</v>
+        <v>35.56953191489362</v>
       </c>
       <c r="Q32" t="b">
         <v>0</v>
@@ -2794,48 +2794,48 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>565.8</v>
+        <v>543.95</v>
       </c>
       <c r="D33" t="n">
-        <v>-0.0249870756505256</v>
+        <v>-0.1378189887462354</v>
       </c>
       <c r="E33" t="n">
-        <v>-0.1044634377967711</v>
+        <v>-0.0963535177340311</v>
       </c>
       <c r="F33" t="n">
-        <v>0.3165794066317626</v>
+        <v>0.1429922252574071</v>
       </c>
       <c r="G33" t="n">
-        <v>0.1816146589309166</v>
+        <v>0.1635648665953814</v>
       </c>
       <c r="H33" t="n">
-        <v>0.3204476129006495</v>
+        <v>0.1978319569994994</v>
       </c>
       <c r="I33" t="n">
-        <v>27.457514161946</v>
+        <v>44.98910675381264</v>
       </c>
       <c r="J33" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="K33" t="n">
         <v>49.98</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M33" t="n">
         <v>49.98</v>
       </c>
       <c r="N33" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="O33" t="n">
         <v>80.85106382978722</v>
       </c>
       <c r="P33" t="n">
-        <v>44.16221276595745</v>
+        <v>52.16221276595745</v>
       </c>
       <c r="Q33" t="b">
         <v>0</v>
@@ -2871,10 +2871,10 @@
         <v>-0.2401052253975846</v>
       </c>
       <c r="G34" t="n">
-        <v>-0.3750699730984306</v>
+        <v>-0.2195325840596104</v>
       </c>
       <c r="H34" t="n">
-        <v>-0.2362370191286977</v>
+        <v>-0.1852654936554923</v>
       </c>
       <c r="I34" t="n">
         <v>63.3225806451613</v>
@@ -2887,7 +2887,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M34" t="n">
@@ -2897,10 +2897,10 @@
         <v>80</v>
       </c>
       <c r="O34" t="n">
-        <v>6.382978723404255</v>
+        <v>17.02127659574468</v>
       </c>
       <c r="P34" t="n">
-        <v>53.62859574468086</v>
+        <v>55.75625531914894</v>
       </c>
       <c r="Q34" t="b">
         <v>0</v>
@@ -2924,48 +2924,48 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>113.3</v>
+        <v>109.14</v>
       </c>
       <c r="D35" t="n">
-        <v>-0.1335270724992352</v>
+        <v>-0.1325013909864081</v>
       </c>
       <c r="E35" t="n">
-        <v>0.0055915505458417</v>
+        <v>-0.0156038603770182</v>
       </c>
       <c r="F35" t="n">
-        <v>0.494525788154597</v>
+        <v>0.1063355296502788</v>
       </c>
       <c r="G35" t="n">
-        <v>0.359561040453751</v>
+        <v>0.126908170988253</v>
       </c>
       <c r="H35" t="n">
-        <v>0.4983939944234838</v>
+        <v>0.161175261392371</v>
       </c>
       <c r="I35" t="n">
-        <v>39.08828923238146</v>
+        <v>42.75874906924796</v>
       </c>
       <c r="J35" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K35" t="n">
         <v>49.07</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M35" t="n">
         <v>49.07</v>
       </c>
       <c r="N35" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O35" t="n">
-        <v>89.36170212765957</v>
+        <v>76.59574468085107</v>
       </c>
       <c r="P35" t="n">
-        <v>49.50034042553192</v>
+        <v>50.94714893617022</v>
       </c>
       <c r="Q35" t="b">
         <v>0</v>
@@ -2989,25 +2989,25 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>498.1</v>
+        <v>465</v>
       </c>
       <c r="D36" t="n">
-        <v>-0.0935395814376706</v>
+        <v>-0.0433083016150601</v>
       </c>
       <c r="E36" t="n">
-        <v>-0.09854311826983971</v>
+        <v>-0.1528511568591728</v>
       </c>
       <c r="F36" t="n">
-        <v>0.1943412060903968</v>
+        <v>0.028533510285335</v>
       </c>
       <c r="G36" t="n">
-        <v>0.0593764583895508</v>
+        <v>0.0491061516233092</v>
       </c>
       <c r="H36" t="n">
-        <v>0.1982094123592837</v>
+        <v>0.0833732420274272</v>
       </c>
       <c r="I36" t="n">
-        <v>36.03682595352917</v>
+        <v>33.50762527233114</v>
       </c>
       <c r="J36" t="n">
         <v>30</v>
@@ -3017,7 +3017,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M36" t="n">
@@ -3027,10 +3027,10 @@
         <v>30</v>
       </c>
       <c r="O36" t="n">
-        <v>72.3404255319149</v>
+        <v>68.08510638297872</v>
       </c>
       <c r="P36" t="n">
-        <v>45.58808510638298</v>
+        <v>44.73702127659575</v>
       </c>
       <c r="Q36" t="b">
         <v>0</v>
@@ -3054,48 +3054,48 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2197.7</v>
+        <v>2183</v>
       </c>
       <c r="D37" t="n">
-        <v>0.1565016050097352</v>
+        <v>-0.06329113924050631</v>
       </c>
       <c r="E37" t="n">
-        <v>0.4207123925269893</v>
+        <v>0.3173616559048942</v>
       </c>
       <c r="F37" t="n">
-        <v>0.723821476194211</v>
+        <v>0.6919857386451713</v>
       </c>
       <c r="G37" t="n">
-        <v>0.588856728493365</v>
+        <v>0.7125583799831455</v>
       </c>
       <c r="H37" t="n">
-        <v>0.7276896824630978</v>
+        <v>0.7468254703872635</v>
       </c>
       <c r="I37" t="n">
-        <v>46.03960396039601</v>
+        <v>47.6534296028881</v>
       </c>
       <c r="J37" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K37" t="n">
         <v>48.59</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M37" t="n">
         <v>48.59</v>
       </c>
       <c r="N37" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O37" t="n">
         <v>100</v>
       </c>
       <c r="P37" t="n">
-        <v>63.43600000000001</v>
+        <v>71.43600000000001</v>
       </c>
       <c r="Q37" t="b">
         <v>0</v>
@@ -3119,48 +3119,48 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>830.85</v>
+        <v>795.15</v>
       </c>
       <c r="D38" t="n">
-        <v>-0.0958210904342148</v>
+        <v>-0.182659197204091</v>
       </c>
       <c r="E38" t="n">
-        <v>-0.1528853996737357</v>
+        <v>-0.1828271928472329</v>
       </c>
       <c r="F38" t="n">
-        <v>-0.2015664039976935</v>
+        <v>-0.2431467732724157</v>
       </c>
       <c r="G38" t="n">
-        <v>-0.3365311516985395</v>
+        <v>-0.2225741319344415</v>
       </c>
       <c r="H38" t="n">
-        <v>-0.1976981977288067</v>
+        <v>-0.1883070415303235</v>
       </c>
       <c r="I38" t="n">
-        <v>29.82805429864254</v>
+        <v>41.92412357931806</v>
       </c>
       <c r="J38" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="K38" t="n">
         <v>49.87</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M38" t="n">
         <v>49.87</v>
       </c>
       <c r="N38" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="O38" t="n">
-        <v>10.63829787234042</v>
+        <v>14.8936170212766</v>
       </c>
       <c r="P38" t="n">
-        <v>30.07565957446808</v>
+        <v>38.92672340425532</v>
       </c>
       <c r="Q38" t="b">
         <v>0</v>
@@ -3184,48 +3184,48 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>2928.7</v>
+        <v>3102.1</v>
       </c>
       <c r="D39" t="n">
-        <v>-0.058204971540663</v>
+        <v>0.008747398543184201</v>
       </c>
       <c r="E39" t="n">
-        <v>0.07400344713777519</v>
+        <v>0.0930970083512456</v>
       </c>
       <c r="F39" t="n">
-        <v>0.2043837644446271</v>
+        <v>0.2254483684917436</v>
       </c>
       <c r="G39" t="n">
-        <v>0.06941901674378111</v>
+        <v>0.2460210098297178</v>
       </c>
       <c r="H39" t="n">
-        <v>0.2082519707135139</v>
+        <v>0.2802881002338359</v>
       </c>
       <c r="I39" t="n">
-        <v>39.47118644067795</v>
+        <v>53.98535417546823</v>
       </c>
       <c r="J39" t="n">
-        <v>30</v>
+        <v>80</v>
       </c>
       <c r="K39" t="n">
         <v>48.69</v>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M39" t="n">
         <v>48.69</v>
       </c>
       <c r="N39" t="n">
-        <v>30</v>
+        <v>80</v>
       </c>
       <c r="O39" t="n">
-        <v>74.46808510638297</v>
+        <v>87.2340425531915</v>
       </c>
       <c r="P39" t="n">
-        <v>46.3696170212766</v>
+        <v>68.9228085106383</v>
       </c>
       <c r="Q39" t="b">
         <v>0</v>
@@ -3249,48 +3249,48 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>195.74</v>
+        <v>185.82</v>
       </c>
       <c r="D40" t="n">
-        <v>-0.09892740413386721</v>
+        <v>-0.1464792614027835</v>
       </c>
       <c r="E40" t="n">
-        <v>-0.0484200291686921</v>
+        <v>-0.0304706250652196</v>
       </c>
       <c r="F40" t="n">
-        <v>-0.0883092687470888</v>
+        <v>-0.1755257786848877</v>
       </c>
       <c r="G40" t="n">
-        <v>-0.2232740164479348</v>
+        <v>-0.1549531373469135</v>
       </c>
       <c r="H40" t="n">
-        <v>-0.084441062478202</v>
+        <v>-0.1206860469427955</v>
       </c>
       <c r="I40" t="n">
-        <v>22.19707879037237</v>
+        <v>40.83181542197934</v>
       </c>
       <c r="J40" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="K40" t="n">
         <v>45.44</v>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M40" t="n">
         <v>45.44</v>
       </c>
       <c r="N40" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="O40" t="n">
-        <v>31.91489361702128</v>
+        <v>23.40425531914894</v>
       </c>
       <c r="P40" t="n">
-        <v>32.55897872340425</v>
+        <v>38.85685106382979</v>
       </c>
       <c r="Q40" t="b">
         <v>0</v>
@@ -3314,25 +3314,25 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>848.4</v>
+        <v>799</v>
       </c>
       <c r="D41" t="n">
-        <v>-0.1073232323232323</v>
+        <v>-0.138776610078146</v>
       </c>
       <c r="E41" t="n">
-        <v>-0.1384615384615385</v>
+        <v>-0.1522096662952942</v>
       </c>
       <c r="F41" t="n">
-        <v>-0.1003658342611738</v>
+        <v>-0.2199550912818509</v>
       </c>
       <c r="G41" t="n">
-        <v>-0.2353305819620198</v>
+        <v>-0.1993824499438767</v>
       </c>
       <c r="H41" t="n">
-        <v>-0.09649762799228701</v>
+        <v>-0.1651153595397587</v>
       </c>
       <c r="I41" t="n">
-        <v>26.14439324116745</v>
+        <v>27.5675675675676</v>
       </c>
       <c r="J41" t="n">
         <v>20</v>
@@ -3342,7 +3342,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M41" t="n">
@@ -3352,10 +3352,10 @@
         <v>20</v>
       </c>
       <c r="O41" t="n">
-        <v>27.65957446808511</v>
+        <v>19.14893617021277</v>
       </c>
       <c r="P41" t="n">
-        <v>32.75191489361702</v>
+        <v>31.04978723404255</v>
       </c>
       <c r="Q41" t="b">
         <v>0</v>
@@ -3379,48 +3379,48 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>594.75</v>
+        <v>525.55</v>
       </c>
       <c r="D42" t="n">
-        <v>0.0123404255319148</v>
+        <v>-0.2231911905993644</v>
       </c>
       <c r="E42" t="n">
-        <v>-0.2108405758641278</v>
+        <v>-0.2653760134190662</v>
       </c>
       <c r="F42" t="n">
-        <v>-0.2394501278772378</v>
+        <v>-0.3267358442223931</v>
       </c>
       <c r="G42" t="n">
-        <v>-0.3744148755780838</v>
+        <v>-0.3061632028844189</v>
       </c>
       <c r="H42" t="n">
-        <v>-0.235581921608351</v>
+        <v>-0.2718961124803009</v>
       </c>
       <c r="I42" t="n">
-        <v>40.33149171270718</v>
+        <v>38.38383838383837</v>
       </c>
       <c r="J42" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K42" t="n">
         <v>47.66</v>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M42" t="n">
         <v>47.66</v>
       </c>
       <c r="N42" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O42" t="n">
-        <v>8.51063829787234</v>
+        <v>4.25531914893617</v>
       </c>
       <c r="P42" t="n">
-        <v>36.76612765957447</v>
+        <v>31.91506382978724</v>
       </c>
       <c r="Q42" t="b">
         <v>0</v>
@@ -3444,25 +3444,25 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>425.35</v>
+        <v>410.45</v>
       </c>
       <c r="D43" t="n">
-        <v>-0.10168954593453</v>
+        <v>-0.0178272313950705</v>
       </c>
       <c r="E43" t="n">
-        <v>-0.0951925122314401</v>
+        <v>-0.1063575005443066</v>
       </c>
       <c r="F43" t="n">
-        <v>-0.0346118928733545</v>
+        <v>-0.1105211832267851</v>
       </c>
       <c r="G43" t="n">
-        <v>-0.1695766405742005</v>
+        <v>-0.08994854188881091</v>
       </c>
       <c r="H43" t="n">
-        <v>-0.0307436866044676</v>
+        <v>-0.0556814514846929</v>
       </c>
       <c r="I43" t="n">
-        <v>45.54455445544556</v>
+        <v>40.36970781156825</v>
       </c>
       <c r="J43" t="n">
         <v>40</v>
@@ -3472,7 +3472,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M43" t="n">
@@ -3482,10 +3482,10 @@
         <v>40</v>
       </c>
       <c r="O43" t="n">
-        <v>36.17021276595745</v>
+        <v>42.5531914893617</v>
       </c>
       <c r="P43" t="n">
-        <v>43.82604255319149</v>
+        <v>45.10263829787234</v>
       </c>
       <c r="Q43" t="b">
         <v>0</v>
@@ -3509,48 +3509,48 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>240.95</v>
+        <v>238.9</v>
       </c>
       <c r="D44" t="n">
-        <v>-0.0987469609126614</v>
+        <v>-0.1361417465196167</v>
       </c>
       <c r="E44" t="n">
-        <v>-0.1448092280390417</v>
+        <v>-0.1623422159887797</v>
       </c>
       <c r="F44" t="n">
-        <v>-0.061903834923107</v>
+        <v>-0.0979799886728337</v>
       </c>
       <c r="G44" t="n">
-        <v>-0.196868582623953</v>
+        <v>-0.0774073473348595</v>
       </c>
       <c r="H44" t="n">
-        <v>-0.0580356286542201</v>
+        <v>-0.0431402569307415</v>
       </c>
       <c r="I44" t="n">
-        <v>19.35714285714286</v>
+        <v>46.77242888402625</v>
       </c>
       <c r="J44" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="K44" t="n">
         <v>47.2</v>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M44" t="n">
         <v>47.2</v>
       </c>
       <c r="N44" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="O44" t="n">
-        <v>34.04255319148936</v>
+        <v>46.80851063829788</v>
       </c>
       <c r="P44" t="n">
-        <v>33.68851063829788</v>
+        <v>44.24170212765958</v>
       </c>
       <c r="Q44" t="b">
         <v>0</v>
@@ -3574,48 +3574,48 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>100.25</v>
+        <v>92.33</v>
       </c>
       <c r="D45" t="n">
-        <v>-0.1127533410036285</v>
+        <v>-0.1465939550790276</v>
       </c>
       <c r="E45" t="n">
-        <v>-0.1929640959587828</v>
+        <v>-0.1683480453972257</v>
       </c>
       <c r="F45" t="n">
-        <v>-0.299147091722595</v>
+        <v>-0.316074074074074</v>
       </c>
       <c r="G45" t="n">
-        <v>-0.434111839423441</v>
+        <v>-0.2955014327360998</v>
       </c>
       <c r="H45" t="n">
-        <v>-0.2952788854537082</v>
+        <v>-0.2612343423319818</v>
       </c>
       <c r="I45" t="n">
-        <v>19.27570093457948</v>
+        <v>31.15942028985505</v>
       </c>
       <c r="J45" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="K45" t="n">
         <v>59.6</v>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M45" t="n">
         <v>59.6</v>
       </c>
       <c r="N45" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="O45" t="n">
-        <v>2.127659574468085</v>
+        <v>6.382978723404255</v>
       </c>
       <c r="P45" t="n">
-        <v>32.26553191489362</v>
+        <v>37.11659574468086</v>
       </c>
       <c r="Q45" t="b">
         <v>0</v>
@@ -3639,48 +3639,48 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>514.65</v>
+        <v>493.4</v>
       </c>
       <c r="D46" t="n">
-        <v>-0.1616712819677471</v>
+        <v>-0.1059164628069222</v>
       </c>
       <c r="E46" t="n">
-        <v>-0.1933385579937304</v>
+        <v>-0.2267669644256387</v>
       </c>
       <c r="F46" t="n">
-        <v>-0.0096218608678918</v>
+        <v>-0.1265710745264648</v>
       </c>
       <c r="G46" t="n">
-        <v>-0.1445866085687378</v>
+        <v>-0.1059984331884906</v>
       </c>
       <c r="H46" t="n">
-        <v>-0.005753654599005</v>
+        <v>-0.0717313427843726</v>
       </c>
       <c r="I46" t="n">
-        <v>28.31991951710265</v>
+        <v>45.43721056932715</v>
       </c>
       <c r="J46" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="K46" t="n">
         <v>49.61</v>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M46" t="n">
         <v>49.61</v>
       </c>
       <c r="N46" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="O46" t="n">
-        <v>44.68085106382978</v>
+        <v>36.17021276595745</v>
       </c>
       <c r="P46" t="n">
-        <v>36.78017021276596</v>
+        <v>43.07804255319149</v>
       </c>
       <c r="Q46" t="b">
         <v>0</v>
@@ -3704,48 +3704,48 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>880.25</v>
+        <v>1089.55</v>
       </c>
       <c r="D47" t="n">
-        <v>0.0270096838175242</v>
+        <v>0.21276714158504</v>
       </c>
       <c r="E47" t="n">
-        <v>-0.0143329040927159</v>
+        <v>0.3153256473712802</v>
       </c>
       <c r="F47" t="n">
-        <v>0.2068138195777351</v>
+        <v>0.4779571351058056</v>
       </c>
       <c r="G47" t="n">
-        <v>0.0718490718768891</v>
+        <v>0.4985297764437798</v>
       </c>
       <c r="H47" t="n">
-        <v>0.210682025846622</v>
+        <v>0.5327968668478978</v>
       </c>
       <c r="I47" t="n">
-        <v>53.79574003276898</v>
+        <v>76.0805057411947</v>
       </c>
       <c r="J47" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K47" t="n">
         <v>46.83</v>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M47" t="n">
         <v>46.83</v>
       </c>
       <c r="N47" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O47" t="n">
-        <v>76.59574468085107</v>
+        <v>95.74468085106383</v>
       </c>
       <c r="P47" t="n">
-        <v>58.05114893617021</v>
+        <v>65.88093617021276</v>
       </c>
       <c r="Q47" t="b">
         <v>0</v>
@@ -3769,48 +3769,48 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>14376</v>
+        <v>13592</v>
       </c>
       <c r="D48" t="n">
-        <v>-0.0620473673908787</v>
+        <v>-0.1284386021160628</v>
       </c>
       <c r="E48" t="n">
-        <v>0.1381521653075765</v>
+        <v>-0.081187047928074</v>
       </c>
       <c r="F48" t="n">
-        <v>0.0445397079125191</v>
+        <v>-0.0421423537702607</v>
       </c>
       <c r="G48" t="n">
-        <v>-0.09042503978832681</v>
+        <v>-0.0215697124322865</v>
       </c>
       <c r="H48" t="n">
-        <v>0.048407914181406</v>
+        <v>0.0126973779718314</v>
       </c>
       <c r="I48" t="n">
-        <v>26.40127388535032</v>
+        <v>37.02397743300423</v>
       </c>
       <c r="J48" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="K48" t="n">
         <v>50.29</v>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M48" t="n">
         <v>50.29</v>
       </c>
       <c r="N48" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="O48" t="n">
-        <v>48.93617021276596</v>
+        <v>61.70212765957447</v>
       </c>
       <c r="P48" t="n">
-        <v>37.9032340425532</v>
+        <v>44.4564255319149</v>
       </c>
       <c r="Q48" t="b">
         <v>0</v>
@@ -3936,57 +3936,57 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>LUMAXTECH</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Forgings</t>
+          <t>Lighting</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1923.9</v>
+        <v>1623.3</v>
       </c>
       <c r="D2" t="n">
-        <v>0.2092394720301698</v>
+        <v>-0.0232264275828871</v>
       </c>
       <c r="E2" t="n">
-        <v>0.3775597880567092</v>
+        <v>0.06459863588667369</v>
       </c>
       <c r="F2" t="n">
-        <v>0.6694724054147865</v>
+        <v>0.4412678682411435</v>
       </c>
       <c r="G2" t="n">
-        <v>0.5345076577139405</v>
+        <v>0.4618405095791177</v>
       </c>
       <c r="H2" t="n">
-        <v>0.6733406116836733</v>
+        <v>0.4961075999832357</v>
       </c>
       <c r="I2" t="n">
-        <v>74.69975980784629</v>
+        <v>57.3173835581573</v>
       </c>
       <c r="J2" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K2" t="n">
-        <v>54.83</v>
+        <v>54.51</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M2" t="n">
-        <v>54.83</v>
+        <v>54.51</v>
       </c>
       <c r="N2" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O2" t="n">
-        <v>97.87234042553192</v>
+        <v>93.61702127659576</v>
       </c>
       <c r="P2" t="n">
-        <v>69.50646808510639</v>
+        <v>72.52740425531915</v>
       </c>
       <c r="Q2" t="b">
         <v>0</v>
@@ -4001,57 +4001,57 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DIVGIITTS</t>
+          <t>SANSERA</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Transmission</t>
+          <t>Forgings</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>721.05</v>
+        <v>2183</v>
       </c>
       <c r="D3" t="n">
-        <v>0.152942117045091</v>
+        <v>-0.06329113924050631</v>
       </c>
       <c r="E3" t="n">
-        <v>0.1205998912114381</v>
+        <v>0.3173616559048942</v>
       </c>
       <c r="F3" t="n">
-        <v>0.1096491228070175</v>
+        <v>0.6919857386451713</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.0253156248938284</v>
+        <v>0.7125583799831455</v>
       </c>
       <c r="H3" t="n">
-        <v>0.1135173290759044</v>
+        <v>0.7468254703872635</v>
       </c>
       <c r="I3" t="n">
-        <v>46.48203592814371</v>
+        <v>47.6534296028881</v>
       </c>
       <c r="J3" t="n">
         <v>80</v>
       </c>
       <c r="K3" t="n">
-        <v>49.92</v>
+        <v>48.59</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M3" t="n">
-        <v>49.92</v>
+        <v>48.59</v>
       </c>
       <c r="N3" t="n">
         <v>80</v>
       </c>
       <c r="O3" t="n">
-        <v>63.82978723404256</v>
+        <v>100</v>
       </c>
       <c r="P3" t="n">
-        <v>64.73395744680852</v>
+        <v>71.43600000000001</v>
       </c>
       <c r="Q3" t="b">
         <v>0</v>
@@ -4066,57 +4066,57 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BHARATSE</t>
+          <t>SHRIPISTON</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Seating</t>
+          <t>Engine/Parts</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>176.48</v>
+        <v>3102.1</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1158320687910976</v>
+        <v>0.008747398543184201</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.0170983013088277</v>
+        <v>0.0930970083512456</v>
       </c>
       <c r="F4" t="n">
-        <v>0.618637072365404</v>
+        <v>0.2254483684917436</v>
       </c>
       <c r="G4" t="n">
-        <v>0.483672324664558</v>
+        <v>0.2460210098297178</v>
       </c>
       <c r="H4" t="n">
-        <v>0.6225052786342908</v>
+        <v>0.2802881002338359</v>
       </c>
       <c r="I4" t="n">
-        <v>55.20238191035647</v>
+        <v>53.98535417546823</v>
       </c>
       <c r="J4" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K4" t="n">
-        <v>52.61</v>
+        <v>48.69</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M4" t="n">
-        <v>52.61</v>
+        <v>48.69</v>
       </c>
       <c r="N4" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O4" t="n">
-        <v>93.61702127659576</v>
+        <v>87.2340425531915</v>
       </c>
       <c r="P4" t="n">
-        <v>63.76740425531915</v>
+        <v>68.9228085106383</v>
       </c>
       <c r="Q4" t="b">
         <v>0</v>
@@ -4131,57 +4131,57 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SANSERA</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Forgings</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>2197.7</v>
+        <v>511.45</v>
       </c>
       <c r="D5" t="n">
-        <v>0.1565016050097352</v>
+        <v>-0.045891241488667</v>
       </c>
       <c r="E5" t="n">
-        <v>0.4207123925269893</v>
+        <v>0.0377396773866287</v>
       </c>
       <c r="F5" t="n">
-        <v>0.723821476194211</v>
+        <v>0.1494549949432519</v>
       </c>
       <c r="G5" t="n">
-        <v>0.588856728493365</v>
+        <v>0.1700276362812262</v>
       </c>
       <c r="H5" t="n">
-        <v>0.7276896824630978</v>
+        <v>0.2042947266853442</v>
       </c>
       <c r="I5" t="n">
-        <v>46.03960396039601</v>
+        <v>50.15782828282829</v>
       </c>
       <c r="J5" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K5" t="n">
-        <v>48.59</v>
+        <v>49.66</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M5" t="n">
-        <v>48.59</v>
+        <v>49.66</v>
       </c>
       <c r="N5" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O5" t="n">
-        <v>100</v>
+        <v>82.97872340425532</v>
       </c>
       <c r="P5" t="n">
-        <v>63.43600000000001</v>
+        <v>68.45974468085107</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
@@ -4196,63 +4196,63 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AUTOAXLES</t>
+          <t>ASKAUTOLTD</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Axles</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1987</v>
+        <v>444.15</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.0579813208173328</v>
+        <v>0.0255137381667049</v>
       </c>
       <c r="E6" t="n">
-        <v>0.2024933430162188</v>
+        <v>-0.0730460189919649</v>
       </c>
       <c r="F6" t="n">
-        <v>0.2149932738168032</v>
+        <v>-0.1285195722554694</v>
       </c>
       <c r="G6" t="n">
-        <v>0.0800285261159572</v>
+        <v>-0.1079469309174951</v>
       </c>
       <c r="H6" t="n">
-        <v>0.21886148008569</v>
+        <v>-0.0736798405133771</v>
       </c>
       <c r="I6" t="n">
-        <v>45.62982005141387</v>
+        <v>69.83381502890172</v>
       </c>
       <c r="J6" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K6" t="n">
-        <v>58.77</v>
+        <v>71.28</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M6" t="n">
-        <v>58.77</v>
+        <v>71.28</v>
       </c>
       <c r="N6" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O6" t="n">
-        <v>78.72340425531915</v>
+        <v>34.04255319148936</v>
       </c>
       <c r="P6" t="n">
-        <v>63.25268085106384</v>
+        <v>67.32051063829788</v>
       </c>
       <c r="Q6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S6" t="b">
         <v>0</v>
@@ -4261,57 +4261,57 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>GNA</t>
+          <t>WHEELS</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Axles</t>
+          <t>Wheels</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>426.25</v>
+        <v>1089.55</v>
       </c>
       <c r="D7" t="n">
-        <v>0.0248857898533301</v>
+        <v>0.21276714158504</v>
       </c>
       <c r="E7" t="n">
-        <v>0.3633455941148249</v>
+        <v>0.3153256473712802</v>
       </c>
       <c r="F7" t="n">
-        <v>0.4046795188663701</v>
+        <v>0.4779571351058056</v>
       </c>
       <c r="G7" t="n">
-        <v>0.2697147711655241</v>
+        <v>0.4985297764437798</v>
       </c>
       <c r="H7" t="n">
-        <v>0.4085477251352569</v>
+        <v>0.5327968668478978</v>
       </c>
       <c r="I7" t="n">
-        <v>47.02058504875406</v>
+        <v>76.0805057411947</v>
       </c>
       <c r="J7" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K7" t="n">
-        <v>54.47</v>
+        <v>46.83</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M7" t="n">
-        <v>54.47</v>
+        <v>46.83</v>
       </c>
       <c r="N7" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O7" t="n">
-        <v>85.1063829787234</v>
+        <v>95.74468085106383</v>
       </c>
       <c r="P7" t="n">
-        <v>62.80927659574468</v>
+        <v>65.88093617021276</v>
       </c>
       <c r="Q7" t="b">
         <v>0</v>
@@ -4326,63 +4326,63 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>LUMAXIND</t>
+          <t>JBMA</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Lighting</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>5576.5</v>
+        <v>572.65</v>
       </c>
       <c r="D8" t="n">
-        <v>0.0538599640933572</v>
+        <v>0.0089859924235751</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0908219553225617</v>
+        <v>-0.0294890263536987</v>
       </c>
       <c r="F8" t="n">
-        <v>0.6683120923831749</v>
+        <v>-0.0634557200098128</v>
       </c>
       <c r="G8" t="n">
-        <v>0.5333473446823289</v>
+        <v>-0.0428830786718386</v>
       </c>
       <c r="H8" t="n">
-        <v>0.6721802986520617</v>
+        <v>-0.0086159882677205</v>
       </c>
       <c r="I8" t="n">
-        <v>33.83625351503353</v>
+        <v>60.2561852956659</v>
       </c>
       <c r="J8" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="K8" t="n">
-        <v>57.69</v>
+        <v>56.91</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M8" t="n">
-        <v>57.69</v>
+        <v>56.91</v>
       </c>
       <c r="N8" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="O8" t="n">
-        <v>95.74468085106383</v>
+        <v>55.31914893617022</v>
       </c>
       <c r="P8" t="n">
-        <v>62.22493617021277</v>
+        <v>65.82782978723404</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
       </c>
       <c r="R8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S8" t="b">
         <v>0</v>
@@ -4391,57 +4391,57 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>JAMNAAUTO</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Suspension</t>
+          <t>Forgings</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>132.57</v>
+        <v>1736.5</v>
       </c>
       <c r="D9" t="n">
-        <v>0.017968210089841</v>
+        <v>-0.0521288209606987</v>
       </c>
       <c r="E9" t="n">
-        <v>0.2102428336680664</v>
+        <v>0.2350640113798008</v>
       </c>
       <c r="F9" t="n">
-        <v>0.457293613279103</v>
+        <v>0.5304953287502205</v>
       </c>
       <c r="G9" t="n">
-        <v>0.322328865578257</v>
+        <v>0.5510679700881947</v>
       </c>
       <c r="H9" t="n">
-        <v>0.4611618195479898</v>
+        <v>0.5853350604923128</v>
       </c>
       <c r="I9" t="n">
-        <v>47.25532330533308</v>
+        <v>37.49420670477369</v>
       </c>
       <c r="J9" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="K9" t="n">
-        <v>48.3</v>
+        <v>54.83</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M9" t="n">
-        <v>48.3</v>
+        <v>54.83</v>
       </c>
       <c r="N9" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="O9" t="n">
-        <v>87.2340425531915</v>
+        <v>97.87234042553192</v>
       </c>
       <c r="P9" t="n">
-        <v>60.7668085106383</v>
+        <v>61.50646808510639</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -4456,63 +4456,63 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>WHEELS</t>
+          <t>TIINDIA</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Wheels</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>880.25</v>
+        <v>2682.4</v>
       </c>
       <c r="D10" t="n">
-        <v>0.0270096838175242</v>
+        <v>0.0562293274531422</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.0143329040927159</v>
+        <v>0.0058874264071699</v>
       </c>
       <c r="F10" t="n">
-        <v>0.2068138195777351</v>
+        <v>-0.1198031173092698</v>
       </c>
       <c r="G10" t="n">
-        <v>0.0718490718768891</v>
+        <v>-0.0992304759712956</v>
       </c>
       <c r="H10" t="n">
-        <v>0.210682025846622</v>
+        <v>-0.0649633855671776</v>
       </c>
       <c r="I10" t="n">
-        <v>53.79574003276898</v>
+        <v>44.36388353914127</v>
       </c>
       <c r="J10" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K10" t="n">
-        <v>46.83</v>
+        <v>48.73</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M10" t="n">
-        <v>46.83</v>
+        <v>48.73</v>
       </c>
       <c r="N10" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O10" t="n">
-        <v>76.59574468085107</v>
+        <v>38.29787234042553</v>
       </c>
       <c r="P10" t="n">
-        <v>58.05114893617021</v>
+        <v>59.15157446808512</v>
       </c>
       <c r="Q10" t="b">
         <v>0</v>
       </c>
       <c r="R10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S10" t="b">
         <v>0</v>
@@ -4521,7 +4521,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>MINDACORP</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -4530,48 +4530,48 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>514.95</v>
+        <v>543.95</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.033592943605142</v>
+        <v>-0.0612649926654585</v>
       </c>
       <c r="E11" t="n">
-        <v>0.0540374577832361</v>
+        <v>-0.071995223065768</v>
       </c>
       <c r="F11" t="n">
-        <v>0.1696763202725724</v>
+        <v>0.0716115051221435</v>
       </c>
       <c r="G11" t="n">
-        <v>0.0347115725717264</v>
+        <v>0.0921841464601177</v>
       </c>
       <c r="H11" t="n">
-        <v>0.1735445265414592</v>
+        <v>0.1264512368642357</v>
       </c>
       <c r="I11" t="n">
-        <v>43.58341559723593</v>
+        <v>54.80591497227357</v>
       </c>
       <c r="J11" t="n">
         <v>60</v>
       </c>
       <c r="K11" t="n">
-        <v>49.66</v>
+        <v>49.42</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M11" t="n">
-        <v>49.66</v>
+        <v>49.42</v>
       </c>
       <c r="N11" t="n">
         <v>60</v>
       </c>
       <c r="O11" t="n">
-        <v>70.21276595744681</v>
+        <v>74.46808510638297</v>
       </c>
       <c r="P11" t="n">
-        <v>57.90655319148937</v>
+        <v>58.6616170212766</v>
       </c>
       <c r="Q11" t="b">
         <v>0</v>
@@ -4586,63 +4586,63 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TIINDIA</t>
+          <t>DIVGIITTS</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Transmission</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>2722.9</v>
+        <v>697.65</v>
       </c>
       <c r="D12" t="n">
-        <v>0.0324182907408812</v>
+        <v>-0.0896457232335095</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.1018570439027607</v>
+        <v>0.1612983770287139</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.098884733759142</v>
+        <v>0.0669062547790182</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.233849481459988</v>
+        <v>0.0874788961169924</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.0950165274902552</v>
+        <v>0.1217459865211104</v>
       </c>
       <c r="I12" t="n">
-        <v>67.22469666717861</v>
+        <v>49.20332525112573</v>
       </c>
       <c r="J12" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K12" t="n">
-        <v>48.73</v>
+        <v>49.92</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M12" t="n">
-        <v>48.73</v>
+        <v>49.92</v>
       </c>
       <c r="N12" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O12" t="n">
-        <v>29.78723404255319</v>
+        <v>72.3404255319149</v>
       </c>
       <c r="P12" t="n">
-        <v>57.44944680851064</v>
+        <v>58.43608510638298</v>
       </c>
       <c r="Q12" t="b">
         <v>0</v>
       </c>
       <c r="R12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S12" t="b">
         <v>0</v>
@@ -4651,63 +4651,63 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MOTHERSON</t>
+          <t>RANEENGINE</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Engine/Parts</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>122.77</v>
+        <v>317.75</v>
       </c>
       <c r="D13" t="n">
-        <v>0.0012232914695806</v>
+        <v>0.1790352504638219</v>
       </c>
       <c r="E13" t="n">
-        <v>0.1267437591776798</v>
+        <v>-0.156154561147258</v>
       </c>
       <c r="F13" t="n">
-        <v>0.3600310180569404</v>
+        <v>-0.2401052253975846</v>
       </c>
       <c r="G13" t="n">
-        <v>0.2250662703560944</v>
+        <v>-0.2195325840596104</v>
       </c>
       <c r="H13" t="n">
-        <v>0.3638992243258272</v>
+        <v>-0.1852654936554923</v>
       </c>
       <c r="I13" t="n">
-        <v>36.94247923715782</v>
+        <v>63.3225806451613</v>
       </c>
       <c r="J13" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="K13" t="n">
-        <v>51.57</v>
+        <v>50.88</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M13" t="n">
-        <v>51.57</v>
+        <v>50.88</v>
       </c>
       <c r="N13" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="O13" t="n">
-        <v>82.97872340425532</v>
+        <v>17.02127659574468</v>
       </c>
       <c r="P13" t="n">
-        <v>57.22374468085107</v>
+        <v>55.75625531914894</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
       </c>
       <c r="R13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S13" t="b">
         <v>0</v>
@@ -4716,7 +4716,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>LUMAXTECH</t>
+          <t>LUMAXIND</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -4725,48 +4725,48 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1531.9</v>
+        <v>5148.5</v>
       </c>
       <c r="D14" t="n">
-        <v>0.0025523560209423</v>
+        <v>-0.1565781498288092</v>
       </c>
       <c r="E14" t="n">
-        <v>0.1208751006073023</v>
+        <v>-0.09189522885616019</v>
       </c>
       <c r="F14" t="n">
-        <v>0.4965806955842127</v>
+        <v>0.2336759878273788</v>
       </c>
       <c r="G14" t="n">
-        <v>0.3616159478833667</v>
+        <v>0.254248629165353</v>
       </c>
       <c r="H14" t="n">
-        <v>0.5004489018530995</v>
+        <v>0.2885157195694711</v>
       </c>
       <c r="I14" t="n">
-        <v>42.36420670298829</v>
+        <v>38.56340288924559</v>
       </c>
       <c r="J14" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K14" t="n">
-        <v>54.51</v>
+        <v>57.69</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M14" t="n">
-        <v>54.51</v>
+        <v>57.69</v>
       </c>
       <c r="N14" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O14" t="n">
-        <v>91.48936170212764</v>
+        <v>89.36170212765957</v>
       </c>
       <c r="P14" t="n">
-        <v>56.10187234042553</v>
+        <v>52.94834042553191</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
@@ -4781,63 +4781,63 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>RANEENGINE</t>
+          <t>PRICOLLTD</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Engine/Parts</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>317.75</v>
+        <v>543.95</v>
       </c>
       <c r="D15" t="n">
-        <v>0.1790352504638219</v>
+        <v>-0.1378189887462354</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.156154561147258</v>
+        <v>-0.0963535177340311</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.2401052253975846</v>
+        <v>0.1429922252574071</v>
       </c>
       <c r="G15" t="n">
-        <v>-0.3750699730984306</v>
+        <v>0.1635648665953814</v>
       </c>
       <c r="H15" t="n">
-        <v>-0.2362370191286977</v>
+        <v>0.1978319569994994</v>
       </c>
       <c r="I15" t="n">
-        <v>63.3225806451613</v>
+        <v>44.98910675381264</v>
       </c>
       <c r="J15" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="K15" t="n">
-        <v>50.88</v>
+        <v>49.98</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M15" t="n">
-        <v>50.88</v>
+        <v>49.98</v>
       </c>
       <c r="N15" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="O15" t="n">
-        <v>6.382978723404255</v>
+        <v>80.85106382978722</v>
       </c>
       <c r="P15" t="n">
-        <v>53.62859574468086</v>
+        <v>52.16221276595745</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
       </c>
       <c r="R15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S15" t="b">
         <v>0</v>
@@ -4846,57 +4846,57 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>RICOAUTO</t>
+          <t>GNA</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Castings</t>
+          <t>Axles</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>113.3</v>
+        <v>396.15</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.1335270724992352</v>
+        <v>-0.0439242186557259</v>
       </c>
       <c r="E16" t="n">
-        <v>0.0055915505458417</v>
+        <v>0.2727710843373494</v>
       </c>
       <c r="F16" t="n">
-        <v>0.494525788154597</v>
+        <v>0.2610218048702848</v>
       </c>
       <c r="G16" t="n">
-        <v>0.359561040453751</v>
+        <v>0.281594446208259</v>
       </c>
       <c r="H16" t="n">
-        <v>0.4983939944234838</v>
+        <v>0.315861536612377</v>
       </c>
       <c r="I16" t="n">
-        <v>39.08828923238146</v>
+        <v>39.38129996524157</v>
       </c>
       <c r="J16" t="n">
         <v>30</v>
       </c>
       <c r="K16" t="n">
-        <v>49.07</v>
+        <v>54.47</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="M16" t="n">
-        <v>49.07</v>
+        <v>54.47</v>
       </c>
       <c r="N16" t="n">
         <v>30</v>
       </c>
       <c r="O16" t="n">
-        <v>89.36170212765957</v>
+        <v>91.48936170212764</v>
       </c>
       <c r="P16" t="n">
-        <v>49.50034042553192</v>
+        <v>52.08587234042552</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>
@@ -4919,7 +4919,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5368,6 +5368,25 @@
       </c>
       <c r="E26" t="n">
         <v>0.1735265188095714</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2025-02-11</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>6</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0.06729471111296829</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0.0542595245326515</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.0130351865803167</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: auto-refresh NSE data and pipeline outputs (2026-03-26)
</commit_message>
<xml_diff>
--- a/working-sector/output/auto_components_comprehensive_report.xlsx
+++ b/working-sector/output/auto_components_comprehensive_report.xlsx
@@ -435,7 +435,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
     </row>
@@ -447,7 +447,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
     </row>
@@ -782,22 +782,22 @@
         <v>1736.5</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.0521288209606987</v>
+        <v>-0.06554377656998329</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2350640113798008</v>
+        <v>0.2641962725684335</v>
       </c>
       <c r="F2" t="n">
-        <v>0.5304953287502205</v>
+        <v>0.5291475871785842</v>
       </c>
       <c r="G2" t="n">
-        <v>0.5510679700881947</v>
+        <v>0.5497202285165584</v>
       </c>
       <c r="H2" t="n">
-        <v>0.5853350604923128</v>
+        <v>0.5839873189206765</v>
       </c>
       <c r="I2" t="n">
-        <v>37.49420670477369</v>
+        <v>34.93084593116758</v>
       </c>
       <c r="J2" t="n">
         <v>50</v>
@@ -807,7 +807,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M2" t="n">
@@ -817,10 +817,10 @@
         <v>50</v>
       </c>
       <c r="O2" t="n">
-        <v>97.87234042553192</v>
+        <v>95.74468085106383</v>
       </c>
       <c r="P2" t="n">
-        <v>61.50646808510639</v>
+        <v>61.08093617021277</v>
       </c>
       <c r="Q2" t="b">
         <v>0</v>
@@ -847,22 +847,22 @@
         <v>1087.6</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.0906354515050168</v>
+        <v>-0.0763481953290871</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.1452373467463062</v>
+        <v>-0.1355905261484661</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.1691367456073339</v>
+        <v>-0.1524314214463841</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.1485641042693597</v>
+        <v>-0.1318587801084099</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.1142970138652417</v>
+        <v>-0.0975916897042918</v>
       </c>
       <c r="I3" t="n">
-        <v>46.095141185449</v>
+        <v>45.68059471930274</v>
       </c>
       <c r="J3" t="n">
         <v>40</v>
@@ -872,7 +872,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M3" t="n">
@@ -912,22 +912,22 @@
         <v>30390</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.1400679117147708</v>
+        <v>-0.1398245117463912</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.1768689057421452</v>
+        <v>-0.1695586828801748</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.2644318044293839</v>
+        <v>-0.2605839416058394</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.2438591630914097</v>
+        <v>-0.2400113002678652</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.2095920726872917</v>
+        <v>-0.2057442098637472</v>
       </c>
       <c r="I4" t="n">
-        <v>33.62168396770474</v>
+        <v>32.80793928779919</v>
       </c>
       <c r="J4" t="n">
         <v>30</v>
@@ -937,7 +937,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M4" t="n">
@@ -947,10 +947,10 @@
         <v>30</v>
       </c>
       <c r="O4" t="n">
-        <v>10.63829787234042</v>
+        <v>12.76595744680851</v>
       </c>
       <c r="P4" t="n">
-        <v>35.51965957446808</v>
+        <v>35.9451914893617</v>
       </c>
       <c r="Q4" t="b">
         <v>0</v>
@@ -977,22 +977,22 @@
         <v>307.15</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.0923463356973995</v>
+        <v>-0.0857270427146896</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.1920294620544521</v>
+        <v>-0.177093101138647</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.2620134550696781</v>
+        <v>-0.2671200190885231</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.2414408137317039</v>
+        <v>-0.2465473777505489</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.2071737233275858</v>
+        <v>-0.2122802873464309</v>
       </c>
       <c r="I5" t="n">
-        <v>43.0862831858407</v>
+        <v>44.92502883506344</v>
       </c>
       <c r="J5" t="n">
         <v>40</v>
@@ -1002,7 +1002,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M5" t="n">
@@ -1012,10 +1012,10 @@
         <v>40</v>
       </c>
       <c r="O5" t="n">
-        <v>12.76595744680851</v>
+        <v>10.63829787234042</v>
       </c>
       <c r="P5" t="n">
-        <v>39.0011914893617</v>
+        <v>38.57565957446808</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
@@ -1042,22 +1042,22 @@
         <v>113.13</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.1352239718697446</v>
+        <v>-0.1400881726968683</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.033489961554891</v>
+        <v>-0.0188204683434518</v>
       </c>
       <c r="F6" t="n">
-        <v>0.1726961749766766</v>
+        <v>0.1719672640629854</v>
       </c>
       <c r="G6" t="n">
-        <v>0.1932688163146508</v>
+        <v>0.1925399054009596</v>
       </c>
       <c r="H6" t="n">
-        <v>0.2275359067187689</v>
+        <v>0.2268069958050776</v>
       </c>
       <c r="I6" t="n">
-        <v>35.66312133709572</v>
+        <v>38.65882352941176</v>
       </c>
       <c r="J6" t="n">
         <v>30</v>
@@ -1067,7 +1067,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M6" t="n">
@@ -1107,22 +1107,22 @@
         <v>2682.4</v>
       </c>
       <c r="D7" t="n">
-        <v>0.0562293274531422</v>
+        <v>0.0467085495766186</v>
       </c>
       <c r="E7" t="n">
-        <v>0.0058874264071699</v>
+        <v>0.045036621474209</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.1198031173092698</v>
+        <v>-0.1187331624942505</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.0992304759712956</v>
+        <v>-0.0981605211562763</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.0649633855671776</v>
+        <v>-0.0638934307521583</v>
       </c>
       <c r="I7" t="n">
-        <v>44.36388353914127</v>
+        <v>47.54158067257497</v>
       </c>
       <c r="J7" t="n">
         <v>80</v>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M7" t="n">
@@ -1172,22 +1172,22 @@
         <v>511.45</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.045891241488667</v>
+        <v>-0.0339975446217774</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0377396773866287</v>
+        <v>0.0516089236146806</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1494549949432519</v>
+        <v>0.1365555555555555</v>
       </c>
       <c r="G8" t="n">
-        <v>0.1700276362812262</v>
+        <v>0.1571281968935297</v>
       </c>
       <c r="H8" t="n">
-        <v>0.2042947266853442</v>
+        <v>0.1913952872976477</v>
       </c>
       <c r="I8" t="n">
-        <v>50.15782828282829</v>
+        <v>48.86658031088081</v>
       </c>
       <c r="J8" t="n">
         <v>80</v>
@@ -1197,7 +1197,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M8" t="n">
@@ -1237,22 +1237,22 @@
         <v>419.65</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.07464167585446529</v>
+        <v>-0.0771852666300165</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.1952248537731327</v>
+        <v>-0.1935235898914192</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.1397088970889709</v>
+        <v>-0.1359003397508493</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.1191362557509967</v>
+        <v>-0.1153276984128751</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.0848691653468787</v>
+        <v>-0.0810606080087571</v>
       </c>
       <c r="I9" t="n">
-        <v>40.15936254980078</v>
+        <v>41.68734491315136</v>
       </c>
       <c r="J9" t="n">
         <v>40</v>
@@ -1262,7 +1262,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M9" t="n">
@@ -1272,10 +1272,10 @@
         <v>40</v>
       </c>
       <c r="O9" t="n">
-        <v>31.91489361702128</v>
+        <v>36.17021276595745</v>
       </c>
       <c r="P9" t="n">
-        <v>43.75897872340426</v>
+        <v>44.6100425531915</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -1302,22 +1302,22 @@
         <v>129970</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.1083287596048299</v>
+        <v>-0.0971170545328239</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.1516872266823314</v>
+        <v>-0.1532899022801302</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.1554082594144978</v>
+        <v>-0.1366987711723679</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.1348356180765236</v>
+        <v>-0.1161261298343937</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.1005685276724056</v>
+        <v>-0.0818590394302757</v>
       </c>
       <c r="I10" t="n">
-        <v>33.76129339039468</v>
+        <v>35.37030886748589</v>
       </c>
       <c r="J10" t="n">
         <v>30</v>
@@ -1327,7 +1327,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M10" t="n">
@@ -1337,10 +1337,10 @@
         <v>30</v>
       </c>
       <c r="O10" t="n">
-        <v>29.78723404255319</v>
+        <v>34.04255319148936</v>
       </c>
       <c r="P10" t="n">
-        <v>37.72144680851064</v>
+        <v>38.57251063829787</v>
       </c>
       <c r="Q10" t="b">
         <v>0</v>
@@ -1392,7 +1392,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M11" t="n">
@@ -1402,10 +1402,10 @@
         <v>20</v>
       </c>
       <c r="O11" t="n">
-        <v>63.82978723404256</v>
+        <v>65.95744680851064</v>
       </c>
       <c r="P11" t="n">
-        <v>24.76595744680852</v>
+        <v>25.19148936170213</v>
       </c>
       <c r="Q11" t="b">
         <v>0</v>
@@ -1432,22 +1432,22 @@
         <v>444.15</v>
       </c>
       <c r="D12" t="n">
-        <v>0.0255137381667049</v>
+        <v>0.0382187938288918</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.0730460189919649</v>
+        <v>-0.0300283904782703</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.1285195722554694</v>
+        <v>-0.1372377622377621</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.1079469309174951</v>
+        <v>-0.1166651208997879</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.0736798405133771</v>
+        <v>-0.08239803049566991</v>
       </c>
       <c r="I12" t="n">
-        <v>69.83381502890172</v>
+        <v>69.2562592047128</v>
       </c>
       <c r="J12" t="n">
         <v>80</v>
@@ -1457,7 +1457,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M12" t="n">
@@ -1467,10 +1467,10 @@
         <v>80</v>
       </c>
       <c r="O12" t="n">
-        <v>34.04255319148936</v>
+        <v>31.91489361702128</v>
       </c>
       <c r="P12" t="n">
-        <v>67.32051063829788</v>
+        <v>66.89497872340425</v>
       </c>
       <c r="Q12" t="b">
         <v>1</v>
@@ -1497,22 +1497,22 @@
         <v>1650.4</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.1813085966565801</v>
+        <v>-0.1761593370937951</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.0945797673908271</v>
+        <v>-0.1021163157608399</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.0678865921156669</v>
+        <v>-0.0617929623102722</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.0473139507776927</v>
+        <v>-0.041220320972298</v>
       </c>
       <c r="H13" t="n">
-        <v>-0.0130468603735747</v>
+        <v>-0.0069532305681799</v>
       </c>
       <c r="I13" t="n">
-        <v>19.06348649596633</v>
+        <v>19.62093862815885</v>
       </c>
       <c r="J13" t="n">
         <v>20</v>
@@ -1522,7 +1522,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M13" t="n">
@@ -1532,10 +1532,10 @@
         <v>20</v>
       </c>
       <c r="O13" t="n">
-        <v>53.19148936170212</v>
+        <v>55.31914893617022</v>
       </c>
       <c r="P13" t="n">
-        <v>42.14629787234043</v>
+        <v>42.57182978723405</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
@@ -1562,22 +1562,22 @@
         <v>560.75</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.1464342796255423</v>
+        <v>-0.1396240889911776</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.25008358408559</v>
+        <v>-0.2056802889723068</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.0585914547133383</v>
+        <v>-0.1111199175715305</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.0380188133753641</v>
+        <v>-0.0905472762335563</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.0037517229712461</v>
+        <v>-0.0562801858294382</v>
       </c>
       <c r="I14" t="n">
-        <v>44.04982772329711</v>
+        <v>44.35548438751002</v>
       </c>
       <c r="J14" t="n">
         <v>40</v>
@@ -1587,7 +1587,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M14" t="n">
@@ -1597,10 +1597,10 @@
         <v>40</v>
       </c>
       <c r="O14" t="n">
-        <v>57.44680851063831</v>
+        <v>48.93617021276596</v>
       </c>
       <c r="P14" t="n">
-        <v>49.34536170212766</v>
+        <v>47.6432340425532</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
@@ -1627,22 +1627,22 @@
         <v>95.70999999999999</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.1321969353522533</v>
+        <v>-0.1147798742138366</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.0096233443708609</v>
+        <v>-0.0038509575353872</v>
       </c>
       <c r="F15" t="n">
-        <v>0.0413447938200413</v>
+        <v>0.0621462656752858</v>
       </c>
       <c r="G15" t="n">
-        <v>0.0619174351580155</v>
+        <v>0.08271890701326</v>
       </c>
       <c r="H15" t="n">
-        <v>0.0961845255621335</v>
+        <v>0.116985997417378</v>
       </c>
       <c r="I15" t="n">
-        <v>41.2743823146944</v>
+        <v>42.68423883808498</v>
       </c>
       <c r="J15" t="n">
         <v>40</v>
@@ -1652,7 +1652,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M15" t="n">
@@ -1662,10 +1662,10 @@
         <v>40</v>
       </c>
       <c r="O15" t="n">
-        <v>70.21276595744681</v>
+        <v>72.3404255319149</v>
       </c>
       <c r="P15" t="n">
-        <v>50.80655319148936</v>
+        <v>51.23208510638297</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
@@ -1692,22 +1692,22 @@
         <v>158.74</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.2123257083312657</v>
+        <v>-0.2043107769423559</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.0942082738944364</v>
+        <v>-0.0377061105722599</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.07741485528304071</v>
+        <v>-0.0376477720521368</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.0568422139450665</v>
+        <v>-0.0170751307141626</v>
       </c>
       <c r="H16" t="n">
-        <v>-0.0225751235409484</v>
+        <v>0.0171919596899553</v>
       </c>
       <c r="I16" t="n">
-        <v>35.63903520931521</v>
+        <v>37.17466743782533</v>
       </c>
       <c r="J16" t="n">
         <v>30</v>
@@ -1717,7 +1717,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M16" t="n">
@@ -1727,16 +1727,16 @@
         <v>30</v>
       </c>
       <c r="O16" t="n">
-        <v>51.06382978723404</v>
+        <v>59.57446808510638</v>
       </c>
       <c r="P16" t="n">
-        <v>43.2567659574468</v>
+        <v>44.95889361702128</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>
       </c>
       <c r="R16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S16" t="b">
         <v>0</v>
@@ -1757,45 +1757,45 @@
         <v>7049</v>
       </c>
       <c r="D17" t="n">
-        <v>-0.1198651517043326</v>
+        <v>-0.1050593537738843</v>
       </c>
       <c r="E17" t="n">
-        <v>-0.0075325589581133</v>
+        <v>0.0202634245187436</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0117697717812543</v>
+        <v>0.0219644798840159</v>
       </c>
       <c r="G17" t="n">
-        <v>0.0323424131192285</v>
+        <v>0.0425371212219901</v>
       </c>
       <c r="H17" t="n">
-        <v>0.0666095035233466</v>
+        <v>0.07680421162610809</v>
       </c>
       <c r="I17" t="n">
-        <v>38.97757122651041</v>
+        <v>41.25320786997433</v>
       </c>
       <c r="J17" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K17" t="n">
         <v>54.65</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M17" t="n">
         <v>54.65</v>
       </c>
       <c r="N17" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O17" t="n">
-        <v>65.95744680851064</v>
+        <v>68.08510638297872</v>
       </c>
       <c r="P17" t="n">
-        <v>47.05148936170213</v>
+        <v>51.47702127659574</v>
       </c>
       <c r="Q17" t="b">
         <v>0</v>
@@ -1822,22 +1822,22 @@
         <v>697.65</v>
       </c>
       <c r="D18" t="n">
-        <v>-0.0896457232335095</v>
+        <v>-0.07239728759473479</v>
       </c>
       <c r="E18" t="n">
-        <v>0.1612983770287139</v>
+        <v>0.1617818484596169</v>
       </c>
       <c r="F18" t="n">
-        <v>0.0669062547790182</v>
+        <v>0.053215579710145</v>
       </c>
       <c r="G18" t="n">
-        <v>0.0874788961169924</v>
+        <v>0.0737882210481192</v>
       </c>
       <c r="H18" t="n">
-        <v>0.1217459865211104</v>
+        <v>0.1080553114522372</v>
       </c>
       <c r="I18" t="n">
-        <v>49.20332525112573</v>
+        <v>45.66506113375324</v>
       </c>
       <c r="J18" t="n">
         <v>60</v>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M18" t="n">
@@ -1857,10 +1857,10 @@
         <v>60</v>
       </c>
       <c r="O18" t="n">
-        <v>72.3404255319149</v>
+        <v>70.21276595744681</v>
       </c>
       <c r="P18" t="n">
-        <v>58.43608510638298</v>
+        <v>58.01055319148936</v>
       </c>
       <c r="Q18" t="b">
         <v>0</v>
@@ -1887,22 +1887,22 @@
         <v>2333.1</v>
       </c>
       <c r="D19" t="n">
-        <v>-0.0867778299671208</v>
+        <v>-0.1310614525139665</v>
       </c>
       <c r="E19" t="n">
-        <v>-0.1225648740127868</v>
+        <v>-0.1226308664259927</v>
       </c>
       <c r="F19" t="n">
-        <v>-0.1985779060181368</v>
+        <v>-0.1992380560131795</v>
       </c>
       <c r="G19" t="n">
-        <v>-0.1780052646801626</v>
+        <v>-0.1786654146752053</v>
       </c>
       <c r="H19" t="n">
-        <v>-0.1437381742760446</v>
+        <v>-0.1443983242710873</v>
       </c>
       <c r="I19" t="n">
-        <v>35.89414595028067</v>
+        <v>39.51968921066571</v>
       </c>
       <c r="J19" t="n">
         <v>30</v>
@@ -1912,7 +1912,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M19" t="n">
@@ -1952,45 +1952,45 @@
         <v>2083.6</v>
       </c>
       <c r="D20" t="n">
-        <v>-0.0729667200569496</v>
+        <v>-0.0711483594864479</v>
       </c>
       <c r="E20" t="n">
-        <v>-0.07535280021301149</v>
+        <v>-0.0806159819970878</v>
       </c>
       <c r="F20" t="n">
-        <v>-0.0492790655229056</v>
+        <v>-0.0442201834862385</v>
       </c>
       <c r="G20" t="n">
-        <v>-0.0287064241849314</v>
+        <v>-0.0236475421482643</v>
       </c>
       <c r="H20" t="n">
-        <v>0.0055606662191866</v>
+        <v>0.0106195482558536</v>
       </c>
       <c r="I20" t="n">
-        <v>46.00603897886356</v>
+        <v>49.18561995597947</v>
       </c>
       <c r="J20" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K20" t="n">
         <v>49.06</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M20" t="n">
         <v>49.06</v>
       </c>
       <c r="N20" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O20" t="n">
-        <v>59.57446808510638</v>
+        <v>57.44680851063831</v>
       </c>
       <c r="P20" t="n">
-        <v>47.53889361702128</v>
+        <v>55.11336170212766</v>
       </c>
       <c r="Q20" t="b">
         <v>0</v>
@@ -2017,22 +2017,22 @@
         <v>881.25</v>
       </c>
       <c r="D21" t="n">
-        <v>-0.09355070973050809</v>
+        <v>-0.087544004969973</v>
       </c>
       <c r="E21" t="n">
-        <v>-0.081265638031693</v>
+        <v>-0.0508885298869143</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.3033596837944664</v>
+        <v>-0.2794358135731807</v>
       </c>
       <c r="G21" t="n">
-        <v>-0.2827870424564922</v>
+        <v>-0.2588631722352065</v>
       </c>
       <c r="H21" t="n">
-        <v>-0.2485199520523742</v>
+        <v>-0.2245960818310884</v>
       </c>
       <c r="I21" t="n">
-        <v>41.35438182354677</v>
+        <v>44.44973041547733</v>
       </c>
       <c r="J21" t="n">
         <v>40</v>
@@ -2042,7 +2042,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M21" t="n">
@@ -2082,22 +2082,22 @@
         <v>396.15</v>
       </c>
       <c r="D22" t="n">
-        <v>-0.0439242186557259</v>
+        <v>-0.0526126987922994</v>
       </c>
       <c r="E22" t="n">
-        <v>0.2727710843373494</v>
+        <v>0.3187416777629828</v>
       </c>
       <c r="F22" t="n">
-        <v>0.2610218048702848</v>
+        <v>0.2502761559097364</v>
       </c>
       <c r="G22" t="n">
-        <v>0.281594446208259</v>
+        <v>0.2708487972477106</v>
       </c>
       <c r="H22" t="n">
-        <v>0.315861536612377</v>
+        <v>0.3051158876518286</v>
       </c>
       <c r="I22" t="n">
-        <v>39.38129996524157</v>
+        <v>39.50488145048813</v>
       </c>
       <c r="J22" t="n">
         <v>30</v>
@@ -2107,7 +2107,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M22" t="n">
@@ -2147,45 +2147,45 @@
         <v>335.15</v>
       </c>
       <c r="D23" t="n">
-        <v>-0.0921034809697954</v>
+        <v>-0.08416450334745181</v>
       </c>
       <c r="E23" t="n">
-        <v>-0.1009924892703864</v>
+        <v>-0.096508963472166</v>
       </c>
       <c r="F23" t="n">
-        <v>-0.1699071207430341</v>
+        <v>-0.1782518082628418</v>
       </c>
       <c r="G23" t="n">
-        <v>-0.1493344794050599</v>
+        <v>-0.1576791669248676</v>
       </c>
       <c r="H23" t="n">
-        <v>-0.1150673890009419</v>
+        <v>-0.1234120765207495</v>
       </c>
       <c r="I23" t="n">
-        <v>31.39534883720927</v>
+        <v>25.85278276481147</v>
       </c>
       <c r="J23" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="K23" t="n">
         <v>49.7</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M23" t="n">
         <v>49.7</v>
       </c>
       <c r="N23" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="O23" t="n">
-        <v>25.53191489361702</v>
+        <v>23.40425531914894</v>
       </c>
       <c r="P23" t="n">
-        <v>36.98638297872341</v>
+        <v>32.56085106382979</v>
       </c>
       <c r="Q23" t="b">
         <v>0</v>
@@ -2212,22 +2212,22 @@
         <v>121.47</v>
       </c>
       <c r="D24" t="n">
-        <v>-0.1223900007224911</v>
+        <v>-0.1499650104968509</v>
       </c>
       <c r="E24" t="n">
-        <v>-0.005159705159705</v>
+        <v>0.0396268401232453</v>
       </c>
       <c r="F24" t="n">
-        <v>0.1259733036707453</v>
+        <v>0.1158368546757302</v>
       </c>
       <c r="G24" t="n">
-        <v>0.1465459450087195</v>
+        <v>0.1364094960137044</v>
       </c>
       <c r="H24" t="n">
-        <v>0.1808130354128375</v>
+        <v>0.1706765864178224</v>
       </c>
       <c r="I24" t="n">
-        <v>36.21378621378621</v>
+        <v>39.83516483516484</v>
       </c>
       <c r="J24" t="n">
         <v>30</v>
@@ -2237,7 +2237,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M24" t="n">
@@ -2247,10 +2247,10 @@
         <v>30</v>
       </c>
       <c r="O24" t="n">
-        <v>78.72340425531915</v>
+        <v>80.85106382978722</v>
       </c>
       <c r="P24" t="n">
-        <v>47.06468085106384</v>
+        <v>47.49021276595744</v>
       </c>
       <c r="Q24" t="b">
         <v>0</v>
@@ -2277,22 +2277,22 @@
         <v>572.65</v>
       </c>
       <c r="D25" t="n">
-        <v>0.0089859924235751</v>
+        <v>0.0290206648697213</v>
       </c>
       <c r="E25" t="n">
-        <v>-0.0294890263536987</v>
+        <v>0.0094306363476115</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.0634557200098128</v>
+        <v>-0.06802831800797469</v>
       </c>
       <c r="G25" t="n">
-        <v>-0.0428830786718386</v>
+        <v>-0.0474556766700005</v>
       </c>
       <c r="H25" t="n">
-        <v>-0.0086159882677205</v>
+        <v>-0.0131885862658824</v>
       </c>
       <c r="I25" t="n">
-        <v>60.2561852956659</v>
+        <v>59.15238954012625</v>
       </c>
       <c r="J25" t="n">
         <v>80</v>
@@ -2302,7 +2302,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M25" t="n">
@@ -2312,10 +2312,10 @@
         <v>80</v>
       </c>
       <c r="O25" t="n">
-        <v>55.31914893617022</v>
+        <v>53.19148936170212</v>
       </c>
       <c r="P25" t="n">
-        <v>65.82782978723404</v>
+        <v>65.40229787234043</v>
       </c>
       <c r="Q25" t="b">
         <v>0</v>
@@ -2342,22 +2342,22 @@
         <v>125.84</v>
       </c>
       <c r="D26" t="n">
-        <v>-0.0838005096468874</v>
+        <v>-0.07531780439415089</v>
       </c>
       <c r="E26" t="n">
-        <v>-0.1233716475095786</v>
+        <v>-0.1102941176470587</v>
       </c>
       <c r="F26" t="n">
-        <v>-0.0829993441667272</v>
+        <v>-0.1170981547744334</v>
       </c>
       <c r="G26" t="n">
-        <v>-0.062426702828753</v>
+        <v>-0.0965255134364592</v>
       </c>
       <c r="H26" t="n">
-        <v>-0.028159612424635</v>
+        <v>-0.0622584230323411</v>
       </c>
       <c r="I26" t="n">
-        <v>41.5401600883246</v>
+        <v>41.66666666666666</v>
       </c>
       <c r="J26" t="n">
         <v>40</v>
@@ -2367,7 +2367,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M26" t="n">
@@ -2377,10 +2377,10 @@
         <v>40</v>
       </c>
       <c r="O26" t="n">
-        <v>48.93617021276596</v>
+        <v>40.42553191489361</v>
       </c>
       <c r="P26" t="n">
-        <v>46.4032340425532</v>
+        <v>44.70110638297872</v>
       </c>
       <c r="Q26" t="b">
         <v>0</v>
@@ -2407,45 +2407,45 @@
         <v>5148.5</v>
       </c>
       <c r="D27" t="n">
-        <v>-0.1565781498288092</v>
+        <v>-0.1348222087786516</v>
       </c>
       <c r="E27" t="n">
-        <v>-0.09189522885616019</v>
+        <v>-0.08552397868561271</v>
       </c>
       <c r="F27" t="n">
-        <v>0.2336759878273788</v>
+        <v>0.2348003357716752</v>
       </c>
       <c r="G27" t="n">
-        <v>0.254248629165353</v>
+        <v>0.2553729771096494</v>
       </c>
       <c r="H27" t="n">
-        <v>0.2885157195694711</v>
+        <v>0.2896400675137675</v>
       </c>
       <c r="I27" t="n">
-        <v>38.56340288924559</v>
+        <v>40.8936170212766</v>
       </c>
       <c r="J27" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K27" t="n">
         <v>57.69</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M27" t="n">
         <v>57.69</v>
       </c>
       <c r="N27" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O27" t="n">
         <v>89.36170212765957</v>
       </c>
       <c r="P27" t="n">
-        <v>52.94834042553191</v>
+        <v>56.94834042553191</v>
       </c>
       <c r="Q27" t="b">
         <v>0</v>
@@ -2472,22 +2472,22 @@
         <v>1623.3</v>
       </c>
       <c r="D28" t="n">
-        <v>-0.0232264275828871</v>
+        <v>-0.0295330902134274</v>
       </c>
       <c r="E28" t="n">
-        <v>0.06459863588667369</v>
+        <v>0.09100073929699549</v>
       </c>
       <c r="F28" t="n">
-        <v>0.4412678682411435</v>
+        <v>0.5489503816793893</v>
       </c>
       <c r="G28" t="n">
-        <v>0.4618405095791177</v>
+        <v>0.5695230230173635</v>
       </c>
       <c r="H28" t="n">
-        <v>0.4961075999832357</v>
+        <v>0.6037901134214815</v>
       </c>
       <c r="I28" t="n">
-        <v>57.3173835581573</v>
+        <v>55.99580162686958</v>
       </c>
       <c r="J28" t="n">
         <v>80</v>
@@ -2497,7 +2497,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M28" t="n">
@@ -2507,10 +2507,10 @@
         <v>80</v>
       </c>
       <c r="O28" t="n">
-        <v>93.61702127659576</v>
+        <v>97.87234042553192</v>
       </c>
       <c r="P28" t="n">
-        <v>72.52740425531915</v>
+        <v>73.37846808510639</v>
       </c>
       <c r="Q28" t="b">
         <v>0</v>
@@ -2537,22 +2537,22 @@
         <v>543.95</v>
       </c>
       <c r="D29" t="n">
-        <v>-0.0612649926654585</v>
+        <v>-0.0517737296260785</v>
       </c>
       <c r="E29" t="n">
-        <v>-0.071995223065768</v>
+        <v>-0.0655385672564851</v>
       </c>
       <c r="F29" t="n">
-        <v>0.0716115051221435</v>
+        <v>0.0735149003355044</v>
       </c>
       <c r="G29" t="n">
-        <v>0.0921841464601177</v>
+        <v>0.0940875416734786</v>
       </c>
       <c r="H29" t="n">
-        <v>0.1264512368642357</v>
+        <v>0.1283546320775966</v>
       </c>
       <c r="I29" t="n">
-        <v>54.80591497227357</v>
+        <v>57.42414460942543</v>
       </c>
       <c r="J29" t="n">
         <v>60</v>
@@ -2562,7 +2562,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M29" t="n">
@@ -2602,22 +2602,22 @@
         <v>111.94</v>
       </c>
       <c r="D30" t="n">
-        <v>-0.0594067725401227</v>
+        <v>-0.0357481264536135</v>
       </c>
       <c r="E30" t="n">
-        <v>0.0506851886615355</v>
+        <v>0.0496015002344114</v>
       </c>
       <c r="F30" t="n">
-        <v>-0.1103163249085995</v>
+        <v>-0.1141183918961696</v>
       </c>
       <c r="G30" t="n">
-        <v>-0.0897436835706253</v>
+        <v>-0.0935457505581954</v>
       </c>
       <c r="H30" t="n">
-        <v>-0.0554765931665073</v>
+        <v>-0.0592786601540774</v>
       </c>
       <c r="I30" t="n">
-        <v>41.92680301399354</v>
+        <v>42.44075183873605</v>
       </c>
       <c r="J30" t="n">
         <v>40</v>
@@ -2627,7 +2627,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M30" t="n">
@@ -2637,10 +2637,10 @@
         <v>40</v>
       </c>
       <c r="O30" t="n">
-        <v>44.68085106382978</v>
+        <v>42.5531914893617</v>
       </c>
       <c r="P30" t="n">
-        <v>45.88817021276596</v>
+        <v>45.46263829787234</v>
       </c>
       <c r="Q30" t="b">
         <v>0</v>
@@ -2667,22 +2667,22 @@
         <v>37.98</v>
       </c>
       <c r="D31" t="n">
-        <v>-0.1459410838767709</v>
+        <v>-0.1290988305434534</v>
       </c>
       <c r="E31" t="n">
-        <v>-0.1671052631578948</v>
+        <v>-0.1522321428571429</v>
       </c>
       <c r="F31" t="n">
-        <v>-0.1167441860465117</v>
+        <v>-0.1140657802659202</v>
       </c>
       <c r="G31" t="n">
-        <v>-0.0961715447085375</v>
+        <v>-0.093493138927946</v>
       </c>
       <c r="H31" t="n">
-        <v>-0.0619044543044194</v>
+        <v>-0.059226048523828</v>
       </c>
       <c r="I31" t="n">
-        <v>30.71120689655172</v>
+        <v>31.70189098998885</v>
       </c>
       <c r="J31" t="n">
         <v>30</v>
@@ -2692,7 +2692,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M31" t="n">
@@ -2702,10 +2702,10 @@
         <v>30</v>
       </c>
       <c r="O31" t="n">
-        <v>40.42553191489361</v>
+        <v>44.68085106382978</v>
       </c>
       <c r="P31" t="n">
-        <v>39.68110638297873</v>
+        <v>40.53217021276596</v>
       </c>
       <c r="Q31" t="b">
         <v>0</v>
@@ -2732,22 +2732,22 @@
         <v>686.55</v>
       </c>
       <c r="D32" t="n">
-        <v>-0.1282458256618627</v>
+        <v>-0.09444041416606209</v>
       </c>
       <c r="E32" t="n">
-        <v>-0.1817531732316309</v>
+        <v>-0.1418125</v>
       </c>
       <c r="F32" t="n">
-        <v>-0.3496732026143792</v>
+        <v>-0.348005698005698</v>
       </c>
       <c r="G32" t="n">
-        <v>-0.3291005612764049</v>
+        <v>-0.3274330566677238</v>
       </c>
       <c r="H32" t="n">
-        <v>-0.2948334708722869</v>
+        <v>-0.2931659662636058</v>
       </c>
       <c r="I32" t="n">
-        <v>47.40046838407492</v>
+        <v>45.03181595692608</v>
       </c>
       <c r="J32" t="n">
         <v>40</v>
@@ -2757,7 +2757,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M32" t="n">
@@ -2797,22 +2797,22 @@
         <v>543.95</v>
       </c>
       <c r="D33" t="n">
-        <v>-0.1378189887462354</v>
+        <v>-0.1213149180195459</v>
       </c>
       <c r="E33" t="n">
-        <v>-0.0963535177340311</v>
+        <v>-0.1059335963182116</v>
       </c>
       <c r="F33" t="n">
-        <v>0.1429922252574071</v>
+        <v>0.1106687085247575</v>
       </c>
       <c r="G33" t="n">
-        <v>0.1635648665953814</v>
+        <v>0.1312413498627317</v>
       </c>
       <c r="H33" t="n">
-        <v>0.1978319569994994</v>
+        <v>0.1655084402668497</v>
       </c>
       <c r="I33" t="n">
-        <v>44.98910675381264</v>
+        <v>43.93560921454346</v>
       </c>
       <c r="J33" t="n">
         <v>40</v>
@@ -2822,7 +2822,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M33" t="n">
@@ -2832,10 +2832,10 @@
         <v>40</v>
       </c>
       <c r="O33" t="n">
-        <v>80.85106382978722</v>
+        <v>78.72340425531915</v>
       </c>
       <c r="P33" t="n">
-        <v>52.16221276595745</v>
+        <v>51.73668085106384</v>
       </c>
       <c r="Q33" t="b">
         <v>0</v>
@@ -2887,7 +2887,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M34" t="n">
@@ -2927,22 +2927,22 @@
         <v>109.14</v>
       </c>
       <c r="D35" t="n">
-        <v>-0.1325013909864081</v>
+        <v>-0.1294568078487676</v>
       </c>
       <c r="E35" t="n">
-        <v>-0.0156038603770182</v>
+        <v>0.0423073249928374</v>
       </c>
       <c r="F35" t="n">
-        <v>0.1063355296502788</v>
+        <v>0.0943547578461847</v>
       </c>
       <c r="G35" t="n">
-        <v>0.126908170988253</v>
+        <v>0.1149273991841589</v>
       </c>
       <c r="H35" t="n">
-        <v>0.161175261392371</v>
+        <v>0.1491944895882769</v>
       </c>
       <c r="I35" t="n">
-        <v>42.75874906924796</v>
+        <v>45.84830339321358</v>
       </c>
       <c r="J35" t="n">
         <v>40</v>
@@ -2952,7 +2952,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M35" t="n">
@@ -2992,22 +2992,22 @@
         <v>465</v>
       </c>
       <c r="D36" t="n">
-        <v>-0.0433083016150601</v>
+        <v>-0.0435050910212896</v>
       </c>
       <c r="E36" t="n">
-        <v>-0.1528511568591728</v>
+        <v>-0.1223931301311692</v>
       </c>
       <c r="F36" t="n">
-        <v>0.028533510285335</v>
+        <v>-0.0094791777612098</v>
       </c>
       <c r="G36" t="n">
-        <v>0.0491061516233092</v>
+        <v>0.0110934635767643</v>
       </c>
       <c r="H36" t="n">
-        <v>0.0833732420274272</v>
+        <v>0.0453605539808823</v>
       </c>
       <c r="I36" t="n">
-        <v>33.50762527233114</v>
+        <v>34.95454545454545</v>
       </c>
       <c r="J36" t="n">
         <v>30</v>
@@ -3017,7 +3017,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M36" t="n">
@@ -3027,10 +3027,10 @@
         <v>30</v>
       </c>
       <c r="O36" t="n">
-        <v>68.08510638297872</v>
+        <v>63.82978723404256</v>
       </c>
       <c r="P36" t="n">
-        <v>44.73702127659575</v>
+        <v>43.88595744680851</v>
       </c>
       <c r="Q36" t="b">
         <v>0</v>
@@ -3057,22 +3057,22 @@
         <v>2183</v>
       </c>
       <c r="D37" t="n">
-        <v>-0.06329113924050631</v>
+        <v>-0.0692816030697079</v>
       </c>
       <c r="E37" t="n">
-        <v>0.3173616559048942</v>
+        <v>0.3397569657542654</v>
       </c>
       <c r="F37" t="n">
-        <v>0.6919857386451713</v>
+        <v>0.6758790112083526</v>
       </c>
       <c r="G37" t="n">
-        <v>0.7125583799831455</v>
+        <v>0.6964516525463268</v>
       </c>
       <c r="H37" t="n">
-        <v>0.7468254703872635</v>
+        <v>0.7307187429504448</v>
       </c>
       <c r="I37" t="n">
-        <v>47.6534296028881</v>
+        <v>49.29617925883368</v>
       </c>
       <c r="J37" t="n">
         <v>80</v>
@@ -3082,7 +3082,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M37" t="n">
@@ -3122,22 +3122,22 @@
         <v>795.15</v>
       </c>
       <c r="D38" t="n">
-        <v>-0.182659197204091</v>
+        <v>-0.1638801261829653</v>
       </c>
       <c r="E38" t="n">
-        <v>-0.1828271928472329</v>
+        <v>-0.1621621621621621</v>
       </c>
       <c r="F38" t="n">
-        <v>-0.2431467732724157</v>
+        <v>-0.2573550014009527</v>
       </c>
       <c r="G38" t="n">
-        <v>-0.2225741319344415</v>
+        <v>-0.2367823600629784</v>
       </c>
       <c r="H38" t="n">
-        <v>-0.1883070415303235</v>
+        <v>-0.2025152696588604</v>
       </c>
       <c r="I38" t="n">
-        <v>41.92412357931806</v>
+        <v>44.00201612903225</v>
       </c>
       <c r="J38" t="n">
         <v>40</v>
@@ -3147,7 +3147,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M38" t="n">
@@ -3187,22 +3187,22 @@
         <v>3102.1</v>
       </c>
       <c r="D39" t="n">
-        <v>0.008747398543184201</v>
+        <v>-0.0255999497424299</v>
       </c>
       <c r="E39" t="n">
-        <v>0.0930970083512456</v>
+        <v>0.0189193627853505</v>
       </c>
       <c r="F39" t="n">
-        <v>0.2254483684917436</v>
+        <v>0.2005960213638824</v>
       </c>
       <c r="G39" t="n">
-        <v>0.2460210098297178</v>
+        <v>0.2211686627018566</v>
       </c>
       <c r="H39" t="n">
-        <v>0.2802881002338359</v>
+        <v>0.2554357531059746</v>
       </c>
       <c r="I39" t="n">
-        <v>53.98535417546823</v>
+        <v>56.375</v>
       </c>
       <c r="J39" t="n">
         <v>80</v>
@@ -3212,7 +3212,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M39" t="n">
@@ -3252,22 +3252,22 @@
         <v>185.82</v>
       </c>
       <c r="D40" t="n">
-        <v>-0.1464792614027835</v>
+        <v>-0.1299339794915016</v>
       </c>
       <c r="E40" t="n">
-        <v>-0.0304706250652196</v>
+        <v>-0.0195230054875475</v>
       </c>
       <c r="F40" t="n">
-        <v>-0.1755257786848877</v>
+        <v>-0.177787610619469</v>
       </c>
       <c r="G40" t="n">
-        <v>-0.1549531373469135</v>
+        <v>-0.1572149692814948</v>
       </c>
       <c r="H40" t="n">
-        <v>-0.1206860469427955</v>
+        <v>-0.1229478788773767</v>
       </c>
       <c r="I40" t="n">
-        <v>40.83181542197934</v>
+        <v>42.21594475831763</v>
       </c>
       <c r="J40" t="n">
         <v>40</v>
@@ -3277,7 +3277,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M40" t="n">
@@ -3287,10 +3287,10 @@
         <v>40</v>
       </c>
       <c r="O40" t="n">
-        <v>23.40425531914894</v>
+        <v>25.53191489361702</v>
       </c>
       <c r="P40" t="n">
-        <v>38.85685106382979</v>
+        <v>39.2823829787234</v>
       </c>
       <c r="Q40" t="b">
         <v>0</v>
@@ -3317,22 +3317,22 @@
         <v>799</v>
       </c>
       <c r="D41" t="n">
-        <v>-0.138776610078146</v>
+        <v>-0.1343914197497426</v>
       </c>
       <c r="E41" t="n">
-        <v>-0.1522096662952942</v>
+        <v>-0.1340630757559336</v>
       </c>
       <c r="F41" t="n">
-        <v>-0.2199550912818509</v>
+        <v>-0.212264615991324</v>
       </c>
       <c r="G41" t="n">
-        <v>-0.1993824499438767</v>
+        <v>-0.1916919746533498</v>
       </c>
       <c r="H41" t="n">
-        <v>-0.1651153595397587</v>
+        <v>-0.1574248842492318</v>
       </c>
       <c r="I41" t="n">
-        <v>27.5675675675676</v>
+        <v>28.65168539325848</v>
       </c>
       <c r="J41" t="n">
         <v>20</v>
@@ -3342,7 +3342,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M41" t="n">
@@ -3382,22 +3382,22 @@
         <v>525.55</v>
       </c>
       <c r="D42" t="n">
-        <v>-0.2231911905993644</v>
+        <v>-0.2168243797034498</v>
       </c>
       <c r="E42" t="n">
-        <v>-0.2653760134190662</v>
+        <v>-0.2383885225708282</v>
       </c>
       <c r="F42" t="n">
-        <v>-0.3267358442223931</v>
+        <v>-0.3193679984458978</v>
       </c>
       <c r="G42" t="n">
-        <v>-0.3061632028844189</v>
+        <v>-0.2987953571079236</v>
       </c>
       <c r="H42" t="n">
-        <v>-0.2718961124803009</v>
+        <v>-0.2645282667038056</v>
       </c>
       <c r="I42" t="n">
-        <v>38.38383838383837</v>
+        <v>31.49732620320856</v>
       </c>
       <c r="J42" t="n">
         <v>30</v>
@@ -3407,7 +3407,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M42" t="n">
@@ -3447,22 +3447,22 @@
         <v>410.45</v>
       </c>
       <c r="D43" t="n">
-        <v>-0.0178272313950705</v>
+        <v>-0.0303567210016537</v>
       </c>
       <c r="E43" t="n">
-        <v>-0.1063575005443066</v>
+        <v>-0.0836124134851529</v>
       </c>
       <c r="F43" t="n">
-        <v>-0.1105211832267851</v>
+        <v>-0.1100390286209886</v>
       </c>
       <c r="G43" t="n">
-        <v>-0.08994854188881091</v>
+        <v>-0.0894663872830144</v>
       </c>
       <c r="H43" t="n">
-        <v>-0.0556814514846929</v>
+        <v>-0.0551992968788964</v>
       </c>
       <c r="I43" t="n">
-        <v>40.36970781156825</v>
+        <v>40.98062953995155</v>
       </c>
       <c r="J43" t="n">
         <v>40</v>
@@ -3472,7 +3472,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M43" t="n">
@@ -3482,10 +3482,10 @@
         <v>40</v>
       </c>
       <c r="O43" t="n">
-        <v>42.5531914893617</v>
+        <v>51.06382978723404</v>
       </c>
       <c r="P43" t="n">
-        <v>45.10263829787234</v>
+        <v>46.8047659574468</v>
       </c>
       <c r="Q43" t="b">
         <v>0</v>
@@ -3512,22 +3512,22 @@
         <v>238.9</v>
       </c>
       <c r="D44" t="n">
-        <v>-0.1361417465196167</v>
+        <v>-0.0943896891584533</v>
       </c>
       <c r="E44" t="n">
-        <v>-0.1623422159887797</v>
+        <v>-0.1467857142857143</v>
       </c>
       <c r="F44" t="n">
-        <v>-0.0979799886728337</v>
+        <v>-0.1120609552127857</v>
       </c>
       <c r="G44" t="n">
-        <v>-0.0774073473348595</v>
+        <v>-0.09148831387481141</v>
       </c>
       <c r="H44" t="n">
-        <v>-0.0431402569307415</v>
+        <v>-0.0572212234706934</v>
       </c>
       <c r="I44" t="n">
-        <v>46.77242888402625</v>
+        <v>48.8292404340377</v>
       </c>
       <c r="J44" t="n">
         <v>40</v>
@@ -3537,7 +3537,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M44" t="n">
@@ -3577,22 +3577,22 @@
         <v>92.33</v>
       </c>
       <c r="D45" t="n">
-        <v>-0.1465939550790276</v>
+        <v>-0.1387930230388956</v>
       </c>
       <c r="E45" t="n">
-        <v>-0.1683480453972257</v>
+        <v>-0.1602546612096408</v>
       </c>
       <c r="F45" t="n">
-        <v>-0.316074074074074</v>
+        <v>-0.3137866963953921</v>
       </c>
       <c r="G45" t="n">
-        <v>-0.2955014327360998</v>
+        <v>-0.2932140550574179</v>
       </c>
       <c r="H45" t="n">
-        <v>-0.2612343423319818</v>
+        <v>-0.2589469646532999</v>
       </c>
       <c r="I45" t="n">
-        <v>31.15942028985505</v>
+        <v>32.43123336291035</v>
       </c>
       <c r="J45" t="n">
         <v>30</v>
@@ -3602,7 +3602,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M45" t="n">
@@ -3642,22 +3642,22 @@
         <v>493.4</v>
       </c>
       <c r="D46" t="n">
-        <v>-0.1059164628069222</v>
+        <v>-0.0963369963369963</v>
       </c>
       <c r="E46" t="n">
-        <v>-0.2267669644256387</v>
+        <v>-0.2063057990830853</v>
       </c>
       <c r="F46" t="n">
-        <v>-0.1265710745264648</v>
+        <v>-0.1380906629399948</v>
       </c>
       <c r="G46" t="n">
-        <v>-0.1059984331884906</v>
+        <v>-0.1175180216020206</v>
       </c>
       <c r="H46" t="n">
-        <v>-0.0717313427843726</v>
+        <v>-0.0832509311979026</v>
       </c>
       <c r="I46" t="n">
-        <v>45.43721056932715</v>
+        <v>44.06590337894443</v>
       </c>
       <c r="J46" t="n">
         <v>40</v>
@@ -3667,7 +3667,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M46" t="n">
@@ -3677,10 +3677,10 @@
         <v>40</v>
       </c>
       <c r="O46" t="n">
-        <v>36.17021276595745</v>
+        <v>29.78723404255319</v>
       </c>
       <c r="P46" t="n">
-        <v>43.07804255319149</v>
+        <v>41.80144680851064</v>
       </c>
       <c r="Q46" t="b">
         <v>0</v>
@@ -3707,22 +3707,22 @@
         <v>1089.55</v>
       </c>
       <c r="D47" t="n">
-        <v>0.21276714158504</v>
+        <v>0.2215370816749817</v>
       </c>
       <c r="E47" t="n">
-        <v>0.3153256473712802</v>
+        <v>0.3412322274881516</v>
       </c>
       <c r="F47" t="n">
-        <v>0.4779571351058056</v>
+        <v>0.4680994408138517</v>
       </c>
       <c r="G47" t="n">
-        <v>0.4985297764437798</v>
+        <v>0.4886720821518259</v>
       </c>
       <c r="H47" t="n">
-        <v>0.5327968668478978</v>
+        <v>0.5229391725559439</v>
       </c>
       <c r="I47" t="n">
-        <v>76.0805057411947</v>
+        <v>77.51051524710832</v>
       </c>
       <c r="J47" t="n">
         <v>70</v>
@@ -3732,7 +3732,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M47" t="n">
@@ -3742,10 +3742,10 @@
         <v>70</v>
       </c>
       <c r="O47" t="n">
-        <v>95.74468085106383</v>
+        <v>93.61702127659576</v>
       </c>
       <c r="P47" t="n">
-        <v>65.88093617021276</v>
+        <v>65.45540425531915</v>
       </c>
       <c r="Q47" t="b">
         <v>0</v>
@@ -3772,22 +3772,22 @@
         <v>13592</v>
       </c>
       <c r="D48" t="n">
-        <v>-0.1284386021160628</v>
+        <v>-0.1396923855940249</v>
       </c>
       <c r="E48" t="n">
-        <v>-0.081187047928074</v>
+        <v>-0.07644220968947479</v>
       </c>
       <c r="F48" t="n">
-        <v>-0.0421423537702607</v>
+        <v>-0.0152151862048978</v>
       </c>
       <c r="G48" t="n">
-        <v>-0.0215697124322865</v>
+        <v>0.0053574551330763</v>
       </c>
       <c r="H48" t="n">
-        <v>0.0126973779718314</v>
+        <v>0.0396245455371944</v>
       </c>
       <c r="I48" t="n">
-        <v>37.02397743300423</v>
+        <v>35.93974175035869</v>
       </c>
       <c r="J48" t="n">
         <v>30</v>
@@ -3797,7 +3797,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M48" t="n">
@@ -3948,22 +3948,22 @@
         <v>1623.3</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.0232264275828871</v>
+        <v>-0.0295330902134274</v>
       </c>
       <c r="E2" t="n">
-        <v>0.06459863588667369</v>
+        <v>0.09100073929699549</v>
       </c>
       <c r="F2" t="n">
-        <v>0.4412678682411435</v>
+        <v>0.5489503816793893</v>
       </c>
       <c r="G2" t="n">
-        <v>0.4618405095791177</v>
+        <v>0.5695230230173635</v>
       </c>
       <c r="H2" t="n">
-        <v>0.4961075999832357</v>
+        <v>0.6037901134214815</v>
       </c>
       <c r="I2" t="n">
-        <v>57.3173835581573</v>
+        <v>55.99580162686958</v>
       </c>
       <c r="J2" t="n">
         <v>80</v>
@@ -3973,7 +3973,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M2" t="n">
@@ -3983,10 +3983,10 @@
         <v>80</v>
       </c>
       <c r="O2" t="n">
-        <v>93.61702127659576</v>
+        <v>97.87234042553192</v>
       </c>
       <c r="P2" t="n">
-        <v>72.52740425531915</v>
+        <v>73.37846808510639</v>
       </c>
       <c r="Q2" t="b">
         <v>0</v>
@@ -4013,22 +4013,22 @@
         <v>2183</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.06329113924050631</v>
+        <v>-0.0692816030697079</v>
       </c>
       <c r="E3" t="n">
-        <v>0.3173616559048942</v>
+        <v>0.3397569657542654</v>
       </c>
       <c r="F3" t="n">
-        <v>0.6919857386451713</v>
+        <v>0.6758790112083526</v>
       </c>
       <c r="G3" t="n">
-        <v>0.7125583799831455</v>
+        <v>0.6964516525463268</v>
       </c>
       <c r="H3" t="n">
-        <v>0.7468254703872635</v>
+        <v>0.7307187429504448</v>
       </c>
       <c r="I3" t="n">
-        <v>47.6534296028881</v>
+        <v>49.29617925883368</v>
       </c>
       <c r="J3" t="n">
         <v>80</v>
@@ -4038,7 +4038,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M3" t="n">
@@ -4078,22 +4078,22 @@
         <v>3102.1</v>
       </c>
       <c r="D4" t="n">
-        <v>0.008747398543184201</v>
+        <v>-0.0255999497424299</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0930970083512456</v>
+        <v>0.0189193627853505</v>
       </c>
       <c r="F4" t="n">
-        <v>0.2254483684917436</v>
+        <v>0.2005960213638824</v>
       </c>
       <c r="G4" t="n">
-        <v>0.2460210098297178</v>
+        <v>0.2211686627018566</v>
       </c>
       <c r="H4" t="n">
-        <v>0.2802881002338359</v>
+        <v>0.2554357531059746</v>
       </c>
       <c r="I4" t="n">
-        <v>53.98535417546823</v>
+        <v>56.375</v>
       </c>
       <c r="J4" t="n">
         <v>80</v>
@@ -4103,7 +4103,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M4" t="n">
@@ -4143,22 +4143,22 @@
         <v>511.45</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.045891241488667</v>
+        <v>-0.0339975446217774</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0377396773866287</v>
+        <v>0.0516089236146806</v>
       </c>
       <c r="F5" t="n">
-        <v>0.1494549949432519</v>
+        <v>0.1365555555555555</v>
       </c>
       <c r="G5" t="n">
-        <v>0.1700276362812262</v>
+        <v>0.1571281968935297</v>
       </c>
       <c r="H5" t="n">
-        <v>0.2042947266853442</v>
+        <v>0.1913952872976477</v>
       </c>
       <c r="I5" t="n">
-        <v>50.15782828282829</v>
+        <v>48.86658031088081</v>
       </c>
       <c r="J5" t="n">
         <v>80</v>
@@ -4168,7 +4168,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M5" t="n">
@@ -4208,22 +4208,22 @@
         <v>444.15</v>
       </c>
       <c r="D6" t="n">
-        <v>0.0255137381667049</v>
+        <v>0.0382187938288918</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.0730460189919649</v>
+        <v>-0.0300283904782703</v>
       </c>
       <c r="F6" t="n">
-        <v>-0.1285195722554694</v>
+        <v>-0.1372377622377621</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.1079469309174951</v>
+        <v>-0.1166651208997879</v>
       </c>
       <c r="H6" t="n">
-        <v>-0.0736798405133771</v>
+        <v>-0.08239803049566991</v>
       </c>
       <c r="I6" t="n">
-        <v>69.83381502890172</v>
+        <v>69.2562592047128</v>
       </c>
       <c r="J6" t="n">
         <v>80</v>
@@ -4233,7 +4233,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M6" t="n">
@@ -4243,10 +4243,10 @@
         <v>80</v>
       </c>
       <c r="O6" t="n">
-        <v>34.04255319148936</v>
+        <v>31.91489361702128</v>
       </c>
       <c r="P6" t="n">
-        <v>67.32051063829788</v>
+        <v>66.89497872340425</v>
       </c>
       <c r="Q6" t="b">
         <v>1</v>
@@ -4273,22 +4273,22 @@
         <v>1089.55</v>
       </c>
       <c r="D7" t="n">
-        <v>0.21276714158504</v>
+        <v>0.2215370816749817</v>
       </c>
       <c r="E7" t="n">
-        <v>0.3153256473712802</v>
+        <v>0.3412322274881516</v>
       </c>
       <c r="F7" t="n">
-        <v>0.4779571351058056</v>
+        <v>0.4680994408138517</v>
       </c>
       <c r="G7" t="n">
-        <v>0.4985297764437798</v>
+        <v>0.4886720821518259</v>
       </c>
       <c r="H7" t="n">
-        <v>0.5327968668478978</v>
+        <v>0.5229391725559439</v>
       </c>
       <c r="I7" t="n">
-        <v>76.0805057411947</v>
+        <v>77.51051524710832</v>
       </c>
       <c r="J7" t="n">
         <v>70</v>
@@ -4298,7 +4298,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M7" t="n">
@@ -4308,10 +4308,10 @@
         <v>70</v>
       </c>
       <c r="O7" t="n">
-        <v>95.74468085106383</v>
+        <v>93.61702127659576</v>
       </c>
       <c r="P7" t="n">
-        <v>65.88093617021276</v>
+        <v>65.45540425531915</v>
       </c>
       <c r="Q7" t="b">
         <v>0</v>
@@ -4338,22 +4338,22 @@
         <v>572.65</v>
       </c>
       <c r="D8" t="n">
-        <v>0.0089859924235751</v>
+        <v>0.0290206648697213</v>
       </c>
       <c r="E8" t="n">
-        <v>-0.0294890263536987</v>
+        <v>0.0094306363476115</v>
       </c>
       <c r="F8" t="n">
-        <v>-0.0634557200098128</v>
+        <v>-0.06802831800797469</v>
       </c>
       <c r="G8" t="n">
-        <v>-0.0428830786718386</v>
+        <v>-0.0474556766700005</v>
       </c>
       <c r="H8" t="n">
-        <v>-0.0086159882677205</v>
+        <v>-0.0131885862658824</v>
       </c>
       <c r="I8" t="n">
-        <v>60.2561852956659</v>
+        <v>59.15238954012625</v>
       </c>
       <c r="J8" t="n">
         <v>80</v>
@@ -4363,7 +4363,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M8" t="n">
@@ -4373,10 +4373,10 @@
         <v>80</v>
       </c>
       <c r="O8" t="n">
-        <v>55.31914893617022</v>
+        <v>53.19148936170212</v>
       </c>
       <c r="P8" t="n">
-        <v>65.82782978723404</v>
+        <v>65.40229787234043</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
@@ -4403,22 +4403,22 @@
         <v>1736.5</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.0521288209606987</v>
+        <v>-0.06554377656998329</v>
       </c>
       <c r="E9" t="n">
-        <v>0.2350640113798008</v>
+        <v>0.2641962725684335</v>
       </c>
       <c r="F9" t="n">
-        <v>0.5304953287502205</v>
+        <v>0.5291475871785842</v>
       </c>
       <c r="G9" t="n">
-        <v>0.5510679700881947</v>
+        <v>0.5497202285165584</v>
       </c>
       <c r="H9" t="n">
-        <v>0.5853350604923128</v>
+        <v>0.5839873189206765</v>
       </c>
       <c r="I9" t="n">
-        <v>37.49420670477369</v>
+        <v>34.93084593116758</v>
       </c>
       <c r="J9" t="n">
         <v>50</v>
@@ -4428,7 +4428,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M9" t="n">
@@ -4438,10 +4438,10 @@
         <v>50</v>
       </c>
       <c r="O9" t="n">
-        <v>97.87234042553192</v>
+        <v>95.74468085106383</v>
       </c>
       <c r="P9" t="n">
-        <v>61.50646808510639</v>
+        <v>61.08093617021277</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -4468,22 +4468,22 @@
         <v>2682.4</v>
       </c>
       <c r="D10" t="n">
-        <v>0.0562293274531422</v>
+        <v>0.0467085495766186</v>
       </c>
       <c r="E10" t="n">
-        <v>0.0058874264071699</v>
+        <v>0.045036621474209</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.1198031173092698</v>
+        <v>-0.1187331624942505</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.0992304759712956</v>
+        <v>-0.0981605211562763</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.0649633855671776</v>
+        <v>-0.0638934307521583</v>
       </c>
       <c r="I10" t="n">
-        <v>44.36388353914127</v>
+        <v>47.54158067257497</v>
       </c>
       <c r="J10" t="n">
         <v>80</v>
@@ -4493,7 +4493,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M10" t="n">
@@ -4533,22 +4533,22 @@
         <v>543.95</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.0612649926654585</v>
+        <v>-0.0517737296260785</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.071995223065768</v>
+        <v>-0.0655385672564851</v>
       </c>
       <c r="F11" t="n">
-        <v>0.0716115051221435</v>
+        <v>0.0735149003355044</v>
       </c>
       <c r="G11" t="n">
-        <v>0.0921841464601177</v>
+        <v>0.0940875416734786</v>
       </c>
       <c r="H11" t="n">
-        <v>0.1264512368642357</v>
+        <v>0.1283546320775966</v>
       </c>
       <c r="I11" t="n">
-        <v>54.80591497227357</v>
+        <v>57.42414460942543</v>
       </c>
       <c r="J11" t="n">
         <v>60</v>
@@ -4558,7 +4558,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M11" t="n">
@@ -4598,22 +4598,22 @@
         <v>697.65</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.0896457232335095</v>
+        <v>-0.07239728759473479</v>
       </c>
       <c r="E12" t="n">
-        <v>0.1612983770287139</v>
+        <v>0.1617818484596169</v>
       </c>
       <c r="F12" t="n">
-        <v>0.0669062547790182</v>
+        <v>0.053215579710145</v>
       </c>
       <c r="G12" t="n">
-        <v>0.0874788961169924</v>
+        <v>0.0737882210481192</v>
       </c>
       <c r="H12" t="n">
-        <v>0.1217459865211104</v>
+        <v>0.1080553114522372</v>
       </c>
       <c r="I12" t="n">
-        <v>49.20332525112573</v>
+        <v>45.66506113375324</v>
       </c>
       <c r="J12" t="n">
         <v>60</v>
@@ -4623,7 +4623,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M12" t="n">
@@ -4633,10 +4633,10 @@
         <v>60</v>
       </c>
       <c r="O12" t="n">
-        <v>72.3404255319149</v>
+        <v>70.21276595744681</v>
       </c>
       <c r="P12" t="n">
-        <v>58.43608510638298</v>
+        <v>58.01055319148936</v>
       </c>
       <c r="Q12" t="b">
         <v>0</v>
@@ -4651,63 +4651,63 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>RANEENGINE</t>
+          <t>LUMAXIND</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Engine/Parts</t>
+          <t>Lighting</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>317.75</v>
+        <v>5148.5</v>
       </c>
       <c r="D13" t="n">
-        <v>0.1790352504638219</v>
+        <v>-0.1348222087786516</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.156154561147258</v>
+        <v>-0.08552397868561271</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.2401052253975846</v>
+        <v>0.2348003357716752</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.2195325840596104</v>
+        <v>0.2553729771096494</v>
       </c>
       <c r="H13" t="n">
-        <v>-0.1852654936554923</v>
+        <v>0.2896400675137675</v>
       </c>
       <c r="I13" t="n">
-        <v>63.3225806451613</v>
+        <v>40.8936170212766</v>
       </c>
       <c r="J13" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="K13" t="n">
-        <v>50.88</v>
+        <v>57.69</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M13" t="n">
-        <v>50.88</v>
+        <v>57.69</v>
       </c>
       <c r="N13" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="O13" t="n">
-        <v>17.02127659574468</v>
+        <v>89.36170212765957</v>
       </c>
       <c r="P13" t="n">
-        <v>55.75625531914894</v>
+        <v>56.94834042553191</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
       </c>
       <c r="R13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S13" t="b">
         <v>0</v>
@@ -4716,63 +4716,63 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>LUMAXIND</t>
+          <t>RANEENGINE</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Lighting</t>
+          <t>Engine/Parts</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>5148.5</v>
+        <v>317.75</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.1565781498288092</v>
+        <v>0.1790352504638219</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.09189522885616019</v>
+        <v>-0.156154561147258</v>
       </c>
       <c r="F14" t="n">
-        <v>0.2336759878273788</v>
+        <v>-0.2401052253975846</v>
       </c>
       <c r="G14" t="n">
-        <v>0.254248629165353</v>
+        <v>-0.2195325840596104</v>
       </c>
       <c r="H14" t="n">
-        <v>0.2885157195694711</v>
+        <v>-0.1852654936554923</v>
       </c>
       <c r="I14" t="n">
-        <v>38.56340288924559</v>
+        <v>63.3225806451613</v>
       </c>
       <c r="J14" t="n">
-        <v>30</v>
+        <v>80</v>
       </c>
       <c r="K14" t="n">
-        <v>57.69</v>
+        <v>50.88</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M14" t="n">
-        <v>57.69</v>
+        <v>50.88</v>
       </c>
       <c r="N14" t="n">
-        <v>30</v>
+        <v>80</v>
       </c>
       <c r="O14" t="n">
-        <v>89.36170212765957</v>
+        <v>17.02127659574468</v>
       </c>
       <c r="P14" t="n">
-        <v>52.94834042553191</v>
+        <v>55.75625531914894</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
       </c>
       <c r="R14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S14" t="b">
         <v>0</v>
@@ -4781,57 +4781,57 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PRICOLLTD</t>
+          <t>FIEMIND</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Lighting</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>543.95</v>
+        <v>2083.6</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.1378189887462354</v>
+        <v>-0.0711483594864479</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.0963535177340311</v>
+        <v>-0.0806159819970878</v>
       </c>
       <c r="F15" t="n">
-        <v>0.1429922252574071</v>
+        <v>-0.0442201834862385</v>
       </c>
       <c r="G15" t="n">
-        <v>0.1635648665953814</v>
+        <v>-0.0236475421482643</v>
       </c>
       <c r="H15" t="n">
-        <v>0.1978319569994994</v>
+        <v>0.0106195482558536</v>
       </c>
       <c r="I15" t="n">
-        <v>44.98910675381264</v>
+        <v>49.18561995597947</v>
       </c>
       <c r="J15" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K15" t="n">
-        <v>49.98</v>
+        <v>49.06</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M15" t="n">
-        <v>49.98</v>
+        <v>49.06</v>
       </c>
       <c r="N15" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O15" t="n">
-        <v>80.85106382978722</v>
+        <v>57.44680851063831</v>
       </c>
       <c r="P15" t="n">
-        <v>52.16221276595745</v>
+        <v>55.11336170212766</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
@@ -4858,22 +4858,22 @@
         <v>396.15</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.0439242186557259</v>
+        <v>-0.0526126987922994</v>
       </c>
       <c r="E16" t="n">
-        <v>0.2727710843373494</v>
+        <v>0.3187416777629828</v>
       </c>
       <c r="F16" t="n">
-        <v>0.2610218048702848</v>
+        <v>0.2502761559097364</v>
       </c>
       <c r="G16" t="n">
-        <v>0.281594446208259</v>
+        <v>0.2708487972477106</v>
       </c>
       <c r="H16" t="n">
-        <v>0.315861536612377</v>
+        <v>0.3051158876518286</v>
       </c>
       <c r="I16" t="n">
-        <v>39.38129996524157</v>
+        <v>39.50488145048813</v>
       </c>
       <c r="J16" t="n">
         <v>30</v>
@@ -4883,7 +4883,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="M16" t="n">

</xml_diff>

<commit_message>
chore: auto-refresh NSE data and pipeline outputs (2026-03-27)
</commit_message>
<xml_diff>
--- a/working-sector/output/auto_components_comprehensive_report.xlsx
+++ b/working-sector/output/auto_components_comprehensive_report.xlsx
@@ -435,7 +435,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
     </row>
@@ -447,7 +447,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
     </row>
@@ -779,25 +779,25 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1736.5</v>
+        <v>1725.1</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.06554377656998329</v>
+        <v>-0.0930073606729758</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2641962725684335</v>
+        <v>0.2470902913323212</v>
       </c>
       <c r="F2" t="n">
-        <v>0.5291475871785842</v>
+        <v>0.5247480996994871</v>
       </c>
       <c r="G2" t="n">
-        <v>0.5497202285165584</v>
+        <v>0.5453207410374613</v>
       </c>
       <c r="H2" t="n">
-        <v>0.5839873189206765</v>
+        <v>0.5795878314415793</v>
       </c>
       <c r="I2" t="n">
-        <v>34.93084593116758</v>
+        <v>37.99860041987404</v>
       </c>
       <c r="J2" t="n">
         <v>50</v>
@@ -807,7 +807,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M2" t="n">
@@ -817,10 +817,10 @@
         <v>50</v>
       </c>
       <c r="O2" t="n">
-        <v>95.74468085106383</v>
+        <v>97.87234042553192</v>
       </c>
       <c r="P2" t="n">
-        <v>61.08093617021277</v>
+        <v>61.50646808510639</v>
       </c>
       <c r="Q2" t="b">
         <v>0</v>
@@ -844,25 +844,25 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1087.6</v>
+        <v>1048.7</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.0763481953290871</v>
+        <v>-0.1388569551650517</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.1355905261484661</v>
+        <v>-0.1485751400503369</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.1524314214463841</v>
+        <v>-0.1798701806522249</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.1318587801084099</v>
+        <v>-0.1592975393142507</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.0975916897042918</v>
+        <v>-0.1250304489101327</v>
       </c>
       <c r="I3" t="n">
-        <v>45.68059471930274</v>
+        <v>45.71575166752181</v>
       </c>
       <c r="J3" t="n">
         <v>40</v>
@@ -872,7 +872,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M3" t="n">
@@ -909,25 +909,25 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>30390</v>
+        <v>29615</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.1398245117463912</v>
+        <v>-0.1901832102816516</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.1695586828801748</v>
+        <v>-0.1948069603045132</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.2605839416058394</v>
+        <v>-0.273073146784487</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.2400113002678652</v>
+        <v>-0.2525005054465128</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.2057442098637472</v>
+        <v>-0.2182334150423948</v>
       </c>
       <c r="I4" t="n">
-        <v>32.80793928779919</v>
+        <v>36.94937541091387</v>
       </c>
       <c r="J4" t="n">
         <v>30</v>
@@ -937,7 +937,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M4" t="n">
@@ -974,25 +974,25 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>307.15</v>
+        <v>300.85</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.0857270427146896</v>
+        <v>-0.1081962353638654</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.177093101138647</v>
+        <v>-0.1942956614890196</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.2671200190885231</v>
+        <v>-0.2583507950203376</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.2465473777505489</v>
+        <v>-0.2377781536823634</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.2122802873464309</v>
+        <v>-0.2035110632782454</v>
       </c>
       <c r="I5" t="n">
-        <v>44.92502883506344</v>
+        <v>45.31704479348461</v>
       </c>
       <c r="J5" t="n">
         <v>40</v>
@@ -1002,7 +1002,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M5" t="n">
@@ -1012,10 +1012,10 @@
         <v>40</v>
       </c>
       <c r="O5" t="n">
-        <v>10.63829787234042</v>
+        <v>14.8936170212766</v>
       </c>
       <c r="P5" t="n">
-        <v>38.57565957446808</v>
+        <v>39.42672340425532</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
@@ -1039,25 +1039,25 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>113.13</v>
+        <v>109.38</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.1400881726968683</v>
+        <v>-0.179075352746923</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.0188204683434518</v>
+        <v>-0.0631263383297644</v>
       </c>
       <c r="F6" t="n">
-        <v>0.1719672640629854</v>
+        <v>0.1596692111959288</v>
       </c>
       <c r="G6" t="n">
-        <v>0.1925399054009596</v>
+        <v>0.180241852533903</v>
       </c>
       <c r="H6" t="n">
-        <v>0.2268069958050776</v>
+        <v>0.214508942938021</v>
       </c>
       <c r="I6" t="n">
-        <v>38.65882352941176</v>
+        <v>39.62855764592377</v>
       </c>
       <c r="J6" t="n">
         <v>30</v>
@@ -1067,7 +1067,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M6" t="n">
@@ -1104,48 +1104,48 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2682.4</v>
+        <v>2566.3</v>
       </c>
       <c r="D7" t="n">
-        <v>0.0467085495766186</v>
+        <v>-0.0200099285905218</v>
       </c>
       <c r="E7" t="n">
-        <v>0.045036621474209</v>
+        <v>-0.0335542667771333</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.1187331624942505</v>
+        <v>-0.143681804531349</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.0981605211562763</v>
+        <v>-0.1231091631933748</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.0638934307521583</v>
+        <v>-0.08884207278925681</v>
       </c>
       <c r="I7" t="n">
-        <v>47.54158067257497</v>
+        <v>47.43791641429439</v>
       </c>
       <c r="J7" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K7" t="n">
         <v>48.73</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M7" t="n">
         <v>48.73</v>
       </c>
       <c r="N7" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O7" t="n">
-        <v>38.29787234042553</v>
+        <v>36.17021276595745</v>
       </c>
       <c r="P7" t="n">
-        <v>59.15157446808512</v>
+        <v>50.7260425531915</v>
       </c>
       <c r="Q7" t="b">
         <v>0</v>
@@ -1169,48 +1169,48 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>511.45</v>
+        <v>488.75</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.0339975446217774</v>
+        <v>-0.0982472324723247</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0516089236146806</v>
+        <v>0.0200354794949391</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1365555555555555</v>
+        <v>0.1159949765955017</v>
       </c>
       <c r="G8" t="n">
-        <v>0.1571281968935297</v>
+        <v>0.1365676179334759</v>
       </c>
       <c r="H8" t="n">
-        <v>0.1913952872976477</v>
+        <v>0.1708347083375939</v>
       </c>
       <c r="I8" t="n">
-        <v>48.86658031088081</v>
+        <v>46.33097942892233</v>
       </c>
       <c r="J8" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="K8" t="n">
         <v>49.66</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M8" t="n">
         <v>49.66</v>
       </c>
       <c r="N8" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="O8" t="n">
         <v>82.97872340425532</v>
       </c>
       <c r="P8" t="n">
-        <v>68.45974468085107</v>
+        <v>52.45974468085107</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
@@ -1234,25 +1234,25 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>419.65</v>
+        <v>412.45</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.0771852666300165</v>
+        <v>-0.1096600107933082</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.1935235898914192</v>
+        <v>-0.2137819290888296</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.1359003397508493</v>
+        <v>-0.1504634397528321</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.1153276984128751</v>
+        <v>-0.1298907984148579</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.0810606080087571</v>
+        <v>-0.0956237080107399</v>
       </c>
       <c r="I9" t="n">
-        <v>41.68734491315136</v>
+        <v>42.37074401008826</v>
       </c>
       <c r="J9" t="n">
         <v>40</v>
@@ -1262,7 +1262,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M9" t="n">
@@ -1272,10 +1272,10 @@
         <v>40</v>
       </c>
       <c r="O9" t="n">
-        <v>36.17021276595745</v>
+        <v>34.04255319148936</v>
       </c>
       <c r="P9" t="n">
-        <v>44.6100425531915</v>
+        <v>44.18451063829788</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -1299,25 +1299,25 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>129970</v>
+        <v>129575</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.0971170545328239</v>
+        <v>-0.1220313717518718</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.1532899022801302</v>
+        <v>-0.1494633890183465</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.1366987711723679</v>
+        <v>-0.1341752697871772</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.1161261298343937</v>
+        <v>-0.1136026284492029</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.0818590394302757</v>
+        <v>-0.07933553804508491</v>
       </c>
       <c r="I10" t="n">
-        <v>35.37030886748589</v>
+        <v>39.9624765478424</v>
       </c>
       <c r="J10" t="n">
         <v>30</v>
@@ -1327,7 +1327,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M10" t="n">
@@ -1337,10 +1337,10 @@
         <v>30</v>
       </c>
       <c r="O10" t="n">
-        <v>34.04255319148936</v>
+        <v>40.42553191489361</v>
       </c>
       <c r="P10" t="n">
-        <v>38.57251063829787</v>
+        <v>39.84910638297872</v>
       </c>
       <c r="Q10" t="b">
         <v>0</v>
@@ -1392,7 +1392,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M11" t="n">
@@ -1402,10 +1402,10 @@
         <v>20</v>
       </c>
       <c r="O11" t="n">
-        <v>65.95744680851064</v>
+        <v>61.70212765957447</v>
       </c>
       <c r="P11" t="n">
-        <v>25.19148936170213</v>
+        <v>24.3404255319149</v>
       </c>
       <c r="Q11" t="b">
         <v>0</v>
@@ -1429,48 +1429,48 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>444.15</v>
+        <v>438.75</v>
       </c>
       <c r="D12" t="n">
-        <v>0.0382187938288918</v>
+        <v>0.0277582572030921</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.0300283904782703</v>
+        <v>-0.0647980390067142</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.1372377622377621</v>
+        <v>-0.15625</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.1166651208997879</v>
+        <v>-0.1356773586620258</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.08239803049566991</v>
+        <v>-0.1014102682579077</v>
       </c>
       <c r="I12" t="n">
-        <v>69.2562592047128</v>
+        <v>72.65353418308227</v>
       </c>
       <c r="J12" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K12" t="n">
         <v>71.28</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M12" t="n">
         <v>71.28</v>
       </c>
       <c r="N12" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O12" t="n">
         <v>31.91489361702128</v>
       </c>
       <c r="P12" t="n">
-        <v>66.89497872340425</v>
+        <v>62.89497872340426</v>
       </c>
       <c r="Q12" t="b">
         <v>1</v>
@@ -1494,25 +1494,25 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1650.4</v>
+        <v>1585.4</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.1761593370937951</v>
+        <v>-0.2271242626627017</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.1021163157608399</v>
+        <v>-0.1379010331702012</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.0617929623102722</v>
+        <v>-0.0852757904454188</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.041220320972298</v>
+        <v>-0.0647031491074446</v>
       </c>
       <c r="H13" t="n">
-        <v>-0.0069532305681799</v>
+        <v>-0.0304360587033266</v>
       </c>
       <c r="I13" t="n">
-        <v>19.62093862815885</v>
+        <v>18.72846312887664</v>
       </c>
       <c r="J13" t="n">
         <v>20</v>
@@ -1522,7 +1522,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M13" t="n">
@@ -1532,10 +1532,10 @@
         <v>20</v>
       </c>
       <c r="O13" t="n">
-        <v>55.31914893617022</v>
+        <v>57.44680851063831</v>
       </c>
       <c r="P13" t="n">
-        <v>42.57182978723405</v>
+        <v>42.99736170212766</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
@@ -1559,25 +1559,25 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>560.75</v>
+        <v>531.65</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.1396240889911776</v>
+        <v>-0.1689073002970142</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.2056802889723068</v>
+        <v>-0.2702127659574468</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.1111199175715305</v>
+        <v>-0.1257913343747431</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.0905472762335563</v>
+        <v>-0.1052186930367689</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.0562801858294382</v>
+        <v>-0.0709516026326508</v>
       </c>
       <c r="I14" t="n">
-        <v>44.35548438751002</v>
+        <v>42.39795918367346</v>
       </c>
       <c r="J14" t="n">
         <v>40</v>
@@ -1587,7 +1587,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M14" t="n">
@@ -1597,10 +1597,10 @@
         <v>40</v>
       </c>
       <c r="O14" t="n">
-        <v>48.93617021276596</v>
+        <v>46.80851063829788</v>
       </c>
       <c r="P14" t="n">
-        <v>47.6432340425532</v>
+        <v>47.21770212765958</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
@@ -1624,25 +1624,25 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>95.70999999999999</v>
+        <v>89.41</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.1147798742138366</v>
+        <v>-0.1747277090640576</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.0038509575353872</v>
+        <v>-0.0652378463146891</v>
       </c>
       <c r="F15" t="n">
-        <v>0.0621462656752858</v>
+        <v>0.0273468918763644</v>
       </c>
       <c r="G15" t="n">
-        <v>0.08271890701326</v>
+        <v>0.0479195332143386</v>
       </c>
       <c r="H15" t="n">
-        <v>0.116985997417378</v>
+        <v>0.08218662361845661</v>
       </c>
       <c r="I15" t="n">
-        <v>42.68423883808498</v>
+        <v>41.1353032659409</v>
       </c>
       <c r="J15" t="n">
         <v>40</v>
@@ -1652,7 +1652,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M15" t="n">
@@ -1689,25 +1689,25 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>158.74</v>
+        <v>149.85</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.2043107769423559</v>
+        <v>-0.2340523410345532</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.0377061105722599</v>
+        <v>-0.1126835622927522</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.0376477720521368</v>
+        <v>-0.0820826952526799</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.0170751307141626</v>
+        <v>-0.0615100539147057</v>
       </c>
       <c r="H16" t="n">
-        <v>0.0171919596899553</v>
+        <v>-0.0272429635105877</v>
       </c>
       <c r="I16" t="n">
-        <v>37.17466743782533</v>
+        <v>35.57985053971767</v>
       </c>
       <c r="J16" t="n">
         <v>30</v>
@@ -1717,7 +1717,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M16" t="n">
@@ -1736,7 +1736,7 @@
         <v>0</v>
       </c>
       <c r="R16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S16" t="b">
         <v>0</v>
@@ -1754,25 +1754,25 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>7049</v>
+        <v>6924</v>
       </c>
       <c r="D17" t="n">
-        <v>-0.1050593537738843</v>
+        <v>-0.1117382937780628</v>
       </c>
       <c r="E17" t="n">
-        <v>0.0202634245187436</v>
+        <v>-0.0214810627473148</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0219644798840159</v>
+        <v>0.0129471143296027</v>
       </c>
       <c r="G17" t="n">
-        <v>0.0425371212219901</v>
+        <v>0.0335197556675769</v>
       </c>
       <c r="H17" t="n">
-        <v>0.07680421162610809</v>
+        <v>0.0677868460716949</v>
       </c>
       <c r="I17" t="n">
-        <v>41.25320786997433</v>
+        <v>42.07197382769901</v>
       </c>
       <c r="J17" t="n">
         <v>40</v>
@@ -1782,7 +1782,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M17" t="n">
@@ -1792,10 +1792,10 @@
         <v>40</v>
       </c>
       <c r="O17" t="n">
-        <v>68.08510638297872</v>
+        <v>70.21276595744681</v>
       </c>
       <c r="P17" t="n">
-        <v>51.47702127659574</v>
+        <v>51.90255319148936</v>
       </c>
       <c r="Q17" t="b">
         <v>0</v>
@@ -1819,25 +1819,25 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>697.65</v>
+        <v>674.75</v>
       </c>
       <c r="D18" t="n">
-        <v>-0.07239728759473479</v>
+        <v>-0.059909439219784</v>
       </c>
       <c r="E18" t="n">
-        <v>0.1617818484596169</v>
+        <v>0.1113398665898048</v>
       </c>
       <c r="F18" t="n">
-        <v>0.053215579710145</v>
+        <v>-0.0029553010712966</v>
       </c>
       <c r="G18" t="n">
-        <v>0.0737882210481192</v>
+        <v>0.0176173402666776</v>
       </c>
       <c r="H18" t="n">
-        <v>0.1080553114522372</v>
+        <v>0.0518844306707956</v>
       </c>
       <c r="I18" t="n">
-        <v>45.66506113375324</v>
+        <v>40.25722339675829</v>
       </c>
       <c r="J18" t="n">
         <v>60</v>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M18" t="n">
@@ -1857,10 +1857,10 @@
         <v>60</v>
       </c>
       <c r="O18" t="n">
-        <v>70.21276595744681</v>
+        <v>65.95744680851064</v>
       </c>
       <c r="P18" t="n">
-        <v>58.01055319148936</v>
+        <v>57.15948936170213</v>
       </c>
       <c r="Q18" t="b">
         <v>0</v>
@@ -1884,25 +1884,25 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2333.1</v>
+        <v>2260</v>
       </c>
       <c r="D19" t="n">
-        <v>-0.1310614525139665</v>
+        <v>-0.1553927797294267</v>
       </c>
       <c r="E19" t="n">
-        <v>-0.1226308664259927</v>
+        <v>-0.1388835968755953</v>
       </c>
       <c r="F19" t="n">
-        <v>-0.1992380560131795</v>
+        <v>-0.2295104322923769</v>
       </c>
       <c r="G19" t="n">
-        <v>-0.1786654146752053</v>
+        <v>-0.2089377909544026</v>
       </c>
       <c r="H19" t="n">
-        <v>-0.1443983242710873</v>
+        <v>-0.1746707005502846</v>
       </c>
       <c r="I19" t="n">
-        <v>39.51968921066571</v>
+        <v>36.59254414650099</v>
       </c>
       <c r="J19" t="n">
         <v>30</v>
@@ -1912,7 +1912,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M19" t="n">
@@ -1949,54 +1949,54 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2083.6</v>
+        <v>1966.1</v>
       </c>
       <c r="D20" t="n">
-        <v>-0.0711483594864479</v>
+        <v>-0.1309287008796359</v>
       </c>
       <c r="E20" t="n">
-        <v>-0.0806159819970878</v>
+        <v>-0.1352860975502484</v>
       </c>
       <c r="F20" t="n">
-        <v>-0.0442201834862385</v>
+        <v>-0.0962952748667034</v>
       </c>
       <c r="G20" t="n">
-        <v>-0.0236475421482643</v>
+        <v>-0.0757226335287292</v>
       </c>
       <c r="H20" t="n">
-        <v>0.0106195482558536</v>
+        <v>-0.0414555431246111</v>
       </c>
       <c r="I20" t="n">
-        <v>49.18561995597947</v>
+        <v>45.03560392314927</v>
       </c>
       <c r="J20" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="K20" t="n">
         <v>49.06</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M20" t="n">
         <v>49.06</v>
       </c>
       <c r="N20" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="O20" t="n">
-        <v>57.44680851063831</v>
+        <v>53.19148936170212</v>
       </c>
       <c r="P20" t="n">
-        <v>55.11336170212766</v>
+        <v>46.26229787234043</v>
       </c>
       <c r="Q20" t="b">
         <v>0</v>
       </c>
       <c r="R20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S20" t="b">
         <v>0</v>
@@ -2014,25 +2014,25 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>881.25</v>
+        <v>823.1</v>
       </c>
       <c r="D21" t="n">
-        <v>-0.087544004969973</v>
+        <v>-0.1863384737050217</v>
       </c>
       <c r="E21" t="n">
-        <v>-0.0508885298869143</v>
+        <v>-0.1568326162671584</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.2794358135731807</v>
+        <v>-0.3265423007691049</v>
       </c>
       <c r="G21" t="n">
-        <v>-0.2588631722352065</v>
+        <v>-0.3059696594311307</v>
       </c>
       <c r="H21" t="n">
-        <v>-0.2245960818310884</v>
+        <v>-0.2717025690270127</v>
       </c>
       <c r="I21" t="n">
-        <v>44.44973041547733</v>
+        <v>42.23293656772639</v>
       </c>
       <c r="J21" t="n">
         <v>40</v>
@@ -2042,7 +2042,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M21" t="n">
@@ -2079,25 +2079,25 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>396.15</v>
+        <v>377.85</v>
       </c>
       <c r="D22" t="n">
-        <v>-0.0526126987922994</v>
+        <v>-0.1040901007705986</v>
       </c>
       <c r="E22" t="n">
-        <v>0.3187416777629828</v>
+        <v>0.2341989220970115</v>
       </c>
       <c r="F22" t="n">
-        <v>0.2502761559097364</v>
+        <v>0.2218270008084075</v>
       </c>
       <c r="G22" t="n">
-        <v>0.2708487972477106</v>
+        <v>0.2423996421463817</v>
       </c>
       <c r="H22" t="n">
-        <v>0.3051158876518286</v>
+        <v>0.2766667325504998</v>
       </c>
       <c r="I22" t="n">
-        <v>39.50488145048813</v>
+        <v>33.32275468105364</v>
       </c>
       <c r="J22" t="n">
         <v>30</v>
@@ -2107,7 +2107,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M22" t="n">
@@ -2144,25 +2144,25 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>335.15</v>
+        <v>322.35</v>
       </c>
       <c r="D23" t="n">
-        <v>-0.08416450334745181</v>
+        <v>-0.1374096869146372</v>
       </c>
       <c r="E23" t="n">
-        <v>-0.096508963472166</v>
+        <v>-0.1297246220302375</v>
       </c>
       <c r="F23" t="n">
-        <v>-0.1782518082628418</v>
+        <v>-0.2039757994814174</v>
       </c>
       <c r="G23" t="n">
-        <v>-0.1576791669248676</v>
+        <v>-0.1834031581434432</v>
       </c>
       <c r="H23" t="n">
-        <v>-0.1234120765207495</v>
+        <v>-0.1491360677393252</v>
       </c>
       <c r="I23" t="n">
-        <v>25.85278276481147</v>
+        <v>23.52941176470587</v>
       </c>
       <c r="J23" t="n">
         <v>20</v>
@@ -2172,7 +2172,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M23" t="n">
@@ -2209,48 +2209,48 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>121.47</v>
+        <v>116.62</v>
       </c>
       <c r="D24" t="n">
-        <v>-0.1499650104968509</v>
+        <v>-0.1895197720480922</v>
       </c>
       <c r="E24" t="n">
-        <v>0.0396268401232453</v>
+        <v>-0.0477668000326609</v>
       </c>
       <c r="F24" t="n">
-        <v>0.1158368546757302</v>
+        <v>0.0995662832359043</v>
       </c>
       <c r="G24" t="n">
-        <v>0.1364094960137044</v>
+        <v>0.1201389245738785</v>
       </c>
       <c r="H24" t="n">
-        <v>0.1706765864178224</v>
+        <v>0.1544060149779965</v>
       </c>
       <c r="I24" t="n">
-        <v>39.83516483516484</v>
+        <v>44.2432872253865</v>
       </c>
       <c r="J24" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K24" t="n">
         <v>48.3</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M24" t="n">
         <v>48.3</v>
       </c>
       <c r="N24" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O24" t="n">
         <v>80.85106382978722</v>
       </c>
       <c r="P24" t="n">
-        <v>47.49021276595744</v>
+        <v>51.49021276595744</v>
       </c>
       <c r="Q24" t="b">
         <v>0</v>
@@ -2274,48 +2274,48 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>572.65</v>
+        <v>546.65</v>
       </c>
       <c r="D25" t="n">
-        <v>0.0290206648697213</v>
+        <v>-0.0176116452511457</v>
       </c>
       <c r="E25" t="n">
-        <v>0.0094306363476115</v>
+        <v>-0.0434820647419073</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.06802831800797469</v>
+        <v>-0.09860664523043949</v>
       </c>
       <c r="G25" t="n">
-        <v>-0.0474556766700005</v>
+        <v>-0.0780340038924652</v>
       </c>
       <c r="H25" t="n">
-        <v>-0.0131885862658824</v>
+        <v>-0.0437669134883472</v>
       </c>
       <c r="I25" t="n">
-        <v>59.15238954012625</v>
+        <v>56.43496214728149</v>
       </c>
       <c r="J25" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K25" t="n">
         <v>56.91</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M25" t="n">
         <v>56.91</v>
       </c>
       <c r="N25" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O25" t="n">
-        <v>53.19148936170212</v>
+        <v>51.06382978723404</v>
       </c>
       <c r="P25" t="n">
-        <v>65.40229787234043</v>
+        <v>56.9767659574468</v>
       </c>
       <c r="Q25" t="b">
         <v>0</v>
@@ -2339,48 +2339,48 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>125.84</v>
+        <v>120.82</v>
       </c>
       <c r="D26" t="n">
-        <v>-0.07531780439415089</v>
+        <v>-0.1401323749199344</v>
       </c>
       <c r="E26" t="n">
-        <v>-0.1102941176470587</v>
+        <v>-0.1724090691143229</v>
       </c>
       <c r="F26" t="n">
-        <v>-0.1170981547744334</v>
+        <v>-0.157696597880647</v>
       </c>
       <c r="G26" t="n">
-        <v>-0.0965255134364592</v>
+        <v>-0.1371239565426728</v>
       </c>
       <c r="H26" t="n">
-        <v>-0.0622584230323411</v>
+        <v>-0.1028568661385548</v>
       </c>
       <c r="I26" t="n">
-        <v>41.66666666666666</v>
+        <v>39.0909090909091</v>
       </c>
       <c r="J26" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K26" t="n">
         <v>51.54</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M26" t="n">
         <v>51.54</v>
       </c>
       <c r="N26" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O26" t="n">
-        <v>40.42553191489361</v>
+        <v>29.78723404255319</v>
       </c>
       <c r="P26" t="n">
-        <v>44.70110638297872</v>
+        <v>38.57344680851064</v>
       </c>
       <c r="Q26" t="b">
         <v>0</v>
@@ -2404,25 +2404,25 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>5148.5</v>
+        <v>4880</v>
       </c>
       <c r="D27" t="n">
-        <v>-0.1348222087786516</v>
+        <v>-0.214752357352042</v>
       </c>
       <c r="E27" t="n">
-        <v>-0.08552397868561271</v>
+        <v>-0.152041702867072</v>
       </c>
       <c r="F27" t="n">
-        <v>0.2348003357716752</v>
+        <v>0.1645110485372021</v>
       </c>
       <c r="G27" t="n">
-        <v>0.2553729771096494</v>
+        <v>0.1850836898751763</v>
       </c>
       <c r="H27" t="n">
-        <v>0.2896400675137675</v>
+        <v>0.2193507802792943</v>
       </c>
       <c r="I27" t="n">
-        <v>40.8936170212766</v>
+        <v>42.24175824175824</v>
       </c>
       <c r="J27" t="n">
         <v>40</v>
@@ -2432,7 +2432,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M27" t="n">
@@ -2442,10 +2442,10 @@
         <v>40</v>
       </c>
       <c r="O27" t="n">
-        <v>89.36170212765957</v>
+        <v>87.2340425531915</v>
       </c>
       <c r="P27" t="n">
-        <v>56.94834042553191</v>
+        <v>56.5228085106383</v>
       </c>
       <c r="Q27" t="b">
         <v>0</v>
@@ -2469,25 +2469,25 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1623.3</v>
+        <v>1608.8</v>
       </c>
       <c r="D28" t="n">
-        <v>-0.0295330902134274</v>
+        <v>-0.064107038976149</v>
       </c>
       <c r="E28" t="n">
-        <v>0.09100073929699549</v>
+        <v>0.0642323212277566</v>
       </c>
       <c r="F28" t="n">
-        <v>0.5489503816793893</v>
+        <v>0.5187387897668272</v>
       </c>
       <c r="G28" t="n">
-        <v>0.5695230230173635</v>
+        <v>0.5393114311048014</v>
       </c>
       <c r="H28" t="n">
-        <v>0.6037901134214815</v>
+        <v>0.5735785215089194</v>
       </c>
       <c r="I28" t="n">
-        <v>55.99580162686958</v>
+        <v>59.15453915453915</v>
       </c>
       <c r="J28" t="n">
         <v>80</v>
@@ -2497,7 +2497,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M28" t="n">
@@ -2507,10 +2507,10 @@
         <v>80</v>
       </c>
       <c r="O28" t="n">
-        <v>97.87234042553192</v>
+        <v>95.74468085106383</v>
       </c>
       <c r="P28" t="n">
-        <v>73.37846808510639</v>
+        <v>72.95293617021277</v>
       </c>
       <c r="Q28" t="b">
         <v>0</v>
@@ -2534,25 +2534,25 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>543.95</v>
+        <v>528.7</v>
       </c>
       <c r="D29" t="n">
-        <v>-0.0517737296260785</v>
+        <v>-0.0871104204437536</v>
       </c>
       <c r="E29" t="n">
-        <v>-0.0655385672564851</v>
+        <v>-0.090643274853801</v>
       </c>
       <c r="F29" t="n">
-        <v>0.0735149003355044</v>
+        <v>0.0521393034825872</v>
       </c>
       <c r="G29" t="n">
-        <v>0.0940875416734786</v>
+        <v>0.0727119448205614</v>
       </c>
       <c r="H29" t="n">
-        <v>0.1283546320775966</v>
+        <v>0.1069790352246794</v>
       </c>
       <c r="I29" t="n">
-        <v>57.42414460942543</v>
+        <v>60.57201225740555</v>
       </c>
       <c r="J29" t="n">
         <v>60</v>
@@ -2562,7 +2562,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M29" t="n">
@@ -2572,10 +2572,10 @@
         <v>60</v>
       </c>
       <c r="O29" t="n">
-        <v>74.46808510638297</v>
+        <v>78.72340425531915</v>
       </c>
       <c r="P29" t="n">
-        <v>58.6616170212766</v>
+        <v>59.51268085106384</v>
       </c>
       <c r="Q29" t="b">
         <v>0</v>
@@ -2599,25 +2599,25 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>111.94</v>
+        <v>109.22</v>
       </c>
       <c r="D30" t="n">
-        <v>-0.0357481264536135</v>
+        <v>-0.0545360110803323</v>
       </c>
       <c r="E30" t="n">
-        <v>0.0496015002344114</v>
+        <v>0.0213203665606882</v>
       </c>
       <c r="F30" t="n">
-        <v>-0.1141183918961696</v>
+        <v>-0.1213900732040865</v>
       </c>
       <c r="G30" t="n">
-        <v>-0.0935457505581954</v>
+        <v>-0.1008174318661123</v>
       </c>
       <c r="H30" t="n">
-        <v>-0.0592786601540774</v>
+        <v>-0.0665503414619943</v>
       </c>
       <c r="I30" t="n">
-        <v>42.44075183873605</v>
+        <v>40.5096203848154</v>
       </c>
       <c r="J30" t="n">
         <v>40</v>
@@ -2627,7 +2627,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M30" t="n">
@@ -2637,10 +2637,10 @@
         <v>40</v>
       </c>
       <c r="O30" t="n">
-        <v>42.5531914893617</v>
+        <v>48.93617021276596</v>
       </c>
       <c r="P30" t="n">
-        <v>45.46263829787234</v>
+        <v>46.73923404255319</v>
       </c>
       <c r="Q30" t="b">
         <v>0</v>
@@ -2664,25 +2664,25 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>37.98</v>
+        <v>37.9</v>
       </c>
       <c r="D31" t="n">
-        <v>-0.1290988305434534</v>
+        <v>-0.1301354142758779</v>
       </c>
       <c r="E31" t="n">
-        <v>-0.1522321428571429</v>
+        <v>-0.153072625698324</v>
       </c>
       <c r="F31" t="n">
-        <v>-0.1140657802659202</v>
+        <v>-0.1415628539071347</v>
       </c>
       <c r="G31" t="n">
-        <v>-0.093493138927946</v>
+        <v>-0.1209902125691605</v>
       </c>
       <c r="H31" t="n">
-        <v>-0.059226048523828</v>
+        <v>-0.08672312216504249</v>
       </c>
       <c r="I31" t="n">
-        <v>31.70189098998885</v>
+        <v>35.9848484848485</v>
       </c>
       <c r="J31" t="n">
         <v>30</v>
@@ -2692,7 +2692,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M31" t="n">
@@ -2702,10 +2702,10 @@
         <v>30</v>
       </c>
       <c r="O31" t="n">
-        <v>44.68085106382978</v>
+        <v>38.29787234042553</v>
       </c>
       <c r="P31" t="n">
-        <v>40.53217021276596</v>
+        <v>39.25557446808512</v>
       </c>
       <c r="Q31" t="b">
         <v>0</v>
@@ -2729,25 +2729,25 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>686.55</v>
+        <v>652.9</v>
       </c>
       <c r="D32" t="n">
-        <v>-0.09444041416606209</v>
+        <v>-0.1403554970375247</v>
       </c>
       <c r="E32" t="n">
-        <v>-0.1418125</v>
+        <v>-0.2071645415907711</v>
       </c>
       <c r="F32" t="n">
-        <v>-0.348005698005698</v>
+        <v>-0.3728146013448608</v>
       </c>
       <c r="G32" t="n">
-        <v>-0.3274330566677238</v>
+        <v>-0.3522419600068865</v>
       </c>
       <c r="H32" t="n">
-        <v>-0.2931659662636058</v>
+        <v>-0.3179748696027685</v>
       </c>
       <c r="I32" t="n">
-        <v>45.03181595692608</v>
+        <v>44.20951465641519</v>
       </c>
       <c r="J32" t="n">
         <v>40</v>
@@ -2757,7 +2757,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M32" t="n">
@@ -2794,25 +2794,25 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>543.95</v>
+        <v>525.3</v>
       </c>
       <c r="D33" t="n">
-        <v>-0.1213149180195459</v>
+        <v>-0.1585776069197501</v>
       </c>
       <c r="E33" t="n">
-        <v>-0.1059335963182116</v>
+        <v>-0.1609966459032105</v>
       </c>
       <c r="F33" t="n">
-        <v>0.1106687085247575</v>
+        <v>0.0501799280287884</v>
       </c>
       <c r="G33" t="n">
-        <v>0.1312413498627317</v>
+        <v>0.07075256936676259</v>
       </c>
       <c r="H33" t="n">
-        <v>0.1655084402668497</v>
+        <v>0.1050196597708806</v>
       </c>
       <c r="I33" t="n">
-        <v>43.93560921454346</v>
+        <v>44.67965001411233</v>
       </c>
       <c r="J33" t="n">
         <v>40</v>
@@ -2822,7 +2822,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M33" t="n">
@@ -2832,10 +2832,10 @@
         <v>40</v>
       </c>
       <c r="O33" t="n">
-        <v>78.72340425531915</v>
+        <v>76.59574468085107</v>
       </c>
       <c r="P33" t="n">
-        <v>51.73668085106384</v>
+        <v>51.31114893617022</v>
       </c>
       <c r="Q33" t="b">
         <v>0</v>
@@ -2887,7 +2887,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M34" t="n">
@@ -2897,10 +2897,10 @@
         <v>80</v>
       </c>
       <c r="O34" t="n">
-        <v>17.02127659574468</v>
+        <v>19.14893617021277</v>
       </c>
       <c r="P34" t="n">
-        <v>55.75625531914894</v>
+        <v>56.18178723404256</v>
       </c>
       <c r="Q34" t="b">
         <v>0</v>
@@ -2924,25 +2924,25 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>109.14</v>
+        <v>105.08</v>
       </c>
       <c r="D35" t="n">
-        <v>-0.1294568078487676</v>
+        <v>-0.1788058768365114</v>
       </c>
       <c r="E35" t="n">
-        <v>0.0423073249928374</v>
+        <v>0.0136008488473038</v>
       </c>
       <c r="F35" t="n">
-        <v>0.0943547578461847</v>
+        <v>0.0489119584747452</v>
       </c>
       <c r="G35" t="n">
-        <v>0.1149273991841589</v>
+        <v>0.0694845998127194</v>
       </c>
       <c r="H35" t="n">
-        <v>0.1491944895882769</v>
+        <v>0.1037516902168375</v>
       </c>
       <c r="I35" t="n">
-        <v>45.84830339321358</v>
+        <v>49.75092051115443</v>
       </c>
       <c r="J35" t="n">
         <v>40</v>
@@ -2952,7 +2952,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M35" t="n">
@@ -2962,10 +2962,10 @@
         <v>40</v>
       </c>
       <c r="O35" t="n">
-        <v>76.59574468085107</v>
+        <v>74.46808510638297</v>
       </c>
       <c r="P35" t="n">
-        <v>50.94714893617022</v>
+        <v>50.5216170212766</v>
       </c>
       <c r="Q35" t="b">
         <v>0</v>
@@ -2989,25 +2989,25 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>465</v>
+        <v>462.7</v>
       </c>
       <c r="D36" t="n">
-        <v>-0.0435050910212896</v>
+        <v>-0.0722807017543859</v>
       </c>
       <c r="E36" t="n">
-        <v>-0.1223931301311692</v>
+        <v>-0.1741923969302159</v>
       </c>
       <c r="F36" t="n">
-        <v>-0.0094791777612098</v>
+        <v>0.0011900897976848</v>
       </c>
       <c r="G36" t="n">
-        <v>0.0110934635767643</v>
+        <v>0.021762731135659</v>
       </c>
       <c r="H36" t="n">
-        <v>0.0453605539808823</v>
+        <v>0.056029821539777</v>
       </c>
       <c r="I36" t="n">
-        <v>34.95454545454545</v>
+        <v>34.98635122838944</v>
       </c>
       <c r="J36" t="n">
         <v>30</v>
@@ -3017,7 +3017,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M36" t="n">
@@ -3027,10 +3027,10 @@
         <v>30</v>
       </c>
       <c r="O36" t="n">
-        <v>63.82978723404256</v>
+        <v>68.08510638297872</v>
       </c>
       <c r="P36" t="n">
-        <v>43.88595744680851</v>
+        <v>44.73702127659575</v>
       </c>
       <c r="Q36" t="b">
         <v>0</v>
@@ -3054,25 +3054,25 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2183</v>
+        <v>2159.2</v>
       </c>
       <c r="D37" t="n">
-        <v>-0.0692816030697079</v>
+        <v>-0.0825189088127815</v>
       </c>
       <c r="E37" t="n">
-        <v>0.3397569657542654</v>
+        <v>0.2840915848944394</v>
       </c>
       <c r="F37" t="n">
-        <v>0.6758790112083526</v>
+        <v>0.6443530576498362</v>
       </c>
       <c r="G37" t="n">
-        <v>0.6964516525463268</v>
+        <v>0.6649256989878104</v>
       </c>
       <c r="H37" t="n">
-        <v>0.7307187429504448</v>
+        <v>0.6991927893919284</v>
       </c>
       <c r="I37" t="n">
-        <v>49.29617925883368</v>
+        <v>53.22580645161288</v>
       </c>
       <c r="J37" t="n">
         <v>80</v>
@@ -3082,7 +3082,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M37" t="n">
@@ -3119,25 +3119,25 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>795.15</v>
+        <v>757.1</v>
       </c>
       <c r="D38" t="n">
-        <v>-0.1638801261829653</v>
+        <v>-0.2093363270847474</v>
       </c>
       <c r="E38" t="n">
-        <v>-0.1621621621621621</v>
+        <v>-0.2153184432813391</v>
       </c>
       <c r="F38" t="n">
-        <v>-0.2573550014009527</v>
+        <v>-0.2846749811035526</v>
       </c>
       <c r="G38" t="n">
-        <v>-0.2367823600629784</v>
+        <v>-0.2641023397655784</v>
       </c>
       <c r="H38" t="n">
-        <v>-0.2025152696588604</v>
+        <v>-0.2298352493614603</v>
       </c>
       <c r="I38" t="n">
-        <v>44.00201612903225</v>
+        <v>41.20516047828823</v>
       </c>
       <c r="J38" t="n">
         <v>40</v>
@@ -3147,7 +3147,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M38" t="n">
@@ -3157,10 +3157,10 @@
         <v>40</v>
       </c>
       <c r="O38" t="n">
-        <v>14.8936170212766</v>
+        <v>10.63829787234042</v>
       </c>
       <c r="P38" t="n">
-        <v>38.92672340425532</v>
+        <v>38.07565957446808</v>
       </c>
       <c r="Q38" t="b">
         <v>0</v>
@@ -3184,25 +3184,25 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>3102.1</v>
+        <v>3033.5</v>
       </c>
       <c r="D39" t="n">
-        <v>-0.0255999497424299</v>
+        <v>-0.0419114395805697</v>
       </c>
       <c r="E39" t="n">
-        <v>0.0189193627853505</v>
+        <v>-0.0298698391378042</v>
       </c>
       <c r="F39" t="n">
-        <v>0.2005960213638824</v>
+        <v>0.1788365134263396</v>
       </c>
       <c r="G39" t="n">
-        <v>0.2211686627018566</v>
+        <v>0.1994091547643138</v>
       </c>
       <c r="H39" t="n">
-        <v>0.2554357531059746</v>
+        <v>0.2336762451684318</v>
       </c>
       <c r="I39" t="n">
-        <v>56.375</v>
+        <v>58.48653596765581</v>
       </c>
       <c r="J39" t="n">
         <v>80</v>
@@ -3212,7 +3212,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M39" t="n">
@@ -3222,10 +3222,10 @@
         <v>80</v>
       </c>
       <c r="O39" t="n">
-        <v>87.2340425531915</v>
+        <v>89.36170212765957</v>
       </c>
       <c r="P39" t="n">
-        <v>68.9228085106383</v>
+        <v>69.34834042553192</v>
       </c>
       <c r="Q39" t="b">
         <v>0</v>
@@ -3249,25 +3249,25 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>185.82</v>
+        <v>178.97</v>
       </c>
       <c r="D40" t="n">
-        <v>-0.1299339794915016</v>
+        <v>-0.1683936620045537</v>
       </c>
       <c r="E40" t="n">
-        <v>-0.0195230054875475</v>
+        <v>-0.0308133867648651</v>
       </c>
       <c r="F40" t="n">
-        <v>-0.177787610619469</v>
+        <v>-0.2002770454443898</v>
       </c>
       <c r="G40" t="n">
-        <v>-0.1572149692814948</v>
+        <v>-0.1797044041064156</v>
       </c>
       <c r="H40" t="n">
-        <v>-0.1229478788773767</v>
+        <v>-0.1454373137022976</v>
       </c>
       <c r="I40" t="n">
-        <v>42.21594475831763</v>
+        <v>43.10897435897437</v>
       </c>
       <c r="J40" t="n">
         <v>40</v>
@@ -3277,7 +3277,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M40" t="n">
@@ -3314,25 +3314,25 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>799</v>
+        <v>762.65</v>
       </c>
       <c r="D41" t="n">
-        <v>-0.1343914197497426</v>
+        <v>-0.1622913005272407</v>
       </c>
       <c r="E41" t="n">
-        <v>-0.1340630757559336</v>
+        <v>-0.1883680093651891</v>
       </c>
       <c r="F41" t="n">
-        <v>-0.212264615991324</v>
+        <v>-0.2498770532113702</v>
       </c>
       <c r="G41" t="n">
-        <v>-0.1916919746533498</v>
+        <v>-0.229304411873396</v>
       </c>
       <c r="H41" t="n">
-        <v>-0.1574248842492318</v>
+        <v>-0.195037321469278</v>
       </c>
       <c r="I41" t="n">
-        <v>28.65168539325848</v>
+        <v>23.986975397974</v>
       </c>
       <c r="J41" t="n">
         <v>20</v>
@@ -3342,7 +3342,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M41" t="n">
@@ -3352,10 +3352,10 @@
         <v>20</v>
       </c>
       <c r="O41" t="n">
-        <v>19.14893617021277</v>
+        <v>17.02127659574468</v>
       </c>
       <c r="P41" t="n">
-        <v>31.04978723404255</v>
+        <v>30.62425531914894</v>
       </c>
       <c r="Q41" t="b">
         <v>0</v>
@@ -3379,25 +3379,25 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>525.55</v>
+        <v>496</v>
       </c>
       <c r="D42" t="n">
-        <v>-0.2168243797034498</v>
+        <v>-0.2457994373907093</v>
       </c>
       <c r="E42" t="n">
-        <v>-0.2383885225708282</v>
+        <v>-0.2622341216718726</v>
       </c>
       <c r="F42" t="n">
-        <v>-0.3193679984458978</v>
+        <v>-0.3624678663239075</v>
       </c>
       <c r="G42" t="n">
-        <v>-0.2987953571079236</v>
+        <v>-0.3418952249859333</v>
       </c>
       <c r="H42" t="n">
-        <v>-0.2645282667038056</v>
+        <v>-0.3076281345818152</v>
       </c>
       <c r="I42" t="n">
-        <v>31.49732620320856</v>
+        <v>33.40896199659673</v>
       </c>
       <c r="J42" t="n">
         <v>30</v>
@@ -3407,7 +3407,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M42" t="n">
@@ -3444,48 +3444,48 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>410.45</v>
+        <v>414.45</v>
       </c>
       <c r="D43" t="n">
-        <v>-0.0303567210016537</v>
+        <v>-0.07694877505567931</v>
       </c>
       <c r="E43" t="n">
-        <v>-0.0836124134851529</v>
+        <v>-0.09725549989109129</v>
       </c>
       <c r="F43" t="n">
-        <v>-0.1100390286209886</v>
+        <v>-0.0862087972660126</v>
       </c>
       <c r="G43" t="n">
-        <v>-0.0894663872830144</v>
+        <v>-0.0656361559280384</v>
       </c>
       <c r="H43" t="n">
-        <v>-0.0551992968788964</v>
+        <v>-0.0313690655239203</v>
       </c>
       <c r="I43" t="n">
-        <v>40.98062953995155</v>
+        <v>51.39171758316361</v>
       </c>
       <c r="J43" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K43" t="n">
         <v>51.48</v>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M43" t="n">
         <v>51.48</v>
       </c>
       <c r="N43" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O43" t="n">
-        <v>51.06382978723404</v>
+        <v>55.31914893617022</v>
       </c>
       <c r="P43" t="n">
-        <v>46.8047659574468</v>
+        <v>55.65582978723404</v>
       </c>
       <c r="Q43" t="b">
         <v>0</v>
@@ -3509,25 +3509,25 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>238.9</v>
+        <v>233</v>
       </c>
       <c r="D44" t="n">
-        <v>-0.0943896891584533</v>
+        <v>-0.1243893273205563</v>
       </c>
       <c r="E44" t="n">
-        <v>-0.1467857142857143</v>
+        <v>-0.1712608927618708</v>
       </c>
       <c r="F44" t="n">
-        <v>-0.1120609552127857</v>
+        <v>-0.1309212980231258</v>
       </c>
       <c r="G44" t="n">
-        <v>-0.09148831387481141</v>
+        <v>-0.1103486566851515</v>
       </c>
       <c r="H44" t="n">
-        <v>-0.0572212234706934</v>
+        <v>-0.07608156628103351</v>
       </c>
       <c r="I44" t="n">
-        <v>48.8292404340377</v>
+        <v>43.38358458961473</v>
       </c>
       <c r="J44" t="n">
         <v>40</v>
@@ -3537,7 +3537,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M44" t="n">
@@ -3547,10 +3547,10 @@
         <v>40</v>
       </c>
       <c r="O44" t="n">
-        <v>46.80851063829788</v>
+        <v>44.68085106382978</v>
       </c>
       <c r="P44" t="n">
-        <v>44.24170212765958</v>
+        <v>43.81617021276596</v>
       </c>
       <c r="Q44" t="b">
         <v>0</v>
@@ -3574,48 +3574,48 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>92.33</v>
+        <v>86.55</v>
       </c>
       <c r="D45" t="n">
-        <v>-0.1387930230388956</v>
+        <v>-0.2008310249307479</v>
       </c>
       <c r="E45" t="n">
-        <v>-0.1602546612096408</v>
+        <v>-0.2118921872154434</v>
       </c>
       <c r="F45" t="n">
-        <v>-0.3137866963953921</v>
+        <v>-0.3525099124710107</v>
       </c>
       <c r="G45" t="n">
-        <v>-0.2932140550574179</v>
+        <v>-0.3319372711330365</v>
       </c>
       <c r="H45" t="n">
-        <v>-0.2589469646532999</v>
+        <v>-0.2976701807289185</v>
       </c>
       <c r="I45" t="n">
-        <v>32.43123336291035</v>
+        <v>26.31389488840891</v>
       </c>
       <c r="J45" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="K45" t="n">
         <v>59.6</v>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M45" t="n">
         <v>59.6</v>
       </c>
       <c r="N45" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="O45" t="n">
         <v>6.382978723404255</v>
       </c>
       <c r="P45" t="n">
-        <v>37.11659574468086</v>
+        <v>33.11659574468086</v>
       </c>
       <c r="Q45" t="b">
         <v>0</v>
@@ -3639,25 +3639,25 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>493.4</v>
+        <v>487.6</v>
       </c>
       <c r="D46" t="n">
-        <v>-0.0963369963369963</v>
+        <v>-0.1153846153846154</v>
       </c>
       <c r="E46" t="n">
-        <v>-0.2063057990830853</v>
+        <v>-0.2353771365846009</v>
       </c>
       <c r="F46" t="n">
-        <v>-0.1380906629399948</v>
+        <v>-0.1309926929246123</v>
       </c>
       <c r="G46" t="n">
-        <v>-0.1175180216020206</v>
+        <v>-0.1104200515866381</v>
       </c>
       <c r="H46" t="n">
-        <v>-0.0832509311979026</v>
+        <v>-0.0761529611825201</v>
       </c>
       <c r="I46" t="n">
-        <v>44.06590337894443</v>
+        <v>51.3337670787248</v>
       </c>
       <c r="J46" t="n">
         <v>40</v>
@@ -3667,7 +3667,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M46" t="n">
@@ -3677,10 +3677,10 @@
         <v>40</v>
       </c>
       <c r="O46" t="n">
-        <v>29.78723404255319</v>
+        <v>42.5531914893617</v>
       </c>
       <c r="P46" t="n">
-        <v>41.80144680851064</v>
+        <v>44.35463829787234</v>
       </c>
       <c r="Q46" t="b">
         <v>0</v>
@@ -3704,25 +3704,25 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>1089.55</v>
+        <v>1082.1</v>
       </c>
       <c r="D47" t="n">
-        <v>0.2215370816749817</v>
+        <v>0.2112833715788882</v>
       </c>
       <c r="E47" t="n">
-        <v>0.3412322274881516</v>
+        <v>0.3170642648490749</v>
       </c>
       <c r="F47" t="n">
-        <v>0.4680994408138517</v>
+        <v>0.4677517802644964</v>
       </c>
       <c r="G47" t="n">
-        <v>0.4886720821518259</v>
+        <v>0.4883244216024706</v>
       </c>
       <c r="H47" t="n">
-        <v>0.5229391725559439</v>
+        <v>0.5225915120065886</v>
       </c>
       <c r="I47" t="n">
-        <v>77.51051524710832</v>
+        <v>73.51181999430361</v>
       </c>
       <c r="J47" t="n">
         <v>70</v>
@@ -3732,7 +3732,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M47" t="n">
@@ -3769,48 +3769,48 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>13592</v>
+        <v>13678</v>
       </c>
       <c r="D48" t="n">
-        <v>-0.1396923855940249</v>
+        <v>-0.1184583655581335</v>
       </c>
       <c r="E48" t="n">
-        <v>-0.07644220968947479</v>
+        <v>-0.0502048468856329</v>
       </c>
       <c r="F48" t="n">
-        <v>-0.0152151862048978</v>
+        <v>-0.0031338823700896</v>
       </c>
       <c r="G48" t="n">
-        <v>0.0053574551330763</v>
+        <v>0.0174387589678846</v>
       </c>
       <c r="H48" t="n">
-        <v>0.0396245455371944</v>
+        <v>0.0517058493720026</v>
       </c>
       <c r="I48" t="n">
-        <v>35.93974175035869</v>
+        <v>43.48521183053557</v>
       </c>
       <c r="J48" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K48" t="n">
         <v>50.29</v>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M48" t="n">
         <v>50.29</v>
       </c>
       <c r="N48" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O48" t="n">
-        <v>61.70212765957447</v>
+        <v>63.82978723404256</v>
       </c>
       <c r="P48" t="n">
-        <v>44.4564255319149</v>
+        <v>48.88195744680851</v>
       </c>
       <c r="Q48" t="b">
         <v>0</v>
@@ -3945,25 +3945,25 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1623.3</v>
+        <v>1608.8</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.0295330902134274</v>
+        <v>-0.064107038976149</v>
       </c>
       <c r="E2" t="n">
-        <v>0.09100073929699549</v>
+        <v>0.0642323212277566</v>
       </c>
       <c r="F2" t="n">
-        <v>0.5489503816793893</v>
+        <v>0.5187387897668272</v>
       </c>
       <c r="G2" t="n">
-        <v>0.5695230230173635</v>
+        <v>0.5393114311048014</v>
       </c>
       <c r="H2" t="n">
-        <v>0.6037901134214815</v>
+        <v>0.5735785215089194</v>
       </c>
       <c r="I2" t="n">
-        <v>55.99580162686958</v>
+        <v>59.15453915453915</v>
       </c>
       <c r="J2" t="n">
         <v>80</v>
@@ -3973,7 +3973,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M2" t="n">
@@ -3983,10 +3983,10 @@
         <v>80</v>
       </c>
       <c r="O2" t="n">
-        <v>97.87234042553192</v>
+        <v>95.74468085106383</v>
       </c>
       <c r="P2" t="n">
-        <v>73.37846808510639</v>
+        <v>72.95293617021277</v>
       </c>
       <c r="Q2" t="b">
         <v>0</v>
@@ -4010,25 +4010,25 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2183</v>
+        <v>2159.2</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.0692816030697079</v>
+        <v>-0.0825189088127815</v>
       </c>
       <c r="E3" t="n">
-        <v>0.3397569657542654</v>
+        <v>0.2840915848944394</v>
       </c>
       <c r="F3" t="n">
-        <v>0.6758790112083526</v>
+        <v>0.6443530576498362</v>
       </c>
       <c r="G3" t="n">
-        <v>0.6964516525463268</v>
+        <v>0.6649256989878104</v>
       </c>
       <c r="H3" t="n">
-        <v>0.7307187429504448</v>
+        <v>0.6991927893919284</v>
       </c>
       <c r="I3" t="n">
-        <v>49.29617925883368</v>
+        <v>53.22580645161288</v>
       </c>
       <c r="J3" t="n">
         <v>80</v>
@@ -4038,7 +4038,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M3" t="n">
@@ -4075,25 +4075,25 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>3102.1</v>
+        <v>3033.5</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.0255999497424299</v>
+        <v>-0.0419114395805697</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0189193627853505</v>
+        <v>-0.0298698391378042</v>
       </c>
       <c r="F4" t="n">
-        <v>0.2005960213638824</v>
+        <v>0.1788365134263396</v>
       </c>
       <c r="G4" t="n">
-        <v>0.2211686627018566</v>
+        <v>0.1994091547643138</v>
       </c>
       <c r="H4" t="n">
-        <v>0.2554357531059746</v>
+        <v>0.2336762451684318</v>
       </c>
       <c r="I4" t="n">
-        <v>56.375</v>
+        <v>58.48653596765581</v>
       </c>
       <c r="J4" t="n">
         <v>80</v>
@@ -4103,7 +4103,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M4" t="n">
@@ -4113,10 +4113,10 @@
         <v>80</v>
       </c>
       <c r="O4" t="n">
-        <v>87.2340425531915</v>
+        <v>89.36170212765957</v>
       </c>
       <c r="P4" t="n">
-        <v>68.9228085106383</v>
+        <v>69.34834042553192</v>
       </c>
       <c r="Q4" t="b">
         <v>0</v>
@@ -4131,57 +4131,57 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>WHEELS</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Wheels</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>511.45</v>
+        <v>1082.1</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.0339975446217774</v>
+        <v>0.2112833715788882</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0516089236146806</v>
+        <v>0.3170642648490749</v>
       </c>
       <c r="F5" t="n">
-        <v>0.1365555555555555</v>
+        <v>0.4677517802644964</v>
       </c>
       <c r="G5" t="n">
-        <v>0.1571281968935297</v>
+        <v>0.4883244216024706</v>
       </c>
       <c r="H5" t="n">
-        <v>0.1913952872976477</v>
+        <v>0.5225915120065886</v>
       </c>
       <c r="I5" t="n">
-        <v>48.86658031088081</v>
+        <v>73.51181999430361</v>
       </c>
       <c r="J5" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K5" t="n">
-        <v>49.66</v>
+        <v>46.83</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M5" t="n">
-        <v>49.66</v>
+        <v>46.83</v>
       </c>
       <c r="N5" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O5" t="n">
-        <v>82.97872340425532</v>
+        <v>93.61702127659576</v>
       </c>
       <c r="P5" t="n">
-        <v>68.45974468085107</v>
+        <v>65.45540425531915</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
@@ -4205,48 +4205,48 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>444.15</v>
+        <v>438.75</v>
       </c>
       <c r="D6" t="n">
-        <v>0.0382187938288918</v>
+        <v>0.0277582572030921</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.0300283904782703</v>
+        <v>-0.0647980390067142</v>
       </c>
       <c r="F6" t="n">
-        <v>-0.1372377622377621</v>
+        <v>-0.15625</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.1166651208997879</v>
+        <v>-0.1356773586620258</v>
       </c>
       <c r="H6" t="n">
-        <v>-0.08239803049566991</v>
+        <v>-0.1014102682579077</v>
       </c>
       <c r="I6" t="n">
-        <v>69.2562592047128</v>
+        <v>72.65353418308227</v>
       </c>
       <c r="J6" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K6" t="n">
         <v>71.28</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M6" t="n">
         <v>71.28</v>
       </c>
       <c r="N6" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O6" t="n">
         <v>31.91489361702128</v>
       </c>
       <c r="P6" t="n">
-        <v>66.89497872340425</v>
+        <v>62.89497872340426</v>
       </c>
       <c r="Q6" t="b">
         <v>1</v>
@@ -4261,57 +4261,57 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>WHEELS</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Wheels</t>
+          <t>Forgings</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1089.55</v>
+        <v>1725.1</v>
       </c>
       <c r="D7" t="n">
-        <v>0.2215370816749817</v>
+        <v>-0.0930073606729758</v>
       </c>
       <c r="E7" t="n">
-        <v>0.3412322274881516</v>
+        <v>0.2470902913323212</v>
       </c>
       <c r="F7" t="n">
-        <v>0.4680994408138517</v>
+        <v>0.5247480996994871</v>
       </c>
       <c r="G7" t="n">
-        <v>0.4886720821518259</v>
+        <v>0.5453207410374613</v>
       </c>
       <c r="H7" t="n">
-        <v>0.5229391725559439</v>
+        <v>0.5795878314415793</v>
       </c>
       <c r="I7" t="n">
-        <v>77.51051524710832</v>
+        <v>37.99860041987404</v>
       </c>
       <c r="J7" t="n">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="K7" t="n">
-        <v>46.83</v>
+        <v>54.83</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M7" t="n">
-        <v>46.83</v>
+        <v>54.83</v>
       </c>
       <c r="N7" t="n">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="O7" t="n">
-        <v>93.61702127659576</v>
+        <v>97.87234042553192</v>
       </c>
       <c r="P7" t="n">
-        <v>65.45540425531915</v>
+        <v>61.50646808510639</v>
       </c>
       <c r="Q7" t="b">
         <v>0</v>
@@ -4326,63 +4326,63 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>JBMA</t>
+          <t>MINDACORP</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>572.65</v>
+        <v>528.7</v>
       </c>
       <c r="D8" t="n">
-        <v>0.0290206648697213</v>
+        <v>-0.0871104204437536</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0094306363476115</v>
+        <v>-0.090643274853801</v>
       </c>
       <c r="F8" t="n">
-        <v>-0.06802831800797469</v>
+        <v>0.0521393034825872</v>
       </c>
       <c r="G8" t="n">
-        <v>-0.0474556766700005</v>
+        <v>0.0727119448205614</v>
       </c>
       <c r="H8" t="n">
-        <v>-0.0131885862658824</v>
+        <v>0.1069790352246794</v>
       </c>
       <c r="I8" t="n">
-        <v>59.15238954012625</v>
+        <v>60.57201225740555</v>
       </c>
       <c r="J8" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K8" t="n">
-        <v>56.91</v>
+        <v>49.42</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M8" t="n">
-        <v>56.91</v>
+        <v>49.42</v>
       </c>
       <c r="N8" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O8" t="n">
-        <v>53.19148936170212</v>
+        <v>78.72340425531915</v>
       </c>
       <c r="P8" t="n">
-        <v>65.40229787234043</v>
+        <v>59.51268085106384</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
       </c>
       <c r="R8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S8" t="b">
         <v>0</v>
@@ -4391,57 +4391,57 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>DIVGIITTS</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Forgings</t>
+          <t>Transmission</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1736.5</v>
+        <v>674.75</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.06554377656998329</v>
+        <v>-0.059909439219784</v>
       </c>
       <c r="E9" t="n">
-        <v>0.2641962725684335</v>
+        <v>0.1113398665898048</v>
       </c>
       <c r="F9" t="n">
-        <v>0.5291475871785842</v>
+        <v>-0.0029553010712966</v>
       </c>
       <c r="G9" t="n">
-        <v>0.5497202285165584</v>
+        <v>0.0176173402666776</v>
       </c>
       <c r="H9" t="n">
-        <v>0.5839873189206765</v>
+        <v>0.0518844306707956</v>
       </c>
       <c r="I9" t="n">
-        <v>34.93084593116758</v>
+        <v>40.25722339675829</v>
       </c>
       <c r="J9" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="K9" t="n">
-        <v>54.83</v>
+        <v>49.92</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M9" t="n">
-        <v>54.83</v>
+        <v>49.92</v>
       </c>
       <c r="N9" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="O9" t="n">
-        <v>95.74468085106383</v>
+        <v>65.95744680851064</v>
       </c>
       <c r="P9" t="n">
-        <v>61.08093617021277</v>
+        <v>57.15948936170213</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -4456,7 +4456,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TIINDIA</t>
+          <t>JBMA</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -4465,48 +4465,48 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>2682.4</v>
+        <v>546.65</v>
       </c>
       <c r="D10" t="n">
-        <v>0.0467085495766186</v>
+        <v>-0.0176116452511457</v>
       </c>
       <c r="E10" t="n">
-        <v>0.045036621474209</v>
+        <v>-0.0434820647419073</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.1187331624942505</v>
+        <v>-0.09860664523043949</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.0981605211562763</v>
+        <v>-0.0780340038924652</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.0638934307521583</v>
+        <v>-0.0437669134883472</v>
       </c>
       <c r="I10" t="n">
-        <v>47.54158067257497</v>
+        <v>56.43496214728149</v>
       </c>
       <c r="J10" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K10" t="n">
-        <v>48.73</v>
+        <v>56.91</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M10" t="n">
-        <v>48.73</v>
+        <v>56.91</v>
       </c>
       <c r="N10" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O10" t="n">
-        <v>38.29787234042553</v>
+        <v>51.06382978723404</v>
       </c>
       <c r="P10" t="n">
-        <v>59.15157446808512</v>
+        <v>56.9767659574468</v>
       </c>
       <c r="Q10" t="b">
         <v>0</v>
@@ -4521,57 +4521,57 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MINDACORP</t>
+          <t>LUMAXIND</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Lighting</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>543.95</v>
+        <v>4880</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.0517737296260785</v>
+        <v>-0.214752357352042</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.0655385672564851</v>
+        <v>-0.152041702867072</v>
       </c>
       <c r="F11" t="n">
-        <v>0.0735149003355044</v>
+        <v>0.1645110485372021</v>
       </c>
       <c r="G11" t="n">
-        <v>0.0940875416734786</v>
+        <v>0.1850836898751763</v>
       </c>
       <c r="H11" t="n">
-        <v>0.1283546320775966</v>
+        <v>0.2193507802792943</v>
       </c>
       <c r="I11" t="n">
-        <v>57.42414460942543</v>
+        <v>42.24175824175824</v>
       </c>
       <c r="J11" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="K11" t="n">
-        <v>49.42</v>
+        <v>57.69</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M11" t="n">
-        <v>49.42</v>
+        <v>57.69</v>
       </c>
       <c r="N11" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="O11" t="n">
-        <v>74.46808510638297</v>
+        <v>87.2340425531915</v>
       </c>
       <c r="P11" t="n">
-        <v>58.6616170212766</v>
+        <v>56.5228085106383</v>
       </c>
       <c r="Q11" t="b">
         <v>0</v>
@@ -4586,63 +4586,63 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>DIVGIITTS</t>
+          <t>RANEENGINE</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Transmission</t>
+          <t>Engine/Parts</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>697.65</v>
+        <v>317.75</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.07239728759473479</v>
+        <v>0.1790352504638219</v>
       </c>
       <c r="E12" t="n">
-        <v>0.1617818484596169</v>
+        <v>-0.156154561147258</v>
       </c>
       <c r="F12" t="n">
-        <v>0.053215579710145</v>
+        <v>-0.2401052253975846</v>
       </c>
       <c r="G12" t="n">
-        <v>0.0737882210481192</v>
+        <v>-0.2195325840596104</v>
       </c>
       <c r="H12" t="n">
-        <v>0.1080553114522372</v>
+        <v>-0.1852654936554923</v>
       </c>
       <c r="I12" t="n">
-        <v>45.66506113375324</v>
+        <v>63.3225806451613</v>
       </c>
       <c r="J12" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K12" t="n">
-        <v>49.92</v>
+        <v>50.88</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M12" t="n">
-        <v>49.92</v>
+        <v>50.88</v>
       </c>
       <c r="N12" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O12" t="n">
-        <v>70.21276595744681</v>
+        <v>19.14893617021277</v>
       </c>
       <c r="P12" t="n">
-        <v>58.01055319148936</v>
+        <v>56.18178723404256</v>
       </c>
       <c r="Q12" t="b">
         <v>0</v>
       </c>
       <c r="R12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S12" t="b">
         <v>0</v>
@@ -4651,63 +4651,63 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>LUMAXIND</t>
+          <t>SUPRAJIT</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Lighting</t>
+          <t>Cables</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>5148.5</v>
+        <v>414.45</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.1348222087786516</v>
+        <v>-0.07694877505567931</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.08552397868561271</v>
+        <v>-0.09725549989109129</v>
       </c>
       <c r="F13" t="n">
-        <v>0.2348003357716752</v>
+        <v>-0.0862087972660126</v>
       </c>
       <c r="G13" t="n">
-        <v>0.2553729771096494</v>
+        <v>-0.0656361559280384</v>
       </c>
       <c r="H13" t="n">
-        <v>0.2896400675137675</v>
+        <v>-0.0313690655239203</v>
       </c>
       <c r="I13" t="n">
-        <v>40.8936170212766</v>
+        <v>51.39171758316361</v>
       </c>
       <c r="J13" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K13" t="n">
-        <v>57.69</v>
+        <v>51.48</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M13" t="n">
-        <v>57.69</v>
+        <v>51.48</v>
       </c>
       <c r="N13" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O13" t="n">
-        <v>89.36170212765957</v>
+        <v>55.31914893617022</v>
       </c>
       <c r="P13" t="n">
-        <v>56.94834042553191</v>
+        <v>55.65582978723404</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
       </c>
       <c r="R13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S13" t="b">
         <v>0</v>
@@ -4716,63 +4716,63 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>RANEENGINE</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Engine/Parts</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>317.75</v>
+        <v>488.75</v>
       </c>
       <c r="D14" t="n">
-        <v>0.1790352504638219</v>
+        <v>-0.0982472324723247</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.156154561147258</v>
+        <v>0.0200354794949391</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.2401052253975846</v>
+        <v>0.1159949765955017</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.2195325840596104</v>
+        <v>0.1365676179334759</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.1852654936554923</v>
+        <v>0.1708347083375939</v>
       </c>
       <c r="I14" t="n">
-        <v>63.3225806451613</v>
+        <v>46.33097942892233</v>
       </c>
       <c r="J14" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="K14" t="n">
-        <v>50.88</v>
+        <v>49.66</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M14" t="n">
-        <v>50.88</v>
+        <v>49.66</v>
       </c>
       <c r="N14" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="O14" t="n">
-        <v>17.02127659574468</v>
+        <v>82.97872340425532</v>
       </c>
       <c r="P14" t="n">
-        <v>55.75625531914894</v>
+        <v>52.45974468085107</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
       </c>
       <c r="R14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S14" t="b">
         <v>0</v>
@@ -4781,57 +4781,57 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>FIEMIND</t>
+          <t>GNA</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Lighting</t>
+          <t>Axles</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2083.6</v>
+        <v>377.85</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.0711483594864479</v>
+        <v>-0.1040901007705986</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.0806159819970878</v>
+        <v>0.2341989220970115</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.0442201834862385</v>
+        <v>0.2218270008084075</v>
       </c>
       <c r="G15" t="n">
-        <v>-0.0236475421482643</v>
+        <v>0.2423996421463817</v>
       </c>
       <c r="H15" t="n">
-        <v>0.0106195482558536</v>
+        <v>0.2766667325504998</v>
       </c>
       <c r="I15" t="n">
-        <v>49.18561995597947</v>
+        <v>33.32275468105364</v>
       </c>
       <c r="J15" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="K15" t="n">
-        <v>49.06</v>
+        <v>54.47</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M15" t="n">
-        <v>49.06</v>
+        <v>54.47</v>
       </c>
       <c r="N15" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="O15" t="n">
-        <v>57.44680851063831</v>
+        <v>91.48936170212764</v>
       </c>
       <c r="P15" t="n">
-        <v>55.11336170212766</v>
+        <v>52.08587234042552</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
@@ -4846,57 +4846,57 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>GNA</t>
+          <t>CRAFTSMAN</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Axles</t>
+          <t>Castings</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>396.15</v>
+        <v>6924</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.0526126987922994</v>
+        <v>-0.1117382937780628</v>
       </c>
       <c r="E16" t="n">
-        <v>0.3187416777629828</v>
+        <v>-0.0214810627473148</v>
       </c>
       <c r="F16" t="n">
-        <v>0.2502761559097364</v>
+        <v>0.0129471143296027</v>
       </c>
       <c r="G16" t="n">
-        <v>0.2708487972477106</v>
+        <v>0.0335197556675769</v>
       </c>
       <c r="H16" t="n">
-        <v>0.3051158876518286</v>
+        <v>0.0677868460716949</v>
       </c>
       <c r="I16" t="n">
-        <v>39.50488145048813</v>
+        <v>42.07197382769901</v>
       </c>
       <c r="J16" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K16" t="n">
-        <v>54.47</v>
+        <v>54.65</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M16" t="n">
-        <v>54.47</v>
+        <v>54.65</v>
       </c>
       <c r="N16" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O16" t="n">
-        <v>91.48936170212764</v>
+        <v>70.21276595744681</v>
       </c>
       <c r="P16" t="n">
-        <v>52.08587234042552</v>
+        <v>51.90255319148936</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
feat: NSE market report for 2026-03-27
https://claude.ai/code/session_01D6UEzdFERzfpopPdoSiiyt
</commit_message>
<xml_diff>
--- a/working-sector/output/auto_components_comprehensive_report.xlsx
+++ b/working-sector/output/auto_components_comprehensive_report.xlsx
@@ -435,7 +435,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
     </row>
@@ -447,7 +447,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
     </row>
@@ -779,25 +779,25 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1736.5</v>
+        <v>1725.1</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.0521288209606987</v>
+        <v>-0.0930073606729758</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2350640113798008</v>
+        <v>0.2470902913323212</v>
       </c>
       <c r="F2" t="n">
-        <v>0.5304953287502205</v>
+        <v>0.5247480996994871</v>
       </c>
       <c r="G2" t="n">
-        <v>0.5510679700881947</v>
+        <v>0.5453207410374613</v>
       </c>
       <c r="H2" t="n">
-        <v>0.5853350604923128</v>
+        <v>0.5795878314415793</v>
       </c>
       <c r="I2" t="n">
-        <v>37.49420670477369</v>
+        <v>37.99860041987404</v>
       </c>
       <c r="J2" t="n">
         <v>50</v>
@@ -807,7 +807,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M2" t="n">
@@ -844,25 +844,25 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1087.6</v>
+        <v>1048.7</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.0906354515050168</v>
+        <v>-0.1388569551650517</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.1452373467463062</v>
+        <v>-0.1485751400503369</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.1691367456073339</v>
+        <v>-0.1798701806522249</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.1485641042693597</v>
+        <v>-0.1592975393142507</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.1142970138652417</v>
+        <v>-0.1250304489101327</v>
       </c>
       <c r="I3" t="n">
-        <v>46.095141185449</v>
+        <v>45.71575166752181</v>
       </c>
       <c r="J3" t="n">
         <v>40</v>
@@ -872,7 +872,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M3" t="n">
@@ -909,25 +909,25 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>30390</v>
+        <v>29615</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.1400679117147708</v>
+        <v>-0.1901832102816516</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.1768689057421452</v>
+        <v>-0.1948069603045132</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.2644318044293839</v>
+        <v>-0.273073146784487</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.2438591630914097</v>
+        <v>-0.2525005054465128</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.2095920726872917</v>
+        <v>-0.2182334150423948</v>
       </c>
       <c r="I4" t="n">
-        <v>33.62168396770474</v>
+        <v>36.94937541091387</v>
       </c>
       <c r="J4" t="n">
         <v>30</v>
@@ -937,7 +937,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M4" t="n">
@@ -947,10 +947,10 @@
         <v>30</v>
       </c>
       <c r="O4" t="n">
-        <v>10.63829787234042</v>
+        <v>12.76595744680851</v>
       </c>
       <c r="P4" t="n">
-        <v>35.51965957446808</v>
+        <v>35.9451914893617</v>
       </c>
       <c r="Q4" t="b">
         <v>0</v>
@@ -974,25 +974,25 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>307.15</v>
+        <v>300.85</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.0923463356973995</v>
+        <v>-0.1081962353638654</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.1920294620544521</v>
+        <v>-0.1942956614890196</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.2620134550696781</v>
+        <v>-0.2583507950203376</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.2414408137317039</v>
+        <v>-0.2377781536823634</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.2071737233275858</v>
+        <v>-0.2035110632782454</v>
       </c>
       <c r="I5" t="n">
-        <v>43.0862831858407</v>
+        <v>45.31704479348461</v>
       </c>
       <c r="J5" t="n">
         <v>40</v>
@@ -1002,7 +1002,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M5" t="n">
@@ -1012,10 +1012,10 @@
         <v>40</v>
       </c>
       <c r="O5" t="n">
-        <v>12.76595744680851</v>
+        <v>14.8936170212766</v>
       </c>
       <c r="P5" t="n">
-        <v>39.0011914893617</v>
+        <v>39.42672340425532</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
@@ -1039,25 +1039,25 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>113.13</v>
+        <v>109.38</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.1352239718697446</v>
+        <v>-0.179075352746923</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.033489961554891</v>
+        <v>-0.0631263383297644</v>
       </c>
       <c r="F6" t="n">
-        <v>0.1726961749766766</v>
+        <v>0.1596692111959288</v>
       </c>
       <c r="G6" t="n">
-        <v>0.1932688163146508</v>
+        <v>0.180241852533903</v>
       </c>
       <c r="H6" t="n">
-        <v>0.2275359067187689</v>
+        <v>0.214508942938021</v>
       </c>
       <c r="I6" t="n">
-        <v>35.66312133709572</v>
+        <v>39.62855764592377</v>
       </c>
       <c r="J6" t="n">
         <v>30</v>
@@ -1067,7 +1067,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M6" t="n">
@@ -1104,48 +1104,48 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2682.4</v>
+        <v>2566.3</v>
       </c>
       <c r="D7" t="n">
-        <v>0.0562293274531422</v>
+        <v>-0.0200099285905218</v>
       </c>
       <c r="E7" t="n">
-        <v>0.0058874264071699</v>
+        <v>-0.0335542667771333</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.1198031173092698</v>
+        <v>-0.143681804531349</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.0992304759712956</v>
+        <v>-0.1231091631933748</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.0649633855671776</v>
+        <v>-0.08884207278925681</v>
       </c>
       <c r="I7" t="n">
-        <v>44.36388353914127</v>
+        <v>47.43791641429439</v>
       </c>
       <c r="J7" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K7" t="n">
         <v>48.73</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M7" t="n">
         <v>48.73</v>
       </c>
       <c r="N7" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O7" t="n">
-        <v>38.29787234042553</v>
+        <v>36.17021276595745</v>
       </c>
       <c r="P7" t="n">
-        <v>59.15157446808512</v>
+        <v>50.7260425531915</v>
       </c>
       <c r="Q7" t="b">
         <v>0</v>
@@ -1169,48 +1169,48 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>511.45</v>
+        <v>488.75</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.045891241488667</v>
+        <v>-0.0982472324723247</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0377396773866287</v>
+        <v>0.0200354794949391</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1494549949432519</v>
+        <v>0.1159949765955017</v>
       </c>
       <c r="G8" t="n">
-        <v>0.1700276362812262</v>
+        <v>0.1365676179334759</v>
       </c>
       <c r="H8" t="n">
-        <v>0.2042947266853442</v>
+        <v>0.1708347083375939</v>
       </c>
       <c r="I8" t="n">
-        <v>50.15782828282829</v>
+        <v>46.33097942892233</v>
       </c>
       <c r="J8" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="K8" t="n">
         <v>49.66</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M8" t="n">
         <v>49.66</v>
       </c>
       <c r="N8" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="O8" t="n">
         <v>82.97872340425532</v>
       </c>
       <c r="P8" t="n">
-        <v>68.45974468085107</v>
+        <v>52.45974468085107</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
@@ -1234,25 +1234,25 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>419.65</v>
+        <v>412.45</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.07464167585446529</v>
+        <v>-0.1096600107933082</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.1952248537731327</v>
+        <v>-0.2137819290888296</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.1397088970889709</v>
+        <v>-0.1504634397528321</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.1191362557509967</v>
+        <v>-0.1298907984148579</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.0848691653468787</v>
+        <v>-0.0956237080107399</v>
       </c>
       <c r="I9" t="n">
-        <v>40.15936254980078</v>
+        <v>42.37074401008826</v>
       </c>
       <c r="J9" t="n">
         <v>40</v>
@@ -1262,7 +1262,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M9" t="n">
@@ -1272,10 +1272,10 @@
         <v>40</v>
       </c>
       <c r="O9" t="n">
-        <v>31.91489361702128</v>
+        <v>34.04255319148936</v>
       </c>
       <c r="P9" t="n">
-        <v>43.75897872340426</v>
+        <v>44.18451063829788</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -1299,25 +1299,25 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>129970</v>
+        <v>129575</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.1083287596048299</v>
+        <v>-0.1220313717518718</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.1516872266823314</v>
+        <v>-0.1494633890183465</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.1554082594144978</v>
+        <v>-0.1341752697871772</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.1348356180765236</v>
+        <v>-0.1136026284492029</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.1005685276724056</v>
+        <v>-0.07933553804508491</v>
       </c>
       <c r="I10" t="n">
-        <v>33.76129339039468</v>
+        <v>39.9624765478424</v>
       </c>
       <c r="J10" t="n">
         <v>30</v>
@@ -1327,7 +1327,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M10" t="n">
@@ -1337,10 +1337,10 @@
         <v>30</v>
       </c>
       <c r="O10" t="n">
-        <v>29.78723404255319</v>
+        <v>40.42553191489361</v>
       </c>
       <c r="P10" t="n">
-        <v>37.72144680851064</v>
+        <v>39.84910638297872</v>
       </c>
       <c r="Q10" t="b">
         <v>0</v>
@@ -1392,7 +1392,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M11" t="n">
@@ -1402,10 +1402,10 @@
         <v>20</v>
       </c>
       <c r="O11" t="n">
-        <v>63.82978723404256</v>
+        <v>61.70212765957447</v>
       </c>
       <c r="P11" t="n">
-        <v>24.76595744680852</v>
+        <v>24.3404255319149</v>
       </c>
       <c r="Q11" t="b">
         <v>0</v>
@@ -1429,48 +1429,48 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>444.15</v>
+        <v>438.75</v>
       </c>
       <c r="D12" t="n">
-        <v>0.0255137381667049</v>
+        <v>0.0277582572030921</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.0730460189919649</v>
+        <v>-0.0647980390067142</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.1285195722554694</v>
+        <v>-0.15625</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.1079469309174951</v>
+        <v>-0.1356773586620258</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.0736798405133771</v>
+        <v>-0.1014102682579077</v>
       </c>
       <c r="I12" t="n">
-        <v>69.83381502890172</v>
+        <v>72.65353418308227</v>
       </c>
       <c r="J12" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K12" t="n">
         <v>71.28</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M12" t="n">
         <v>71.28</v>
       </c>
       <c r="N12" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O12" t="n">
-        <v>34.04255319148936</v>
+        <v>31.91489361702128</v>
       </c>
       <c r="P12" t="n">
-        <v>67.32051063829788</v>
+        <v>62.89497872340426</v>
       </c>
       <c r="Q12" t="b">
         <v>1</v>
@@ -1494,25 +1494,25 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1650.4</v>
+        <v>1585.4</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.1813085966565801</v>
+        <v>-0.2271242626627017</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.0945797673908271</v>
+        <v>-0.1379010331702012</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.0678865921156669</v>
+        <v>-0.0852757904454188</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.0473139507776927</v>
+        <v>-0.0647031491074446</v>
       </c>
       <c r="H13" t="n">
-        <v>-0.0130468603735747</v>
+        <v>-0.0304360587033266</v>
       </c>
       <c r="I13" t="n">
-        <v>19.06348649596633</v>
+        <v>18.72846312887664</v>
       </c>
       <c r="J13" t="n">
         <v>20</v>
@@ -1522,7 +1522,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M13" t="n">
@@ -1532,10 +1532,10 @@
         <v>20</v>
       </c>
       <c r="O13" t="n">
-        <v>53.19148936170212</v>
+        <v>57.44680851063831</v>
       </c>
       <c r="P13" t="n">
-        <v>42.14629787234043</v>
+        <v>42.99736170212766</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
@@ -1559,25 +1559,25 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>560.75</v>
+        <v>531.65</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.1464342796255423</v>
+        <v>-0.1689073002970142</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.25008358408559</v>
+        <v>-0.2702127659574468</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.0585914547133383</v>
+        <v>-0.1257913343747431</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.0380188133753641</v>
+        <v>-0.1052186930367689</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.0037517229712461</v>
+        <v>-0.0709516026326508</v>
       </c>
       <c r="I14" t="n">
-        <v>44.04982772329711</v>
+        <v>42.39795918367346</v>
       </c>
       <c r="J14" t="n">
         <v>40</v>
@@ -1587,7 +1587,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M14" t="n">
@@ -1597,10 +1597,10 @@
         <v>40</v>
       </c>
       <c r="O14" t="n">
-        <v>57.44680851063831</v>
+        <v>46.80851063829788</v>
       </c>
       <c r="P14" t="n">
-        <v>49.34536170212766</v>
+        <v>47.21770212765958</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
@@ -1624,25 +1624,25 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>95.70999999999999</v>
+        <v>89.41</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.1321969353522533</v>
+        <v>-0.1747277090640576</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.0096233443708609</v>
+        <v>-0.0652378463146891</v>
       </c>
       <c r="F15" t="n">
-        <v>0.0413447938200413</v>
+        <v>0.0273468918763644</v>
       </c>
       <c r="G15" t="n">
-        <v>0.0619174351580155</v>
+        <v>0.0479195332143386</v>
       </c>
       <c r="H15" t="n">
-        <v>0.0961845255621335</v>
+        <v>0.08218662361845661</v>
       </c>
       <c r="I15" t="n">
-        <v>41.2743823146944</v>
+        <v>41.1353032659409</v>
       </c>
       <c r="J15" t="n">
         <v>40</v>
@@ -1652,7 +1652,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M15" t="n">
@@ -1662,10 +1662,10 @@
         <v>40</v>
       </c>
       <c r="O15" t="n">
-        <v>70.21276595744681</v>
+        <v>72.3404255319149</v>
       </c>
       <c r="P15" t="n">
-        <v>50.80655319148936</v>
+        <v>51.23208510638297</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
@@ -1689,25 +1689,25 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>158.74</v>
+        <v>149.85</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.2123257083312657</v>
+        <v>-0.2340523410345532</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.0942082738944364</v>
+        <v>-0.1126835622927522</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.07741485528304071</v>
+        <v>-0.0820826952526799</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.0568422139450665</v>
+        <v>-0.0615100539147057</v>
       </c>
       <c r="H16" t="n">
-        <v>-0.0225751235409484</v>
+        <v>-0.0272429635105877</v>
       </c>
       <c r="I16" t="n">
-        <v>35.63903520931521</v>
+        <v>35.57985053971767</v>
       </c>
       <c r="J16" t="n">
         <v>30</v>
@@ -1717,7 +1717,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M16" t="n">
@@ -1727,10 +1727,10 @@
         <v>30</v>
       </c>
       <c r="O16" t="n">
-        <v>51.06382978723404</v>
+        <v>59.57446808510638</v>
       </c>
       <c r="P16" t="n">
-        <v>43.2567659574468</v>
+        <v>44.95889361702128</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>
@@ -1754,48 +1754,48 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>7049</v>
+        <v>6924</v>
       </c>
       <c r="D17" t="n">
-        <v>-0.1198651517043326</v>
+        <v>-0.1117382937780628</v>
       </c>
       <c r="E17" t="n">
-        <v>-0.0075325589581133</v>
+        <v>-0.0214810627473148</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0117697717812543</v>
+        <v>0.0129471143296027</v>
       </c>
       <c r="G17" t="n">
-        <v>0.0323424131192285</v>
+        <v>0.0335197556675769</v>
       </c>
       <c r="H17" t="n">
-        <v>0.0666095035233466</v>
+        <v>0.0677868460716949</v>
       </c>
       <c r="I17" t="n">
-        <v>38.97757122651041</v>
+        <v>42.07197382769901</v>
       </c>
       <c r="J17" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K17" t="n">
         <v>54.65</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M17" t="n">
         <v>54.65</v>
       </c>
       <c r="N17" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O17" t="n">
-        <v>65.95744680851064</v>
+        <v>70.21276595744681</v>
       </c>
       <c r="P17" t="n">
-        <v>47.05148936170213</v>
+        <v>51.90255319148936</v>
       </c>
       <c r="Q17" t="b">
         <v>0</v>
@@ -1819,25 +1819,25 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>697.65</v>
+        <v>674.75</v>
       </c>
       <c r="D18" t="n">
-        <v>-0.0896457232335095</v>
+        <v>-0.059909439219784</v>
       </c>
       <c r="E18" t="n">
-        <v>0.1612983770287139</v>
+        <v>0.1113398665898048</v>
       </c>
       <c r="F18" t="n">
-        <v>0.0669062547790182</v>
+        <v>-0.0029553010712966</v>
       </c>
       <c r="G18" t="n">
-        <v>0.0874788961169924</v>
+        <v>0.0176173402666776</v>
       </c>
       <c r="H18" t="n">
-        <v>0.1217459865211104</v>
+        <v>0.0518844306707956</v>
       </c>
       <c r="I18" t="n">
-        <v>49.20332525112573</v>
+        <v>40.25722339675829</v>
       </c>
       <c r="J18" t="n">
         <v>60</v>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M18" t="n">
@@ -1857,10 +1857,10 @@
         <v>60</v>
       </c>
       <c r="O18" t="n">
-        <v>72.3404255319149</v>
+        <v>65.95744680851064</v>
       </c>
       <c r="P18" t="n">
-        <v>58.43608510638298</v>
+        <v>57.15948936170213</v>
       </c>
       <c r="Q18" t="b">
         <v>0</v>
@@ -1884,25 +1884,25 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2333.1</v>
+        <v>2260</v>
       </c>
       <c r="D19" t="n">
-        <v>-0.0867778299671208</v>
+        <v>-0.1553927797294267</v>
       </c>
       <c r="E19" t="n">
-        <v>-0.1225648740127868</v>
+        <v>-0.1388835968755953</v>
       </c>
       <c r="F19" t="n">
-        <v>-0.1985779060181368</v>
+        <v>-0.2295104322923769</v>
       </c>
       <c r="G19" t="n">
-        <v>-0.1780052646801626</v>
+        <v>-0.2089377909544026</v>
       </c>
       <c r="H19" t="n">
-        <v>-0.1437381742760446</v>
+        <v>-0.1746707005502846</v>
       </c>
       <c r="I19" t="n">
-        <v>35.89414595028067</v>
+        <v>36.59254414650099</v>
       </c>
       <c r="J19" t="n">
         <v>30</v>
@@ -1912,7 +1912,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M19" t="n">
@@ -1949,25 +1949,25 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2083.6</v>
+        <v>1966.1</v>
       </c>
       <c r="D20" t="n">
-        <v>-0.0729667200569496</v>
+        <v>-0.1309287008796359</v>
       </c>
       <c r="E20" t="n">
-        <v>-0.07535280021301149</v>
+        <v>-0.1352860975502484</v>
       </c>
       <c r="F20" t="n">
-        <v>-0.0492790655229056</v>
+        <v>-0.0962952748667034</v>
       </c>
       <c r="G20" t="n">
-        <v>-0.0287064241849314</v>
+        <v>-0.0757226335287292</v>
       </c>
       <c r="H20" t="n">
-        <v>0.0055606662191866</v>
+        <v>-0.0414555431246111</v>
       </c>
       <c r="I20" t="n">
-        <v>46.00603897886356</v>
+        <v>45.03560392314927</v>
       </c>
       <c r="J20" t="n">
         <v>40</v>
@@ -1977,7 +1977,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M20" t="n">
@@ -1987,16 +1987,16 @@
         <v>40</v>
       </c>
       <c r="O20" t="n">
-        <v>59.57446808510638</v>
+        <v>53.19148936170212</v>
       </c>
       <c r="P20" t="n">
-        <v>47.53889361702128</v>
+        <v>46.26229787234043</v>
       </c>
       <c r="Q20" t="b">
         <v>0</v>
       </c>
       <c r="R20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S20" t="b">
         <v>0</v>
@@ -2014,25 +2014,25 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>881.25</v>
+        <v>823.1</v>
       </c>
       <c r="D21" t="n">
-        <v>-0.09355070973050809</v>
+        <v>-0.1863384737050217</v>
       </c>
       <c r="E21" t="n">
-        <v>-0.081265638031693</v>
+        <v>-0.1568326162671584</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.3033596837944664</v>
+        <v>-0.3265423007691049</v>
       </c>
       <c r="G21" t="n">
-        <v>-0.2827870424564922</v>
+        <v>-0.3059696594311307</v>
       </c>
       <c r="H21" t="n">
-        <v>-0.2485199520523742</v>
+        <v>-0.2717025690270127</v>
       </c>
       <c r="I21" t="n">
-        <v>41.35438182354677</v>
+        <v>42.23293656772639</v>
       </c>
       <c r="J21" t="n">
         <v>40</v>
@@ -2042,7 +2042,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M21" t="n">
@@ -2079,25 +2079,25 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>396.15</v>
+        <v>377.85</v>
       </c>
       <c r="D22" t="n">
-        <v>-0.0439242186557259</v>
+        <v>-0.1040901007705986</v>
       </c>
       <c r="E22" t="n">
-        <v>0.2727710843373494</v>
+        <v>0.2341989220970115</v>
       </c>
       <c r="F22" t="n">
-        <v>0.2610218048702848</v>
+        <v>0.2218270008084075</v>
       </c>
       <c r="G22" t="n">
-        <v>0.281594446208259</v>
+        <v>0.2423996421463817</v>
       </c>
       <c r="H22" t="n">
-        <v>0.315861536612377</v>
+        <v>0.2766667325504998</v>
       </c>
       <c r="I22" t="n">
-        <v>39.38129996524157</v>
+        <v>33.32275468105364</v>
       </c>
       <c r="J22" t="n">
         <v>30</v>
@@ -2107,7 +2107,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M22" t="n">
@@ -2144,48 +2144,48 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>335.15</v>
+        <v>322.35</v>
       </c>
       <c r="D23" t="n">
-        <v>-0.0921034809697954</v>
+        <v>-0.1374096869146372</v>
       </c>
       <c r="E23" t="n">
-        <v>-0.1009924892703864</v>
+        <v>-0.1297246220302375</v>
       </c>
       <c r="F23" t="n">
-        <v>-0.1699071207430341</v>
+        <v>-0.2039757994814174</v>
       </c>
       <c r="G23" t="n">
-        <v>-0.1493344794050599</v>
+        <v>-0.1834031581434432</v>
       </c>
       <c r="H23" t="n">
-        <v>-0.1150673890009419</v>
+        <v>-0.1491360677393252</v>
       </c>
       <c r="I23" t="n">
-        <v>31.39534883720927</v>
+        <v>23.52941176470587</v>
       </c>
       <c r="J23" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="K23" t="n">
         <v>49.7</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M23" t="n">
         <v>49.7</v>
       </c>
       <c r="N23" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="O23" t="n">
-        <v>25.53191489361702</v>
+        <v>23.40425531914894</v>
       </c>
       <c r="P23" t="n">
-        <v>36.98638297872341</v>
+        <v>32.56085106382979</v>
       </c>
       <c r="Q23" t="b">
         <v>0</v>
@@ -2209,48 +2209,48 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>121.47</v>
+        <v>116.62</v>
       </c>
       <c r="D24" t="n">
-        <v>-0.1223900007224911</v>
+        <v>-0.1895197720480922</v>
       </c>
       <c r="E24" t="n">
-        <v>-0.005159705159705</v>
+        <v>-0.0477668000326609</v>
       </c>
       <c r="F24" t="n">
-        <v>0.1259733036707453</v>
+        <v>0.0995662832359043</v>
       </c>
       <c r="G24" t="n">
-        <v>0.1465459450087195</v>
+        <v>0.1201389245738785</v>
       </c>
       <c r="H24" t="n">
-        <v>0.1808130354128375</v>
+        <v>0.1544060149779965</v>
       </c>
       <c r="I24" t="n">
-        <v>36.21378621378621</v>
+        <v>44.2432872253865</v>
       </c>
       <c r="J24" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K24" t="n">
         <v>48.3</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M24" t="n">
         <v>48.3</v>
       </c>
       <c r="N24" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O24" t="n">
-        <v>78.72340425531915</v>
+        <v>80.85106382978722</v>
       </c>
       <c r="P24" t="n">
-        <v>47.06468085106384</v>
+        <v>51.49021276595744</v>
       </c>
       <c r="Q24" t="b">
         <v>0</v>
@@ -2274,48 +2274,48 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>572.65</v>
+        <v>546.65</v>
       </c>
       <c r="D25" t="n">
-        <v>0.0089859924235751</v>
+        <v>-0.0176116452511457</v>
       </c>
       <c r="E25" t="n">
-        <v>-0.0294890263536987</v>
+        <v>-0.0434820647419073</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.0634557200098128</v>
+        <v>-0.09860664523043949</v>
       </c>
       <c r="G25" t="n">
-        <v>-0.0428830786718386</v>
+        <v>-0.0780340038924652</v>
       </c>
       <c r="H25" t="n">
-        <v>-0.0086159882677205</v>
+        <v>-0.0437669134883472</v>
       </c>
       <c r="I25" t="n">
-        <v>60.2561852956659</v>
+        <v>56.43496214728149</v>
       </c>
       <c r="J25" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K25" t="n">
         <v>56.91</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M25" t="n">
         <v>56.91</v>
       </c>
       <c r="N25" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O25" t="n">
-        <v>55.31914893617022</v>
+        <v>51.06382978723404</v>
       </c>
       <c r="P25" t="n">
-        <v>65.82782978723404</v>
+        <v>56.9767659574468</v>
       </c>
       <c r="Q25" t="b">
         <v>0</v>
@@ -2339,48 +2339,48 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>125.84</v>
+        <v>120.82</v>
       </c>
       <c r="D26" t="n">
-        <v>-0.0838005096468874</v>
+        <v>-0.1401323749199344</v>
       </c>
       <c r="E26" t="n">
-        <v>-0.1233716475095786</v>
+        <v>-0.1724090691143229</v>
       </c>
       <c r="F26" t="n">
-        <v>-0.0829993441667272</v>
+        <v>-0.157696597880647</v>
       </c>
       <c r="G26" t="n">
-        <v>-0.062426702828753</v>
+        <v>-0.1371239565426728</v>
       </c>
       <c r="H26" t="n">
-        <v>-0.028159612424635</v>
+        <v>-0.1028568661385548</v>
       </c>
       <c r="I26" t="n">
-        <v>41.5401600883246</v>
+        <v>39.0909090909091</v>
       </c>
       <c r="J26" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K26" t="n">
         <v>51.54</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M26" t="n">
         <v>51.54</v>
       </c>
       <c r="N26" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O26" t="n">
-        <v>48.93617021276596</v>
+        <v>29.78723404255319</v>
       </c>
       <c r="P26" t="n">
-        <v>46.4032340425532</v>
+        <v>38.57344680851064</v>
       </c>
       <c r="Q26" t="b">
         <v>0</v>
@@ -2404,48 +2404,48 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>5148.5</v>
+        <v>4880</v>
       </c>
       <c r="D27" t="n">
-        <v>-0.1565781498288092</v>
+        <v>-0.214752357352042</v>
       </c>
       <c r="E27" t="n">
-        <v>-0.09189522885616019</v>
+        <v>-0.152041702867072</v>
       </c>
       <c r="F27" t="n">
-        <v>0.2336759878273788</v>
+        <v>0.1645110485372021</v>
       </c>
       <c r="G27" t="n">
-        <v>0.254248629165353</v>
+        <v>0.1850836898751763</v>
       </c>
       <c r="H27" t="n">
-        <v>0.2885157195694711</v>
+        <v>0.2193507802792943</v>
       </c>
       <c r="I27" t="n">
-        <v>38.56340288924559</v>
+        <v>42.24175824175824</v>
       </c>
       <c r="J27" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K27" t="n">
         <v>57.69</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M27" t="n">
         <v>57.69</v>
       </c>
       <c r="N27" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O27" t="n">
-        <v>89.36170212765957</v>
+        <v>87.2340425531915</v>
       </c>
       <c r="P27" t="n">
-        <v>52.94834042553191</v>
+        <v>56.5228085106383</v>
       </c>
       <c r="Q27" t="b">
         <v>0</v>
@@ -2469,25 +2469,25 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1623.3</v>
+        <v>1608.8</v>
       </c>
       <c r="D28" t="n">
-        <v>-0.0232264275828871</v>
+        <v>-0.064107038976149</v>
       </c>
       <c r="E28" t="n">
-        <v>0.06459863588667369</v>
+        <v>0.0642323212277566</v>
       </c>
       <c r="F28" t="n">
-        <v>0.4412678682411435</v>
+        <v>0.5187387897668272</v>
       </c>
       <c r="G28" t="n">
-        <v>0.4618405095791177</v>
+        <v>0.5393114311048014</v>
       </c>
       <c r="H28" t="n">
-        <v>0.4961075999832357</v>
+        <v>0.5735785215089194</v>
       </c>
       <c r="I28" t="n">
-        <v>57.3173835581573</v>
+        <v>59.15453915453915</v>
       </c>
       <c r="J28" t="n">
         <v>80</v>
@@ -2497,7 +2497,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M28" t="n">
@@ -2507,10 +2507,10 @@
         <v>80</v>
       </c>
       <c r="O28" t="n">
-        <v>93.61702127659576</v>
+        <v>95.74468085106383</v>
       </c>
       <c r="P28" t="n">
-        <v>72.52740425531915</v>
+        <v>72.95293617021277</v>
       </c>
       <c r="Q28" t="b">
         <v>0</v>
@@ -2534,25 +2534,25 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>543.95</v>
+        <v>528.7</v>
       </c>
       <c r="D29" t="n">
-        <v>-0.0612649926654585</v>
+        <v>-0.0871104204437536</v>
       </c>
       <c r="E29" t="n">
-        <v>-0.071995223065768</v>
+        <v>-0.090643274853801</v>
       </c>
       <c r="F29" t="n">
-        <v>0.0716115051221435</v>
+        <v>0.0521393034825872</v>
       </c>
       <c r="G29" t="n">
-        <v>0.0921841464601177</v>
+        <v>0.0727119448205614</v>
       </c>
       <c r="H29" t="n">
-        <v>0.1264512368642357</v>
+        <v>0.1069790352246794</v>
       </c>
       <c r="I29" t="n">
-        <v>54.80591497227357</v>
+        <v>60.57201225740555</v>
       </c>
       <c r="J29" t="n">
         <v>60</v>
@@ -2562,7 +2562,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M29" t="n">
@@ -2572,10 +2572,10 @@
         <v>60</v>
       </c>
       <c r="O29" t="n">
-        <v>74.46808510638297</v>
+        <v>78.72340425531915</v>
       </c>
       <c r="P29" t="n">
-        <v>58.6616170212766</v>
+        <v>59.51268085106384</v>
       </c>
       <c r="Q29" t="b">
         <v>0</v>
@@ -2599,25 +2599,25 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>111.94</v>
+        <v>109.22</v>
       </c>
       <c r="D30" t="n">
-        <v>-0.0594067725401227</v>
+        <v>-0.0545360110803323</v>
       </c>
       <c r="E30" t="n">
-        <v>0.0506851886615355</v>
+        <v>0.0213203665606882</v>
       </c>
       <c r="F30" t="n">
-        <v>-0.1103163249085995</v>
+        <v>-0.1213900732040865</v>
       </c>
       <c r="G30" t="n">
-        <v>-0.0897436835706253</v>
+        <v>-0.1008174318661123</v>
       </c>
       <c r="H30" t="n">
-        <v>-0.0554765931665073</v>
+        <v>-0.0665503414619943</v>
       </c>
       <c r="I30" t="n">
-        <v>41.92680301399354</v>
+        <v>40.5096203848154</v>
       </c>
       <c r="J30" t="n">
         <v>40</v>
@@ -2627,7 +2627,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M30" t="n">
@@ -2637,10 +2637,10 @@
         <v>40</v>
       </c>
       <c r="O30" t="n">
-        <v>44.68085106382978</v>
+        <v>48.93617021276596</v>
       </c>
       <c r="P30" t="n">
-        <v>45.88817021276596</v>
+        <v>46.73923404255319</v>
       </c>
       <c r="Q30" t="b">
         <v>0</v>
@@ -2664,25 +2664,25 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>37.98</v>
+        <v>37.9</v>
       </c>
       <c r="D31" t="n">
-        <v>-0.1459410838767709</v>
+        <v>-0.1301354142758779</v>
       </c>
       <c r="E31" t="n">
-        <v>-0.1671052631578948</v>
+        <v>-0.153072625698324</v>
       </c>
       <c r="F31" t="n">
-        <v>-0.1167441860465117</v>
+        <v>-0.1415628539071347</v>
       </c>
       <c r="G31" t="n">
-        <v>-0.0961715447085375</v>
+        <v>-0.1209902125691605</v>
       </c>
       <c r="H31" t="n">
-        <v>-0.0619044543044194</v>
+        <v>-0.08672312216504249</v>
       </c>
       <c r="I31" t="n">
-        <v>30.71120689655172</v>
+        <v>35.9848484848485</v>
       </c>
       <c r="J31" t="n">
         <v>30</v>
@@ -2692,7 +2692,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M31" t="n">
@@ -2702,10 +2702,10 @@
         <v>30</v>
       </c>
       <c r="O31" t="n">
-        <v>40.42553191489361</v>
+        <v>38.29787234042553</v>
       </c>
       <c r="P31" t="n">
-        <v>39.68110638297873</v>
+        <v>39.25557446808512</v>
       </c>
       <c r="Q31" t="b">
         <v>0</v>
@@ -2729,25 +2729,25 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>686.55</v>
+        <v>652.9</v>
       </c>
       <c r="D32" t="n">
-        <v>-0.1282458256618627</v>
+        <v>-0.1403554970375247</v>
       </c>
       <c r="E32" t="n">
-        <v>-0.1817531732316309</v>
+        <v>-0.2071645415907711</v>
       </c>
       <c r="F32" t="n">
-        <v>-0.3496732026143792</v>
+        <v>-0.3728146013448608</v>
       </c>
       <c r="G32" t="n">
-        <v>-0.3291005612764049</v>
+        <v>-0.3522419600068865</v>
       </c>
       <c r="H32" t="n">
-        <v>-0.2948334708722869</v>
+        <v>-0.3179748696027685</v>
       </c>
       <c r="I32" t="n">
-        <v>47.40046838407492</v>
+        <v>44.20951465641519</v>
       </c>
       <c r="J32" t="n">
         <v>40</v>
@@ -2757,7 +2757,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M32" t="n">
@@ -2794,25 +2794,25 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>543.95</v>
+        <v>525.3</v>
       </c>
       <c r="D33" t="n">
-        <v>-0.1378189887462354</v>
+        <v>-0.1585776069197501</v>
       </c>
       <c r="E33" t="n">
-        <v>-0.0963535177340311</v>
+        <v>-0.1609966459032105</v>
       </c>
       <c r="F33" t="n">
-        <v>0.1429922252574071</v>
+        <v>0.0501799280287884</v>
       </c>
       <c r="G33" t="n">
-        <v>0.1635648665953814</v>
+        <v>0.07075256936676259</v>
       </c>
       <c r="H33" t="n">
-        <v>0.1978319569994994</v>
+        <v>0.1050196597708806</v>
       </c>
       <c r="I33" t="n">
-        <v>44.98910675381264</v>
+        <v>44.67965001411233</v>
       </c>
       <c r="J33" t="n">
         <v>40</v>
@@ -2822,7 +2822,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M33" t="n">
@@ -2832,10 +2832,10 @@
         <v>40</v>
       </c>
       <c r="O33" t="n">
-        <v>80.85106382978722</v>
+        <v>76.59574468085107</v>
       </c>
       <c r="P33" t="n">
-        <v>52.16221276595745</v>
+        <v>51.31114893617022</v>
       </c>
       <c r="Q33" t="b">
         <v>0</v>
@@ -2887,7 +2887,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M34" t="n">
@@ -2897,10 +2897,10 @@
         <v>80</v>
       </c>
       <c r="O34" t="n">
-        <v>17.02127659574468</v>
+        <v>19.14893617021277</v>
       </c>
       <c r="P34" t="n">
-        <v>55.75625531914894</v>
+        <v>56.18178723404256</v>
       </c>
       <c r="Q34" t="b">
         <v>0</v>
@@ -2924,25 +2924,25 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>109.14</v>
+        <v>105.08</v>
       </c>
       <c r="D35" t="n">
-        <v>-0.1325013909864081</v>
+        <v>-0.1788058768365114</v>
       </c>
       <c r="E35" t="n">
-        <v>-0.0156038603770182</v>
+        <v>0.0136008488473038</v>
       </c>
       <c r="F35" t="n">
-        <v>0.1063355296502788</v>
+        <v>0.0489119584747452</v>
       </c>
       <c r="G35" t="n">
-        <v>0.126908170988253</v>
+        <v>0.0694845998127194</v>
       </c>
       <c r="H35" t="n">
-        <v>0.161175261392371</v>
+        <v>0.1037516902168375</v>
       </c>
       <c r="I35" t="n">
-        <v>42.75874906924796</v>
+        <v>49.75092051115443</v>
       </c>
       <c r="J35" t="n">
         <v>40</v>
@@ -2952,7 +2952,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M35" t="n">
@@ -2962,10 +2962,10 @@
         <v>40</v>
       </c>
       <c r="O35" t="n">
-        <v>76.59574468085107</v>
+        <v>74.46808510638297</v>
       </c>
       <c r="P35" t="n">
-        <v>50.94714893617022</v>
+        <v>50.5216170212766</v>
       </c>
       <c r="Q35" t="b">
         <v>0</v>
@@ -2989,25 +2989,25 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>465</v>
+        <v>462.7</v>
       </c>
       <c r="D36" t="n">
-        <v>-0.0433083016150601</v>
+        <v>-0.0722807017543859</v>
       </c>
       <c r="E36" t="n">
-        <v>-0.1528511568591728</v>
+        <v>-0.1741923969302159</v>
       </c>
       <c r="F36" t="n">
-        <v>0.028533510285335</v>
+        <v>0.0011900897976848</v>
       </c>
       <c r="G36" t="n">
-        <v>0.0491061516233092</v>
+        <v>0.021762731135659</v>
       </c>
       <c r="H36" t="n">
-        <v>0.0833732420274272</v>
+        <v>0.056029821539777</v>
       </c>
       <c r="I36" t="n">
-        <v>33.50762527233114</v>
+        <v>34.98635122838944</v>
       </c>
       <c r="J36" t="n">
         <v>30</v>
@@ -3017,7 +3017,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M36" t="n">
@@ -3054,25 +3054,25 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2183</v>
+        <v>2159.2</v>
       </c>
       <c r="D37" t="n">
-        <v>-0.06329113924050631</v>
+        <v>-0.0825189088127815</v>
       </c>
       <c r="E37" t="n">
-        <v>0.3173616559048942</v>
+        <v>0.2840915848944394</v>
       </c>
       <c r="F37" t="n">
-        <v>0.6919857386451713</v>
+        <v>0.6443530576498362</v>
       </c>
       <c r="G37" t="n">
-        <v>0.7125583799831455</v>
+        <v>0.6649256989878104</v>
       </c>
       <c r="H37" t="n">
-        <v>0.7468254703872635</v>
+        <v>0.6991927893919284</v>
       </c>
       <c r="I37" t="n">
-        <v>47.6534296028881</v>
+        <v>53.22580645161288</v>
       </c>
       <c r="J37" t="n">
         <v>80</v>
@@ -3082,7 +3082,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M37" t="n">
@@ -3119,25 +3119,25 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>795.15</v>
+        <v>757.1</v>
       </c>
       <c r="D38" t="n">
-        <v>-0.182659197204091</v>
+        <v>-0.2093363270847474</v>
       </c>
       <c r="E38" t="n">
-        <v>-0.1828271928472329</v>
+        <v>-0.2153184432813391</v>
       </c>
       <c r="F38" t="n">
-        <v>-0.2431467732724157</v>
+        <v>-0.2846749811035526</v>
       </c>
       <c r="G38" t="n">
-        <v>-0.2225741319344415</v>
+        <v>-0.2641023397655784</v>
       </c>
       <c r="H38" t="n">
-        <v>-0.1883070415303235</v>
+        <v>-0.2298352493614603</v>
       </c>
       <c r="I38" t="n">
-        <v>41.92412357931806</v>
+        <v>41.20516047828823</v>
       </c>
       <c r="J38" t="n">
         <v>40</v>
@@ -3147,7 +3147,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M38" t="n">
@@ -3157,10 +3157,10 @@
         <v>40</v>
       </c>
       <c r="O38" t="n">
-        <v>14.8936170212766</v>
+        <v>10.63829787234042</v>
       </c>
       <c r="P38" t="n">
-        <v>38.92672340425532</v>
+        <v>38.07565957446808</v>
       </c>
       <c r="Q38" t="b">
         <v>0</v>
@@ -3184,25 +3184,25 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>3102.1</v>
+        <v>3033.5</v>
       </c>
       <c r="D39" t="n">
-        <v>0.008747398543184201</v>
+        <v>-0.0419114395805697</v>
       </c>
       <c r="E39" t="n">
-        <v>0.0930970083512456</v>
+        <v>-0.0298698391378042</v>
       </c>
       <c r="F39" t="n">
-        <v>0.2254483684917436</v>
+        <v>0.1788365134263396</v>
       </c>
       <c r="G39" t="n">
-        <v>0.2460210098297178</v>
+        <v>0.1994091547643138</v>
       </c>
       <c r="H39" t="n">
-        <v>0.2802881002338359</v>
+        <v>0.2336762451684318</v>
       </c>
       <c r="I39" t="n">
-        <v>53.98535417546823</v>
+        <v>58.48653596765581</v>
       </c>
       <c r="J39" t="n">
         <v>80</v>
@@ -3212,7 +3212,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M39" t="n">
@@ -3222,10 +3222,10 @@
         <v>80</v>
       </c>
       <c r="O39" t="n">
-        <v>87.2340425531915</v>
+        <v>89.36170212765957</v>
       </c>
       <c r="P39" t="n">
-        <v>68.9228085106383</v>
+        <v>69.34834042553192</v>
       </c>
       <c r="Q39" t="b">
         <v>0</v>
@@ -3249,25 +3249,25 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>185.82</v>
+        <v>178.97</v>
       </c>
       <c r="D40" t="n">
-        <v>-0.1464792614027835</v>
+        <v>-0.1683936620045537</v>
       </c>
       <c r="E40" t="n">
-        <v>-0.0304706250652196</v>
+        <v>-0.0308133867648651</v>
       </c>
       <c r="F40" t="n">
-        <v>-0.1755257786848877</v>
+        <v>-0.2002770454443898</v>
       </c>
       <c r="G40" t="n">
-        <v>-0.1549531373469135</v>
+        <v>-0.1797044041064156</v>
       </c>
       <c r="H40" t="n">
-        <v>-0.1206860469427955</v>
+        <v>-0.1454373137022976</v>
       </c>
       <c r="I40" t="n">
-        <v>40.83181542197934</v>
+        <v>43.10897435897437</v>
       </c>
       <c r="J40" t="n">
         <v>40</v>
@@ -3277,7 +3277,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M40" t="n">
@@ -3287,10 +3287,10 @@
         <v>40</v>
       </c>
       <c r="O40" t="n">
-        <v>23.40425531914894</v>
+        <v>25.53191489361702</v>
       </c>
       <c r="P40" t="n">
-        <v>38.85685106382979</v>
+        <v>39.2823829787234</v>
       </c>
       <c r="Q40" t="b">
         <v>0</v>
@@ -3314,25 +3314,25 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>799</v>
+        <v>762.65</v>
       </c>
       <c r="D41" t="n">
-        <v>-0.138776610078146</v>
+        <v>-0.1622913005272407</v>
       </c>
       <c r="E41" t="n">
-        <v>-0.1522096662952942</v>
+        <v>-0.1883680093651891</v>
       </c>
       <c r="F41" t="n">
-        <v>-0.2199550912818509</v>
+        <v>-0.2498770532113702</v>
       </c>
       <c r="G41" t="n">
-        <v>-0.1993824499438767</v>
+        <v>-0.229304411873396</v>
       </c>
       <c r="H41" t="n">
-        <v>-0.1651153595397587</v>
+        <v>-0.195037321469278</v>
       </c>
       <c r="I41" t="n">
-        <v>27.5675675675676</v>
+        <v>23.986975397974</v>
       </c>
       <c r="J41" t="n">
         <v>20</v>
@@ -3342,7 +3342,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M41" t="n">
@@ -3352,10 +3352,10 @@
         <v>20</v>
       </c>
       <c r="O41" t="n">
-        <v>19.14893617021277</v>
+        <v>17.02127659574468</v>
       </c>
       <c r="P41" t="n">
-        <v>31.04978723404255</v>
+        <v>30.62425531914894</v>
       </c>
       <c r="Q41" t="b">
         <v>0</v>
@@ -3379,25 +3379,25 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>525.55</v>
+        <v>496</v>
       </c>
       <c r="D42" t="n">
-        <v>-0.2231911905993644</v>
+        <v>-0.2457994373907093</v>
       </c>
       <c r="E42" t="n">
-        <v>-0.2653760134190662</v>
+        <v>-0.2622341216718726</v>
       </c>
       <c r="F42" t="n">
-        <v>-0.3267358442223931</v>
+        <v>-0.3624678663239075</v>
       </c>
       <c r="G42" t="n">
-        <v>-0.3061632028844189</v>
+        <v>-0.3418952249859333</v>
       </c>
       <c r="H42" t="n">
-        <v>-0.2718961124803009</v>
+        <v>-0.3076281345818152</v>
       </c>
       <c r="I42" t="n">
-        <v>38.38383838383837</v>
+        <v>33.40896199659673</v>
       </c>
       <c r="J42" t="n">
         <v>30</v>
@@ -3407,7 +3407,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M42" t="n">
@@ -3444,48 +3444,48 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>410.45</v>
+        <v>414.45</v>
       </c>
       <c r="D43" t="n">
-        <v>-0.0178272313950705</v>
+        <v>-0.07694877505567931</v>
       </c>
       <c r="E43" t="n">
-        <v>-0.1063575005443066</v>
+        <v>-0.09725549989109129</v>
       </c>
       <c r="F43" t="n">
-        <v>-0.1105211832267851</v>
+        <v>-0.0862087972660126</v>
       </c>
       <c r="G43" t="n">
-        <v>-0.08994854188881091</v>
+        <v>-0.0656361559280384</v>
       </c>
       <c r="H43" t="n">
-        <v>-0.0556814514846929</v>
+        <v>-0.0313690655239203</v>
       </c>
       <c r="I43" t="n">
-        <v>40.36970781156825</v>
+        <v>51.39171758316361</v>
       </c>
       <c r="J43" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K43" t="n">
         <v>51.48</v>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M43" t="n">
         <v>51.48</v>
       </c>
       <c r="N43" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O43" t="n">
-        <v>42.5531914893617</v>
+        <v>55.31914893617022</v>
       </c>
       <c r="P43" t="n">
-        <v>45.10263829787234</v>
+        <v>55.65582978723404</v>
       </c>
       <c r="Q43" t="b">
         <v>0</v>
@@ -3509,25 +3509,25 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>238.9</v>
+        <v>233</v>
       </c>
       <c r="D44" t="n">
-        <v>-0.1361417465196167</v>
+        <v>-0.1243893273205563</v>
       </c>
       <c r="E44" t="n">
-        <v>-0.1623422159887797</v>
+        <v>-0.1712608927618708</v>
       </c>
       <c r="F44" t="n">
-        <v>-0.0979799886728337</v>
+        <v>-0.1309212980231258</v>
       </c>
       <c r="G44" t="n">
-        <v>-0.0774073473348595</v>
+        <v>-0.1103486566851515</v>
       </c>
       <c r="H44" t="n">
-        <v>-0.0431402569307415</v>
+        <v>-0.07608156628103351</v>
       </c>
       <c r="I44" t="n">
-        <v>46.77242888402625</v>
+        <v>43.38358458961473</v>
       </c>
       <c r="J44" t="n">
         <v>40</v>
@@ -3537,7 +3537,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M44" t="n">
@@ -3547,10 +3547,10 @@
         <v>40</v>
       </c>
       <c r="O44" t="n">
-        <v>46.80851063829788</v>
+        <v>44.68085106382978</v>
       </c>
       <c r="P44" t="n">
-        <v>44.24170212765958</v>
+        <v>43.81617021276596</v>
       </c>
       <c r="Q44" t="b">
         <v>0</v>
@@ -3574,48 +3574,48 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>92.33</v>
+        <v>86.55</v>
       </c>
       <c r="D45" t="n">
-        <v>-0.1465939550790276</v>
+        <v>-0.2008310249307479</v>
       </c>
       <c r="E45" t="n">
-        <v>-0.1683480453972257</v>
+        <v>-0.2118921872154434</v>
       </c>
       <c r="F45" t="n">
-        <v>-0.316074074074074</v>
+        <v>-0.3525099124710107</v>
       </c>
       <c r="G45" t="n">
-        <v>-0.2955014327360998</v>
+        <v>-0.3319372711330365</v>
       </c>
       <c r="H45" t="n">
-        <v>-0.2612343423319818</v>
+        <v>-0.2976701807289185</v>
       </c>
       <c r="I45" t="n">
-        <v>31.15942028985505</v>
+        <v>26.31389488840891</v>
       </c>
       <c r="J45" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="K45" t="n">
         <v>59.6</v>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M45" t="n">
         <v>59.6</v>
       </c>
       <c r="N45" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="O45" t="n">
         <v>6.382978723404255</v>
       </c>
       <c r="P45" t="n">
-        <v>37.11659574468086</v>
+        <v>33.11659574468086</v>
       </c>
       <c r="Q45" t="b">
         <v>0</v>
@@ -3639,25 +3639,25 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>493.4</v>
+        <v>487.6</v>
       </c>
       <c r="D46" t="n">
-        <v>-0.1059164628069222</v>
+        <v>-0.1153846153846154</v>
       </c>
       <c r="E46" t="n">
-        <v>-0.2267669644256387</v>
+        <v>-0.2353771365846009</v>
       </c>
       <c r="F46" t="n">
-        <v>-0.1265710745264648</v>
+        <v>-0.1309926929246123</v>
       </c>
       <c r="G46" t="n">
-        <v>-0.1059984331884906</v>
+        <v>-0.1104200515866381</v>
       </c>
       <c r="H46" t="n">
-        <v>-0.0717313427843726</v>
+        <v>-0.0761529611825201</v>
       </c>
       <c r="I46" t="n">
-        <v>45.43721056932715</v>
+        <v>51.3337670787248</v>
       </c>
       <c r="J46" t="n">
         <v>40</v>
@@ -3667,7 +3667,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M46" t="n">
@@ -3677,10 +3677,10 @@
         <v>40</v>
       </c>
       <c r="O46" t="n">
-        <v>36.17021276595745</v>
+        <v>42.5531914893617</v>
       </c>
       <c r="P46" t="n">
-        <v>43.07804255319149</v>
+        <v>44.35463829787234</v>
       </c>
       <c r="Q46" t="b">
         <v>0</v>
@@ -3704,25 +3704,25 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>1089.55</v>
+        <v>1082.1</v>
       </c>
       <c r="D47" t="n">
-        <v>0.21276714158504</v>
+        <v>0.2112833715788882</v>
       </c>
       <c r="E47" t="n">
-        <v>0.3153256473712802</v>
+        <v>0.3170642648490749</v>
       </c>
       <c r="F47" t="n">
-        <v>0.4779571351058056</v>
+        <v>0.4677517802644964</v>
       </c>
       <c r="G47" t="n">
-        <v>0.4985297764437798</v>
+        <v>0.4883244216024706</v>
       </c>
       <c r="H47" t="n">
-        <v>0.5327968668478978</v>
+        <v>0.5225915120065886</v>
       </c>
       <c r="I47" t="n">
-        <v>76.0805057411947</v>
+        <v>73.51181999430361</v>
       </c>
       <c r="J47" t="n">
         <v>70</v>
@@ -3732,7 +3732,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M47" t="n">
@@ -3742,10 +3742,10 @@
         <v>70</v>
       </c>
       <c r="O47" t="n">
-        <v>95.74468085106383</v>
+        <v>93.61702127659576</v>
       </c>
       <c r="P47" t="n">
-        <v>65.88093617021276</v>
+        <v>65.45540425531915</v>
       </c>
       <c r="Q47" t="b">
         <v>0</v>
@@ -3769,48 +3769,48 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>13592</v>
+        <v>13678</v>
       </c>
       <c r="D48" t="n">
-        <v>-0.1284386021160628</v>
+        <v>-0.1184583655581335</v>
       </c>
       <c r="E48" t="n">
-        <v>-0.081187047928074</v>
+        <v>-0.0502048468856329</v>
       </c>
       <c r="F48" t="n">
-        <v>-0.0421423537702607</v>
+        <v>-0.0031338823700896</v>
       </c>
       <c r="G48" t="n">
-        <v>-0.0215697124322865</v>
+        <v>0.0174387589678846</v>
       </c>
       <c r="H48" t="n">
-        <v>0.0126973779718314</v>
+        <v>0.0517058493720026</v>
       </c>
       <c r="I48" t="n">
-        <v>37.02397743300423</v>
+        <v>43.48521183053557</v>
       </c>
       <c r="J48" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K48" t="n">
         <v>50.29</v>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M48" t="n">
         <v>50.29</v>
       </c>
       <c r="N48" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O48" t="n">
-        <v>61.70212765957447</v>
+        <v>63.82978723404256</v>
       </c>
       <c r="P48" t="n">
-        <v>44.4564255319149</v>
+        <v>48.88195744680851</v>
       </c>
       <c r="Q48" t="b">
         <v>0</v>
@@ -3945,25 +3945,25 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1623.3</v>
+        <v>1608.8</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.0232264275828871</v>
+        <v>-0.064107038976149</v>
       </c>
       <c r="E2" t="n">
-        <v>0.06459863588667369</v>
+        <v>0.0642323212277566</v>
       </c>
       <c r="F2" t="n">
-        <v>0.4412678682411435</v>
+        <v>0.5187387897668272</v>
       </c>
       <c r="G2" t="n">
-        <v>0.4618405095791177</v>
+        <v>0.5393114311048014</v>
       </c>
       <c r="H2" t="n">
-        <v>0.4961075999832357</v>
+        <v>0.5735785215089194</v>
       </c>
       <c r="I2" t="n">
-        <v>57.3173835581573</v>
+        <v>59.15453915453915</v>
       </c>
       <c r="J2" t="n">
         <v>80</v>
@@ -3973,7 +3973,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M2" t="n">
@@ -3983,10 +3983,10 @@
         <v>80</v>
       </c>
       <c r="O2" t="n">
-        <v>93.61702127659576</v>
+        <v>95.74468085106383</v>
       </c>
       <c r="P2" t="n">
-        <v>72.52740425531915</v>
+        <v>72.95293617021277</v>
       </c>
       <c r="Q2" t="b">
         <v>0</v>
@@ -4010,25 +4010,25 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2183</v>
+        <v>2159.2</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.06329113924050631</v>
+        <v>-0.0825189088127815</v>
       </c>
       <c r="E3" t="n">
-        <v>0.3173616559048942</v>
+        <v>0.2840915848944394</v>
       </c>
       <c r="F3" t="n">
-        <v>0.6919857386451713</v>
+        <v>0.6443530576498362</v>
       </c>
       <c r="G3" t="n">
-        <v>0.7125583799831455</v>
+        <v>0.6649256989878104</v>
       </c>
       <c r="H3" t="n">
-        <v>0.7468254703872635</v>
+        <v>0.6991927893919284</v>
       </c>
       <c r="I3" t="n">
-        <v>47.6534296028881</v>
+        <v>53.22580645161288</v>
       </c>
       <c r="J3" t="n">
         <v>80</v>
@@ -4038,7 +4038,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M3" t="n">
@@ -4075,25 +4075,25 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>3102.1</v>
+        <v>3033.5</v>
       </c>
       <c r="D4" t="n">
-        <v>0.008747398543184201</v>
+        <v>-0.0419114395805697</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0930970083512456</v>
+        <v>-0.0298698391378042</v>
       </c>
       <c r="F4" t="n">
-        <v>0.2254483684917436</v>
+        <v>0.1788365134263396</v>
       </c>
       <c r="G4" t="n">
-        <v>0.2460210098297178</v>
+        <v>0.1994091547643138</v>
       </c>
       <c r="H4" t="n">
-        <v>0.2802881002338359</v>
+        <v>0.2336762451684318</v>
       </c>
       <c r="I4" t="n">
-        <v>53.98535417546823</v>
+        <v>58.48653596765581</v>
       </c>
       <c r="J4" t="n">
         <v>80</v>
@@ -4103,7 +4103,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M4" t="n">
@@ -4113,10 +4113,10 @@
         <v>80</v>
       </c>
       <c r="O4" t="n">
-        <v>87.2340425531915</v>
+        <v>89.36170212765957</v>
       </c>
       <c r="P4" t="n">
-        <v>68.9228085106383</v>
+        <v>69.34834042553192</v>
       </c>
       <c r="Q4" t="b">
         <v>0</v>
@@ -4131,57 +4131,57 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>WHEELS</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Wheels</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>511.45</v>
+        <v>1082.1</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.045891241488667</v>
+        <v>0.2112833715788882</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0377396773866287</v>
+        <v>0.3170642648490749</v>
       </c>
       <c r="F5" t="n">
-        <v>0.1494549949432519</v>
+        <v>0.4677517802644964</v>
       </c>
       <c r="G5" t="n">
-        <v>0.1700276362812262</v>
+        <v>0.4883244216024706</v>
       </c>
       <c r="H5" t="n">
-        <v>0.2042947266853442</v>
+        <v>0.5225915120065886</v>
       </c>
       <c r="I5" t="n">
-        <v>50.15782828282829</v>
+        <v>73.51181999430361</v>
       </c>
       <c r="J5" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K5" t="n">
-        <v>49.66</v>
+        <v>46.83</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M5" t="n">
-        <v>49.66</v>
+        <v>46.83</v>
       </c>
       <c r="N5" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O5" t="n">
-        <v>82.97872340425532</v>
+        <v>93.61702127659576</v>
       </c>
       <c r="P5" t="n">
-        <v>68.45974468085107</v>
+        <v>65.45540425531915</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
@@ -4205,48 +4205,48 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>444.15</v>
+        <v>438.75</v>
       </c>
       <c r="D6" t="n">
-        <v>0.0255137381667049</v>
+        <v>0.0277582572030921</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.0730460189919649</v>
+        <v>-0.0647980390067142</v>
       </c>
       <c r="F6" t="n">
-        <v>-0.1285195722554694</v>
+        <v>-0.15625</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.1079469309174951</v>
+        <v>-0.1356773586620258</v>
       </c>
       <c r="H6" t="n">
-        <v>-0.0736798405133771</v>
+        <v>-0.1014102682579077</v>
       </c>
       <c r="I6" t="n">
-        <v>69.83381502890172</v>
+        <v>72.65353418308227</v>
       </c>
       <c r="J6" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K6" t="n">
         <v>71.28</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M6" t="n">
         <v>71.28</v>
       </c>
       <c r="N6" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O6" t="n">
-        <v>34.04255319148936</v>
+        <v>31.91489361702128</v>
       </c>
       <c r="P6" t="n">
-        <v>67.32051063829788</v>
+        <v>62.89497872340426</v>
       </c>
       <c r="Q6" t="b">
         <v>1</v>
@@ -4261,57 +4261,57 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>WHEELS</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Wheels</t>
+          <t>Forgings</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1089.55</v>
+        <v>1725.1</v>
       </c>
       <c r="D7" t="n">
-        <v>0.21276714158504</v>
+        <v>-0.0930073606729758</v>
       </c>
       <c r="E7" t="n">
-        <v>0.3153256473712802</v>
+        <v>0.2470902913323212</v>
       </c>
       <c r="F7" t="n">
-        <v>0.4779571351058056</v>
+        <v>0.5247480996994871</v>
       </c>
       <c r="G7" t="n">
-        <v>0.4985297764437798</v>
+        <v>0.5453207410374613</v>
       </c>
       <c r="H7" t="n">
-        <v>0.5327968668478978</v>
+        <v>0.5795878314415793</v>
       </c>
       <c r="I7" t="n">
-        <v>76.0805057411947</v>
+        <v>37.99860041987404</v>
       </c>
       <c r="J7" t="n">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="K7" t="n">
-        <v>46.83</v>
+        <v>54.83</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M7" t="n">
-        <v>46.83</v>
+        <v>54.83</v>
       </c>
       <c r="N7" t="n">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="O7" t="n">
-        <v>95.74468085106383</v>
+        <v>97.87234042553192</v>
       </c>
       <c r="P7" t="n">
-        <v>65.88093617021276</v>
+        <v>61.50646808510639</v>
       </c>
       <c r="Q7" t="b">
         <v>0</v>
@@ -4326,63 +4326,63 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>JBMA</t>
+          <t>MINDACORP</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>572.65</v>
+        <v>528.7</v>
       </c>
       <c r="D8" t="n">
-        <v>0.0089859924235751</v>
+        <v>-0.0871104204437536</v>
       </c>
       <c r="E8" t="n">
-        <v>-0.0294890263536987</v>
+        <v>-0.090643274853801</v>
       </c>
       <c r="F8" t="n">
-        <v>-0.0634557200098128</v>
+        <v>0.0521393034825872</v>
       </c>
       <c r="G8" t="n">
-        <v>-0.0428830786718386</v>
+        <v>0.0727119448205614</v>
       </c>
       <c r="H8" t="n">
-        <v>-0.0086159882677205</v>
+        <v>0.1069790352246794</v>
       </c>
       <c r="I8" t="n">
-        <v>60.2561852956659</v>
+        <v>60.57201225740555</v>
       </c>
       <c r="J8" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K8" t="n">
-        <v>56.91</v>
+        <v>49.42</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M8" t="n">
-        <v>56.91</v>
+        <v>49.42</v>
       </c>
       <c r="N8" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O8" t="n">
-        <v>55.31914893617022</v>
+        <v>78.72340425531915</v>
       </c>
       <c r="P8" t="n">
-        <v>65.82782978723404</v>
+        <v>59.51268085106384</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
       </c>
       <c r="R8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S8" t="b">
         <v>0</v>
@@ -4391,57 +4391,57 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>DIVGIITTS</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Forgings</t>
+          <t>Transmission</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1736.5</v>
+        <v>674.75</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.0521288209606987</v>
+        <v>-0.059909439219784</v>
       </c>
       <c r="E9" t="n">
-        <v>0.2350640113798008</v>
+        <v>0.1113398665898048</v>
       </c>
       <c r="F9" t="n">
-        <v>0.5304953287502205</v>
+        <v>-0.0029553010712966</v>
       </c>
       <c r="G9" t="n">
-        <v>0.5510679700881947</v>
+        <v>0.0176173402666776</v>
       </c>
       <c r="H9" t="n">
-        <v>0.5853350604923128</v>
+        <v>0.0518844306707956</v>
       </c>
       <c r="I9" t="n">
-        <v>37.49420670477369</v>
+        <v>40.25722339675829</v>
       </c>
       <c r="J9" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="K9" t="n">
-        <v>54.83</v>
+        <v>49.92</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M9" t="n">
-        <v>54.83</v>
+        <v>49.92</v>
       </c>
       <c r="N9" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="O9" t="n">
-        <v>97.87234042553192</v>
+        <v>65.95744680851064</v>
       </c>
       <c r="P9" t="n">
-        <v>61.50646808510639</v>
+        <v>57.15948936170213</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -4456,7 +4456,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TIINDIA</t>
+          <t>JBMA</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -4465,48 +4465,48 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>2682.4</v>
+        <v>546.65</v>
       </c>
       <c r="D10" t="n">
-        <v>0.0562293274531422</v>
+        <v>-0.0176116452511457</v>
       </c>
       <c r="E10" t="n">
-        <v>0.0058874264071699</v>
+        <v>-0.0434820647419073</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.1198031173092698</v>
+        <v>-0.09860664523043949</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.0992304759712956</v>
+        <v>-0.0780340038924652</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.0649633855671776</v>
+        <v>-0.0437669134883472</v>
       </c>
       <c r="I10" t="n">
-        <v>44.36388353914127</v>
+        <v>56.43496214728149</v>
       </c>
       <c r="J10" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K10" t="n">
-        <v>48.73</v>
+        <v>56.91</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M10" t="n">
-        <v>48.73</v>
+        <v>56.91</v>
       </c>
       <c r="N10" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O10" t="n">
-        <v>38.29787234042553</v>
+        <v>51.06382978723404</v>
       </c>
       <c r="P10" t="n">
-        <v>59.15157446808512</v>
+        <v>56.9767659574468</v>
       </c>
       <c r="Q10" t="b">
         <v>0</v>
@@ -4521,57 +4521,57 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MINDACORP</t>
+          <t>LUMAXIND</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Lighting</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>543.95</v>
+        <v>4880</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.0612649926654585</v>
+        <v>-0.214752357352042</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.071995223065768</v>
+        <v>-0.152041702867072</v>
       </c>
       <c r="F11" t="n">
-        <v>0.0716115051221435</v>
+        <v>0.1645110485372021</v>
       </c>
       <c r="G11" t="n">
-        <v>0.0921841464601177</v>
+        <v>0.1850836898751763</v>
       </c>
       <c r="H11" t="n">
-        <v>0.1264512368642357</v>
+        <v>0.2193507802792943</v>
       </c>
       <c r="I11" t="n">
-        <v>54.80591497227357</v>
+        <v>42.24175824175824</v>
       </c>
       <c r="J11" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="K11" t="n">
-        <v>49.42</v>
+        <v>57.69</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M11" t="n">
-        <v>49.42</v>
+        <v>57.69</v>
       </c>
       <c r="N11" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="O11" t="n">
-        <v>74.46808510638297</v>
+        <v>87.2340425531915</v>
       </c>
       <c r="P11" t="n">
-        <v>58.6616170212766</v>
+        <v>56.5228085106383</v>
       </c>
       <c r="Q11" t="b">
         <v>0</v>
@@ -4586,63 +4586,63 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>DIVGIITTS</t>
+          <t>RANEENGINE</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Transmission</t>
+          <t>Engine/Parts</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>697.65</v>
+        <v>317.75</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.0896457232335095</v>
+        <v>0.1790352504638219</v>
       </c>
       <c r="E12" t="n">
-        <v>0.1612983770287139</v>
+        <v>-0.156154561147258</v>
       </c>
       <c r="F12" t="n">
-        <v>0.0669062547790182</v>
+        <v>-0.2401052253975846</v>
       </c>
       <c r="G12" t="n">
-        <v>0.0874788961169924</v>
+        <v>-0.2195325840596104</v>
       </c>
       <c r="H12" t="n">
-        <v>0.1217459865211104</v>
+        <v>-0.1852654936554923</v>
       </c>
       <c r="I12" t="n">
-        <v>49.20332525112573</v>
+        <v>63.3225806451613</v>
       </c>
       <c r="J12" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K12" t="n">
-        <v>49.92</v>
+        <v>50.88</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M12" t="n">
-        <v>49.92</v>
+        <v>50.88</v>
       </c>
       <c r="N12" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O12" t="n">
-        <v>72.3404255319149</v>
+        <v>19.14893617021277</v>
       </c>
       <c r="P12" t="n">
-        <v>58.43608510638298</v>
+        <v>56.18178723404256</v>
       </c>
       <c r="Q12" t="b">
         <v>0</v>
       </c>
       <c r="R12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S12" t="b">
         <v>0</v>
@@ -4651,57 +4651,57 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>RANEENGINE</t>
+          <t>SUPRAJIT</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Engine/Parts</t>
+          <t>Cables</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>317.75</v>
+        <v>414.45</v>
       </c>
       <c r="D13" t="n">
-        <v>0.1790352504638219</v>
+        <v>-0.07694877505567931</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.156154561147258</v>
+        <v>-0.09725549989109129</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.2401052253975846</v>
+        <v>-0.0862087972660126</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.2195325840596104</v>
+        <v>-0.0656361559280384</v>
       </c>
       <c r="H13" t="n">
-        <v>-0.1852654936554923</v>
+        <v>-0.0313690655239203</v>
       </c>
       <c r="I13" t="n">
-        <v>63.3225806451613</v>
+        <v>51.39171758316361</v>
       </c>
       <c r="J13" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K13" t="n">
-        <v>50.88</v>
+        <v>51.48</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M13" t="n">
-        <v>50.88</v>
+        <v>51.48</v>
       </c>
       <c r="N13" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O13" t="n">
-        <v>17.02127659574468</v>
+        <v>55.31914893617022</v>
       </c>
       <c r="P13" t="n">
-        <v>55.75625531914894</v>
+        <v>55.65582978723404</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
@@ -4716,57 +4716,57 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>LUMAXIND</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Lighting</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>5148.5</v>
+        <v>488.75</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.1565781498288092</v>
+        <v>-0.0982472324723247</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.09189522885616019</v>
+        <v>0.0200354794949391</v>
       </c>
       <c r="F14" t="n">
-        <v>0.2336759878273788</v>
+        <v>0.1159949765955017</v>
       </c>
       <c r="G14" t="n">
-        <v>0.254248629165353</v>
+        <v>0.1365676179334759</v>
       </c>
       <c r="H14" t="n">
-        <v>0.2885157195694711</v>
+        <v>0.1708347083375939</v>
       </c>
       <c r="I14" t="n">
-        <v>38.56340288924559</v>
+        <v>46.33097942892233</v>
       </c>
       <c r="J14" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K14" t="n">
-        <v>57.69</v>
+        <v>49.66</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M14" t="n">
-        <v>57.69</v>
+        <v>49.66</v>
       </c>
       <c r="N14" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O14" t="n">
-        <v>89.36170212765957</v>
+        <v>82.97872340425532</v>
       </c>
       <c r="P14" t="n">
-        <v>52.94834042553191</v>
+        <v>52.45974468085107</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
@@ -4781,57 +4781,57 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PRICOLLTD</t>
+          <t>GNA</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Axles</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>543.95</v>
+        <v>377.85</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.1378189887462354</v>
+        <v>-0.1040901007705986</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.0963535177340311</v>
+        <v>0.2341989220970115</v>
       </c>
       <c r="F15" t="n">
-        <v>0.1429922252574071</v>
+        <v>0.2218270008084075</v>
       </c>
       <c r="G15" t="n">
-        <v>0.1635648665953814</v>
+        <v>0.2423996421463817</v>
       </c>
       <c r="H15" t="n">
-        <v>0.1978319569994994</v>
+        <v>0.2766667325504998</v>
       </c>
       <c r="I15" t="n">
-        <v>44.98910675381264</v>
+        <v>33.32275468105364</v>
       </c>
       <c r="J15" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K15" t="n">
-        <v>49.98</v>
+        <v>54.47</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M15" t="n">
-        <v>49.98</v>
+        <v>54.47</v>
       </c>
       <c r="N15" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O15" t="n">
-        <v>80.85106382978722</v>
+        <v>91.48936170212764</v>
       </c>
       <c r="P15" t="n">
-        <v>52.16221276595745</v>
+        <v>52.08587234042552</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
@@ -4846,57 +4846,57 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>GNA</t>
+          <t>CRAFTSMAN</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Axles</t>
+          <t>Castings</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>396.15</v>
+        <v>6924</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.0439242186557259</v>
+        <v>-0.1117382937780628</v>
       </c>
       <c r="E16" t="n">
-        <v>0.2727710843373494</v>
+        <v>-0.0214810627473148</v>
       </c>
       <c r="F16" t="n">
-        <v>0.2610218048702848</v>
+        <v>0.0129471143296027</v>
       </c>
       <c r="G16" t="n">
-        <v>0.281594446208259</v>
+        <v>0.0335197556675769</v>
       </c>
       <c r="H16" t="n">
-        <v>0.315861536612377</v>
+        <v>0.0677868460716949</v>
       </c>
       <c r="I16" t="n">
-        <v>39.38129996524157</v>
+        <v>42.07197382769901</v>
       </c>
       <c r="J16" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K16" t="n">
-        <v>54.47</v>
+        <v>54.65</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="M16" t="n">
-        <v>54.47</v>
+        <v>54.65</v>
       </c>
       <c r="N16" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O16" t="n">
-        <v>91.48936170212764</v>
+        <v>70.21276595744681</v>
       </c>
       <c r="P16" t="n">
-        <v>52.08587234042552</v>
+        <v>51.90255319148936</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
chore: auto-refresh NSE data and pipeline outputs (2026-03-30)
</commit_message>
<xml_diff>
--- a/working-sector/output/auto_components_comprehensive_report.xlsx
+++ b/working-sector/output/auto_components_comprehensive_report.xlsx
@@ -435,7 +435,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
     </row>
@@ -447,7 +447,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
     </row>
@@ -779,48 +779,48 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1725.1</v>
+        <v>1674.6</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.0930073606729758</v>
+        <v>-0.124163179916318</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2470902913323212</v>
+        <v>0.2101459748518572</v>
       </c>
       <c r="F2" t="n">
-        <v>0.5247480996994871</v>
+        <v>0.4732119292689363</v>
       </c>
       <c r="G2" t="n">
-        <v>0.5453207410374613</v>
+        <v>0.5588154238072776</v>
       </c>
       <c r="H2" t="n">
-        <v>0.5795878314415793</v>
+        <v>0.573634153097961</v>
       </c>
       <c r="I2" t="n">
-        <v>37.99860041987404</v>
+        <v>36.07973421926911</v>
       </c>
       <c r="J2" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="K2" t="n">
         <v>54.83</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M2" t="n">
         <v>54.83</v>
       </c>
       <c r="N2" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="O2" t="n">
         <v>97.87234042553192</v>
       </c>
       <c r="P2" t="n">
-        <v>61.50646808510639</v>
+        <v>53.50646808510639</v>
       </c>
       <c r="Q2" t="b">
         <v>0</v>
@@ -844,48 +844,48 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1048.7</v>
+        <v>1031.6</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.1388569551650517</v>
+        <v>-0.1617097350885746</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.1485751400503369</v>
+        <v>-0.1567072672279899</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.1798701806522249</v>
+        <v>-0.2056060372709071</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.1592975393142507</v>
+        <v>-0.1200025427325658</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.1250304489101327</v>
+        <v>-0.1051838134418824</v>
       </c>
       <c r="I3" t="n">
-        <v>45.71575166752181</v>
+        <v>38.93190921228303</v>
       </c>
       <c r="J3" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K3" t="n">
         <v>49.36</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M3" t="n">
         <v>49.36</v>
       </c>
       <c r="N3" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O3" t="n">
-        <v>27.65957446808511</v>
+        <v>31.91489361702128</v>
       </c>
       <c r="P3" t="n">
-        <v>41.27591489361702</v>
+        <v>38.12697872340426</v>
       </c>
       <c r="Q3" t="b">
         <v>0</v>
@@ -909,48 +909,48 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>29615</v>
+        <v>28745</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.1901832102816516</v>
+        <v>-0.2176102340772999</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.1948069603045132</v>
+        <v>-0.2103021978021978</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.273073146784487</v>
+        <v>-0.2973600586653629</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.2525005054465128</v>
+        <v>-0.2117565641270217</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.2182334150423948</v>
+        <v>-0.1969378348363383</v>
       </c>
       <c r="I4" t="n">
-        <v>36.94937541091387</v>
+        <v>29.14321450906817</v>
       </c>
       <c r="J4" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="K4" t="n">
         <v>53.48</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M4" t="n">
         <v>53.48</v>
       </c>
       <c r="N4" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="O4" t="n">
-        <v>12.76595744680851</v>
+        <v>14.8936170212766</v>
       </c>
       <c r="P4" t="n">
-        <v>35.9451914893617</v>
+        <v>32.37072340425532</v>
       </c>
       <c r="Q4" t="b">
         <v>0</v>
@@ -974,48 +974,48 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>300.85</v>
+        <v>287.9</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.1081962353638654</v>
+        <v>-0.1528615565690747</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.1942956614890196</v>
+        <v>-0.222732181425486</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.2583507950203376</v>
+        <v>-0.3024833434282253</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.2377781536823634</v>
+        <v>-0.2168798488898841</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.2035110632782454</v>
+        <v>-0.2020611195992007</v>
       </c>
       <c r="I5" t="n">
-        <v>45.31704479348461</v>
+        <v>33.9393939393939</v>
       </c>
       <c r="J5" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K5" t="n">
         <v>51.12</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M5" t="n">
         <v>51.12</v>
       </c>
       <c r="N5" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O5" t="n">
-        <v>14.8936170212766</v>
+        <v>12.76595744680851</v>
       </c>
       <c r="P5" t="n">
-        <v>39.42672340425532</v>
+        <v>35.0011914893617</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
@@ -1039,48 +1039,48 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>109.38</v>
+        <v>105.08</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.179075352746923</v>
+        <v>-0.2234129037026088</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.0631263383297644</v>
+        <v>-0.0963192294461644</v>
       </c>
       <c r="F6" t="n">
-        <v>0.1596692111959288</v>
+        <v>0.1107822410147991</v>
       </c>
       <c r="G6" t="n">
-        <v>0.180241852533903</v>
+        <v>0.1963857355531404</v>
       </c>
       <c r="H6" t="n">
-        <v>0.214508942938021</v>
+        <v>0.2112044648438238</v>
       </c>
       <c r="I6" t="n">
-        <v>39.62855764592377</v>
+        <v>27.27498140342178</v>
       </c>
       <c r="J6" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="K6" t="n">
         <v>51.57</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M6" t="n">
         <v>51.57</v>
       </c>
       <c r="N6" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="O6" t="n">
         <v>85.1063829787234</v>
       </c>
       <c r="P6" t="n">
-        <v>49.64927659574468</v>
+        <v>45.64927659574468</v>
       </c>
       <c r="Q6" t="b">
         <v>0</v>
@@ -1104,25 +1104,25 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2566.3</v>
+        <v>2517.3</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.0200099285905218</v>
+        <v>-0.0746241223394478</v>
       </c>
       <c r="E7" t="n">
-        <v>-0.0335542667771333</v>
+        <v>-0.0420868373986833</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.143681804531349</v>
+        <v>-0.1582625560088275</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.1231091631933748</v>
+        <v>-0.0726590614704862</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.08884207278925681</v>
+        <v>-0.0578403321798028</v>
       </c>
       <c r="I7" t="n">
-        <v>47.43791641429439</v>
+        <v>42.44338498212158</v>
       </c>
       <c r="J7" t="n">
         <v>60</v>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M7" t="n">
@@ -1142,10 +1142,10 @@
         <v>60</v>
       </c>
       <c r="O7" t="n">
-        <v>36.17021276595745</v>
+        <v>44.68085106382978</v>
       </c>
       <c r="P7" t="n">
-        <v>50.7260425531915</v>
+        <v>52.42817021276596</v>
       </c>
       <c r="Q7" t="b">
         <v>0</v>
@@ -1169,25 +1169,25 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>488.75</v>
+        <v>481.5</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.0982472324723247</v>
+        <v>-0.1170807738149812</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0200354794949391</v>
+        <v>0.0211006255964372</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1159949765955017</v>
+        <v>0.0915892087961913</v>
       </c>
       <c r="G8" t="n">
-        <v>0.1365676179334759</v>
+        <v>0.1771927033345326</v>
       </c>
       <c r="H8" t="n">
-        <v>0.1708347083375939</v>
+        <v>0.192011432625216</v>
       </c>
       <c r="I8" t="n">
-        <v>46.33097942892233</v>
+        <v>40.49041182018234</v>
       </c>
       <c r="J8" t="n">
         <v>40</v>
@@ -1197,7 +1197,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M8" t="n">
@@ -1234,48 +1234,48 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>412.45</v>
+        <v>412.3</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.1096600107933082</v>
+        <v>-0.105348811977867</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.2137819290888296</v>
+        <v>-0.2082573211713874</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.1504634397528321</v>
+        <v>-0.146023198011599</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.1298907984148579</v>
+        <v>-0.0604197034732577</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.0956237080107399</v>
+        <v>-0.0456009741825743</v>
       </c>
       <c r="I9" t="n">
-        <v>42.37074401008826</v>
+        <v>38.6058981233244</v>
       </c>
       <c r="J9" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K9" t="n">
         <v>53.44</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M9" t="n">
         <v>53.44</v>
       </c>
       <c r="N9" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O9" t="n">
-        <v>34.04255319148936</v>
+        <v>48.93617021276596</v>
       </c>
       <c r="P9" t="n">
-        <v>44.18451063829788</v>
+        <v>43.1632340425532</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -1299,25 +1299,25 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>129575</v>
+        <v>128495</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.1220313717518718</v>
+        <v>-0.1046892419175028</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.1494633890183465</v>
+        <v>-0.1528267677600131</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.1341752697871772</v>
+        <v>-0.1323767724510466</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.1136026284492029</v>
+        <v>-0.0467732779127053</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.07933553804508491</v>
+        <v>-0.0319545486220219</v>
       </c>
       <c r="I10" t="n">
-        <v>39.9624765478424</v>
+        <v>32.67638943634213</v>
       </c>
       <c r="J10" t="n">
         <v>30</v>
@@ -1327,7 +1327,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M10" t="n">
@@ -1337,10 +1337,10 @@
         <v>30</v>
       </c>
       <c r="O10" t="n">
-        <v>40.42553191489361</v>
+        <v>51.06382978723404</v>
       </c>
       <c r="P10" t="n">
-        <v>39.84910638297872</v>
+        <v>41.97676595744681</v>
       </c>
       <c r="Q10" t="b">
         <v>0</v>
@@ -1376,10 +1376,10 @@
         <v>-0.0042030657656173</v>
       </c>
       <c r="G11" t="n">
-        <v>0.0163695755723568</v>
+        <v>0.0814004287727239</v>
       </c>
       <c r="H11" t="n">
-        <v>0.0506366659764748</v>
+        <v>0.09621915806340731</v>
       </c>
       <c r="I11" t="n">
         <v>27.6054590570719</v>
@@ -1392,7 +1392,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M11" t="n">
@@ -1402,10 +1402,10 @@
         <v>20</v>
       </c>
       <c r="O11" t="n">
-        <v>61.70212765957447</v>
+        <v>70.21276595744681</v>
       </c>
       <c r="P11" t="n">
-        <v>24.3404255319149</v>
+        <v>26.04255319148936</v>
       </c>
       <c r="Q11" t="b">
         <v>0</v>
@@ -1429,25 +1429,25 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>438.75</v>
+        <v>444.75</v>
       </c>
       <c r="D12" t="n">
-        <v>0.0277582572030921</v>
+        <v>0.0481970304030168</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.0647980390067142</v>
+        <v>-0.0331521739130434</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.15625</v>
+        <v>-0.1549496484894545</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.1356773586620258</v>
+        <v>-0.06934615395111331</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.1014102682579077</v>
+        <v>-0.0545274246604299</v>
       </c>
       <c r="I12" t="n">
-        <v>72.65353418308227</v>
+        <v>70.92402464065708</v>
       </c>
       <c r="J12" t="n">
         <v>70</v>
@@ -1457,7 +1457,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M12" t="n">
@@ -1467,10 +1467,10 @@
         <v>70</v>
       </c>
       <c r="O12" t="n">
-        <v>31.91489361702128</v>
+        <v>46.80851063829788</v>
       </c>
       <c r="P12" t="n">
-        <v>62.89497872340426</v>
+        <v>65.87370212765957</v>
       </c>
       <c r="Q12" t="b">
         <v>1</v>
@@ -1494,25 +1494,25 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1585.4</v>
+        <v>1547.1</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.2271242626627017</v>
+        <v>-0.23795685154172</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.1379010331702012</v>
+        <v>-0.1317207318442025</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.0852757904454188</v>
+        <v>-0.100157040656081</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.0647031491074446</v>
+        <v>-0.0145535461177397</v>
       </c>
       <c r="H13" t="n">
-        <v>-0.0304360587033266</v>
+        <v>0.0002651831729436</v>
       </c>
       <c r="I13" t="n">
-        <v>18.72846312887664</v>
+        <v>18.14388249040228</v>
       </c>
       <c r="J13" t="n">
         <v>20</v>
@@ -1522,7 +1522,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M13" t="n">
@@ -1541,7 +1541,7 @@
         <v>0</v>
       </c>
       <c r="R13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S13" t="b">
         <v>0</v>
@@ -1559,48 +1559,48 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>531.65</v>
+        <v>504.35</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.1689073002970142</v>
+        <v>-0.201029702970297</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.2702127659574468</v>
+        <v>-0.2905471936981291</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.1257913343747431</v>
+        <v>-0.1714309183505832</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.1052186930367689</v>
+        <v>-0.0858274238122419</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.0709516026326508</v>
+        <v>-0.0710086945215585</v>
       </c>
       <c r="I14" t="n">
-        <v>42.39795918367346</v>
+        <v>34.31717029749359</v>
       </c>
       <c r="J14" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K14" t="n">
         <v>54.64</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M14" t="n">
         <v>54.64</v>
       </c>
       <c r="N14" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O14" t="n">
-        <v>46.80851063829788</v>
+        <v>38.29787234042553</v>
       </c>
       <c r="P14" t="n">
-        <v>47.21770212765958</v>
+        <v>41.51557446808511</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
@@ -1624,48 +1624,48 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>89.41</v>
+        <v>86.22</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.1747277090640576</v>
+        <v>-0.2070265796008461</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.0652378463146891</v>
+        <v>-0.1849891294073165</v>
       </c>
       <c r="F15" t="n">
-        <v>0.0273468918763644</v>
+        <v>-0.012484251517581</v>
       </c>
       <c r="G15" t="n">
-        <v>0.0479195332143386</v>
+        <v>0.0731192430207602</v>
       </c>
       <c r="H15" t="n">
-        <v>0.08218662361845661</v>
+        <v>0.0879379723114436</v>
       </c>
       <c r="I15" t="n">
-        <v>41.1353032659409</v>
+        <v>27.45098039215688</v>
       </c>
       <c r="J15" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="K15" t="n">
         <v>51.91</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M15" t="n">
         <v>51.91</v>
       </c>
       <c r="N15" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="O15" t="n">
-        <v>72.3404255319149</v>
+        <v>68.08510638297872</v>
       </c>
       <c r="P15" t="n">
-        <v>51.23208510638297</v>
+        <v>42.38102127659575</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
@@ -1689,48 +1689,48 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>149.85</v>
+        <v>140.81</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.2340523410345532</v>
+        <v>-0.2751467105940491</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.1126835622927522</v>
+        <v>-0.1720468042570705</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.0820826952526799</v>
+        <v>-0.1217488929083765</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.0615100539147057</v>
+        <v>-0.0361453983700352</v>
       </c>
       <c r="H16" t="n">
-        <v>-0.0272429635105877</v>
+        <v>-0.0213266690793518</v>
       </c>
       <c r="I16" t="n">
-        <v>35.57985053971767</v>
+        <v>26.96097753251871</v>
       </c>
       <c r="J16" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="K16" t="n">
         <v>52.61</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M16" t="n">
         <v>52.61</v>
       </c>
       <c r="N16" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="O16" t="n">
-        <v>59.57446808510638</v>
+        <v>55.31914893617022</v>
       </c>
       <c r="P16" t="n">
-        <v>44.95889361702128</v>
+        <v>40.10782978723405</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>
@@ -1754,48 +1754,48 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>6924</v>
+        <v>6977</v>
       </c>
       <c r="D17" t="n">
-        <v>-0.1117382937780628</v>
+        <v>-0.1002643626281514</v>
       </c>
       <c r="E17" t="n">
-        <v>-0.0214810627473148</v>
+        <v>0.0007171543316122</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0129471143296027</v>
+        <v>0.0120394545982014</v>
       </c>
       <c r="G17" t="n">
-        <v>0.0335197556675769</v>
+        <v>0.0976429491365427</v>
       </c>
       <c r="H17" t="n">
-        <v>0.0677868460716949</v>
+        <v>0.1124616784272261</v>
       </c>
       <c r="I17" t="n">
-        <v>42.07197382769901</v>
+        <v>39.96383363471971</v>
       </c>
       <c r="J17" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K17" t="n">
         <v>54.65</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M17" t="n">
         <v>54.65</v>
       </c>
       <c r="N17" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O17" t="n">
-        <v>70.21276595744681</v>
+        <v>74.46808510638297</v>
       </c>
       <c r="P17" t="n">
-        <v>51.90255319148936</v>
+        <v>48.7536170212766</v>
       </c>
       <c r="Q17" t="b">
         <v>0</v>
@@ -1819,48 +1819,48 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>674.75</v>
+        <v>615.8</v>
       </c>
       <c r="D18" t="n">
-        <v>-0.059909439219784</v>
+        <v>-0.1860956912503305</v>
       </c>
       <c r="E18" t="n">
-        <v>0.1113398665898048</v>
+        <v>0.0378360158422514</v>
       </c>
       <c r="F18" t="n">
-        <v>-0.0029553010712966</v>
+        <v>-0.0836991295290529</v>
       </c>
       <c r="G18" t="n">
-        <v>0.0176173402666776</v>
+        <v>0.0019043650092883</v>
       </c>
       <c r="H18" t="n">
-        <v>0.0518844306707956</v>
+        <v>0.0167230942999717</v>
       </c>
       <c r="I18" t="n">
-        <v>40.25722339675829</v>
+        <v>29.6598430044636</v>
       </c>
       <c r="J18" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="K18" t="n">
         <v>49.92</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M18" t="n">
         <v>49.92</v>
       </c>
       <c r="N18" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="O18" t="n">
-        <v>65.95744680851064</v>
+        <v>59.57446808510638</v>
       </c>
       <c r="P18" t="n">
-        <v>57.15948936170213</v>
+        <v>39.88289361702128</v>
       </c>
       <c r="Q18" t="b">
         <v>0</v>
@@ -1884,48 +1884,48 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2260</v>
+        <v>2213.9</v>
       </c>
       <c r="D19" t="n">
-        <v>-0.1553927797294267</v>
+        <v>-0.1630500529260546</v>
       </c>
       <c r="E19" t="n">
-        <v>-0.1388835968755953</v>
+        <v>-0.138090788756521</v>
       </c>
       <c r="F19" t="n">
-        <v>-0.2295104322923769</v>
+        <v>-0.2540265516544241</v>
       </c>
       <c r="G19" t="n">
-        <v>-0.2089377909544026</v>
+        <v>-0.1684230571160828</v>
       </c>
       <c r="H19" t="n">
-        <v>-0.1746707005502846</v>
+        <v>-0.1536043278253994</v>
       </c>
       <c r="I19" t="n">
-        <v>36.59254414650099</v>
+        <v>28.77544320420225</v>
       </c>
       <c r="J19" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="K19" t="n">
         <v>51.27</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M19" t="n">
         <v>51.27</v>
       </c>
       <c r="N19" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="O19" t="n">
         <v>21.27659574468085</v>
       </c>
       <c r="P19" t="n">
-        <v>36.76331914893618</v>
+        <v>32.76331914893618</v>
       </c>
       <c r="Q19" t="b">
         <v>0</v>
@@ -1949,54 +1949,54 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>1966.1</v>
+        <v>1910.9</v>
       </c>
       <c r="D20" t="n">
-        <v>-0.1309287008796359</v>
+        <v>-0.1355740522934949</v>
       </c>
       <c r="E20" t="n">
-        <v>-0.1352860975502484</v>
+        <v>-0.1480606330806955</v>
       </c>
       <c r="F20" t="n">
-        <v>-0.0962952748667034</v>
+        <v>-0.064614029076313</v>
       </c>
       <c r="G20" t="n">
-        <v>-0.0757226335287292</v>
+        <v>0.0209894654620281</v>
       </c>
       <c r="H20" t="n">
-        <v>-0.0414555431246111</v>
+        <v>0.0358081947527115</v>
       </c>
       <c r="I20" t="n">
-        <v>45.03560392314927</v>
+        <v>33.63350485991995</v>
       </c>
       <c r="J20" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K20" t="n">
         <v>49.06</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M20" t="n">
         <v>49.06</v>
       </c>
       <c r="N20" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O20" t="n">
-        <v>53.19148936170212</v>
+        <v>61.70212765957447</v>
       </c>
       <c r="P20" t="n">
-        <v>46.26229787234043</v>
+        <v>43.9644255319149</v>
       </c>
       <c r="Q20" t="b">
         <v>0</v>
       </c>
       <c r="R20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S20" t="b">
         <v>0</v>
@@ -2014,48 +2014,48 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>823.1</v>
+        <v>826.35</v>
       </c>
       <c r="D21" t="n">
-        <v>-0.1863384737050217</v>
+        <v>-0.1824387830818699</v>
       </c>
       <c r="E21" t="n">
-        <v>-0.1568326162671584</v>
+        <v>-0.1344401382633288</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.3265423007691049</v>
+        <v>-0.3123491720063244</v>
       </c>
       <c r="G21" t="n">
-        <v>-0.3059696594311307</v>
+        <v>-0.2267456774679831</v>
       </c>
       <c r="H21" t="n">
-        <v>-0.2717025690270127</v>
+        <v>-0.2119269481772997</v>
       </c>
       <c r="I21" t="n">
-        <v>42.23293656772639</v>
+        <v>38.13135388091013</v>
       </c>
       <c r="J21" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K21" t="n">
         <v>48.43</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M21" t="n">
         <v>48.43</v>
       </c>
       <c r="N21" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O21" t="n">
-        <v>8.51063829787234</v>
+        <v>10.63829787234042</v>
       </c>
       <c r="P21" t="n">
-        <v>37.07412765957447</v>
+        <v>33.49965957446808</v>
       </c>
       <c r="Q21" t="b">
         <v>0</v>
@@ -2079,48 +2079,48 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>377.85</v>
+        <v>356.7</v>
       </c>
       <c r="D22" t="n">
-        <v>-0.1040901007705986</v>
+        <v>-0.1540377090003557</v>
       </c>
       <c r="E22" t="n">
-        <v>0.2341989220970115</v>
+        <v>0.1714285714285714</v>
       </c>
       <c r="F22" t="n">
-        <v>0.2218270008084075</v>
+        <v>0.1581168831168831</v>
       </c>
       <c r="G22" t="n">
-        <v>0.2423996421463817</v>
+        <v>0.2437203776552243</v>
       </c>
       <c r="H22" t="n">
-        <v>0.2766667325504998</v>
+        <v>0.2585391069459077</v>
       </c>
       <c r="I22" t="n">
-        <v>33.32275468105364</v>
+        <v>29.85499004833665</v>
       </c>
       <c r="J22" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="K22" t="n">
         <v>54.47</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M22" t="n">
         <v>54.47</v>
       </c>
       <c r="N22" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="O22" t="n">
-        <v>91.48936170212764</v>
+        <v>89.36170212765957</v>
       </c>
       <c r="P22" t="n">
-        <v>52.08587234042552</v>
+        <v>47.66034042553191</v>
       </c>
       <c r="Q22" t="b">
         <v>0</v>
@@ -2144,25 +2144,25 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>322.35</v>
+        <v>314.25</v>
       </c>
       <c r="D23" t="n">
-        <v>-0.1374096869146372</v>
+        <v>-0.1529649595687331</v>
       </c>
       <c r="E23" t="n">
-        <v>-0.1297246220302375</v>
+        <v>-0.1369129360065916</v>
       </c>
       <c r="F23" t="n">
-        <v>-0.2039757994814174</v>
+        <v>-0.220899962811454</v>
       </c>
       <c r="G23" t="n">
-        <v>-0.1834031581434432</v>
+        <v>-0.1352964682731128</v>
       </c>
       <c r="H23" t="n">
-        <v>-0.1491360677393252</v>
+        <v>-0.1204777389824294</v>
       </c>
       <c r="I23" t="n">
-        <v>23.52941176470587</v>
+        <v>18.96678966789663</v>
       </c>
       <c r="J23" t="n">
         <v>20</v>
@@ -2172,7 +2172,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M23" t="n">
@@ -2182,10 +2182,10 @@
         <v>20</v>
       </c>
       <c r="O23" t="n">
-        <v>23.40425531914894</v>
+        <v>29.78723404255319</v>
       </c>
       <c r="P23" t="n">
-        <v>32.56085106382979</v>
+        <v>33.83744680851064</v>
       </c>
       <c r="Q23" t="b">
         <v>0</v>
@@ -2209,48 +2209,48 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>116.62</v>
+        <v>111.92</v>
       </c>
       <c r="D24" t="n">
-        <v>-0.1895197720480922</v>
+        <v>-0.2450590219224283</v>
       </c>
       <c r="E24" t="n">
-        <v>-0.0477668000326609</v>
+        <v>-0.0872614581634317</v>
       </c>
       <c r="F24" t="n">
-        <v>0.0995662832359043</v>
+        <v>0.0388935301216002</v>
       </c>
       <c r="G24" t="n">
-        <v>0.1201389245738785</v>
+        <v>0.1244970246599415</v>
       </c>
       <c r="H24" t="n">
-        <v>0.1544060149779965</v>
+        <v>0.1393157539506249</v>
       </c>
       <c r="I24" t="n">
-        <v>44.2432872253865</v>
+        <v>35.49618320610686</v>
       </c>
       <c r="J24" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K24" t="n">
         <v>48.3</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M24" t="n">
         <v>48.3</v>
       </c>
       <c r="N24" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O24" t="n">
-        <v>80.85106382978722</v>
+        <v>78.72340425531915</v>
       </c>
       <c r="P24" t="n">
-        <v>51.49021276595744</v>
+        <v>47.06468085106384</v>
       </c>
       <c r="Q24" t="b">
         <v>0</v>
@@ -2274,48 +2274,48 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>546.65</v>
+        <v>515.25</v>
       </c>
       <c r="D25" t="n">
-        <v>-0.0176116452511457</v>
+        <v>-0.0810593900481542</v>
       </c>
       <c r="E25" t="n">
-        <v>-0.0434820647419073</v>
+        <v>-0.0777698228029354</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.09860664523043949</v>
+        <v>-0.1602835723598435</v>
       </c>
       <c r="G25" t="n">
-        <v>-0.0780340038924652</v>
+        <v>-0.07468007782150229</v>
       </c>
       <c r="H25" t="n">
-        <v>-0.0437669134883472</v>
+        <v>-0.0598613485308189</v>
       </c>
       <c r="I25" t="n">
-        <v>56.43496214728149</v>
+        <v>48.86731391585761</v>
       </c>
       <c r="J25" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="K25" t="n">
         <v>56.91</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M25" t="n">
         <v>56.91</v>
       </c>
       <c r="N25" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="O25" t="n">
-        <v>51.06382978723404</v>
+        <v>42.5531914893617</v>
       </c>
       <c r="P25" t="n">
-        <v>56.9767659574468</v>
+        <v>47.27463829787234</v>
       </c>
       <c r="Q25" t="b">
         <v>0</v>
@@ -2339,48 +2339,48 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>120.82</v>
+        <v>117.55</v>
       </c>
       <c r="D26" t="n">
-        <v>-0.1401323749199344</v>
+        <v>-0.1683175321918777</v>
       </c>
       <c r="E26" t="n">
-        <v>-0.1724090691143229</v>
+        <v>-0.1842470506592644</v>
       </c>
       <c r="F26" t="n">
-        <v>-0.157696597880647</v>
+        <v>-0.2612957958901527</v>
       </c>
       <c r="G26" t="n">
-        <v>-0.1371239565426728</v>
+        <v>-0.1756923013518114</v>
       </c>
       <c r="H26" t="n">
-        <v>-0.1028568661385548</v>
+        <v>-0.160873572061128</v>
       </c>
       <c r="I26" t="n">
-        <v>39.0909090909091</v>
+        <v>28.11407048695187</v>
       </c>
       <c r="J26" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="K26" t="n">
         <v>51.54</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M26" t="n">
         <v>51.54</v>
       </c>
       <c r="N26" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="O26" t="n">
-        <v>29.78723404255319</v>
+        <v>17.02127659574468</v>
       </c>
       <c r="P26" t="n">
-        <v>38.57344680851064</v>
+        <v>32.02025531914894</v>
       </c>
       <c r="Q26" t="b">
         <v>0</v>
@@ -2404,48 +2404,48 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>4880</v>
+        <v>4654</v>
       </c>
       <c r="D27" t="n">
-        <v>-0.214752357352042</v>
+        <v>-0.2341489904392041</v>
       </c>
       <c r="E27" t="n">
-        <v>-0.152041702867072</v>
+        <v>-0.1699661137863385</v>
       </c>
       <c r="F27" t="n">
-        <v>0.1645110485372021</v>
+        <v>0.1235032831208962</v>
       </c>
       <c r="G27" t="n">
-        <v>0.1850836898751763</v>
+        <v>0.2091067776592374</v>
       </c>
       <c r="H27" t="n">
-        <v>0.2193507802792943</v>
+        <v>0.2239255069499208</v>
       </c>
       <c r="I27" t="n">
-        <v>42.24175824175824</v>
+        <v>39.25653594771242</v>
       </c>
       <c r="J27" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K27" t="n">
         <v>57.69</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M27" t="n">
         <v>57.69</v>
       </c>
       <c r="N27" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O27" t="n">
         <v>87.2340425531915</v>
       </c>
       <c r="P27" t="n">
-        <v>56.5228085106383</v>
+        <v>52.5228085106383</v>
       </c>
       <c r="Q27" t="b">
         <v>0</v>
@@ -2469,48 +2469,48 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1608.8</v>
+        <v>1522.2</v>
       </c>
       <c r="D28" t="n">
-        <v>-0.064107038976149</v>
+        <v>-0.1292758265644663</v>
       </c>
       <c r="E28" t="n">
-        <v>0.0642323212277566</v>
+        <v>0.0291393414914475</v>
       </c>
       <c r="F28" t="n">
-        <v>0.5187387897668272</v>
+        <v>0.4243473378871525</v>
       </c>
       <c r="G28" t="n">
-        <v>0.5393114311048014</v>
+        <v>0.5099508324254938</v>
       </c>
       <c r="H28" t="n">
-        <v>0.5735785215089194</v>
+        <v>0.5247695617161772</v>
       </c>
       <c r="I28" t="n">
-        <v>59.15453915453915</v>
+        <v>51.17172493276988</v>
       </c>
       <c r="J28" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="K28" t="n">
         <v>54.51</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M28" t="n">
         <v>54.51</v>
       </c>
       <c r="N28" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="O28" t="n">
         <v>95.74468085106383</v>
       </c>
       <c r="P28" t="n">
-        <v>72.95293617021277</v>
+        <v>56.95293617021277</v>
       </c>
       <c r="Q28" t="b">
         <v>0</v>
@@ -2534,48 +2534,48 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>528.7</v>
+        <v>505.65</v>
       </c>
       <c r="D29" t="n">
-        <v>-0.0871104204437536</v>
+        <v>-0.1166914140973012</v>
       </c>
       <c r="E29" t="n">
-        <v>-0.090643274853801</v>
+        <v>-0.1371160409556314</v>
       </c>
       <c r="F29" t="n">
-        <v>0.0521393034825872</v>
+        <v>0.0032738095238094</v>
       </c>
       <c r="G29" t="n">
-        <v>0.0727119448205614</v>
+        <v>0.08887730406215059</v>
       </c>
       <c r="H29" t="n">
-        <v>0.1069790352246794</v>
+        <v>0.103696033352834</v>
       </c>
       <c r="I29" t="n">
-        <v>60.57201225740555</v>
+        <v>49.5638629283489</v>
       </c>
       <c r="J29" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="K29" t="n">
         <v>49.42</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M29" t="n">
         <v>49.42</v>
       </c>
       <c r="N29" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="O29" t="n">
-        <v>78.72340425531915</v>
+        <v>72.3404255319149</v>
       </c>
       <c r="P29" t="n">
-        <v>59.51268085106384</v>
+        <v>50.23608510638298</v>
       </c>
       <c r="Q29" t="b">
         <v>0</v>
@@ -2599,48 +2599,48 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>109.22</v>
+        <v>102.65</v>
       </c>
       <c r="D30" t="n">
-        <v>-0.0545360110803323</v>
+        <v>-0.1111014894354001</v>
       </c>
       <c r="E30" t="n">
-        <v>0.0213203665606882</v>
+        <v>-0.041370937616735</v>
       </c>
       <c r="F30" t="n">
-        <v>-0.1213900732040865</v>
+        <v>-0.1795875959079284</v>
       </c>
       <c r="G30" t="n">
-        <v>-0.1008174318661123</v>
+        <v>-0.0939841013695871</v>
       </c>
       <c r="H30" t="n">
-        <v>-0.0665503414619943</v>
+        <v>-0.0791653720789037</v>
       </c>
       <c r="I30" t="n">
-        <v>40.5096203848154</v>
+        <v>28.93339768339769</v>
       </c>
       <c r="J30" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="K30" t="n">
         <v>52.38</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M30" t="n">
         <v>52.38</v>
       </c>
       <c r="N30" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="O30" t="n">
-        <v>48.93617021276596</v>
+        <v>36.17021276595745</v>
       </c>
       <c r="P30" t="n">
-        <v>46.73923404255319</v>
+        <v>36.18604255319149</v>
       </c>
       <c r="Q30" t="b">
         <v>0</v>
@@ -2664,48 +2664,48 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>37.9</v>
+        <v>36.9</v>
       </c>
       <c r="D31" t="n">
-        <v>-0.1301354142758779</v>
+        <v>-0.1400605919366114</v>
       </c>
       <c r="E31" t="n">
-        <v>-0.153072625698324</v>
+        <v>-0.1709728150977308</v>
       </c>
       <c r="F31" t="n">
-        <v>-0.1415628539071347</v>
+        <v>-0.1830861191056011</v>
       </c>
       <c r="G31" t="n">
-        <v>-0.1209902125691605</v>
+        <v>-0.0974826245672598</v>
       </c>
       <c r="H31" t="n">
-        <v>-0.08672312216504249</v>
+        <v>-0.0826638952765764</v>
       </c>
       <c r="I31" t="n">
-        <v>35.9848484848485</v>
+        <v>26.86746987951804</v>
       </c>
       <c r="J31" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="K31" t="n">
         <v>48.99</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M31" t="n">
         <v>48.99</v>
       </c>
       <c r="N31" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="O31" t="n">
-        <v>38.29787234042553</v>
+        <v>34.04255319148936</v>
       </c>
       <c r="P31" t="n">
-        <v>39.25557446808512</v>
+        <v>34.40451063829788</v>
       </c>
       <c r="Q31" t="b">
         <v>0</v>
@@ -2729,48 +2729,48 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>652.9</v>
+        <v>610.8</v>
       </c>
       <c r="D32" t="n">
-        <v>-0.1403554970375247</v>
+        <v>-0.2010986855012753</v>
       </c>
       <c r="E32" t="n">
-        <v>-0.2071645415907711</v>
+        <v>-0.2512411890897947</v>
       </c>
       <c r="F32" t="n">
-        <v>-0.3728146013448608</v>
+        <v>-0.455469376838727</v>
       </c>
       <c r="G32" t="n">
-        <v>-0.3522419600068865</v>
+        <v>-0.3698658823003857</v>
       </c>
       <c r="H32" t="n">
-        <v>-0.3179748696027685</v>
+        <v>-0.3550471530097023</v>
       </c>
       <c r="I32" t="n">
-        <v>44.20951465641519</v>
+        <v>32.94573643410853</v>
       </c>
       <c r="J32" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K32" t="n">
         <v>47.86</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M32" t="n">
         <v>47.86</v>
       </c>
       <c r="N32" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O32" t="n">
         <v>2.127659574468085</v>
       </c>
       <c r="P32" t="n">
-        <v>35.56953191489362</v>
+        <v>31.56953191489362</v>
       </c>
       <c r="Q32" t="b">
         <v>0</v>
@@ -2794,48 +2794,48 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>525.3</v>
+        <v>513.9</v>
       </c>
       <c r="D33" t="n">
-        <v>-0.1585776069197501</v>
+        <v>-0.1680427391937835</v>
       </c>
       <c r="E33" t="n">
-        <v>-0.1609966459032105</v>
+        <v>-0.1588509698011294</v>
       </c>
       <c r="F33" t="n">
-        <v>0.0501799280287884</v>
+        <v>0.0446183555239352</v>
       </c>
       <c r="G33" t="n">
-        <v>0.07075256936676259</v>
+        <v>0.1302218500622765</v>
       </c>
       <c r="H33" t="n">
-        <v>0.1050196597708806</v>
+        <v>0.1450405793529599</v>
       </c>
       <c r="I33" t="n">
-        <v>44.67965001411233</v>
+        <v>36.24708624708624</v>
       </c>
       <c r="J33" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K33" t="n">
         <v>49.98</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M33" t="n">
         <v>49.98</v>
       </c>
       <c r="N33" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O33" t="n">
-        <v>76.59574468085107</v>
+        <v>80.85106382978722</v>
       </c>
       <c r="P33" t="n">
-        <v>51.31114893617022</v>
+        <v>48.16221276595745</v>
       </c>
       <c r="Q33" t="b">
         <v>0</v>
@@ -2871,10 +2871,10 @@
         <v>-0.2401052253975846</v>
       </c>
       <c r="G34" t="n">
-        <v>-0.2195325840596104</v>
+        <v>-0.1545017308592433</v>
       </c>
       <c r="H34" t="n">
-        <v>-0.1852654936554923</v>
+        <v>-0.1396830015685599</v>
       </c>
       <c r="I34" t="n">
         <v>63.3225806451613</v>
@@ -2887,7 +2887,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M34" t="n">
@@ -2897,10 +2897,10 @@
         <v>80</v>
       </c>
       <c r="O34" t="n">
-        <v>19.14893617021277</v>
+        <v>25.53191489361702</v>
       </c>
       <c r="P34" t="n">
-        <v>56.18178723404256</v>
+        <v>57.45838297872341</v>
       </c>
       <c r="Q34" t="b">
         <v>0</v>
@@ -2924,48 +2924,48 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>105.08</v>
+        <v>100.49</v>
       </c>
       <c r="D35" t="n">
-        <v>-0.1788058768365114</v>
+        <v>-0.2342452183189819</v>
       </c>
       <c r="E35" t="n">
-        <v>0.0136008488473038</v>
+        <v>-0.0049509852460639</v>
       </c>
       <c r="F35" t="n">
-        <v>0.0489119584747452</v>
+        <v>-0.012771392081737</v>
       </c>
       <c r="G35" t="n">
-        <v>0.0694845998127194</v>
+        <v>0.07283210245660419</v>
       </c>
       <c r="H35" t="n">
-        <v>0.1037516902168375</v>
+        <v>0.08765083174728761</v>
       </c>
       <c r="I35" t="n">
-        <v>49.75092051115443</v>
+        <v>37.08399366085577</v>
       </c>
       <c r="J35" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K35" t="n">
         <v>49.07</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M35" t="n">
         <v>49.07</v>
       </c>
       <c r="N35" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O35" t="n">
-        <v>74.46808510638297</v>
+        <v>65.95744680851064</v>
       </c>
       <c r="P35" t="n">
-        <v>50.5216170212766</v>
+        <v>44.81948936170213</v>
       </c>
       <c r="Q35" t="b">
         <v>0</v>
@@ -2989,48 +2989,48 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>462.7</v>
+        <v>437</v>
       </c>
       <c r="D36" t="n">
-        <v>-0.0722807017543859</v>
+        <v>-0.1254752851711026</v>
       </c>
       <c r="E36" t="n">
-        <v>-0.1741923969302159</v>
+        <v>-0.1989000916590284</v>
       </c>
       <c r="F36" t="n">
-        <v>0.0011900897976848</v>
+        <v>-0.0486557091542397</v>
       </c>
       <c r="G36" t="n">
-        <v>0.021762731135659</v>
+        <v>0.0369477853841014</v>
       </c>
       <c r="H36" t="n">
-        <v>0.056029821539777</v>
+        <v>0.0517665146747848</v>
       </c>
       <c r="I36" t="n">
-        <v>34.98635122838944</v>
+        <v>24.3380062305296</v>
       </c>
       <c r="J36" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="K36" t="n">
         <v>47.8</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M36" t="n">
         <v>47.8</v>
       </c>
       <c r="N36" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="O36" t="n">
-        <v>68.08510638297872</v>
+        <v>63.82978723404256</v>
       </c>
       <c r="P36" t="n">
-        <v>44.73702127659575</v>
+        <v>39.88595744680851</v>
       </c>
       <c r="Q36" t="b">
         <v>0</v>
@@ -3054,48 +3054,48 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2159.2</v>
+        <v>2074.5</v>
       </c>
       <c r="D37" t="n">
-        <v>-0.0825189088127815</v>
+        <v>-0.09370904325032769</v>
       </c>
       <c r="E37" t="n">
-        <v>0.2840915848944394</v>
+        <v>0.2601749483659337</v>
       </c>
       <c r="F37" t="n">
-        <v>0.6443530576498362</v>
+        <v>0.5212290093128986</v>
       </c>
       <c r="G37" t="n">
-        <v>0.6649256989878104</v>
+        <v>0.6068325038512399</v>
       </c>
       <c r="H37" t="n">
-        <v>0.6991927893919284</v>
+        <v>0.6216512331419233</v>
       </c>
       <c r="I37" t="n">
-        <v>53.22580645161288</v>
+        <v>44.29001140960482</v>
       </c>
       <c r="J37" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K37" t="n">
         <v>48.59</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M37" t="n">
         <v>48.59</v>
       </c>
       <c r="N37" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O37" t="n">
         <v>100</v>
       </c>
       <c r="P37" t="n">
-        <v>71.43600000000001</v>
+        <v>63.43600000000001</v>
       </c>
       <c r="Q37" t="b">
         <v>0</v>
@@ -3119,48 +3119,48 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>757.1</v>
+        <v>708</v>
       </c>
       <c r="D38" t="n">
-        <v>-0.2093363270847474</v>
+        <v>-0.2565758387147582</v>
       </c>
       <c r="E38" t="n">
-        <v>-0.2153184432813391</v>
+        <v>-0.2639950101356619</v>
       </c>
       <c r="F38" t="n">
-        <v>-0.2846749811035526</v>
+        <v>-0.3304964539007092</v>
       </c>
       <c r="G38" t="n">
-        <v>-0.2641023397655784</v>
+        <v>-0.244892959362368</v>
       </c>
       <c r="H38" t="n">
-        <v>-0.2298352493614603</v>
+        <v>-0.2300742300716846</v>
       </c>
       <c r="I38" t="n">
-        <v>41.20516047828823</v>
+        <v>32.34408602150538</v>
       </c>
       <c r="J38" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K38" t="n">
         <v>49.87</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M38" t="n">
         <v>49.87</v>
       </c>
       <c r="N38" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O38" t="n">
-        <v>10.63829787234042</v>
+        <v>8.51063829787234</v>
       </c>
       <c r="P38" t="n">
-        <v>38.07565957446808</v>
+        <v>33.65012765957447</v>
       </c>
       <c r="Q38" t="b">
         <v>0</v>
@@ -3184,25 +3184,25 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>3033.5</v>
+        <v>3016.5</v>
       </c>
       <c r="D39" t="n">
-        <v>-0.0419114395805697</v>
+        <v>-0.0412852784134248</v>
       </c>
       <c r="E39" t="n">
-        <v>-0.0298698391378042</v>
+        <v>-0.0407975069956754</v>
       </c>
       <c r="F39" t="n">
-        <v>0.1788365134263396</v>
+        <v>0.1704563091727458</v>
       </c>
       <c r="G39" t="n">
-        <v>0.1994091547643138</v>
+        <v>0.256059803711087</v>
       </c>
       <c r="H39" t="n">
-        <v>0.2336762451684318</v>
+        <v>0.2708785330017704</v>
       </c>
       <c r="I39" t="n">
-        <v>58.48653596765581</v>
+        <v>49.47330512289548</v>
       </c>
       <c r="J39" t="n">
         <v>80</v>
@@ -3212,7 +3212,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M39" t="n">
@@ -3222,10 +3222,10 @@
         <v>80</v>
       </c>
       <c r="O39" t="n">
-        <v>89.36170212765957</v>
+        <v>91.48936170212764</v>
       </c>
       <c r="P39" t="n">
-        <v>69.34834042553192</v>
+        <v>69.77387234042553</v>
       </c>
       <c r="Q39" t="b">
         <v>0</v>
@@ -3249,48 +3249,48 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>178.97</v>
+        <v>170.43</v>
       </c>
       <c r="D40" t="n">
-        <v>-0.1683936620045537</v>
+        <v>-0.2010968921389396</v>
       </c>
       <c r="E40" t="n">
-        <v>-0.0308133867648651</v>
+        <v>-0.0822294022617123</v>
       </c>
       <c r="F40" t="n">
-        <v>-0.2002770454443898</v>
+        <v>-0.24263431542461</v>
       </c>
       <c r="G40" t="n">
-        <v>-0.1797044041064156</v>
+        <v>-0.1570308208862687</v>
       </c>
       <c r="H40" t="n">
-        <v>-0.1454373137022976</v>
+        <v>-0.1422120915955853</v>
       </c>
       <c r="I40" t="n">
-        <v>43.10897435897437</v>
+        <v>33.58467802744686</v>
       </c>
       <c r="J40" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K40" t="n">
         <v>45.44</v>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M40" t="n">
         <v>45.44</v>
       </c>
       <c r="N40" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O40" t="n">
-        <v>25.53191489361702</v>
+        <v>23.40425531914894</v>
       </c>
       <c r="P40" t="n">
-        <v>39.2823829787234</v>
+        <v>34.85685106382979</v>
       </c>
       <c r="Q40" t="b">
         <v>0</v>
@@ -3314,25 +3314,25 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>762.65</v>
+        <v>749.05</v>
       </c>
       <c r="D41" t="n">
-        <v>-0.1622913005272407</v>
+        <v>-0.1764608872519377</v>
       </c>
       <c r="E41" t="n">
-        <v>-0.1883680093651891</v>
+        <v>-0.2013115103694621</v>
       </c>
       <c r="F41" t="n">
-        <v>-0.2498770532113702</v>
+        <v>-0.2612919132149902</v>
       </c>
       <c r="G41" t="n">
-        <v>-0.229304411873396</v>
+        <v>-0.1756884186766489</v>
       </c>
       <c r="H41" t="n">
-        <v>-0.195037321469278</v>
+        <v>-0.1608696893859655</v>
       </c>
       <c r="I41" t="n">
-        <v>23.986975397974</v>
+        <v>16.82439537329127</v>
       </c>
       <c r="J41" t="n">
         <v>20</v>
@@ -3342,7 +3342,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M41" t="n">
@@ -3352,10 +3352,10 @@
         <v>20</v>
       </c>
       <c r="O41" t="n">
-        <v>17.02127659574468</v>
+        <v>19.14893617021277</v>
       </c>
       <c r="P41" t="n">
-        <v>30.62425531914894</v>
+        <v>31.04978723404255</v>
       </c>
       <c r="Q41" t="b">
         <v>0</v>
@@ -3379,48 +3379,48 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>496</v>
+        <v>465.05</v>
       </c>
       <c r="D42" t="n">
-        <v>-0.2457994373907093</v>
+        <v>-0.2665404936519201</v>
       </c>
       <c r="E42" t="n">
-        <v>-0.2622341216718726</v>
+        <v>-0.3102195194304361</v>
       </c>
       <c r="F42" t="n">
-        <v>-0.3624678663239075</v>
+        <v>-0.396822308690013</v>
       </c>
       <c r="G42" t="n">
-        <v>-0.3418952249859333</v>
+        <v>-0.3112188141516717</v>
       </c>
       <c r="H42" t="n">
-        <v>-0.3076281345818152</v>
+        <v>-0.2964000848609883</v>
       </c>
       <c r="I42" t="n">
-        <v>33.40896199659673</v>
+        <v>21.0904255319149</v>
       </c>
       <c r="J42" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="K42" t="n">
         <v>47.66</v>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M42" t="n">
         <v>47.66</v>
       </c>
       <c r="N42" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="O42" t="n">
-        <v>4.25531914893617</v>
+        <v>6.382978723404255</v>
       </c>
       <c r="P42" t="n">
-        <v>31.91506382978724</v>
+        <v>28.34059574468085</v>
       </c>
       <c r="Q42" t="b">
         <v>0</v>
@@ -3444,48 +3444,48 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>414.45</v>
+        <v>400.1</v>
       </c>
       <c r="D43" t="n">
-        <v>-0.07694877505567931</v>
+        <v>-0.0895437478666514</v>
       </c>
       <c r="E43" t="n">
-        <v>-0.09725549989109129</v>
+        <v>-0.1194982394366196</v>
       </c>
       <c r="F43" t="n">
-        <v>-0.0862087972660126</v>
+        <v>-0.1314446977097578</v>
       </c>
       <c r="G43" t="n">
-        <v>-0.0656361559280384</v>
+        <v>-0.0458412031714166</v>
       </c>
       <c r="H43" t="n">
-        <v>-0.0313690655239203</v>
+        <v>-0.0310224738807332</v>
       </c>
       <c r="I43" t="n">
-        <v>51.39171758316361</v>
+        <v>37.07653701380177</v>
       </c>
       <c r="J43" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="K43" t="n">
         <v>51.48</v>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M43" t="n">
         <v>51.48</v>
       </c>
       <c r="N43" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="O43" t="n">
-        <v>55.31914893617022</v>
+        <v>53.19148936170212</v>
       </c>
       <c r="P43" t="n">
-        <v>55.65582978723404</v>
+        <v>43.23029787234042</v>
       </c>
       <c r="Q43" t="b">
         <v>0</v>
@@ -3509,25 +3509,25 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>233</v>
+        <v>231.8</v>
       </c>
       <c r="D44" t="n">
-        <v>-0.1243893273205563</v>
+        <v>-0.1117072236060546</v>
       </c>
       <c r="E44" t="n">
-        <v>-0.1712608927618708</v>
+        <v>-0.1733238231098429</v>
       </c>
       <c r="F44" t="n">
-        <v>-0.1309212980231258</v>
+        <v>-0.1634788884879104</v>
       </c>
       <c r="G44" t="n">
-        <v>-0.1103486566851515</v>
+        <v>-0.0778753939495692</v>
       </c>
       <c r="H44" t="n">
-        <v>-0.07608156628103351</v>
+        <v>-0.06305666465888581</v>
       </c>
       <c r="I44" t="n">
-        <v>43.38358458961473</v>
+        <v>41.42212189616253</v>
       </c>
       <c r="J44" t="n">
         <v>40</v>
@@ -3537,7 +3537,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M44" t="n">
@@ -3547,10 +3547,10 @@
         <v>40</v>
       </c>
       <c r="O44" t="n">
-        <v>44.68085106382978</v>
+        <v>40.42553191489361</v>
       </c>
       <c r="P44" t="n">
-        <v>43.81617021276596</v>
+        <v>42.96510638297872</v>
       </c>
       <c r="Q44" t="b">
         <v>0</v>
@@ -3574,25 +3574,25 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>86.55</v>
+        <v>80.68000000000001</v>
       </c>
       <c r="D45" t="n">
-        <v>-0.2008310249307479</v>
+        <v>-0.2593408611034609</v>
       </c>
       <c r="E45" t="n">
-        <v>-0.2118921872154434</v>
+        <v>-0.285954509248606</v>
       </c>
       <c r="F45" t="n">
-        <v>-0.3525099124710107</v>
+        <v>-0.4100614214682655</v>
       </c>
       <c r="G45" t="n">
-        <v>-0.3319372711330365</v>
+        <v>-0.3244579269299242</v>
       </c>
       <c r="H45" t="n">
-        <v>-0.2976701807289185</v>
+        <v>-0.3096391976392408</v>
       </c>
       <c r="I45" t="n">
-        <v>26.31389488840891</v>
+        <v>20.61482820976488</v>
       </c>
       <c r="J45" t="n">
         <v>20</v>
@@ -3602,7 +3602,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M45" t="n">
@@ -3612,10 +3612,10 @@
         <v>20</v>
       </c>
       <c r="O45" t="n">
-        <v>6.382978723404255</v>
+        <v>4.25531914893617</v>
       </c>
       <c r="P45" t="n">
-        <v>33.11659574468086</v>
+        <v>32.69106382978724</v>
       </c>
       <c r="Q45" t="b">
         <v>0</v>
@@ -3639,25 +3639,25 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>487.6</v>
+        <v>467.4</v>
       </c>
       <c r="D46" t="n">
-        <v>-0.1153846153846154</v>
+        <v>-0.1497180280152812</v>
       </c>
       <c r="E46" t="n">
-        <v>-0.2353771365846009</v>
+        <v>-0.2607354685646501</v>
       </c>
       <c r="F46" t="n">
-        <v>-0.1309926929246123</v>
+        <v>-0.2237169905331341</v>
       </c>
       <c r="G46" t="n">
-        <v>-0.1104200515866381</v>
+        <v>-0.1381134959947928</v>
       </c>
       <c r="H46" t="n">
-        <v>-0.0761529611825201</v>
+        <v>-0.1232947667041094</v>
       </c>
       <c r="I46" t="n">
-        <v>51.3337670787248</v>
+        <v>40.42019441831294</v>
       </c>
       <c r="J46" t="n">
         <v>40</v>
@@ -3667,7 +3667,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M46" t="n">
@@ -3677,10 +3677,10 @@
         <v>40</v>
       </c>
       <c r="O46" t="n">
-        <v>42.5531914893617</v>
+        <v>27.65957446808511</v>
       </c>
       <c r="P46" t="n">
-        <v>44.35463829787234</v>
+        <v>41.37591489361702</v>
       </c>
       <c r="Q46" t="b">
         <v>0</v>
@@ -3704,48 +3704,48 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>1082.1</v>
+        <v>997.25</v>
       </c>
       <c r="D47" t="n">
-        <v>0.2112833715788882</v>
+        <v>0.1026037923599978</v>
       </c>
       <c r="E47" t="n">
-        <v>0.3170642648490749</v>
+        <v>0.1977540235407158</v>
       </c>
       <c r="F47" t="n">
-        <v>0.4677517802644964</v>
+        <v>0.3620842723485624</v>
       </c>
       <c r="G47" t="n">
-        <v>0.4883244216024706</v>
+        <v>0.4476877668869037</v>
       </c>
       <c r="H47" t="n">
-        <v>0.5225915120065886</v>
+        <v>0.4625064961775871</v>
       </c>
       <c r="I47" t="n">
-        <v>73.51181999430361</v>
+        <v>58.16770551570036</v>
       </c>
       <c r="J47" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K47" t="n">
         <v>46.83</v>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M47" t="n">
         <v>46.83</v>
       </c>
       <c r="N47" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O47" t="n">
         <v>93.61702127659576</v>
       </c>
       <c r="P47" t="n">
-        <v>65.45540425531915</v>
+        <v>69.45540425531915</v>
       </c>
       <c r="Q47" t="b">
         <v>0</v>
@@ -3769,25 +3769,25 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>13678</v>
+        <v>13768</v>
       </c>
       <c r="D48" t="n">
-        <v>-0.1184583655581335</v>
+        <v>-0.1120856442667355</v>
       </c>
       <c r="E48" t="n">
-        <v>-0.0502048468856329</v>
+        <v>-0.0412923891093934</v>
       </c>
       <c r="F48" t="n">
-        <v>-0.0031338823700896</v>
+        <v>0.0181172816682688</v>
       </c>
       <c r="G48" t="n">
-        <v>0.0174387589678846</v>
+        <v>0.1037207762066101</v>
       </c>
       <c r="H48" t="n">
-        <v>0.0517058493720026</v>
+        <v>0.1185395054972935</v>
       </c>
       <c r="I48" t="n">
-        <v>43.48521183053557</v>
+        <v>45.60588463027487</v>
       </c>
       <c r="J48" t="n">
         <v>40</v>
@@ -3797,7 +3797,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M48" t="n">
@@ -3807,10 +3807,10 @@
         <v>40</v>
       </c>
       <c r="O48" t="n">
-        <v>63.82978723404256</v>
+        <v>76.59574468085107</v>
       </c>
       <c r="P48" t="n">
-        <v>48.88195744680851</v>
+        <v>51.43514893617021</v>
       </c>
       <c r="Q48" t="b">
         <v>0</v>
@@ -3936,57 +3936,57 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>LUMAXTECH</t>
+          <t>SHRIPISTON</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Lighting</t>
+          <t>Engine/Parts</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1608.8</v>
+        <v>3016.5</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.064107038976149</v>
+        <v>-0.0412852784134248</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0642323212277566</v>
+        <v>-0.0407975069956754</v>
       </c>
       <c r="F2" t="n">
-        <v>0.5187387897668272</v>
+        <v>0.1704563091727458</v>
       </c>
       <c r="G2" t="n">
-        <v>0.5393114311048014</v>
+        <v>0.256059803711087</v>
       </c>
       <c r="H2" t="n">
-        <v>0.5735785215089194</v>
+        <v>0.2708785330017704</v>
       </c>
       <c r="I2" t="n">
-        <v>59.15453915453915</v>
+        <v>49.47330512289548</v>
       </c>
       <c r="J2" t="n">
         <v>80</v>
       </c>
       <c r="K2" t="n">
-        <v>54.51</v>
+        <v>48.69</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M2" t="n">
-        <v>54.51</v>
+        <v>48.69</v>
       </c>
       <c r="N2" t="n">
         <v>80</v>
       </c>
       <c r="O2" t="n">
-        <v>95.74468085106383</v>
+        <v>91.48936170212764</v>
       </c>
       <c r="P2" t="n">
-        <v>72.95293617021277</v>
+        <v>69.77387234042553</v>
       </c>
       <c r="Q2" t="b">
         <v>0</v>
@@ -4001,57 +4001,57 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SANSERA</t>
+          <t>WHEELS</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Forgings</t>
+          <t>Wheels</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2159.2</v>
+        <v>997.25</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.0825189088127815</v>
+        <v>0.1026037923599978</v>
       </c>
       <c r="E3" t="n">
-        <v>0.2840915848944394</v>
+        <v>0.1977540235407158</v>
       </c>
       <c r="F3" t="n">
-        <v>0.6443530576498362</v>
+        <v>0.3620842723485624</v>
       </c>
       <c r="G3" t="n">
-        <v>0.6649256989878104</v>
+        <v>0.4476877668869037</v>
       </c>
       <c r="H3" t="n">
-        <v>0.6991927893919284</v>
+        <v>0.4625064961775871</v>
       </c>
       <c r="I3" t="n">
-        <v>53.22580645161288</v>
+        <v>58.16770551570036</v>
       </c>
       <c r="J3" t="n">
         <v>80</v>
       </c>
       <c r="K3" t="n">
-        <v>48.59</v>
+        <v>46.83</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M3" t="n">
-        <v>48.59</v>
+        <v>46.83</v>
       </c>
       <c r="N3" t="n">
         <v>80</v>
       </c>
       <c r="O3" t="n">
-        <v>100</v>
+        <v>93.61702127659576</v>
       </c>
       <c r="P3" t="n">
-        <v>71.43600000000001</v>
+        <v>69.45540425531915</v>
       </c>
       <c r="Q3" t="b">
         <v>0</v>
@@ -4066,63 +4066,63 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SHRIPISTON</t>
+          <t>ASKAUTOLTD</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Engine/Parts</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>3033.5</v>
+        <v>444.75</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.0419114395805697</v>
+        <v>0.0481970304030168</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.0298698391378042</v>
+        <v>-0.0331521739130434</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1788365134263396</v>
+        <v>-0.1549496484894545</v>
       </c>
       <c r="G4" t="n">
-        <v>0.1994091547643138</v>
+        <v>-0.06934615395111331</v>
       </c>
       <c r="H4" t="n">
-        <v>0.2336762451684318</v>
+        <v>-0.0545274246604299</v>
       </c>
       <c r="I4" t="n">
-        <v>58.48653596765581</v>
+        <v>70.92402464065708</v>
       </c>
       <c r="J4" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K4" t="n">
-        <v>48.69</v>
+        <v>71.28</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M4" t="n">
-        <v>48.69</v>
+        <v>71.28</v>
       </c>
       <c r="N4" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O4" t="n">
-        <v>89.36170212765957</v>
+        <v>46.80851063829788</v>
       </c>
       <c r="P4" t="n">
-        <v>69.34834042553192</v>
+        <v>65.87370212765957</v>
       </c>
       <c r="Q4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S4" t="b">
         <v>0</v>
@@ -4131,57 +4131,57 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>WHEELS</t>
+          <t>SANSERA</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Wheels</t>
+          <t>Forgings</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1082.1</v>
+        <v>2074.5</v>
       </c>
       <c r="D5" t="n">
-        <v>0.2112833715788882</v>
+        <v>-0.09370904325032769</v>
       </c>
       <c r="E5" t="n">
-        <v>0.3170642648490749</v>
+        <v>0.2601749483659337</v>
       </c>
       <c r="F5" t="n">
-        <v>0.4677517802644964</v>
+        <v>0.5212290093128986</v>
       </c>
       <c r="G5" t="n">
-        <v>0.4883244216024706</v>
+        <v>0.6068325038512399</v>
       </c>
       <c r="H5" t="n">
-        <v>0.5225915120065886</v>
+        <v>0.6216512331419233</v>
       </c>
       <c r="I5" t="n">
-        <v>73.51181999430361</v>
+        <v>44.29001140960482</v>
       </c>
       <c r="J5" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="K5" t="n">
-        <v>46.83</v>
+        <v>48.59</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M5" t="n">
-        <v>46.83</v>
+        <v>48.59</v>
       </c>
       <c r="N5" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="O5" t="n">
-        <v>93.61702127659576</v>
+        <v>100</v>
       </c>
       <c r="P5" t="n">
-        <v>65.45540425531915</v>
+        <v>63.43600000000001</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
@@ -4196,60 +4196,60 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ASKAUTOLTD</t>
+          <t>RANEENGINE</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Engine/Parts</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>438.75</v>
+        <v>317.75</v>
       </c>
       <c r="D6" t="n">
-        <v>0.0277582572030921</v>
+        <v>0.1790352504638219</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.0647980390067142</v>
+        <v>-0.156154561147258</v>
       </c>
       <c r="F6" t="n">
-        <v>-0.15625</v>
+        <v>-0.2401052253975846</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.1356773586620258</v>
+        <v>-0.1545017308592433</v>
       </c>
       <c r="H6" t="n">
-        <v>-0.1014102682579077</v>
+        <v>-0.1396830015685599</v>
       </c>
       <c r="I6" t="n">
-        <v>72.65353418308227</v>
+        <v>63.3225806451613</v>
       </c>
       <c r="J6" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K6" t="n">
-        <v>71.28</v>
+        <v>50.88</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M6" t="n">
-        <v>71.28</v>
+        <v>50.88</v>
       </c>
       <c r="N6" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O6" t="n">
-        <v>31.91489361702128</v>
+        <v>25.53191489361702</v>
       </c>
       <c r="P6" t="n">
-        <v>62.89497872340426</v>
+        <v>57.45838297872341</v>
       </c>
       <c r="Q6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R6" t="b">
         <v>0</v>
@@ -4261,57 +4261,57 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>LUMAXTECH</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Forgings</t>
+          <t>Lighting</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1725.1</v>
+        <v>1522.2</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.0930073606729758</v>
+        <v>-0.1292758265644663</v>
       </c>
       <c r="E7" t="n">
-        <v>0.2470902913323212</v>
+        <v>0.0291393414914475</v>
       </c>
       <c r="F7" t="n">
-        <v>0.5247480996994871</v>
+        <v>0.4243473378871525</v>
       </c>
       <c r="G7" t="n">
-        <v>0.5453207410374613</v>
+        <v>0.5099508324254938</v>
       </c>
       <c r="H7" t="n">
-        <v>0.5795878314415793</v>
+        <v>0.5247695617161772</v>
       </c>
       <c r="I7" t="n">
-        <v>37.99860041987404</v>
+        <v>51.17172493276988</v>
       </c>
       <c r="J7" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="K7" t="n">
-        <v>54.83</v>
+        <v>54.51</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M7" t="n">
-        <v>54.83</v>
+        <v>54.51</v>
       </c>
       <c r="N7" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="O7" t="n">
-        <v>97.87234042553192</v>
+        <v>95.74468085106383</v>
       </c>
       <c r="P7" t="n">
-        <v>61.50646808510639</v>
+        <v>56.95293617021277</v>
       </c>
       <c r="Q7" t="b">
         <v>0</v>
@@ -4326,57 +4326,57 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MINDACORP</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Forgings</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>528.7</v>
+        <v>1674.6</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.0871104204437536</v>
+        <v>-0.124163179916318</v>
       </c>
       <c r="E8" t="n">
-        <v>-0.090643274853801</v>
+        <v>0.2101459748518572</v>
       </c>
       <c r="F8" t="n">
-        <v>0.0521393034825872</v>
+        <v>0.4732119292689363</v>
       </c>
       <c r="G8" t="n">
-        <v>0.0727119448205614</v>
+        <v>0.5588154238072776</v>
       </c>
       <c r="H8" t="n">
-        <v>0.1069790352246794</v>
+        <v>0.573634153097961</v>
       </c>
       <c r="I8" t="n">
-        <v>60.57201225740555</v>
+        <v>36.07973421926911</v>
       </c>
       <c r="J8" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="K8" t="n">
-        <v>49.42</v>
+        <v>54.83</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M8" t="n">
-        <v>49.42</v>
+        <v>54.83</v>
       </c>
       <c r="N8" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="O8" t="n">
-        <v>78.72340425531915</v>
+        <v>97.87234042553192</v>
       </c>
       <c r="P8" t="n">
-        <v>59.51268085106384</v>
+        <v>53.50646808510639</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
@@ -4391,57 +4391,57 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>DIVGIITTS</t>
+          <t>LUMAXIND</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Transmission</t>
+          <t>Lighting</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>674.75</v>
+        <v>4654</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.059909439219784</v>
+        <v>-0.2341489904392041</v>
       </c>
       <c r="E9" t="n">
-        <v>0.1113398665898048</v>
+        <v>-0.1699661137863385</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.0029553010712966</v>
+        <v>0.1235032831208962</v>
       </c>
       <c r="G9" t="n">
-        <v>0.0176173402666776</v>
+        <v>0.2091067776592374</v>
       </c>
       <c r="H9" t="n">
-        <v>0.0518844306707956</v>
+        <v>0.2239255069499208</v>
       </c>
       <c r="I9" t="n">
-        <v>40.25722339675829</v>
+        <v>39.25653594771242</v>
       </c>
       <c r="J9" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="K9" t="n">
-        <v>49.92</v>
+        <v>57.69</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M9" t="n">
-        <v>49.92</v>
+        <v>57.69</v>
       </c>
       <c r="N9" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="O9" t="n">
-        <v>65.95744680851064</v>
+        <v>87.2340425531915</v>
       </c>
       <c r="P9" t="n">
-        <v>57.15948936170213</v>
+        <v>52.5228085106383</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -4456,63 +4456,63 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>JBMA</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>546.65</v>
+        <v>481.5</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.0176116452511457</v>
+        <v>-0.1170807738149812</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.0434820647419073</v>
+        <v>0.0211006255964372</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.09860664523043949</v>
+        <v>0.0915892087961913</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.0780340038924652</v>
+        <v>0.1771927033345326</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.0437669134883472</v>
+        <v>0.192011432625216</v>
       </c>
       <c r="I10" t="n">
-        <v>56.43496214728149</v>
+        <v>40.49041182018234</v>
       </c>
       <c r="J10" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="K10" t="n">
-        <v>56.91</v>
+        <v>49.66</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M10" t="n">
-        <v>56.91</v>
+        <v>49.66</v>
       </c>
       <c r="N10" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="O10" t="n">
-        <v>51.06382978723404</v>
+        <v>82.97872340425532</v>
       </c>
       <c r="P10" t="n">
-        <v>56.9767659574468</v>
+        <v>52.45974468085107</v>
       </c>
       <c r="Q10" t="b">
         <v>0</v>
       </c>
       <c r="R10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S10" t="b">
         <v>0</v>
@@ -4521,63 +4521,63 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>LUMAXIND</t>
+          <t>TIINDIA</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Lighting</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>4880</v>
+        <v>2517.3</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.214752357352042</v>
+        <v>-0.0746241223394478</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.152041702867072</v>
+        <v>-0.0420868373986833</v>
       </c>
       <c r="F11" t="n">
-        <v>0.1645110485372021</v>
+        <v>-0.1582625560088275</v>
       </c>
       <c r="G11" t="n">
-        <v>0.1850836898751763</v>
+        <v>-0.0726590614704862</v>
       </c>
       <c r="H11" t="n">
-        <v>0.2193507802792943</v>
+        <v>-0.0578403321798028</v>
       </c>
       <c r="I11" t="n">
-        <v>42.24175824175824</v>
+        <v>42.44338498212158</v>
       </c>
       <c r="J11" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K11" t="n">
-        <v>57.69</v>
+        <v>48.73</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M11" t="n">
-        <v>57.69</v>
+        <v>48.73</v>
       </c>
       <c r="N11" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O11" t="n">
-        <v>87.2340425531915</v>
+        <v>44.68085106382978</v>
       </c>
       <c r="P11" t="n">
-        <v>56.5228085106383</v>
+        <v>52.42817021276596</v>
       </c>
       <c r="Q11" t="b">
         <v>0</v>
       </c>
       <c r="R11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S11" t="b">
         <v>0</v>
@@ -4586,63 +4586,63 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>RANEENGINE</t>
+          <t>ZFCVINDIA</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Engine/Parts</t>
+          <t>Brakes/Transmission</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>317.75</v>
+        <v>13768</v>
       </c>
       <c r="D12" t="n">
-        <v>0.1790352504638219</v>
+        <v>-0.1120856442667355</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.156154561147258</v>
+        <v>-0.0412923891093934</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.2401052253975846</v>
+        <v>0.0181172816682688</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.2195325840596104</v>
+        <v>0.1037207762066101</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.1852654936554923</v>
+        <v>0.1185395054972935</v>
       </c>
       <c r="I12" t="n">
-        <v>63.3225806451613</v>
+        <v>45.60588463027487</v>
       </c>
       <c r="J12" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="K12" t="n">
-        <v>50.88</v>
+        <v>50.29</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M12" t="n">
-        <v>50.88</v>
+        <v>50.29</v>
       </c>
       <c r="N12" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="O12" t="n">
-        <v>19.14893617021277</v>
+        <v>76.59574468085107</v>
       </c>
       <c r="P12" t="n">
-        <v>56.18178723404256</v>
+        <v>51.43514893617021</v>
       </c>
       <c r="Q12" t="b">
         <v>0</v>
       </c>
       <c r="R12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S12" t="b">
         <v>0</v>
@@ -4651,63 +4651,63 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>SUPRAJIT</t>
+          <t>MINDACORP</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Cables</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>414.45</v>
+        <v>505.65</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.07694877505567931</v>
+        <v>-0.1166914140973012</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.09725549989109129</v>
+        <v>-0.1371160409556314</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.0862087972660126</v>
+        <v>0.0032738095238094</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.0656361559280384</v>
+        <v>0.08887730406215059</v>
       </c>
       <c r="H13" t="n">
-        <v>-0.0313690655239203</v>
+        <v>0.103696033352834</v>
       </c>
       <c r="I13" t="n">
-        <v>51.39171758316361</v>
+        <v>49.5638629283489</v>
       </c>
       <c r="J13" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="K13" t="n">
-        <v>51.48</v>
+        <v>49.42</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M13" t="n">
-        <v>51.48</v>
+        <v>49.42</v>
       </c>
       <c r="N13" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="O13" t="n">
-        <v>55.31914893617022</v>
+        <v>72.3404255319149</v>
       </c>
       <c r="P13" t="n">
-        <v>55.65582978723404</v>
+        <v>50.23608510638298</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
       </c>
       <c r="R13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S13" t="b">
         <v>0</v>
@@ -4716,57 +4716,57 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>CRAFTSMAN</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Castings</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>488.75</v>
+        <v>6977</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.0982472324723247</v>
+        <v>-0.1002643626281514</v>
       </c>
       <c r="E14" t="n">
-        <v>0.0200354794949391</v>
+        <v>0.0007171543316122</v>
       </c>
       <c r="F14" t="n">
-        <v>0.1159949765955017</v>
+        <v>0.0120394545982014</v>
       </c>
       <c r="G14" t="n">
-        <v>0.1365676179334759</v>
+        <v>0.0976429491365427</v>
       </c>
       <c r="H14" t="n">
-        <v>0.1708347083375939</v>
+        <v>0.1124616784272261</v>
       </c>
       <c r="I14" t="n">
-        <v>46.33097942892233</v>
+        <v>39.96383363471971</v>
       </c>
       <c r="J14" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K14" t="n">
-        <v>49.66</v>
+        <v>54.65</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M14" t="n">
-        <v>49.66</v>
+        <v>54.65</v>
       </c>
       <c r="N14" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O14" t="n">
-        <v>82.97872340425532</v>
+        <v>74.46808510638297</v>
       </c>
       <c r="P14" t="n">
-        <v>52.45974468085107</v>
+        <v>48.7536170212766</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
@@ -4781,57 +4781,57 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>GNA</t>
+          <t>PRICOLLTD</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Axles</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>377.85</v>
+        <v>513.9</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.1040901007705986</v>
+        <v>-0.1680427391937835</v>
       </c>
       <c r="E15" t="n">
-        <v>0.2341989220970115</v>
+        <v>-0.1588509698011294</v>
       </c>
       <c r="F15" t="n">
-        <v>0.2218270008084075</v>
+        <v>0.0446183555239352</v>
       </c>
       <c r="G15" t="n">
-        <v>0.2423996421463817</v>
+        <v>0.1302218500622765</v>
       </c>
       <c r="H15" t="n">
-        <v>0.2766667325504998</v>
+        <v>0.1450405793529599</v>
       </c>
       <c r="I15" t="n">
-        <v>33.32275468105364</v>
+        <v>36.24708624708624</v>
       </c>
       <c r="J15" t="n">
         <v>30</v>
       </c>
       <c r="K15" t="n">
-        <v>54.47</v>
+        <v>49.98</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M15" t="n">
-        <v>54.47</v>
+        <v>49.98</v>
       </c>
       <c r="N15" t="n">
         <v>30</v>
       </c>
       <c r="O15" t="n">
-        <v>91.48936170212764</v>
+        <v>80.85106382978722</v>
       </c>
       <c r="P15" t="n">
-        <v>52.08587234042552</v>
+        <v>48.16221276595745</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
@@ -4846,57 +4846,57 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CRAFTSMAN</t>
+          <t>GNA</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Castings</t>
+          <t>Axles</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>6924</v>
+        <v>356.7</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.1117382937780628</v>
+        <v>-0.1540377090003557</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.0214810627473148</v>
+        <v>0.1714285714285714</v>
       </c>
       <c r="F16" t="n">
-        <v>0.0129471143296027</v>
+        <v>0.1581168831168831</v>
       </c>
       <c r="G16" t="n">
-        <v>0.0335197556675769</v>
+        <v>0.2437203776552243</v>
       </c>
       <c r="H16" t="n">
-        <v>0.0677868460716949</v>
+        <v>0.2585391069459077</v>
       </c>
       <c r="I16" t="n">
-        <v>42.07197382769901</v>
+        <v>29.85499004833665</v>
       </c>
       <c r="J16" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="K16" t="n">
-        <v>54.65</v>
+        <v>54.47</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="M16" t="n">
-        <v>54.65</v>
+        <v>54.47</v>
       </c>
       <c r="N16" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="O16" t="n">
-        <v>70.21276595744681</v>
+        <v>89.36170212765957</v>
       </c>
       <c r="P16" t="n">
-        <v>51.90255319148936</v>
+        <v>47.66034042553191</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
chore: auto-refresh NSE data and pipeline outputs (2026-03-31)
</commit_message>
<xml_diff>
--- a/working-sector/output/auto_components_comprehensive_report.xlsx
+++ b/working-sector/output/auto_components_comprehensive_report.xlsx
@@ -435,7 +435,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
     </row>
@@ -447,7 +447,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
     </row>
@@ -782,22 +782,22 @@
         <v>1674.6</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.124163179916318</v>
+        <v>-0.1237965676015069</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2101459748518572</v>
+        <v>0.1898536308085829</v>
       </c>
       <c r="F2" t="n">
-        <v>0.4732119292689363</v>
+        <v>0.3922514133688062</v>
       </c>
       <c r="G2" t="n">
-        <v>0.5588154238072776</v>
+        <v>0.4778549079071474</v>
       </c>
       <c r="H2" t="n">
-        <v>0.573634153097961</v>
+        <v>0.4926736371978308</v>
       </c>
       <c r="I2" t="n">
-        <v>36.07973421926911</v>
+        <v>39.00161608906448</v>
       </c>
       <c r="J2" t="n">
         <v>30</v>
@@ -807,7 +807,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M2" t="n">
@@ -847,45 +847,45 @@
         <v>1031.6</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.1617097350885746</v>
+        <v>-0.132015145140934</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.1567072672279899</v>
+        <v>-0.1646287148756985</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.2056060372709071</v>
+        <v>-0.2124589663333079</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.1200025427325658</v>
+        <v>-0.1268554717949667</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.1051838134418824</v>
+        <v>-0.1120367425042833</v>
       </c>
       <c r="I3" t="n">
-        <v>38.93190921228303</v>
+        <v>42.66900790166812</v>
       </c>
       <c r="J3" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K3" t="n">
         <v>49.36</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M3" t="n">
         <v>49.36</v>
       </c>
       <c r="N3" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O3" t="n">
-        <v>31.91489361702128</v>
+        <v>36.17021276595745</v>
       </c>
       <c r="P3" t="n">
-        <v>38.12697872340426</v>
+        <v>42.97804255319149</v>
       </c>
       <c r="Q3" t="b">
         <v>0</v>
@@ -912,45 +912,45 @@
         <v>28745</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.2176102340772999</v>
+        <v>-0.210844200411805</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.2103021978021978</v>
+        <v>-0.2205802603036876</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.2973600586653629</v>
+        <v>-0.3049208076411558</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.2117565641270217</v>
+        <v>-0.2193173131028145</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.1969378348363383</v>
+        <v>-0.2044985838121311</v>
       </c>
       <c r="I4" t="n">
-        <v>29.14321450906817</v>
+        <v>30.53735255570118</v>
       </c>
       <c r="J4" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="K4" t="n">
         <v>53.48</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M4" t="n">
         <v>53.48</v>
       </c>
       <c r="N4" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="O4" t="n">
         <v>14.8936170212766</v>
       </c>
       <c r="P4" t="n">
-        <v>32.37072340425532</v>
+        <v>36.37072340425532</v>
       </c>
       <c r="Q4" t="b">
         <v>0</v>
@@ -977,22 +977,22 @@
         <v>287.9</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.1528615565690747</v>
+        <v>-0.1387974872868681</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.222732181425486</v>
+        <v>-0.2314468766684464</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.3024833434282253</v>
+        <v>-0.3263133263133264</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.2168798488898841</v>
+        <v>-0.2407098317749851</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.2020611195992007</v>
+        <v>-0.2258911024843017</v>
       </c>
       <c r="I5" t="n">
-        <v>33.9393939393939</v>
+        <v>36.15023474178401</v>
       </c>
       <c r="J5" t="n">
         <v>30</v>
@@ -1002,7 +1002,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M5" t="n">
@@ -1012,10 +1012,10 @@
         <v>30</v>
       </c>
       <c r="O5" t="n">
-        <v>12.76595744680851</v>
+        <v>10.63829787234042</v>
       </c>
       <c r="P5" t="n">
-        <v>35.0011914893617</v>
+        <v>34.57565957446808</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
@@ -1042,22 +1042,22 @@
         <v>105.08</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.2234129037026088</v>
+        <v>-0.2119394030298486</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.0963192294461644</v>
+        <v>-0.1228714524207011</v>
       </c>
       <c r="F6" t="n">
-        <v>0.1107822410147991</v>
+        <v>0.0660444354266005</v>
       </c>
       <c r="G6" t="n">
-        <v>0.1963857355531404</v>
+        <v>0.1516479299649418</v>
       </c>
       <c r="H6" t="n">
-        <v>0.2112044648438238</v>
+        <v>0.1664666592556252</v>
       </c>
       <c r="I6" t="n">
-        <v>27.27498140342178</v>
+        <v>28.7131297311407</v>
       </c>
       <c r="J6" t="n">
         <v>20</v>
@@ -1067,7 +1067,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M6" t="n">
@@ -1107,22 +1107,22 @@
         <v>2517.3</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.0746241223394478</v>
+        <v>-0.0857485290913052</v>
       </c>
       <c r="E7" t="n">
-        <v>-0.0420868373986833</v>
+        <v>-0.0504696163856511</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.1582625560088275</v>
+        <v>-0.1806464212479249</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.0726590614704862</v>
+        <v>-0.0950429267095837</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.0578403321798028</v>
+        <v>-0.0802241974189003</v>
       </c>
       <c r="I7" t="n">
-        <v>42.44338498212158</v>
+        <v>46.79984229202262</v>
       </c>
       <c r="J7" t="n">
         <v>60</v>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M7" t="n">
@@ -1142,10 +1142,10 @@
         <v>60</v>
       </c>
       <c r="O7" t="n">
-        <v>44.68085106382978</v>
+        <v>42.5531914893617</v>
       </c>
       <c r="P7" t="n">
-        <v>52.42817021276596</v>
+        <v>52.00263829787234</v>
       </c>
       <c r="Q7" t="b">
         <v>0</v>
@@ -1172,45 +1172,45 @@
         <v>481.5</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.1170807738149812</v>
+        <v>-0.0991580916744621</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0211006255964372</v>
+        <v>-0.0034150884818379</v>
       </c>
       <c r="F8" t="n">
-        <v>0.0915892087961913</v>
+        <v>0.059755694948828</v>
       </c>
       <c r="G8" t="n">
-        <v>0.1771927033345326</v>
+        <v>0.1453591894871693</v>
       </c>
       <c r="H8" t="n">
-        <v>0.192011432625216</v>
+        <v>0.1601779187778527</v>
       </c>
       <c r="I8" t="n">
-        <v>40.49041182018234</v>
+        <v>38.7180317254775</v>
       </c>
       <c r="J8" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K8" t="n">
         <v>49.66</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M8" t="n">
         <v>49.66</v>
       </c>
       <c r="N8" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O8" t="n">
         <v>82.97872340425532</v>
       </c>
       <c r="P8" t="n">
-        <v>52.45974468085107</v>
+        <v>48.45974468085107</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
@@ -1237,22 +1237,22 @@
         <v>412.3</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.105348811977867</v>
+        <v>-0.0919502257460631</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.2082573211713874</v>
+        <v>-0.1980159502042404</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.146023198011599</v>
+        <v>-0.1410416666666666</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.0604197034732577</v>
+        <v>-0.0554381721283253</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.0456009741825743</v>
+        <v>-0.0406194428376419</v>
       </c>
       <c r="I9" t="n">
-        <v>38.6058981233244</v>
+        <v>39.8707891093678</v>
       </c>
       <c r="J9" t="n">
         <v>30</v>
@@ -1262,7 +1262,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M9" t="n">
@@ -1302,22 +1302,22 @@
         <v>128495</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.1046892419175028</v>
+        <v>-0.088590984856545</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.1528267677600131</v>
+        <v>-0.1632261005470174</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.1323767724510466</v>
+        <v>-0.1263301036885942</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.0467732779127053</v>
+        <v>-0.0407266091502529</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.0319545486220219</v>
+        <v>-0.0259078798595695</v>
       </c>
       <c r="I10" t="n">
-        <v>32.67638943634213</v>
+        <v>34.05916187345933</v>
       </c>
       <c r="J10" t="n">
         <v>30</v>
@@ -1327,7 +1327,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M10" t="n">
@@ -1392,7 +1392,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M11" t="n">
@@ -1432,45 +1432,45 @@
         <v>444.75</v>
       </c>
       <c r="D12" t="n">
-        <v>0.0481970304030168</v>
+        <v>0.0707836764174791</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.0331521739130434</v>
+        <v>-0.0402460077686663</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.1549496484894545</v>
+        <v>-0.174018014671743</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.06934615395111331</v>
+        <v>-0.0884145201334017</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.0545274246604299</v>
+        <v>-0.07359579084271831</v>
       </c>
       <c r="I12" t="n">
-        <v>70.92402464065708</v>
+        <v>68.07935076645629</v>
       </c>
       <c r="J12" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K12" t="n">
         <v>71.28</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M12" t="n">
         <v>71.28</v>
       </c>
       <c r="N12" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O12" t="n">
-        <v>46.80851063829788</v>
+        <v>44.68085106382978</v>
       </c>
       <c r="P12" t="n">
-        <v>65.87370212765957</v>
+        <v>69.44817021276596</v>
       </c>
       <c r="Q12" t="b">
         <v>1</v>
@@ -1497,22 +1497,22 @@
         <v>1547.1</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.23795685154172</v>
+        <v>-0.2437307523097228</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.1317207318442025</v>
+        <v>-0.1586818206536517</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.100157040656081</v>
+        <v>-0.0912775330396475</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.0145535461177397</v>
+        <v>-0.0056740385013063</v>
       </c>
       <c r="H13" t="n">
-        <v>0.0002651831729436</v>
+        <v>0.009144690789377</v>
       </c>
       <c r="I13" t="n">
-        <v>18.14388249040228</v>
+        <v>19.14743702659856</v>
       </c>
       <c r="J13" t="n">
         <v>20</v>
@@ -1522,7 +1522,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M13" t="n">
@@ -1532,10 +1532,10 @@
         <v>20</v>
       </c>
       <c r="O13" t="n">
-        <v>57.44680851063831</v>
+        <v>59.57446808510638</v>
       </c>
       <c r="P13" t="n">
-        <v>42.99736170212766</v>
+        <v>43.42289361702128</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
@@ -1562,22 +1562,22 @@
         <v>504.35</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.201029702970297</v>
+        <v>-0.1903844610321855</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.2905471936981291</v>
+        <v>-0.2867345495686607</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.1714309183505832</v>
+        <v>-0.2022933965994463</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.0858274238122419</v>
+        <v>-0.116689902061105</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.0710086945215585</v>
+        <v>-0.1018711727704216</v>
       </c>
       <c r="I14" t="n">
-        <v>34.31717029749359</v>
+        <v>32.83832335329343</v>
       </c>
       <c r="J14" t="n">
         <v>30</v>
@@ -1587,7 +1587,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M14" t="n">
@@ -1597,10 +1597,10 @@
         <v>30</v>
       </c>
       <c r="O14" t="n">
-        <v>38.29787234042553</v>
+        <v>40.42553191489361</v>
       </c>
       <c r="P14" t="n">
-        <v>41.51557446808511</v>
+        <v>41.94110638297872</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
@@ -1627,22 +1627,22 @@
         <v>86.22</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.2070265796008461</v>
+        <v>-0.1924697948862039</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.1849891294073165</v>
+        <v>-0.2105118578884717</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.012484251517581</v>
+        <v>-0.0038128249566724</v>
       </c>
       <c r="G15" t="n">
-        <v>0.0731192430207602</v>
+        <v>0.08179066958166881</v>
       </c>
       <c r="H15" t="n">
-        <v>0.0879379723114436</v>
+        <v>0.0966093988723522</v>
       </c>
       <c r="I15" t="n">
-        <v>27.45098039215688</v>
+        <v>28.62149532710282</v>
       </c>
       <c r="J15" t="n">
         <v>20</v>
@@ -1652,7 +1652,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M15" t="n">
@@ -1662,10 +1662,10 @@
         <v>20</v>
       </c>
       <c r="O15" t="n">
-        <v>68.08510638297872</v>
+        <v>72.3404255319149</v>
       </c>
       <c r="P15" t="n">
-        <v>42.38102127659575</v>
+        <v>43.23208510638298</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
@@ -1692,22 +1692,22 @@
         <v>140.81</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.2751467105940491</v>
+        <v>-0.2591676750670805</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.1720468042570705</v>
+        <v>-0.1727278068268609</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.1217488929083765</v>
+        <v>-0.0876635998444991</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.0361453983700352</v>
+        <v>-0.0020601053061578</v>
       </c>
       <c r="H16" t="n">
-        <v>-0.0213266690793518</v>
+        <v>0.0127586239845255</v>
       </c>
       <c r="I16" t="n">
-        <v>26.96097753251871</v>
+        <v>28.28784119106699</v>
       </c>
       <c r="J16" t="n">
         <v>20</v>
@@ -1717,7 +1717,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M16" t="n">
@@ -1727,16 +1727,16 @@
         <v>20</v>
       </c>
       <c r="O16" t="n">
-        <v>55.31914893617022</v>
+        <v>61.70212765957447</v>
       </c>
       <c r="P16" t="n">
-        <v>40.10782978723405</v>
+        <v>41.38442553191489</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>
       </c>
       <c r="R16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S16" t="b">
         <v>0</v>
@@ -1757,45 +1757,45 @@
         <v>6977</v>
       </c>
       <c r="D17" t="n">
-        <v>-0.1002643626281514</v>
+        <v>-0.07294711666223749</v>
       </c>
       <c r="E17" t="n">
-        <v>0.0007171543316122</v>
+        <v>-0.007680273076376</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0120394545982014</v>
+        <v>0.0204768173175369</v>
       </c>
       <c r="G17" t="n">
-        <v>0.0976429491365427</v>
+        <v>0.1060803118558781</v>
       </c>
       <c r="H17" t="n">
-        <v>0.1124616784272261</v>
+        <v>0.1208990411465615</v>
       </c>
       <c r="I17" t="n">
-        <v>39.96383363471971</v>
+        <v>41.76706827309237</v>
       </c>
       <c r="J17" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K17" t="n">
         <v>54.65</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M17" t="n">
         <v>54.65</v>
       </c>
       <c r="N17" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O17" t="n">
-        <v>74.46808510638297</v>
+        <v>76.59574468085107</v>
       </c>
       <c r="P17" t="n">
-        <v>48.7536170212766</v>
+        <v>53.17914893617021</v>
       </c>
       <c r="Q17" t="b">
         <v>0</v>
@@ -1822,45 +1822,45 @@
         <v>615.8</v>
       </c>
       <c r="D18" t="n">
-        <v>-0.1860956912503305</v>
+        <v>-0.147386638975424</v>
       </c>
       <c r="E18" t="n">
-        <v>0.0378360158422514</v>
+        <v>0.0355671403346506</v>
       </c>
       <c r="F18" t="n">
-        <v>-0.0836991295290529</v>
+        <v>-0.0946114827611557</v>
       </c>
       <c r="G18" t="n">
-        <v>0.0019043650092883</v>
+        <v>-0.0090079882228144</v>
       </c>
       <c r="H18" t="n">
-        <v>0.0167230942999717</v>
+        <v>0.0058107410678689</v>
       </c>
       <c r="I18" t="n">
-        <v>29.6598430044636</v>
+        <v>32.1220203367228</v>
       </c>
       <c r="J18" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="K18" t="n">
         <v>49.92</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M18" t="n">
         <v>49.92</v>
       </c>
       <c r="N18" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="O18" t="n">
-        <v>59.57446808510638</v>
+        <v>57.44680851063831</v>
       </c>
       <c r="P18" t="n">
-        <v>39.88289361702128</v>
+        <v>43.45736170212766</v>
       </c>
       <c r="Q18" t="b">
         <v>0</v>
@@ -1887,22 +1887,22 @@
         <v>2213.9</v>
       </c>
       <c r="D19" t="n">
-        <v>-0.1630500529260546</v>
+        <v>-0.1682383439155426</v>
       </c>
       <c r="E19" t="n">
-        <v>-0.138090788756521</v>
+        <v>-0.1350939563230064</v>
       </c>
       <c r="F19" t="n">
-        <v>-0.2540265516544241</v>
+        <v>-0.2633102622121654</v>
       </c>
       <c r="G19" t="n">
-        <v>-0.1684230571160828</v>
+        <v>-0.1777067676738242</v>
       </c>
       <c r="H19" t="n">
-        <v>-0.1536043278253994</v>
+        <v>-0.1628880383831408</v>
       </c>
       <c r="I19" t="n">
-        <v>28.77544320420225</v>
+        <v>27.25901089689862</v>
       </c>
       <c r="J19" t="n">
         <v>20</v>
@@ -1912,7 +1912,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M19" t="n">
@@ -1952,22 +1952,22 @@
         <v>1910.9</v>
       </c>
       <c r="D20" t="n">
-        <v>-0.1355740522934949</v>
+        <v>-0.1220307833677922</v>
       </c>
       <c r="E20" t="n">
-        <v>-0.1480606330806955</v>
+        <v>-0.1591939103269238</v>
       </c>
       <c r="F20" t="n">
-        <v>-0.064614029076313</v>
+        <v>-0.1192385693215338</v>
       </c>
       <c r="G20" t="n">
-        <v>0.0209894654620281</v>
+        <v>-0.0336350747831926</v>
       </c>
       <c r="H20" t="n">
-        <v>0.0358081947527115</v>
+        <v>-0.0188163454925092</v>
       </c>
       <c r="I20" t="n">
-        <v>33.63350485991995</v>
+        <v>35.07751937984497</v>
       </c>
       <c r="J20" t="n">
         <v>30</v>
@@ -1977,7 +1977,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M20" t="n">
@@ -1987,16 +1987,16 @@
         <v>30</v>
       </c>
       <c r="O20" t="n">
-        <v>61.70212765957447</v>
+        <v>55.31914893617022</v>
       </c>
       <c r="P20" t="n">
-        <v>43.9644255319149</v>
+        <v>42.68782978723405</v>
       </c>
       <c r="Q20" t="b">
         <v>0</v>
       </c>
       <c r="R20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S20" t="b">
         <v>0</v>
@@ -2017,45 +2017,45 @@
         <v>826.35</v>
       </c>
       <c r="D21" t="n">
-        <v>-0.1824387830818699</v>
+        <v>-0.1726571886263516</v>
       </c>
       <c r="E21" t="n">
-        <v>-0.1344401382633288</v>
+        <v>-0.1417220606564186</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.3123491720063244</v>
+        <v>-0.3232740971255424</v>
       </c>
       <c r="G21" t="n">
-        <v>-0.2267456774679831</v>
+        <v>-0.2376706025872011</v>
       </c>
       <c r="H21" t="n">
-        <v>-0.2119269481772997</v>
+        <v>-0.2228518732965178</v>
       </c>
       <c r="I21" t="n">
-        <v>38.13135388091013</v>
+        <v>40.18024145553478</v>
       </c>
       <c r="J21" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K21" t="n">
         <v>48.43</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M21" t="n">
         <v>48.43</v>
       </c>
       <c r="N21" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O21" t="n">
-        <v>10.63829787234042</v>
+        <v>12.76595744680851</v>
       </c>
       <c r="P21" t="n">
-        <v>33.49965957446808</v>
+        <v>37.9251914893617</v>
       </c>
       <c r="Q21" t="b">
         <v>0</v>
@@ -2082,45 +2082,45 @@
         <v>356.7</v>
       </c>
       <c r="D22" t="n">
-        <v>-0.1540377090003557</v>
+        <v>-0.1486873508353222</v>
       </c>
       <c r="E22" t="n">
-        <v>0.1714285714285714</v>
+        <v>0.167021102568297</v>
       </c>
       <c r="F22" t="n">
-        <v>0.1581168831168831</v>
+        <v>0.1361681796464404</v>
       </c>
       <c r="G22" t="n">
-        <v>0.2437203776552243</v>
+        <v>0.2217716741847817</v>
       </c>
       <c r="H22" t="n">
-        <v>0.2585391069459077</v>
+        <v>0.2365904034754651</v>
       </c>
       <c r="I22" t="n">
-        <v>29.85499004833665</v>
+        <v>30.99173553719008</v>
       </c>
       <c r="J22" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="K22" t="n">
         <v>54.47</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M22" t="n">
         <v>54.47</v>
       </c>
       <c r="N22" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="O22" t="n">
-        <v>89.36170212765957</v>
+        <v>91.48936170212764</v>
       </c>
       <c r="P22" t="n">
-        <v>47.66034042553191</v>
+        <v>52.08587234042552</v>
       </c>
       <c r="Q22" t="b">
         <v>0</v>
@@ -2147,22 +2147,22 @@
         <v>314.25</v>
       </c>
       <c r="D23" t="n">
-        <v>-0.1529649595687331</v>
+        <v>-0.1496414558246516</v>
       </c>
       <c r="E23" t="n">
-        <v>-0.1369129360065916</v>
+        <v>-0.1480276535176902</v>
       </c>
       <c r="F23" t="n">
-        <v>-0.220899962811454</v>
+        <v>-0.2276972229048905</v>
       </c>
       <c r="G23" t="n">
-        <v>-0.1352964682731128</v>
+        <v>-0.1420937283665493</v>
       </c>
       <c r="H23" t="n">
-        <v>-0.1204777389824294</v>
+        <v>-0.1272749990758659</v>
       </c>
       <c r="I23" t="n">
-        <v>18.96678966789663</v>
+        <v>19.20777279521669</v>
       </c>
       <c r="J23" t="n">
         <v>20</v>
@@ -2172,7 +2172,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M23" t="n">
@@ -2182,10 +2182,10 @@
         <v>20</v>
       </c>
       <c r="O23" t="n">
-        <v>29.78723404255319</v>
+        <v>27.65957446808511</v>
       </c>
       <c r="P23" t="n">
-        <v>33.83744680851064</v>
+        <v>33.41191489361702</v>
       </c>
       <c r="Q23" t="b">
         <v>0</v>
@@ -2212,22 +2212,22 @@
         <v>111.92</v>
       </c>
       <c r="D24" t="n">
-        <v>-0.2450590219224283</v>
+        <v>-0.2408600691853761</v>
       </c>
       <c r="E24" t="n">
-        <v>-0.0872614581634317</v>
+        <v>-0.1084202979367482</v>
       </c>
       <c r="F24" t="n">
-        <v>0.0388935301216002</v>
+        <v>0.0512868683073455</v>
       </c>
       <c r="G24" t="n">
-        <v>0.1244970246599415</v>
+        <v>0.1368903628456867</v>
       </c>
       <c r="H24" t="n">
-        <v>0.1393157539506249</v>
+        <v>0.1517090921363701</v>
       </c>
       <c r="I24" t="n">
-        <v>35.49618320610686</v>
+        <v>37.34939759036145</v>
       </c>
       <c r="J24" t="n">
         <v>30</v>
@@ -2237,7 +2237,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M24" t="n">
@@ -2247,10 +2247,10 @@
         <v>30</v>
       </c>
       <c r="O24" t="n">
-        <v>78.72340425531915</v>
+        <v>80.85106382978722</v>
       </c>
       <c r="P24" t="n">
-        <v>47.06468085106384</v>
+        <v>47.49021276595744</v>
       </c>
       <c r="Q24" t="b">
         <v>0</v>
@@ -2277,22 +2277,22 @@
         <v>515.25</v>
       </c>
       <c r="D25" t="n">
-        <v>-0.0810593900481542</v>
+        <v>-0.06547565067561439</v>
       </c>
       <c r="E25" t="n">
-        <v>-0.0777698228029354</v>
+        <v>-0.0882951428824205</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.1602835723598435</v>
+        <v>-0.1726878612716762</v>
       </c>
       <c r="G25" t="n">
-        <v>-0.07468007782150229</v>
+        <v>-0.0870843667333349</v>
       </c>
       <c r="H25" t="n">
-        <v>-0.0598613485308189</v>
+        <v>-0.07226563744265151</v>
       </c>
       <c r="I25" t="n">
-        <v>48.86731391585761</v>
+        <v>50.56932350971199</v>
       </c>
       <c r="J25" t="n">
         <v>40</v>
@@ -2302,7 +2302,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M25" t="n">
@@ -2312,10 +2312,10 @@
         <v>40</v>
       </c>
       <c r="O25" t="n">
-        <v>42.5531914893617</v>
+        <v>46.80851063829788</v>
       </c>
       <c r="P25" t="n">
-        <v>47.27463829787234</v>
+        <v>48.12570212765957</v>
       </c>
       <c r="Q25" t="b">
         <v>0</v>
@@ -2342,22 +2342,22 @@
         <v>117.55</v>
       </c>
       <c r="D26" t="n">
-        <v>-0.1683175321918777</v>
+        <v>-0.21255359056806</v>
       </c>
       <c r="E26" t="n">
-        <v>-0.1842470506592644</v>
+        <v>-0.1915405777166438</v>
       </c>
       <c r="F26" t="n">
-        <v>-0.2612957958901527</v>
+        <v>-0.2586870151983351</v>
       </c>
       <c r="G26" t="n">
-        <v>-0.1756923013518114</v>
+        <v>-0.1730835206599938</v>
       </c>
       <c r="H26" t="n">
-        <v>-0.160873572061128</v>
+        <v>-0.1582647913693105</v>
       </c>
       <c r="I26" t="n">
-        <v>28.11407048695187</v>
+        <v>23.59164998570205</v>
       </c>
       <c r="J26" t="n">
         <v>20</v>
@@ -2367,7 +2367,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M26" t="n">
@@ -2377,10 +2377,10 @@
         <v>20</v>
       </c>
       <c r="O26" t="n">
-        <v>17.02127659574468</v>
+        <v>23.40425531914894</v>
       </c>
       <c r="P26" t="n">
-        <v>32.02025531914894</v>
+        <v>33.29685106382978</v>
       </c>
       <c r="Q26" t="b">
         <v>0</v>
@@ -2407,22 +2407,22 @@
         <v>4654</v>
       </c>
       <c r="D27" t="n">
-        <v>-0.2341489904392041</v>
+        <v>-0.2302221340081708</v>
       </c>
       <c r="E27" t="n">
-        <v>-0.1699661137863385</v>
+        <v>-0.1675163223325284</v>
       </c>
       <c r="F27" t="n">
-        <v>0.1235032831208962</v>
+        <v>0.114944180920895</v>
       </c>
       <c r="G27" t="n">
-        <v>0.2091067776592374</v>
+        <v>0.2005476754592363</v>
       </c>
       <c r="H27" t="n">
-        <v>0.2239255069499208</v>
+        <v>0.2153664047499197</v>
       </c>
       <c r="I27" t="n">
-        <v>39.25653594771242</v>
+        <v>37.80844834797156</v>
       </c>
       <c r="J27" t="n">
         <v>30</v>
@@ -2432,7 +2432,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M27" t="n">
@@ -2472,22 +2472,22 @@
         <v>1522.2</v>
       </c>
       <c r="D28" t="n">
-        <v>-0.1292758265644663</v>
+        <v>-0.1338340730624786</v>
       </c>
       <c r="E28" t="n">
-        <v>0.0291393414914475</v>
+        <v>0.0300446609825417</v>
       </c>
       <c r="F28" t="n">
-        <v>0.4243473378871525</v>
+        <v>0.3264203555245732</v>
       </c>
       <c r="G28" t="n">
-        <v>0.5099508324254938</v>
+        <v>0.4120238500629145</v>
       </c>
       <c r="H28" t="n">
-        <v>0.5247695617161772</v>
+        <v>0.4268425793535979</v>
       </c>
       <c r="I28" t="n">
-        <v>51.17172493276988</v>
+        <v>53.46534653465347</v>
       </c>
       <c r="J28" t="n">
         <v>40</v>
@@ -2497,7 +2497,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M28" t="n">
@@ -2507,10 +2507,10 @@
         <v>40</v>
       </c>
       <c r="O28" t="n">
-        <v>95.74468085106383</v>
+        <v>93.61702127659576</v>
       </c>
       <c r="P28" t="n">
-        <v>56.95293617021277</v>
+        <v>56.52740425531916</v>
       </c>
       <c r="Q28" t="b">
         <v>0</v>
@@ -2537,22 +2537,22 @@
         <v>505.65</v>
       </c>
       <c r="D29" t="n">
-        <v>-0.1166914140973012</v>
+        <v>-0.08982089820898199</v>
       </c>
       <c r="E29" t="n">
-        <v>-0.1371160409556314</v>
+        <v>-0.1342350826127899</v>
       </c>
       <c r="F29" t="n">
-        <v>0.0032738095238094</v>
+        <v>-0.0287168651555898</v>
       </c>
       <c r="G29" t="n">
-        <v>0.08887730406215059</v>
+        <v>0.0568866293827514</v>
       </c>
       <c r="H29" t="n">
-        <v>0.103696033352834</v>
+        <v>0.0717053586734348</v>
       </c>
       <c r="I29" t="n">
-        <v>49.5638629283489</v>
+        <v>53.85917400135408</v>
       </c>
       <c r="J29" t="n">
         <v>40</v>
@@ -2562,7 +2562,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M29" t="n">
@@ -2572,10 +2572,10 @@
         <v>40</v>
       </c>
       <c r="O29" t="n">
-        <v>72.3404255319149</v>
+        <v>65.95744680851064</v>
       </c>
       <c r="P29" t="n">
-        <v>50.23608510638298</v>
+        <v>48.95948936170213</v>
       </c>
       <c r="Q29" t="b">
         <v>0</v>
@@ -2602,22 +2602,22 @@
         <v>102.65</v>
       </c>
       <c r="D30" t="n">
-        <v>-0.1111014894354001</v>
+        <v>-0.1160006889424732</v>
       </c>
       <c r="E30" t="n">
-        <v>-0.041370937616735</v>
+        <v>-0.0297731568998108</v>
       </c>
       <c r="F30" t="n">
-        <v>-0.1795875959079284</v>
+        <v>-0.2266837426548139</v>
       </c>
       <c r="G30" t="n">
-        <v>-0.0939841013695871</v>
+        <v>-0.1410802481164726</v>
       </c>
       <c r="H30" t="n">
-        <v>-0.0791653720789037</v>
+        <v>-0.1262615188257893</v>
       </c>
       <c r="I30" t="n">
-        <v>28.93339768339769</v>
+        <v>15.27617951668582</v>
       </c>
       <c r="J30" t="n">
         <v>20</v>
@@ -2627,7 +2627,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M30" t="n">
@@ -2637,10 +2637,10 @@
         <v>20</v>
       </c>
       <c r="O30" t="n">
-        <v>36.17021276595745</v>
+        <v>29.78723404255319</v>
       </c>
       <c r="P30" t="n">
-        <v>36.18604255319149</v>
+        <v>34.90944680851064</v>
       </c>
       <c r="Q30" t="b">
         <v>0</v>
@@ -2667,22 +2667,22 @@
         <v>36.9</v>
       </c>
       <c r="D31" t="n">
-        <v>-0.1400605919366114</v>
+        <v>-0.1458333333333333</v>
       </c>
       <c r="E31" t="n">
-        <v>-0.1709728150977308</v>
+        <v>-0.1916757940854326</v>
       </c>
       <c r="F31" t="n">
-        <v>-0.1830861191056011</v>
+        <v>-0.2192128650021159</v>
       </c>
       <c r="G31" t="n">
-        <v>-0.0974826245672598</v>
+        <v>-0.1336093704637746</v>
       </c>
       <c r="H31" t="n">
-        <v>-0.0826638952765764</v>
+        <v>-0.1187906411730912</v>
       </c>
       <c r="I31" t="n">
-        <v>26.86746987951804</v>
+        <v>28.8113695090439</v>
       </c>
       <c r="J31" t="n">
         <v>20</v>
@@ -2692,7 +2692,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M31" t="n">
@@ -2732,22 +2732,22 @@
         <v>610.8</v>
       </c>
       <c r="D32" t="n">
-        <v>-0.2010986855012753</v>
+        <v>-0.191261171797418</v>
       </c>
       <c r="E32" t="n">
-        <v>-0.2512411890897947</v>
+        <v>-0.2524782768327011</v>
       </c>
       <c r="F32" t="n">
-        <v>-0.455469376838727</v>
+        <v>-0.4510649770827717</v>
       </c>
       <c r="G32" t="n">
-        <v>-0.3698658823003857</v>
+        <v>-0.3654614825444304</v>
       </c>
       <c r="H32" t="n">
-        <v>-0.3550471530097023</v>
+        <v>-0.350642753253747</v>
       </c>
       <c r="I32" t="n">
-        <v>32.94573643410853</v>
+        <v>34.18047289689559</v>
       </c>
       <c r="J32" t="n">
         <v>30</v>
@@ -2757,7 +2757,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M32" t="n">
@@ -2797,22 +2797,22 @@
         <v>513.9</v>
       </c>
       <c r="D33" t="n">
-        <v>-0.1680427391937835</v>
+        <v>-0.1474784339747843</v>
       </c>
       <c r="E33" t="n">
-        <v>-0.1588509698011294</v>
+        <v>-0.1615271659324523</v>
       </c>
       <c r="F33" t="n">
-        <v>0.0446183555239352</v>
+        <v>0.0279027902790278</v>
       </c>
       <c r="G33" t="n">
-        <v>0.1302218500622765</v>
+        <v>0.1135062848173691</v>
       </c>
       <c r="H33" t="n">
-        <v>0.1450405793529599</v>
+        <v>0.1283250141080525</v>
       </c>
       <c r="I33" t="n">
-        <v>36.24708624708624</v>
+        <v>38.44252163164401</v>
       </c>
       <c r="J33" t="n">
         <v>30</v>
@@ -2822,7 +2822,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M33" t="n">
@@ -2832,10 +2832,10 @@
         <v>30</v>
       </c>
       <c r="O33" t="n">
-        <v>80.85106382978722</v>
+        <v>78.72340425531915</v>
       </c>
       <c r="P33" t="n">
-        <v>48.16221276595745</v>
+        <v>47.73668085106383</v>
       </c>
       <c r="Q33" t="b">
         <v>0</v>
@@ -2887,7 +2887,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M34" t="n">
@@ -2927,22 +2927,22 @@
         <v>100.49</v>
       </c>
       <c r="D35" t="n">
-        <v>-0.2342452183189819</v>
+        <v>-0.2399788231734987</v>
       </c>
       <c r="E35" t="n">
-        <v>-0.0049509852460639</v>
+        <v>-0.1389031705227078</v>
       </c>
       <c r="F35" t="n">
-        <v>-0.012771392081737</v>
+        <v>-0.0174049085753398</v>
       </c>
       <c r="G35" t="n">
-        <v>0.07283210245660419</v>
+        <v>0.06819858596300141</v>
       </c>
       <c r="H35" t="n">
-        <v>0.08765083174728761</v>
+        <v>0.0830173152536848</v>
       </c>
       <c r="I35" t="n">
-        <v>37.08399366085577</v>
+        <v>37.14285714285714</v>
       </c>
       <c r="J35" t="n">
         <v>30</v>
@@ -2952,7 +2952,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M35" t="n">
@@ -2962,10 +2962,10 @@
         <v>30</v>
       </c>
       <c r="O35" t="n">
-        <v>65.95744680851064</v>
+        <v>68.08510638297872</v>
       </c>
       <c r="P35" t="n">
-        <v>44.81948936170213</v>
+        <v>45.24502127659574</v>
       </c>
       <c r="Q35" t="b">
         <v>0</v>
@@ -2992,22 +2992,22 @@
         <v>437</v>
       </c>
       <c r="D36" t="n">
-        <v>-0.1254752851711026</v>
+        <v>-0.1373864982234505</v>
       </c>
       <c r="E36" t="n">
-        <v>-0.1989000916590284</v>
+        <v>-0.1999999999999999</v>
       </c>
       <c r="F36" t="n">
-        <v>-0.0486557091542397</v>
+        <v>-0.0541125541125541</v>
       </c>
       <c r="G36" t="n">
-        <v>0.0369477853841014</v>
+        <v>0.0314909404257871</v>
       </c>
       <c r="H36" t="n">
-        <v>0.0517665146747848</v>
+        <v>0.0463096697164705</v>
       </c>
       <c r="I36" t="n">
-        <v>24.3380062305296</v>
+        <v>22.58964143426293</v>
       </c>
       <c r="J36" t="n">
         <v>20</v>
@@ -3017,7 +3017,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M36" t="n">
@@ -3057,22 +3057,22 @@
         <v>2074.5</v>
       </c>
       <c r="D37" t="n">
-        <v>-0.09370904325032769</v>
+        <v>-0.1142942532661599</v>
       </c>
       <c r="E37" t="n">
-        <v>0.2601749483659337</v>
+        <v>0.2366616989567809</v>
       </c>
       <c r="F37" t="n">
-        <v>0.5212290093128986</v>
+        <v>0.4839055793991416</v>
       </c>
       <c r="G37" t="n">
-        <v>0.6068325038512399</v>
+        <v>0.5695090739374828</v>
       </c>
       <c r="H37" t="n">
-        <v>0.6216512331419233</v>
+        <v>0.5843278032281662</v>
       </c>
       <c r="I37" t="n">
-        <v>44.29001140960482</v>
+        <v>44.60927705808609</v>
       </c>
       <c r="J37" t="n">
         <v>60</v>
@@ -3082,7 +3082,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M37" t="n">
@@ -3122,22 +3122,22 @@
         <v>708</v>
       </c>
       <c r="D38" t="n">
-        <v>-0.2565758387147582</v>
+        <v>-0.2403433476394849</v>
       </c>
       <c r="E38" t="n">
-        <v>-0.2639950101356619</v>
+        <v>-0.2650646182591997</v>
       </c>
       <c r="F38" t="n">
-        <v>-0.3304964539007092</v>
+        <v>-0.3343987966531917</v>
       </c>
       <c r="G38" t="n">
-        <v>-0.244892959362368</v>
+        <v>-0.2487953021148504</v>
       </c>
       <c r="H38" t="n">
-        <v>-0.2300742300716846</v>
+        <v>-0.233976572824167</v>
       </c>
       <c r="I38" t="n">
-        <v>32.34408602150538</v>
+        <v>33.44699777613046</v>
       </c>
       <c r="J38" t="n">
         <v>30</v>
@@ -3147,7 +3147,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M38" t="n">
@@ -3187,22 +3187,22 @@
         <v>3016.5</v>
       </c>
       <c r="D39" t="n">
-        <v>-0.0412852784134248</v>
+        <v>-0.0322114921877506</v>
       </c>
       <c r="E39" t="n">
-        <v>-0.0407975069956754</v>
+        <v>-0.0366620892281162</v>
       </c>
       <c r="F39" t="n">
-        <v>0.1704563091727458</v>
+        <v>0.1256437047540861</v>
       </c>
       <c r="G39" t="n">
-        <v>0.256059803711087</v>
+        <v>0.2112471992924274</v>
       </c>
       <c r="H39" t="n">
-        <v>0.2708785330017704</v>
+        <v>0.2260659285831108</v>
       </c>
       <c r="I39" t="n">
-        <v>49.47330512289548</v>
+        <v>48.94468704512374</v>
       </c>
       <c r="J39" t="n">
         <v>80</v>
@@ -3212,7 +3212,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M39" t="n">
@@ -3222,10 +3222,10 @@
         <v>80</v>
       </c>
       <c r="O39" t="n">
-        <v>91.48936170212764</v>
+        <v>89.36170212765957</v>
       </c>
       <c r="P39" t="n">
-        <v>69.77387234042553</v>
+        <v>69.34834042553192</v>
       </c>
       <c r="Q39" t="b">
         <v>0</v>
@@ -3252,22 +3252,22 @@
         <v>170.43</v>
       </c>
       <c r="D40" t="n">
-        <v>-0.2010968921389396</v>
+        <v>-0.2072654542071724</v>
       </c>
       <c r="E40" t="n">
-        <v>-0.0822294022617123</v>
+        <v>-0.09586206896551711</v>
       </c>
       <c r="F40" t="n">
-        <v>-0.24263431542461</v>
+        <v>-0.2931148900871008</v>
       </c>
       <c r="G40" t="n">
-        <v>-0.1570308208862687</v>
+        <v>-0.2075113955487595</v>
       </c>
       <c r="H40" t="n">
-        <v>-0.1422120915955853</v>
+        <v>-0.1926926662580761</v>
       </c>
       <c r="I40" t="n">
-        <v>33.58467802744686</v>
+        <v>30.17282384651975</v>
       </c>
       <c r="J40" t="n">
         <v>30</v>
@@ -3277,7 +3277,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M40" t="n">
@@ -3287,10 +3287,10 @@
         <v>30</v>
       </c>
       <c r="O40" t="n">
-        <v>23.40425531914894</v>
+        <v>17.02127659574468</v>
       </c>
       <c r="P40" t="n">
-        <v>34.85685106382979</v>
+        <v>33.58025531914893</v>
       </c>
       <c r="Q40" t="b">
         <v>0</v>
@@ -3317,22 +3317,22 @@
         <v>749.05</v>
       </c>
       <c r="D41" t="n">
-        <v>-0.1764608872519377</v>
+        <v>-0.1421290728969821</v>
       </c>
       <c r="E41" t="n">
-        <v>-0.2013115103694621</v>
+        <v>-0.2044078597981944</v>
       </c>
       <c r="F41" t="n">
-        <v>-0.2612919132149902</v>
+        <v>-0.2681485100146556</v>
       </c>
       <c r="G41" t="n">
-        <v>-0.1756884186766489</v>
+        <v>-0.1825450154763144</v>
       </c>
       <c r="H41" t="n">
-        <v>-0.1608696893859655</v>
+        <v>-0.167726286185631</v>
       </c>
       <c r="I41" t="n">
-        <v>16.82439537329127</v>
+        <v>17.72525849335302</v>
       </c>
       <c r="J41" t="n">
         <v>20</v>
@@ -3342,7 +3342,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M41" t="n">
@@ -3382,22 +3382,22 @@
         <v>465.05</v>
       </c>
       <c r="D42" t="n">
-        <v>-0.2665404936519201</v>
+        <v>-0.2315128480542013</v>
       </c>
       <c r="E42" t="n">
-        <v>-0.3102195194304361</v>
+        <v>-0.3104240806642941</v>
       </c>
       <c r="F42" t="n">
-        <v>-0.396822308690013</v>
+        <v>-0.3986940780967157</v>
       </c>
       <c r="G42" t="n">
-        <v>-0.3112188141516717</v>
+        <v>-0.3130905835583745</v>
       </c>
       <c r="H42" t="n">
-        <v>-0.2964000848609883</v>
+        <v>-0.2982718542676911</v>
       </c>
       <c r="I42" t="n">
-        <v>21.0904255319149</v>
+        <v>21.97893569844792</v>
       </c>
       <c r="J42" t="n">
         <v>20</v>
@@ -3407,7 +3407,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M42" t="n">
@@ -3447,22 +3447,22 @@
         <v>400.1</v>
       </c>
       <c r="D43" t="n">
-        <v>-0.0895437478666514</v>
+        <v>-0.0834955904249227</v>
       </c>
       <c r="E43" t="n">
-        <v>-0.1194982394366196</v>
+        <v>-0.1173615707037282</v>
       </c>
       <c r="F43" t="n">
-        <v>-0.1314446977097578</v>
+        <v>-0.1262284341559291</v>
       </c>
       <c r="G43" t="n">
-        <v>-0.0458412031714166</v>
+        <v>-0.0406249396175878</v>
       </c>
       <c r="H43" t="n">
-        <v>-0.0310224738807332</v>
+        <v>-0.0258062103269044</v>
       </c>
       <c r="I43" t="n">
-        <v>37.07653701380177</v>
+        <v>37.40506329113924</v>
       </c>
       <c r="J43" t="n">
         <v>30</v>
@@ -3472,7 +3472,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M43" t="n">
@@ -3512,22 +3512,22 @@
         <v>231.8</v>
       </c>
       <c r="D44" t="n">
-        <v>-0.1117072236060546</v>
+        <v>-0.1070878274268105</v>
       </c>
       <c r="E44" t="n">
-        <v>-0.1733238231098429</v>
+        <v>-0.1774308019872249</v>
       </c>
       <c r="F44" t="n">
-        <v>-0.1634788884879104</v>
+        <v>-0.2077922077922078</v>
       </c>
       <c r="G44" t="n">
-        <v>-0.0778753939495692</v>
+        <v>-0.1221887132538666</v>
       </c>
       <c r="H44" t="n">
-        <v>-0.06305666465888581</v>
+        <v>-0.1073699839631832</v>
       </c>
       <c r="I44" t="n">
-        <v>41.42212189616253</v>
+        <v>43.82089552238806</v>
       </c>
       <c r="J44" t="n">
         <v>40</v>
@@ -3537,7 +3537,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M44" t="n">
@@ -3547,10 +3547,10 @@
         <v>40</v>
       </c>
       <c r="O44" t="n">
-        <v>40.42553191489361</v>
+        <v>38.29787234042553</v>
       </c>
       <c r="P44" t="n">
-        <v>42.96510638297872</v>
+        <v>42.53957446808511</v>
       </c>
       <c r="Q44" t="b">
         <v>0</v>
@@ -3577,22 +3577,22 @@
         <v>80.68000000000001</v>
       </c>
       <c r="D45" t="n">
-        <v>-0.2593408611034609</v>
+        <v>-0.2570218252141081</v>
       </c>
       <c r="E45" t="n">
-        <v>-0.285954509248606</v>
+        <v>-0.2844345898004434</v>
       </c>
       <c r="F45" t="n">
-        <v>-0.4100614214682655</v>
+        <v>-0.4064592069447509</v>
       </c>
       <c r="G45" t="n">
-        <v>-0.3244579269299242</v>
+        <v>-0.3208557124064096</v>
       </c>
       <c r="H45" t="n">
-        <v>-0.3096391976392408</v>
+        <v>-0.3060369831157262</v>
       </c>
       <c r="I45" t="n">
-        <v>20.61482820976488</v>
+        <v>19.02858899477402</v>
       </c>
       <c r="J45" t="n">
         <v>20</v>
@@ -3602,7 +3602,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M45" t="n">
@@ -3642,22 +3642,22 @@
         <v>467.4</v>
       </c>
       <c r="D46" t="n">
-        <v>-0.1497180280152812</v>
+        <v>-0.1359645068860339</v>
       </c>
       <c r="E46" t="n">
-        <v>-0.2607354685646501</v>
+        <v>-0.2780909722758515</v>
       </c>
       <c r="F46" t="n">
-        <v>-0.2237169905331341</v>
+        <v>-0.2258385093167702</v>
       </c>
       <c r="G46" t="n">
-        <v>-0.1381134959947928</v>
+        <v>-0.1402350147784289</v>
       </c>
       <c r="H46" t="n">
-        <v>-0.1232947667041094</v>
+        <v>-0.1254162854877455</v>
       </c>
       <c r="I46" t="n">
-        <v>40.42019441831294</v>
+        <v>41.35386589669552</v>
       </c>
       <c r="J46" t="n">
         <v>40</v>
@@ -3667,7 +3667,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M46" t="n">
@@ -3677,10 +3677,10 @@
         <v>40</v>
       </c>
       <c r="O46" t="n">
-        <v>27.65957446808511</v>
+        <v>31.91489361702128</v>
       </c>
       <c r="P46" t="n">
-        <v>41.37591489361702</v>
+        <v>42.22697872340426</v>
       </c>
       <c r="Q46" t="b">
         <v>0</v>
@@ -3707,22 +3707,22 @@
         <v>997.25</v>
       </c>
       <c r="D47" t="n">
-        <v>0.1026037923599978</v>
+        <v>0.1058438678199158</v>
       </c>
       <c r="E47" t="n">
-        <v>0.1977540235407158</v>
+        <v>0.1868491520380839</v>
       </c>
       <c r="F47" t="n">
-        <v>0.3620842723485624</v>
+        <v>0.3300213390237396</v>
       </c>
       <c r="G47" t="n">
-        <v>0.4476877668869037</v>
+        <v>0.4156248335620809</v>
       </c>
       <c r="H47" t="n">
-        <v>0.4625064961775871</v>
+        <v>0.4304435628527643</v>
       </c>
       <c r="I47" t="n">
-        <v>58.16770551570036</v>
+        <v>59.49001683906664</v>
       </c>
       <c r="J47" t="n">
         <v>80</v>
@@ -3732,7 +3732,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M47" t="n">
@@ -3742,10 +3742,10 @@
         <v>80</v>
       </c>
       <c r="O47" t="n">
-        <v>93.61702127659576</v>
+        <v>95.74468085106383</v>
       </c>
       <c r="P47" t="n">
-        <v>69.45540425531915</v>
+        <v>69.88093617021276</v>
       </c>
       <c r="Q47" t="b">
         <v>0</v>
@@ -3772,22 +3772,22 @@
         <v>13768</v>
       </c>
       <c r="D48" t="n">
-        <v>-0.1120856442667355</v>
+        <v>-0.0920601424426272</v>
       </c>
       <c r="E48" t="n">
-        <v>-0.0412923891093934</v>
+        <v>-0.0336889387984278</v>
       </c>
       <c r="F48" t="n">
-        <v>0.0181172816682688</v>
+        <v>0.0051102350708132</v>
       </c>
       <c r="G48" t="n">
-        <v>0.1037207762066101</v>
+        <v>0.0907137296091544</v>
       </c>
       <c r="H48" t="n">
-        <v>0.1185395054972935</v>
+        <v>0.1055324588998378</v>
       </c>
       <c r="I48" t="n">
-        <v>45.60588463027487</v>
+        <v>45.800933125972</v>
       </c>
       <c r="J48" t="n">
         <v>40</v>
@@ -3797,7 +3797,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M48" t="n">
@@ -3807,10 +3807,10 @@
         <v>40</v>
       </c>
       <c r="O48" t="n">
-        <v>76.59574468085107</v>
+        <v>74.46808510638297</v>
       </c>
       <c r="P48" t="n">
-        <v>51.43514893617021</v>
+        <v>51.0096170212766</v>
       </c>
       <c r="Q48" t="b">
         <v>0</v>
@@ -3936,57 +3936,57 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SHRIPISTON</t>
+          <t>WHEELS</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Engine/Parts</t>
+          <t>Wheels</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>3016.5</v>
+        <v>997.25</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.0412852784134248</v>
+        <v>0.1058438678199158</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.0407975069956754</v>
+        <v>0.1868491520380839</v>
       </c>
       <c r="F2" t="n">
-        <v>0.1704563091727458</v>
+        <v>0.3300213390237396</v>
       </c>
       <c r="G2" t="n">
-        <v>0.256059803711087</v>
+        <v>0.4156248335620809</v>
       </c>
       <c r="H2" t="n">
-        <v>0.2708785330017704</v>
+        <v>0.4304435628527643</v>
       </c>
       <c r="I2" t="n">
-        <v>49.47330512289548</v>
+        <v>59.49001683906664</v>
       </c>
       <c r="J2" t="n">
         <v>80</v>
       </c>
       <c r="K2" t="n">
-        <v>48.69</v>
+        <v>46.83</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M2" t="n">
-        <v>48.69</v>
+        <v>46.83</v>
       </c>
       <c r="N2" t="n">
         <v>80</v>
       </c>
       <c r="O2" t="n">
-        <v>91.48936170212764</v>
+        <v>95.74468085106383</v>
       </c>
       <c r="P2" t="n">
-        <v>69.77387234042553</v>
+        <v>69.88093617021276</v>
       </c>
       <c r="Q2" t="b">
         <v>0</v>
@@ -4001,63 +4001,63 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>WHEELS</t>
+          <t>ASKAUTOLTD</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Wheels</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>997.25</v>
+        <v>444.75</v>
       </c>
       <c r="D3" t="n">
-        <v>0.1026037923599978</v>
+        <v>0.0707836764174791</v>
       </c>
       <c r="E3" t="n">
-        <v>0.1977540235407158</v>
+        <v>-0.0402460077686663</v>
       </c>
       <c r="F3" t="n">
-        <v>0.3620842723485624</v>
+        <v>-0.174018014671743</v>
       </c>
       <c r="G3" t="n">
-        <v>0.4476877668869037</v>
+        <v>-0.0884145201334017</v>
       </c>
       <c r="H3" t="n">
-        <v>0.4625064961775871</v>
+        <v>-0.07359579084271831</v>
       </c>
       <c r="I3" t="n">
-        <v>58.16770551570036</v>
+        <v>68.07935076645629</v>
       </c>
       <c r="J3" t="n">
         <v>80</v>
       </c>
       <c r="K3" t="n">
-        <v>46.83</v>
+        <v>71.28</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M3" t="n">
-        <v>46.83</v>
+        <v>71.28</v>
       </c>
       <c r="N3" t="n">
         <v>80</v>
       </c>
       <c r="O3" t="n">
-        <v>93.61702127659576</v>
+        <v>44.68085106382978</v>
       </c>
       <c r="P3" t="n">
-        <v>69.45540425531915</v>
+        <v>69.44817021276596</v>
       </c>
       <c r="Q3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S3" t="b">
         <v>0</v>
@@ -4066,63 +4066,63 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ASKAUTOLTD</t>
+          <t>SHRIPISTON</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Engine/Parts</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>444.75</v>
+        <v>3016.5</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0481970304030168</v>
+        <v>-0.0322114921877506</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.0331521739130434</v>
+        <v>-0.0366620892281162</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.1549496484894545</v>
+        <v>0.1256437047540861</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.06934615395111331</v>
+        <v>0.2112471992924274</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.0545274246604299</v>
+        <v>0.2260659285831108</v>
       </c>
       <c r="I4" t="n">
-        <v>70.92402464065708</v>
+        <v>48.94468704512374</v>
       </c>
       <c r="J4" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K4" t="n">
-        <v>71.28</v>
+        <v>48.69</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M4" t="n">
-        <v>71.28</v>
+        <v>48.69</v>
       </c>
       <c r="N4" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O4" t="n">
-        <v>46.80851063829788</v>
+        <v>89.36170212765957</v>
       </c>
       <c r="P4" t="n">
-        <v>65.87370212765957</v>
+        <v>69.34834042553192</v>
       </c>
       <c r="Q4" t="b">
+        <v>0</v>
+      </c>
+      <c r="R4" t="b">
         <v>1</v>
-      </c>
-      <c r="R4" t="b">
-        <v>0</v>
       </c>
       <c r="S4" t="b">
         <v>0</v>
@@ -4143,22 +4143,22 @@
         <v>2074.5</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.09370904325032769</v>
+        <v>-0.1142942532661599</v>
       </c>
       <c r="E5" t="n">
-        <v>0.2601749483659337</v>
+        <v>0.2366616989567809</v>
       </c>
       <c r="F5" t="n">
-        <v>0.5212290093128986</v>
+        <v>0.4839055793991416</v>
       </c>
       <c r="G5" t="n">
-        <v>0.6068325038512399</v>
+        <v>0.5695090739374828</v>
       </c>
       <c r="H5" t="n">
-        <v>0.6216512331419233</v>
+        <v>0.5843278032281662</v>
       </c>
       <c r="I5" t="n">
-        <v>44.29001140960482</v>
+        <v>44.60927705808609</v>
       </c>
       <c r="J5" t="n">
         <v>60</v>
@@ -4168,7 +4168,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M5" t="n">
@@ -4233,7 +4233,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M6" t="n">
@@ -4273,22 +4273,22 @@
         <v>1522.2</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.1292758265644663</v>
+        <v>-0.1338340730624786</v>
       </c>
       <c r="E7" t="n">
-        <v>0.0291393414914475</v>
+        <v>0.0300446609825417</v>
       </c>
       <c r="F7" t="n">
-        <v>0.4243473378871525</v>
+        <v>0.3264203555245732</v>
       </c>
       <c r="G7" t="n">
-        <v>0.5099508324254938</v>
+        <v>0.4120238500629145</v>
       </c>
       <c r="H7" t="n">
-        <v>0.5247695617161772</v>
+        <v>0.4268425793535979</v>
       </c>
       <c r="I7" t="n">
-        <v>51.17172493276988</v>
+        <v>53.46534653465347</v>
       </c>
       <c r="J7" t="n">
         <v>40</v>
@@ -4298,7 +4298,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M7" t="n">
@@ -4308,10 +4308,10 @@
         <v>40</v>
       </c>
       <c r="O7" t="n">
-        <v>95.74468085106383</v>
+        <v>93.61702127659576</v>
       </c>
       <c r="P7" t="n">
-        <v>56.95293617021277</v>
+        <v>56.52740425531916</v>
       </c>
       <c r="Q7" t="b">
         <v>0</v>
@@ -4338,22 +4338,22 @@
         <v>1674.6</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.124163179916318</v>
+        <v>-0.1237965676015069</v>
       </c>
       <c r="E8" t="n">
-        <v>0.2101459748518572</v>
+        <v>0.1898536308085829</v>
       </c>
       <c r="F8" t="n">
-        <v>0.4732119292689363</v>
+        <v>0.3922514133688062</v>
       </c>
       <c r="G8" t="n">
-        <v>0.5588154238072776</v>
+        <v>0.4778549079071474</v>
       </c>
       <c r="H8" t="n">
-        <v>0.573634153097961</v>
+        <v>0.4926736371978308</v>
       </c>
       <c r="I8" t="n">
-        <v>36.07973421926911</v>
+        <v>39.00161608906448</v>
       </c>
       <c r="J8" t="n">
         <v>30</v>
@@ -4363,7 +4363,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M8" t="n">
@@ -4391,57 +4391,57 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>LUMAXIND</t>
+          <t>CRAFTSMAN</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Lighting</t>
+          <t>Castings</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>4654</v>
+        <v>6977</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.2341489904392041</v>
+        <v>-0.07294711666223749</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.1699661137863385</v>
+        <v>-0.007680273076376</v>
       </c>
       <c r="F9" t="n">
-        <v>0.1235032831208962</v>
+        <v>0.0204768173175369</v>
       </c>
       <c r="G9" t="n">
-        <v>0.2091067776592374</v>
+        <v>0.1060803118558781</v>
       </c>
       <c r="H9" t="n">
-        <v>0.2239255069499208</v>
+        <v>0.1208990411465615</v>
       </c>
       <c r="I9" t="n">
-        <v>39.25653594771242</v>
+        <v>41.76706827309237</v>
       </c>
       <c r="J9" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K9" t="n">
-        <v>57.69</v>
+        <v>54.65</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M9" t="n">
-        <v>57.69</v>
+        <v>54.65</v>
       </c>
       <c r="N9" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O9" t="n">
-        <v>87.2340425531915</v>
+        <v>76.59574468085107</v>
       </c>
       <c r="P9" t="n">
-        <v>52.5228085106383</v>
+        <v>53.17914893617021</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -4456,57 +4456,57 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>LUMAXIND</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Lighting</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>481.5</v>
+        <v>4654</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.1170807738149812</v>
+        <v>-0.2302221340081708</v>
       </c>
       <c r="E10" t="n">
-        <v>0.0211006255964372</v>
+        <v>-0.1675163223325284</v>
       </c>
       <c r="F10" t="n">
-        <v>0.0915892087961913</v>
+        <v>0.114944180920895</v>
       </c>
       <c r="G10" t="n">
-        <v>0.1771927033345326</v>
+        <v>0.2005476754592363</v>
       </c>
       <c r="H10" t="n">
-        <v>0.192011432625216</v>
+        <v>0.2153664047499197</v>
       </c>
       <c r="I10" t="n">
-        <v>40.49041182018234</v>
+        <v>37.80844834797156</v>
       </c>
       <c r="J10" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K10" t="n">
-        <v>49.66</v>
+        <v>57.69</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M10" t="n">
-        <v>49.66</v>
+        <v>57.69</v>
       </c>
       <c r="N10" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O10" t="n">
-        <v>82.97872340425532</v>
+        <v>87.2340425531915</v>
       </c>
       <c r="P10" t="n">
-        <v>52.45974468085107</v>
+        <v>52.5228085106383</v>
       </c>
       <c r="Q10" t="b">
         <v>0</v>
@@ -4521,63 +4521,63 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TIINDIA</t>
+          <t>GNA</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Axles</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>2517.3</v>
+        <v>356.7</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.0746241223394478</v>
+        <v>-0.1486873508353222</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.0420868373986833</v>
+        <v>0.167021102568297</v>
       </c>
       <c r="F11" t="n">
-        <v>-0.1582625560088275</v>
+        <v>0.1361681796464404</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.0726590614704862</v>
+        <v>0.2217716741847817</v>
       </c>
       <c r="H11" t="n">
-        <v>-0.0578403321798028</v>
+        <v>0.2365904034754651</v>
       </c>
       <c r="I11" t="n">
-        <v>42.44338498212158</v>
+        <v>30.99173553719008</v>
       </c>
       <c r="J11" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="K11" t="n">
-        <v>48.73</v>
+        <v>54.47</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M11" t="n">
-        <v>48.73</v>
+        <v>54.47</v>
       </c>
       <c r="N11" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="O11" t="n">
-        <v>44.68085106382978</v>
+        <v>91.48936170212764</v>
       </c>
       <c r="P11" t="n">
-        <v>52.42817021276596</v>
+        <v>52.08587234042552</v>
       </c>
       <c r="Q11" t="b">
         <v>0</v>
       </c>
       <c r="R11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S11" t="b">
         <v>0</v>
@@ -4586,63 +4586,63 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ZFCVINDIA</t>
+          <t>TIINDIA</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Brakes/Transmission</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>13768</v>
+        <v>2517.3</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.1120856442667355</v>
+        <v>-0.0857485290913052</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.0412923891093934</v>
+        <v>-0.0504696163856511</v>
       </c>
       <c r="F12" t="n">
-        <v>0.0181172816682688</v>
+        <v>-0.1806464212479249</v>
       </c>
       <c r="G12" t="n">
-        <v>0.1037207762066101</v>
+        <v>-0.0950429267095837</v>
       </c>
       <c r="H12" t="n">
-        <v>0.1185395054972935</v>
+        <v>-0.0802241974189003</v>
       </c>
       <c r="I12" t="n">
-        <v>45.60588463027487</v>
+        <v>46.79984229202262</v>
       </c>
       <c r="J12" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K12" t="n">
-        <v>50.29</v>
+        <v>48.73</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M12" t="n">
-        <v>50.29</v>
+        <v>48.73</v>
       </c>
       <c r="N12" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O12" t="n">
-        <v>76.59574468085107</v>
+        <v>42.5531914893617</v>
       </c>
       <c r="P12" t="n">
-        <v>51.43514893617021</v>
+        <v>52.00263829787234</v>
       </c>
       <c r="Q12" t="b">
         <v>0</v>
       </c>
       <c r="R12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S12" t="b">
         <v>0</v>
@@ -4651,57 +4651,57 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MINDACORP</t>
+          <t>ZFCVINDIA</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Brakes/Transmission</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>505.65</v>
+        <v>13768</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.1166914140973012</v>
+        <v>-0.0920601424426272</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.1371160409556314</v>
+        <v>-0.0336889387984278</v>
       </c>
       <c r="F13" t="n">
-        <v>0.0032738095238094</v>
+        <v>0.0051102350708132</v>
       </c>
       <c r="G13" t="n">
-        <v>0.08887730406215059</v>
+        <v>0.0907137296091544</v>
       </c>
       <c r="H13" t="n">
-        <v>0.103696033352834</v>
+        <v>0.1055324588998378</v>
       </c>
       <c r="I13" t="n">
-        <v>49.5638629283489</v>
+        <v>45.800933125972</v>
       </c>
       <c r="J13" t="n">
         <v>40</v>
       </c>
       <c r="K13" t="n">
-        <v>49.42</v>
+        <v>50.29</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M13" t="n">
-        <v>49.42</v>
+        <v>50.29</v>
       </c>
       <c r="N13" t="n">
         <v>40</v>
       </c>
       <c r="O13" t="n">
-        <v>72.3404255319149</v>
+        <v>74.46808510638297</v>
       </c>
       <c r="P13" t="n">
-        <v>50.23608510638298</v>
+        <v>51.0096170212766</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
@@ -4716,57 +4716,57 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CRAFTSMAN</t>
+          <t>MINDACORP</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Castings</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>6977</v>
+        <v>505.65</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.1002643626281514</v>
+        <v>-0.08982089820898199</v>
       </c>
       <c r="E14" t="n">
-        <v>0.0007171543316122</v>
+        <v>-0.1342350826127899</v>
       </c>
       <c r="F14" t="n">
-        <v>0.0120394545982014</v>
+        <v>-0.0287168651555898</v>
       </c>
       <c r="G14" t="n">
-        <v>0.0976429491365427</v>
+        <v>0.0568866293827514</v>
       </c>
       <c r="H14" t="n">
-        <v>0.1124616784272261</v>
+        <v>0.0717053586734348</v>
       </c>
       <c r="I14" t="n">
-        <v>39.96383363471971</v>
+        <v>53.85917400135408</v>
       </c>
       <c r="J14" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K14" t="n">
-        <v>54.65</v>
+        <v>49.42</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M14" t="n">
-        <v>54.65</v>
+        <v>49.42</v>
       </c>
       <c r="N14" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O14" t="n">
-        <v>74.46808510638297</v>
+        <v>65.95744680851064</v>
       </c>
       <c r="P14" t="n">
-        <v>48.7536170212766</v>
+        <v>48.95948936170213</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
@@ -4781,7 +4781,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PRICOLLTD</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -4790,48 +4790,48 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>513.9</v>
+        <v>481.5</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.1680427391937835</v>
+        <v>-0.0991580916744621</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.1588509698011294</v>
+        <v>-0.0034150884818379</v>
       </c>
       <c r="F15" t="n">
-        <v>0.0446183555239352</v>
+        <v>0.059755694948828</v>
       </c>
       <c r="G15" t="n">
-        <v>0.1302218500622765</v>
+        <v>0.1453591894871693</v>
       </c>
       <c r="H15" t="n">
-        <v>0.1450405793529599</v>
+        <v>0.1601779187778527</v>
       </c>
       <c r="I15" t="n">
-        <v>36.24708624708624</v>
+        <v>38.7180317254775</v>
       </c>
       <c r="J15" t="n">
         <v>30</v>
       </c>
       <c r="K15" t="n">
-        <v>49.98</v>
+        <v>49.66</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M15" t="n">
-        <v>49.98</v>
+        <v>49.66</v>
       </c>
       <c r="N15" t="n">
         <v>30</v>
       </c>
       <c r="O15" t="n">
-        <v>80.85106382978722</v>
+        <v>82.97872340425532</v>
       </c>
       <c r="P15" t="n">
-        <v>48.16221276595745</v>
+        <v>48.45974468085107</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
@@ -4846,63 +4846,63 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>GNA</t>
+          <t>JBMA</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Axles</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>356.7</v>
+        <v>515.25</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.1540377090003557</v>
+        <v>-0.06547565067561439</v>
       </c>
       <c r="E16" t="n">
-        <v>0.1714285714285714</v>
+        <v>-0.0882951428824205</v>
       </c>
       <c r="F16" t="n">
-        <v>0.1581168831168831</v>
+        <v>-0.1726878612716762</v>
       </c>
       <c r="G16" t="n">
-        <v>0.2437203776552243</v>
+        <v>-0.0870843667333349</v>
       </c>
       <c r="H16" t="n">
-        <v>0.2585391069459077</v>
+        <v>-0.07226563744265151</v>
       </c>
       <c r="I16" t="n">
-        <v>29.85499004833665</v>
+        <v>50.56932350971199</v>
       </c>
       <c r="J16" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="K16" t="n">
-        <v>54.47</v>
+        <v>56.91</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M16" t="n">
-        <v>54.47</v>
+        <v>56.91</v>
       </c>
       <c r="N16" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="O16" t="n">
-        <v>89.36170212765957</v>
+        <v>46.80851063829788</v>
       </c>
       <c r="P16" t="n">
-        <v>47.66034042553191</v>
+        <v>48.12570212765957</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>
       </c>
       <c r="R16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S16" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
chore: auto-refresh NSE data and pipeline outputs (2026-04-01)
</commit_message>
<xml_diff>
--- a/working-sector/output/auto_components_comprehensive_report.xlsx
+++ b/working-sector/output/auto_components_comprehensive_report.xlsx
@@ -435,7 +435,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
     </row>
@@ -447,7 +447,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
     </row>
@@ -779,25 +779,25 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1674.6</v>
+        <v>1668.4</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.1237965676015069</v>
+        <v>-0.1122226360879049</v>
       </c>
       <c r="E2" t="n">
-        <v>0.1898536308085829</v>
+        <v>0.1694939015841863</v>
       </c>
       <c r="F2" t="n">
-        <v>0.3922514133688062</v>
+        <v>0.4118642633494118</v>
       </c>
       <c r="G2" t="n">
-        <v>0.4778549079071474</v>
+        <v>0.4974677578877531</v>
       </c>
       <c r="H2" t="n">
-        <v>0.4926736371978308</v>
+        <v>0.5122864871784365</v>
       </c>
       <c r="I2" t="n">
-        <v>39.00161608906448</v>
+        <v>39.8093841642229</v>
       </c>
       <c r="J2" t="n">
         <v>30</v>
@@ -807,7 +807,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M2" t="n">
@@ -844,25 +844,25 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1031.6</v>
+        <v>1043.4</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.132015145140934</v>
+        <v>-0.08505787443002449</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.1646287148756985</v>
+        <v>-0.164009294127073</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.2124589663333079</v>
+        <v>-0.1873198847262247</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.1268554717949667</v>
+        <v>-0.1017163901878834</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.1120367425042833</v>
+        <v>-0.0868976608972</v>
       </c>
       <c r="I3" t="n">
-        <v>42.66900790166812</v>
+        <v>46.31207757860712</v>
       </c>
       <c r="J3" t="n">
         <v>40</v>
@@ -872,7 +872,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M3" t="n">
@@ -882,10 +882,10 @@
         <v>40</v>
       </c>
       <c r="O3" t="n">
-        <v>36.17021276595745</v>
+        <v>40.42553191489361</v>
       </c>
       <c r="P3" t="n">
-        <v>42.97804255319149</v>
+        <v>43.82910638297872</v>
       </c>
       <c r="Q3" t="b">
         <v>0</v>
@@ -909,48 +909,48 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>28745</v>
+        <v>30635</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.210844200411805</v>
+        <v>-0.1338705117331071</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.2205802603036876</v>
+        <v>-0.1655998910527032</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.3049208076411558</v>
+        <v>-0.2617182793107603</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.2193173131028145</v>
+        <v>-0.176114784772419</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.2044985838121311</v>
+        <v>-0.1612960554817356</v>
       </c>
       <c r="I4" t="n">
-        <v>30.53735255570118</v>
+        <v>46.32272228320527</v>
       </c>
       <c r="J4" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K4" t="n">
         <v>53.48</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M4" t="n">
         <v>53.48</v>
       </c>
       <c r="N4" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O4" t="n">
-        <v>14.8936170212766</v>
+        <v>19.14893617021277</v>
       </c>
       <c r="P4" t="n">
-        <v>36.37072340425532</v>
+        <v>41.22178723404255</v>
       </c>
       <c r="Q4" t="b">
         <v>0</v>
@@ -974,48 +974,48 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>287.9</v>
+        <v>299.85</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.1387974872868681</v>
+        <v>-0.0710966542750929</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.2314468766684464</v>
+        <v>-0.1977257525083611</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.3263133263133264</v>
+        <v>-0.2973637961335675</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.2407098317749851</v>
+        <v>-0.2117603015952263</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.2258911024843017</v>
+        <v>-0.1969415723045429</v>
       </c>
       <c r="I5" t="n">
-        <v>36.15023474178401</v>
+        <v>44.69419759539991</v>
       </c>
       <c r="J5" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K5" t="n">
         <v>51.12</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M5" t="n">
         <v>51.12</v>
       </c>
       <c r="N5" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O5" t="n">
-        <v>10.63829787234042</v>
+        <v>14.8936170212766</v>
       </c>
       <c r="P5" t="n">
-        <v>34.57565957446808</v>
+        <v>39.42672340425532</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
@@ -1039,48 +1039,48 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>105.08</v>
+        <v>107.62</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.2119394030298486</v>
+        <v>-0.1634667703070346</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.1228714524207011</v>
+        <v>-0.1127782357790601</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0660444354266005</v>
+        <v>0.08905079943331309</v>
       </c>
       <c r="G6" t="n">
-        <v>0.1516479299649418</v>
+        <v>0.1746542939716544</v>
       </c>
       <c r="H6" t="n">
-        <v>0.1664666592556252</v>
+        <v>0.1894730232623378</v>
       </c>
       <c r="I6" t="n">
-        <v>28.7131297311407</v>
+        <v>34.16603583144084</v>
       </c>
       <c r="J6" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="K6" t="n">
         <v>51.57</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M6" t="n">
         <v>51.57</v>
       </c>
       <c r="N6" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="O6" t="n">
-        <v>85.1063829787234</v>
+        <v>80.85106382978722</v>
       </c>
       <c r="P6" t="n">
-        <v>45.64927659574468</v>
+        <v>48.79821276595744</v>
       </c>
       <c r="Q6" t="b">
         <v>0</v>
@@ -1104,48 +1104,48 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2517.3</v>
+        <v>2572.7</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.0857485290913052</v>
+        <v>-0.0933535382012968</v>
       </c>
       <c r="E7" t="n">
-        <v>-0.0504696163856511</v>
+        <v>-0.0312170507606567</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.1806464212479249</v>
+        <v>-0.183658575281612</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.0950429267095837</v>
+        <v>-0.0980550807432707</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.0802241974189003</v>
+        <v>-0.0832363514525873</v>
       </c>
       <c r="I7" t="n">
-        <v>46.79984229202262</v>
+        <v>51.4375</v>
       </c>
       <c r="J7" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K7" t="n">
         <v>48.73</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M7" t="n">
         <v>48.73</v>
       </c>
       <c r="N7" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O7" t="n">
         <v>42.5531914893617</v>
       </c>
       <c r="P7" t="n">
-        <v>52.00263829787234</v>
+        <v>60.00263829787234</v>
       </c>
       <c r="Q7" t="b">
         <v>0</v>
@@ -1169,48 +1169,48 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>481.5</v>
+        <v>497.25</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.0991580916744621</v>
+        <v>-0.0386660222329627</v>
       </c>
       <c r="E8" t="n">
-        <v>-0.0034150884818379</v>
+        <v>0.0096446700507615</v>
       </c>
       <c r="F8" t="n">
-        <v>0.059755694948828</v>
+        <v>0.1161616161616161</v>
       </c>
       <c r="G8" t="n">
-        <v>0.1453591894871693</v>
+        <v>0.2017651106999574</v>
       </c>
       <c r="H8" t="n">
-        <v>0.1601779187778527</v>
+        <v>0.2165838399906408</v>
       </c>
       <c r="I8" t="n">
-        <v>38.7180317254775</v>
+        <v>46.02497715504112</v>
       </c>
       <c r="J8" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K8" t="n">
         <v>49.66</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M8" t="n">
         <v>49.66</v>
       </c>
       <c r="N8" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O8" t="n">
-        <v>82.97872340425532</v>
+        <v>85.1063829787234</v>
       </c>
       <c r="P8" t="n">
-        <v>48.45974468085107</v>
+        <v>52.88527659574468</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
@@ -1234,48 +1234,48 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>412.3</v>
+        <v>415.25</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.0919502257460631</v>
+        <v>-0.0571071752951861</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.1980159502042404</v>
+        <v>-0.1857843137254902</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.1410416666666666</v>
+        <v>-0.1374117158288325</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.0554381721283253</v>
+        <v>-0.0518082212904912</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.0406194428376419</v>
+        <v>-0.0369894919998078</v>
       </c>
       <c r="I9" t="n">
-        <v>39.8707891093678</v>
+        <v>48.73284054910245</v>
       </c>
       <c r="J9" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K9" t="n">
         <v>53.44</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M9" t="n">
         <v>53.44</v>
       </c>
       <c r="N9" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O9" t="n">
-        <v>48.93617021276596</v>
+        <v>44.68085106382978</v>
       </c>
       <c r="P9" t="n">
-        <v>43.1632340425532</v>
+        <v>46.31217021276596</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -1299,25 +1299,25 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>128495</v>
+        <v>129095</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.088590984856545</v>
+        <v>-0.0700882405906717</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.1632261005470174</v>
+        <v>-0.1537528679121599</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.1263301036885942</v>
+        <v>-0.1354184107423902</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.0407266091502529</v>
+        <v>-0.0498149162040489</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.0259078798595695</v>
+        <v>-0.0349961869133655</v>
       </c>
       <c r="I10" t="n">
-        <v>34.05916187345933</v>
+        <v>30.78913324708927</v>
       </c>
       <c r="J10" t="n">
         <v>30</v>
@@ -1327,7 +1327,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M10" t="n">
@@ -1337,10 +1337,10 @@
         <v>30</v>
       </c>
       <c r="O10" t="n">
-        <v>51.06382978723404</v>
+        <v>46.80851063829788</v>
       </c>
       <c r="P10" t="n">
-        <v>41.97676595744681</v>
+        <v>41.12570212765957</v>
       </c>
       <c r="Q10" t="b">
         <v>0</v>
@@ -1392,7 +1392,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M11" t="n">
@@ -1402,10 +1402,10 @@
         <v>20</v>
       </c>
       <c r="O11" t="n">
-        <v>70.21276595744681</v>
+        <v>63.82978723404256</v>
       </c>
       <c r="P11" t="n">
-        <v>26.04255319148936</v>
+        <v>24.76595744680852</v>
       </c>
       <c r="Q11" t="b">
         <v>0</v>
@@ -1429,25 +1429,25 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>444.75</v>
+        <v>435.7</v>
       </c>
       <c r="D12" t="n">
-        <v>0.0707836764174791</v>
+        <v>0.0889777555611095</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.0402460077686663</v>
+        <v>-0.06431869429829271</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.174018014671743</v>
+        <v>-0.1885650433001211</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.0884145201334017</v>
+        <v>-0.1029615487617798</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.07359579084271831</v>
+        <v>-0.0881428194710964</v>
       </c>
       <c r="I12" t="n">
-        <v>68.07935076645629</v>
+        <v>62.39424703891709</v>
       </c>
       <c r="J12" t="n">
         <v>80</v>
@@ -1457,7 +1457,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M12" t="n">
@@ -1467,10 +1467,10 @@
         <v>80</v>
       </c>
       <c r="O12" t="n">
-        <v>44.68085106382978</v>
+        <v>38.29787234042553</v>
       </c>
       <c r="P12" t="n">
-        <v>69.44817021276596</v>
+        <v>68.17157446808511</v>
       </c>
       <c r="Q12" t="b">
         <v>1</v>
@@ -1494,48 +1494,48 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1547.1</v>
+        <v>1623.6</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.2437307523097228</v>
+        <v>-0.190950767390871</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.1586818206536517</v>
+        <v>-0.131950384944397</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.0912775330396475</v>
+        <v>-0.054397204426325</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.0056740385013063</v>
+        <v>0.0312062901120162</v>
       </c>
       <c r="H13" t="n">
-        <v>0.009144690789377</v>
+        <v>0.0460250194026996</v>
       </c>
       <c r="I13" t="n">
-        <v>19.14743702659856</v>
+        <v>32.51404494382022</v>
       </c>
       <c r="J13" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="K13" t="n">
         <v>58.77</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M13" t="n">
         <v>58.77</v>
       </c>
       <c r="N13" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="O13" t="n">
-        <v>59.57446808510638</v>
+        <v>57.44680851063831</v>
       </c>
       <c r="P13" t="n">
-        <v>43.42289361702128</v>
+        <v>46.99736170212766</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
@@ -1559,48 +1559,48 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>504.35</v>
+        <v>539.65</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.1903844610321855</v>
+        <v>-0.0908861185983828</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.2867345495686607</v>
+        <v>-0.240624780130866</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.2022933965994463</v>
+        <v>-0.13036822173878</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.116689902061105</v>
+        <v>-0.0447647272004387</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.1018711727704216</v>
+        <v>-0.0299459979097553</v>
       </c>
       <c r="I14" t="n">
-        <v>32.83832335329343</v>
+        <v>42.6839293053843</v>
       </c>
       <c r="J14" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K14" t="n">
         <v>54.64</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M14" t="n">
         <v>54.64</v>
       </c>
       <c r="N14" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O14" t="n">
-        <v>40.42553191489361</v>
+        <v>48.93617021276596</v>
       </c>
       <c r="P14" t="n">
-        <v>41.94110638297872</v>
+        <v>47.6432340425532</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
@@ -1624,48 +1624,48 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>86.22</v>
+        <v>90.78</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.1924697948862039</v>
+        <v>-0.1249277038750722</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.2105118578884717</v>
+        <v>-0.1415602836879432</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.0038128249566724</v>
+        <v>0.0273879583521956</v>
       </c>
       <c r="G15" t="n">
-        <v>0.08179066958166881</v>
+        <v>0.1129914528905369</v>
       </c>
       <c r="H15" t="n">
-        <v>0.0966093988723522</v>
+        <v>0.1278101821812203</v>
       </c>
       <c r="I15" t="n">
-        <v>28.62149532710282</v>
+        <v>39.73436635307139</v>
       </c>
       <c r="J15" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="K15" t="n">
         <v>51.91</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M15" t="n">
         <v>51.91</v>
       </c>
       <c r="N15" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="O15" t="n">
         <v>72.3404255319149</v>
       </c>
       <c r="P15" t="n">
-        <v>43.23208510638298</v>
+        <v>47.23208510638297</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
@@ -1689,48 +1689,48 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>140.81</v>
+        <v>155.84</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.2591676750670805</v>
+        <v>-0.1383866865704649</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.1727278068268609</v>
+        <v>-0.1245927423884957</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.0876635998444991</v>
+        <v>-0.0333705495596079</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.0020601053061578</v>
+        <v>0.0522329449787333</v>
       </c>
       <c r="H16" t="n">
-        <v>0.0127586239845255</v>
+        <v>0.0670516742694167</v>
       </c>
       <c r="I16" t="n">
-        <v>28.28784119106699</v>
+        <v>41.96670995159958</v>
       </c>
       <c r="J16" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="K16" t="n">
         <v>52.61</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M16" t="n">
         <v>52.61</v>
       </c>
       <c r="N16" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="O16" t="n">
         <v>61.70212765957447</v>
       </c>
       <c r="P16" t="n">
-        <v>41.38442553191489</v>
+        <v>49.38442553191489</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>
@@ -1754,48 +1754,48 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>6977</v>
+        <v>6838</v>
       </c>
       <c r="D17" t="n">
-        <v>-0.07294711666223749</v>
+        <v>-0.1081838930551026</v>
       </c>
       <c r="E17" t="n">
-        <v>-0.007680273076376</v>
+        <v>-0.0253705815279361</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0204768173175369</v>
+        <v>0.0095224034841663</v>
       </c>
       <c r="G17" t="n">
-        <v>0.1060803118558781</v>
+        <v>0.09512589802250759</v>
       </c>
       <c r="H17" t="n">
-        <v>0.1208990411465615</v>
+        <v>0.1099446273131909</v>
       </c>
       <c r="I17" t="n">
-        <v>41.76706827309237</v>
+        <v>38.41490794791199</v>
       </c>
       <c r="J17" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K17" t="n">
         <v>54.65</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M17" t="n">
         <v>54.65</v>
       </c>
       <c r="N17" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O17" t="n">
-        <v>76.59574468085107</v>
+        <v>70.21276595744681</v>
       </c>
       <c r="P17" t="n">
-        <v>53.17914893617021</v>
+        <v>47.90255319148936</v>
       </c>
       <c r="Q17" t="b">
         <v>0</v>
@@ -1819,25 +1819,25 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>615.8</v>
+        <v>631.85</v>
       </c>
       <c r="D18" t="n">
-        <v>-0.147386638975424</v>
+        <v>-0.0540459615240661</v>
       </c>
       <c r="E18" t="n">
-        <v>0.0355671403346506</v>
+        <v>0.06461668070766639</v>
       </c>
       <c r="F18" t="n">
-        <v>-0.0946114827611557</v>
+        <v>-0.0445334946317858</v>
       </c>
       <c r="G18" t="n">
-        <v>-0.0090079882228144</v>
+        <v>0.0410699999065554</v>
       </c>
       <c r="H18" t="n">
-        <v>0.0058107410678689</v>
+        <v>0.0558887291972388</v>
       </c>
       <c r="I18" t="n">
-        <v>32.1220203367228</v>
+        <v>36.88269073010667</v>
       </c>
       <c r="J18" t="n">
         <v>30</v>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M18" t="n">
@@ -1857,10 +1857,10 @@
         <v>30</v>
       </c>
       <c r="O18" t="n">
-        <v>57.44680851063831</v>
+        <v>59.57446808510638</v>
       </c>
       <c r="P18" t="n">
-        <v>43.45736170212766</v>
+        <v>43.88289361702128</v>
       </c>
       <c r="Q18" t="b">
         <v>0</v>
@@ -1884,48 +1884,48 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2213.9</v>
+        <v>2252</v>
       </c>
       <c r="D19" t="n">
-        <v>-0.1682383439155426</v>
+        <v>-0.1515014505858859</v>
       </c>
       <c r="E19" t="n">
-        <v>-0.1350939563230064</v>
+        <v>-0.1471958192903396</v>
       </c>
       <c r="F19" t="n">
-        <v>-0.2633102622121654</v>
+        <v>-0.2445994901381993</v>
       </c>
       <c r="G19" t="n">
-        <v>-0.1777067676738242</v>
+        <v>-0.1589959955998581</v>
       </c>
       <c r="H19" t="n">
-        <v>-0.1628880383831408</v>
+        <v>-0.1441772663091747</v>
       </c>
       <c r="I19" t="n">
-        <v>27.25901089689862</v>
+        <v>32.90703393999017</v>
       </c>
       <c r="J19" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="K19" t="n">
         <v>51.27</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M19" t="n">
         <v>51.27</v>
       </c>
       <c r="N19" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="O19" t="n">
         <v>21.27659574468085</v>
       </c>
       <c r="P19" t="n">
-        <v>32.76331914893618</v>
+        <v>36.76331914893618</v>
       </c>
       <c r="Q19" t="b">
         <v>0</v>
@@ -1949,54 +1949,54 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>1910.9</v>
+        <v>1974.7</v>
       </c>
       <c r="D20" t="n">
-        <v>-0.1220307833677922</v>
+        <v>-0.09230062054700069</v>
       </c>
       <c r="E20" t="n">
-        <v>-0.1591939103269238</v>
+        <v>-0.1405005440696408</v>
       </c>
       <c r="F20" t="n">
-        <v>-0.1192385693215338</v>
+        <v>-0.095460583573817</v>
       </c>
       <c r="G20" t="n">
-        <v>-0.0336350747831926</v>
+        <v>-0.0098570890354757</v>
       </c>
       <c r="H20" t="n">
-        <v>-0.0188163454925092</v>
+        <v>0.0049616402552076</v>
       </c>
       <c r="I20" t="n">
-        <v>35.07751937984497</v>
+        <v>41.24948282995449</v>
       </c>
       <c r="J20" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K20" t="n">
         <v>49.06</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M20" t="n">
         <v>49.06</v>
       </c>
       <c r="N20" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O20" t="n">
-        <v>55.31914893617022</v>
+        <v>53.19148936170212</v>
       </c>
       <c r="P20" t="n">
-        <v>42.68782978723405</v>
+        <v>46.26229787234043</v>
       </c>
       <c r="Q20" t="b">
         <v>0</v>
       </c>
       <c r="R20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S20" t="b">
         <v>0</v>
@@ -2014,48 +2014,48 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>826.35</v>
+        <v>866.2</v>
       </c>
       <c r="D21" t="n">
-        <v>-0.1726571886263516</v>
+        <v>-0.0916050547952387</v>
       </c>
       <c r="E21" t="n">
-        <v>-0.1417220606564186</v>
+        <v>-0.1047028423772609</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.3232740971255424</v>
+        <v>-0.3118843342866221</v>
       </c>
       <c r="G21" t="n">
-        <v>-0.2376706025872011</v>
+        <v>-0.2262808397482808</v>
       </c>
       <c r="H21" t="n">
-        <v>-0.2228518732965178</v>
+        <v>-0.2114621104575974</v>
       </c>
       <c r="I21" t="n">
-        <v>40.18024145553478</v>
+        <v>47.93689320388352</v>
       </c>
       <c r="J21" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K21" t="n">
         <v>48.43</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M21" t="n">
         <v>48.43</v>
       </c>
       <c r="N21" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O21" t="n">
-        <v>12.76595744680851</v>
+        <v>8.51063829787234</v>
       </c>
       <c r="P21" t="n">
-        <v>37.9251914893617</v>
+        <v>45.07412765957447</v>
       </c>
       <c r="Q21" t="b">
         <v>0</v>
@@ -2079,25 +2079,25 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>356.7</v>
+        <v>378.45</v>
       </c>
       <c r="D22" t="n">
-        <v>-0.1486873508353222</v>
+        <v>-0.1175236096537251</v>
       </c>
       <c r="E22" t="n">
-        <v>0.167021102568297</v>
+        <v>0.2455158795458283</v>
       </c>
       <c r="F22" t="n">
-        <v>0.1361681796464404</v>
+        <v>0.2012378987462306</v>
       </c>
       <c r="G22" t="n">
-        <v>0.2217716741847817</v>
+        <v>0.2868413932845719</v>
       </c>
       <c r="H22" t="n">
-        <v>0.2365904034754651</v>
+        <v>0.3016601225752553</v>
       </c>
       <c r="I22" t="n">
-        <v>30.99173553719008</v>
+        <v>39.91935483870968</v>
       </c>
       <c r="J22" t="n">
         <v>30</v>
@@ -2107,7 +2107,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M22" t="n">
@@ -2144,48 +2144,48 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>314.25</v>
+        <v>330.85</v>
       </c>
       <c r="D23" t="n">
-        <v>-0.1496414558246516</v>
+        <v>-0.0775128955806495</v>
       </c>
       <c r="E23" t="n">
-        <v>-0.1480276535176902</v>
+        <v>-0.1134780278670952</v>
       </c>
       <c r="F23" t="n">
-        <v>-0.2276972229048905</v>
+        <v>-0.1961856171039844</v>
       </c>
       <c r="G23" t="n">
-        <v>-0.1420937283665493</v>
+        <v>-0.1105821225656431</v>
       </c>
       <c r="H23" t="n">
-        <v>-0.1272749990758659</v>
+        <v>-0.0957633932749597</v>
       </c>
       <c r="I23" t="n">
-        <v>19.20777279521669</v>
+        <v>35.56763285024155</v>
       </c>
       <c r="J23" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="K23" t="n">
         <v>49.7</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M23" t="n">
         <v>49.7</v>
       </c>
       <c r="N23" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="O23" t="n">
-        <v>27.65957446808511</v>
+        <v>34.04255319148936</v>
       </c>
       <c r="P23" t="n">
-        <v>33.41191489361702</v>
+        <v>38.68851063829788</v>
       </c>
       <c r="Q23" t="b">
         <v>0</v>
@@ -2209,48 +2209,48 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>111.92</v>
+        <v>119.95</v>
       </c>
       <c r="D24" t="n">
-        <v>-0.2408600691853761</v>
+        <v>-0.1636452377632128</v>
       </c>
       <c r="E24" t="n">
-        <v>-0.1084202979367482</v>
+        <v>-0.038785159067233</v>
       </c>
       <c r="F24" t="n">
-        <v>0.0512868683073455</v>
+        <v>0.09144676979071879</v>
       </c>
       <c r="G24" t="n">
-        <v>0.1368903628456867</v>
+        <v>0.1770502643290601</v>
       </c>
       <c r="H24" t="n">
-        <v>0.1517090921363701</v>
+        <v>0.1918689936197435</v>
       </c>
       <c r="I24" t="n">
-        <v>37.34939759036145</v>
+        <v>47.70744384629664</v>
       </c>
       <c r="J24" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K24" t="n">
         <v>48.3</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M24" t="n">
         <v>48.3</v>
       </c>
       <c r="N24" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O24" t="n">
-        <v>80.85106382978722</v>
+        <v>82.97872340425532</v>
       </c>
       <c r="P24" t="n">
-        <v>47.49021276595744</v>
+        <v>51.91574468085106</v>
       </c>
       <c r="Q24" t="b">
         <v>0</v>
@@ -2274,48 +2274,48 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>515.25</v>
+        <v>561.1</v>
       </c>
       <c r="D25" t="n">
-        <v>-0.06547565067561439</v>
+        <v>0.0641001327517543</v>
       </c>
       <c r="E25" t="n">
-        <v>-0.0882951428824205</v>
+        <v>-0.0170797932907068</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.1726878612716762</v>
+        <v>-0.1047467092142001</v>
       </c>
       <c r="G25" t="n">
-        <v>-0.0870843667333349</v>
+        <v>-0.0191432146758588</v>
       </c>
       <c r="H25" t="n">
-        <v>-0.07226563744265151</v>
+        <v>-0.0043244853851754</v>
       </c>
       <c r="I25" t="n">
-        <v>50.56932350971199</v>
+        <v>56.87363038714392</v>
       </c>
       <c r="J25" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="K25" t="n">
         <v>56.91</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M25" t="n">
         <v>56.91</v>
       </c>
       <c r="N25" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="O25" t="n">
-        <v>46.80851063829788</v>
+        <v>51.06382978723404</v>
       </c>
       <c r="P25" t="n">
-        <v>48.12570212765957</v>
+        <v>64.9767659574468</v>
       </c>
       <c r="Q25" t="b">
         <v>0</v>
@@ -2339,48 +2339,48 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>117.55</v>
+        <v>125.34</v>
       </c>
       <c r="D26" t="n">
-        <v>-0.21255359056806</v>
+        <v>-0.0956057435601414</v>
       </c>
       <c r="E26" t="n">
-        <v>-0.1915405777166438</v>
+        <v>-0.1258804658623333</v>
       </c>
       <c r="F26" t="n">
-        <v>-0.2586870151983351</v>
+        <v>-0.3110915686490051</v>
       </c>
       <c r="G26" t="n">
-        <v>-0.1730835206599938</v>
+        <v>-0.2254880741106638</v>
       </c>
       <c r="H26" t="n">
-        <v>-0.1582647913693105</v>
+        <v>-0.2106693448199804</v>
       </c>
       <c r="I26" t="n">
-        <v>23.59164998570205</v>
+        <v>38.27248866618948</v>
       </c>
       <c r="J26" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="K26" t="n">
         <v>51.54</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M26" t="n">
         <v>51.54</v>
       </c>
       <c r="N26" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="O26" t="n">
-        <v>23.40425531914894</v>
+        <v>10.63829787234042</v>
       </c>
       <c r="P26" t="n">
-        <v>33.29685106382978</v>
+        <v>34.74365957446808</v>
       </c>
       <c r="Q26" t="b">
         <v>0</v>
@@ -2404,48 +2404,48 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>4654</v>
+        <v>4805.4</v>
       </c>
       <c r="D27" t="n">
-        <v>-0.2302221340081708</v>
+        <v>-0.1923697478991597</v>
       </c>
       <c r="E27" t="n">
-        <v>-0.1675163223325284</v>
+        <v>-0.1256550218340612</v>
       </c>
       <c r="F27" t="n">
-        <v>0.114944180920895</v>
+        <v>0.1459436256975246</v>
       </c>
       <c r="G27" t="n">
-        <v>0.2005476754592363</v>
+        <v>0.2315471202358658</v>
       </c>
       <c r="H27" t="n">
-        <v>0.2153664047499197</v>
+        <v>0.2463658495265492</v>
       </c>
       <c r="I27" t="n">
-        <v>37.80844834797156</v>
+        <v>46.77362169828044</v>
       </c>
       <c r="J27" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K27" t="n">
         <v>57.69</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M27" t="n">
         <v>57.69</v>
       </c>
       <c r="N27" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O27" t="n">
-        <v>87.2340425531915</v>
+        <v>89.36170212765957</v>
       </c>
       <c r="P27" t="n">
-        <v>52.5228085106383</v>
+        <v>56.94834042553191</v>
       </c>
       <c r="Q27" t="b">
         <v>0</v>
@@ -2469,48 +2469,48 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1522.2</v>
+        <v>1593.5</v>
       </c>
       <c r="D28" t="n">
-        <v>-0.1338340730624786</v>
+        <v>-0.0423102349900835</v>
       </c>
       <c r="E28" t="n">
-        <v>0.0300446609825417</v>
+        <v>0.07574427867413749</v>
       </c>
       <c r="F28" t="n">
-        <v>0.3264203555245732</v>
+        <v>0.3990342405618963</v>
       </c>
       <c r="G28" t="n">
-        <v>0.4120238500629145</v>
+        <v>0.4846377351002375</v>
       </c>
       <c r="H28" t="n">
-        <v>0.4268425793535979</v>
+        <v>0.4994564643909209</v>
       </c>
       <c r="I28" t="n">
-        <v>53.46534653465347</v>
+        <v>63.56641468682506</v>
       </c>
       <c r="J28" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="K28" t="n">
         <v>54.51</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M28" t="n">
         <v>54.51</v>
       </c>
       <c r="N28" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="O28" t="n">
-        <v>93.61702127659576</v>
+        <v>95.74468085106383</v>
       </c>
       <c r="P28" t="n">
-        <v>56.52740425531916</v>
+        <v>72.95293617021277</v>
       </c>
       <c r="Q28" t="b">
         <v>0</v>
@@ -2534,48 +2534,48 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>505.65</v>
+        <v>514.15</v>
       </c>
       <c r="D29" t="n">
-        <v>-0.08982089820898199</v>
+        <v>-0.0492788461538461</v>
       </c>
       <c r="E29" t="n">
-        <v>-0.1342350826127899</v>
+        <v>-0.1210359859817079</v>
       </c>
       <c r="F29" t="n">
-        <v>-0.0287168651555898</v>
+        <v>-0.0021348859776807</v>
       </c>
       <c r="G29" t="n">
-        <v>0.0568866293827514</v>
+        <v>0.0834686085606605</v>
       </c>
       <c r="H29" t="n">
-        <v>0.0717053586734348</v>
+        <v>0.0982873378513439</v>
       </c>
       <c r="I29" t="n">
-        <v>53.85917400135408</v>
+        <v>61.53039832285116</v>
       </c>
       <c r="J29" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K29" t="n">
         <v>49.42</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M29" t="n">
         <v>49.42</v>
       </c>
       <c r="N29" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O29" t="n">
         <v>65.95744680851064</v>
       </c>
       <c r="P29" t="n">
-        <v>48.95948936170213</v>
+        <v>56.95948936170213</v>
       </c>
       <c r="Q29" t="b">
         <v>0</v>
@@ -2599,25 +2599,25 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>102.65</v>
+        <v>107.84</v>
       </c>
       <c r="D30" t="n">
-        <v>-0.1160006889424732</v>
+        <v>-0.0438020925696045</v>
       </c>
       <c r="E30" t="n">
-        <v>-0.0297731568998108</v>
+        <v>0.0170706403847968</v>
       </c>
       <c r="F30" t="n">
-        <v>-0.2266837426548139</v>
+        <v>-0.1954640405848999</v>
       </c>
       <c r="G30" t="n">
-        <v>-0.1410802481164726</v>
+        <v>-0.1098605460465587</v>
       </c>
       <c r="H30" t="n">
-        <v>-0.1262615188257893</v>
+        <v>-0.09504181675587529</v>
       </c>
       <c r="I30" t="n">
-        <v>15.27617951668582</v>
+        <v>26.06075822244538</v>
       </c>
       <c r="J30" t="n">
         <v>20</v>
@@ -2627,7 +2627,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M30" t="n">
@@ -2637,10 +2637,10 @@
         <v>20</v>
       </c>
       <c r="O30" t="n">
-        <v>29.78723404255319</v>
+        <v>36.17021276595745</v>
       </c>
       <c r="P30" t="n">
-        <v>34.90944680851064</v>
+        <v>36.18604255319149</v>
       </c>
       <c r="Q30" t="b">
         <v>0</v>
@@ -2664,48 +2664,48 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>36.9</v>
+        <v>38.2</v>
       </c>
       <c r="D31" t="n">
-        <v>-0.1458333333333333</v>
+        <v>-0.09585798816568029</v>
       </c>
       <c r="E31" t="n">
-        <v>-0.1916757940854326</v>
+        <v>-0.1679372685689391</v>
       </c>
       <c r="F31" t="n">
-        <v>-0.2192128650021159</v>
+        <v>-0.2282828282828282</v>
       </c>
       <c r="G31" t="n">
-        <v>-0.1336093704637746</v>
+        <v>-0.1426793337444869</v>
       </c>
       <c r="H31" t="n">
-        <v>-0.1187906411730912</v>
+        <v>-0.1278606044538035</v>
       </c>
       <c r="I31" t="n">
-        <v>28.8113695090439</v>
+        <v>39.57399103139014</v>
       </c>
       <c r="J31" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="K31" t="n">
         <v>48.99</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M31" t="n">
         <v>48.99</v>
       </c>
       <c r="N31" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="O31" t="n">
-        <v>34.04255319148936</v>
+        <v>27.65957446808511</v>
       </c>
       <c r="P31" t="n">
-        <v>34.40451063829788</v>
+        <v>37.12791489361702</v>
       </c>
       <c r="Q31" t="b">
         <v>0</v>
@@ -2729,48 +2729,48 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>610.8</v>
+        <v>664.15</v>
       </c>
       <c r="D32" t="n">
-        <v>-0.191261171797418</v>
+        <v>-0.0936817685589519</v>
       </c>
       <c r="E32" t="n">
-        <v>-0.2524782768327011</v>
+        <v>-0.1893194995422643</v>
       </c>
       <c r="F32" t="n">
-        <v>-0.4510649770827717</v>
+        <v>-0.4078020508247882</v>
       </c>
       <c r="G32" t="n">
-        <v>-0.3654614825444304</v>
+        <v>-0.322198556286447</v>
       </c>
       <c r="H32" t="n">
-        <v>-0.350642753253747</v>
+        <v>-0.3073798269957636</v>
       </c>
       <c r="I32" t="n">
-        <v>34.18047289689559</v>
+        <v>45.96112311015118</v>
       </c>
       <c r="J32" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K32" t="n">
         <v>47.86</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M32" t="n">
         <v>47.86</v>
       </c>
       <c r="N32" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O32" t="n">
         <v>2.127659574468085</v>
       </c>
       <c r="P32" t="n">
-        <v>31.56953191489362</v>
+        <v>35.56953191489362</v>
       </c>
       <c r="Q32" t="b">
         <v>0</v>
@@ -2794,48 +2794,48 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>513.9</v>
+        <v>537.9</v>
       </c>
       <c r="D33" t="n">
-        <v>-0.1474784339747843</v>
+        <v>-0.0800410466906106</v>
       </c>
       <c r="E33" t="n">
-        <v>-0.1615271659324523</v>
+        <v>-0.113034875092753</v>
       </c>
       <c r="F33" t="n">
-        <v>0.0279027902790278</v>
+        <v>0.0354186717998075</v>
       </c>
       <c r="G33" t="n">
-        <v>0.1135062848173691</v>
+        <v>0.1210221663381487</v>
       </c>
       <c r="H33" t="n">
-        <v>0.1283250141080525</v>
+        <v>0.1358408956288321</v>
       </c>
       <c r="I33" t="n">
-        <v>38.44252163164401</v>
+        <v>48.93556627873971</v>
       </c>
       <c r="J33" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="K33" t="n">
         <v>49.98</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M33" t="n">
         <v>49.98</v>
       </c>
       <c r="N33" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="O33" t="n">
-        <v>78.72340425531915</v>
+        <v>74.46808510638297</v>
       </c>
       <c r="P33" t="n">
-        <v>47.73668085106383</v>
+        <v>58.8856170212766</v>
       </c>
       <c r="Q33" t="b">
         <v>0</v>
@@ -2887,7 +2887,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M34" t="n">
@@ -2897,10 +2897,10 @@
         <v>80</v>
       </c>
       <c r="O34" t="n">
-        <v>25.53191489361702</v>
+        <v>23.40425531914894</v>
       </c>
       <c r="P34" t="n">
-        <v>57.45838297872341</v>
+        <v>57.03285106382979</v>
       </c>
       <c r="Q34" t="b">
         <v>0</v>
@@ -2924,48 +2924,48 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>100.49</v>
+        <v>108.49</v>
       </c>
       <c r="D35" t="n">
-        <v>-0.2399788231734987</v>
+        <v>-0.1324270291883247</v>
       </c>
       <c r="E35" t="n">
-        <v>-0.1389031705227078</v>
+        <v>-0.0847815083516113</v>
       </c>
       <c r="F35" t="n">
-        <v>-0.0174049085753398</v>
+        <v>0.0542221358468564</v>
       </c>
       <c r="G35" t="n">
-        <v>0.06819858596300141</v>
+        <v>0.1398256303851976</v>
       </c>
       <c r="H35" t="n">
-        <v>0.0830173152536848</v>
+        <v>0.154644359675881</v>
       </c>
       <c r="I35" t="n">
-        <v>37.14285714285714</v>
+        <v>46.81259600614439</v>
       </c>
       <c r="J35" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="K35" t="n">
         <v>49.07</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M35" t="n">
         <v>49.07</v>
       </c>
       <c r="N35" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="O35" t="n">
-        <v>68.08510638297872</v>
+        <v>78.72340425531915</v>
       </c>
       <c r="P35" t="n">
-        <v>45.24502127659574</v>
+        <v>59.37268085106383</v>
       </c>
       <c r="Q35" t="b">
         <v>0</v>
@@ -2989,48 +2989,48 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>437</v>
+        <v>460.4</v>
       </c>
       <c r="D36" t="n">
-        <v>-0.1373864982234505</v>
+        <v>-0.08714186576782</v>
       </c>
       <c r="E36" t="n">
-        <v>-0.1999999999999999</v>
+        <v>-0.1794689003742648</v>
       </c>
       <c r="F36" t="n">
-        <v>-0.0541125541125541</v>
+        <v>0.0073296138278087</v>
       </c>
       <c r="G36" t="n">
-        <v>0.0314909404257871</v>
+        <v>0.0929331083661499</v>
       </c>
       <c r="H36" t="n">
-        <v>0.0463096697164705</v>
+        <v>0.1077518376568333</v>
       </c>
       <c r="I36" t="n">
-        <v>22.58964143426293</v>
+        <v>38.56184798807747</v>
       </c>
       <c r="J36" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="K36" t="n">
         <v>47.8</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M36" t="n">
         <v>47.8</v>
       </c>
       <c r="N36" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="O36" t="n">
-        <v>63.82978723404256</v>
+        <v>68.08510638297872</v>
       </c>
       <c r="P36" t="n">
-        <v>39.88595744680851</v>
+        <v>44.73702127659575</v>
       </c>
       <c r="Q36" t="b">
         <v>0</v>
@@ -3054,48 +3054,48 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2074.5</v>
+        <v>2142.4</v>
       </c>
       <c r="D37" t="n">
-        <v>-0.1142942532661599</v>
+        <v>-0.0392394277770303</v>
       </c>
       <c r="E37" t="n">
-        <v>0.2366616989567809</v>
+        <v>0.2608286252354048</v>
       </c>
       <c r="F37" t="n">
-        <v>0.4839055793991416</v>
+        <v>0.5370928397187547</v>
       </c>
       <c r="G37" t="n">
-        <v>0.5695090739374828</v>
+        <v>0.6226963342570959</v>
       </c>
       <c r="H37" t="n">
-        <v>0.5843278032281662</v>
+        <v>0.6375150635477793</v>
       </c>
       <c r="I37" t="n">
-        <v>44.60927705808609</v>
+        <v>53.38727076591155</v>
       </c>
       <c r="J37" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K37" t="n">
         <v>48.59</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M37" t="n">
         <v>48.59</v>
       </c>
       <c r="N37" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O37" t="n">
         <v>100</v>
       </c>
       <c r="P37" t="n">
-        <v>63.43600000000001</v>
+        <v>71.43600000000001</v>
       </c>
       <c r="Q37" t="b">
         <v>0</v>
@@ -3119,48 +3119,48 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>708</v>
+        <v>742.05</v>
       </c>
       <c r="D38" t="n">
-        <v>-0.2403433476394849</v>
+        <v>-0.172050209205021</v>
       </c>
       <c r="E38" t="n">
-        <v>-0.2650646182591997</v>
+        <v>-0.2190591454430647</v>
       </c>
       <c r="F38" t="n">
-        <v>-0.3343987966531917</v>
+        <v>-0.2986294896030246</v>
       </c>
       <c r="G38" t="n">
-        <v>-0.2487953021148504</v>
+        <v>-0.2130259950646833</v>
       </c>
       <c r="H38" t="n">
-        <v>-0.233976572824167</v>
+        <v>-0.1982072657739999</v>
       </c>
       <c r="I38" t="n">
-        <v>33.44699777613046</v>
+        <v>40.37668408028594</v>
       </c>
       <c r="J38" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K38" t="n">
         <v>49.87</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M38" t="n">
         <v>49.87</v>
       </c>
       <c r="N38" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O38" t="n">
-        <v>8.51063829787234</v>
+        <v>12.76595744680851</v>
       </c>
       <c r="P38" t="n">
-        <v>33.65012765957447</v>
+        <v>38.5011914893617</v>
       </c>
       <c r="Q38" t="b">
         <v>0</v>
@@ -3184,25 +3184,25 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>3016.5</v>
+        <v>3025.2</v>
       </c>
       <c r="D39" t="n">
-        <v>-0.0322114921877506</v>
+        <v>-0.0165149544863459</v>
       </c>
       <c r="E39" t="n">
-        <v>-0.0366620892281162</v>
+        <v>-0.0247896586183553</v>
       </c>
       <c r="F39" t="n">
-        <v>0.1256437047540861</v>
+        <v>0.1217323593755792</v>
       </c>
       <c r="G39" t="n">
-        <v>0.2112471992924274</v>
+        <v>0.2073358539139205</v>
       </c>
       <c r="H39" t="n">
-        <v>0.2260659285831108</v>
+        <v>0.2221545832046039</v>
       </c>
       <c r="I39" t="n">
-        <v>48.94468704512374</v>
+        <v>52.32580398162328</v>
       </c>
       <c r="J39" t="n">
         <v>80</v>
@@ -3212,7 +3212,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M39" t="n">
@@ -3222,10 +3222,10 @@
         <v>80</v>
       </c>
       <c r="O39" t="n">
-        <v>89.36170212765957</v>
+        <v>87.2340425531915</v>
       </c>
       <c r="P39" t="n">
-        <v>69.34834042553192</v>
+        <v>68.9228085106383</v>
       </c>
       <c r="Q39" t="b">
         <v>0</v>
@@ -3249,48 +3249,48 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>170.43</v>
+        <v>187.9</v>
       </c>
       <c r="D40" t="n">
-        <v>-0.2072654542071724</v>
+        <v>-0.08697764820213801</v>
       </c>
       <c r="E40" t="n">
-        <v>-0.09586206896551711</v>
+        <v>-0.0035530572201304</v>
       </c>
       <c r="F40" t="n">
-        <v>-0.2931148900871008</v>
+        <v>-0.2307062436028658</v>
       </c>
       <c r="G40" t="n">
-        <v>-0.2075113955487595</v>
+        <v>-0.1451027490645245</v>
       </c>
       <c r="H40" t="n">
-        <v>-0.1926926662580761</v>
+        <v>-0.1302840197738412</v>
       </c>
       <c r="I40" t="n">
-        <v>30.17282384651975</v>
+        <v>46.99369125788593</v>
       </c>
       <c r="J40" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="K40" t="n">
         <v>45.44</v>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M40" t="n">
         <v>45.44</v>
       </c>
       <c r="N40" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="O40" t="n">
-        <v>17.02127659574468</v>
+        <v>25.53191489361702</v>
       </c>
       <c r="P40" t="n">
-        <v>33.58025531914893</v>
+        <v>47.2823829787234</v>
       </c>
       <c r="Q40" t="b">
         <v>0</v>
@@ -3314,25 +3314,25 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>749.05</v>
+        <v>752.9</v>
       </c>
       <c r="D41" t="n">
-        <v>-0.1421290728969821</v>
+        <v>-0.1110455162642423</v>
       </c>
       <c r="E41" t="n">
-        <v>-0.2044078597981944</v>
+        <v>-0.1957055870099349</v>
       </c>
       <c r="F41" t="n">
-        <v>-0.2681485100146556</v>
+        <v>-0.2619351044015293</v>
       </c>
       <c r="G41" t="n">
-        <v>-0.1825450154763144</v>
+        <v>-0.176331609863188</v>
       </c>
       <c r="H41" t="n">
-        <v>-0.167726286185631</v>
+        <v>-0.1615128805725046</v>
       </c>
       <c r="I41" t="n">
-        <v>17.72525849335302</v>
+        <v>20.93984962406016</v>
       </c>
       <c r="J41" t="n">
         <v>20</v>
@@ -3342,7 +3342,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M41" t="n">
@@ -3352,10 +3352,10 @@
         <v>20</v>
       </c>
       <c r="O41" t="n">
-        <v>19.14893617021277</v>
+        <v>17.02127659574468</v>
       </c>
       <c r="P41" t="n">
-        <v>31.04978723404255</v>
+        <v>30.62425531914894</v>
       </c>
       <c r="Q41" t="b">
         <v>0</v>
@@ -3379,48 +3379,48 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>465.05</v>
+        <v>497.65</v>
       </c>
       <c r="D42" t="n">
-        <v>-0.2315128480542013</v>
+        <v>-0.1480784045193871</v>
       </c>
       <c r="E42" t="n">
-        <v>-0.3104240806642941</v>
+        <v>-0.2617564159620235</v>
       </c>
       <c r="F42" t="n">
-        <v>-0.3986940780967157</v>
+        <v>-0.3572074399380006</v>
       </c>
       <c r="G42" t="n">
-        <v>-0.3130905835583745</v>
+        <v>-0.2716039453996594</v>
       </c>
       <c r="H42" t="n">
-        <v>-0.2982718542676911</v>
+        <v>-0.256785216108976</v>
       </c>
       <c r="I42" t="n">
-        <v>21.97893569844792</v>
+        <v>32.13596914175506</v>
       </c>
       <c r="J42" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="K42" t="n">
         <v>47.66</v>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M42" t="n">
         <v>47.66</v>
       </c>
       <c r="N42" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="O42" t="n">
-        <v>6.382978723404255</v>
+        <v>4.25531914893617</v>
       </c>
       <c r="P42" t="n">
-        <v>28.34059574468085</v>
+        <v>31.91506382978724</v>
       </c>
       <c r="Q42" t="b">
         <v>0</v>
@@ -3444,54 +3444,54 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>400.1</v>
+        <v>421.95</v>
       </c>
       <c r="D43" t="n">
-        <v>-0.0834955904249227</v>
+        <v>-0.0212247738343772</v>
       </c>
       <c r="E43" t="n">
-        <v>-0.1173615707037282</v>
+        <v>-0.0511580841016415</v>
       </c>
       <c r="F43" t="n">
-        <v>-0.1262284341559291</v>
+        <v>-0.0810192747468147</v>
       </c>
       <c r="G43" t="n">
-        <v>-0.0406249396175878</v>
+        <v>0.0045842197915265</v>
       </c>
       <c r="H43" t="n">
-        <v>-0.0258062103269044</v>
+        <v>0.0194029490822099</v>
       </c>
       <c r="I43" t="n">
-        <v>37.40506329113924</v>
+        <v>56.05234460196291</v>
       </c>
       <c r="J43" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="K43" t="n">
         <v>51.48</v>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M43" t="n">
         <v>51.48</v>
       </c>
       <c r="N43" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="O43" t="n">
-        <v>53.19148936170212</v>
+        <v>55.31914893617022</v>
       </c>
       <c r="P43" t="n">
-        <v>43.23029787234042</v>
+        <v>55.65582978723404</v>
       </c>
       <c r="Q43" t="b">
         <v>0</v>
       </c>
       <c r="R43" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S43" t="b">
         <v>0</v>
@@ -3509,48 +3509,48 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>231.8</v>
+        <v>243.31</v>
       </c>
       <c r="D44" t="n">
-        <v>-0.1070878274268105</v>
+        <v>-0.0398184688239936</v>
       </c>
       <c r="E44" t="n">
-        <v>-0.1774308019872249</v>
+        <v>-0.1333570792520035</v>
       </c>
       <c r="F44" t="n">
-        <v>-0.2077922077922078</v>
+        <v>-0.2099042052281213</v>
       </c>
       <c r="G44" t="n">
-        <v>-0.1221887132538666</v>
+        <v>-0.1243007106897801</v>
       </c>
       <c r="H44" t="n">
-        <v>-0.1073699839631832</v>
+        <v>-0.1094819813990967</v>
       </c>
       <c r="I44" t="n">
-        <v>43.82089552238806</v>
+        <v>45.10558861276397</v>
       </c>
       <c r="J44" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K44" t="n">
         <v>47.2</v>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M44" t="n">
         <v>47.2</v>
       </c>
       <c r="N44" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O44" t="n">
-        <v>38.29787234042553</v>
+        <v>31.91489361702128</v>
       </c>
       <c r="P44" t="n">
-        <v>42.53957446808511</v>
+        <v>49.26297872340426</v>
       </c>
       <c r="Q44" t="b">
         <v>0</v>
@@ -3574,25 +3574,25 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>80.68000000000001</v>
+        <v>86.75</v>
       </c>
       <c r="D45" t="n">
-        <v>-0.2570218252141081</v>
+        <v>-0.1530801522991312</v>
       </c>
       <c r="E45" t="n">
-        <v>-0.2844345898004434</v>
+        <v>-0.2473538087801492</v>
       </c>
       <c r="F45" t="n">
-        <v>-0.4064592069447509</v>
+        <v>-0.3546827345086663</v>
       </c>
       <c r="G45" t="n">
-        <v>-0.3208557124064096</v>
+        <v>-0.269079239970325</v>
       </c>
       <c r="H45" t="n">
-        <v>-0.3060369831157262</v>
+        <v>-0.2542605106796416</v>
       </c>
       <c r="I45" t="n">
-        <v>19.02858899477402</v>
+        <v>28.92606583917967</v>
       </c>
       <c r="J45" t="n">
         <v>20</v>
@@ -3602,7 +3602,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M45" t="n">
@@ -3612,10 +3612,10 @@
         <v>20</v>
       </c>
       <c r="O45" t="n">
-        <v>4.25531914893617</v>
+        <v>6.382978723404255</v>
       </c>
       <c r="P45" t="n">
-        <v>32.69106382978724</v>
+        <v>33.11659574468086</v>
       </c>
       <c r="Q45" t="b">
         <v>0</v>
@@ -3639,25 +3639,25 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>467.4</v>
+        <v>478.35</v>
       </c>
       <c r="D46" t="n">
-        <v>-0.1359645068860339</v>
+        <v>-0.08929081389814369</v>
       </c>
       <c r="E46" t="n">
-        <v>-0.2780909722758515</v>
+        <v>-0.2642467122971621</v>
       </c>
       <c r="F46" t="n">
-        <v>-0.2258385093167702</v>
+        <v>-0.2194664273476381</v>
       </c>
       <c r="G46" t="n">
-        <v>-0.1402350147784289</v>
+        <v>-0.1338629328092968</v>
       </c>
       <c r="H46" t="n">
-        <v>-0.1254162854877455</v>
+        <v>-0.1190442035186134</v>
       </c>
       <c r="I46" t="n">
-        <v>41.35386589669552</v>
+        <v>44.87334137515078</v>
       </c>
       <c r="J46" t="n">
         <v>40</v>
@@ -3667,7 +3667,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M46" t="n">
@@ -3677,10 +3677,10 @@
         <v>40</v>
       </c>
       <c r="O46" t="n">
-        <v>31.91489361702128</v>
+        <v>29.78723404255319</v>
       </c>
       <c r="P46" t="n">
-        <v>42.22697872340426</v>
+        <v>41.80144680851064</v>
       </c>
       <c r="Q46" t="b">
         <v>0</v>
@@ -3704,25 +3704,25 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>997.25</v>
+        <v>987.55</v>
       </c>
       <c r="D47" t="n">
-        <v>0.1058438678199158</v>
+        <v>0.1265685603467943</v>
       </c>
       <c r="E47" t="n">
-        <v>0.1868491520380839</v>
+        <v>0.1727229545184656</v>
       </c>
       <c r="F47" t="n">
-        <v>0.3300213390237396</v>
+        <v>0.3409600108629234</v>
       </c>
       <c r="G47" t="n">
-        <v>0.4156248335620809</v>
+        <v>0.4265635054012646</v>
       </c>
       <c r="H47" t="n">
-        <v>0.4304435628527643</v>
+        <v>0.441382234691948</v>
       </c>
       <c r="I47" t="n">
-        <v>59.49001683906664</v>
+        <v>56.88173344631399</v>
       </c>
       <c r="J47" t="n">
         <v>80</v>
@@ -3732,7 +3732,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M47" t="n">
@@ -3742,10 +3742,10 @@
         <v>80</v>
       </c>
       <c r="O47" t="n">
-        <v>95.74468085106383</v>
+        <v>93.61702127659576</v>
       </c>
       <c r="P47" t="n">
-        <v>69.88093617021276</v>
+        <v>69.45540425531915</v>
       </c>
       <c r="Q47" t="b">
         <v>0</v>
@@ -3769,48 +3769,48 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>13768</v>
+        <v>14375</v>
       </c>
       <c r="D48" t="n">
-        <v>-0.0920601424426272</v>
+        <v>-0.0216429592322874</v>
       </c>
       <c r="E48" t="n">
-        <v>-0.0336889387984278</v>
+        <v>0.017915309446254</v>
       </c>
       <c r="F48" t="n">
-        <v>0.0051102350708132</v>
+        <v>0.0471299533799534</v>
       </c>
       <c r="G48" t="n">
-        <v>0.0907137296091544</v>
+        <v>0.1327334479182946</v>
       </c>
       <c r="H48" t="n">
-        <v>0.1055324588998378</v>
+        <v>0.147552177208978</v>
       </c>
       <c r="I48" t="n">
-        <v>45.800933125972</v>
+        <v>56.38029058749211</v>
       </c>
       <c r="J48" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K48" t="n">
         <v>50.29</v>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M48" t="n">
         <v>50.29</v>
       </c>
       <c r="N48" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O48" t="n">
-        <v>74.46808510638297</v>
+        <v>76.59574468085107</v>
       </c>
       <c r="P48" t="n">
-        <v>51.0096170212766</v>
+        <v>59.43514893617021</v>
       </c>
       <c r="Q48" t="b">
         <v>0</v>
@@ -3936,48 +3936,48 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>WHEELS</t>
+          <t>LUMAXTECH</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Wheels</t>
+          <t>Lighting</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>997.25</v>
+        <v>1593.5</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1058438678199158</v>
+        <v>-0.0423102349900835</v>
       </c>
       <c r="E2" t="n">
-        <v>0.1868491520380839</v>
+        <v>0.07574427867413749</v>
       </c>
       <c r="F2" t="n">
-        <v>0.3300213390237396</v>
+        <v>0.3990342405618963</v>
       </c>
       <c r="G2" t="n">
-        <v>0.4156248335620809</v>
+        <v>0.4846377351002375</v>
       </c>
       <c r="H2" t="n">
-        <v>0.4304435628527643</v>
+        <v>0.4994564643909209</v>
       </c>
       <c r="I2" t="n">
-        <v>59.49001683906664</v>
+        <v>63.56641468682506</v>
       </c>
       <c r="J2" t="n">
         <v>80</v>
       </c>
       <c r="K2" t="n">
-        <v>46.83</v>
+        <v>54.51</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M2" t="n">
-        <v>46.83</v>
+        <v>54.51</v>
       </c>
       <c r="N2" t="n">
         <v>80</v>
@@ -3986,7 +3986,7 @@
         <v>95.74468085106383</v>
       </c>
       <c r="P2" t="n">
-        <v>69.88093617021276</v>
+        <v>72.95293617021277</v>
       </c>
       <c r="Q2" t="b">
         <v>0</v>
@@ -4001,63 +4001,63 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ASKAUTOLTD</t>
+          <t>SANSERA</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Forgings</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>444.75</v>
+        <v>2142.4</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0707836764174791</v>
+        <v>-0.0392394277770303</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.0402460077686663</v>
+        <v>0.2608286252354048</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.174018014671743</v>
+        <v>0.5370928397187547</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.0884145201334017</v>
+        <v>0.6226963342570959</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.07359579084271831</v>
+        <v>0.6375150635477793</v>
       </c>
       <c r="I3" t="n">
-        <v>68.07935076645629</v>
+        <v>53.38727076591155</v>
       </c>
       <c r="J3" t="n">
         <v>80</v>
       </c>
       <c r="K3" t="n">
-        <v>71.28</v>
+        <v>48.59</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M3" t="n">
-        <v>71.28</v>
+        <v>48.59</v>
       </c>
       <c r="N3" t="n">
         <v>80</v>
       </c>
       <c r="O3" t="n">
-        <v>44.68085106382978</v>
+        <v>100</v>
       </c>
       <c r="P3" t="n">
-        <v>69.44817021276596</v>
+        <v>71.43600000000001</v>
       </c>
       <c r="Q3" t="b">
+        <v>0</v>
+      </c>
+      <c r="R3" t="b">
         <v>1</v>
-      </c>
-      <c r="R3" t="b">
-        <v>0</v>
       </c>
       <c r="S3" t="b">
         <v>0</v>
@@ -4066,57 +4066,57 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SHRIPISTON</t>
+          <t>WHEELS</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Engine/Parts</t>
+          <t>Wheels</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>3016.5</v>
+        <v>987.55</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.0322114921877506</v>
+        <v>0.1265685603467943</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.0366620892281162</v>
+        <v>0.1727229545184656</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1256437047540861</v>
+        <v>0.3409600108629234</v>
       </c>
       <c r="G4" t="n">
-        <v>0.2112471992924274</v>
+        <v>0.4265635054012646</v>
       </c>
       <c r="H4" t="n">
-        <v>0.2260659285831108</v>
+        <v>0.441382234691948</v>
       </c>
       <c r="I4" t="n">
-        <v>48.94468704512374</v>
+        <v>56.88173344631399</v>
       </c>
       <c r="J4" t="n">
         <v>80</v>
       </c>
       <c r="K4" t="n">
-        <v>48.69</v>
+        <v>46.83</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M4" t="n">
-        <v>48.69</v>
+        <v>46.83</v>
       </c>
       <c r="N4" t="n">
         <v>80</v>
       </c>
       <c r="O4" t="n">
-        <v>89.36170212765957</v>
+        <v>93.61702127659576</v>
       </c>
       <c r="P4" t="n">
-        <v>69.34834042553192</v>
+        <v>69.45540425531915</v>
       </c>
       <c r="Q4" t="b">
         <v>0</v>
@@ -4131,57 +4131,57 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SANSERA</t>
+          <t>SHRIPISTON</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Forgings</t>
+          <t>Engine/Parts</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>2074.5</v>
+        <v>3025.2</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.1142942532661599</v>
+        <v>-0.0165149544863459</v>
       </c>
       <c r="E5" t="n">
-        <v>0.2366616989567809</v>
+        <v>-0.0247896586183553</v>
       </c>
       <c r="F5" t="n">
-        <v>0.4839055793991416</v>
+        <v>0.1217323593755792</v>
       </c>
       <c r="G5" t="n">
-        <v>0.5695090739374828</v>
+        <v>0.2073358539139205</v>
       </c>
       <c r="H5" t="n">
-        <v>0.5843278032281662</v>
+        <v>0.2221545832046039</v>
       </c>
       <c r="I5" t="n">
-        <v>44.60927705808609</v>
+        <v>52.32580398162328</v>
       </c>
       <c r="J5" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K5" t="n">
-        <v>48.59</v>
+        <v>48.69</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M5" t="n">
-        <v>48.59</v>
+        <v>48.69</v>
       </c>
       <c r="N5" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O5" t="n">
-        <v>100</v>
+        <v>87.2340425531915</v>
       </c>
       <c r="P5" t="n">
-        <v>63.43600000000001</v>
+        <v>68.9228085106383</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
@@ -4196,60 +4196,60 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>RANEENGINE</t>
+          <t>ASKAUTOLTD</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Engine/Parts</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>317.75</v>
+        <v>435.7</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1790352504638219</v>
+        <v>0.0889777555611095</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.156154561147258</v>
+        <v>-0.06431869429829271</v>
       </c>
       <c r="F6" t="n">
-        <v>-0.2401052253975846</v>
+        <v>-0.1885650433001211</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.1545017308592433</v>
+        <v>-0.1029615487617798</v>
       </c>
       <c r="H6" t="n">
-        <v>-0.1396830015685599</v>
+        <v>-0.0881428194710964</v>
       </c>
       <c r="I6" t="n">
-        <v>63.3225806451613</v>
+        <v>62.39424703891709</v>
       </c>
       <c r="J6" t="n">
         <v>80</v>
       </c>
       <c r="K6" t="n">
-        <v>50.88</v>
+        <v>71.28</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M6" t="n">
-        <v>50.88</v>
+        <v>71.28</v>
       </c>
       <c r="N6" t="n">
         <v>80</v>
       </c>
       <c r="O6" t="n">
-        <v>25.53191489361702</v>
+        <v>38.29787234042553</v>
       </c>
       <c r="P6" t="n">
-        <v>57.45838297872341</v>
+        <v>68.17157446808511</v>
       </c>
       <c r="Q6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R6" t="b">
         <v>0</v>
@@ -4261,63 +4261,63 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>LUMAXTECH</t>
+          <t>JBMA</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Lighting</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1522.2</v>
+        <v>561.1</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.1338340730624786</v>
+        <v>0.0641001327517543</v>
       </c>
       <c r="E7" t="n">
-        <v>0.0300446609825417</v>
+        <v>-0.0170797932907068</v>
       </c>
       <c r="F7" t="n">
-        <v>0.3264203555245732</v>
+        <v>-0.1047467092142001</v>
       </c>
       <c r="G7" t="n">
-        <v>0.4120238500629145</v>
+        <v>-0.0191432146758588</v>
       </c>
       <c r="H7" t="n">
-        <v>0.4268425793535979</v>
+        <v>-0.0043244853851754</v>
       </c>
       <c r="I7" t="n">
-        <v>53.46534653465347</v>
+        <v>56.87363038714392</v>
       </c>
       <c r="J7" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="K7" t="n">
-        <v>54.51</v>
+        <v>56.91</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M7" t="n">
-        <v>54.51</v>
+        <v>56.91</v>
       </c>
       <c r="N7" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="O7" t="n">
-        <v>93.61702127659576</v>
+        <v>51.06382978723404</v>
       </c>
       <c r="P7" t="n">
-        <v>56.52740425531916</v>
+        <v>64.9767659574468</v>
       </c>
       <c r="Q7" t="b">
         <v>0</v>
       </c>
       <c r="R7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S7" t="b">
         <v>0</v>
@@ -4326,63 +4326,63 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>TIINDIA</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Forgings</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1674.6</v>
+        <v>2572.7</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.1237965676015069</v>
+        <v>-0.0933535382012968</v>
       </c>
       <c r="E8" t="n">
-        <v>0.1898536308085829</v>
+        <v>-0.0312170507606567</v>
       </c>
       <c r="F8" t="n">
-        <v>0.3922514133688062</v>
+        <v>-0.183658575281612</v>
       </c>
       <c r="G8" t="n">
-        <v>0.4778549079071474</v>
+        <v>-0.0980550807432707</v>
       </c>
       <c r="H8" t="n">
-        <v>0.4926736371978308</v>
+        <v>-0.0832363514525873</v>
       </c>
       <c r="I8" t="n">
-        <v>39.00161608906448</v>
+        <v>51.4375</v>
       </c>
       <c r="J8" t="n">
-        <v>30</v>
+        <v>80</v>
       </c>
       <c r="K8" t="n">
-        <v>54.83</v>
+        <v>48.73</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M8" t="n">
-        <v>54.83</v>
+        <v>48.73</v>
       </c>
       <c r="N8" t="n">
-        <v>30</v>
+        <v>80</v>
       </c>
       <c r="O8" t="n">
-        <v>97.87234042553192</v>
+        <v>42.5531914893617</v>
       </c>
       <c r="P8" t="n">
-        <v>53.50646808510639</v>
+        <v>60.00263829787234</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
       </c>
       <c r="R8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S8" t="b">
         <v>0</v>
@@ -4391,57 +4391,57 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CRAFTSMAN</t>
+          <t>ZFCVINDIA</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Castings</t>
+          <t>Brakes/Transmission</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>6977</v>
+        <v>14375</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.07294711666223749</v>
+        <v>-0.0216429592322874</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.007680273076376</v>
+        <v>0.017915309446254</v>
       </c>
       <c r="F9" t="n">
-        <v>0.0204768173175369</v>
+        <v>0.0471299533799534</v>
       </c>
       <c r="G9" t="n">
-        <v>0.1060803118558781</v>
+        <v>0.1327334479182946</v>
       </c>
       <c r="H9" t="n">
-        <v>0.1208990411465615</v>
+        <v>0.147552177208978</v>
       </c>
       <c r="I9" t="n">
-        <v>41.76706827309237</v>
+        <v>56.38029058749211</v>
       </c>
       <c r="J9" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K9" t="n">
-        <v>54.65</v>
+        <v>50.29</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M9" t="n">
-        <v>54.65</v>
+        <v>50.29</v>
       </c>
       <c r="N9" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O9" t="n">
         <v>76.59574468085107</v>
       </c>
       <c r="P9" t="n">
-        <v>53.17914893617021</v>
+        <v>59.43514893617021</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -4456,57 +4456,57 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>LUMAXIND</t>
+          <t>RICOAUTO</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Lighting</t>
+          <t>Castings</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>4654</v>
+        <v>108.49</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.2302221340081708</v>
+        <v>-0.1324270291883247</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.1675163223325284</v>
+        <v>-0.0847815083516113</v>
       </c>
       <c r="F10" t="n">
-        <v>0.114944180920895</v>
+        <v>0.0542221358468564</v>
       </c>
       <c r="G10" t="n">
-        <v>0.2005476754592363</v>
+        <v>0.1398256303851976</v>
       </c>
       <c r="H10" t="n">
-        <v>0.2153664047499197</v>
+        <v>0.154644359675881</v>
       </c>
       <c r="I10" t="n">
-        <v>37.80844834797156</v>
+        <v>46.81259600614439</v>
       </c>
       <c r="J10" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="K10" t="n">
-        <v>57.69</v>
+        <v>49.07</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M10" t="n">
-        <v>57.69</v>
+        <v>49.07</v>
       </c>
       <c r="N10" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="O10" t="n">
-        <v>87.2340425531915</v>
+        <v>78.72340425531915</v>
       </c>
       <c r="P10" t="n">
-        <v>52.5228085106383</v>
+        <v>59.37268085106383</v>
       </c>
       <c r="Q10" t="b">
         <v>0</v>
@@ -4521,57 +4521,57 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>GNA</t>
+          <t>PRICOLLTD</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Axles</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>356.7</v>
+        <v>537.9</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.1486873508353222</v>
+        <v>-0.0800410466906106</v>
       </c>
       <c r="E11" t="n">
-        <v>0.167021102568297</v>
+        <v>-0.113034875092753</v>
       </c>
       <c r="F11" t="n">
-        <v>0.1361681796464404</v>
+        <v>0.0354186717998075</v>
       </c>
       <c r="G11" t="n">
-        <v>0.2217716741847817</v>
+        <v>0.1210221663381487</v>
       </c>
       <c r="H11" t="n">
-        <v>0.2365904034754651</v>
+        <v>0.1358408956288321</v>
       </c>
       <c r="I11" t="n">
-        <v>30.99173553719008</v>
+        <v>48.93556627873971</v>
       </c>
       <c r="J11" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="K11" t="n">
-        <v>54.47</v>
+        <v>49.98</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M11" t="n">
-        <v>54.47</v>
+        <v>49.98</v>
       </c>
       <c r="N11" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="O11" t="n">
-        <v>91.48936170212764</v>
+        <v>74.46808510638297</v>
       </c>
       <c r="P11" t="n">
-        <v>52.08587234042552</v>
+        <v>58.8856170212766</v>
       </c>
       <c r="Q11" t="b">
         <v>0</v>
@@ -4586,57 +4586,57 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TIINDIA</t>
+          <t>RANEENGINE</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Engine/Parts</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>2517.3</v>
+        <v>317.75</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.0857485290913052</v>
+        <v>0.1790352504638219</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.0504696163856511</v>
+        <v>-0.156154561147258</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.1806464212479249</v>
+        <v>-0.2401052253975846</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.0950429267095837</v>
+        <v>-0.1545017308592433</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.0802241974189003</v>
+        <v>-0.1396830015685599</v>
       </c>
       <c r="I12" t="n">
-        <v>46.79984229202262</v>
+        <v>63.3225806451613</v>
       </c>
       <c r="J12" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K12" t="n">
-        <v>48.73</v>
+        <v>50.88</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M12" t="n">
-        <v>48.73</v>
+        <v>50.88</v>
       </c>
       <c r="N12" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O12" t="n">
-        <v>42.5531914893617</v>
+        <v>23.40425531914894</v>
       </c>
       <c r="P12" t="n">
-        <v>52.00263829787234</v>
+        <v>57.03285106382979</v>
       </c>
       <c r="Q12" t="b">
         <v>0</v>
@@ -4651,57 +4651,57 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ZFCVINDIA</t>
+          <t>MINDACORP</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Brakes/Transmission</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>13768</v>
+        <v>514.15</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.0920601424426272</v>
+        <v>-0.0492788461538461</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.0336889387984278</v>
+        <v>-0.1210359859817079</v>
       </c>
       <c r="F13" t="n">
-        <v>0.0051102350708132</v>
+        <v>-0.0021348859776807</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0907137296091544</v>
+        <v>0.0834686085606605</v>
       </c>
       <c r="H13" t="n">
-        <v>0.1055324588998378</v>
+        <v>0.0982873378513439</v>
       </c>
       <c r="I13" t="n">
-        <v>45.800933125972</v>
+        <v>61.53039832285116</v>
       </c>
       <c r="J13" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K13" t="n">
-        <v>50.29</v>
+        <v>49.42</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M13" t="n">
-        <v>50.29</v>
+        <v>49.42</v>
       </c>
       <c r="N13" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O13" t="n">
-        <v>74.46808510638297</v>
+        <v>65.95744680851064</v>
       </c>
       <c r="P13" t="n">
-        <v>51.0096170212766</v>
+        <v>56.95948936170213</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
@@ -4716,57 +4716,57 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>MINDACORP</t>
+          <t>LUMAXIND</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Lighting</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>505.65</v>
+        <v>4805.4</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.08982089820898199</v>
+        <v>-0.1923697478991597</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.1342350826127899</v>
+        <v>-0.1256550218340612</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.0287168651555898</v>
+        <v>0.1459436256975246</v>
       </c>
       <c r="G14" t="n">
-        <v>0.0568866293827514</v>
+        <v>0.2315471202358658</v>
       </c>
       <c r="H14" t="n">
-        <v>0.0717053586734348</v>
+        <v>0.2463658495265492</v>
       </c>
       <c r="I14" t="n">
-        <v>53.85917400135408</v>
+        <v>46.77362169828044</v>
       </c>
       <c r="J14" t="n">
         <v>40</v>
       </c>
       <c r="K14" t="n">
-        <v>49.42</v>
+        <v>57.69</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M14" t="n">
-        <v>49.42</v>
+        <v>57.69</v>
       </c>
       <c r="N14" t="n">
         <v>40</v>
       </c>
       <c r="O14" t="n">
-        <v>65.95744680851064</v>
+        <v>89.36170212765957</v>
       </c>
       <c r="P14" t="n">
-        <v>48.95948936170213</v>
+        <v>56.94834042553191</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
@@ -4781,57 +4781,57 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>SUPRAJIT</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Cables</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>481.5</v>
+        <v>421.95</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.0991580916744621</v>
+        <v>-0.0212247738343772</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.0034150884818379</v>
+        <v>-0.0511580841016415</v>
       </c>
       <c r="F15" t="n">
-        <v>0.059755694948828</v>
+        <v>-0.0810192747468147</v>
       </c>
       <c r="G15" t="n">
-        <v>0.1453591894871693</v>
+        <v>0.0045842197915265</v>
       </c>
       <c r="H15" t="n">
-        <v>0.1601779187778527</v>
+        <v>0.0194029490822099</v>
       </c>
       <c r="I15" t="n">
-        <v>38.7180317254775</v>
+        <v>56.05234460196291</v>
       </c>
       <c r="J15" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="K15" t="n">
-        <v>49.66</v>
+        <v>51.48</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M15" t="n">
-        <v>49.66</v>
+        <v>51.48</v>
       </c>
       <c r="N15" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="O15" t="n">
-        <v>82.97872340425532</v>
+        <v>55.31914893617022</v>
       </c>
       <c r="P15" t="n">
-        <v>48.45974468085107</v>
+        <v>55.65582978723404</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
@@ -4846,63 +4846,63 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>JBMA</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Forgings</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>515.25</v>
+        <v>1668.4</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.06547565067561439</v>
+        <v>-0.1122226360879049</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.0882951428824205</v>
+        <v>0.1694939015841863</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.1726878612716762</v>
+        <v>0.4118642633494118</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.0870843667333349</v>
+        <v>0.4974677578877531</v>
       </c>
       <c r="H16" t="n">
-        <v>-0.07226563744265151</v>
+        <v>0.5122864871784365</v>
       </c>
       <c r="I16" t="n">
-        <v>50.56932350971199</v>
+        <v>39.8093841642229</v>
       </c>
       <c r="J16" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K16" t="n">
-        <v>56.91</v>
+        <v>54.83</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="M16" t="n">
-        <v>56.91</v>
+        <v>54.83</v>
       </c>
       <c r="N16" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O16" t="n">
-        <v>46.80851063829788</v>
+        <v>97.87234042553192</v>
       </c>
       <c r="P16" t="n">
-        <v>48.12570212765957</v>
+        <v>53.50646808510639</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>
       </c>
       <c r="R16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S16" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
chore: auto-refresh NSE data and pipeline outputs (2026-04-02)
</commit_message>
<xml_diff>
--- a/working-sector/output/auto_components_comprehensive_report.xlsx
+++ b/working-sector/output/auto_components_comprehensive_report.xlsx
@@ -435,7 +435,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -447,7 +447,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -779,48 +779,48 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1668.4</v>
+        <v>1642.6</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.1122226360879049</v>
+        <v>-0.1081550656966011</v>
       </c>
       <c r="E2" t="n">
-        <v>0.1694939015841863</v>
+        <v>0.1171109902067464</v>
       </c>
       <c r="F2" t="n">
-        <v>0.4118642633494118</v>
+        <v>0.3689474122843568</v>
       </c>
       <c r="G2" t="n">
-        <v>0.4974677578877531</v>
+        <v>0.4480394542590838</v>
       </c>
       <c r="H2" t="n">
-        <v>0.5122864871784365</v>
+        <v>0.4519115173868244</v>
       </c>
       <c r="I2" t="n">
-        <v>39.8093841642229</v>
+        <v>46.51959734418505</v>
       </c>
       <c r="J2" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K2" t="n">
         <v>54.83</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M2" t="n">
         <v>54.83</v>
       </c>
       <c r="N2" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O2" t="n">
-        <v>97.87234042553192</v>
+        <v>95.74468085106383</v>
       </c>
       <c r="P2" t="n">
-        <v>53.50646808510639</v>
+        <v>57.08093617021277</v>
       </c>
       <c r="Q2" t="b">
         <v>0</v>
@@ -844,25 +844,25 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1043.4</v>
+        <v>1025.4</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.08505787443002449</v>
+        <v>-0.088128056914184</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.164009294127073</v>
+        <v>-0.2025198320111991</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.1873198847262247</v>
+        <v>-0.1924712553157976</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.1017163901878834</v>
+        <v>-0.1133792133410706</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.0868976608972</v>
+        <v>-0.10950715021333</v>
       </c>
       <c r="I3" t="n">
-        <v>46.31207757860712</v>
+        <v>52.01320132013202</v>
       </c>
       <c r="J3" t="n">
         <v>40</v>
@@ -872,7 +872,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M3" t="n">
@@ -882,10 +882,10 @@
         <v>40</v>
       </c>
       <c r="O3" t="n">
-        <v>40.42553191489361</v>
+        <v>34.04255319148936</v>
       </c>
       <c r="P3" t="n">
-        <v>43.82910638297872</v>
+        <v>42.55251063829788</v>
       </c>
       <c r="Q3" t="b">
         <v>0</v>
@@ -909,48 +909,48 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>30635</v>
+        <v>32135</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.1338705117331071</v>
+        <v>-0.0375861036238395</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.1655998910527032</v>
+        <v>-0.1083518312985571</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.2617182793107603</v>
+        <v>-0.2163150835263991</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.176114784772419</v>
+        <v>-0.1372230415516721</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.1612960554817356</v>
+        <v>-0.1333509784239315</v>
       </c>
       <c r="I4" t="n">
-        <v>46.32272228320527</v>
+        <v>60.27397260273973</v>
       </c>
       <c r="J4" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K4" t="n">
         <v>53.48</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M4" t="n">
         <v>53.48</v>
       </c>
       <c r="N4" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O4" t="n">
-        <v>19.14893617021277</v>
+        <v>27.65957446808511</v>
       </c>
       <c r="P4" t="n">
-        <v>41.22178723404255</v>
+        <v>50.92391489361702</v>
       </c>
       <c r="Q4" t="b">
         <v>0</v>
@@ -974,25 +974,25 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>299.85</v>
+        <v>299.25</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.0710966542750929</v>
+        <v>-0.0468227424749163</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.1977257525083611</v>
+        <v>-0.1737990060739922</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.2973637961335675</v>
+        <v>-0.2912966252220248</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.2117603015952263</v>
+        <v>-0.2122045832472977</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.1969415723045429</v>
+        <v>-0.2083325201195571</v>
       </c>
       <c r="I5" t="n">
-        <v>44.69419759539991</v>
+        <v>51.59927579963788</v>
       </c>
       <c r="J5" t="n">
         <v>40</v>
@@ -1002,7 +1002,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M5" t="n">
@@ -1012,10 +1012,10 @@
         <v>40</v>
       </c>
       <c r="O5" t="n">
-        <v>14.8936170212766</v>
+        <v>12.76595744680851</v>
       </c>
       <c r="P5" t="n">
-        <v>39.42672340425532</v>
+        <v>39.0011914893617</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
@@ -1039,25 +1039,25 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>107.62</v>
+        <v>106.81</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.1634667703070346</v>
+        <v>-0.1307779947916666</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.1127782357790601</v>
+        <v>-0.1094714023678505</v>
       </c>
       <c r="F6" t="n">
-        <v>0.08905079943331309</v>
+        <v>0.0617296222664016</v>
       </c>
       <c r="G6" t="n">
-        <v>0.1746542939716544</v>
+        <v>0.1408216642411287</v>
       </c>
       <c r="H6" t="n">
-        <v>0.1894730232623378</v>
+        <v>0.1446937273688693</v>
       </c>
       <c r="I6" t="n">
-        <v>34.16603583144084</v>
+        <v>39.71839249046643</v>
       </c>
       <c r="J6" t="n">
         <v>30</v>
@@ -1067,7 +1067,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M6" t="n">
@@ -1077,10 +1077,10 @@
         <v>30</v>
       </c>
       <c r="O6" t="n">
-        <v>80.85106382978722</v>
+        <v>78.72340425531915</v>
       </c>
       <c r="P6" t="n">
-        <v>48.79821276595744</v>
+        <v>48.37268085106383</v>
       </c>
       <c r="Q6" t="b">
         <v>0</v>
@@ -1104,25 +1104,25 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2572.7</v>
+        <v>2567.3</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.0933535382012968</v>
+        <v>-0.0735448017032945</v>
       </c>
       <c r="E7" t="n">
-        <v>-0.0312170507606567</v>
+        <v>-0.0179029111357635</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.183658575281612</v>
+        <v>-0.2064232944885783</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.0980550807432707</v>
+        <v>-0.1273312525138512</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.0832363514525873</v>
+        <v>-0.1234591893861106</v>
       </c>
       <c r="I7" t="n">
-        <v>51.4375</v>
+        <v>57.64112620815244</v>
       </c>
       <c r="J7" t="n">
         <v>80</v>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M7" t="n">
@@ -1142,10 +1142,10 @@
         <v>80</v>
       </c>
       <c r="O7" t="n">
-        <v>42.5531914893617</v>
+        <v>29.78723404255319</v>
       </c>
       <c r="P7" t="n">
-        <v>60.00263829787234</v>
+        <v>57.44944680851064</v>
       </c>
       <c r="Q7" t="b">
         <v>0</v>
@@ -1169,25 +1169,25 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>497.25</v>
+        <v>496.55</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.0386660222329627</v>
+        <v>-0.009672915835660101</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0096446700507615</v>
+        <v>0.0357738840216939</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1161616161616161</v>
+        <v>0.1033218531274302</v>
       </c>
       <c r="G8" t="n">
-        <v>0.2017651106999574</v>
+        <v>0.1824138951021573</v>
       </c>
       <c r="H8" t="n">
-        <v>0.2165838399906408</v>
+        <v>0.1862859582298979</v>
       </c>
       <c r="I8" t="n">
-        <v>46.02497715504112</v>
+        <v>53.73399715504979</v>
       </c>
       <c r="J8" t="n">
         <v>40</v>
@@ -1197,7 +1197,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M8" t="n">
@@ -1207,10 +1207,10 @@
         <v>40</v>
       </c>
       <c r="O8" t="n">
-        <v>85.1063829787234</v>
+        <v>87.2340425531915</v>
       </c>
       <c r="P8" t="n">
-        <v>52.88527659574468</v>
+        <v>53.31080851063831</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
@@ -1234,25 +1234,25 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>415.25</v>
+        <v>409.45</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.0571071752951861</v>
+        <v>-0.0506607929515419</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.1857843137254902</v>
+        <v>-0.1811</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.1374117158288325</v>
+        <v>-0.1461787092065478</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.0518082212904912</v>
+        <v>-0.0670866672318207</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.0369894919998078</v>
+        <v>-0.0632146041040802</v>
       </c>
       <c r="I9" t="n">
-        <v>48.73284054910245</v>
+        <v>55.5021046301864</v>
       </c>
       <c r="J9" t="n">
         <v>40</v>
@@ -1262,7 +1262,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M9" t="n">
@@ -1272,10 +1272,10 @@
         <v>40</v>
       </c>
       <c r="O9" t="n">
-        <v>44.68085106382978</v>
+        <v>46.80851063829788</v>
       </c>
       <c r="P9" t="n">
-        <v>46.31217021276596</v>
+        <v>46.73770212765958</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -1299,25 +1299,25 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>129095</v>
+        <v>126390</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.0700882405906717</v>
+        <v>-0.0641243983709737</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.1537528679121599</v>
+        <v>-0.1731379411860913</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.1354184107423902</v>
+        <v>-0.1298750473305566</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.0498149162040489</v>
+        <v>-0.0507830053558295</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.0349961869133655</v>
+        <v>-0.046910942228089</v>
       </c>
       <c r="I10" t="n">
-        <v>30.78913324708927</v>
+        <v>31.30206049978081</v>
       </c>
       <c r="J10" t="n">
         <v>30</v>
@@ -1327,7 +1327,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M10" t="n">
@@ -1337,10 +1337,10 @@
         <v>30</v>
       </c>
       <c r="O10" t="n">
-        <v>46.80851063829788</v>
+        <v>48.93617021276596</v>
       </c>
       <c r="P10" t="n">
-        <v>41.12570212765957</v>
+        <v>41.55123404255319</v>
       </c>
       <c r="Q10" t="b">
         <v>0</v>
@@ -1376,10 +1376,10 @@
         <v>-0.0042030657656173</v>
       </c>
       <c r="G11" t="n">
-        <v>0.0814004287727239</v>
+        <v>0.0748889762091097</v>
       </c>
       <c r="H11" t="n">
-        <v>0.09621915806340731</v>
+        <v>0.0787610393368503</v>
       </c>
       <c r="I11" t="n">
         <v>27.6054590570719</v>
@@ -1392,7 +1392,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M11" t="n">
@@ -1402,10 +1402,10 @@
         <v>20</v>
       </c>
       <c r="O11" t="n">
-        <v>63.82978723404256</v>
+        <v>65.95744680851064</v>
       </c>
       <c r="P11" t="n">
-        <v>24.76595744680852</v>
+        <v>25.19148936170213</v>
       </c>
       <c r="Q11" t="b">
         <v>0</v>
@@ -1429,25 +1429,25 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>435.7</v>
+        <v>436.5</v>
       </c>
       <c r="D12" t="n">
-        <v>0.0889777555611095</v>
+        <v>0.1303897449177782</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.06431869429829271</v>
+        <v>-0.08806016922594791</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.1885650433001211</v>
+        <v>-0.1646732370108122</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.1029615487617798</v>
+        <v>-0.08558119503608511</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.0881428194710964</v>
+        <v>-0.0817091319083446</v>
       </c>
       <c r="I12" t="n">
-        <v>62.39424703891709</v>
+        <v>64.88250652741513</v>
       </c>
       <c r="J12" t="n">
         <v>80</v>
@@ -1457,7 +1457,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M12" t="n">
@@ -1467,10 +1467,10 @@
         <v>80</v>
       </c>
       <c r="O12" t="n">
-        <v>38.29787234042553</v>
+        <v>42.5531914893617</v>
       </c>
       <c r="P12" t="n">
-        <v>68.17157446808511</v>
+        <v>69.02263829787233</v>
       </c>
       <c r="Q12" t="b">
         <v>1</v>
@@ -1494,25 +1494,25 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1623.6</v>
+        <v>1659.1</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.190950767390871</v>
+        <v>-0.1711545186591397</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.131950384944397</v>
+        <v>-0.11867197875166</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.054397204426325</v>
+        <v>-0.025778038755138</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0312062901120162</v>
+        <v>0.053314003219589</v>
       </c>
       <c r="H13" t="n">
-        <v>0.0460250194026996</v>
+        <v>0.0571860663473295</v>
       </c>
       <c r="I13" t="n">
-        <v>32.51404494382022</v>
+        <v>39.78727239949522</v>
       </c>
       <c r="J13" t="n">
         <v>30</v>
@@ -1522,7 +1522,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M13" t="n">
@@ -1532,10 +1532,10 @@
         <v>30</v>
       </c>
       <c r="O13" t="n">
-        <v>57.44680851063831</v>
+        <v>61.70212765957447</v>
       </c>
       <c r="P13" t="n">
-        <v>46.99736170212766</v>
+        <v>47.8484255319149</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
@@ -1559,25 +1559,25 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>539.65</v>
+        <v>520.9</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.0908861185983828</v>
+        <v>-0.09044875152785049</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.240624780130866</v>
+        <v>-0.2438121506859258</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.13036822173878</v>
+        <v>-0.1601096420509513</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.0447647272004387</v>
+        <v>-0.0810176000762242</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.0299459979097553</v>
+        <v>-0.0771455369484837</v>
       </c>
       <c r="I14" t="n">
-        <v>42.6839293053843</v>
+        <v>43.87410223912125</v>
       </c>
       <c r="J14" t="n">
         <v>40</v>
@@ -1587,7 +1587,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M14" t="n">
@@ -1597,10 +1597,10 @@
         <v>40</v>
       </c>
       <c r="O14" t="n">
-        <v>48.93617021276596</v>
+        <v>44.68085106382978</v>
       </c>
       <c r="P14" t="n">
-        <v>47.6432340425532</v>
+        <v>46.79217021276596</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
@@ -1624,25 +1624,25 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>90.78</v>
+        <v>90.09999999999999</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.1249277038750722</v>
+        <v>-0.0949271722752386</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.1415602836879432</v>
+        <v>-0.2509145327569005</v>
       </c>
       <c r="F15" t="n">
-        <v>0.0273879583521956</v>
+        <v>0.028538812785388</v>
       </c>
       <c r="G15" t="n">
-        <v>0.1129914528905369</v>
+        <v>0.1076308547601151</v>
       </c>
       <c r="H15" t="n">
-        <v>0.1278101821812203</v>
+        <v>0.1115029178878557</v>
       </c>
       <c r="I15" t="n">
-        <v>39.73436635307139</v>
+        <v>39.75636766334441</v>
       </c>
       <c r="J15" t="n">
         <v>30</v>
@@ -1652,7 +1652,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M15" t="n">
@@ -1662,10 +1662,10 @@
         <v>30</v>
       </c>
       <c r="O15" t="n">
-        <v>72.3404255319149</v>
+        <v>76.59574468085107</v>
       </c>
       <c r="P15" t="n">
-        <v>47.23208510638297</v>
+        <v>48.08314893617021</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
@@ -1689,25 +1689,25 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>155.84</v>
+        <v>156.33</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.1383866865704649</v>
+        <v>-0.1047929908950351</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.1245927423884957</v>
+        <v>-0.0920020909566124</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.0333705495596079</v>
+        <v>-0.0738744075829384</v>
       </c>
       <c r="G16" t="n">
-        <v>0.0522329449787333</v>
+        <v>0.0052176343917886</v>
       </c>
       <c r="H16" t="n">
-        <v>0.0670516742694167</v>
+        <v>0.0090896975195292</v>
       </c>
       <c r="I16" t="n">
-        <v>41.96670995159958</v>
+        <v>48.29804341999465</v>
       </c>
       <c r="J16" t="n">
         <v>40</v>
@@ -1717,7 +1717,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M16" t="n">
@@ -1727,10 +1727,10 @@
         <v>40</v>
       </c>
       <c r="O16" t="n">
-        <v>61.70212765957447</v>
+        <v>55.31914893617022</v>
       </c>
       <c r="P16" t="n">
-        <v>49.38442553191489</v>
+        <v>48.10782978723404</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>
@@ -1754,48 +1754,48 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>6838</v>
+        <v>6789</v>
       </c>
       <c r="D17" t="n">
-        <v>-0.1081838930551026</v>
+        <v>-0.0852253587549687</v>
       </c>
       <c r="E17" t="n">
-        <v>-0.0253705815279361</v>
+        <v>-0.1171077443266792</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0095224034841663</v>
+        <v>0.019752159218926</v>
       </c>
       <c r="G17" t="n">
-        <v>0.09512589802250759</v>
+        <v>0.0988442011936531</v>
       </c>
       <c r="H17" t="n">
-        <v>0.1099446273131909</v>
+        <v>0.1027162643213936</v>
       </c>
       <c r="I17" t="n">
-        <v>38.41490794791199</v>
+        <v>53.60275689223057</v>
       </c>
       <c r="J17" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K17" t="n">
         <v>54.65</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M17" t="n">
         <v>54.65</v>
       </c>
       <c r="N17" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O17" t="n">
-        <v>70.21276595744681</v>
+        <v>74.46808510638297</v>
       </c>
       <c r="P17" t="n">
-        <v>47.90255319148936</v>
+        <v>52.7536170212766</v>
       </c>
       <c r="Q17" t="b">
         <v>0</v>
@@ -1819,48 +1819,48 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>631.85</v>
+        <v>633.8</v>
       </c>
       <c r="D18" t="n">
-        <v>-0.0540459615240661</v>
+        <v>-0.08436867957237799</v>
       </c>
       <c r="E18" t="n">
-        <v>0.06461668070766639</v>
+        <v>0.0360441356763383</v>
       </c>
       <c r="F18" t="n">
-        <v>-0.0445334946317858</v>
+        <v>-0.0464154066049801</v>
       </c>
       <c r="G18" t="n">
-        <v>0.0410699999065554</v>
+        <v>0.0326766353697469</v>
       </c>
       <c r="H18" t="n">
-        <v>0.0558887291972388</v>
+        <v>0.0365486984974875</v>
       </c>
       <c r="I18" t="n">
-        <v>36.88269073010667</v>
+        <v>42.69977595220314</v>
       </c>
       <c r="J18" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K18" t="n">
         <v>49.92</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M18" t="n">
         <v>49.92</v>
       </c>
       <c r="N18" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O18" t="n">
         <v>59.57446808510638</v>
       </c>
       <c r="P18" t="n">
-        <v>43.88289361702128</v>
+        <v>47.88289361702128</v>
       </c>
       <c r="Q18" t="b">
         <v>0</v>
@@ -1884,25 +1884,25 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2252</v>
+        <v>2251.9</v>
       </c>
       <c r="D19" t="n">
-        <v>-0.1515014505858859</v>
+        <v>-0.1010379241516965</v>
       </c>
       <c r="E19" t="n">
-        <v>-0.1471958192903396</v>
+        <v>-0.1305069693810572</v>
       </c>
       <c r="F19" t="n">
-        <v>-0.2445994901381993</v>
+        <v>-0.2595357095883203</v>
       </c>
       <c r="G19" t="n">
-        <v>-0.1589959955998581</v>
+        <v>-0.1804436676135932</v>
       </c>
       <c r="H19" t="n">
-        <v>-0.1441772663091747</v>
+        <v>-0.1765716044858526</v>
       </c>
       <c r="I19" t="n">
-        <v>32.90703393999017</v>
+        <v>36.29951166576236</v>
       </c>
       <c r="J19" t="n">
         <v>30</v>
@@ -1912,7 +1912,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M19" t="n">
@@ -1922,10 +1922,10 @@
         <v>30</v>
       </c>
       <c r="O19" t="n">
-        <v>21.27659574468085</v>
+        <v>17.02127659574468</v>
       </c>
       <c r="P19" t="n">
-        <v>36.76331914893618</v>
+        <v>35.91225531914894</v>
       </c>
       <c r="Q19" t="b">
         <v>0</v>
@@ -1949,25 +1949,25 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>1974.7</v>
+        <v>1985.3</v>
       </c>
       <c r="D20" t="n">
-        <v>-0.09230062054700069</v>
+        <v>-0.06850279172336129</v>
       </c>
       <c r="E20" t="n">
-        <v>-0.1405005440696408</v>
+        <v>-0.1217041231640417</v>
       </c>
       <c r="F20" t="n">
-        <v>-0.095460583573817</v>
+        <v>-0.06802178199230111</v>
       </c>
       <c r="G20" t="n">
-        <v>-0.0098570890354757</v>
+        <v>0.0110702599824259</v>
       </c>
       <c r="H20" t="n">
-        <v>0.0049616402552076</v>
+        <v>0.0149423231101665</v>
       </c>
       <c r="I20" t="n">
-        <v>41.24948282995449</v>
+        <v>45.41721660067459</v>
       </c>
       <c r="J20" t="n">
         <v>40</v>
@@ -1977,7 +1977,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M20" t="n">
@@ -1987,10 +1987,10 @@
         <v>40</v>
       </c>
       <c r="O20" t="n">
-        <v>53.19148936170212</v>
+        <v>57.44680851063831</v>
       </c>
       <c r="P20" t="n">
-        <v>46.26229787234043</v>
+        <v>47.11336170212766</v>
       </c>
       <c r="Q20" t="b">
         <v>0</v>
@@ -2014,25 +2014,25 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>866.2</v>
+        <v>876.7</v>
       </c>
       <c r="D21" t="n">
-        <v>-0.0916050547952387</v>
+        <v>-0.0550255995688493</v>
       </c>
       <c r="E21" t="n">
-        <v>-0.1047028423772609</v>
+        <v>-0.1318082788671023</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.3118843342866221</v>
+        <v>-0.3058041016707578</v>
       </c>
       <c r="G21" t="n">
-        <v>-0.2262808397482808</v>
+        <v>-0.2267120596960307</v>
       </c>
       <c r="H21" t="n">
-        <v>-0.2114621104575974</v>
+        <v>-0.2228399965682901</v>
       </c>
       <c r="I21" t="n">
-        <v>47.93689320388352</v>
+        <v>55.66567558638918</v>
       </c>
       <c r="J21" t="n">
         <v>60</v>
@@ -2042,7 +2042,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M21" t="n">
@@ -2079,48 +2079,48 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>378.45</v>
+        <v>371.3</v>
       </c>
       <c r="D22" t="n">
-        <v>-0.1175236096537251</v>
+        <v>-0.1005329457364341</v>
       </c>
       <c r="E22" t="n">
-        <v>0.2455158795458283</v>
+        <v>0.2453463021968809</v>
       </c>
       <c r="F22" t="n">
-        <v>0.2012378987462306</v>
+        <v>0.1856937569854704</v>
       </c>
       <c r="G22" t="n">
-        <v>0.2868413932845719</v>
+        <v>0.2647857989601975</v>
       </c>
       <c r="H22" t="n">
-        <v>0.3016601225752553</v>
+        <v>0.268657862087938</v>
       </c>
       <c r="I22" t="n">
-        <v>39.91935483870968</v>
+        <v>44.83695652173915</v>
       </c>
       <c r="J22" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K22" t="n">
         <v>54.47</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M22" t="n">
         <v>54.47</v>
       </c>
       <c r="N22" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O22" t="n">
         <v>91.48936170212764</v>
       </c>
       <c r="P22" t="n">
-        <v>52.08587234042552</v>
+        <v>56.08587234042552</v>
       </c>
       <c r="Q22" t="b">
         <v>0</v>
@@ -2144,25 +2144,25 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>330.85</v>
+        <v>333.55</v>
       </c>
       <c r="D23" t="n">
-        <v>-0.0775128955806495</v>
+        <v>-0.0618759668119814</v>
       </c>
       <c r="E23" t="n">
-        <v>-0.1134780278670952</v>
+        <v>-0.1119542066027688</v>
       </c>
       <c r="F23" t="n">
-        <v>-0.1961856171039844</v>
+        <v>-0.1923728813559322</v>
       </c>
       <c r="G23" t="n">
-        <v>-0.1105821225656431</v>
+        <v>-0.1132808393812051</v>
       </c>
       <c r="H23" t="n">
-        <v>-0.0957633932749597</v>
+        <v>-0.1094087762534645</v>
       </c>
       <c r="I23" t="n">
-        <v>35.56763285024155</v>
+        <v>39.49631449631451</v>
       </c>
       <c r="J23" t="n">
         <v>30</v>
@@ -2172,7 +2172,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M23" t="n">
@@ -2182,10 +2182,10 @@
         <v>30</v>
       </c>
       <c r="O23" t="n">
-        <v>34.04255319148936</v>
+        <v>36.17021276595745</v>
       </c>
       <c r="P23" t="n">
-        <v>38.68851063829788</v>
+        <v>39.1140425531915</v>
       </c>
       <c r="Q23" t="b">
         <v>0</v>
@@ -2209,25 +2209,25 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>119.95</v>
+        <v>116.04</v>
       </c>
       <c r="D24" t="n">
-        <v>-0.1636452377632128</v>
+        <v>-0.1542274052478133</v>
       </c>
       <c r="E24" t="n">
-        <v>-0.038785159067233</v>
+        <v>-0.08326749881497859</v>
       </c>
       <c r="F24" t="n">
-        <v>0.09144676979071879</v>
+        <v>0.0725575376652187</v>
       </c>
       <c r="G24" t="n">
-        <v>0.1770502643290601</v>
+        <v>0.1516495796399458</v>
       </c>
       <c r="H24" t="n">
-        <v>0.1918689936197435</v>
+        <v>0.1555216427676864</v>
       </c>
       <c r="I24" t="n">
-        <v>47.70744384629664</v>
+        <v>48.56386999244142</v>
       </c>
       <c r="J24" t="n">
         <v>40</v>
@@ -2237,7 +2237,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M24" t="n">
@@ -2274,25 +2274,25 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>561.1</v>
+        <v>561.7</v>
       </c>
       <c r="D25" t="n">
-        <v>0.0641001327517543</v>
+        <v>0.1057086614173228</v>
       </c>
       <c r="E25" t="n">
-        <v>-0.0170797932907068</v>
+        <v>-0.1046465290507691</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.1047467092142001</v>
+        <v>-0.1103191573612101</v>
       </c>
       <c r="G25" t="n">
-        <v>-0.0191432146758588</v>
+        <v>-0.031227115386483</v>
       </c>
       <c r="H25" t="n">
-        <v>-0.0043244853851754</v>
+        <v>-0.0273550522587424</v>
       </c>
       <c r="I25" t="n">
-        <v>56.87363038714392</v>
+        <v>60.43020736614052</v>
       </c>
       <c r="J25" t="n">
         <v>80</v>
@@ -2302,7 +2302,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M25" t="n">
@@ -2339,48 +2339,48 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>125.34</v>
+        <v>127.14</v>
       </c>
       <c r="D26" t="n">
-        <v>-0.0956057435601414</v>
+        <v>-0.0173892881984696</v>
       </c>
       <c r="E26" t="n">
-        <v>-0.1258804658623333</v>
+        <v>-0.0973375931842385</v>
       </c>
       <c r="F26" t="n">
-        <v>-0.3110915686490051</v>
+        <v>-0.2498672488052392</v>
       </c>
       <c r="G26" t="n">
-        <v>-0.2254880741106638</v>
+        <v>-0.1707752068305121</v>
       </c>
       <c r="H26" t="n">
-        <v>-0.2106693448199804</v>
+        <v>-0.1669031437027716</v>
       </c>
       <c r="I26" t="n">
-        <v>38.27248866618948</v>
+        <v>45.95569294178259</v>
       </c>
       <c r="J26" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K26" t="n">
         <v>51.54</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M26" t="n">
         <v>51.54</v>
       </c>
       <c r="N26" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O26" t="n">
-        <v>10.63829787234042</v>
+        <v>19.14893617021277</v>
       </c>
       <c r="P26" t="n">
-        <v>34.74365957446808</v>
+        <v>40.44578723404256</v>
       </c>
       <c r="Q26" t="b">
         <v>0</v>
@@ -2404,25 +2404,25 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>4805.4</v>
+        <v>4785</v>
       </c>
       <c r="D27" t="n">
-        <v>-0.1923697478991597</v>
+        <v>-0.1530223913620674</v>
       </c>
       <c r="E27" t="n">
-        <v>-0.1256550218340612</v>
+        <v>-0.0829819854350325</v>
       </c>
       <c r="F27" t="n">
-        <v>0.1459436256975246</v>
+        <v>0.1431233426503262</v>
       </c>
       <c r="G27" t="n">
-        <v>0.2315471202358658</v>
+        <v>0.2222153846250533</v>
       </c>
       <c r="H27" t="n">
-        <v>0.2463658495265492</v>
+        <v>0.2260874477527938</v>
       </c>
       <c r="I27" t="n">
-        <v>46.77362169828044</v>
+        <v>49.33389426447903</v>
       </c>
       <c r="J27" t="n">
         <v>40</v>
@@ -2432,7 +2432,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M27" t="n">
@@ -2469,25 +2469,25 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1593.5</v>
+        <v>1613.9</v>
       </c>
       <c r="D28" t="n">
-        <v>-0.0423102349900835</v>
+        <v>0.0522918432548737</v>
       </c>
       <c r="E28" t="n">
-        <v>0.07574427867413749</v>
+        <v>0.0449336354807381</v>
       </c>
       <c r="F28" t="n">
-        <v>0.3990342405618963</v>
+        <v>0.4464061659795664</v>
       </c>
       <c r="G28" t="n">
-        <v>0.4846377351002375</v>
+        <v>0.5254982079542935</v>
       </c>
       <c r="H28" t="n">
-        <v>0.4994564643909209</v>
+        <v>0.529370271082034</v>
       </c>
       <c r="I28" t="n">
-        <v>63.56641468682506</v>
+        <v>62.49826316520774</v>
       </c>
       <c r="J28" t="n">
         <v>80</v>
@@ -2497,7 +2497,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M28" t="n">
@@ -2507,10 +2507,10 @@
         <v>80</v>
       </c>
       <c r="O28" t="n">
-        <v>95.74468085106383</v>
+        <v>97.87234042553192</v>
       </c>
       <c r="P28" t="n">
-        <v>72.95293617021277</v>
+        <v>73.37846808510639</v>
       </c>
       <c r="Q28" t="b">
         <v>0</v>
@@ -2534,48 +2534,48 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>514.15</v>
+        <v>501.4</v>
       </c>
       <c r="D29" t="n">
-        <v>-0.0492788461538461</v>
+        <v>-0.0452251737598781</v>
       </c>
       <c r="E29" t="n">
-        <v>-0.1210359859817079</v>
+        <v>-0.1266329907681589</v>
       </c>
       <c r="F29" t="n">
-        <v>-0.0021348859776807</v>
+        <v>-0.0166699352814276</v>
       </c>
       <c r="G29" t="n">
-        <v>0.0834686085606605</v>
+        <v>0.0624221066932993</v>
       </c>
       <c r="H29" t="n">
-        <v>0.0982873378513439</v>
+        <v>0.0662941698210399</v>
       </c>
       <c r="I29" t="n">
-        <v>61.53039832285116</v>
+        <v>56.60559305689488</v>
       </c>
       <c r="J29" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="K29" t="n">
         <v>49.42</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M29" t="n">
         <v>49.42</v>
       </c>
       <c r="N29" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="O29" t="n">
-        <v>65.95744680851064</v>
+        <v>63.82978723404256</v>
       </c>
       <c r="P29" t="n">
-        <v>56.95948936170213</v>
+        <v>48.53395744680852</v>
       </c>
       <c r="Q29" t="b">
         <v>0</v>
@@ -2599,48 +2599,48 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>107.84</v>
+        <v>108.6</v>
       </c>
       <c r="D30" t="n">
-        <v>-0.0438020925696045</v>
+        <v>-0.0553235908141962</v>
       </c>
       <c r="E30" t="n">
-        <v>0.0170706403847968</v>
+        <v>0.0155227230222554</v>
       </c>
       <c r="F30" t="n">
-        <v>-0.1954640405848999</v>
+        <v>-0.1831515607371192</v>
       </c>
       <c r="G30" t="n">
-        <v>-0.1098605460465587</v>
+        <v>-0.1040595187623921</v>
       </c>
       <c r="H30" t="n">
-        <v>-0.09504181675587529</v>
+        <v>-0.1001874556346515</v>
       </c>
       <c r="I30" t="n">
-        <v>26.06075822244538</v>
+        <v>30.56241426611795</v>
       </c>
       <c r="J30" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="K30" t="n">
         <v>52.38</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M30" t="n">
         <v>52.38</v>
       </c>
       <c r="N30" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="O30" t="n">
-        <v>36.17021276595745</v>
+        <v>38.29787234042553</v>
       </c>
       <c r="P30" t="n">
-        <v>36.18604255319149</v>
+        <v>40.61157446808511</v>
       </c>
       <c r="Q30" t="b">
         <v>0</v>
@@ -2664,25 +2664,25 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>38.2</v>
+        <v>37.07</v>
       </c>
       <c r="D31" t="n">
-        <v>-0.09585798816568029</v>
+        <v>-0.1054536679536679</v>
       </c>
       <c r="E31" t="n">
-        <v>-0.1679372685689391</v>
+        <v>-0.2359851607584502</v>
       </c>
       <c r="F31" t="n">
-        <v>-0.2282828282828282</v>
+        <v>-0.2420772848088325</v>
       </c>
       <c r="G31" t="n">
-        <v>-0.1426793337444869</v>
+        <v>-0.1629852428341054</v>
       </c>
       <c r="H31" t="n">
-        <v>-0.1278606044538035</v>
+        <v>-0.1591131797063648</v>
       </c>
       <c r="I31" t="n">
-        <v>39.57399103139014</v>
+        <v>38.91951488423375</v>
       </c>
       <c r="J31" t="n">
         <v>30</v>
@@ -2692,7 +2692,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M31" t="n">
@@ -2702,10 +2702,10 @@
         <v>30</v>
       </c>
       <c r="O31" t="n">
-        <v>27.65957446808511</v>
+        <v>21.27659574468085</v>
       </c>
       <c r="P31" t="n">
-        <v>37.12791489361702</v>
+        <v>35.85131914893617</v>
       </c>
       <c r="Q31" t="b">
         <v>0</v>
@@ -2729,25 +2729,25 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>664.15</v>
+        <v>659.5</v>
       </c>
       <c r="D32" t="n">
-        <v>-0.0936817685589519</v>
+        <v>-0.06513572896732581</v>
       </c>
       <c r="E32" t="n">
-        <v>-0.1893194995422643</v>
+        <v>-0.2085208520852085</v>
       </c>
       <c r="F32" t="n">
-        <v>-0.4078020508247882</v>
+        <v>-0.4136214101538188</v>
       </c>
       <c r="G32" t="n">
-        <v>-0.322198556286447</v>
+        <v>-0.3345293681790917</v>
       </c>
       <c r="H32" t="n">
-        <v>-0.3073798269957636</v>
+        <v>-0.3306573050513511</v>
       </c>
       <c r="I32" t="n">
-        <v>45.96112311015118</v>
+        <v>50.82802547770701</v>
       </c>
       <c r="J32" t="n">
         <v>40</v>
@@ -2757,7 +2757,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M32" t="n">
@@ -2794,48 +2794,48 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>537.9</v>
+        <v>529.85</v>
       </c>
       <c r="D33" t="n">
-        <v>-0.0800410466906106</v>
+        <v>-0.0617141845227554</v>
       </c>
       <c r="E33" t="n">
-        <v>-0.113034875092753</v>
+        <v>-0.1985327484495538</v>
       </c>
       <c r="F33" t="n">
-        <v>0.0354186717998075</v>
+        <v>0.0150383141762453</v>
       </c>
       <c r="G33" t="n">
-        <v>0.1210221663381487</v>
+        <v>0.0941303561509724</v>
       </c>
       <c r="H33" t="n">
-        <v>0.1358408956288321</v>
+        <v>0.098002419278713</v>
       </c>
       <c r="I33" t="n">
-        <v>48.93556627873971</v>
+        <v>54.07779171894605</v>
       </c>
       <c r="J33" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="K33" t="n">
         <v>49.98</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M33" t="n">
         <v>49.98</v>
       </c>
       <c r="N33" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="O33" t="n">
-        <v>74.46808510638297</v>
+        <v>70.21276595744681</v>
       </c>
       <c r="P33" t="n">
-        <v>58.8856170212766</v>
+        <v>50.03455319148937</v>
       </c>
       <c r="Q33" t="b">
         <v>0</v>
@@ -2871,10 +2871,10 @@
         <v>-0.2401052253975846</v>
       </c>
       <c r="G34" t="n">
-        <v>-0.1545017308592433</v>
+        <v>-0.1610131834228575</v>
       </c>
       <c r="H34" t="n">
-        <v>-0.1396830015685599</v>
+        <v>-0.1571411202951169</v>
       </c>
       <c r="I34" t="n">
         <v>63.3225806451613</v>
@@ -2887,7 +2887,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M34" t="n">
@@ -2924,25 +2924,25 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>108.49</v>
+        <v>108.75</v>
       </c>
       <c r="D35" t="n">
-        <v>-0.1324270291883247</v>
+        <v>-0.0693196405648266</v>
       </c>
       <c r="E35" t="n">
-        <v>-0.0847815083516113</v>
+        <v>-0.2015418502202642</v>
       </c>
       <c r="F35" t="n">
-        <v>0.0542221358468564</v>
+        <v>0.06890112050324371</v>
       </c>
       <c r="G35" t="n">
-        <v>0.1398256303851976</v>
+        <v>0.1479931624779707</v>
       </c>
       <c r="H35" t="n">
-        <v>0.154644359675881</v>
+        <v>0.1518652256057113</v>
       </c>
       <c r="I35" t="n">
-        <v>46.81259600614439</v>
+        <v>53.28719723183392</v>
       </c>
       <c r="J35" t="n">
         <v>60</v>
@@ -2952,7 +2952,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M35" t="n">
@@ -2962,10 +2962,10 @@
         <v>60</v>
       </c>
       <c r="O35" t="n">
-        <v>78.72340425531915</v>
+        <v>80.85106382978722</v>
       </c>
       <c r="P35" t="n">
-        <v>59.37268085106383</v>
+        <v>59.79821276595744</v>
       </c>
       <c r="Q35" t="b">
         <v>0</v>
@@ -2989,48 +2989,48 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>460.4</v>
+        <v>461.35</v>
       </c>
       <c r="D36" t="n">
-        <v>-0.08714186576782</v>
+        <v>-0.0760989286071893</v>
       </c>
       <c r="E36" t="n">
-        <v>-0.1794689003742648</v>
+        <v>-0.1613343028540265</v>
       </c>
       <c r="F36" t="n">
-        <v>0.0073296138278087</v>
+        <v>0.0002168021680217</v>
       </c>
       <c r="G36" t="n">
-        <v>0.0929331083661499</v>
+        <v>0.0793088441427488</v>
       </c>
       <c r="H36" t="n">
-        <v>0.1077518376568333</v>
+        <v>0.08318090727048939</v>
       </c>
       <c r="I36" t="n">
-        <v>38.56184798807747</v>
+        <v>41.17187500000001</v>
       </c>
       <c r="J36" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K36" t="n">
         <v>47.8</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M36" t="n">
         <v>47.8</v>
       </c>
       <c r="N36" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O36" t="n">
         <v>68.08510638297872</v>
       </c>
       <c r="P36" t="n">
-        <v>44.73702127659575</v>
+        <v>48.73702127659575</v>
       </c>
       <c r="Q36" t="b">
         <v>0</v>
@@ -3054,25 +3054,25 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2142.4</v>
+        <v>2136.6</v>
       </c>
       <c r="D37" t="n">
-        <v>-0.0392394277770303</v>
+        <v>-0.0145288501452884</v>
       </c>
       <c r="E37" t="n">
-        <v>0.2608286252354048</v>
+        <v>0.2740608228980321</v>
       </c>
       <c r="F37" t="n">
-        <v>0.5370928397187547</v>
+        <v>0.5095379398050019</v>
       </c>
       <c r="G37" t="n">
-        <v>0.6226963342570959</v>
+        <v>0.588629981779729</v>
       </c>
       <c r="H37" t="n">
-        <v>0.6375150635477793</v>
+        <v>0.5925020449074696</v>
       </c>
       <c r="I37" t="n">
-        <v>53.38727076591155</v>
+        <v>61.35631043887923</v>
       </c>
       <c r="J37" t="n">
         <v>80</v>
@@ -3082,7 +3082,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M37" t="n">
@@ -3119,25 +3119,25 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>742.05</v>
+        <v>736.1</v>
       </c>
       <c r="D38" t="n">
-        <v>-0.172050209205021</v>
+        <v>-0.1459070603933399</v>
       </c>
       <c r="E38" t="n">
-        <v>-0.2190591454430647</v>
+        <v>-0.2172063593342904</v>
       </c>
       <c r="F38" t="n">
-        <v>-0.2986294896030246</v>
+        <v>-0.3016791575751825</v>
       </c>
       <c r="G38" t="n">
-        <v>-0.2130259950646833</v>
+        <v>-0.2225871156004554</v>
       </c>
       <c r="H38" t="n">
-        <v>-0.1982072657739999</v>
+        <v>-0.2187150524727148</v>
       </c>
       <c r="I38" t="n">
-        <v>40.37668408028594</v>
+        <v>43.53045798132504</v>
       </c>
       <c r="J38" t="n">
         <v>40</v>
@@ -3147,7 +3147,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M38" t="n">
@@ -3157,10 +3157,10 @@
         <v>40</v>
       </c>
       <c r="O38" t="n">
-        <v>12.76595744680851</v>
+        <v>10.63829787234042</v>
       </c>
       <c r="P38" t="n">
-        <v>38.5011914893617</v>
+        <v>38.07565957446808</v>
       </c>
       <c r="Q38" t="b">
         <v>0</v>
@@ -3184,48 +3184,48 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>3025.2</v>
+        <v>2928.4</v>
       </c>
       <c r="D39" t="n">
-        <v>-0.0165149544863459</v>
+        <v>-0.0138407139249031</v>
       </c>
       <c r="E39" t="n">
-        <v>-0.0247896586183553</v>
+        <v>-0.0956145768993205</v>
       </c>
       <c r="F39" t="n">
-        <v>0.1217323593755792</v>
+        <v>0.1000338078960221</v>
       </c>
       <c r="G39" t="n">
-        <v>0.2073358539139205</v>
+        <v>0.1791258498707492</v>
       </c>
       <c r="H39" t="n">
-        <v>0.2221545832046039</v>
+        <v>0.1829979129984897</v>
       </c>
       <c r="I39" t="n">
-        <v>52.32580398162328</v>
+        <v>53.54029967681912</v>
       </c>
       <c r="J39" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="K39" t="n">
         <v>48.69</v>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M39" t="n">
         <v>48.69</v>
       </c>
       <c r="N39" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="O39" t="n">
-        <v>87.2340425531915</v>
+        <v>85.1063829787234</v>
       </c>
       <c r="P39" t="n">
-        <v>68.9228085106383</v>
+        <v>52.49727659574468</v>
       </c>
       <c r="Q39" t="b">
         <v>0</v>
@@ -3249,25 +3249,25 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>187.9</v>
+        <v>189.25</v>
       </c>
       <c r="D40" t="n">
-        <v>-0.08697764820213801</v>
+        <v>-0.0346357886145684</v>
       </c>
       <c r="E40" t="n">
-        <v>-0.0035530572201304</v>
+        <v>-0.0229736706246772</v>
       </c>
       <c r="F40" t="n">
-        <v>-0.2307062436028658</v>
+        <v>-0.2244170320888487</v>
       </c>
       <c r="G40" t="n">
-        <v>-0.1451027490645245</v>
+        <v>-0.1453249901141217</v>
       </c>
       <c r="H40" t="n">
-        <v>-0.1302840197738412</v>
+        <v>-0.1414529269863811</v>
       </c>
       <c r="I40" t="n">
-        <v>46.99369125788593</v>
+        <v>54.87893286936349</v>
       </c>
       <c r="J40" t="n">
         <v>60</v>
@@ -3277,7 +3277,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M40" t="n">
@@ -3314,25 +3314,25 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>752.9</v>
+        <v>749.9</v>
       </c>
       <c r="D41" t="n">
-        <v>-0.1110455162642423</v>
+        <v>-0.1028831199904294</v>
       </c>
       <c r="E41" t="n">
-        <v>-0.1957055870099349</v>
+        <v>-0.1976675760980045</v>
       </c>
       <c r="F41" t="n">
-        <v>-0.2619351044015293</v>
+        <v>-0.2616914443241115</v>
       </c>
       <c r="G41" t="n">
-        <v>-0.176331609863188</v>
+        <v>-0.1825994023493844</v>
       </c>
       <c r="H41" t="n">
-        <v>-0.1615128805725046</v>
+        <v>-0.1787273392216438</v>
       </c>
       <c r="I41" t="n">
-        <v>20.93984962406016</v>
+        <v>21.74931667317455</v>
       </c>
       <c r="J41" t="n">
         <v>20</v>
@@ -3342,7 +3342,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M41" t="n">
@@ -3352,10 +3352,10 @@
         <v>20</v>
       </c>
       <c r="O41" t="n">
-        <v>17.02127659574468</v>
+        <v>14.8936170212766</v>
       </c>
       <c r="P41" t="n">
-        <v>30.62425531914894</v>
+        <v>30.19872340425532</v>
       </c>
       <c r="Q41" t="b">
         <v>0</v>
@@ -3379,25 +3379,25 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>497.65</v>
+        <v>497.15</v>
       </c>
       <c r="D42" t="n">
-        <v>-0.1480784045193871</v>
+        <v>-0.126887952230418</v>
       </c>
       <c r="E42" t="n">
-        <v>-0.2617564159620235</v>
+        <v>-0.2757666253915071</v>
       </c>
       <c r="F42" t="n">
-        <v>-0.3572074399380006</v>
+        <v>-0.354434489027399</v>
       </c>
       <c r="G42" t="n">
-        <v>-0.2716039453996594</v>
+        <v>-0.2753424470526719</v>
       </c>
       <c r="H42" t="n">
-        <v>-0.256785216108976</v>
+        <v>-0.2714703839249314</v>
       </c>
       <c r="I42" t="n">
-        <v>32.13596914175506</v>
+        <v>36.97642163661581</v>
       </c>
       <c r="J42" t="n">
         <v>30</v>
@@ -3407,7 +3407,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M42" t="n">
@@ -3417,10 +3417,10 @@
         <v>30</v>
       </c>
       <c r="O42" t="n">
-        <v>4.25531914893617</v>
+        <v>6.382978723404255</v>
       </c>
       <c r="P42" t="n">
-        <v>31.91506382978724</v>
+        <v>32.34059574468085</v>
       </c>
       <c r="Q42" t="b">
         <v>0</v>
@@ -3444,25 +3444,25 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>421.95</v>
+        <v>411.55</v>
       </c>
       <c r="D43" t="n">
-        <v>-0.0212247738343772</v>
+        <v>-0.0267234243821686</v>
       </c>
       <c r="E43" t="n">
-        <v>-0.0511580841016415</v>
+        <v>-0.1120819848975188</v>
       </c>
       <c r="F43" t="n">
-        <v>-0.0810192747468147</v>
+        <v>-0.1023991275899672</v>
       </c>
       <c r="G43" t="n">
-        <v>0.0045842197915265</v>
+        <v>-0.0233070856152401</v>
       </c>
       <c r="H43" t="n">
-        <v>0.0194029490822099</v>
+        <v>-0.0194350224874996</v>
       </c>
       <c r="I43" t="n">
-        <v>56.05234460196291</v>
+        <v>54.21940928270043</v>
       </c>
       <c r="J43" t="n">
         <v>60</v>
@@ -3472,7 +3472,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M43" t="n">
@@ -3482,16 +3482,16 @@
         <v>60</v>
       </c>
       <c r="O43" t="n">
-        <v>55.31914893617022</v>
+        <v>53.19148936170212</v>
       </c>
       <c r="P43" t="n">
-        <v>55.65582978723404</v>
+        <v>55.23029787234042</v>
       </c>
       <c r="Q43" t="b">
         <v>0</v>
       </c>
       <c r="R43" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S43" t="b">
         <v>0</v>
@@ -3509,25 +3509,25 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>243.31</v>
+        <v>246.66</v>
       </c>
       <c r="D44" t="n">
-        <v>-0.0398184688239936</v>
+        <v>0.0161071060762101</v>
       </c>
       <c r="E44" t="n">
-        <v>-0.1333570792520035</v>
+        <v>-0.1028914348063284</v>
       </c>
       <c r="F44" t="n">
-        <v>-0.2099042052281213</v>
+        <v>-0.1753259779338014</v>
       </c>
       <c r="G44" t="n">
-        <v>-0.1243007106897801</v>
+        <v>-0.0962339359590743</v>
       </c>
       <c r="H44" t="n">
-        <v>-0.1094819813990967</v>
+        <v>-0.09236187283133369</v>
       </c>
       <c r="I44" t="n">
-        <v>45.10558861276397</v>
+        <v>49.41771556287495</v>
       </c>
       <c r="J44" t="n">
         <v>60</v>
@@ -3537,7 +3537,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M44" t="n">
@@ -3547,10 +3547,10 @@
         <v>60</v>
       </c>
       <c r="O44" t="n">
-        <v>31.91489361702128</v>
+        <v>40.42553191489361</v>
       </c>
       <c r="P44" t="n">
-        <v>49.26297872340426</v>
+        <v>50.96510638297872</v>
       </c>
       <c r="Q44" t="b">
         <v>0</v>
@@ -3574,48 +3574,48 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>86.75</v>
+        <v>89.8</v>
       </c>
       <c r="D45" t="n">
-        <v>-0.1530801522991312</v>
+        <v>-0.1173579712993906</v>
       </c>
       <c r="E45" t="n">
-        <v>-0.2473538087801492</v>
+        <v>-0.1866678742867493</v>
       </c>
       <c r="F45" t="n">
-        <v>-0.3546827345086663</v>
+        <v>-0.3683173888576252</v>
       </c>
       <c r="G45" t="n">
-        <v>-0.269079239970325</v>
+        <v>-0.2892253468828981</v>
       </c>
       <c r="H45" t="n">
-        <v>-0.2542605106796416</v>
+        <v>-0.2853532837551575</v>
       </c>
       <c r="I45" t="n">
-        <v>28.92606583917967</v>
+        <v>36.57370517928285</v>
       </c>
       <c r="J45" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="K45" t="n">
         <v>59.6</v>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M45" t="n">
         <v>59.6</v>
       </c>
       <c r="N45" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="O45" t="n">
-        <v>6.382978723404255</v>
+        <v>4.25531914893617</v>
       </c>
       <c r="P45" t="n">
-        <v>33.11659574468086</v>
+        <v>36.69106382978724</v>
       </c>
       <c r="Q45" t="b">
         <v>0</v>
@@ -3639,25 +3639,25 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>478.35</v>
+        <v>490</v>
       </c>
       <c r="D46" t="n">
-        <v>-0.08929081389814369</v>
+        <v>-0.0479891198756557</v>
       </c>
       <c r="E46" t="n">
-        <v>-0.2642467122971621</v>
+        <v>-0.170335252285811</v>
       </c>
       <c r="F46" t="n">
-        <v>-0.2194664273476381</v>
+        <v>-0.1958644457208501</v>
       </c>
       <c r="G46" t="n">
-        <v>-0.1338629328092968</v>
+        <v>-0.116772403746123</v>
       </c>
       <c r="H46" t="n">
-        <v>-0.1190442035186134</v>
+        <v>-0.1129003406183825</v>
       </c>
       <c r="I46" t="n">
-        <v>44.87334137515078</v>
+        <v>52.84003684372122</v>
       </c>
       <c r="J46" t="n">
         <v>40</v>
@@ -3667,7 +3667,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M46" t="n">
@@ -3677,10 +3677,10 @@
         <v>40</v>
       </c>
       <c r="O46" t="n">
-        <v>29.78723404255319</v>
+        <v>31.91489361702128</v>
       </c>
       <c r="P46" t="n">
-        <v>41.80144680851064</v>
+        <v>42.22697872340426</v>
       </c>
       <c r="Q46" t="b">
         <v>0</v>
@@ -3704,48 +3704,48 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>987.55</v>
+        <v>974.35</v>
       </c>
       <c r="D47" t="n">
-        <v>0.1265685603467943</v>
+        <v>0.1176301904106447</v>
       </c>
       <c r="E47" t="n">
-        <v>0.1727229545184656</v>
+        <v>0.1325700337091713</v>
       </c>
       <c r="F47" t="n">
-        <v>0.3409600108629234</v>
+        <v>0.3150010122140494</v>
       </c>
       <c r="G47" t="n">
-        <v>0.4265635054012646</v>
+        <v>0.3940930541887765</v>
       </c>
       <c r="H47" t="n">
-        <v>0.441382234691948</v>
+        <v>0.397965117316517</v>
       </c>
       <c r="I47" t="n">
-        <v>56.88173344631399</v>
+        <v>59.59416613823716</v>
       </c>
       <c r="J47" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K47" t="n">
         <v>46.83</v>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M47" t="n">
         <v>46.83</v>
       </c>
       <c r="N47" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O47" t="n">
         <v>93.61702127659576</v>
       </c>
       <c r="P47" t="n">
-        <v>69.45540425531915</v>
+        <v>61.45540425531915</v>
       </c>
       <c r="Q47" t="b">
         <v>0</v>
@@ -3769,25 +3769,25 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>14375</v>
+        <v>13974</v>
       </c>
       <c r="D48" t="n">
-        <v>-0.0216429592322874</v>
+        <v>-0.0170230725942599</v>
       </c>
       <c r="E48" t="n">
-        <v>0.017915309446254</v>
+        <v>-0.0607608549536228</v>
       </c>
       <c r="F48" t="n">
-        <v>0.0471299533799534</v>
+        <v>0.0185873605947954</v>
       </c>
       <c r="G48" t="n">
-        <v>0.1327334479182946</v>
+        <v>0.0976794025695225</v>
       </c>
       <c r="H48" t="n">
-        <v>0.147552177208978</v>
+        <v>0.1015514656972631</v>
       </c>
       <c r="I48" t="n">
-        <v>56.38029058749211</v>
+        <v>55.78125</v>
       </c>
       <c r="J48" t="n">
         <v>60</v>
@@ -3797,7 +3797,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M48" t="n">
@@ -3807,10 +3807,10 @@
         <v>60</v>
       </c>
       <c r="O48" t="n">
-        <v>76.59574468085107</v>
+        <v>72.3404255319149</v>
       </c>
       <c r="P48" t="n">
-        <v>59.43514893617021</v>
+        <v>58.58408510638298</v>
       </c>
       <c r="Q48" t="b">
         <v>0</v>
@@ -3945,25 +3945,25 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1593.5</v>
+        <v>1613.9</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.0423102349900835</v>
+        <v>0.0522918432548737</v>
       </c>
       <c r="E2" t="n">
-        <v>0.07574427867413749</v>
+        <v>0.0449336354807381</v>
       </c>
       <c r="F2" t="n">
-        <v>0.3990342405618963</v>
+        <v>0.4464061659795664</v>
       </c>
       <c r="G2" t="n">
-        <v>0.4846377351002375</v>
+        <v>0.5254982079542935</v>
       </c>
       <c r="H2" t="n">
-        <v>0.4994564643909209</v>
+        <v>0.529370271082034</v>
       </c>
       <c r="I2" t="n">
-        <v>63.56641468682506</v>
+        <v>62.49826316520774</v>
       </c>
       <c r="J2" t="n">
         <v>80</v>
@@ -3973,7 +3973,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M2" t="n">
@@ -3983,10 +3983,10 @@
         <v>80</v>
       </c>
       <c r="O2" t="n">
-        <v>95.74468085106383</v>
+        <v>97.87234042553192</v>
       </c>
       <c r="P2" t="n">
-        <v>72.95293617021277</v>
+        <v>73.37846808510639</v>
       </c>
       <c r="Q2" t="b">
         <v>0</v>
@@ -4010,25 +4010,25 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2142.4</v>
+        <v>2136.6</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.0392394277770303</v>
+        <v>-0.0145288501452884</v>
       </c>
       <c r="E3" t="n">
-        <v>0.2608286252354048</v>
+        <v>0.2740608228980321</v>
       </c>
       <c r="F3" t="n">
-        <v>0.5370928397187547</v>
+        <v>0.5095379398050019</v>
       </c>
       <c r="G3" t="n">
-        <v>0.6226963342570959</v>
+        <v>0.588629981779729</v>
       </c>
       <c r="H3" t="n">
-        <v>0.6375150635477793</v>
+        <v>0.5925020449074696</v>
       </c>
       <c r="I3" t="n">
-        <v>53.38727076591155</v>
+        <v>61.35631043887923</v>
       </c>
       <c r="J3" t="n">
         <v>80</v>
@@ -4038,7 +4038,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M3" t="n">
@@ -4066,63 +4066,63 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>WHEELS</t>
+          <t>ASKAUTOLTD</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Wheels</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>987.55</v>
+        <v>436.5</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1265685603467943</v>
+        <v>0.1303897449177782</v>
       </c>
       <c r="E4" t="n">
-        <v>0.1727229545184656</v>
+        <v>-0.08806016922594791</v>
       </c>
       <c r="F4" t="n">
-        <v>0.3409600108629234</v>
+        <v>-0.1646732370108122</v>
       </c>
       <c r="G4" t="n">
-        <v>0.4265635054012646</v>
+        <v>-0.08558119503608511</v>
       </c>
       <c r="H4" t="n">
-        <v>0.441382234691948</v>
+        <v>-0.0817091319083446</v>
       </c>
       <c r="I4" t="n">
-        <v>56.88173344631399</v>
+        <v>64.88250652741513</v>
       </c>
       <c r="J4" t="n">
         <v>80</v>
       </c>
       <c r="K4" t="n">
-        <v>46.83</v>
+        <v>71.28</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M4" t="n">
-        <v>46.83</v>
+        <v>71.28</v>
       </c>
       <c r="N4" t="n">
         <v>80</v>
       </c>
       <c r="O4" t="n">
-        <v>93.61702127659576</v>
+        <v>42.5531914893617</v>
       </c>
       <c r="P4" t="n">
-        <v>69.45540425531915</v>
+        <v>69.02263829787233</v>
       </c>
       <c r="Q4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S4" t="b">
         <v>0</v>
@@ -4131,63 +4131,63 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SHRIPISTON</t>
+          <t>JBMA</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Engine/Parts</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>3025.2</v>
+        <v>561.7</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.0165149544863459</v>
+        <v>0.1057086614173228</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.0247896586183553</v>
+        <v>-0.1046465290507691</v>
       </c>
       <c r="F5" t="n">
-        <v>0.1217323593755792</v>
+        <v>-0.1103191573612101</v>
       </c>
       <c r="G5" t="n">
-        <v>0.2073358539139205</v>
+        <v>-0.031227115386483</v>
       </c>
       <c r="H5" t="n">
-        <v>0.2221545832046039</v>
+        <v>-0.0273550522587424</v>
       </c>
       <c r="I5" t="n">
-        <v>52.32580398162328</v>
+        <v>60.43020736614052</v>
       </c>
       <c r="J5" t="n">
         <v>80</v>
       </c>
       <c r="K5" t="n">
-        <v>48.69</v>
+        <v>56.91</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M5" t="n">
-        <v>48.69</v>
+        <v>56.91</v>
       </c>
       <c r="N5" t="n">
         <v>80</v>
       </c>
       <c r="O5" t="n">
-        <v>87.2340425531915</v>
+        <v>51.06382978723404</v>
       </c>
       <c r="P5" t="n">
-        <v>68.9228085106383</v>
+        <v>64.9767659574468</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
       </c>
       <c r="R5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S5" t="b">
         <v>0</v>
@@ -4196,63 +4196,63 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ASKAUTOLTD</t>
+          <t>WHEELS</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Wheels</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>435.7</v>
+        <v>974.35</v>
       </c>
       <c r="D6" t="n">
-        <v>0.0889777555611095</v>
+        <v>0.1176301904106447</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.06431869429829271</v>
+        <v>0.1325700337091713</v>
       </c>
       <c r="F6" t="n">
-        <v>-0.1885650433001211</v>
+        <v>0.3150010122140494</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.1029615487617798</v>
+        <v>0.3940930541887765</v>
       </c>
       <c r="H6" t="n">
-        <v>-0.0881428194710964</v>
+        <v>0.397965117316517</v>
       </c>
       <c r="I6" t="n">
-        <v>62.39424703891709</v>
+        <v>59.59416613823716</v>
       </c>
       <c r="J6" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K6" t="n">
-        <v>71.28</v>
+        <v>46.83</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M6" t="n">
-        <v>71.28</v>
+        <v>46.83</v>
       </c>
       <c r="N6" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O6" t="n">
-        <v>38.29787234042553</v>
+        <v>93.61702127659576</v>
       </c>
       <c r="P6" t="n">
-        <v>68.17157446808511</v>
+        <v>61.45540425531915</v>
       </c>
       <c r="Q6" t="b">
+        <v>0</v>
+      </c>
+      <c r="R6" t="b">
         <v>1</v>
-      </c>
-      <c r="R6" t="b">
-        <v>0</v>
       </c>
       <c r="S6" t="b">
         <v>0</v>
@@ -4261,63 +4261,63 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>JBMA</t>
+          <t>RICOAUTO</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Castings</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>561.1</v>
+        <v>108.75</v>
       </c>
       <c r="D7" t="n">
-        <v>0.0641001327517543</v>
+        <v>-0.0693196405648266</v>
       </c>
       <c r="E7" t="n">
-        <v>-0.0170797932907068</v>
+        <v>-0.2015418502202642</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.1047467092142001</v>
+        <v>0.06890112050324371</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.0191432146758588</v>
+        <v>0.1479931624779707</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.0043244853851754</v>
+        <v>0.1518652256057113</v>
       </c>
       <c r="I7" t="n">
-        <v>56.87363038714392</v>
+        <v>53.28719723183392</v>
       </c>
       <c r="J7" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K7" t="n">
-        <v>56.91</v>
+        <v>49.07</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M7" t="n">
-        <v>56.91</v>
+        <v>49.07</v>
       </c>
       <c r="N7" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O7" t="n">
-        <v>51.06382978723404</v>
+        <v>80.85106382978722</v>
       </c>
       <c r="P7" t="n">
-        <v>64.9767659574468</v>
+        <v>59.79821276595744</v>
       </c>
       <c r="Q7" t="b">
         <v>0</v>
       </c>
       <c r="R7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S7" t="b">
         <v>0</v>
@@ -4326,63 +4326,63 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TIINDIA</t>
+          <t>ZFCVINDIA</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Brakes/Transmission</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>2572.7</v>
+        <v>13974</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.0933535382012968</v>
+        <v>-0.0170230725942599</v>
       </c>
       <c r="E8" t="n">
-        <v>-0.0312170507606567</v>
+        <v>-0.0607608549536228</v>
       </c>
       <c r="F8" t="n">
-        <v>-0.183658575281612</v>
+        <v>0.0185873605947954</v>
       </c>
       <c r="G8" t="n">
-        <v>-0.0980550807432707</v>
+        <v>0.0976794025695225</v>
       </c>
       <c r="H8" t="n">
-        <v>-0.0832363514525873</v>
+        <v>0.1015514656972631</v>
       </c>
       <c r="I8" t="n">
-        <v>51.4375</v>
+        <v>55.78125</v>
       </c>
       <c r="J8" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K8" t="n">
-        <v>48.73</v>
+        <v>50.29</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M8" t="n">
-        <v>48.73</v>
+        <v>50.29</v>
       </c>
       <c r="N8" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O8" t="n">
-        <v>42.5531914893617</v>
+        <v>72.3404255319149</v>
       </c>
       <c r="P8" t="n">
-        <v>60.00263829787234</v>
+        <v>58.58408510638298</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
       </c>
       <c r="R8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S8" t="b">
         <v>0</v>
@@ -4391,63 +4391,63 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ZFCVINDIA</t>
+          <t>TIINDIA</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Brakes/Transmission</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>14375</v>
+        <v>2567.3</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.0216429592322874</v>
+        <v>-0.0735448017032945</v>
       </c>
       <c r="E9" t="n">
-        <v>0.017915309446254</v>
+        <v>-0.0179029111357635</v>
       </c>
       <c r="F9" t="n">
-        <v>0.0471299533799534</v>
+        <v>-0.2064232944885783</v>
       </c>
       <c r="G9" t="n">
-        <v>0.1327334479182946</v>
+        <v>-0.1273312525138512</v>
       </c>
       <c r="H9" t="n">
-        <v>0.147552177208978</v>
+        <v>-0.1234591893861106</v>
       </c>
       <c r="I9" t="n">
-        <v>56.38029058749211</v>
+        <v>57.64112620815244</v>
       </c>
       <c r="J9" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K9" t="n">
-        <v>50.29</v>
+        <v>48.73</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M9" t="n">
-        <v>50.29</v>
+        <v>48.73</v>
       </c>
       <c r="N9" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O9" t="n">
-        <v>76.59574468085107</v>
+        <v>29.78723404255319</v>
       </c>
       <c r="P9" t="n">
-        <v>59.43514893617021</v>
+        <v>57.44944680851064</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
       </c>
       <c r="R9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S9" t="b">
         <v>0</v>
@@ -4456,57 +4456,57 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>RICOAUTO</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Castings</t>
+          <t>Forgings</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>108.49</v>
+        <v>1642.6</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.1324270291883247</v>
+        <v>-0.1081550656966011</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.0847815083516113</v>
+        <v>0.1171109902067464</v>
       </c>
       <c r="F10" t="n">
-        <v>0.0542221358468564</v>
+        <v>0.3689474122843568</v>
       </c>
       <c r="G10" t="n">
-        <v>0.1398256303851976</v>
+        <v>0.4480394542590838</v>
       </c>
       <c r="H10" t="n">
-        <v>0.154644359675881</v>
+        <v>0.4519115173868244</v>
       </c>
       <c r="I10" t="n">
-        <v>46.81259600614439</v>
+        <v>46.51959734418505</v>
       </c>
       <c r="J10" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="K10" t="n">
-        <v>49.07</v>
+        <v>54.83</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M10" t="n">
-        <v>49.07</v>
+        <v>54.83</v>
       </c>
       <c r="N10" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="O10" t="n">
-        <v>78.72340425531915</v>
+        <v>95.74468085106383</v>
       </c>
       <c r="P10" t="n">
-        <v>59.37268085106383</v>
+        <v>57.08093617021277</v>
       </c>
       <c r="Q10" t="b">
         <v>0</v>
@@ -4521,63 +4521,63 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>PRICOLLTD</t>
+          <t>RANEENGINE</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Engine/Parts</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>537.9</v>
+        <v>317.75</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.0800410466906106</v>
+        <v>0.1790352504638219</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.113034875092753</v>
+        <v>-0.156154561147258</v>
       </c>
       <c r="F11" t="n">
-        <v>0.0354186717998075</v>
+        <v>-0.2401052253975846</v>
       </c>
       <c r="G11" t="n">
-        <v>0.1210221663381487</v>
+        <v>-0.1610131834228575</v>
       </c>
       <c r="H11" t="n">
-        <v>0.1358408956288321</v>
+        <v>-0.1571411202951169</v>
       </c>
       <c r="I11" t="n">
-        <v>48.93556627873971</v>
+        <v>63.3225806451613</v>
       </c>
       <c r="J11" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K11" t="n">
-        <v>49.98</v>
+        <v>50.88</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M11" t="n">
-        <v>49.98</v>
+        <v>50.88</v>
       </c>
       <c r="N11" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O11" t="n">
-        <v>74.46808510638297</v>
+        <v>23.40425531914894</v>
       </c>
       <c r="P11" t="n">
-        <v>58.8856170212766</v>
+        <v>57.03285106382979</v>
       </c>
       <c r="Q11" t="b">
         <v>0</v>
       </c>
       <c r="R11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S11" t="b">
         <v>0</v>
@@ -4586,63 +4586,63 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>RANEENGINE</t>
+          <t>LUMAXIND</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Engine/Parts</t>
+          <t>Lighting</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>317.75</v>
+        <v>4785</v>
       </c>
       <c r="D12" t="n">
-        <v>0.1790352504638219</v>
+        <v>-0.1530223913620674</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.156154561147258</v>
+        <v>-0.0829819854350325</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.2401052253975846</v>
+        <v>0.1431233426503262</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.1545017308592433</v>
+        <v>0.2222153846250533</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.1396830015685599</v>
+        <v>0.2260874477527938</v>
       </c>
       <c r="I12" t="n">
-        <v>63.3225806451613</v>
+        <v>49.33389426447903</v>
       </c>
       <c r="J12" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="K12" t="n">
-        <v>50.88</v>
+        <v>57.69</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M12" t="n">
-        <v>50.88</v>
+        <v>57.69</v>
       </c>
       <c r="N12" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="O12" t="n">
-        <v>23.40425531914894</v>
+        <v>89.36170212765957</v>
       </c>
       <c r="P12" t="n">
-        <v>57.03285106382979</v>
+        <v>56.94834042553191</v>
       </c>
       <c r="Q12" t="b">
         <v>0</v>
       </c>
       <c r="R12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S12" t="b">
         <v>0</v>
@@ -4651,57 +4651,57 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MINDACORP</t>
+          <t>GNA</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Axles</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>514.15</v>
+        <v>371.3</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.0492788461538461</v>
+        <v>-0.1005329457364341</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.1210359859817079</v>
+        <v>0.2453463021968809</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.0021348859776807</v>
+        <v>0.1856937569854704</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0834686085606605</v>
+        <v>0.2647857989601975</v>
       </c>
       <c r="H13" t="n">
-        <v>0.0982873378513439</v>
+        <v>0.268657862087938</v>
       </c>
       <c r="I13" t="n">
-        <v>61.53039832285116</v>
+        <v>44.83695652173915</v>
       </c>
       <c r="J13" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="K13" t="n">
-        <v>49.42</v>
+        <v>54.47</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M13" t="n">
-        <v>49.42</v>
+        <v>54.47</v>
       </c>
       <c r="N13" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="O13" t="n">
-        <v>65.95744680851064</v>
+        <v>91.48936170212764</v>
       </c>
       <c r="P13" t="n">
-        <v>56.95948936170213</v>
+        <v>56.08587234042552</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
@@ -4716,63 +4716,63 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>LUMAXIND</t>
+          <t>SUPRAJIT</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Lighting</t>
+          <t>Cables</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>4805.4</v>
+        <v>411.55</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.1923697478991597</v>
+        <v>-0.0267234243821686</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.1256550218340612</v>
+        <v>-0.1120819848975188</v>
       </c>
       <c r="F14" t="n">
-        <v>0.1459436256975246</v>
+        <v>-0.1023991275899672</v>
       </c>
       <c r="G14" t="n">
-        <v>0.2315471202358658</v>
+        <v>-0.0233070856152401</v>
       </c>
       <c r="H14" t="n">
-        <v>0.2463658495265492</v>
+        <v>-0.0194350224874996</v>
       </c>
       <c r="I14" t="n">
-        <v>46.77362169828044</v>
+        <v>54.21940928270043</v>
       </c>
       <c r="J14" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K14" t="n">
-        <v>57.69</v>
+        <v>51.48</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M14" t="n">
-        <v>57.69</v>
+        <v>51.48</v>
       </c>
       <c r="N14" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O14" t="n">
-        <v>89.36170212765957</v>
+        <v>53.19148936170212</v>
       </c>
       <c r="P14" t="n">
-        <v>56.94834042553191</v>
+        <v>55.23029787234042</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
       </c>
       <c r="R14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S14" t="b">
         <v>0</v>
@@ -4781,57 +4781,57 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SUPRAJIT</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Cables</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>421.95</v>
+        <v>496.55</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.0212247738343772</v>
+        <v>-0.009672915835660101</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.0511580841016415</v>
+        <v>0.0357738840216939</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.0810192747468147</v>
+        <v>0.1033218531274302</v>
       </c>
       <c r="G15" t="n">
-        <v>0.0045842197915265</v>
+        <v>0.1824138951021573</v>
       </c>
       <c r="H15" t="n">
-        <v>0.0194029490822099</v>
+        <v>0.1862859582298979</v>
       </c>
       <c r="I15" t="n">
-        <v>56.05234460196291</v>
+        <v>53.73399715504979</v>
       </c>
       <c r="J15" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="K15" t="n">
-        <v>51.48</v>
+        <v>49.66</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M15" t="n">
-        <v>51.48</v>
+        <v>49.66</v>
       </c>
       <c r="N15" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="O15" t="n">
-        <v>55.31914893617022</v>
+        <v>87.2340425531915</v>
       </c>
       <c r="P15" t="n">
-        <v>55.65582978723404</v>
+        <v>53.31080851063831</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
@@ -4846,57 +4846,57 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>CRAFTSMAN</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Forgings</t>
+          <t>Castings</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1668.4</v>
+        <v>6789</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.1122226360879049</v>
+        <v>-0.0852253587549687</v>
       </c>
       <c r="E16" t="n">
-        <v>0.1694939015841863</v>
+        <v>-0.1171077443266792</v>
       </c>
       <c r="F16" t="n">
-        <v>0.4118642633494118</v>
+        <v>0.019752159218926</v>
       </c>
       <c r="G16" t="n">
-        <v>0.4974677578877531</v>
+        <v>0.0988442011936531</v>
       </c>
       <c r="H16" t="n">
-        <v>0.5122864871784365</v>
+        <v>0.1027162643213936</v>
       </c>
       <c r="I16" t="n">
-        <v>39.8093841642229</v>
+        <v>53.60275689223057</v>
       </c>
       <c r="J16" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K16" t="n">
-        <v>54.83</v>
+        <v>54.65</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="M16" t="n">
-        <v>54.83</v>
+        <v>54.65</v>
       </c>
       <c r="N16" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O16" t="n">
-        <v>97.87234042553192</v>
+        <v>74.46808510638297</v>
       </c>
       <c r="P16" t="n">
-        <v>53.50646808510639</v>
+        <v>52.7536170212766</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
chore: auto-refresh NSE data and pipeline outputs (2026-04-03)
</commit_message>
<xml_diff>
--- a/working-sector/output/auto_components_comprehensive_report.xlsx
+++ b/working-sector/output/auto_components_comprehensive_report.xlsx
@@ -435,7 +435,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
     </row>
@@ -791,10 +791,10 @@
         <v>0.3689474122843568</v>
       </c>
       <c r="G2" t="n">
-        <v>0.4480394542590838</v>
+        <v>0.4829467208333394</v>
       </c>
       <c r="H2" t="n">
-        <v>0.4519115173868244</v>
+        <v>0.4537557379504254</v>
       </c>
       <c r="I2" t="n">
         <v>46.51959734418505</v>
@@ -856,10 +856,10 @@
         <v>-0.1924712553157976</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.1133792133410706</v>
+        <v>-0.078471946766815</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.10950715021333</v>
+        <v>-0.107662929649729</v>
       </c>
       <c r="I3" t="n">
         <v>52.01320132013202</v>
@@ -921,10 +921,10 @@
         <v>-0.2163150835263991</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.1372230415516721</v>
+        <v>-0.1023157749774165</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.1333509784239315</v>
+        <v>-0.1315067578603305</v>
       </c>
       <c r="I4" t="n">
         <v>60.27397260273973</v>
@@ -986,10 +986,10 @@
         <v>-0.2912966252220248</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.2122045832472977</v>
+        <v>-0.1772973166730421</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.2083325201195571</v>
+        <v>-0.2064882995559561</v>
       </c>
       <c r="I5" t="n">
         <v>51.59927579963788</v>
@@ -1051,10 +1051,10 @@
         <v>0.0617296222664016</v>
       </c>
       <c r="G6" t="n">
-        <v>0.1408216642411287</v>
+        <v>0.1757289308153843</v>
       </c>
       <c r="H6" t="n">
-        <v>0.1446937273688693</v>
+        <v>0.1465379479324703</v>
       </c>
       <c r="I6" t="n">
         <v>39.71839249046643</v>
@@ -1116,10 +1116,10 @@
         <v>-0.2064232944885783</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.1273312525138512</v>
+        <v>-0.0924239859395956</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.1234591893861106</v>
+        <v>-0.1216149688225096</v>
       </c>
       <c r="I7" t="n">
         <v>57.64112620815244</v>
@@ -1181,10 +1181,10 @@
         <v>0.1033218531274302</v>
       </c>
       <c r="G8" t="n">
-        <v>0.1824138951021573</v>
+        <v>0.2173211616764129</v>
       </c>
       <c r="H8" t="n">
-        <v>0.1862859582298979</v>
+        <v>0.1881301787934989</v>
       </c>
       <c r="I8" t="n">
         <v>53.73399715504979</v>
@@ -1246,10 +1246,10 @@
         <v>-0.1461787092065478</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.0670866672318207</v>
+        <v>-0.0321794006575651</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.0632146041040802</v>
+        <v>-0.0613703835404791</v>
       </c>
       <c r="I9" t="n">
         <v>55.5021046301864</v>
@@ -1311,10 +1311,10 @@
         <v>-0.1298750473305566</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.0507830053558295</v>
+        <v>-0.015875738781574</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.046910942228089</v>
+        <v>-0.0450667216644879</v>
       </c>
       <c r="I10" t="n">
         <v>31.30206049978081</v>
@@ -1376,10 +1376,10 @@
         <v>-0.0042030657656173</v>
       </c>
       <c r="G11" t="n">
-        <v>0.0748889762091097</v>
+        <v>0.1097962427833653</v>
       </c>
       <c r="H11" t="n">
-        <v>0.0787610393368503</v>
+        <v>0.0806052599004513</v>
       </c>
       <c r="I11" t="n">
         <v>27.6054590570719</v>
@@ -1441,10 +1441,10 @@
         <v>-0.1646732370108122</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.08558119503608511</v>
+        <v>-0.0506739284618296</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.0817091319083446</v>
+        <v>-0.07986491134474361</v>
       </c>
       <c r="I12" t="n">
         <v>64.88250652741513</v>
@@ -1506,10 +1506,10 @@
         <v>-0.025778038755138</v>
       </c>
       <c r="G13" t="n">
-        <v>0.053314003219589</v>
+        <v>0.0882212697938445</v>
       </c>
       <c r="H13" t="n">
-        <v>0.0571860663473295</v>
+        <v>0.0590302869109305</v>
       </c>
       <c r="I13" t="n">
         <v>39.78727239949522</v>
@@ -1571,10 +1571,10 @@
         <v>-0.1601096420509513</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.0810176000762242</v>
+        <v>-0.0461103335019686</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.0771455369484837</v>
+        <v>-0.07530131638488261</v>
       </c>
       <c r="I14" t="n">
         <v>43.87410223912125</v>
@@ -1636,10 +1636,10 @@
         <v>0.028538812785388</v>
       </c>
       <c r="G15" t="n">
-        <v>0.1076308547601151</v>
+        <v>0.1425381213343707</v>
       </c>
       <c r="H15" t="n">
-        <v>0.1115029178878557</v>
+        <v>0.1133471384514567</v>
       </c>
       <c r="I15" t="n">
         <v>39.75636766334441</v>
@@ -1701,10 +1701,10 @@
         <v>-0.0738744075829384</v>
       </c>
       <c r="G16" t="n">
-        <v>0.0052176343917886</v>
+        <v>0.0401249009660442</v>
       </c>
       <c r="H16" t="n">
-        <v>0.0090896975195292</v>
+        <v>0.0109339180831302</v>
       </c>
       <c r="I16" t="n">
         <v>48.29804341999465</v>
@@ -1766,10 +1766,10 @@
         <v>0.019752159218926</v>
       </c>
       <c r="G17" t="n">
-        <v>0.0988442011936531</v>
+        <v>0.1337514677679087</v>
       </c>
       <c r="H17" t="n">
-        <v>0.1027162643213936</v>
+        <v>0.1045604848849947</v>
       </c>
       <c r="I17" t="n">
         <v>53.60275689223057</v>
@@ -1831,10 +1831,10 @@
         <v>-0.0464154066049801</v>
       </c>
       <c r="G18" t="n">
-        <v>0.0326766353697469</v>
+        <v>0.0675839019440025</v>
       </c>
       <c r="H18" t="n">
-        <v>0.0365486984974875</v>
+        <v>0.0383929190610885</v>
       </c>
       <c r="I18" t="n">
         <v>42.69977595220314</v>
@@ -1896,10 +1896,10 @@
         <v>-0.2595357095883203</v>
       </c>
       <c r="G19" t="n">
-        <v>-0.1804436676135932</v>
+        <v>-0.1455364010393376</v>
       </c>
       <c r="H19" t="n">
-        <v>-0.1765716044858526</v>
+        <v>-0.1747273839222516</v>
       </c>
       <c r="I19" t="n">
         <v>36.29951166576236</v>
@@ -1961,10 +1961,10 @@
         <v>-0.06802178199230111</v>
       </c>
       <c r="G20" t="n">
-        <v>0.0110702599824259</v>
+        <v>0.0459775265566815</v>
       </c>
       <c r="H20" t="n">
-        <v>0.0149423231101665</v>
+        <v>0.0167865436737675</v>
       </c>
       <c r="I20" t="n">
         <v>45.41721660067459</v>
@@ -2026,10 +2026,10 @@
         <v>-0.3058041016707578</v>
       </c>
       <c r="G21" t="n">
-        <v>-0.2267120596960307</v>
+        <v>-0.1918047931217751</v>
       </c>
       <c r="H21" t="n">
-        <v>-0.2228399965682901</v>
+        <v>-0.2209957760046891</v>
       </c>
       <c r="I21" t="n">
         <v>55.66567558638918</v>
@@ -2091,10 +2091,10 @@
         <v>0.1856937569854704</v>
       </c>
       <c r="G22" t="n">
-        <v>0.2647857989601975</v>
+        <v>0.2996930655344531</v>
       </c>
       <c r="H22" t="n">
-        <v>0.268657862087938</v>
+        <v>0.2705020826515391</v>
       </c>
       <c r="I22" t="n">
         <v>44.83695652173915</v>
@@ -2156,10 +2156,10 @@
         <v>-0.1923728813559322</v>
       </c>
       <c r="G23" t="n">
-        <v>-0.1132808393812051</v>
+        <v>-0.0783735728069495</v>
       </c>
       <c r="H23" t="n">
-        <v>-0.1094087762534645</v>
+        <v>-0.1075645556898635</v>
       </c>
       <c r="I23" t="n">
         <v>39.49631449631451</v>
@@ -2221,10 +2221,10 @@
         <v>0.0725575376652187</v>
       </c>
       <c r="G24" t="n">
-        <v>0.1516495796399458</v>
+        <v>0.1865568462142014</v>
       </c>
       <c r="H24" t="n">
-        <v>0.1555216427676864</v>
+        <v>0.1573658633312874</v>
       </c>
       <c r="I24" t="n">
         <v>48.56386999244142</v>
@@ -2286,10 +2286,10 @@
         <v>-0.1103191573612101</v>
       </c>
       <c r="G25" t="n">
-        <v>-0.031227115386483</v>
+        <v>0.0036801511877725</v>
       </c>
       <c r="H25" t="n">
-        <v>-0.0273550522587424</v>
+        <v>-0.0255108316951414</v>
       </c>
       <c r="I25" t="n">
         <v>60.43020736614052</v>
@@ -2351,10 +2351,10 @@
         <v>-0.2498672488052392</v>
       </c>
       <c r="G26" t="n">
-        <v>-0.1707752068305121</v>
+        <v>-0.1358679402562566</v>
       </c>
       <c r="H26" t="n">
-        <v>-0.1669031437027716</v>
+        <v>-0.1650589231391706</v>
       </c>
       <c r="I26" t="n">
         <v>45.95569294178259</v>
@@ -2416,10 +2416,10 @@
         <v>0.1431233426503262</v>
       </c>
       <c r="G27" t="n">
-        <v>0.2222153846250533</v>
+        <v>0.2571226511993089</v>
       </c>
       <c r="H27" t="n">
-        <v>0.2260874477527938</v>
+        <v>0.2279316683163949</v>
       </c>
       <c r="I27" t="n">
         <v>49.33389426447903</v>
@@ -2481,10 +2481,10 @@
         <v>0.4464061659795664</v>
       </c>
       <c r="G28" t="n">
-        <v>0.5254982079542935</v>
+        <v>0.5604054745285491</v>
       </c>
       <c r="H28" t="n">
-        <v>0.529370271082034</v>
+        <v>0.5312144916456351</v>
       </c>
       <c r="I28" t="n">
         <v>62.49826316520774</v>
@@ -2546,10 +2546,10 @@
         <v>-0.0166699352814276</v>
       </c>
       <c r="G29" t="n">
-        <v>0.0624221066932993</v>
+        <v>0.09732937326755491</v>
       </c>
       <c r="H29" t="n">
-        <v>0.0662941698210399</v>
+        <v>0.0681383903846409</v>
       </c>
       <c r="I29" t="n">
         <v>56.60559305689488</v>
@@ -2611,10 +2611,10 @@
         <v>-0.1831515607371192</v>
       </c>
       <c r="G30" t="n">
-        <v>-0.1040595187623921</v>
+        <v>-0.0691522521881365</v>
       </c>
       <c r="H30" t="n">
-        <v>-0.1001874556346515</v>
+        <v>-0.0983432350710505</v>
       </c>
       <c r="I30" t="n">
         <v>30.56241426611795</v>
@@ -2676,10 +2676,10 @@
         <v>-0.2420772848088325</v>
       </c>
       <c r="G31" t="n">
-        <v>-0.1629852428341054</v>
+        <v>-0.1280779762598498</v>
       </c>
       <c r="H31" t="n">
-        <v>-0.1591131797063648</v>
+        <v>-0.1572689591427638</v>
       </c>
       <c r="I31" t="n">
         <v>38.91951488423375</v>
@@ -2741,10 +2741,10 @@
         <v>-0.4136214101538188</v>
       </c>
       <c r="G32" t="n">
-        <v>-0.3345293681790917</v>
+        <v>-0.2996221016048361</v>
       </c>
       <c r="H32" t="n">
-        <v>-0.3306573050513511</v>
+        <v>-0.3288130844877501</v>
       </c>
       <c r="I32" t="n">
         <v>50.82802547770701</v>
@@ -2806,10 +2806,10 @@
         <v>0.0150383141762453</v>
       </c>
       <c r="G33" t="n">
-        <v>0.0941303561509724</v>
+        <v>0.129037622725228</v>
       </c>
       <c r="H33" t="n">
-        <v>0.098002419278713</v>
+        <v>0.099846639842314</v>
       </c>
       <c r="I33" t="n">
         <v>54.07779171894605</v>
@@ -2871,10 +2871,10 @@
         <v>-0.2401052253975846</v>
       </c>
       <c r="G34" t="n">
-        <v>-0.1610131834228575</v>
+        <v>-0.1261059168486019</v>
       </c>
       <c r="H34" t="n">
-        <v>-0.1571411202951169</v>
+        <v>-0.1552968997315159</v>
       </c>
       <c r="I34" t="n">
         <v>63.3225806451613</v>
@@ -2936,10 +2936,10 @@
         <v>0.06890112050324371</v>
       </c>
       <c r="G35" t="n">
-        <v>0.1479931624779707</v>
+        <v>0.1829004290522263</v>
       </c>
       <c r="H35" t="n">
-        <v>0.1518652256057113</v>
+        <v>0.1537094461693123</v>
       </c>
       <c r="I35" t="n">
         <v>53.28719723183392</v>
@@ -3001,10 +3001,10 @@
         <v>0.0002168021680217</v>
       </c>
       <c r="G36" t="n">
-        <v>0.0793088441427488</v>
+        <v>0.1142161107170044</v>
       </c>
       <c r="H36" t="n">
-        <v>0.08318090727048939</v>
+        <v>0.0850251278340904</v>
       </c>
       <c r="I36" t="n">
         <v>41.17187500000001</v>
@@ -3066,10 +3066,10 @@
         <v>0.5095379398050019</v>
       </c>
       <c r="G37" t="n">
-        <v>0.588629981779729</v>
+        <v>0.6235372483539846</v>
       </c>
       <c r="H37" t="n">
-        <v>0.5925020449074696</v>
+        <v>0.5943462654710706</v>
       </c>
       <c r="I37" t="n">
         <v>61.35631043887923</v>
@@ -3131,10 +3131,10 @@
         <v>-0.3016791575751825</v>
       </c>
       <c r="G38" t="n">
-        <v>-0.2225871156004554</v>
+        <v>-0.1876798490261998</v>
       </c>
       <c r="H38" t="n">
-        <v>-0.2187150524727148</v>
+        <v>-0.2168708319091138</v>
       </c>
       <c r="I38" t="n">
         <v>43.53045798132504</v>
@@ -3196,10 +3196,10 @@
         <v>0.1000338078960221</v>
       </c>
       <c r="G39" t="n">
-        <v>0.1791258498707492</v>
+        <v>0.2140331164450047</v>
       </c>
       <c r="H39" t="n">
-        <v>0.1829979129984897</v>
+        <v>0.1848421335620907</v>
       </c>
       <c r="I39" t="n">
         <v>53.54029967681912</v>
@@ -3261,10 +3261,10 @@
         <v>-0.2244170320888487</v>
       </c>
       <c r="G40" t="n">
-        <v>-0.1453249901141217</v>
+        <v>-0.1104177235398661</v>
       </c>
       <c r="H40" t="n">
-        <v>-0.1414529269863811</v>
+        <v>-0.1396087064227801</v>
       </c>
       <c r="I40" t="n">
         <v>54.87893286936349</v>
@@ -3326,10 +3326,10 @@
         <v>-0.2616914443241115</v>
       </c>
       <c r="G41" t="n">
-        <v>-0.1825994023493844</v>
+        <v>-0.1476921357751288</v>
       </c>
       <c r="H41" t="n">
-        <v>-0.1787273392216438</v>
+        <v>-0.1768831186580428</v>
       </c>
       <c r="I41" t="n">
         <v>21.74931667317455</v>
@@ -3391,10 +3391,10 @@
         <v>-0.354434489027399</v>
       </c>
       <c r="G42" t="n">
-        <v>-0.2753424470526719</v>
+        <v>-0.2404351804784164</v>
       </c>
       <c r="H42" t="n">
-        <v>-0.2714703839249314</v>
+        <v>-0.2696261633613304</v>
       </c>
       <c r="I42" t="n">
         <v>36.97642163661581</v>
@@ -3456,10 +3456,10 @@
         <v>-0.1023991275899672</v>
       </c>
       <c r="G43" t="n">
-        <v>-0.0233070856152401</v>
+        <v>0.0116001809590153</v>
       </c>
       <c r="H43" t="n">
-        <v>-0.0194350224874996</v>
+        <v>-0.0175908019238986</v>
       </c>
       <c r="I43" t="n">
         <v>54.21940928270043</v>
@@ -3521,10 +3521,10 @@
         <v>-0.1753259779338014</v>
       </c>
       <c r="G44" t="n">
-        <v>-0.0962339359590743</v>
+        <v>-0.0613266693848187</v>
       </c>
       <c r="H44" t="n">
-        <v>-0.09236187283133369</v>
+        <v>-0.0905176522677327</v>
       </c>
       <c r="I44" t="n">
         <v>49.41771556287495</v>
@@ -3586,10 +3586,10 @@
         <v>-0.3683173888576252</v>
       </c>
       <c r="G45" t="n">
-        <v>-0.2892253468828981</v>
+        <v>-0.2543180803086425</v>
       </c>
       <c r="H45" t="n">
-        <v>-0.2853532837551575</v>
+        <v>-0.2835090631915565</v>
       </c>
       <c r="I45" t="n">
         <v>36.57370517928285</v>
@@ -3651,10 +3651,10 @@
         <v>-0.1958644457208501</v>
       </c>
       <c r="G46" t="n">
-        <v>-0.116772403746123</v>
+        <v>-0.0818651371718675</v>
       </c>
       <c r="H46" t="n">
-        <v>-0.1129003406183825</v>
+        <v>-0.1110561200547815</v>
       </c>
       <c r="I46" t="n">
         <v>52.84003684372122</v>
@@ -3716,10 +3716,10 @@
         <v>0.3150010122140494</v>
       </c>
       <c r="G47" t="n">
-        <v>0.3940930541887765</v>
+        <v>0.4290003207630321</v>
       </c>
       <c r="H47" t="n">
-        <v>0.397965117316517</v>
+        <v>0.3998093378801181</v>
       </c>
       <c r="I47" t="n">
         <v>59.59416613823716</v>
@@ -3781,10 +3781,10 @@
         <v>0.0185873605947954</v>
       </c>
       <c r="G48" t="n">
-        <v>0.0976794025695225</v>
+        <v>0.1325866691437781</v>
       </c>
       <c r="H48" t="n">
-        <v>0.1015514656972631</v>
+        <v>0.1033956862608641</v>
       </c>
       <c r="I48" t="n">
         <v>55.78125</v>
@@ -3957,10 +3957,10 @@
         <v>0.4464061659795664</v>
       </c>
       <c r="G2" t="n">
-        <v>0.5254982079542935</v>
+        <v>0.5604054745285491</v>
       </c>
       <c r="H2" t="n">
-        <v>0.529370271082034</v>
+        <v>0.5312144916456351</v>
       </c>
       <c r="I2" t="n">
         <v>62.49826316520774</v>
@@ -4022,10 +4022,10 @@
         <v>0.5095379398050019</v>
       </c>
       <c r="G3" t="n">
-        <v>0.588629981779729</v>
+        <v>0.6235372483539846</v>
       </c>
       <c r="H3" t="n">
-        <v>0.5925020449074696</v>
+        <v>0.5943462654710706</v>
       </c>
       <c r="I3" t="n">
         <v>61.35631043887923</v>
@@ -4087,10 +4087,10 @@
         <v>-0.1646732370108122</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.08558119503608511</v>
+        <v>-0.0506739284618296</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.0817091319083446</v>
+        <v>-0.07986491134474361</v>
       </c>
       <c r="I4" t="n">
         <v>64.88250652741513</v>
@@ -4152,10 +4152,10 @@
         <v>-0.1103191573612101</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.031227115386483</v>
+        <v>0.0036801511877725</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.0273550522587424</v>
+        <v>-0.0255108316951414</v>
       </c>
       <c r="I5" t="n">
         <v>60.43020736614052</v>
@@ -4217,10 +4217,10 @@
         <v>0.3150010122140494</v>
       </c>
       <c r="G6" t="n">
-        <v>0.3940930541887765</v>
+        <v>0.4290003207630321</v>
       </c>
       <c r="H6" t="n">
-        <v>0.397965117316517</v>
+        <v>0.3998093378801181</v>
       </c>
       <c r="I6" t="n">
         <v>59.59416613823716</v>
@@ -4282,10 +4282,10 @@
         <v>0.06890112050324371</v>
       </c>
       <c r="G7" t="n">
-        <v>0.1479931624779707</v>
+        <v>0.1829004290522263</v>
       </c>
       <c r="H7" t="n">
-        <v>0.1518652256057113</v>
+        <v>0.1537094461693123</v>
       </c>
       <c r="I7" t="n">
         <v>53.28719723183392</v>
@@ -4347,10 +4347,10 @@
         <v>0.0185873605947954</v>
       </c>
       <c r="G8" t="n">
-        <v>0.0976794025695225</v>
+        <v>0.1325866691437781</v>
       </c>
       <c r="H8" t="n">
-        <v>0.1015514656972631</v>
+        <v>0.1033956862608641</v>
       </c>
       <c r="I8" t="n">
         <v>55.78125</v>
@@ -4412,10 +4412,10 @@
         <v>-0.2064232944885783</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.1273312525138512</v>
+        <v>-0.0924239859395956</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.1234591893861106</v>
+        <v>-0.1216149688225096</v>
       </c>
       <c r="I9" t="n">
         <v>57.64112620815244</v>
@@ -4477,10 +4477,10 @@
         <v>0.3689474122843568</v>
       </c>
       <c r="G10" t="n">
-        <v>0.4480394542590838</v>
+        <v>0.4829467208333394</v>
       </c>
       <c r="H10" t="n">
-        <v>0.4519115173868244</v>
+        <v>0.4537557379504254</v>
       </c>
       <c r="I10" t="n">
         <v>46.51959734418505</v>
@@ -4542,10 +4542,10 @@
         <v>-0.2401052253975846</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.1610131834228575</v>
+        <v>-0.1261059168486019</v>
       </c>
       <c r="H11" t="n">
-        <v>-0.1571411202951169</v>
+        <v>-0.1552968997315159</v>
       </c>
       <c r="I11" t="n">
         <v>63.3225806451613</v>
@@ -4607,10 +4607,10 @@
         <v>0.1431233426503262</v>
       </c>
       <c r="G12" t="n">
-        <v>0.2222153846250533</v>
+        <v>0.2571226511993089</v>
       </c>
       <c r="H12" t="n">
-        <v>0.2260874477527938</v>
+        <v>0.2279316683163949</v>
       </c>
       <c r="I12" t="n">
         <v>49.33389426447903</v>
@@ -4672,10 +4672,10 @@
         <v>0.1856937569854704</v>
       </c>
       <c r="G13" t="n">
-        <v>0.2647857989601975</v>
+        <v>0.2996930655344531</v>
       </c>
       <c r="H13" t="n">
-        <v>0.268657862087938</v>
+        <v>0.2705020826515391</v>
       </c>
       <c r="I13" t="n">
         <v>44.83695652173915</v>
@@ -4737,10 +4737,10 @@
         <v>-0.1023991275899672</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.0233070856152401</v>
+        <v>0.0116001809590153</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.0194350224874996</v>
+        <v>-0.0175908019238986</v>
       </c>
       <c r="I14" t="n">
         <v>54.21940928270043</v>
@@ -4802,10 +4802,10 @@
         <v>0.1033218531274302</v>
       </c>
       <c r="G15" t="n">
-        <v>0.1824138951021573</v>
+        <v>0.2173211616764129</v>
       </c>
       <c r="H15" t="n">
-        <v>0.1862859582298979</v>
+        <v>0.1881301787934989</v>
       </c>
       <c r="I15" t="n">
         <v>53.73399715504979</v>
@@ -4867,10 +4867,10 @@
         <v>0.019752159218926</v>
       </c>
       <c r="G16" t="n">
-        <v>0.0988442011936531</v>
+        <v>0.1337514677679087</v>
       </c>
       <c r="H16" t="n">
-        <v>0.1027162643213936</v>
+        <v>0.1045604848849947</v>
       </c>
       <c r="I16" t="n">
         <v>53.60275689223057</v>

</xml_diff>

<commit_message>
chore: auto-refresh NSE data and pipeline outputs (2026-04-06)
</commit_message>
<xml_diff>
--- a/working-sector/output/auto_components_comprehensive_report.xlsx
+++ b/working-sector/output/auto_components_comprehensive_report.xlsx
@@ -435,7 +435,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-06</t>
         </is>
       </c>
     </row>
@@ -447,7 +447,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
     </row>
@@ -782,22 +782,22 @@
         <v>1642.6</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.1081550656966011</v>
+        <v>-0.1347450484618627</v>
       </c>
       <c r="E2" t="n">
-        <v>0.1171109902067464</v>
+        <v>0.1216880633706636</v>
       </c>
       <c r="F2" t="n">
-        <v>0.3689474122843568</v>
+        <v>0.3553923591055365</v>
       </c>
       <c r="G2" t="n">
-        <v>0.4829467208333394</v>
+        <v>0.459580715584889</v>
       </c>
       <c r="H2" t="n">
-        <v>0.4537557379504254</v>
+        <v>0.4318681250397126</v>
       </c>
       <c r="I2" t="n">
-        <v>46.51959734418505</v>
+        <v>43.88764044943819</v>
       </c>
       <c r="J2" t="n">
         <v>40</v>
@@ -807,7 +807,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M2" t="n">
@@ -847,22 +847,22 @@
         <v>1025.4</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.088128056914184</v>
+        <v>-0.0830725207904854</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.2025198320111991</v>
+        <v>-0.2030776404756352</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.1924712553157976</v>
+        <v>-0.200280767430978</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.078471946766815</v>
+        <v>-0.0960924109516255</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.107662929649729</v>
+        <v>-0.1238050014968019</v>
       </c>
       <c r="I3" t="n">
-        <v>52.01320132013202</v>
+        <v>51.15888478333896</v>
       </c>
       <c r="J3" t="n">
         <v>40</v>
@@ -872,7 +872,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M3" t="n">
@@ -882,10 +882,10 @@
         <v>40</v>
       </c>
       <c r="O3" t="n">
-        <v>34.04255319148936</v>
+        <v>31.91489361702128</v>
       </c>
       <c r="P3" t="n">
-        <v>42.55251063829788</v>
+        <v>42.12697872340426</v>
       </c>
       <c r="Q3" t="b">
         <v>0</v>
@@ -912,22 +912,22 @@
         <v>32135</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.0375861036238395</v>
+        <v>-0.0329521516701775</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.1083518312985571</v>
+        <v>-0.1108190370780298</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.2163150835263991</v>
+        <v>-0.2095683187799778</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.1023157749774165</v>
+        <v>-0.1053799623006254</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.1315067578603305</v>
+        <v>-0.1330925528458018</v>
       </c>
       <c r="I4" t="n">
-        <v>60.27397260273973</v>
+        <v>59.54935622317596</v>
       </c>
       <c r="J4" t="n">
         <v>60</v>
@@ -937,7 +937,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M4" t="n">
@@ -977,22 +977,22 @@
         <v>299.25</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.0468227424749163</v>
+        <v>-0.06381980290943209</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.1737990060739922</v>
+        <v>-0.17618719889883</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.2912966252220248</v>
+        <v>-0.2920511000709723</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.1772973166730421</v>
+        <v>-0.1878627435916199</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.2064882995559561</v>
+        <v>-0.2155753341367963</v>
       </c>
       <c r="I5" t="n">
-        <v>51.59927579963788</v>
+        <v>52.51842751842753</v>
       </c>
       <c r="J5" t="n">
         <v>40</v>
@@ -1002,7 +1002,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M5" t="n">
@@ -1042,45 +1042,45 @@
         <v>106.81</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.1307779947916666</v>
+        <v>-0.1545828716162736</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.1094714023678505</v>
+        <v>-0.1282239634345412</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0617296222664016</v>
+        <v>0.0609913579020562</v>
       </c>
       <c r="G6" t="n">
-        <v>0.1757289308153843</v>
+        <v>0.1651797143814086</v>
       </c>
       <c r="H6" t="n">
-        <v>0.1465379479324703</v>
+        <v>0.1374671238362322</v>
       </c>
       <c r="I6" t="n">
-        <v>39.71839249046643</v>
+        <v>40.30961595713011</v>
       </c>
       <c r="J6" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K6" t="n">
         <v>51.57</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M6" t="n">
         <v>51.57</v>
       </c>
       <c r="N6" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O6" t="n">
         <v>78.72340425531915</v>
       </c>
       <c r="P6" t="n">
-        <v>48.37268085106383</v>
+        <v>52.37268085106383</v>
       </c>
       <c r="Q6" t="b">
         <v>0</v>
@@ -1107,22 +1107,22 @@
         <v>2567.3</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.0735448017032945</v>
+        <v>-0.0771415219813795</v>
       </c>
       <c r="E7" t="n">
-        <v>-0.0179029111357635</v>
+        <v>-0.0211979107095199</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.2064232944885783</v>
+        <v>-0.2005418366393672</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.0924239859395956</v>
+        <v>-0.0963534801600147</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.1216149688225096</v>
+        <v>-0.1240660707051911</v>
       </c>
       <c r="I7" t="n">
-        <v>57.64112620815244</v>
+        <v>60.69321533923305</v>
       </c>
       <c r="J7" t="n">
         <v>80</v>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M7" t="n">
@@ -1172,22 +1172,22 @@
         <v>496.55</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.009672915835660101</v>
+        <v>-0.0281827967511497</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0357738840216939</v>
+        <v>0.0469112376133249</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1033218531274302</v>
+        <v>0.1286509830662576</v>
       </c>
       <c r="G8" t="n">
-        <v>0.2173211616764129</v>
+        <v>0.2328393395456101</v>
       </c>
       <c r="H8" t="n">
-        <v>0.1881301787934989</v>
+        <v>0.2051267490004337</v>
       </c>
       <c r="I8" t="n">
-        <v>53.73399715504979</v>
+        <v>52.67369952710077</v>
       </c>
       <c r="J8" t="n">
         <v>40</v>
@@ -1197,7 +1197,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M8" t="n">
@@ -1237,22 +1237,22 @@
         <v>409.45</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.0506607929515419</v>
+        <v>-0.0785416901091482</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.1811</v>
+        <v>-0.1714892755969242</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.1461787092065478</v>
+        <v>-0.1430514859773964</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.0321794006575651</v>
+        <v>-0.038863129498044</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.0613703835404791</v>
+        <v>-0.0665757200432204</v>
       </c>
       <c r="I9" t="n">
-        <v>55.5021046301864</v>
+        <v>47.62915782024061</v>
       </c>
       <c r="J9" t="n">
         <v>40</v>
@@ -1262,7 +1262,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M9" t="n">
@@ -1302,22 +1302,22 @@
         <v>126390</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.0641243983709737</v>
+        <v>-0.0985985807509896</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.1731379411860913</v>
+        <v>-0.165935262480615</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.1298750473305566</v>
+        <v>-0.1371518296013107</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.015875738781574</v>
+        <v>-0.0329634731219583</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.0450667216644879</v>
+        <v>-0.0606760636671347</v>
       </c>
       <c r="I10" t="n">
-        <v>31.30206049978081</v>
+        <v>35.28539659006671</v>
       </c>
       <c r="J10" t="n">
         <v>30</v>
@@ -1327,7 +1327,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M10" t="n">
@@ -1376,10 +1376,10 @@
         <v>-0.0042030657656173</v>
       </c>
       <c r="G11" t="n">
-        <v>0.1097962427833653</v>
+        <v>0.09998529071373501</v>
       </c>
       <c r="H11" t="n">
-        <v>0.0806052599004513</v>
+        <v>0.07227270016855861</v>
       </c>
       <c r="I11" t="n">
         <v>27.6054590570719</v>
@@ -1392,7 +1392,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M11" t="n">
@@ -1432,22 +1432,22 @@
         <v>436.5</v>
       </c>
       <c r="D12" t="n">
-        <v>0.1303897449177782</v>
+        <v>0.1213872832369942</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.08806016922594791</v>
+        <v>-0.08739284967593559</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.1646732370108122</v>
+        <v>-0.1526739784528777</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.0506739284618296</v>
+        <v>-0.0484856219735253</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.07986491134474361</v>
+        <v>-0.07619821251870169</v>
       </c>
       <c r="I12" t="n">
-        <v>64.88250652741513</v>
+        <v>63.01558203483042</v>
       </c>
       <c r="J12" t="n">
         <v>80</v>
@@ -1457,7 +1457,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M12" t="n">
@@ -1467,10 +1467,10 @@
         <v>80</v>
       </c>
       <c r="O12" t="n">
-        <v>42.5531914893617</v>
+        <v>44.68085106382978</v>
       </c>
       <c r="P12" t="n">
-        <v>69.02263829787233</v>
+        <v>69.44817021276596</v>
       </c>
       <c r="Q12" t="b">
         <v>1</v>
@@ -1497,45 +1497,45 @@
         <v>1659.1</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.1711545186591397</v>
+        <v>-0.171775159744409</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.11867197875166</v>
+        <v>-0.118250425170068</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.025778038755138</v>
+        <v>-0.0412597515169026</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0882212697938445</v>
+        <v>0.0629286049624497</v>
       </c>
       <c r="H13" t="n">
-        <v>0.0590302869109305</v>
+        <v>0.0352160144172734</v>
       </c>
       <c r="I13" t="n">
-        <v>39.78727239949522</v>
+        <v>44.29058799919726</v>
       </c>
       <c r="J13" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K13" t="n">
         <v>58.77</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M13" t="n">
         <v>58.77</v>
       </c>
       <c r="N13" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O13" t="n">
-        <v>61.70212765957447</v>
+        <v>59.57446808510638</v>
       </c>
       <c r="P13" t="n">
-        <v>47.8484255319149</v>
+        <v>51.42289361702128</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
@@ -1562,22 +1562,22 @@
         <v>520.9</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.09044875152785049</v>
+        <v>-0.1068244170096023</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.2438121506859258</v>
+        <v>-0.236888368004688</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.1601096420509513</v>
+        <v>-0.158549390194653</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.0461103335019686</v>
+        <v>-0.0543610337153006</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.07530131638488261</v>
+        <v>-0.082073624260477</v>
       </c>
       <c r="I14" t="n">
-        <v>43.87410223912125</v>
+        <v>40.75808249721292</v>
       </c>
       <c r="J14" t="n">
         <v>40</v>
@@ -1587,7 +1587,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M14" t="n">
@@ -1597,10 +1597,10 @@
         <v>40</v>
       </c>
       <c r="O14" t="n">
-        <v>44.68085106382978</v>
+        <v>42.5531914893617</v>
       </c>
       <c r="P14" t="n">
-        <v>46.79217021276596</v>
+        <v>46.36663829787234</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
@@ -1627,45 +1627,45 @@
         <v>90.09999999999999</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.0949271722752386</v>
+        <v>-0.1202890060535052</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.2509145327569005</v>
+        <v>-0.3856538933587891</v>
       </c>
       <c r="F15" t="n">
-        <v>0.028538812785388</v>
+        <v>0.0258453831264944</v>
       </c>
       <c r="G15" t="n">
-        <v>0.1425381213343707</v>
+        <v>0.1300337396058468</v>
       </c>
       <c r="H15" t="n">
-        <v>0.1133471384514567</v>
+        <v>0.1023211490606704</v>
       </c>
       <c r="I15" t="n">
-        <v>39.75636766334441</v>
+        <v>42.86567164179105</v>
       </c>
       <c r="J15" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K15" t="n">
         <v>51.91</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M15" t="n">
         <v>51.91</v>
       </c>
       <c r="N15" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O15" t="n">
-        <v>76.59574468085107</v>
+        <v>74.46808510638297</v>
       </c>
       <c r="P15" t="n">
-        <v>48.08314893617021</v>
+        <v>51.65761702127659</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
@@ -1692,22 +1692,22 @@
         <v>156.33</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.1047929908950351</v>
+        <v>-0.1288866599799397</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.0920020909566124</v>
+        <v>-0.09594031922276181</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.0738744075829384</v>
+        <v>-0.0666308436324556</v>
       </c>
       <c r="G16" t="n">
-        <v>0.0401249009660442</v>
+        <v>0.0375575128468967</v>
       </c>
       <c r="H16" t="n">
-        <v>0.0109339180831302</v>
+        <v>0.009844922301720399</v>
       </c>
       <c r="I16" t="n">
-        <v>48.29804341999465</v>
+        <v>47.22298221614229</v>
       </c>
       <c r="J16" t="n">
         <v>40</v>
@@ -1717,7 +1717,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M16" t="n">
@@ -1727,10 +1727,10 @@
         <v>40</v>
       </c>
       <c r="O16" t="n">
-        <v>55.31914893617022</v>
+        <v>57.44680851063831</v>
       </c>
       <c r="P16" t="n">
-        <v>48.10782978723404</v>
+        <v>48.53336170212766</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>
@@ -1757,22 +1757,22 @@
         <v>6789</v>
       </c>
       <c r="D17" t="n">
-        <v>-0.0852253587549687</v>
+        <v>-0.1060635986569227</v>
       </c>
       <c r="E17" t="n">
-        <v>-0.1171077443266792</v>
+        <v>-0.1208805438653285</v>
       </c>
       <c r="F17" t="n">
-        <v>0.019752159218926</v>
+        <v>0.0016967908520841</v>
       </c>
       <c r="G17" t="n">
-        <v>0.1337514677679087</v>
+        <v>0.1058851473314366</v>
       </c>
       <c r="H17" t="n">
-        <v>0.1045604848849947</v>
+        <v>0.0781725567862602</v>
       </c>
       <c r="I17" t="n">
-        <v>53.60275689223057</v>
+        <v>49.88155668358714</v>
       </c>
       <c r="J17" t="n">
         <v>40</v>
@@ -1782,7 +1782,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M17" t="n">
@@ -1792,10 +1792,10 @@
         <v>40</v>
       </c>
       <c r="O17" t="n">
-        <v>74.46808510638297</v>
+        <v>70.21276595744681</v>
       </c>
       <c r="P17" t="n">
-        <v>52.7536170212766</v>
+        <v>51.90255319148936</v>
       </c>
       <c r="Q17" t="b">
         <v>0</v>
@@ -1822,22 +1822,22 @@
         <v>633.8</v>
       </c>
       <c r="D18" t="n">
-        <v>-0.08436867957237799</v>
+        <v>-0.09747241011035961</v>
       </c>
       <c r="E18" t="n">
-        <v>0.0360441356763383</v>
+        <v>0.0367220086693382</v>
       </c>
       <c r="F18" t="n">
-        <v>-0.0464154066049801</v>
+        <v>-0.0405691795337572</v>
       </c>
       <c r="G18" t="n">
-        <v>0.0675839019440025</v>
+        <v>0.0636191769455951</v>
       </c>
       <c r="H18" t="n">
-        <v>0.0383929190610885</v>
+        <v>0.0359065864004187</v>
       </c>
       <c r="I18" t="n">
-        <v>42.69977595220314</v>
+        <v>45.17084732372111</v>
       </c>
       <c r="J18" t="n">
         <v>40</v>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M18" t="n">
@@ -1857,10 +1857,10 @@
         <v>40</v>
       </c>
       <c r="O18" t="n">
-        <v>59.57446808510638</v>
+        <v>61.70212765957447</v>
       </c>
       <c r="P18" t="n">
-        <v>47.88289361702128</v>
+        <v>48.3084255319149</v>
       </c>
       <c r="Q18" t="b">
         <v>0</v>
@@ -1887,22 +1887,22 @@
         <v>2251.9</v>
       </c>
       <c r="D19" t="n">
-        <v>-0.1010379241516965</v>
+        <v>-0.1024711040255081</v>
       </c>
       <c r="E19" t="n">
-        <v>-0.1305069693810572</v>
+        <v>-0.1145407360805284</v>
       </c>
       <c r="F19" t="n">
-        <v>-0.2595357095883203</v>
+        <v>-0.2303038589055609</v>
       </c>
       <c r="G19" t="n">
-        <v>-0.1455364010393376</v>
+        <v>-0.1261155024262085</v>
       </c>
       <c r="H19" t="n">
-        <v>-0.1747273839222516</v>
+        <v>-0.1538280929713849</v>
       </c>
       <c r="I19" t="n">
-        <v>36.29951166576236</v>
+        <v>37.10482529118138</v>
       </c>
       <c r="J19" t="n">
         <v>30</v>
@@ -1912,7 +1912,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M19" t="n">
@@ -1922,10 +1922,10 @@
         <v>30</v>
       </c>
       <c r="O19" t="n">
-        <v>17.02127659574468</v>
+        <v>23.40425531914894</v>
       </c>
       <c r="P19" t="n">
-        <v>35.91225531914894</v>
+        <v>37.18885106382979</v>
       </c>
       <c r="Q19" t="b">
         <v>0</v>
@@ -1952,22 +1952,22 @@
         <v>1985.3</v>
       </c>
       <c r="D20" t="n">
-        <v>-0.06850279172336129</v>
+        <v>-0.0730693808945747</v>
       </c>
       <c r="E20" t="n">
-        <v>-0.1217041231640417</v>
+        <v>-0.1090517434815779</v>
       </c>
       <c r="F20" t="n">
-        <v>-0.06802178199230111</v>
+        <v>-0.082408948049547</v>
       </c>
       <c r="G20" t="n">
-        <v>0.0459775265566815</v>
+        <v>0.0217794084298054</v>
       </c>
       <c r="H20" t="n">
-        <v>0.0167865436737675</v>
+        <v>-0.0059331821153709</v>
       </c>
       <c r="I20" t="n">
-        <v>45.41721660067459</v>
+        <v>48.45877014551714</v>
       </c>
       <c r="J20" t="n">
         <v>40</v>
@@ -1977,7 +1977,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M20" t="n">
@@ -1987,16 +1987,16 @@
         <v>40</v>
       </c>
       <c r="O20" t="n">
-        <v>57.44680851063831</v>
+        <v>53.19148936170212</v>
       </c>
       <c r="P20" t="n">
-        <v>47.11336170212766</v>
+        <v>46.26229787234043</v>
       </c>
       <c r="Q20" t="b">
         <v>0</v>
       </c>
       <c r="R20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S20" t="b">
         <v>0</v>
@@ -2017,22 +2017,22 @@
         <v>876.7</v>
       </c>
       <c r="D21" t="n">
-        <v>-0.0550255995688493</v>
+        <v>-0.06719157312337069</v>
       </c>
       <c r="E21" t="n">
-        <v>-0.1318082788671023</v>
+        <v>-0.1561266724420059</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.3058041016707578</v>
+        <v>-0.2949738640932851</v>
       </c>
       <c r="G21" t="n">
-        <v>-0.1918047931217751</v>
+        <v>-0.1907855076139326</v>
       </c>
       <c r="H21" t="n">
-        <v>-0.2209957760046891</v>
+        <v>-0.218498098159109</v>
       </c>
       <c r="I21" t="n">
-        <v>55.66567558638918</v>
+        <v>57.90378006872851</v>
       </c>
       <c r="J21" t="n">
         <v>60</v>
@@ -2042,7 +2042,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M21" t="n">
@@ -2052,10 +2052,10 @@
         <v>60</v>
       </c>
       <c r="O21" t="n">
-        <v>8.51063829787234</v>
+        <v>10.63829787234042</v>
       </c>
       <c r="P21" t="n">
-        <v>45.07412765957447</v>
+        <v>45.49965957446808</v>
       </c>
       <c r="Q21" t="b">
         <v>0</v>
@@ -2082,22 +2082,22 @@
         <v>371.3</v>
       </c>
       <c r="D22" t="n">
-        <v>-0.1005329457364341</v>
+        <v>-0.1298336067494726</v>
       </c>
       <c r="E22" t="n">
-        <v>0.2453463021968809</v>
+        <v>0.2223868312757202</v>
       </c>
       <c r="F22" t="n">
-        <v>0.1856937569854704</v>
+        <v>0.2027858762552641</v>
       </c>
       <c r="G22" t="n">
-        <v>0.2996930655344531</v>
+        <v>0.3069742327346165</v>
       </c>
       <c r="H22" t="n">
-        <v>0.2705020826515391</v>
+        <v>0.2792616421894401</v>
       </c>
       <c r="I22" t="n">
-        <v>44.83695652173915</v>
+        <v>46.1466749533872</v>
       </c>
       <c r="J22" t="n">
         <v>40</v>
@@ -2107,7 +2107,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M22" t="n">
@@ -2147,45 +2147,45 @@
         <v>333.55</v>
       </c>
       <c r="D23" t="n">
-        <v>-0.0618759668119814</v>
+        <v>-0.0671234792336735</v>
       </c>
       <c r="E23" t="n">
-        <v>-0.1119542066027688</v>
+        <v>-0.1446339274265931</v>
       </c>
       <c r="F23" t="n">
-        <v>-0.1923728813559322</v>
+        <v>-0.1919815891472868</v>
       </c>
       <c r="G23" t="n">
-        <v>-0.0783735728069495</v>
+        <v>-0.0877932326679343</v>
       </c>
       <c r="H23" t="n">
-        <v>-0.1075645556898635</v>
+        <v>-0.1155058232131107</v>
       </c>
       <c r="I23" t="n">
-        <v>39.49631449631451</v>
+        <v>46.7296511627907</v>
       </c>
       <c r="J23" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K23" t="n">
         <v>49.7</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M23" t="n">
         <v>49.7</v>
       </c>
       <c r="N23" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O23" t="n">
         <v>36.17021276595745</v>
       </c>
       <c r="P23" t="n">
-        <v>39.1140425531915</v>
+        <v>43.1140425531915</v>
       </c>
       <c r="Q23" t="b">
         <v>0</v>
@@ -2212,22 +2212,22 @@
         <v>116.04</v>
       </c>
       <c r="D24" t="n">
-        <v>-0.1542274052478133</v>
+        <v>-0.1593131927841773</v>
       </c>
       <c r="E24" t="n">
-        <v>-0.08326749881497859</v>
+        <v>-0.0828327537148275</v>
       </c>
       <c r="F24" t="n">
-        <v>0.0725575376652187</v>
+        <v>0.07964272422776331</v>
       </c>
       <c r="G24" t="n">
-        <v>0.1865568462142014</v>
+        <v>0.1838310807071157</v>
       </c>
       <c r="H24" t="n">
-        <v>0.1573658633312874</v>
+        <v>0.1561184901619393</v>
       </c>
       <c r="I24" t="n">
-        <v>48.56386999244142</v>
+        <v>47.2378367900756</v>
       </c>
       <c r="J24" t="n">
         <v>40</v>
@@ -2237,7 +2237,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M24" t="n">
@@ -2277,22 +2277,22 @@
         <v>561.7</v>
       </c>
       <c r="D25" t="n">
-        <v>0.1057086614173228</v>
+        <v>0.09237650719564371</v>
       </c>
       <c r="E25" t="n">
-        <v>-0.1046465290507691</v>
+        <v>-0.1022136977543354</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.1103191573612101</v>
+        <v>-0.1025005991851082</v>
       </c>
       <c r="G25" t="n">
-        <v>0.0036801511877725</v>
+        <v>0.0016877572942441</v>
       </c>
       <c r="H25" t="n">
-        <v>-0.0255108316951414</v>
+        <v>-0.0260248332509321</v>
       </c>
       <c r="I25" t="n">
-        <v>60.43020736614052</v>
+        <v>61.984126984127</v>
       </c>
       <c r="J25" t="n">
         <v>80</v>
@@ -2302,7 +2302,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M25" t="n">
@@ -2342,45 +2342,45 @@
         <v>127.14</v>
       </c>
       <c r="D26" t="n">
-        <v>-0.0173892881984696</v>
+        <v>-0.0365992270970675</v>
       </c>
       <c r="E26" t="n">
-        <v>-0.0973375931842385</v>
+        <v>-0.09906462585034009</v>
       </c>
       <c r="F26" t="n">
-        <v>-0.2498672488052392</v>
+        <v>-0.2308064613709237</v>
       </c>
       <c r="G26" t="n">
-        <v>-0.1358679402562566</v>
+        <v>-0.1266181048915713</v>
       </c>
       <c r="H26" t="n">
-        <v>-0.1650589231391706</v>
+        <v>-0.1543306954367477</v>
       </c>
       <c r="I26" t="n">
-        <v>45.95569294178259</v>
+        <v>46.12202688728027</v>
       </c>
       <c r="J26" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K26" t="n">
         <v>51.54</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M26" t="n">
         <v>51.54</v>
       </c>
       <c r="N26" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O26" t="n">
-        <v>19.14893617021277</v>
+        <v>21.27659574468085</v>
       </c>
       <c r="P26" t="n">
-        <v>40.44578723404256</v>
+        <v>48.87131914893617</v>
       </c>
       <c r="Q26" t="b">
         <v>0</v>
@@ -2407,22 +2407,22 @@
         <v>4785</v>
       </c>
       <c r="D27" t="n">
-        <v>-0.1530223913620674</v>
+        <v>-0.1632421089446533</v>
       </c>
       <c r="E27" t="n">
-        <v>-0.0829819854350325</v>
+        <v>-0.0564921620822241</v>
       </c>
       <c r="F27" t="n">
-        <v>0.1431233426503262</v>
+        <v>0.1548208036683962</v>
       </c>
       <c r="G27" t="n">
-        <v>0.2571226511993089</v>
+        <v>0.2590091601477486</v>
       </c>
       <c r="H27" t="n">
-        <v>0.2279316683163949</v>
+        <v>0.2312965696025722</v>
       </c>
       <c r="I27" t="n">
-        <v>49.33389426447903</v>
+        <v>47.14745465184318</v>
       </c>
       <c r="J27" t="n">
         <v>40</v>
@@ -2432,7 +2432,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M27" t="n">
@@ -2472,22 +2472,22 @@
         <v>1613.9</v>
       </c>
       <c r="D28" t="n">
-        <v>0.0522918432548737</v>
+        <v>0.0700125969634688</v>
       </c>
       <c r="E28" t="n">
-        <v>0.0449336354807381</v>
+        <v>-0.0016701719658541</v>
       </c>
       <c r="F28" t="n">
-        <v>0.4464061659795664</v>
+        <v>0.5053633056617854</v>
       </c>
       <c r="G28" t="n">
-        <v>0.5604054745285491</v>
+        <v>0.6095516621411379</v>
       </c>
       <c r="H28" t="n">
-        <v>0.5312144916456351</v>
+        <v>0.5818390715959615</v>
       </c>
       <c r="I28" t="n">
-        <v>62.49826316520774</v>
+        <v>61.51433052901754</v>
       </c>
       <c r="J28" t="n">
         <v>80</v>
@@ -2497,7 +2497,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M28" t="n">
@@ -2537,22 +2537,22 @@
         <v>501.4</v>
       </c>
       <c r="D29" t="n">
-        <v>-0.0452251737598781</v>
+        <v>-0.0510078546418094</v>
       </c>
       <c r="E29" t="n">
-        <v>-0.1266329907681589</v>
+        <v>-0.1427594460591554</v>
       </c>
       <c r="F29" t="n">
-        <v>-0.0166699352814276</v>
+        <v>-0.0110453648915187</v>
       </c>
       <c r="G29" t="n">
-        <v>0.09732937326755491</v>
+        <v>0.0931429915878336</v>
       </c>
       <c r="H29" t="n">
-        <v>0.0681383903846409</v>
+        <v>0.06543040104265729</v>
       </c>
       <c r="I29" t="n">
-        <v>56.60559305689488</v>
+        <v>56.53573728267867</v>
       </c>
       <c r="J29" t="n">
         <v>40</v>
@@ -2562,7 +2562,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M29" t="n">
@@ -2602,22 +2602,22 @@
         <v>108.6</v>
       </c>
       <c r="D30" t="n">
-        <v>-0.0553235908141962</v>
+        <v>-0.0791928099033407</v>
       </c>
       <c r="E30" t="n">
-        <v>0.0155227230222554</v>
+        <v>-0.021180712032447</v>
       </c>
       <c r="F30" t="n">
-        <v>-0.1831515607371192</v>
+        <v>-0.1863340076421668</v>
       </c>
       <c r="G30" t="n">
-        <v>-0.0691522521881365</v>
+        <v>-0.0821456511628143</v>
       </c>
       <c r="H30" t="n">
-        <v>-0.0983432350710505</v>
+        <v>-0.1098582417079907</v>
       </c>
       <c r="I30" t="n">
-        <v>30.56241426611795</v>
+        <v>30.10218171775749</v>
       </c>
       <c r="J30" t="n">
         <v>30</v>
@@ -2627,7 +2627,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M30" t="n">
@@ -2667,22 +2667,22 @@
         <v>37.07</v>
       </c>
       <c r="D31" t="n">
-        <v>-0.1054536679536679</v>
+        <v>-0.1080365736284889</v>
       </c>
       <c r="E31" t="n">
-        <v>-0.2359851607584502</v>
+        <v>-0.2422322158626328</v>
       </c>
       <c r="F31" t="n">
-        <v>-0.2420772848088325</v>
+        <v>-0.251111111111111</v>
       </c>
       <c r="G31" t="n">
-        <v>-0.1280779762598498</v>
+        <v>-0.1469227546317586</v>
       </c>
       <c r="H31" t="n">
-        <v>-0.1572689591427638</v>
+        <v>-0.174635345176935</v>
       </c>
       <c r="I31" t="n">
-        <v>38.91951488423375</v>
+        <v>38.44444444444445</v>
       </c>
       <c r="J31" t="n">
         <v>30</v>
@@ -2692,7 +2692,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M31" t="n">
@@ -2702,10 +2702,10 @@
         <v>30</v>
       </c>
       <c r="O31" t="n">
-        <v>21.27659574468085</v>
+        <v>17.02127659574468</v>
       </c>
       <c r="P31" t="n">
-        <v>35.85131914893617</v>
+        <v>35.00025531914894</v>
       </c>
       <c r="Q31" t="b">
         <v>0</v>
@@ -2732,22 +2732,22 @@
         <v>659.5</v>
       </c>
       <c r="D32" t="n">
-        <v>-0.06513572896732581</v>
+        <v>-0.0621444823663254</v>
       </c>
       <c r="E32" t="n">
-        <v>-0.2085208520852085</v>
+        <v>-0.1807453416149068</v>
       </c>
       <c r="F32" t="n">
-        <v>-0.4136214101538188</v>
+        <v>-0.3854254030379275</v>
       </c>
       <c r="G32" t="n">
-        <v>-0.2996221016048361</v>
+        <v>-0.281237046558575</v>
       </c>
       <c r="H32" t="n">
-        <v>-0.3288130844877501</v>
+        <v>-0.3089496371037514</v>
       </c>
       <c r="I32" t="n">
-        <v>50.82802547770701</v>
+        <v>51.68393782383419</v>
       </c>
       <c r="J32" t="n">
         <v>40</v>
@@ -2757,7 +2757,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M32" t="n">
@@ -2797,22 +2797,22 @@
         <v>529.85</v>
       </c>
       <c r="D33" t="n">
-        <v>-0.0617141845227554</v>
+        <v>-0.057793189294923</v>
       </c>
       <c r="E33" t="n">
-        <v>-0.1985327484495538</v>
+        <v>-0.1978046934140802</v>
       </c>
       <c r="F33" t="n">
-        <v>0.0150383141762453</v>
+        <v>0.020315809743886</v>
       </c>
       <c r="G33" t="n">
-        <v>0.129037622725228</v>
+        <v>0.1245041662232384</v>
       </c>
       <c r="H33" t="n">
-        <v>0.099846639842314</v>
+        <v>0.096791575678062</v>
       </c>
       <c r="I33" t="n">
-        <v>54.07779171894605</v>
+        <v>51.41055426485231</v>
       </c>
       <c r="J33" t="n">
         <v>40</v>
@@ -2822,7 +2822,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M33" t="n">
@@ -2832,10 +2832,10 @@
         <v>40</v>
       </c>
       <c r="O33" t="n">
-        <v>70.21276595744681</v>
+        <v>72.3404255319149</v>
       </c>
       <c r="P33" t="n">
-        <v>50.03455319148937</v>
+        <v>50.46008510638298</v>
       </c>
       <c r="Q33" t="b">
         <v>0</v>
@@ -2871,10 +2871,10 @@
         <v>-0.2401052253975846</v>
       </c>
       <c r="G34" t="n">
-        <v>-0.1261059168486019</v>
+        <v>-0.1359168689182321</v>
       </c>
       <c r="H34" t="n">
-        <v>-0.1552968997315159</v>
+        <v>-0.1636294594634085</v>
       </c>
       <c r="I34" t="n">
         <v>63.3225806451613</v>
@@ -2887,7 +2887,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M34" t="n">
@@ -2897,10 +2897,10 @@
         <v>80</v>
       </c>
       <c r="O34" t="n">
-        <v>23.40425531914894</v>
+        <v>19.14893617021277</v>
       </c>
       <c r="P34" t="n">
-        <v>57.03285106382979</v>
+        <v>56.18178723404256</v>
       </c>
       <c r="Q34" t="b">
         <v>0</v>
@@ -2927,22 +2927,22 @@
         <v>108.75</v>
       </c>
       <c r="D35" t="n">
-        <v>-0.0693196405648266</v>
+        <v>-0.0698768388641806</v>
       </c>
       <c r="E35" t="n">
-        <v>-0.2015418502202642</v>
+        <v>-0.2122419413256067</v>
       </c>
       <c r="F35" t="n">
-        <v>0.06890112050324371</v>
+        <v>0.0752422384813129</v>
       </c>
       <c r="G35" t="n">
-        <v>0.1829004290522263</v>
+        <v>0.1794305949606653</v>
       </c>
       <c r="H35" t="n">
-        <v>0.1537094461693123</v>
+        <v>0.151718004415489</v>
       </c>
       <c r="I35" t="n">
-        <v>53.28719723183392</v>
+        <v>53.20623916811091</v>
       </c>
       <c r="J35" t="n">
         <v>60</v>
@@ -2952,7 +2952,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M35" t="n">
@@ -2992,22 +2992,22 @@
         <v>461.35</v>
       </c>
       <c r="D36" t="n">
-        <v>-0.0760989286071893</v>
+        <v>-0.0825295813860992</v>
       </c>
       <c r="E36" t="n">
-        <v>-0.1613343028540265</v>
+        <v>-0.14880073800738</v>
       </c>
       <c r="F36" t="n">
-        <v>0.0002168021680217</v>
+        <v>-0.0034560967707094</v>
       </c>
       <c r="G36" t="n">
-        <v>0.1142161107170044</v>
+        <v>0.1007322597086429</v>
       </c>
       <c r="H36" t="n">
-        <v>0.0850251278340904</v>
+        <v>0.0730196691634665</v>
       </c>
       <c r="I36" t="n">
-        <v>41.17187500000001</v>
+        <v>41.07981220657278</v>
       </c>
       <c r="J36" t="n">
         <v>40</v>
@@ -3017,7 +3017,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M36" t="n">
@@ -3057,22 +3057,22 @@
         <v>2136.6</v>
       </c>
       <c r="D37" t="n">
-        <v>-0.0145288501452884</v>
+        <v>-0.0434704749966422</v>
       </c>
       <c r="E37" t="n">
-        <v>0.2740608228980321</v>
+        <v>0.2101954120645708</v>
       </c>
       <c r="F37" t="n">
-        <v>0.5095379398050019</v>
+        <v>0.5090048732255101</v>
       </c>
       <c r="G37" t="n">
-        <v>0.6235372483539846</v>
+        <v>0.6131932297048626</v>
       </c>
       <c r="H37" t="n">
-        <v>0.5943462654710706</v>
+        <v>0.5854806391596862</v>
       </c>
       <c r="I37" t="n">
-        <v>61.35631043887923</v>
+        <v>57.48772504091652</v>
       </c>
       <c r="J37" t="n">
         <v>80</v>
@@ -3082,7 +3082,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M37" t="n">
@@ -3122,22 +3122,22 @@
         <v>736.1</v>
       </c>
       <c r="D38" t="n">
-        <v>-0.1459070603933399</v>
+        <v>-0.1294938505203405</v>
       </c>
       <c r="E38" t="n">
-        <v>-0.2172063593342904</v>
+        <v>-0.2180794561291692</v>
       </c>
       <c r="F38" t="n">
-        <v>-0.3016791575751825</v>
+        <v>-0.2971450396257041</v>
       </c>
       <c r="G38" t="n">
-        <v>-0.1876798490261998</v>
+        <v>-0.1929566831463517</v>
       </c>
       <c r="H38" t="n">
-        <v>-0.2168708319091138</v>
+        <v>-0.2206692736915281</v>
       </c>
       <c r="I38" t="n">
-        <v>43.53045798132504</v>
+        <v>45.77618453865336</v>
       </c>
       <c r="J38" t="n">
         <v>40</v>
@@ -3147,7 +3147,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M38" t="n">
@@ -3157,10 +3157,10 @@
         <v>40</v>
       </c>
       <c r="O38" t="n">
-        <v>10.63829787234042</v>
+        <v>8.51063829787234</v>
       </c>
       <c r="P38" t="n">
-        <v>38.07565957446808</v>
+        <v>37.65012765957447</v>
       </c>
       <c r="Q38" t="b">
         <v>0</v>
@@ -3187,22 +3187,22 @@
         <v>2928.4</v>
       </c>
       <c r="D39" t="n">
-        <v>-0.0138407139249031</v>
+        <v>-0.0202415604402957</v>
       </c>
       <c r="E39" t="n">
-        <v>-0.0956145768993205</v>
+        <v>-0.0688120071228695</v>
       </c>
       <c r="F39" t="n">
-        <v>0.1000338078960221</v>
+        <v>0.1211332312404287</v>
       </c>
       <c r="G39" t="n">
-        <v>0.2140331164450047</v>
+        <v>0.2253215877197811</v>
       </c>
       <c r="H39" t="n">
-        <v>0.1848421335620907</v>
+        <v>0.1976089971746047</v>
       </c>
       <c r="I39" t="n">
-        <v>53.54029967681912</v>
+        <v>49.24574729859849</v>
       </c>
       <c r="J39" t="n">
         <v>40</v>
@@ -3212,7 +3212,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M39" t="n">
@@ -3252,22 +3252,22 @@
         <v>189.25</v>
       </c>
       <c r="D40" t="n">
-        <v>-0.0346357886145684</v>
+        <v>-0.0437089439110661</v>
       </c>
       <c r="E40" t="n">
-        <v>-0.0229736706246772</v>
+        <v>-0.0984231337239769</v>
       </c>
       <c r="F40" t="n">
-        <v>-0.2244170320888487</v>
+        <v>-0.2290300240355236</v>
       </c>
       <c r="G40" t="n">
-        <v>-0.1104177235398661</v>
+        <v>-0.1248416675561712</v>
       </c>
       <c r="H40" t="n">
-        <v>-0.1396087064227801</v>
+        <v>-0.1525542581013476</v>
       </c>
       <c r="I40" t="n">
-        <v>54.87893286936349</v>
+        <v>57.81273865892775</v>
       </c>
       <c r="J40" t="n">
         <v>60</v>
@@ -3277,7 +3277,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M40" t="n">
@@ -3317,22 +3317,22 @@
         <v>749.9</v>
       </c>
       <c r="D41" t="n">
-        <v>-0.1028831199904294</v>
+        <v>-0.120815991558708</v>
       </c>
       <c r="E41" t="n">
-        <v>-0.1976675760980045</v>
+        <v>-0.2074195423558632</v>
       </c>
       <c r="F41" t="n">
-        <v>-0.2616914443241115</v>
+        <v>-0.2589188655005435</v>
       </c>
       <c r="G41" t="n">
-        <v>-0.1476921357751288</v>
+        <v>-0.1547305090211911</v>
       </c>
       <c r="H41" t="n">
-        <v>-0.1768831186580428</v>
+        <v>-0.1824430995663675</v>
       </c>
       <c r="I41" t="n">
-        <v>21.74931667317455</v>
+        <v>24.41911442349847</v>
       </c>
       <c r="J41" t="n">
         <v>20</v>
@@ -3342,7 +3342,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M41" t="n">
@@ -3382,22 +3382,22 @@
         <v>497.15</v>
       </c>
       <c r="D42" t="n">
-        <v>-0.126887952230418</v>
+        <v>-0.1336586215910081</v>
       </c>
       <c r="E42" t="n">
-        <v>-0.2757666253915071</v>
+        <v>-0.2803792429615691</v>
       </c>
       <c r="F42" t="n">
-        <v>-0.354434489027399</v>
+        <v>-0.3509791122715405</v>
       </c>
       <c r="G42" t="n">
-        <v>-0.2404351804784164</v>
+        <v>-0.2467907557921881</v>
       </c>
       <c r="H42" t="n">
-        <v>-0.2696261633613304</v>
+        <v>-0.2745033463373645</v>
       </c>
       <c r="I42" t="n">
-        <v>36.97642163661581</v>
+        <v>35.14130745075647</v>
       </c>
       <c r="J42" t="n">
         <v>30</v>
@@ -3407,7 +3407,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M42" t="n">
@@ -3447,22 +3447,22 @@
         <v>411.55</v>
       </c>
       <c r="D43" t="n">
-        <v>-0.0267234243821686</v>
+        <v>-0.0352789498359118</v>
       </c>
       <c r="E43" t="n">
-        <v>-0.1120819848975188</v>
+        <v>-0.1257567711099309</v>
       </c>
       <c r="F43" t="n">
-        <v>-0.1023991275899672</v>
+        <v>-0.078688157600179</v>
       </c>
       <c r="G43" t="n">
-        <v>0.0116001809590153</v>
+        <v>0.0255001988791734</v>
       </c>
       <c r="H43" t="n">
-        <v>-0.0175908019238986</v>
+        <v>-0.0022123916660029</v>
       </c>
       <c r="I43" t="n">
-        <v>54.21940928270043</v>
+        <v>51.85801442041044</v>
       </c>
       <c r="J43" t="n">
         <v>60</v>
@@ -3472,7 +3472,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M43" t="n">
@@ -3482,10 +3482,10 @@
         <v>60</v>
       </c>
       <c r="O43" t="n">
-        <v>53.19148936170212</v>
+        <v>55.31914893617022</v>
       </c>
       <c r="P43" t="n">
-        <v>55.23029787234042</v>
+        <v>55.65582978723404</v>
       </c>
       <c r="Q43" t="b">
         <v>0</v>
@@ -3512,22 +3512,22 @@
         <v>246.66</v>
       </c>
       <c r="D44" t="n">
-        <v>0.0161071060762101</v>
+        <v>0.0075980392156862</v>
       </c>
       <c r="E44" t="n">
-        <v>-0.1028914348063284</v>
+        <v>-0.1025650354738949</v>
       </c>
       <c r="F44" t="n">
-        <v>-0.1753259779338014</v>
+        <v>-0.171030078978323</v>
       </c>
       <c r="G44" t="n">
-        <v>-0.0613266693848187</v>
+        <v>-0.0668417224989705</v>
       </c>
       <c r="H44" t="n">
-        <v>-0.0905176522677327</v>
+        <v>-0.0945543130441469</v>
       </c>
       <c r="I44" t="n">
-        <v>49.41771556287495</v>
+        <v>55.70879193740883</v>
       </c>
       <c r="J44" t="n">
         <v>60</v>
@@ -3537,7 +3537,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M44" t="n">
@@ -3577,22 +3577,22 @@
         <v>89.8</v>
       </c>
       <c r="D45" t="n">
-        <v>-0.1173579712993906</v>
+        <v>-0.1123850943955718</v>
       </c>
       <c r="E45" t="n">
-        <v>-0.1866678742867493</v>
+        <v>-0.1757687012391006</v>
       </c>
       <c r="F45" t="n">
-        <v>-0.3683173888576252</v>
+        <v>-0.3556257175660161</v>
       </c>
       <c r="G45" t="n">
-        <v>-0.2543180803086425</v>
+        <v>-0.2514373610866637</v>
       </c>
       <c r="H45" t="n">
-        <v>-0.2835090631915565</v>
+        <v>-0.2791499516318401</v>
       </c>
       <c r="I45" t="n">
-        <v>36.57370517928285</v>
+        <v>39.30916357407933</v>
       </c>
       <c r="J45" t="n">
         <v>30</v>
@@ -3602,7 +3602,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M45" t="n">
@@ -3642,45 +3642,45 @@
         <v>490</v>
       </c>
       <c r="D46" t="n">
-        <v>-0.0479891198756557</v>
+        <v>-0.0394981868078015</v>
       </c>
       <c r="E46" t="n">
-        <v>-0.170335252285811</v>
+        <v>-0.1932164320408331</v>
       </c>
       <c r="F46" t="n">
-        <v>-0.1958644457208501</v>
+        <v>-0.1967871485943774</v>
       </c>
       <c r="G46" t="n">
-        <v>-0.0818651371718675</v>
+        <v>-0.09259879211502491</v>
       </c>
       <c r="H46" t="n">
-        <v>-0.1110561200547815</v>
+        <v>-0.1203113826602013</v>
       </c>
       <c r="I46" t="n">
-        <v>52.84003684372122</v>
+        <v>53.46380863622242</v>
       </c>
       <c r="J46" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K46" t="n">
         <v>49.61</v>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M46" t="n">
         <v>49.61</v>
       </c>
       <c r="N46" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O46" t="n">
-        <v>31.91489361702128</v>
+        <v>34.04255319148936</v>
       </c>
       <c r="P46" t="n">
-        <v>42.22697872340426</v>
+        <v>50.65251063829788</v>
       </c>
       <c r="Q46" t="b">
         <v>0</v>
@@ -3707,22 +3707,22 @@
         <v>974.35</v>
       </c>
       <c r="D47" t="n">
-        <v>0.1176301904106447</v>
+        <v>0.09798287130944321</v>
       </c>
       <c r="E47" t="n">
-        <v>0.1325700337091713</v>
+        <v>0.126611551136035</v>
       </c>
       <c r="F47" t="n">
-        <v>0.3150010122140494</v>
+        <v>0.3098743026147745</v>
       </c>
       <c r="G47" t="n">
-        <v>0.4290003207630321</v>
+        <v>0.414062659094127</v>
       </c>
       <c r="H47" t="n">
-        <v>0.3998093378801181</v>
+        <v>0.3863500685489506</v>
       </c>
       <c r="I47" t="n">
-        <v>59.59416613823716</v>
+        <v>57.26931330472104</v>
       </c>
       <c r="J47" t="n">
         <v>60</v>
@@ -3732,7 +3732,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M47" t="n">
@@ -3772,22 +3772,22 @@
         <v>13974</v>
       </c>
       <c r="D48" t="n">
-        <v>-0.0170230725942599</v>
+        <v>-0.0247068676716918</v>
       </c>
       <c r="E48" t="n">
-        <v>-0.0607608549536228</v>
+        <v>-0.051259420191459</v>
       </c>
       <c r="F48" t="n">
-        <v>0.0185873605947954</v>
+        <v>0.0315198937034029</v>
       </c>
       <c r="G48" t="n">
-        <v>0.1325866691437781</v>
+        <v>0.1357082501827553</v>
       </c>
       <c r="H48" t="n">
-        <v>0.1033956862608641</v>
+        <v>0.1079956596375789</v>
       </c>
       <c r="I48" t="n">
-        <v>55.78125</v>
+        <v>54.85003190810466</v>
       </c>
       <c r="J48" t="n">
         <v>60</v>
@@ -3797,7 +3797,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M48" t="n">
@@ -3807,10 +3807,10 @@
         <v>60</v>
       </c>
       <c r="O48" t="n">
-        <v>72.3404255319149</v>
+        <v>76.59574468085107</v>
       </c>
       <c r="P48" t="n">
-        <v>58.58408510638298</v>
+        <v>59.43514893617021</v>
       </c>
       <c r="Q48" t="b">
         <v>0</v>
@@ -3948,22 +3948,22 @@
         <v>1613.9</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0522918432548737</v>
+        <v>0.0700125969634688</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0449336354807381</v>
+        <v>-0.0016701719658541</v>
       </c>
       <c r="F2" t="n">
-        <v>0.4464061659795664</v>
+        <v>0.5053633056617854</v>
       </c>
       <c r="G2" t="n">
-        <v>0.5604054745285491</v>
+        <v>0.6095516621411379</v>
       </c>
       <c r="H2" t="n">
-        <v>0.5312144916456351</v>
+        <v>0.5818390715959615</v>
       </c>
       <c r="I2" t="n">
-        <v>62.49826316520774</v>
+        <v>61.51433052901754</v>
       </c>
       <c r="J2" t="n">
         <v>80</v>
@@ -3973,7 +3973,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M2" t="n">
@@ -4013,22 +4013,22 @@
         <v>2136.6</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.0145288501452884</v>
+        <v>-0.0434704749966422</v>
       </c>
       <c r="E3" t="n">
-        <v>0.2740608228980321</v>
+        <v>0.2101954120645708</v>
       </c>
       <c r="F3" t="n">
-        <v>0.5095379398050019</v>
+        <v>0.5090048732255101</v>
       </c>
       <c r="G3" t="n">
-        <v>0.6235372483539846</v>
+        <v>0.6131932297048626</v>
       </c>
       <c r="H3" t="n">
-        <v>0.5943462654710706</v>
+        <v>0.5854806391596862</v>
       </c>
       <c r="I3" t="n">
-        <v>61.35631043887923</v>
+        <v>57.48772504091652</v>
       </c>
       <c r="J3" t="n">
         <v>80</v>
@@ -4038,7 +4038,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M3" t="n">
@@ -4078,22 +4078,22 @@
         <v>436.5</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1303897449177782</v>
+        <v>0.1213872832369942</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.08806016922594791</v>
+        <v>-0.08739284967593559</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.1646732370108122</v>
+        <v>-0.1526739784528777</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.0506739284618296</v>
+        <v>-0.0484856219735253</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.07986491134474361</v>
+        <v>-0.07619821251870169</v>
       </c>
       <c r="I4" t="n">
-        <v>64.88250652741513</v>
+        <v>63.01558203483042</v>
       </c>
       <c r="J4" t="n">
         <v>80</v>
@@ -4103,7 +4103,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M4" t="n">
@@ -4113,10 +4113,10 @@
         <v>80</v>
       </c>
       <c r="O4" t="n">
-        <v>42.5531914893617</v>
+        <v>44.68085106382978</v>
       </c>
       <c r="P4" t="n">
-        <v>69.02263829787233</v>
+        <v>69.44817021276596</v>
       </c>
       <c r="Q4" t="b">
         <v>1</v>
@@ -4143,22 +4143,22 @@
         <v>561.7</v>
       </c>
       <c r="D5" t="n">
-        <v>0.1057086614173228</v>
+        <v>0.09237650719564371</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.1046465290507691</v>
+        <v>-0.1022136977543354</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.1103191573612101</v>
+        <v>-0.1025005991851082</v>
       </c>
       <c r="G5" t="n">
-        <v>0.0036801511877725</v>
+        <v>0.0016877572942441</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.0255108316951414</v>
+        <v>-0.0260248332509321</v>
       </c>
       <c r="I5" t="n">
-        <v>60.43020736614052</v>
+        <v>61.984126984127</v>
       </c>
       <c r="J5" t="n">
         <v>80</v>
@@ -4168,7 +4168,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M5" t="n">
@@ -4208,22 +4208,22 @@
         <v>974.35</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1176301904106447</v>
+        <v>0.09798287130944321</v>
       </c>
       <c r="E6" t="n">
-        <v>0.1325700337091713</v>
+        <v>0.126611551136035</v>
       </c>
       <c r="F6" t="n">
-        <v>0.3150010122140494</v>
+        <v>0.3098743026147745</v>
       </c>
       <c r="G6" t="n">
-        <v>0.4290003207630321</v>
+        <v>0.414062659094127</v>
       </c>
       <c r="H6" t="n">
-        <v>0.3998093378801181</v>
+        <v>0.3863500685489506</v>
       </c>
       <c r="I6" t="n">
-        <v>59.59416613823716</v>
+        <v>57.26931330472104</v>
       </c>
       <c r="J6" t="n">
         <v>60</v>
@@ -4233,7 +4233,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M6" t="n">
@@ -4273,22 +4273,22 @@
         <v>108.75</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.0693196405648266</v>
+        <v>-0.0698768388641806</v>
       </c>
       <c r="E7" t="n">
-        <v>-0.2015418502202642</v>
+        <v>-0.2122419413256067</v>
       </c>
       <c r="F7" t="n">
-        <v>0.06890112050324371</v>
+        <v>0.0752422384813129</v>
       </c>
       <c r="G7" t="n">
-        <v>0.1829004290522263</v>
+        <v>0.1794305949606653</v>
       </c>
       <c r="H7" t="n">
-        <v>0.1537094461693123</v>
+        <v>0.151718004415489</v>
       </c>
       <c r="I7" t="n">
-        <v>53.28719723183392</v>
+        <v>53.20623916811091</v>
       </c>
       <c r="J7" t="n">
         <v>60</v>
@@ -4298,7 +4298,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M7" t="n">
@@ -4338,22 +4338,22 @@
         <v>13974</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.0170230725942599</v>
+        <v>-0.0247068676716918</v>
       </c>
       <c r="E8" t="n">
-        <v>-0.0607608549536228</v>
+        <v>-0.051259420191459</v>
       </c>
       <c r="F8" t="n">
-        <v>0.0185873605947954</v>
+        <v>0.0315198937034029</v>
       </c>
       <c r="G8" t="n">
-        <v>0.1325866691437781</v>
+        <v>0.1357082501827553</v>
       </c>
       <c r="H8" t="n">
-        <v>0.1033956862608641</v>
+        <v>0.1079956596375789</v>
       </c>
       <c r="I8" t="n">
-        <v>55.78125</v>
+        <v>54.85003190810466</v>
       </c>
       <c r="J8" t="n">
         <v>60</v>
@@ -4363,7 +4363,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M8" t="n">
@@ -4373,10 +4373,10 @@
         <v>60</v>
       </c>
       <c r="O8" t="n">
-        <v>72.3404255319149</v>
+        <v>76.59574468085107</v>
       </c>
       <c r="P8" t="n">
-        <v>58.58408510638298</v>
+        <v>59.43514893617021</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
@@ -4403,22 +4403,22 @@
         <v>2567.3</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.0735448017032945</v>
+        <v>-0.0771415219813795</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.0179029111357635</v>
+        <v>-0.0211979107095199</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.2064232944885783</v>
+        <v>-0.2005418366393672</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.0924239859395956</v>
+        <v>-0.0963534801600147</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.1216149688225096</v>
+        <v>-0.1240660707051911</v>
       </c>
       <c r="I9" t="n">
-        <v>57.64112620815244</v>
+        <v>60.69321533923305</v>
       </c>
       <c r="J9" t="n">
         <v>80</v>
@@ -4428,7 +4428,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M9" t="n">
@@ -4468,22 +4468,22 @@
         <v>1642.6</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.1081550656966011</v>
+        <v>-0.1347450484618627</v>
       </c>
       <c r="E10" t="n">
-        <v>0.1171109902067464</v>
+        <v>0.1216880633706636</v>
       </c>
       <c r="F10" t="n">
-        <v>0.3689474122843568</v>
+        <v>0.3553923591055365</v>
       </c>
       <c r="G10" t="n">
-        <v>0.4829467208333394</v>
+        <v>0.459580715584889</v>
       </c>
       <c r="H10" t="n">
-        <v>0.4537557379504254</v>
+        <v>0.4318681250397126</v>
       </c>
       <c r="I10" t="n">
-        <v>46.51959734418505</v>
+        <v>43.88764044943819</v>
       </c>
       <c r="J10" t="n">
         <v>40</v>
@@ -4493,7 +4493,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M10" t="n">
@@ -4521,63 +4521,63 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>RANEENGINE</t>
+          <t>LUMAXIND</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Engine/Parts</t>
+          <t>Lighting</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>317.75</v>
+        <v>4785</v>
       </c>
       <c r="D11" t="n">
-        <v>0.1790352504638219</v>
+        <v>-0.1632421089446533</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.156154561147258</v>
+        <v>-0.0564921620822241</v>
       </c>
       <c r="F11" t="n">
-        <v>-0.2401052253975846</v>
+        <v>0.1548208036683962</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.1261059168486019</v>
+        <v>0.2590091601477486</v>
       </c>
       <c r="H11" t="n">
-        <v>-0.1552968997315159</v>
+        <v>0.2312965696025722</v>
       </c>
       <c r="I11" t="n">
-        <v>63.3225806451613</v>
+        <v>47.14745465184318</v>
       </c>
       <c r="J11" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="K11" t="n">
-        <v>50.88</v>
+        <v>57.69</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M11" t="n">
-        <v>50.88</v>
+        <v>57.69</v>
       </c>
       <c r="N11" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="O11" t="n">
-        <v>23.40425531914894</v>
+        <v>89.36170212765957</v>
       </c>
       <c r="P11" t="n">
-        <v>57.03285106382979</v>
+        <v>56.94834042553191</v>
       </c>
       <c r="Q11" t="b">
         <v>0</v>
       </c>
       <c r="R11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S11" t="b">
         <v>0</v>
@@ -4586,63 +4586,63 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>LUMAXIND</t>
+          <t>RANEENGINE</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Lighting</t>
+          <t>Engine/Parts</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>4785</v>
+        <v>317.75</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.1530223913620674</v>
+        <v>0.1790352504638219</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.0829819854350325</v>
+        <v>-0.156154561147258</v>
       </c>
       <c r="F12" t="n">
-        <v>0.1431233426503262</v>
+        <v>-0.2401052253975846</v>
       </c>
       <c r="G12" t="n">
-        <v>0.2571226511993089</v>
+        <v>-0.1359168689182321</v>
       </c>
       <c r="H12" t="n">
-        <v>0.2279316683163949</v>
+        <v>-0.1636294594634085</v>
       </c>
       <c r="I12" t="n">
-        <v>49.33389426447903</v>
+        <v>63.3225806451613</v>
       </c>
       <c r="J12" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="K12" t="n">
-        <v>57.69</v>
+        <v>50.88</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M12" t="n">
-        <v>57.69</v>
+        <v>50.88</v>
       </c>
       <c r="N12" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="O12" t="n">
-        <v>89.36170212765957</v>
+        <v>19.14893617021277</v>
       </c>
       <c r="P12" t="n">
-        <v>56.94834042553191</v>
+        <v>56.18178723404256</v>
       </c>
       <c r="Q12" t="b">
         <v>0</v>
       </c>
       <c r="R12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S12" t="b">
         <v>0</v>
@@ -4663,22 +4663,22 @@
         <v>371.3</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.1005329457364341</v>
+        <v>-0.1298336067494726</v>
       </c>
       <c r="E13" t="n">
-        <v>0.2453463021968809</v>
+        <v>0.2223868312757202</v>
       </c>
       <c r="F13" t="n">
-        <v>0.1856937569854704</v>
+        <v>0.2027858762552641</v>
       </c>
       <c r="G13" t="n">
-        <v>0.2996930655344531</v>
+        <v>0.3069742327346165</v>
       </c>
       <c r="H13" t="n">
-        <v>0.2705020826515391</v>
+        <v>0.2792616421894401</v>
       </c>
       <c r="I13" t="n">
-        <v>44.83695652173915</v>
+        <v>46.1466749533872</v>
       </c>
       <c r="J13" t="n">
         <v>40</v>
@@ -4688,7 +4688,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M13" t="n">
@@ -4728,22 +4728,22 @@
         <v>411.55</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.0267234243821686</v>
+        <v>-0.0352789498359118</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.1120819848975188</v>
+        <v>-0.1257567711099309</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.1023991275899672</v>
+        <v>-0.078688157600179</v>
       </c>
       <c r="G14" t="n">
-        <v>0.0116001809590153</v>
+        <v>0.0255001988791734</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.0175908019238986</v>
+        <v>-0.0022123916660029</v>
       </c>
       <c r="I14" t="n">
-        <v>54.21940928270043</v>
+        <v>51.85801442041044</v>
       </c>
       <c r="J14" t="n">
         <v>60</v>
@@ -4753,7 +4753,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M14" t="n">
@@ -4763,10 +4763,10 @@
         <v>60</v>
       </c>
       <c r="O14" t="n">
-        <v>53.19148936170212</v>
+        <v>55.31914893617022</v>
       </c>
       <c r="P14" t="n">
-        <v>55.23029787234042</v>
+        <v>55.65582978723404</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
@@ -4793,22 +4793,22 @@
         <v>496.55</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.009672915835660101</v>
+        <v>-0.0281827967511497</v>
       </c>
       <c r="E15" t="n">
-        <v>0.0357738840216939</v>
+        <v>0.0469112376133249</v>
       </c>
       <c r="F15" t="n">
-        <v>0.1033218531274302</v>
+        <v>0.1286509830662576</v>
       </c>
       <c r="G15" t="n">
-        <v>0.2173211616764129</v>
+        <v>0.2328393395456101</v>
       </c>
       <c r="H15" t="n">
-        <v>0.1881301787934989</v>
+        <v>0.2051267490004337</v>
       </c>
       <c r="I15" t="n">
-        <v>53.73399715504979</v>
+        <v>52.67369952710077</v>
       </c>
       <c r="J15" t="n">
         <v>40</v>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M15" t="n">
@@ -4846,57 +4846,57 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CRAFTSMAN</t>
+          <t>SHRIPISTON</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Castings</t>
+          <t>Engine/Parts</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>6789</v>
+        <v>2928.4</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.0852253587549687</v>
+        <v>-0.0202415604402957</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.1171077443266792</v>
+        <v>-0.0688120071228695</v>
       </c>
       <c r="F16" t="n">
-        <v>0.019752159218926</v>
+        <v>0.1211332312404287</v>
       </c>
       <c r="G16" t="n">
-        <v>0.1337514677679087</v>
+        <v>0.2253215877197811</v>
       </c>
       <c r="H16" t="n">
-        <v>0.1045604848849947</v>
+        <v>0.1976089971746047</v>
       </c>
       <c r="I16" t="n">
-        <v>53.60275689223057</v>
+        <v>49.24574729859849</v>
       </c>
       <c r="J16" t="n">
         <v>40</v>
       </c>
       <c r="K16" t="n">
-        <v>54.65</v>
+        <v>48.69</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="M16" t="n">
-        <v>54.65</v>
+        <v>48.69</v>
       </c>
       <c r="N16" t="n">
         <v>40</v>
       </c>
       <c r="O16" t="n">
-        <v>74.46808510638297</v>
+        <v>85.1063829787234</v>
       </c>
       <c r="P16" t="n">
-        <v>52.7536170212766</v>
+        <v>52.49727659574468</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
chore: auto-refresh NSE data and pipeline outputs (2026-04-07)
</commit_message>
<xml_diff>
--- a/working-sector/output/auto_components_comprehensive_report.xlsx
+++ b/working-sector/output/auto_components_comprehensive_report.xlsx
@@ -435,7 +435,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
     </row>
@@ -447,7 +447,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
     </row>
@@ -779,48 +779,48 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1642.6</v>
+        <v>1671.3</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.1347450484618627</v>
+        <v>-0.1025613488696772</v>
       </c>
       <c r="E2" t="n">
-        <v>0.1216880633706636</v>
+        <v>0.127504553734062</v>
       </c>
       <c r="F2" t="n">
-        <v>0.3553923591055365</v>
+        <v>0.3508729388942773</v>
       </c>
       <c r="G2" t="n">
-        <v>0.459580715584889</v>
+        <v>0.4425720737588798</v>
       </c>
       <c r="H2" t="n">
-        <v>0.4318681250397126</v>
+        <v>0.4279158635523904</v>
       </c>
       <c r="I2" t="n">
-        <v>43.88764044943819</v>
+        <v>31.83183183183183</v>
       </c>
       <c r="J2" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K2" t="n">
         <v>54.83</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M2" t="n">
         <v>54.83</v>
       </c>
       <c r="N2" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O2" t="n">
         <v>95.74468085106383</v>
       </c>
       <c r="P2" t="n">
-        <v>57.08093617021277</v>
+        <v>53.08093617021277</v>
       </c>
       <c r="Q2" t="b">
         <v>0</v>
@@ -844,25 +844,25 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1025.4</v>
+        <v>1021.4</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.0830725207904854</v>
+        <v>-0.056094630810461</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.2030776404756352</v>
+        <v>-0.2358222355229686</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.200280767430978</v>
+        <v>-0.2152132155205532</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.0960924109516255</v>
+        <v>-0.1235140806559507</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.1238050014968019</v>
+        <v>-0.1381702908624401</v>
       </c>
       <c r="I3" t="n">
-        <v>51.15888478333896</v>
+        <v>41.12021857923496</v>
       </c>
       <c r="J3" t="n">
         <v>40</v>
@@ -872,7 +872,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M3" t="n">
@@ -882,10 +882,10 @@
         <v>40</v>
       </c>
       <c r="O3" t="n">
-        <v>31.91489361702128</v>
+        <v>36.17021276595745</v>
       </c>
       <c r="P3" t="n">
-        <v>42.12697872340426</v>
+        <v>42.97804255319149</v>
       </c>
       <c r="Q3" t="b">
         <v>0</v>
@@ -909,25 +909,25 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>32135</v>
+        <v>33445</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.0329521516701775</v>
+        <v>0.058386075949367</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.1108190370780298</v>
+        <v>-0.1461577738064845</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.2095683187799778</v>
+        <v>-0.1521105336544556</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.1053799623006254</v>
+        <v>-0.060411398789853</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.1330925528458018</v>
+        <v>-0.07506760899634241</v>
       </c>
       <c r="I4" t="n">
-        <v>59.54935622317596</v>
+        <v>62.18781218781219</v>
       </c>
       <c r="J4" t="n">
         <v>60</v>
@@ -937,7 +937,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M4" t="n">
@@ -947,10 +947,10 @@
         <v>60</v>
       </c>
       <c r="O4" t="n">
-        <v>27.65957446808511</v>
+        <v>44.68085106382978</v>
       </c>
       <c r="P4" t="n">
-        <v>50.92391489361702</v>
+        <v>54.32817021276595</v>
       </c>
       <c r="Q4" t="b">
         <v>0</v>
@@ -974,25 +974,25 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>299.25</v>
+        <v>297.25</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.06381980290943209</v>
+        <v>-0.0377144707024926</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.17618719889883</v>
+        <v>-0.1907160359379254</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.2920511000709723</v>
+        <v>-0.2848550463130037</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.1878627435916199</v>
+        <v>-0.1931559114484011</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.2155753341367963</v>
+        <v>-0.2078121216548906</v>
       </c>
       <c r="I5" t="n">
-        <v>52.51842751842753</v>
+        <v>41.76217765042979</v>
       </c>
       <c r="J5" t="n">
         <v>40</v>
@@ -1002,7 +1002,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M5" t="n">
@@ -1012,10 +1012,10 @@
         <v>40</v>
       </c>
       <c r="O5" t="n">
-        <v>12.76595744680851</v>
+        <v>10.63829787234042</v>
       </c>
       <c r="P5" t="n">
-        <v>39.0011914893617</v>
+        <v>38.57565957446808</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
@@ -1039,48 +1039,48 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>106.81</v>
+        <v>108.44</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.1545828716162736</v>
+        <v>-0.08086116290896769</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.1282239634345412</v>
+        <v>-0.1097611033576881</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0609913579020562</v>
+        <v>0.0058436137649569</v>
       </c>
       <c r="G6" t="n">
-        <v>0.1651797143814086</v>
+        <v>0.0975427486295594</v>
       </c>
       <c r="H6" t="n">
-        <v>0.1374671238362322</v>
+        <v>0.08288653842307001</v>
       </c>
       <c r="I6" t="n">
-        <v>40.30961595713011</v>
+        <v>34.81794538361508</v>
       </c>
       <c r="J6" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K6" t="n">
         <v>51.57</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M6" t="n">
         <v>51.57</v>
       </c>
       <c r="N6" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O6" t="n">
-        <v>78.72340425531915</v>
+        <v>70.21276595744681</v>
       </c>
       <c r="P6" t="n">
-        <v>52.37268085106383</v>
+        <v>46.67055319148936</v>
       </c>
       <c r="Q6" t="b">
         <v>0</v>
@@ -1104,25 +1104,25 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2567.3</v>
+        <v>2588.2</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.0771415219813795</v>
+        <v>-0.0078202867438472</v>
       </c>
       <c r="E7" t="n">
-        <v>-0.0211979107095199</v>
+        <v>0.0230039525691698</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.2005418366393672</v>
+        <v>-0.2283473957246355</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.0963534801600147</v>
+        <v>-0.136648260860033</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.1240660707051911</v>
+        <v>-0.1513044710665224</v>
       </c>
       <c r="I7" t="n">
-        <v>60.69321533923305</v>
+        <v>52.53784505788068</v>
       </c>
       <c r="J7" t="n">
         <v>80</v>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M7" t="n">
@@ -1169,48 +1169,48 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>496.55</v>
+        <v>515.15</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.0281827967511497</v>
+        <v>0.0288595965648092</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0469112376133249</v>
+        <v>0.0701080182800166</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1286509830662576</v>
+        <v>0.1869815668202763</v>
       </c>
       <c r="G8" t="n">
-        <v>0.2328393395456101</v>
+        <v>0.2786807016848789</v>
       </c>
       <c r="H8" t="n">
-        <v>0.2051267490004337</v>
+        <v>0.2640244914783894</v>
       </c>
       <c r="I8" t="n">
-        <v>52.67369952710077</v>
+        <v>51.25515174222554</v>
       </c>
       <c r="J8" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="K8" t="n">
         <v>49.66</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M8" t="n">
         <v>49.66</v>
       </c>
       <c r="N8" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="O8" t="n">
-        <v>87.2340425531915</v>
+        <v>89.36170212765957</v>
       </c>
       <c r="P8" t="n">
-        <v>53.31080851063831</v>
+        <v>69.73634042553192</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
@@ -1234,25 +1234,25 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>409.45</v>
+        <v>412.85</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.0785416901091482</v>
+        <v>-0.0412215513237342</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.1714892755969242</v>
+        <v>-0.1837682878608145</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.1430514859773964</v>
+        <v>-0.1384599332220366</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.038863129498044</v>
+        <v>-0.046760798357434</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.0665757200432204</v>
+        <v>-0.0614170085639235</v>
       </c>
       <c r="I9" t="n">
-        <v>47.62915782024061</v>
+        <v>44.49760765550241</v>
       </c>
       <c r="J9" t="n">
         <v>40</v>
@@ -1262,7 +1262,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M9" t="n">
@@ -1272,10 +1272,10 @@
         <v>40</v>
       </c>
       <c r="O9" t="n">
-        <v>46.80851063829788</v>
+        <v>48.93617021276596</v>
       </c>
       <c r="P9" t="n">
-        <v>46.73770212765958</v>
+        <v>47.1632340425532</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -1299,25 +1299,25 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>126390</v>
+        <v>127175</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.0985985807509896</v>
+        <v>-0.0574393181397072</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.165935262480615</v>
+        <v>-0.1544496526046341</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.1371518296013107</v>
+        <v>-0.1372116689280869</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.0329634731219583</v>
+        <v>-0.0455125340634843</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.0606760636671347</v>
+        <v>-0.0601687442699737</v>
       </c>
       <c r="I10" t="n">
-        <v>35.28539659006671</v>
+        <v>32.7599486521181</v>
       </c>
       <c r="J10" t="n">
         <v>30</v>
@@ -1327,7 +1327,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M10" t="n">
@@ -1337,10 +1337,10 @@
         <v>30</v>
       </c>
       <c r="O10" t="n">
-        <v>48.93617021276596</v>
+        <v>51.06382978723404</v>
       </c>
       <c r="P10" t="n">
-        <v>41.55123404255319</v>
+        <v>41.97676595744681</v>
       </c>
       <c r="Q10" t="b">
         <v>0</v>
@@ -1376,10 +1376,10 @@
         <v>-0.0042030657656173</v>
       </c>
       <c r="G11" t="n">
-        <v>0.09998529071373501</v>
+        <v>0.0874960690989852</v>
       </c>
       <c r="H11" t="n">
-        <v>0.07227270016855861</v>
+        <v>0.0728398588924957</v>
       </c>
       <c r="I11" t="n">
         <v>27.6054590570719</v>
@@ -1392,7 +1392,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M11" t="n">
@@ -1402,10 +1402,10 @@
         <v>20</v>
       </c>
       <c r="O11" t="n">
-        <v>65.95744680851064</v>
+        <v>63.82978723404256</v>
       </c>
       <c r="P11" t="n">
-        <v>25.19148936170213</v>
+        <v>24.76595744680852</v>
       </c>
       <c r="Q11" t="b">
         <v>0</v>
@@ -1429,25 +1429,25 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>436.5</v>
+        <v>433.15</v>
       </c>
       <c r="D12" t="n">
-        <v>0.1213872832369942</v>
+        <v>0.1395685345961588</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.08739284967593559</v>
+        <v>-0.0898297961756671</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.1526739784528777</v>
+        <v>-0.1839675960813865</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.0484856219735253</v>
+        <v>-0.092268461216784</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.07619821251870169</v>
+        <v>-0.1069246714232734</v>
       </c>
       <c r="I12" t="n">
-        <v>63.01558203483042</v>
+        <v>57.83071464774454</v>
       </c>
       <c r="J12" t="n">
         <v>80</v>
@@ -1457,7 +1457,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M12" t="n">
@@ -1467,10 +1467,10 @@
         <v>80</v>
       </c>
       <c r="O12" t="n">
-        <v>44.68085106382978</v>
+        <v>38.29787234042553</v>
       </c>
       <c r="P12" t="n">
-        <v>69.44817021276596</v>
+        <v>68.17157446808511</v>
       </c>
       <c r="Q12" t="b">
         <v>1</v>
@@ -1494,25 +1494,25 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1659.1</v>
+        <v>1663.7</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.171775159744409</v>
+        <v>-0.1461198932457401</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.118250425170068</v>
+        <v>-0.1674839871897517</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.0412597515169026</v>
+        <v>-0.0475727043737118</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0629286049624497</v>
+        <v>0.0441264304908907</v>
       </c>
       <c r="H13" t="n">
-        <v>0.0352160144172734</v>
+        <v>0.0294702202844012</v>
       </c>
       <c r="I13" t="n">
-        <v>44.29058799919726</v>
+        <v>41.5429646665273</v>
       </c>
       <c r="J13" t="n">
         <v>40</v>
@@ -1522,7 +1522,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M13" t="n">
@@ -1532,10 +1532,10 @@
         <v>40</v>
       </c>
       <c r="O13" t="n">
-        <v>59.57446808510638</v>
+        <v>55.31914893617022</v>
       </c>
       <c r="P13" t="n">
-        <v>51.42289361702128</v>
+        <v>50.57182978723405</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
@@ -1559,25 +1559,25 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>520.9</v>
+        <v>535.7</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.1068244170096023</v>
+        <v>-0.0458633894380621</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.236888368004688</v>
+        <v>-0.243735441519023</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.158549390194653</v>
+        <v>-0.2319162663990249</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.0543610337153006</v>
+        <v>-0.1402171315344224</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.082073624260477</v>
+        <v>-0.1548733417409118</v>
       </c>
       <c r="I14" t="n">
-        <v>40.75808249721292</v>
+        <v>41.4298601714028</v>
       </c>
       <c r="J14" t="n">
         <v>40</v>
@@ -1587,7 +1587,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M14" t="n">
@@ -1597,10 +1597,10 @@
         <v>40</v>
       </c>
       <c r="O14" t="n">
-        <v>42.5531914893617</v>
+        <v>27.65957446808511</v>
       </c>
       <c r="P14" t="n">
-        <v>46.36663829787234</v>
+        <v>43.38791489361702</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
@@ -1624,48 +1624,48 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>90.09999999999999</v>
+        <v>94.84999999999999</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.1202890060535052</v>
+        <v>-0.0145454545454546</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.3856538933587891</v>
+        <v>-0.1670325810134364</v>
       </c>
       <c r="F15" t="n">
-        <v>0.0258453831264944</v>
+        <v>0.0645342312008978</v>
       </c>
       <c r="G15" t="n">
-        <v>0.1300337396058468</v>
+        <v>0.1562333660655004</v>
       </c>
       <c r="H15" t="n">
-        <v>0.1023211490606704</v>
+        <v>0.1415771558590109</v>
       </c>
       <c r="I15" t="n">
-        <v>42.86567164179105</v>
+        <v>41.91198786039452</v>
       </c>
       <c r="J15" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K15" t="n">
         <v>51.91</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M15" t="n">
         <v>51.91</v>
       </c>
       <c r="N15" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O15" t="n">
-        <v>74.46808510638297</v>
+        <v>82.97872340425532</v>
       </c>
       <c r="P15" t="n">
-        <v>51.65761702127659</v>
+        <v>61.35974468085107</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
@@ -1689,48 +1689,48 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>156.33</v>
+        <v>163.02</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.1288866599799397</v>
+        <v>-0.0449352627570448</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.09594031922276181</v>
+        <v>-0.0628880202345366</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.0666308436324556</v>
+        <v>-0.0256992589050919</v>
       </c>
       <c r="G16" t="n">
-        <v>0.0375575128468967</v>
+        <v>0.0659998759595106</v>
       </c>
       <c r="H16" t="n">
-        <v>0.009844922301720399</v>
+        <v>0.0513436657530211</v>
       </c>
       <c r="I16" t="n">
-        <v>47.22298221614229</v>
+        <v>47.6952277657267</v>
       </c>
       <c r="J16" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K16" t="n">
         <v>52.61</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M16" t="n">
         <v>52.61</v>
       </c>
       <c r="N16" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O16" t="n">
-        <v>57.44680851063831</v>
+        <v>59.57446808510638</v>
       </c>
       <c r="P16" t="n">
-        <v>48.53336170212766</v>
+        <v>56.95889361702128</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>
@@ -1754,25 +1754,25 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>6789</v>
+        <v>6744.5</v>
       </c>
       <c r="D17" t="n">
-        <v>-0.1060635986569227</v>
+        <v>-0.0745111492281304</v>
       </c>
       <c r="E17" t="n">
-        <v>-0.1208805438653285</v>
+        <v>-0.1571482129467633</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0016967908520841</v>
+        <v>0.0234446130500758</v>
       </c>
       <c r="G17" t="n">
-        <v>0.1058851473314366</v>
+        <v>0.1151437479146784</v>
       </c>
       <c r="H17" t="n">
-        <v>0.0781725567862602</v>
+        <v>0.1004875377081889</v>
       </c>
       <c r="I17" t="n">
-        <v>49.88155668358714</v>
+        <v>44.77339181286549</v>
       </c>
       <c r="J17" t="n">
         <v>40</v>
@@ -1782,7 +1782,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M17" t="n">
@@ -1792,10 +1792,10 @@
         <v>40</v>
       </c>
       <c r="O17" t="n">
-        <v>70.21276595744681</v>
+        <v>76.59574468085107</v>
       </c>
       <c r="P17" t="n">
-        <v>51.90255319148936</v>
+        <v>53.17914893617021</v>
       </c>
       <c r="Q17" t="b">
         <v>0</v>
@@ -1819,48 +1819,48 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>633.8</v>
+        <v>642.1</v>
       </c>
       <c r="D18" t="n">
-        <v>-0.09747241011035961</v>
+        <v>-0.1204712006026983</v>
       </c>
       <c r="E18" t="n">
-        <v>0.0367220086693382</v>
+        <v>0.0395013760725271</v>
       </c>
       <c r="F18" t="n">
-        <v>-0.0405691795337572</v>
+        <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>0.0636191769455951</v>
+        <v>0.0916991348646025</v>
       </c>
       <c r="H18" t="n">
-        <v>0.0359065864004187</v>
+        <v>0.0770429246581131</v>
       </c>
       <c r="I18" t="n">
-        <v>45.17084732372111</v>
+        <v>39.33547695605573</v>
       </c>
       <c r="J18" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K18" t="n">
         <v>49.92</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M18" t="n">
         <v>49.92</v>
       </c>
       <c r="N18" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O18" t="n">
-        <v>61.70212765957447</v>
+        <v>68.08510638297872</v>
       </c>
       <c r="P18" t="n">
-        <v>48.3084255319149</v>
+        <v>45.58502127659575</v>
       </c>
       <c r="Q18" t="b">
         <v>0</v>
@@ -1884,25 +1884,25 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2251.9</v>
+        <v>2217.6</v>
       </c>
       <c r="D19" t="n">
-        <v>-0.1024711040255081</v>
+        <v>-0.0851485148514852</v>
       </c>
       <c r="E19" t="n">
-        <v>-0.1145407360805284</v>
+        <v>-0.1298069376863915</v>
       </c>
       <c r="F19" t="n">
-        <v>-0.2303038589055609</v>
+        <v>-0.2256172085064776</v>
       </c>
       <c r="G19" t="n">
-        <v>-0.1261155024262085</v>
+        <v>-0.133918073641875</v>
       </c>
       <c r="H19" t="n">
-        <v>-0.1538280929713849</v>
+        <v>-0.1485742838483644</v>
       </c>
       <c r="I19" t="n">
-        <v>37.10482529118138</v>
+        <v>35.75210825652088</v>
       </c>
       <c r="J19" t="n">
         <v>30</v>
@@ -1912,7 +1912,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M19" t="n">
@@ -1922,10 +1922,10 @@
         <v>30</v>
       </c>
       <c r="O19" t="n">
-        <v>23.40425531914894</v>
+        <v>31.91489361702128</v>
       </c>
       <c r="P19" t="n">
-        <v>37.18885106382979</v>
+        <v>38.89097872340426</v>
       </c>
       <c r="Q19" t="b">
         <v>0</v>
@@ -1949,54 +1949,54 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>1985.3</v>
+        <v>2031</v>
       </c>
       <c r="D20" t="n">
-        <v>-0.0730693808945747</v>
+        <v>-0.0044117647058823</v>
       </c>
       <c r="E20" t="n">
-        <v>-0.1090517434815779</v>
+        <v>-0.1354135626410114</v>
       </c>
       <c r="F20" t="n">
-        <v>-0.082408948049547</v>
+        <v>-0.0279040827071268</v>
       </c>
       <c r="G20" t="n">
-        <v>0.0217794084298054</v>
+        <v>0.0637950521574757</v>
       </c>
       <c r="H20" t="n">
-        <v>-0.0059331821153709</v>
+        <v>0.0491388419509862</v>
       </c>
       <c r="I20" t="n">
-        <v>48.45877014551714</v>
+        <v>46.4618401699624</v>
       </c>
       <c r="J20" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K20" t="n">
         <v>49.06</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M20" t="n">
         <v>49.06</v>
       </c>
       <c r="N20" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O20" t="n">
-        <v>53.19148936170212</v>
+        <v>57.44680851063831</v>
       </c>
       <c r="P20" t="n">
-        <v>46.26229787234043</v>
+        <v>55.11336170212766</v>
       </c>
       <c r="Q20" t="b">
         <v>0</v>
       </c>
       <c r="R20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S20" t="b">
         <v>0</v>
@@ -2014,25 +2014,25 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>876.7</v>
+        <v>889.45</v>
       </c>
       <c r="D21" t="n">
-        <v>-0.06719157312337069</v>
+        <v>0.0169210541359401</v>
       </c>
       <c r="E21" t="n">
-        <v>-0.1561266724420059</v>
+        <v>-0.1597865104855468</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.2949738640932851</v>
+        <v>-0.3170684889434889</v>
       </c>
       <c r="G21" t="n">
-        <v>-0.1907855076139326</v>
+        <v>-0.2253693540788863</v>
       </c>
       <c r="H21" t="n">
-        <v>-0.218498098159109</v>
+        <v>-0.2400255642853758</v>
       </c>
       <c r="I21" t="n">
-        <v>57.90378006872851</v>
+        <v>53.37773549000951</v>
       </c>
       <c r="J21" t="n">
         <v>60</v>
@@ -2042,7 +2042,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M21" t="n">
@@ -2052,10 +2052,10 @@
         <v>60</v>
       </c>
       <c r="O21" t="n">
-        <v>10.63829787234042</v>
+        <v>6.382978723404255</v>
       </c>
       <c r="P21" t="n">
-        <v>45.49965957446808</v>
+        <v>44.64859574468085</v>
       </c>
       <c r="Q21" t="b">
         <v>0</v>
@@ -2079,25 +2079,25 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>371.3</v>
+        <v>379.7</v>
       </c>
       <c r="D22" t="n">
-        <v>-0.1298336067494726</v>
+        <v>-0.1177973977695167</v>
       </c>
       <c r="E22" t="n">
-        <v>0.2223868312757202</v>
+        <v>0.1012180974477958</v>
       </c>
       <c r="F22" t="n">
-        <v>0.2027858762552641</v>
+        <v>0.2230632952166209</v>
       </c>
       <c r="G22" t="n">
-        <v>0.3069742327346165</v>
+        <v>0.3147624300812235</v>
       </c>
       <c r="H22" t="n">
-        <v>0.2792616421894401</v>
+        <v>0.300106219874734</v>
       </c>
       <c r="I22" t="n">
-        <v>46.1466749533872</v>
+        <v>44.93295915185531</v>
       </c>
       <c r="J22" t="n">
         <v>40</v>
@@ -2107,7 +2107,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M22" t="n">
@@ -2117,10 +2117,10 @@
         <v>40</v>
       </c>
       <c r="O22" t="n">
-        <v>91.48936170212764</v>
+        <v>93.61702127659576</v>
       </c>
       <c r="P22" t="n">
-        <v>56.08587234042552</v>
+        <v>56.51140425531915</v>
       </c>
       <c r="Q22" t="b">
         <v>0</v>
@@ -2144,48 +2144,48 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>333.55</v>
+        <v>342.35</v>
       </c>
       <c r="D23" t="n">
-        <v>-0.0671234792336735</v>
+        <v>-0.0349541930937279</v>
       </c>
       <c r="E23" t="n">
-        <v>-0.1446339274265931</v>
+        <v>-0.1141156682623882</v>
       </c>
       <c r="F23" t="n">
-        <v>-0.1919815891472868</v>
+        <v>-0.170362292499697</v>
       </c>
       <c r="G23" t="n">
-        <v>-0.0877932326679343</v>
+        <v>-0.07866315763509441</v>
       </c>
       <c r="H23" t="n">
-        <v>-0.1155058232131107</v>
+        <v>-0.0933193678415839</v>
       </c>
       <c r="I23" t="n">
-        <v>46.7296511627907</v>
+        <v>50.82074852265266</v>
       </c>
       <c r="J23" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K23" t="n">
         <v>49.7</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M23" t="n">
         <v>49.7</v>
       </c>
       <c r="N23" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O23" t="n">
-        <v>36.17021276595745</v>
+        <v>40.42553191489361</v>
       </c>
       <c r="P23" t="n">
-        <v>43.1140425531915</v>
+        <v>51.96510638297872</v>
       </c>
       <c r="Q23" t="b">
         <v>0</v>
@@ -2209,25 +2209,25 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>116.04</v>
+        <v>114.82</v>
       </c>
       <c r="D24" t="n">
-        <v>-0.1593131927841773</v>
+        <v>-0.0610075237160615</v>
       </c>
       <c r="E24" t="n">
-        <v>-0.0828327537148275</v>
+        <v>-0.1417893714029449</v>
       </c>
       <c r="F24" t="n">
-        <v>0.07964272422776331</v>
+        <v>0.0566905945150009</v>
       </c>
       <c r="G24" t="n">
-        <v>0.1838310807071157</v>
+        <v>0.1483897293796034</v>
       </c>
       <c r="H24" t="n">
-        <v>0.1561184901619393</v>
+        <v>0.133733519173114</v>
       </c>
       <c r="I24" t="n">
-        <v>47.2378367900756</v>
+        <v>41.09001837109614</v>
       </c>
       <c r="J24" t="n">
         <v>40</v>
@@ -2237,7 +2237,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M24" t="n">
@@ -2247,10 +2247,10 @@
         <v>40</v>
       </c>
       <c r="O24" t="n">
-        <v>82.97872340425532</v>
+        <v>80.85106382978722</v>
       </c>
       <c r="P24" t="n">
-        <v>51.91574468085106</v>
+        <v>51.49021276595744</v>
       </c>
       <c r="Q24" t="b">
         <v>0</v>
@@ -2274,25 +2274,25 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>561.7</v>
+        <v>560.35</v>
       </c>
       <c r="D25" t="n">
-        <v>0.09237650719564371</v>
+        <v>0.1003436426116839</v>
       </c>
       <c r="E25" t="n">
-        <v>-0.1022136977543354</v>
+        <v>-0.139643789344388</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.1025005991851082</v>
+        <v>-0.2394299287410926</v>
       </c>
       <c r="G25" t="n">
-        <v>0.0016877572942441</v>
+        <v>-0.14773079387649</v>
       </c>
       <c r="H25" t="n">
-        <v>-0.0260248332509321</v>
+        <v>-0.1623870040829794</v>
       </c>
       <c r="I25" t="n">
-        <v>61.984126984127</v>
+        <v>44.39853076216713</v>
       </c>
       <c r="J25" t="n">
         <v>80</v>
@@ -2302,7 +2302,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M25" t="n">
@@ -2312,10 +2312,10 @@
         <v>80</v>
       </c>
       <c r="O25" t="n">
-        <v>51.06382978723404</v>
+        <v>25.53191489361702</v>
       </c>
       <c r="P25" t="n">
-        <v>64.9767659574468</v>
+        <v>59.8703829787234</v>
       </c>
       <c r="Q25" t="b">
         <v>0</v>
@@ -2339,25 +2339,25 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>127.14</v>
+        <v>127.49</v>
       </c>
       <c r="D26" t="n">
-        <v>-0.0365992270970675</v>
+        <v>-0.0133880204302739</v>
       </c>
       <c r="E26" t="n">
-        <v>-0.09906462585034009</v>
+        <v>-0.2017406549370735</v>
       </c>
       <c r="F26" t="n">
-        <v>-0.2308064613709237</v>
+        <v>-0.2566614191592327</v>
       </c>
       <c r="G26" t="n">
-        <v>-0.1266181048915713</v>
+        <v>-0.1649622842946301</v>
       </c>
       <c r="H26" t="n">
-        <v>-0.1543306954367477</v>
+        <v>-0.1796184945011195</v>
       </c>
       <c r="I26" t="n">
-        <v>46.12202688728027</v>
+        <v>45.45696775912602</v>
       </c>
       <c r="J26" t="n">
         <v>60</v>
@@ -2367,7 +2367,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M26" t="n">
@@ -2377,10 +2377,10 @@
         <v>60</v>
       </c>
       <c r="O26" t="n">
-        <v>21.27659574468085</v>
+        <v>17.02127659574468</v>
       </c>
       <c r="P26" t="n">
-        <v>48.87131914893617</v>
+        <v>48.02025531914894</v>
       </c>
       <c r="Q26" t="b">
         <v>0</v>
@@ -2404,48 +2404,48 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>4785</v>
+        <v>4800</v>
       </c>
       <c r="D27" t="n">
-        <v>-0.1632421089446533</v>
+        <v>-0.0827441238295433</v>
       </c>
       <c r="E27" t="n">
-        <v>-0.0564921620822241</v>
+        <v>-0.1638359027959237</v>
       </c>
       <c r="F27" t="n">
-        <v>0.1548208036683962</v>
+        <v>0.1446558878237231</v>
       </c>
       <c r="G27" t="n">
-        <v>0.2590091601477486</v>
+        <v>0.2363550226883257</v>
       </c>
       <c r="H27" t="n">
-        <v>0.2312965696025722</v>
+        <v>0.2216988124818363</v>
       </c>
       <c r="I27" t="n">
-        <v>47.14745465184318</v>
+        <v>36.84502049407333</v>
       </c>
       <c r="J27" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K27" t="n">
         <v>57.69</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M27" t="n">
         <v>57.69</v>
       </c>
       <c r="N27" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O27" t="n">
-        <v>89.36170212765957</v>
+        <v>87.2340425531915</v>
       </c>
       <c r="P27" t="n">
-        <v>56.94834042553191</v>
+        <v>52.5228085106383</v>
       </c>
       <c r="Q27" t="b">
         <v>0</v>
@@ -2469,25 +2469,25 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1613.9</v>
+        <v>1634.4</v>
       </c>
       <c r="D28" t="n">
-        <v>0.0700125969634688</v>
+        <v>0.1067921717342723</v>
       </c>
       <c r="E28" t="n">
-        <v>-0.0016701719658541</v>
+        <v>-0.0282996432818073</v>
       </c>
       <c r="F28" t="n">
-        <v>0.5053633056617854</v>
+        <v>0.4808371840173959</v>
       </c>
       <c r="G28" t="n">
-        <v>0.6095516621411379</v>
+        <v>0.5725363188819985</v>
       </c>
       <c r="H28" t="n">
-        <v>0.5818390715959615</v>
+        <v>0.5578801086755091</v>
       </c>
       <c r="I28" t="n">
-        <v>61.51433052901754</v>
+        <v>48.72545642438856</v>
       </c>
       <c r="J28" t="n">
         <v>80</v>
@@ -2497,7 +2497,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M28" t="n">
@@ -2534,25 +2534,25 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>501.4</v>
+        <v>505.2</v>
       </c>
       <c r="D29" t="n">
-        <v>-0.0510078546418094</v>
+        <v>0.0151713051341304</v>
       </c>
       <c r="E29" t="n">
-        <v>-0.1427594460591554</v>
+        <v>-0.1622585191940966</v>
       </c>
       <c r="F29" t="n">
-        <v>-0.0110453648915187</v>
+        <v>-0.0087314823898754</v>
       </c>
       <c r="G29" t="n">
-        <v>0.0931429915878336</v>
+        <v>0.08296765247472709</v>
       </c>
       <c r="H29" t="n">
-        <v>0.06543040104265729</v>
+        <v>0.0683114422682377</v>
       </c>
       <c r="I29" t="n">
-        <v>56.53573728267867</v>
+        <v>49.92997198879552</v>
       </c>
       <c r="J29" t="n">
         <v>40</v>
@@ -2562,7 +2562,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M29" t="n">
@@ -2572,10 +2572,10 @@
         <v>40</v>
       </c>
       <c r="O29" t="n">
-        <v>63.82978723404256</v>
+        <v>61.70212765957447</v>
       </c>
       <c r="P29" t="n">
-        <v>48.53395744680852</v>
+        <v>48.1084255319149</v>
       </c>
       <c r="Q29" t="b">
         <v>0</v>
@@ -2599,48 +2599,48 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>108.6</v>
+        <v>110.21</v>
       </c>
       <c r="D30" t="n">
-        <v>-0.0791928099033407</v>
+        <v>-0.0541537933401991</v>
       </c>
       <c r="E30" t="n">
-        <v>-0.021180712032447</v>
+        <v>-0.0367942667365845</v>
       </c>
       <c r="F30" t="n">
-        <v>-0.1863340076421668</v>
+        <v>-0.1456589147286822</v>
       </c>
       <c r="G30" t="n">
-        <v>-0.0821456511628143</v>
+        <v>-0.0539597798640796</v>
       </c>
       <c r="H30" t="n">
-        <v>-0.1098582417079907</v>
+        <v>-0.068615990070569</v>
       </c>
       <c r="I30" t="n">
-        <v>30.10218171775749</v>
+        <v>29.11852096401451</v>
       </c>
       <c r="J30" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="K30" t="n">
         <v>52.38</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M30" t="n">
         <v>52.38</v>
       </c>
       <c r="N30" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="O30" t="n">
-        <v>38.29787234042553</v>
+        <v>46.80851063829788</v>
       </c>
       <c r="P30" t="n">
-        <v>40.61157446808511</v>
+        <v>38.31370212765957</v>
       </c>
       <c r="Q30" t="b">
         <v>0</v>
@@ -2664,48 +2664,48 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>37.07</v>
+        <v>37.01</v>
       </c>
       <c r="D31" t="n">
-        <v>-0.1080365736284889</v>
+        <v>-0.07751744765702891</v>
       </c>
       <c r="E31" t="n">
-        <v>-0.2422322158626328</v>
+        <v>-0.2889529298751201</v>
       </c>
       <c r="F31" t="n">
-        <v>-0.251111111111111</v>
+        <v>-0.2419090536665301</v>
       </c>
       <c r="G31" t="n">
-        <v>-0.1469227546317586</v>
+        <v>-0.1502099188019275</v>
       </c>
       <c r="H31" t="n">
-        <v>-0.174635345176935</v>
+        <v>-0.164866129008417</v>
       </c>
       <c r="I31" t="n">
-        <v>38.44444444444445</v>
+        <v>40.17660044150109</v>
       </c>
       <c r="J31" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K31" t="n">
         <v>48.99</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M31" t="n">
         <v>48.99</v>
       </c>
       <c r="N31" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O31" t="n">
-        <v>17.02127659574468</v>
+        <v>19.14893617021277</v>
       </c>
       <c r="P31" t="n">
-        <v>35.00025531914894</v>
+        <v>39.42578723404256</v>
       </c>
       <c r="Q31" t="b">
         <v>0</v>
@@ -2729,48 +2729,48 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>659.5</v>
+        <v>667.7</v>
       </c>
       <c r="D32" t="n">
-        <v>-0.0621444823663254</v>
+        <v>-0.0309846890646541</v>
       </c>
       <c r="E32" t="n">
-        <v>-0.1807453416149068</v>
+        <v>-0.1788722867859558</v>
       </c>
       <c r="F32" t="n">
-        <v>-0.3854254030379275</v>
+        <v>-0.4076998137141843</v>
       </c>
       <c r="G32" t="n">
-        <v>-0.281237046558575</v>
+        <v>-0.3160006788495817</v>
       </c>
       <c r="H32" t="n">
-        <v>-0.3089496371037514</v>
+        <v>-0.3306568890560711</v>
       </c>
       <c r="I32" t="n">
-        <v>51.68393782383419</v>
+        <v>42.81333844384822</v>
       </c>
       <c r="J32" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K32" t="n">
         <v>47.86</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M32" t="n">
         <v>47.86</v>
       </c>
       <c r="N32" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O32" t="n">
         <v>2.127659574468085</v>
       </c>
       <c r="P32" t="n">
-        <v>35.56953191489362</v>
+        <v>43.56953191489362</v>
       </c>
       <c r="Q32" t="b">
         <v>0</v>
@@ -2794,48 +2794,48 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>529.85</v>
+        <v>539.1</v>
       </c>
       <c r="D33" t="n">
-        <v>-0.057793189294923</v>
+        <v>-0.0092805292658273</v>
       </c>
       <c r="E33" t="n">
-        <v>-0.1978046934140802</v>
+        <v>-0.2039279385705847</v>
       </c>
       <c r="F33" t="n">
-        <v>0.020315809743886</v>
+        <v>0.0129650507328071</v>
       </c>
       <c r="G33" t="n">
-        <v>0.1245041662232384</v>
+        <v>0.1046641855974097</v>
       </c>
       <c r="H33" t="n">
-        <v>0.096791575678062</v>
+        <v>0.0900079753909203</v>
       </c>
       <c r="I33" t="n">
-        <v>51.41055426485231</v>
+        <v>47.57804090419806</v>
       </c>
       <c r="J33" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K33" t="n">
         <v>49.98</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M33" t="n">
         <v>49.98</v>
       </c>
       <c r="N33" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O33" t="n">
         <v>72.3404255319149</v>
       </c>
       <c r="P33" t="n">
-        <v>50.46008510638298</v>
+        <v>58.46008510638298</v>
       </c>
       <c r="Q33" t="b">
         <v>0</v>
@@ -2871,10 +2871,10 @@
         <v>-0.2401052253975846</v>
       </c>
       <c r="G34" t="n">
-        <v>-0.1359168689182321</v>
+        <v>-0.148406090532982</v>
       </c>
       <c r="H34" t="n">
-        <v>-0.1636294594634085</v>
+        <v>-0.1630623007394714</v>
       </c>
       <c r="I34" t="n">
         <v>63.3225806451613</v>
@@ -2887,7 +2887,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M34" t="n">
@@ -2897,10 +2897,10 @@
         <v>80</v>
       </c>
       <c r="O34" t="n">
-        <v>19.14893617021277</v>
+        <v>21.27659574468085</v>
       </c>
       <c r="P34" t="n">
-        <v>56.18178723404256</v>
+        <v>56.60731914893617</v>
       </c>
       <c r="Q34" t="b">
         <v>0</v>
@@ -2924,25 +2924,25 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>108.75</v>
+        <v>108.18</v>
       </c>
       <c r="D35" t="n">
-        <v>-0.0698768388641806</v>
+        <v>0.02725287247175</v>
       </c>
       <c r="E35" t="n">
-        <v>-0.2122419413256067</v>
+        <v>-0.177338403041825</v>
       </c>
       <c r="F35" t="n">
-        <v>0.0752422384813129</v>
+        <v>0.0179730874188388</v>
       </c>
       <c r="G35" t="n">
-        <v>0.1794305949606653</v>
+        <v>0.1096722222834414</v>
       </c>
       <c r="H35" t="n">
-        <v>0.151718004415489</v>
+        <v>0.0950160120769519</v>
       </c>
       <c r="I35" t="n">
-        <v>53.20623916811091</v>
+        <v>44.05444126074499</v>
       </c>
       <c r="J35" t="n">
         <v>60</v>
@@ -2952,7 +2952,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M35" t="n">
@@ -2962,10 +2962,10 @@
         <v>60</v>
       </c>
       <c r="O35" t="n">
-        <v>80.85106382978722</v>
+        <v>74.46808510638297</v>
       </c>
       <c r="P35" t="n">
-        <v>59.79821276595744</v>
+        <v>58.5216170212766</v>
       </c>
       <c r="Q35" t="b">
         <v>0</v>
@@ -2989,48 +2989,48 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>461.35</v>
+        <v>472.6</v>
       </c>
       <c r="D36" t="n">
-        <v>-0.0825295813860992</v>
+        <v>-0.046600766592697</v>
       </c>
       <c r="E36" t="n">
-        <v>-0.14880073800738</v>
+        <v>-0.1853128770901568</v>
       </c>
       <c r="F36" t="n">
-        <v>-0.0034560967707094</v>
+        <v>0.0264986967854041</v>
       </c>
       <c r="G36" t="n">
-        <v>0.1007322597086429</v>
+        <v>0.1181978316500067</v>
       </c>
       <c r="H36" t="n">
-        <v>0.0730196691634665</v>
+        <v>0.1035416214435173</v>
       </c>
       <c r="I36" t="n">
-        <v>41.07981220657278</v>
+        <v>44.093567251462</v>
       </c>
       <c r="J36" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K36" t="n">
         <v>47.8</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M36" t="n">
         <v>47.8</v>
       </c>
       <c r="N36" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O36" t="n">
-        <v>68.08510638297872</v>
+        <v>78.72340425531915</v>
       </c>
       <c r="P36" t="n">
-        <v>48.73702127659575</v>
+        <v>58.86468085106384</v>
       </c>
       <c r="Q36" t="b">
         <v>0</v>
@@ -3054,25 +3054,25 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2136.6</v>
+        <v>2150.6</v>
       </c>
       <c r="D37" t="n">
-        <v>-0.0434704749966422</v>
+        <v>0.0256581457458984</v>
       </c>
       <c r="E37" t="n">
-        <v>0.2101954120645708</v>
+        <v>0.1125711329539576</v>
       </c>
       <c r="F37" t="n">
-        <v>0.5090048732255101</v>
+        <v>0.5363623374767823</v>
       </c>
       <c r="G37" t="n">
-        <v>0.6131932297048626</v>
+        <v>0.6280614723413849</v>
       </c>
       <c r="H37" t="n">
-        <v>0.5854806391596862</v>
+        <v>0.6134052621348954</v>
       </c>
       <c r="I37" t="n">
-        <v>57.48772504091652</v>
+        <v>45.81015299026424</v>
       </c>
       <c r="J37" t="n">
         <v>80</v>
@@ -3082,7 +3082,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M37" t="n">
@@ -3119,48 +3119,48 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>736.1</v>
+        <v>759.9</v>
       </c>
       <c r="D38" t="n">
-        <v>-0.1294938505203405</v>
+        <v>-0.0653136531365313</v>
       </c>
       <c r="E38" t="n">
-        <v>-0.2180794561291692</v>
+        <v>-0.2206553510076406</v>
       </c>
       <c r="F38" t="n">
-        <v>-0.2971450396257041</v>
+        <v>-0.278621606227454</v>
       </c>
       <c r="G38" t="n">
-        <v>-0.1929566831463517</v>
+        <v>-0.1869224713628514</v>
       </c>
       <c r="H38" t="n">
-        <v>-0.2206692736915281</v>
+        <v>-0.2015786815693409</v>
       </c>
       <c r="I38" t="n">
-        <v>45.77618453865336</v>
+        <v>37.99679201568346</v>
       </c>
       <c r="J38" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K38" t="n">
         <v>49.87</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M38" t="n">
         <v>49.87</v>
       </c>
       <c r="N38" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O38" t="n">
-        <v>8.51063829787234</v>
+        <v>12.76595744680851</v>
       </c>
       <c r="P38" t="n">
-        <v>37.65012765957447</v>
+        <v>34.5011914893617</v>
       </c>
       <c r="Q38" t="b">
         <v>0</v>
@@ -3184,25 +3184,25 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>2928.4</v>
+        <v>2976.4</v>
       </c>
       <c r="D39" t="n">
-        <v>-0.0202415604402957</v>
+        <v>0.0588402703664177</v>
       </c>
       <c r="E39" t="n">
-        <v>-0.0688120071228695</v>
+        <v>-0.1142457518673928</v>
       </c>
       <c r="F39" t="n">
-        <v>0.1211332312404287</v>
+        <v>0.1133388194808109</v>
       </c>
       <c r="G39" t="n">
-        <v>0.2253215877197811</v>
+        <v>0.2050379543454135</v>
       </c>
       <c r="H39" t="n">
-        <v>0.1976089971746047</v>
+        <v>0.190381744138924</v>
       </c>
       <c r="I39" t="n">
-        <v>49.24574729859849</v>
+        <v>45.91883264933881</v>
       </c>
       <c r="J39" t="n">
         <v>40</v>
@@ -3212,7 +3212,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M39" t="n">
@@ -3249,25 +3249,25 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>189.25</v>
+        <v>191.18</v>
       </c>
       <c r="D40" t="n">
-        <v>-0.0437089439110661</v>
+        <v>0.0192461481047077</v>
       </c>
       <c r="E40" t="n">
-        <v>-0.0984231337239769</v>
+        <v>-0.1062596419054742</v>
       </c>
       <c r="F40" t="n">
-        <v>-0.2290300240355236</v>
+        <v>-0.2244533690316822</v>
       </c>
       <c r="G40" t="n">
-        <v>-0.1248416675561712</v>
+        <v>-0.1327542341670796</v>
       </c>
       <c r="H40" t="n">
-        <v>-0.1525542581013476</v>
+        <v>-0.1474104443735691</v>
       </c>
       <c r="I40" t="n">
-        <v>57.81273865892775</v>
+        <v>53.69656328583402</v>
       </c>
       <c r="J40" t="n">
         <v>60</v>
@@ -3277,7 +3277,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M40" t="n">
@@ -3287,10 +3287,10 @@
         <v>60</v>
       </c>
       <c r="O40" t="n">
-        <v>25.53191489361702</v>
+        <v>34.04255319148936</v>
       </c>
       <c r="P40" t="n">
-        <v>47.2823829787234</v>
+        <v>48.98451063829788</v>
       </c>
       <c r="Q40" t="b">
         <v>0</v>
@@ -3314,25 +3314,25 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>749.9</v>
+        <v>750.05</v>
       </c>
       <c r="D41" t="n">
-        <v>-0.120815991558708</v>
+        <v>-0.1012521718291294</v>
       </c>
       <c r="E41" t="n">
-        <v>-0.2074195423558632</v>
+        <v>-0.2012247071352503</v>
       </c>
       <c r="F41" t="n">
-        <v>-0.2589188655005435</v>
+        <v>-0.2591367048597393</v>
       </c>
       <c r="G41" t="n">
-        <v>-0.1547305090211911</v>
+        <v>-0.1674375699951367</v>
       </c>
       <c r="H41" t="n">
-        <v>-0.1824430995663675</v>
+        <v>-0.1820937802016261</v>
       </c>
       <c r="I41" t="n">
-        <v>24.41911442349847</v>
+        <v>23.96411789833407</v>
       </c>
       <c r="J41" t="n">
         <v>20</v>
@@ -3342,7 +3342,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M41" t="n">
@@ -3379,48 +3379,48 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>497.15</v>
+        <v>532.4</v>
       </c>
       <c r="D42" t="n">
-        <v>-0.1336586215910081</v>
+        <v>-0.0398557258791704</v>
       </c>
       <c r="E42" t="n">
-        <v>-0.2803792429615691</v>
+        <v>-0.2330187999711878</v>
       </c>
       <c r="F42" t="n">
-        <v>-0.3509791122715405</v>
+        <v>-0.2996119187002565</v>
       </c>
       <c r="G42" t="n">
-        <v>-0.2467907557921881</v>
+        <v>-0.2079127838356539</v>
       </c>
       <c r="H42" t="n">
-        <v>-0.2745033463373645</v>
+        <v>-0.2225689940421433</v>
       </c>
       <c r="I42" t="n">
-        <v>35.14130745075647</v>
+        <v>46.41249669049509</v>
       </c>
       <c r="J42" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="K42" t="n">
         <v>47.66</v>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M42" t="n">
         <v>47.66</v>
       </c>
       <c r="N42" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="O42" t="n">
-        <v>6.382978723404255</v>
+        <v>8.51063829787234</v>
       </c>
       <c r="P42" t="n">
-        <v>32.34059574468085</v>
+        <v>44.76612765957447</v>
       </c>
       <c r="Q42" t="b">
         <v>0</v>
@@ -3444,25 +3444,25 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>411.55</v>
+        <v>418.2</v>
       </c>
       <c r="D43" t="n">
-        <v>-0.0352789498359118</v>
+        <v>0.0140640155189137</v>
       </c>
       <c r="E43" t="n">
-        <v>-0.1257567711099309</v>
+        <v>-0.1208745007357577</v>
       </c>
       <c r="F43" t="n">
-        <v>-0.078688157600179</v>
+        <v>-0.0631720430107526</v>
       </c>
       <c r="G43" t="n">
-        <v>0.0255001988791734</v>
+        <v>0.0285270918538499</v>
       </c>
       <c r="H43" t="n">
-        <v>-0.0022123916660029</v>
+        <v>0.0138708816473605</v>
       </c>
       <c r="I43" t="n">
-        <v>51.85801442041044</v>
+        <v>56.33059788980072</v>
       </c>
       <c r="J43" t="n">
         <v>60</v>
@@ -3472,7 +3472,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M43" t="n">
@@ -3482,16 +3482,16 @@
         <v>60</v>
       </c>
       <c r="O43" t="n">
-        <v>55.31914893617022</v>
+        <v>53.19148936170212</v>
       </c>
       <c r="P43" t="n">
-        <v>55.65582978723404</v>
+        <v>55.23029787234042</v>
       </c>
       <c r="Q43" t="b">
         <v>0</v>
       </c>
       <c r="R43" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S43" t="b">
         <v>0</v>
@@ -3509,25 +3509,25 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>246.66</v>
+        <v>249.2</v>
       </c>
       <c r="D44" t="n">
-        <v>0.0075980392156862</v>
+        <v>0.017765979170921</v>
       </c>
       <c r="E44" t="n">
-        <v>-0.1025650354738949</v>
+        <v>-0.090178897407813</v>
       </c>
       <c r="F44" t="n">
-        <v>-0.171030078978323</v>
+        <v>-0.1619303850681016</v>
       </c>
       <c r="G44" t="n">
-        <v>-0.0668417224989705</v>
+        <v>-0.070231250203499</v>
       </c>
       <c r="H44" t="n">
-        <v>-0.0945543130441469</v>
+        <v>-0.0848874604099885</v>
       </c>
       <c r="I44" t="n">
-        <v>55.70879193740883</v>
+        <v>52.7207711442786</v>
       </c>
       <c r="J44" t="n">
         <v>60</v>
@@ -3537,7 +3537,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M44" t="n">
@@ -3547,10 +3547,10 @@
         <v>60</v>
       </c>
       <c r="O44" t="n">
-        <v>40.42553191489361</v>
+        <v>42.5531914893617</v>
       </c>
       <c r="P44" t="n">
-        <v>50.96510638297872</v>
+        <v>51.39063829787234</v>
       </c>
       <c r="Q44" t="b">
         <v>0</v>
@@ -3574,25 +3574,25 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>89.8</v>
+        <v>91.27</v>
       </c>
       <c r="D45" t="n">
-        <v>-0.1123850943955718</v>
+        <v>-0.08464547186841841</v>
       </c>
       <c r="E45" t="n">
-        <v>-0.1757687012391006</v>
+        <v>-0.1984015457579484</v>
       </c>
       <c r="F45" t="n">
-        <v>-0.3556257175660161</v>
+        <v>-0.3353480920477716</v>
       </c>
       <c r="G45" t="n">
-        <v>-0.2514373610866637</v>
+        <v>-0.243648957183169</v>
       </c>
       <c r="H45" t="n">
-        <v>-0.2791499516318401</v>
+        <v>-0.2583051673896585</v>
       </c>
       <c r="I45" t="n">
-        <v>39.30916357407933</v>
+        <v>35.08396946564882</v>
       </c>
       <c r="J45" t="n">
         <v>30</v>
@@ -3602,7 +3602,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M45" t="n">
@@ -3639,48 +3639,48 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>490</v>
+        <v>473.15</v>
       </c>
       <c r="D46" t="n">
-        <v>-0.0394981868078015</v>
+        <v>-0.0214064115822131</v>
       </c>
       <c r="E46" t="n">
-        <v>-0.1932164320408331</v>
+        <v>-0.2452544265433083</v>
       </c>
       <c r="F46" t="n">
-        <v>-0.1967871485943774</v>
+        <v>-0.2396143029329048</v>
       </c>
       <c r="G46" t="n">
-        <v>-0.09259879211502491</v>
+        <v>-0.1479151680683023</v>
       </c>
       <c r="H46" t="n">
-        <v>-0.1203113826602013</v>
+        <v>-0.1625713782747917</v>
       </c>
       <c r="I46" t="n">
-        <v>53.46380863622242</v>
+        <v>30.67623724971668</v>
       </c>
       <c r="J46" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="K46" t="n">
         <v>49.61</v>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M46" t="n">
         <v>49.61</v>
       </c>
       <c r="N46" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="O46" t="n">
-        <v>34.04255319148936</v>
+        <v>23.40425531914894</v>
       </c>
       <c r="P46" t="n">
-        <v>50.65251063829788</v>
+        <v>36.52485106382979</v>
       </c>
       <c r="Q46" t="b">
         <v>0</v>
@@ -3704,25 +3704,25 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>974.35</v>
+        <v>960.35</v>
       </c>
       <c r="D47" t="n">
-        <v>0.09798287130944321</v>
+        <v>0.0472737186477645</v>
       </c>
       <c r="E47" t="n">
-        <v>0.126611551136035</v>
+        <v>0.104802991084268</v>
       </c>
       <c r="F47" t="n">
-        <v>0.3098743026147745</v>
+        <v>0.2167110097554796</v>
       </c>
       <c r="G47" t="n">
-        <v>0.414062659094127</v>
+        <v>0.3084101446200822</v>
       </c>
       <c r="H47" t="n">
-        <v>0.3863500685489506</v>
+        <v>0.2937539344135927</v>
       </c>
       <c r="I47" t="n">
-        <v>57.26931330472104</v>
+        <v>48.28730748805098</v>
       </c>
       <c r="J47" t="n">
         <v>60</v>
@@ -3732,7 +3732,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M47" t="n">
@@ -3742,10 +3742,10 @@
         <v>60</v>
       </c>
       <c r="O47" t="n">
-        <v>93.61702127659576</v>
+        <v>91.48936170212764</v>
       </c>
       <c r="P47" t="n">
-        <v>61.45540425531915</v>
+        <v>61.02987234042553</v>
       </c>
       <c r="Q47" t="b">
         <v>0</v>
@@ -3769,48 +3769,48 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>13974</v>
+        <v>13649</v>
       </c>
       <c r="D48" t="n">
-        <v>-0.0247068676716918</v>
+        <v>-0.0253499000285633</v>
       </c>
       <c r="E48" t="n">
-        <v>-0.051259420191459</v>
+        <v>-0.0972286526886698</v>
       </c>
       <c r="F48" t="n">
-        <v>0.0315198937034029</v>
+        <v>-0.0006589544589251</v>
       </c>
       <c r="G48" t="n">
-        <v>0.1357082501827553</v>
+        <v>0.09104018040567741</v>
       </c>
       <c r="H48" t="n">
-        <v>0.1079956596375789</v>
+        <v>0.0763839701991879</v>
       </c>
       <c r="I48" t="n">
-        <v>54.85003190810466</v>
+        <v>48.91404099112878</v>
       </c>
       <c r="J48" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="K48" t="n">
         <v>50.29</v>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M48" t="n">
         <v>50.29</v>
       </c>
       <c r="N48" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="O48" t="n">
-        <v>76.59574468085107</v>
+        <v>65.95744680851064</v>
       </c>
       <c r="P48" t="n">
-        <v>59.43514893617021</v>
+        <v>49.30748936170212</v>
       </c>
       <c r="Q48" t="b">
         <v>0</v>
@@ -3945,25 +3945,25 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1613.9</v>
+        <v>1634.4</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0700125969634688</v>
+        <v>0.1067921717342723</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.0016701719658541</v>
+        <v>-0.0282996432818073</v>
       </c>
       <c r="F2" t="n">
-        <v>0.5053633056617854</v>
+        <v>0.4808371840173959</v>
       </c>
       <c r="G2" t="n">
-        <v>0.6095516621411379</v>
+        <v>0.5725363188819985</v>
       </c>
       <c r="H2" t="n">
-        <v>0.5818390715959615</v>
+        <v>0.5578801086755091</v>
       </c>
       <c r="I2" t="n">
-        <v>61.51433052901754</v>
+        <v>48.72545642438856</v>
       </c>
       <c r="J2" t="n">
         <v>80</v>
@@ -3973,7 +3973,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M2" t="n">
@@ -4010,25 +4010,25 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2136.6</v>
+        <v>2150.6</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.0434704749966422</v>
+        <v>0.0256581457458984</v>
       </c>
       <c r="E3" t="n">
-        <v>0.2101954120645708</v>
+        <v>0.1125711329539576</v>
       </c>
       <c r="F3" t="n">
-        <v>0.5090048732255101</v>
+        <v>0.5363623374767823</v>
       </c>
       <c r="G3" t="n">
-        <v>0.6131932297048626</v>
+        <v>0.6280614723413849</v>
       </c>
       <c r="H3" t="n">
-        <v>0.5854806391596862</v>
+        <v>0.6134052621348954</v>
       </c>
       <c r="I3" t="n">
-        <v>57.48772504091652</v>
+        <v>45.81015299026424</v>
       </c>
       <c r="J3" t="n">
         <v>80</v>
@@ -4038,7 +4038,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M3" t="n">
@@ -4066,63 +4066,63 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ASKAUTOLTD</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>436.5</v>
+        <v>515.15</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1213872832369942</v>
+        <v>0.0288595965648092</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.08739284967593559</v>
+        <v>0.0701080182800166</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.1526739784528777</v>
+        <v>0.1869815668202763</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.0484856219735253</v>
+        <v>0.2786807016848789</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.07619821251870169</v>
+        <v>0.2640244914783894</v>
       </c>
       <c r="I4" t="n">
-        <v>63.01558203483042</v>
+        <v>51.25515174222554</v>
       </c>
       <c r="J4" t="n">
         <v>80</v>
       </c>
       <c r="K4" t="n">
-        <v>71.28</v>
+        <v>49.66</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M4" t="n">
-        <v>71.28</v>
+        <v>49.66</v>
       </c>
       <c r="N4" t="n">
         <v>80</v>
       </c>
       <c r="O4" t="n">
-        <v>44.68085106382978</v>
+        <v>89.36170212765957</v>
       </c>
       <c r="P4" t="n">
-        <v>69.44817021276596</v>
+        <v>69.73634042553192</v>
       </c>
       <c r="Q4" t="b">
+        <v>0</v>
+      </c>
+      <c r="R4" t="b">
         <v>1</v>
-      </c>
-      <c r="R4" t="b">
-        <v>0</v>
       </c>
       <c r="S4" t="b">
         <v>0</v>
@@ -4131,7 +4131,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>JBMA</t>
+          <t>ASKAUTOLTD</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -4140,51 +4140,51 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>561.7</v>
+        <v>433.15</v>
       </c>
       <c r="D5" t="n">
-        <v>0.09237650719564371</v>
+        <v>0.1395685345961588</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.1022136977543354</v>
+        <v>-0.0898297961756671</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.1025005991851082</v>
+        <v>-0.1839675960813865</v>
       </c>
       <c r="G5" t="n">
-        <v>0.0016877572942441</v>
+        <v>-0.092268461216784</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.0260248332509321</v>
+        <v>-0.1069246714232734</v>
       </c>
       <c r="I5" t="n">
-        <v>61.984126984127</v>
+        <v>57.83071464774454</v>
       </c>
       <c r="J5" t="n">
         <v>80</v>
       </c>
       <c r="K5" t="n">
-        <v>56.91</v>
+        <v>71.28</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M5" t="n">
-        <v>56.91</v>
+        <v>71.28</v>
       </c>
       <c r="N5" t="n">
         <v>80</v>
       </c>
       <c r="O5" t="n">
-        <v>51.06382978723404</v>
+        <v>38.29787234042553</v>
       </c>
       <c r="P5" t="n">
-        <v>64.9767659574468</v>
+        <v>68.17157446808511</v>
       </c>
       <c r="Q5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R5" t="b">
         <v>0</v>
@@ -4196,57 +4196,57 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>WHEELS</t>
+          <t>BHARATGEAR</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Wheels</t>
+          <t>Gears</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>974.35</v>
+        <v>94.84999999999999</v>
       </c>
       <c r="D6" t="n">
-        <v>0.09798287130944321</v>
+        <v>-0.0145454545454546</v>
       </c>
       <c r="E6" t="n">
-        <v>0.126611551136035</v>
+        <v>-0.1670325810134364</v>
       </c>
       <c r="F6" t="n">
-        <v>0.3098743026147745</v>
+        <v>0.0645342312008978</v>
       </c>
       <c r="G6" t="n">
-        <v>0.414062659094127</v>
+        <v>0.1562333660655004</v>
       </c>
       <c r="H6" t="n">
-        <v>0.3863500685489506</v>
+        <v>0.1415771558590109</v>
       </c>
       <c r="I6" t="n">
-        <v>57.26931330472104</v>
+        <v>41.91198786039452</v>
       </c>
       <c r="J6" t="n">
         <v>60</v>
       </c>
       <c r="K6" t="n">
-        <v>46.83</v>
+        <v>51.91</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M6" t="n">
-        <v>46.83</v>
+        <v>51.91</v>
       </c>
       <c r="N6" t="n">
         <v>60</v>
       </c>
       <c r="O6" t="n">
-        <v>93.61702127659576</v>
+        <v>82.97872340425532</v>
       </c>
       <c r="P6" t="n">
-        <v>61.45540425531915</v>
+        <v>61.35974468085107</v>
       </c>
       <c r="Q6" t="b">
         <v>0</v>
@@ -4261,57 +4261,57 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>RICOAUTO</t>
+          <t>WHEELS</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Castings</t>
+          <t>Wheels</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>108.75</v>
+        <v>960.35</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.0698768388641806</v>
+        <v>0.0472737186477645</v>
       </c>
       <c r="E7" t="n">
-        <v>-0.2122419413256067</v>
+        <v>0.104802991084268</v>
       </c>
       <c r="F7" t="n">
-        <v>0.0752422384813129</v>
+        <v>0.2167110097554796</v>
       </c>
       <c r="G7" t="n">
-        <v>0.1794305949606653</v>
+        <v>0.3084101446200822</v>
       </c>
       <c r="H7" t="n">
-        <v>0.151718004415489</v>
+        <v>0.2937539344135927</v>
       </c>
       <c r="I7" t="n">
-        <v>53.20623916811091</v>
+        <v>48.28730748805098</v>
       </c>
       <c r="J7" t="n">
         <v>60</v>
       </c>
       <c r="K7" t="n">
-        <v>49.07</v>
+        <v>46.83</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M7" t="n">
-        <v>49.07</v>
+        <v>46.83</v>
       </c>
       <c r="N7" t="n">
         <v>60</v>
       </c>
       <c r="O7" t="n">
-        <v>80.85106382978722</v>
+        <v>91.48936170212764</v>
       </c>
       <c r="P7" t="n">
-        <v>59.79821276595744</v>
+        <v>61.02987234042553</v>
       </c>
       <c r="Q7" t="b">
         <v>0</v>
@@ -4326,63 +4326,63 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ZFCVINDIA</t>
+          <t>JBMA</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Brakes/Transmission</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>13974</v>
+        <v>560.35</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.0247068676716918</v>
+        <v>0.1003436426116839</v>
       </c>
       <c r="E8" t="n">
-        <v>-0.051259420191459</v>
+        <v>-0.139643789344388</v>
       </c>
       <c r="F8" t="n">
-        <v>0.0315198937034029</v>
+        <v>-0.2394299287410926</v>
       </c>
       <c r="G8" t="n">
-        <v>0.1357082501827553</v>
+        <v>-0.14773079387649</v>
       </c>
       <c r="H8" t="n">
-        <v>0.1079956596375789</v>
+        <v>-0.1623870040829794</v>
       </c>
       <c r="I8" t="n">
-        <v>54.85003190810466</v>
+        <v>44.39853076216713</v>
       </c>
       <c r="J8" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K8" t="n">
-        <v>50.29</v>
+        <v>56.91</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M8" t="n">
-        <v>50.29</v>
+        <v>56.91</v>
       </c>
       <c r="N8" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O8" t="n">
-        <v>76.59574468085107</v>
+        <v>25.53191489361702</v>
       </c>
       <c r="P8" t="n">
-        <v>59.43514893617021</v>
+        <v>59.8703829787234</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
       </c>
       <c r="R8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S8" t="b">
         <v>0</v>
@@ -4391,7 +4391,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TIINDIA</t>
+          <t>SANDHAR</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -4400,54 +4400,54 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>2567.3</v>
+        <v>472.6</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.0771415219813795</v>
+        <v>-0.046600766592697</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.0211979107095199</v>
+        <v>-0.1853128770901568</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.2005418366393672</v>
+        <v>0.0264986967854041</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.0963534801600147</v>
+        <v>0.1181978316500067</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.1240660707051911</v>
+        <v>0.1035416214435173</v>
       </c>
       <c r="I9" t="n">
-        <v>60.69321533923305</v>
+        <v>44.093567251462</v>
       </c>
       <c r="J9" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K9" t="n">
-        <v>48.73</v>
+        <v>47.8</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M9" t="n">
-        <v>48.73</v>
+        <v>47.8</v>
       </c>
       <c r="N9" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O9" t="n">
-        <v>29.78723404255319</v>
+        <v>78.72340425531915</v>
       </c>
       <c r="P9" t="n">
-        <v>57.44944680851064</v>
+        <v>58.86468085106384</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
       </c>
       <c r="R9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S9" t="b">
         <v>0</v>
@@ -4456,57 +4456,57 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>RICOAUTO</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Forgings</t>
+          <t>Castings</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1642.6</v>
+        <v>108.18</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.1347450484618627</v>
+        <v>0.02725287247175</v>
       </c>
       <c r="E10" t="n">
-        <v>0.1216880633706636</v>
+        <v>-0.177338403041825</v>
       </c>
       <c r="F10" t="n">
-        <v>0.3553923591055365</v>
+        <v>0.0179730874188388</v>
       </c>
       <c r="G10" t="n">
-        <v>0.459580715584889</v>
+        <v>0.1096722222834414</v>
       </c>
       <c r="H10" t="n">
-        <v>0.4318681250397126</v>
+        <v>0.0950160120769519</v>
       </c>
       <c r="I10" t="n">
-        <v>43.88764044943819</v>
+        <v>44.05444126074499</v>
       </c>
       <c r="J10" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K10" t="n">
-        <v>54.83</v>
+        <v>49.07</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M10" t="n">
-        <v>54.83</v>
+        <v>49.07</v>
       </c>
       <c r="N10" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O10" t="n">
-        <v>95.74468085106383</v>
+        <v>74.46808510638297</v>
       </c>
       <c r="P10" t="n">
-        <v>57.08093617021277</v>
+        <v>58.5216170212766</v>
       </c>
       <c r="Q10" t="b">
         <v>0</v>
@@ -4521,57 +4521,57 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>LUMAXIND</t>
+          <t>PRICOLLTD</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Lighting</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>4785</v>
+        <v>539.1</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.1632421089446533</v>
+        <v>-0.0092805292658273</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.0564921620822241</v>
+        <v>-0.2039279385705847</v>
       </c>
       <c r="F11" t="n">
-        <v>0.1548208036683962</v>
+        <v>0.0129650507328071</v>
       </c>
       <c r="G11" t="n">
-        <v>0.2590091601477486</v>
+        <v>0.1046641855974097</v>
       </c>
       <c r="H11" t="n">
-        <v>0.2312965696025722</v>
+        <v>0.0900079753909203</v>
       </c>
       <c r="I11" t="n">
-        <v>47.14745465184318</v>
+        <v>47.57804090419806</v>
       </c>
       <c r="J11" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K11" t="n">
-        <v>57.69</v>
+        <v>49.98</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M11" t="n">
-        <v>57.69</v>
+        <v>49.98</v>
       </c>
       <c r="N11" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O11" t="n">
-        <v>89.36170212765957</v>
+        <v>72.3404255319149</v>
       </c>
       <c r="P11" t="n">
-        <v>56.94834042553191</v>
+        <v>58.46008510638298</v>
       </c>
       <c r="Q11" t="b">
         <v>0</v>
@@ -4586,57 +4586,57 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>RANEENGINE</t>
+          <t>TIINDIA</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Engine/Parts</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>317.75</v>
+        <v>2588.2</v>
       </c>
       <c r="D12" t="n">
-        <v>0.1790352504638219</v>
+        <v>-0.0078202867438472</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.156154561147258</v>
+        <v>0.0230039525691698</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.2401052253975846</v>
+        <v>-0.2283473957246355</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.1359168689182321</v>
+        <v>-0.136648260860033</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.1636294594634085</v>
+        <v>-0.1513044710665224</v>
       </c>
       <c r="I12" t="n">
-        <v>63.3225806451613</v>
+        <v>52.53784505788068</v>
       </c>
       <c r="J12" t="n">
         <v>80</v>
       </c>
       <c r="K12" t="n">
-        <v>50.88</v>
+        <v>48.73</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M12" t="n">
-        <v>50.88</v>
+        <v>48.73</v>
       </c>
       <c r="N12" t="n">
         <v>80</v>
       </c>
       <c r="O12" t="n">
-        <v>19.14893617021277</v>
+        <v>29.78723404255319</v>
       </c>
       <c r="P12" t="n">
-        <v>56.18178723404256</v>
+        <v>57.44944680851064</v>
       </c>
       <c r="Q12" t="b">
         <v>0</v>
@@ -4651,57 +4651,57 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>GNA</t>
+          <t>BHARATSE</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Axles</t>
+          <t>Seating</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>371.3</v>
+        <v>163.02</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.1298336067494726</v>
+        <v>-0.0449352627570448</v>
       </c>
       <c r="E13" t="n">
-        <v>0.2223868312757202</v>
+        <v>-0.0628880202345366</v>
       </c>
       <c r="F13" t="n">
-        <v>0.2027858762552641</v>
+        <v>-0.0256992589050919</v>
       </c>
       <c r="G13" t="n">
-        <v>0.3069742327346165</v>
+        <v>0.0659998759595106</v>
       </c>
       <c r="H13" t="n">
-        <v>0.2792616421894401</v>
+        <v>0.0513436657530211</v>
       </c>
       <c r="I13" t="n">
-        <v>46.1466749533872</v>
+        <v>47.6952277657267</v>
       </c>
       <c r="J13" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K13" t="n">
-        <v>54.47</v>
+        <v>52.61</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M13" t="n">
-        <v>54.47</v>
+        <v>52.61</v>
       </c>
       <c r="N13" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O13" t="n">
-        <v>91.48936170212764</v>
+        <v>59.57446808510638</v>
       </c>
       <c r="P13" t="n">
-        <v>56.08587234042552</v>
+        <v>56.95889361702128</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
@@ -4716,57 +4716,57 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SUPRAJIT</t>
+          <t>RANEENGINE</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Cables</t>
+          <t>Engine/Parts</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>411.55</v>
+        <v>317.75</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.0352789498359118</v>
+        <v>0.1790352504638219</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.1257567711099309</v>
+        <v>-0.156154561147258</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.078688157600179</v>
+        <v>-0.2401052253975846</v>
       </c>
       <c r="G14" t="n">
-        <v>0.0255001988791734</v>
+        <v>-0.148406090532982</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.0022123916660029</v>
+        <v>-0.1630623007394714</v>
       </c>
       <c r="I14" t="n">
-        <v>51.85801442041044</v>
+        <v>63.3225806451613</v>
       </c>
       <c r="J14" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K14" t="n">
-        <v>51.48</v>
+        <v>50.88</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M14" t="n">
-        <v>51.48</v>
+        <v>50.88</v>
       </c>
       <c r="N14" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O14" t="n">
-        <v>55.31914893617022</v>
+        <v>21.27659574468085</v>
       </c>
       <c r="P14" t="n">
-        <v>55.65582978723404</v>
+        <v>56.60731914893617</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
@@ -4781,57 +4781,57 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>GNA</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Axles</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>496.55</v>
+        <v>379.7</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.0281827967511497</v>
+        <v>-0.1177973977695167</v>
       </c>
       <c r="E15" t="n">
-        <v>0.0469112376133249</v>
+        <v>0.1012180974477958</v>
       </c>
       <c r="F15" t="n">
-        <v>0.1286509830662576</v>
+        <v>0.2230632952166209</v>
       </c>
       <c r="G15" t="n">
-        <v>0.2328393395456101</v>
+        <v>0.3147624300812235</v>
       </c>
       <c r="H15" t="n">
-        <v>0.2051267490004337</v>
+        <v>0.300106219874734</v>
       </c>
       <c r="I15" t="n">
-        <v>52.67369952710077</v>
+        <v>44.93295915185531</v>
       </c>
       <c r="J15" t="n">
         <v>40</v>
       </c>
       <c r="K15" t="n">
-        <v>49.66</v>
+        <v>54.47</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M15" t="n">
-        <v>49.66</v>
+        <v>54.47</v>
       </c>
       <c r="N15" t="n">
         <v>40</v>
       </c>
       <c r="O15" t="n">
-        <v>87.2340425531915</v>
+        <v>93.61702127659576</v>
       </c>
       <c r="P15" t="n">
-        <v>53.31080851063831</v>
+        <v>56.51140425531915</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
@@ -4846,57 +4846,57 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>SHRIPISTON</t>
+          <t>SUPRAJIT</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Engine/Parts</t>
+          <t>Cables</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2928.4</v>
+        <v>418.2</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.0202415604402957</v>
+        <v>0.0140640155189137</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.0688120071228695</v>
+        <v>-0.1208745007357577</v>
       </c>
       <c r="F16" t="n">
-        <v>0.1211332312404287</v>
+        <v>-0.0631720430107526</v>
       </c>
       <c r="G16" t="n">
-        <v>0.2253215877197811</v>
+        <v>0.0285270918538499</v>
       </c>
       <c r="H16" t="n">
-        <v>0.1976089971746047</v>
+        <v>0.0138708816473605</v>
       </c>
       <c r="I16" t="n">
-        <v>49.24574729859849</v>
+        <v>56.33059788980072</v>
       </c>
       <c r="J16" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K16" t="n">
-        <v>48.69</v>
+        <v>51.48</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="M16" t="n">
-        <v>48.69</v>
+        <v>51.48</v>
       </c>
       <c r="N16" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O16" t="n">
-        <v>85.1063829787234</v>
+        <v>53.19148936170212</v>
       </c>
       <c r="P16" t="n">
-        <v>52.49727659574468</v>
+        <v>55.23029787234042</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
chore: auto-refresh NSE data and pipeline outputs (2026-04-08)
</commit_message>
<xml_diff>
--- a/working-sector/output/auto_components_comprehensive_report.xlsx
+++ b/working-sector/output/auto_components_comprehensive_report.xlsx
@@ -435,7 +435,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
     </row>
@@ -447,7 +447,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
     </row>
@@ -779,48 +779,48 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1671.3</v>
+        <v>1781.4</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.1025613488696772</v>
+        <v>-0.0330040169362718</v>
       </c>
       <c r="E2" t="n">
-        <v>0.127504553734062</v>
+        <v>0.2079745032888045</v>
       </c>
       <c r="F2" t="n">
-        <v>0.3508729388942773</v>
+        <v>0.4102279924002534</v>
       </c>
       <c r="G2" t="n">
-        <v>0.4425720737588798</v>
+        <v>0.4379533709367348</v>
       </c>
       <c r="H2" t="n">
-        <v>0.4279158635523904</v>
+        <v>0.4520218991598677</v>
       </c>
       <c r="I2" t="n">
-        <v>31.83183183183183</v>
+        <v>58.97502601456814</v>
       </c>
       <c r="J2" t="n">
-        <v>30</v>
+        <v>80</v>
       </c>
       <c r="K2" t="n">
         <v>54.83</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M2" t="n">
         <v>54.83</v>
       </c>
       <c r="N2" t="n">
-        <v>30</v>
+        <v>80</v>
       </c>
       <c r="O2" t="n">
         <v>95.74468085106383</v>
       </c>
       <c r="P2" t="n">
-        <v>53.08093617021277</v>
+        <v>73.08093617021277</v>
       </c>
       <c r="Q2" t="b">
         <v>0</v>
@@ -844,48 +844,48 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1021.4</v>
+        <v>1090.2</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.056094630810461</v>
+        <v>-0.0218034993270525</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.2358222355229686</v>
+        <v>-0.1746536452418805</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.2152132155205532</v>
+        <v>-0.1747785935962454</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.1235140806559507</v>
+        <v>-0.1470532150597641</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.1381702908624401</v>
+        <v>-0.1329846868366312</v>
       </c>
       <c r="I3" t="n">
-        <v>41.12021857923496</v>
+        <v>57.73573390296002</v>
       </c>
       <c r="J3" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K3" t="n">
         <v>49.36</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M3" t="n">
         <v>49.36</v>
       </c>
       <c r="N3" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O3" t="n">
         <v>36.17021276595745</v>
       </c>
       <c r="P3" t="n">
-        <v>42.97804255319149</v>
+        <v>50.97804255319149</v>
       </c>
       <c r="Q3" t="b">
         <v>0</v>
@@ -909,48 +909,48 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>33445</v>
+        <v>35935</v>
       </c>
       <c r="D4" t="n">
-        <v>0.058386075949367</v>
+        <v>0.1201683291770574</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.1461577738064845</v>
+        <v>-0.0776437371663244</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.1521105336544556</v>
+        <v>-0.0998246492985972</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.060411398789853</v>
+        <v>-0.07209927076211579</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.07506760899634241</v>
+        <v>-0.0580307425389829</v>
       </c>
       <c r="I4" t="n">
-        <v>62.18781218781219</v>
+        <v>74.93551160791057</v>
       </c>
       <c r="J4" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K4" t="n">
         <v>53.48</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M4" t="n">
         <v>53.48</v>
       </c>
       <c r="N4" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O4" t="n">
-        <v>44.68085106382978</v>
+        <v>51.06382978723404</v>
       </c>
       <c r="P4" t="n">
-        <v>54.32817021276595</v>
+        <v>59.6047659574468</v>
       </c>
       <c r="Q4" t="b">
         <v>0</v>
@@ -974,48 +974,48 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>297.25</v>
+        <v>314.15</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.0377144707024926</v>
+        <v>-0.0091468222677811</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.1907160359379254</v>
+        <v>-0.1364760857614074</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.2848550463130037</v>
+        <v>-0.248804399808704</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.1931559114484011</v>
+        <v>-0.2210790212722226</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.2078121216548906</v>
+        <v>-0.2070104930490898</v>
       </c>
       <c r="I5" t="n">
-        <v>41.76217765042979</v>
+        <v>57.70676691729321</v>
       </c>
       <c r="J5" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K5" t="n">
         <v>51.12</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M5" t="n">
         <v>51.12</v>
       </c>
       <c r="N5" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O5" t="n">
-        <v>10.63829787234042</v>
+        <v>14.8936170212766</v>
       </c>
       <c r="P5" t="n">
-        <v>38.57565957446808</v>
+        <v>47.42672340425532</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
@@ -1039,48 +1039,48 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>108.44</v>
+        <v>118.11</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.08086116290896769</v>
+        <v>-0.042946276638846</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.1097611033576881</v>
+        <v>-0.0225109658197467</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0058436137649569</v>
+        <v>0.07480207480207469</v>
       </c>
       <c r="G6" t="n">
-        <v>0.0975427486295594</v>
+        <v>0.1025274533385561</v>
       </c>
       <c r="H6" t="n">
-        <v>0.08288653842307001</v>
+        <v>0.116595981561689</v>
       </c>
       <c r="I6" t="n">
-        <v>34.81794538361508</v>
+        <v>59.24418604651163</v>
       </c>
       <c r="J6" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="K6" t="n">
         <v>51.57</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M6" t="n">
         <v>51.57</v>
       </c>
       <c r="N6" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="O6" t="n">
         <v>70.21276595744681</v>
       </c>
       <c r="P6" t="n">
-        <v>46.67055319148936</v>
+        <v>58.67055319148936</v>
       </c>
       <c r="Q6" t="b">
         <v>0</v>
@@ -1104,25 +1104,25 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2588.2</v>
+        <v>2727.1</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.0078202867438472</v>
+        <v>0.0313906433190878</v>
       </c>
       <c r="E7" t="n">
-        <v>0.0230039525691698</v>
+        <v>0.06987053746567271</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.2283473957246355</v>
+        <v>-0.1989484196921631</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.136648260860033</v>
+        <v>-0.1712230411556817</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.1513044710665224</v>
+        <v>-0.1571545129325489</v>
       </c>
       <c r="I7" t="n">
-        <v>52.53784505788068</v>
+        <v>64.69360369762936</v>
       </c>
       <c r="J7" t="n">
         <v>80</v>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M7" t="n">
@@ -1142,10 +1142,10 @@
         <v>80</v>
       </c>
       <c r="O7" t="n">
-        <v>29.78723404255319</v>
+        <v>25.53191489361702</v>
       </c>
       <c r="P7" t="n">
-        <v>57.44944680851064</v>
+        <v>56.59838297872341</v>
       </c>
       <c r="Q7" t="b">
         <v>0</v>
@@ -1169,25 +1169,25 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>515.15</v>
+        <v>533.7</v>
       </c>
       <c r="D8" t="n">
-        <v>0.0288595965648092</v>
+        <v>0.0428920371275036</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0701080182800166</v>
+        <v>0.1201595130653794</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1869815668202763</v>
+        <v>0.2338457981736217</v>
       </c>
       <c r="G8" t="n">
-        <v>0.2786807016848789</v>
+        <v>0.2615711767101031</v>
       </c>
       <c r="H8" t="n">
-        <v>0.2640244914783894</v>
+        <v>0.275639704933236</v>
       </c>
       <c r="I8" t="n">
-        <v>51.25515174222554</v>
+        <v>62.59899208063357</v>
       </c>
       <c r="J8" t="n">
         <v>80</v>
@@ -1197,7 +1197,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M8" t="n">
@@ -1207,10 +1207,10 @@
         <v>80</v>
       </c>
       <c r="O8" t="n">
-        <v>89.36170212765957</v>
+        <v>87.2340425531915</v>
       </c>
       <c r="P8" t="n">
-        <v>69.73634042553192</v>
+        <v>69.31080851063831</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
@@ -1234,48 +1234,48 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>412.85</v>
+        <v>436.1</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.0412215513237342</v>
+        <v>-0.003883051621745</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.1837682878608145</v>
+        <v>-0.1605389797882579</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.1384599332220366</v>
+        <v>-0.1031362467866323</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.046760798357434</v>
+        <v>-0.07541086825015091</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.0614170085639235</v>
+        <v>-0.0613423400270181</v>
       </c>
       <c r="I9" t="n">
-        <v>44.49760765550241</v>
+        <v>59.7197898423818</v>
       </c>
       <c r="J9" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K9" t="n">
         <v>53.44</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M9" t="n">
         <v>53.44</v>
       </c>
       <c r="N9" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O9" t="n">
         <v>48.93617021276596</v>
       </c>
       <c r="P9" t="n">
-        <v>47.1632340425532</v>
+        <v>55.1632340425532</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -1299,48 +1299,48 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>127175</v>
+        <v>133050</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.0574393181397072</v>
+        <v>-0.0308482354226609</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.1544496526046341</v>
+        <v>-0.1141516029162089</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.1372116689280869</v>
+        <v>-0.1182318245079196</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.0455125340634843</v>
+        <v>-0.0905064459714383</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.0601687442699737</v>
+        <v>-0.0764379177483054</v>
       </c>
       <c r="I10" t="n">
-        <v>32.7599486521181</v>
+        <v>55.69188820722564</v>
       </c>
       <c r="J10" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="K10" t="n">
         <v>49.41</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M10" t="n">
         <v>49.41</v>
       </c>
       <c r="N10" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="O10" t="n">
-        <v>51.06382978723404</v>
+        <v>46.80851063829788</v>
       </c>
       <c r="P10" t="n">
-        <v>41.97676595744681</v>
+        <v>53.12570212765957</v>
       </c>
       <c r="Q10" t="b">
         <v>0</v>
@@ -1376,10 +1376,10 @@
         <v>-0.0042030657656173</v>
       </c>
       <c r="G11" t="n">
-        <v>0.0874960690989852</v>
+        <v>0.023522312770864</v>
       </c>
       <c r="H11" t="n">
-        <v>0.0728398588924957</v>
+        <v>0.0375908409939969</v>
       </c>
       <c r="I11" t="n">
         <v>27.6054590570719</v>
@@ -1392,7 +1392,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M11" t="n">
@@ -1402,10 +1402,10 @@
         <v>20</v>
       </c>
       <c r="O11" t="n">
-        <v>63.82978723404256</v>
+        <v>57.44680851063831</v>
       </c>
       <c r="P11" t="n">
-        <v>24.76595744680852</v>
+        <v>23.48936170212766</v>
       </c>
       <c r="Q11" t="b">
         <v>0</v>
@@ -1429,25 +1429,25 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>433.15</v>
+        <v>440.5</v>
       </c>
       <c r="D12" t="n">
-        <v>0.1395685345961588</v>
+        <v>0.1185881157948196</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.0898297961756671</v>
+        <v>-0.0717521862817406</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.1839675960813865</v>
+        <v>-0.1760194537972316</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.092268461216784</v>
+        <v>-0.1482940752607502</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.1069246714232734</v>
+        <v>-0.1342255470376173</v>
       </c>
       <c r="I12" t="n">
-        <v>57.83071464774454</v>
+        <v>60.43747028055159</v>
       </c>
       <c r="J12" t="n">
         <v>80</v>
@@ -1457,7 +1457,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M12" t="n">
@@ -1467,10 +1467,10 @@
         <v>80</v>
       </c>
       <c r="O12" t="n">
-        <v>38.29787234042553</v>
+        <v>34.04255319148936</v>
       </c>
       <c r="P12" t="n">
-        <v>68.17157446808511</v>
+        <v>67.32051063829788</v>
       </c>
       <c r="Q12" t="b">
         <v>1</v>
@@ -1494,48 +1494,48 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1663.7</v>
+        <v>1713.1</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.1461198932457401</v>
+        <v>-0.1118311903774368</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.1674839871897517</v>
+        <v>-0.1335727291118754</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.0475727043737118</v>
+        <v>-0.0373138522056758</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0441264304908907</v>
+        <v>-0.0095884736691944</v>
       </c>
       <c r="H13" t="n">
-        <v>0.0294702202844012</v>
+        <v>0.0044800545539384</v>
       </c>
       <c r="I13" t="n">
-        <v>41.5429646665273</v>
+        <v>55.34240463975014</v>
       </c>
       <c r="J13" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K13" t="n">
         <v>58.77</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M13" t="n">
         <v>58.77</v>
       </c>
       <c r="N13" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O13" t="n">
         <v>55.31914893617022</v>
       </c>
       <c r="P13" t="n">
-        <v>50.57182978723405</v>
+        <v>58.57182978723405</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
@@ -1559,48 +1559,48 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>535.7</v>
+        <v>573.9</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.0458633894380621</v>
+        <v>0.0045510239803956</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.243735441519023</v>
+        <v>-0.1780292179891149</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.2319162663990249</v>
+        <v>-0.168682552328529</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.1402171315344224</v>
+        <v>-0.1409571737920476</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.1548733417409118</v>
+        <v>-0.1268886455689147</v>
       </c>
       <c r="I14" t="n">
-        <v>41.4298601714028</v>
+        <v>54.97780596068484</v>
       </c>
       <c r="J14" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K14" t="n">
         <v>54.64</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M14" t="n">
         <v>54.64</v>
       </c>
       <c r="N14" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O14" t="n">
-        <v>27.65957446808511</v>
+        <v>38.29787234042553</v>
       </c>
       <c r="P14" t="n">
-        <v>43.38791489361702</v>
+        <v>53.51557446808511</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
@@ -1624,25 +1624,25 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>94.84999999999999</v>
+        <v>98.94</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.0145454545454546</v>
+        <v>-0.0330336200156371</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.1670325810134364</v>
+        <v>-0.1055058312991592</v>
       </c>
       <c r="F15" t="n">
-        <v>0.0645342312008978</v>
+        <v>0.1005561735261399</v>
       </c>
       <c r="G15" t="n">
-        <v>0.1562333660655004</v>
+        <v>0.1282815520626213</v>
       </c>
       <c r="H15" t="n">
-        <v>0.1415771558590109</v>
+        <v>0.1423500802857542</v>
       </c>
       <c r="I15" t="n">
-        <v>41.91198786039452</v>
+        <v>53.67316341829085</v>
       </c>
       <c r="J15" t="n">
         <v>60</v>
@@ -1652,7 +1652,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M15" t="n">
@@ -1662,10 +1662,10 @@
         <v>60</v>
       </c>
       <c r="O15" t="n">
-        <v>82.97872340425532</v>
+        <v>78.72340425531915</v>
       </c>
       <c r="P15" t="n">
-        <v>61.35974468085107</v>
+        <v>60.50868085106383</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
@@ -1689,48 +1689,48 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>163.02</v>
+        <v>176.72</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.0449352627570448</v>
+        <v>0.004775983625199</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.0628880202345366</v>
+        <v>0.0193228355540173</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.0256992589050919</v>
+        <v>0.1117961623151935</v>
       </c>
       <c r="G16" t="n">
-        <v>0.0659998759595106</v>
+        <v>0.1395215408516749</v>
       </c>
       <c r="H16" t="n">
-        <v>0.0513436657530211</v>
+        <v>0.1535900690748077</v>
       </c>
       <c r="I16" t="n">
-        <v>47.6952277657267</v>
+        <v>63.04656262092092</v>
       </c>
       <c r="J16" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K16" t="n">
         <v>52.61</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M16" t="n">
         <v>52.61</v>
       </c>
       <c r="N16" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O16" t="n">
-        <v>59.57446808510638</v>
+        <v>80.85106382978722</v>
       </c>
       <c r="P16" t="n">
-        <v>56.95889361702128</v>
+        <v>69.21421276595744</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>
@@ -1754,48 +1754,48 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>6744.5</v>
+        <v>7351.5</v>
       </c>
       <c r="D17" t="n">
-        <v>-0.0745111492281304</v>
+        <v>-0.009365314647621499</v>
       </c>
       <c r="E17" t="n">
-        <v>-0.1571482129467633</v>
+        <v>-0.0835255251511563</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0234446130500758</v>
+        <v>0.0893531895976884</v>
       </c>
       <c r="G17" t="n">
-        <v>0.1151437479146784</v>
+        <v>0.1170785681341698</v>
       </c>
       <c r="H17" t="n">
-        <v>0.1004875377081889</v>
+        <v>0.1311470963573027</v>
       </c>
       <c r="I17" t="n">
-        <v>44.77339181286549</v>
+        <v>62.77992277992279</v>
       </c>
       <c r="J17" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K17" t="n">
         <v>54.65</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M17" t="n">
         <v>54.65</v>
       </c>
       <c r="N17" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O17" t="n">
         <v>76.59574468085107</v>
       </c>
       <c r="P17" t="n">
-        <v>53.17914893617021</v>
+        <v>61.17914893617021</v>
       </c>
       <c r="Q17" t="b">
         <v>0</v>
@@ -1819,48 +1819,48 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>642.1</v>
+        <v>673.25</v>
       </c>
       <c r="D18" t="n">
-        <v>-0.1204712006026983</v>
+        <v>-0.0998729861621766</v>
       </c>
       <c r="E18" t="n">
-        <v>0.0395013760725271</v>
+        <v>0.0887846688768496</v>
       </c>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>0.0214686693976633</v>
       </c>
       <c r="G18" t="n">
-        <v>0.0916991348646025</v>
+        <v>0.0491940479341447</v>
       </c>
       <c r="H18" t="n">
-        <v>0.0770429246581131</v>
+        <v>0.06326257615727759</v>
       </c>
       <c r="I18" t="n">
-        <v>39.33547695605573</v>
+        <v>48.40488381252461</v>
       </c>
       <c r="J18" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="K18" t="n">
         <v>49.92</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M18" t="n">
         <v>49.92</v>
       </c>
       <c r="N18" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="O18" t="n">
-        <v>68.08510638297872</v>
+        <v>59.57446808510638</v>
       </c>
       <c r="P18" t="n">
-        <v>45.58502127659575</v>
+        <v>55.88289361702128</v>
       </c>
       <c r="Q18" t="b">
         <v>0</v>
@@ -1884,48 +1884,48 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2217.6</v>
+        <v>2359.1</v>
       </c>
       <c r="D19" t="n">
-        <v>-0.0851485148514852</v>
+        <v>-0.0458645096056623</v>
       </c>
       <c r="E19" t="n">
-        <v>-0.1298069376863915</v>
+        <v>-0.0818836349484335</v>
       </c>
       <c r="F19" t="n">
-        <v>-0.2256172085064776</v>
+        <v>-0.1926972828690711</v>
       </c>
       <c r="G19" t="n">
-        <v>-0.133918073641875</v>
+        <v>-0.1649719043325898</v>
       </c>
       <c r="H19" t="n">
-        <v>-0.1485742838483644</v>
+        <v>-0.1509033761094569</v>
       </c>
       <c r="I19" t="n">
-        <v>35.75210825652088</v>
+        <v>57.36049601417182</v>
       </c>
       <c r="J19" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="K19" t="n">
         <v>51.27</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M19" t="n">
         <v>51.27</v>
       </c>
       <c r="N19" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="O19" t="n">
-        <v>31.91489361702128</v>
+        <v>27.65957446808511</v>
       </c>
       <c r="P19" t="n">
-        <v>38.89097872340426</v>
+        <v>50.03991489361702</v>
       </c>
       <c r="Q19" t="b">
         <v>0</v>
@@ -1949,48 +1949,48 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2031</v>
+        <v>2161.3</v>
       </c>
       <c r="D20" t="n">
-        <v>-0.0044117647058823</v>
+        <v>0.0100004673115565</v>
       </c>
       <c r="E20" t="n">
-        <v>-0.1354135626410114</v>
+        <v>-0.0674404556437693</v>
       </c>
       <c r="F20" t="n">
-        <v>-0.0279040827071268</v>
+        <v>0.0299752192146398</v>
       </c>
       <c r="G20" t="n">
-        <v>0.0637950521574757</v>
+        <v>0.0577005977511212</v>
       </c>
       <c r="H20" t="n">
-        <v>0.0491388419509862</v>
+        <v>0.0717691259742541</v>
       </c>
       <c r="I20" t="n">
-        <v>46.4618401699624</v>
+        <v>61.93606214520467</v>
       </c>
       <c r="J20" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K20" t="n">
         <v>49.06</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M20" t="n">
         <v>49.06</v>
       </c>
       <c r="N20" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O20" t="n">
-        <v>57.44680851063831</v>
+        <v>63.82978723404256</v>
       </c>
       <c r="P20" t="n">
-        <v>55.11336170212766</v>
+        <v>64.38995744680851</v>
       </c>
       <c r="Q20" t="b">
         <v>0</v>
@@ -2014,48 +2014,48 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>889.45</v>
+        <v>918.95</v>
       </c>
       <c r="D21" t="n">
-        <v>0.0169210541359401</v>
+        <v>0.0211690187798645</v>
       </c>
       <c r="E21" t="n">
-        <v>-0.1597865104855468</v>
+        <v>-0.1203694840624102</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.3170684889434889</v>
+        <v>-0.3023458852110537</v>
       </c>
       <c r="G21" t="n">
-        <v>-0.2253693540788863</v>
+        <v>-0.2746205066745724</v>
       </c>
       <c r="H21" t="n">
-        <v>-0.2400255642853758</v>
+        <v>-0.2605519784514395</v>
       </c>
       <c r="I21" t="n">
-        <v>53.37773549000951</v>
+        <v>65.32614970175102</v>
       </c>
       <c r="J21" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K21" t="n">
         <v>48.43</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M21" t="n">
         <v>48.43</v>
       </c>
       <c r="N21" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O21" t="n">
         <v>6.382978723404255</v>
       </c>
       <c r="P21" t="n">
-        <v>44.64859574468085</v>
+        <v>52.64859574468085</v>
       </c>
       <c r="Q21" t="b">
         <v>0</v>
@@ -2079,48 +2079,48 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>379.7</v>
+        <v>409.75</v>
       </c>
       <c r="D22" t="n">
-        <v>-0.1177973977695167</v>
+        <v>-0.0416325575956029</v>
       </c>
       <c r="E22" t="n">
-        <v>0.1012180974477958</v>
+        <v>0.0915023974427278</v>
       </c>
       <c r="F22" t="n">
-        <v>0.2230632952166209</v>
+        <v>0.314354450681636</v>
       </c>
       <c r="G22" t="n">
-        <v>0.3147624300812235</v>
+        <v>0.3420798292181174</v>
       </c>
       <c r="H22" t="n">
-        <v>0.300106219874734</v>
+        <v>0.3561483574412503</v>
       </c>
       <c r="I22" t="n">
-        <v>44.93295915185531</v>
+        <v>58.62761986792995</v>
       </c>
       <c r="J22" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="K22" t="n">
         <v>54.47</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M22" t="n">
         <v>54.47</v>
       </c>
       <c r="N22" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="O22" t="n">
         <v>93.61702127659576</v>
       </c>
       <c r="P22" t="n">
-        <v>56.51140425531915</v>
+        <v>72.51140425531915</v>
       </c>
       <c r="Q22" t="b">
         <v>0</v>
@@ -2144,25 +2144,25 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>342.35</v>
+        <v>353.05</v>
       </c>
       <c r="D23" t="n">
-        <v>-0.0349541930937279</v>
+        <v>-0.009121526803255699</v>
       </c>
       <c r="E23" t="n">
-        <v>-0.1141156682623882</v>
+        <v>-0.1100327703554322</v>
       </c>
       <c r="F23" t="n">
-        <v>-0.170362292499697</v>
+        <v>-0.1536617523672538</v>
       </c>
       <c r="G23" t="n">
-        <v>-0.07866315763509441</v>
+        <v>-0.1259363738307725</v>
       </c>
       <c r="H23" t="n">
-        <v>-0.0933193678415839</v>
+        <v>-0.1118678456076396</v>
       </c>
       <c r="I23" t="n">
-        <v>50.82074852265266</v>
+        <v>55.7590076786769</v>
       </c>
       <c r="J23" t="n">
         <v>60</v>
@@ -2172,7 +2172,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M23" t="n">
@@ -2209,48 +2209,48 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>114.82</v>
+        <v>121.07</v>
       </c>
       <c r="D24" t="n">
-        <v>-0.0610075237160615</v>
+        <v>-0.0418645140867363</v>
       </c>
       <c r="E24" t="n">
-        <v>-0.1417893714029449</v>
+        <v>-0.1073508810735088</v>
       </c>
       <c r="F24" t="n">
-        <v>0.0566905945150009</v>
+        <v>0.1197743248242693</v>
       </c>
       <c r="G24" t="n">
-        <v>0.1483897293796034</v>
+        <v>0.1474997033607507</v>
       </c>
       <c r="H24" t="n">
-        <v>0.133733519173114</v>
+        <v>0.1615682315838835</v>
       </c>
       <c r="I24" t="n">
-        <v>41.09001837109614</v>
+        <v>54.14614121510672</v>
       </c>
       <c r="J24" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K24" t="n">
         <v>48.3</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M24" t="n">
         <v>48.3</v>
       </c>
       <c r="N24" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O24" t="n">
-        <v>80.85106382978722</v>
+        <v>82.97872340425532</v>
       </c>
       <c r="P24" t="n">
-        <v>51.49021276595744</v>
+        <v>59.91574468085106</v>
       </c>
       <c r="Q24" t="b">
         <v>0</v>
@@ -2274,25 +2274,25 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>560.35</v>
+        <v>580.25</v>
       </c>
       <c r="D25" t="n">
-        <v>0.1003436426116839</v>
+        <v>0.1110579224509333</v>
       </c>
       <c r="E25" t="n">
-        <v>-0.139643789344388</v>
+        <v>-0.0940671350507416</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.2394299287410926</v>
+        <v>-0.1917960860784178</v>
       </c>
       <c r="G25" t="n">
-        <v>-0.14773079387649</v>
+        <v>-0.1640707075419364</v>
       </c>
       <c r="H25" t="n">
-        <v>-0.1623870040829794</v>
+        <v>-0.1500021793188035</v>
       </c>
       <c r="I25" t="n">
-        <v>44.39853076216713</v>
+        <v>57.75136206042595</v>
       </c>
       <c r="J25" t="n">
         <v>80</v>
@@ -2302,7 +2302,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M25" t="n">
@@ -2312,10 +2312,10 @@
         <v>80</v>
       </c>
       <c r="O25" t="n">
-        <v>25.53191489361702</v>
+        <v>29.78723404255319</v>
       </c>
       <c r="P25" t="n">
-        <v>59.8703829787234</v>
+        <v>60.72144680851064</v>
       </c>
       <c r="Q25" t="b">
         <v>0</v>
@@ -2339,25 +2339,25 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>127.49</v>
+        <v>133.21</v>
       </c>
       <c r="D26" t="n">
-        <v>-0.0133880204302739</v>
+        <v>-0.0045583619787773</v>
       </c>
       <c r="E26" t="n">
-        <v>-0.2017406549370735</v>
+        <v>-0.1639364840268624</v>
       </c>
       <c r="F26" t="n">
-        <v>-0.2566614191592327</v>
+        <v>-0.2276337913840087</v>
       </c>
       <c r="G26" t="n">
-        <v>-0.1649622842946301</v>
+        <v>-0.1999084128475273</v>
       </c>
       <c r="H26" t="n">
-        <v>-0.1796184945011195</v>
+        <v>-0.1858398846243945</v>
       </c>
       <c r="I26" t="n">
-        <v>45.45696775912602</v>
+        <v>57.96437659033079</v>
       </c>
       <c r="J26" t="n">
         <v>60</v>
@@ -2367,7 +2367,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M26" t="n">
@@ -2377,10 +2377,10 @@
         <v>60</v>
       </c>
       <c r="O26" t="n">
-        <v>17.02127659574468</v>
+        <v>19.14893617021277</v>
       </c>
       <c r="P26" t="n">
-        <v>48.02025531914894</v>
+        <v>48.44578723404256</v>
       </c>
       <c r="Q26" t="b">
         <v>0</v>
@@ -2404,48 +2404,48 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>4800</v>
+        <v>5251</v>
       </c>
       <c r="D27" t="n">
-        <v>-0.0827441238295433</v>
+        <v>0.0137065637065636</v>
       </c>
       <c r="E27" t="n">
-        <v>-0.1638359027959237</v>
+        <v>-0.0608960028614862</v>
       </c>
       <c r="F27" t="n">
-        <v>0.1446558878237231</v>
+        <v>0.2508337303477845</v>
       </c>
       <c r="G27" t="n">
-        <v>0.2363550226883257</v>
+        <v>0.2785591088842659</v>
       </c>
       <c r="H27" t="n">
-        <v>0.2216988124818363</v>
+        <v>0.2926276371073988</v>
       </c>
       <c r="I27" t="n">
-        <v>36.84502049407333</v>
+        <v>57.68773580029976</v>
       </c>
       <c r="J27" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="K27" t="n">
         <v>57.69</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M27" t="n">
         <v>57.69</v>
       </c>
       <c r="N27" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="O27" t="n">
-        <v>87.2340425531915</v>
+        <v>89.36170212765957</v>
       </c>
       <c r="P27" t="n">
-        <v>52.5228085106383</v>
+        <v>64.94834042553191</v>
       </c>
       <c r="Q27" t="b">
         <v>0</v>
@@ -2469,25 +2469,25 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1634.4</v>
+        <v>1691.7</v>
       </c>
       <c r="D28" t="n">
-        <v>0.1067921717342723</v>
+        <v>0.1248753241571911</v>
       </c>
       <c r="E28" t="n">
-        <v>-0.0282996432818073</v>
+        <v>0.0125089777352167</v>
       </c>
       <c r="F28" t="n">
-        <v>0.4808371840173959</v>
+        <v>0.5525881057268724</v>
       </c>
       <c r="G28" t="n">
-        <v>0.5725363188819985</v>
+        <v>0.5803134842633538</v>
       </c>
       <c r="H28" t="n">
-        <v>0.5578801086755091</v>
+        <v>0.5943820124864867</v>
       </c>
       <c r="I28" t="n">
-        <v>48.72545642438856</v>
+        <v>60.31914893617022</v>
       </c>
       <c r="J28" t="n">
         <v>80</v>
@@ -2497,7 +2497,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M28" t="n">
@@ -2534,48 +2534,48 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>505.2</v>
+        <v>532.55</v>
       </c>
       <c r="D29" t="n">
-        <v>0.0151713051341304</v>
+        <v>0.0502908983334975</v>
       </c>
       <c r="E29" t="n">
-        <v>-0.1622585191940966</v>
+        <v>-0.1093736934526299</v>
       </c>
       <c r="F29" t="n">
-        <v>-0.0087314823898754</v>
+        <v>0.0280888030888029</v>
       </c>
       <c r="G29" t="n">
-        <v>0.08296765247472709</v>
+        <v>0.0558141816252842</v>
       </c>
       <c r="H29" t="n">
-        <v>0.0683114422682377</v>
+        <v>0.0698827098484171</v>
       </c>
       <c r="I29" t="n">
-        <v>49.92997198879552</v>
+        <v>59.66132446325973</v>
       </c>
       <c r="J29" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K29" t="n">
         <v>49.42</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M29" t="n">
         <v>49.42</v>
       </c>
       <c r="N29" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O29" t="n">
         <v>61.70212765957447</v>
       </c>
       <c r="P29" t="n">
-        <v>48.1084255319149</v>
+        <v>56.1084255319149</v>
       </c>
       <c r="Q29" t="b">
         <v>0</v>
@@ -2599,48 +2599,48 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>110.21</v>
+        <v>113.62</v>
       </c>
       <c r="D30" t="n">
-        <v>-0.0541537933401991</v>
+        <v>-0.0540338023478477</v>
       </c>
       <c r="E30" t="n">
-        <v>-0.0367942667365845</v>
+        <v>-0.0091567105607395</v>
       </c>
       <c r="F30" t="n">
-        <v>-0.1456589147286822</v>
+        <v>-0.1337297956694113</v>
       </c>
       <c r="G30" t="n">
-        <v>-0.0539597798640796</v>
+        <v>-0.1060044171329299</v>
       </c>
       <c r="H30" t="n">
-        <v>-0.068615990070569</v>
+        <v>-0.091935888909797</v>
       </c>
       <c r="I30" t="n">
-        <v>29.11852096401451</v>
+        <v>43.70979270907792</v>
       </c>
       <c r="J30" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="K30" t="n">
         <v>52.38</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M30" t="n">
         <v>52.38</v>
       </c>
       <c r="N30" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="O30" t="n">
-        <v>46.80851063829788</v>
+        <v>42.5531914893617</v>
       </c>
       <c r="P30" t="n">
-        <v>38.31370212765957</v>
+        <v>45.46263829787234</v>
       </c>
       <c r="Q30" t="b">
         <v>0</v>
@@ -2664,48 +2664,48 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>37.01</v>
+        <v>38.76</v>
       </c>
       <c r="D31" t="n">
-        <v>-0.07751744765702891</v>
+        <v>-0.04860088365243</v>
       </c>
       <c r="E31" t="n">
-        <v>-0.2889529298751201</v>
+        <v>-0.2423768569194683</v>
       </c>
       <c r="F31" t="n">
-        <v>-0.2419090536665301</v>
+        <v>-0.2145896656534954</v>
       </c>
       <c r="G31" t="n">
-        <v>-0.1502099188019275</v>
+        <v>-0.186864287117014</v>
       </c>
       <c r="H31" t="n">
-        <v>-0.164866129008417</v>
+        <v>-0.1727957588938812</v>
       </c>
       <c r="I31" t="n">
-        <v>40.17660044150109</v>
+        <v>58.01937567276639</v>
       </c>
       <c r="J31" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K31" t="n">
         <v>48.99</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M31" t="n">
         <v>48.99</v>
       </c>
       <c r="N31" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O31" t="n">
-        <v>19.14893617021277</v>
+        <v>21.27659574468085</v>
       </c>
       <c r="P31" t="n">
-        <v>39.42578723404256</v>
+        <v>47.85131914893617</v>
       </c>
       <c r="Q31" t="b">
         <v>0</v>
@@ -2729,48 +2729,48 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>667.7</v>
+        <v>716.6</v>
       </c>
       <c r="D32" t="n">
-        <v>-0.0309846890646541</v>
+        <v>-0.0058268590455049</v>
       </c>
       <c r="E32" t="n">
-        <v>-0.1788722867859558</v>
+        <v>-0.1012166060454031</v>
       </c>
       <c r="F32" t="n">
-        <v>-0.4076998137141843</v>
+        <v>-0.3518451519536902</v>
       </c>
       <c r="G32" t="n">
-        <v>-0.3160006788495817</v>
+        <v>-0.3241197734172089</v>
       </c>
       <c r="H32" t="n">
-        <v>-0.3306568890560711</v>
+        <v>-0.310051245194076</v>
       </c>
       <c r="I32" t="n">
-        <v>42.81333844384822</v>
+        <v>56.80933852140078</v>
       </c>
       <c r="J32" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K32" t="n">
         <v>47.86</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M32" t="n">
         <v>47.86</v>
       </c>
       <c r="N32" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O32" t="n">
         <v>2.127659574468085</v>
       </c>
       <c r="P32" t="n">
-        <v>43.56953191489362</v>
+        <v>51.56953191489362</v>
       </c>
       <c r="Q32" t="b">
         <v>0</v>
@@ -2794,48 +2794,48 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>539.1</v>
+        <v>569.35</v>
       </c>
       <c r="D33" t="n">
-        <v>-0.0092805292658273</v>
+        <v>0.0147032614507218</v>
       </c>
       <c r="E33" t="n">
-        <v>-0.2039279385705847</v>
+        <v>-0.1281010719754977</v>
       </c>
       <c r="F33" t="n">
-        <v>0.0129650507328071</v>
+        <v>0.079745875213351</v>
       </c>
       <c r="G33" t="n">
-        <v>0.1046641855974097</v>
+        <v>0.1074712537498324</v>
       </c>
       <c r="H33" t="n">
-        <v>0.0900079753909203</v>
+        <v>0.1215397819729653</v>
       </c>
       <c r="I33" t="n">
-        <v>47.57804090419806</v>
+        <v>60.8764186633039</v>
       </c>
       <c r="J33" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K33" t="n">
         <v>49.98</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M33" t="n">
         <v>49.98</v>
       </c>
       <c r="N33" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O33" t="n">
-        <v>72.3404255319149</v>
+        <v>74.46808510638297</v>
       </c>
       <c r="P33" t="n">
-        <v>58.46008510638298</v>
+        <v>66.8856170212766</v>
       </c>
       <c r="Q33" t="b">
         <v>0</v>
@@ -2871,10 +2871,10 @@
         <v>-0.2401052253975846</v>
       </c>
       <c r="G34" t="n">
-        <v>-0.148406090532982</v>
+        <v>-0.2123798468611032</v>
       </c>
       <c r="H34" t="n">
-        <v>-0.1630623007394714</v>
+        <v>-0.1983113186379703</v>
       </c>
       <c r="I34" t="n">
         <v>63.3225806451613</v>
@@ -2887,7 +2887,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M34" t="n">
@@ -2897,10 +2897,10 @@
         <v>80</v>
       </c>
       <c r="O34" t="n">
-        <v>21.27659574468085</v>
+        <v>17.02127659574468</v>
       </c>
       <c r="P34" t="n">
-        <v>56.60731914893617</v>
+        <v>55.75625531914894</v>
       </c>
       <c r="Q34" t="b">
         <v>0</v>
@@ -2924,25 +2924,25 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>108.18</v>
+        <v>115.68</v>
       </c>
       <c r="D35" t="n">
-        <v>0.02725287247175</v>
+        <v>0.0337801608579089</v>
       </c>
       <c r="E35" t="n">
-        <v>-0.177338403041825</v>
+        <v>-0.0897072710103871</v>
       </c>
       <c r="F35" t="n">
-        <v>0.0179730874188388</v>
+        <v>0.0777974471256872</v>
       </c>
       <c r="G35" t="n">
-        <v>0.1096722222834414</v>
+        <v>0.1055228256621686</v>
       </c>
       <c r="H35" t="n">
-        <v>0.0950160120769519</v>
+        <v>0.1195913538853015</v>
       </c>
       <c r="I35" t="n">
-        <v>44.05444126074499</v>
+        <v>60.9297957266964</v>
       </c>
       <c r="J35" t="n">
         <v>60</v>
@@ -2952,7 +2952,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M35" t="n">
@@ -2962,10 +2962,10 @@
         <v>60</v>
       </c>
       <c r="O35" t="n">
-        <v>74.46808510638297</v>
+        <v>72.3404255319149</v>
       </c>
       <c r="P35" t="n">
-        <v>58.5216170212766</v>
+        <v>58.09608510638298</v>
       </c>
       <c r="Q35" t="b">
         <v>0</v>
@@ -2989,25 +2989,25 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>472.6</v>
+        <v>486.4</v>
       </c>
       <c r="D36" t="n">
-        <v>-0.046600766592697</v>
+        <v>-0.032809703718433</v>
       </c>
       <c r="E36" t="n">
-        <v>-0.1853128770901568</v>
+        <v>-0.1578947368421053</v>
       </c>
       <c r="F36" t="n">
-        <v>0.0264986967854041</v>
+        <v>0.0496331463098835</v>
       </c>
       <c r="G36" t="n">
-        <v>0.1181978316500067</v>
+        <v>0.07735852484636491</v>
       </c>
       <c r="H36" t="n">
-        <v>0.1035416214435173</v>
+        <v>0.0914270530694978</v>
       </c>
       <c r="I36" t="n">
-        <v>44.093567251462</v>
+        <v>55.15484123872992</v>
       </c>
       <c r="J36" t="n">
         <v>60</v>
@@ -3017,7 +3017,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M36" t="n">
@@ -3027,10 +3027,10 @@
         <v>60</v>
       </c>
       <c r="O36" t="n">
-        <v>78.72340425531915</v>
+        <v>65.95744680851064</v>
       </c>
       <c r="P36" t="n">
-        <v>58.86468085106384</v>
+        <v>56.31148936170213</v>
       </c>
       <c r="Q36" t="b">
         <v>0</v>
@@ -3054,25 +3054,25 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2150.6</v>
+        <v>2248.1</v>
       </c>
       <c r="D37" t="n">
-        <v>0.0256581457458984</v>
+        <v>0.0290671061063809</v>
       </c>
       <c r="E37" t="n">
-        <v>0.1125711329539576</v>
+        <v>0.1677834917666614</v>
       </c>
       <c r="F37" t="n">
-        <v>0.5363623374767823</v>
+        <v>0.5730879574557415</v>
       </c>
       <c r="G37" t="n">
-        <v>0.6280614723413849</v>
+        <v>0.6008133359922229</v>
       </c>
       <c r="H37" t="n">
-        <v>0.6134052621348954</v>
+        <v>0.6148818642153557</v>
       </c>
       <c r="I37" t="n">
-        <v>45.81015299026424</v>
+        <v>59.29697766097239</v>
       </c>
       <c r="J37" t="n">
         <v>80</v>
@@ -3082,7 +3082,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M37" t="n">
@@ -3119,48 +3119,48 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>759.9</v>
+        <v>802.2</v>
       </c>
       <c r="D38" t="n">
-        <v>-0.0653136531365313</v>
+        <v>-0.0348312578956866</v>
       </c>
       <c r="E38" t="n">
-        <v>-0.2206553510076406</v>
+        <v>-0.1580162686958802</v>
       </c>
       <c r="F38" t="n">
-        <v>-0.278621606227454</v>
+        <v>-0.2519582245430809</v>
       </c>
       <c r="G38" t="n">
-        <v>-0.1869224713628514</v>
+        <v>-0.2242328460065995</v>
       </c>
       <c r="H38" t="n">
-        <v>-0.2015786815693409</v>
+        <v>-0.2101643177834666</v>
       </c>
       <c r="I38" t="n">
-        <v>37.99679201568346</v>
+        <v>52.30985420692079</v>
       </c>
       <c r="J38" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="K38" t="n">
         <v>49.87</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M38" t="n">
         <v>49.87</v>
       </c>
       <c r="N38" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="O38" t="n">
         <v>12.76595744680851</v>
       </c>
       <c r="P38" t="n">
-        <v>34.5011914893617</v>
+        <v>46.5011914893617</v>
       </c>
       <c r="Q38" t="b">
         <v>0</v>
@@ -3184,48 +3184,48 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>2976.4</v>
+        <v>3130.9</v>
       </c>
       <c r="D39" t="n">
-        <v>0.0588402703664177</v>
+        <v>0.0339145366884618</v>
       </c>
       <c r="E39" t="n">
-        <v>-0.1142457518673928</v>
+        <v>-0.0614526814352948</v>
       </c>
       <c r="F39" t="n">
-        <v>0.1133388194808109</v>
+        <v>0.1742489592318943</v>
       </c>
       <c r="G39" t="n">
-        <v>0.2050379543454135</v>
+        <v>0.2019743377683757</v>
       </c>
       <c r="H39" t="n">
-        <v>0.190381744138924</v>
+        <v>0.2160428659915085</v>
       </c>
       <c r="I39" t="n">
-        <v>45.91883264933881</v>
+        <v>60.13812452789469</v>
       </c>
       <c r="J39" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="K39" t="n">
         <v>48.69</v>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M39" t="n">
         <v>48.69</v>
       </c>
       <c r="N39" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="O39" t="n">
         <v>85.1063829787234</v>
       </c>
       <c r="P39" t="n">
-        <v>52.49727659574468</v>
+        <v>68.49727659574468</v>
       </c>
       <c r="Q39" t="b">
         <v>0</v>
@@ -3249,48 +3249,48 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>191.18</v>
+        <v>201.5</v>
       </c>
       <c r="D40" t="n">
-        <v>0.0192461481047077</v>
+        <v>0.0483870967741935</v>
       </c>
       <c r="E40" t="n">
-        <v>-0.1062596419054742</v>
+        <v>-0.0562060889929741</v>
       </c>
       <c r="F40" t="n">
-        <v>-0.2244533690316822</v>
+        <v>-0.1763744124259145</v>
       </c>
       <c r="G40" t="n">
-        <v>-0.1327542341670796</v>
+        <v>-0.1486490338894331</v>
       </c>
       <c r="H40" t="n">
-        <v>-0.1474104443735691</v>
+        <v>-0.1345805056663003</v>
       </c>
       <c r="I40" t="n">
-        <v>53.69656328583402</v>
+        <v>67.86858974358975</v>
       </c>
       <c r="J40" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K40" t="n">
         <v>45.44</v>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M40" t="n">
         <v>45.44</v>
       </c>
       <c r="N40" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O40" t="n">
-        <v>34.04255319148936</v>
+        <v>31.91489361702128</v>
       </c>
       <c r="P40" t="n">
-        <v>48.98451063829788</v>
+        <v>56.55897872340426</v>
       </c>
       <c r="Q40" t="b">
         <v>0</v>
@@ -3314,48 +3314,48 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>750.05</v>
+        <v>780.25</v>
       </c>
       <c r="D41" t="n">
-        <v>-0.1012521718291294</v>
+        <v>-0.0752044565603887</v>
       </c>
       <c r="E41" t="n">
-        <v>-0.2012247071352503</v>
+        <v>-0.1691070763005164</v>
       </c>
       <c r="F41" t="n">
-        <v>-0.2591367048597393</v>
+        <v>-0.2596546161874941</v>
       </c>
       <c r="G41" t="n">
-        <v>-0.1674375699951367</v>
+        <v>-0.2319292376510127</v>
       </c>
       <c r="H41" t="n">
-        <v>-0.1820937802016261</v>
+        <v>-0.2178607094278798</v>
       </c>
       <c r="I41" t="n">
-        <v>23.96411789833407</v>
+        <v>37.80573025856047</v>
       </c>
       <c r="J41" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="K41" t="n">
         <v>48.05</v>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M41" t="n">
         <v>48.05</v>
       </c>
       <c r="N41" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="O41" t="n">
-        <v>14.8936170212766</v>
+        <v>10.63829787234042</v>
       </c>
       <c r="P41" t="n">
-        <v>30.19872340425532</v>
+        <v>33.34765957446808</v>
       </c>
       <c r="Q41" t="b">
         <v>0</v>
@@ -3379,25 +3379,25 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>532.4</v>
+        <v>561.1</v>
       </c>
       <c r="D42" t="n">
-        <v>-0.0398557258791704</v>
+        <v>-0.0220479302832243</v>
       </c>
       <c r="E42" t="n">
-        <v>-0.2330187999711878</v>
+        <v>-0.1818910840562805</v>
       </c>
       <c r="F42" t="n">
-        <v>-0.2996119187002565</v>
+        <v>-0.2675890875864769</v>
       </c>
       <c r="G42" t="n">
-        <v>-0.2079127838356539</v>
+        <v>-0.2398637090499955</v>
       </c>
       <c r="H42" t="n">
-        <v>-0.2225689940421433</v>
+        <v>-0.2257951808268626</v>
       </c>
       <c r="I42" t="n">
-        <v>46.41249669049509</v>
+        <v>56.5080135988344</v>
       </c>
       <c r="J42" t="n">
         <v>60</v>
@@ -3407,7 +3407,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M42" t="n">
@@ -3444,54 +3444,54 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>418.2</v>
+        <v>427.4</v>
       </c>
       <c r="D43" t="n">
-        <v>0.0140640155189137</v>
+        <v>0.0159258378892321</v>
       </c>
       <c r="E43" t="n">
-        <v>-0.1208745007357577</v>
+        <v>-0.0892819092265075</v>
       </c>
       <c r="F43" t="n">
-        <v>-0.0631720430107526</v>
+        <v>-0.0513816446565309</v>
       </c>
       <c r="G43" t="n">
-        <v>0.0285270918538499</v>
+        <v>-0.0236562661200495</v>
       </c>
       <c r="H43" t="n">
-        <v>0.0138708816473605</v>
+        <v>-0.009587737896916601</v>
       </c>
       <c r="I43" t="n">
-        <v>56.33059788980072</v>
+        <v>67.87196206283343</v>
       </c>
       <c r="J43" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K43" t="n">
         <v>51.48</v>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M43" t="n">
         <v>51.48</v>
       </c>
       <c r="N43" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O43" t="n">
         <v>53.19148936170212</v>
       </c>
       <c r="P43" t="n">
-        <v>55.23029787234042</v>
+        <v>63.23029787234042</v>
       </c>
       <c r="Q43" t="b">
         <v>0</v>
       </c>
       <c r="R43" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S43" t="b">
         <v>0</v>
@@ -3509,25 +3509,25 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>249.2</v>
+        <v>253.91</v>
       </c>
       <c r="D44" t="n">
-        <v>0.017765979170921</v>
+        <v>0.0279757085020242</v>
       </c>
       <c r="E44" t="n">
-        <v>-0.090178897407813</v>
+        <v>-0.0630627306273062</v>
       </c>
       <c r="F44" t="n">
-        <v>-0.1619303850681016</v>
+        <v>-0.1328210382513661</v>
       </c>
       <c r="G44" t="n">
-        <v>-0.070231250203499</v>
+        <v>-0.1050956597148847</v>
       </c>
       <c r="H44" t="n">
-        <v>-0.0848874604099885</v>
+        <v>-0.0910271314917519</v>
       </c>
       <c r="I44" t="n">
-        <v>52.7207711442786</v>
+        <v>66.15279205207261</v>
       </c>
       <c r="J44" t="n">
         <v>60</v>
@@ -3537,7 +3537,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M44" t="n">
@@ -3547,10 +3547,10 @@
         <v>60</v>
       </c>
       <c r="O44" t="n">
-        <v>42.5531914893617</v>
+        <v>44.68085106382978</v>
       </c>
       <c r="P44" t="n">
-        <v>51.39063829787234</v>
+        <v>51.81617021276596</v>
       </c>
       <c r="Q44" t="b">
         <v>0</v>
@@ -3574,48 +3574,48 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>91.27</v>
+        <v>96.31999999999999</v>
       </c>
       <c r="D45" t="n">
-        <v>-0.08464547186841841</v>
+        <v>-0.0385306448392893</v>
       </c>
       <c r="E45" t="n">
-        <v>-0.1984015457579484</v>
+        <v>-0.1406138472519629</v>
       </c>
       <c r="F45" t="n">
-        <v>-0.3353480920477716</v>
+        <v>-0.3058518304987028</v>
       </c>
       <c r="G45" t="n">
-        <v>-0.243648957183169</v>
+        <v>-0.2781264519622214</v>
       </c>
       <c r="H45" t="n">
-        <v>-0.2583051673896585</v>
+        <v>-0.2640579237390885</v>
       </c>
       <c r="I45" t="n">
-        <v>35.08396946564882</v>
+        <v>48.97838318033756</v>
       </c>
       <c r="J45" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="K45" t="n">
         <v>59.6</v>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M45" t="n">
         <v>59.6</v>
       </c>
       <c r="N45" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="O45" t="n">
         <v>4.25531914893617</v>
       </c>
       <c r="P45" t="n">
-        <v>36.69106382978724</v>
+        <v>48.69106382978724</v>
       </c>
       <c r="Q45" t="b">
         <v>0</v>
@@ -3639,48 +3639,48 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>473.15</v>
+        <v>500.4</v>
       </c>
       <c r="D46" t="n">
-        <v>-0.0214064115822131</v>
+        <v>0.0049201727081031</v>
       </c>
       <c r="E46" t="n">
-        <v>-0.2452544265433083</v>
+        <v>-0.189110354885756</v>
       </c>
       <c r="F46" t="n">
-        <v>-0.2396143029329048</v>
+        <v>-0.2071615305394913</v>
       </c>
       <c r="G46" t="n">
-        <v>-0.1479151680683023</v>
+        <v>-0.17943615200301</v>
       </c>
       <c r="H46" t="n">
-        <v>-0.1625713782747917</v>
+        <v>-0.1653676237798771</v>
       </c>
       <c r="I46" t="n">
-        <v>30.67623724971668</v>
+        <v>48.83051457358763</v>
       </c>
       <c r="J46" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="K46" t="n">
         <v>49.61</v>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M46" t="n">
         <v>49.61</v>
       </c>
       <c r="N46" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="O46" t="n">
         <v>23.40425531914894</v>
       </c>
       <c r="P46" t="n">
-        <v>36.52485106382979</v>
+        <v>48.52485106382979</v>
       </c>
       <c r="Q46" t="b">
         <v>0</v>
@@ -3704,48 +3704,48 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>960.35</v>
+        <v>991.9</v>
       </c>
       <c r="D47" t="n">
-        <v>0.0472737186477645</v>
+        <v>0.0690881655529209</v>
       </c>
       <c r="E47" t="n">
-        <v>0.104802991084268</v>
+        <v>0.1271590909090909</v>
       </c>
       <c r="F47" t="n">
-        <v>0.2167110097554796</v>
+        <v>0.2530318342597271</v>
       </c>
       <c r="G47" t="n">
-        <v>0.3084101446200822</v>
+        <v>0.2807572127962084</v>
       </c>
       <c r="H47" t="n">
-        <v>0.2937539344135927</v>
+        <v>0.2948257410193413</v>
       </c>
       <c r="I47" t="n">
-        <v>48.28730748805098</v>
+        <v>50.1790739319519</v>
       </c>
       <c r="J47" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K47" t="n">
         <v>46.83</v>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M47" t="n">
         <v>46.83</v>
       </c>
       <c r="N47" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O47" t="n">
         <v>91.48936170212764</v>
       </c>
       <c r="P47" t="n">
-        <v>61.02987234042553</v>
+        <v>69.02987234042553</v>
       </c>
       <c r="Q47" t="b">
         <v>0</v>
@@ -3769,48 +3769,48 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>13649</v>
+        <v>14439</v>
       </c>
       <c r="D48" t="n">
-        <v>-0.0253499000285633</v>
+        <v>0.0317256162915327</v>
       </c>
       <c r="E48" t="n">
-        <v>-0.0972286526886698</v>
+        <v>-0.0562128243676057</v>
       </c>
       <c r="F48" t="n">
-        <v>-0.0006589544589251</v>
+        <v>0.051485581124381</v>
       </c>
       <c r="G48" t="n">
-        <v>0.09104018040567741</v>
+        <v>0.0792109596608624</v>
       </c>
       <c r="H48" t="n">
-        <v>0.0763839701991879</v>
+        <v>0.0932794878839953</v>
       </c>
       <c r="I48" t="n">
-        <v>48.91404099112878</v>
+        <v>64.13422818791946</v>
       </c>
       <c r="J48" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K48" t="n">
         <v>50.29</v>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M48" t="n">
         <v>50.29</v>
       </c>
       <c r="N48" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O48" t="n">
-        <v>65.95744680851064</v>
+        <v>68.08510638297872</v>
       </c>
       <c r="P48" t="n">
-        <v>49.30748936170212</v>
+        <v>57.73302127659574</v>
       </c>
       <c r="Q48" t="b">
         <v>0</v>
@@ -3945,25 +3945,25 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1634.4</v>
+        <v>1691.7</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1067921717342723</v>
+        <v>0.1248753241571911</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.0282996432818073</v>
+        <v>0.0125089777352167</v>
       </c>
       <c r="F2" t="n">
-        <v>0.4808371840173959</v>
+        <v>0.5525881057268724</v>
       </c>
       <c r="G2" t="n">
-        <v>0.5725363188819985</v>
+        <v>0.5803134842633538</v>
       </c>
       <c r="H2" t="n">
-        <v>0.5578801086755091</v>
+        <v>0.5943820124864867</v>
       </c>
       <c r="I2" t="n">
-        <v>48.72545642438856</v>
+        <v>60.31914893617022</v>
       </c>
       <c r="J2" t="n">
         <v>80</v>
@@ -3973,7 +3973,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M2" t="n">
@@ -4001,7 +4001,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SANSERA</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -4010,48 +4010,48 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2150.6</v>
+        <v>1781.4</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0256581457458984</v>
+        <v>-0.0330040169362718</v>
       </c>
       <c r="E3" t="n">
-        <v>0.1125711329539576</v>
+        <v>0.2079745032888045</v>
       </c>
       <c r="F3" t="n">
-        <v>0.5363623374767823</v>
+        <v>0.4102279924002534</v>
       </c>
       <c r="G3" t="n">
-        <v>0.6280614723413849</v>
+        <v>0.4379533709367348</v>
       </c>
       <c r="H3" t="n">
-        <v>0.6134052621348954</v>
+        <v>0.4520218991598677</v>
       </c>
       <c r="I3" t="n">
-        <v>45.81015299026424</v>
+        <v>58.97502601456814</v>
       </c>
       <c r="J3" t="n">
         <v>80</v>
       </c>
       <c r="K3" t="n">
-        <v>48.59</v>
+        <v>54.83</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M3" t="n">
-        <v>48.59</v>
+        <v>54.83</v>
       </c>
       <c r="N3" t="n">
         <v>80</v>
       </c>
       <c r="O3" t="n">
-        <v>100</v>
+        <v>95.74468085106383</v>
       </c>
       <c r="P3" t="n">
-        <v>71.43600000000001</v>
+        <v>73.08093617021277</v>
       </c>
       <c r="Q3" t="b">
         <v>0</v>
@@ -4066,57 +4066,57 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>GNA</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Axles</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>515.15</v>
+        <v>409.75</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0288595965648092</v>
+        <v>-0.0416325575956029</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0701080182800166</v>
+        <v>0.0915023974427278</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1869815668202763</v>
+        <v>0.314354450681636</v>
       </c>
       <c r="G4" t="n">
-        <v>0.2786807016848789</v>
+        <v>0.3420798292181174</v>
       </c>
       <c r="H4" t="n">
-        <v>0.2640244914783894</v>
+        <v>0.3561483574412503</v>
       </c>
       <c r="I4" t="n">
-        <v>51.25515174222554</v>
+        <v>58.62761986792995</v>
       </c>
       <c r="J4" t="n">
         <v>80</v>
       </c>
       <c r="K4" t="n">
-        <v>49.66</v>
+        <v>54.47</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M4" t="n">
-        <v>49.66</v>
+        <v>54.47</v>
       </c>
       <c r="N4" t="n">
         <v>80</v>
       </c>
       <c r="O4" t="n">
-        <v>89.36170212765957</v>
+        <v>93.61702127659576</v>
       </c>
       <c r="P4" t="n">
-        <v>69.73634042553192</v>
+        <v>72.51140425531915</v>
       </c>
       <c r="Q4" t="b">
         <v>0</v>
@@ -4131,63 +4131,63 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ASKAUTOLTD</t>
+          <t>SANSERA</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Forgings</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>433.15</v>
+        <v>2248.1</v>
       </c>
       <c r="D5" t="n">
-        <v>0.1395685345961588</v>
+        <v>0.0290671061063809</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.0898297961756671</v>
+        <v>0.1677834917666614</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.1839675960813865</v>
+        <v>0.5730879574557415</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.092268461216784</v>
+        <v>0.6008133359922229</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.1069246714232734</v>
+        <v>0.6148818642153557</v>
       </c>
       <c r="I5" t="n">
-        <v>57.83071464774454</v>
+        <v>59.29697766097239</v>
       </c>
       <c r="J5" t="n">
         <v>80</v>
       </c>
       <c r="K5" t="n">
-        <v>71.28</v>
+        <v>48.59</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M5" t="n">
-        <v>71.28</v>
+        <v>48.59</v>
       </c>
       <c r="N5" t="n">
         <v>80</v>
       </c>
       <c r="O5" t="n">
-        <v>38.29787234042553</v>
+        <v>100</v>
       </c>
       <c r="P5" t="n">
-        <v>68.17157446808511</v>
+        <v>71.43600000000001</v>
       </c>
       <c r="Q5" t="b">
+        <v>0</v>
+      </c>
+      <c r="R5" t="b">
         <v>1</v>
-      </c>
-      <c r="R5" t="b">
-        <v>0</v>
       </c>
       <c r="S5" t="b">
         <v>0</v>
@@ -4196,57 +4196,57 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BHARATGEAR</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Gears</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>94.84999999999999</v>
+        <v>533.7</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.0145454545454546</v>
+        <v>0.0428920371275036</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.1670325810134364</v>
+        <v>0.1201595130653794</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0645342312008978</v>
+        <v>0.2338457981736217</v>
       </c>
       <c r="G6" t="n">
-        <v>0.1562333660655004</v>
+        <v>0.2615711767101031</v>
       </c>
       <c r="H6" t="n">
-        <v>0.1415771558590109</v>
+        <v>0.275639704933236</v>
       </c>
       <c r="I6" t="n">
-        <v>41.91198786039452</v>
+        <v>62.59899208063357</v>
       </c>
       <c r="J6" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K6" t="n">
-        <v>51.91</v>
+        <v>49.66</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M6" t="n">
-        <v>51.91</v>
+        <v>49.66</v>
       </c>
       <c r="N6" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O6" t="n">
-        <v>82.97872340425532</v>
+        <v>87.2340425531915</v>
       </c>
       <c r="P6" t="n">
-        <v>61.35974468085107</v>
+        <v>69.31080851063831</v>
       </c>
       <c r="Q6" t="b">
         <v>0</v>
@@ -4261,57 +4261,57 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>WHEELS</t>
+          <t>BHARATSE</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Wheels</t>
+          <t>Seating</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>960.35</v>
+        <v>176.72</v>
       </c>
       <c r="D7" t="n">
-        <v>0.0472737186477645</v>
+        <v>0.004775983625199</v>
       </c>
       <c r="E7" t="n">
-        <v>0.104802991084268</v>
+        <v>0.0193228355540173</v>
       </c>
       <c r="F7" t="n">
-        <v>0.2167110097554796</v>
+        <v>0.1117961623151935</v>
       </c>
       <c r="G7" t="n">
-        <v>0.3084101446200822</v>
+        <v>0.1395215408516749</v>
       </c>
       <c r="H7" t="n">
-        <v>0.2937539344135927</v>
+        <v>0.1535900690748077</v>
       </c>
       <c r="I7" t="n">
-        <v>48.28730748805098</v>
+        <v>63.04656262092092</v>
       </c>
       <c r="J7" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K7" t="n">
-        <v>46.83</v>
+        <v>52.61</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M7" t="n">
-        <v>46.83</v>
+        <v>52.61</v>
       </c>
       <c r="N7" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O7" t="n">
-        <v>91.48936170212764</v>
+        <v>80.85106382978722</v>
       </c>
       <c r="P7" t="n">
-        <v>61.02987234042553</v>
+        <v>69.21421276595744</v>
       </c>
       <c r="Q7" t="b">
         <v>0</v>
@@ -4326,63 +4326,63 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>JBMA</t>
+          <t>WHEELS</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Wheels</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>560.35</v>
+        <v>991.9</v>
       </c>
       <c r="D8" t="n">
-        <v>0.1003436426116839</v>
+        <v>0.0690881655529209</v>
       </c>
       <c r="E8" t="n">
-        <v>-0.139643789344388</v>
+        <v>0.1271590909090909</v>
       </c>
       <c r="F8" t="n">
-        <v>-0.2394299287410926</v>
+        <v>0.2530318342597271</v>
       </c>
       <c r="G8" t="n">
-        <v>-0.14773079387649</v>
+        <v>0.2807572127962084</v>
       </c>
       <c r="H8" t="n">
-        <v>-0.1623870040829794</v>
+        <v>0.2948257410193413</v>
       </c>
       <c r="I8" t="n">
-        <v>44.39853076216713</v>
+        <v>50.1790739319519</v>
       </c>
       <c r="J8" t="n">
         <v>80</v>
       </c>
       <c r="K8" t="n">
-        <v>56.91</v>
+        <v>46.83</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M8" t="n">
-        <v>56.91</v>
+        <v>46.83</v>
       </c>
       <c r="N8" t="n">
         <v>80</v>
       </c>
       <c r="O8" t="n">
-        <v>25.53191489361702</v>
+        <v>91.48936170212764</v>
       </c>
       <c r="P8" t="n">
-        <v>59.8703829787234</v>
+        <v>69.02987234042553</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
       </c>
       <c r="R8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S8" t="b">
         <v>0</v>
@@ -4391,57 +4391,57 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SANDHAR</t>
+          <t>SHRIPISTON</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Engine/Parts</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>472.6</v>
+        <v>3130.9</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.046600766592697</v>
+        <v>0.0339145366884618</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.1853128770901568</v>
+        <v>-0.0614526814352948</v>
       </c>
       <c r="F9" t="n">
-        <v>0.0264986967854041</v>
+        <v>0.1742489592318943</v>
       </c>
       <c r="G9" t="n">
-        <v>0.1181978316500067</v>
+        <v>0.2019743377683757</v>
       </c>
       <c r="H9" t="n">
-        <v>0.1035416214435173</v>
+        <v>0.2160428659915085</v>
       </c>
       <c r="I9" t="n">
-        <v>44.093567251462</v>
+        <v>60.13812452789469</v>
       </c>
       <c r="J9" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K9" t="n">
-        <v>47.8</v>
+        <v>48.69</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M9" t="n">
-        <v>47.8</v>
+        <v>48.69</v>
       </c>
       <c r="N9" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O9" t="n">
-        <v>78.72340425531915</v>
+        <v>85.1063829787234</v>
       </c>
       <c r="P9" t="n">
-        <v>58.86468085106384</v>
+        <v>68.49727659574468</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -4456,63 +4456,63 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>RICOAUTO</t>
+          <t>ASKAUTOLTD</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Castings</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>108.18</v>
+        <v>440.5</v>
       </c>
       <c r="D10" t="n">
-        <v>0.02725287247175</v>
+        <v>0.1185881157948196</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.177338403041825</v>
+        <v>-0.0717521862817406</v>
       </c>
       <c r="F10" t="n">
-        <v>0.0179730874188388</v>
+        <v>-0.1760194537972316</v>
       </c>
       <c r="G10" t="n">
-        <v>0.1096722222834414</v>
+        <v>-0.1482940752607502</v>
       </c>
       <c r="H10" t="n">
-        <v>0.0950160120769519</v>
+        <v>-0.1342255470376173</v>
       </c>
       <c r="I10" t="n">
-        <v>44.05444126074499</v>
+        <v>60.43747028055159</v>
       </c>
       <c r="J10" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K10" t="n">
-        <v>49.07</v>
+        <v>71.28</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M10" t="n">
-        <v>49.07</v>
+        <v>71.28</v>
       </c>
       <c r="N10" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O10" t="n">
-        <v>74.46808510638297</v>
+        <v>34.04255319148936</v>
       </c>
       <c r="P10" t="n">
-        <v>58.5216170212766</v>
+        <v>67.32051063829788</v>
       </c>
       <c r="Q10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S10" t="b">
         <v>0</v>
@@ -4530,48 +4530,48 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>539.1</v>
+        <v>569.35</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.0092805292658273</v>
+        <v>0.0147032614507218</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.2039279385705847</v>
+        <v>-0.1281010719754977</v>
       </c>
       <c r="F11" t="n">
-        <v>0.0129650507328071</v>
+        <v>0.079745875213351</v>
       </c>
       <c r="G11" t="n">
-        <v>0.1046641855974097</v>
+        <v>0.1074712537498324</v>
       </c>
       <c r="H11" t="n">
-        <v>0.0900079753909203</v>
+        <v>0.1215397819729653</v>
       </c>
       <c r="I11" t="n">
-        <v>47.57804090419806</v>
+        <v>60.8764186633039</v>
       </c>
       <c r="J11" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K11" t="n">
         <v>49.98</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M11" t="n">
         <v>49.98</v>
       </c>
       <c r="N11" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O11" t="n">
-        <v>72.3404255319149</v>
+        <v>74.46808510638297</v>
       </c>
       <c r="P11" t="n">
-        <v>58.46008510638298</v>
+        <v>66.8856170212766</v>
       </c>
       <c r="Q11" t="b">
         <v>0</v>
@@ -4586,63 +4586,63 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TIINDIA</t>
+          <t>LUMAXIND</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Lighting</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>2588.2</v>
+        <v>5251</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.0078202867438472</v>
+        <v>0.0137065637065636</v>
       </c>
       <c r="E12" t="n">
-        <v>0.0230039525691698</v>
+        <v>-0.0608960028614862</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.2283473957246355</v>
+        <v>0.2508337303477845</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.136648260860033</v>
+        <v>0.2785591088842659</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.1513044710665224</v>
+        <v>0.2926276371073988</v>
       </c>
       <c r="I12" t="n">
-        <v>52.53784505788068</v>
+        <v>57.68773580029976</v>
       </c>
       <c r="J12" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K12" t="n">
-        <v>48.73</v>
+        <v>57.69</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M12" t="n">
-        <v>48.73</v>
+        <v>57.69</v>
       </c>
       <c r="N12" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O12" t="n">
-        <v>29.78723404255319</v>
+        <v>89.36170212765957</v>
       </c>
       <c r="P12" t="n">
-        <v>57.44944680851064</v>
+        <v>64.94834042553191</v>
       </c>
       <c r="Q12" t="b">
         <v>0</v>
       </c>
       <c r="R12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S12" t="b">
         <v>0</v>
@@ -4651,57 +4651,57 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>BHARATSE</t>
+          <t>FIEMIND</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Seating</t>
+          <t>Lighting</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>163.02</v>
+        <v>2161.3</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.0449352627570448</v>
+        <v>0.0100004673115565</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.0628880202345366</v>
+        <v>-0.0674404556437693</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.0256992589050919</v>
+        <v>0.0299752192146398</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0659998759595106</v>
+        <v>0.0577005977511212</v>
       </c>
       <c r="H13" t="n">
-        <v>0.0513436657530211</v>
+        <v>0.0717691259742541</v>
       </c>
       <c r="I13" t="n">
-        <v>47.6952277657267</v>
+        <v>61.93606214520467</v>
       </c>
       <c r="J13" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K13" t="n">
-        <v>52.61</v>
+        <v>49.06</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M13" t="n">
-        <v>52.61</v>
+        <v>49.06</v>
       </c>
       <c r="N13" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O13" t="n">
-        <v>59.57446808510638</v>
+        <v>63.82978723404256</v>
       </c>
       <c r="P13" t="n">
-        <v>56.95889361702128</v>
+        <v>64.38995744680851</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
@@ -4716,57 +4716,57 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>RANEENGINE</t>
+          <t>SUPRAJIT</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Engine/Parts</t>
+          <t>Cables</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>317.75</v>
+        <v>427.4</v>
       </c>
       <c r="D14" t="n">
-        <v>0.1790352504638219</v>
+        <v>0.0159258378892321</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.156154561147258</v>
+        <v>-0.0892819092265075</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.2401052253975846</v>
+        <v>-0.0513816446565309</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.148406090532982</v>
+        <v>-0.0236562661200495</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.1630623007394714</v>
+        <v>-0.009587737896916601</v>
       </c>
       <c r="I14" t="n">
-        <v>63.3225806451613</v>
+        <v>67.87196206283343</v>
       </c>
       <c r="J14" t="n">
         <v>80</v>
       </c>
       <c r="K14" t="n">
-        <v>50.88</v>
+        <v>51.48</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M14" t="n">
-        <v>50.88</v>
+        <v>51.48</v>
       </c>
       <c r="N14" t="n">
         <v>80</v>
       </c>
       <c r="O14" t="n">
-        <v>21.27659574468085</v>
+        <v>53.19148936170212</v>
       </c>
       <c r="P14" t="n">
-        <v>56.60731914893617</v>
+        <v>63.23029787234042</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
@@ -4781,57 +4781,57 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>GNA</t>
+          <t>CRAFTSMAN</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Axles</t>
+          <t>Castings</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>379.7</v>
+        <v>7351.5</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.1177973977695167</v>
+        <v>-0.009365314647621499</v>
       </c>
       <c r="E15" t="n">
-        <v>0.1012180974477958</v>
+        <v>-0.0835255251511563</v>
       </c>
       <c r="F15" t="n">
-        <v>0.2230632952166209</v>
+        <v>0.0893531895976884</v>
       </c>
       <c r="G15" t="n">
-        <v>0.3147624300812235</v>
+        <v>0.1170785681341698</v>
       </c>
       <c r="H15" t="n">
-        <v>0.300106219874734</v>
+        <v>0.1311470963573027</v>
       </c>
       <c r="I15" t="n">
-        <v>44.93295915185531</v>
+        <v>62.77992277992279</v>
       </c>
       <c r="J15" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K15" t="n">
-        <v>54.47</v>
+        <v>54.65</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M15" t="n">
-        <v>54.47</v>
+        <v>54.65</v>
       </c>
       <c r="N15" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O15" t="n">
-        <v>93.61702127659576</v>
+        <v>76.59574468085107</v>
       </c>
       <c r="P15" t="n">
-        <v>56.51140425531915</v>
+        <v>61.17914893617021</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
@@ -4846,63 +4846,63 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>SUPRAJIT</t>
+          <t>JBMA</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Cables</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>418.2</v>
+        <v>580.25</v>
       </c>
       <c r="D16" t="n">
-        <v>0.0140640155189137</v>
+        <v>0.1110579224509333</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.1208745007357577</v>
+        <v>-0.0940671350507416</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.0631720430107526</v>
+        <v>-0.1917960860784178</v>
       </c>
       <c r="G16" t="n">
-        <v>0.0285270918538499</v>
+        <v>-0.1640707075419364</v>
       </c>
       <c r="H16" t="n">
-        <v>0.0138708816473605</v>
+        <v>-0.1500021793188035</v>
       </c>
       <c r="I16" t="n">
-        <v>56.33059788980072</v>
+        <v>57.75136206042595</v>
       </c>
       <c r="J16" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K16" t="n">
-        <v>51.48</v>
+        <v>56.91</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M16" t="n">
-        <v>51.48</v>
+        <v>56.91</v>
       </c>
       <c r="N16" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O16" t="n">
-        <v>53.19148936170212</v>
+        <v>29.78723404255319</v>
       </c>
       <c r="P16" t="n">
-        <v>55.23029787234042</v>
+        <v>60.72144680851064</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>
       </c>
       <c r="R16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S16" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
chore: auto-refresh NSE data and pipeline outputs (2026-04-09)
</commit_message>
<xml_diff>
--- a/working-sector/output/auto_components_comprehensive_report.xlsx
+++ b/working-sector/output/auto_components_comprehensive_report.xlsx
@@ -435,7 +435,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
     </row>
@@ -447,7 +447,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
     </row>
@@ -779,25 +779,25 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1781.4</v>
+        <v>1739.4</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.0330040169362718</v>
+        <v>-0.0321072839574869</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2079745032888045</v>
+        <v>0.1725765134151273</v>
       </c>
       <c r="F2" t="n">
-        <v>0.4102279924002534</v>
+        <v>0.3711177676178465</v>
       </c>
       <c r="G2" t="n">
-        <v>0.4379533709367348</v>
+        <v>0.4070265988267989</v>
       </c>
       <c r="H2" t="n">
-        <v>0.4520218991598677</v>
+        <v>0.4208261579974242</v>
       </c>
       <c r="I2" t="n">
-        <v>58.97502601456814</v>
+        <v>53.27849588719154</v>
       </c>
       <c r="J2" t="n">
         <v>80</v>
@@ -807,7 +807,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M2" t="n">
@@ -844,25 +844,25 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1090.2</v>
+        <v>1054.6</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.0218034993270525</v>
+        <v>-0.0250531570675789</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.1746536452418805</v>
+        <v>-0.1999696555909574</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.1747785935962454</v>
+        <v>-0.1909474491752973</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.1470532150597641</v>
+        <v>-0.155038617966345</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.1329846868366312</v>
+        <v>-0.1412390587957197</v>
       </c>
       <c r="I3" t="n">
-        <v>57.73573390296002</v>
+        <v>48.1536628945801</v>
       </c>
       <c r="J3" t="n">
         <v>60</v>
@@ -872,7 +872,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M3" t="n">
@@ -882,10 +882,10 @@
         <v>60</v>
       </c>
       <c r="O3" t="n">
-        <v>36.17021276595745</v>
+        <v>25.53191489361702</v>
       </c>
       <c r="P3" t="n">
-        <v>50.97804255319149</v>
+        <v>48.8503829787234</v>
       </c>
       <c r="Q3" t="b">
         <v>0</v>
@@ -909,25 +909,25 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>35935</v>
+        <v>36770</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1201683291770574</v>
+        <v>0.1593883020652688</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.0776437371663244</v>
+        <v>-0.0606718610295057</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.0998246492985972</v>
+        <v>-0.0755499685732243</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.07209927076211579</v>
+        <v>-0.0396411373642719</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.0580307425389829</v>
+        <v>-0.0258415781936467</v>
       </c>
       <c r="I4" t="n">
-        <v>74.93551160791057</v>
+        <v>76.12612612612612</v>
       </c>
       <c r="J4" t="n">
         <v>70</v>
@@ -937,7 +937,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M4" t="n">
@@ -974,25 +974,25 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>314.15</v>
+        <v>311.25</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.0091468222677811</v>
+        <v>-0.0008025682182986</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.1364760857614074</v>
+        <v>-0.133973288814691</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.248804399808704</v>
+        <v>-0.2568051575931233</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.2210790212722226</v>
+        <v>-0.2208963263841709</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.2070104930490898</v>
+        <v>-0.2070967672135456</v>
       </c>
       <c r="I5" t="n">
-        <v>57.70676691729321</v>
+        <v>55.25030525030527</v>
       </c>
       <c r="J5" t="n">
         <v>60</v>
@@ -1002,7 +1002,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M5" t="n">
@@ -1012,10 +1012,10 @@
         <v>60</v>
       </c>
       <c r="O5" t="n">
-        <v>14.8936170212766</v>
+        <v>10.63829787234042</v>
       </c>
       <c r="P5" t="n">
-        <v>47.42672340425532</v>
+        <v>46.57565957446808</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
@@ -1039,25 +1039,25 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>118.11</v>
+        <v>116.9</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.042946276638846</v>
+        <v>-0.0369882197874618</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.0225109658197467</v>
+        <v>-0.0205278592375365</v>
       </c>
       <c r="F6" t="n">
-        <v>0.07480207480207469</v>
+        <v>0.0691421254801536</v>
       </c>
       <c r="G6" t="n">
-        <v>0.1025274533385561</v>
+        <v>0.105050956689106</v>
       </c>
       <c r="H6" t="n">
-        <v>0.116595981561689</v>
+        <v>0.1188505158597312</v>
       </c>
       <c r="I6" t="n">
-        <v>59.24418604651163</v>
+        <v>57.48942172073343</v>
       </c>
       <c r="J6" t="n">
         <v>60</v>
@@ -1067,7 +1067,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M6" t="n">
@@ -1104,25 +1104,25 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2727.1</v>
+        <v>2743.3</v>
       </c>
       <c r="D7" t="n">
-        <v>0.0313906433190878</v>
+        <v>0.06909586905689789</v>
       </c>
       <c r="E7" t="n">
-        <v>0.06987053746567271</v>
+        <v>0.0854237556382053</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.1989484196921631</v>
+        <v>-0.1900501919102449</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.1712230411556817</v>
+        <v>-0.1541413607012925</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.1571545129325489</v>
+        <v>-0.1403418015306673</v>
       </c>
       <c r="I7" t="n">
-        <v>64.69360369762936</v>
+        <v>65.1559741024132</v>
       </c>
       <c r="J7" t="n">
         <v>80</v>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M7" t="n">
@@ -1142,10 +1142,10 @@
         <v>80</v>
       </c>
       <c r="O7" t="n">
-        <v>25.53191489361702</v>
+        <v>27.65957446808511</v>
       </c>
       <c r="P7" t="n">
-        <v>56.59838297872341</v>
+        <v>57.02391489361703</v>
       </c>
       <c r="Q7" t="b">
         <v>0</v>
@@ -1169,25 +1169,25 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>533.7</v>
+        <v>523.05</v>
       </c>
       <c r="D8" t="n">
-        <v>0.0428920371275036</v>
+        <v>0.0129756947806718</v>
       </c>
       <c r="E8" t="n">
-        <v>0.1201595130653794</v>
+        <v>0.1039468130012661</v>
       </c>
       <c r="F8" t="n">
-        <v>0.2338457981736217</v>
+        <v>0.2035204786010123</v>
       </c>
       <c r="G8" t="n">
-        <v>0.2615711767101031</v>
+        <v>0.2394293098099646</v>
       </c>
       <c r="H8" t="n">
-        <v>0.275639704933236</v>
+        <v>0.2532288689805899</v>
       </c>
       <c r="I8" t="n">
-        <v>62.59899208063357</v>
+        <v>55.91549295774645</v>
       </c>
       <c r="J8" t="n">
         <v>80</v>
@@ -1197,7 +1197,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M8" t="n">
@@ -1207,10 +1207,10 @@
         <v>80</v>
       </c>
       <c r="O8" t="n">
-        <v>87.2340425531915</v>
+        <v>85.1063829787234</v>
       </c>
       <c r="P8" t="n">
-        <v>69.31080851063831</v>
+        <v>68.88527659574468</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
@@ -1234,25 +1234,25 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>436.1</v>
+        <v>440.35</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.003883051621745</v>
+        <v>0.0140472078295912</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.1605389797882579</v>
+        <v>-0.1491643319486039</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.1031362467866323</v>
+        <v>-0.0891508946116453</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.07541086825015091</v>
+        <v>-0.0532420634026929</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.0613423400270181</v>
+        <v>-0.0394425042320677</v>
       </c>
       <c r="I9" t="n">
-        <v>59.7197898423818</v>
+        <v>61.01694915254237</v>
       </c>
       <c r="J9" t="n">
         <v>60</v>
@@ -1262,7 +1262,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M9" t="n">
@@ -1299,25 +1299,25 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>133050</v>
+        <v>134020</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.0308482354226609</v>
+        <v>-0.0164030677773292</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.1141516029162089</v>
+        <v>-0.1073367302760848</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.1182318245079196</v>
+        <v>-0.1079012181321973</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.0905064459714383</v>
+        <v>-0.0719923869232449</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.0764379177483054</v>
+        <v>-0.0581928277526196</v>
       </c>
       <c r="I10" t="n">
-        <v>55.69188820722564</v>
+        <v>66.24092161282243</v>
       </c>
       <c r="J10" t="n">
         <v>60</v>
@@ -1327,7 +1327,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M10" t="n">
@@ -1376,10 +1376,10 @@
         <v>-0.0042030657656173</v>
       </c>
       <c r="G11" t="n">
-        <v>0.023522312770864</v>
+        <v>0.031705765443335</v>
       </c>
       <c r="H11" t="n">
-        <v>0.0375908409939969</v>
+        <v>0.0455053246139602</v>
       </c>
       <c r="I11" t="n">
         <v>27.6054590570719</v>
@@ -1392,7 +1392,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M11" t="n">
@@ -1402,10 +1402,10 @@
         <v>20</v>
       </c>
       <c r="O11" t="n">
-        <v>57.44680851063831</v>
+        <v>59.57446808510638</v>
       </c>
       <c r="P11" t="n">
-        <v>23.48936170212766</v>
+        <v>23.91489361702128</v>
       </c>
       <c r="Q11" t="b">
         <v>0</v>
@@ -1429,25 +1429,25 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>440.5</v>
+        <v>438.6</v>
       </c>
       <c r="D12" t="n">
-        <v>0.1185881157948196</v>
+        <v>0.08389966637835169</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.0717521862817406</v>
+        <v>-0.0646193218170184</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.1760194537972316</v>
+        <v>-0.1791896696921493</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.1482940752607502</v>
+        <v>-0.1432808384831969</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.1342255470376173</v>
+        <v>-0.1294812793125717</v>
       </c>
       <c r="I12" t="n">
-        <v>60.43747028055159</v>
+        <v>65.04605936540432</v>
       </c>
       <c r="J12" t="n">
         <v>80</v>
@@ -1457,7 +1457,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M12" t="n">
@@ -1494,25 +1494,25 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1713.1</v>
+        <v>1688.8</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.1118311903774368</v>
+        <v>-0.1099399177822283</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.1335727291118754</v>
+        <v>-0.143697393773451</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.0373138522056758</v>
+        <v>-0.0563781639380902</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.0095884736691944</v>
+        <v>-0.0204693327291378</v>
       </c>
       <c r="H13" t="n">
-        <v>0.0044800545539384</v>
+        <v>-0.0066697735585126</v>
       </c>
       <c r="I13" t="n">
-        <v>55.34240463975014</v>
+        <v>52.34557418807046</v>
       </c>
       <c r="J13" t="n">
         <v>60</v>
@@ -1522,7 +1522,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M13" t="n">
@@ -1532,16 +1532,16 @@
         <v>60</v>
       </c>
       <c r="O13" t="n">
-        <v>55.31914893617022</v>
+        <v>53.19148936170212</v>
       </c>
       <c r="P13" t="n">
-        <v>58.57182978723405</v>
+        <v>58.14629787234043</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
       </c>
       <c r="R13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S13" t="b">
         <v>0</v>
@@ -1559,25 +1559,25 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>573.9</v>
+        <v>566.25</v>
       </c>
       <c r="D14" t="n">
-        <v>0.0045510239803956</v>
+        <v>-0.0169270833333333</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.1780292179891149</v>
+        <v>-0.1846065231478149</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.168682552328529</v>
+        <v>-0.238655462184874</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.1409571737920476</v>
+        <v>-0.2027466309759216</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.1268886455689147</v>
+        <v>-0.1889470718052963</v>
       </c>
       <c r="I14" t="n">
-        <v>54.97780596068484</v>
+        <v>52.60535603072452</v>
       </c>
       <c r="J14" t="n">
         <v>60</v>
@@ -1587,7 +1587,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M14" t="n">
@@ -1597,10 +1597,10 @@
         <v>60</v>
       </c>
       <c r="O14" t="n">
-        <v>38.29787234042553</v>
+        <v>17.02127659574468</v>
       </c>
       <c r="P14" t="n">
-        <v>53.51557446808511</v>
+        <v>49.26025531914894</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
@@ -1624,25 +1624,25 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>98.94</v>
+        <v>99.45</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.0330336200156371</v>
+        <v>-0.0139797739440808</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.1055058312991592</v>
+        <v>-0.0851807561401893</v>
       </c>
       <c r="F15" t="n">
-        <v>0.1005561735261399</v>
+        <v>0.097197705207414</v>
       </c>
       <c r="G15" t="n">
-        <v>0.1282815520626213</v>
+        <v>0.1331065364163663</v>
       </c>
       <c r="H15" t="n">
-        <v>0.1423500802857542</v>
+        <v>0.1469060955869916</v>
       </c>
       <c r="I15" t="n">
-        <v>53.67316341829085</v>
+        <v>52.09302325581396</v>
       </c>
       <c r="J15" t="n">
         <v>60</v>
@@ -1652,7 +1652,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M15" t="n">
@@ -1689,25 +1689,25 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>176.72</v>
+        <v>176.74</v>
       </c>
       <c r="D16" t="n">
-        <v>0.004775983625199</v>
+        <v>0.0257094771052173</v>
       </c>
       <c r="E16" t="n">
-        <v>0.0193228355540173</v>
+        <v>0.0405039444248203</v>
       </c>
       <c r="F16" t="n">
-        <v>0.1117961623151935</v>
+        <v>0.1704635761589403</v>
       </c>
       <c r="G16" t="n">
-        <v>0.1395215408516749</v>
+        <v>0.2063724073678927</v>
       </c>
       <c r="H16" t="n">
-        <v>0.1535900690748077</v>
+        <v>0.220171966538518</v>
       </c>
       <c r="I16" t="n">
-        <v>63.04656262092092</v>
+        <v>61.80000000000001</v>
       </c>
       <c r="J16" t="n">
         <v>80</v>
@@ -1717,7 +1717,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M16" t="n">
@@ -1727,10 +1727,10 @@
         <v>80</v>
       </c>
       <c r="O16" t="n">
-        <v>80.85106382978722</v>
+        <v>82.97872340425532</v>
       </c>
       <c r="P16" t="n">
-        <v>69.21421276595744</v>
+        <v>69.63974468085107</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>
@@ -1754,48 +1754,48 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>7351.5</v>
+        <v>7408.5</v>
       </c>
       <c r="D17" t="n">
-        <v>-0.009365314647621499</v>
+        <v>0.01133028462221</v>
       </c>
       <c r="E17" t="n">
-        <v>-0.0835255251511563</v>
+        <v>-0.0509223674096848</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0893531895976884</v>
+        <v>0.08924501948099681</v>
       </c>
       <c r="G17" t="n">
-        <v>0.1170785681341698</v>
+        <v>0.1251538506899492</v>
       </c>
       <c r="H17" t="n">
-        <v>0.1311470963573027</v>
+        <v>0.1389534098605744</v>
       </c>
       <c r="I17" t="n">
         <v>62.77992277992279</v>
       </c>
       <c r="J17" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K17" t="n">
         <v>54.65</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M17" t="n">
         <v>54.65</v>
       </c>
       <c r="N17" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O17" t="n">
         <v>76.59574468085107</v>
       </c>
       <c r="P17" t="n">
-        <v>61.17914893617021</v>
+        <v>69.17914893617021</v>
       </c>
       <c r="Q17" t="b">
         <v>0</v>
@@ -1819,25 +1819,25 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>673.25</v>
+        <v>677.45</v>
       </c>
       <c r="D18" t="n">
-        <v>-0.0998729861621766</v>
+        <v>-0.0630661779959891</v>
       </c>
       <c r="E18" t="n">
-        <v>0.0887846688768496</v>
+        <v>0.120400231538907</v>
       </c>
       <c r="F18" t="n">
-        <v>0.0214686693976633</v>
+        <v>0.0304989351992699</v>
       </c>
       <c r="G18" t="n">
-        <v>0.0491940479341447</v>
+        <v>0.0664077664082223</v>
       </c>
       <c r="H18" t="n">
-        <v>0.06326257615727759</v>
+        <v>0.08020732557884749</v>
       </c>
       <c r="I18" t="n">
-        <v>48.40488381252461</v>
+        <v>44.12454681168694</v>
       </c>
       <c r="J18" t="n">
         <v>60</v>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M18" t="n">
@@ -1857,10 +1857,10 @@
         <v>60</v>
       </c>
       <c r="O18" t="n">
-        <v>59.57446808510638</v>
+        <v>61.70212765957447</v>
       </c>
       <c r="P18" t="n">
-        <v>55.88289361702128</v>
+        <v>56.3084255319149</v>
       </c>
       <c r="Q18" t="b">
         <v>0</v>
@@ -1884,25 +1884,25 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2359.1</v>
+        <v>2379.6</v>
       </c>
       <c r="D19" t="n">
-        <v>-0.0458645096056623</v>
+        <v>-0.042491549975857</v>
       </c>
       <c r="E19" t="n">
-        <v>-0.0818836349484335</v>
+        <v>-0.0845227561266496</v>
       </c>
       <c r="F19" t="n">
-        <v>-0.1926972828690711</v>
+        <v>-0.1738934212810275</v>
       </c>
       <c r="G19" t="n">
-        <v>-0.1649719043325898</v>
+        <v>-0.1379845900720752</v>
       </c>
       <c r="H19" t="n">
-        <v>-0.1509033761094569</v>
+        <v>-0.1241850309014499</v>
       </c>
       <c r="I19" t="n">
-        <v>57.36049601417182</v>
+        <v>58.55002583089372</v>
       </c>
       <c r="J19" t="n">
         <v>60</v>
@@ -1912,7 +1912,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M19" t="n">
@@ -1922,10 +1922,10 @@
         <v>60</v>
       </c>
       <c r="O19" t="n">
-        <v>27.65957446808511</v>
+        <v>38.29787234042553</v>
       </c>
       <c r="P19" t="n">
-        <v>50.03991489361702</v>
+        <v>52.16757446808511</v>
       </c>
       <c r="Q19" t="b">
         <v>0</v>
@@ -1949,25 +1949,25 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2161.3</v>
+        <v>2158.2</v>
       </c>
       <c r="D20" t="n">
-        <v>0.0100004673115565</v>
+        <v>0.02231064374023</v>
       </c>
       <c r="E20" t="n">
-        <v>-0.0674404556437693</v>
+        <v>-0.0914372316241476</v>
       </c>
       <c r="F20" t="n">
-        <v>0.0299752192146398</v>
+        <v>0.0660936573799642</v>
       </c>
       <c r="G20" t="n">
-        <v>0.0577005977511212</v>
+        <v>0.1020024885889165</v>
       </c>
       <c r="H20" t="n">
-        <v>0.0717691259742541</v>
+        <v>0.1158020477595418</v>
       </c>
       <c r="I20" t="n">
-        <v>61.93606214520467</v>
+        <v>60.1514215080346</v>
       </c>
       <c r="J20" t="n">
         <v>80</v>
@@ -1977,7 +1977,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M20" t="n">
@@ -1987,10 +1987,10 @@
         <v>80</v>
       </c>
       <c r="O20" t="n">
-        <v>63.82978723404256</v>
+        <v>68.08510638297872</v>
       </c>
       <c r="P20" t="n">
-        <v>64.38995744680851</v>
+        <v>65.24102127659575</v>
       </c>
       <c r="Q20" t="b">
         <v>0</v>
@@ -2014,48 +2014,48 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>918.95</v>
+        <v>907.2</v>
       </c>
       <c r="D21" t="n">
-        <v>0.0211690187798645</v>
+        <v>0.0261282660332542</v>
       </c>
       <c r="E21" t="n">
-        <v>-0.1203694840624102</v>
+        <v>-0.1212708252615265</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.3023458852110537</v>
+        <v>-0.3082202226628031</v>
       </c>
       <c r="G21" t="n">
-        <v>-0.2746205066745724</v>
+        <v>-0.2723113914538507</v>
       </c>
       <c r="H21" t="n">
-        <v>-0.2605519784514395</v>
+        <v>-0.2585118322832255</v>
       </c>
       <c r="I21" t="n">
-        <v>65.32614970175102</v>
+        <v>58.9231699939504</v>
       </c>
       <c r="J21" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K21" t="n">
         <v>48.43</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M21" t="n">
         <v>48.43</v>
       </c>
       <c r="N21" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O21" t="n">
         <v>6.382978723404255</v>
       </c>
       <c r="P21" t="n">
-        <v>52.64859574468085</v>
+        <v>44.64859574468085</v>
       </c>
       <c r="Q21" t="b">
         <v>0</v>
@@ -2079,25 +2079,25 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>409.75</v>
+        <v>409.65</v>
       </c>
       <c r="D22" t="n">
-        <v>-0.0416325575956029</v>
+        <v>-0.0271906910472572</v>
       </c>
       <c r="E22" t="n">
-        <v>0.0915023974427278</v>
+        <v>0.0656867845993756</v>
       </c>
       <c r="F22" t="n">
-        <v>0.314354450681636</v>
+        <v>0.3096227621483374</v>
       </c>
       <c r="G22" t="n">
-        <v>0.3420798292181174</v>
+        <v>0.3455315933572898</v>
       </c>
       <c r="H22" t="n">
-        <v>0.3561483574412503</v>
+        <v>0.359331152527915</v>
       </c>
       <c r="I22" t="n">
-        <v>58.62761986792995</v>
+        <v>60.09417304296643</v>
       </c>
       <c r="J22" t="n">
         <v>80</v>
@@ -2107,7 +2107,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M22" t="n">
@@ -2144,25 +2144,25 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>353.05</v>
+        <v>348.95</v>
       </c>
       <c r="D23" t="n">
-        <v>-0.009121526803255699</v>
+        <v>-0.0182866788577859</v>
       </c>
       <c r="E23" t="n">
-        <v>-0.1100327703554322</v>
+        <v>-0.1169176262178919</v>
       </c>
       <c r="F23" t="n">
-        <v>-0.1536617523672538</v>
+        <v>-0.1679780639008107</v>
       </c>
       <c r="G23" t="n">
-        <v>-0.1259363738307725</v>
+        <v>-0.1320692326918583</v>
       </c>
       <c r="H23" t="n">
-        <v>-0.1118678456076396</v>
+        <v>-0.118269673521233</v>
       </c>
       <c r="I23" t="n">
-        <v>55.7590076786769</v>
+        <v>54.85183033120276</v>
       </c>
       <c r="J23" t="n">
         <v>60</v>
@@ -2172,7 +2172,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M23" t="n">
@@ -2209,25 +2209,25 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>121.07</v>
+        <v>121.95</v>
       </c>
       <c r="D24" t="n">
-        <v>-0.0418645140867363</v>
+        <v>-0.0156590523851803</v>
       </c>
       <c r="E24" t="n">
-        <v>-0.1073508810735088</v>
+        <v>-0.0770453341406189</v>
       </c>
       <c r="F24" t="n">
-        <v>0.1197743248242693</v>
+        <v>0.1200404114621602</v>
       </c>
       <c r="G24" t="n">
-        <v>0.1474997033607507</v>
+        <v>0.1559492426711126</v>
       </c>
       <c r="H24" t="n">
-        <v>0.1615682315838835</v>
+        <v>0.1697488018417379</v>
       </c>
       <c r="I24" t="n">
-        <v>54.14614121510672</v>
+        <v>52.41746538871138</v>
       </c>
       <c r="J24" t="n">
         <v>60</v>
@@ -2237,7 +2237,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M24" t="n">
@@ -2247,10 +2247,10 @@
         <v>60</v>
       </c>
       <c r="O24" t="n">
-        <v>82.97872340425532</v>
+        <v>80.85106382978722</v>
       </c>
       <c r="P24" t="n">
-        <v>59.91574468085106</v>
+        <v>59.49021276595744</v>
       </c>
       <c r="Q24" t="b">
         <v>0</v>
@@ -2274,25 +2274,25 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>580.25</v>
+        <v>604.95</v>
       </c>
       <c r="D25" t="n">
-        <v>0.1110579224509333</v>
+        <v>0.1818892253589918</v>
       </c>
       <c r="E25" t="n">
-        <v>-0.0940671350507416</v>
+        <v>-0.09084761045987361</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.1917960860784178</v>
+        <v>-0.1780012229091649</v>
       </c>
       <c r="G25" t="n">
-        <v>-0.1640707075419364</v>
+        <v>-0.1420923917002126</v>
       </c>
       <c r="H25" t="n">
-        <v>-0.1500021793188035</v>
+        <v>-0.1282928325295873</v>
       </c>
       <c r="I25" t="n">
-        <v>57.75136206042595</v>
+        <v>59.04944791166589</v>
       </c>
       <c r="J25" t="n">
         <v>80</v>
@@ -2302,7 +2302,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M25" t="n">
@@ -2312,10 +2312,10 @@
         <v>80</v>
       </c>
       <c r="O25" t="n">
-        <v>29.78723404255319</v>
+        <v>36.17021276595745</v>
       </c>
       <c r="P25" t="n">
-        <v>60.72144680851064</v>
+        <v>61.99804255319149</v>
       </c>
       <c r="Q25" t="b">
         <v>0</v>
@@ -2339,25 +2339,25 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>133.21</v>
+        <v>130.94</v>
       </c>
       <c r="D26" t="n">
-        <v>-0.0045583619787773</v>
+        <v>-0.0373474489045729</v>
       </c>
       <c r="E26" t="n">
-        <v>-0.1639364840268624</v>
+        <v>-0.1775125628140703</v>
       </c>
       <c r="F26" t="n">
-        <v>-0.2276337913840087</v>
+        <v>-0.2459979269837613</v>
       </c>
       <c r="G26" t="n">
-        <v>-0.1999084128475273</v>
+        <v>-0.2100890957748089</v>
       </c>
       <c r="H26" t="n">
-        <v>-0.1858398846243945</v>
+        <v>-0.1962895366041837</v>
       </c>
       <c r="I26" t="n">
-        <v>57.96437659033079</v>
+        <v>54.44848484848485</v>
       </c>
       <c r="J26" t="n">
         <v>60</v>
@@ -2367,7 +2367,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M26" t="n">
@@ -2377,10 +2377,10 @@
         <v>60</v>
       </c>
       <c r="O26" t="n">
-        <v>19.14893617021277</v>
+        <v>12.76595744680851</v>
       </c>
       <c r="P26" t="n">
-        <v>48.44578723404256</v>
+        <v>47.1691914893617</v>
       </c>
       <c r="Q26" t="b">
         <v>0</v>
@@ -2404,25 +2404,25 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>5251</v>
+        <v>5304</v>
       </c>
       <c r="D27" t="n">
-        <v>0.0137065637065636</v>
+        <v>0.0127935841130417</v>
       </c>
       <c r="E27" t="n">
-        <v>-0.0608960028614862</v>
+        <v>-0.0519259987487711</v>
       </c>
       <c r="F27" t="n">
-        <v>0.2508337303477845</v>
+        <v>0.2074578277596923</v>
       </c>
       <c r="G27" t="n">
-        <v>0.2785591088842659</v>
+        <v>0.2433666589686447</v>
       </c>
       <c r="H27" t="n">
-        <v>0.2926276371073988</v>
+        <v>0.25716621813927</v>
       </c>
       <c r="I27" t="n">
-        <v>57.68773580029976</v>
+        <v>56.58836629725861</v>
       </c>
       <c r="J27" t="n">
         <v>60</v>
@@ -2432,7 +2432,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M27" t="n">
@@ -2442,10 +2442,10 @@
         <v>60</v>
       </c>
       <c r="O27" t="n">
-        <v>89.36170212765957</v>
+        <v>87.2340425531915</v>
       </c>
       <c r="P27" t="n">
-        <v>64.94834042553191</v>
+        <v>64.5228085106383</v>
       </c>
       <c r="Q27" t="b">
         <v>0</v>
@@ -2469,25 +2469,25 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1691.7</v>
+        <v>1725.6</v>
       </c>
       <c r="D28" t="n">
-        <v>0.1248753241571911</v>
+        <v>0.1735582154515775</v>
       </c>
       <c r="E28" t="n">
-        <v>0.0125089777352167</v>
+        <v>0.033479068096065</v>
       </c>
       <c r="F28" t="n">
-        <v>0.5525881057268724</v>
+        <v>0.5505436247641295</v>
       </c>
       <c r="G28" t="n">
-        <v>0.5803134842633538</v>
+        <v>0.5864524559730819</v>
       </c>
       <c r="H28" t="n">
-        <v>0.5943820124864867</v>
+        <v>0.6002520151437072</v>
       </c>
       <c r="I28" t="n">
-        <v>60.31914893617022</v>
+        <v>63.34236369793431</v>
       </c>
       <c r="J28" t="n">
         <v>80</v>
@@ -2497,7 +2497,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M28" t="n">
@@ -2507,10 +2507,10 @@
         <v>80</v>
       </c>
       <c r="O28" t="n">
-        <v>97.87234042553192</v>
+        <v>100</v>
       </c>
       <c r="P28" t="n">
-        <v>73.37846808510639</v>
+        <v>73.804</v>
       </c>
       <c r="Q28" t="b">
         <v>0</v>
@@ -2534,25 +2534,25 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>532.55</v>
+        <v>514.4</v>
       </c>
       <c r="D29" t="n">
-        <v>0.0502908983334975</v>
+        <v>0.0407688416793119</v>
       </c>
       <c r="E29" t="n">
-        <v>-0.1093736934526299</v>
+        <v>-0.1369127516778524</v>
       </c>
       <c r="F29" t="n">
-        <v>0.0280888030888029</v>
+        <v>-0.0326281147155618</v>
       </c>
       <c r="G29" t="n">
-        <v>0.0558141816252842</v>
+        <v>0.0032807164933905</v>
       </c>
       <c r="H29" t="n">
-        <v>0.0698827098484171</v>
+        <v>0.0170802756640158</v>
       </c>
       <c r="I29" t="n">
-        <v>59.66132446325973</v>
+        <v>53.27643171806167</v>
       </c>
       <c r="J29" t="n">
         <v>60</v>
@@ -2562,7 +2562,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M29" t="n">
@@ -2572,10 +2572,10 @@
         <v>60</v>
       </c>
       <c r="O29" t="n">
-        <v>61.70212765957447</v>
+        <v>57.44680851063831</v>
       </c>
       <c r="P29" t="n">
-        <v>56.1084255319149</v>
+        <v>55.25736170212766</v>
       </c>
       <c r="Q29" t="b">
         <v>0</v>
@@ -2599,48 +2599,48 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>113.62</v>
+        <v>114.05</v>
       </c>
       <c r="D30" t="n">
-        <v>-0.0540338023478477</v>
+        <v>-0.1004811104976733</v>
       </c>
       <c r="E30" t="n">
-        <v>-0.0091567105607395</v>
+        <v>-0.0610077391733904</v>
       </c>
       <c r="F30" t="n">
-        <v>-0.1337297956694113</v>
+        <v>-0.1215435569591004</v>
       </c>
       <c r="G30" t="n">
-        <v>-0.1060044171329299</v>
+        <v>-0.08563472575014799</v>
       </c>
       <c r="H30" t="n">
-        <v>-0.091935888909797</v>
+        <v>-0.0718351665795228</v>
       </c>
       <c r="I30" t="n">
-        <v>43.70979270907792</v>
+        <v>42.60204081632653</v>
       </c>
       <c r="J30" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K30" t="n">
         <v>52.38</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M30" t="n">
         <v>52.38</v>
       </c>
       <c r="N30" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O30" t="n">
-        <v>42.5531914893617</v>
+        <v>44.68085106382978</v>
       </c>
       <c r="P30" t="n">
-        <v>45.46263829787234</v>
+        <v>53.88817021276596</v>
       </c>
       <c r="Q30" t="b">
         <v>0</v>
@@ -2664,25 +2664,25 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>38.76</v>
+        <v>38.58</v>
       </c>
       <c r="D31" t="n">
-        <v>-0.04860088365243</v>
+        <v>-0.039820806371329</v>
       </c>
       <c r="E31" t="n">
-        <v>-0.2423768569194683</v>
+        <v>-0.2320859872611466</v>
       </c>
       <c r="F31" t="n">
-        <v>-0.2145896656534954</v>
+        <v>-0.2061728395061729</v>
       </c>
       <c r="G31" t="n">
-        <v>-0.186864287117014</v>
+        <v>-0.1702640082972205</v>
       </c>
       <c r="H31" t="n">
-        <v>-0.1727957588938812</v>
+        <v>-0.1564644491265953</v>
       </c>
       <c r="I31" t="n">
-        <v>58.01937567276639</v>
+        <v>58.71459694989108</v>
       </c>
       <c r="J31" t="n">
         <v>60</v>
@@ -2692,7 +2692,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M31" t="n">
@@ -2702,10 +2702,10 @@
         <v>60</v>
       </c>
       <c r="O31" t="n">
-        <v>21.27659574468085</v>
+        <v>23.40425531914894</v>
       </c>
       <c r="P31" t="n">
-        <v>47.85131914893617</v>
+        <v>48.27685106382979</v>
       </c>
       <c r="Q31" t="b">
         <v>0</v>
@@ -2729,25 +2729,25 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>716.6</v>
+        <v>715.35</v>
       </c>
       <c r="D32" t="n">
-        <v>-0.0058268590455049</v>
+        <v>0.0087428611718254</v>
       </c>
       <c r="E32" t="n">
-        <v>-0.1012166060454031</v>
+        <v>-0.086923224200651</v>
       </c>
       <c r="F32" t="n">
-        <v>-0.3518451519536902</v>
+        <v>-0.361009379187137</v>
       </c>
       <c r="G32" t="n">
-        <v>-0.3241197734172089</v>
+        <v>-0.3251005479781846</v>
       </c>
       <c r="H32" t="n">
-        <v>-0.310051245194076</v>
+        <v>-0.3113009888075594</v>
       </c>
       <c r="I32" t="n">
-        <v>56.80933852140078</v>
+        <v>56.02495543672015</v>
       </c>
       <c r="J32" t="n">
         <v>80</v>
@@ -2757,7 +2757,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M32" t="n">
@@ -2794,25 +2794,25 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>569.35</v>
+        <v>571.5</v>
       </c>
       <c r="D33" t="n">
-        <v>0.0147032614507218</v>
+        <v>0.0366406675131507</v>
       </c>
       <c r="E33" t="n">
-        <v>-0.1281010719754977</v>
+        <v>-0.1407953093287228</v>
       </c>
       <c r="F33" t="n">
-        <v>0.079745875213351</v>
+        <v>0.06992417860151651</v>
       </c>
       <c r="G33" t="n">
-        <v>0.1074712537498324</v>
+        <v>0.1058330098104689</v>
       </c>
       <c r="H33" t="n">
-        <v>0.1215397819729653</v>
+        <v>0.1196325689810942</v>
       </c>
       <c r="I33" t="n">
-        <v>60.8764186633039</v>
+        <v>61.90028222013171</v>
       </c>
       <c r="J33" t="n">
         <v>80</v>
@@ -2822,7 +2822,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M33" t="n">
@@ -2832,10 +2832,10 @@
         <v>80</v>
       </c>
       <c r="O33" t="n">
-        <v>74.46808510638297</v>
+        <v>72.3404255319149</v>
       </c>
       <c r="P33" t="n">
-        <v>66.8856170212766</v>
+        <v>66.46008510638299</v>
       </c>
       <c r="Q33" t="b">
         <v>0</v>
@@ -2871,10 +2871,10 @@
         <v>-0.2401052253975846</v>
       </c>
       <c r="G34" t="n">
-        <v>-0.2123798468611032</v>
+        <v>-0.2041963941886322</v>
       </c>
       <c r="H34" t="n">
-        <v>-0.1983113186379703</v>
+        <v>-0.1903968350180069</v>
       </c>
       <c r="I34" t="n">
         <v>63.3225806451613</v>
@@ -2887,7 +2887,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M34" t="n">
@@ -2897,10 +2897,10 @@
         <v>80</v>
       </c>
       <c r="O34" t="n">
-        <v>17.02127659574468</v>
+        <v>14.8936170212766</v>
       </c>
       <c r="P34" t="n">
-        <v>55.75625531914894</v>
+        <v>55.33072340425532</v>
       </c>
       <c r="Q34" t="b">
         <v>0</v>
@@ -2924,25 +2924,25 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>115.68</v>
+        <v>114.52</v>
       </c>
       <c r="D35" t="n">
-        <v>0.0337801608579089</v>
+        <v>0.0240543682375034</v>
       </c>
       <c r="E35" t="n">
-        <v>-0.0897072710103871</v>
+        <v>-0.1472822040208489</v>
       </c>
       <c r="F35" t="n">
-        <v>0.0777974471256872</v>
+        <v>0.07895232711513089</v>
       </c>
       <c r="G35" t="n">
-        <v>0.1055228256621686</v>
+        <v>0.1148611583240832</v>
       </c>
       <c r="H35" t="n">
-        <v>0.1195913538853015</v>
+        <v>0.1286607174947085</v>
       </c>
       <c r="I35" t="n">
-        <v>60.9297957266964</v>
+        <v>56.52173913043476</v>
       </c>
       <c r="J35" t="n">
         <v>60</v>
@@ -2952,7 +2952,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M35" t="n">
@@ -2962,10 +2962,10 @@
         <v>60</v>
       </c>
       <c r="O35" t="n">
-        <v>72.3404255319149</v>
+        <v>74.46808510638297</v>
       </c>
       <c r="P35" t="n">
-        <v>58.09608510638298</v>
+        <v>58.5216170212766</v>
       </c>
       <c r="Q35" t="b">
         <v>0</v>
@@ -2989,25 +2989,25 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>486.4</v>
+        <v>484.7</v>
       </c>
       <c r="D36" t="n">
-        <v>-0.032809703718433</v>
+        <v>-0.0417160933175168</v>
       </c>
       <c r="E36" t="n">
-        <v>-0.1578947368421053</v>
+        <v>-0.1716653849440313</v>
       </c>
       <c r="F36" t="n">
-        <v>0.0496331463098835</v>
+        <v>0.0349097896871997</v>
       </c>
       <c r="G36" t="n">
-        <v>0.07735852484636491</v>
+        <v>0.0708186208961521</v>
       </c>
       <c r="H36" t="n">
-        <v>0.0914270530694978</v>
+        <v>0.08461818006677729</v>
       </c>
       <c r="I36" t="n">
-        <v>55.15484123872992</v>
+        <v>52.9552715654952</v>
       </c>
       <c r="J36" t="n">
         <v>60</v>
@@ -3017,7 +3017,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M36" t="n">
@@ -3027,10 +3027,10 @@
         <v>60</v>
       </c>
       <c r="O36" t="n">
-        <v>65.95744680851064</v>
+        <v>63.82978723404256</v>
       </c>
       <c r="P36" t="n">
-        <v>56.31148936170213</v>
+        <v>55.88595744680852</v>
       </c>
       <c r="Q36" t="b">
         <v>0</v>
@@ -3054,25 +3054,25 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2248.1</v>
+        <v>2251.7</v>
       </c>
       <c r="D37" t="n">
-        <v>0.0290671061063809</v>
+        <v>0.0339808054369288</v>
       </c>
       <c r="E37" t="n">
-        <v>0.1677834917666614</v>
+        <v>0.1575673452601274</v>
       </c>
       <c r="F37" t="n">
-        <v>0.5730879574557415</v>
+        <v>0.4941605839416056</v>
       </c>
       <c r="G37" t="n">
-        <v>0.6008133359922229</v>
+        <v>0.5300694151505581</v>
       </c>
       <c r="H37" t="n">
-        <v>0.6148818642153557</v>
+        <v>0.5438689743211833</v>
       </c>
       <c r="I37" t="n">
-        <v>59.29697766097239</v>
+        <v>56.48050579557426</v>
       </c>
       <c r="J37" t="n">
         <v>80</v>
@@ -3082,7 +3082,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M37" t="n">
@@ -3092,10 +3092,10 @@
         <v>80</v>
       </c>
       <c r="O37" t="n">
-        <v>100</v>
+        <v>97.87234042553192</v>
       </c>
       <c r="P37" t="n">
-        <v>71.43600000000001</v>
+        <v>71.0104680851064</v>
       </c>
       <c r="Q37" t="b">
         <v>0</v>
@@ -3119,25 +3119,25 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>802.2</v>
+        <v>822.75</v>
       </c>
       <c r="D38" t="n">
-        <v>-0.0348312578956866</v>
+        <v>0.0037821021167572</v>
       </c>
       <c r="E38" t="n">
-        <v>-0.1580162686958802</v>
+        <v>-0.1313872466216217</v>
       </c>
       <c r="F38" t="n">
-        <v>-0.2519582245430809</v>
+        <v>-0.2243329876496653</v>
       </c>
       <c r="G38" t="n">
-        <v>-0.2242328460065995</v>
+        <v>-0.1884241564407129</v>
       </c>
       <c r="H38" t="n">
-        <v>-0.2101643177834666</v>
+        <v>-0.1746245972700877</v>
       </c>
       <c r="I38" t="n">
-        <v>52.30985420692079</v>
+        <v>56.01652892561984</v>
       </c>
       <c r="J38" t="n">
         <v>60</v>
@@ -3147,7 +3147,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M38" t="n">
@@ -3157,10 +3157,10 @@
         <v>60</v>
       </c>
       <c r="O38" t="n">
-        <v>12.76595744680851</v>
+        <v>19.14893617021277</v>
       </c>
       <c r="P38" t="n">
-        <v>46.5011914893617</v>
+        <v>47.77778723404256</v>
       </c>
       <c r="Q38" t="b">
         <v>0</v>
@@ -3184,25 +3184,25 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>3130.9</v>
+        <v>3223.7</v>
       </c>
       <c r="D39" t="n">
-        <v>0.0339145366884618</v>
+        <v>0.0605322893706616</v>
       </c>
       <c r="E39" t="n">
-        <v>-0.0614526814352948</v>
+        <v>-0.0446597913703177</v>
       </c>
       <c r="F39" t="n">
-        <v>0.1742489592318943</v>
+        <v>0.2131486847552024</v>
       </c>
       <c r="G39" t="n">
-        <v>0.2019743377683757</v>
+        <v>0.2490575159641548</v>
       </c>
       <c r="H39" t="n">
-        <v>0.2160428659915085</v>
+        <v>0.26285707513478</v>
       </c>
       <c r="I39" t="n">
-        <v>60.13812452789469</v>
+        <v>55.89253731343283</v>
       </c>
       <c r="J39" t="n">
         <v>80</v>
@@ -3212,7 +3212,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M39" t="n">
@@ -3222,10 +3222,10 @@
         <v>80</v>
       </c>
       <c r="O39" t="n">
-        <v>85.1063829787234</v>
+        <v>89.36170212765957</v>
       </c>
       <c r="P39" t="n">
-        <v>68.49727659574468</v>
+        <v>69.34834042553192</v>
       </c>
       <c r="Q39" t="b">
         <v>0</v>
@@ -3249,25 +3249,25 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>201.5</v>
+        <v>203.24</v>
       </c>
       <c r="D40" t="n">
-        <v>0.0483870967741935</v>
+        <v>0.0399099467867376</v>
       </c>
       <c r="E40" t="n">
-        <v>-0.0562060889929741</v>
+        <v>-0.0524058187243564</v>
       </c>
       <c r="F40" t="n">
-        <v>-0.1763744124259145</v>
+        <v>-0.1801532876159741</v>
       </c>
       <c r="G40" t="n">
-        <v>-0.1486490338894331</v>
+        <v>-0.1442444564070217</v>
       </c>
       <c r="H40" t="n">
-        <v>-0.1345805056663003</v>
+        <v>-0.1304448972363965</v>
       </c>
       <c r="I40" t="n">
-        <v>67.86858974358975</v>
+        <v>65.35936420179684</v>
       </c>
       <c r="J40" t="n">
         <v>80</v>
@@ -3277,7 +3277,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M40" t="n">
@@ -3287,10 +3287,10 @@
         <v>80</v>
       </c>
       <c r="O40" t="n">
-        <v>31.91489361702128</v>
+        <v>29.78723404255319</v>
       </c>
       <c r="P40" t="n">
-        <v>56.55897872340426</v>
+        <v>56.13344680851064</v>
       </c>
       <c r="Q40" t="b">
         <v>0</v>
@@ -3314,25 +3314,25 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>780.25</v>
+        <v>780.85</v>
       </c>
       <c r="D41" t="n">
-        <v>-0.0752044565603887</v>
+        <v>-0.06647139697531231</v>
       </c>
       <c r="E41" t="n">
-        <v>-0.1691070763005164</v>
+        <v>-0.18029603191266</v>
       </c>
       <c r="F41" t="n">
-        <v>-0.2596546161874941</v>
+        <v>-0.2599981046247157</v>
       </c>
       <c r="G41" t="n">
-        <v>-0.2319292376510127</v>
+        <v>-0.2240892734157633</v>
       </c>
       <c r="H41" t="n">
-        <v>-0.2178607094278798</v>
+        <v>-0.2102897142451381</v>
       </c>
       <c r="I41" t="n">
-        <v>37.80573025856047</v>
+        <v>38.64358883786651</v>
       </c>
       <c r="J41" t="n">
         <v>30</v>
@@ -3342,7 +3342,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M41" t="n">
@@ -3352,10 +3352,10 @@
         <v>30</v>
       </c>
       <c r="O41" t="n">
-        <v>10.63829787234042</v>
+        <v>8.51063829787234</v>
       </c>
       <c r="P41" t="n">
-        <v>33.34765957446808</v>
+        <v>32.92212765957446</v>
       </c>
       <c r="Q41" t="b">
         <v>0</v>
@@ -3379,48 +3379,48 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>561.1</v>
+        <v>628.85</v>
       </c>
       <c r="D42" t="n">
-        <v>-0.0220479302832243</v>
+        <v>0.1107480349730638</v>
       </c>
       <c r="E42" t="n">
-        <v>-0.1818910840562805</v>
+        <v>-0.0945284377249819</v>
       </c>
       <c r="F42" t="n">
-        <v>-0.2675890875864769</v>
+        <v>-0.1801173402868318</v>
       </c>
       <c r="G42" t="n">
-        <v>-0.2398637090499955</v>
+        <v>-0.1442085090778794</v>
       </c>
       <c r="H42" t="n">
-        <v>-0.2257951808268626</v>
+        <v>-0.1304089499072541</v>
       </c>
       <c r="I42" t="n">
-        <v>56.5080135988344</v>
+        <v>68.36242109171927</v>
       </c>
       <c r="J42" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K42" t="n">
         <v>47.66</v>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M42" t="n">
         <v>47.66</v>
       </c>
       <c r="N42" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O42" t="n">
-        <v>8.51063829787234</v>
+        <v>31.91489361702128</v>
       </c>
       <c r="P42" t="n">
-        <v>44.76612765957447</v>
+        <v>57.44697872340426</v>
       </c>
       <c r="Q42" t="b">
         <v>0</v>
@@ -3444,25 +3444,25 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>427.4</v>
+        <v>431.75</v>
       </c>
       <c r="D43" t="n">
-        <v>0.0159258378892321</v>
+        <v>0.0279761904761903</v>
       </c>
       <c r="E43" t="n">
-        <v>-0.0892819092265075</v>
+        <v>-0.07676681278734079</v>
       </c>
       <c r="F43" t="n">
-        <v>-0.0513816446565309</v>
+        <v>-0.05005500550055</v>
       </c>
       <c r="G43" t="n">
-        <v>-0.0236562661200495</v>
+        <v>-0.0141461742915977</v>
       </c>
       <c r="H43" t="n">
-        <v>-0.009587737896916601</v>
+        <v>-0.0003466151209724</v>
       </c>
       <c r="I43" t="n">
-        <v>67.87196206283343</v>
+        <v>67.50599520383693</v>
       </c>
       <c r="J43" t="n">
         <v>80</v>
@@ -3472,7 +3472,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M43" t="n">
@@ -3482,10 +3482,10 @@
         <v>80</v>
       </c>
       <c r="O43" t="n">
-        <v>53.19148936170212</v>
+        <v>55.31914893617022</v>
       </c>
       <c r="P43" t="n">
-        <v>63.23029787234042</v>
+        <v>63.65582978723404</v>
       </c>
       <c r="Q43" t="b">
         <v>0</v>
@@ -3509,48 +3509,48 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>253.91</v>
+        <v>258.44</v>
       </c>
       <c r="D44" t="n">
-        <v>0.0279757085020242</v>
+        <v>0.067272351848028</v>
       </c>
       <c r="E44" t="n">
-        <v>-0.0630627306273062</v>
+        <v>-0.0372881355932203</v>
       </c>
       <c r="F44" t="n">
-        <v>-0.1328210382513661</v>
+        <v>-0.123189143341815</v>
       </c>
       <c r="G44" t="n">
-        <v>-0.1050956597148847</v>
+        <v>-0.08728031213286259</v>
       </c>
       <c r="H44" t="n">
-        <v>-0.0910271314917519</v>
+        <v>-0.0734807529622374</v>
       </c>
       <c r="I44" t="n">
-        <v>66.15279205207261</v>
+        <v>67.82283015795473</v>
       </c>
       <c r="J44" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K44" t="n">
         <v>47.2</v>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M44" t="n">
         <v>47.2</v>
       </c>
       <c r="N44" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O44" t="n">
-        <v>44.68085106382978</v>
+        <v>42.5531914893617</v>
       </c>
       <c r="P44" t="n">
-        <v>51.81617021276596</v>
+        <v>59.39063829787234</v>
       </c>
       <c r="Q44" t="b">
         <v>0</v>
@@ -3574,25 +3574,25 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>96.31999999999999</v>
+        <v>94.26000000000001</v>
       </c>
       <c r="D45" t="n">
-        <v>-0.0385306448392893</v>
+        <v>-0.0651591788158285</v>
       </c>
       <c r="E45" t="n">
-        <v>-0.1406138472519629</v>
+        <v>-0.1468139029688631</v>
       </c>
       <c r="F45" t="n">
-        <v>-0.3058518304987028</v>
+        <v>-0.3420813847979339</v>
       </c>
       <c r="G45" t="n">
-        <v>-0.2781264519622214</v>
+        <v>-0.3061725535889815</v>
       </c>
       <c r="H45" t="n">
-        <v>-0.2640579237390885</v>
+        <v>-0.2923729944183563</v>
       </c>
       <c r="I45" t="n">
-        <v>48.97838318033756</v>
+        <v>45.60067681895093</v>
       </c>
       <c r="J45" t="n">
         <v>60</v>
@@ -3602,7 +3602,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M45" t="n">
@@ -3639,25 +3639,25 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>500.4</v>
+        <v>499.7</v>
       </c>
       <c r="D46" t="n">
-        <v>0.0049201727081031</v>
+        <v>0.0108222918984524</v>
       </c>
       <c r="E46" t="n">
-        <v>-0.189110354885756</v>
+        <v>-0.170209232813019</v>
       </c>
       <c r="F46" t="n">
-        <v>-0.2071615305394913</v>
+        <v>-0.2221962798661375</v>
       </c>
       <c r="G46" t="n">
-        <v>-0.17943615200301</v>
+        <v>-0.1862874486571851</v>
       </c>
       <c r="H46" t="n">
-        <v>-0.1653676237798771</v>
+        <v>-0.1724878894865599</v>
       </c>
       <c r="I46" t="n">
-        <v>48.83051457358763</v>
+        <v>50.55886736214605</v>
       </c>
       <c r="J46" t="n">
         <v>60</v>
@@ -3667,7 +3667,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M46" t="n">
@@ -3677,10 +3677,10 @@
         <v>60</v>
       </c>
       <c r="O46" t="n">
-        <v>23.40425531914894</v>
+        <v>21.27659574468085</v>
       </c>
       <c r="P46" t="n">
-        <v>48.52485106382979</v>
+        <v>48.09931914893617</v>
       </c>
       <c r="Q46" t="b">
         <v>0</v>
@@ -3704,25 +3704,25 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>991.9</v>
+        <v>1001.35</v>
       </c>
       <c r="D47" t="n">
-        <v>0.0690881655529209</v>
+        <v>0.0903794849458268</v>
       </c>
       <c r="E47" t="n">
-        <v>0.1271590909090909</v>
+        <v>0.1397757668886234</v>
       </c>
       <c r="F47" t="n">
-        <v>0.2530318342597271</v>
+        <v>0.2329618912762421</v>
       </c>
       <c r="G47" t="n">
-        <v>0.2807572127962084</v>
+        <v>0.2688707224851945</v>
       </c>
       <c r="H47" t="n">
-        <v>0.2948257410193413</v>
+        <v>0.2826702816558197</v>
       </c>
       <c r="I47" t="n">
-        <v>50.1790739319519</v>
+        <v>46.44575828406435</v>
       </c>
       <c r="J47" t="n">
         <v>80</v>
@@ -3732,7 +3732,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M47" t="n">
@@ -3769,25 +3769,25 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>14439</v>
+        <v>14248</v>
       </c>
       <c r="D48" t="n">
-        <v>0.0317256162915327</v>
+        <v>0.018878718535469</v>
       </c>
       <c r="E48" t="n">
-        <v>-0.0562128243676057</v>
+        <v>-0.0425374638801155</v>
       </c>
       <c r="F48" t="n">
-        <v>0.051485581124381</v>
+        <v>0.0502727406752174</v>
       </c>
       <c r="G48" t="n">
-        <v>0.0792109596608624</v>
+        <v>0.08618157188416981</v>
       </c>
       <c r="H48" t="n">
-        <v>0.0932794878839953</v>
+        <v>0.0999811310547951</v>
       </c>
       <c r="I48" t="n">
-        <v>64.13422818791946</v>
+        <v>56.38389031705226</v>
       </c>
       <c r="J48" t="n">
         <v>60</v>
@@ -3797,7 +3797,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M48" t="n">
@@ -3807,10 +3807,10 @@
         <v>60</v>
       </c>
       <c r="O48" t="n">
-        <v>68.08510638297872</v>
+        <v>65.95744680851064</v>
       </c>
       <c r="P48" t="n">
-        <v>57.73302127659574</v>
+        <v>57.30748936170212</v>
       </c>
       <c r="Q48" t="b">
         <v>0</v>
@@ -3945,25 +3945,25 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1691.7</v>
+        <v>1725.6</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1248753241571911</v>
+        <v>0.1735582154515775</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0125089777352167</v>
+        <v>0.033479068096065</v>
       </c>
       <c r="F2" t="n">
-        <v>0.5525881057268724</v>
+        <v>0.5505436247641295</v>
       </c>
       <c r="G2" t="n">
-        <v>0.5803134842633538</v>
+        <v>0.5864524559730819</v>
       </c>
       <c r="H2" t="n">
-        <v>0.5943820124864867</v>
+        <v>0.6002520151437072</v>
       </c>
       <c r="I2" t="n">
-        <v>60.31914893617022</v>
+        <v>63.34236369793431</v>
       </c>
       <c r="J2" t="n">
         <v>80</v>
@@ -3973,7 +3973,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M2" t="n">
@@ -3983,10 +3983,10 @@
         <v>80</v>
       </c>
       <c r="O2" t="n">
-        <v>97.87234042553192</v>
+        <v>100</v>
       </c>
       <c r="P2" t="n">
-        <v>73.37846808510639</v>
+        <v>73.804</v>
       </c>
       <c r="Q2" t="b">
         <v>0</v>
@@ -4010,25 +4010,25 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1781.4</v>
+        <v>1739.4</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.0330040169362718</v>
+        <v>-0.0321072839574869</v>
       </c>
       <c r="E3" t="n">
-        <v>0.2079745032888045</v>
+        <v>0.1725765134151273</v>
       </c>
       <c r="F3" t="n">
-        <v>0.4102279924002534</v>
+        <v>0.3711177676178465</v>
       </c>
       <c r="G3" t="n">
-        <v>0.4379533709367348</v>
+        <v>0.4070265988267989</v>
       </c>
       <c r="H3" t="n">
-        <v>0.4520218991598677</v>
+        <v>0.4208261579974242</v>
       </c>
       <c r="I3" t="n">
-        <v>58.97502601456814</v>
+        <v>53.27849588719154</v>
       </c>
       <c r="J3" t="n">
         <v>80</v>
@@ -4038,7 +4038,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M3" t="n">
@@ -4075,25 +4075,25 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>409.75</v>
+        <v>409.65</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.0416325575956029</v>
+        <v>-0.0271906910472572</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0915023974427278</v>
+        <v>0.0656867845993756</v>
       </c>
       <c r="F4" t="n">
-        <v>0.314354450681636</v>
+        <v>0.3096227621483374</v>
       </c>
       <c r="G4" t="n">
-        <v>0.3420798292181174</v>
+        <v>0.3455315933572898</v>
       </c>
       <c r="H4" t="n">
-        <v>0.3561483574412503</v>
+        <v>0.359331152527915</v>
       </c>
       <c r="I4" t="n">
-        <v>58.62761986792995</v>
+        <v>60.09417304296643</v>
       </c>
       <c r="J4" t="n">
         <v>80</v>
@@ -4103,7 +4103,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M4" t="n">
@@ -4140,25 +4140,25 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>2248.1</v>
+        <v>2251.7</v>
       </c>
       <c r="D5" t="n">
-        <v>0.0290671061063809</v>
+        <v>0.0339808054369288</v>
       </c>
       <c r="E5" t="n">
-        <v>0.1677834917666614</v>
+        <v>0.1575673452601274</v>
       </c>
       <c r="F5" t="n">
-        <v>0.5730879574557415</v>
+        <v>0.4941605839416056</v>
       </c>
       <c r="G5" t="n">
-        <v>0.6008133359922229</v>
+        <v>0.5300694151505581</v>
       </c>
       <c r="H5" t="n">
-        <v>0.6148818642153557</v>
+        <v>0.5438689743211833</v>
       </c>
       <c r="I5" t="n">
-        <v>59.29697766097239</v>
+        <v>56.48050579557426</v>
       </c>
       <c r="J5" t="n">
         <v>80</v>
@@ -4168,7 +4168,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M5" t="n">
@@ -4178,10 +4178,10 @@
         <v>80</v>
       </c>
       <c r="O5" t="n">
-        <v>100</v>
+        <v>97.87234042553192</v>
       </c>
       <c r="P5" t="n">
-        <v>71.43600000000001</v>
+        <v>71.0104680851064</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
@@ -4196,57 +4196,57 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>BHARATSE</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Seating</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>533.7</v>
+        <v>176.74</v>
       </c>
       <c r="D6" t="n">
-        <v>0.0428920371275036</v>
+        <v>0.0257094771052173</v>
       </c>
       <c r="E6" t="n">
-        <v>0.1201595130653794</v>
+        <v>0.0405039444248203</v>
       </c>
       <c r="F6" t="n">
-        <v>0.2338457981736217</v>
+        <v>0.1704635761589403</v>
       </c>
       <c r="G6" t="n">
-        <v>0.2615711767101031</v>
+        <v>0.2063724073678927</v>
       </c>
       <c r="H6" t="n">
-        <v>0.275639704933236</v>
+        <v>0.220171966538518</v>
       </c>
       <c r="I6" t="n">
-        <v>62.59899208063357</v>
+        <v>61.80000000000001</v>
       </c>
       <c r="J6" t="n">
         <v>80</v>
       </c>
       <c r="K6" t="n">
-        <v>49.66</v>
+        <v>52.61</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M6" t="n">
-        <v>49.66</v>
+        <v>52.61</v>
       </c>
       <c r="N6" t="n">
         <v>80</v>
       </c>
       <c r="O6" t="n">
-        <v>87.2340425531915</v>
+        <v>82.97872340425532</v>
       </c>
       <c r="P6" t="n">
-        <v>69.31080851063831</v>
+        <v>69.63974468085107</v>
       </c>
       <c r="Q6" t="b">
         <v>0</v>
@@ -4261,57 +4261,57 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BHARATSE</t>
+          <t>SHRIPISTON</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Seating</t>
+          <t>Engine/Parts</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>176.72</v>
+        <v>3223.7</v>
       </c>
       <c r="D7" t="n">
-        <v>0.004775983625199</v>
+        <v>0.0605322893706616</v>
       </c>
       <c r="E7" t="n">
-        <v>0.0193228355540173</v>
+        <v>-0.0446597913703177</v>
       </c>
       <c r="F7" t="n">
-        <v>0.1117961623151935</v>
+        <v>0.2131486847552024</v>
       </c>
       <c r="G7" t="n">
-        <v>0.1395215408516749</v>
+        <v>0.2490575159641548</v>
       </c>
       <c r="H7" t="n">
-        <v>0.1535900690748077</v>
+        <v>0.26285707513478</v>
       </c>
       <c r="I7" t="n">
-        <v>63.04656262092092</v>
+        <v>55.89253731343283</v>
       </c>
       <c r="J7" t="n">
         <v>80</v>
       </c>
       <c r="K7" t="n">
-        <v>52.61</v>
+        <v>48.69</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M7" t="n">
-        <v>52.61</v>
+        <v>48.69</v>
       </c>
       <c r="N7" t="n">
         <v>80</v>
       </c>
       <c r="O7" t="n">
-        <v>80.85106382978722</v>
+        <v>89.36170212765957</v>
       </c>
       <c r="P7" t="n">
-        <v>69.21421276595744</v>
+        <v>69.34834042553192</v>
       </c>
       <c r="Q7" t="b">
         <v>0</v>
@@ -4326,57 +4326,57 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>WHEELS</t>
+          <t>CRAFTSMAN</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Wheels</t>
+          <t>Castings</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>991.9</v>
+        <v>7408.5</v>
       </c>
       <c r="D8" t="n">
-        <v>0.0690881655529209</v>
+        <v>0.01133028462221</v>
       </c>
       <c r="E8" t="n">
-        <v>0.1271590909090909</v>
+        <v>-0.0509223674096848</v>
       </c>
       <c r="F8" t="n">
-        <v>0.2530318342597271</v>
+        <v>0.08924501948099681</v>
       </c>
       <c r="G8" t="n">
-        <v>0.2807572127962084</v>
+        <v>0.1251538506899492</v>
       </c>
       <c r="H8" t="n">
-        <v>0.2948257410193413</v>
+        <v>0.1389534098605744</v>
       </c>
       <c r="I8" t="n">
-        <v>50.1790739319519</v>
+        <v>62.77992277992279</v>
       </c>
       <c r="J8" t="n">
         <v>80</v>
       </c>
       <c r="K8" t="n">
-        <v>46.83</v>
+        <v>54.65</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M8" t="n">
-        <v>46.83</v>
+        <v>54.65</v>
       </c>
       <c r="N8" t="n">
         <v>80</v>
       </c>
       <c r="O8" t="n">
-        <v>91.48936170212764</v>
+        <v>76.59574468085107</v>
       </c>
       <c r="P8" t="n">
-        <v>69.02987234042553</v>
+        <v>69.17914893617021</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
@@ -4391,57 +4391,57 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SHRIPISTON</t>
+          <t>WHEELS</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Engine/Parts</t>
+          <t>Wheels</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>3130.9</v>
+        <v>1001.35</v>
       </c>
       <c r="D9" t="n">
-        <v>0.0339145366884618</v>
+        <v>0.0903794849458268</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.0614526814352948</v>
+        <v>0.1397757668886234</v>
       </c>
       <c r="F9" t="n">
-        <v>0.1742489592318943</v>
+        <v>0.2329618912762421</v>
       </c>
       <c r="G9" t="n">
-        <v>0.2019743377683757</v>
+        <v>0.2688707224851945</v>
       </c>
       <c r="H9" t="n">
-        <v>0.2160428659915085</v>
+        <v>0.2826702816558197</v>
       </c>
       <c r="I9" t="n">
-        <v>60.13812452789469</v>
+        <v>46.44575828406435</v>
       </c>
       <c r="J9" t="n">
         <v>80</v>
       </c>
       <c r="K9" t="n">
-        <v>48.69</v>
+        <v>46.83</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M9" t="n">
-        <v>48.69</v>
+        <v>46.83</v>
       </c>
       <c r="N9" t="n">
         <v>80</v>
       </c>
       <c r="O9" t="n">
-        <v>85.1063829787234</v>
+        <v>91.48936170212764</v>
       </c>
       <c r="P9" t="n">
-        <v>68.49727659574468</v>
+        <v>69.02987234042553</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -4456,63 +4456,63 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ASKAUTOLTD</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>440.5</v>
+        <v>523.05</v>
       </c>
       <c r="D10" t="n">
-        <v>0.1185881157948196</v>
+        <v>0.0129756947806718</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.0717521862817406</v>
+        <v>0.1039468130012661</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.1760194537972316</v>
+        <v>0.2035204786010123</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.1482940752607502</v>
+        <v>0.2394293098099646</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.1342255470376173</v>
+        <v>0.2532288689805899</v>
       </c>
       <c r="I10" t="n">
-        <v>60.43747028055159</v>
+        <v>55.91549295774645</v>
       </c>
       <c r="J10" t="n">
         <v>80</v>
       </c>
       <c r="K10" t="n">
-        <v>71.28</v>
+        <v>49.66</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M10" t="n">
-        <v>71.28</v>
+        <v>49.66</v>
       </c>
       <c r="N10" t="n">
         <v>80</v>
       </c>
       <c r="O10" t="n">
-        <v>34.04255319148936</v>
+        <v>85.1063829787234</v>
       </c>
       <c r="P10" t="n">
-        <v>67.32051063829788</v>
+        <v>68.88527659574468</v>
       </c>
       <c r="Q10" t="b">
+        <v>0</v>
+      </c>
+      <c r="R10" t="b">
         <v>1</v>
-      </c>
-      <c r="R10" t="b">
-        <v>0</v>
       </c>
       <c r="S10" t="b">
         <v>0</v>
@@ -4521,63 +4521,63 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>PRICOLLTD</t>
+          <t>ASKAUTOLTD</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>569.35</v>
+        <v>438.6</v>
       </c>
       <c r="D11" t="n">
-        <v>0.0147032614507218</v>
+        <v>0.08389966637835169</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.1281010719754977</v>
+        <v>-0.0646193218170184</v>
       </c>
       <c r="F11" t="n">
-        <v>0.079745875213351</v>
+        <v>-0.1791896696921493</v>
       </c>
       <c r="G11" t="n">
-        <v>0.1074712537498324</v>
+        <v>-0.1432808384831969</v>
       </c>
       <c r="H11" t="n">
-        <v>0.1215397819729653</v>
+        <v>-0.1294812793125717</v>
       </c>
       <c r="I11" t="n">
-        <v>60.8764186633039</v>
+        <v>65.04605936540432</v>
       </c>
       <c r="J11" t="n">
         <v>80</v>
       </c>
       <c r="K11" t="n">
-        <v>49.98</v>
+        <v>71.28</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M11" t="n">
-        <v>49.98</v>
+        <v>71.28</v>
       </c>
       <c r="N11" t="n">
         <v>80</v>
       </c>
       <c r="O11" t="n">
-        <v>74.46808510638297</v>
+        <v>34.04255319148936</v>
       </c>
       <c r="P11" t="n">
-        <v>66.8856170212766</v>
+        <v>67.32051063829788</v>
       </c>
       <c r="Q11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S11" t="b">
         <v>0</v>
@@ -4586,57 +4586,57 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>LUMAXIND</t>
+          <t>PRICOLLTD</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Lighting</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>5251</v>
+        <v>571.5</v>
       </c>
       <c r="D12" t="n">
-        <v>0.0137065637065636</v>
+        <v>0.0366406675131507</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.0608960028614862</v>
+        <v>-0.1407953093287228</v>
       </c>
       <c r="F12" t="n">
-        <v>0.2508337303477845</v>
+        <v>0.06992417860151651</v>
       </c>
       <c r="G12" t="n">
-        <v>0.2785591088842659</v>
+        <v>0.1058330098104689</v>
       </c>
       <c r="H12" t="n">
-        <v>0.2926276371073988</v>
+        <v>0.1196325689810942</v>
       </c>
       <c r="I12" t="n">
-        <v>57.68773580029976</v>
+        <v>61.90028222013171</v>
       </c>
       <c r="J12" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K12" t="n">
-        <v>57.69</v>
+        <v>49.98</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M12" t="n">
-        <v>57.69</v>
+        <v>49.98</v>
       </c>
       <c r="N12" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O12" t="n">
-        <v>89.36170212765957</v>
+        <v>72.3404255319149</v>
       </c>
       <c r="P12" t="n">
-        <v>64.94834042553191</v>
+        <v>66.46008510638299</v>
       </c>
       <c r="Q12" t="b">
         <v>0</v>
@@ -4660,25 +4660,25 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>2161.3</v>
+        <v>2158.2</v>
       </c>
       <c r="D13" t="n">
-        <v>0.0100004673115565</v>
+        <v>0.02231064374023</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.0674404556437693</v>
+        <v>-0.0914372316241476</v>
       </c>
       <c r="F13" t="n">
-        <v>0.0299752192146398</v>
+        <v>0.0660936573799642</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0577005977511212</v>
+        <v>0.1020024885889165</v>
       </c>
       <c r="H13" t="n">
-        <v>0.0717691259742541</v>
+        <v>0.1158020477595418</v>
       </c>
       <c r="I13" t="n">
-        <v>61.93606214520467</v>
+        <v>60.1514215080346</v>
       </c>
       <c r="J13" t="n">
         <v>80</v>
@@ -4688,7 +4688,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M13" t="n">
@@ -4698,10 +4698,10 @@
         <v>80</v>
       </c>
       <c r="O13" t="n">
-        <v>63.82978723404256</v>
+        <v>68.08510638297872</v>
       </c>
       <c r="P13" t="n">
-        <v>64.38995744680851</v>
+        <v>65.24102127659575</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
@@ -4716,63 +4716,63 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SUPRAJIT</t>
+          <t>LUMAXIND</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Cables</t>
+          <t>Lighting</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>427.4</v>
+        <v>5304</v>
       </c>
       <c r="D14" t="n">
-        <v>0.0159258378892321</v>
+        <v>0.0127935841130417</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.0892819092265075</v>
+        <v>-0.0519259987487711</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.0513816446565309</v>
+        <v>0.2074578277596923</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.0236562661200495</v>
+        <v>0.2433666589686447</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.009587737896916601</v>
+        <v>0.25716621813927</v>
       </c>
       <c r="I14" t="n">
-        <v>67.87196206283343</v>
+        <v>56.58836629725861</v>
       </c>
       <c r="J14" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K14" t="n">
-        <v>51.48</v>
+        <v>57.69</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M14" t="n">
-        <v>51.48</v>
+        <v>57.69</v>
       </c>
       <c r="N14" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O14" t="n">
-        <v>53.19148936170212</v>
+        <v>87.2340425531915</v>
       </c>
       <c r="P14" t="n">
-        <v>63.23029787234042</v>
+        <v>64.5228085106383</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
       </c>
       <c r="R14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S14" t="b">
         <v>0</v>
@@ -4781,63 +4781,63 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CRAFTSMAN</t>
+          <t>SUPRAJIT</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Castings</t>
+          <t>Cables</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>7351.5</v>
+        <v>431.75</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.009365314647621499</v>
+        <v>0.0279761904761903</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.0835255251511563</v>
+        <v>-0.07676681278734079</v>
       </c>
       <c r="F15" t="n">
-        <v>0.0893531895976884</v>
+        <v>-0.05005500550055</v>
       </c>
       <c r="G15" t="n">
-        <v>0.1170785681341698</v>
+        <v>-0.0141461742915977</v>
       </c>
       <c r="H15" t="n">
-        <v>0.1311470963573027</v>
+        <v>-0.0003466151209724</v>
       </c>
       <c r="I15" t="n">
-        <v>62.77992277992279</v>
+        <v>67.50599520383693</v>
       </c>
       <c r="J15" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K15" t="n">
-        <v>54.65</v>
+        <v>51.48</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M15" t="n">
-        <v>54.65</v>
+        <v>51.48</v>
       </c>
       <c r="N15" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O15" t="n">
-        <v>76.59574468085107</v>
+        <v>55.31914893617022</v>
       </c>
       <c r="P15" t="n">
-        <v>61.17914893617021</v>
+        <v>63.65582978723404</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
       </c>
       <c r="R15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S15" t="b">
         <v>0</v>
@@ -4855,25 +4855,25 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>580.25</v>
+        <v>604.95</v>
       </c>
       <c r="D16" t="n">
-        <v>0.1110579224509333</v>
+        <v>0.1818892253589918</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.0940671350507416</v>
+        <v>-0.09084761045987361</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.1917960860784178</v>
+        <v>-0.1780012229091649</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.1640707075419364</v>
+        <v>-0.1420923917002126</v>
       </c>
       <c r="H16" t="n">
-        <v>-0.1500021793188035</v>
+        <v>-0.1282928325295873</v>
       </c>
       <c r="I16" t="n">
-        <v>57.75136206042595</v>
+        <v>59.04944791166589</v>
       </c>
       <c r="J16" t="n">
         <v>80</v>
@@ -4883,7 +4883,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="M16" t="n">
@@ -4893,10 +4893,10 @@
         <v>80</v>
       </c>
       <c r="O16" t="n">
-        <v>29.78723404255319</v>
+        <v>36.17021276595745</v>
       </c>
       <c r="P16" t="n">
-        <v>60.72144680851064</v>
+        <v>61.99804255319149</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>
@@ -4919,7 +4919,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5387,6 +5387,25 @@
       </c>
       <c r="E27" t="n">
         <v>0.0130351865803167</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2025-03-13</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>4</v>
+      </c>
+      <c r="C28" t="n">
+        <v>0.6558098012315705</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0.0862171793595323</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0.5695926218720382</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: auto-refresh NSE data and pipeline outputs (2026-04-10)
</commit_message>
<xml_diff>
--- a/working-sector/output/auto_components_comprehensive_report.xlsx
+++ b/working-sector/output/auto_components_comprehensive_report.xlsx
@@ -435,7 +435,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -447,7 +447,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -779,25 +779,25 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1739.4</v>
+        <v>1798.8</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.0321072839574869</v>
+        <v>0.0107889413351314</v>
       </c>
       <c r="E2" t="n">
-        <v>0.1725765134151273</v>
+        <v>0.2370538477408708</v>
       </c>
       <c r="F2" t="n">
-        <v>0.3711177676178465</v>
+        <v>0.4179410373640233</v>
       </c>
       <c r="G2" t="n">
-        <v>0.4070265988267989</v>
+        <v>0.4224158913006803</v>
       </c>
       <c r="H2" t="n">
-        <v>0.4208261579974242</v>
+        <v>0.4553766686245629</v>
       </c>
       <c r="I2" t="n">
-        <v>53.27849588719154</v>
+        <v>67.79620853080567</v>
       </c>
       <c r="J2" t="n">
         <v>80</v>
@@ -807,7 +807,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M2" t="n">
@@ -844,25 +844,25 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1054.6</v>
+        <v>1078</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.0250531570675789</v>
+        <v>0.008890968647636799</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.1999696555909574</v>
+        <v>-0.1511811023622047</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.1909474491752973</v>
+        <v>-0.1787292396769769</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.155038617966345</v>
+        <v>-0.1742543857403199</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.1412390587957197</v>
+        <v>-0.1412936084164373</v>
       </c>
       <c r="I3" t="n">
-        <v>48.1536628945801</v>
+        <v>57.53807895554864</v>
       </c>
       <c r="J3" t="n">
         <v>60</v>
@@ -872,7 +872,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M3" t="n">
@@ -882,10 +882,10 @@
         <v>60</v>
       </c>
       <c r="O3" t="n">
-        <v>25.53191489361702</v>
+        <v>27.65957446808511</v>
       </c>
       <c r="P3" t="n">
-        <v>48.8503829787234</v>
+        <v>49.27591489361702</v>
       </c>
       <c r="Q3" t="b">
         <v>0</v>
@@ -909,48 +909,48 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>36770</v>
+        <v>37330</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1593883020652688</v>
+        <v>0.1924612681680242</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.0606718610295057</v>
+        <v>-0.0344024831867563</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.0755499685732243</v>
+        <v>-0.064059170114078</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.0396411373642719</v>
+        <v>-0.0595843161774209</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.0258415781936467</v>
+        <v>-0.0266235388535384</v>
       </c>
       <c r="I4" t="n">
-        <v>76.12612612612612</v>
+        <v>85.5840208423795</v>
       </c>
       <c r="J4" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="K4" t="n">
         <v>53.48</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M4" t="n">
         <v>53.48</v>
       </c>
       <c r="N4" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="O4" t="n">
         <v>51.06382978723404</v>
       </c>
       <c r="P4" t="n">
-        <v>59.6047659574468</v>
+        <v>55.6047659574468</v>
       </c>
       <c r="Q4" t="b">
         <v>0</v>
@@ -974,48 +974,48 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>311.25</v>
+        <v>324.5</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.0008025682182986</v>
+        <v>0.0467741935483871</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.133973288814691</v>
+        <v>-0.0802154195011338</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.2568051575931233</v>
+        <v>-0.2367399741267787</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.2208963263841709</v>
+        <v>-0.2322651201901217</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.2070967672135456</v>
+        <v>-0.1993043428662391</v>
       </c>
       <c r="I5" t="n">
-        <v>55.25030525030527</v>
+        <v>70.27027027027027</v>
       </c>
       <c r="J5" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K5" t="n">
         <v>51.12</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M5" t="n">
         <v>51.12</v>
       </c>
       <c r="N5" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O5" t="n">
-        <v>10.63829787234042</v>
+        <v>14.8936170212766</v>
       </c>
       <c r="P5" t="n">
-        <v>46.57565957446808</v>
+        <v>51.42672340425532</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
@@ -1039,48 +1039,48 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>116.9</v>
+        <v>122.16</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.0369882197874618</v>
+        <v>0.0165598735125238</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.0205278592375365</v>
+        <v>0.034290068580137</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0691421254801536</v>
+        <v>0.1209396219489813</v>
       </c>
       <c r="G6" t="n">
-        <v>0.105050956689106</v>
+        <v>0.1254144758856383</v>
       </c>
       <c r="H6" t="n">
-        <v>0.1188505158597312</v>
+        <v>0.1583752532095209</v>
       </c>
       <c r="I6" t="n">
-        <v>57.48942172073343</v>
+        <v>71.80061607392888</v>
       </c>
       <c r="J6" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K6" t="n">
         <v>51.57</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M6" t="n">
         <v>51.57</v>
       </c>
       <c r="N6" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O6" t="n">
-        <v>70.21276595744681</v>
+        <v>76.59574468085107</v>
       </c>
       <c r="P6" t="n">
-        <v>58.67055319148936</v>
+        <v>63.94714893617022</v>
       </c>
       <c r="Q6" t="b">
         <v>0</v>
@@ -1104,48 +1104,48 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2743.3</v>
+        <v>2744.8</v>
       </c>
       <c r="D7" t="n">
-        <v>0.06909586905689789</v>
+        <v>0.0765188061340551</v>
       </c>
       <c r="E7" t="n">
-        <v>0.0854237556382053</v>
+        <v>0.09463609172482559</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.1900501919102449</v>
+        <v>-0.1903005988377237</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.1541413607012925</v>
+        <v>-0.1858257449010667</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.1403418015306673</v>
+        <v>-0.1528649675771841</v>
       </c>
       <c r="I7" t="n">
-        <v>65.1559741024132</v>
+        <v>72.26740403383218</v>
       </c>
       <c r="J7" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K7" t="n">
         <v>48.73</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M7" t="n">
         <v>48.73</v>
       </c>
       <c r="N7" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O7" t="n">
-        <v>27.65957446808511</v>
+        <v>23.40425531914894</v>
       </c>
       <c r="P7" t="n">
-        <v>57.02391489361703</v>
+        <v>52.17285106382979</v>
       </c>
       <c r="Q7" t="b">
         <v>0</v>
@@ -1169,48 +1169,48 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>523.05</v>
+        <v>554.25</v>
       </c>
       <c r="D8" t="n">
-        <v>0.0129756947806718</v>
+        <v>0.08612580834803051</v>
       </c>
       <c r="E8" t="n">
-        <v>0.1039468130012661</v>
+        <v>0.1974721832127037</v>
       </c>
       <c r="F8" t="n">
-        <v>0.2035204786010123</v>
+        <v>0.2579437131184747</v>
       </c>
       <c r="G8" t="n">
-        <v>0.2394293098099646</v>
+        <v>0.2624185670551318</v>
       </c>
       <c r="H8" t="n">
-        <v>0.2532288689805899</v>
+        <v>0.2953793443790143</v>
       </c>
       <c r="I8" t="n">
-        <v>55.91549295774645</v>
+        <v>72.81105990783408</v>
       </c>
       <c r="J8" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K8" t="n">
         <v>49.66</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M8" t="n">
         <v>49.66</v>
       </c>
       <c r="N8" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O8" t="n">
         <v>85.1063829787234</v>
       </c>
       <c r="P8" t="n">
-        <v>68.88527659574468</v>
+        <v>64.88527659574468</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
@@ -1234,48 +1234,48 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>440.35</v>
+        <v>438.15</v>
       </c>
       <c r="D9" t="n">
-        <v>0.0140472078295912</v>
+        <v>0.0490841613791452</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.1491643319486039</v>
+        <v>-0.1573228195018753</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.0891508946116453</v>
+        <v>-0.0957589516045815</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.0532420634026929</v>
+        <v>-0.0912840976679245</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.0394425042320677</v>
+        <v>-0.0583233203440419</v>
       </c>
       <c r="I9" t="n">
-        <v>61.01694915254237</v>
+        <v>77.86589762076422</v>
       </c>
       <c r="J9" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="K9" t="n">
         <v>53.44</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M9" t="n">
         <v>53.44</v>
       </c>
       <c r="N9" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="O9" t="n">
-        <v>48.93617021276596</v>
+        <v>42.5531914893617</v>
       </c>
       <c r="P9" t="n">
-        <v>55.1632340425532</v>
+        <v>49.88663829787235</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -1299,48 +1299,48 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>134020</v>
+        <v>136705</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.0164030677773292</v>
+        <v>-0.009419948552588601</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.1073367302760848</v>
+        <v>-0.08078940290478751</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.1079012181321973</v>
+        <v>-0.08282455551828249</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.0719923869232449</v>
+        <v>-0.07834970158162539</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.0581928277526196</v>
+        <v>-0.0453889242577428</v>
       </c>
       <c r="I10" t="n">
-        <v>66.24092161282243</v>
+        <v>79.19362867098059</v>
       </c>
       <c r="J10" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="K10" t="n">
         <v>49.41</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M10" t="n">
         <v>49.41</v>
       </c>
       <c r="N10" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="O10" t="n">
-        <v>46.80851063829788</v>
+        <v>48.93617021276596</v>
       </c>
       <c r="P10" t="n">
-        <v>53.12570212765957</v>
+        <v>49.55123404255319</v>
       </c>
       <c r="Q10" t="b">
         <v>0</v>
@@ -1376,10 +1376,10 @@
         <v>-0.0042030657656173</v>
       </c>
       <c r="G11" t="n">
-        <v>0.031705765443335</v>
+        <v>0.0002717881710396</v>
       </c>
       <c r="H11" t="n">
-        <v>0.0455053246139602</v>
+        <v>0.0332325654949222</v>
       </c>
       <c r="I11" t="n">
         <v>27.6054590570719</v>
@@ -1392,7 +1392,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M11" t="n">
@@ -1429,48 +1429,48 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>438.6</v>
+        <v>440.15</v>
       </c>
       <c r="D12" t="n">
-        <v>0.08389966637835169</v>
+        <v>0.08304625984251961</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.0646193218170184</v>
+        <v>-0.0640085061137692</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.1791896696921493</v>
+        <v>-0.1540457428406688</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.1432808384831969</v>
+        <v>-0.1495708889040118</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.1294812793125717</v>
+        <v>-0.1166101115801292</v>
       </c>
       <c r="I12" t="n">
-        <v>65.04605936540432</v>
+        <v>76.76886792452831</v>
       </c>
       <c r="J12" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K12" t="n">
         <v>71.28</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M12" t="n">
         <v>71.28</v>
       </c>
       <c r="N12" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O12" t="n">
-        <v>34.04255319148936</v>
+        <v>38.29787234042553</v>
       </c>
       <c r="P12" t="n">
-        <v>67.32051063829788</v>
+        <v>64.17157446808511</v>
       </c>
       <c r="Q12" t="b">
         <v>1</v>
@@ -1494,25 +1494,25 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1688.8</v>
+        <v>1721</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.1099399177822283</v>
+        <v>-0.0558481457098968</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.143697393773451</v>
+        <v>-0.1000836645053336</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.0563781639380902</v>
+        <v>-0.0277385458448674</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.0204693327291378</v>
+        <v>-0.0232636919082104</v>
       </c>
       <c r="H13" t="n">
-        <v>-0.0066697735585126</v>
+        <v>0.0096970854156721</v>
       </c>
       <c r="I13" t="n">
-        <v>52.34557418807046</v>
+        <v>68.26640548481879</v>
       </c>
       <c r="J13" t="n">
         <v>60</v>
@@ -1522,7 +1522,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M13" t="n">
@@ -1532,16 +1532,16 @@
         <v>60</v>
       </c>
       <c r="O13" t="n">
-        <v>53.19148936170212</v>
+        <v>57.44680851063831</v>
       </c>
       <c r="P13" t="n">
-        <v>58.14629787234043</v>
+        <v>58.99736170212766</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
       </c>
       <c r="R13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S13" t="b">
         <v>0</v>
@@ -1559,25 +1559,25 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>566.25</v>
+        <v>590.35</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.0169270833333333</v>
+        <v>0.0262494567579314</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.1846065231478149</v>
+        <v>-0.1351450336946967</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.238655462184874</v>
+        <v>-0.2641321283889062</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.2027466309759216</v>
+        <v>-0.2596572744522492</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.1889470718052963</v>
+        <v>-0.2266964971283666</v>
       </c>
       <c r="I14" t="n">
-        <v>52.60535603072452</v>
+        <v>64.55479452054794</v>
       </c>
       <c r="J14" t="n">
         <v>60</v>
@@ -1587,7 +1587,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M14" t="n">
@@ -1597,10 +1597,10 @@
         <v>60</v>
       </c>
       <c r="O14" t="n">
-        <v>17.02127659574468</v>
+        <v>6.382978723404255</v>
       </c>
       <c r="P14" t="n">
-        <v>49.26025531914894</v>
+        <v>47.13259574468086</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
@@ -1624,25 +1624,25 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>99.45</v>
+        <v>101.95</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.0139797739440808</v>
+        <v>0.0381873727087576</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.0851807561401893</v>
+        <v>-0.0378444696111739</v>
       </c>
       <c r="F15" t="n">
-        <v>0.097197705207414</v>
+        <v>0.1475686627645205</v>
       </c>
       <c r="G15" t="n">
-        <v>0.1331065364163663</v>
+        <v>0.1520435167011775</v>
       </c>
       <c r="H15" t="n">
-        <v>0.1469060955869916</v>
+        <v>0.1850042940250601</v>
       </c>
       <c r="I15" t="n">
-        <v>52.09302325581396</v>
+        <v>65.49032914828641</v>
       </c>
       <c r="J15" t="n">
         <v>60</v>
@@ -1652,7 +1652,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M15" t="n">
@@ -1689,48 +1689,48 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>176.74</v>
+        <v>176.93</v>
       </c>
       <c r="D16" t="n">
-        <v>0.0257094771052173</v>
+        <v>0.0441428149896725</v>
       </c>
       <c r="E16" t="n">
-        <v>0.0405039444248203</v>
+        <v>0.0601593864221943</v>
       </c>
       <c r="F16" t="n">
-        <v>0.1704635761589403</v>
+        <v>0.2036054421768707</v>
       </c>
       <c r="G16" t="n">
-        <v>0.2063724073678927</v>
+        <v>0.2080802961135277</v>
       </c>
       <c r="H16" t="n">
-        <v>0.220171966538518</v>
+        <v>0.2410410734374103</v>
       </c>
       <c r="I16" t="n">
-        <v>61.80000000000001</v>
+        <v>72.18861485962464</v>
       </c>
       <c r="J16" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K16" t="n">
         <v>52.61</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M16" t="n">
         <v>52.61</v>
       </c>
       <c r="N16" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O16" t="n">
         <v>82.97872340425532</v>
       </c>
       <c r="P16" t="n">
-        <v>69.63974468085107</v>
+        <v>65.63974468085107</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>
@@ -1754,48 +1754,48 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>7408.5</v>
+        <v>7430</v>
       </c>
       <c r="D17" t="n">
-        <v>0.01133028462221</v>
+        <v>0.0103345118302964</v>
       </c>
       <c r="E17" t="n">
-        <v>-0.0509223674096848</v>
+        <v>-0.0309116994913264</v>
       </c>
       <c r="F17" t="n">
-        <v>0.08924501948099681</v>
+        <v>0.0970837947582132</v>
       </c>
       <c r="G17" t="n">
-        <v>0.1251538506899492</v>
+        <v>0.1015586486948703</v>
       </c>
       <c r="H17" t="n">
-        <v>0.1389534098605744</v>
+        <v>0.1345194260187528</v>
       </c>
       <c r="I17" t="n">
-        <v>62.77992277992279</v>
+        <v>77.63528307788552</v>
       </c>
       <c r="J17" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K17" t="n">
         <v>54.65</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M17" t="n">
         <v>54.65</v>
       </c>
       <c r="N17" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O17" t="n">
-        <v>76.59574468085107</v>
+        <v>72.3404255319149</v>
       </c>
       <c r="P17" t="n">
-        <v>69.17914893617021</v>
+        <v>64.32808510638299</v>
       </c>
       <c r="Q17" t="b">
         <v>0</v>
@@ -1819,25 +1819,25 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>677.45</v>
+        <v>673.45</v>
       </c>
       <c r="D18" t="n">
-        <v>-0.0630661779959891</v>
+        <v>-0.0538774936779993</v>
       </c>
       <c r="E18" t="n">
-        <v>0.120400231538907</v>
+        <v>0.1302341193253335</v>
       </c>
       <c r="F18" t="n">
-        <v>0.0304989351992699</v>
+        <v>0.0278540903540902</v>
       </c>
       <c r="G18" t="n">
-        <v>0.0664077664082223</v>
+        <v>0.0323289442907472</v>
       </c>
       <c r="H18" t="n">
-        <v>0.08020732557884749</v>
+        <v>0.0652897216146298</v>
       </c>
       <c r="I18" t="n">
-        <v>44.12454681168694</v>
+        <v>53.88020833333336</v>
       </c>
       <c r="J18" t="n">
         <v>60</v>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M18" t="n">
@@ -1884,48 +1884,48 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2379.6</v>
+        <v>2433</v>
       </c>
       <c r="D19" t="n">
-        <v>-0.042491549975857</v>
+        <v>-0.0111765901239585</v>
       </c>
       <c r="E19" t="n">
-        <v>-0.0845227561266496</v>
+        <v>-0.0682444852941175</v>
       </c>
       <c r="F19" t="n">
-        <v>-0.1738934212810275</v>
+        <v>-0.1644343704924789</v>
       </c>
       <c r="G19" t="n">
-        <v>-0.1379845900720752</v>
+        <v>-0.1599595165558218</v>
       </c>
       <c r="H19" t="n">
-        <v>-0.1241850309014499</v>
+        <v>-0.1269987392319392</v>
       </c>
       <c r="I19" t="n">
-        <v>58.55002583089372</v>
+        <v>69.82605608803692</v>
       </c>
       <c r="J19" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K19" t="n">
         <v>51.27</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M19" t="n">
         <v>51.27</v>
       </c>
       <c r="N19" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O19" t="n">
-        <v>38.29787234042553</v>
+        <v>31.91489361702128</v>
       </c>
       <c r="P19" t="n">
-        <v>52.16757446808511</v>
+        <v>58.89097872340426</v>
       </c>
       <c r="Q19" t="b">
         <v>0</v>
@@ -1949,48 +1949,48 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2158.2</v>
+        <v>2216.6</v>
       </c>
       <c r="D20" t="n">
-        <v>0.02231064374023</v>
+        <v>0.0547202131709174</v>
       </c>
       <c r="E20" t="n">
-        <v>-0.0914372316241476</v>
+        <v>-0.0474021229962612</v>
       </c>
       <c r="F20" t="n">
-        <v>0.0660936573799642</v>
+        <v>0.0796882610813443</v>
       </c>
       <c r="G20" t="n">
-        <v>0.1020024885889165</v>
+        <v>0.08416311501800131</v>
       </c>
       <c r="H20" t="n">
-        <v>0.1158020477595418</v>
+        <v>0.1171238923418839</v>
       </c>
       <c r="I20" t="n">
-        <v>60.1514215080346</v>
+        <v>71.80433039294304</v>
       </c>
       <c r="J20" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K20" t="n">
         <v>49.06</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M20" t="n">
         <v>49.06</v>
       </c>
       <c r="N20" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O20" t="n">
-        <v>68.08510638297872</v>
+        <v>70.21276595744681</v>
       </c>
       <c r="P20" t="n">
-        <v>65.24102127659575</v>
+        <v>61.66655319148936</v>
       </c>
       <c r="Q20" t="b">
         <v>0</v>
@@ -2014,48 +2014,48 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>907.2</v>
+        <v>933.5</v>
       </c>
       <c r="D21" t="n">
-        <v>0.0261282660332542</v>
+        <v>0.0610365992270971</v>
       </c>
       <c r="E21" t="n">
-        <v>-0.1212708252615265</v>
+        <v>-0.0783887846776582</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.3082202226628031</v>
+        <v>-0.2515834201876051</v>
       </c>
       <c r="G21" t="n">
-        <v>-0.2723113914538507</v>
+        <v>-0.2471085662509481</v>
       </c>
       <c r="H21" t="n">
-        <v>-0.2585118322832255</v>
+        <v>-0.2141477889270655</v>
       </c>
       <c r="I21" t="n">
-        <v>58.9231699939504</v>
+        <v>71.15146512587702</v>
       </c>
       <c r="J21" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K21" t="n">
         <v>48.43</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M21" t="n">
         <v>48.43</v>
       </c>
       <c r="N21" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O21" t="n">
-        <v>6.382978723404255</v>
+        <v>8.51063829787234</v>
       </c>
       <c r="P21" t="n">
-        <v>44.64859574468085</v>
+        <v>49.07412765957447</v>
       </c>
       <c r="Q21" t="b">
         <v>0</v>
@@ -2079,48 +2079,48 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>409.65</v>
+        <v>443</v>
       </c>
       <c r="D22" t="n">
-        <v>-0.0271906910472572</v>
+        <v>0.0650318547902393</v>
       </c>
       <c r="E22" t="n">
-        <v>0.0656867845993756</v>
+        <v>0.2054421768707484</v>
       </c>
       <c r="F22" t="n">
-        <v>0.3096227621483374</v>
+        <v>0.3809226932668328</v>
       </c>
       <c r="G22" t="n">
-        <v>0.3455315933572898</v>
+        <v>0.3853975472034898</v>
       </c>
       <c r="H22" t="n">
-        <v>0.359331152527915</v>
+        <v>0.4183583245273724</v>
       </c>
       <c r="I22" t="n">
-        <v>60.09417304296643</v>
+        <v>73.69423286180631</v>
       </c>
       <c r="J22" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K22" t="n">
         <v>54.47</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M22" t="n">
         <v>54.47</v>
       </c>
       <c r="N22" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O22" t="n">
         <v>93.61702127659576</v>
       </c>
       <c r="P22" t="n">
-        <v>72.51140425531915</v>
+        <v>68.51140425531915</v>
       </c>
       <c r="Q22" t="b">
         <v>0</v>
@@ -2144,25 +2144,25 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>348.95</v>
+        <v>357.9</v>
       </c>
       <c r="D23" t="n">
-        <v>-0.0182866788577859</v>
+        <v>0.0088794926004227</v>
       </c>
       <c r="E23" t="n">
-        <v>-0.1169176262178919</v>
+        <v>-0.07002728335715221</v>
       </c>
       <c r="F23" t="n">
-        <v>-0.1679780639008107</v>
+        <v>-0.1407994238386749</v>
       </c>
       <c r="G23" t="n">
-        <v>-0.1320692326918583</v>
+        <v>-0.1363245699020179</v>
       </c>
       <c r="H23" t="n">
-        <v>-0.118269673521233</v>
+        <v>-0.1033637925781353</v>
       </c>
       <c r="I23" t="n">
-        <v>54.85183033120276</v>
+        <v>67.93708408953418</v>
       </c>
       <c r="J23" t="n">
         <v>60</v>
@@ -2172,7 +2172,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M23" t="n">
@@ -2209,25 +2209,25 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>121.95</v>
+        <v>124.8</v>
       </c>
       <c r="D24" t="n">
-        <v>-0.0156590523851803</v>
+        <v>0.0194412677667048</v>
       </c>
       <c r="E24" t="n">
-        <v>-0.0770453341406189</v>
+        <v>-0.027355623100304</v>
       </c>
       <c r="F24" t="n">
-        <v>0.1200404114621602</v>
+        <v>0.1587743732590529</v>
       </c>
       <c r="G24" t="n">
-        <v>0.1559492426711126</v>
+        <v>0.16324922719571</v>
       </c>
       <c r="H24" t="n">
-        <v>0.1697488018417379</v>
+        <v>0.1962100045195925</v>
       </c>
       <c r="I24" t="n">
-        <v>52.41746538871138</v>
+        <v>64.52067669172934</v>
       </c>
       <c r="J24" t="n">
         <v>60</v>
@@ -2237,7 +2237,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M24" t="n">
@@ -2274,25 +2274,25 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>604.95</v>
+        <v>611.45</v>
       </c>
       <c r="D25" t="n">
-        <v>0.1818892253589918</v>
+        <v>0.1894757319326916</v>
       </c>
       <c r="E25" t="n">
-        <v>-0.09084761045987361</v>
+        <v>-0.0406370126304228</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.1780012229091649</v>
+        <v>-0.1689432551817872</v>
       </c>
       <c r="G25" t="n">
-        <v>-0.1420923917002126</v>
+        <v>-0.1644684012451301</v>
       </c>
       <c r="H25" t="n">
-        <v>-0.1282928325295873</v>
+        <v>-0.1315076239212476</v>
       </c>
       <c r="I25" t="n">
-        <v>59.04944791166589</v>
+        <v>68.79150066401063</v>
       </c>
       <c r="J25" t="n">
         <v>80</v>
@@ -2302,7 +2302,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M25" t="n">
@@ -2312,10 +2312,10 @@
         <v>80</v>
       </c>
       <c r="O25" t="n">
-        <v>36.17021276595745</v>
+        <v>29.78723404255319</v>
       </c>
       <c r="P25" t="n">
-        <v>61.99804255319149</v>
+        <v>60.72144680851064</v>
       </c>
       <c r="Q25" t="b">
         <v>0</v>
@@ -2339,25 +2339,25 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>130.94</v>
+        <v>133.88</v>
       </c>
       <c r="D26" t="n">
-        <v>-0.0373474489045729</v>
+        <v>-0.009543537767256</v>
       </c>
       <c r="E26" t="n">
-        <v>-0.1775125628140703</v>
+        <v>-0.1223861029170764</v>
       </c>
       <c r="F26" t="n">
-        <v>-0.2459979269837613</v>
+        <v>-0.2373682711478212</v>
       </c>
       <c r="G26" t="n">
-        <v>-0.2100890957748089</v>
+        <v>-0.2328934172111642</v>
       </c>
       <c r="H26" t="n">
-        <v>-0.1962895366041837</v>
+        <v>-0.1999326398872816</v>
       </c>
       <c r="I26" t="n">
-        <v>54.44848484848485</v>
+        <v>68.64864864864862</v>
       </c>
       <c r="J26" t="n">
         <v>60</v>
@@ -2367,7 +2367,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M26" t="n">
@@ -2404,48 +2404,48 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>5304</v>
+        <v>5571.6</v>
       </c>
       <c r="D27" t="n">
-        <v>0.0127935841130417</v>
+        <v>0.1253484144617249</v>
       </c>
       <c r="E27" t="n">
-        <v>-0.0519259987487711</v>
+        <v>0.0054317423080394</v>
       </c>
       <c r="F27" t="n">
-        <v>0.2074578277596923</v>
+        <v>0.3048854747294955</v>
       </c>
       <c r="G27" t="n">
-        <v>0.2433666589686447</v>
+        <v>0.3093603286661526</v>
       </c>
       <c r="H27" t="n">
-        <v>0.25716621813927</v>
+        <v>0.3423211059900352</v>
       </c>
       <c r="I27" t="n">
-        <v>56.58836629725861</v>
+        <v>70.03147953830012</v>
       </c>
       <c r="J27" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K27" t="n">
         <v>57.69</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M27" t="n">
         <v>57.69</v>
       </c>
       <c r="N27" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O27" t="n">
-        <v>87.2340425531915</v>
+        <v>89.36170212765957</v>
       </c>
       <c r="P27" t="n">
-        <v>64.5228085106383</v>
+        <v>68.94834042553191</v>
       </c>
       <c r="Q27" t="b">
         <v>0</v>
@@ -2469,48 +2469,48 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1725.6</v>
+        <v>1823.3</v>
       </c>
       <c r="D28" t="n">
-        <v>0.1735582154515775</v>
+        <v>0.3093716337522441</v>
       </c>
       <c r="E28" t="n">
-        <v>0.033479068096065</v>
+        <v>0.1515821385713383</v>
       </c>
       <c r="F28" t="n">
-        <v>0.5505436247641295</v>
+        <v>0.6435009915269514</v>
       </c>
       <c r="G28" t="n">
-        <v>0.5864524559730819</v>
+        <v>0.6479758454636084</v>
       </c>
       <c r="H28" t="n">
-        <v>0.6002520151437072</v>
+        <v>0.680936622787491</v>
       </c>
       <c r="I28" t="n">
-        <v>63.34236369793431</v>
+        <v>78.54170134842684</v>
       </c>
       <c r="J28" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K28" t="n">
         <v>54.51</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M28" t="n">
         <v>54.51</v>
       </c>
       <c r="N28" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O28" t="n">
         <v>100</v>
       </c>
       <c r="P28" t="n">
-        <v>73.804</v>
+        <v>69.804</v>
       </c>
       <c r="Q28" t="b">
         <v>0</v>
@@ -2534,25 +2534,25 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>514.4</v>
+        <v>514.35</v>
       </c>
       <c r="D29" t="n">
-        <v>0.0407688416793119</v>
+        <v>0.0690013509300635</v>
       </c>
       <c r="E29" t="n">
-        <v>-0.1369127516778524</v>
+        <v>-0.1233915636983382</v>
       </c>
       <c r="F29" t="n">
-        <v>-0.0326281147155618</v>
+        <v>-0.0321761219305674</v>
       </c>
       <c r="G29" t="n">
-        <v>0.0032807164933905</v>
+        <v>-0.0277012679939103</v>
       </c>
       <c r="H29" t="n">
-        <v>0.0170802756640158</v>
+        <v>0.0052595093299722</v>
       </c>
       <c r="I29" t="n">
-        <v>53.27643171806167</v>
+        <v>56.91176470588235</v>
       </c>
       <c r="J29" t="n">
         <v>60</v>
@@ -2562,7 +2562,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M29" t="n">
@@ -2572,10 +2572,10 @@
         <v>60</v>
       </c>
       <c r="O29" t="n">
-        <v>57.44680851063831</v>
+        <v>55.31914893617022</v>
       </c>
       <c r="P29" t="n">
-        <v>55.25736170212766</v>
+        <v>54.83182978723404</v>
       </c>
       <c r="Q29" t="b">
         <v>0</v>
@@ -2599,48 +2599,48 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>114.05</v>
+        <v>119.83</v>
       </c>
       <c r="D30" t="n">
-        <v>-0.1004811104976733</v>
+        <v>-0.0557875659916475</v>
       </c>
       <c r="E30" t="n">
-        <v>-0.0610077391733904</v>
+        <v>-0.0211566737461199</v>
       </c>
       <c r="F30" t="n">
-        <v>-0.1215435569591004</v>
+        <v>-0.094939577039275</v>
       </c>
       <c r="G30" t="n">
-        <v>-0.08563472575014799</v>
+        <v>-0.09046472310261799</v>
       </c>
       <c r="H30" t="n">
-        <v>-0.0718351665795228</v>
+        <v>-0.0575039457787354</v>
       </c>
       <c r="I30" t="n">
-        <v>42.60204081632653</v>
+        <v>63.114161849711</v>
       </c>
       <c r="J30" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K30" t="n">
         <v>52.38</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M30" t="n">
         <v>52.38</v>
       </c>
       <c r="N30" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O30" t="n">
-        <v>44.68085106382978</v>
+        <v>46.80851063829788</v>
       </c>
       <c r="P30" t="n">
-        <v>53.88817021276596</v>
+        <v>62.31370212765957</v>
       </c>
       <c r="Q30" t="b">
         <v>0</v>
@@ -2664,25 +2664,25 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>38.58</v>
+        <v>39.33</v>
       </c>
       <c r="D31" t="n">
-        <v>-0.039820806371329</v>
+        <v>-0.0182226660009986</v>
       </c>
       <c r="E31" t="n">
-        <v>-0.2320859872611466</v>
+        <v>-0.1917385943279901</v>
       </c>
       <c r="F31" t="n">
-        <v>-0.2061728395061729</v>
+        <v>-0.1887376237623762</v>
       </c>
       <c r="G31" t="n">
-        <v>-0.1702640082972205</v>
+        <v>-0.1842627698257192</v>
       </c>
       <c r="H31" t="n">
-        <v>-0.1564644491265953</v>
+        <v>-0.1513019925018366</v>
       </c>
       <c r="I31" t="n">
-        <v>58.71459694989108</v>
+        <v>69.45701357466061</v>
       </c>
       <c r="J31" t="n">
         <v>60</v>
@@ -2692,7 +2692,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M31" t="n">
@@ -2702,10 +2702,10 @@
         <v>60</v>
       </c>
       <c r="O31" t="n">
-        <v>23.40425531914894</v>
+        <v>25.53191489361702</v>
       </c>
       <c r="P31" t="n">
-        <v>48.27685106382979</v>
+        <v>48.70238297872341</v>
       </c>
       <c r="Q31" t="b">
         <v>0</v>
@@ -2729,25 +2729,25 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>715.35</v>
+        <v>733.75</v>
       </c>
       <c r="D32" t="n">
-        <v>0.0087428611718254</v>
+        <v>0.0600260040450735</v>
       </c>
       <c r="E32" t="n">
-        <v>-0.086923224200651</v>
+        <v>-0.07947559904654369</v>
       </c>
       <c r="F32" t="n">
-        <v>-0.361009379187137</v>
+        <v>-0.370117606661516</v>
       </c>
       <c r="G32" t="n">
-        <v>-0.3251005479781846</v>
+        <v>-0.365642752724859</v>
       </c>
       <c r="H32" t="n">
-        <v>-0.3113009888075594</v>
+        <v>-0.3326819754009764</v>
       </c>
       <c r="I32" t="n">
-        <v>56.02495543672015</v>
+        <v>68.2542768273717</v>
       </c>
       <c r="J32" t="n">
         <v>80</v>
@@ -2757,7 +2757,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M32" t="n">
@@ -2794,48 +2794,48 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>571.5</v>
+        <v>583.75</v>
       </c>
       <c r="D33" t="n">
-        <v>0.0366406675131507</v>
+        <v>0.0777254684759531</v>
       </c>
       <c r="E33" t="n">
-        <v>-0.1407953093287228</v>
+        <v>-0.1101371951219511</v>
       </c>
       <c r="F33" t="n">
-        <v>0.06992417860151651</v>
+        <v>0.06982497938238789</v>
       </c>
       <c r="G33" t="n">
-        <v>0.1058330098104689</v>
+        <v>0.07429983331904499</v>
       </c>
       <c r="H33" t="n">
-        <v>0.1196325689810942</v>
+        <v>0.1072606106429275</v>
       </c>
       <c r="I33" t="n">
-        <v>61.90028222013171</v>
+        <v>74.43810801744381</v>
       </c>
       <c r="J33" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K33" t="n">
         <v>49.98</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M33" t="n">
         <v>49.98</v>
       </c>
       <c r="N33" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O33" t="n">
-        <v>72.3404255319149</v>
+        <v>65.95744680851064</v>
       </c>
       <c r="P33" t="n">
-        <v>66.46008510638299</v>
+        <v>61.18348936170213</v>
       </c>
       <c r="Q33" t="b">
         <v>0</v>
@@ -2871,10 +2871,10 @@
         <v>-0.2401052253975846</v>
       </c>
       <c r="G34" t="n">
-        <v>-0.2041963941886322</v>
+        <v>-0.2356303714609275</v>
       </c>
       <c r="H34" t="n">
-        <v>-0.1903968350180069</v>
+        <v>-0.202669594137045</v>
       </c>
       <c r="I34" t="n">
         <v>63.3225806451613</v>
@@ -2887,7 +2887,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M34" t="n">
@@ -2897,10 +2897,10 @@
         <v>80</v>
       </c>
       <c r="O34" t="n">
-        <v>14.8936170212766</v>
+        <v>10.63829787234042</v>
       </c>
       <c r="P34" t="n">
-        <v>55.33072340425532</v>
+        <v>54.47965957446809</v>
       </c>
       <c r="Q34" t="b">
         <v>0</v>
@@ -2924,25 +2924,25 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>114.52</v>
+        <v>116.72</v>
       </c>
       <c r="D35" t="n">
-        <v>0.0240543682375034</v>
+        <v>0.0439137823092745</v>
       </c>
       <c r="E35" t="n">
-        <v>-0.1472822040208489</v>
+        <v>-0.1056624013485556</v>
       </c>
       <c r="F35" t="n">
-        <v>0.07895232711513089</v>
+        <v>0.1084520417853751</v>
       </c>
       <c r="G35" t="n">
-        <v>0.1148611583240832</v>
+        <v>0.1129268957220321</v>
       </c>
       <c r="H35" t="n">
-        <v>0.1286607174947085</v>
+        <v>0.1458876730459147</v>
       </c>
       <c r="I35" t="n">
-        <v>56.52173913043476</v>
+        <v>68.52352623039479</v>
       </c>
       <c r="J35" t="n">
         <v>60</v>
@@ -2952,7 +2952,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M35" t="n">
@@ -2989,48 +2989,48 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>484.7</v>
+        <v>492.5</v>
       </c>
       <c r="D36" t="n">
-        <v>-0.0417160933175168</v>
+        <v>0.0028507432294848</v>
       </c>
       <c r="E36" t="n">
-        <v>-0.1716653849440313</v>
+        <v>-0.1471861471861472</v>
       </c>
       <c r="F36" t="n">
-        <v>0.0349097896871997</v>
+        <v>0.0760323355909984</v>
       </c>
       <c r="G36" t="n">
-        <v>0.0708186208961521</v>
+        <v>0.0805071895276554</v>
       </c>
       <c r="H36" t="n">
-        <v>0.08461818006677729</v>
+        <v>0.113467966851538</v>
       </c>
       <c r="I36" t="n">
-        <v>52.9552715654952</v>
+        <v>71.38728323699422</v>
       </c>
       <c r="J36" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="K36" t="n">
         <v>47.8</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M36" t="n">
         <v>47.8</v>
       </c>
       <c r="N36" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="O36" t="n">
-        <v>63.82978723404256</v>
+        <v>68.08510638297872</v>
       </c>
       <c r="P36" t="n">
-        <v>55.88595744680852</v>
+        <v>52.73702127659575</v>
       </c>
       <c r="Q36" t="b">
         <v>0</v>
@@ -3054,48 +3054,48 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2251.7</v>
+        <v>2337.5</v>
       </c>
       <c r="D37" t="n">
-        <v>0.0339808054369288</v>
+        <v>0.1240142335064435</v>
       </c>
       <c r="E37" t="n">
-        <v>0.1575673452601274</v>
+        <v>0.2342256718939752</v>
       </c>
       <c r="F37" t="n">
-        <v>0.4941605839416056</v>
+        <v>0.5838867055156525</v>
       </c>
       <c r="G37" t="n">
-        <v>0.5300694151505581</v>
+        <v>0.5883615594523095</v>
       </c>
       <c r="H37" t="n">
-        <v>0.5438689743211833</v>
+        <v>0.6213223367761921</v>
       </c>
       <c r="I37" t="n">
-        <v>56.48050579557426</v>
+        <v>78.09085681426104</v>
       </c>
       <c r="J37" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K37" t="n">
         <v>48.59</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M37" t="n">
         <v>48.59</v>
       </c>
       <c r="N37" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O37" t="n">
         <v>97.87234042553192</v>
       </c>
       <c r="P37" t="n">
-        <v>71.0104680851064</v>
+        <v>67.0104680851064</v>
       </c>
       <c r="Q37" t="b">
         <v>0</v>
@@ -3119,25 +3119,25 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>822.75</v>
+        <v>831.3</v>
       </c>
       <c r="D38" t="n">
-        <v>0.0037821021167572</v>
+        <v>0.0237054368573363</v>
       </c>
       <c r="E38" t="n">
-        <v>-0.1313872466216217</v>
+        <v>-0.1033813298818961</v>
       </c>
       <c r="F38" t="n">
-        <v>-0.2243329876496653</v>
+        <v>-0.2138263665594856</v>
       </c>
       <c r="G38" t="n">
-        <v>-0.1884241564407129</v>
+        <v>-0.2093515126228285</v>
       </c>
       <c r="H38" t="n">
-        <v>-0.1746245972700877</v>
+        <v>-0.176390735298946</v>
       </c>
       <c r="I38" t="n">
-        <v>56.01652892561984</v>
+        <v>65.65842862412396</v>
       </c>
       <c r="J38" t="n">
         <v>60</v>
@@ -3147,7 +3147,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M38" t="n">
@@ -3184,48 +3184,48 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>3223.7</v>
+        <v>3608.2</v>
       </c>
       <c r="D39" t="n">
-        <v>0.0605322893706616</v>
+        <v>0.2121884028757643</v>
       </c>
       <c r="E39" t="n">
-        <v>-0.0446597913703177</v>
+        <v>0.0986541623530845</v>
       </c>
       <c r="F39" t="n">
-        <v>0.2131486847552024</v>
+        <v>0.3754431441314374</v>
       </c>
       <c r="G39" t="n">
-        <v>0.2490575159641548</v>
+        <v>0.3799179980680944</v>
       </c>
       <c r="H39" t="n">
-        <v>0.26285707513478</v>
+        <v>0.412878775391977</v>
       </c>
       <c r="I39" t="n">
-        <v>55.89253731343283</v>
+        <v>82.37681159420292</v>
       </c>
       <c r="J39" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K39" t="n">
         <v>48.69</v>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M39" t="n">
         <v>48.69</v>
       </c>
       <c r="N39" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O39" t="n">
-        <v>89.36170212765957</v>
+        <v>91.48936170212764</v>
       </c>
       <c r="P39" t="n">
-        <v>69.34834042553192</v>
+        <v>61.77387234042553</v>
       </c>
       <c r="Q39" t="b">
         <v>0</v>
@@ -3249,48 +3249,48 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>203.24</v>
+        <v>210.21</v>
       </c>
       <c r="D40" t="n">
-        <v>0.0399099467867376</v>
+        <v>0.0916030534351146</v>
       </c>
       <c r="E40" t="n">
-        <v>-0.0524058187243564</v>
+        <v>0.0213789417423837</v>
       </c>
       <c r="F40" t="n">
-        <v>-0.1801532876159741</v>
+        <v>-0.156155915057605</v>
       </c>
       <c r="G40" t="n">
-        <v>-0.1442444564070217</v>
+        <v>-0.151681061120948</v>
       </c>
       <c r="H40" t="n">
-        <v>-0.1304448972363965</v>
+        <v>-0.1187202837970654</v>
       </c>
       <c r="I40" t="n">
-        <v>65.35936420179684</v>
+        <v>74.43096859943513</v>
       </c>
       <c r="J40" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K40" t="n">
         <v>45.44</v>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M40" t="n">
         <v>45.44</v>
       </c>
       <c r="N40" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O40" t="n">
-        <v>29.78723404255319</v>
+        <v>36.17021276595745</v>
       </c>
       <c r="P40" t="n">
-        <v>56.13344680851064</v>
+        <v>53.4100425531915</v>
       </c>
       <c r="Q40" t="b">
         <v>0</v>
@@ -3314,48 +3314,48 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>780.85</v>
+        <v>802.75</v>
       </c>
       <c r="D41" t="n">
-        <v>-0.06647139697531231</v>
+        <v>-0.0330643218501566</v>
       </c>
       <c r="E41" t="n">
-        <v>-0.18029603191266</v>
+        <v>-0.1436876633420449</v>
       </c>
       <c r="F41" t="n">
-        <v>-0.2599981046247157</v>
+        <v>-0.2308613586279583</v>
       </c>
       <c r="G41" t="n">
-        <v>-0.2240892734157633</v>
+        <v>-0.2263865046913012</v>
       </c>
       <c r="H41" t="n">
-        <v>-0.2102897142451381</v>
+        <v>-0.1934257273674187</v>
       </c>
       <c r="I41" t="n">
-        <v>38.64358883786651</v>
+        <v>51.98506956226672</v>
       </c>
       <c r="J41" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="K41" t="n">
         <v>48.05</v>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M41" t="n">
         <v>48.05</v>
       </c>
       <c r="N41" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="O41" t="n">
-        <v>8.51063829787234</v>
+        <v>17.02127659574468</v>
       </c>
       <c r="P41" t="n">
-        <v>32.92212765957446</v>
+        <v>46.62425531914894</v>
       </c>
       <c r="Q41" t="b">
         <v>0</v>
@@ -3379,48 +3379,48 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>628.85</v>
+        <v>622.8</v>
       </c>
       <c r="D42" t="n">
-        <v>0.1107480349730638</v>
+        <v>0.089287275907302</v>
       </c>
       <c r="E42" t="n">
-        <v>-0.0945284377249819</v>
+        <v>-0.0839829386674511</v>
       </c>
       <c r="F42" t="n">
-        <v>-0.1801173402868318</v>
+        <v>-0.1979911145451033</v>
       </c>
       <c r="G42" t="n">
-        <v>-0.1442085090778794</v>
+        <v>-0.1935162606084463</v>
       </c>
       <c r="H42" t="n">
-        <v>-0.1304089499072541</v>
+        <v>-0.1605554832845637</v>
       </c>
       <c r="I42" t="n">
-        <v>68.36242109171927</v>
+        <v>71.85792349726773</v>
       </c>
       <c r="J42" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K42" t="n">
         <v>47.66</v>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M42" t="n">
         <v>47.66</v>
       </c>
       <c r="N42" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O42" t="n">
-        <v>31.91489361702128</v>
+        <v>21.27659574468085</v>
       </c>
       <c r="P42" t="n">
-        <v>57.44697872340426</v>
+        <v>51.31931914893617</v>
       </c>
       <c r="Q42" t="b">
         <v>0</v>
@@ -3444,48 +3444,48 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>431.75</v>
+        <v>436.65</v>
       </c>
       <c r="D43" t="n">
-        <v>0.0279761904761903</v>
+        <v>0.0627966411098939</v>
       </c>
       <c r="E43" t="n">
-        <v>-0.07676681278734079</v>
+        <v>-0.0482781168265039</v>
       </c>
       <c r="F43" t="n">
-        <v>-0.05005500550055</v>
+        <v>-0.0418038183015141</v>
       </c>
       <c r="G43" t="n">
-        <v>-0.0141461742915977</v>
+        <v>-0.0373289643648571</v>
       </c>
       <c r="H43" t="n">
-        <v>-0.0003466151209724</v>
+        <v>-0.0043681870409745</v>
       </c>
       <c r="I43" t="n">
-        <v>67.50599520383693</v>
+        <v>71.20418848167542</v>
       </c>
       <c r="J43" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K43" t="n">
         <v>51.48</v>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M43" t="n">
         <v>51.48</v>
       </c>
       <c r="N43" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O43" t="n">
-        <v>55.31914893617022</v>
+        <v>53.19148936170212</v>
       </c>
       <c r="P43" t="n">
-        <v>63.65582978723404</v>
+        <v>59.23029787234042</v>
       </c>
       <c r="Q43" t="b">
         <v>0</v>
@@ -3509,48 +3509,48 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>258.44</v>
+        <v>265.7</v>
       </c>
       <c r="D44" t="n">
-        <v>0.067272351848028</v>
+        <v>0.055621771950735</v>
       </c>
       <c r="E44" t="n">
-        <v>-0.0372881355932203</v>
+        <v>-0.0385380857608106</v>
       </c>
       <c r="F44" t="n">
-        <v>-0.123189143341815</v>
+        <v>-0.0954893617021277</v>
       </c>
       <c r="G44" t="n">
-        <v>-0.08728031213286259</v>
+        <v>-0.0910145077654707</v>
       </c>
       <c r="H44" t="n">
-        <v>-0.0734807529622374</v>
+        <v>-0.0580537304415881</v>
       </c>
       <c r="I44" t="n">
-        <v>67.82283015795473</v>
+        <v>86.53573956121728</v>
       </c>
       <c r="J44" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K44" t="n">
         <v>47.2</v>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M44" t="n">
         <v>47.2</v>
       </c>
       <c r="N44" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O44" t="n">
-        <v>42.5531914893617</v>
+        <v>44.68085106382978</v>
       </c>
       <c r="P44" t="n">
-        <v>59.39063829787234</v>
+        <v>51.81617021276596</v>
       </c>
       <c r="Q44" t="b">
         <v>0</v>
@@ -3574,25 +3574,25 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>94.26000000000001</v>
+        <v>98.81</v>
       </c>
       <c r="D45" t="n">
-        <v>-0.0651591788158285</v>
+        <v>-0.0347758132265312</v>
       </c>
       <c r="E45" t="n">
-        <v>-0.1468139029688631</v>
+        <v>-0.0844992124525155</v>
       </c>
       <c r="F45" t="n">
-        <v>-0.3420813847979339</v>
+        <v>-0.3098414472305649</v>
       </c>
       <c r="G45" t="n">
-        <v>-0.3061725535889815</v>
+        <v>-0.3053665932939079</v>
       </c>
       <c r="H45" t="n">
-        <v>-0.2923729944183563</v>
+        <v>-0.2724058159700253</v>
       </c>
       <c r="I45" t="n">
-        <v>45.60067681895093</v>
+        <v>59.3356242840779</v>
       </c>
       <c r="J45" t="n">
         <v>60</v>
@@ -3602,7 +3602,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M45" t="n">
@@ -3639,48 +3639,48 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>499.7</v>
+        <v>526.35</v>
       </c>
       <c r="D46" t="n">
-        <v>0.0108222918984524</v>
+        <v>0.0625820127182799</v>
       </c>
       <c r="E46" t="n">
-        <v>-0.170209232813019</v>
+        <v>-0.1181940023454514</v>
       </c>
       <c r="F46" t="n">
-        <v>-0.2221962798661375</v>
+        <v>-0.1631290245647507</v>
       </c>
       <c r="G46" t="n">
-        <v>-0.1862874486571851</v>
+        <v>-0.1586541706280937</v>
       </c>
       <c r="H46" t="n">
-        <v>-0.1724878894865599</v>
+        <v>-0.1256933933042111</v>
       </c>
       <c r="I46" t="n">
-        <v>50.55886736214605</v>
+        <v>68.45345889170591</v>
       </c>
       <c r="J46" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K46" t="n">
         <v>49.61</v>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M46" t="n">
         <v>49.61</v>
       </c>
       <c r="N46" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O46" t="n">
-        <v>21.27659574468085</v>
+        <v>34.04255319148936</v>
       </c>
       <c r="P46" t="n">
-        <v>48.09931914893617</v>
+        <v>58.65251063829788</v>
       </c>
       <c r="Q46" t="b">
         <v>0</v>
@@ -3704,25 +3704,25 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>1001.35</v>
+        <v>1043.85</v>
       </c>
       <c r="D47" t="n">
-        <v>0.0903794849458268</v>
+        <v>0.1215751584828621</v>
       </c>
       <c r="E47" t="n">
-        <v>0.1397757668886234</v>
+        <v>0.2331364441819254</v>
       </c>
       <c r="F47" t="n">
-        <v>0.2329618912762421</v>
+        <v>0.2750091608647855</v>
       </c>
       <c r="G47" t="n">
-        <v>0.2688707224851945</v>
+        <v>0.2794840148014426</v>
       </c>
       <c r="H47" t="n">
-        <v>0.2826702816558197</v>
+        <v>0.3124447921253251</v>
       </c>
       <c r="I47" t="n">
-        <v>46.44575828406435</v>
+        <v>58.38972517608065</v>
       </c>
       <c r="J47" t="n">
         <v>80</v>
@@ -3732,7 +3732,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M47" t="n">
@@ -3742,10 +3742,10 @@
         <v>80</v>
       </c>
       <c r="O47" t="n">
-        <v>91.48936170212764</v>
+        <v>87.2340425531915</v>
       </c>
       <c r="P47" t="n">
-        <v>69.02987234042553</v>
+        <v>68.17880851063831</v>
       </c>
       <c r="Q47" t="b">
         <v>0</v>
@@ -3769,25 +3769,25 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>14248</v>
+        <v>14364</v>
       </c>
       <c r="D48" t="n">
-        <v>0.018878718535469</v>
+        <v>0.0281296972299762</v>
       </c>
       <c r="E48" t="n">
-        <v>-0.0425374638801155</v>
+        <v>-0.0070510161758606</v>
       </c>
       <c r="F48" t="n">
-        <v>0.0502727406752174</v>
+        <v>0.06803479812625469</v>
       </c>
       <c r="G48" t="n">
-        <v>0.08618157188416981</v>
+        <v>0.07250965206291179</v>
       </c>
       <c r="H48" t="n">
-        <v>0.0999811310547951</v>
+        <v>0.1054704293867944</v>
       </c>
       <c r="I48" t="n">
-        <v>56.38389031705226</v>
+        <v>66.58171392163109</v>
       </c>
       <c r="J48" t="n">
         <v>60</v>
@@ -3797,7 +3797,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M48" t="n">
@@ -3807,10 +3807,10 @@
         <v>60</v>
       </c>
       <c r="O48" t="n">
-        <v>65.95744680851064</v>
+        <v>63.82978723404256</v>
       </c>
       <c r="P48" t="n">
-        <v>57.30748936170212</v>
+        <v>56.88195744680851</v>
       </c>
       <c r="Q48" t="b">
         <v>0</v>
@@ -3936,57 +3936,57 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>LUMAXTECH</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Lighting</t>
+          <t>Forgings</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1725.6</v>
+        <v>1798.8</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1735582154515775</v>
+        <v>0.0107889413351314</v>
       </c>
       <c r="E2" t="n">
-        <v>0.033479068096065</v>
+        <v>0.2370538477408708</v>
       </c>
       <c r="F2" t="n">
-        <v>0.5505436247641295</v>
+        <v>0.4179410373640233</v>
       </c>
       <c r="G2" t="n">
-        <v>0.5864524559730819</v>
+        <v>0.4224158913006803</v>
       </c>
       <c r="H2" t="n">
-        <v>0.6002520151437072</v>
+        <v>0.4553766686245629</v>
       </c>
       <c r="I2" t="n">
-        <v>63.34236369793431</v>
+        <v>67.79620853080567</v>
       </c>
       <c r="J2" t="n">
         <v>80</v>
       </c>
       <c r="K2" t="n">
-        <v>54.51</v>
+        <v>54.83</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M2" t="n">
-        <v>54.51</v>
+        <v>54.83</v>
       </c>
       <c r="N2" t="n">
         <v>80</v>
       </c>
       <c r="O2" t="n">
-        <v>100</v>
+        <v>95.74468085106383</v>
       </c>
       <c r="P2" t="n">
-        <v>73.804</v>
+        <v>73.08093617021277</v>
       </c>
       <c r="Q2" t="b">
         <v>0</v>
@@ -4001,57 +4001,57 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>LUMAXTECH</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Forgings</t>
+          <t>Lighting</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1739.4</v>
+        <v>1823.3</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.0321072839574869</v>
+        <v>0.3093716337522441</v>
       </c>
       <c r="E3" t="n">
-        <v>0.1725765134151273</v>
+        <v>0.1515821385713383</v>
       </c>
       <c r="F3" t="n">
-        <v>0.3711177676178465</v>
+        <v>0.6435009915269514</v>
       </c>
       <c r="G3" t="n">
-        <v>0.4070265988267989</v>
+        <v>0.6479758454636084</v>
       </c>
       <c r="H3" t="n">
-        <v>0.4208261579974242</v>
+        <v>0.680936622787491</v>
       </c>
       <c r="I3" t="n">
-        <v>53.27849588719154</v>
+        <v>78.54170134842684</v>
       </c>
       <c r="J3" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K3" t="n">
-        <v>54.83</v>
+        <v>54.51</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M3" t="n">
-        <v>54.83</v>
+        <v>54.51</v>
       </c>
       <c r="N3" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O3" t="n">
-        <v>95.74468085106383</v>
+        <v>100</v>
       </c>
       <c r="P3" t="n">
-        <v>73.08093617021277</v>
+        <v>69.804</v>
       </c>
       <c r="Q3" t="b">
         <v>0</v>
@@ -4066,57 +4066,57 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>GNA</t>
+          <t>LUMAXIND</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Axles</t>
+          <t>Lighting</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>409.65</v>
+        <v>5571.6</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.0271906910472572</v>
+        <v>0.1253484144617249</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0656867845993756</v>
+        <v>0.0054317423080394</v>
       </c>
       <c r="F4" t="n">
-        <v>0.3096227621483374</v>
+        <v>0.3048854747294955</v>
       </c>
       <c r="G4" t="n">
-        <v>0.3455315933572898</v>
+        <v>0.3093603286661526</v>
       </c>
       <c r="H4" t="n">
-        <v>0.359331152527915</v>
+        <v>0.3423211059900352</v>
       </c>
       <c r="I4" t="n">
-        <v>60.09417304296643</v>
+        <v>70.03147953830012</v>
       </c>
       <c r="J4" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K4" t="n">
-        <v>54.47</v>
+        <v>57.69</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M4" t="n">
-        <v>54.47</v>
+        <v>57.69</v>
       </c>
       <c r="N4" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O4" t="n">
-        <v>93.61702127659576</v>
+        <v>89.36170212765957</v>
       </c>
       <c r="P4" t="n">
-        <v>72.51140425531915</v>
+        <v>68.94834042553191</v>
       </c>
       <c r="Q4" t="b">
         <v>0</v>
@@ -4131,57 +4131,57 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SANSERA</t>
+          <t>GNA</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Forgings</t>
+          <t>Axles</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>2251.7</v>
+        <v>443</v>
       </c>
       <c r="D5" t="n">
-        <v>0.0339808054369288</v>
+        <v>0.0650318547902393</v>
       </c>
       <c r="E5" t="n">
-        <v>0.1575673452601274</v>
+        <v>0.2054421768707484</v>
       </c>
       <c r="F5" t="n">
-        <v>0.4941605839416056</v>
+        <v>0.3809226932668328</v>
       </c>
       <c r="G5" t="n">
-        <v>0.5300694151505581</v>
+        <v>0.3853975472034898</v>
       </c>
       <c r="H5" t="n">
-        <v>0.5438689743211833</v>
+        <v>0.4183583245273724</v>
       </c>
       <c r="I5" t="n">
-        <v>56.48050579557426</v>
+        <v>73.69423286180631</v>
       </c>
       <c r="J5" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K5" t="n">
-        <v>48.59</v>
+        <v>54.47</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M5" t="n">
-        <v>48.59</v>
+        <v>54.47</v>
       </c>
       <c r="N5" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O5" t="n">
-        <v>97.87234042553192</v>
+        <v>93.61702127659576</v>
       </c>
       <c r="P5" t="n">
-        <v>71.0104680851064</v>
+        <v>68.51140425531915</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
@@ -4196,57 +4196,57 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BHARATSE</t>
+          <t>WHEELS</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Seating</t>
+          <t>Wheels</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>176.74</v>
+        <v>1043.85</v>
       </c>
       <c r="D6" t="n">
-        <v>0.0257094771052173</v>
+        <v>0.1215751584828621</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0405039444248203</v>
+        <v>0.2331364441819254</v>
       </c>
       <c r="F6" t="n">
-        <v>0.1704635761589403</v>
+        <v>0.2750091608647855</v>
       </c>
       <c r="G6" t="n">
-        <v>0.2063724073678927</v>
+        <v>0.2794840148014426</v>
       </c>
       <c r="H6" t="n">
-        <v>0.220171966538518</v>
+        <v>0.3124447921253251</v>
       </c>
       <c r="I6" t="n">
-        <v>61.80000000000001</v>
+        <v>58.38972517608065</v>
       </c>
       <c r="J6" t="n">
         <v>80</v>
       </c>
       <c r="K6" t="n">
-        <v>52.61</v>
+        <v>46.83</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M6" t="n">
-        <v>52.61</v>
+        <v>46.83</v>
       </c>
       <c r="N6" t="n">
         <v>80</v>
       </c>
       <c r="O6" t="n">
-        <v>82.97872340425532</v>
+        <v>87.2340425531915</v>
       </c>
       <c r="P6" t="n">
-        <v>69.63974468085107</v>
+        <v>68.17880851063831</v>
       </c>
       <c r="Q6" t="b">
         <v>0</v>
@@ -4261,57 +4261,57 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SHRIPISTON</t>
+          <t>SANSERA</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Engine/Parts</t>
+          <t>Forgings</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>3223.7</v>
+        <v>2337.5</v>
       </c>
       <c r="D7" t="n">
-        <v>0.0605322893706616</v>
+        <v>0.1240142335064435</v>
       </c>
       <c r="E7" t="n">
-        <v>-0.0446597913703177</v>
+        <v>0.2342256718939752</v>
       </c>
       <c r="F7" t="n">
-        <v>0.2131486847552024</v>
+        <v>0.5838867055156525</v>
       </c>
       <c r="G7" t="n">
-        <v>0.2490575159641548</v>
+        <v>0.5883615594523095</v>
       </c>
       <c r="H7" t="n">
-        <v>0.26285707513478</v>
+        <v>0.6213223367761921</v>
       </c>
       <c r="I7" t="n">
-        <v>55.89253731343283</v>
+        <v>78.09085681426104</v>
       </c>
       <c r="J7" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K7" t="n">
-        <v>48.69</v>
+        <v>48.59</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M7" t="n">
-        <v>48.69</v>
+        <v>48.59</v>
       </c>
       <c r="N7" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O7" t="n">
-        <v>89.36170212765957</v>
+        <v>97.87234042553192</v>
       </c>
       <c r="P7" t="n">
-        <v>69.34834042553192</v>
+        <v>67.0104680851064</v>
       </c>
       <c r="Q7" t="b">
         <v>0</v>
@@ -4326,57 +4326,57 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CRAFTSMAN</t>
+          <t>BHARATSE</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Castings</t>
+          <t>Seating</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>7408.5</v>
+        <v>176.93</v>
       </c>
       <c r="D8" t="n">
-        <v>0.01133028462221</v>
+        <v>0.0441428149896725</v>
       </c>
       <c r="E8" t="n">
-        <v>-0.0509223674096848</v>
+        <v>0.0601593864221943</v>
       </c>
       <c r="F8" t="n">
-        <v>0.08924501948099681</v>
+        <v>0.2036054421768707</v>
       </c>
       <c r="G8" t="n">
-        <v>0.1251538506899492</v>
+        <v>0.2080802961135277</v>
       </c>
       <c r="H8" t="n">
-        <v>0.1389534098605744</v>
+        <v>0.2410410734374103</v>
       </c>
       <c r="I8" t="n">
-        <v>62.77992277992279</v>
+        <v>72.18861485962464</v>
       </c>
       <c r="J8" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K8" t="n">
-        <v>54.65</v>
+        <v>52.61</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M8" t="n">
-        <v>54.65</v>
+        <v>52.61</v>
       </c>
       <c r="N8" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O8" t="n">
-        <v>76.59574468085107</v>
+        <v>82.97872340425532</v>
       </c>
       <c r="P8" t="n">
-        <v>69.17914893617021</v>
+        <v>65.63974468085107</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
@@ -4391,57 +4391,57 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>WHEELS</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Wheels</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1001.35</v>
+        <v>554.25</v>
       </c>
       <c r="D9" t="n">
-        <v>0.0903794849458268</v>
+        <v>0.08612580834803051</v>
       </c>
       <c r="E9" t="n">
-        <v>0.1397757668886234</v>
+        <v>0.1974721832127037</v>
       </c>
       <c r="F9" t="n">
-        <v>0.2329618912762421</v>
+        <v>0.2579437131184747</v>
       </c>
       <c r="G9" t="n">
-        <v>0.2688707224851945</v>
+        <v>0.2624185670551318</v>
       </c>
       <c r="H9" t="n">
-        <v>0.2826702816558197</v>
+        <v>0.2953793443790143</v>
       </c>
       <c r="I9" t="n">
-        <v>46.44575828406435</v>
+        <v>72.81105990783408</v>
       </c>
       <c r="J9" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K9" t="n">
-        <v>46.83</v>
+        <v>49.66</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M9" t="n">
-        <v>46.83</v>
+        <v>49.66</v>
       </c>
       <c r="N9" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O9" t="n">
-        <v>91.48936170212764</v>
+        <v>85.1063829787234</v>
       </c>
       <c r="P9" t="n">
-        <v>69.02987234042553</v>
+        <v>64.88527659574468</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -4456,57 +4456,57 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>CRAFTSMAN</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Castings</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>523.05</v>
+        <v>7430</v>
       </c>
       <c r="D10" t="n">
-        <v>0.0129756947806718</v>
+        <v>0.0103345118302964</v>
       </c>
       <c r="E10" t="n">
-        <v>0.1039468130012661</v>
+        <v>-0.0309116994913264</v>
       </c>
       <c r="F10" t="n">
-        <v>0.2035204786010123</v>
+        <v>0.0970837947582132</v>
       </c>
       <c r="G10" t="n">
-        <v>0.2394293098099646</v>
+        <v>0.1015586486948703</v>
       </c>
       <c r="H10" t="n">
-        <v>0.2532288689805899</v>
+        <v>0.1345194260187528</v>
       </c>
       <c r="I10" t="n">
-        <v>55.91549295774645</v>
+        <v>77.63528307788552</v>
       </c>
       <c r="J10" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K10" t="n">
-        <v>49.66</v>
+        <v>54.65</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M10" t="n">
-        <v>49.66</v>
+        <v>54.65</v>
       </c>
       <c r="N10" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O10" t="n">
-        <v>85.1063829787234</v>
+        <v>72.3404255319149</v>
       </c>
       <c r="P10" t="n">
-        <v>68.88527659574468</v>
+        <v>64.32808510638299</v>
       </c>
       <c r="Q10" t="b">
         <v>0</v>
@@ -4530,48 +4530,48 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>438.6</v>
+        <v>440.15</v>
       </c>
       <c r="D11" t="n">
-        <v>0.08389966637835169</v>
+        <v>0.08304625984251961</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.0646193218170184</v>
+        <v>-0.0640085061137692</v>
       </c>
       <c r="F11" t="n">
-        <v>-0.1791896696921493</v>
+        <v>-0.1540457428406688</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.1432808384831969</v>
+        <v>-0.1495708889040118</v>
       </c>
       <c r="H11" t="n">
-        <v>-0.1294812793125717</v>
+        <v>-0.1166101115801292</v>
       </c>
       <c r="I11" t="n">
-        <v>65.04605936540432</v>
+        <v>76.76886792452831</v>
       </c>
       <c r="J11" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K11" t="n">
         <v>71.28</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M11" t="n">
         <v>71.28</v>
       </c>
       <c r="N11" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O11" t="n">
-        <v>34.04255319148936</v>
+        <v>38.29787234042553</v>
       </c>
       <c r="P11" t="n">
-        <v>67.32051063829788</v>
+        <v>64.17157446808511</v>
       </c>
       <c r="Q11" t="b">
         <v>1</v>
@@ -4586,7 +4586,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>PRICOLLTD</t>
+          <t>MOTHERSON</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -4595,48 +4595,48 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>571.5</v>
+        <v>122.16</v>
       </c>
       <c r="D12" t="n">
-        <v>0.0366406675131507</v>
+        <v>0.0165598735125238</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.1407953093287228</v>
+        <v>0.034290068580137</v>
       </c>
       <c r="F12" t="n">
-        <v>0.06992417860151651</v>
+        <v>0.1209396219489813</v>
       </c>
       <c r="G12" t="n">
-        <v>0.1058330098104689</v>
+        <v>0.1254144758856383</v>
       </c>
       <c r="H12" t="n">
-        <v>0.1196325689810942</v>
+        <v>0.1583752532095209</v>
       </c>
       <c r="I12" t="n">
-        <v>61.90028222013171</v>
+        <v>71.80061607392888</v>
       </c>
       <c r="J12" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K12" t="n">
-        <v>49.98</v>
+        <v>51.57</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M12" t="n">
-        <v>49.98</v>
+        <v>51.57</v>
       </c>
       <c r="N12" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O12" t="n">
-        <v>72.3404255319149</v>
+        <v>76.59574468085107</v>
       </c>
       <c r="P12" t="n">
-        <v>66.46008510638299</v>
+        <v>63.94714893617022</v>
       </c>
       <c r="Q12" t="b">
         <v>0</v>
@@ -4651,63 +4651,63 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>FIEMIND</t>
+          <t>MENONBE</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Lighting</t>
+          <t>Bearings</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>2158.2</v>
+        <v>119.83</v>
       </c>
       <c r="D13" t="n">
-        <v>0.02231064374023</v>
+        <v>-0.0557875659916475</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.0914372316241476</v>
+        <v>-0.0211566737461199</v>
       </c>
       <c r="F13" t="n">
-        <v>0.0660936573799642</v>
+        <v>-0.094939577039275</v>
       </c>
       <c r="G13" t="n">
-        <v>0.1020024885889165</v>
+        <v>-0.09046472310261799</v>
       </c>
       <c r="H13" t="n">
-        <v>0.1158020477595418</v>
+        <v>-0.0575039457787354</v>
       </c>
       <c r="I13" t="n">
-        <v>60.1514215080346</v>
+        <v>63.114161849711</v>
       </c>
       <c r="J13" t="n">
         <v>80</v>
       </c>
       <c r="K13" t="n">
-        <v>49.06</v>
+        <v>52.38</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M13" t="n">
-        <v>49.06</v>
+        <v>52.38</v>
       </c>
       <c r="N13" t="n">
         <v>80</v>
       </c>
       <c r="O13" t="n">
-        <v>68.08510638297872</v>
+        <v>46.80851063829788</v>
       </c>
       <c r="P13" t="n">
-        <v>65.24102127659575</v>
+        <v>62.31370212765957</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
       </c>
       <c r="R13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S13" t="b">
         <v>0</v>
@@ -4716,57 +4716,57 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>LUMAXIND</t>
+          <t>SHRIPISTON</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Lighting</t>
+          <t>Engine/Parts</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>5304</v>
+        <v>3608.2</v>
       </c>
       <c r="D14" t="n">
-        <v>0.0127935841130417</v>
+        <v>0.2121884028757643</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.0519259987487711</v>
+        <v>0.0986541623530845</v>
       </c>
       <c r="F14" t="n">
-        <v>0.2074578277596923</v>
+        <v>0.3754431441314374</v>
       </c>
       <c r="G14" t="n">
-        <v>0.2433666589686447</v>
+        <v>0.3799179980680944</v>
       </c>
       <c r="H14" t="n">
-        <v>0.25716621813927</v>
+        <v>0.412878775391977</v>
       </c>
       <c r="I14" t="n">
-        <v>56.58836629725861</v>
+        <v>82.37681159420292</v>
       </c>
       <c r="J14" t="n">
         <v>60</v>
       </c>
       <c r="K14" t="n">
-        <v>57.69</v>
+        <v>48.69</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M14" t="n">
-        <v>57.69</v>
+        <v>48.69</v>
       </c>
       <c r="N14" t="n">
         <v>60</v>
       </c>
       <c r="O14" t="n">
-        <v>87.2340425531915</v>
+        <v>91.48936170212764</v>
       </c>
       <c r="P14" t="n">
-        <v>64.5228085106383</v>
+        <v>61.77387234042553</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
@@ -4781,63 +4781,63 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SUPRAJIT</t>
+          <t>FIEMIND</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Cables</t>
+          <t>Lighting</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>431.75</v>
+        <v>2216.6</v>
       </c>
       <c r="D15" t="n">
-        <v>0.0279761904761903</v>
+        <v>0.0547202131709174</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.07676681278734079</v>
+        <v>-0.0474021229962612</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.05005500550055</v>
+        <v>0.0796882610813443</v>
       </c>
       <c r="G15" t="n">
-        <v>-0.0141461742915977</v>
+        <v>0.08416311501800131</v>
       </c>
       <c r="H15" t="n">
-        <v>-0.0003466151209724</v>
+        <v>0.1171238923418839</v>
       </c>
       <c r="I15" t="n">
-        <v>67.50599520383693</v>
+        <v>71.80433039294304</v>
       </c>
       <c r="J15" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K15" t="n">
-        <v>51.48</v>
+        <v>49.06</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M15" t="n">
-        <v>51.48</v>
+        <v>49.06</v>
       </c>
       <c r="N15" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O15" t="n">
-        <v>55.31914893617022</v>
+        <v>70.21276595744681</v>
       </c>
       <c r="P15" t="n">
-        <v>63.65582978723404</v>
+        <v>61.66655319148936</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
       </c>
       <c r="R15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S15" t="b">
         <v>0</v>
@@ -4846,63 +4846,63 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>JBMA</t>
+          <t>PRICOLLTD</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>604.95</v>
+        <v>583.75</v>
       </c>
       <c r="D16" t="n">
-        <v>0.1818892253589918</v>
+        <v>0.0777254684759531</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.09084761045987361</v>
+        <v>-0.1101371951219511</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.1780012229091649</v>
+        <v>0.06982497938238789</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.1420923917002126</v>
+        <v>0.07429983331904499</v>
       </c>
       <c r="H16" t="n">
-        <v>-0.1282928325295873</v>
+        <v>0.1072606106429275</v>
       </c>
       <c r="I16" t="n">
-        <v>59.04944791166589</v>
+        <v>74.43810801744381</v>
       </c>
       <c r="J16" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K16" t="n">
-        <v>56.91</v>
+        <v>49.98</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="M16" t="n">
-        <v>56.91</v>
+        <v>49.98</v>
       </c>
       <c r="N16" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O16" t="n">
-        <v>36.17021276595745</v>
+        <v>65.95744680851064</v>
       </c>
       <c r="P16" t="n">
-        <v>61.99804255319149</v>
+        <v>61.18348936170213</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>
       </c>
       <c r="R16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S16" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
chore: auto-refresh NSE data and pipeline outputs (2026-04-13)
</commit_message>
<xml_diff>
--- a/working-sector/output/auto_components_comprehensive_report.xlsx
+++ b/working-sector/output/auto_components_comprehensive_report.xlsx
@@ -435,7 +435,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
     </row>
@@ -447,7 +447,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
     </row>
@@ -779,25 +779,25 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1798.8</v>
+        <v>1801.3</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0107889413351314</v>
+        <v>0.0753387857441347</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2370538477408708</v>
+        <v>0.2470058843890619</v>
       </c>
       <c r="F2" t="n">
-        <v>0.4179410373640233</v>
+        <v>0.4153374715172466</v>
       </c>
       <c r="G2" t="n">
-        <v>0.4224158913006803</v>
+        <v>0.4544531553648288</v>
       </c>
       <c r="H2" t="n">
-        <v>0.4553766686245629</v>
+        <v>0.4662696774455371</v>
       </c>
       <c r="I2" t="n">
-        <v>67.79620853080567</v>
+        <v>62.69558056546801</v>
       </c>
       <c r="J2" t="n">
         <v>80</v>
@@ -807,7 +807,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M2" t="n">
@@ -844,25 +844,25 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1078</v>
+        <v>1078.2</v>
       </c>
       <c r="D3" t="n">
-        <v>0.008890968647636799</v>
+        <v>0.0641531780497433</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.1511811023622047</v>
+        <v>-0.1373019683149303</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.1787292396769769</v>
+        <v>-0.1829961354853375</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.1742543857403199</v>
+        <v>-0.1438804516377554</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.1412936084164373</v>
+        <v>-0.132063929557047</v>
       </c>
       <c r="I3" t="n">
-        <v>57.53807895554864</v>
+        <v>51.21428571428571</v>
       </c>
       <c r="J3" t="n">
         <v>60</v>
@@ -872,7 +872,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M3" t="n">
@@ -909,48 +909,48 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>37330</v>
+        <v>36615</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1924612681680242</v>
+        <v>0.2130197117773729</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.0344024831867563</v>
+        <v>-0.0363205684958547</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.064059170114078</v>
+        <v>-0.0797939180698668</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.0595843161774209</v>
+        <v>-0.0406782342222846</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.0266235388535384</v>
+        <v>-0.0288617121415762</v>
       </c>
       <c r="I4" t="n">
-        <v>85.5840208423795</v>
+        <v>78.95436420026584</v>
       </c>
       <c r="J4" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K4" t="n">
         <v>53.48</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M4" t="n">
         <v>53.48</v>
       </c>
       <c r="N4" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O4" t="n">
-        <v>51.06382978723404</v>
+        <v>53.19148936170212</v>
       </c>
       <c r="P4" t="n">
-        <v>55.6047659574468</v>
+        <v>60.03029787234042</v>
       </c>
       <c r="Q4" t="b">
         <v>0</v>
@@ -974,48 +974,48 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>324.5</v>
+        <v>324.8</v>
       </c>
       <c r="D5" t="n">
-        <v>0.0467741935483871</v>
+        <v>0.0950775455158461</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.0802154195011338</v>
+        <v>-0.0624909799393851</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.2367399741267787</v>
+        <v>-0.2164053075995174</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.2322651201901217</v>
+        <v>-0.1772896237519353</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.1993043428662391</v>
+        <v>-0.1654731016712269</v>
       </c>
       <c r="I5" t="n">
-        <v>70.27027027027027</v>
+        <v>67.34828496042218</v>
       </c>
       <c r="J5" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K5" t="n">
         <v>51.12</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M5" t="n">
         <v>51.12</v>
       </c>
       <c r="N5" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O5" t="n">
-        <v>14.8936170212766</v>
+        <v>21.27659574468085</v>
       </c>
       <c r="P5" t="n">
-        <v>51.42672340425532</v>
+        <v>56.70331914893617</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
@@ -1039,48 +1039,48 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>122.16</v>
+        <v>119.11</v>
       </c>
       <c r="D6" t="n">
-        <v>0.0165598735125238</v>
+        <v>0.046476893340362</v>
       </c>
       <c r="E6" t="n">
-        <v>0.034290068580137</v>
+        <v>0.0300069180214459</v>
       </c>
       <c r="F6" t="n">
-        <v>0.1209396219489813</v>
+        <v>0.09195086175284189</v>
       </c>
       <c r="G6" t="n">
-        <v>0.1254144758856383</v>
+        <v>0.131066545600424</v>
       </c>
       <c r="H6" t="n">
-        <v>0.1583752532095209</v>
+        <v>0.1428830676811324</v>
       </c>
       <c r="I6" t="n">
-        <v>71.80061607392888</v>
+        <v>61.65984804208066</v>
       </c>
       <c r="J6" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="K6" t="n">
         <v>51.57</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M6" t="n">
         <v>51.57</v>
       </c>
       <c r="N6" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="O6" t="n">
-        <v>76.59574468085107</v>
+        <v>74.46808510638297</v>
       </c>
       <c r="P6" t="n">
-        <v>63.94714893617022</v>
+        <v>59.5216170212766</v>
       </c>
       <c r="Q6" t="b">
         <v>0</v>
@@ -1104,48 +1104,48 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2744.8</v>
+        <v>2715.5</v>
       </c>
       <c r="D7" t="n">
-        <v>0.0765188061340551</v>
+        <v>0.1046700838011553</v>
       </c>
       <c r="E7" t="n">
-        <v>0.09463609172482559</v>
+        <v>0.1072375127420999</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.1903005988377237</v>
+        <v>-0.1844610625581884</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.1858257449010667</v>
+        <v>-0.1453453787106062</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.1528649675771841</v>
+        <v>-0.1335288566298978</v>
       </c>
       <c r="I7" t="n">
-        <v>72.26740403383218</v>
+        <v>63.44007319304669</v>
       </c>
       <c r="J7" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K7" t="n">
         <v>48.73</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M7" t="n">
         <v>48.73</v>
       </c>
       <c r="N7" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O7" t="n">
-        <v>23.40425531914894</v>
+        <v>25.53191489361702</v>
       </c>
       <c r="P7" t="n">
-        <v>52.17285106382979</v>
+        <v>56.59838297872341</v>
       </c>
       <c r="Q7" t="b">
         <v>0</v>
@@ -1169,25 +1169,25 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>554.25</v>
+        <v>569.3</v>
       </c>
       <c r="D8" t="n">
-        <v>0.08612580834803051</v>
+        <v>0.1712786750334327</v>
       </c>
       <c r="E8" t="n">
-        <v>0.1974721832127037</v>
+        <v>0.2385510714674208</v>
       </c>
       <c r="F8" t="n">
-        <v>0.2579437131184747</v>
+        <v>0.305135259055479</v>
       </c>
       <c r="G8" t="n">
-        <v>0.2624185670551318</v>
+        <v>0.3442509429030611</v>
       </c>
       <c r="H8" t="n">
-        <v>0.2953793443790143</v>
+        <v>0.3560674649837695</v>
       </c>
       <c r="I8" t="n">
-        <v>72.81105990783408</v>
+        <v>73.72773536895671</v>
       </c>
       <c r="J8" t="n">
         <v>70</v>
@@ -1197,7 +1197,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M8" t="n">
@@ -1207,10 +1207,10 @@
         <v>70</v>
       </c>
       <c r="O8" t="n">
-        <v>85.1063829787234</v>
+        <v>89.36170212765957</v>
       </c>
       <c r="P8" t="n">
-        <v>64.88527659574468</v>
+        <v>65.73634042553192</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
@@ -1234,48 +1234,48 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>438.15</v>
+        <v>432.4</v>
       </c>
       <c r="D9" t="n">
-        <v>0.0490841613791452</v>
+        <v>0.0801898576067947</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.1573228195018753</v>
+        <v>-0.1427438540840603</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.0957589516045815</v>
+        <v>-0.1003848954540725</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.0912840976679245</v>
+        <v>-0.0612692116064904</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.0583233203440419</v>
+        <v>-0.049452689525782</v>
       </c>
       <c r="I9" t="n">
-        <v>77.86589762076422</v>
+        <v>69.81402002861229</v>
       </c>
       <c r="J9" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="K9" t="n">
         <v>53.44</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M9" t="n">
         <v>53.44</v>
       </c>
       <c r="N9" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="O9" t="n">
-        <v>42.5531914893617</v>
+        <v>46.80851063829788</v>
       </c>
       <c r="P9" t="n">
-        <v>49.88663829787235</v>
+        <v>54.73770212765958</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -1299,48 +1299,48 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>136705</v>
+        <v>134315</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.009419948552588601</v>
+        <v>-0.0044841387488882</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.08078940290478751</v>
+        <v>-0.086882626873789</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.08282455551828249</v>
+        <v>-0.1028021776159781</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.07834970158162539</v>
+        <v>-0.0636864937683959</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.0453889242577428</v>
+        <v>-0.0518699716876875</v>
       </c>
       <c r="I10" t="n">
-        <v>79.19362867098059</v>
+        <v>66.83493185259969</v>
       </c>
       <c r="J10" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="K10" t="n">
         <v>49.41</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M10" t="n">
         <v>49.41</v>
       </c>
       <c r="N10" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="O10" t="n">
-        <v>48.93617021276596</v>
+        <v>44.68085106382978</v>
       </c>
       <c r="P10" t="n">
-        <v>49.55123404255319</v>
+        <v>52.70017021276595</v>
       </c>
       <c r="Q10" t="b">
         <v>0</v>
@@ -1376,10 +1376,10 @@
         <v>-0.0042030657656173</v>
       </c>
       <c r="G11" t="n">
-        <v>0.0002717881710396</v>
+        <v>0.0349126180819647</v>
       </c>
       <c r="H11" t="n">
-        <v>0.0332325654949222</v>
+        <v>0.0467291401626731</v>
       </c>
       <c r="I11" t="n">
         <v>27.6054590570719</v>
@@ -1392,7 +1392,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M11" t="n">
@@ -1429,48 +1429,48 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>440.15</v>
+        <v>435.5</v>
       </c>
       <c r="D12" t="n">
-        <v>0.08304625984251961</v>
+        <v>0.0825254784986329</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.0640085061137692</v>
+        <v>-0.08277169334456611</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.1540457428406688</v>
+        <v>-0.1571511515386104</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.1495708889040118</v>
+        <v>-0.1180354676910283</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.1166101115801292</v>
+        <v>-0.1062189456103199</v>
       </c>
       <c r="I12" t="n">
-        <v>76.76886792452831</v>
+        <v>64.6589259796807</v>
       </c>
       <c r="J12" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K12" t="n">
         <v>71.28</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M12" t="n">
         <v>71.28</v>
       </c>
       <c r="N12" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O12" t="n">
-        <v>38.29787234042553</v>
+        <v>34.04255319148936</v>
       </c>
       <c r="P12" t="n">
-        <v>64.17157446808511</v>
+        <v>67.32051063829788</v>
       </c>
       <c r="Q12" t="b">
         <v>1</v>
@@ -1494,25 +1494,25 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1721</v>
+        <v>1690.5</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.0558481457098968</v>
+        <v>-0.0462085308056872</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.1000836645053336</v>
+        <v>-0.1161246470772769</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.0277385458448674</v>
+        <v>-0.0392702887019776</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.0232636919082104</v>
+        <v>-0.0001546048543955</v>
       </c>
       <c r="H13" t="n">
-        <v>0.0096970854156721</v>
+        <v>0.0116619172263128</v>
       </c>
       <c r="I13" t="n">
-        <v>68.26640548481879</v>
+        <v>62.83658310120704</v>
       </c>
       <c r="J13" t="n">
         <v>60</v>
@@ -1522,7 +1522,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M13" t="n">
@@ -1559,25 +1559,25 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>590.35</v>
+        <v>578.8</v>
       </c>
       <c r="D14" t="n">
-        <v>0.0262494567579314</v>
+        <v>0.0525550100018183</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.1351450336946967</v>
+        <v>-0.1339218913661529</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.2641321283889062</v>
+        <v>-0.3073240785064625</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.2596572744522492</v>
+        <v>-0.2682083946588803</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.2266964971283666</v>
+        <v>-0.256391872578172</v>
       </c>
       <c r="I14" t="n">
-        <v>64.55479452054794</v>
+        <v>56.36994219653178</v>
       </c>
       <c r="J14" t="n">
         <v>60</v>
@@ -1587,7 +1587,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M14" t="n">
@@ -1624,48 +1624,48 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>101.95</v>
+        <v>105.26</v>
       </c>
       <c r="D15" t="n">
-        <v>0.0381873727087576</v>
+        <v>0.07958974358974361</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.0378444696111739</v>
+        <v>0.0024761904761905</v>
       </c>
       <c r="F15" t="n">
-        <v>0.1475686627645205</v>
+        <v>0.1725520775314695</v>
       </c>
       <c r="G15" t="n">
-        <v>0.1520435167011775</v>
+        <v>0.2116677613790516</v>
       </c>
       <c r="H15" t="n">
-        <v>0.1850042940250601</v>
+        <v>0.22348428345976</v>
       </c>
       <c r="I15" t="n">
-        <v>65.49032914828641</v>
+        <v>67.98866855524079</v>
       </c>
       <c r="J15" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K15" t="n">
         <v>51.91</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M15" t="n">
         <v>51.91</v>
       </c>
       <c r="N15" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O15" t="n">
-        <v>78.72340425531915</v>
+        <v>82.97872340425532</v>
       </c>
       <c r="P15" t="n">
-        <v>60.50868085106383</v>
+        <v>69.35974468085107</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
@@ -1689,48 +1689,48 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>176.93</v>
+        <v>174.84</v>
       </c>
       <c r="D16" t="n">
-        <v>0.0441428149896725</v>
+        <v>0.1005224397305972</v>
       </c>
       <c r="E16" t="n">
-        <v>0.0601593864221943</v>
+        <v>0.0730330182889407</v>
       </c>
       <c r="F16" t="n">
-        <v>0.2036054421768707</v>
+        <v>0.1355458855621225</v>
       </c>
       <c r="G16" t="n">
-        <v>0.2080802961135277</v>
+        <v>0.1746615694097046</v>
       </c>
       <c r="H16" t="n">
-        <v>0.2410410734374103</v>
+        <v>0.186478091490413</v>
       </c>
       <c r="I16" t="n">
-        <v>72.18861485962464</v>
+        <v>66.25653126580144</v>
       </c>
       <c r="J16" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K16" t="n">
         <v>52.61</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M16" t="n">
         <v>52.61</v>
       </c>
       <c r="N16" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O16" t="n">
-        <v>82.97872340425532</v>
+        <v>78.72340425531915</v>
       </c>
       <c r="P16" t="n">
-        <v>65.63974468085107</v>
+        <v>68.78868085106383</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>
@@ -1754,25 +1754,25 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>7430</v>
+        <v>7398.5</v>
       </c>
       <c r="D17" t="n">
-        <v>0.0103345118302964</v>
+        <v>0.1085555888522624</v>
       </c>
       <c r="E17" t="n">
-        <v>-0.0309116994913264</v>
+        <v>-0.0291956436163233</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0970837947582132</v>
+        <v>0.0917072450936993</v>
       </c>
       <c r="G17" t="n">
-        <v>0.1015586486948703</v>
+        <v>0.1308229289412814</v>
       </c>
       <c r="H17" t="n">
-        <v>0.1345194260187528</v>
+        <v>0.1426394510219898</v>
       </c>
       <c r="I17" t="n">
-        <v>77.63528307788552</v>
+        <v>70.8286464191976</v>
       </c>
       <c r="J17" t="n">
         <v>70</v>
@@ -1782,7 +1782,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M17" t="n">
@@ -1819,48 +1819,48 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>673.45</v>
+        <v>689.2</v>
       </c>
       <c r="D18" t="n">
-        <v>-0.0538774936779993</v>
+        <v>0.0242235101798187</v>
       </c>
       <c r="E18" t="n">
-        <v>0.1302341193253335</v>
+        <v>0.1711129991503823</v>
       </c>
       <c r="F18" t="n">
-        <v>0.0278540903540902</v>
+        <v>0.0390471883009198</v>
       </c>
       <c r="G18" t="n">
-        <v>0.0323289442907472</v>
+        <v>0.0781628721485019</v>
       </c>
       <c r="H18" t="n">
-        <v>0.0652897216146298</v>
+        <v>0.08997939422921029</v>
       </c>
       <c r="I18" t="n">
-        <v>53.88020833333336</v>
+        <v>47.66548463356975</v>
       </c>
       <c r="J18" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K18" t="n">
         <v>49.92</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M18" t="n">
         <v>49.92</v>
       </c>
       <c r="N18" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O18" t="n">
         <v>61.70212765957447</v>
       </c>
       <c r="P18" t="n">
-        <v>56.3084255319149</v>
+        <v>64.30842553191489</v>
       </c>
       <c r="Q18" t="b">
         <v>0</v>
@@ -1884,48 +1884,48 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2433</v>
+        <v>2391.8</v>
       </c>
       <c r="D19" t="n">
-        <v>-0.0111765901239585</v>
+        <v>-0.0048264957976199</v>
       </c>
       <c r="E19" t="n">
-        <v>-0.0682444852941175</v>
+        <v>-0.0877955758962623</v>
       </c>
       <c r="F19" t="n">
-        <v>-0.1644343704924789</v>
+        <v>-0.1693696822364992</v>
       </c>
       <c r="G19" t="n">
-        <v>-0.1599595165558218</v>
+        <v>-0.1302539983889171</v>
       </c>
       <c r="H19" t="n">
-        <v>-0.1269987392319392</v>
+        <v>-0.1184374763082087</v>
       </c>
       <c r="I19" t="n">
-        <v>69.82605608803692</v>
+        <v>63.17991631799165</v>
       </c>
       <c r="J19" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K19" t="n">
         <v>51.27</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M19" t="n">
         <v>51.27</v>
       </c>
       <c r="N19" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O19" t="n">
         <v>31.91489361702128</v>
       </c>
       <c r="P19" t="n">
-        <v>58.89097872340426</v>
+        <v>50.89097872340426</v>
       </c>
       <c r="Q19" t="b">
         <v>0</v>
@@ -1949,48 +1949,48 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2216.6</v>
+        <v>2164.9</v>
       </c>
       <c r="D20" t="n">
-        <v>0.0547202131709174</v>
+        <v>0.0571833186834651</v>
       </c>
       <c r="E20" t="n">
-        <v>-0.0474021229962612</v>
+        <v>-0.0295844726343628</v>
       </c>
       <c r="F20" t="n">
-        <v>0.0796882610813443</v>
+        <v>0.0601860920666015</v>
       </c>
       <c r="G20" t="n">
-        <v>0.08416311501800131</v>
+        <v>0.0993017759141836</v>
       </c>
       <c r="H20" t="n">
-        <v>0.1171238923418839</v>
+        <v>0.111118297994892</v>
       </c>
       <c r="I20" t="n">
-        <v>71.80433039294304</v>
+        <v>62.61298274445357</v>
       </c>
       <c r="J20" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K20" t="n">
         <v>49.06</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M20" t="n">
         <v>49.06</v>
       </c>
       <c r="N20" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O20" t="n">
-        <v>70.21276595744681</v>
+        <v>65.95744680851064</v>
       </c>
       <c r="P20" t="n">
-        <v>61.66655319148936</v>
+        <v>64.81548936170213</v>
       </c>
       <c r="Q20" t="b">
         <v>0</v>
@@ -2014,48 +2014,48 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>933.5</v>
+        <v>927.65</v>
       </c>
       <c r="D21" t="n">
-        <v>0.0610365992270971</v>
+        <v>0.101198955365622</v>
       </c>
       <c r="E21" t="n">
-        <v>-0.0783887846776582</v>
+        <v>-0.0497336611350134</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.2515834201876051</v>
+        <v>-0.2767989397364934</v>
       </c>
       <c r="G21" t="n">
-        <v>-0.2471085662509481</v>
+        <v>-0.2376832558889112</v>
       </c>
       <c r="H21" t="n">
-        <v>-0.2141477889270655</v>
+        <v>-0.2258667338082028</v>
       </c>
       <c r="I21" t="n">
-        <v>71.15146512587702</v>
+        <v>65.43463381245722</v>
       </c>
       <c r="J21" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K21" t="n">
         <v>48.43</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M21" t="n">
         <v>48.43</v>
       </c>
       <c r="N21" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O21" t="n">
         <v>8.51063829787234</v>
       </c>
       <c r="P21" t="n">
-        <v>49.07412765957447</v>
+        <v>53.07412765957447</v>
       </c>
       <c r="Q21" t="b">
         <v>0</v>
@@ -2079,48 +2079,48 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>443</v>
+        <v>440.1</v>
       </c>
       <c r="D22" t="n">
-        <v>0.0650318547902393</v>
+        <v>0.1331101956745624</v>
       </c>
       <c r="E22" t="n">
-        <v>0.2054421768707484</v>
+        <v>0.2255639097744359</v>
       </c>
       <c r="F22" t="n">
-        <v>0.3809226932668328</v>
+        <v>0.3894238358326756</v>
       </c>
       <c r="G22" t="n">
-        <v>0.3853975472034898</v>
+        <v>0.4285395196802577</v>
       </c>
       <c r="H22" t="n">
-        <v>0.4183583245273724</v>
+        <v>0.4403560417609661</v>
       </c>
       <c r="I22" t="n">
-        <v>73.69423286180631</v>
+        <v>69.98535871156662</v>
       </c>
       <c r="J22" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K22" t="n">
         <v>54.47</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M22" t="n">
         <v>54.47</v>
       </c>
       <c r="N22" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O22" t="n">
-        <v>93.61702127659576</v>
+        <v>91.48936170212764</v>
       </c>
       <c r="P22" t="n">
-        <v>68.51140425531915</v>
+        <v>72.08587234042552</v>
       </c>
       <c r="Q22" t="b">
         <v>0</v>
@@ -2144,48 +2144,48 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>357.9</v>
+        <v>370.2</v>
       </c>
       <c r="D23" t="n">
-        <v>0.0088794926004227</v>
+        <v>0.0557536004562955</v>
       </c>
       <c r="E23" t="n">
-        <v>-0.07002728335715221</v>
+        <v>-0.0259176424154716</v>
       </c>
       <c r="F23" t="n">
-        <v>-0.1407994238386749</v>
+        <v>-0.1266808209483368</v>
       </c>
       <c r="G23" t="n">
-        <v>-0.1363245699020179</v>
+        <v>-0.0875651371007547</v>
       </c>
       <c r="H23" t="n">
-        <v>-0.1033637925781353</v>
+        <v>-0.0757486150200463</v>
       </c>
       <c r="I23" t="n">
-        <v>67.93708408953418</v>
+        <v>70.57190449750139</v>
       </c>
       <c r="J23" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K23" t="n">
         <v>49.7</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M23" t="n">
         <v>49.7</v>
       </c>
       <c r="N23" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O23" t="n">
-        <v>40.42553191489361</v>
+        <v>42.5531914893617</v>
       </c>
       <c r="P23" t="n">
-        <v>51.96510638297872</v>
+        <v>56.39063829787234</v>
       </c>
       <c r="Q23" t="b">
         <v>0</v>
@@ -2209,25 +2209,25 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>124.8</v>
+        <v>122.92</v>
       </c>
       <c r="D24" t="n">
-        <v>0.0194412677667048</v>
+        <v>0.0455937393671317</v>
       </c>
       <c r="E24" t="n">
-        <v>-0.027355623100304</v>
+        <v>-0.0433496770176667</v>
       </c>
       <c r="F24" t="n">
-        <v>0.1587743732590529</v>
+        <v>0.1396254403856851</v>
       </c>
       <c r="G24" t="n">
-        <v>0.16324922719571</v>
+        <v>0.1787411242332672</v>
       </c>
       <c r="H24" t="n">
-        <v>0.1962100045195925</v>
+        <v>0.1905576463139756</v>
       </c>
       <c r="I24" t="n">
-        <v>64.52067669172934</v>
+        <v>56.55066530194473</v>
       </c>
       <c r="J24" t="n">
         <v>60</v>
@@ -2237,7 +2237,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M24" t="n">
@@ -2274,25 +2274,25 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>611.45</v>
+        <v>624.6</v>
       </c>
       <c r="D25" t="n">
-        <v>0.1894757319326916</v>
+        <v>0.2636050981185516</v>
       </c>
       <c r="E25" t="n">
-        <v>-0.0406370126304228</v>
+        <v>0.0177611210689261</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.1689432551817872</v>
+        <v>-0.1391951488423374</v>
       </c>
       <c r="G25" t="n">
-        <v>-0.1644684012451301</v>
+        <v>-0.1000794649947552</v>
       </c>
       <c r="H25" t="n">
-        <v>-0.1315076239212476</v>
+        <v>-0.0882629429140469</v>
       </c>
       <c r="I25" t="n">
-        <v>68.79150066401063</v>
+        <v>65.42083578575632</v>
       </c>
       <c r="J25" t="n">
         <v>80</v>
@@ -2302,7 +2302,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M25" t="n">
@@ -2312,10 +2312,10 @@
         <v>80</v>
       </c>
       <c r="O25" t="n">
-        <v>29.78723404255319</v>
+        <v>36.17021276595745</v>
       </c>
       <c r="P25" t="n">
-        <v>60.72144680851064</v>
+        <v>61.99804255319149</v>
       </c>
       <c r="Q25" t="b">
         <v>0</v>
@@ -2339,25 +2339,25 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>133.88</v>
+        <v>132.2</v>
       </c>
       <c r="D26" t="n">
-        <v>-0.009543537767256</v>
+        <v>0.0147374884863369</v>
       </c>
       <c r="E26" t="n">
-        <v>-0.1223861029170764</v>
+        <v>-0.1213027583914921</v>
       </c>
       <c r="F26" t="n">
-        <v>-0.2373682711478212</v>
+        <v>-0.2413634798576839</v>
       </c>
       <c r="G26" t="n">
-        <v>-0.2328934172111642</v>
+        <v>-0.2022477960101018</v>
       </c>
       <c r="H26" t="n">
-        <v>-0.1999326398872816</v>
+        <v>-0.1904312739293934</v>
       </c>
       <c r="I26" t="n">
-        <v>68.64864864864862</v>
+        <v>62.08963745361115</v>
       </c>
       <c r="J26" t="n">
         <v>60</v>
@@ -2367,7 +2367,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M26" t="n">
@@ -2377,10 +2377,10 @@
         <v>60</v>
       </c>
       <c r="O26" t="n">
-        <v>12.76595744680851</v>
+        <v>10.63829787234042</v>
       </c>
       <c r="P26" t="n">
-        <v>47.1691914893617</v>
+        <v>46.74365957446808</v>
       </c>
       <c r="Q26" t="b">
         <v>0</v>
@@ -2404,48 +2404,48 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>5571.6</v>
+        <v>5399.4</v>
       </c>
       <c r="D27" t="n">
-        <v>0.1253484144617249</v>
+        <v>0.1217201620442505</v>
       </c>
       <c r="E27" t="n">
-        <v>0.0054317423080394</v>
+        <v>-0.0133576975788031</v>
       </c>
       <c r="F27" t="n">
-        <v>0.3048854747294955</v>
+        <v>0.2355889150781482</v>
       </c>
       <c r="G27" t="n">
-        <v>0.3093603286661526</v>
+        <v>0.2747045989257304</v>
       </c>
       <c r="H27" t="n">
-        <v>0.3423211059900352</v>
+        <v>0.2865211210064388</v>
       </c>
       <c r="I27" t="n">
-        <v>70.03147953830012</v>
+        <v>60.04729402912881</v>
       </c>
       <c r="J27" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="K27" t="n">
         <v>57.69</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M27" t="n">
         <v>57.69</v>
       </c>
       <c r="N27" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="O27" t="n">
-        <v>89.36170212765957</v>
+        <v>85.1063829787234</v>
       </c>
       <c r="P27" t="n">
-        <v>68.94834042553191</v>
+        <v>64.09727659574469</v>
       </c>
       <c r="Q27" t="b">
         <v>0</v>
@@ -2469,25 +2469,25 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1823.3</v>
+        <v>1847.8</v>
       </c>
       <c r="D28" t="n">
-        <v>0.3093716337522441</v>
+        <v>0.2885634588563459</v>
       </c>
       <c r="E28" t="n">
-        <v>0.1515821385713383</v>
+        <v>0.2070024168789599</v>
       </c>
       <c r="F28" t="n">
-        <v>0.6435009915269514</v>
+        <v>0.65336435218325</v>
       </c>
       <c r="G28" t="n">
-        <v>0.6479758454636084</v>
+        <v>0.6924800360308321</v>
       </c>
       <c r="H28" t="n">
-        <v>0.680936622787491</v>
+        <v>0.7042965581115405</v>
       </c>
       <c r="I28" t="n">
-        <v>78.54170134842684</v>
+        <v>75.85237916822781</v>
       </c>
       <c r="J28" t="n">
         <v>70</v>
@@ -2497,7 +2497,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M28" t="n">
@@ -2534,54 +2534,54 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>514.35</v>
+        <v>509.25</v>
       </c>
       <c r="D29" t="n">
-        <v>0.0690013509300635</v>
+        <v>0.059062077570968</v>
       </c>
       <c r="E29" t="n">
-        <v>-0.1233915636983382</v>
+        <v>-0.1197061365600691</v>
       </c>
       <c r="F29" t="n">
-        <v>-0.0321761219305674</v>
+        <v>-0.0728265817023213</v>
       </c>
       <c r="G29" t="n">
-        <v>-0.0277012679939103</v>
+        <v>-0.0337108978547392</v>
       </c>
       <c r="H29" t="n">
-        <v>0.0052595093299722</v>
+        <v>-0.0218943757740308</v>
       </c>
       <c r="I29" t="n">
-        <v>56.91176470588235</v>
+        <v>45.90956161546426</v>
       </c>
       <c r="J29" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="K29" t="n">
         <v>49.42</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M29" t="n">
         <v>49.42</v>
       </c>
       <c r="N29" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="O29" t="n">
         <v>55.31914893617022</v>
       </c>
       <c r="P29" t="n">
-        <v>54.83182978723404</v>
+        <v>46.83182978723404</v>
       </c>
       <c r="Q29" t="b">
         <v>0</v>
       </c>
       <c r="R29" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S29" t="b">
         <v>0</v>
@@ -2599,25 +2599,25 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>119.83</v>
+        <v>117.86</v>
       </c>
       <c r="D30" t="n">
-        <v>-0.0557875659916475</v>
+        <v>-0.0399934837501018</v>
       </c>
       <c r="E30" t="n">
-        <v>-0.0211566737461199</v>
+        <v>-0.0036351339927297</v>
       </c>
       <c r="F30" t="n">
-        <v>-0.094939577039275</v>
+        <v>-0.090094958696827</v>
       </c>
       <c r="G30" t="n">
-        <v>-0.09046472310261799</v>
+        <v>-0.0509792748492449</v>
       </c>
       <c r="H30" t="n">
-        <v>-0.0575039457787354</v>
+        <v>-0.0391627527685365</v>
       </c>
       <c r="I30" t="n">
-        <v>63.114161849711</v>
+        <v>59.78781656399726</v>
       </c>
       <c r="J30" t="n">
         <v>80</v>
@@ -2627,7 +2627,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M30" t="n">
@@ -2637,10 +2637,10 @@
         <v>80</v>
       </c>
       <c r="O30" t="n">
-        <v>46.80851063829788</v>
+        <v>51.06382978723404</v>
       </c>
       <c r="P30" t="n">
-        <v>62.31370212765957</v>
+        <v>63.1647659574468</v>
       </c>
       <c r="Q30" t="b">
         <v>0</v>
@@ -2664,25 +2664,25 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>39.33</v>
+        <v>38.53</v>
       </c>
       <c r="D31" t="n">
-        <v>-0.0182226660009986</v>
+        <v>-0.0140736949846468</v>
       </c>
       <c r="E31" t="n">
-        <v>-0.1917385943279901</v>
+        <v>-0.1946070234113712</v>
       </c>
       <c r="F31" t="n">
-        <v>-0.1887376237623762</v>
+        <v>-0.2049112670243499</v>
       </c>
       <c r="G31" t="n">
-        <v>-0.1842627698257192</v>
+        <v>-0.1657955831767678</v>
       </c>
       <c r="H31" t="n">
-        <v>-0.1513019925018366</v>
+        <v>-0.1539790610960594</v>
       </c>
       <c r="I31" t="n">
-        <v>69.45701357466061</v>
+        <v>56.35910224438904</v>
       </c>
       <c r="J31" t="n">
         <v>60</v>
@@ -2692,7 +2692,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M31" t="n">
@@ -2702,10 +2702,10 @@
         <v>60</v>
       </c>
       <c r="O31" t="n">
-        <v>25.53191489361702</v>
+        <v>23.40425531914894</v>
       </c>
       <c r="P31" t="n">
-        <v>48.70238297872341</v>
+        <v>48.27685106382979</v>
       </c>
       <c r="Q31" t="b">
         <v>0</v>
@@ -2729,25 +2729,25 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>733.75</v>
+        <v>728.1</v>
       </c>
       <c r="D32" t="n">
-        <v>0.0600260040450735</v>
+        <v>0.1127922971114168</v>
       </c>
       <c r="E32" t="n">
-        <v>-0.07947559904654369</v>
+        <v>-0.0672559569561875</v>
       </c>
       <c r="F32" t="n">
-        <v>-0.370117606661516</v>
+        <v>-0.3301747930082797</v>
       </c>
       <c r="G32" t="n">
-        <v>-0.365642752724859</v>
+        <v>-0.2910591091606975</v>
       </c>
       <c r="H32" t="n">
-        <v>-0.3326819754009764</v>
+        <v>-0.2792425870799891</v>
       </c>
       <c r="I32" t="n">
-        <v>68.2542768273717</v>
+        <v>62.90630975143405</v>
       </c>
       <c r="J32" t="n">
         <v>80</v>
@@ -2757,7 +2757,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M32" t="n">
@@ -2794,48 +2794,48 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>583.75</v>
+        <v>573.1</v>
       </c>
       <c r="D33" t="n">
-        <v>0.0777254684759531</v>
+        <v>0.1088323498113572</v>
       </c>
       <c r="E33" t="n">
-        <v>-0.1101371951219511</v>
+        <v>-0.085089399744572</v>
       </c>
       <c r="F33" t="n">
-        <v>0.06982497938238789</v>
+        <v>0.0615911827359452</v>
       </c>
       <c r="G33" t="n">
-        <v>0.07429983331904499</v>
+        <v>0.1007068665835273</v>
       </c>
       <c r="H33" t="n">
-        <v>0.1072606106429275</v>
+        <v>0.1125233886642357</v>
       </c>
       <c r="I33" t="n">
-        <v>74.43810801744381</v>
+        <v>65.30249110320284</v>
       </c>
       <c r="J33" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K33" t="n">
         <v>49.98</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M33" t="n">
         <v>49.98</v>
       </c>
       <c r="N33" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O33" t="n">
-        <v>65.95744680851064</v>
+        <v>68.08510638297872</v>
       </c>
       <c r="P33" t="n">
-        <v>61.18348936170213</v>
+        <v>65.60902127659575</v>
       </c>
       <c r="Q33" t="b">
         <v>0</v>
@@ -2871,10 +2871,10 @@
         <v>-0.2401052253975846</v>
       </c>
       <c r="G34" t="n">
-        <v>-0.2356303714609275</v>
+        <v>-0.2009895415500024</v>
       </c>
       <c r="H34" t="n">
-        <v>-0.202669594137045</v>
+        <v>-0.1891730194692941</v>
       </c>
       <c r="I34" t="n">
         <v>63.3225806451613</v>
@@ -2887,7 +2887,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M34" t="n">
@@ -2897,10 +2897,10 @@
         <v>80</v>
       </c>
       <c r="O34" t="n">
-        <v>10.63829787234042</v>
+        <v>12.76595744680851</v>
       </c>
       <c r="P34" t="n">
-        <v>54.47965957446809</v>
+        <v>54.90519148936171</v>
       </c>
       <c r="Q34" t="b">
         <v>0</v>
@@ -2924,25 +2924,25 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>116.72</v>
+        <v>116.31</v>
       </c>
       <c r="D35" t="n">
-        <v>0.0439137823092745</v>
+        <v>0.1002743354460315</v>
       </c>
       <c r="E35" t="n">
-        <v>-0.1056624013485556</v>
+        <v>-0.08127962085308039</v>
       </c>
       <c r="F35" t="n">
-        <v>0.1084520417853751</v>
+        <v>0.1136537725009574</v>
       </c>
       <c r="G35" t="n">
-        <v>0.1129268957220321</v>
+        <v>0.1527694563485395</v>
       </c>
       <c r="H35" t="n">
-        <v>0.1458876730459147</v>
+        <v>0.1645859784292479</v>
       </c>
       <c r="I35" t="n">
-        <v>68.52352623039479</v>
+        <v>62.16640502354787</v>
       </c>
       <c r="J35" t="n">
         <v>60</v>
@@ -2952,7 +2952,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M35" t="n">
@@ -2962,10 +2962,10 @@
         <v>60</v>
       </c>
       <c r="O35" t="n">
-        <v>74.46808510638297</v>
+        <v>76.59574468085107</v>
       </c>
       <c r="P35" t="n">
-        <v>58.5216170212766</v>
+        <v>58.94714893617022</v>
       </c>
       <c r="Q35" t="b">
         <v>0</v>
@@ -2989,48 +2989,48 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>492.5</v>
+        <v>484.4</v>
       </c>
       <c r="D36" t="n">
-        <v>0.0028507432294848</v>
+        <v>0.0009298481248063</v>
       </c>
       <c r="E36" t="n">
-        <v>-0.1471861471861472</v>
+        <v>-0.1246046805819102</v>
       </c>
       <c r="F36" t="n">
-        <v>0.0760323355909984</v>
+        <v>0.0481445418154278</v>
       </c>
       <c r="G36" t="n">
-        <v>0.0805071895276554</v>
+        <v>0.08726022566300989</v>
       </c>
       <c r="H36" t="n">
-        <v>0.113467966851538</v>
+        <v>0.0990767477437183</v>
       </c>
       <c r="I36" t="n">
-        <v>71.38728323699422</v>
+        <v>63.13993174061433</v>
       </c>
       <c r="J36" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="K36" t="n">
         <v>47.8</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M36" t="n">
         <v>47.8</v>
       </c>
       <c r="N36" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="O36" t="n">
-        <v>68.08510638297872</v>
+        <v>63.82978723404256</v>
       </c>
       <c r="P36" t="n">
-        <v>52.73702127659575</v>
+        <v>55.88595744680852</v>
       </c>
       <c r="Q36" t="b">
         <v>0</v>
@@ -3054,25 +3054,25 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2337.5</v>
+        <v>2346.2</v>
       </c>
       <c r="D37" t="n">
-        <v>0.1240142335064435</v>
+        <v>0.2010852871915633</v>
       </c>
       <c r="E37" t="n">
-        <v>0.2342256718939752</v>
+        <v>0.2942409532215357</v>
       </c>
       <c r="F37" t="n">
-        <v>0.5838867055156525</v>
+        <v>0.5693645484949832</v>
       </c>
       <c r="G37" t="n">
-        <v>0.5883615594523095</v>
+        <v>0.6084802323425653</v>
       </c>
       <c r="H37" t="n">
-        <v>0.6213223367761921</v>
+        <v>0.6202967544232737</v>
       </c>
       <c r="I37" t="n">
-        <v>78.09085681426104</v>
+        <v>75.09261276966656</v>
       </c>
       <c r="J37" t="n">
         <v>70</v>
@@ -3082,7 +3082,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M37" t="n">
@@ -3119,25 +3119,25 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>831.3</v>
+        <v>814</v>
       </c>
       <c r="D38" t="n">
-        <v>0.0237054368573363</v>
+        <v>0.0439243347226674</v>
       </c>
       <c r="E38" t="n">
-        <v>-0.1033813298818961</v>
+        <v>-0.1032279387462818</v>
       </c>
       <c r="F38" t="n">
-        <v>-0.2138263665594856</v>
+        <v>-0.2398206948076204</v>
       </c>
       <c r="G38" t="n">
-        <v>-0.2093515126228285</v>
+        <v>-0.2007050109600383</v>
       </c>
       <c r="H38" t="n">
-        <v>-0.176390735298946</v>
+        <v>-0.1888884888793299</v>
       </c>
       <c r="I38" t="n">
-        <v>65.65842862412396</v>
+        <v>59.08080059303188</v>
       </c>
       <c r="J38" t="n">
         <v>60</v>
@@ -3147,7 +3147,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M38" t="n">
@@ -3157,10 +3157,10 @@
         <v>60</v>
       </c>
       <c r="O38" t="n">
-        <v>19.14893617021277</v>
+        <v>14.8936170212766</v>
       </c>
       <c r="P38" t="n">
-        <v>47.77778723404256</v>
+        <v>46.92672340425532</v>
       </c>
       <c r="Q38" t="b">
         <v>0</v>
@@ -3184,25 +3184,25 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>3608.2</v>
+        <v>3610.5</v>
       </c>
       <c r="D39" t="n">
-        <v>0.2121884028757643</v>
+        <v>0.2641364097895733</v>
       </c>
       <c r="E39" t="n">
-        <v>0.0986541623530845</v>
+        <v>0.1335237975637322</v>
       </c>
       <c r="F39" t="n">
-        <v>0.3754431441314374</v>
+        <v>0.3922952336881073</v>
       </c>
       <c r="G39" t="n">
-        <v>0.3799179980680944</v>
+        <v>0.4314109175356895</v>
       </c>
       <c r="H39" t="n">
-        <v>0.412878775391977</v>
+        <v>0.4432274396163979</v>
       </c>
       <c r="I39" t="n">
-        <v>82.37681159420292</v>
+        <v>81.59806295399518</v>
       </c>
       <c r="J39" t="n">
         <v>60</v>
@@ -3212,7 +3212,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M39" t="n">
@@ -3222,10 +3222,10 @@
         <v>60</v>
       </c>
       <c r="O39" t="n">
-        <v>91.48936170212764</v>
+        <v>93.61702127659576</v>
       </c>
       <c r="P39" t="n">
-        <v>61.77387234042553</v>
+        <v>62.19940425531915</v>
       </c>
       <c r="Q39" t="b">
         <v>0</v>
@@ -3249,25 +3249,25 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>210.21</v>
+        <v>212.66</v>
       </c>
       <c r="D40" t="n">
-        <v>0.0916030534351146</v>
+        <v>0.1651325882095111</v>
       </c>
       <c r="E40" t="n">
-        <v>0.0213789417423837</v>
+        <v>0.0678383128295254</v>
       </c>
       <c r="F40" t="n">
-        <v>-0.156155915057605</v>
+        <v>-0.1284783410515962</v>
       </c>
       <c r="G40" t="n">
-        <v>-0.151681061120948</v>
+        <v>-0.0893626572040141</v>
       </c>
       <c r="H40" t="n">
-        <v>-0.1187202837970654</v>
+        <v>-0.0775461351233057</v>
       </c>
       <c r="I40" t="n">
-        <v>74.43096859943513</v>
+        <v>75.09305712898528</v>
       </c>
       <c r="J40" t="n">
         <v>70</v>
@@ -3277,7 +3277,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M40" t="n">
@@ -3287,10 +3287,10 @@
         <v>70</v>
       </c>
       <c r="O40" t="n">
-        <v>36.17021276595745</v>
+        <v>40.42553191489361</v>
       </c>
       <c r="P40" t="n">
-        <v>53.4100425531915</v>
+        <v>54.26110638297872</v>
       </c>
       <c r="Q40" t="b">
         <v>0</v>
@@ -3314,25 +3314,25 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>802.75</v>
+        <v>791.2</v>
       </c>
       <c r="D41" t="n">
-        <v>-0.0330643218501566</v>
+        <v>-0.0377622377622377</v>
       </c>
       <c r="E41" t="n">
-        <v>-0.1436876633420449</v>
+        <v>-0.149567367119901</v>
       </c>
       <c r="F41" t="n">
-        <v>-0.2308613586279583</v>
+        <v>-0.2379117703717973</v>
       </c>
       <c r="G41" t="n">
-        <v>-0.2263865046913012</v>
+        <v>-0.1987960865242152</v>
       </c>
       <c r="H41" t="n">
-        <v>-0.1934257273674187</v>
+        <v>-0.1869795644435068</v>
       </c>
       <c r="I41" t="n">
-        <v>51.98506956226672</v>
+        <v>48.69675778766691</v>
       </c>
       <c r="J41" t="n">
         <v>60</v>
@@ -3342,7 +3342,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M41" t="n">
@@ -3379,48 +3379,48 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>622.8</v>
+        <v>614.2</v>
       </c>
       <c r="D42" t="n">
-        <v>0.089287275907302</v>
+        <v>0.1288366109171108</v>
       </c>
       <c r="E42" t="n">
-        <v>-0.0839829386674511</v>
+        <v>-0.0596340809921149</v>
       </c>
       <c r="F42" t="n">
-        <v>-0.1979911145451033</v>
+        <v>-0.2190718372536554</v>
       </c>
       <c r="G42" t="n">
-        <v>-0.1935162606084463</v>
+        <v>-0.1799561534060733</v>
       </c>
       <c r="H42" t="n">
-        <v>-0.1605554832845637</v>
+        <v>-0.1681396313253649</v>
       </c>
       <c r="I42" t="n">
-        <v>71.85792349726773</v>
+        <v>67.73935638616831</v>
       </c>
       <c r="J42" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K42" t="n">
         <v>47.66</v>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M42" t="n">
         <v>47.66</v>
       </c>
       <c r="N42" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O42" t="n">
-        <v>21.27659574468085</v>
+        <v>19.14893617021277</v>
       </c>
       <c r="P42" t="n">
-        <v>51.31931914893617</v>
+        <v>54.89378723404256</v>
       </c>
       <c r="Q42" t="b">
         <v>0</v>
@@ -3444,48 +3444,48 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>436.65</v>
+        <v>411.6</v>
       </c>
       <c r="D43" t="n">
-        <v>0.0627966411098939</v>
+        <v>0.0199479618386817</v>
       </c>
       <c r="E43" t="n">
-        <v>-0.0482781168265039</v>
+        <v>-0.1053146397130746</v>
       </c>
       <c r="F43" t="n">
-        <v>-0.0418038183015141</v>
+        <v>-0.1342938269008307</v>
       </c>
       <c r="G43" t="n">
-        <v>-0.0373289643648571</v>
+        <v>-0.0951781430532485</v>
       </c>
       <c r="H43" t="n">
-        <v>-0.0043681870409745</v>
+        <v>-0.0833616209725401</v>
       </c>
       <c r="I43" t="n">
-        <v>71.20418848167542</v>
+        <v>54.72727272727276</v>
       </c>
       <c r="J43" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="K43" t="n">
         <v>51.48</v>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M43" t="n">
         <v>51.48</v>
       </c>
       <c r="N43" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="O43" t="n">
-        <v>53.19148936170212</v>
+        <v>38.29787234042553</v>
       </c>
       <c r="P43" t="n">
-        <v>59.23029787234042</v>
+        <v>52.25157446808511</v>
       </c>
       <c r="Q43" t="b">
         <v>0</v>
@@ -3509,25 +3509,25 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>265.7</v>
+        <v>265.8</v>
       </c>
       <c r="D44" t="n">
-        <v>0.055621771950735</v>
+        <v>0.0732889158086009</v>
       </c>
       <c r="E44" t="n">
-        <v>-0.0385380857608106</v>
+        <v>-0.0151908114116338</v>
       </c>
       <c r="F44" t="n">
-        <v>-0.0954893617021277</v>
+        <v>-0.0917478216299332</v>
       </c>
       <c r="G44" t="n">
-        <v>-0.0910145077654707</v>
+        <v>-0.052632137782351</v>
       </c>
       <c r="H44" t="n">
-        <v>-0.0580537304415881</v>
+        <v>-0.0408156157016427</v>
       </c>
       <c r="I44" t="n">
-        <v>86.53573956121728</v>
+        <v>87.0979207392927</v>
       </c>
       <c r="J44" t="n">
         <v>60</v>
@@ -3537,7 +3537,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M44" t="n">
@@ -3547,10 +3547,10 @@
         <v>60</v>
       </c>
       <c r="O44" t="n">
-        <v>44.68085106382978</v>
+        <v>48.93617021276596</v>
       </c>
       <c r="P44" t="n">
-        <v>51.81617021276596</v>
+        <v>52.6672340425532</v>
       </c>
       <c r="Q44" t="b">
         <v>0</v>
@@ -3574,25 +3574,25 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>98.81</v>
+        <v>98</v>
       </c>
       <c r="D45" t="n">
-        <v>-0.0347758132265312</v>
+        <v>-0.0191172054849364</v>
       </c>
       <c r="E45" t="n">
-        <v>-0.0844992124525155</v>
+        <v>-0.0853089415717752</v>
       </c>
       <c r="F45" t="n">
-        <v>-0.3098414472305649</v>
+        <v>-0.3099077529751425</v>
       </c>
       <c r="G45" t="n">
-        <v>-0.3053665932939079</v>
+        <v>-0.2707920691275604</v>
       </c>
       <c r="H45" t="n">
-        <v>-0.2724058159700253</v>
+        <v>-0.258975547046852</v>
       </c>
       <c r="I45" t="n">
-        <v>59.3356242840779</v>
+        <v>57.35795454545456</v>
       </c>
       <c r="J45" t="n">
         <v>60</v>
@@ -3602,7 +3602,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M45" t="n">
@@ -3639,48 +3639,48 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>526.35</v>
+        <v>518.35</v>
       </c>
       <c r="D46" t="n">
-        <v>0.0625820127182799</v>
+        <v>0.07821112844513781</v>
       </c>
       <c r="E46" t="n">
-        <v>-0.1181940023454514</v>
+        <v>-0.1093642611683848</v>
       </c>
       <c r="F46" t="n">
-        <v>-0.1631290245647507</v>
+        <v>-0.1811216429699841</v>
       </c>
       <c r="G46" t="n">
-        <v>-0.1586541706280937</v>
+        <v>-0.142005959122402</v>
       </c>
       <c r="H46" t="n">
-        <v>-0.1256933933042111</v>
+        <v>-0.1301894370416936</v>
       </c>
       <c r="I46" t="n">
-        <v>68.45345889170591</v>
+        <v>61.02079395085067</v>
       </c>
       <c r="J46" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K46" t="n">
         <v>49.61</v>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M46" t="n">
         <v>49.61</v>
       </c>
       <c r="N46" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O46" t="n">
-        <v>34.04255319148936</v>
+        <v>29.78723404255319</v>
       </c>
       <c r="P46" t="n">
-        <v>58.65251063829788</v>
+        <v>49.80144680851064</v>
       </c>
       <c r="Q46" t="b">
         <v>0</v>
@@ -3704,25 +3704,25 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>1043.85</v>
+        <v>1022.05</v>
       </c>
       <c r="D47" t="n">
-        <v>0.1215751584828621</v>
+        <v>0.1372538110604204</v>
       </c>
       <c r="E47" t="n">
-        <v>0.2331364441819254</v>
+        <v>0.2600789051904819</v>
       </c>
       <c r="F47" t="n">
-        <v>0.2750091608647855</v>
+        <v>0.2660885723134096</v>
       </c>
       <c r="G47" t="n">
-        <v>0.2794840148014426</v>
+        <v>0.3052042561609918</v>
       </c>
       <c r="H47" t="n">
-        <v>0.3124447921253251</v>
+        <v>0.3170207782417001</v>
       </c>
       <c r="I47" t="n">
-        <v>58.38972517608065</v>
+        <v>49.39104915627291</v>
       </c>
       <c r="J47" t="n">
         <v>80</v>
@@ -3732,7 +3732,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M47" t="n">
@@ -3769,25 +3769,25 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>14364</v>
+        <v>14069</v>
       </c>
       <c r="D48" t="n">
-        <v>0.0281296972299762</v>
+        <v>0.0341811231990591</v>
       </c>
       <c r="E48" t="n">
-        <v>-0.0070510161758606</v>
+        <v>-0.0122858747542825</v>
       </c>
       <c r="F48" t="n">
-        <v>0.06803479812625469</v>
+        <v>0.0626132930513594</v>
       </c>
       <c r="G48" t="n">
-        <v>0.07250965206291179</v>
+        <v>0.1017289768989415</v>
       </c>
       <c r="H48" t="n">
-        <v>0.1054704293867944</v>
+        <v>0.1135454989796499</v>
       </c>
       <c r="I48" t="n">
-        <v>66.58171392163109</v>
+        <v>63.29497274379164</v>
       </c>
       <c r="J48" t="n">
         <v>60</v>
@@ -3797,7 +3797,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M48" t="n">
@@ -3807,10 +3807,10 @@
         <v>60</v>
       </c>
       <c r="O48" t="n">
-        <v>63.82978723404256</v>
+        <v>70.21276595744681</v>
       </c>
       <c r="P48" t="n">
-        <v>56.88195744680851</v>
+        <v>58.15855319148936</v>
       </c>
       <c r="Q48" t="b">
         <v>0</v>
@@ -3945,25 +3945,25 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1798.8</v>
+        <v>1801.3</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0107889413351314</v>
+        <v>0.0753387857441347</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2370538477408708</v>
+        <v>0.2470058843890619</v>
       </c>
       <c r="F2" t="n">
-        <v>0.4179410373640233</v>
+        <v>0.4153374715172466</v>
       </c>
       <c r="G2" t="n">
-        <v>0.4224158913006803</v>
+        <v>0.4544531553648288</v>
       </c>
       <c r="H2" t="n">
-        <v>0.4553766686245629</v>
+        <v>0.4662696774455371</v>
       </c>
       <c r="I2" t="n">
-        <v>67.79620853080567</v>
+        <v>62.69558056546801</v>
       </c>
       <c r="J2" t="n">
         <v>80</v>
@@ -3973,7 +3973,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M2" t="n">
@@ -4001,57 +4001,57 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>LUMAXTECH</t>
+          <t>GNA</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Lighting</t>
+          <t>Axles</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1823.3</v>
+        <v>440.1</v>
       </c>
       <c r="D3" t="n">
-        <v>0.3093716337522441</v>
+        <v>0.1331101956745624</v>
       </c>
       <c r="E3" t="n">
-        <v>0.1515821385713383</v>
+        <v>0.2255639097744359</v>
       </c>
       <c r="F3" t="n">
-        <v>0.6435009915269514</v>
+        <v>0.3894238358326756</v>
       </c>
       <c r="G3" t="n">
-        <v>0.6479758454636084</v>
+        <v>0.4285395196802577</v>
       </c>
       <c r="H3" t="n">
-        <v>0.680936622787491</v>
+        <v>0.4403560417609661</v>
       </c>
       <c r="I3" t="n">
-        <v>78.54170134842684</v>
+        <v>69.98535871156662</v>
       </c>
       <c r="J3" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K3" t="n">
-        <v>54.51</v>
+        <v>54.47</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M3" t="n">
-        <v>54.51</v>
+        <v>54.47</v>
       </c>
       <c r="N3" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O3" t="n">
-        <v>100</v>
+        <v>91.48936170212764</v>
       </c>
       <c r="P3" t="n">
-        <v>69.804</v>
+        <v>72.08587234042552</v>
       </c>
       <c r="Q3" t="b">
         <v>0</v>
@@ -4066,7 +4066,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>LUMAXIND</t>
+          <t>LUMAXTECH</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -4075,48 +4075,48 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>5571.6</v>
+        <v>1847.8</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1253484144617249</v>
+        <v>0.2885634588563459</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0054317423080394</v>
+        <v>0.2070024168789599</v>
       </c>
       <c r="F4" t="n">
-        <v>0.3048854747294955</v>
+        <v>0.65336435218325</v>
       </c>
       <c r="G4" t="n">
-        <v>0.3093603286661526</v>
+        <v>0.6924800360308321</v>
       </c>
       <c r="H4" t="n">
-        <v>0.3423211059900352</v>
+        <v>0.7042965581115405</v>
       </c>
       <c r="I4" t="n">
-        <v>70.03147953830012</v>
+        <v>75.85237916822781</v>
       </c>
       <c r="J4" t="n">
         <v>70</v>
       </c>
       <c r="K4" t="n">
-        <v>57.69</v>
+        <v>54.51</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M4" t="n">
-        <v>57.69</v>
+        <v>54.51</v>
       </c>
       <c r="N4" t="n">
         <v>70</v>
       </c>
       <c r="O4" t="n">
-        <v>89.36170212765957</v>
+        <v>100</v>
       </c>
       <c r="P4" t="n">
-        <v>68.94834042553191</v>
+        <v>69.804</v>
       </c>
       <c r="Q4" t="b">
         <v>0</v>
@@ -4131,57 +4131,57 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>GNA</t>
+          <t>BHARATGEAR</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Axles</t>
+          <t>Gears</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>443</v>
+        <v>105.26</v>
       </c>
       <c r="D5" t="n">
-        <v>0.0650318547902393</v>
+        <v>0.07958974358974361</v>
       </c>
       <c r="E5" t="n">
-        <v>0.2054421768707484</v>
+        <v>0.0024761904761905</v>
       </c>
       <c r="F5" t="n">
-        <v>0.3809226932668328</v>
+        <v>0.1725520775314695</v>
       </c>
       <c r="G5" t="n">
-        <v>0.3853975472034898</v>
+        <v>0.2116677613790516</v>
       </c>
       <c r="H5" t="n">
-        <v>0.4183583245273724</v>
+        <v>0.22348428345976</v>
       </c>
       <c r="I5" t="n">
-        <v>73.69423286180631</v>
+        <v>67.98866855524079</v>
       </c>
       <c r="J5" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K5" t="n">
-        <v>54.47</v>
+        <v>51.91</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M5" t="n">
-        <v>54.47</v>
+        <v>51.91</v>
       </c>
       <c r="N5" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O5" t="n">
-        <v>93.61702127659576</v>
+        <v>82.97872340425532</v>
       </c>
       <c r="P5" t="n">
-        <v>68.51140425531915</v>
+        <v>69.35974468085107</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
@@ -4196,57 +4196,57 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>WHEELS</t>
+          <t>BHARATSE</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Wheels</t>
+          <t>Seating</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1043.85</v>
+        <v>174.84</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1215751584828621</v>
+        <v>0.1005224397305972</v>
       </c>
       <c r="E6" t="n">
-        <v>0.2331364441819254</v>
+        <v>0.0730330182889407</v>
       </c>
       <c r="F6" t="n">
-        <v>0.2750091608647855</v>
+        <v>0.1355458855621225</v>
       </c>
       <c r="G6" t="n">
-        <v>0.2794840148014426</v>
+        <v>0.1746615694097046</v>
       </c>
       <c r="H6" t="n">
-        <v>0.3124447921253251</v>
+        <v>0.186478091490413</v>
       </c>
       <c r="I6" t="n">
-        <v>58.38972517608065</v>
+        <v>66.25653126580144</v>
       </c>
       <c r="J6" t="n">
         <v>80</v>
       </c>
       <c r="K6" t="n">
-        <v>46.83</v>
+        <v>52.61</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M6" t="n">
-        <v>46.83</v>
+        <v>52.61</v>
       </c>
       <c r="N6" t="n">
         <v>80</v>
       </c>
       <c r="O6" t="n">
-        <v>87.2340425531915</v>
+        <v>78.72340425531915</v>
       </c>
       <c r="P6" t="n">
-        <v>68.17880851063831</v>
+        <v>68.78868085106383</v>
       </c>
       <c r="Q6" t="b">
         <v>0</v>
@@ -4261,57 +4261,57 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SANSERA</t>
+          <t>WHEELS</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Forgings</t>
+          <t>Wheels</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2337.5</v>
+        <v>1022.05</v>
       </c>
       <c r="D7" t="n">
-        <v>0.1240142335064435</v>
+        <v>0.1372538110604204</v>
       </c>
       <c r="E7" t="n">
-        <v>0.2342256718939752</v>
+        <v>0.2600789051904819</v>
       </c>
       <c r="F7" t="n">
-        <v>0.5838867055156525</v>
+        <v>0.2660885723134096</v>
       </c>
       <c r="G7" t="n">
-        <v>0.5883615594523095</v>
+        <v>0.3052042561609918</v>
       </c>
       <c r="H7" t="n">
-        <v>0.6213223367761921</v>
+        <v>0.3170207782417001</v>
       </c>
       <c r="I7" t="n">
-        <v>78.09085681426104</v>
+        <v>49.39104915627291</v>
       </c>
       <c r="J7" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K7" t="n">
-        <v>48.59</v>
+        <v>46.83</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M7" t="n">
-        <v>48.59</v>
+        <v>46.83</v>
       </c>
       <c r="N7" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O7" t="n">
-        <v>97.87234042553192</v>
+        <v>87.2340425531915</v>
       </c>
       <c r="P7" t="n">
-        <v>67.0104680851064</v>
+        <v>68.17880851063831</v>
       </c>
       <c r="Q7" t="b">
         <v>0</v>
@@ -4326,63 +4326,63 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BHARATSE</t>
+          <t>ASKAUTOLTD</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Seating</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>176.93</v>
+        <v>435.5</v>
       </c>
       <c r="D8" t="n">
-        <v>0.0441428149896725</v>
+        <v>0.0825254784986329</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0601593864221943</v>
+        <v>-0.08277169334456611</v>
       </c>
       <c r="F8" t="n">
-        <v>0.2036054421768707</v>
+        <v>-0.1571511515386104</v>
       </c>
       <c r="G8" t="n">
-        <v>0.2080802961135277</v>
+        <v>-0.1180354676910283</v>
       </c>
       <c r="H8" t="n">
-        <v>0.2410410734374103</v>
+        <v>-0.1062189456103199</v>
       </c>
       <c r="I8" t="n">
-        <v>72.18861485962464</v>
+        <v>64.6589259796807</v>
       </c>
       <c r="J8" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K8" t="n">
-        <v>52.61</v>
+        <v>71.28</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M8" t="n">
-        <v>52.61</v>
+        <v>71.28</v>
       </c>
       <c r="N8" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O8" t="n">
-        <v>82.97872340425532</v>
+        <v>34.04255319148936</v>
       </c>
       <c r="P8" t="n">
-        <v>65.63974468085107</v>
+        <v>67.32051063829788</v>
       </c>
       <c r="Q8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S8" t="b">
         <v>0</v>
@@ -4391,57 +4391,57 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>SANSERA</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Forgings</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>554.25</v>
+        <v>2346.2</v>
       </c>
       <c r="D9" t="n">
-        <v>0.08612580834803051</v>
+        <v>0.2010852871915633</v>
       </c>
       <c r="E9" t="n">
-        <v>0.1974721832127037</v>
+        <v>0.2942409532215357</v>
       </c>
       <c r="F9" t="n">
-        <v>0.2579437131184747</v>
+        <v>0.5693645484949832</v>
       </c>
       <c r="G9" t="n">
-        <v>0.2624185670551318</v>
+        <v>0.6084802323425653</v>
       </c>
       <c r="H9" t="n">
-        <v>0.2953793443790143</v>
+        <v>0.6202967544232737</v>
       </c>
       <c r="I9" t="n">
-        <v>72.81105990783408</v>
+        <v>75.09261276966656</v>
       </c>
       <c r="J9" t="n">
         <v>70</v>
       </c>
       <c r="K9" t="n">
-        <v>49.66</v>
+        <v>48.59</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M9" t="n">
-        <v>49.66</v>
+        <v>48.59</v>
       </c>
       <c r="N9" t="n">
         <v>70</v>
       </c>
       <c r="O9" t="n">
-        <v>85.1063829787234</v>
+        <v>97.87234042553192</v>
       </c>
       <c r="P9" t="n">
-        <v>64.88527659574468</v>
+        <v>67.0104680851064</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -4456,57 +4456,57 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CRAFTSMAN</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Castings</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>7430</v>
+        <v>569.3</v>
       </c>
       <c r="D10" t="n">
-        <v>0.0103345118302964</v>
+        <v>0.1712786750334327</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.0309116994913264</v>
+        <v>0.2385510714674208</v>
       </c>
       <c r="F10" t="n">
-        <v>0.0970837947582132</v>
+        <v>0.305135259055479</v>
       </c>
       <c r="G10" t="n">
-        <v>0.1015586486948703</v>
+        <v>0.3442509429030611</v>
       </c>
       <c r="H10" t="n">
-        <v>0.1345194260187528</v>
+        <v>0.3560674649837695</v>
       </c>
       <c r="I10" t="n">
-        <v>77.63528307788552</v>
+        <v>73.72773536895671</v>
       </c>
       <c r="J10" t="n">
         <v>70</v>
       </c>
       <c r="K10" t="n">
-        <v>54.65</v>
+        <v>49.66</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M10" t="n">
-        <v>54.65</v>
+        <v>49.66</v>
       </c>
       <c r="N10" t="n">
         <v>70</v>
       </c>
       <c r="O10" t="n">
-        <v>72.3404255319149</v>
+        <v>89.36170212765957</v>
       </c>
       <c r="P10" t="n">
-        <v>64.32808510638299</v>
+        <v>65.73634042553192</v>
       </c>
       <c r="Q10" t="b">
         <v>0</v>
@@ -4521,63 +4521,63 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ASKAUTOLTD</t>
+          <t>PRICOLLTD</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>440.15</v>
+        <v>573.1</v>
       </c>
       <c r="D11" t="n">
-        <v>0.08304625984251961</v>
+        <v>0.1088323498113572</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.0640085061137692</v>
+        <v>-0.085089399744572</v>
       </c>
       <c r="F11" t="n">
-        <v>-0.1540457428406688</v>
+        <v>0.0615911827359452</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.1495708889040118</v>
+        <v>0.1007068665835273</v>
       </c>
       <c r="H11" t="n">
-        <v>-0.1166101115801292</v>
+        <v>0.1125233886642357</v>
       </c>
       <c r="I11" t="n">
-        <v>76.76886792452831</v>
+        <v>65.30249110320284</v>
       </c>
       <c r="J11" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K11" t="n">
-        <v>71.28</v>
+        <v>49.98</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M11" t="n">
-        <v>71.28</v>
+        <v>49.98</v>
       </c>
       <c r="N11" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O11" t="n">
-        <v>38.29787234042553</v>
+        <v>68.08510638297872</v>
       </c>
       <c r="P11" t="n">
-        <v>64.17157446808511</v>
+        <v>65.60902127659575</v>
       </c>
       <c r="Q11" t="b">
+        <v>0</v>
+      </c>
+      <c r="R11" t="b">
         <v>1</v>
-      </c>
-      <c r="R11" t="b">
-        <v>0</v>
       </c>
       <c r="S11" t="b">
         <v>0</v>
@@ -4586,57 +4586,57 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>MOTHERSON</t>
+          <t>FIEMIND</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Lighting</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>122.16</v>
+        <v>2164.9</v>
       </c>
       <c r="D12" t="n">
-        <v>0.0165598735125238</v>
+        <v>0.0571833186834651</v>
       </c>
       <c r="E12" t="n">
-        <v>0.034290068580137</v>
+        <v>-0.0295844726343628</v>
       </c>
       <c r="F12" t="n">
-        <v>0.1209396219489813</v>
+        <v>0.0601860920666015</v>
       </c>
       <c r="G12" t="n">
-        <v>0.1254144758856383</v>
+        <v>0.0993017759141836</v>
       </c>
       <c r="H12" t="n">
-        <v>0.1583752532095209</v>
+        <v>0.111118297994892</v>
       </c>
       <c r="I12" t="n">
-        <v>71.80061607392888</v>
+        <v>62.61298274445357</v>
       </c>
       <c r="J12" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K12" t="n">
-        <v>51.57</v>
+        <v>49.06</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M12" t="n">
-        <v>51.57</v>
+        <v>49.06</v>
       </c>
       <c r="N12" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O12" t="n">
-        <v>76.59574468085107</v>
+        <v>65.95744680851064</v>
       </c>
       <c r="P12" t="n">
-        <v>63.94714893617022</v>
+        <v>64.81548936170213</v>
       </c>
       <c r="Q12" t="b">
         <v>0</v>
@@ -4651,63 +4651,63 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MENONBE</t>
+          <t>CRAFTSMAN</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Bearings</t>
+          <t>Castings</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>119.83</v>
+        <v>7398.5</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.0557875659916475</v>
+        <v>0.1085555888522624</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.0211566737461199</v>
+        <v>-0.0291956436163233</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.094939577039275</v>
+        <v>0.0917072450936993</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.09046472310261799</v>
+        <v>0.1308229289412814</v>
       </c>
       <c r="H13" t="n">
-        <v>-0.0575039457787354</v>
+        <v>0.1426394510219898</v>
       </c>
       <c r="I13" t="n">
-        <v>63.114161849711</v>
+        <v>70.8286464191976</v>
       </c>
       <c r="J13" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K13" t="n">
-        <v>52.38</v>
+        <v>54.65</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M13" t="n">
-        <v>52.38</v>
+        <v>54.65</v>
       </c>
       <c r="N13" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O13" t="n">
-        <v>46.80851063829788</v>
+        <v>72.3404255319149</v>
       </c>
       <c r="P13" t="n">
-        <v>62.31370212765957</v>
+        <v>64.32808510638299</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
       </c>
       <c r="R13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S13" t="b">
         <v>0</v>
@@ -4716,57 +4716,57 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SHRIPISTON</t>
+          <t>DIVGIITTS</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Engine/Parts</t>
+          <t>Transmission</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>3608.2</v>
+        <v>689.2</v>
       </c>
       <c r="D14" t="n">
-        <v>0.2121884028757643</v>
+        <v>0.0242235101798187</v>
       </c>
       <c r="E14" t="n">
-        <v>0.0986541623530845</v>
+        <v>0.1711129991503823</v>
       </c>
       <c r="F14" t="n">
-        <v>0.3754431441314374</v>
+        <v>0.0390471883009198</v>
       </c>
       <c r="G14" t="n">
-        <v>0.3799179980680944</v>
+        <v>0.0781628721485019</v>
       </c>
       <c r="H14" t="n">
-        <v>0.412878775391977</v>
+        <v>0.08997939422921029</v>
       </c>
       <c r="I14" t="n">
-        <v>82.37681159420292</v>
+        <v>47.66548463356975</v>
       </c>
       <c r="J14" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K14" t="n">
-        <v>48.69</v>
+        <v>49.92</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M14" t="n">
-        <v>48.69</v>
+        <v>49.92</v>
       </c>
       <c r="N14" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O14" t="n">
-        <v>91.48936170212764</v>
+        <v>61.70212765957447</v>
       </c>
       <c r="P14" t="n">
-        <v>61.77387234042553</v>
+        <v>64.30842553191489</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
@@ -4781,7 +4781,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>FIEMIND</t>
+          <t>LUMAXIND</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -4790,48 +4790,48 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2216.6</v>
+        <v>5399.4</v>
       </c>
       <c r="D15" t="n">
-        <v>0.0547202131709174</v>
+        <v>0.1217201620442505</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.0474021229962612</v>
+        <v>-0.0133576975788031</v>
       </c>
       <c r="F15" t="n">
-        <v>0.0796882610813443</v>
+        <v>0.2355889150781482</v>
       </c>
       <c r="G15" t="n">
-        <v>0.08416311501800131</v>
+        <v>0.2747045989257304</v>
       </c>
       <c r="H15" t="n">
-        <v>0.1171238923418839</v>
+        <v>0.2865211210064388</v>
       </c>
       <c r="I15" t="n">
-        <v>71.80433039294304</v>
+        <v>60.04729402912881</v>
       </c>
       <c r="J15" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="K15" t="n">
-        <v>49.06</v>
+        <v>57.69</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M15" t="n">
-        <v>49.06</v>
+        <v>57.69</v>
       </c>
       <c r="N15" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="O15" t="n">
-        <v>70.21276595744681</v>
+        <v>85.1063829787234</v>
       </c>
       <c r="P15" t="n">
-        <v>61.66655319148936</v>
+        <v>64.09727659574469</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
@@ -4846,63 +4846,63 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>PRICOLLTD</t>
+          <t>MENONBE</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Bearings</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>583.75</v>
+        <v>117.86</v>
       </c>
       <c r="D16" t="n">
-        <v>0.0777254684759531</v>
+        <v>-0.0399934837501018</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.1101371951219511</v>
+        <v>-0.0036351339927297</v>
       </c>
       <c r="F16" t="n">
-        <v>0.06982497938238789</v>
+        <v>-0.090094958696827</v>
       </c>
       <c r="G16" t="n">
-        <v>0.07429983331904499</v>
+        <v>-0.0509792748492449</v>
       </c>
       <c r="H16" t="n">
-        <v>0.1072606106429275</v>
+        <v>-0.0391627527685365</v>
       </c>
       <c r="I16" t="n">
-        <v>74.43810801744381</v>
+        <v>59.78781656399726</v>
       </c>
       <c r="J16" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K16" t="n">
-        <v>49.98</v>
+        <v>52.38</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="M16" t="n">
-        <v>49.98</v>
+        <v>52.38</v>
       </c>
       <c r="N16" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O16" t="n">
-        <v>65.95744680851064</v>
+        <v>51.06382978723404</v>
       </c>
       <c r="P16" t="n">
-        <v>61.18348936170213</v>
+        <v>63.1647659574468</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>
       </c>
       <c r="R16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S16" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
chore: auto-refresh NSE data and pipeline outputs (2026-04-14)
</commit_message>
<xml_diff>
--- a/working-sector/output/auto_components_comprehensive_report.xlsx
+++ b/working-sector/output/auto_components_comprehensive_report.xlsx
@@ -435,7 +435,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
     </row>
@@ -447,7 +447,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
     </row>
@@ -782,22 +782,22 @@
         <v>1801.3</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0753387857441347</v>
+        <v>0.0614614024749557</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2470058843890619</v>
+        <v>0.2366469861320885</v>
       </c>
       <c r="F2" t="n">
-        <v>0.4153374715172466</v>
+        <v>0.4341560509554139</v>
       </c>
       <c r="G2" t="n">
-        <v>0.4544531553648288</v>
+        <v>0.473271734802996</v>
       </c>
       <c r="H2" t="n">
-        <v>0.4662696774455371</v>
+        <v>0.4850882568837044</v>
       </c>
       <c r="I2" t="n">
-        <v>62.69558056546801</v>
+        <v>59.62566844919785</v>
       </c>
       <c r="J2" t="n">
         <v>80</v>
@@ -807,7 +807,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M2" t="n">
@@ -847,22 +847,22 @@
         <v>1078.2</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0641531780497433</v>
+        <v>0.0586156111929307</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.1373019683149303</v>
+        <v>-0.1089256198347107</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.1829961354853375</v>
+        <v>-0.178639445417841</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.1438804516377554</v>
+        <v>-0.1395237615702589</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.132063929557047</v>
+        <v>-0.1277072394895505</v>
       </c>
       <c r="I3" t="n">
-        <v>51.21428571428571</v>
+        <v>48.21834723275212</v>
       </c>
       <c r="J3" t="n">
         <v>60</v>
@@ -872,7 +872,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M3" t="n">
@@ -882,10 +882,10 @@
         <v>60</v>
       </c>
       <c r="O3" t="n">
-        <v>27.65957446808511</v>
+        <v>29.78723404255319</v>
       </c>
       <c r="P3" t="n">
-        <v>49.27591489361702</v>
+        <v>49.70144680851064</v>
       </c>
       <c r="Q3" t="b">
         <v>0</v>
@@ -912,22 +912,22 @@
         <v>36615</v>
       </c>
       <c r="D4" t="n">
-        <v>0.2130197117773729</v>
+        <v>0.2062263218580136</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.0363205684958547</v>
+        <v>-0.0277482740308019</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.0797939180698668</v>
+        <v>-0.0746777862016679</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.0406782342222846</v>
+        <v>-0.0355621023540858</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.0288617121415762</v>
+        <v>-0.0237455802733774</v>
       </c>
       <c r="I4" t="n">
-        <v>78.95436420026584</v>
+        <v>78.35990888382688</v>
       </c>
       <c r="J4" t="n">
         <v>70</v>
@@ -937,7 +937,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M4" t="n">
@@ -977,22 +977,22 @@
         <v>324.8</v>
       </c>
       <c r="D5" t="n">
-        <v>0.0950775455158461</v>
+        <v>0.1004573945451465</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.0624909799393851</v>
+        <v>-0.0712038890477552</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.2164053075995174</v>
+        <v>-0.1957409929429243</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.1772896237519353</v>
+        <v>-0.1566253090953422</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.1654731016712269</v>
+        <v>-0.1448087870146338</v>
       </c>
       <c r="I5" t="n">
-        <v>67.34828496042218</v>
+        <v>63.14221891288162</v>
       </c>
       <c r="J5" t="n">
         <v>80</v>
@@ -1002,7 +1002,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M5" t="n">
@@ -1042,22 +1042,22 @@
         <v>119.11</v>
       </c>
       <c r="D6" t="n">
-        <v>0.046476893340362</v>
+        <v>0.0510942463819272</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0300069180214459</v>
+        <v>0.0358292025393511</v>
       </c>
       <c r="F6" t="n">
-        <v>0.09195086175284189</v>
+        <v>0.0833105957253297</v>
       </c>
       <c r="G6" t="n">
-        <v>0.131066545600424</v>
+        <v>0.1224262795729118</v>
       </c>
       <c r="H6" t="n">
-        <v>0.1428830676811324</v>
+        <v>0.1342428016536202</v>
       </c>
       <c r="I6" t="n">
-        <v>61.65984804208066</v>
+        <v>59.27995034140286</v>
       </c>
       <c r="J6" t="n">
         <v>60</v>
@@ -1067,7 +1067,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M6" t="n">
@@ -1077,10 +1077,10 @@
         <v>60</v>
       </c>
       <c r="O6" t="n">
-        <v>74.46808510638297</v>
+        <v>70.21276595744681</v>
       </c>
       <c r="P6" t="n">
-        <v>59.5216170212766</v>
+        <v>58.67055319148936</v>
       </c>
       <c r="Q6" t="b">
         <v>0</v>
@@ -1107,22 +1107,22 @@
         <v>2715.5</v>
       </c>
       <c r="D7" t="n">
-        <v>0.1046700838011553</v>
+        <v>0.1210419848903934</v>
       </c>
       <c r="E7" t="n">
-        <v>0.1072375127420999</v>
+        <v>0.1273716112425791</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.1844610625581884</v>
+        <v>-0.1894271812781708</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.1453453787106062</v>
+        <v>-0.1503114974305887</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.1335288566298978</v>
+        <v>-0.1384949753498803</v>
       </c>
       <c r="I7" t="n">
-        <v>63.44007319304669</v>
+        <v>53.82482089207303</v>
       </c>
       <c r="J7" t="n">
         <v>80</v>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M7" t="n">
@@ -1142,10 +1142,10 @@
         <v>80</v>
       </c>
       <c r="O7" t="n">
-        <v>25.53191489361702</v>
+        <v>27.65957446808511</v>
       </c>
       <c r="P7" t="n">
-        <v>56.59838297872341</v>
+        <v>57.02391489361703</v>
       </c>
       <c r="Q7" t="b">
         <v>0</v>
@@ -1172,22 +1172,22 @@
         <v>569.3</v>
       </c>
       <c r="D8" t="n">
-        <v>0.1712786750334327</v>
+        <v>0.1637367130008176</v>
       </c>
       <c r="E8" t="n">
-        <v>0.2385510714674208</v>
+        <v>0.2461420597570316</v>
       </c>
       <c r="F8" t="n">
-        <v>0.305135259055479</v>
+        <v>0.3535425582501186</v>
       </c>
       <c r="G8" t="n">
-        <v>0.3442509429030611</v>
+        <v>0.3926582420977007</v>
       </c>
       <c r="H8" t="n">
-        <v>0.3560674649837695</v>
+        <v>0.4044747641784091</v>
       </c>
       <c r="I8" t="n">
-        <v>73.72773536895671</v>
+        <v>70.59451762192948</v>
       </c>
       <c r="J8" t="n">
         <v>70</v>
@@ -1197,7 +1197,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M8" t="n">
@@ -1237,22 +1237,22 @@
         <v>432.4</v>
       </c>
       <c r="D9" t="n">
-        <v>0.0801898576067947</v>
+        <v>0.0474806201550386</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.1427438540840603</v>
+        <v>-0.1415525114155251</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.1003848954540725</v>
+        <v>-0.1110197368421053</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.0612692116064904</v>
+        <v>-0.0719040529945231</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.049452689525782</v>
+        <v>-0.0600875309138148</v>
       </c>
       <c r="I9" t="n">
-        <v>69.81402002861229</v>
+        <v>61.60145586897178</v>
       </c>
       <c r="J9" t="n">
         <v>60</v>
@@ -1262,7 +1262,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M9" t="n">
@@ -1272,10 +1272,10 @@
         <v>60</v>
       </c>
       <c r="O9" t="n">
-        <v>46.80851063829788</v>
+        <v>48.93617021276596</v>
       </c>
       <c r="P9" t="n">
-        <v>54.73770212765958</v>
+        <v>55.1632340425532</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -1302,22 +1302,22 @@
         <v>134315</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.0044841387488882</v>
+        <v>0.0148853375646982</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.086882626873789</v>
+        <v>-0.096950953037281</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.1028021776159781</v>
+        <v>-0.1212626758259731</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.0636864937683959</v>
+        <v>-0.082146991978391</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.0518699716876875</v>
+        <v>-0.0703304698976826</v>
       </c>
       <c r="I10" t="n">
-        <v>66.83493185259969</v>
+        <v>62.4249356591364</v>
       </c>
       <c r="J10" t="n">
         <v>60</v>
@@ -1327,7 +1327,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M10" t="n">
@@ -1337,10 +1337,10 @@
         <v>60</v>
       </c>
       <c r="O10" t="n">
-        <v>44.68085106382978</v>
+        <v>42.5531914893617</v>
       </c>
       <c r="P10" t="n">
-        <v>52.70017021276595</v>
+        <v>52.27463829787234</v>
       </c>
       <c r="Q10" t="b">
         <v>0</v>
@@ -1392,7 +1392,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M11" t="n">
@@ -1432,45 +1432,45 @@
         <v>435.5</v>
       </c>
       <c r="D12" t="n">
-        <v>0.0825254784986329</v>
+        <v>0.0671404067630481</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.08277169334456611</v>
+        <v>-0.0592936602224861</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.1571511515386104</v>
+        <v>-0.1535471331389698</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.1180354676910283</v>
+        <v>-0.1144314492913877</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.1062189456103199</v>
+        <v>-0.1026149272106793</v>
       </c>
       <c r="I12" t="n">
-        <v>64.6589259796807</v>
+        <v>39.20099875156056</v>
       </c>
       <c r="J12" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K12" t="n">
         <v>71.28</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M12" t="n">
         <v>71.28</v>
       </c>
       <c r="N12" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O12" t="n">
-        <v>34.04255319148936</v>
+        <v>36.17021276595745</v>
       </c>
       <c r="P12" t="n">
-        <v>67.32051063829788</v>
+        <v>63.74604255319149</v>
       </c>
       <c r="Q12" t="b">
         <v>1</v>
@@ -1497,22 +1497,22 @@
         <v>1690.5</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.0462085308056872</v>
+        <v>-0.0148601398601398</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.1161246470772769</v>
+        <v>-0.1214074112572111</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.0392702887019776</v>
+        <v>-0.0563773374267373</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.0001546048543955</v>
+        <v>-0.0172616535791552</v>
       </c>
       <c r="H13" t="n">
-        <v>0.0116619172263128</v>
+        <v>-0.0054451314984468</v>
       </c>
       <c r="I13" t="n">
-        <v>62.83658310120704</v>
+        <v>55.56480710519011</v>
       </c>
       <c r="J13" t="n">
         <v>60</v>
@@ -1522,7 +1522,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M13" t="n">
@@ -1532,16 +1532,16 @@
         <v>60</v>
       </c>
       <c r="O13" t="n">
-        <v>57.44680851063831</v>
+        <v>55.31914893617022</v>
       </c>
       <c r="P13" t="n">
-        <v>58.99736170212766</v>
+        <v>58.57182978723405</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
       </c>
       <c r="R13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S13" t="b">
         <v>0</v>
@@ -1562,22 +1562,22 @@
         <v>578.8</v>
       </c>
       <c r="D14" t="n">
-        <v>0.0525550100018183</v>
+        <v>0.0292522450431225</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.1339218913661529</v>
+        <v>-0.0990738578877734</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.3073240785064625</v>
+        <v>-0.2973596358118362</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.2682083946588803</v>
+        <v>-0.2582439519642541</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.256391872578172</v>
+        <v>-0.2464274298835457</v>
       </c>
       <c r="I14" t="n">
-        <v>56.36994219653178</v>
+        <v>54.3651753325272</v>
       </c>
       <c r="J14" t="n">
         <v>60</v>
@@ -1587,7 +1587,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M14" t="n">
@@ -1597,10 +1597,10 @@
         <v>60</v>
       </c>
       <c r="O14" t="n">
-        <v>6.382978723404255</v>
+        <v>4.25531914893617</v>
       </c>
       <c r="P14" t="n">
-        <v>47.13259574468086</v>
+        <v>46.70706382978724</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
@@ -1627,22 +1627,22 @@
         <v>105.26</v>
       </c>
       <c r="D15" t="n">
-        <v>0.07958974358974361</v>
+        <v>0.1094013490725127</v>
       </c>
       <c r="E15" t="n">
-        <v>0.0024761904761905</v>
+        <v>-0.0207461159177596</v>
       </c>
       <c r="F15" t="n">
-        <v>0.1725520775314695</v>
+        <v>0.1872321227159938</v>
       </c>
       <c r="G15" t="n">
-        <v>0.2116677613790516</v>
+        <v>0.226347806563576</v>
       </c>
       <c r="H15" t="n">
-        <v>0.22348428345976</v>
+        <v>0.2381643286442843</v>
       </c>
       <c r="I15" t="n">
-        <v>67.98866855524079</v>
+        <v>65.97524255603882</v>
       </c>
       <c r="J15" t="n">
         <v>80</v>
@@ -1652,7 +1652,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M15" t="n">
@@ -1692,22 +1692,22 @@
         <v>174.84</v>
       </c>
       <c r="D16" t="n">
-        <v>0.1005224397305972</v>
+        <v>0.0900928985597606</v>
       </c>
       <c r="E16" t="n">
-        <v>0.0730330182889407</v>
+        <v>0.0945971326613661</v>
       </c>
       <c r="F16" t="n">
-        <v>0.1355458855621225</v>
+        <v>0.08717821166521569</v>
       </c>
       <c r="G16" t="n">
-        <v>0.1746615694097046</v>
+        <v>0.1262938955127979</v>
       </c>
       <c r="H16" t="n">
-        <v>0.186478091490413</v>
+        <v>0.1381104175935062</v>
       </c>
       <c r="I16" t="n">
-        <v>66.25653126580144</v>
+        <v>64.33915211970074</v>
       </c>
       <c r="J16" t="n">
         <v>80</v>
@@ -1717,7 +1717,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M16" t="n">
@@ -1727,10 +1727,10 @@
         <v>80</v>
       </c>
       <c r="O16" t="n">
-        <v>78.72340425531915</v>
+        <v>74.46808510638297</v>
       </c>
       <c r="P16" t="n">
-        <v>68.78868085106383</v>
+        <v>67.93761702127659</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>
@@ -1757,45 +1757,45 @@
         <v>7398.5</v>
       </c>
       <c r="D17" t="n">
-        <v>0.1085555888522624</v>
+        <v>0.0892160471107839</v>
       </c>
       <c r="E17" t="n">
-        <v>-0.0291956436163233</v>
+        <v>-0.0129410979921286</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0917072450936993</v>
+        <v>0.0917877960599129</v>
       </c>
       <c r="G17" t="n">
-        <v>0.1308229289412814</v>
+        <v>0.130903479907495</v>
       </c>
       <c r="H17" t="n">
-        <v>0.1426394510219898</v>
+        <v>0.1427200019882034</v>
       </c>
       <c r="I17" t="n">
-        <v>70.8286464191976</v>
+        <v>65.49889135254989</v>
       </c>
       <c r="J17" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K17" t="n">
         <v>54.65</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M17" t="n">
         <v>54.65</v>
       </c>
       <c r="N17" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O17" t="n">
-        <v>72.3404255319149</v>
+        <v>76.59574468085107</v>
       </c>
       <c r="P17" t="n">
-        <v>64.32808510638299</v>
+        <v>69.17914893617021</v>
       </c>
       <c r="Q17" t="b">
         <v>0</v>
@@ -1822,22 +1822,22 @@
         <v>689.2</v>
       </c>
       <c r="D18" t="n">
-        <v>0.0242235101798187</v>
+        <v>0.0470186099506266</v>
       </c>
       <c r="E18" t="n">
-        <v>0.1711129991503823</v>
+        <v>0.1804401815534813</v>
       </c>
       <c r="F18" t="n">
-        <v>0.0390471883009198</v>
+        <v>0.0355345203215387</v>
       </c>
       <c r="G18" t="n">
-        <v>0.0781628721485019</v>
+        <v>0.0746502041691208</v>
       </c>
       <c r="H18" t="n">
-        <v>0.08997939422921029</v>
+        <v>0.08646672624982921</v>
       </c>
       <c r="I18" t="n">
-        <v>47.66548463356975</v>
+        <v>47.49481174029056</v>
       </c>
       <c r="J18" t="n">
         <v>80</v>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M18" t="n">
@@ -1887,22 +1887,22 @@
         <v>2391.8</v>
       </c>
       <c r="D19" t="n">
-        <v>-0.0048264957976199</v>
+        <v>0.0001672660366311</v>
       </c>
       <c r="E19" t="n">
-        <v>-0.0877955758962623</v>
+        <v>-0.07045975671369149</v>
       </c>
       <c r="F19" t="n">
-        <v>-0.1693696822364992</v>
+        <v>-0.1624763638910288</v>
       </c>
       <c r="G19" t="n">
-        <v>-0.1302539983889171</v>
+        <v>-0.1233606800434466</v>
       </c>
       <c r="H19" t="n">
-        <v>-0.1184374763082087</v>
+        <v>-0.1115441579627383</v>
       </c>
       <c r="I19" t="n">
-        <v>63.17991631799165</v>
+        <v>56.10060278528375</v>
       </c>
       <c r="J19" t="n">
         <v>60</v>
@@ -1912,7 +1912,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M19" t="n">
@@ -1952,22 +1952,22 @@
         <v>2164.9</v>
       </c>
       <c r="D20" t="n">
-        <v>0.0571833186834651</v>
+        <v>0.0797506234413965</v>
       </c>
       <c r="E20" t="n">
-        <v>-0.0295844726343628</v>
+        <v>-0.0255660080118826</v>
       </c>
       <c r="F20" t="n">
-        <v>0.0601860920666015</v>
+        <v>0.08543494610178</v>
       </c>
       <c r="G20" t="n">
-        <v>0.0993017759141836</v>
+        <v>0.1245506299493621</v>
       </c>
       <c r="H20" t="n">
-        <v>0.111118297994892</v>
+        <v>0.1363671520300705</v>
       </c>
       <c r="I20" t="n">
-        <v>62.61298274445357</v>
+        <v>57.57971284728698</v>
       </c>
       <c r="J20" t="n">
         <v>80</v>
@@ -1977,7 +1977,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M20" t="n">
@@ -1987,10 +1987,10 @@
         <v>80</v>
       </c>
       <c r="O20" t="n">
-        <v>65.95744680851064</v>
+        <v>72.3404255319149</v>
       </c>
       <c r="P20" t="n">
-        <v>64.81548936170213</v>
+        <v>66.09208510638298</v>
       </c>
       <c r="Q20" t="b">
         <v>0</v>
@@ -2017,22 +2017,22 @@
         <v>927.65</v>
       </c>
       <c r="D21" t="n">
-        <v>0.101198955365622</v>
+        <v>0.1167087998073912</v>
       </c>
       <c r="E21" t="n">
-        <v>-0.0497336611350134</v>
+        <v>-0.0326903023983315</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.2767989397364934</v>
+        <v>-0.2783741734733567</v>
       </c>
       <c r="G21" t="n">
-        <v>-0.2376832558889112</v>
+        <v>-0.2392584896257745</v>
       </c>
       <c r="H21" t="n">
-        <v>-0.2258667338082028</v>
+        <v>-0.2274419675450661</v>
       </c>
       <c r="I21" t="n">
-        <v>65.43463381245722</v>
+        <v>61.72309247094492</v>
       </c>
       <c r="J21" t="n">
         <v>80</v>
@@ -2042,7 +2042,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M21" t="n">
@@ -2082,22 +2082,22 @@
         <v>440.1</v>
       </c>
       <c r="D22" t="n">
-        <v>0.1331101956745624</v>
+        <v>0.1469898358092261</v>
       </c>
       <c r="E22" t="n">
-        <v>0.2255639097744359</v>
+        <v>0.2606702950443997</v>
       </c>
       <c r="F22" t="n">
-        <v>0.3894238358326756</v>
+        <v>0.3791914760263239</v>
       </c>
       <c r="G22" t="n">
-        <v>0.4285395196802577</v>
+        <v>0.4183071598739061</v>
       </c>
       <c r="H22" t="n">
-        <v>0.4403560417609661</v>
+        <v>0.4301236819546145</v>
       </c>
       <c r="I22" t="n">
-        <v>69.98535871156662</v>
+        <v>65.00512120177535</v>
       </c>
       <c r="J22" t="n">
         <v>80</v>
@@ -2107,7 +2107,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M22" t="n">
@@ -2147,45 +2147,45 @@
         <v>370.2</v>
       </c>
       <c r="D23" t="n">
-        <v>0.0557536004562955</v>
+        <v>0.0951042745156041</v>
       </c>
       <c r="E23" t="n">
-        <v>-0.0259176424154716</v>
+        <v>-0.0146393398988554</v>
       </c>
       <c r="F23" t="n">
-        <v>-0.1266808209483368</v>
+        <v>-0.12129124139568</v>
       </c>
       <c r="G23" t="n">
-        <v>-0.0875651371007547</v>
+        <v>-0.0821755575480979</v>
       </c>
       <c r="H23" t="n">
-        <v>-0.0757486150200463</v>
+        <v>-0.0703590354673895</v>
       </c>
       <c r="I23" t="n">
-        <v>70.57190449750139</v>
+        <v>69.90346394094266</v>
       </c>
       <c r="J23" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K23" t="n">
         <v>49.7</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M23" t="n">
         <v>49.7</v>
       </c>
       <c r="N23" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O23" t="n">
-        <v>42.5531914893617</v>
+        <v>40.42553191489361</v>
       </c>
       <c r="P23" t="n">
-        <v>56.39063829787234</v>
+        <v>59.96510638297872</v>
       </c>
       <c r="Q23" t="b">
         <v>0</v>
@@ -2212,22 +2212,22 @@
         <v>122.92</v>
       </c>
       <c r="D24" t="n">
-        <v>0.0455937393671317</v>
+        <v>0.0338968794684162</v>
       </c>
       <c r="E24" t="n">
-        <v>-0.0433496770176667</v>
+        <v>-0.024521863344179</v>
       </c>
       <c r="F24" t="n">
-        <v>0.1396254403856851</v>
+        <v>0.173684713071708</v>
       </c>
       <c r="G24" t="n">
-        <v>0.1787411242332672</v>
+        <v>0.2128003969192902</v>
       </c>
       <c r="H24" t="n">
-        <v>0.1905576463139756</v>
+        <v>0.2246169189999985</v>
       </c>
       <c r="I24" t="n">
-        <v>56.55066530194473</v>
+        <v>52.04744422479526</v>
       </c>
       <c r="J24" t="n">
         <v>60</v>
@@ -2237,7 +2237,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M24" t="n">
@@ -2277,22 +2277,22 @@
         <v>624.6</v>
       </c>
       <c r="D25" t="n">
-        <v>0.2636050981185516</v>
+        <v>0.2846565199506377</v>
       </c>
       <c r="E25" t="n">
-        <v>0.0177611210689261</v>
+        <v>0.0414339308045019</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.1391951488423374</v>
+        <v>-0.1578805446946205</v>
       </c>
       <c r="G25" t="n">
-        <v>-0.1000794649947552</v>
+        <v>-0.1187648608470384</v>
       </c>
       <c r="H25" t="n">
-        <v>-0.0882629429140469</v>
+        <v>-0.10694833876633</v>
       </c>
       <c r="I25" t="n">
-        <v>65.42083578575632</v>
+        <v>65.32900560637357</v>
       </c>
       <c r="J25" t="n">
         <v>80</v>
@@ -2302,7 +2302,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M25" t="n">
@@ -2312,10 +2312,10 @@
         <v>80</v>
       </c>
       <c r="O25" t="n">
-        <v>36.17021276595745</v>
+        <v>34.04255319148936</v>
       </c>
       <c r="P25" t="n">
-        <v>61.99804255319149</v>
+        <v>61.57251063829787</v>
       </c>
       <c r="Q25" t="b">
         <v>0</v>
@@ -2342,22 +2342,22 @@
         <v>132.2</v>
       </c>
       <c r="D26" t="n">
-        <v>0.0147374884863369</v>
+        <v>0.0158291071154141</v>
       </c>
       <c r="E26" t="n">
-        <v>-0.1213027583914921</v>
+        <v>-0.09902542084100049</v>
       </c>
       <c r="F26" t="n">
-        <v>-0.2413634798576839</v>
+        <v>-0.2737460858100313</v>
       </c>
       <c r="G26" t="n">
-        <v>-0.2022477960101018</v>
+        <v>-0.2346304019624492</v>
       </c>
       <c r="H26" t="n">
-        <v>-0.1904312739293934</v>
+        <v>-0.2228138798817408</v>
       </c>
       <c r="I26" t="n">
-        <v>62.08963745361115</v>
+        <v>59.6597812879708</v>
       </c>
       <c r="J26" t="n">
         <v>60</v>
@@ -2367,7 +2367,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M26" t="n">
@@ -2407,22 +2407,22 @@
         <v>5399.4</v>
       </c>
       <c r="D27" t="n">
-        <v>0.1217201620442505</v>
+        <v>0.1014687882496938</v>
       </c>
       <c r="E27" t="n">
-        <v>-0.0133576975788031</v>
+        <v>-0.0341829889991951</v>
       </c>
       <c r="F27" t="n">
-        <v>0.2355889150781482</v>
+        <v>0.263076635164218</v>
       </c>
       <c r="G27" t="n">
-        <v>0.2747045989257304</v>
+        <v>0.3021923190118001</v>
       </c>
       <c r="H27" t="n">
-        <v>0.2865211210064388</v>
+        <v>0.3140088410925085</v>
       </c>
       <c r="I27" t="n">
-        <v>60.04729402912881</v>
+        <v>57.21931288484777</v>
       </c>
       <c r="J27" t="n">
         <v>60</v>
@@ -2432,7 +2432,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M27" t="n">
@@ -2472,22 +2472,22 @@
         <v>1847.8</v>
       </c>
       <c r="D28" t="n">
-        <v>0.2885634588563459</v>
+        <v>0.2722390526025886</v>
       </c>
       <c r="E28" t="n">
-        <v>0.2070024168789599</v>
+        <v>0.2227368978295394</v>
       </c>
       <c r="F28" t="n">
-        <v>0.65336435218325</v>
+        <v>0.6757050875124693</v>
       </c>
       <c r="G28" t="n">
-        <v>0.6924800360308321</v>
+        <v>0.7148207713600514</v>
       </c>
       <c r="H28" t="n">
-        <v>0.7042965581115405</v>
+        <v>0.7266372934407598</v>
       </c>
       <c r="I28" t="n">
-        <v>75.85237916822781</v>
+        <v>73.27389591540536</v>
       </c>
       <c r="J28" t="n">
         <v>70</v>
@@ -2497,7 +2497,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M28" t="n">
@@ -2537,51 +2537,51 @@
         <v>509.25</v>
       </c>
       <c r="D29" t="n">
-        <v>0.059062077570968</v>
+        <v>0.0585117439201827</v>
       </c>
       <c r="E29" t="n">
-        <v>-0.1197061365600691</v>
+        <v>-0.1216041397153945</v>
       </c>
       <c r="F29" t="n">
-        <v>-0.0728265817023213</v>
+        <v>-0.0442004504504504</v>
       </c>
       <c r="G29" t="n">
-        <v>-0.0337108978547392</v>
+        <v>-0.0050847666028682</v>
       </c>
       <c r="H29" t="n">
-        <v>-0.0218943757740308</v>
+        <v>0.0067317554778401</v>
       </c>
       <c r="I29" t="n">
-        <v>45.90956161546426</v>
+        <v>35.77868852459015</v>
       </c>
       <c r="J29" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K29" t="n">
         <v>49.42</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M29" t="n">
         <v>49.42</v>
       </c>
       <c r="N29" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O29" t="n">
-        <v>55.31914893617022</v>
+        <v>57.44680851063831</v>
       </c>
       <c r="P29" t="n">
-        <v>46.83182978723404</v>
+        <v>43.25736170212766</v>
       </c>
       <c r="Q29" t="b">
         <v>0</v>
       </c>
       <c r="R29" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S29" t="b">
         <v>0</v>
@@ -2602,22 +2602,22 @@
         <v>117.86</v>
       </c>
       <c r="D30" t="n">
-        <v>-0.0399934837501018</v>
+        <v>-0.0418665149174863</v>
       </c>
       <c r="E30" t="n">
-        <v>-0.0036351339927297</v>
+        <v>-0.0577230572433642</v>
       </c>
       <c r="F30" t="n">
-        <v>-0.090094958696827</v>
+        <v>-0.0919876733436055</v>
       </c>
       <c r="G30" t="n">
-        <v>-0.0509792748492449</v>
+        <v>-0.0528719894960234</v>
       </c>
       <c r="H30" t="n">
-        <v>-0.0391627527685365</v>
+        <v>-0.041055467415315</v>
       </c>
       <c r="I30" t="n">
-        <v>59.78781656399726</v>
+        <v>60.19986216402481</v>
       </c>
       <c r="J30" t="n">
         <v>80</v>
@@ -2627,7 +2627,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M30" t="n">
@@ -2667,22 +2667,22 @@
         <v>38.53</v>
       </c>
       <c r="D31" t="n">
-        <v>-0.0140736949846468</v>
+        <v>-0.0158365261813536</v>
       </c>
       <c r="E31" t="n">
-        <v>-0.1946070234113712</v>
+        <v>-0.1760051325919589</v>
       </c>
       <c r="F31" t="n">
-        <v>-0.2049112670243499</v>
+        <v>-0.1902059688944934</v>
       </c>
       <c r="G31" t="n">
-        <v>-0.1657955831767678</v>
+        <v>-0.1510902850469113</v>
       </c>
       <c r="H31" t="n">
-        <v>-0.1539790610960594</v>
+        <v>-0.1392737629662029</v>
       </c>
       <c r="I31" t="n">
-        <v>56.35910224438904</v>
+        <v>53.64238410596029</v>
       </c>
       <c r="J31" t="n">
         <v>60</v>
@@ -2692,7 +2692,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M31" t="n">
@@ -2702,10 +2702,10 @@
         <v>60</v>
       </c>
       <c r="O31" t="n">
-        <v>23.40425531914894</v>
+        <v>25.53191489361702</v>
       </c>
       <c r="P31" t="n">
-        <v>48.27685106382979</v>
+        <v>48.70238297872341</v>
       </c>
       <c r="Q31" t="b">
         <v>0</v>
@@ -2732,22 +2732,22 @@
         <v>728.1</v>
       </c>
       <c r="D32" t="n">
-        <v>0.1127922971114168</v>
+        <v>0.1217069788938529</v>
       </c>
       <c r="E32" t="n">
-        <v>-0.0672559569561875</v>
+        <v>-0.0362673726009264</v>
       </c>
       <c r="F32" t="n">
-        <v>-0.3301747930082797</v>
+        <v>-0.313760603204524</v>
       </c>
       <c r="G32" t="n">
-        <v>-0.2910591091606975</v>
+        <v>-0.2746449193569419</v>
       </c>
       <c r="H32" t="n">
-        <v>-0.2792425870799891</v>
+        <v>-0.2628283972762335</v>
       </c>
       <c r="I32" t="n">
-        <v>62.90630975143405</v>
+        <v>59.61138098542681</v>
       </c>
       <c r="J32" t="n">
         <v>80</v>
@@ -2757,7 +2757,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M32" t="n">
@@ -2797,22 +2797,22 @@
         <v>573.1</v>
       </c>
       <c r="D33" t="n">
-        <v>0.1088323498113572</v>
+        <v>0.0903729071537291</v>
       </c>
       <c r="E33" t="n">
-        <v>-0.085089399744572</v>
+        <v>-0.1023572715169551</v>
       </c>
       <c r="F33" t="n">
-        <v>0.0615911827359452</v>
+        <v>0.0587474598189545</v>
       </c>
       <c r="G33" t="n">
-        <v>0.1007068665835273</v>
+        <v>0.0978631436665367</v>
       </c>
       <c r="H33" t="n">
-        <v>0.1125233886642357</v>
+        <v>0.109679665747245</v>
       </c>
       <c r="I33" t="n">
-        <v>65.30249110320284</v>
+        <v>61.50809317015396</v>
       </c>
       <c r="J33" t="n">
         <v>80</v>
@@ -2822,7 +2822,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M33" t="n">
@@ -2832,10 +2832,10 @@
         <v>80</v>
       </c>
       <c r="O33" t="n">
-        <v>68.08510638297872</v>
+        <v>65.95744680851064</v>
       </c>
       <c r="P33" t="n">
-        <v>65.60902127659575</v>
+        <v>65.18348936170213</v>
       </c>
       <c r="Q33" t="b">
         <v>0</v>
@@ -2887,7 +2887,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M34" t="n">
@@ -2897,10 +2897,10 @@
         <v>80</v>
       </c>
       <c r="O34" t="n">
-        <v>12.76595744680851</v>
+        <v>14.8936170212766</v>
       </c>
       <c r="P34" t="n">
-        <v>54.90519148936171</v>
+        <v>55.33072340425532</v>
       </c>
       <c r="Q34" t="b">
         <v>0</v>
@@ -2927,22 +2927,22 @@
         <v>116.31</v>
       </c>
       <c r="D35" t="n">
-        <v>0.1002743354460315</v>
+        <v>0.0994422913318839</v>
       </c>
       <c r="E35" t="n">
-        <v>-0.08127962085308039</v>
+        <v>-0.07873267326732659</v>
       </c>
       <c r="F35" t="n">
-        <v>0.1136537725009574</v>
+        <v>0.1137604136742314</v>
       </c>
       <c r="G35" t="n">
-        <v>0.1527694563485395</v>
+        <v>0.1528760975218135</v>
       </c>
       <c r="H35" t="n">
-        <v>0.1645859784292479</v>
+        <v>0.1646926196025219</v>
       </c>
       <c r="I35" t="n">
-        <v>62.16640502354787</v>
+        <v>61.4646626159258</v>
       </c>
       <c r="J35" t="n">
         <v>60</v>
@@ -2952,7 +2952,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M35" t="n">
@@ -2962,10 +2962,10 @@
         <v>60</v>
       </c>
       <c r="O35" t="n">
-        <v>76.59574468085107</v>
+        <v>78.72340425531915</v>
       </c>
       <c r="P35" t="n">
-        <v>58.94714893617022</v>
+        <v>59.37268085106383</v>
       </c>
       <c r="Q35" t="b">
         <v>0</v>
@@ -2992,22 +2992,22 @@
         <v>484.4</v>
       </c>
       <c r="D36" t="n">
-        <v>0.0009298481248063</v>
+        <v>0.0005163688939378</v>
       </c>
       <c r="E36" t="n">
-        <v>-0.1246046805819102</v>
+        <v>-0.1223842739378567</v>
       </c>
       <c r="F36" t="n">
-        <v>0.0481445418154278</v>
+        <v>0.0594925634295713</v>
       </c>
       <c r="G36" t="n">
-        <v>0.08726022566300989</v>
+        <v>0.09860824727715339</v>
       </c>
       <c r="H36" t="n">
-        <v>0.0990767477437183</v>
+        <v>0.1104247693578618</v>
       </c>
       <c r="I36" t="n">
-        <v>63.13993174061433</v>
+        <v>60.21052631578947</v>
       </c>
       <c r="J36" t="n">
         <v>60</v>
@@ -3017,7 +3017,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M36" t="n">
@@ -3027,10 +3027,10 @@
         <v>60</v>
       </c>
       <c r="O36" t="n">
-        <v>63.82978723404256</v>
+        <v>68.08510638297872</v>
       </c>
       <c r="P36" t="n">
-        <v>55.88595744680852</v>
+        <v>56.73702127659575</v>
       </c>
       <c r="Q36" t="b">
         <v>0</v>
@@ -3057,22 +3057,22 @@
         <v>2346.2</v>
       </c>
       <c r="D37" t="n">
-        <v>0.2010852871915633</v>
+        <v>0.1575883165581211</v>
       </c>
       <c r="E37" t="n">
-        <v>0.2942409532215357</v>
+        <v>0.2773301393728222</v>
       </c>
       <c r="F37" t="n">
-        <v>0.5693645484949832</v>
+        <v>0.5689447639427576</v>
       </c>
       <c r="G37" t="n">
-        <v>0.6084802323425653</v>
+        <v>0.6080604477903397</v>
       </c>
       <c r="H37" t="n">
-        <v>0.6202967544232737</v>
+        <v>0.6198769698710481</v>
       </c>
       <c r="I37" t="n">
-        <v>75.09261276966656</v>
+        <v>70.82695252679936</v>
       </c>
       <c r="J37" t="n">
         <v>70</v>
@@ -3082,7 +3082,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M37" t="n">
@@ -3122,22 +3122,22 @@
         <v>814</v>
       </c>
       <c r="D38" t="n">
-        <v>0.0439243347226674</v>
+        <v>0.0665618448637315</v>
       </c>
       <c r="E38" t="n">
-        <v>-0.1032279387462818</v>
+        <v>-0.08338494454141079</v>
       </c>
       <c r="F38" t="n">
-        <v>-0.2398206948076204</v>
+        <v>-0.2510121457489878</v>
       </c>
       <c r="G38" t="n">
-        <v>-0.2007050109600383</v>
+        <v>-0.2118964619014056</v>
       </c>
       <c r="H38" t="n">
-        <v>-0.1888884888793299</v>
+        <v>-0.2000799398206972</v>
       </c>
       <c r="I38" t="n">
-        <v>59.08080059303188</v>
+        <v>53.93281869392865</v>
       </c>
       <c r="J38" t="n">
         <v>60</v>
@@ -3147,7 +3147,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M38" t="n">
@@ -3157,10 +3157,10 @@
         <v>60</v>
       </c>
       <c r="O38" t="n">
-        <v>14.8936170212766</v>
+        <v>12.76595744680851</v>
       </c>
       <c r="P38" t="n">
-        <v>46.92672340425532</v>
+        <v>46.5011914893617</v>
       </c>
       <c r="Q38" t="b">
         <v>0</v>
@@ -3187,45 +3187,45 @@
         <v>3610.5</v>
       </c>
       <c r="D39" t="n">
-        <v>0.2641364097895733</v>
+        <v>0.227017841971113</v>
       </c>
       <c r="E39" t="n">
-        <v>0.1335237975637322</v>
+        <v>0.1632514981635413</v>
       </c>
       <c r="F39" t="n">
-        <v>0.3922952336881073</v>
+        <v>0.3884936353497672</v>
       </c>
       <c r="G39" t="n">
-        <v>0.4314109175356895</v>
+        <v>0.4276093191973493</v>
       </c>
       <c r="H39" t="n">
-        <v>0.4432274396163979</v>
+        <v>0.4394258412780577</v>
       </c>
       <c r="I39" t="n">
-        <v>81.59806295399518</v>
+        <v>79.11131470453508</v>
       </c>
       <c r="J39" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K39" t="n">
         <v>48.69</v>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M39" t="n">
         <v>48.69</v>
       </c>
       <c r="N39" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O39" t="n">
         <v>93.61702127659576</v>
       </c>
       <c r="P39" t="n">
-        <v>62.19940425531915</v>
+        <v>66.19940425531915</v>
       </c>
       <c r="Q39" t="b">
         <v>0</v>
@@ -3252,22 +3252,22 @@
         <v>212.66</v>
       </c>
       <c r="D40" t="n">
-        <v>0.1651325882095111</v>
+        <v>0.1879119651435592</v>
       </c>
       <c r="E40" t="n">
-        <v>0.0678383128295254</v>
+        <v>0.0723073820088746</v>
       </c>
       <c r="F40" t="n">
-        <v>-0.1284783410515962</v>
+        <v>-0.118398142774231</v>
       </c>
       <c r="G40" t="n">
-        <v>-0.0893626572040141</v>
+        <v>-0.0792824589266488</v>
       </c>
       <c r="H40" t="n">
-        <v>-0.0775461351233057</v>
+        <v>-0.06746593684594041</v>
       </c>
       <c r="I40" t="n">
-        <v>75.09305712898528</v>
+        <v>73.29052412356822</v>
       </c>
       <c r="J40" t="n">
         <v>70</v>
@@ -3277,7 +3277,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M40" t="n">
@@ -3287,10 +3287,10 @@
         <v>70</v>
       </c>
       <c r="O40" t="n">
-        <v>40.42553191489361</v>
+        <v>44.68085106382978</v>
       </c>
       <c r="P40" t="n">
-        <v>54.26110638297872</v>
+        <v>55.11217021276596</v>
       </c>
       <c r="Q40" t="b">
         <v>0</v>
@@ -3317,22 +3317,22 @@
         <v>791.2</v>
       </c>
       <c r="D41" t="n">
-        <v>-0.0377622377622377</v>
+        <v>-0.0210949582431178</v>
       </c>
       <c r="E41" t="n">
-        <v>-0.149567367119901</v>
+        <v>-0.1422376409366867</v>
       </c>
       <c r="F41" t="n">
-        <v>-0.2379117703717973</v>
+        <v>-0.2319937876140555</v>
       </c>
       <c r="G41" t="n">
-        <v>-0.1987960865242152</v>
+        <v>-0.1928781037664734</v>
       </c>
       <c r="H41" t="n">
-        <v>-0.1869795644435068</v>
+        <v>-0.181061581685765</v>
       </c>
       <c r="I41" t="n">
-        <v>48.69675778766691</v>
+        <v>47.46093750000001</v>
       </c>
       <c r="J41" t="n">
         <v>60</v>
@@ -3342,7 +3342,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M41" t="n">
@@ -3382,22 +3382,22 @@
         <v>614.2</v>
       </c>
       <c r="D42" t="n">
-        <v>0.1288366109171108</v>
+        <v>0.118353969410051</v>
       </c>
       <c r="E42" t="n">
-        <v>-0.0596340809921149</v>
+        <v>-0.0389610389610389</v>
       </c>
       <c r="F42" t="n">
-        <v>-0.2190718372536554</v>
+        <v>-0.2104891059836749</v>
       </c>
       <c r="G42" t="n">
-        <v>-0.1799561534060733</v>
+        <v>-0.1713734221360928</v>
       </c>
       <c r="H42" t="n">
-        <v>-0.1681396313253649</v>
+        <v>-0.1595569000553844</v>
       </c>
       <c r="I42" t="n">
-        <v>67.73935638616831</v>
+        <v>67.7264547090582</v>
       </c>
       <c r="J42" t="n">
         <v>80</v>
@@ -3407,7 +3407,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M42" t="n">
@@ -3447,45 +3447,45 @@
         <v>411.6</v>
       </c>
       <c r="D43" t="n">
-        <v>0.0199479618386817</v>
+        <v>0.008329250367466999</v>
       </c>
       <c r="E43" t="n">
-        <v>-0.1053146397130746</v>
+        <v>-0.1051201217523642</v>
       </c>
       <c r="F43" t="n">
-        <v>-0.1342938269008307</v>
+        <v>-0.1129310344827585</v>
       </c>
       <c r="G43" t="n">
-        <v>-0.0951781430532485</v>
+        <v>-0.0738153506351764</v>
       </c>
       <c r="H43" t="n">
-        <v>-0.0833616209725401</v>
+        <v>-0.061998828554468</v>
       </c>
       <c r="I43" t="n">
-        <v>54.72727272727276</v>
+        <v>50.57071960297768</v>
       </c>
       <c r="J43" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="K43" t="n">
         <v>51.48</v>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M43" t="n">
         <v>51.48</v>
       </c>
       <c r="N43" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="O43" t="n">
-        <v>38.29787234042553</v>
+        <v>46.80851063829788</v>
       </c>
       <c r="P43" t="n">
-        <v>52.25157446808511</v>
+        <v>45.95370212765958</v>
       </c>
       <c r="Q43" t="b">
         <v>0</v>
@@ -3512,22 +3512,22 @@
         <v>265.8</v>
       </c>
       <c r="D44" t="n">
-        <v>0.0732889158086009</v>
+        <v>0.1165721487082545</v>
       </c>
       <c r="E44" t="n">
-        <v>-0.0151908114116338</v>
+        <v>0.0009414422895877</v>
       </c>
       <c r="F44" t="n">
-        <v>-0.0917478216299332</v>
+        <v>-0.1326480665687713</v>
       </c>
       <c r="G44" t="n">
-        <v>-0.052632137782351</v>
+        <v>-0.0935323827211892</v>
       </c>
       <c r="H44" t="n">
-        <v>-0.0408156157016427</v>
+        <v>-0.08171586064048079</v>
       </c>
       <c r="I44" t="n">
-        <v>87.0979207392927</v>
+        <v>82.47223563495898</v>
       </c>
       <c r="J44" t="n">
         <v>60</v>
@@ -3537,7 +3537,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M44" t="n">
@@ -3547,10 +3547,10 @@
         <v>60</v>
       </c>
       <c r="O44" t="n">
-        <v>48.93617021276596</v>
+        <v>38.29787234042553</v>
       </c>
       <c r="P44" t="n">
-        <v>52.6672340425532</v>
+        <v>50.53957446808511</v>
       </c>
       <c r="Q44" t="b">
         <v>0</v>
@@ -3577,22 +3577,22 @@
         <v>98</v>
       </c>
       <c r="D45" t="n">
-        <v>-0.0191172054849364</v>
+        <v>0.0072977695549387</v>
       </c>
       <c r="E45" t="n">
-        <v>-0.0853089415717752</v>
+        <v>-0.1000918273645546</v>
       </c>
       <c r="F45" t="n">
-        <v>-0.3099077529751425</v>
+        <v>-0.2947103274559193</v>
       </c>
       <c r="G45" t="n">
-        <v>-0.2707920691275604</v>
+        <v>-0.2555946436083371</v>
       </c>
       <c r="H45" t="n">
-        <v>-0.258975547046852</v>
+        <v>-0.2437781215276288</v>
       </c>
       <c r="I45" t="n">
-        <v>57.35795454545456</v>
+        <v>58.16767502160761</v>
       </c>
       <c r="J45" t="n">
         <v>60</v>
@@ -3602,7 +3602,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M45" t="n">
@@ -3612,10 +3612,10 @@
         <v>60</v>
       </c>
       <c r="O45" t="n">
-        <v>4.25531914893617</v>
+        <v>6.382978723404255</v>
       </c>
       <c r="P45" t="n">
-        <v>48.69106382978724</v>
+        <v>49.11659574468086</v>
       </c>
       <c r="Q45" t="b">
         <v>0</v>
@@ -3642,22 +3642,22 @@
         <v>518.35</v>
       </c>
       <c r="D46" t="n">
-        <v>0.07821112844513781</v>
+        <v>0.0824892972747206</v>
       </c>
       <c r="E46" t="n">
-        <v>-0.1093642611683848</v>
+        <v>-0.0935560024481944</v>
       </c>
       <c r="F46" t="n">
-        <v>-0.1811216429699841</v>
+        <v>-0.1902679059595406</v>
       </c>
       <c r="G46" t="n">
-        <v>-0.142005959122402</v>
+        <v>-0.1511522221119585</v>
       </c>
       <c r="H46" t="n">
-        <v>-0.1301894370416936</v>
+        <v>-0.1393357000312501</v>
       </c>
       <c r="I46" t="n">
-        <v>61.02079395085067</v>
+        <v>59.74228816868411</v>
       </c>
       <c r="J46" t="n">
         <v>60</v>
@@ -3667,7 +3667,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M46" t="n">
@@ -3677,10 +3677,10 @@
         <v>60</v>
       </c>
       <c r="O46" t="n">
-        <v>29.78723404255319</v>
+        <v>23.40425531914894</v>
       </c>
       <c r="P46" t="n">
-        <v>49.80144680851064</v>
+        <v>48.52485106382979</v>
       </c>
       <c r="Q46" t="b">
         <v>0</v>
@@ -3707,45 +3707,45 @@
         <v>1022.05</v>
       </c>
       <c r="D47" t="n">
-        <v>0.1372538110604204</v>
+        <v>0.1107428136716839</v>
       </c>
       <c r="E47" t="n">
-        <v>0.2600789051904819</v>
+        <v>0.2711274174491636</v>
       </c>
       <c r="F47" t="n">
-        <v>0.2660885723134096</v>
+        <v>0.2812460824871503</v>
       </c>
       <c r="G47" t="n">
-        <v>0.3052042561609918</v>
+        <v>0.3203617663347324</v>
       </c>
       <c r="H47" t="n">
-        <v>0.3170207782417001</v>
+        <v>0.3321782884154408</v>
       </c>
       <c r="I47" t="n">
-        <v>49.39104915627291</v>
+        <v>37.83345349675558</v>
       </c>
       <c r="J47" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K47" t="n">
         <v>46.83</v>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M47" t="n">
         <v>46.83</v>
       </c>
       <c r="N47" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O47" t="n">
         <v>87.2340425531915</v>
       </c>
       <c r="P47" t="n">
-        <v>68.17880851063831</v>
+        <v>64.17880851063831</v>
       </c>
       <c r="Q47" t="b">
         <v>0</v>
@@ -3772,22 +3772,22 @@
         <v>14069</v>
       </c>
       <c r="D48" t="n">
-        <v>0.0341811231990591</v>
+        <v>0.0291880029261155</v>
       </c>
       <c r="E48" t="n">
-        <v>-0.0122858747542825</v>
+        <v>0.0075914917997566</v>
       </c>
       <c r="F48" t="n">
-        <v>0.0626132930513594</v>
+        <v>0.0554388597149286</v>
       </c>
       <c r="G48" t="n">
-        <v>0.1017289768989415</v>
+        <v>0.09455454356251081</v>
       </c>
       <c r="H48" t="n">
-        <v>0.1135454989796499</v>
+        <v>0.1063710656432191</v>
       </c>
       <c r="I48" t="n">
-        <v>63.29497274379164</v>
+        <v>58.22130299896587</v>
       </c>
       <c r="J48" t="n">
         <v>60</v>
@@ -3797,7 +3797,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M48" t="n">
@@ -3807,10 +3807,10 @@
         <v>60</v>
       </c>
       <c r="O48" t="n">
-        <v>70.21276595744681</v>
+        <v>63.82978723404256</v>
       </c>
       <c r="P48" t="n">
-        <v>58.15855319148936</v>
+        <v>56.88195744680851</v>
       </c>
       <c r="Q48" t="b">
         <v>0</v>
@@ -3948,22 +3948,22 @@
         <v>1801.3</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0753387857441347</v>
+        <v>0.0614614024749557</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2470058843890619</v>
+        <v>0.2366469861320885</v>
       </c>
       <c r="F2" t="n">
-        <v>0.4153374715172466</v>
+        <v>0.4341560509554139</v>
       </c>
       <c r="G2" t="n">
-        <v>0.4544531553648288</v>
+        <v>0.473271734802996</v>
       </c>
       <c r="H2" t="n">
-        <v>0.4662696774455371</v>
+        <v>0.4850882568837044</v>
       </c>
       <c r="I2" t="n">
-        <v>62.69558056546801</v>
+        <v>59.62566844919785</v>
       </c>
       <c r="J2" t="n">
         <v>80</v>
@@ -3973,7 +3973,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M2" t="n">
@@ -4013,22 +4013,22 @@
         <v>440.1</v>
       </c>
       <c r="D3" t="n">
-        <v>0.1331101956745624</v>
+        <v>0.1469898358092261</v>
       </c>
       <c r="E3" t="n">
-        <v>0.2255639097744359</v>
+        <v>0.2606702950443997</v>
       </c>
       <c r="F3" t="n">
-        <v>0.3894238358326756</v>
+        <v>0.3791914760263239</v>
       </c>
       <c r="G3" t="n">
-        <v>0.4285395196802577</v>
+        <v>0.4183071598739061</v>
       </c>
       <c r="H3" t="n">
-        <v>0.4403560417609661</v>
+        <v>0.4301236819546145</v>
       </c>
       <c r="I3" t="n">
-        <v>69.98535871156662</v>
+        <v>65.00512120177535</v>
       </c>
       <c r="J3" t="n">
         <v>80</v>
@@ -4038,7 +4038,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M3" t="n">
@@ -4078,22 +4078,22 @@
         <v>1847.8</v>
       </c>
       <c r="D4" t="n">
-        <v>0.2885634588563459</v>
+        <v>0.2722390526025886</v>
       </c>
       <c r="E4" t="n">
-        <v>0.2070024168789599</v>
+        <v>0.2227368978295394</v>
       </c>
       <c r="F4" t="n">
-        <v>0.65336435218325</v>
+        <v>0.6757050875124693</v>
       </c>
       <c r="G4" t="n">
-        <v>0.6924800360308321</v>
+        <v>0.7148207713600514</v>
       </c>
       <c r="H4" t="n">
-        <v>0.7042965581115405</v>
+        <v>0.7266372934407598</v>
       </c>
       <c r="I4" t="n">
-        <v>75.85237916822781</v>
+        <v>73.27389591540536</v>
       </c>
       <c r="J4" t="n">
         <v>70</v>
@@ -4103,7 +4103,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M4" t="n">
@@ -4143,22 +4143,22 @@
         <v>105.26</v>
       </c>
       <c r="D5" t="n">
-        <v>0.07958974358974361</v>
+        <v>0.1094013490725127</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0024761904761905</v>
+        <v>-0.0207461159177596</v>
       </c>
       <c r="F5" t="n">
-        <v>0.1725520775314695</v>
+        <v>0.1872321227159938</v>
       </c>
       <c r="G5" t="n">
-        <v>0.2116677613790516</v>
+        <v>0.226347806563576</v>
       </c>
       <c r="H5" t="n">
-        <v>0.22348428345976</v>
+        <v>0.2381643286442843</v>
       </c>
       <c r="I5" t="n">
-        <v>67.98866855524079</v>
+        <v>65.97524255603882</v>
       </c>
       <c r="J5" t="n">
         <v>80</v>
@@ -4168,7 +4168,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M5" t="n">
@@ -4196,57 +4196,57 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BHARATSE</t>
+          <t>CRAFTSMAN</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Seating</t>
+          <t>Castings</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>174.84</v>
+        <v>7398.5</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1005224397305972</v>
+        <v>0.0892160471107839</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0730330182889407</v>
+        <v>-0.0129410979921286</v>
       </c>
       <c r="F6" t="n">
-        <v>0.1355458855621225</v>
+        <v>0.0917877960599129</v>
       </c>
       <c r="G6" t="n">
-        <v>0.1746615694097046</v>
+        <v>0.130903479907495</v>
       </c>
       <c r="H6" t="n">
-        <v>0.186478091490413</v>
+        <v>0.1427200019882034</v>
       </c>
       <c r="I6" t="n">
-        <v>66.25653126580144</v>
+        <v>65.49889135254989</v>
       </c>
       <c r="J6" t="n">
         <v>80</v>
       </c>
       <c r="K6" t="n">
-        <v>52.61</v>
+        <v>54.65</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M6" t="n">
-        <v>52.61</v>
+        <v>54.65</v>
       </c>
       <c r="N6" t="n">
         <v>80</v>
       </c>
       <c r="O6" t="n">
-        <v>78.72340425531915</v>
+        <v>76.59574468085107</v>
       </c>
       <c r="P6" t="n">
-        <v>68.78868085106383</v>
+        <v>69.17914893617021</v>
       </c>
       <c r="Q6" t="b">
         <v>0</v>
@@ -4261,57 +4261,57 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>WHEELS</t>
+          <t>BHARATSE</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Wheels</t>
+          <t>Seating</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1022.05</v>
+        <v>174.84</v>
       </c>
       <c r="D7" t="n">
-        <v>0.1372538110604204</v>
+        <v>0.0900928985597606</v>
       </c>
       <c r="E7" t="n">
-        <v>0.2600789051904819</v>
+        <v>0.0945971326613661</v>
       </c>
       <c r="F7" t="n">
-        <v>0.2660885723134096</v>
+        <v>0.08717821166521569</v>
       </c>
       <c r="G7" t="n">
-        <v>0.3052042561609918</v>
+        <v>0.1262938955127979</v>
       </c>
       <c r="H7" t="n">
-        <v>0.3170207782417001</v>
+        <v>0.1381104175935062</v>
       </c>
       <c r="I7" t="n">
-        <v>49.39104915627291</v>
+        <v>64.33915211970074</v>
       </c>
       <c r="J7" t="n">
         <v>80</v>
       </c>
       <c r="K7" t="n">
-        <v>46.83</v>
+        <v>52.61</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M7" t="n">
-        <v>46.83</v>
+        <v>52.61</v>
       </c>
       <c r="N7" t="n">
         <v>80</v>
       </c>
       <c r="O7" t="n">
-        <v>87.2340425531915</v>
+        <v>74.46808510638297</v>
       </c>
       <c r="P7" t="n">
-        <v>68.17880851063831</v>
+        <v>67.93761702127659</v>
       </c>
       <c r="Q7" t="b">
         <v>0</v>
@@ -4326,63 +4326,63 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ASKAUTOLTD</t>
+          <t>SANSERA</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Forgings</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>435.5</v>
+        <v>2346.2</v>
       </c>
       <c r="D8" t="n">
-        <v>0.0825254784986329</v>
+        <v>0.1575883165581211</v>
       </c>
       <c r="E8" t="n">
-        <v>-0.08277169334456611</v>
+        <v>0.2773301393728222</v>
       </c>
       <c r="F8" t="n">
-        <v>-0.1571511515386104</v>
+        <v>0.5689447639427576</v>
       </c>
       <c r="G8" t="n">
-        <v>-0.1180354676910283</v>
+        <v>0.6080604477903397</v>
       </c>
       <c r="H8" t="n">
-        <v>-0.1062189456103199</v>
+        <v>0.6198769698710481</v>
       </c>
       <c r="I8" t="n">
-        <v>64.6589259796807</v>
+        <v>70.82695252679936</v>
       </c>
       <c r="J8" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K8" t="n">
-        <v>71.28</v>
+        <v>48.59</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M8" t="n">
-        <v>71.28</v>
+        <v>48.59</v>
       </c>
       <c r="N8" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O8" t="n">
-        <v>34.04255319148936</v>
+        <v>97.87234042553192</v>
       </c>
       <c r="P8" t="n">
-        <v>67.32051063829788</v>
+        <v>67.0104680851064</v>
       </c>
       <c r="Q8" t="b">
+        <v>0</v>
+      </c>
+      <c r="R8" t="b">
         <v>1</v>
-      </c>
-      <c r="R8" t="b">
-        <v>0</v>
       </c>
       <c r="S8" t="b">
         <v>0</v>
@@ -4391,57 +4391,57 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SANSERA</t>
+          <t>SHRIPISTON</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Forgings</t>
+          <t>Engine/Parts</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>2346.2</v>
+        <v>3610.5</v>
       </c>
       <c r="D9" t="n">
-        <v>0.2010852871915633</v>
+        <v>0.227017841971113</v>
       </c>
       <c r="E9" t="n">
-        <v>0.2942409532215357</v>
+        <v>0.1632514981635413</v>
       </c>
       <c r="F9" t="n">
-        <v>0.5693645484949832</v>
+        <v>0.3884936353497672</v>
       </c>
       <c r="G9" t="n">
-        <v>0.6084802323425653</v>
+        <v>0.4276093191973493</v>
       </c>
       <c r="H9" t="n">
-        <v>0.6202967544232737</v>
+        <v>0.4394258412780577</v>
       </c>
       <c r="I9" t="n">
-        <v>75.09261276966656</v>
+        <v>79.11131470453508</v>
       </c>
       <c r="J9" t="n">
         <v>70</v>
       </c>
       <c r="K9" t="n">
-        <v>48.59</v>
+        <v>48.69</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M9" t="n">
-        <v>48.59</v>
+        <v>48.69</v>
       </c>
       <c r="N9" t="n">
         <v>70</v>
       </c>
       <c r="O9" t="n">
-        <v>97.87234042553192</v>
+        <v>93.61702127659576</v>
       </c>
       <c r="P9" t="n">
-        <v>67.0104680851064</v>
+        <v>66.19940425531915</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -4456,57 +4456,57 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>FIEMIND</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Lighting</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>569.3</v>
+        <v>2164.9</v>
       </c>
       <c r="D10" t="n">
-        <v>0.1712786750334327</v>
+        <v>0.0797506234413965</v>
       </c>
       <c r="E10" t="n">
-        <v>0.2385510714674208</v>
+        <v>-0.0255660080118826</v>
       </c>
       <c r="F10" t="n">
-        <v>0.305135259055479</v>
+        <v>0.08543494610178</v>
       </c>
       <c r="G10" t="n">
-        <v>0.3442509429030611</v>
+        <v>0.1245506299493621</v>
       </c>
       <c r="H10" t="n">
-        <v>0.3560674649837695</v>
+        <v>0.1363671520300705</v>
       </c>
       <c r="I10" t="n">
-        <v>73.72773536895671</v>
+        <v>57.57971284728698</v>
       </c>
       <c r="J10" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K10" t="n">
-        <v>49.66</v>
+        <v>49.06</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M10" t="n">
-        <v>49.66</v>
+        <v>49.06</v>
       </c>
       <c r="N10" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O10" t="n">
-        <v>89.36170212765957</v>
+        <v>72.3404255319149</v>
       </c>
       <c r="P10" t="n">
-        <v>65.73634042553192</v>
+        <v>66.09208510638298</v>
       </c>
       <c r="Q10" t="b">
         <v>0</v>
@@ -4521,7 +4521,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>PRICOLLTD</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -4530,48 +4530,48 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>573.1</v>
+        <v>569.3</v>
       </c>
       <c r="D11" t="n">
-        <v>0.1088323498113572</v>
+        <v>0.1637367130008176</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.085089399744572</v>
+        <v>0.2461420597570316</v>
       </c>
       <c r="F11" t="n">
-        <v>0.0615911827359452</v>
+        <v>0.3535425582501186</v>
       </c>
       <c r="G11" t="n">
-        <v>0.1007068665835273</v>
+        <v>0.3926582420977007</v>
       </c>
       <c r="H11" t="n">
-        <v>0.1125233886642357</v>
+        <v>0.4044747641784091</v>
       </c>
       <c r="I11" t="n">
-        <v>65.30249110320284</v>
+        <v>70.59451762192948</v>
       </c>
       <c r="J11" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K11" t="n">
-        <v>49.98</v>
+        <v>49.66</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M11" t="n">
-        <v>49.98</v>
+        <v>49.66</v>
       </c>
       <c r="N11" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O11" t="n">
-        <v>68.08510638297872</v>
+        <v>89.36170212765957</v>
       </c>
       <c r="P11" t="n">
-        <v>65.60902127659575</v>
+        <v>65.73634042553192</v>
       </c>
       <c r="Q11" t="b">
         <v>0</v>
@@ -4586,48 +4586,48 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>FIEMIND</t>
+          <t>PRICOLLTD</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Lighting</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>2164.9</v>
+        <v>573.1</v>
       </c>
       <c r="D12" t="n">
-        <v>0.0571833186834651</v>
+        <v>0.0903729071537291</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.0295844726343628</v>
+        <v>-0.1023572715169551</v>
       </c>
       <c r="F12" t="n">
-        <v>0.0601860920666015</v>
+        <v>0.0587474598189545</v>
       </c>
       <c r="G12" t="n">
-        <v>0.0993017759141836</v>
+        <v>0.0978631436665367</v>
       </c>
       <c r="H12" t="n">
-        <v>0.111118297994892</v>
+        <v>0.109679665747245</v>
       </c>
       <c r="I12" t="n">
-        <v>62.61298274445357</v>
+        <v>61.50809317015396</v>
       </c>
       <c r="J12" t="n">
         <v>80</v>
       </c>
       <c r="K12" t="n">
-        <v>49.06</v>
+        <v>49.98</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M12" t="n">
-        <v>49.06</v>
+        <v>49.98</v>
       </c>
       <c r="N12" t="n">
         <v>80</v>
@@ -4636,7 +4636,7 @@
         <v>65.95744680851064</v>
       </c>
       <c r="P12" t="n">
-        <v>64.81548936170213</v>
+        <v>65.18348936170213</v>
       </c>
       <c r="Q12" t="b">
         <v>0</v>
@@ -4651,57 +4651,57 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CRAFTSMAN</t>
+          <t>DIVGIITTS</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Castings</t>
+          <t>Transmission</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>7398.5</v>
+        <v>689.2</v>
       </c>
       <c r="D13" t="n">
-        <v>0.1085555888522624</v>
+        <v>0.0470186099506266</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.0291956436163233</v>
+        <v>0.1804401815534813</v>
       </c>
       <c r="F13" t="n">
-        <v>0.0917072450936993</v>
+        <v>0.0355345203215387</v>
       </c>
       <c r="G13" t="n">
-        <v>0.1308229289412814</v>
+        <v>0.0746502041691208</v>
       </c>
       <c r="H13" t="n">
-        <v>0.1426394510219898</v>
+        <v>0.08646672624982921</v>
       </c>
       <c r="I13" t="n">
-        <v>70.8286464191976</v>
+        <v>47.49481174029056</v>
       </c>
       <c r="J13" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K13" t="n">
-        <v>54.65</v>
+        <v>49.92</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M13" t="n">
-        <v>54.65</v>
+        <v>49.92</v>
       </c>
       <c r="N13" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O13" t="n">
-        <v>72.3404255319149</v>
+        <v>61.70212765957447</v>
       </c>
       <c r="P13" t="n">
-        <v>64.32808510638299</v>
+        <v>64.30842553191489</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
@@ -4716,57 +4716,57 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>DIVGIITTS</t>
+          <t>WHEELS</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Transmission</t>
+          <t>Wheels</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>689.2</v>
+        <v>1022.05</v>
       </c>
       <c r="D14" t="n">
-        <v>0.0242235101798187</v>
+        <v>0.1107428136716839</v>
       </c>
       <c r="E14" t="n">
-        <v>0.1711129991503823</v>
+        <v>0.2711274174491636</v>
       </c>
       <c r="F14" t="n">
-        <v>0.0390471883009198</v>
+        <v>0.2812460824871503</v>
       </c>
       <c r="G14" t="n">
-        <v>0.0781628721485019</v>
+        <v>0.3203617663347324</v>
       </c>
       <c r="H14" t="n">
-        <v>0.08997939422921029</v>
+        <v>0.3321782884154408</v>
       </c>
       <c r="I14" t="n">
-        <v>47.66548463356975</v>
+        <v>37.83345349675558</v>
       </c>
       <c r="J14" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K14" t="n">
-        <v>49.92</v>
+        <v>46.83</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M14" t="n">
-        <v>49.92</v>
+        <v>46.83</v>
       </c>
       <c r="N14" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O14" t="n">
-        <v>61.70212765957447</v>
+        <v>87.2340425531915</v>
       </c>
       <c r="P14" t="n">
-        <v>64.30842553191489</v>
+        <v>64.17880851063831</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
@@ -4793,22 +4793,22 @@
         <v>5399.4</v>
       </c>
       <c r="D15" t="n">
-        <v>0.1217201620442505</v>
+        <v>0.1014687882496938</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.0133576975788031</v>
+        <v>-0.0341829889991951</v>
       </c>
       <c r="F15" t="n">
-        <v>0.2355889150781482</v>
+        <v>0.263076635164218</v>
       </c>
       <c r="G15" t="n">
-        <v>0.2747045989257304</v>
+        <v>0.3021923190118001</v>
       </c>
       <c r="H15" t="n">
-        <v>0.2865211210064388</v>
+        <v>0.3140088410925085</v>
       </c>
       <c r="I15" t="n">
-        <v>60.04729402912881</v>
+        <v>57.21931288484777</v>
       </c>
       <c r="J15" t="n">
         <v>60</v>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M15" t="n">
@@ -4846,60 +4846,60 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>MENONBE</t>
+          <t>ASKAUTOLTD</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Bearings</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>117.86</v>
+        <v>435.5</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.0399934837501018</v>
+        <v>0.0671404067630481</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.0036351339927297</v>
+        <v>-0.0592936602224861</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.090094958696827</v>
+        <v>-0.1535471331389698</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.0509792748492449</v>
+        <v>-0.1144314492913877</v>
       </c>
       <c r="H16" t="n">
-        <v>-0.0391627527685365</v>
+        <v>-0.1026149272106793</v>
       </c>
       <c r="I16" t="n">
-        <v>59.78781656399726</v>
+        <v>39.20099875156056</v>
       </c>
       <c r="J16" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K16" t="n">
-        <v>52.38</v>
+        <v>71.28</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="M16" t="n">
-        <v>52.38</v>
+        <v>71.28</v>
       </c>
       <c r="N16" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O16" t="n">
-        <v>51.06382978723404</v>
+        <v>36.17021276595745</v>
       </c>
       <c r="P16" t="n">
-        <v>63.1647659574468</v>
+        <v>63.74604255319149</v>
       </c>
       <c r="Q16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R16" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
chore: auto-refresh NSE data and pipeline outputs (2026-04-15)
</commit_message>
<xml_diff>
--- a/working-sector/output/auto_components_comprehensive_report.xlsx
+++ b/working-sector/output/auto_components_comprehensive_report.xlsx
@@ -435,7 +435,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -447,7 +447,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -779,25 +779,25 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1801.3</v>
+        <v>1831.6</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0614614024749557</v>
+        <v>0.0490263459335624</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2366469861320885</v>
+        <v>0.2542628227076628</v>
       </c>
       <c r="F2" t="n">
-        <v>0.4341560509554139</v>
+        <v>0.4641087130295762</v>
       </c>
       <c r="G2" t="n">
-        <v>0.473271734802996</v>
+        <v>0.4938416460402579</v>
       </c>
       <c r="H2" t="n">
-        <v>0.4850882568837044</v>
+        <v>0.5003485403716336</v>
       </c>
       <c r="I2" t="n">
-        <v>59.62566844919785</v>
+        <v>62.95993458708093</v>
       </c>
       <c r="J2" t="n">
         <v>80</v>
@@ -807,7 +807,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M2" t="n">
@@ -844,25 +844,25 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1078.2</v>
+        <v>1100.1</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0586156111929307</v>
+        <v>0.0447293447293446</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.1089256198347107</v>
+        <v>-0.08386075949367081</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.178639445417841</v>
+        <v>-0.164755903120492</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.1395237615702589</v>
+        <v>-0.1350229701098103</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.1277072394895505</v>
+        <v>-0.1285160757784347</v>
       </c>
       <c r="I3" t="n">
-        <v>48.21834723275212</v>
+        <v>52.18760938046901</v>
       </c>
       <c r="J3" t="n">
         <v>60</v>
@@ -872,7 +872,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M3" t="n">
@@ -909,25 +909,25 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>36615</v>
+        <v>37080</v>
       </c>
       <c r="D4" t="n">
-        <v>0.2062263218580136</v>
+        <v>0.209985315712188</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.0277482740308019</v>
+        <v>-0.0217649386624455</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.0746777862016679</v>
+        <v>-0.0586443259710586</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.0355621023540858</v>
+        <v>-0.0289113929603769</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.0237455802733774</v>
+        <v>-0.0224044986290012</v>
       </c>
       <c r="I4" t="n">
-        <v>78.35990888382688</v>
+        <v>79.23951048951048</v>
       </c>
       <c r="J4" t="n">
         <v>70</v>
@@ -937,7 +937,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M4" t="n">
@@ -947,10 +947,10 @@
         <v>70</v>
       </c>
       <c r="O4" t="n">
-        <v>53.19148936170212</v>
+        <v>51.06382978723404</v>
       </c>
       <c r="P4" t="n">
-        <v>60.03029787234042</v>
+        <v>59.6047659574468</v>
       </c>
       <c r="Q4" t="b">
         <v>0</v>
@@ -974,25 +974,25 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>324.8</v>
+        <v>330</v>
       </c>
       <c r="D5" t="n">
-        <v>0.1004573945451465</v>
+        <v>0.093077177873468</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.0712038890477552</v>
+        <v>-0.0462427745664739</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.1957409929429243</v>
+        <v>-0.1816491010539367</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.1566253090953422</v>
+        <v>-0.151916168043255</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.1448087870146338</v>
+        <v>-0.1454092737118794</v>
       </c>
       <c r="I5" t="n">
-        <v>63.14221891288162</v>
+        <v>65.79129232895647</v>
       </c>
       <c r="J5" t="n">
         <v>80</v>
@@ -1002,7 +1002,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M5" t="n">
@@ -1012,10 +1012,10 @@
         <v>80</v>
       </c>
       <c r="O5" t="n">
-        <v>21.27659574468085</v>
+        <v>23.40425531914894</v>
       </c>
       <c r="P5" t="n">
-        <v>56.70331914893617</v>
+        <v>57.12885106382979</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
@@ -1039,48 +1039,48 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>119.11</v>
+        <v>123.55</v>
       </c>
       <c r="D6" t="n">
-        <v>0.0510942463819272</v>
+        <v>0.0666493999827333</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0358292025393511</v>
+        <v>0.0750021752371008</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0833105957253297</v>
+        <v>0.1023376159885796</v>
       </c>
       <c r="G6" t="n">
-        <v>0.1224262795729118</v>
+        <v>0.1320705489992613</v>
       </c>
       <c r="H6" t="n">
-        <v>0.1342428016536202</v>
+        <v>0.1385774433306369</v>
       </c>
       <c r="I6" t="n">
-        <v>59.27995034140286</v>
+        <v>64.21167484997272</v>
       </c>
       <c r="J6" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K6" t="n">
         <v>51.57</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M6" t="n">
         <v>51.57</v>
       </c>
       <c r="N6" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O6" t="n">
-        <v>70.21276595744681</v>
+        <v>72.3404255319149</v>
       </c>
       <c r="P6" t="n">
-        <v>58.67055319148936</v>
+        <v>67.09608510638299</v>
       </c>
       <c r="Q6" t="b">
         <v>0</v>
@@ -1104,25 +1104,25 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2715.5</v>
+        <v>2755</v>
       </c>
       <c r="D7" t="n">
-        <v>0.1210419848903934</v>
+        <v>0.1127266852457691</v>
       </c>
       <c r="E7" t="n">
-        <v>0.1273716112425791</v>
+        <v>0.1540233736857537</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.1894271812781708</v>
+        <v>-0.1659097789887981</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.1503114974305887</v>
+        <v>-0.1361768459781164</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.1384949753498803</v>
+        <v>-0.1296699516467407</v>
       </c>
       <c r="I7" t="n">
-        <v>53.82482089207303</v>
+        <v>57.68742058449809</v>
       </c>
       <c r="J7" t="n">
         <v>80</v>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M7" t="n">
@@ -1169,25 +1169,25 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>569.3</v>
+        <v>585.7</v>
       </c>
       <c r="D8" t="n">
-        <v>0.1637367130008176</v>
+        <v>0.1665006970722964</v>
       </c>
       <c r="E8" t="n">
-        <v>0.2461420597570316</v>
+        <v>0.2814790504321192</v>
       </c>
       <c r="F8" t="n">
-        <v>0.3535425582501186</v>
+        <v>0.390055773110241</v>
       </c>
       <c r="G8" t="n">
-        <v>0.3926582420977007</v>
+        <v>0.4197887061209226</v>
       </c>
       <c r="H8" t="n">
-        <v>0.4044747641784091</v>
+        <v>0.4262956004522983</v>
       </c>
       <c r="I8" t="n">
-        <v>70.59451762192948</v>
+        <v>73.66911061523747</v>
       </c>
       <c r="J8" t="n">
         <v>70</v>
@@ -1197,7 +1197,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M8" t="n">
@@ -1207,10 +1207,10 @@
         <v>70</v>
       </c>
       <c r="O8" t="n">
-        <v>89.36170212765957</v>
+        <v>91.48936170212764</v>
       </c>
       <c r="P8" t="n">
-        <v>65.73634042553192</v>
+        <v>66.16187234042553</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
@@ -1234,25 +1234,25 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>432.4</v>
+        <v>441.6</v>
       </c>
       <c r="D9" t="n">
-        <v>0.0474806201550386</v>
+        <v>0.0465694987557767</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.1415525114155251</v>
+        <v>-0.1515850144092219</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.1110197368421053</v>
+        <v>-0.0970248440854718</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.0719040529945231</v>
+        <v>-0.0672919110747901</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.0600875309138148</v>
+        <v>-0.0607850167434145</v>
       </c>
       <c r="I9" t="n">
-        <v>61.60145586897178</v>
+        <v>67.10833982852691</v>
       </c>
       <c r="J9" t="n">
         <v>60</v>
@@ -1262,7 +1262,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M9" t="n">
@@ -1272,10 +1272,10 @@
         <v>60</v>
       </c>
       <c r="O9" t="n">
-        <v>48.93617021276596</v>
+        <v>46.80851063829788</v>
       </c>
       <c r="P9" t="n">
-        <v>55.1632340425532</v>
+        <v>54.73770212765958</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -1299,48 +1299,48 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>134315</v>
+        <v>137900</v>
       </c>
       <c r="D10" t="n">
-        <v>0.0148853375646982</v>
+        <v>0.0387947269303201</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.096950953037281</v>
+        <v>-0.0664139191659332</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.1212626758259731</v>
+        <v>-0.1156571648443262</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.082146991978391</v>
+        <v>-0.0859242318336445</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.0703304698976826</v>
+        <v>-0.0794173375022688</v>
       </c>
       <c r="I10" t="n">
-        <v>62.4249356591364</v>
+        <v>68.81822496440437</v>
       </c>
       <c r="J10" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K10" t="n">
         <v>49.41</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M10" t="n">
         <v>49.41</v>
       </c>
       <c r="N10" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O10" t="n">
         <v>42.5531914893617</v>
       </c>
       <c r="P10" t="n">
-        <v>52.27463829787234</v>
+        <v>60.27463829787234</v>
       </c>
       <c r="Q10" t="b">
         <v>0</v>
@@ -1376,10 +1376,10 @@
         <v>-0.0042030657656173</v>
       </c>
       <c r="G11" t="n">
-        <v>0.0349126180819647</v>
+        <v>0.0255298672450643</v>
       </c>
       <c r="H11" t="n">
-        <v>0.0467291401626731</v>
+        <v>0.0320367615764399</v>
       </c>
       <c r="I11" t="n">
         <v>27.6054590570719</v>
@@ -1392,7 +1392,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M11" t="n">
@@ -1429,48 +1429,48 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>435.5</v>
+        <v>440.15</v>
       </c>
       <c r="D12" t="n">
-        <v>0.0671404067630481</v>
+        <v>0.08411330049261059</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.0592936602224861</v>
+        <v>-0.0548636461241142</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.1535471331389698</v>
+        <v>-0.1780578898225957</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.1144314492913877</v>
+        <v>-0.148324956811914</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.1026149272106793</v>
+        <v>-0.1418180624805384</v>
       </c>
       <c r="I12" t="n">
-        <v>39.20099875156056</v>
+        <v>45.52572706935123</v>
       </c>
       <c r="J12" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K12" t="n">
         <v>71.28</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M12" t="n">
         <v>71.28</v>
       </c>
       <c r="N12" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O12" t="n">
-        <v>36.17021276595745</v>
+        <v>25.53191489361702</v>
       </c>
       <c r="P12" t="n">
-        <v>63.74604255319149</v>
+        <v>65.6183829787234</v>
       </c>
       <c r="Q12" t="b">
         <v>1</v>
@@ -1494,25 +1494,25 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1690.5</v>
+        <v>1727.2</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.0148601398601398</v>
+        <v>0.0046533271288971</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.1214074112572111</v>
+        <v>-0.0945690920528412</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.0563773374267373</v>
+        <v>-0.0475350170949597</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.0172616535791552</v>
+        <v>-0.017802084084278</v>
       </c>
       <c r="H13" t="n">
-        <v>-0.0054451314984468</v>
+        <v>-0.0112951897529024</v>
       </c>
       <c r="I13" t="n">
-        <v>55.56480710519011</v>
+        <v>59.67254408060453</v>
       </c>
       <c r="J13" t="n">
         <v>60</v>
@@ -1522,7 +1522,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M13" t="n">
@@ -1559,48 +1559,48 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>578.8</v>
+        <v>596.9</v>
       </c>
       <c r="D14" t="n">
-        <v>0.0292522450431225</v>
+        <v>0.0350268770591293</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.0990738578877734</v>
+        <v>-0.0800647299067581</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.2973596358118362</v>
+        <v>-0.2676972150656361</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.2582439519642541</v>
+        <v>-0.2379642820549544</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.2464274298835457</v>
+        <v>-0.2314573877235788</v>
       </c>
       <c r="I14" t="n">
-        <v>54.3651753325272</v>
+        <v>58.03869246164109</v>
       </c>
       <c r="J14" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K14" t="n">
         <v>54.64</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M14" t="n">
         <v>54.64</v>
       </c>
       <c r="N14" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O14" t="n">
-        <v>4.25531914893617</v>
+        <v>8.51063829787234</v>
       </c>
       <c r="P14" t="n">
-        <v>46.70706382978724</v>
+        <v>55.55812765957447</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
@@ -1624,48 +1624,48 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>105.26</v>
+        <v>111.65</v>
       </c>
       <c r="D15" t="n">
-        <v>0.1094013490725127</v>
+        <v>0.1548407116259826</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.0207461159177596</v>
+        <v>0.0538984330753258</v>
       </c>
       <c r="F15" t="n">
-        <v>0.1872321227159938</v>
+        <v>0.2647258722247394</v>
       </c>
       <c r="G15" t="n">
-        <v>0.226347806563576</v>
+        <v>0.2944588052354211</v>
       </c>
       <c r="H15" t="n">
-        <v>0.2381643286442843</v>
+        <v>0.3009656995667967</v>
       </c>
       <c r="I15" t="n">
-        <v>65.97524255603882</v>
+        <v>71.96802646085999</v>
       </c>
       <c r="J15" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K15" t="n">
         <v>51.91</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M15" t="n">
         <v>51.91</v>
       </c>
       <c r="N15" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O15" t="n">
-        <v>82.97872340425532</v>
+        <v>85.1063829787234</v>
       </c>
       <c r="P15" t="n">
-        <v>69.35974468085107</v>
+        <v>65.78527659574468</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
@@ -1689,25 +1689,25 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>174.84</v>
+        <v>184.81</v>
       </c>
       <c r="D16" t="n">
-        <v>0.0900928985597606</v>
+        <v>0.1359641035097425</v>
       </c>
       <c r="E16" t="n">
-        <v>0.0945971326613661</v>
+        <v>0.140098704503393</v>
       </c>
       <c r="F16" t="n">
-        <v>0.08717821166521569</v>
+        <v>0.0944569465829681</v>
       </c>
       <c r="G16" t="n">
-        <v>0.1262938955127979</v>
+        <v>0.1241898795936498</v>
       </c>
       <c r="H16" t="n">
-        <v>0.1381104175935062</v>
+        <v>0.1306967739250254</v>
       </c>
       <c r="I16" t="n">
-        <v>64.33915211970074</v>
+        <v>69.71713810316139</v>
       </c>
       <c r="J16" t="n">
         <v>80</v>
@@ -1717,7 +1717,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M16" t="n">
@@ -1727,10 +1727,10 @@
         <v>80</v>
       </c>
       <c r="O16" t="n">
-        <v>74.46808510638297</v>
+        <v>68.08510638297872</v>
       </c>
       <c r="P16" t="n">
-        <v>67.93761702127659</v>
+        <v>66.66102127659575</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>
@@ -1754,25 +1754,25 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>7398.5</v>
+        <v>7433.5</v>
       </c>
       <c r="D17" t="n">
-        <v>0.0892160471107839</v>
+        <v>0.07467110018794269</v>
       </c>
       <c r="E17" t="n">
-        <v>-0.0129410979921286</v>
+        <v>-0.0329148507122877</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0917877960599129</v>
+        <v>0.0924388272466749</v>
       </c>
       <c r="G17" t="n">
-        <v>0.130903479907495</v>
+        <v>0.1221717602573566</v>
       </c>
       <c r="H17" t="n">
-        <v>0.1427200019882034</v>
+        <v>0.1286786545887323</v>
       </c>
       <c r="I17" t="n">
-        <v>65.49889135254989</v>
+        <v>66.53763440860214</v>
       </c>
       <c r="J17" t="n">
         <v>80</v>
@@ -1782,7 +1782,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M17" t="n">
@@ -1792,10 +1792,10 @@
         <v>80</v>
       </c>
       <c r="O17" t="n">
-        <v>76.59574468085107</v>
+        <v>65.95744680851064</v>
       </c>
       <c r="P17" t="n">
-        <v>69.17914893617021</v>
+        <v>67.05148936170212</v>
       </c>
       <c r="Q17" t="b">
         <v>0</v>
@@ -1819,25 +1819,25 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>689.2</v>
+        <v>777.75</v>
       </c>
       <c r="D18" t="n">
-        <v>0.0470186099506266</v>
+        <v>0.1547884187082404</v>
       </c>
       <c r="E18" t="n">
-        <v>0.1804401815534813</v>
+        <v>0.3238297872340425</v>
       </c>
       <c r="F18" t="n">
-        <v>0.0355345203215387</v>
+        <v>0.1768933948702429</v>
       </c>
       <c r="G18" t="n">
-        <v>0.0746502041691208</v>
+        <v>0.2066263278809246</v>
       </c>
       <c r="H18" t="n">
-        <v>0.08646672624982921</v>
+        <v>0.2131332222123002</v>
       </c>
       <c r="I18" t="n">
-        <v>47.49481174029056</v>
+        <v>65.57153965785382</v>
       </c>
       <c r="J18" t="n">
         <v>80</v>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M18" t="n">
@@ -1857,10 +1857,10 @@
         <v>80</v>
       </c>
       <c r="O18" t="n">
-        <v>61.70212765957447</v>
+        <v>80.85106382978722</v>
       </c>
       <c r="P18" t="n">
-        <v>64.30842553191489</v>
+        <v>68.13821276595745</v>
       </c>
       <c r="Q18" t="b">
         <v>0</v>
@@ -1884,25 +1884,25 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2391.8</v>
+        <v>2412.4</v>
       </c>
       <c r="D19" t="n">
-        <v>0.0001672660366311</v>
+        <v>0.0362097848030584</v>
       </c>
       <c r="E19" t="n">
-        <v>-0.07045975671369149</v>
+        <v>-0.0677795811113687</v>
       </c>
       <c r="F19" t="n">
-        <v>-0.1624763638910288</v>
+        <v>-0.153722023433663</v>
       </c>
       <c r="G19" t="n">
-        <v>-0.1233606800434466</v>
+        <v>-0.1239890904229813</v>
       </c>
       <c r="H19" t="n">
-        <v>-0.1115441579627383</v>
+        <v>-0.1174821960916057</v>
       </c>
       <c r="I19" t="n">
-        <v>56.10060278528375</v>
+        <v>57.90312936017543</v>
       </c>
       <c r="J19" t="n">
         <v>60</v>
@@ -1912,7 +1912,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M19" t="n">
@@ -1922,10 +1922,10 @@
         <v>60</v>
       </c>
       <c r="O19" t="n">
-        <v>31.91489361702128</v>
+        <v>36.17021276595745</v>
       </c>
       <c r="P19" t="n">
-        <v>50.89097872340426</v>
+        <v>51.7420425531915</v>
       </c>
       <c r="Q19" t="b">
         <v>0</v>
@@ -1949,25 +1949,25 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2164.9</v>
+        <v>2241.3</v>
       </c>
       <c r="D20" t="n">
-        <v>0.0797506234413965</v>
+        <v>0.1188598242811502</v>
       </c>
       <c r="E20" t="n">
-        <v>-0.0255660080118826</v>
+        <v>-0.0063838276366536</v>
       </c>
       <c r="F20" t="n">
-        <v>0.08543494610178</v>
+        <v>0.1097742127153893</v>
       </c>
       <c r="G20" t="n">
-        <v>0.1245506299493621</v>
+        <v>0.139507145726071</v>
       </c>
       <c r="H20" t="n">
-        <v>0.1363671520300705</v>
+        <v>0.1460140400574466</v>
       </c>
       <c r="I20" t="n">
-        <v>57.57971284728698</v>
+        <v>62.86926717806433</v>
       </c>
       <c r="J20" t="n">
         <v>80</v>
@@ -1977,7 +1977,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M20" t="n">
@@ -1987,10 +1987,10 @@
         <v>80</v>
       </c>
       <c r="O20" t="n">
-        <v>72.3404255319149</v>
+        <v>74.46808510638297</v>
       </c>
       <c r="P20" t="n">
-        <v>66.09208510638298</v>
+        <v>66.51761702127659</v>
       </c>
       <c r="Q20" t="b">
         <v>0</v>
@@ -2014,25 +2014,25 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>927.65</v>
+        <v>964.4</v>
       </c>
       <c r="D21" t="n">
-        <v>0.1167087998073912</v>
+        <v>0.1425186589266673</v>
       </c>
       <c r="E21" t="n">
-        <v>-0.0326903023983315</v>
+        <v>0.0123871509552802</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.2783741734733567</v>
+        <v>-0.2521132221791392</v>
       </c>
       <c r="G21" t="n">
-        <v>-0.2392584896257745</v>
+        <v>-0.2223802891684575</v>
       </c>
       <c r="H21" t="n">
-        <v>-0.2274419675450661</v>
+        <v>-0.2158733948370819</v>
       </c>
       <c r="I21" t="n">
-        <v>61.72309247094492</v>
+        <v>67.71787769017686</v>
       </c>
       <c r="J21" t="n">
         <v>80</v>
@@ -2042,7 +2042,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M21" t="n">
@@ -2052,10 +2052,10 @@
         <v>80</v>
       </c>
       <c r="O21" t="n">
-        <v>8.51063829787234</v>
+        <v>12.76595744680851</v>
       </c>
       <c r="P21" t="n">
-        <v>53.07412765957447</v>
+        <v>53.9251914893617</v>
       </c>
       <c r="Q21" t="b">
         <v>0</v>
@@ -2079,25 +2079,25 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>440.1</v>
+        <v>443.7</v>
       </c>
       <c r="D22" t="n">
-        <v>0.1469898358092261</v>
+        <v>0.136381098732232</v>
       </c>
       <c r="E22" t="n">
-        <v>0.2606702950443997</v>
+        <v>0.2630230572160545</v>
       </c>
       <c r="F22" t="n">
-        <v>0.3791914760263239</v>
+        <v>0.3515077672860187</v>
       </c>
       <c r="G22" t="n">
-        <v>0.4183071598739061</v>
+        <v>0.3812407002967004</v>
       </c>
       <c r="H22" t="n">
-        <v>0.4301236819546145</v>
+        <v>0.387747594628076</v>
       </c>
       <c r="I22" t="n">
-        <v>65.00512120177535</v>
+        <v>65.84471842719094</v>
       </c>
       <c r="J22" t="n">
         <v>80</v>
@@ -2107,7 +2107,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M22" t="n">
@@ -2117,10 +2117,10 @@
         <v>80</v>
       </c>
       <c r="O22" t="n">
-        <v>91.48936170212764</v>
+        <v>89.36170212765957</v>
       </c>
       <c r="P22" t="n">
-        <v>72.08587234042552</v>
+        <v>71.66034042553191</v>
       </c>
       <c r="Q22" t="b">
         <v>0</v>
@@ -2144,48 +2144,48 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>370.2</v>
+        <v>381.25</v>
       </c>
       <c r="D23" t="n">
-        <v>0.0951042745156041</v>
+        <v>0.1154183733177296</v>
       </c>
       <c r="E23" t="n">
-        <v>-0.0146393398988554</v>
+        <v>-0.0102544132917964</v>
       </c>
       <c r="F23" t="n">
-        <v>-0.12129124139568</v>
+        <v>-0.096135609293504</v>
       </c>
       <c r="G23" t="n">
-        <v>-0.0821755575480979</v>
+        <v>-0.0664026762828223</v>
       </c>
       <c r="H23" t="n">
-        <v>-0.0703590354673895</v>
+        <v>-0.0598957819514467</v>
       </c>
       <c r="I23" t="n">
-        <v>69.90346394094266</v>
+        <v>73.2593340060545</v>
       </c>
       <c r="J23" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K23" t="n">
         <v>49.7</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M23" t="n">
         <v>49.7</v>
       </c>
       <c r="N23" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O23" t="n">
-        <v>40.42553191489361</v>
+        <v>48.93617021276596</v>
       </c>
       <c r="P23" t="n">
-        <v>59.96510638297872</v>
+        <v>57.6672340425532</v>
       </c>
       <c r="Q23" t="b">
         <v>0</v>
@@ -2209,25 +2209,25 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>122.92</v>
+        <v>123.81</v>
       </c>
       <c r="D24" t="n">
-        <v>0.0338968794684162</v>
+        <v>0.034249436137332</v>
       </c>
       <c r="E24" t="n">
-        <v>-0.024521863344179</v>
+        <v>-0.0727231875374476</v>
       </c>
       <c r="F24" t="n">
-        <v>0.173684713071708</v>
+        <v>0.1537601341906624</v>
       </c>
       <c r="G24" t="n">
-        <v>0.2128003969192902</v>
+        <v>0.1834930672013441</v>
       </c>
       <c r="H24" t="n">
-        <v>0.2246169189999985</v>
+        <v>0.1899999615327198</v>
       </c>
       <c r="I24" t="n">
-        <v>52.04744422479526</v>
+        <v>53.22314049586777</v>
       </c>
       <c r="J24" t="n">
         <v>60</v>
@@ -2237,7 +2237,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M24" t="n">
@@ -2247,10 +2247,10 @@
         <v>60</v>
       </c>
       <c r="O24" t="n">
-        <v>80.85106382978722</v>
+        <v>78.72340425531915</v>
       </c>
       <c r="P24" t="n">
-        <v>59.49021276595744</v>
+        <v>59.06468085106384</v>
       </c>
       <c r="Q24" t="b">
         <v>0</v>
@@ -2274,25 +2274,25 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>624.6</v>
+        <v>628.15</v>
       </c>
       <c r="D25" t="n">
-        <v>0.2846565199506377</v>
+        <v>0.2762088581877284</v>
       </c>
       <c r="E25" t="n">
-        <v>0.0414339308045019</v>
+        <v>0.0336514727661674</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.1578805446946205</v>
+        <v>-0.1490788404226497</v>
       </c>
       <c r="G25" t="n">
-        <v>-0.1187648608470384</v>
+        <v>-0.119345907411968</v>
       </c>
       <c r="H25" t="n">
-        <v>-0.10694833876633</v>
+        <v>-0.1128390130805924</v>
       </c>
       <c r="I25" t="n">
-        <v>65.32900560637357</v>
+        <v>66.04046242774567</v>
       </c>
       <c r="J25" t="n">
         <v>80</v>
@@ -2302,7 +2302,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M25" t="n">
@@ -2312,10 +2312,10 @@
         <v>80</v>
       </c>
       <c r="O25" t="n">
-        <v>34.04255319148936</v>
+        <v>38.29787234042553</v>
       </c>
       <c r="P25" t="n">
-        <v>61.57251063829787</v>
+        <v>62.42357446808511</v>
       </c>
       <c r="Q25" t="b">
         <v>0</v>
@@ -2339,25 +2339,25 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>132.2</v>
+        <v>133.18</v>
       </c>
       <c r="D26" t="n">
-        <v>0.0158291071154141</v>
+        <v>0.0345684766565681</v>
       </c>
       <c r="E26" t="n">
-        <v>-0.09902542084100049</v>
+        <v>-0.0985515094084201</v>
       </c>
       <c r="F26" t="n">
-        <v>-0.2737460858100313</v>
+        <v>-0.2795629124743048</v>
       </c>
       <c r="G26" t="n">
-        <v>-0.2346304019624492</v>
+        <v>-0.2498299794636231</v>
       </c>
       <c r="H26" t="n">
-        <v>-0.2228138798817408</v>
+        <v>-0.2433230851322475</v>
       </c>
       <c r="I26" t="n">
-        <v>59.6597812879708</v>
+        <v>60.82595870206488</v>
       </c>
       <c r="J26" t="n">
         <v>60</v>
@@ -2367,7 +2367,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M26" t="n">
@@ -2377,10 +2377,10 @@
         <v>60</v>
       </c>
       <c r="O26" t="n">
-        <v>10.63829787234042</v>
+        <v>6.382978723404255</v>
       </c>
       <c r="P26" t="n">
-        <v>46.74365957446808</v>
+        <v>45.89259574468085</v>
       </c>
       <c r="Q26" t="b">
         <v>0</v>
@@ -2404,48 +2404,48 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>5399.4</v>
+        <v>5475</v>
       </c>
       <c r="D27" t="n">
-        <v>0.1014687882496938</v>
+        <v>0.080307813733228</v>
       </c>
       <c r="E27" t="n">
-        <v>-0.0341829889991951</v>
+        <v>0.0004568296025582</v>
       </c>
       <c r="F27" t="n">
-        <v>0.263076635164218</v>
+        <v>0.1908905033279679</v>
       </c>
       <c r="G27" t="n">
-        <v>0.3021923190118001</v>
+        <v>0.2206234363386496</v>
       </c>
       <c r="H27" t="n">
-        <v>0.3140088410925085</v>
+        <v>0.2271303306700253</v>
       </c>
       <c r="I27" t="n">
-        <v>57.21931288484777</v>
+        <v>59.00292284784646</v>
       </c>
       <c r="J27" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K27" t="n">
         <v>57.69</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M27" t="n">
         <v>57.69</v>
       </c>
       <c r="N27" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O27" t="n">
-        <v>85.1063829787234</v>
+        <v>82.97872340425532</v>
       </c>
       <c r="P27" t="n">
-        <v>64.09727659574469</v>
+        <v>71.67174468085106</v>
       </c>
       <c r="Q27" t="b">
         <v>0</v>
@@ -2469,48 +2469,48 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1847.8</v>
+        <v>1779.3</v>
       </c>
       <c r="D28" t="n">
-        <v>0.2722390526025886</v>
+        <v>0.139043595160361</v>
       </c>
       <c r="E28" t="n">
-        <v>0.2227368978295394</v>
+        <v>0.187228931740842</v>
       </c>
       <c r="F28" t="n">
-        <v>0.6757050875124693</v>
+        <v>0.5124957497449845</v>
       </c>
       <c r="G28" t="n">
-        <v>0.7148207713600514</v>
+        <v>0.5422286827556662</v>
       </c>
       <c r="H28" t="n">
-        <v>0.7266372934407598</v>
+        <v>0.5487355770870418</v>
       </c>
       <c r="I28" t="n">
-        <v>73.27389591540536</v>
+        <v>64.161220043573</v>
       </c>
       <c r="J28" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K28" t="n">
         <v>54.51</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M28" t="n">
         <v>54.51</v>
       </c>
       <c r="N28" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O28" t="n">
-        <v>100</v>
+        <v>97.87234042553192</v>
       </c>
       <c r="P28" t="n">
-        <v>69.804</v>
+        <v>73.37846808510639</v>
       </c>
       <c r="Q28" t="b">
         <v>0</v>
@@ -2534,54 +2534,54 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>509.25</v>
+        <v>515.05</v>
       </c>
       <c r="D29" t="n">
-        <v>0.0585117439201827</v>
+        <v>0.0525186471850411</v>
       </c>
       <c r="E29" t="n">
-        <v>-0.1216041397153945</v>
+        <v>-0.1042608695652175</v>
       </c>
       <c r="F29" t="n">
-        <v>-0.0442004504504504</v>
+        <v>-0.0363891487371376</v>
       </c>
       <c r="G29" t="n">
-        <v>-0.0050847666028682</v>
+        <v>-0.0066562157264559</v>
       </c>
       <c r="H29" t="n">
-        <v>0.0067317554778401</v>
+        <v>-0.0001493213950802</v>
       </c>
       <c r="I29" t="n">
-        <v>35.77868852459015</v>
+        <v>38.69327073552422</v>
       </c>
       <c r="J29" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="K29" t="n">
         <v>49.42</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M29" t="n">
         <v>49.42</v>
       </c>
       <c r="N29" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="O29" t="n">
         <v>57.44680851063831</v>
       </c>
       <c r="P29" t="n">
-        <v>43.25736170212766</v>
+        <v>51.25736170212766</v>
       </c>
       <c r="Q29" t="b">
         <v>0</v>
       </c>
       <c r="R29" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S29" t="b">
         <v>0</v>
@@ -2599,48 +2599,48 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>117.86</v>
+        <v>127.71</v>
       </c>
       <c r="D30" t="n">
-        <v>-0.0418665149174863</v>
+        <v>0.0056697377746279</v>
       </c>
       <c r="E30" t="n">
-        <v>-0.0577230572433642</v>
+        <v>0.0069384215091066</v>
       </c>
       <c r="F30" t="n">
-        <v>-0.0919876733436055</v>
+        <v>-0.0556089625083191</v>
       </c>
       <c r="G30" t="n">
-        <v>-0.0528719894960234</v>
+        <v>-0.0258760294976374</v>
       </c>
       <c r="H30" t="n">
-        <v>-0.041055467415315</v>
+        <v>-0.0193691351662618</v>
       </c>
       <c r="I30" t="n">
-        <v>60.19986216402481</v>
+        <v>70.28556727553382</v>
       </c>
       <c r="J30" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K30" t="n">
         <v>52.38</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M30" t="n">
         <v>52.38</v>
       </c>
       <c r="N30" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O30" t="n">
-        <v>51.06382978723404</v>
+        <v>53.19148936170212</v>
       </c>
       <c r="P30" t="n">
-        <v>63.1647659574468</v>
+        <v>59.59029787234042</v>
       </c>
       <c r="Q30" t="b">
         <v>0</v>
@@ -2664,25 +2664,25 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>38.53</v>
+        <v>39.02</v>
       </c>
       <c r="D31" t="n">
-        <v>-0.0158365261813536</v>
+        <v>0.0077479338842976</v>
       </c>
       <c r="E31" t="n">
-        <v>-0.1760051325919589</v>
+        <v>-0.1465441819772527</v>
       </c>
       <c r="F31" t="n">
-        <v>-0.1902059688944934</v>
+        <v>-0.1872526556967297</v>
       </c>
       <c r="G31" t="n">
-        <v>-0.1510902850469113</v>
+        <v>-0.157519722686048</v>
       </c>
       <c r="H31" t="n">
-        <v>-0.1392737629662029</v>
+        <v>-0.1510128283546724</v>
       </c>
       <c r="I31" t="n">
-        <v>53.64238410596029</v>
+        <v>56.46766169154233</v>
       </c>
       <c r="J31" t="n">
         <v>60</v>
@@ -2692,7 +2692,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M31" t="n">
@@ -2702,10 +2702,10 @@
         <v>60</v>
       </c>
       <c r="O31" t="n">
-        <v>25.53191489361702</v>
+        <v>21.27659574468085</v>
       </c>
       <c r="P31" t="n">
-        <v>48.70238297872341</v>
+        <v>47.85131914893617</v>
       </c>
       <c r="Q31" t="b">
         <v>0</v>
@@ -2729,25 +2729,25 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>728.1</v>
+        <v>753</v>
       </c>
       <c r="D32" t="n">
-        <v>0.1217069788938529</v>
+        <v>0.1313950867703404</v>
       </c>
       <c r="E32" t="n">
-        <v>-0.0362673726009264</v>
+        <v>0.008842443729903501</v>
       </c>
       <c r="F32" t="n">
-        <v>-0.313760603204524</v>
+        <v>-0.3045164865613744</v>
       </c>
       <c r="G32" t="n">
-        <v>-0.2746449193569419</v>
+        <v>-0.2747835535506927</v>
       </c>
       <c r="H32" t="n">
-        <v>-0.2628283972762335</v>
+        <v>-0.2682766592193171</v>
       </c>
       <c r="I32" t="n">
-        <v>59.61138098542681</v>
+        <v>63.78344741754824</v>
       </c>
       <c r="J32" t="n">
         <v>80</v>
@@ -2757,7 +2757,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M32" t="n">
@@ -2794,25 +2794,25 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>573.1</v>
+        <v>577.7</v>
       </c>
       <c r="D33" t="n">
-        <v>0.0903729071537291</v>
+        <v>0.09943857645827391</v>
       </c>
       <c r="E33" t="n">
-        <v>-0.1023572715169551</v>
+        <v>-0.0760495801679327</v>
       </c>
       <c r="F33" t="n">
-        <v>0.0587474598189545</v>
+        <v>0.0619485294117647</v>
       </c>
       <c r="G33" t="n">
-        <v>0.0978631436665367</v>
+        <v>0.0916814624224464</v>
       </c>
       <c r="H33" t="n">
-        <v>0.109679665747245</v>
+        <v>0.098188356753822</v>
       </c>
       <c r="I33" t="n">
-        <v>61.50809317015396</v>
+        <v>62.85714285714286</v>
       </c>
       <c r="J33" t="n">
         <v>80</v>
@@ -2822,7 +2822,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M33" t="n">
@@ -2832,10 +2832,10 @@
         <v>80</v>
       </c>
       <c r="O33" t="n">
-        <v>65.95744680851064</v>
+        <v>61.70212765957447</v>
       </c>
       <c r="P33" t="n">
-        <v>65.18348936170213</v>
+        <v>64.33242553191489</v>
       </c>
       <c r="Q33" t="b">
         <v>0</v>
@@ -2871,10 +2871,10 @@
         <v>-0.2401052253975846</v>
       </c>
       <c r="G34" t="n">
-        <v>-0.2009895415500024</v>
+        <v>-0.2103722923869029</v>
       </c>
       <c r="H34" t="n">
-        <v>-0.1891730194692941</v>
+        <v>-0.2038653980555272</v>
       </c>
       <c r="I34" t="n">
         <v>63.3225806451613</v>
@@ -2887,7 +2887,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M34" t="n">
@@ -2924,48 +2924,48 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>116.31</v>
+        <v>118.08</v>
       </c>
       <c r="D35" t="n">
-        <v>0.0994422913318839</v>
+        <v>0.0816158285243198</v>
       </c>
       <c r="E35" t="n">
-        <v>-0.07873267326732659</v>
+        <v>-0.0780762023735166</v>
       </c>
       <c r="F35" t="n">
-        <v>0.1137604136742314</v>
+        <v>0.1400984841170223</v>
       </c>
       <c r="G35" t="n">
-        <v>0.1528760975218135</v>
+        <v>0.169831417127704</v>
       </c>
       <c r="H35" t="n">
-        <v>0.1646926196025219</v>
+        <v>0.1763383114590796</v>
       </c>
       <c r="I35" t="n">
-        <v>61.4646626159258</v>
+        <v>63.52905569007262</v>
       </c>
       <c r="J35" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K35" t="n">
         <v>49.07</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M35" t="n">
         <v>49.07</v>
       </c>
       <c r="N35" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O35" t="n">
-        <v>78.72340425531915</v>
+        <v>76.59574468085107</v>
       </c>
       <c r="P35" t="n">
-        <v>59.37268085106383</v>
+        <v>66.94714893617021</v>
       </c>
       <c r="Q35" t="b">
         <v>0</v>
@@ -2989,48 +2989,48 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>484.4</v>
+        <v>499.65</v>
       </c>
       <c r="D36" t="n">
-        <v>0.0005163688939378</v>
+        <v>0.03974612423265</v>
       </c>
       <c r="E36" t="n">
-        <v>-0.1223842739378567</v>
+        <v>-0.1064115174818921</v>
       </c>
       <c r="F36" t="n">
-        <v>0.0594925634295713</v>
+        <v>0.0966856892010534</v>
       </c>
       <c r="G36" t="n">
-        <v>0.09860824727715339</v>
+        <v>0.1264186222117351</v>
       </c>
       <c r="H36" t="n">
-        <v>0.1104247693578618</v>
+        <v>0.1329255165431108</v>
       </c>
       <c r="I36" t="n">
-        <v>60.21052631578947</v>
+        <v>65.71428571428571</v>
       </c>
       <c r="J36" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K36" t="n">
         <v>47.8</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M36" t="n">
         <v>47.8</v>
       </c>
       <c r="N36" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O36" t="n">
-        <v>68.08510638297872</v>
+        <v>70.21276595744681</v>
       </c>
       <c r="P36" t="n">
-        <v>56.73702127659575</v>
+        <v>65.16255319148937</v>
       </c>
       <c r="Q36" t="b">
         <v>0</v>
@@ -3054,48 +3054,48 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2346.2</v>
+        <v>2340.8</v>
       </c>
       <c r="D37" t="n">
-        <v>0.1575883165581211</v>
+        <v>0.1235480464625131</v>
       </c>
       <c r="E37" t="n">
-        <v>0.2773301393728222</v>
+        <v>0.2843191045758808</v>
       </c>
       <c r="F37" t="n">
-        <v>0.5689447639427576</v>
+        <v>0.5624082232011749</v>
       </c>
       <c r="G37" t="n">
-        <v>0.6080604477903397</v>
+        <v>0.5921411562118566</v>
       </c>
       <c r="H37" t="n">
-        <v>0.6198769698710481</v>
+        <v>0.5986480505432322</v>
       </c>
       <c r="I37" t="n">
-        <v>70.82695252679936</v>
+        <v>69.86404833836862</v>
       </c>
       <c r="J37" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K37" t="n">
         <v>48.59</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M37" t="n">
         <v>48.59</v>
       </c>
       <c r="N37" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O37" t="n">
-        <v>97.87234042553192</v>
+        <v>100</v>
       </c>
       <c r="P37" t="n">
-        <v>67.0104680851064</v>
+        <v>71.43600000000001</v>
       </c>
       <c r="Q37" t="b">
         <v>0</v>
@@ -3119,48 +3119,48 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>814</v>
+        <v>847.3</v>
       </c>
       <c r="D38" t="n">
-        <v>0.0665618448637315</v>
+        <v>0.09209254366179009</v>
       </c>
       <c r="E38" t="n">
-        <v>-0.08338494454141079</v>
+        <v>-0.0254198297676558</v>
       </c>
       <c r="F38" t="n">
-        <v>-0.2510121457489878</v>
+        <v>-0.2526900687952019</v>
       </c>
       <c r="G38" t="n">
-        <v>-0.2118964619014056</v>
+        <v>-0.2229571357845202</v>
       </c>
       <c r="H38" t="n">
-        <v>-0.2000799398206972</v>
+        <v>-0.2164502414531446</v>
       </c>
       <c r="I38" t="n">
-        <v>53.93281869392865</v>
+        <v>59.55303169078587</v>
       </c>
       <c r="J38" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K38" t="n">
         <v>49.87</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M38" t="n">
         <v>49.87</v>
       </c>
       <c r="N38" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O38" t="n">
-        <v>12.76595744680851</v>
+        <v>10.63829787234042</v>
       </c>
       <c r="P38" t="n">
-        <v>46.5011914893617</v>
+        <v>54.07565957446808</v>
       </c>
       <c r="Q38" t="b">
         <v>0</v>
@@ -3184,25 +3184,25 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>3610.5</v>
+        <v>3645</v>
       </c>
       <c r="D39" t="n">
-        <v>0.227017841971113</v>
+        <v>0.2211873492361296</v>
       </c>
       <c r="E39" t="n">
-        <v>0.1632514981635413</v>
+        <v>0.1967299231728938</v>
       </c>
       <c r="F39" t="n">
-        <v>0.3884936353497672</v>
+        <v>0.400414937759336</v>
       </c>
       <c r="G39" t="n">
-        <v>0.4276093191973493</v>
+        <v>0.4301478707700177</v>
       </c>
       <c r="H39" t="n">
-        <v>0.4394258412780577</v>
+        <v>0.4366547651013933</v>
       </c>
       <c r="I39" t="n">
-        <v>79.11131470453508</v>
+        <v>79.90525504021156</v>
       </c>
       <c r="J39" t="n">
         <v>70</v>
@@ -3212,7 +3212,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M39" t="n">
@@ -3249,25 +3249,25 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>212.66</v>
+        <v>214.77</v>
       </c>
       <c r="D40" t="n">
-        <v>0.1879119651435592</v>
+        <v>0.1859848694019548</v>
       </c>
       <c r="E40" t="n">
-        <v>0.0723073820088746</v>
+        <v>0.0684543057559325</v>
       </c>
       <c r="F40" t="n">
-        <v>-0.118398142774231</v>
+        <v>-0.1079127725856697</v>
       </c>
       <c r="G40" t="n">
-        <v>-0.0792824589266488</v>
+        <v>-0.078179839574988</v>
       </c>
       <c r="H40" t="n">
-        <v>-0.06746593684594041</v>
+        <v>-0.0716729452436124</v>
       </c>
       <c r="I40" t="n">
-        <v>73.29052412356822</v>
+        <v>74.23405323957812</v>
       </c>
       <c r="J40" t="n">
         <v>70</v>
@@ -3277,7 +3277,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M40" t="n">
@@ -3314,25 +3314,25 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>791.2</v>
+        <v>807.35</v>
       </c>
       <c r="D41" t="n">
-        <v>-0.0210949582431178</v>
+        <v>-0.0206817079087821</v>
       </c>
       <c r="E41" t="n">
-        <v>-0.1422376409366867</v>
+        <v>-0.130245084837059</v>
       </c>
       <c r="F41" t="n">
-        <v>-0.2319937876140555</v>
+        <v>-0.2162411416367342</v>
       </c>
       <c r="G41" t="n">
-        <v>-0.1928781037664734</v>
+        <v>-0.1865082086260525</v>
       </c>
       <c r="H41" t="n">
-        <v>-0.181061581685765</v>
+        <v>-0.1800013142946769</v>
       </c>
       <c r="I41" t="n">
-        <v>47.46093750000001</v>
+        <v>52.45949926362298</v>
       </c>
       <c r="J41" t="n">
         <v>60</v>
@@ -3342,7 +3342,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M41" t="n">
@@ -3379,25 +3379,25 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>614.2</v>
+        <v>626.25</v>
       </c>
       <c r="D42" t="n">
-        <v>0.118353969410051</v>
+        <v>0.1777150916784202</v>
       </c>
       <c r="E42" t="n">
-        <v>-0.0389610389610389</v>
+        <v>-0.0336393796774939</v>
       </c>
       <c r="F42" t="n">
-        <v>-0.2104891059836749</v>
+        <v>-0.1942228512609367</v>
       </c>
       <c r="G42" t="n">
-        <v>-0.1713734221360928</v>
+        <v>-0.164489918250255</v>
       </c>
       <c r="H42" t="n">
-        <v>-0.1595569000553844</v>
+        <v>-0.1579830239188794</v>
       </c>
       <c r="I42" t="n">
-        <v>67.7264547090582</v>
+        <v>69.21022510492179</v>
       </c>
       <c r="J42" t="n">
         <v>80</v>
@@ -3407,7 +3407,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M42" t="n">
@@ -3444,48 +3444,48 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>411.6</v>
+        <v>415.75</v>
       </c>
       <c r="D43" t="n">
-        <v>0.008329250367466999</v>
+        <v>0.0340753637607262</v>
       </c>
       <c r="E43" t="n">
-        <v>-0.1051201217523642</v>
+        <v>-0.0941279006427715</v>
       </c>
       <c r="F43" t="n">
-        <v>-0.1129310344827585</v>
+        <v>-0.1584008097165992</v>
       </c>
       <c r="G43" t="n">
-        <v>-0.0738153506351764</v>
+        <v>-0.1286678767059175</v>
       </c>
       <c r="H43" t="n">
-        <v>-0.061998828554468</v>
+        <v>-0.1221609823745418</v>
       </c>
       <c r="I43" t="n">
-        <v>50.57071960297768</v>
+        <v>52.52621544327933</v>
       </c>
       <c r="J43" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K43" t="n">
         <v>51.48</v>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M43" t="n">
         <v>51.48</v>
       </c>
       <c r="N43" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O43" t="n">
-        <v>46.80851063829788</v>
+        <v>31.91489361702128</v>
       </c>
       <c r="P43" t="n">
-        <v>45.95370212765958</v>
+        <v>50.97497872340426</v>
       </c>
       <c r="Q43" t="b">
         <v>0</v>
@@ -3509,25 +3509,25 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>265.8</v>
+        <v>266.71</v>
       </c>
       <c r="D44" t="n">
-        <v>0.1165721487082545</v>
+        <v>0.1354193273733501</v>
       </c>
       <c r="E44" t="n">
-        <v>0.0009414422895877</v>
+        <v>0.0015396169733381</v>
       </c>
       <c r="F44" t="n">
-        <v>-0.1326480665687713</v>
+        <v>-0.141583521081429</v>
       </c>
       <c r="G44" t="n">
-        <v>-0.0935323827211892</v>
+        <v>-0.1118505880707473</v>
       </c>
       <c r="H44" t="n">
-        <v>-0.08171586064048079</v>
+        <v>-0.1053436937393716</v>
       </c>
       <c r="I44" t="n">
-        <v>82.47223563495898</v>
+        <v>82.84904323175053</v>
       </c>
       <c r="J44" t="n">
         <v>60</v>
@@ -3537,7 +3537,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M44" t="n">
@@ -3547,10 +3547,10 @@
         <v>60</v>
       </c>
       <c r="O44" t="n">
-        <v>38.29787234042553</v>
+        <v>40.42553191489361</v>
       </c>
       <c r="P44" t="n">
-        <v>50.53957446808511</v>
+        <v>50.96510638297872</v>
       </c>
       <c r="Q44" t="b">
         <v>0</v>
@@ -3574,25 +3574,25 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>98</v>
+        <v>99.70999999999999</v>
       </c>
       <c r="D45" t="n">
-        <v>0.0072977695549387</v>
+        <v>0.0136220392396053</v>
       </c>
       <c r="E45" t="n">
-        <v>-0.1000918273645546</v>
+        <v>-0.0725513905683192</v>
       </c>
       <c r="F45" t="n">
-        <v>-0.2947103274559193</v>
+        <v>-0.3025809610407778</v>
       </c>
       <c r="G45" t="n">
-        <v>-0.2555946436083371</v>
+        <v>-0.2728480280300961</v>
       </c>
       <c r="H45" t="n">
-        <v>-0.2437781215276288</v>
+        <v>-0.2663411336987205</v>
       </c>
       <c r="I45" t="n">
-        <v>58.16767502160761</v>
+        <v>60.13179571663922</v>
       </c>
       <c r="J45" t="n">
         <v>60</v>
@@ -3602,7 +3602,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M45" t="n">
@@ -3612,10 +3612,10 @@
         <v>60</v>
       </c>
       <c r="O45" t="n">
-        <v>6.382978723404255</v>
+        <v>4.25531914893617</v>
       </c>
       <c r="P45" t="n">
-        <v>49.11659574468086</v>
+        <v>48.69106382978724</v>
       </c>
       <c r="Q45" t="b">
         <v>0</v>
@@ -3639,48 +3639,48 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>518.35</v>
+        <v>539.55</v>
       </c>
       <c r="D46" t="n">
-        <v>0.0824892972747206</v>
+        <v>0.09165402124430951</v>
       </c>
       <c r="E46" t="n">
-        <v>-0.0935560024481944</v>
+        <v>-0.0423322683706071</v>
       </c>
       <c r="F46" t="n">
-        <v>-0.1902679059595406</v>
+        <v>-0.1545753682231276</v>
       </c>
       <c r="G46" t="n">
-        <v>-0.1511522221119585</v>
+        <v>-0.1248424352124459</v>
       </c>
       <c r="H46" t="n">
-        <v>-0.1393357000312501</v>
+        <v>-0.1183355408810703</v>
       </c>
       <c r="I46" t="n">
-        <v>59.74228816868411</v>
+        <v>65.46063651591288</v>
       </c>
       <c r="J46" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K46" t="n">
         <v>49.61</v>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M46" t="n">
         <v>49.61</v>
       </c>
       <c r="N46" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O46" t="n">
-        <v>23.40425531914894</v>
+        <v>34.04255319148936</v>
       </c>
       <c r="P46" t="n">
-        <v>48.52485106382979</v>
+        <v>58.65251063829788</v>
       </c>
       <c r="Q46" t="b">
         <v>0</v>
@@ -3704,48 +3704,48 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>1022.05</v>
+        <v>1032.65</v>
       </c>
       <c r="D47" t="n">
-        <v>0.1107428136716839</v>
+        <v>0.0824990827611511</v>
       </c>
       <c r="E47" t="n">
-        <v>0.2711274174491636</v>
+        <v>0.2714232947549864</v>
       </c>
       <c r="F47" t="n">
-        <v>0.2812460824871503</v>
+        <v>0.2762157819934501</v>
       </c>
       <c r="G47" t="n">
-        <v>0.3203617663347324</v>
+        <v>0.3059487150041318</v>
       </c>
       <c r="H47" t="n">
-        <v>0.3321782884154408</v>
+        <v>0.3124556093355074</v>
       </c>
       <c r="I47" t="n">
-        <v>37.83345349675558</v>
+        <v>40.1215277777778</v>
       </c>
       <c r="J47" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K47" t="n">
         <v>46.83</v>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M47" t="n">
         <v>46.83</v>
       </c>
       <c r="N47" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O47" t="n">
         <v>87.2340425531915</v>
       </c>
       <c r="P47" t="n">
-        <v>64.17880851063831</v>
+        <v>68.17880851063831</v>
       </c>
       <c r="Q47" t="b">
         <v>0</v>
@@ -3769,25 +3769,25 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>14069</v>
+        <v>14010</v>
       </c>
       <c r="D48" t="n">
-        <v>0.0291880029261155</v>
+        <v>0.0301470588235293</v>
       </c>
       <c r="E48" t="n">
-        <v>0.0075914917997566</v>
+        <v>-0.0087030354489492</v>
       </c>
       <c r="F48" t="n">
-        <v>0.0554388597149286</v>
+        <v>0.0777752134779599</v>
       </c>
       <c r="G48" t="n">
-        <v>0.09455454356251081</v>
+        <v>0.1075081464886416</v>
       </c>
       <c r="H48" t="n">
-        <v>0.1063710656432191</v>
+        <v>0.1140150408200172</v>
       </c>
       <c r="I48" t="n">
-        <v>58.22130299896587</v>
+        <v>57.06081081081081</v>
       </c>
       <c r="J48" t="n">
         <v>60</v>
@@ -3797,7 +3797,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M48" t="n">
@@ -3936,57 +3936,57 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>LUMAXTECH</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Forgings</t>
+          <t>Lighting</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1801.3</v>
+        <v>1779.3</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0614614024749557</v>
+        <v>0.139043595160361</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2366469861320885</v>
+        <v>0.187228931740842</v>
       </c>
       <c r="F2" t="n">
-        <v>0.4341560509554139</v>
+        <v>0.5124957497449845</v>
       </c>
       <c r="G2" t="n">
-        <v>0.473271734802996</v>
+        <v>0.5422286827556662</v>
       </c>
       <c r="H2" t="n">
-        <v>0.4850882568837044</v>
+        <v>0.5487355770870418</v>
       </c>
       <c r="I2" t="n">
-        <v>59.62566844919785</v>
+        <v>64.161220043573</v>
       </c>
       <c r="J2" t="n">
         <v>80</v>
       </c>
       <c r="K2" t="n">
-        <v>54.83</v>
+        <v>54.51</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M2" t="n">
-        <v>54.83</v>
+        <v>54.51</v>
       </c>
       <c r="N2" t="n">
         <v>80</v>
       </c>
       <c r="O2" t="n">
-        <v>95.74468085106383</v>
+        <v>97.87234042553192</v>
       </c>
       <c r="P2" t="n">
-        <v>73.08093617021277</v>
+        <v>73.37846808510639</v>
       </c>
       <c r="Q2" t="b">
         <v>0</v>
@@ -4001,57 +4001,57 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GNA</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Axles</t>
+          <t>Forgings</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>440.1</v>
+        <v>1831.6</v>
       </c>
       <c r="D3" t="n">
-        <v>0.1469898358092261</v>
+        <v>0.0490263459335624</v>
       </c>
       <c r="E3" t="n">
-        <v>0.2606702950443997</v>
+        <v>0.2542628227076628</v>
       </c>
       <c r="F3" t="n">
-        <v>0.3791914760263239</v>
+        <v>0.4641087130295762</v>
       </c>
       <c r="G3" t="n">
-        <v>0.4183071598739061</v>
+        <v>0.4938416460402579</v>
       </c>
       <c r="H3" t="n">
-        <v>0.4301236819546145</v>
+        <v>0.5003485403716336</v>
       </c>
       <c r="I3" t="n">
-        <v>65.00512120177535</v>
+        <v>62.95993458708093</v>
       </c>
       <c r="J3" t="n">
         <v>80</v>
       </c>
       <c r="K3" t="n">
-        <v>54.47</v>
+        <v>54.83</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M3" t="n">
-        <v>54.47</v>
+        <v>54.83</v>
       </c>
       <c r="N3" t="n">
         <v>80</v>
       </c>
       <c r="O3" t="n">
-        <v>91.48936170212764</v>
+        <v>95.74468085106383</v>
       </c>
       <c r="P3" t="n">
-        <v>72.08587234042552</v>
+        <v>73.08093617021277</v>
       </c>
       <c r="Q3" t="b">
         <v>0</v>
@@ -4066,7 +4066,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>LUMAXTECH</t>
+          <t>LUMAXIND</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -4075,48 +4075,48 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1847.8</v>
+        <v>5475</v>
       </c>
       <c r="D4" t="n">
-        <v>0.2722390526025886</v>
+        <v>0.080307813733228</v>
       </c>
       <c r="E4" t="n">
-        <v>0.2227368978295394</v>
+        <v>0.0004568296025582</v>
       </c>
       <c r="F4" t="n">
-        <v>0.6757050875124693</v>
+        <v>0.1908905033279679</v>
       </c>
       <c r="G4" t="n">
-        <v>0.7148207713600514</v>
+        <v>0.2206234363386496</v>
       </c>
       <c r="H4" t="n">
-        <v>0.7266372934407598</v>
+        <v>0.2271303306700253</v>
       </c>
       <c r="I4" t="n">
-        <v>73.27389591540536</v>
+        <v>59.00292284784646</v>
       </c>
       <c r="J4" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K4" t="n">
-        <v>54.51</v>
+        <v>57.69</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M4" t="n">
-        <v>54.51</v>
+        <v>57.69</v>
       </c>
       <c r="N4" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O4" t="n">
-        <v>100</v>
+        <v>82.97872340425532</v>
       </c>
       <c r="P4" t="n">
-        <v>69.804</v>
+        <v>71.67174468085106</v>
       </c>
       <c r="Q4" t="b">
         <v>0</v>
@@ -4131,57 +4131,57 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BHARATGEAR</t>
+          <t>GNA</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Gears</t>
+          <t>Axles</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>105.26</v>
+        <v>443.7</v>
       </c>
       <c r="D5" t="n">
-        <v>0.1094013490725127</v>
+        <v>0.136381098732232</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.0207461159177596</v>
+        <v>0.2630230572160545</v>
       </c>
       <c r="F5" t="n">
-        <v>0.1872321227159938</v>
+        <v>0.3515077672860187</v>
       </c>
       <c r="G5" t="n">
-        <v>0.226347806563576</v>
+        <v>0.3812407002967004</v>
       </c>
       <c r="H5" t="n">
-        <v>0.2381643286442843</v>
+        <v>0.387747594628076</v>
       </c>
       <c r="I5" t="n">
-        <v>65.97524255603882</v>
+        <v>65.84471842719094</v>
       </c>
       <c r="J5" t="n">
         <v>80</v>
       </c>
       <c r="K5" t="n">
-        <v>51.91</v>
+        <v>54.47</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M5" t="n">
-        <v>51.91</v>
+        <v>54.47</v>
       </c>
       <c r="N5" t="n">
         <v>80</v>
       </c>
       <c r="O5" t="n">
-        <v>82.97872340425532</v>
+        <v>89.36170212765957</v>
       </c>
       <c r="P5" t="n">
-        <v>69.35974468085107</v>
+        <v>71.66034042553191</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
@@ -4196,57 +4196,57 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CRAFTSMAN</t>
+          <t>SANSERA</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Castings</t>
+          <t>Forgings</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>7398.5</v>
+        <v>2340.8</v>
       </c>
       <c r="D6" t="n">
-        <v>0.0892160471107839</v>
+        <v>0.1235480464625131</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.0129410979921286</v>
+        <v>0.2843191045758808</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0917877960599129</v>
+        <v>0.5624082232011749</v>
       </c>
       <c r="G6" t="n">
-        <v>0.130903479907495</v>
+        <v>0.5921411562118566</v>
       </c>
       <c r="H6" t="n">
-        <v>0.1427200019882034</v>
+        <v>0.5986480505432322</v>
       </c>
       <c r="I6" t="n">
-        <v>65.49889135254989</v>
+        <v>69.86404833836862</v>
       </c>
       <c r="J6" t="n">
         <v>80</v>
       </c>
       <c r="K6" t="n">
-        <v>54.65</v>
+        <v>48.59</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M6" t="n">
-        <v>54.65</v>
+        <v>48.59</v>
       </c>
       <c r="N6" t="n">
         <v>80</v>
       </c>
       <c r="O6" t="n">
-        <v>76.59574468085107</v>
+        <v>100</v>
       </c>
       <c r="P6" t="n">
-        <v>69.17914893617021</v>
+        <v>71.43600000000001</v>
       </c>
       <c r="Q6" t="b">
         <v>0</v>
@@ -4261,57 +4261,57 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BHARATSE</t>
+          <t>WHEELS</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Seating</t>
+          <t>Wheels</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>174.84</v>
+        <v>1032.65</v>
       </c>
       <c r="D7" t="n">
-        <v>0.0900928985597606</v>
+        <v>0.0824990827611511</v>
       </c>
       <c r="E7" t="n">
-        <v>0.0945971326613661</v>
+        <v>0.2714232947549864</v>
       </c>
       <c r="F7" t="n">
-        <v>0.08717821166521569</v>
+        <v>0.2762157819934501</v>
       </c>
       <c r="G7" t="n">
-        <v>0.1262938955127979</v>
+        <v>0.3059487150041318</v>
       </c>
       <c r="H7" t="n">
-        <v>0.1381104175935062</v>
+        <v>0.3124556093355074</v>
       </c>
       <c r="I7" t="n">
-        <v>64.33915211970074</v>
+        <v>40.1215277777778</v>
       </c>
       <c r="J7" t="n">
         <v>80</v>
       </c>
       <c r="K7" t="n">
-        <v>52.61</v>
+        <v>46.83</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M7" t="n">
-        <v>52.61</v>
+        <v>46.83</v>
       </c>
       <c r="N7" t="n">
         <v>80</v>
       </c>
       <c r="O7" t="n">
-        <v>74.46808510638297</v>
+        <v>87.2340425531915</v>
       </c>
       <c r="P7" t="n">
-        <v>67.93761702127659</v>
+        <v>68.17880851063831</v>
       </c>
       <c r="Q7" t="b">
         <v>0</v>
@@ -4326,57 +4326,57 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SANSERA</t>
+          <t>DIVGIITTS</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Forgings</t>
+          <t>Transmission</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>2346.2</v>
+        <v>777.75</v>
       </c>
       <c r="D8" t="n">
-        <v>0.1575883165581211</v>
+        <v>0.1547884187082404</v>
       </c>
       <c r="E8" t="n">
-        <v>0.2773301393728222</v>
+        <v>0.3238297872340425</v>
       </c>
       <c r="F8" t="n">
-        <v>0.5689447639427576</v>
+        <v>0.1768933948702429</v>
       </c>
       <c r="G8" t="n">
-        <v>0.6080604477903397</v>
+        <v>0.2066263278809246</v>
       </c>
       <c r="H8" t="n">
-        <v>0.6198769698710481</v>
+        <v>0.2131332222123002</v>
       </c>
       <c r="I8" t="n">
-        <v>70.82695252679936</v>
+        <v>65.57153965785382</v>
       </c>
       <c r="J8" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K8" t="n">
-        <v>48.59</v>
+        <v>49.92</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M8" t="n">
-        <v>48.59</v>
+        <v>49.92</v>
       </c>
       <c r="N8" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O8" t="n">
-        <v>97.87234042553192</v>
+        <v>80.85106382978722</v>
       </c>
       <c r="P8" t="n">
-        <v>67.0104680851064</v>
+        <v>68.13821276595745</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
@@ -4391,57 +4391,57 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SHRIPISTON</t>
+          <t>MOTHERSON</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Engine/Parts</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>3610.5</v>
+        <v>123.55</v>
       </c>
       <c r="D9" t="n">
-        <v>0.227017841971113</v>
+        <v>0.0666493999827333</v>
       </c>
       <c r="E9" t="n">
-        <v>0.1632514981635413</v>
+        <v>0.0750021752371008</v>
       </c>
       <c r="F9" t="n">
-        <v>0.3884936353497672</v>
+        <v>0.1023376159885796</v>
       </c>
       <c r="G9" t="n">
-        <v>0.4276093191973493</v>
+        <v>0.1320705489992613</v>
       </c>
       <c r="H9" t="n">
-        <v>0.4394258412780577</v>
+        <v>0.1385774433306369</v>
       </c>
       <c r="I9" t="n">
-        <v>79.11131470453508</v>
+        <v>64.21167484997272</v>
       </c>
       <c r="J9" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K9" t="n">
-        <v>48.69</v>
+        <v>51.57</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M9" t="n">
-        <v>48.69</v>
+        <v>51.57</v>
       </c>
       <c r="N9" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O9" t="n">
-        <v>93.61702127659576</v>
+        <v>72.3404255319149</v>
       </c>
       <c r="P9" t="n">
-        <v>66.19940425531915</v>
+        <v>67.09608510638299</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -4456,57 +4456,57 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>FIEMIND</t>
+          <t>CRAFTSMAN</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Lighting</t>
+          <t>Castings</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>2164.9</v>
+        <v>7433.5</v>
       </c>
       <c r="D10" t="n">
-        <v>0.0797506234413965</v>
+        <v>0.07467110018794269</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.0255660080118826</v>
+        <v>-0.0329148507122877</v>
       </c>
       <c r="F10" t="n">
-        <v>0.08543494610178</v>
+        <v>0.0924388272466749</v>
       </c>
       <c r="G10" t="n">
-        <v>0.1245506299493621</v>
+        <v>0.1221717602573566</v>
       </c>
       <c r="H10" t="n">
-        <v>0.1363671520300705</v>
+        <v>0.1286786545887323</v>
       </c>
       <c r="I10" t="n">
-        <v>57.57971284728698</v>
+        <v>66.53763440860214</v>
       </c>
       <c r="J10" t="n">
         <v>80</v>
       </c>
       <c r="K10" t="n">
-        <v>49.06</v>
+        <v>54.65</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M10" t="n">
-        <v>49.06</v>
+        <v>54.65</v>
       </c>
       <c r="N10" t="n">
         <v>80</v>
       </c>
       <c r="O10" t="n">
-        <v>72.3404255319149</v>
+        <v>65.95744680851064</v>
       </c>
       <c r="P10" t="n">
-        <v>66.09208510638298</v>
+        <v>67.05148936170212</v>
       </c>
       <c r="Q10" t="b">
         <v>0</v>
@@ -4521,57 +4521,57 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>RICOAUTO</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Castings</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>569.3</v>
+        <v>118.08</v>
       </c>
       <c r="D11" t="n">
-        <v>0.1637367130008176</v>
+        <v>0.0816158285243198</v>
       </c>
       <c r="E11" t="n">
-        <v>0.2461420597570316</v>
+        <v>-0.0780762023735166</v>
       </c>
       <c r="F11" t="n">
-        <v>0.3535425582501186</v>
+        <v>0.1400984841170223</v>
       </c>
       <c r="G11" t="n">
-        <v>0.3926582420977007</v>
+        <v>0.169831417127704</v>
       </c>
       <c r="H11" t="n">
-        <v>0.4044747641784091</v>
+        <v>0.1763383114590796</v>
       </c>
       <c r="I11" t="n">
-        <v>70.59451762192948</v>
+        <v>63.52905569007262</v>
       </c>
       <c r="J11" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K11" t="n">
-        <v>49.66</v>
+        <v>49.07</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M11" t="n">
-        <v>49.66</v>
+        <v>49.07</v>
       </c>
       <c r="N11" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O11" t="n">
-        <v>89.36170212765957</v>
+        <v>76.59574468085107</v>
       </c>
       <c r="P11" t="n">
-        <v>65.73634042553192</v>
+        <v>66.94714893617021</v>
       </c>
       <c r="Q11" t="b">
         <v>0</v>
@@ -4586,57 +4586,57 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>PRICOLLTD</t>
+          <t>BHARATSE</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Seating</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>573.1</v>
+        <v>184.81</v>
       </c>
       <c r="D12" t="n">
-        <v>0.0903729071537291</v>
+        <v>0.1359641035097425</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.1023572715169551</v>
+        <v>0.140098704503393</v>
       </c>
       <c r="F12" t="n">
-        <v>0.0587474598189545</v>
+        <v>0.0944569465829681</v>
       </c>
       <c r="G12" t="n">
-        <v>0.0978631436665367</v>
+        <v>0.1241898795936498</v>
       </c>
       <c r="H12" t="n">
-        <v>0.109679665747245</v>
+        <v>0.1306967739250254</v>
       </c>
       <c r="I12" t="n">
-        <v>61.50809317015396</v>
+        <v>69.71713810316139</v>
       </c>
       <c r="J12" t="n">
         <v>80</v>
       </c>
       <c r="K12" t="n">
-        <v>49.98</v>
+        <v>52.61</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M12" t="n">
-        <v>49.98</v>
+        <v>52.61</v>
       </c>
       <c r="N12" t="n">
         <v>80</v>
       </c>
       <c r="O12" t="n">
-        <v>65.95744680851064</v>
+        <v>68.08510638297872</v>
       </c>
       <c r="P12" t="n">
-        <v>65.18348936170213</v>
+        <v>66.66102127659575</v>
       </c>
       <c r="Q12" t="b">
         <v>0</v>
@@ -4651,57 +4651,57 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>DIVGIITTS</t>
+          <t>FIEMIND</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Transmission</t>
+          <t>Lighting</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>689.2</v>
+        <v>2241.3</v>
       </c>
       <c r="D13" t="n">
-        <v>0.0470186099506266</v>
+        <v>0.1188598242811502</v>
       </c>
       <c r="E13" t="n">
-        <v>0.1804401815534813</v>
+        <v>-0.0063838276366536</v>
       </c>
       <c r="F13" t="n">
-        <v>0.0355345203215387</v>
+        <v>0.1097742127153893</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0746502041691208</v>
+        <v>0.139507145726071</v>
       </c>
       <c r="H13" t="n">
-        <v>0.08646672624982921</v>
+        <v>0.1460140400574466</v>
       </c>
       <c r="I13" t="n">
-        <v>47.49481174029056</v>
+        <v>62.86926717806433</v>
       </c>
       <c r="J13" t="n">
         <v>80</v>
       </c>
       <c r="K13" t="n">
-        <v>49.92</v>
+        <v>49.06</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M13" t="n">
-        <v>49.92</v>
+        <v>49.06</v>
       </c>
       <c r="N13" t="n">
         <v>80</v>
       </c>
       <c r="O13" t="n">
-        <v>61.70212765957447</v>
+        <v>74.46808510638297</v>
       </c>
       <c r="P13" t="n">
-        <v>64.30842553191489</v>
+        <v>66.51761702127659</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
@@ -4716,57 +4716,57 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>WHEELS</t>
+          <t>SHRIPISTON</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Wheels</t>
+          <t>Engine/Parts</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1022.05</v>
+        <v>3645</v>
       </c>
       <c r="D14" t="n">
-        <v>0.1107428136716839</v>
+        <v>0.2211873492361296</v>
       </c>
       <c r="E14" t="n">
-        <v>0.2711274174491636</v>
+        <v>0.1967299231728938</v>
       </c>
       <c r="F14" t="n">
-        <v>0.2812460824871503</v>
+        <v>0.400414937759336</v>
       </c>
       <c r="G14" t="n">
-        <v>0.3203617663347324</v>
+        <v>0.4301478707700177</v>
       </c>
       <c r="H14" t="n">
-        <v>0.3321782884154408</v>
+        <v>0.4366547651013933</v>
       </c>
       <c r="I14" t="n">
-        <v>37.83345349675558</v>
+        <v>79.90525504021156</v>
       </c>
       <c r="J14" t="n">
         <v>70</v>
       </c>
       <c r="K14" t="n">
-        <v>46.83</v>
+        <v>48.69</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M14" t="n">
-        <v>46.83</v>
+        <v>48.69</v>
       </c>
       <c r="N14" t="n">
         <v>70</v>
       </c>
       <c r="O14" t="n">
-        <v>87.2340425531915</v>
+        <v>93.61702127659576</v>
       </c>
       <c r="P14" t="n">
-        <v>64.17880851063831</v>
+        <v>66.19940425531915</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
@@ -4781,57 +4781,57 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>LUMAXIND</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Lighting</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>5399.4</v>
+        <v>585.7</v>
       </c>
       <c r="D15" t="n">
-        <v>0.1014687882496938</v>
+        <v>0.1665006970722964</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.0341829889991951</v>
+        <v>0.2814790504321192</v>
       </c>
       <c r="F15" t="n">
-        <v>0.263076635164218</v>
+        <v>0.390055773110241</v>
       </c>
       <c r="G15" t="n">
-        <v>0.3021923190118001</v>
+        <v>0.4197887061209226</v>
       </c>
       <c r="H15" t="n">
-        <v>0.3140088410925085</v>
+        <v>0.4262956004522983</v>
       </c>
       <c r="I15" t="n">
-        <v>57.21931288484777</v>
+        <v>73.66911061523747</v>
       </c>
       <c r="J15" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K15" t="n">
-        <v>57.69</v>
+        <v>49.66</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M15" t="n">
-        <v>57.69</v>
+        <v>49.66</v>
       </c>
       <c r="N15" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O15" t="n">
-        <v>85.1063829787234</v>
+        <v>91.48936170212764</v>
       </c>
       <c r="P15" t="n">
-        <v>64.09727659574469</v>
+        <v>66.16187234042553</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
@@ -4846,63 +4846,63 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ASKAUTOLTD</t>
+          <t>BHARATGEAR</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Gears</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>435.5</v>
+        <v>111.65</v>
       </c>
       <c r="D16" t="n">
-        <v>0.0671404067630481</v>
+        <v>0.1548407116259826</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.0592936602224861</v>
+        <v>0.0538984330753258</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.1535471331389698</v>
+        <v>0.2647258722247394</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.1144314492913877</v>
+        <v>0.2944588052354211</v>
       </c>
       <c r="H16" t="n">
-        <v>-0.1026149272106793</v>
+        <v>0.3009656995667967</v>
       </c>
       <c r="I16" t="n">
-        <v>39.20099875156056</v>
+        <v>71.96802646085999</v>
       </c>
       <c r="J16" t="n">
         <v>70</v>
       </c>
       <c r="K16" t="n">
-        <v>71.28</v>
+        <v>51.91</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="M16" t="n">
-        <v>71.28</v>
+        <v>51.91</v>
       </c>
       <c r="N16" t="n">
         <v>70</v>
       </c>
       <c r="O16" t="n">
-        <v>36.17021276595745</v>
+        <v>85.1063829787234</v>
       </c>
       <c r="P16" t="n">
-        <v>63.74604255319149</v>
+        <v>65.78527659574468</v>
       </c>
       <c r="Q16" t="b">
+        <v>0</v>
+      </c>
+      <c r="R16" t="b">
         <v>1</v>
-      </c>
-      <c r="R16" t="b">
-        <v>0</v>
       </c>
       <c r="S16" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
chore: auto-refresh NSE data and pipeline outputs (2026-04-16)
</commit_message>
<xml_diff>
--- a/working-sector/output/auto_components_comprehensive_report.xlsx
+++ b/working-sector/output/auto_components_comprehensive_report.xlsx
@@ -435,7 +435,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
     </row>
@@ -791,10 +791,10 @@
         <v>0.4641087130295762</v>
       </c>
       <c r="G2" t="n">
-        <v>0.4938416460402579</v>
+        <v>0.49874546802009</v>
       </c>
       <c r="H2" t="n">
-        <v>0.5003485403716336</v>
+        <v>0.5007855984281281</v>
       </c>
       <c r="I2" t="n">
         <v>62.95993458708093</v>
@@ -856,10 +856,10 @@
         <v>-0.164755903120492</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.1350229701098103</v>
+        <v>-0.1301191481299782</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.1285160757784347</v>
+        <v>-0.1280790177219402</v>
       </c>
       <c r="I3" t="n">
         <v>52.18760938046901</v>
@@ -921,10 +921,10 @@
         <v>-0.0586443259710586</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.0289113929603769</v>
+        <v>-0.0240075709805448</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.0224044986290012</v>
+        <v>-0.0219674405725067</v>
       </c>
       <c r="I4" t="n">
         <v>79.23951048951048</v>
@@ -986,10 +986,10 @@
         <v>-0.1816491010539367</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.151916168043255</v>
+        <v>-0.1470123460634229</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.1454092737118794</v>
+        <v>-0.1449722156553848</v>
       </c>
       <c r="I5" t="n">
         <v>65.79129232895647</v>
@@ -1051,10 +1051,10 @@
         <v>0.1023376159885796</v>
       </c>
       <c r="G6" t="n">
-        <v>0.1320705489992613</v>
+        <v>0.1369743709790933</v>
       </c>
       <c r="H6" t="n">
-        <v>0.1385774433306369</v>
+        <v>0.1390145013871314</v>
       </c>
       <c r="I6" t="n">
         <v>64.21167484997272</v>
@@ -1116,10 +1116,10 @@
         <v>-0.1659097789887981</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.1361768459781164</v>
+        <v>-0.1312730239982843</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.1296699516467407</v>
+        <v>-0.1292328935902462</v>
       </c>
       <c r="I7" t="n">
         <v>57.68742058449809</v>
@@ -1181,10 +1181,10 @@
         <v>0.390055773110241</v>
       </c>
       <c r="G8" t="n">
-        <v>0.4197887061209226</v>
+        <v>0.4246925281007547</v>
       </c>
       <c r="H8" t="n">
-        <v>0.4262956004522983</v>
+        <v>0.4267326585087928</v>
       </c>
       <c r="I8" t="n">
         <v>73.66911061523747</v>
@@ -1246,10 +1246,10 @@
         <v>-0.0970248440854718</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.0672919110747901</v>
+        <v>-0.062388089094958</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.0607850167434145</v>
+        <v>-0.06034795868692</v>
       </c>
       <c r="I9" t="n">
         <v>67.10833982852691</v>
@@ -1311,10 +1311,10 @@
         <v>-0.1156571648443262</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.0859242318336445</v>
+        <v>-0.0810204098538124</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.0794173375022688</v>
+        <v>-0.07898027944577431</v>
       </c>
       <c r="I10" t="n">
         <v>68.81822496440437</v>
@@ -1376,10 +1376,10 @@
         <v>-0.0042030657656173</v>
       </c>
       <c r="G11" t="n">
-        <v>0.0255298672450643</v>
+        <v>0.0304336892248964</v>
       </c>
       <c r="H11" t="n">
-        <v>0.0320367615764399</v>
+        <v>0.0324738196329345</v>
       </c>
       <c r="I11" t="n">
         <v>27.6054590570719</v>
@@ -1441,10 +1441,10 @@
         <v>-0.1780578898225957</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.148324956811914</v>
+        <v>-0.1434211348320819</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.1418180624805384</v>
+        <v>-0.1413810044240439</v>
       </c>
       <c r="I12" t="n">
         <v>45.52572706935123</v>
@@ -1506,10 +1506,10 @@
         <v>-0.0475350170949597</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.017802084084278</v>
+        <v>-0.012898262104446</v>
       </c>
       <c r="H13" t="n">
-        <v>-0.0112951897529024</v>
+        <v>-0.0108581316964079</v>
       </c>
       <c r="I13" t="n">
         <v>59.67254408060453</v>
@@ -1571,10 +1571,10 @@
         <v>-0.2676972150656361</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.2379642820549544</v>
+        <v>-0.2330604600751223</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.2314573877235788</v>
+        <v>-0.2310203296670843</v>
       </c>
       <c r="I14" t="n">
         <v>58.03869246164109</v>
@@ -1636,10 +1636,10 @@
         <v>0.2647258722247394</v>
       </c>
       <c r="G15" t="n">
-        <v>0.2944588052354211</v>
+        <v>0.2993626272152532</v>
       </c>
       <c r="H15" t="n">
-        <v>0.3009656995667967</v>
+        <v>0.3014027576232913</v>
       </c>
       <c r="I15" t="n">
         <v>71.96802646085999</v>
@@ -1701,10 +1701,10 @@
         <v>0.0944569465829681</v>
       </c>
       <c r="G16" t="n">
-        <v>0.1241898795936498</v>
+        <v>0.1290937015734818</v>
       </c>
       <c r="H16" t="n">
-        <v>0.1306967739250254</v>
+        <v>0.1311338319815199</v>
       </c>
       <c r="I16" t="n">
         <v>69.71713810316139</v>
@@ -1766,10 +1766,10 @@
         <v>0.0924388272466749</v>
       </c>
       <c r="G17" t="n">
-        <v>0.1221717602573566</v>
+        <v>0.1270755822371887</v>
       </c>
       <c r="H17" t="n">
-        <v>0.1286786545887323</v>
+        <v>0.1291157126452268</v>
       </c>
       <c r="I17" t="n">
         <v>66.53763440860214</v>
@@ -1831,10 +1831,10 @@
         <v>0.1768933948702429</v>
       </c>
       <c r="G18" t="n">
-        <v>0.2066263278809246</v>
+        <v>0.2115301498607567</v>
       </c>
       <c r="H18" t="n">
-        <v>0.2131332222123002</v>
+        <v>0.2135702802687947</v>
       </c>
       <c r="I18" t="n">
         <v>65.57153965785382</v>
@@ -1896,10 +1896,10 @@
         <v>-0.153722023433663</v>
       </c>
       <c r="G19" t="n">
-        <v>-0.1239890904229813</v>
+        <v>-0.1190852684431492</v>
       </c>
       <c r="H19" t="n">
-        <v>-0.1174821960916057</v>
+        <v>-0.1170451380351111</v>
       </c>
       <c r="I19" t="n">
         <v>57.90312936017543</v>
@@ -1961,10 +1961,10 @@
         <v>0.1097742127153893</v>
       </c>
       <c r="G20" t="n">
-        <v>0.139507145726071</v>
+        <v>0.1444109677059031</v>
       </c>
       <c r="H20" t="n">
-        <v>0.1460140400574466</v>
+        <v>0.1464510981139412</v>
       </c>
       <c r="I20" t="n">
         <v>62.86926717806433</v>
@@ -2026,10 +2026,10 @@
         <v>-0.2521132221791392</v>
       </c>
       <c r="G21" t="n">
-        <v>-0.2223802891684575</v>
+        <v>-0.2174764671886254</v>
       </c>
       <c r="H21" t="n">
-        <v>-0.2158733948370819</v>
+        <v>-0.2154363367805873</v>
       </c>
       <c r="I21" t="n">
         <v>67.71787769017686</v>
@@ -2091,10 +2091,10 @@
         <v>0.3515077672860187</v>
       </c>
       <c r="G22" t="n">
-        <v>0.3812407002967004</v>
+        <v>0.3861445222765325</v>
       </c>
       <c r="H22" t="n">
-        <v>0.387747594628076</v>
+        <v>0.3881846526845706</v>
       </c>
       <c r="I22" t="n">
         <v>65.84471842719094</v>
@@ -2156,10 +2156,10 @@
         <v>-0.096135609293504</v>
       </c>
       <c r="G23" t="n">
-        <v>-0.0664026762828223</v>
+        <v>-0.0614988543029902</v>
       </c>
       <c r="H23" t="n">
-        <v>-0.0598957819514467</v>
+        <v>-0.0594587238949522</v>
       </c>
       <c r="I23" t="n">
         <v>73.2593340060545</v>
@@ -2221,10 +2221,10 @@
         <v>0.1537601341906624</v>
       </c>
       <c r="G24" t="n">
-        <v>0.1834930672013441</v>
+        <v>0.1883968891811762</v>
       </c>
       <c r="H24" t="n">
-        <v>0.1899999615327198</v>
+        <v>0.1904370195892143</v>
       </c>
       <c r="I24" t="n">
         <v>53.22314049586777</v>
@@ -2286,10 +2286,10 @@
         <v>-0.1490788404226497</v>
       </c>
       <c r="G25" t="n">
-        <v>-0.119345907411968</v>
+        <v>-0.1144420854321359</v>
       </c>
       <c r="H25" t="n">
-        <v>-0.1128390130805924</v>
+        <v>-0.1124019550240978</v>
       </c>
       <c r="I25" t="n">
         <v>66.04046242774567</v>
@@ -2351,10 +2351,10 @@
         <v>-0.2795629124743048</v>
       </c>
       <c r="G26" t="n">
-        <v>-0.2498299794636231</v>
+        <v>-0.2449261574837911</v>
       </c>
       <c r="H26" t="n">
-        <v>-0.2433230851322475</v>
+        <v>-0.242886027075753</v>
       </c>
       <c r="I26" t="n">
         <v>60.82595870206488</v>
@@ -2416,10 +2416,10 @@
         <v>0.1908905033279679</v>
       </c>
       <c r="G27" t="n">
-        <v>0.2206234363386496</v>
+        <v>0.2255272583184817</v>
       </c>
       <c r="H27" t="n">
-        <v>0.2271303306700253</v>
+        <v>0.2275673887265198</v>
       </c>
       <c r="I27" t="n">
         <v>59.00292284784646</v>
@@ -2481,10 +2481,10 @@
         <v>0.5124957497449845</v>
       </c>
       <c r="G28" t="n">
-        <v>0.5422286827556662</v>
+        <v>0.5471325047354982</v>
       </c>
       <c r="H28" t="n">
-        <v>0.5487355770870418</v>
+        <v>0.5491726351435363</v>
       </c>
       <c r="I28" t="n">
         <v>64.161220043573</v>
@@ -2546,10 +2546,10 @@
         <v>-0.0363891487371376</v>
       </c>
       <c r="G29" t="n">
-        <v>-0.0066562157264559</v>
+        <v>-0.0017523937466238</v>
       </c>
       <c r="H29" t="n">
-        <v>-0.0001493213950802</v>
+        <v>0.0002877366614142</v>
       </c>
       <c r="I29" t="n">
         <v>38.69327073552422</v>
@@ -2581,7 +2581,7 @@
         <v>0</v>
       </c>
       <c r="R29" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S29" t="b">
         <v>0</v>
@@ -2611,10 +2611,10 @@
         <v>-0.0556089625083191</v>
       </c>
       <c r="G30" t="n">
-        <v>-0.0258760294976374</v>
+        <v>-0.0209722075178053</v>
       </c>
       <c r="H30" t="n">
-        <v>-0.0193691351662618</v>
+        <v>-0.0189320771097672</v>
       </c>
       <c r="I30" t="n">
         <v>70.28556727553382</v>
@@ -2676,10 +2676,10 @@
         <v>-0.1872526556967297</v>
       </c>
       <c r="G31" t="n">
-        <v>-0.157519722686048</v>
+        <v>-0.152615900706216</v>
       </c>
       <c r="H31" t="n">
-        <v>-0.1510128283546724</v>
+        <v>-0.1505757702981779</v>
       </c>
       <c r="I31" t="n">
         <v>56.46766169154233</v>
@@ -2741,10 +2741,10 @@
         <v>-0.3045164865613744</v>
       </c>
       <c r="G32" t="n">
-        <v>-0.2747835535506927</v>
+        <v>-0.2698797315708606</v>
       </c>
       <c r="H32" t="n">
-        <v>-0.2682766592193171</v>
+        <v>-0.2678396011628225</v>
       </c>
       <c r="I32" t="n">
         <v>63.78344741754824</v>
@@ -2806,10 +2806,10 @@
         <v>0.0619485294117647</v>
       </c>
       <c r="G33" t="n">
-        <v>0.0916814624224464</v>
+        <v>0.0965852844022785</v>
       </c>
       <c r="H33" t="n">
-        <v>0.098188356753822</v>
+        <v>0.0986254148103166</v>
       </c>
       <c r="I33" t="n">
         <v>62.85714285714286</v>
@@ -2871,10 +2871,10 @@
         <v>-0.2401052253975846</v>
       </c>
       <c r="G34" t="n">
-        <v>-0.2103722923869029</v>
+        <v>-0.2054684704070708</v>
       </c>
       <c r="H34" t="n">
-        <v>-0.2038653980555272</v>
+        <v>-0.2034283399990327</v>
       </c>
       <c r="I34" t="n">
         <v>63.3225806451613</v>
@@ -2936,10 +2936,10 @@
         <v>0.1400984841170223</v>
       </c>
       <c r="G35" t="n">
-        <v>0.169831417127704</v>
+        <v>0.174735239107536</v>
       </c>
       <c r="H35" t="n">
-        <v>0.1763383114590796</v>
+        <v>0.1767753695155741</v>
       </c>
       <c r="I35" t="n">
         <v>63.52905569007262</v>
@@ -3001,10 +3001,10 @@
         <v>0.0966856892010534</v>
       </c>
       <c r="G36" t="n">
-        <v>0.1264186222117351</v>
+        <v>0.1313224441915672</v>
       </c>
       <c r="H36" t="n">
-        <v>0.1329255165431108</v>
+        <v>0.1333625745996053</v>
       </c>
       <c r="I36" t="n">
         <v>65.71428571428571</v>
@@ -3066,10 +3066,10 @@
         <v>0.5624082232011749</v>
       </c>
       <c r="G37" t="n">
-        <v>0.5921411562118566</v>
+        <v>0.5970449781916887</v>
       </c>
       <c r="H37" t="n">
-        <v>0.5986480505432322</v>
+        <v>0.5990851085997267</v>
       </c>
       <c r="I37" t="n">
         <v>69.86404833836862</v>
@@ -3131,10 +3131,10 @@
         <v>-0.2526900687952019</v>
       </c>
       <c r="G38" t="n">
-        <v>-0.2229571357845202</v>
+        <v>-0.2180533138046881</v>
       </c>
       <c r="H38" t="n">
-        <v>-0.2164502414531446</v>
+        <v>-0.2160131833966501</v>
       </c>
       <c r="I38" t="n">
         <v>59.55303169078587</v>
@@ -3196,10 +3196,10 @@
         <v>0.400414937759336</v>
       </c>
       <c r="G39" t="n">
-        <v>0.4301478707700177</v>
+        <v>0.4350516927498498</v>
       </c>
       <c r="H39" t="n">
-        <v>0.4366547651013933</v>
+        <v>0.4370918231578878</v>
       </c>
       <c r="I39" t="n">
         <v>79.90525504021156</v>
@@ -3261,10 +3261,10 @@
         <v>-0.1079127725856697</v>
       </c>
       <c r="G40" t="n">
-        <v>-0.078179839574988</v>
+        <v>-0.07327601759515601</v>
       </c>
       <c r="H40" t="n">
-        <v>-0.0716729452436124</v>
+        <v>-0.0712358871871179</v>
       </c>
       <c r="I40" t="n">
         <v>74.23405323957812</v>
@@ -3326,10 +3326,10 @@
         <v>-0.2162411416367342</v>
       </c>
       <c r="G41" t="n">
-        <v>-0.1865082086260525</v>
+        <v>-0.1816043866462204</v>
       </c>
       <c r="H41" t="n">
-        <v>-0.1800013142946769</v>
+        <v>-0.1795642562381824</v>
       </c>
       <c r="I41" t="n">
         <v>52.45949926362298</v>
@@ -3391,10 +3391,10 @@
         <v>-0.1942228512609367</v>
       </c>
       <c r="G42" t="n">
-        <v>-0.164489918250255</v>
+        <v>-0.1595860962704229</v>
       </c>
       <c r="H42" t="n">
-        <v>-0.1579830239188794</v>
+        <v>-0.1575459658623849</v>
       </c>
       <c r="I42" t="n">
         <v>69.21022510492179</v>
@@ -3456,10 +3456,10 @@
         <v>-0.1584008097165992</v>
       </c>
       <c r="G43" t="n">
-        <v>-0.1286678767059175</v>
+        <v>-0.1237640547260854</v>
       </c>
       <c r="H43" t="n">
-        <v>-0.1221609823745418</v>
+        <v>-0.1217239243180473</v>
       </c>
       <c r="I43" t="n">
         <v>52.52621544327933</v>
@@ -3521,10 +3521,10 @@
         <v>-0.141583521081429</v>
       </c>
       <c r="G44" t="n">
-        <v>-0.1118505880707473</v>
+        <v>-0.1069467660909152</v>
       </c>
       <c r="H44" t="n">
-        <v>-0.1053436937393716</v>
+        <v>-0.1049066356828771</v>
       </c>
       <c r="I44" t="n">
         <v>82.84904323175053</v>
@@ -3586,10 +3586,10 @@
         <v>-0.3025809610407778</v>
       </c>
       <c r="G45" t="n">
-        <v>-0.2728480280300961</v>
+        <v>-0.267944206050264</v>
       </c>
       <c r="H45" t="n">
-        <v>-0.2663411336987205</v>
+        <v>-0.2659040756422259</v>
       </c>
       <c r="I45" t="n">
         <v>60.13179571663922</v>
@@ -3651,10 +3651,10 @@
         <v>-0.1545753682231276</v>
       </c>
       <c r="G46" t="n">
-        <v>-0.1248424352124459</v>
+        <v>-0.1199386132326139</v>
       </c>
       <c r="H46" t="n">
-        <v>-0.1183355408810703</v>
+        <v>-0.1178984828245758</v>
       </c>
       <c r="I46" t="n">
         <v>65.46063651591288</v>
@@ -3716,10 +3716,10 @@
         <v>0.2762157819934501</v>
       </c>
       <c r="G47" t="n">
-        <v>0.3059487150041318</v>
+        <v>0.3108525369839638</v>
       </c>
       <c r="H47" t="n">
-        <v>0.3124556093355074</v>
+        <v>0.3128926673920019</v>
       </c>
       <c r="I47" t="n">
         <v>40.1215277777778</v>
@@ -3781,10 +3781,10 @@
         <v>0.0777752134779599</v>
       </c>
       <c r="G48" t="n">
-        <v>0.1075081464886416</v>
+        <v>0.1124119684684736</v>
       </c>
       <c r="H48" t="n">
-        <v>0.1140150408200172</v>
+        <v>0.1144520988765117</v>
       </c>
       <c r="I48" t="n">
         <v>57.06081081081081</v>
@@ -3957,10 +3957,10 @@
         <v>0.5124957497449845</v>
       </c>
       <c r="G2" t="n">
-        <v>0.5422286827556662</v>
+        <v>0.5471325047354982</v>
       </c>
       <c r="H2" t="n">
-        <v>0.5487355770870418</v>
+        <v>0.5491726351435363</v>
       </c>
       <c r="I2" t="n">
         <v>64.161220043573</v>
@@ -4022,10 +4022,10 @@
         <v>0.4641087130295762</v>
       </c>
       <c r="G3" t="n">
-        <v>0.4938416460402579</v>
+        <v>0.49874546802009</v>
       </c>
       <c r="H3" t="n">
-        <v>0.5003485403716336</v>
+        <v>0.5007855984281281</v>
       </c>
       <c r="I3" t="n">
         <v>62.95993458708093</v>
@@ -4087,10 +4087,10 @@
         <v>0.1908905033279679</v>
       </c>
       <c r="G4" t="n">
-        <v>0.2206234363386496</v>
+        <v>0.2255272583184817</v>
       </c>
       <c r="H4" t="n">
-        <v>0.2271303306700253</v>
+        <v>0.2275673887265198</v>
       </c>
       <c r="I4" t="n">
         <v>59.00292284784646</v>
@@ -4152,10 +4152,10 @@
         <v>0.3515077672860187</v>
       </c>
       <c r="G5" t="n">
-        <v>0.3812407002967004</v>
+        <v>0.3861445222765325</v>
       </c>
       <c r="H5" t="n">
-        <v>0.387747594628076</v>
+        <v>0.3881846526845706</v>
       </c>
       <c r="I5" t="n">
         <v>65.84471842719094</v>
@@ -4217,10 +4217,10 @@
         <v>0.5624082232011749</v>
       </c>
       <c r="G6" t="n">
-        <v>0.5921411562118566</v>
+        <v>0.5970449781916887</v>
       </c>
       <c r="H6" t="n">
-        <v>0.5986480505432322</v>
+        <v>0.5990851085997267</v>
       </c>
       <c r="I6" t="n">
         <v>69.86404833836862</v>
@@ -4282,10 +4282,10 @@
         <v>0.2762157819934501</v>
       </c>
       <c r="G7" t="n">
-        <v>0.3059487150041318</v>
+        <v>0.3108525369839638</v>
       </c>
       <c r="H7" t="n">
-        <v>0.3124556093355074</v>
+        <v>0.3128926673920019</v>
       </c>
       <c r="I7" t="n">
         <v>40.1215277777778</v>
@@ -4347,10 +4347,10 @@
         <v>0.1768933948702429</v>
       </c>
       <c r="G8" t="n">
-        <v>0.2066263278809246</v>
+        <v>0.2115301498607567</v>
       </c>
       <c r="H8" t="n">
-        <v>0.2131332222123002</v>
+        <v>0.2135702802687947</v>
       </c>
       <c r="I8" t="n">
         <v>65.57153965785382</v>
@@ -4412,10 +4412,10 @@
         <v>0.1023376159885796</v>
       </c>
       <c r="G9" t="n">
-        <v>0.1320705489992613</v>
+        <v>0.1369743709790933</v>
       </c>
       <c r="H9" t="n">
-        <v>0.1385774433306369</v>
+        <v>0.1390145013871314</v>
       </c>
       <c r="I9" t="n">
         <v>64.21167484997272</v>
@@ -4477,10 +4477,10 @@
         <v>0.0924388272466749</v>
       </c>
       <c r="G10" t="n">
-        <v>0.1221717602573566</v>
+        <v>0.1270755822371887</v>
       </c>
       <c r="H10" t="n">
-        <v>0.1286786545887323</v>
+        <v>0.1291157126452268</v>
       </c>
       <c r="I10" t="n">
         <v>66.53763440860214</v>
@@ -4542,10 +4542,10 @@
         <v>0.1400984841170223</v>
       </c>
       <c r="G11" t="n">
-        <v>0.169831417127704</v>
+        <v>0.174735239107536</v>
       </c>
       <c r="H11" t="n">
-        <v>0.1763383114590796</v>
+        <v>0.1767753695155741</v>
       </c>
       <c r="I11" t="n">
         <v>63.52905569007262</v>
@@ -4607,10 +4607,10 @@
         <v>0.0944569465829681</v>
       </c>
       <c r="G12" t="n">
-        <v>0.1241898795936498</v>
+        <v>0.1290937015734818</v>
       </c>
       <c r="H12" t="n">
-        <v>0.1306967739250254</v>
+        <v>0.1311338319815199</v>
       </c>
       <c r="I12" t="n">
         <v>69.71713810316139</v>
@@ -4672,10 +4672,10 @@
         <v>0.1097742127153893</v>
       </c>
       <c r="G13" t="n">
-        <v>0.139507145726071</v>
+        <v>0.1444109677059031</v>
       </c>
       <c r="H13" t="n">
-        <v>0.1460140400574466</v>
+        <v>0.1464510981139412</v>
       </c>
       <c r="I13" t="n">
         <v>62.86926717806433</v>
@@ -4737,10 +4737,10 @@
         <v>0.400414937759336</v>
       </c>
       <c r="G14" t="n">
-        <v>0.4301478707700177</v>
+        <v>0.4350516927498498</v>
       </c>
       <c r="H14" t="n">
-        <v>0.4366547651013933</v>
+        <v>0.4370918231578878</v>
       </c>
       <c r="I14" t="n">
         <v>79.90525504021156</v>
@@ -4802,10 +4802,10 @@
         <v>0.390055773110241</v>
       </c>
       <c r="G15" t="n">
-        <v>0.4197887061209226</v>
+        <v>0.4246925281007547</v>
       </c>
       <c r="H15" t="n">
-        <v>0.4262956004522983</v>
+        <v>0.4267326585087928</v>
       </c>
       <c r="I15" t="n">
         <v>73.66911061523747</v>
@@ -4867,10 +4867,10 @@
         <v>0.2647258722247394</v>
       </c>
       <c r="G16" t="n">
-        <v>0.2944588052354211</v>
+        <v>0.2993626272152532</v>
       </c>
       <c r="H16" t="n">
-        <v>0.3009656995667967</v>
+        <v>0.3014027576232913</v>
       </c>
       <c r="I16" t="n">
         <v>71.96802646085999</v>

</xml_diff>

<commit_message>
chore: auto-refresh NSE data and pipeline outputs (2026-04-17)
</commit_message>
<xml_diff>
--- a/working-sector/output/auto_components_comprehensive_report.xlsx
+++ b/working-sector/output/auto_components_comprehensive_report.xlsx
@@ -435,7 +435,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -447,7 +447,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -779,48 +779,48 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1831.6</v>
+        <v>1860.5</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0490263459335624</v>
+        <v>0.08648680214903059</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2542628227076628</v>
+        <v>0.2765884451763414</v>
       </c>
       <c r="F2" t="n">
-        <v>0.4641087130295762</v>
+        <v>0.5325370675453047</v>
       </c>
       <c r="G2" t="n">
-        <v>0.49874546802009</v>
+        <v>0.5613601009900163</v>
       </c>
       <c r="H2" t="n">
-        <v>0.5007855984281281</v>
+        <v>0.5588179547727297</v>
       </c>
       <c r="I2" t="n">
-        <v>62.95993458708093</v>
+        <v>77.83767595088349</v>
       </c>
       <c r="J2" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K2" t="n">
         <v>54.83</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M2" t="n">
         <v>54.83</v>
       </c>
       <c r="N2" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O2" t="n">
-        <v>95.74468085106383</v>
+        <v>97.87234042553192</v>
       </c>
       <c r="P2" t="n">
-        <v>73.08093617021277</v>
+        <v>69.50646808510639</v>
       </c>
       <c r="Q2" t="b">
         <v>0</v>
@@ -844,25 +844,25 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1100.1</v>
+        <v>1097.8</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0447293447293446</v>
+        <v>0.0560846560846559</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.08386075949367081</v>
+        <v>-0.0728040540540541</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.164755903120492</v>
+        <v>-0.1458803392204154</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.1301191481299782</v>
+        <v>-0.1170573057757038</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.1280790177219402</v>
+        <v>-0.1195994519929904</v>
       </c>
       <c r="I3" t="n">
-        <v>52.18760938046901</v>
+        <v>63.20830007980843</v>
       </c>
       <c r="J3" t="n">
         <v>60</v>
@@ -872,7 +872,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M3" t="n">
@@ -882,10 +882,10 @@
         <v>60</v>
       </c>
       <c r="O3" t="n">
-        <v>29.78723404255319</v>
+        <v>27.65957446808511</v>
       </c>
       <c r="P3" t="n">
-        <v>49.70144680851064</v>
+        <v>49.27591489361702</v>
       </c>
       <c r="Q3" t="b">
         <v>0</v>
@@ -909,54 +909,54 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>37080</v>
+        <v>37505</v>
       </c>
       <c r="D4" t="n">
-        <v>0.209985315712188</v>
+        <v>0.244566119130579</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.0217649386624455</v>
+        <v>0.01818922220714</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.0586443259710586</v>
+        <v>-0.0219063763202503</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.0240075709805448</v>
+        <v>0.0069166571244612</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.0219674405725067</v>
+        <v>0.0043745109071745</v>
       </c>
       <c r="I4" t="n">
-        <v>79.23951048951048</v>
+        <v>92.85714285714286</v>
       </c>
       <c r="J4" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="K4" t="n">
         <v>53.48</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M4" t="n">
         <v>53.48</v>
       </c>
       <c r="N4" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="O4" t="n">
-        <v>51.06382978723404</v>
+        <v>53.19148936170212</v>
       </c>
       <c r="P4" t="n">
-        <v>59.6047659574468</v>
+        <v>56.03029787234042</v>
       </c>
       <c r="Q4" t="b">
         <v>0</v>
       </c>
       <c r="R4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S4" t="b">
         <v>0</v>
@@ -977,45 +977,45 @@
         <v>330</v>
       </c>
       <c r="D5" t="n">
-        <v>0.093077177873468</v>
+        <v>0.0932582408481033</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.0462427745664739</v>
+        <v>-0.040976460331299</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.1816491010539367</v>
+        <v>-0.1506884570840304</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.1470123460634229</v>
+        <v>-0.1218654236393188</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.1449722156553848</v>
+        <v>-0.1244075698566055</v>
       </c>
       <c r="I5" t="n">
-        <v>65.79129232895647</v>
+        <v>87.65652951699467</v>
       </c>
       <c r="J5" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K5" t="n">
         <v>51.12</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M5" t="n">
         <v>51.12</v>
       </c>
       <c r="N5" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O5" t="n">
         <v>23.40425531914894</v>
       </c>
       <c r="P5" t="n">
-        <v>57.12885106382979</v>
+        <v>49.12885106382979</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
@@ -1039,48 +1039,48 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>123.55</v>
+        <v>125.03</v>
       </c>
       <c r="D6" t="n">
-        <v>0.0666493999827333</v>
+        <v>0.1188366890380312</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0750021752371008</v>
+        <v>0.0892063768620958</v>
       </c>
       <c r="F6" t="n">
-        <v>0.1023376159885796</v>
+        <v>0.1698166167664672</v>
       </c>
       <c r="G6" t="n">
-        <v>0.1369743709790933</v>
+        <v>0.1986396502111788</v>
       </c>
       <c r="H6" t="n">
-        <v>0.1390145013871314</v>
+        <v>0.1960975039938921</v>
       </c>
       <c r="I6" t="n">
-        <v>64.21167484997272</v>
+        <v>81.61648177496039</v>
       </c>
       <c r="J6" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K6" t="n">
         <v>51.57</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M6" t="n">
         <v>51.57</v>
       </c>
       <c r="N6" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O6" t="n">
-        <v>72.3404255319149</v>
+        <v>78.72340425531915</v>
       </c>
       <c r="P6" t="n">
-        <v>67.09608510638299</v>
+        <v>60.37268085106383</v>
       </c>
       <c r="Q6" t="b">
         <v>0</v>
@@ -1104,48 +1104,48 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2755</v>
+        <v>2790.2</v>
       </c>
       <c r="D7" t="n">
-        <v>0.1127266852457691</v>
+        <v>0.1028458498023714</v>
       </c>
       <c r="E7" t="n">
-        <v>0.1540233736857537</v>
+        <v>0.1910697515580979</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.1659097789887981</v>
+        <v>-0.09952881946685591</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.1312730239982843</v>
+        <v>-0.07070578602214431</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.1292328935902462</v>
+        <v>-0.073247932239431</v>
       </c>
       <c r="I7" t="n">
-        <v>57.68742058449809</v>
+        <v>89.37950937950943</v>
       </c>
       <c r="J7" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K7" t="n">
         <v>48.73</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M7" t="n">
         <v>48.73</v>
       </c>
       <c r="N7" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O7" t="n">
-        <v>27.65957446808511</v>
+        <v>34.04255319148936</v>
       </c>
       <c r="P7" t="n">
-        <v>57.02391489361703</v>
+        <v>50.30051063829788</v>
       </c>
       <c r="Q7" t="b">
         <v>0</v>
@@ -1169,48 +1169,48 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>585.7</v>
+        <v>593.85</v>
       </c>
       <c r="D8" t="n">
-        <v>0.1665006970722964</v>
+        <v>0.1907960697814317</v>
       </c>
       <c r="E8" t="n">
-        <v>0.2814790504321192</v>
+        <v>0.2906976744186047</v>
       </c>
       <c r="F8" t="n">
-        <v>0.390055773110241</v>
+        <v>0.4650302207968422</v>
       </c>
       <c r="G8" t="n">
-        <v>0.4246925281007547</v>
+        <v>0.4938532542415538</v>
       </c>
       <c r="H8" t="n">
-        <v>0.4267326585087928</v>
+        <v>0.4913111080242671</v>
       </c>
       <c r="I8" t="n">
-        <v>73.66911061523747</v>
+        <v>88.80829015544036</v>
       </c>
       <c r="J8" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="K8" t="n">
         <v>49.66</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M8" t="n">
         <v>49.66</v>
       </c>
       <c r="N8" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="O8" t="n">
-        <v>91.48936170212764</v>
+        <v>95.74468085106383</v>
       </c>
       <c r="P8" t="n">
-        <v>66.16187234042553</v>
+        <v>63.01293617021277</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
@@ -1234,48 +1234,48 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>441.6</v>
+        <v>445.4</v>
       </c>
       <c r="D9" t="n">
-        <v>0.0465694987557767</v>
+        <v>0.0618667302419835</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.1515850144092219</v>
+        <v>-0.1241765804738964</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.0970248440854718</v>
+        <v>-0.0432821394050049</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.062388089094958</v>
+        <v>-0.0144591059602933</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.06034795868692</v>
+        <v>-0.0170012521775799</v>
       </c>
       <c r="I9" t="n">
-        <v>67.10833982852691</v>
+        <v>77.31023102310225</v>
       </c>
       <c r="J9" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K9" t="n">
         <v>53.44</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M9" t="n">
         <v>53.44</v>
       </c>
       <c r="N9" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O9" t="n">
-        <v>46.80851063829788</v>
+        <v>44.68085106382978</v>
       </c>
       <c r="P9" t="n">
-        <v>54.73770212765958</v>
+        <v>58.31217021276596</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -1299,48 +1299,48 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>137900</v>
+        <v>139855</v>
       </c>
       <c r="D10" t="n">
-        <v>0.0387947269303201</v>
+        <v>0.0713164043050289</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.0664139191659332</v>
+        <v>-0.0208975077009241</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.1156571648443262</v>
+        <v>-0.0413339274085752</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.0810204098538124</v>
+        <v>-0.0125108939638636</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.07898027944577431</v>
+        <v>-0.0150530401811502</v>
       </c>
       <c r="I10" t="n">
-        <v>68.81822496440437</v>
+        <v>76.35730858468678</v>
       </c>
       <c r="J10" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K10" t="n">
         <v>49.41</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M10" t="n">
         <v>49.41</v>
       </c>
       <c r="N10" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O10" t="n">
-        <v>42.5531914893617</v>
+        <v>46.80851063829788</v>
       </c>
       <c r="P10" t="n">
-        <v>60.27463829787234</v>
+        <v>57.12570212765957</v>
       </c>
       <c r="Q10" t="b">
         <v>0</v>
@@ -1376,10 +1376,10 @@
         <v>-0.0042030657656173</v>
       </c>
       <c r="G11" t="n">
-        <v>0.0304336892248964</v>
+        <v>0.0246199676790942</v>
       </c>
       <c r="H11" t="n">
-        <v>0.0324738196329345</v>
+        <v>0.0220778214618075</v>
       </c>
       <c r="I11" t="n">
         <v>27.6054590570719</v>
@@ -1392,7 +1392,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M11" t="n">
@@ -1402,10 +1402,10 @@
         <v>20</v>
       </c>
       <c r="O11" t="n">
-        <v>59.57446808510638</v>
+        <v>55.31914893617022</v>
       </c>
       <c r="P11" t="n">
-        <v>23.91489361702128</v>
+        <v>23.06382978723404</v>
       </c>
       <c r="Q11" t="b">
         <v>0</v>
@@ -1429,25 +1429,25 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>440.15</v>
+        <v>436.8</v>
       </c>
       <c r="D12" t="n">
-        <v>0.08411330049261059</v>
+        <v>0.043602914824991</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.0548636461241142</v>
+        <v>-0.0586206896551724</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.1780578898225957</v>
+        <v>-0.192680898253396</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.1434211348320819</v>
+        <v>-0.1638578648086844</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.1413810044240439</v>
+        <v>-0.1664000110259711</v>
       </c>
       <c r="I12" t="n">
-        <v>45.52572706935123</v>
+        <v>40.02509410288583</v>
       </c>
       <c r="J12" t="n">
         <v>80</v>
@@ -1457,7 +1457,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M12" t="n">
@@ -1467,10 +1467,10 @@
         <v>80</v>
       </c>
       <c r="O12" t="n">
-        <v>25.53191489361702</v>
+        <v>12.76595744680851</v>
       </c>
       <c r="P12" t="n">
-        <v>65.6183829787234</v>
+        <v>63.0651914893617</v>
       </c>
       <c r="Q12" t="b">
         <v>1</v>
@@ -1494,25 +1494,25 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1727.2</v>
+        <v>1881.9</v>
       </c>
       <c r="D13" t="n">
-        <v>0.0046533271288971</v>
+        <v>0.130134518376171</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.0945690920528412</v>
+        <v>-0.0376374328816159</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.0475350170949597</v>
+        <v>0.083294957402717</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.012898262104446</v>
+        <v>0.1121179908474286</v>
       </c>
       <c r="H13" t="n">
-        <v>-0.0108581316964079</v>
+        <v>0.109575844630142</v>
       </c>
       <c r="I13" t="n">
-        <v>59.67254408060453</v>
+        <v>87.3327386262266</v>
       </c>
       <c r="J13" t="n">
         <v>60</v>
@@ -1522,7 +1522,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M13" t="n">
@@ -1532,16 +1532,16 @@
         <v>60</v>
       </c>
       <c r="O13" t="n">
-        <v>55.31914893617022</v>
+        <v>61.70212765957447</v>
       </c>
       <c r="P13" t="n">
-        <v>58.57182978723405</v>
+        <v>59.8484255319149</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
       </c>
       <c r="R13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S13" t="b">
         <v>0</v>
@@ -1559,48 +1559,48 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>596.9</v>
+        <v>624.95</v>
       </c>
       <c r="D14" t="n">
-        <v>0.0350268770591293</v>
+        <v>0.1355501044789679</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.0800647299067581</v>
+        <v>-0.0080945956670104</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.2676972150656361</v>
+        <v>-0.2737783975364591</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.2330604600751223</v>
+        <v>-0.2449553640917475</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.2310203296670843</v>
+        <v>-0.2474975103090342</v>
       </c>
       <c r="I14" t="n">
-        <v>58.03869246164109</v>
+        <v>80.68702290076334</v>
       </c>
       <c r="J14" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K14" t="n">
         <v>54.64</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M14" t="n">
         <v>54.64</v>
       </c>
       <c r="N14" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O14" t="n">
-        <v>8.51063829787234</v>
+        <v>2.127659574468085</v>
       </c>
       <c r="P14" t="n">
-        <v>55.55812765957447</v>
+        <v>46.28153191489362</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
@@ -1624,48 +1624,48 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>111.65</v>
+        <v>112.64</v>
       </c>
       <c r="D15" t="n">
-        <v>0.1548407116259826</v>
+        <v>0.1673748574981863</v>
       </c>
       <c r="E15" t="n">
-        <v>0.0538984330753258</v>
+        <v>0.069807199164213</v>
       </c>
       <c r="F15" t="n">
-        <v>0.2647258722247394</v>
+        <v>0.2639138240574505</v>
       </c>
       <c r="G15" t="n">
-        <v>0.2993626272152532</v>
+        <v>0.2927368575021621</v>
       </c>
       <c r="H15" t="n">
-        <v>0.3014027576232913</v>
+        <v>0.2901947112848755</v>
       </c>
       <c r="I15" t="n">
-        <v>71.96802646085999</v>
+        <v>94.62837837837836</v>
       </c>
       <c r="J15" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="K15" t="n">
         <v>51.91</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M15" t="n">
         <v>51.91</v>
       </c>
       <c r="N15" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="O15" t="n">
         <v>85.1063829787234</v>
       </c>
       <c r="P15" t="n">
-        <v>65.78527659574468</v>
+        <v>61.78527659574468</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
@@ -1689,48 +1689,48 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>184.81</v>
+        <v>183.46</v>
       </c>
       <c r="D16" t="n">
-        <v>0.1359641035097425</v>
+        <v>0.1723432807208127</v>
       </c>
       <c r="E16" t="n">
-        <v>0.140098704503393</v>
+        <v>0.156819471593417</v>
       </c>
       <c r="F16" t="n">
-        <v>0.0944569465829681</v>
+        <v>0.0260052569766791</v>
       </c>
       <c r="G16" t="n">
-        <v>0.1290937015734818</v>
+        <v>0.0548282904213907</v>
       </c>
       <c r="H16" t="n">
-        <v>0.1311338319815199</v>
+        <v>0.052286144204104</v>
       </c>
       <c r="I16" t="n">
-        <v>69.71713810316139</v>
+        <v>92.31990474300456</v>
       </c>
       <c r="J16" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K16" t="n">
         <v>52.61</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M16" t="n">
         <v>52.61</v>
       </c>
       <c r="N16" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O16" t="n">
-        <v>68.08510638297872</v>
+        <v>59.57446808510638</v>
       </c>
       <c r="P16" t="n">
-        <v>66.66102127659575</v>
+        <v>56.95889361702128</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>
@@ -1754,48 +1754,48 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>7433.5</v>
+        <v>7691</v>
       </c>
       <c r="D17" t="n">
-        <v>0.07467110018794269</v>
+        <v>0.1219547775346463</v>
       </c>
       <c r="E17" t="n">
-        <v>-0.0329148507122877</v>
+        <v>-0.0099124613800205</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0924388272466749</v>
+        <v>0.1446643845810389</v>
       </c>
       <c r="G17" t="n">
-        <v>0.1270755822371887</v>
+        <v>0.1734874180257505</v>
       </c>
       <c r="H17" t="n">
-        <v>0.1291157126452268</v>
+        <v>0.1709452718084638</v>
       </c>
       <c r="I17" t="n">
-        <v>66.53763440860214</v>
+        <v>78.74396135265701</v>
       </c>
       <c r="J17" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K17" t="n">
         <v>54.65</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M17" t="n">
         <v>54.65</v>
       </c>
       <c r="N17" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O17" t="n">
-        <v>65.95744680851064</v>
+        <v>70.21276595744681</v>
       </c>
       <c r="P17" t="n">
-        <v>67.05148936170212</v>
+        <v>63.90255319148936</v>
       </c>
       <c r="Q17" t="b">
         <v>0</v>
@@ -1819,48 +1819,48 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>777.75</v>
+        <v>776.1</v>
       </c>
       <c r="D18" t="n">
-        <v>0.1547884187082404</v>
+        <v>0.1390621560137961</v>
       </c>
       <c r="E18" t="n">
-        <v>0.3238297872340425</v>
+        <v>0.3027276542173731</v>
       </c>
       <c r="F18" t="n">
-        <v>0.1768933948702429</v>
+        <v>0.1537946926336133</v>
       </c>
       <c r="G18" t="n">
-        <v>0.2115301498607567</v>
+        <v>0.1826177260783249</v>
       </c>
       <c r="H18" t="n">
-        <v>0.2135702802687947</v>
+        <v>0.1800755798610382</v>
       </c>
       <c r="I18" t="n">
-        <v>65.57153965785382</v>
+        <v>92.18421052631584</v>
       </c>
       <c r="J18" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K18" t="n">
         <v>49.92</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M18" t="n">
         <v>49.92</v>
       </c>
       <c r="N18" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O18" t="n">
-        <v>80.85106382978722</v>
+        <v>72.3404255319149</v>
       </c>
       <c r="P18" t="n">
-        <v>68.13821276595745</v>
+        <v>58.43608510638298</v>
       </c>
       <c r="Q18" t="b">
         <v>0</v>
@@ -1884,48 +1884,48 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2412.4</v>
+        <v>2384.4</v>
       </c>
       <c r="D19" t="n">
-        <v>0.0362097848030584</v>
+        <v>0.0476274165202108</v>
       </c>
       <c r="E19" t="n">
-        <v>-0.0677795811113687</v>
+        <v>-0.0560570071258906</v>
       </c>
       <c r="F19" t="n">
-        <v>-0.153722023433663</v>
+        <v>-0.1283494790714676</v>
       </c>
       <c r="G19" t="n">
-        <v>-0.1190852684431492</v>
+        <v>-0.099526445626756</v>
       </c>
       <c r="H19" t="n">
-        <v>-0.1170451380351111</v>
+        <v>-0.1020685918440427</v>
       </c>
       <c r="I19" t="n">
-        <v>57.90312936017543</v>
+        <v>70.74714042346068</v>
       </c>
       <c r="J19" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="K19" t="n">
         <v>51.27</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M19" t="n">
         <v>51.27</v>
       </c>
       <c r="N19" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="O19" t="n">
-        <v>36.17021276595745</v>
+        <v>29.78723404255319</v>
       </c>
       <c r="P19" t="n">
-        <v>51.7420425531915</v>
+        <v>46.46544680851064</v>
       </c>
       <c r="Q19" t="b">
         <v>0</v>
@@ -1949,48 +1949,48 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2241.3</v>
+        <v>2259.1</v>
       </c>
       <c r="D20" t="n">
-        <v>0.1188598242811502</v>
+        <v>0.1287034723957032</v>
       </c>
       <c r="E20" t="n">
-        <v>-0.0063838276366536</v>
+        <v>0.0359992662569934</v>
       </c>
       <c r="F20" t="n">
-        <v>0.1097742127153893</v>
+        <v>0.1647847383346223</v>
       </c>
       <c r="G20" t="n">
-        <v>0.1444109677059031</v>
+        <v>0.1936077717793339</v>
       </c>
       <c r="H20" t="n">
-        <v>0.1464510981139412</v>
+        <v>0.1910656255620473</v>
       </c>
       <c r="I20" t="n">
-        <v>62.86926717806433</v>
+        <v>86.76097972972968</v>
       </c>
       <c r="J20" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K20" t="n">
         <v>49.06</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M20" t="n">
         <v>49.06</v>
       </c>
       <c r="N20" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O20" t="n">
-        <v>74.46808510638297</v>
+        <v>76.59574468085107</v>
       </c>
       <c r="P20" t="n">
-        <v>66.51761702127659</v>
+        <v>58.94314893617022</v>
       </c>
       <c r="Q20" t="b">
         <v>0</v>
@@ -2014,48 +2014,48 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>964.4</v>
+        <v>1014.35</v>
       </c>
       <c r="D21" t="n">
-        <v>0.1425186589266673</v>
+        <v>0.208566662695103</v>
       </c>
       <c r="E21" t="n">
-        <v>0.0123871509552802</v>
+        <v>0.1021949364337717</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.2521132221791392</v>
+        <v>-0.1680200131233595</v>
       </c>
       <c r="G21" t="n">
-        <v>-0.2174764671886254</v>
+        <v>-0.1391969796786479</v>
       </c>
       <c r="H21" t="n">
-        <v>-0.2154363367805873</v>
+        <v>-0.1417391258959346</v>
       </c>
       <c r="I21" t="n">
-        <v>67.71787769017686</v>
+        <v>92.11469534050178</v>
       </c>
       <c r="J21" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K21" t="n">
         <v>48.43</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M21" t="n">
         <v>48.43</v>
       </c>
       <c r="N21" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O21" t="n">
-        <v>12.76595744680851</v>
+        <v>19.14893617021277</v>
       </c>
       <c r="P21" t="n">
-        <v>53.9251914893617</v>
+        <v>47.20178723404256</v>
       </c>
       <c r="Q21" t="b">
         <v>0</v>
@@ -2079,48 +2079,48 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>443.7</v>
+        <v>435.9</v>
       </c>
       <c r="D22" t="n">
-        <v>0.136381098732232</v>
+        <v>0.1480115880958652</v>
       </c>
       <c r="E22" t="n">
-        <v>0.2630230572160545</v>
+        <v>0.2301396923945251</v>
       </c>
       <c r="F22" t="n">
-        <v>0.3515077672860187</v>
+        <v>0.4122792807387008</v>
       </c>
       <c r="G22" t="n">
-        <v>0.3861445222765325</v>
+        <v>0.4411023141834124</v>
       </c>
       <c r="H22" t="n">
-        <v>0.3881846526845706</v>
+        <v>0.4385601679661257</v>
       </c>
       <c r="I22" t="n">
-        <v>65.84471842719094</v>
+        <v>83.44594594594594</v>
       </c>
       <c r="J22" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K22" t="n">
         <v>54.47</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M22" t="n">
         <v>54.47</v>
       </c>
       <c r="N22" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O22" t="n">
-        <v>89.36170212765957</v>
+        <v>93.61702127659576</v>
       </c>
       <c r="P22" t="n">
-        <v>71.66034042553191</v>
+        <v>64.51140425531915</v>
       </c>
       <c r="Q22" t="b">
         <v>0</v>
@@ -2144,54 +2144,54 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>381.25</v>
+        <v>401.6</v>
       </c>
       <c r="D23" t="n">
-        <v>0.1154183733177296</v>
+        <v>0.1698223128459073</v>
       </c>
       <c r="E23" t="n">
-        <v>-0.0102544132917964</v>
+        <v>0.0186429930247304</v>
       </c>
       <c r="F23" t="n">
-        <v>-0.096135609293504</v>
+        <v>0.0004982561036372</v>
       </c>
       <c r="G23" t="n">
-        <v>-0.0614988543029902</v>
+        <v>0.0293212895483488</v>
       </c>
       <c r="H23" t="n">
-        <v>-0.0594587238949522</v>
+        <v>0.0267791433310622</v>
       </c>
       <c r="I23" t="n">
-        <v>73.2593340060545</v>
+        <v>89.83128134974922</v>
       </c>
       <c r="J23" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="K23" t="n">
         <v>49.7</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M23" t="n">
         <v>49.7</v>
       </c>
       <c r="N23" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="O23" t="n">
-        <v>48.93617021276596</v>
+        <v>57.44680851063831</v>
       </c>
       <c r="P23" t="n">
-        <v>57.6672340425532</v>
+        <v>55.36936170212766</v>
       </c>
       <c r="Q23" t="b">
         <v>0</v>
       </c>
       <c r="R23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S23" t="b">
         <v>0</v>
@@ -2209,48 +2209,48 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>123.81</v>
+        <v>128.56</v>
       </c>
       <c r="D24" t="n">
-        <v>0.034249436137332</v>
+        <v>0.0985217465607108</v>
       </c>
       <c r="E24" t="n">
-        <v>-0.0727231875374476</v>
+        <v>0.0052388771600593</v>
       </c>
       <c r="F24" t="n">
-        <v>0.1537601341906624</v>
+        <v>0.2618767177071064</v>
       </c>
       <c r="G24" t="n">
-        <v>0.1883968891811762</v>
+        <v>0.290699751151818</v>
       </c>
       <c r="H24" t="n">
-        <v>0.1904370195892143</v>
+        <v>0.2881576049345313</v>
       </c>
       <c r="I24" t="n">
-        <v>53.22314049586777</v>
+        <v>76.41269841269843</v>
       </c>
       <c r="J24" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K24" t="n">
         <v>48.3</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M24" t="n">
         <v>48.3</v>
       </c>
       <c r="N24" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O24" t="n">
-        <v>78.72340425531915</v>
+        <v>82.97872340425532</v>
       </c>
       <c r="P24" t="n">
-        <v>59.06468085106384</v>
+        <v>63.91574468085106</v>
       </c>
       <c r="Q24" t="b">
         <v>0</v>
@@ -2274,48 +2274,48 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>628.15</v>
+        <v>624.2</v>
       </c>
       <c r="D25" t="n">
-        <v>0.2762088581877284</v>
+        <v>0.1370798797704708</v>
       </c>
       <c r="E25" t="n">
-        <v>0.0336514727661674</v>
+        <v>0.0529689608636978</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.1490788404226497</v>
+        <v>-0.0802328151477196</v>
       </c>
       <c r="G25" t="n">
-        <v>-0.1144420854321359</v>
+        <v>-0.051409781703008</v>
       </c>
       <c r="H25" t="n">
-        <v>-0.1124019550240978</v>
+        <v>-0.0539519279202946</v>
       </c>
       <c r="I25" t="n">
-        <v>66.04046242774567</v>
+        <v>95.49060542797496</v>
       </c>
       <c r="J25" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K25" t="n">
         <v>56.91</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M25" t="n">
         <v>56.91</v>
       </c>
       <c r="N25" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O25" t="n">
         <v>38.29787234042553</v>
       </c>
       <c r="P25" t="n">
-        <v>62.42357446808511</v>
+        <v>54.42357446808511</v>
       </c>
       <c r="Q25" t="b">
         <v>0</v>
@@ -2339,48 +2339,48 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>133.18</v>
+        <v>132.83</v>
       </c>
       <c r="D26" t="n">
-        <v>0.0345684766565681</v>
+        <v>0.0463174478141001</v>
       </c>
       <c r="E26" t="n">
-        <v>-0.0985515094084201</v>
+        <v>-0.078912696761667</v>
       </c>
       <c r="F26" t="n">
-        <v>-0.2795629124743048</v>
+        <v>-0.1930133657351153</v>
       </c>
       <c r="G26" t="n">
-        <v>-0.2449261574837911</v>
+        <v>-0.1641903322904037</v>
       </c>
       <c r="H26" t="n">
-        <v>-0.242886027075753</v>
+        <v>-0.1667324785076903</v>
       </c>
       <c r="I26" t="n">
-        <v>60.82595870206488</v>
+        <v>78.72180451127812</v>
       </c>
       <c r="J26" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="K26" t="n">
         <v>51.54</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M26" t="n">
         <v>51.54</v>
       </c>
       <c r="N26" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="O26" t="n">
-        <v>6.382978723404255</v>
+        <v>10.63829787234042</v>
       </c>
       <c r="P26" t="n">
-        <v>45.89259574468085</v>
+        <v>42.74365957446808</v>
       </c>
       <c r="Q26" t="b">
         <v>0</v>
@@ -2404,48 +2404,48 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>5475</v>
+        <v>5573.4</v>
       </c>
       <c r="D27" t="n">
-        <v>0.080307813733228</v>
+        <v>0.1251438376905218</v>
       </c>
       <c r="E27" t="n">
-        <v>0.0004568296025582</v>
+        <v>0.0136218968809673</v>
       </c>
       <c r="F27" t="n">
-        <v>0.1908905033279679</v>
+        <v>0.1247805291517829</v>
       </c>
       <c r="G27" t="n">
-        <v>0.2255272583184817</v>
+        <v>0.1536035625964945</v>
       </c>
       <c r="H27" t="n">
-        <v>0.2275673887265198</v>
+        <v>0.1510614163792079</v>
       </c>
       <c r="I27" t="n">
-        <v>59.00292284784646</v>
+        <v>82.43720011289864</v>
       </c>
       <c r="J27" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K27" t="n">
         <v>57.69</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M27" t="n">
         <v>57.69</v>
       </c>
       <c r="N27" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O27" t="n">
-        <v>82.97872340425532</v>
+        <v>65.95744680851064</v>
       </c>
       <c r="P27" t="n">
-        <v>71.67174468085106</v>
+        <v>60.26748936170213</v>
       </c>
       <c r="Q27" t="b">
         <v>0</v>
@@ -2469,48 +2469,48 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1779.3</v>
+        <v>1794.9</v>
       </c>
       <c r="D28" t="n">
-        <v>0.139043595160361</v>
+        <v>0.1394020186631119</v>
       </c>
       <c r="E28" t="n">
-        <v>0.187228931740842</v>
+        <v>0.1649143302180686</v>
       </c>
       <c r="F28" t="n">
-        <v>0.5124957497449845</v>
+        <v>0.3569970514855975</v>
       </c>
       <c r="G28" t="n">
-        <v>0.5471325047354982</v>
+        <v>0.3858200849303091</v>
       </c>
       <c r="H28" t="n">
-        <v>0.5491726351435363</v>
+        <v>0.3832779387130225</v>
       </c>
       <c r="I28" t="n">
-        <v>64.161220043573</v>
+        <v>78.84493336154011</v>
       </c>
       <c r="J28" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K28" t="n">
         <v>54.51</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M28" t="n">
         <v>54.51</v>
       </c>
       <c r="N28" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O28" t="n">
-        <v>97.87234042553192</v>
+        <v>89.36170212765957</v>
       </c>
       <c r="P28" t="n">
-        <v>73.37846808510639</v>
+        <v>67.67634042553192</v>
       </c>
       <c r="Q28" t="b">
         <v>0</v>
@@ -2534,54 +2534,54 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>515.05</v>
+        <v>532.8</v>
       </c>
       <c r="D29" t="n">
-        <v>0.0525186471850411</v>
+        <v>0.06432281262485</v>
       </c>
       <c r="E29" t="n">
-        <v>-0.1042608695652175</v>
+        <v>-0.0499286733238231</v>
       </c>
       <c r="F29" t="n">
-        <v>-0.0363891487371376</v>
+        <v>-0.06337347279599199</v>
       </c>
       <c r="G29" t="n">
-        <v>-0.0017523937466238</v>
+        <v>-0.0345504393512804</v>
       </c>
       <c r="H29" t="n">
-        <v>0.0002877366614142</v>
+        <v>-0.037092585568567</v>
       </c>
       <c r="I29" t="n">
-        <v>38.69327073552422</v>
+        <v>60.769535898453</v>
       </c>
       <c r="J29" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="K29" t="n">
         <v>49.42</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M29" t="n">
         <v>49.42</v>
       </c>
       <c r="N29" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="O29" t="n">
-        <v>57.44680851063831</v>
+        <v>42.5531914893617</v>
       </c>
       <c r="P29" t="n">
-        <v>51.25736170212766</v>
+        <v>52.27863829787234</v>
       </c>
       <c r="Q29" t="b">
         <v>0</v>
       </c>
       <c r="R29" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S29" t="b">
         <v>0</v>
@@ -2599,48 +2599,48 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>127.71</v>
+        <v>125.86</v>
       </c>
       <c r="D30" t="n">
-        <v>0.0056697377746279</v>
+        <v>0.0744408400204883</v>
       </c>
       <c r="E30" t="n">
-        <v>0.0069384215091066</v>
+        <v>-0.0391632949080082</v>
       </c>
       <c r="F30" t="n">
-        <v>-0.0556089625083191</v>
+        <v>-0.0263035741915518</v>
       </c>
       <c r="G30" t="n">
-        <v>-0.0209722075178053</v>
+        <v>0.0025194592531597</v>
       </c>
       <c r="H30" t="n">
-        <v>-0.0189320771097672</v>
+        <v>-2.268696412688342e-05</v>
       </c>
       <c r="I30" t="n">
-        <v>70.28556727553382</v>
+        <v>86.39071809344621</v>
       </c>
       <c r="J30" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="K30" t="n">
         <v>52.38</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M30" t="n">
         <v>52.38</v>
       </c>
       <c r="N30" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="O30" t="n">
-        <v>53.19148936170212</v>
+        <v>48.93617021276596</v>
       </c>
       <c r="P30" t="n">
-        <v>59.59029787234042</v>
+        <v>54.73923404255319</v>
       </c>
       <c r="Q30" t="b">
         <v>0</v>
@@ -2664,25 +2664,25 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>39.02</v>
+        <v>39.52</v>
       </c>
       <c r="D31" t="n">
-        <v>0.0077479338842976</v>
+        <v>0.0603702709954387</v>
       </c>
       <c r="E31" t="n">
-        <v>-0.1465441819772527</v>
+        <v>-0.1285556780595369</v>
       </c>
       <c r="F31" t="n">
-        <v>-0.1872526556967297</v>
+        <v>-0.1490094745908698</v>
       </c>
       <c r="G31" t="n">
-        <v>-0.152615900706216</v>
+        <v>-0.1201864411461582</v>
       </c>
       <c r="H31" t="n">
-        <v>-0.1505757702981779</v>
+        <v>-0.1227285873634449</v>
       </c>
       <c r="I31" t="n">
-        <v>56.46766169154233</v>
+        <v>67.56032171581771</v>
       </c>
       <c r="J31" t="n">
         <v>60</v>
@@ -2692,7 +2692,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M31" t="n">
@@ -2702,10 +2702,10 @@
         <v>60</v>
       </c>
       <c r="O31" t="n">
-        <v>21.27659574468085</v>
+        <v>25.53191489361702</v>
       </c>
       <c r="P31" t="n">
-        <v>47.85131914893617</v>
+        <v>48.70238297872341</v>
       </c>
       <c r="Q31" t="b">
         <v>0</v>
@@ -2729,48 +2729,48 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>753</v>
+        <v>754.5</v>
       </c>
       <c r="D32" t="n">
-        <v>0.1313950867703404</v>
+        <v>0.1126677481197462</v>
       </c>
       <c r="E32" t="n">
-        <v>0.008842443729903501</v>
+        <v>0.0319359912466663</v>
       </c>
       <c r="F32" t="n">
-        <v>-0.3045164865613744</v>
+        <v>-0.2673334628083122</v>
       </c>
       <c r="G32" t="n">
-        <v>-0.2698797315708606</v>
+        <v>-0.2385104293636006</v>
       </c>
       <c r="H32" t="n">
-        <v>-0.2678396011628225</v>
+        <v>-0.2410525755808873</v>
       </c>
       <c r="I32" t="n">
-        <v>63.78344741754824</v>
+        <v>92.81883194278906</v>
       </c>
       <c r="J32" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K32" t="n">
         <v>47.86</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M32" t="n">
         <v>47.86</v>
       </c>
       <c r="N32" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O32" t="n">
-        <v>2.127659574468085</v>
+        <v>6.382978723404255</v>
       </c>
       <c r="P32" t="n">
-        <v>51.56953191489362</v>
+        <v>44.42059574468086</v>
       </c>
       <c r="Q32" t="b">
         <v>0</v>
@@ -2794,48 +2794,48 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>577.7</v>
+        <v>586.8</v>
       </c>
       <c r="D33" t="n">
-        <v>0.09943857645827391</v>
+        <v>0.0971300364588201</v>
       </c>
       <c r="E33" t="n">
-        <v>-0.0760495801679327</v>
+        <v>-0.0331191300049431</v>
       </c>
       <c r="F33" t="n">
-        <v>0.0619485294117647</v>
+        <v>0.0909090909090908</v>
       </c>
       <c r="G33" t="n">
-        <v>0.0965852844022785</v>
+        <v>0.1197321243538024</v>
       </c>
       <c r="H33" t="n">
-        <v>0.0986254148103166</v>
+        <v>0.1171899781365157</v>
       </c>
       <c r="I33" t="n">
-        <v>62.85714285714286</v>
+        <v>83.04623753399822</v>
       </c>
       <c r="J33" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K33" t="n">
         <v>49.98</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M33" t="n">
         <v>49.98</v>
       </c>
       <c r="N33" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O33" t="n">
-        <v>61.70212765957447</v>
+        <v>63.82978723404256</v>
       </c>
       <c r="P33" t="n">
-        <v>64.33242553191489</v>
+        <v>56.75795744680852</v>
       </c>
       <c r="Q33" t="b">
         <v>0</v>
@@ -2871,10 +2871,10 @@
         <v>-0.2401052253975846</v>
       </c>
       <c r="G34" t="n">
-        <v>-0.2054684704070708</v>
+        <v>-0.211282191952873</v>
       </c>
       <c r="H34" t="n">
-        <v>-0.2034283399990327</v>
+        <v>-0.2138243381701596</v>
       </c>
       <c r="I34" t="n">
         <v>63.3225806451613</v>
@@ -2887,7 +2887,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M34" t="n">
@@ -2897,10 +2897,10 @@
         <v>80</v>
       </c>
       <c r="O34" t="n">
-        <v>14.8936170212766</v>
+        <v>8.51063829787234</v>
       </c>
       <c r="P34" t="n">
-        <v>55.33072340425532</v>
+        <v>54.05412765957447</v>
       </c>
       <c r="Q34" t="b">
         <v>0</v>
@@ -2924,48 +2924,48 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>118.08</v>
+        <v>119.08</v>
       </c>
       <c r="D35" t="n">
-        <v>0.0816158285243198</v>
+        <v>0.119488577606468</v>
       </c>
       <c r="E35" t="n">
-        <v>-0.0780762023735166</v>
+        <v>-0.0226526592252134</v>
       </c>
       <c r="F35" t="n">
-        <v>0.1400984841170223</v>
+        <v>0.2673478075776927</v>
       </c>
       <c r="G35" t="n">
-        <v>0.174735239107536</v>
+        <v>0.2961708410224043</v>
       </c>
       <c r="H35" t="n">
-        <v>0.1767753695155741</v>
+        <v>0.2936286948051176</v>
       </c>
       <c r="I35" t="n">
-        <v>63.52905569007262</v>
+        <v>85.51776843714175</v>
       </c>
       <c r="J35" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K35" t="n">
         <v>49.07</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M35" t="n">
         <v>49.07</v>
       </c>
       <c r="N35" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O35" t="n">
-        <v>76.59574468085107</v>
+        <v>87.2340425531915</v>
       </c>
       <c r="P35" t="n">
-        <v>66.94714893617021</v>
+        <v>61.07480851063831</v>
       </c>
       <c r="Q35" t="b">
         <v>0</v>
@@ -2989,48 +2989,48 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>499.65</v>
+        <v>506.85</v>
       </c>
       <c r="D36" t="n">
-        <v>0.03974612423265</v>
+        <v>0.0709984152139462</v>
       </c>
       <c r="E36" t="n">
-        <v>-0.1064115174818921</v>
+        <v>-0.0803773927243036</v>
       </c>
       <c r="F36" t="n">
-        <v>0.0966856892010534</v>
+        <v>0.1269594219010561</v>
       </c>
       <c r="G36" t="n">
-        <v>0.1313224441915672</v>
+        <v>0.1557824553457677</v>
       </c>
       <c r="H36" t="n">
-        <v>0.1333625745996053</v>
+        <v>0.153240309128481</v>
       </c>
       <c r="I36" t="n">
-        <v>65.71428571428571</v>
+        <v>89.04415874790385</v>
       </c>
       <c r="J36" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K36" t="n">
         <v>47.8</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M36" t="n">
         <v>47.8</v>
       </c>
       <c r="N36" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O36" t="n">
-        <v>70.21276595744681</v>
+        <v>68.08510638297872</v>
       </c>
       <c r="P36" t="n">
-        <v>65.16255319148937</v>
+        <v>56.73702127659575</v>
       </c>
       <c r="Q36" t="b">
         <v>0</v>
@@ -3054,48 +3054,48 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2340.8</v>
+        <v>2378.3</v>
       </c>
       <c r="D37" t="n">
-        <v>0.1235480464625131</v>
+        <v>0.1140100238887067</v>
       </c>
       <c r="E37" t="n">
-        <v>0.2843191045758808</v>
+        <v>0.2907304895256704</v>
       </c>
       <c r="F37" t="n">
-        <v>0.5624082232011749</v>
+        <v>0.701702919290212</v>
       </c>
       <c r="G37" t="n">
-        <v>0.5970449781916887</v>
+        <v>0.7305259527349236</v>
       </c>
       <c r="H37" t="n">
-        <v>0.5990851085997267</v>
+        <v>0.7279838065176369</v>
       </c>
       <c r="I37" t="n">
-        <v>69.86404833836862</v>
+        <v>91.77667766776686</v>
       </c>
       <c r="J37" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K37" t="n">
         <v>48.59</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M37" t="n">
         <v>48.59</v>
       </c>
       <c r="N37" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O37" t="n">
         <v>100</v>
       </c>
       <c r="P37" t="n">
-        <v>71.43600000000001</v>
+        <v>63.43600000000001</v>
       </c>
       <c r="Q37" t="b">
         <v>0</v>
@@ -3119,48 +3119,48 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>847.3</v>
+        <v>869</v>
       </c>
       <c r="D38" t="n">
-        <v>0.09209254366179009</v>
+        <v>0.1013243774158798</v>
       </c>
       <c r="E38" t="n">
-        <v>-0.0254198297676558</v>
+        <v>0.0216317893251822</v>
       </c>
       <c r="F38" t="n">
-        <v>-0.2526900687952019</v>
+        <v>-0.1861009646904561</v>
       </c>
       <c r="G38" t="n">
-        <v>-0.2180533138046881</v>
+        <v>-0.1572779312457445</v>
       </c>
       <c r="H38" t="n">
-        <v>-0.2160131833966501</v>
+        <v>-0.1598200774630311</v>
       </c>
       <c r="I38" t="n">
-        <v>59.55303169078587</v>
+        <v>88.79518072289162</v>
       </c>
       <c r="J38" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K38" t="n">
         <v>49.87</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M38" t="n">
         <v>49.87</v>
       </c>
       <c r="N38" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O38" t="n">
-        <v>10.63829787234042</v>
+        <v>17.02127659574468</v>
       </c>
       <c r="P38" t="n">
-        <v>54.07565957446808</v>
+        <v>47.35225531914894</v>
       </c>
       <c r="Q38" t="b">
         <v>0</v>
@@ -3184,48 +3184,48 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>3645</v>
+        <v>3735.8</v>
       </c>
       <c r="D39" t="n">
-        <v>0.2211873492361296</v>
+        <v>0.2693849813115869</v>
       </c>
       <c r="E39" t="n">
-        <v>0.1967299231728938</v>
+        <v>0.2945457065631713</v>
       </c>
       <c r="F39" t="n">
-        <v>0.400414937759336</v>
+        <v>0.3830149563157117</v>
       </c>
       <c r="G39" t="n">
-        <v>0.4350516927498498</v>
+        <v>0.4118379897604233</v>
       </c>
       <c r="H39" t="n">
-        <v>0.4370918231578878</v>
+        <v>0.4092958435431366</v>
       </c>
       <c r="I39" t="n">
-        <v>79.90525504021156</v>
+        <v>86.30994447248865</v>
       </c>
       <c r="J39" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="K39" t="n">
         <v>48.69</v>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M39" t="n">
         <v>48.69</v>
       </c>
       <c r="N39" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="O39" t="n">
-        <v>93.61702127659576</v>
+        <v>91.48936170212764</v>
       </c>
       <c r="P39" t="n">
-        <v>66.19940425531915</v>
+        <v>61.77387234042553</v>
       </c>
       <c r="Q39" t="b">
         <v>0</v>
@@ -3249,54 +3249,54 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>214.77</v>
+        <v>220.94</v>
       </c>
       <c r="D40" t="n">
-        <v>0.1859848694019548</v>
+        <v>0.2329241071428571</v>
       </c>
       <c r="E40" t="n">
-        <v>0.0684543057559325</v>
+        <v>0.1164224355735219</v>
       </c>
       <c r="F40" t="n">
-        <v>-0.1079127725856697</v>
+        <v>-0.0255369823137652</v>
       </c>
       <c r="G40" t="n">
-        <v>-0.07327601759515601</v>
+        <v>0.0032860511309463</v>
       </c>
       <c r="H40" t="n">
-        <v>-0.0712358871871179</v>
+        <v>0.0007439049136597</v>
       </c>
       <c r="I40" t="n">
-        <v>74.23405323957812</v>
+        <v>97.42723004694837</v>
       </c>
       <c r="J40" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="K40" t="n">
         <v>45.44</v>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M40" t="n">
         <v>45.44</v>
       </c>
       <c r="N40" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="O40" t="n">
-        <v>44.68085106382978</v>
+        <v>51.06382978723404</v>
       </c>
       <c r="P40" t="n">
-        <v>55.11217021276596</v>
+        <v>52.38876595744681</v>
       </c>
       <c r="Q40" t="b">
         <v>0</v>
       </c>
       <c r="R40" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S40" t="b">
         <v>0</v>
@@ -3314,48 +3314,48 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>807.35</v>
+        <v>828.9</v>
       </c>
       <c r="D41" t="n">
-        <v>-0.0206817079087821</v>
+        <v>0.0168680610930502</v>
       </c>
       <c r="E41" t="n">
-        <v>-0.130245084837059</v>
+        <v>-0.1117183732518887</v>
       </c>
       <c r="F41" t="n">
-        <v>-0.2162411416367342</v>
+        <v>-0.1538383013474887</v>
       </c>
       <c r="G41" t="n">
-        <v>-0.1816043866462204</v>
+        <v>-0.1250152679027771</v>
       </c>
       <c r="H41" t="n">
-        <v>-0.1795642562381824</v>
+        <v>-0.1275574141200638</v>
       </c>
       <c r="I41" t="n">
-        <v>52.45949926362298</v>
+        <v>78.24548991864168</v>
       </c>
       <c r="J41" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="K41" t="n">
         <v>48.05</v>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M41" t="n">
         <v>48.05</v>
       </c>
       <c r="N41" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="O41" t="n">
-        <v>17.02127659574468</v>
+        <v>21.27659574468085</v>
       </c>
       <c r="P41" t="n">
-        <v>46.62425531914894</v>
+        <v>43.47531914893617</v>
       </c>
       <c r="Q41" t="b">
         <v>0</v>
@@ -3379,48 +3379,48 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>626.25</v>
+        <v>619.25</v>
       </c>
       <c r="D42" t="n">
-        <v>0.1777150916784202</v>
+        <v>0.1589930750514692</v>
       </c>
       <c r="E42" t="n">
-        <v>-0.0336393796774939</v>
+        <v>-0.053424029348823</v>
       </c>
       <c r="F42" t="n">
-        <v>-0.1942228512609367</v>
+        <v>-0.1895694280853291</v>
       </c>
       <c r="G42" t="n">
-        <v>-0.1595860962704229</v>
+        <v>-0.1607463946406175</v>
       </c>
       <c r="H42" t="n">
-        <v>-0.1575459658623849</v>
+        <v>-0.1632885408579042</v>
       </c>
       <c r="I42" t="n">
-        <v>69.21022510492179</v>
+        <v>85.28604118993132</v>
       </c>
       <c r="J42" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K42" t="n">
         <v>47.66</v>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M42" t="n">
         <v>47.66</v>
       </c>
       <c r="N42" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O42" t="n">
-        <v>19.14893617021277</v>
+        <v>14.8936170212766</v>
       </c>
       <c r="P42" t="n">
-        <v>54.89378723404256</v>
+        <v>46.04272340425532</v>
       </c>
       <c r="Q42" t="b">
         <v>0</v>
@@ -3444,48 +3444,48 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>415.75</v>
+        <v>425.2</v>
       </c>
       <c r="D43" t="n">
-        <v>0.0340753637607262</v>
+        <v>0.07035871617369401</v>
       </c>
       <c r="E43" t="n">
-        <v>-0.0941279006427715</v>
+        <v>-0.085296332150156</v>
       </c>
       <c r="F43" t="n">
-        <v>-0.1584008097165992</v>
+        <v>-0.07845687039445159</v>
       </c>
       <c r="G43" t="n">
-        <v>-0.1237640547260854</v>
+        <v>-0.0496338369497399</v>
       </c>
       <c r="H43" t="n">
-        <v>-0.1217239243180473</v>
+        <v>-0.0521759831670266</v>
       </c>
       <c r="I43" t="n">
-        <v>52.52621544327933</v>
+        <v>61.8957345971564</v>
       </c>
       <c r="J43" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K43" t="n">
         <v>51.48</v>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M43" t="n">
         <v>51.48</v>
       </c>
       <c r="N43" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O43" t="n">
-        <v>31.91489361702128</v>
+        <v>40.42553191489361</v>
       </c>
       <c r="P43" t="n">
-        <v>50.97497872340426</v>
+        <v>60.67710638297872</v>
       </c>
       <c r="Q43" t="b">
         <v>0</v>
@@ -3509,25 +3509,25 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>266.71</v>
+        <v>275.62</v>
       </c>
       <c r="D44" t="n">
-        <v>0.1354193273733501</v>
+        <v>0.172601574133163</v>
       </c>
       <c r="E44" t="n">
-        <v>0.0015396169733381</v>
+        <v>0.013122587759603</v>
       </c>
       <c r="F44" t="n">
-        <v>-0.141583521081429</v>
+        <v>-0.0887088775004132</v>
       </c>
       <c r="G44" t="n">
-        <v>-0.1069467660909152</v>
+        <v>-0.0598858440557016</v>
       </c>
       <c r="H44" t="n">
-        <v>-0.1049066356828771</v>
+        <v>-0.0624279902729882</v>
       </c>
       <c r="I44" t="n">
-        <v>82.84904323175053</v>
+        <v>99.63751699139104</v>
       </c>
       <c r="J44" t="n">
         <v>60</v>
@@ -3537,7 +3537,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M44" t="n">
@@ -3547,10 +3547,10 @@
         <v>60</v>
       </c>
       <c r="O44" t="n">
-        <v>40.42553191489361</v>
+        <v>36.17021276595745</v>
       </c>
       <c r="P44" t="n">
-        <v>50.96510638297872</v>
+        <v>50.1140425531915</v>
       </c>
       <c r="Q44" t="b">
         <v>0</v>
@@ -3574,25 +3574,25 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>99.70999999999999</v>
+        <v>101.7</v>
       </c>
       <c r="D45" t="n">
-        <v>0.0136220392396053</v>
+        <v>0.0483455313885166</v>
       </c>
       <c r="E45" t="n">
-        <v>-0.0725513905683192</v>
+        <v>-0.1775836972343522</v>
       </c>
       <c r="F45" t="n">
-        <v>-0.3025809610407778</v>
+        <v>-0.2702877233263974</v>
       </c>
       <c r="G45" t="n">
-        <v>-0.267944206050264</v>
+        <v>-0.2414646898816858</v>
       </c>
       <c r="H45" t="n">
-        <v>-0.2659040756422259</v>
+        <v>-0.2440068360989724</v>
       </c>
       <c r="I45" t="n">
-        <v>60.13179571663922</v>
+        <v>89.27503736920779</v>
       </c>
       <c r="J45" t="n">
         <v>60</v>
@@ -3602,7 +3602,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M45" t="n">
@@ -3639,48 +3639,48 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>539.55</v>
+        <v>539.2</v>
       </c>
       <c r="D46" t="n">
-        <v>0.09165402124430951</v>
+        <v>0.0705847314603396</v>
       </c>
       <c r="E46" t="n">
-        <v>-0.0423322683706071</v>
+        <v>-0.0400569699127648</v>
       </c>
       <c r="F46" t="n">
-        <v>-0.1545753682231276</v>
+        <v>-0.1044676963959474</v>
       </c>
       <c r="G46" t="n">
-        <v>-0.1199386132326139</v>
+        <v>-0.0756446629512358</v>
       </c>
       <c r="H46" t="n">
-        <v>-0.1178984828245758</v>
+        <v>-0.0781868091685225</v>
       </c>
       <c r="I46" t="n">
-        <v>65.46063651591288</v>
+        <v>76.57290895632869</v>
       </c>
       <c r="J46" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K46" t="n">
         <v>49.61</v>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M46" t="n">
         <v>49.61</v>
       </c>
       <c r="N46" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O46" t="n">
-        <v>34.04255319148936</v>
+        <v>31.91489361702128</v>
       </c>
       <c r="P46" t="n">
-        <v>58.65251063829788</v>
+        <v>54.22697872340426</v>
       </c>
       <c r="Q46" t="b">
         <v>0</v>
@@ -3704,25 +3704,25 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>1032.65</v>
+        <v>1067.05</v>
       </c>
       <c r="D47" t="n">
-        <v>0.0824990827611511</v>
+        <v>0.0772841998990407</v>
       </c>
       <c r="E47" t="n">
-        <v>0.2714232947549864</v>
+        <v>0.3672240374143121</v>
       </c>
       <c r="F47" t="n">
-        <v>0.2762157819934501</v>
+        <v>0.1856111111111111</v>
       </c>
       <c r="G47" t="n">
-        <v>0.3108525369839638</v>
+        <v>0.2144341445558227</v>
       </c>
       <c r="H47" t="n">
-        <v>0.3128926673920019</v>
+        <v>0.2118919983385361</v>
       </c>
       <c r="I47" t="n">
-        <v>40.1215277777778</v>
+        <v>64.55379482902416</v>
       </c>
       <c r="J47" t="n">
         <v>80</v>
@@ -3732,7 +3732,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M47" t="n">
@@ -3742,10 +3742,10 @@
         <v>80</v>
       </c>
       <c r="O47" t="n">
-        <v>87.2340425531915</v>
+        <v>80.85106382978722</v>
       </c>
       <c r="P47" t="n">
-        <v>68.17880851063831</v>
+        <v>66.90221276595744</v>
       </c>
       <c r="Q47" t="b">
         <v>0</v>
@@ -3769,48 +3769,48 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>14010</v>
+        <v>14500</v>
       </c>
       <c r="D48" t="n">
-        <v>0.0301470588235293</v>
+        <v>0.08322127595995819</v>
       </c>
       <c r="E48" t="n">
-        <v>-0.0087030354489492</v>
+        <v>0.0321019289629154</v>
       </c>
       <c r="F48" t="n">
-        <v>0.0777752134779599</v>
+        <v>0.1622314844501442</v>
       </c>
       <c r="G48" t="n">
-        <v>0.1124119684684736</v>
+        <v>0.1910545178948558</v>
       </c>
       <c r="H48" t="n">
-        <v>0.1144520988765117</v>
+        <v>0.1885123716775691</v>
       </c>
       <c r="I48" t="n">
-        <v>57.06081081081081</v>
+        <v>61.17898594990837</v>
       </c>
       <c r="J48" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K48" t="n">
         <v>50.29</v>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M48" t="n">
         <v>50.29</v>
       </c>
       <c r="N48" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O48" t="n">
-        <v>63.82978723404256</v>
+        <v>74.46808510638297</v>
       </c>
       <c r="P48" t="n">
-        <v>56.88195744680851</v>
+        <v>67.0096170212766</v>
       </c>
       <c r="Q48" t="b">
         <v>0</v>
@@ -3936,57 +3936,57 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>LUMAXTECH</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Lighting</t>
+          <t>Forgings</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1779.3</v>
+        <v>1860.5</v>
       </c>
       <c r="D2" t="n">
-        <v>0.139043595160361</v>
+        <v>0.08648680214903059</v>
       </c>
       <c r="E2" t="n">
-        <v>0.187228931740842</v>
+        <v>0.2765884451763414</v>
       </c>
       <c r="F2" t="n">
-        <v>0.5124957497449845</v>
+        <v>0.5325370675453047</v>
       </c>
       <c r="G2" t="n">
-        <v>0.5471325047354982</v>
+        <v>0.5613601009900163</v>
       </c>
       <c r="H2" t="n">
-        <v>0.5491726351435363</v>
+        <v>0.5588179547727297</v>
       </c>
       <c r="I2" t="n">
-        <v>64.161220043573</v>
+        <v>77.83767595088349</v>
       </c>
       <c r="J2" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K2" t="n">
-        <v>54.51</v>
+        <v>54.83</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M2" t="n">
-        <v>54.51</v>
+        <v>54.83</v>
       </c>
       <c r="N2" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O2" t="n">
         <v>97.87234042553192</v>
       </c>
       <c r="P2" t="n">
-        <v>73.37846808510639</v>
+        <v>69.50646808510639</v>
       </c>
       <c r="Q2" t="b">
         <v>0</v>
@@ -4001,57 +4001,57 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>LUMAXTECH</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Forgings</t>
+          <t>Lighting</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1831.6</v>
+        <v>1794.9</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0490263459335624</v>
+        <v>0.1394020186631119</v>
       </c>
       <c r="E3" t="n">
-        <v>0.2542628227076628</v>
+        <v>0.1649143302180686</v>
       </c>
       <c r="F3" t="n">
-        <v>0.4641087130295762</v>
+        <v>0.3569970514855975</v>
       </c>
       <c r="G3" t="n">
-        <v>0.49874546802009</v>
+        <v>0.3858200849303091</v>
       </c>
       <c r="H3" t="n">
-        <v>0.5007855984281281</v>
+        <v>0.3832779387130225</v>
       </c>
       <c r="I3" t="n">
-        <v>62.95993458708093</v>
+        <v>78.84493336154011</v>
       </c>
       <c r="J3" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K3" t="n">
-        <v>54.83</v>
+        <v>54.51</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M3" t="n">
-        <v>54.83</v>
+        <v>54.51</v>
       </c>
       <c r="N3" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O3" t="n">
-        <v>95.74468085106383</v>
+        <v>89.36170212765957</v>
       </c>
       <c r="P3" t="n">
-        <v>73.08093617021277</v>
+        <v>67.67634042553192</v>
       </c>
       <c r="Q3" t="b">
         <v>0</v>
@@ -4066,57 +4066,57 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>LUMAXIND</t>
+          <t>ZFCVINDIA</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Lighting</t>
+          <t>Brakes/Transmission</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>5475</v>
+        <v>14500</v>
       </c>
       <c r="D4" t="n">
-        <v>0.080307813733228</v>
+        <v>0.08322127595995819</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0004568296025582</v>
+        <v>0.0321019289629154</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1908905033279679</v>
+        <v>0.1622314844501442</v>
       </c>
       <c r="G4" t="n">
-        <v>0.2255272583184817</v>
+        <v>0.1910545178948558</v>
       </c>
       <c r="H4" t="n">
-        <v>0.2275673887265198</v>
+        <v>0.1885123716775691</v>
       </c>
       <c r="I4" t="n">
-        <v>59.00292284784646</v>
+        <v>61.17898594990837</v>
       </c>
       <c r="J4" t="n">
         <v>80</v>
       </c>
       <c r="K4" t="n">
-        <v>57.69</v>
+        <v>50.29</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M4" t="n">
-        <v>57.69</v>
+        <v>50.29</v>
       </c>
       <c r="N4" t="n">
         <v>80</v>
       </c>
       <c r="O4" t="n">
-        <v>82.97872340425532</v>
+        <v>74.46808510638297</v>
       </c>
       <c r="P4" t="n">
-        <v>71.67174468085106</v>
+        <v>67.0096170212766</v>
       </c>
       <c r="Q4" t="b">
         <v>0</v>
@@ -4131,57 +4131,57 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>GNA</t>
+          <t>WHEELS</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Axles</t>
+          <t>Wheels</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>443.7</v>
+        <v>1067.05</v>
       </c>
       <c r="D5" t="n">
-        <v>0.136381098732232</v>
+        <v>0.0772841998990407</v>
       </c>
       <c r="E5" t="n">
-        <v>0.2630230572160545</v>
+        <v>0.3672240374143121</v>
       </c>
       <c r="F5" t="n">
-        <v>0.3515077672860187</v>
+        <v>0.1856111111111111</v>
       </c>
       <c r="G5" t="n">
-        <v>0.3861445222765325</v>
+        <v>0.2144341445558227</v>
       </c>
       <c r="H5" t="n">
-        <v>0.3881846526845706</v>
+        <v>0.2118919983385361</v>
       </c>
       <c r="I5" t="n">
-        <v>65.84471842719094</v>
+        <v>64.55379482902416</v>
       </c>
       <c r="J5" t="n">
         <v>80</v>
       </c>
       <c r="K5" t="n">
-        <v>54.47</v>
+        <v>46.83</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M5" t="n">
-        <v>54.47</v>
+        <v>46.83</v>
       </c>
       <c r="N5" t="n">
         <v>80</v>
       </c>
       <c r="O5" t="n">
-        <v>89.36170212765957</v>
+        <v>80.85106382978722</v>
       </c>
       <c r="P5" t="n">
-        <v>71.66034042553191</v>
+        <v>66.90221276595744</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
@@ -4196,57 +4196,57 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SANSERA</t>
+          <t>GNA</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Forgings</t>
+          <t>Axles</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>2340.8</v>
+        <v>435.9</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1235480464625131</v>
+        <v>0.1480115880958652</v>
       </c>
       <c r="E6" t="n">
-        <v>0.2843191045758808</v>
+        <v>0.2301396923945251</v>
       </c>
       <c r="F6" t="n">
-        <v>0.5624082232011749</v>
+        <v>0.4122792807387008</v>
       </c>
       <c r="G6" t="n">
-        <v>0.5970449781916887</v>
+        <v>0.4411023141834124</v>
       </c>
       <c r="H6" t="n">
-        <v>0.5990851085997267</v>
+        <v>0.4385601679661257</v>
       </c>
       <c r="I6" t="n">
-        <v>69.86404833836862</v>
+        <v>83.44594594594594</v>
       </c>
       <c r="J6" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K6" t="n">
-        <v>48.59</v>
+        <v>54.47</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M6" t="n">
-        <v>48.59</v>
+        <v>54.47</v>
       </c>
       <c r="N6" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O6" t="n">
-        <v>100</v>
+        <v>93.61702127659576</v>
       </c>
       <c r="P6" t="n">
-        <v>71.43600000000001</v>
+        <v>64.51140425531915</v>
       </c>
       <c r="Q6" t="b">
         <v>0</v>
@@ -4261,57 +4261,57 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>WHEELS</t>
+          <t>JAMNAAUTO</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Wheels</t>
+          <t>Suspension</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1032.65</v>
+        <v>128.56</v>
       </c>
       <c r="D7" t="n">
-        <v>0.0824990827611511</v>
+        <v>0.0985217465607108</v>
       </c>
       <c r="E7" t="n">
-        <v>0.2714232947549864</v>
+        <v>0.0052388771600593</v>
       </c>
       <c r="F7" t="n">
-        <v>0.2762157819934501</v>
+        <v>0.2618767177071064</v>
       </c>
       <c r="G7" t="n">
-        <v>0.3108525369839638</v>
+        <v>0.290699751151818</v>
       </c>
       <c r="H7" t="n">
-        <v>0.3128926673920019</v>
+        <v>0.2881576049345313</v>
       </c>
       <c r="I7" t="n">
-        <v>40.1215277777778</v>
+        <v>76.41269841269843</v>
       </c>
       <c r="J7" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K7" t="n">
-        <v>46.83</v>
+        <v>48.3</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M7" t="n">
-        <v>46.83</v>
+        <v>48.3</v>
       </c>
       <c r="N7" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O7" t="n">
-        <v>87.2340425531915</v>
+        <v>82.97872340425532</v>
       </c>
       <c r="P7" t="n">
-        <v>68.17880851063831</v>
+        <v>63.91574468085106</v>
       </c>
       <c r="Q7" t="b">
         <v>0</v>
@@ -4326,57 +4326,57 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>DIVGIITTS</t>
+          <t>CRAFTSMAN</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Transmission</t>
+          <t>Castings</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>777.75</v>
+        <v>7691</v>
       </c>
       <c r="D8" t="n">
-        <v>0.1547884187082404</v>
+        <v>0.1219547775346463</v>
       </c>
       <c r="E8" t="n">
-        <v>0.3238297872340425</v>
+        <v>-0.0099124613800205</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1768933948702429</v>
+        <v>0.1446643845810389</v>
       </c>
       <c r="G8" t="n">
-        <v>0.2115301498607567</v>
+        <v>0.1734874180257505</v>
       </c>
       <c r="H8" t="n">
-        <v>0.2135702802687947</v>
+        <v>0.1709452718084638</v>
       </c>
       <c r="I8" t="n">
-        <v>65.57153965785382</v>
+        <v>78.74396135265701</v>
       </c>
       <c r="J8" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K8" t="n">
-        <v>49.92</v>
+        <v>54.65</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M8" t="n">
-        <v>49.92</v>
+        <v>54.65</v>
       </c>
       <c r="N8" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O8" t="n">
-        <v>80.85106382978722</v>
+        <v>70.21276595744681</v>
       </c>
       <c r="P8" t="n">
-        <v>68.13821276595745</v>
+        <v>63.90255319148936</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
@@ -4391,57 +4391,57 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>MOTHERSON</t>
+          <t>SANSERA</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Forgings</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>123.55</v>
+        <v>2378.3</v>
       </c>
       <c r="D9" t="n">
-        <v>0.0666493999827333</v>
+        <v>0.1140100238887067</v>
       </c>
       <c r="E9" t="n">
-        <v>0.0750021752371008</v>
+        <v>0.2907304895256704</v>
       </c>
       <c r="F9" t="n">
-        <v>0.1023376159885796</v>
+        <v>0.701702919290212</v>
       </c>
       <c r="G9" t="n">
-        <v>0.1369743709790933</v>
+        <v>0.7305259527349236</v>
       </c>
       <c r="H9" t="n">
-        <v>0.1390145013871314</v>
+        <v>0.7279838065176369</v>
       </c>
       <c r="I9" t="n">
-        <v>64.21167484997272</v>
+        <v>91.77667766776686</v>
       </c>
       <c r="J9" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K9" t="n">
-        <v>51.57</v>
+        <v>48.59</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M9" t="n">
-        <v>51.57</v>
+        <v>48.59</v>
       </c>
       <c r="N9" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O9" t="n">
-        <v>72.3404255319149</v>
+        <v>100</v>
       </c>
       <c r="P9" t="n">
-        <v>67.09608510638299</v>
+        <v>63.43600000000001</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -4456,63 +4456,63 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CRAFTSMAN</t>
+          <t>ASKAUTOLTD</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Castings</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>7433.5</v>
+        <v>436.8</v>
       </c>
       <c r="D10" t="n">
-        <v>0.07467110018794269</v>
+        <v>0.043602914824991</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.0329148507122877</v>
+        <v>-0.0586206896551724</v>
       </c>
       <c r="F10" t="n">
-        <v>0.0924388272466749</v>
+        <v>-0.192680898253396</v>
       </c>
       <c r="G10" t="n">
-        <v>0.1270755822371887</v>
+        <v>-0.1638578648086844</v>
       </c>
       <c r="H10" t="n">
-        <v>0.1291157126452268</v>
+        <v>-0.1664000110259711</v>
       </c>
       <c r="I10" t="n">
-        <v>66.53763440860214</v>
+        <v>40.02509410288583</v>
       </c>
       <c r="J10" t="n">
         <v>80</v>
       </c>
       <c r="K10" t="n">
-        <v>54.65</v>
+        <v>71.28</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M10" t="n">
-        <v>54.65</v>
+        <v>71.28</v>
       </c>
       <c r="N10" t="n">
         <v>80</v>
       </c>
       <c r="O10" t="n">
-        <v>65.95744680851064</v>
+        <v>12.76595744680851</v>
       </c>
       <c r="P10" t="n">
-        <v>67.05148936170212</v>
+        <v>63.0651914893617</v>
       </c>
       <c r="Q10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S10" t="b">
         <v>0</v>
@@ -4521,57 +4521,57 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>RICOAUTO</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Castings</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>118.08</v>
+        <v>593.85</v>
       </c>
       <c r="D11" t="n">
-        <v>0.0816158285243198</v>
+        <v>0.1907960697814317</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.0780762023735166</v>
+        <v>0.2906976744186047</v>
       </c>
       <c r="F11" t="n">
-        <v>0.1400984841170223</v>
+        <v>0.4650302207968422</v>
       </c>
       <c r="G11" t="n">
-        <v>0.174735239107536</v>
+        <v>0.4938532542415538</v>
       </c>
       <c r="H11" t="n">
-        <v>0.1767753695155741</v>
+        <v>0.4913111080242671</v>
       </c>
       <c r="I11" t="n">
-        <v>63.52905569007262</v>
+        <v>88.80829015544036</v>
       </c>
       <c r="J11" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K11" t="n">
-        <v>49.07</v>
+        <v>49.66</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M11" t="n">
-        <v>49.07</v>
+        <v>49.66</v>
       </c>
       <c r="N11" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O11" t="n">
-        <v>76.59574468085107</v>
+        <v>95.74468085106383</v>
       </c>
       <c r="P11" t="n">
-        <v>66.94714893617021</v>
+        <v>63.01293617021277</v>
       </c>
       <c r="Q11" t="b">
         <v>0</v>
@@ -4586,57 +4586,57 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>BHARATSE</t>
+          <t>BHARATGEAR</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Seating</t>
+          <t>Gears</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>184.81</v>
+        <v>112.64</v>
       </c>
       <c r="D12" t="n">
-        <v>0.1359641035097425</v>
+        <v>0.1673748574981863</v>
       </c>
       <c r="E12" t="n">
-        <v>0.140098704503393</v>
+        <v>0.069807199164213</v>
       </c>
       <c r="F12" t="n">
-        <v>0.0944569465829681</v>
+        <v>0.2639138240574505</v>
       </c>
       <c r="G12" t="n">
-        <v>0.1290937015734818</v>
+        <v>0.2927368575021621</v>
       </c>
       <c r="H12" t="n">
-        <v>0.1311338319815199</v>
+        <v>0.2901947112848755</v>
       </c>
       <c r="I12" t="n">
-        <v>69.71713810316139</v>
+        <v>94.62837837837836</v>
       </c>
       <c r="J12" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K12" t="n">
-        <v>52.61</v>
+        <v>51.91</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M12" t="n">
-        <v>52.61</v>
+        <v>51.91</v>
       </c>
       <c r="N12" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O12" t="n">
-        <v>68.08510638297872</v>
+        <v>85.1063829787234</v>
       </c>
       <c r="P12" t="n">
-        <v>66.66102127659575</v>
+        <v>61.78527659574468</v>
       </c>
       <c r="Q12" t="b">
         <v>0</v>
@@ -4651,57 +4651,57 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>FIEMIND</t>
+          <t>SHRIPISTON</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Lighting</t>
+          <t>Engine/Parts</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>2241.3</v>
+        <v>3735.8</v>
       </c>
       <c r="D13" t="n">
-        <v>0.1188598242811502</v>
+        <v>0.2693849813115869</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.0063838276366536</v>
+        <v>0.2945457065631713</v>
       </c>
       <c r="F13" t="n">
-        <v>0.1097742127153893</v>
+        <v>0.3830149563157117</v>
       </c>
       <c r="G13" t="n">
-        <v>0.1444109677059031</v>
+        <v>0.4118379897604233</v>
       </c>
       <c r="H13" t="n">
-        <v>0.1464510981139412</v>
+        <v>0.4092958435431366</v>
       </c>
       <c r="I13" t="n">
-        <v>62.86926717806433</v>
+        <v>86.30994447248865</v>
       </c>
       <c r="J13" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K13" t="n">
-        <v>49.06</v>
+        <v>48.69</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M13" t="n">
-        <v>49.06</v>
+        <v>48.69</v>
       </c>
       <c r="N13" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O13" t="n">
-        <v>74.46808510638297</v>
+        <v>91.48936170212764</v>
       </c>
       <c r="P13" t="n">
-        <v>66.51761702127659</v>
+        <v>61.77387234042553</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
@@ -4716,57 +4716,57 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SHRIPISTON</t>
+          <t>RICOAUTO</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Engine/Parts</t>
+          <t>Castings</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>3645</v>
+        <v>119.08</v>
       </c>
       <c r="D14" t="n">
-        <v>0.2211873492361296</v>
+        <v>0.119488577606468</v>
       </c>
       <c r="E14" t="n">
-        <v>0.1967299231728938</v>
+        <v>-0.0226526592252134</v>
       </c>
       <c r="F14" t="n">
-        <v>0.400414937759336</v>
+        <v>0.2673478075776927</v>
       </c>
       <c r="G14" t="n">
-        <v>0.4350516927498498</v>
+        <v>0.2961708410224043</v>
       </c>
       <c r="H14" t="n">
-        <v>0.4370918231578878</v>
+        <v>0.2936286948051176</v>
       </c>
       <c r="I14" t="n">
-        <v>79.90525504021156</v>
+        <v>85.51776843714175</v>
       </c>
       <c r="J14" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="K14" t="n">
-        <v>48.69</v>
+        <v>49.07</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M14" t="n">
-        <v>48.69</v>
+        <v>49.07</v>
       </c>
       <c r="N14" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="O14" t="n">
-        <v>93.61702127659576</v>
+        <v>87.2340425531915</v>
       </c>
       <c r="P14" t="n">
-        <v>66.19940425531915</v>
+        <v>61.07480851063831</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
@@ -4781,63 +4781,63 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>SUPRAJIT</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Cables</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>585.7</v>
+        <v>425.2</v>
       </c>
       <c r="D15" t="n">
-        <v>0.1665006970722964</v>
+        <v>0.07035871617369401</v>
       </c>
       <c r="E15" t="n">
-        <v>0.2814790504321192</v>
+        <v>-0.085296332150156</v>
       </c>
       <c r="F15" t="n">
-        <v>0.390055773110241</v>
+        <v>-0.07845687039445159</v>
       </c>
       <c r="G15" t="n">
-        <v>0.4246925281007547</v>
+        <v>-0.0496338369497399</v>
       </c>
       <c r="H15" t="n">
-        <v>0.4267326585087928</v>
+        <v>-0.0521759831670266</v>
       </c>
       <c r="I15" t="n">
-        <v>73.66911061523747</v>
+        <v>61.8957345971564</v>
       </c>
       <c r="J15" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K15" t="n">
-        <v>49.66</v>
+        <v>51.48</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M15" t="n">
-        <v>49.66</v>
+        <v>51.48</v>
       </c>
       <c r="N15" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O15" t="n">
-        <v>91.48936170212764</v>
+        <v>40.42553191489361</v>
       </c>
       <c r="P15" t="n">
-        <v>66.16187234042553</v>
+        <v>60.67710638297872</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
       </c>
       <c r="R15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S15" t="b">
         <v>0</v>
@@ -4846,57 +4846,57 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>BHARATGEAR</t>
+          <t>MOTHERSON</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Gears</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>111.65</v>
+        <v>125.03</v>
       </c>
       <c r="D16" t="n">
-        <v>0.1548407116259826</v>
+        <v>0.1188366890380312</v>
       </c>
       <c r="E16" t="n">
-        <v>0.0538984330753258</v>
+        <v>0.0892063768620958</v>
       </c>
       <c r="F16" t="n">
-        <v>0.2647258722247394</v>
+        <v>0.1698166167664672</v>
       </c>
       <c r="G16" t="n">
-        <v>0.2993626272152532</v>
+        <v>0.1986396502111788</v>
       </c>
       <c r="H16" t="n">
-        <v>0.3014027576232913</v>
+        <v>0.1960975039938921</v>
       </c>
       <c r="I16" t="n">
-        <v>71.96802646085999</v>
+        <v>81.61648177496039</v>
       </c>
       <c r="J16" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="K16" t="n">
-        <v>51.91</v>
+        <v>51.57</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="M16" t="n">
-        <v>51.91</v>
+        <v>51.57</v>
       </c>
       <c r="N16" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="O16" t="n">
-        <v>85.1063829787234</v>
+        <v>78.72340425531915</v>
       </c>
       <c r="P16" t="n">
-        <v>65.78527659574468</v>
+        <v>60.37268085106383</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
chore: auto-refresh NSE data and pipeline outputs (2026-04-20)
</commit_message>
<xml_diff>
--- a/working-sector/output/auto_components_comprehensive_report.xlsx
+++ b/working-sector/output/auto_components_comprehensive_report.xlsx
@@ -435,7 +435,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
     </row>
@@ -447,7 +447,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
     </row>
@@ -779,25 +779,25 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1860.5</v>
+        <v>1866.2</v>
       </c>
       <c r="D2" t="n">
-        <v>0.08648680214903059</v>
+        <v>0.0903885480572597</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2765884451763414</v>
+        <v>0.3187760582291006</v>
       </c>
       <c r="F2" t="n">
-        <v>0.5325370675453047</v>
+        <v>0.5392609699769053</v>
       </c>
       <c r="G2" t="n">
-        <v>0.5613601009900163</v>
+        <v>0.5625353685067882</v>
       </c>
       <c r="H2" t="n">
-        <v>0.5588179547727297</v>
+        <v>0.5613147775893503</v>
       </c>
       <c r="I2" t="n">
-        <v>77.83767595088349</v>
+        <v>78.20965842167257</v>
       </c>
       <c r="J2" t="n">
         <v>70</v>
@@ -807,7 +807,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M2" t="n">
@@ -844,48 +844,48 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1097.8</v>
+        <v>1129.4</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0560846560846559</v>
+        <v>0.058481724461106</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.0728040540540541</v>
+        <v>-0.0220798337518399</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.1458803392204154</v>
+        <v>-0.1304280874653525</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.1170573057757038</v>
+        <v>-0.1071536889354696</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.1195994519929904</v>
+        <v>-0.1083742798529074</v>
       </c>
       <c r="I3" t="n">
-        <v>63.20830007980843</v>
+        <v>67.32813607370656</v>
       </c>
       <c r="J3" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K3" t="n">
         <v>49.36</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M3" t="n">
         <v>49.36</v>
       </c>
       <c r="N3" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O3" t="n">
-        <v>27.65957446808511</v>
+        <v>29.78723404255319</v>
       </c>
       <c r="P3" t="n">
-        <v>49.27591489361702</v>
+        <v>57.70144680851064</v>
       </c>
       <c r="Q3" t="b">
         <v>0</v>
@@ -909,25 +909,25 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>37505</v>
+        <v>37790</v>
       </c>
       <c r="D4" t="n">
-        <v>0.244566119130579</v>
+        <v>0.2435011516946363</v>
       </c>
       <c r="E4" t="n">
-        <v>0.01818922220714</v>
+        <v>0.035058887975897</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.0219063763202503</v>
+        <v>-0.0093065932625507</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0069166571244612</v>
+        <v>0.0139678052673321</v>
       </c>
       <c r="H4" t="n">
-        <v>0.0043745109071745</v>
+        <v>0.0127472143498942</v>
       </c>
       <c r="I4" t="n">
-        <v>92.85714285714286</v>
+        <v>93.05092812946216</v>
       </c>
       <c r="J4" t="n">
         <v>60</v>
@@ -937,7 +937,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M4" t="n">
@@ -974,25 +974,25 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>330</v>
+        <v>329.7</v>
       </c>
       <c r="D5" t="n">
-        <v>0.0932582408481033</v>
+        <v>0.0893771683462745</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.040976460331299</v>
+        <v>-0.0368098159509203</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.1506884570840304</v>
+        <v>-0.1562380038387716</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.1218654236393188</v>
+        <v>-0.1329636053088887</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.1244075698566055</v>
+        <v>-0.1341841962263266</v>
       </c>
       <c r="I5" t="n">
-        <v>87.65652951699467</v>
+        <v>87.18861209964415</v>
       </c>
       <c r="J5" t="n">
         <v>60</v>
@@ -1002,7 +1002,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M5" t="n">
@@ -1012,10 +1012,10 @@
         <v>60</v>
       </c>
       <c r="O5" t="n">
-        <v>23.40425531914894</v>
+        <v>21.27659574468085</v>
       </c>
       <c r="P5" t="n">
-        <v>49.12885106382979</v>
+        <v>48.70331914893617</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
@@ -1039,48 +1039,48 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>125.03</v>
+        <v>123.19</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1188366890380312</v>
+        <v>0.1039519670221345</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0892063768620958</v>
+        <v>0.09667942668921919</v>
       </c>
       <c r="F6" t="n">
-        <v>0.1698166167664672</v>
+        <v>0.1660198769522005</v>
       </c>
       <c r="G6" t="n">
-        <v>0.1986396502111788</v>
+        <v>0.1892942754820834</v>
       </c>
       <c r="H6" t="n">
-        <v>0.1960975039938921</v>
+        <v>0.1880736845646455</v>
       </c>
       <c r="I6" t="n">
-        <v>81.61648177496039</v>
+        <v>77.11889787361486</v>
       </c>
       <c r="J6" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K6" t="n">
         <v>51.57</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M6" t="n">
         <v>51.57</v>
       </c>
       <c r="N6" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O6" t="n">
-        <v>78.72340425531915</v>
+        <v>76.59574468085107</v>
       </c>
       <c r="P6" t="n">
-        <v>60.37268085106383</v>
+        <v>63.94714893617022</v>
       </c>
       <c r="Q6" t="b">
         <v>0</v>
@@ -1104,25 +1104,25 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2790.2</v>
+        <v>2873.1</v>
       </c>
       <c r="D7" t="n">
-        <v>0.1028458498023714</v>
+        <v>0.1323454065345051</v>
       </c>
       <c r="E7" t="n">
-        <v>0.1910697515580979</v>
+        <v>0.2053616378587011</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.09952881946685591</v>
+        <v>-0.0722058965996059</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.07070578602214431</v>
+        <v>-0.048931498069723</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.073247932239431</v>
+        <v>-0.0501520889871609</v>
       </c>
       <c r="I7" t="n">
-        <v>89.37950937950943</v>
+        <v>91.42990218910111</v>
       </c>
       <c r="J7" t="n">
         <v>60</v>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M7" t="n">
@@ -1142,10 +1142,10 @@
         <v>60</v>
       </c>
       <c r="O7" t="n">
-        <v>34.04255319148936</v>
+        <v>38.29787234042553</v>
       </c>
       <c r="P7" t="n">
-        <v>50.30051063829788</v>
+        <v>51.15157446808512</v>
       </c>
       <c r="Q7" t="b">
         <v>0</v>
@@ -1169,48 +1169,48 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>593.85</v>
+        <v>576.55</v>
       </c>
       <c r="D8" t="n">
-        <v>0.1907960697814317</v>
+        <v>0.1388641975308642</v>
       </c>
       <c r="E8" t="n">
-        <v>0.2906976744186047</v>
+        <v>0.2879481737964928</v>
       </c>
       <c r="F8" t="n">
-        <v>0.4650302207968422</v>
+        <v>0.4002428658166361</v>
       </c>
       <c r="G8" t="n">
-        <v>0.4938532542415538</v>
+        <v>0.423517264346519</v>
       </c>
       <c r="H8" t="n">
-        <v>0.4913111080242671</v>
+        <v>0.4222966734290811</v>
       </c>
       <c r="I8" t="n">
-        <v>88.80829015544036</v>
+        <v>79.32736809626651</v>
       </c>
       <c r="J8" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K8" t="n">
         <v>49.66</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M8" t="n">
         <v>49.66</v>
       </c>
       <c r="N8" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O8" t="n">
-        <v>95.74468085106383</v>
+        <v>91.48936170212764</v>
       </c>
       <c r="P8" t="n">
-        <v>63.01293617021277</v>
+        <v>66.16187234042553</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
@@ -1234,25 +1234,25 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>445.4</v>
+        <v>441.4</v>
       </c>
       <c r="D9" t="n">
-        <v>0.0618667302419835</v>
+        <v>0.0488297493168585</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.1241765804738964</v>
+        <v>-0.1345946475835703</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.0432821394050049</v>
+        <v>-0.0667089544349297</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.0144591059602933</v>
+        <v>-0.0434345559050468</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.0170012521775799</v>
+        <v>-0.0446551468224847</v>
       </c>
       <c r="I9" t="n">
-        <v>77.31023102310225</v>
+        <v>72.52321981424143</v>
       </c>
       <c r="J9" t="n">
         <v>70</v>
@@ -1262,7 +1262,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M9" t="n">
@@ -1272,10 +1272,10 @@
         <v>70</v>
       </c>
       <c r="O9" t="n">
-        <v>44.68085106382978</v>
+        <v>40.42553191489361</v>
       </c>
       <c r="P9" t="n">
-        <v>58.31217021276596</v>
+        <v>57.46110638297873</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -1299,25 +1299,25 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>139855</v>
+        <v>139225</v>
       </c>
       <c r="D10" t="n">
-        <v>0.0713164043050289</v>
+        <v>0.0916611126357469</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.0208975077009241</v>
+        <v>-0.0267048830787514</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.0413339274085752</v>
+        <v>-0.0452269921821423</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.0125108939638636</v>
+        <v>-0.0219525936522594</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.0150530401811502</v>
+        <v>-0.0231731845696973</v>
       </c>
       <c r="I10" t="n">
-        <v>76.35730858468678</v>
+        <v>74.18845807033364</v>
       </c>
       <c r="J10" t="n">
         <v>70</v>
@@ -1327,7 +1327,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M10" t="n">
@@ -1337,10 +1337,10 @@
         <v>70</v>
       </c>
       <c r="O10" t="n">
-        <v>46.80851063829788</v>
+        <v>44.68085106382978</v>
       </c>
       <c r="P10" t="n">
-        <v>57.12570212765957</v>
+        <v>56.70017021276595</v>
       </c>
       <c r="Q10" t="b">
         <v>0</v>
@@ -1376,10 +1376,10 @@
         <v>-0.0042030657656173</v>
       </c>
       <c r="G11" t="n">
-        <v>0.0246199676790942</v>
+        <v>0.0190713327642655</v>
       </c>
       <c r="H11" t="n">
-        <v>0.0220778214618075</v>
+        <v>0.0178507418468276</v>
       </c>
       <c r="I11" t="n">
         <v>27.6054590570719</v>
@@ -1392,7 +1392,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M11" t="n">
@@ -1429,25 +1429,25 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>436.8</v>
+        <v>438.25</v>
       </c>
       <c r="D12" t="n">
-        <v>0.043602914824991</v>
+        <v>0.0709921798631476</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.0586206896551724</v>
+        <v>-0.0441657579062159</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.192680898253396</v>
+        <v>-0.1695091908281221</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.1638578648086844</v>
+        <v>-0.1462347922982392</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.1664000110259711</v>
+        <v>-0.147455383215677</v>
       </c>
       <c r="I12" t="n">
-        <v>40.02509410288583</v>
+        <v>42.13075060532687</v>
       </c>
       <c r="J12" t="n">
         <v>80</v>
@@ -1457,7 +1457,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M12" t="n">
@@ -1467,10 +1467,10 @@
         <v>80</v>
       </c>
       <c r="O12" t="n">
-        <v>12.76595744680851</v>
+        <v>19.14893617021277</v>
       </c>
       <c r="P12" t="n">
-        <v>63.0651914893617</v>
+        <v>64.34178723404256</v>
       </c>
       <c r="Q12" t="b">
         <v>1</v>
@@ -1494,48 +1494,48 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1881.9</v>
+        <v>1787.5</v>
       </c>
       <c r="D13" t="n">
-        <v>0.130134518376171</v>
+        <v>0.0724785504289913</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.0376374328816159</v>
+        <v>-0.06944661356655731</v>
       </c>
       <c r="F13" t="n">
-        <v>0.083294957402717</v>
+        <v>0.0347921732082898</v>
       </c>
       <c r="G13" t="n">
-        <v>0.1121179908474286</v>
+        <v>0.0580665717381727</v>
       </c>
       <c r="H13" t="n">
-        <v>0.109575844630142</v>
+        <v>0.0568459808207348</v>
       </c>
       <c r="I13" t="n">
-        <v>87.3327386262266</v>
+        <v>72.14443625644805</v>
       </c>
       <c r="J13" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="K13" t="n">
         <v>58.77</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M13" t="n">
         <v>58.77</v>
       </c>
       <c r="N13" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="O13" t="n">
         <v>61.70212765957447</v>
       </c>
       <c r="P13" t="n">
-        <v>59.8484255319149</v>
+        <v>55.8484255319149</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
@@ -1559,48 +1559,48 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>624.95</v>
+        <v>613.35</v>
       </c>
       <c r="D14" t="n">
-        <v>0.1355501044789679</v>
+        <v>0.107729817590753</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.0080945956670104</v>
+        <v>0.0018784710878796</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.2737783975364591</v>
+        <v>-0.2613800578034682</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.2449553640917475</v>
+        <v>-0.2381056592735853</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.2474975103090342</v>
+        <v>-0.2393262501910231</v>
       </c>
       <c r="I14" t="n">
-        <v>80.68702290076334</v>
+        <v>76.18933205189811</v>
       </c>
       <c r="J14" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K14" t="n">
         <v>54.64</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M14" t="n">
         <v>54.64</v>
       </c>
       <c r="N14" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O14" t="n">
-        <v>2.127659574468085</v>
+        <v>4.25531914893617</v>
       </c>
       <c r="P14" t="n">
-        <v>46.28153191489362</v>
+        <v>50.70706382978724</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
@@ -1624,25 +1624,25 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>112.64</v>
+        <v>108.05</v>
       </c>
       <c r="D15" t="n">
-        <v>0.1673748574981863</v>
+        <v>0.101427115188583</v>
       </c>
       <c r="E15" t="n">
-        <v>0.069807199164213</v>
+        <v>-0.0019397746166636</v>
       </c>
       <c r="F15" t="n">
-        <v>0.2639138240574505</v>
+        <v>0.2033634034970486</v>
       </c>
       <c r="G15" t="n">
-        <v>0.2927368575021621</v>
+        <v>0.2266378020269315</v>
       </c>
       <c r="H15" t="n">
-        <v>0.2901947112848755</v>
+        <v>0.2254172111094936</v>
       </c>
       <c r="I15" t="n">
-        <v>94.62837837837836</v>
+        <v>81.924539338988</v>
       </c>
       <c r="J15" t="n">
         <v>60</v>
@@ -1652,7 +1652,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M15" t="n">
@@ -1662,10 +1662,10 @@
         <v>60</v>
       </c>
       <c r="O15" t="n">
-        <v>85.1063829787234</v>
+        <v>82.97872340425532</v>
       </c>
       <c r="P15" t="n">
-        <v>61.78527659574468</v>
+        <v>61.35974468085107</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
@@ -1689,25 +1689,25 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>183.46</v>
+        <v>180.19</v>
       </c>
       <c r="D16" t="n">
-        <v>0.1723432807208127</v>
+        <v>0.132985412474849</v>
       </c>
       <c r="E16" t="n">
-        <v>0.156819471593417</v>
+        <v>0.1331279084391898</v>
       </c>
       <c r="F16" t="n">
-        <v>0.0260052569766791</v>
+        <v>0.001333703806613</v>
       </c>
       <c r="G16" t="n">
-        <v>0.0548282904213907</v>
+        <v>0.0246081023364959</v>
       </c>
       <c r="H16" t="n">
-        <v>0.052286144204104</v>
+        <v>0.023387511419058</v>
       </c>
       <c r="I16" t="n">
-        <v>92.31990474300456</v>
+        <v>86.69399925456577</v>
       </c>
       <c r="J16" t="n">
         <v>60</v>
@@ -1717,7 +1717,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M16" t="n">
@@ -1727,10 +1727,10 @@
         <v>60</v>
       </c>
       <c r="O16" t="n">
-        <v>59.57446808510638</v>
+        <v>57.44680851063831</v>
       </c>
       <c r="P16" t="n">
-        <v>56.95889361702128</v>
+        <v>56.53336170212766</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>
@@ -1754,25 +1754,25 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>7691</v>
+        <v>7721.5</v>
       </c>
       <c r="D17" t="n">
-        <v>0.1219547775346463</v>
+        <v>0.1171151620370369</v>
       </c>
       <c r="E17" t="n">
-        <v>-0.0099124613800205</v>
+        <v>0.0154523934771173</v>
       </c>
       <c r="F17" t="n">
-        <v>0.1446643845810389</v>
+        <v>0.1366011628762788</v>
       </c>
       <c r="G17" t="n">
-        <v>0.1734874180257505</v>
+        <v>0.1598755614061617</v>
       </c>
       <c r="H17" t="n">
-        <v>0.1709452718084638</v>
+        <v>0.1586549704887239</v>
       </c>
       <c r="I17" t="n">
-        <v>78.74396135265701</v>
+        <v>79.25343811394892</v>
       </c>
       <c r="J17" t="n">
         <v>70</v>
@@ -1782,7 +1782,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M17" t="n">
@@ -1819,25 +1819,25 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>776.1</v>
+        <v>755.45</v>
       </c>
       <c r="D18" t="n">
-        <v>0.1390621560137961</v>
+        <v>0.0715602836879434</v>
       </c>
       <c r="E18" t="n">
-        <v>0.3027276542173731</v>
+        <v>0.2559434746467166</v>
       </c>
       <c r="F18" t="n">
-        <v>0.1537946926336133</v>
+        <v>0.142976019366064</v>
       </c>
       <c r="G18" t="n">
-        <v>0.1826177260783249</v>
+        <v>0.1662504178959469</v>
       </c>
       <c r="H18" t="n">
-        <v>0.1800755798610382</v>
+        <v>0.1650298269785091</v>
       </c>
       <c r="I18" t="n">
-        <v>92.18421052631584</v>
+        <v>83.14740090197014</v>
       </c>
       <c r="J18" t="n">
         <v>60</v>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M18" t="n">
@@ -1884,48 +1884,48 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2384.4</v>
+        <v>2358.1</v>
       </c>
       <c r="D19" t="n">
-        <v>0.0476274165202108</v>
+        <v>0.0341183177652062</v>
       </c>
       <c r="E19" t="n">
-        <v>-0.0560570071258906</v>
+        <v>-0.0743473994111875</v>
       </c>
       <c r="F19" t="n">
-        <v>-0.1283494790714676</v>
+        <v>-0.1410723391855468</v>
       </c>
       <c r="G19" t="n">
-        <v>-0.099526445626756</v>
+        <v>-0.1177979406556639</v>
       </c>
       <c r="H19" t="n">
-        <v>-0.1020685918440427</v>
+        <v>-0.1190185315731018</v>
       </c>
       <c r="I19" t="n">
-        <v>70.74714042346068</v>
+        <v>66.49130832570901</v>
       </c>
       <c r="J19" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="K19" t="n">
         <v>51.27</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M19" t="n">
         <v>51.27</v>
       </c>
       <c r="N19" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="O19" t="n">
-        <v>29.78723404255319</v>
+        <v>25.53191489361702</v>
       </c>
       <c r="P19" t="n">
-        <v>46.46544680851064</v>
+        <v>49.61438297872341</v>
       </c>
       <c r="Q19" t="b">
         <v>0</v>
@@ -1949,25 +1949,25 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2259.1</v>
+        <v>2250.5</v>
       </c>
       <c r="D20" t="n">
-        <v>0.1287034723957032</v>
+        <v>0.1103710282218275</v>
       </c>
       <c r="E20" t="n">
-        <v>0.0359992662569934</v>
+        <v>0.0354267310789049</v>
       </c>
       <c r="F20" t="n">
-        <v>0.1647847383346223</v>
+        <v>0.1801258521237545</v>
       </c>
       <c r="G20" t="n">
-        <v>0.1936077717793339</v>
+        <v>0.2034002506536374</v>
       </c>
       <c r="H20" t="n">
-        <v>0.1910656255620473</v>
+        <v>0.2021796597361995</v>
       </c>
       <c r="I20" t="n">
-        <v>86.76097972972968</v>
+        <v>85.21360431356281</v>
       </c>
       <c r="J20" t="n">
         <v>60</v>
@@ -1977,7 +1977,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M20" t="n">
@@ -1987,10 +1987,10 @@
         <v>60</v>
       </c>
       <c r="O20" t="n">
-        <v>76.59574468085107</v>
+        <v>78.72340425531915</v>
       </c>
       <c r="P20" t="n">
-        <v>58.94314893617022</v>
+        <v>59.36868085106384</v>
       </c>
       <c r="Q20" t="b">
         <v>0</v>
@@ -2014,25 +2014,25 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1014.35</v>
+        <v>1017.85</v>
       </c>
       <c r="D21" t="n">
-        <v>0.208566662695103</v>
+        <v>0.1795005504374529</v>
       </c>
       <c r="E21" t="n">
-        <v>0.1021949364337717</v>
+        <v>0.1000216146114774</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.1680200131233595</v>
+        <v>-0.138437447096665</v>
       </c>
       <c r="G21" t="n">
-        <v>-0.1391969796786479</v>
+        <v>-0.1151630485667821</v>
       </c>
       <c r="H21" t="n">
-        <v>-0.1417391258959346</v>
+        <v>-0.11638363948422</v>
       </c>
       <c r="I21" t="n">
-        <v>92.11469534050178</v>
+        <v>92.236435818262</v>
       </c>
       <c r="J21" t="n">
         <v>60</v>
@@ -2042,7 +2042,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M21" t="n">
@@ -2052,10 +2052,10 @@
         <v>60</v>
       </c>
       <c r="O21" t="n">
-        <v>19.14893617021277</v>
+        <v>27.65957446808511</v>
       </c>
       <c r="P21" t="n">
-        <v>47.20178723404256</v>
+        <v>48.90391489361702</v>
       </c>
       <c r="Q21" t="b">
         <v>0</v>
@@ -2079,25 +2079,25 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>435.9</v>
+        <v>448.5</v>
       </c>
       <c r="D22" t="n">
-        <v>0.1480115880958652</v>
+        <v>0.1948847742107364</v>
       </c>
       <c r="E22" t="n">
-        <v>0.2301396923945251</v>
+        <v>0.2741477272727273</v>
       </c>
       <c r="F22" t="n">
-        <v>0.4122792807387008</v>
+        <v>0.4538087520259319</v>
       </c>
       <c r="G22" t="n">
-        <v>0.4411023141834124</v>
+        <v>0.4770831505558148</v>
       </c>
       <c r="H22" t="n">
-        <v>0.4385601679661257</v>
+        <v>0.475862559638377</v>
       </c>
       <c r="I22" t="n">
-        <v>83.44594594594594</v>
+        <v>85.03816793893128</v>
       </c>
       <c r="J22" t="n">
         <v>60</v>
@@ -2107,7 +2107,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M22" t="n">
@@ -2117,10 +2117,10 @@
         <v>60</v>
       </c>
       <c r="O22" t="n">
-        <v>93.61702127659576</v>
+        <v>95.74468085106383</v>
       </c>
       <c r="P22" t="n">
-        <v>64.51140425531915</v>
+        <v>64.93693617021276</v>
       </c>
       <c r="Q22" t="b">
         <v>0</v>
@@ -2144,25 +2144,25 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>401.6</v>
+        <v>393.15</v>
       </c>
       <c r="D23" t="n">
-        <v>0.1698223128459073</v>
+        <v>0.1542865531415147</v>
       </c>
       <c r="E23" t="n">
-        <v>0.0186429930247304</v>
+        <v>-0.0030429821224801</v>
       </c>
       <c r="F23" t="n">
-        <v>0.0004982561036372</v>
+        <v>0.0035737077217612</v>
       </c>
       <c r="G23" t="n">
-        <v>0.0293212895483488</v>
+        <v>0.0268481062516441</v>
       </c>
       <c r="H23" t="n">
-        <v>0.0267791433310622</v>
+        <v>0.0256275153342062</v>
       </c>
       <c r="I23" t="n">
-        <v>89.83128134974922</v>
+        <v>83.40389500423369</v>
       </c>
       <c r="J23" t="n">
         <v>60</v>
@@ -2172,7 +2172,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M23" t="n">
@@ -2182,10 +2182,10 @@
         <v>60</v>
       </c>
       <c r="O23" t="n">
-        <v>57.44680851063831</v>
+        <v>59.57446808510638</v>
       </c>
       <c r="P23" t="n">
-        <v>55.36936170212766</v>
+        <v>55.79489361702128</v>
       </c>
       <c r="Q23" t="b">
         <v>0</v>
@@ -2209,48 +2209,48 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>128.56</v>
+        <v>126.11</v>
       </c>
       <c r="D24" t="n">
-        <v>0.0985217465607108</v>
+        <v>0.0537266042780748</v>
       </c>
       <c r="E24" t="n">
-        <v>0.0052388771600593</v>
+        <v>0.0314902666448551</v>
       </c>
       <c r="F24" t="n">
-        <v>0.2618767177071064</v>
+        <v>0.253204809698897</v>
       </c>
       <c r="G24" t="n">
-        <v>0.290699751151818</v>
+        <v>0.2764792082287799</v>
       </c>
       <c r="H24" t="n">
-        <v>0.2881576049345313</v>
+        <v>0.275258617311342</v>
       </c>
       <c r="I24" t="n">
-        <v>76.41269841269843</v>
+        <v>70.89837997054492</v>
       </c>
       <c r="J24" t="n">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="K24" t="n">
         <v>48.3</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M24" t="n">
         <v>48.3</v>
       </c>
       <c r="N24" t="n">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="O24" t="n">
-        <v>82.97872340425532</v>
+        <v>85.1063829787234</v>
       </c>
       <c r="P24" t="n">
-        <v>63.91574468085106</v>
+        <v>56.34127659574468</v>
       </c>
       <c r="Q24" t="b">
         <v>0</v>
@@ -2274,25 +2274,25 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>624.2</v>
+        <v>615.65</v>
       </c>
       <c r="D25" t="n">
-        <v>0.1370798797704708</v>
+        <v>0.0853239312472453</v>
       </c>
       <c r="E25" t="n">
-        <v>0.0529689608636978</v>
+        <v>0.0491649625085208</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.0802328151477196</v>
+        <v>-0.081462140992167</v>
       </c>
       <c r="G25" t="n">
-        <v>-0.051409781703008</v>
+        <v>-0.0581877424622842</v>
       </c>
       <c r="H25" t="n">
-        <v>-0.0539519279202946</v>
+        <v>-0.059408333379722</v>
       </c>
       <c r="I25" t="n">
-        <v>95.49060542797496</v>
+        <v>89.12704598597035</v>
       </c>
       <c r="J25" t="n">
         <v>60</v>
@@ -2302,7 +2302,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M25" t="n">
@@ -2312,10 +2312,10 @@
         <v>60</v>
       </c>
       <c r="O25" t="n">
-        <v>38.29787234042553</v>
+        <v>36.17021276595745</v>
       </c>
       <c r="P25" t="n">
-        <v>54.42357446808511</v>
+        <v>53.99804255319149</v>
       </c>
       <c r="Q25" t="b">
         <v>0</v>
@@ -2339,25 +2339,25 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>132.83</v>
+        <v>132.25</v>
       </c>
       <c r="D26" t="n">
-        <v>0.0463174478141001</v>
+        <v>0.0391294099159267</v>
       </c>
       <c r="E26" t="n">
-        <v>-0.078912696761667</v>
+        <v>-0.0689242466910728</v>
       </c>
       <c r="F26" t="n">
-        <v>-0.1930133657351153</v>
+        <v>-0.1894956180670466</v>
       </c>
       <c r="G26" t="n">
-        <v>-0.1641903322904037</v>
+        <v>-0.1662212195371637</v>
       </c>
       <c r="H26" t="n">
-        <v>-0.1667324785076903</v>
+        <v>-0.1674418104546016</v>
       </c>
       <c r="I26" t="n">
-        <v>78.72180451127812</v>
+        <v>77.04194260485642</v>
       </c>
       <c r="J26" t="n">
         <v>50</v>
@@ -2367,7 +2367,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M26" t="n">
@@ -2404,48 +2404,48 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>5573.4</v>
+        <v>5517.1</v>
       </c>
       <c r="D27" t="n">
-        <v>0.1251438376905218</v>
+        <v>0.09130649787360311</v>
       </c>
       <c r="E27" t="n">
-        <v>0.0136218968809673</v>
+        <v>0.0294057281462822</v>
       </c>
       <c r="F27" t="n">
-        <v>0.1247805291517829</v>
+        <v>0.09225713210983751</v>
       </c>
       <c r="G27" t="n">
-        <v>0.1536035625964945</v>
+        <v>0.1155315306397204</v>
       </c>
       <c r="H27" t="n">
-        <v>0.1510614163792079</v>
+        <v>0.1143109397222825</v>
       </c>
       <c r="I27" t="n">
-        <v>82.43720011289864</v>
+        <v>79.28741092636581</v>
       </c>
       <c r="J27" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K27" t="n">
         <v>57.69</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M27" t="n">
         <v>57.69</v>
       </c>
       <c r="N27" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O27" t="n">
-        <v>65.95744680851064</v>
+        <v>63.82978723404256</v>
       </c>
       <c r="P27" t="n">
-        <v>60.26748936170213</v>
+        <v>63.84195744680851</v>
       </c>
       <c r="Q27" t="b">
         <v>0</v>
@@ -2469,25 +2469,25 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1794.9</v>
+        <v>1795.4</v>
       </c>
       <c r="D28" t="n">
-        <v>0.1394020186631119</v>
+        <v>0.1450255102040816</v>
       </c>
       <c r="E28" t="n">
-        <v>0.1649143302180686</v>
+        <v>0.2136821469614007</v>
       </c>
       <c r="F28" t="n">
-        <v>0.3569970514855975</v>
+        <v>0.4365498479756762</v>
       </c>
       <c r="G28" t="n">
-        <v>0.3858200849303091</v>
+        <v>0.4598242465055591</v>
       </c>
       <c r="H28" t="n">
-        <v>0.3832779387130225</v>
+        <v>0.4586036555881212</v>
       </c>
       <c r="I28" t="n">
-        <v>78.84493336154011</v>
+        <v>78.86728655959428</v>
       </c>
       <c r="J28" t="n">
         <v>70</v>
@@ -2497,7 +2497,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M28" t="n">
@@ -2507,10 +2507,10 @@
         <v>70</v>
       </c>
       <c r="O28" t="n">
-        <v>89.36170212765957</v>
+        <v>93.61702127659576</v>
       </c>
       <c r="P28" t="n">
-        <v>67.67634042553192</v>
+        <v>68.52740425531915</v>
       </c>
       <c r="Q28" t="b">
         <v>0</v>
@@ -2534,48 +2534,48 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>532.8</v>
+        <v>537.95</v>
       </c>
       <c r="D29" t="n">
-        <v>0.06432281262485</v>
+        <v>0.070547263681592</v>
       </c>
       <c r="E29" t="n">
-        <v>-0.0499286733238231</v>
+        <v>-0.01257342143906</v>
       </c>
       <c r="F29" t="n">
-        <v>-0.06337347279599199</v>
+        <v>-0.0553165334972342</v>
       </c>
       <c r="G29" t="n">
-        <v>-0.0345504393512804</v>
+        <v>-0.0320421349673513</v>
       </c>
       <c r="H29" t="n">
-        <v>-0.037092585568567</v>
+        <v>-0.0332627258847891</v>
       </c>
       <c r="I29" t="n">
-        <v>60.769535898453</v>
+        <v>62.30945121951223</v>
       </c>
       <c r="J29" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K29" t="n">
         <v>49.42</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M29" t="n">
         <v>49.42</v>
       </c>
       <c r="N29" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O29" t="n">
         <v>42.5531914893617</v>
       </c>
       <c r="P29" t="n">
-        <v>52.27863829787234</v>
+        <v>60.27863829787234</v>
       </c>
       <c r="Q29" t="b">
         <v>0</v>
@@ -2599,25 +2599,25 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>125.86</v>
+        <v>123.98</v>
       </c>
       <c r="D30" t="n">
-        <v>0.0744408400204883</v>
+        <v>0.0496994327321989</v>
       </c>
       <c r="E30" t="n">
-        <v>-0.0391632949080082</v>
+        <v>-0.0244708474309544</v>
       </c>
       <c r="F30" t="n">
-        <v>-0.0263035741915518</v>
+        <v>-0.0332189644416719</v>
       </c>
       <c r="G30" t="n">
-        <v>0.0025194592531597</v>
+        <v>-0.009944565911788999</v>
       </c>
       <c r="H30" t="n">
-        <v>-2.268696412688342e-05</v>
+        <v>-0.0111651568292269</v>
       </c>
       <c r="I30" t="n">
-        <v>86.39071809344621</v>
+        <v>81.58128516434705</v>
       </c>
       <c r="J30" t="n">
         <v>60</v>
@@ -2627,7 +2627,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M30" t="n">
@@ -2664,25 +2664,25 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>39.52</v>
+        <v>39.19</v>
       </c>
       <c r="D31" t="n">
-        <v>0.0603702709954387</v>
+        <v>0.0597620335316386</v>
       </c>
       <c r="E31" t="n">
-        <v>-0.1285556780595369</v>
+        <v>-0.1260035682426405</v>
       </c>
       <c r="F31" t="n">
-        <v>-0.1490094745908698</v>
+        <v>-0.1426383723474076</v>
       </c>
       <c r="G31" t="n">
-        <v>-0.1201864411461582</v>
+        <v>-0.1193639738175247</v>
       </c>
       <c r="H31" t="n">
-        <v>-0.1227285873634449</v>
+        <v>-0.1205845647349626</v>
       </c>
       <c r="I31" t="n">
-        <v>67.56032171581771</v>
+        <v>64.69833119383821</v>
       </c>
       <c r="J31" t="n">
         <v>60</v>
@@ -2692,7 +2692,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M31" t="n">
@@ -2702,10 +2702,10 @@
         <v>60</v>
       </c>
       <c r="O31" t="n">
-        <v>25.53191489361702</v>
+        <v>23.40425531914894</v>
       </c>
       <c r="P31" t="n">
-        <v>48.70238297872341</v>
+        <v>48.27685106382979</v>
       </c>
       <c r="Q31" t="b">
         <v>0</v>
@@ -2729,25 +2729,25 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>754.5</v>
+        <v>748.75</v>
       </c>
       <c r="D32" t="n">
-        <v>0.1126677481197462</v>
+        <v>0.09859878218766061</v>
       </c>
       <c r="E32" t="n">
-        <v>0.0319359912466663</v>
+        <v>0.0484492053490164</v>
       </c>
       <c r="F32" t="n">
-        <v>-0.2673334628083122</v>
+        <v>-0.2663629237703312</v>
       </c>
       <c r="G32" t="n">
-        <v>-0.2385104293636006</v>
+        <v>-0.2430885252404483</v>
       </c>
       <c r="H32" t="n">
-        <v>-0.2410525755808873</v>
+        <v>-0.2443091161578862</v>
       </c>
       <c r="I32" t="n">
-        <v>92.81883194278906</v>
+        <v>89.74358974358977</v>
       </c>
       <c r="J32" t="n">
         <v>60</v>
@@ -2757,7 +2757,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M32" t="n">
@@ -2767,10 +2767,10 @@
         <v>60</v>
       </c>
       <c r="O32" t="n">
-        <v>6.382978723404255</v>
+        <v>2.127659574468085</v>
       </c>
       <c r="P32" t="n">
-        <v>44.42059574468086</v>
+        <v>43.56953191489362</v>
       </c>
       <c r="Q32" t="b">
         <v>0</v>
@@ -2794,25 +2794,25 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>586.8</v>
+        <v>588.45</v>
       </c>
       <c r="D33" t="n">
-        <v>0.0971300364588201</v>
+        <v>0.1028956986224347</v>
       </c>
       <c r="E33" t="n">
-        <v>-0.0331191300049431</v>
+        <v>0.0077061392242485</v>
       </c>
       <c r="F33" t="n">
-        <v>0.0909090909090908</v>
+        <v>0.0999065420560747</v>
       </c>
       <c r="G33" t="n">
-        <v>0.1197321243538024</v>
+        <v>0.1231809405859576</v>
       </c>
       <c r="H33" t="n">
-        <v>0.1171899781365157</v>
+        <v>0.1219603496685197</v>
       </c>
       <c r="I33" t="n">
-        <v>83.04623753399822</v>
+        <v>83.29611433675754</v>
       </c>
       <c r="J33" t="n">
         <v>60</v>
@@ -2822,7 +2822,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M33" t="n">
@@ -2832,10 +2832,10 @@
         <v>60</v>
       </c>
       <c r="O33" t="n">
-        <v>63.82978723404256</v>
+        <v>65.95744680851064</v>
       </c>
       <c r="P33" t="n">
-        <v>56.75795744680852</v>
+        <v>57.18348936170213</v>
       </c>
       <c r="Q33" t="b">
         <v>0</v>
@@ -2871,10 +2871,10 @@
         <v>-0.2401052253975846</v>
       </c>
       <c r="G34" t="n">
-        <v>-0.211282191952873</v>
+        <v>-0.2168308268677017</v>
       </c>
       <c r="H34" t="n">
-        <v>-0.2138243381701596</v>
+        <v>-0.2180514177851396</v>
       </c>
       <c r="I34" t="n">
         <v>63.3225806451613</v>
@@ -2887,7 +2887,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M34" t="n">
@@ -2924,48 +2924,48 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>119.08</v>
+        <v>115.9</v>
       </c>
       <c r="D35" t="n">
-        <v>0.119488577606468</v>
+        <v>0.0615497343835866</v>
       </c>
       <c r="E35" t="n">
-        <v>-0.0226526592252134</v>
+        <v>-0.0358539223026369</v>
       </c>
       <c r="F35" t="n">
-        <v>0.2673478075776927</v>
+        <v>0.2558240329396468</v>
       </c>
       <c r="G35" t="n">
-        <v>0.2961708410224043</v>
+        <v>0.2790984314695297</v>
       </c>
       <c r="H35" t="n">
-        <v>0.2936286948051176</v>
+        <v>0.2778778405520918</v>
       </c>
       <c r="I35" t="n">
-        <v>85.51776843714175</v>
+        <v>76.25212947189098</v>
       </c>
       <c r="J35" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="K35" t="n">
         <v>49.07</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M35" t="n">
         <v>49.07</v>
       </c>
       <c r="N35" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="O35" t="n">
         <v>87.2340425531915</v>
       </c>
       <c r="P35" t="n">
-        <v>61.07480851063831</v>
+        <v>57.07480851063831</v>
       </c>
       <c r="Q35" t="b">
         <v>0</v>
@@ -2989,48 +2989,48 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>506.85</v>
+        <v>494.25</v>
       </c>
       <c r="D36" t="n">
-        <v>0.0709984152139462</v>
+        <v>0.035512256442489</v>
       </c>
       <c r="E36" t="n">
-        <v>-0.0803773927243036</v>
+        <v>-0.0703470328223454</v>
       </c>
       <c r="F36" t="n">
-        <v>0.1269594219010561</v>
+        <v>0.1110486680903675</v>
       </c>
       <c r="G36" t="n">
-        <v>0.1557824553457677</v>
+        <v>0.1343230666202504</v>
       </c>
       <c r="H36" t="n">
-        <v>0.153240309128481</v>
+        <v>0.1331024757028125</v>
       </c>
       <c r="I36" t="n">
-        <v>89.04415874790385</v>
+        <v>78.04997550220479</v>
       </c>
       <c r="J36" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K36" t="n">
         <v>47.8</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M36" t="n">
         <v>47.8</v>
       </c>
       <c r="N36" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O36" t="n">
         <v>68.08510638297872</v>
       </c>
       <c r="P36" t="n">
-        <v>56.73702127659575</v>
+        <v>60.73702127659575</v>
       </c>
       <c r="Q36" t="b">
         <v>0</v>
@@ -3054,48 +3054,48 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2378.3</v>
+        <v>2275.5</v>
       </c>
       <c r="D37" t="n">
-        <v>0.1140100238887067</v>
+        <v>0.0448138114697644</v>
       </c>
       <c r="E37" t="n">
-        <v>0.2907304895256704</v>
+        <v>0.2626935242217414</v>
       </c>
       <c r="F37" t="n">
-        <v>0.701702919290212</v>
+        <v>0.6582859641451684</v>
       </c>
       <c r="G37" t="n">
-        <v>0.7305259527349236</v>
+        <v>0.6815603626750513</v>
       </c>
       <c r="H37" t="n">
-        <v>0.7279838065176369</v>
+        <v>0.6803397717576134</v>
       </c>
       <c r="I37" t="n">
-        <v>91.77667766776686</v>
+        <v>71.54802744425388</v>
       </c>
       <c r="J37" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K37" t="n">
         <v>48.59</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M37" t="n">
         <v>48.59</v>
       </c>
       <c r="N37" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O37" t="n">
         <v>100</v>
       </c>
       <c r="P37" t="n">
-        <v>63.43600000000001</v>
+        <v>67.43600000000001</v>
       </c>
       <c r="Q37" t="b">
         <v>0</v>
@@ -3119,25 +3119,25 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>869</v>
+        <v>860.9</v>
       </c>
       <c r="D38" t="n">
-        <v>0.1013243774158798</v>
+        <v>0.0948051122273796</v>
       </c>
       <c r="E38" t="n">
-        <v>0.0216317893251822</v>
+        <v>0.0241494170830358</v>
       </c>
       <c r="F38" t="n">
-        <v>-0.1861009646904561</v>
+        <v>-0.1769598470363289</v>
       </c>
       <c r="G38" t="n">
-        <v>-0.1572779312457445</v>
+        <v>-0.153685448506446</v>
       </c>
       <c r="H38" t="n">
-        <v>-0.1598200774630311</v>
+        <v>-0.1549060394238839</v>
       </c>
       <c r="I38" t="n">
-        <v>88.79518072289162</v>
+        <v>85.45918367346941</v>
       </c>
       <c r="J38" t="n">
         <v>60</v>
@@ -3147,7 +3147,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M38" t="n">
@@ -3157,10 +3157,10 @@
         <v>60</v>
       </c>
       <c r="O38" t="n">
-        <v>17.02127659574468</v>
+        <v>14.8936170212766</v>
       </c>
       <c r="P38" t="n">
-        <v>47.35225531914894</v>
+        <v>46.92672340425532</v>
       </c>
       <c r="Q38" t="b">
         <v>0</v>
@@ -3184,48 +3184,48 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>3735.8</v>
+        <v>3627.6</v>
       </c>
       <c r="D39" t="n">
-        <v>0.2693849813115869</v>
+        <v>0.1608319999999998</v>
       </c>
       <c r="E39" t="n">
-        <v>0.2945457065631713</v>
+        <v>0.2799379013478231</v>
       </c>
       <c r="F39" t="n">
-        <v>0.3830149563157117</v>
+        <v>0.3458984157607685</v>
       </c>
       <c r="G39" t="n">
-        <v>0.4118379897604233</v>
+        <v>0.3691728142906514</v>
       </c>
       <c r="H39" t="n">
-        <v>0.4092958435431366</v>
+        <v>0.3679522233732135</v>
       </c>
       <c r="I39" t="n">
-        <v>86.30994447248865</v>
+        <v>77.81013925548373</v>
       </c>
       <c r="J39" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K39" t="n">
         <v>48.69</v>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M39" t="n">
         <v>48.69</v>
       </c>
       <c r="N39" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O39" t="n">
-        <v>91.48936170212764</v>
+        <v>89.36170212765957</v>
       </c>
       <c r="P39" t="n">
-        <v>61.77387234042553</v>
+        <v>65.34834042553192</v>
       </c>
       <c r="Q39" t="b">
         <v>0</v>
@@ -3249,25 +3249,25 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>220.94</v>
+        <v>217.76</v>
       </c>
       <c r="D40" t="n">
-        <v>0.2329241071428571</v>
+        <v>0.1741615442683057</v>
       </c>
       <c r="E40" t="n">
-        <v>0.1164224355735219</v>
+        <v>0.1195886889460153</v>
       </c>
       <c r="F40" t="n">
-        <v>-0.0255369823137652</v>
+        <v>-0.0331660968787461</v>
       </c>
       <c r="G40" t="n">
-        <v>0.0032860511309463</v>
+        <v>-0.0098916983488632</v>
       </c>
       <c r="H40" t="n">
-        <v>0.0007439049136597</v>
+        <v>-0.0111122892663011</v>
       </c>
       <c r="I40" t="n">
-        <v>97.42723004694837</v>
+        <v>91.93691298954457</v>
       </c>
       <c r="J40" t="n">
         <v>60</v>
@@ -3277,7 +3277,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M40" t="n">
@@ -3296,7 +3296,7 @@
         <v>0</v>
       </c>
       <c r="R40" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S40" t="b">
         <v>0</v>
@@ -3314,25 +3314,25 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>828.9</v>
+        <v>828.95</v>
       </c>
       <c r="D41" t="n">
-        <v>0.0168680610930502</v>
+        <v>0.0196186961869619</v>
       </c>
       <c r="E41" t="n">
-        <v>-0.1117183732518887</v>
+        <v>-0.1045638671347555</v>
       </c>
       <c r="F41" t="n">
-        <v>-0.1538383013474887</v>
+        <v>-0.1697215544871794</v>
       </c>
       <c r="G41" t="n">
-        <v>-0.1250152679027771</v>
+        <v>-0.1464471559572965</v>
       </c>
       <c r="H41" t="n">
-        <v>-0.1275574141200638</v>
+        <v>-0.1476677468747343</v>
       </c>
       <c r="I41" t="n">
-        <v>78.24548991864168</v>
+        <v>78.25318246110326</v>
       </c>
       <c r="J41" t="n">
         <v>50</v>
@@ -3342,7 +3342,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M41" t="n">
@@ -3352,10 +3352,10 @@
         <v>50</v>
       </c>
       <c r="O41" t="n">
-        <v>21.27659574468085</v>
+        <v>17.02127659574468</v>
       </c>
       <c r="P41" t="n">
-        <v>43.47531914893617</v>
+        <v>42.62425531914894</v>
       </c>
       <c r="Q41" t="b">
         <v>0</v>
@@ -3379,25 +3379,25 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>619.25</v>
+        <v>616.15</v>
       </c>
       <c r="D42" t="n">
-        <v>0.1589930750514692</v>
+        <v>0.1626568544202282</v>
       </c>
       <c r="E42" t="n">
-        <v>-0.053424029348823</v>
+        <v>-0.0281545741324921</v>
       </c>
       <c r="F42" t="n">
-        <v>-0.1895694280853291</v>
+        <v>-0.1869763145741242</v>
       </c>
       <c r="G42" t="n">
-        <v>-0.1607463946406175</v>
+        <v>-0.1637019160442413</v>
       </c>
       <c r="H42" t="n">
-        <v>-0.1632885408579042</v>
+        <v>-0.1649225069616792</v>
       </c>
       <c r="I42" t="n">
-        <v>85.28604118993132</v>
+        <v>84.09296028880863</v>
       </c>
       <c r="J42" t="n">
         <v>60</v>
@@ -3407,7 +3407,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M42" t="n">
@@ -3417,10 +3417,10 @@
         <v>60</v>
       </c>
       <c r="O42" t="n">
-        <v>14.8936170212766</v>
+        <v>12.76595744680851</v>
       </c>
       <c r="P42" t="n">
-        <v>46.04272340425532</v>
+        <v>45.6171914893617</v>
       </c>
       <c r="Q42" t="b">
         <v>0</v>
@@ -3444,48 +3444,48 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>425.2</v>
+        <v>414.4</v>
       </c>
       <c r="D43" t="n">
-        <v>0.07035871617369401</v>
+        <v>0.029437336976773</v>
       </c>
       <c r="E43" t="n">
-        <v>-0.085296332150156</v>
+        <v>-0.085815133465696</v>
       </c>
       <c r="F43" t="n">
-        <v>-0.07845687039445159</v>
+        <v>-0.104580812445981</v>
       </c>
       <c r="G43" t="n">
-        <v>-0.0496338369497399</v>
+        <v>-0.08130641391609809</v>
       </c>
       <c r="H43" t="n">
-        <v>-0.0521759831670266</v>
+        <v>-0.08252700483353601</v>
       </c>
       <c r="I43" t="n">
-        <v>61.8957345971564</v>
+        <v>56.14789337919173</v>
       </c>
       <c r="J43" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="K43" t="n">
         <v>51.48</v>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M43" t="n">
         <v>51.48</v>
       </c>
       <c r="N43" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="O43" t="n">
-        <v>40.42553191489361</v>
+        <v>34.04255319148936</v>
       </c>
       <c r="P43" t="n">
-        <v>60.67710638297872</v>
+        <v>43.40051063829787</v>
       </c>
       <c r="Q43" t="b">
         <v>0</v>
@@ -3509,25 +3509,25 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>275.62</v>
+        <v>281.41</v>
       </c>
       <c r="D44" t="n">
-        <v>0.172601574133163</v>
+        <v>0.1896427816529275</v>
       </c>
       <c r="E44" t="n">
-        <v>0.013122587759603</v>
+        <v>0.142781725888325</v>
       </c>
       <c r="F44" t="n">
-        <v>-0.0887088775004132</v>
+        <v>-0.0421715452688903</v>
       </c>
       <c r="G44" t="n">
-        <v>-0.0598858440557016</v>
+        <v>-0.0188971467390074</v>
       </c>
       <c r="H44" t="n">
-        <v>-0.0624279902729882</v>
+        <v>-0.0201177376564453</v>
       </c>
       <c r="I44" t="n">
-        <v>99.63751699139104</v>
+        <v>99.6795513719207</v>
       </c>
       <c r="J44" t="n">
         <v>60</v>
@@ -3537,7 +3537,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M44" t="n">
@@ -3547,10 +3547,10 @@
         <v>60</v>
       </c>
       <c r="O44" t="n">
-        <v>36.17021276595745</v>
+        <v>46.80851063829788</v>
       </c>
       <c r="P44" t="n">
-        <v>50.1140425531915</v>
+        <v>52.24170212765958</v>
       </c>
       <c r="Q44" t="b">
         <v>0</v>
@@ -3574,25 +3574,25 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>101.7</v>
+        <v>102.88</v>
       </c>
       <c r="D45" t="n">
-        <v>0.0483455313885166</v>
+        <v>0.0564797699733004</v>
       </c>
       <c r="E45" t="n">
-        <v>-0.1775836972343522</v>
+        <v>-0.1286524942830523</v>
       </c>
       <c r="F45" t="n">
-        <v>-0.2702877233263974</v>
+        <v>-0.2450282527335437</v>
       </c>
       <c r="G45" t="n">
-        <v>-0.2414646898816858</v>
+        <v>-0.2217538542036609</v>
       </c>
       <c r="H45" t="n">
-        <v>-0.2440068360989724</v>
+        <v>-0.2229744451210987</v>
       </c>
       <c r="I45" t="n">
-        <v>89.27503736920779</v>
+        <v>89.72798854688621</v>
       </c>
       <c r="J45" t="n">
         <v>60</v>
@@ -3602,7 +3602,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M45" t="n">
@@ -3612,10 +3612,10 @@
         <v>60</v>
       </c>
       <c r="O45" t="n">
-        <v>4.25531914893617</v>
+        <v>6.382978723404255</v>
       </c>
       <c r="P45" t="n">
-        <v>48.69106382978724</v>
+        <v>49.11659574468086</v>
       </c>
       <c r="Q45" t="b">
         <v>0</v>
@@ -3639,48 +3639,48 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>539.2</v>
+        <v>526.15</v>
       </c>
       <c r="D46" t="n">
-        <v>0.0705847314603396</v>
+        <v>0.0561019670814932</v>
       </c>
       <c r="E46" t="n">
-        <v>-0.0400569699127648</v>
+        <v>-0.049841986455982</v>
       </c>
       <c r="F46" t="n">
-        <v>-0.1044676963959474</v>
+        <v>-0.1088245257452574</v>
       </c>
       <c r="G46" t="n">
-        <v>-0.0756446629512358</v>
+        <v>-0.0855501272153745</v>
       </c>
       <c r="H46" t="n">
-        <v>-0.0781868091685225</v>
+        <v>-0.0867707181328124</v>
       </c>
       <c r="I46" t="n">
-        <v>76.57290895632869</v>
+        <v>69.8278771515356</v>
       </c>
       <c r="J46" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K46" t="n">
         <v>49.61</v>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M46" t="n">
         <v>49.61</v>
       </c>
       <c r="N46" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O46" t="n">
         <v>31.91489361702128</v>
       </c>
       <c r="P46" t="n">
-        <v>54.22697872340426</v>
+        <v>58.22697872340426</v>
       </c>
       <c r="Q46" t="b">
         <v>0</v>
@@ -3704,25 +3704,25 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>1067.05</v>
+        <v>1074.35</v>
       </c>
       <c r="D47" t="n">
-        <v>0.0772841998990407</v>
+        <v>0.0459014797507786</v>
       </c>
       <c r="E47" t="n">
-        <v>0.3672240374143121</v>
+        <v>0.3700822546706623</v>
       </c>
       <c r="F47" t="n">
-        <v>0.1856111111111111</v>
+        <v>0.1885717446620201</v>
       </c>
       <c r="G47" t="n">
-        <v>0.2144341445558227</v>
+        <v>0.2118461431919029</v>
       </c>
       <c r="H47" t="n">
-        <v>0.2118919983385361</v>
+        <v>0.2106255522744651</v>
       </c>
       <c r="I47" t="n">
-        <v>64.55379482902416</v>
+        <v>65.60097126669362</v>
       </c>
       <c r="J47" t="n">
         <v>80</v>
@@ -3732,7 +3732,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M47" t="n">
@@ -3769,25 +3769,25 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>14500</v>
+        <v>15032</v>
       </c>
       <c r="D48" t="n">
-        <v>0.08322127595995819</v>
+        <v>0.0891964350409391</v>
       </c>
       <c r="E48" t="n">
-        <v>0.0321019289629154</v>
+        <v>0.0720296676650977</v>
       </c>
       <c r="F48" t="n">
-        <v>0.1622314844501442</v>
+        <v>0.164819837272375</v>
       </c>
       <c r="G48" t="n">
-        <v>0.1910545178948558</v>
+        <v>0.1880942358022579</v>
       </c>
       <c r="H48" t="n">
-        <v>0.1885123716775691</v>
+        <v>0.18687364488482</v>
       </c>
       <c r="I48" t="n">
-        <v>61.17898594990837</v>
+        <v>66.60535995796111</v>
       </c>
       <c r="J48" t="n">
         <v>80</v>
@@ -3797,7 +3797,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M48" t="n">
@@ -3945,25 +3945,25 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1860.5</v>
+        <v>1866.2</v>
       </c>
       <c r="D2" t="n">
-        <v>0.08648680214903059</v>
+        <v>0.0903885480572597</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2765884451763414</v>
+        <v>0.3187760582291006</v>
       </c>
       <c r="F2" t="n">
-        <v>0.5325370675453047</v>
+        <v>0.5392609699769053</v>
       </c>
       <c r="G2" t="n">
-        <v>0.5613601009900163</v>
+        <v>0.5625353685067882</v>
       </c>
       <c r="H2" t="n">
-        <v>0.5588179547727297</v>
+        <v>0.5613147775893503</v>
       </c>
       <c r="I2" t="n">
-        <v>77.83767595088349</v>
+        <v>78.20965842167257</v>
       </c>
       <c r="J2" t="n">
         <v>70</v>
@@ -3973,7 +3973,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M2" t="n">
@@ -4010,25 +4010,25 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1794.9</v>
+        <v>1795.4</v>
       </c>
       <c r="D3" t="n">
-        <v>0.1394020186631119</v>
+        <v>0.1450255102040816</v>
       </c>
       <c r="E3" t="n">
-        <v>0.1649143302180686</v>
+        <v>0.2136821469614007</v>
       </c>
       <c r="F3" t="n">
-        <v>0.3569970514855975</v>
+        <v>0.4365498479756762</v>
       </c>
       <c r="G3" t="n">
-        <v>0.3858200849303091</v>
+        <v>0.4598242465055591</v>
       </c>
       <c r="H3" t="n">
-        <v>0.3832779387130225</v>
+        <v>0.4586036555881212</v>
       </c>
       <c r="I3" t="n">
-        <v>78.84493336154011</v>
+        <v>78.86728655959428</v>
       </c>
       <c r="J3" t="n">
         <v>70</v>
@@ -4038,7 +4038,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M3" t="n">
@@ -4048,10 +4048,10 @@
         <v>70</v>
       </c>
       <c r="O3" t="n">
-        <v>89.36170212765957</v>
+        <v>93.61702127659576</v>
       </c>
       <c r="P3" t="n">
-        <v>67.67634042553192</v>
+        <v>68.52740425531915</v>
       </c>
       <c r="Q3" t="b">
         <v>0</v>
@@ -4066,57 +4066,57 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ZFCVINDIA</t>
+          <t>SANSERA</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Brakes/Transmission</t>
+          <t>Forgings</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>14500</v>
+        <v>2275.5</v>
       </c>
       <c r="D4" t="n">
-        <v>0.08322127595995819</v>
+        <v>0.0448138114697644</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0321019289629154</v>
+        <v>0.2626935242217414</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1622314844501442</v>
+        <v>0.6582859641451684</v>
       </c>
       <c r="G4" t="n">
-        <v>0.1910545178948558</v>
+        <v>0.6815603626750513</v>
       </c>
       <c r="H4" t="n">
-        <v>0.1885123716775691</v>
+        <v>0.6803397717576134</v>
       </c>
       <c r="I4" t="n">
-        <v>61.17898594990837</v>
+        <v>71.54802744425388</v>
       </c>
       <c r="J4" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K4" t="n">
-        <v>50.29</v>
+        <v>48.59</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M4" t="n">
-        <v>50.29</v>
+        <v>48.59</v>
       </c>
       <c r="N4" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O4" t="n">
-        <v>74.46808510638297</v>
+        <v>100</v>
       </c>
       <c r="P4" t="n">
-        <v>67.0096170212766</v>
+        <v>67.43600000000001</v>
       </c>
       <c r="Q4" t="b">
         <v>0</v>
@@ -4131,57 +4131,57 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>WHEELS</t>
+          <t>ZFCVINDIA</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Wheels</t>
+          <t>Brakes/Transmission</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1067.05</v>
+        <v>15032</v>
       </c>
       <c r="D5" t="n">
-        <v>0.0772841998990407</v>
+        <v>0.0891964350409391</v>
       </c>
       <c r="E5" t="n">
-        <v>0.3672240374143121</v>
+        <v>0.0720296676650977</v>
       </c>
       <c r="F5" t="n">
-        <v>0.1856111111111111</v>
+        <v>0.164819837272375</v>
       </c>
       <c r="G5" t="n">
-        <v>0.2144341445558227</v>
+        <v>0.1880942358022579</v>
       </c>
       <c r="H5" t="n">
-        <v>0.2118919983385361</v>
+        <v>0.18687364488482</v>
       </c>
       <c r="I5" t="n">
-        <v>64.55379482902416</v>
+        <v>66.60535995796111</v>
       </c>
       <c r="J5" t="n">
         <v>80</v>
       </c>
       <c r="K5" t="n">
-        <v>46.83</v>
+        <v>50.29</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M5" t="n">
-        <v>46.83</v>
+        <v>50.29</v>
       </c>
       <c r="N5" t="n">
         <v>80</v>
       </c>
       <c r="O5" t="n">
-        <v>80.85106382978722</v>
+        <v>74.46808510638297</v>
       </c>
       <c r="P5" t="n">
-        <v>66.90221276595744</v>
+        <v>67.0096170212766</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
@@ -4196,57 +4196,57 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>GNA</t>
+          <t>WHEELS</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Axles</t>
+          <t>Wheels</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>435.9</v>
+        <v>1074.35</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1480115880958652</v>
+        <v>0.0459014797507786</v>
       </c>
       <c r="E6" t="n">
-        <v>0.2301396923945251</v>
+        <v>0.3700822546706623</v>
       </c>
       <c r="F6" t="n">
-        <v>0.4122792807387008</v>
+        <v>0.1885717446620201</v>
       </c>
       <c r="G6" t="n">
-        <v>0.4411023141834124</v>
+        <v>0.2118461431919029</v>
       </c>
       <c r="H6" t="n">
-        <v>0.4385601679661257</v>
+        <v>0.2106255522744651</v>
       </c>
       <c r="I6" t="n">
-        <v>83.44594594594594</v>
+        <v>65.60097126669362</v>
       </c>
       <c r="J6" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K6" t="n">
-        <v>54.47</v>
+        <v>46.83</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M6" t="n">
-        <v>54.47</v>
+        <v>46.83</v>
       </c>
       <c r="N6" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O6" t="n">
-        <v>93.61702127659576</v>
+        <v>80.85106382978722</v>
       </c>
       <c r="P6" t="n">
-        <v>64.51140425531915</v>
+        <v>66.90221276595744</v>
       </c>
       <c r="Q6" t="b">
         <v>0</v>
@@ -4261,57 +4261,57 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>JAMNAAUTO</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Suspension</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>128.56</v>
+        <v>576.55</v>
       </c>
       <c r="D7" t="n">
-        <v>0.0985217465607108</v>
+        <v>0.1388641975308642</v>
       </c>
       <c r="E7" t="n">
-        <v>0.0052388771600593</v>
+        <v>0.2879481737964928</v>
       </c>
       <c r="F7" t="n">
-        <v>0.2618767177071064</v>
+        <v>0.4002428658166361</v>
       </c>
       <c r="G7" t="n">
-        <v>0.290699751151818</v>
+        <v>0.423517264346519</v>
       </c>
       <c r="H7" t="n">
-        <v>0.2881576049345313</v>
+        <v>0.4222966734290811</v>
       </c>
       <c r="I7" t="n">
-        <v>76.41269841269843</v>
+        <v>79.32736809626651</v>
       </c>
       <c r="J7" t="n">
         <v>70</v>
       </c>
       <c r="K7" t="n">
-        <v>48.3</v>
+        <v>49.66</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M7" t="n">
-        <v>48.3</v>
+        <v>49.66</v>
       </c>
       <c r="N7" t="n">
         <v>70</v>
       </c>
       <c r="O7" t="n">
-        <v>82.97872340425532</v>
+        <v>91.48936170212764</v>
       </c>
       <c r="P7" t="n">
-        <v>63.91574468085106</v>
+        <v>66.16187234042553</v>
       </c>
       <c r="Q7" t="b">
         <v>0</v>
@@ -4326,57 +4326,57 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CRAFTSMAN</t>
+          <t>SHRIPISTON</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Castings</t>
+          <t>Engine/Parts</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>7691</v>
+        <v>3627.6</v>
       </c>
       <c r="D8" t="n">
-        <v>0.1219547775346463</v>
+        <v>0.1608319999999998</v>
       </c>
       <c r="E8" t="n">
-        <v>-0.0099124613800205</v>
+        <v>0.2799379013478231</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1446643845810389</v>
+        <v>0.3458984157607685</v>
       </c>
       <c r="G8" t="n">
-        <v>0.1734874180257505</v>
+        <v>0.3691728142906514</v>
       </c>
       <c r="H8" t="n">
-        <v>0.1709452718084638</v>
+        <v>0.3679522233732135</v>
       </c>
       <c r="I8" t="n">
-        <v>78.74396135265701</v>
+        <v>77.81013925548373</v>
       </c>
       <c r="J8" t="n">
         <v>70</v>
       </c>
       <c r="K8" t="n">
-        <v>54.65</v>
+        <v>48.69</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M8" t="n">
-        <v>54.65</v>
+        <v>48.69</v>
       </c>
       <c r="N8" t="n">
         <v>70</v>
       </c>
       <c r="O8" t="n">
-        <v>70.21276595744681</v>
+        <v>89.36170212765957</v>
       </c>
       <c r="P8" t="n">
-        <v>63.90255319148936</v>
+        <v>65.34834042553192</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
@@ -4391,57 +4391,57 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SANSERA</t>
+          <t>GNA</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Forgings</t>
+          <t>Axles</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>2378.3</v>
+        <v>448.5</v>
       </c>
       <c r="D9" t="n">
-        <v>0.1140100238887067</v>
+        <v>0.1948847742107364</v>
       </c>
       <c r="E9" t="n">
-        <v>0.2907304895256704</v>
+        <v>0.2741477272727273</v>
       </c>
       <c r="F9" t="n">
-        <v>0.701702919290212</v>
+        <v>0.4538087520259319</v>
       </c>
       <c r="G9" t="n">
-        <v>0.7305259527349236</v>
+        <v>0.4770831505558148</v>
       </c>
       <c r="H9" t="n">
-        <v>0.7279838065176369</v>
+        <v>0.475862559638377</v>
       </c>
       <c r="I9" t="n">
-        <v>91.77667766776686</v>
+        <v>85.03816793893128</v>
       </c>
       <c r="J9" t="n">
         <v>60</v>
       </c>
       <c r="K9" t="n">
-        <v>48.59</v>
+        <v>54.47</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M9" t="n">
-        <v>48.59</v>
+        <v>54.47</v>
       </c>
       <c r="N9" t="n">
         <v>60</v>
       </c>
       <c r="O9" t="n">
-        <v>100</v>
+        <v>95.74468085106383</v>
       </c>
       <c r="P9" t="n">
-        <v>63.43600000000001</v>
+        <v>64.93693617021276</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -4465,25 +4465,25 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>436.8</v>
+        <v>438.25</v>
       </c>
       <c r="D10" t="n">
-        <v>0.043602914824991</v>
+        <v>0.0709921798631476</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.0586206896551724</v>
+        <v>-0.0441657579062159</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.192680898253396</v>
+        <v>-0.1695091908281221</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.1638578648086844</v>
+        <v>-0.1462347922982392</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.1664000110259711</v>
+        <v>-0.147455383215677</v>
       </c>
       <c r="I10" t="n">
-        <v>40.02509410288583</v>
+        <v>42.13075060532687</v>
       </c>
       <c r="J10" t="n">
         <v>80</v>
@@ -4493,7 +4493,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M10" t="n">
@@ -4503,10 +4503,10 @@
         <v>80</v>
       </c>
       <c r="O10" t="n">
-        <v>12.76595744680851</v>
+        <v>19.14893617021277</v>
       </c>
       <c r="P10" t="n">
-        <v>63.0651914893617</v>
+        <v>64.34178723404256</v>
       </c>
       <c r="Q10" t="b">
         <v>1</v>
@@ -4521,7 +4521,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>MOTHERSON</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -4530,48 +4530,48 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>593.85</v>
+        <v>123.19</v>
       </c>
       <c r="D11" t="n">
-        <v>0.1907960697814317</v>
+        <v>0.1039519670221345</v>
       </c>
       <c r="E11" t="n">
-        <v>0.2906976744186047</v>
+        <v>0.09667942668921919</v>
       </c>
       <c r="F11" t="n">
-        <v>0.4650302207968422</v>
+        <v>0.1660198769522005</v>
       </c>
       <c r="G11" t="n">
-        <v>0.4938532542415538</v>
+        <v>0.1892942754820834</v>
       </c>
       <c r="H11" t="n">
-        <v>0.4913111080242671</v>
+        <v>0.1880736845646455</v>
       </c>
       <c r="I11" t="n">
-        <v>88.80829015544036</v>
+        <v>77.11889787361486</v>
       </c>
       <c r="J11" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K11" t="n">
-        <v>49.66</v>
+        <v>51.57</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M11" t="n">
-        <v>49.66</v>
+        <v>51.57</v>
       </c>
       <c r="N11" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O11" t="n">
-        <v>95.74468085106383</v>
+        <v>76.59574468085107</v>
       </c>
       <c r="P11" t="n">
-        <v>63.01293617021277</v>
+        <v>63.94714893617022</v>
       </c>
       <c r="Q11" t="b">
         <v>0</v>
@@ -4586,57 +4586,57 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>BHARATGEAR</t>
+          <t>CRAFTSMAN</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Gears</t>
+          <t>Castings</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>112.64</v>
+        <v>7721.5</v>
       </c>
       <c r="D12" t="n">
-        <v>0.1673748574981863</v>
+        <v>0.1171151620370369</v>
       </c>
       <c r="E12" t="n">
-        <v>0.069807199164213</v>
+        <v>0.0154523934771173</v>
       </c>
       <c r="F12" t="n">
-        <v>0.2639138240574505</v>
+        <v>0.1366011628762788</v>
       </c>
       <c r="G12" t="n">
-        <v>0.2927368575021621</v>
+        <v>0.1598755614061617</v>
       </c>
       <c r="H12" t="n">
-        <v>0.2901947112848755</v>
+        <v>0.1586549704887239</v>
       </c>
       <c r="I12" t="n">
-        <v>94.62837837837836</v>
+        <v>79.25343811394892</v>
       </c>
       <c r="J12" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K12" t="n">
-        <v>51.91</v>
+        <v>54.65</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M12" t="n">
-        <v>51.91</v>
+        <v>54.65</v>
       </c>
       <c r="N12" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O12" t="n">
-        <v>85.1063829787234</v>
+        <v>70.21276595744681</v>
       </c>
       <c r="P12" t="n">
-        <v>61.78527659574468</v>
+        <v>63.90255319148936</v>
       </c>
       <c r="Q12" t="b">
         <v>0</v>
@@ -4651,57 +4651,57 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>SHRIPISTON</t>
+          <t>LUMAXIND</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Engine/Parts</t>
+          <t>Lighting</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>3735.8</v>
+        <v>5517.1</v>
       </c>
       <c r="D13" t="n">
-        <v>0.2693849813115869</v>
+        <v>0.09130649787360311</v>
       </c>
       <c r="E13" t="n">
-        <v>0.2945457065631713</v>
+        <v>0.0294057281462822</v>
       </c>
       <c r="F13" t="n">
-        <v>0.3830149563157117</v>
+        <v>0.09225713210983751</v>
       </c>
       <c r="G13" t="n">
-        <v>0.4118379897604233</v>
+        <v>0.1155315306397204</v>
       </c>
       <c r="H13" t="n">
-        <v>0.4092958435431366</v>
+        <v>0.1143109397222825</v>
       </c>
       <c r="I13" t="n">
-        <v>86.30994447248865</v>
+        <v>79.28741092636581</v>
       </c>
       <c r="J13" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K13" t="n">
-        <v>48.69</v>
+        <v>57.69</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M13" t="n">
-        <v>48.69</v>
+        <v>57.69</v>
       </c>
       <c r="N13" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O13" t="n">
-        <v>91.48936170212764</v>
+        <v>63.82978723404256</v>
       </c>
       <c r="P13" t="n">
-        <v>61.77387234042553</v>
+        <v>63.84195744680851</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
@@ -4716,57 +4716,57 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>RICOAUTO</t>
+          <t>BHARATGEAR</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Castings</t>
+          <t>Gears</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>119.08</v>
+        <v>108.05</v>
       </c>
       <c r="D14" t="n">
-        <v>0.119488577606468</v>
+        <v>0.101427115188583</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.0226526592252134</v>
+        <v>-0.0019397746166636</v>
       </c>
       <c r="F14" t="n">
-        <v>0.2673478075776927</v>
+        <v>0.2033634034970486</v>
       </c>
       <c r="G14" t="n">
-        <v>0.2961708410224043</v>
+        <v>0.2266378020269315</v>
       </c>
       <c r="H14" t="n">
-        <v>0.2936286948051176</v>
+        <v>0.2254172111094936</v>
       </c>
       <c r="I14" t="n">
-        <v>85.51776843714175</v>
+        <v>81.924539338988</v>
       </c>
       <c r="J14" t="n">
         <v>60</v>
       </c>
       <c r="K14" t="n">
-        <v>49.07</v>
+        <v>51.91</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M14" t="n">
-        <v>49.07</v>
+        <v>51.91</v>
       </c>
       <c r="N14" t="n">
         <v>60</v>
       </c>
       <c r="O14" t="n">
-        <v>87.2340425531915</v>
+        <v>82.97872340425532</v>
       </c>
       <c r="P14" t="n">
-        <v>61.07480851063831</v>
+        <v>61.35974468085107</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
@@ -4781,63 +4781,63 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SUPRAJIT</t>
+          <t>SANDHAR</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Cables</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>425.2</v>
+        <v>494.25</v>
       </c>
       <c r="D15" t="n">
-        <v>0.07035871617369401</v>
+        <v>0.035512256442489</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.085296332150156</v>
+        <v>-0.0703470328223454</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.07845687039445159</v>
+        <v>0.1110486680903675</v>
       </c>
       <c r="G15" t="n">
-        <v>-0.0496338369497399</v>
+        <v>0.1343230666202504</v>
       </c>
       <c r="H15" t="n">
-        <v>-0.0521759831670266</v>
+        <v>0.1331024757028125</v>
       </c>
       <c r="I15" t="n">
-        <v>61.8957345971564</v>
+        <v>78.04997550220479</v>
       </c>
       <c r="J15" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K15" t="n">
-        <v>51.48</v>
+        <v>47.8</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M15" t="n">
-        <v>51.48</v>
+        <v>47.8</v>
       </c>
       <c r="N15" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O15" t="n">
-        <v>40.42553191489361</v>
+        <v>68.08510638297872</v>
       </c>
       <c r="P15" t="n">
-        <v>60.67710638297872</v>
+        <v>60.73702127659575</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
       </c>
       <c r="R15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S15" t="b">
         <v>0</v>
@@ -4846,7 +4846,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>MOTHERSON</t>
+          <t>MINDACORP</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -4855,54 +4855,54 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>125.03</v>
+        <v>537.95</v>
       </c>
       <c r="D16" t="n">
-        <v>0.1188366890380312</v>
+        <v>0.070547263681592</v>
       </c>
       <c r="E16" t="n">
-        <v>0.0892063768620958</v>
+        <v>-0.01257342143906</v>
       </c>
       <c r="F16" t="n">
-        <v>0.1698166167664672</v>
+        <v>-0.0553165334972342</v>
       </c>
       <c r="G16" t="n">
-        <v>0.1986396502111788</v>
+        <v>-0.0320421349673513</v>
       </c>
       <c r="H16" t="n">
-        <v>0.1960975039938921</v>
+        <v>-0.0332627258847891</v>
       </c>
       <c r="I16" t="n">
-        <v>81.61648177496039</v>
+        <v>62.30945121951223</v>
       </c>
       <c r="J16" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K16" t="n">
-        <v>51.57</v>
+        <v>49.42</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="M16" t="n">
-        <v>51.57</v>
+        <v>49.42</v>
       </c>
       <c r="N16" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O16" t="n">
-        <v>78.72340425531915</v>
+        <v>42.5531914893617</v>
       </c>
       <c r="P16" t="n">
-        <v>60.37268085106383</v>
+        <v>60.27863829787234</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>
       </c>
       <c r="R16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S16" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
chore: auto-refresh NSE data and pipeline outputs (2026-04-21)
</commit_message>
<xml_diff>
--- a/working-sector/output/auto_components_comprehensive_report.xlsx
+++ b/working-sector/output/auto_components_comprehensive_report.xlsx
@@ -435,7 +435,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
     </row>
@@ -447,7 +447,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
     </row>
@@ -779,48 +779,48 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1866.2</v>
+        <v>1895.8</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0903885480572597</v>
+        <v>0.1499454082251607</v>
       </c>
       <c r="E2" t="n">
-        <v>0.3187760582291006</v>
+        <v>0.3598737536762069</v>
       </c>
       <c r="F2" t="n">
-        <v>0.5392609699769053</v>
+        <v>0.5544440800262382</v>
       </c>
       <c r="G2" t="n">
-        <v>0.5625353685067882</v>
+        <v>0.5799455541157523</v>
       </c>
       <c r="H2" t="n">
-        <v>0.5613147775893503</v>
+        <v>0.5665725673950768</v>
       </c>
       <c r="I2" t="n">
-        <v>78.20965842167257</v>
+        <v>81.32231404958674</v>
       </c>
       <c r="J2" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="K2" t="n">
         <v>54.83</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M2" t="n">
         <v>54.83</v>
       </c>
       <c r="N2" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="O2" t="n">
         <v>97.87234042553192</v>
       </c>
       <c r="P2" t="n">
-        <v>69.50646808510639</v>
+        <v>65.50646808510639</v>
       </c>
       <c r="Q2" t="b">
         <v>0</v>
@@ -844,25 +844,25 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1129.4</v>
+        <v>1149.6</v>
       </c>
       <c r="D3" t="n">
-        <v>0.058481724461106</v>
+        <v>0.1166585721223893</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.0220798337518399</v>
+        <v>0.0260621206711886</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.1304280874653525</v>
+        <v>-0.1319842947749926</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.1071536889354696</v>
+        <v>-0.1064828206854785</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.1083742798529074</v>
+        <v>-0.119855807406154</v>
       </c>
       <c r="I3" t="n">
-        <v>67.32813607370656</v>
+        <v>68.27253957329656</v>
       </c>
       <c r="J3" t="n">
         <v>80</v>
@@ -872,7 +872,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M3" t="n">
@@ -909,25 +909,25 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>37790</v>
+        <v>38100</v>
       </c>
       <c r="D4" t="n">
-        <v>0.2435011516946363</v>
+        <v>0.307705508838167</v>
       </c>
       <c r="E4" t="n">
-        <v>0.035058887975897</v>
+        <v>0.0709768095572733</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.0093065932625507</v>
+        <v>-0.0057411273486429</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0139678052673321</v>
+        <v>0.0197603467408711</v>
       </c>
       <c r="H4" t="n">
-        <v>0.0127472143498942</v>
+        <v>0.0063873600201955</v>
       </c>
       <c r="I4" t="n">
-        <v>93.05092812946216</v>
+        <v>91.82072829131651</v>
       </c>
       <c r="J4" t="n">
         <v>60</v>
@@ -937,7 +937,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M4" t="n">
@@ -947,10 +947,10 @@
         <v>60</v>
       </c>
       <c r="O4" t="n">
-        <v>53.19148936170212</v>
+        <v>57.44680851063831</v>
       </c>
       <c r="P4" t="n">
-        <v>56.03029787234042</v>
+        <v>56.88136170212766</v>
       </c>
       <c r="Q4" t="b">
         <v>0</v>
@@ -974,25 +974,25 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>329.7</v>
+        <v>333.1</v>
       </c>
       <c r="D5" t="n">
-        <v>0.0893771683462745</v>
+        <v>0.1456577815993123</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.0368098159509203</v>
+        <v>0.007866868381240601</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.1562380038387716</v>
+        <v>-0.156815592962916</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.1329636053088887</v>
+        <v>-0.1313141188734019</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.1341841962263266</v>
+        <v>-0.1446871055940775</v>
       </c>
       <c r="I5" t="n">
-        <v>87.18861209964415</v>
+        <v>84.88982161594964</v>
       </c>
       <c r="J5" t="n">
         <v>60</v>
@@ -1002,7 +1002,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M5" t="n">
@@ -1012,10 +1012,10 @@
         <v>60</v>
       </c>
       <c r="O5" t="n">
-        <v>21.27659574468085</v>
+        <v>23.40425531914894</v>
       </c>
       <c r="P5" t="n">
-        <v>48.70331914893617</v>
+        <v>49.12885106382979</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
@@ -1039,25 +1039,25 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>123.19</v>
+        <v>124.7</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1039519670221345</v>
+        <v>0.1699033680457828</v>
       </c>
       <c r="E6" t="n">
-        <v>0.09667942668921919</v>
+        <v>0.1558068403003059</v>
       </c>
       <c r="F6" t="n">
-        <v>0.1660198769522005</v>
+        <v>0.1764150943396227</v>
       </c>
       <c r="G6" t="n">
-        <v>0.1892942754820834</v>
+        <v>0.2019165684291368</v>
       </c>
       <c r="H6" t="n">
-        <v>0.1880736845646455</v>
+        <v>0.1885435817084613</v>
       </c>
       <c r="I6" t="n">
-        <v>77.11889787361486</v>
+        <v>76.39060568603213</v>
       </c>
       <c r="J6" t="n">
         <v>70</v>
@@ -1067,7 +1067,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M6" t="n">
@@ -1104,25 +1104,25 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2873.1</v>
+        <v>2885.2</v>
       </c>
       <c r="D7" t="n">
-        <v>0.1323454065345051</v>
+        <v>0.1676244435451233</v>
       </c>
       <c r="E7" t="n">
-        <v>0.2053616378587011</v>
+        <v>0.2385490448594118</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.0722058965996059</v>
+        <v>-0.0644920722414967</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.048931498069723</v>
+        <v>-0.0389905981519826</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.0501520889871609</v>
+        <v>-0.0523635848726582</v>
       </c>
       <c r="I7" t="n">
-        <v>91.42990218910111</v>
+        <v>90.46879046879052</v>
       </c>
       <c r="J7" t="n">
         <v>60</v>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M7" t="n">
@@ -1142,10 +1142,10 @@
         <v>60</v>
       </c>
       <c r="O7" t="n">
-        <v>38.29787234042553</v>
+        <v>40.42553191489361</v>
       </c>
       <c r="P7" t="n">
-        <v>51.15157446808512</v>
+        <v>51.57710638297873</v>
       </c>
       <c r="Q7" t="b">
         <v>0</v>
@@ -1169,25 +1169,25 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>576.55</v>
+        <v>581.3</v>
       </c>
       <c r="D8" t="n">
-        <v>0.1388641975308642</v>
+        <v>0.198680276317146</v>
       </c>
       <c r="E8" t="n">
-        <v>0.2879481737964928</v>
+        <v>0.3035093620361027</v>
       </c>
       <c r="F8" t="n">
-        <v>0.4002428658166361</v>
+        <v>0.4049546827794561</v>
       </c>
       <c r="G8" t="n">
-        <v>0.423517264346519</v>
+        <v>0.4304561568689702</v>
       </c>
       <c r="H8" t="n">
-        <v>0.4222966734290811</v>
+        <v>0.4170831701482946</v>
       </c>
       <c r="I8" t="n">
-        <v>79.32736809626651</v>
+        <v>77.82191327375034</v>
       </c>
       <c r="J8" t="n">
         <v>70</v>
@@ -1197,7 +1197,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M8" t="n">
@@ -1207,10 +1207,10 @@
         <v>70</v>
       </c>
       <c r="O8" t="n">
-        <v>91.48936170212764</v>
+        <v>93.61702127659576</v>
       </c>
       <c r="P8" t="n">
-        <v>66.16187234042553</v>
+        <v>66.58740425531916</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
@@ -1234,25 +1234,25 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>441.4</v>
+        <v>441.95</v>
       </c>
       <c r="D9" t="n">
-        <v>0.0488297493168585</v>
+        <v>0.1062578222778471</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.1345946475835703</v>
+        <v>-0.1276154757204896</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.0667089544349297</v>
+        <v>-0.0549556292098791</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.0434345559050468</v>
+        <v>-0.029454155120365</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.0446551468224847</v>
+        <v>-0.0428271418410406</v>
       </c>
       <c r="I9" t="n">
-        <v>72.52321981424143</v>
+        <v>71.46302250803853</v>
       </c>
       <c r="J9" t="n">
         <v>70</v>
@@ -1262,7 +1262,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M9" t="n">
@@ -1272,10 +1272,10 @@
         <v>70</v>
       </c>
       <c r="O9" t="n">
-        <v>40.42553191489361</v>
+        <v>46.80851063829788</v>
       </c>
       <c r="P9" t="n">
-        <v>57.46110638297873</v>
+        <v>58.73770212765958</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -1299,25 +1299,25 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>139225</v>
+        <v>139665</v>
       </c>
       <c r="D10" t="n">
-        <v>0.0916611126357469</v>
+        <v>0.1175435087017402</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.0267048830787514</v>
+        <v>-0.0249240758194575</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.0452269921821423</v>
+        <v>-0.0610125050423557</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.0219525936522594</v>
+        <v>-0.0355110309528416</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.0231731845696973</v>
+        <v>-0.0488840176735172</v>
       </c>
       <c r="I10" t="n">
-        <v>74.18845807033364</v>
+        <v>74.00090826521344</v>
       </c>
       <c r="J10" t="n">
         <v>70</v>
@@ -1327,7 +1327,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M10" t="n">
@@ -1337,10 +1337,10 @@
         <v>70</v>
       </c>
       <c r="O10" t="n">
-        <v>44.68085106382978</v>
+        <v>42.5531914893617</v>
       </c>
       <c r="P10" t="n">
-        <v>56.70017021276595</v>
+        <v>56.27463829787234</v>
       </c>
       <c r="Q10" t="b">
         <v>0</v>
@@ -1376,10 +1376,10 @@
         <v>-0.0042030657656173</v>
       </c>
       <c r="G11" t="n">
-        <v>0.0190713327642655</v>
+        <v>0.0212984083238967</v>
       </c>
       <c r="H11" t="n">
-        <v>0.0178507418468276</v>
+        <v>0.0079254216032211</v>
       </c>
       <c r="I11" t="n">
         <v>27.6054590570719</v>
@@ -1392,7 +1392,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M11" t="n">
@@ -1402,10 +1402,10 @@
         <v>20</v>
       </c>
       <c r="O11" t="n">
-        <v>55.31914893617022</v>
+        <v>59.57446808510638</v>
       </c>
       <c r="P11" t="n">
-        <v>23.06382978723404</v>
+        <v>23.91489361702128</v>
       </c>
       <c r="Q11" t="b">
         <v>0</v>
@@ -1429,48 +1429,48 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>438.25</v>
+        <v>438.15</v>
       </c>
       <c r="D12" t="n">
-        <v>0.0709921798631476</v>
+        <v>0.1099430018999365</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.0441657579062159</v>
+        <v>-0.0118403247631935</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.1695091908281221</v>
+        <v>-0.1740810556079171</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.1462347922982392</v>
+        <v>-0.148579581518403</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.147455383215677</v>
+        <v>-0.1619525682390785</v>
       </c>
       <c r="I12" t="n">
-        <v>42.13075060532687</v>
+        <v>53.78670788253476</v>
       </c>
       <c r="J12" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K12" t="n">
         <v>71.28</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M12" t="n">
         <v>71.28</v>
       </c>
       <c r="N12" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O12" t="n">
-        <v>19.14893617021277</v>
+        <v>17.02127659574468</v>
       </c>
       <c r="P12" t="n">
-        <v>64.34178723404256</v>
+        <v>55.91625531914894</v>
       </c>
       <c r="Q12" t="b">
         <v>1</v>
@@ -1494,48 +1494,48 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1787.5</v>
+        <v>1803.9</v>
       </c>
       <c r="D13" t="n">
-        <v>0.0724785504289913</v>
+        <v>0.1476650973406286</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.06944661356655731</v>
+        <v>-0.0297439759036144</v>
       </c>
       <c r="F13" t="n">
-        <v>0.0347921732082898</v>
+        <v>0.0288011862666819</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0580665717381727</v>
+        <v>0.054302660356196</v>
       </c>
       <c r="H13" t="n">
-        <v>0.0568459808207348</v>
+        <v>0.0409296736355204</v>
       </c>
       <c r="I13" t="n">
-        <v>72.14443625644805</v>
+        <v>68.67619639527658</v>
       </c>
       <c r="J13" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="K13" t="n">
         <v>58.77</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M13" t="n">
         <v>58.77</v>
       </c>
       <c r="N13" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="O13" t="n">
         <v>61.70212765957447</v>
       </c>
       <c r="P13" t="n">
-        <v>55.8484255319149</v>
+        <v>59.8484255319149</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
@@ -1559,25 +1559,25 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>613.35</v>
+        <v>612.6</v>
       </c>
       <c r="D14" t="n">
-        <v>0.107729817590753</v>
+        <v>0.1727768737436583</v>
       </c>
       <c r="E14" t="n">
-        <v>0.0018784710878796</v>
+        <v>0.0672473867595819</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.2613800578034682</v>
+        <v>-0.2875501540966447</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.2381056592735853</v>
+        <v>-0.2620486800071306</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.2393262501910231</v>
+        <v>-0.2754216667278062</v>
       </c>
       <c r="I14" t="n">
-        <v>76.18933205189811</v>
+        <v>71.01699798329011</v>
       </c>
       <c r="J14" t="n">
         <v>70</v>
@@ -1587,7 +1587,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M14" t="n">
@@ -1597,10 +1597,10 @@
         <v>70</v>
       </c>
       <c r="O14" t="n">
-        <v>4.25531914893617</v>
+        <v>2.127659574468085</v>
       </c>
       <c r="P14" t="n">
-        <v>50.70706382978724</v>
+        <v>50.28153191489362</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
@@ -1624,48 +1624,48 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>108.05</v>
+        <v>108.92</v>
       </c>
       <c r="D15" t="n">
-        <v>0.101427115188583</v>
+        <v>0.1734539969834088</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.0019397746166636</v>
+        <v>-0.0137631293009778</v>
       </c>
       <c r="F15" t="n">
-        <v>0.2033634034970486</v>
+        <v>0.2253346833164584</v>
       </c>
       <c r="G15" t="n">
-        <v>0.2266378020269315</v>
+        <v>0.2508361574059725</v>
       </c>
       <c r="H15" t="n">
-        <v>0.2254172111094936</v>
+        <v>0.237463170685297</v>
       </c>
       <c r="I15" t="n">
-        <v>81.924539338988</v>
+        <v>79.73770491803278</v>
       </c>
       <c r="J15" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K15" t="n">
         <v>51.91</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M15" t="n">
         <v>51.91</v>
       </c>
       <c r="N15" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O15" t="n">
         <v>82.97872340425532</v>
       </c>
       <c r="P15" t="n">
-        <v>61.35974468085107</v>
+        <v>65.35974468085107</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
@@ -1689,25 +1689,25 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>180.19</v>
+        <v>180.77</v>
       </c>
       <c r="D16" t="n">
-        <v>0.132985412474849</v>
+        <v>0.2187837108953614</v>
       </c>
       <c r="E16" t="n">
-        <v>0.1331279084391898</v>
+        <v>0.1949365415124273</v>
       </c>
       <c r="F16" t="n">
-        <v>0.001333703806613</v>
+        <v>-0.0296312201406407</v>
       </c>
       <c r="G16" t="n">
-        <v>0.0246081023364959</v>
+        <v>-0.0041297460511267</v>
       </c>
       <c r="H16" t="n">
-        <v>0.023387511419058</v>
+        <v>-0.0175027327718022</v>
       </c>
       <c r="I16" t="n">
-        <v>86.69399925456577</v>
+        <v>81.79035960214229</v>
       </c>
       <c r="J16" t="n">
         <v>60</v>
@@ -1717,7 +1717,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M16" t="n">
@@ -1727,16 +1727,16 @@
         <v>60</v>
       </c>
       <c r="O16" t="n">
-        <v>57.44680851063831</v>
+        <v>51.06382978723404</v>
       </c>
       <c r="P16" t="n">
-        <v>56.53336170212766</v>
+        <v>55.2567659574468</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>
       </c>
       <c r="R16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S16" t="b">
         <v>0</v>
@@ -1754,48 +1754,48 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>7721.5</v>
+        <v>7653</v>
       </c>
       <c r="D17" t="n">
-        <v>0.1171151620370369</v>
+        <v>0.169021614603223</v>
       </c>
       <c r="E17" t="n">
-        <v>0.0154523934771173</v>
+        <v>0.0327935222672064</v>
       </c>
       <c r="F17" t="n">
-        <v>0.1366011628762788</v>
+        <v>0.1394327402665078</v>
       </c>
       <c r="G17" t="n">
-        <v>0.1598755614061617</v>
+        <v>0.1649342143560219</v>
       </c>
       <c r="H17" t="n">
-        <v>0.1586549704887239</v>
+        <v>0.1515612276353464</v>
       </c>
       <c r="I17" t="n">
-        <v>79.25343811394892</v>
+        <v>83.90183028286189</v>
       </c>
       <c r="J17" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="K17" t="n">
         <v>54.65</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M17" t="n">
         <v>54.65</v>
       </c>
       <c r="N17" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="O17" t="n">
         <v>70.21276595744681</v>
       </c>
       <c r="P17" t="n">
-        <v>63.90255319148936</v>
+        <v>59.90255319148936</v>
       </c>
       <c r="Q17" t="b">
         <v>0</v>
@@ -1819,48 +1819,48 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>755.45</v>
+        <v>748.1</v>
       </c>
       <c r="D18" t="n">
-        <v>0.0715602836879434</v>
+        <v>0.1359805633588946</v>
       </c>
       <c r="E18" t="n">
-        <v>0.2559434746467166</v>
+        <v>0.2627225926238501</v>
       </c>
       <c r="F18" t="n">
-        <v>0.142976019366064</v>
+        <v>0.1160674324929136</v>
       </c>
       <c r="G18" t="n">
-        <v>0.1662504178959469</v>
+        <v>0.1415689065824277</v>
       </c>
       <c r="H18" t="n">
-        <v>0.1650298269785091</v>
+        <v>0.1281959198617521</v>
       </c>
       <c r="I18" t="n">
-        <v>83.14740090197014</v>
+        <v>78.78187670215402</v>
       </c>
       <c r="J18" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K18" t="n">
         <v>49.92</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M18" t="n">
         <v>49.92</v>
       </c>
       <c r="N18" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O18" t="n">
-        <v>72.3404255319149</v>
+        <v>68.08510638297872</v>
       </c>
       <c r="P18" t="n">
-        <v>58.43608510638298</v>
+        <v>61.58502127659575</v>
       </c>
       <c r="Q18" t="b">
         <v>0</v>
@@ -1884,25 +1884,25 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2358.1</v>
+        <v>2389.8</v>
       </c>
       <c r="D19" t="n">
-        <v>0.0341183177652062</v>
+        <v>0.08155322230267931</v>
       </c>
       <c r="E19" t="n">
-        <v>-0.0743473994111875</v>
+        <v>-0.0341120362137254</v>
       </c>
       <c r="F19" t="n">
-        <v>-0.1410723391855468</v>
+        <v>-0.1503235440517669</v>
       </c>
       <c r="G19" t="n">
-        <v>-0.1177979406556639</v>
+        <v>-0.1248220699622528</v>
       </c>
       <c r="H19" t="n">
-        <v>-0.1190185315731018</v>
+        <v>-0.1381950566829284</v>
       </c>
       <c r="I19" t="n">
-        <v>66.49130832570901</v>
+        <v>65.99350046425253</v>
       </c>
       <c r="J19" t="n">
         <v>60</v>
@@ -1912,7 +1912,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M19" t="n">
@@ -1949,25 +1949,25 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2250.5</v>
+        <v>2267.8</v>
       </c>
       <c r="D20" t="n">
-        <v>0.1103710282218275</v>
+        <v>0.1661438782331465</v>
       </c>
       <c r="E20" t="n">
-        <v>0.0354267310789049</v>
+        <v>0.0712834805611979</v>
       </c>
       <c r="F20" t="n">
-        <v>0.1801258521237545</v>
+        <v>0.1548019146552604</v>
       </c>
       <c r="G20" t="n">
-        <v>0.2034002506536374</v>
+        <v>0.1803033887447744</v>
       </c>
       <c r="H20" t="n">
-        <v>0.2021796597361995</v>
+        <v>0.1669304020240989</v>
       </c>
       <c r="I20" t="n">
-        <v>85.21360431356281</v>
+        <v>83.63552903373879</v>
       </c>
       <c r="J20" t="n">
         <v>60</v>
@@ -1977,7 +1977,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M20" t="n">
@@ -1987,10 +1987,10 @@
         <v>60</v>
       </c>
       <c r="O20" t="n">
-        <v>78.72340425531915</v>
+        <v>72.3404255319149</v>
       </c>
       <c r="P20" t="n">
-        <v>59.36868085106384</v>
+        <v>58.09208510638298</v>
       </c>
       <c r="Q20" t="b">
         <v>0</v>
@@ -2014,25 +2014,25 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1017.85</v>
+        <v>1016</v>
       </c>
       <c r="D21" t="n">
-        <v>0.1795005504374529</v>
+        <v>0.2226233453670276</v>
       </c>
       <c r="E21" t="n">
-        <v>0.1000216146114774</v>
+        <v>0.1477632173520107</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.138437447096665</v>
+        <v>-0.1813713641124807</v>
       </c>
       <c r="G21" t="n">
-        <v>-0.1151630485667821</v>
+        <v>-0.1558698900229667</v>
       </c>
       <c r="H21" t="n">
-        <v>-0.11638363948422</v>
+        <v>-0.1692428767436422</v>
       </c>
       <c r="I21" t="n">
-        <v>92.236435818262</v>
+        <v>89.69263381028085</v>
       </c>
       <c r="J21" t="n">
         <v>60</v>
@@ -2042,7 +2042,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M21" t="n">
@@ -2052,10 +2052,10 @@
         <v>60</v>
       </c>
       <c r="O21" t="n">
-        <v>27.65957446808511</v>
+        <v>14.8936170212766</v>
       </c>
       <c r="P21" t="n">
-        <v>48.90391489361702</v>
+        <v>46.35072340425532</v>
       </c>
       <c r="Q21" t="b">
         <v>0</v>
@@ -2079,25 +2079,25 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>448.5</v>
+        <v>450.65</v>
       </c>
       <c r="D22" t="n">
-        <v>0.1948847742107364</v>
+        <v>0.2662264681090194</v>
       </c>
       <c r="E22" t="n">
-        <v>0.2741477272727273</v>
+        <v>0.3238836662749706</v>
       </c>
       <c r="F22" t="n">
-        <v>0.4538087520259319</v>
+        <v>0.4383977018831788</v>
       </c>
       <c r="G22" t="n">
-        <v>0.4770831505558148</v>
+        <v>0.4638991759726929</v>
       </c>
       <c r="H22" t="n">
-        <v>0.475862559638377</v>
+        <v>0.4505261892520174</v>
       </c>
       <c r="I22" t="n">
-        <v>85.03816793893128</v>
+        <v>82.40574506283662</v>
       </c>
       <c r="J22" t="n">
         <v>60</v>
@@ -2107,7 +2107,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M22" t="n">
@@ -2144,25 +2144,25 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>393.15</v>
+        <v>393.55</v>
       </c>
       <c r="D23" t="n">
-        <v>0.1542865531415147</v>
+        <v>0.198933739527799</v>
       </c>
       <c r="E23" t="n">
-        <v>-0.0030429821224801</v>
+        <v>0.0314506617743415</v>
       </c>
       <c r="F23" t="n">
-        <v>0.0035737077217612</v>
+        <v>-0.0078154544308584</v>
       </c>
       <c r="G23" t="n">
-        <v>0.0268481062516441</v>
+        <v>0.0176860196586556</v>
       </c>
       <c r="H23" t="n">
-        <v>0.0256275153342062</v>
+        <v>0.0043130329379801</v>
       </c>
       <c r="I23" t="n">
-        <v>83.40389500423369</v>
+        <v>80.76545632973502</v>
       </c>
       <c r="J23" t="n">
         <v>60</v>
@@ -2172,7 +2172,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M23" t="n">
@@ -2182,10 +2182,10 @@
         <v>60</v>
       </c>
       <c r="O23" t="n">
-        <v>59.57446808510638</v>
+        <v>55.31914893617022</v>
       </c>
       <c r="P23" t="n">
-        <v>55.79489361702128</v>
+        <v>54.94382978723405</v>
       </c>
       <c r="Q23" t="b">
         <v>0</v>
@@ -2209,48 +2209,48 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>126.11</v>
+        <v>124.33</v>
       </c>
       <c r="D24" t="n">
-        <v>0.0537266042780748</v>
+        <v>0.1057452863749555</v>
       </c>
       <c r="E24" t="n">
-        <v>0.0314902666448551</v>
+        <v>0.0627404051628344</v>
       </c>
       <c r="F24" t="n">
-        <v>0.253204809698897</v>
+        <v>0.2319659135949265</v>
       </c>
       <c r="G24" t="n">
-        <v>0.2764792082287799</v>
+        <v>0.2574673876844406</v>
       </c>
       <c r="H24" t="n">
-        <v>0.275258617311342</v>
+        <v>0.2440944009637651</v>
       </c>
       <c r="I24" t="n">
-        <v>70.89837997054492</v>
+        <v>57.90613718411552</v>
       </c>
       <c r="J24" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="K24" t="n">
         <v>48.3</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M24" t="n">
         <v>48.3</v>
       </c>
       <c r="N24" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="O24" t="n">
         <v>85.1063829787234</v>
       </c>
       <c r="P24" t="n">
-        <v>56.34127659574468</v>
+        <v>60.34127659574468</v>
       </c>
       <c r="Q24" t="b">
         <v>0</v>
@@ -2274,25 +2274,25 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>615.65</v>
+        <v>626</v>
       </c>
       <c r="D25" t="n">
-        <v>0.0853239312472453</v>
+        <v>0.15775846125393</v>
       </c>
       <c r="E25" t="n">
-        <v>0.0491649625085208</v>
+        <v>0.1125921976361858</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.081462140992167</v>
+        <v>-0.08123578190357381</v>
       </c>
       <c r="G25" t="n">
-        <v>-0.0581877424622842</v>
+        <v>-0.0557343078140597</v>
       </c>
       <c r="H25" t="n">
-        <v>-0.059408333379722</v>
+        <v>-0.0691072945347353</v>
       </c>
       <c r="I25" t="n">
-        <v>89.12704598597035</v>
+        <v>84.96767241379307</v>
       </c>
       <c r="J25" t="n">
         <v>60</v>
@@ -2302,7 +2302,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M25" t="n">
@@ -2339,48 +2339,48 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>132.25</v>
+        <v>129.13</v>
       </c>
       <c r="D26" t="n">
-        <v>0.0391294099159267</v>
+        <v>0.0753664223850765</v>
       </c>
       <c r="E26" t="n">
-        <v>-0.0689242466910728</v>
+        <v>-0.06298526957405121</v>
       </c>
       <c r="F26" t="n">
-        <v>-0.1894956180670466</v>
+        <v>-0.2083742030407063</v>
       </c>
       <c r="G26" t="n">
-        <v>-0.1662212195371637</v>
+        <v>-0.1828727289511922</v>
       </c>
       <c r="H26" t="n">
-        <v>-0.1674418104546016</v>
+        <v>-0.1962457156718677</v>
       </c>
       <c r="I26" t="n">
-        <v>77.04194260485642</v>
+        <v>58.41848067525539</v>
       </c>
       <c r="J26" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="K26" t="n">
         <v>51.54</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M26" t="n">
         <v>51.54</v>
       </c>
       <c r="N26" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="O26" t="n">
         <v>10.63829787234042</v>
       </c>
       <c r="P26" t="n">
-        <v>42.74365957446808</v>
+        <v>46.74365957446808</v>
       </c>
       <c r="Q26" t="b">
         <v>0</v>
@@ -2404,25 +2404,25 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>5517.1</v>
+        <v>5506.4</v>
       </c>
       <c r="D27" t="n">
-        <v>0.09130649787360311</v>
+        <v>0.1452579034941763</v>
       </c>
       <c r="E27" t="n">
-        <v>0.0294057281462822</v>
+        <v>0.057804245509557</v>
       </c>
       <c r="F27" t="n">
-        <v>0.09225713210983751</v>
+        <v>0.0758890191481047</v>
       </c>
       <c r="G27" t="n">
-        <v>0.1155315306397204</v>
+        <v>0.1013904932376188</v>
       </c>
       <c r="H27" t="n">
-        <v>0.1143109397222825</v>
+        <v>0.08801750651694321</v>
       </c>
       <c r="I27" t="n">
-        <v>79.28741092636581</v>
+        <v>76.29801920768305</v>
       </c>
       <c r="J27" t="n">
         <v>70</v>
@@ -2432,7 +2432,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M27" t="n">
@@ -2442,10 +2442,10 @@
         <v>70</v>
       </c>
       <c r="O27" t="n">
-        <v>63.82978723404256</v>
+        <v>65.95744680851064</v>
       </c>
       <c r="P27" t="n">
-        <v>63.84195744680851</v>
+        <v>64.26748936170213</v>
       </c>
       <c r="Q27" t="b">
         <v>0</v>
@@ -2469,25 +2469,25 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1795.4</v>
+        <v>1774.8</v>
       </c>
       <c r="D28" t="n">
-        <v>0.1450255102040816</v>
+        <v>0.1988651715752498</v>
       </c>
       <c r="E28" t="n">
-        <v>0.2136821469614007</v>
+        <v>0.302988033184054</v>
       </c>
       <c r="F28" t="n">
-        <v>0.4365498479756762</v>
+        <v>0.3464835748425765</v>
       </c>
       <c r="G28" t="n">
-        <v>0.4598242465055591</v>
+        <v>0.3719850489320906</v>
       </c>
       <c r="H28" t="n">
-        <v>0.4586036555881212</v>
+        <v>0.358612062211415</v>
       </c>
       <c r="I28" t="n">
-        <v>78.86728655959428</v>
+        <v>71.45562130177515</v>
       </c>
       <c r="J28" t="n">
         <v>70</v>
@@ -2497,7 +2497,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M28" t="n">
@@ -2507,10 +2507,10 @@
         <v>70</v>
       </c>
       <c r="O28" t="n">
-        <v>93.61702127659576</v>
+        <v>91.48936170212764</v>
       </c>
       <c r="P28" t="n">
-        <v>68.52740425531915</v>
+        <v>68.10187234042553</v>
       </c>
       <c r="Q28" t="b">
         <v>0</v>
@@ -2534,25 +2534,25 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>537.95</v>
+        <v>544.45</v>
       </c>
       <c r="D29" t="n">
-        <v>0.070547263681592</v>
+        <v>0.1091983294285423</v>
       </c>
       <c r="E29" t="n">
-        <v>-0.01257342143906</v>
+        <v>0.0154807423295719</v>
       </c>
       <c r="F29" t="n">
-        <v>-0.0553165334972342</v>
+        <v>-0.0609692997585372</v>
       </c>
       <c r="G29" t="n">
-        <v>-0.0320421349673513</v>
+        <v>-0.0354678256690231</v>
       </c>
       <c r="H29" t="n">
-        <v>-0.0332627258847891</v>
+        <v>-0.0488408123896987</v>
       </c>
       <c r="I29" t="n">
-        <v>62.30945121951223</v>
+        <v>61.7260061919505</v>
       </c>
       <c r="J29" t="n">
         <v>80</v>
@@ -2562,7 +2562,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M29" t="n">
@@ -2572,10 +2572,10 @@
         <v>80</v>
       </c>
       <c r="O29" t="n">
-        <v>42.5531914893617</v>
+        <v>44.68085106382978</v>
       </c>
       <c r="P29" t="n">
-        <v>60.27863829787234</v>
+        <v>60.70417021276596</v>
       </c>
       <c r="Q29" t="b">
         <v>0</v>
@@ -2599,48 +2599,48 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>123.98</v>
+        <v>125.62</v>
       </c>
       <c r="D30" t="n">
-        <v>0.0496994327321989</v>
+        <v>0.1159278671049126</v>
       </c>
       <c r="E30" t="n">
-        <v>-0.0244708474309544</v>
+        <v>0.0289130968957327</v>
       </c>
       <c r="F30" t="n">
-        <v>-0.0332189644416719</v>
+        <v>-0.0255216817934992</v>
       </c>
       <c r="G30" t="n">
-        <v>-0.009944565911788999</v>
+        <v>-2.020770398514227e-05</v>
       </c>
       <c r="H30" t="n">
-        <v>-0.0111651568292269</v>
+        <v>-0.0133931944246606</v>
       </c>
       <c r="I30" t="n">
-        <v>81.58128516434705</v>
+        <v>79.41760423560557</v>
       </c>
       <c r="J30" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K30" t="n">
         <v>52.38</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M30" t="n">
         <v>52.38</v>
       </c>
       <c r="N30" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O30" t="n">
-        <v>48.93617021276596</v>
+        <v>53.19148936170212</v>
       </c>
       <c r="P30" t="n">
-        <v>54.73923404255319</v>
+        <v>59.59029787234042</v>
       </c>
       <c r="Q30" t="b">
         <v>0</v>
@@ -2664,48 +2664,48 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>39.19</v>
+        <v>40.01</v>
       </c>
       <c r="D31" t="n">
-        <v>0.0597620335316386</v>
+        <v>0.1147952075787126</v>
       </c>
       <c r="E31" t="n">
-        <v>-0.1260035682426405</v>
+        <v>-0.08044127786715689</v>
       </c>
       <c r="F31" t="n">
-        <v>-0.1426383723474076</v>
+        <v>-0.1271815008726005</v>
       </c>
       <c r="G31" t="n">
-        <v>-0.1193639738175247</v>
+        <v>-0.1016800267830864</v>
       </c>
       <c r="H31" t="n">
-        <v>-0.1205845647349626</v>
+        <v>-0.1150530135037619</v>
       </c>
       <c r="I31" t="n">
-        <v>64.69833119383821</v>
+        <v>62.38030095759229</v>
       </c>
       <c r="J31" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K31" t="n">
         <v>48.99</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M31" t="n">
         <v>48.99</v>
       </c>
       <c r="N31" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O31" t="n">
-        <v>23.40425531914894</v>
+        <v>31.91489361702128</v>
       </c>
       <c r="P31" t="n">
-        <v>48.27685106382979</v>
+        <v>57.97897872340426</v>
       </c>
       <c r="Q31" t="b">
         <v>0</v>
@@ -2729,25 +2729,25 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>748.75</v>
+        <v>754.25</v>
       </c>
       <c r="D32" t="n">
-        <v>0.09859878218766061</v>
+        <v>0.1787919043525825</v>
       </c>
       <c r="E32" t="n">
-        <v>0.0484492053490164</v>
+        <v>0.0880698211194459</v>
       </c>
       <c r="F32" t="n">
-        <v>-0.2663629237703312</v>
+        <v>-0.2768456375838926</v>
       </c>
       <c r="G32" t="n">
-        <v>-0.2430885252404483</v>
+        <v>-0.2513441634943785</v>
       </c>
       <c r="H32" t="n">
-        <v>-0.2443091161578862</v>
+        <v>-0.264717150215054</v>
       </c>
       <c r="I32" t="n">
-        <v>89.74358974358977</v>
+        <v>85.83929992044554</v>
       </c>
       <c r="J32" t="n">
         <v>60</v>
@@ -2757,7 +2757,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M32" t="n">
@@ -2767,10 +2767,10 @@
         <v>60</v>
       </c>
       <c r="O32" t="n">
-        <v>2.127659574468085</v>
+        <v>4.25531914893617</v>
       </c>
       <c r="P32" t="n">
-        <v>43.56953191489362</v>
+        <v>43.99506382978724</v>
       </c>
       <c r="Q32" t="b">
         <v>0</v>
@@ -2794,25 +2794,25 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>588.45</v>
+        <v>605.45</v>
       </c>
       <c r="D33" t="n">
-        <v>0.1028956986224347</v>
+        <v>0.1850655705617538</v>
       </c>
       <c r="E33" t="n">
-        <v>0.0077061392242485</v>
+        <v>0.0545153705477663</v>
       </c>
       <c r="F33" t="n">
-        <v>0.0999065420560747</v>
+        <v>0.1565425023877746</v>
       </c>
       <c r="G33" t="n">
-        <v>0.1231809405859576</v>
+        <v>0.1820439764772887</v>
       </c>
       <c r="H33" t="n">
-        <v>0.1219603496685197</v>
+        <v>0.1686709897566132</v>
       </c>
       <c r="I33" t="n">
-        <v>83.29611433675754</v>
+        <v>82.1819914244879</v>
       </c>
       <c r="J33" t="n">
         <v>60</v>
@@ -2822,7 +2822,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M33" t="n">
@@ -2832,10 +2832,10 @@
         <v>60</v>
       </c>
       <c r="O33" t="n">
-        <v>65.95744680851064</v>
+        <v>74.46808510638297</v>
       </c>
       <c r="P33" t="n">
-        <v>57.18348936170213</v>
+        <v>58.8856170212766</v>
       </c>
       <c r="Q33" t="b">
         <v>0</v>
@@ -2871,10 +2871,10 @@
         <v>-0.2401052253975846</v>
       </c>
       <c r="G34" t="n">
-        <v>-0.2168308268677017</v>
+        <v>-0.2146037513080705</v>
       </c>
       <c r="H34" t="n">
-        <v>-0.2180514177851396</v>
+        <v>-0.227976738028746</v>
       </c>
       <c r="I34" t="n">
         <v>63.3225806451613</v>
@@ -2887,7 +2887,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M34" t="n">
@@ -2924,48 +2924,48 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>115.9</v>
+        <v>116.08</v>
       </c>
       <c r="D35" t="n">
-        <v>0.0615497343835866</v>
+        <v>0.1267715006794798</v>
       </c>
       <c r="E35" t="n">
-        <v>-0.0358539223026369</v>
+        <v>-0.00326292289198</v>
       </c>
       <c r="F35" t="n">
-        <v>0.2558240329396468</v>
+        <v>0.2375266524520256</v>
       </c>
       <c r="G35" t="n">
-        <v>0.2790984314695297</v>
+        <v>0.2630281265415397</v>
       </c>
       <c r="H35" t="n">
-        <v>0.2778778405520918</v>
+        <v>0.2496551398208641</v>
       </c>
       <c r="I35" t="n">
-        <v>76.25212947189098</v>
+        <v>67.62656758012076</v>
       </c>
       <c r="J35" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="K35" t="n">
         <v>49.07</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M35" t="n">
         <v>49.07</v>
       </c>
       <c r="N35" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="O35" t="n">
         <v>87.2340425531915</v>
       </c>
       <c r="P35" t="n">
-        <v>57.07480851063831</v>
+        <v>69.07480851063831</v>
       </c>
       <c r="Q35" t="b">
         <v>0</v>
@@ -2989,48 +2989,48 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>494.25</v>
+        <v>488.7</v>
       </c>
       <c r="D36" t="n">
-        <v>0.035512256442489</v>
+        <v>0.0906047757197052</v>
       </c>
       <c r="E36" t="n">
-        <v>-0.0703470328223454</v>
+        <v>-0.0418586413096755</v>
       </c>
       <c r="F36" t="n">
-        <v>0.1110486680903675</v>
+        <v>0.072886937431394</v>
       </c>
       <c r="G36" t="n">
-        <v>0.1343230666202504</v>
+        <v>0.0983884115209081</v>
       </c>
       <c r="H36" t="n">
-        <v>0.1331024757028125</v>
+        <v>0.08501542480023259</v>
       </c>
       <c r="I36" t="n">
-        <v>78.04997550220479</v>
+        <v>66.80522565320663</v>
       </c>
       <c r="J36" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K36" t="n">
         <v>47.8</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M36" t="n">
         <v>47.8</v>
       </c>
       <c r="N36" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O36" t="n">
-        <v>68.08510638297872</v>
+        <v>63.82978723404256</v>
       </c>
       <c r="P36" t="n">
-        <v>60.73702127659575</v>
+        <v>63.88595744680852</v>
       </c>
       <c r="Q36" t="b">
         <v>0</v>
@@ -3054,25 +3054,25 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2275.5</v>
+        <v>2374.6</v>
       </c>
       <c r="D37" t="n">
-        <v>0.0448138114697644</v>
+        <v>0.1615143807474075</v>
       </c>
       <c r="E37" t="n">
-        <v>0.2626935242217414</v>
+        <v>0.3499715747583853</v>
       </c>
       <c r="F37" t="n">
-        <v>0.6582859641451684</v>
+        <v>0.6933609070812237</v>
       </c>
       <c r="G37" t="n">
-        <v>0.6815603626750513</v>
+        <v>0.7188623811707378</v>
       </c>
       <c r="H37" t="n">
-        <v>0.6803397717576134</v>
+        <v>0.7054893944500622</v>
       </c>
       <c r="I37" t="n">
-        <v>71.54802744425388</v>
+        <v>73.33199356913184</v>
       </c>
       <c r="J37" t="n">
         <v>70</v>
@@ -3082,7 +3082,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M37" t="n">
@@ -3119,25 +3119,25 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>860.9</v>
+        <v>864.7</v>
       </c>
       <c r="D38" t="n">
-        <v>0.0948051122273796</v>
+        <v>0.1584941050375135</v>
       </c>
       <c r="E38" t="n">
-        <v>0.0241494170830358</v>
+        <v>0.025558915969875</v>
       </c>
       <c r="F38" t="n">
-        <v>-0.1769598470363289</v>
+        <v>-0.1823167848699762</v>
       </c>
       <c r="G38" t="n">
-        <v>-0.153685448506446</v>
+        <v>-0.1568153107804621</v>
       </c>
       <c r="H38" t="n">
-        <v>-0.1549060394238839</v>
+        <v>-0.1701882975011377</v>
       </c>
       <c r="I38" t="n">
-        <v>85.45918367346941</v>
+        <v>83.08605341246295</v>
       </c>
       <c r="J38" t="n">
         <v>60</v>
@@ -3147,7 +3147,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M38" t="n">
@@ -3157,10 +3157,10 @@
         <v>60</v>
       </c>
       <c r="O38" t="n">
-        <v>14.8936170212766</v>
+        <v>12.76595744680851</v>
       </c>
       <c r="P38" t="n">
-        <v>46.92672340425532</v>
+        <v>46.5011914893617</v>
       </c>
       <c r="Q38" t="b">
         <v>0</v>
@@ -3184,25 +3184,25 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>3627.6</v>
+        <v>3586.8</v>
       </c>
       <c r="D39" t="n">
-        <v>0.1608319999999998</v>
+        <v>0.2208304969366916</v>
       </c>
       <c r="E39" t="n">
-        <v>0.2799379013478231</v>
+        <v>0.3096724723408919</v>
       </c>
       <c r="F39" t="n">
-        <v>0.3458984157607685</v>
+        <v>0.3102944399795426</v>
       </c>
       <c r="G39" t="n">
-        <v>0.3691728142906514</v>
+        <v>0.3357959140690567</v>
       </c>
       <c r="H39" t="n">
-        <v>0.3679522233732135</v>
+        <v>0.3224229273483812</v>
       </c>
       <c r="I39" t="n">
-        <v>77.81013925548373</v>
+        <v>74.83197736116026</v>
       </c>
       <c r="J39" t="n">
         <v>70</v>
@@ -3212,7 +3212,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M39" t="n">
@@ -3249,25 +3249,25 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>217.76</v>
+        <v>217.4</v>
       </c>
       <c r="D40" t="n">
-        <v>0.1741615442683057</v>
+        <v>0.2024336283185841</v>
       </c>
       <c r="E40" t="n">
-        <v>0.1195886889460153</v>
+        <v>0.1419266729698498</v>
       </c>
       <c r="F40" t="n">
-        <v>-0.0331660968787461</v>
+        <v>-0.0504062199702978</v>
       </c>
       <c r="G40" t="n">
-        <v>-0.0098916983488632</v>
+        <v>-0.0249047458807837</v>
       </c>
       <c r="H40" t="n">
-        <v>-0.0111122892663011</v>
+        <v>-0.0382777326014592</v>
       </c>
       <c r="I40" t="n">
-        <v>91.93691298954457</v>
+        <v>87.51271617497457</v>
       </c>
       <c r="J40" t="n">
         <v>60</v>
@@ -3277,7 +3277,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M40" t="n">
@@ -3287,10 +3287,10 @@
         <v>60</v>
       </c>
       <c r="O40" t="n">
-        <v>51.06382978723404</v>
+        <v>48.93617021276596</v>
       </c>
       <c r="P40" t="n">
-        <v>52.38876595744681</v>
+        <v>51.9632340425532</v>
       </c>
       <c r="Q40" t="b">
         <v>0</v>
@@ -3314,25 +3314,25 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>828.95</v>
+        <v>835.25</v>
       </c>
       <c r="D41" t="n">
-        <v>0.0196186961869619</v>
+        <v>0.0481239804241435</v>
       </c>
       <c r="E41" t="n">
-        <v>-0.1045638671347555</v>
+        <v>-0.0918234206806567</v>
       </c>
       <c r="F41" t="n">
-        <v>-0.1697215544871794</v>
+        <v>-0.1733471892319873</v>
       </c>
       <c r="G41" t="n">
-        <v>-0.1464471559572965</v>
+        <v>-0.1478457151424732</v>
       </c>
       <c r="H41" t="n">
-        <v>-0.1476677468747343</v>
+        <v>-0.1612187018631488</v>
       </c>
       <c r="I41" t="n">
-        <v>78.25318246110326</v>
+        <v>78.6235662148071</v>
       </c>
       <c r="J41" t="n">
         <v>50</v>
@@ -3342,7 +3342,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M41" t="n">
@@ -3352,10 +3352,10 @@
         <v>50</v>
       </c>
       <c r="O41" t="n">
-        <v>17.02127659574468</v>
+        <v>19.14893617021277</v>
       </c>
       <c r="P41" t="n">
-        <v>42.62425531914894</v>
+        <v>43.04978723404256</v>
       </c>
       <c r="Q41" t="b">
         <v>0</v>
@@ -3379,25 +3379,25 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>616.15</v>
+        <v>621.2</v>
       </c>
       <c r="D42" t="n">
-        <v>0.1626568544202282</v>
+        <v>0.2161315583398591</v>
       </c>
       <c r="E42" t="n">
-        <v>-0.0281545741324921</v>
+        <v>0.0310373443983402</v>
       </c>
       <c r="F42" t="n">
-        <v>-0.1869763145741242</v>
+        <v>-0.1733315589859604</v>
       </c>
       <c r="G42" t="n">
-        <v>-0.1637019160442413</v>
+        <v>-0.1478300848964463</v>
       </c>
       <c r="H42" t="n">
-        <v>-0.1649225069616792</v>
+        <v>-0.1612030716171218</v>
       </c>
       <c r="I42" t="n">
-        <v>84.09296028880863</v>
+        <v>81.83457871682553</v>
       </c>
       <c r="J42" t="n">
         <v>60</v>
@@ -3407,7 +3407,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M42" t="n">
@@ -3417,10 +3417,10 @@
         <v>60</v>
       </c>
       <c r="O42" t="n">
-        <v>12.76595744680851</v>
+        <v>21.27659574468085</v>
       </c>
       <c r="P42" t="n">
-        <v>45.6171914893617</v>
+        <v>47.31931914893617</v>
       </c>
       <c r="Q42" t="b">
         <v>0</v>
@@ -3444,48 +3444,48 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>414.4</v>
+        <v>422.1</v>
       </c>
       <c r="D43" t="n">
-        <v>0.029437336976773</v>
+        <v>0.0547226386806598</v>
       </c>
       <c r="E43" t="n">
-        <v>-0.085815133465696</v>
+        <v>-0.0369609856262833</v>
       </c>
       <c r="F43" t="n">
-        <v>-0.104580812445981</v>
+        <v>-0.0901056262125457</v>
       </c>
       <c r="G43" t="n">
-        <v>-0.08130641391609809</v>
+        <v>-0.0646041521230316</v>
       </c>
       <c r="H43" t="n">
-        <v>-0.08252700483353601</v>
+        <v>-0.07797713884370711</v>
       </c>
       <c r="I43" t="n">
-        <v>56.14789337919173</v>
+        <v>50.07342143906023</v>
       </c>
       <c r="J43" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="K43" t="n">
         <v>51.48</v>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M43" t="n">
         <v>51.48</v>
       </c>
       <c r="N43" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="O43" t="n">
         <v>34.04255319148936</v>
       </c>
       <c r="P43" t="n">
-        <v>43.40051063829787</v>
+        <v>59.40051063829787</v>
       </c>
       <c r="Q43" t="b">
         <v>0</v>
@@ -3509,25 +3509,25 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>281.41</v>
+        <v>279.95</v>
       </c>
       <c r="D44" t="n">
-        <v>0.1896427816529275</v>
+        <v>0.2475490196078431</v>
       </c>
       <c r="E44" t="n">
-        <v>0.142781725888325</v>
+        <v>0.1827207435572455</v>
       </c>
       <c r="F44" t="n">
-        <v>-0.0421715452688903</v>
+        <v>-0.0665221740580193</v>
       </c>
       <c r="G44" t="n">
-        <v>-0.0188971467390074</v>
+        <v>-0.0410206999685052</v>
       </c>
       <c r="H44" t="n">
-        <v>-0.0201177376564453</v>
+        <v>-0.0543936866891807</v>
       </c>
       <c r="I44" t="n">
-        <v>99.6795513719207</v>
+        <v>95.93781344032088</v>
       </c>
       <c r="J44" t="n">
         <v>60</v>
@@ -3537,7 +3537,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M44" t="n">
@@ -3547,10 +3547,10 @@
         <v>60</v>
       </c>
       <c r="O44" t="n">
-        <v>46.80851063829788</v>
+        <v>38.29787234042553</v>
       </c>
       <c r="P44" t="n">
-        <v>52.24170212765958</v>
+        <v>50.53957446808511</v>
       </c>
       <c r="Q44" t="b">
         <v>0</v>
@@ -3574,25 +3574,25 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>102.88</v>
+        <v>104.01</v>
       </c>
       <c r="D45" t="n">
-        <v>0.0564797699733004</v>
+        <v>0.1269910066096</v>
       </c>
       <c r="E45" t="n">
-        <v>-0.1286524942830523</v>
+        <v>-0.0950143565648655</v>
       </c>
       <c r="F45" t="n">
-        <v>-0.2450282527335437</v>
+        <v>-0.2476128472222222</v>
       </c>
       <c r="G45" t="n">
-        <v>-0.2217538542036609</v>
+        <v>-0.2221113731327081</v>
       </c>
       <c r="H45" t="n">
-        <v>-0.2229744451210987</v>
+        <v>-0.2354843598533836</v>
       </c>
       <c r="I45" t="n">
-        <v>89.72798854688621</v>
+        <v>87.52173913043481</v>
       </c>
       <c r="J45" t="n">
         <v>60</v>
@@ -3602,7 +3602,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M45" t="n">
@@ -3639,25 +3639,25 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>526.15</v>
+        <v>527.65</v>
       </c>
       <c r="D46" t="n">
-        <v>0.0561019670814932</v>
+        <v>0.1099074463609592</v>
       </c>
       <c r="E46" t="n">
-        <v>-0.049841986455982</v>
+        <v>-0.0093870271285083</v>
       </c>
       <c r="F46" t="n">
-        <v>-0.1088245257452574</v>
+        <v>-0.1352126526264033</v>
       </c>
       <c r="G46" t="n">
-        <v>-0.0855501272153745</v>
+        <v>-0.1097111785368892</v>
       </c>
       <c r="H46" t="n">
-        <v>-0.0867707181328124</v>
+        <v>-0.1230841652575648</v>
       </c>
       <c r="I46" t="n">
-        <v>69.8278771515356</v>
+        <v>67.7721701514059</v>
       </c>
       <c r="J46" t="n">
         <v>80</v>
@@ -3667,7 +3667,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M46" t="n">
@@ -3677,10 +3677,10 @@
         <v>80</v>
       </c>
       <c r="O46" t="n">
-        <v>31.91489361702128</v>
+        <v>27.65957446808511</v>
       </c>
       <c r="P46" t="n">
-        <v>58.22697872340426</v>
+        <v>57.37591489361702</v>
       </c>
       <c r="Q46" t="b">
         <v>0</v>
@@ -3704,25 +3704,25 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>1074.35</v>
+        <v>1045.9</v>
       </c>
       <c r="D47" t="n">
-        <v>0.0459014797507786</v>
+        <v>0.0638795646424577</v>
       </c>
       <c r="E47" t="n">
-        <v>0.3700822546706623</v>
+        <v>0.3764558794498915</v>
       </c>
       <c r="F47" t="n">
-        <v>0.1885717446620201</v>
+        <v>0.193200616051566</v>
       </c>
       <c r="G47" t="n">
-        <v>0.2118461431919029</v>
+        <v>0.2187020901410801</v>
       </c>
       <c r="H47" t="n">
-        <v>0.2106255522744651</v>
+        <v>0.2053291034204045</v>
       </c>
       <c r="I47" t="n">
-        <v>65.60097126669362</v>
+        <v>60.97423359037055</v>
       </c>
       <c r="J47" t="n">
         <v>80</v>
@@ -3732,7 +3732,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M47" t="n">
@@ -3769,25 +3769,25 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>15032</v>
+        <v>15380</v>
       </c>
       <c r="D48" t="n">
-        <v>0.0891964350409391</v>
+        <v>0.1543946558582902</v>
       </c>
       <c r="E48" t="n">
-        <v>0.0720296676650977</v>
+        <v>0.1195224923569659</v>
       </c>
       <c r="F48" t="n">
-        <v>0.164819837272375</v>
+        <v>0.1771909682357444</v>
       </c>
       <c r="G48" t="n">
-        <v>0.1880942358022579</v>
+        <v>0.2026924423252585</v>
       </c>
       <c r="H48" t="n">
-        <v>0.18687364488482</v>
+        <v>0.1893194556045829</v>
       </c>
       <c r="I48" t="n">
-        <v>66.60535995796111</v>
+        <v>64.16690160699183</v>
       </c>
       <c r="J48" t="n">
         <v>80</v>
@@ -3797,7 +3797,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M48" t="n">
@@ -3807,10 +3807,10 @@
         <v>80</v>
       </c>
       <c r="O48" t="n">
-        <v>74.46808510638297</v>
+        <v>78.72340425531915</v>
       </c>
       <c r="P48" t="n">
-        <v>67.0096170212766</v>
+        <v>67.86068085106383</v>
       </c>
       <c r="Q48" t="b">
         <v>0</v>
@@ -3936,57 +3936,57 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>RICOAUTO</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Forgings</t>
+          <t>Castings</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1866.2</v>
+        <v>116.08</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0903885480572597</v>
+        <v>0.1267715006794798</v>
       </c>
       <c r="E2" t="n">
-        <v>0.3187760582291006</v>
+        <v>-0.00326292289198</v>
       </c>
       <c r="F2" t="n">
-        <v>0.5392609699769053</v>
+        <v>0.2375266524520256</v>
       </c>
       <c r="G2" t="n">
-        <v>0.5625353685067882</v>
+        <v>0.2630281265415397</v>
       </c>
       <c r="H2" t="n">
-        <v>0.5613147775893503</v>
+        <v>0.2496551398208641</v>
       </c>
       <c r="I2" t="n">
-        <v>78.20965842167257</v>
+        <v>67.62656758012076</v>
       </c>
       <c r="J2" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K2" t="n">
-        <v>54.83</v>
+        <v>49.07</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M2" t="n">
-        <v>54.83</v>
+        <v>49.07</v>
       </c>
       <c r="N2" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O2" t="n">
-        <v>97.87234042553192</v>
+        <v>87.2340425531915</v>
       </c>
       <c r="P2" t="n">
-        <v>69.50646808510639</v>
+        <v>69.07480851063831</v>
       </c>
       <c r="Q2" t="b">
         <v>0</v>
@@ -4010,25 +4010,25 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1795.4</v>
+        <v>1774.8</v>
       </c>
       <c r="D3" t="n">
-        <v>0.1450255102040816</v>
+        <v>0.1988651715752498</v>
       </c>
       <c r="E3" t="n">
-        <v>0.2136821469614007</v>
+        <v>0.302988033184054</v>
       </c>
       <c r="F3" t="n">
-        <v>0.4365498479756762</v>
+        <v>0.3464835748425765</v>
       </c>
       <c r="G3" t="n">
-        <v>0.4598242465055591</v>
+        <v>0.3719850489320906</v>
       </c>
       <c r="H3" t="n">
-        <v>0.4586036555881212</v>
+        <v>0.358612062211415</v>
       </c>
       <c r="I3" t="n">
-        <v>78.86728655959428</v>
+        <v>71.45562130177515</v>
       </c>
       <c r="J3" t="n">
         <v>70</v>
@@ -4038,7 +4038,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M3" t="n">
@@ -4048,10 +4048,10 @@
         <v>70</v>
       </c>
       <c r="O3" t="n">
-        <v>93.61702127659576</v>
+        <v>91.48936170212764</v>
       </c>
       <c r="P3" t="n">
-        <v>68.52740425531915</v>
+        <v>68.10187234042553</v>
       </c>
       <c r="Q3" t="b">
         <v>0</v>
@@ -4066,57 +4066,57 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SANSERA</t>
+          <t>ZFCVINDIA</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Forgings</t>
+          <t>Brakes/Transmission</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>2275.5</v>
+        <v>15380</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0448138114697644</v>
+        <v>0.1543946558582902</v>
       </c>
       <c r="E4" t="n">
-        <v>0.2626935242217414</v>
+        <v>0.1195224923569659</v>
       </c>
       <c r="F4" t="n">
-        <v>0.6582859641451684</v>
+        <v>0.1771909682357444</v>
       </c>
       <c r="G4" t="n">
-        <v>0.6815603626750513</v>
+        <v>0.2026924423252585</v>
       </c>
       <c r="H4" t="n">
-        <v>0.6803397717576134</v>
+        <v>0.1893194556045829</v>
       </c>
       <c r="I4" t="n">
-        <v>71.54802744425388</v>
+        <v>64.16690160699183</v>
       </c>
       <c r="J4" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K4" t="n">
-        <v>48.59</v>
+        <v>50.29</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M4" t="n">
-        <v>48.59</v>
+        <v>50.29</v>
       </c>
       <c r="N4" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O4" t="n">
-        <v>100</v>
+        <v>78.72340425531915</v>
       </c>
       <c r="P4" t="n">
-        <v>67.43600000000001</v>
+        <v>67.86068085106383</v>
       </c>
       <c r="Q4" t="b">
         <v>0</v>
@@ -4131,57 +4131,57 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ZFCVINDIA</t>
+          <t>SANSERA</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Brakes/Transmission</t>
+          <t>Forgings</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>15032</v>
+        <v>2374.6</v>
       </c>
       <c r="D5" t="n">
-        <v>0.0891964350409391</v>
+        <v>0.1615143807474075</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0720296676650977</v>
+        <v>0.3499715747583853</v>
       </c>
       <c r="F5" t="n">
-        <v>0.164819837272375</v>
+        <v>0.6933609070812237</v>
       </c>
       <c r="G5" t="n">
-        <v>0.1880942358022579</v>
+        <v>0.7188623811707378</v>
       </c>
       <c r="H5" t="n">
-        <v>0.18687364488482</v>
+        <v>0.7054893944500622</v>
       </c>
       <c r="I5" t="n">
-        <v>66.60535995796111</v>
+        <v>73.33199356913184</v>
       </c>
       <c r="J5" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K5" t="n">
-        <v>50.29</v>
+        <v>48.59</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M5" t="n">
-        <v>50.29</v>
+        <v>48.59</v>
       </c>
       <c r="N5" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O5" t="n">
-        <v>74.46808510638297</v>
+        <v>100</v>
       </c>
       <c r="P5" t="n">
-        <v>67.0096170212766</v>
+        <v>67.43600000000001</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
@@ -4205,25 +4205,25 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1074.35</v>
+        <v>1045.9</v>
       </c>
       <c r="D6" t="n">
-        <v>0.0459014797507786</v>
+        <v>0.0638795646424577</v>
       </c>
       <c r="E6" t="n">
-        <v>0.3700822546706623</v>
+        <v>0.3764558794498915</v>
       </c>
       <c r="F6" t="n">
-        <v>0.1885717446620201</v>
+        <v>0.193200616051566</v>
       </c>
       <c r="G6" t="n">
-        <v>0.2118461431919029</v>
+        <v>0.2187020901410801</v>
       </c>
       <c r="H6" t="n">
-        <v>0.2106255522744651</v>
+        <v>0.2053291034204045</v>
       </c>
       <c r="I6" t="n">
-        <v>65.60097126669362</v>
+        <v>60.97423359037055</v>
       </c>
       <c r="J6" t="n">
         <v>80</v>
@@ -4233,7 +4233,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M6" t="n">
@@ -4270,25 +4270,25 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>576.55</v>
+        <v>581.3</v>
       </c>
       <c r="D7" t="n">
-        <v>0.1388641975308642</v>
+        <v>0.198680276317146</v>
       </c>
       <c r="E7" t="n">
-        <v>0.2879481737964928</v>
+        <v>0.3035093620361027</v>
       </c>
       <c r="F7" t="n">
-        <v>0.4002428658166361</v>
+        <v>0.4049546827794561</v>
       </c>
       <c r="G7" t="n">
-        <v>0.423517264346519</v>
+        <v>0.4304561568689702</v>
       </c>
       <c r="H7" t="n">
-        <v>0.4222966734290811</v>
+        <v>0.4170831701482946</v>
       </c>
       <c r="I7" t="n">
-        <v>79.32736809626651</v>
+        <v>77.82191327375034</v>
       </c>
       <c r="J7" t="n">
         <v>70</v>
@@ -4298,7 +4298,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M7" t="n">
@@ -4308,10 +4308,10 @@
         <v>70</v>
       </c>
       <c r="O7" t="n">
-        <v>91.48936170212764</v>
+        <v>93.61702127659576</v>
       </c>
       <c r="P7" t="n">
-        <v>66.16187234042553</v>
+        <v>66.58740425531916</v>
       </c>
       <c r="Q7" t="b">
         <v>0</v>
@@ -4326,57 +4326,57 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SHRIPISTON</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Engine/Parts</t>
+          <t>Forgings</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>3627.6</v>
+        <v>1895.8</v>
       </c>
       <c r="D8" t="n">
-        <v>0.1608319999999998</v>
+        <v>0.1499454082251607</v>
       </c>
       <c r="E8" t="n">
-        <v>0.2799379013478231</v>
+        <v>0.3598737536762069</v>
       </c>
       <c r="F8" t="n">
-        <v>0.3458984157607685</v>
+        <v>0.5544440800262382</v>
       </c>
       <c r="G8" t="n">
-        <v>0.3691728142906514</v>
+        <v>0.5799455541157523</v>
       </c>
       <c r="H8" t="n">
-        <v>0.3679522233732135</v>
+        <v>0.5665725673950768</v>
       </c>
       <c r="I8" t="n">
-        <v>77.81013925548373</v>
+        <v>81.32231404958674</v>
       </c>
       <c r="J8" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="K8" t="n">
-        <v>48.69</v>
+        <v>54.83</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M8" t="n">
-        <v>48.69</v>
+        <v>54.83</v>
       </c>
       <c r="N8" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="O8" t="n">
-        <v>89.36170212765957</v>
+        <v>97.87234042553192</v>
       </c>
       <c r="P8" t="n">
-        <v>65.34834042553192</v>
+        <v>65.50646808510639</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
@@ -4391,57 +4391,57 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>GNA</t>
+          <t>BHARATGEAR</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Axles</t>
+          <t>Gears</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>448.5</v>
+        <v>108.92</v>
       </c>
       <c r="D9" t="n">
-        <v>0.1948847742107364</v>
+        <v>0.1734539969834088</v>
       </c>
       <c r="E9" t="n">
-        <v>0.2741477272727273</v>
+        <v>-0.0137631293009778</v>
       </c>
       <c r="F9" t="n">
-        <v>0.4538087520259319</v>
+        <v>0.2253346833164584</v>
       </c>
       <c r="G9" t="n">
-        <v>0.4770831505558148</v>
+        <v>0.2508361574059725</v>
       </c>
       <c r="H9" t="n">
-        <v>0.475862559638377</v>
+        <v>0.237463170685297</v>
       </c>
       <c r="I9" t="n">
-        <v>85.03816793893128</v>
+        <v>79.73770491803278</v>
       </c>
       <c r="J9" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K9" t="n">
-        <v>54.47</v>
+        <v>51.91</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M9" t="n">
-        <v>54.47</v>
+        <v>51.91</v>
       </c>
       <c r="N9" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O9" t="n">
-        <v>95.74468085106383</v>
+        <v>82.97872340425532</v>
       </c>
       <c r="P9" t="n">
-        <v>64.93693617021276</v>
+        <v>65.35974468085107</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -4456,63 +4456,63 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ASKAUTOLTD</t>
+          <t>SHRIPISTON</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Engine/Parts</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>438.25</v>
+        <v>3586.8</v>
       </c>
       <c r="D10" t="n">
-        <v>0.0709921798631476</v>
+        <v>0.2208304969366916</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.0441657579062159</v>
+        <v>0.3096724723408919</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.1695091908281221</v>
+        <v>0.3102944399795426</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.1462347922982392</v>
+        <v>0.3357959140690567</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.147455383215677</v>
+        <v>0.3224229273483812</v>
       </c>
       <c r="I10" t="n">
-        <v>42.13075060532687</v>
+        <v>74.83197736116026</v>
       </c>
       <c r="J10" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K10" t="n">
-        <v>71.28</v>
+        <v>48.69</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M10" t="n">
-        <v>71.28</v>
+        <v>48.69</v>
       </c>
       <c r="N10" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O10" t="n">
-        <v>19.14893617021277</v>
+        <v>89.36170212765957</v>
       </c>
       <c r="P10" t="n">
-        <v>64.34178723404256</v>
+        <v>65.34834042553192</v>
       </c>
       <c r="Q10" t="b">
+        <v>0</v>
+      </c>
+      <c r="R10" t="b">
         <v>1</v>
-      </c>
-      <c r="R10" t="b">
-        <v>0</v>
       </c>
       <c r="S10" t="b">
         <v>0</v>
@@ -4521,57 +4521,57 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MOTHERSON</t>
+          <t>GNA</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Axles</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>123.19</v>
+        <v>450.65</v>
       </c>
       <c r="D11" t="n">
-        <v>0.1039519670221345</v>
+        <v>0.2662264681090194</v>
       </c>
       <c r="E11" t="n">
-        <v>0.09667942668921919</v>
+        <v>0.3238836662749706</v>
       </c>
       <c r="F11" t="n">
-        <v>0.1660198769522005</v>
+        <v>0.4383977018831788</v>
       </c>
       <c r="G11" t="n">
-        <v>0.1892942754820834</v>
+        <v>0.4638991759726929</v>
       </c>
       <c r="H11" t="n">
-        <v>0.1880736845646455</v>
+        <v>0.4505261892520174</v>
       </c>
       <c r="I11" t="n">
-        <v>77.11889787361486</v>
+        <v>82.40574506283662</v>
       </c>
       <c r="J11" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="K11" t="n">
-        <v>51.57</v>
+        <v>54.47</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M11" t="n">
-        <v>51.57</v>
+        <v>54.47</v>
       </c>
       <c r="N11" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="O11" t="n">
-        <v>76.59574468085107</v>
+        <v>95.74468085106383</v>
       </c>
       <c r="P11" t="n">
-        <v>63.94714893617022</v>
+        <v>64.93693617021276</v>
       </c>
       <c r="Q11" t="b">
         <v>0</v>
@@ -4586,57 +4586,57 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CRAFTSMAN</t>
+          <t>LUMAXIND</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Castings</t>
+          <t>Lighting</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>7721.5</v>
+        <v>5506.4</v>
       </c>
       <c r="D12" t="n">
-        <v>0.1171151620370369</v>
+        <v>0.1452579034941763</v>
       </c>
       <c r="E12" t="n">
-        <v>0.0154523934771173</v>
+        <v>0.057804245509557</v>
       </c>
       <c r="F12" t="n">
-        <v>0.1366011628762788</v>
+        <v>0.0758890191481047</v>
       </c>
       <c r="G12" t="n">
-        <v>0.1598755614061617</v>
+        <v>0.1013904932376188</v>
       </c>
       <c r="H12" t="n">
-        <v>0.1586549704887239</v>
+        <v>0.08801750651694321</v>
       </c>
       <c r="I12" t="n">
-        <v>79.25343811394892</v>
+        <v>76.29801920768305</v>
       </c>
       <c r="J12" t="n">
         <v>70</v>
       </c>
       <c r="K12" t="n">
-        <v>54.65</v>
+        <v>57.69</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M12" t="n">
-        <v>54.65</v>
+        <v>57.69</v>
       </c>
       <c r="N12" t="n">
         <v>70</v>
       </c>
       <c r="O12" t="n">
-        <v>70.21276595744681</v>
+        <v>65.95744680851064</v>
       </c>
       <c r="P12" t="n">
-        <v>63.90255319148936</v>
+        <v>64.26748936170213</v>
       </c>
       <c r="Q12" t="b">
         <v>0</v>
@@ -4651,57 +4651,57 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>LUMAXIND</t>
+          <t>MOTHERSON</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Lighting</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>5517.1</v>
+        <v>124.7</v>
       </c>
       <c r="D13" t="n">
-        <v>0.09130649787360311</v>
+        <v>0.1699033680457828</v>
       </c>
       <c r="E13" t="n">
-        <v>0.0294057281462822</v>
+        <v>0.1558068403003059</v>
       </c>
       <c r="F13" t="n">
-        <v>0.09225713210983751</v>
+        <v>0.1764150943396227</v>
       </c>
       <c r="G13" t="n">
-        <v>0.1155315306397204</v>
+        <v>0.2019165684291368</v>
       </c>
       <c r="H13" t="n">
-        <v>0.1143109397222825</v>
+        <v>0.1885435817084613</v>
       </c>
       <c r="I13" t="n">
-        <v>79.28741092636581</v>
+        <v>76.39060568603213</v>
       </c>
       <c r="J13" t="n">
         <v>70</v>
       </c>
       <c r="K13" t="n">
-        <v>57.69</v>
+        <v>51.57</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M13" t="n">
-        <v>57.69</v>
+        <v>51.57</v>
       </c>
       <c r="N13" t="n">
         <v>70</v>
       </c>
       <c r="O13" t="n">
-        <v>63.82978723404256</v>
+        <v>76.59574468085107</v>
       </c>
       <c r="P13" t="n">
-        <v>63.84195744680851</v>
+        <v>63.94714893617022</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
@@ -4716,57 +4716,57 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>BHARATGEAR</t>
+          <t>SANDHAR</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Gears</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>108.05</v>
+        <v>488.7</v>
       </c>
       <c r="D14" t="n">
-        <v>0.101427115188583</v>
+        <v>0.0906047757197052</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.0019397746166636</v>
+        <v>-0.0418586413096755</v>
       </c>
       <c r="F14" t="n">
-        <v>0.2033634034970486</v>
+        <v>0.072886937431394</v>
       </c>
       <c r="G14" t="n">
-        <v>0.2266378020269315</v>
+        <v>0.0983884115209081</v>
       </c>
       <c r="H14" t="n">
-        <v>0.2254172111094936</v>
+        <v>0.08501542480023259</v>
       </c>
       <c r="I14" t="n">
-        <v>81.924539338988</v>
+        <v>66.80522565320663</v>
       </c>
       <c r="J14" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K14" t="n">
-        <v>51.91</v>
+        <v>47.8</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M14" t="n">
-        <v>51.91</v>
+        <v>47.8</v>
       </c>
       <c r="N14" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O14" t="n">
-        <v>82.97872340425532</v>
+        <v>63.82978723404256</v>
       </c>
       <c r="P14" t="n">
-        <v>61.35974468085107</v>
+        <v>63.88595744680852</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
@@ -4781,48 +4781,48 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SANDHAR</t>
+          <t>DIVGIITTS</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Transmission</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>494.25</v>
+        <v>748.1</v>
       </c>
       <c r="D15" t="n">
-        <v>0.035512256442489</v>
+        <v>0.1359805633588946</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.0703470328223454</v>
+        <v>0.2627225926238501</v>
       </c>
       <c r="F15" t="n">
-        <v>0.1110486680903675</v>
+        <v>0.1160674324929136</v>
       </c>
       <c r="G15" t="n">
-        <v>0.1343230666202504</v>
+        <v>0.1415689065824277</v>
       </c>
       <c r="H15" t="n">
-        <v>0.1331024757028125</v>
+        <v>0.1281959198617521</v>
       </c>
       <c r="I15" t="n">
-        <v>78.04997550220479</v>
+        <v>78.78187670215402</v>
       </c>
       <c r="J15" t="n">
         <v>70</v>
       </c>
       <c r="K15" t="n">
-        <v>47.8</v>
+        <v>49.92</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M15" t="n">
-        <v>47.8</v>
+        <v>49.92</v>
       </c>
       <c r="N15" t="n">
         <v>70</v>
@@ -4831,7 +4831,7 @@
         <v>68.08510638297872</v>
       </c>
       <c r="P15" t="n">
-        <v>60.73702127659575</v>
+        <v>61.58502127659575</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
@@ -4855,25 +4855,25 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>537.95</v>
+        <v>544.45</v>
       </c>
       <c r="D16" t="n">
-        <v>0.070547263681592</v>
+        <v>0.1091983294285423</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.01257342143906</v>
+        <v>0.0154807423295719</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.0553165334972342</v>
+        <v>-0.0609692997585372</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.0320421349673513</v>
+        <v>-0.0354678256690231</v>
       </c>
       <c r="H16" t="n">
-        <v>-0.0332627258847891</v>
+        <v>-0.0488408123896987</v>
       </c>
       <c r="I16" t="n">
-        <v>62.30945121951223</v>
+        <v>61.7260061919505</v>
       </c>
       <c r="J16" t="n">
         <v>80</v>
@@ -4883,7 +4883,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="M16" t="n">
@@ -4893,10 +4893,10 @@
         <v>80</v>
       </c>
       <c r="O16" t="n">
-        <v>42.5531914893617</v>
+        <v>44.68085106382978</v>
       </c>
       <c r="P16" t="n">
-        <v>60.27863829787234</v>
+        <v>60.70417021276596</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
chore: auto-refresh NSE data and pipeline outputs (2026-04-22)
</commit_message>
<xml_diff>
--- a/working-sector/output/auto_components_comprehensive_report.xlsx
+++ b/working-sector/output/auto_components_comprehensive_report.xlsx
@@ -435,7 +435,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
     </row>
@@ -447,7 +447,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
     </row>
@@ -779,25 +779,25 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1895.8</v>
+        <v>1903.2</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1499454082251607</v>
+        <v>0.1137640449438202</v>
       </c>
       <c r="E2" t="n">
-        <v>0.3598737536762069</v>
+        <v>0.3791304347826087</v>
       </c>
       <c r="F2" t="n">
-        <v>0.5544440800262382</v>
+        <v>0.5597443042124242</v>
       </c>
       <c r="G2" t="n">
-        <v>0.5799455541157523</v>
+        <v>0.5803810879325622</v>
       </c>
       <c r="H2" t="n">
-        <v>0.5665725673950768</v>
+        <v>0.5678014267303019</v>
       </c>
       <c r="I2" t="n">
-        <v>81.32231404958674</v>
+        <v>87.81195589088799</v>
       </c>
       <c r="J2" t="n">
         <v>60</v>
@@ -807,7 +807,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M2" t="n">
@@ -844,48 +844,48 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1149.6</v>
+        <v>1151.3</v>
       </c>
       <c r="D3" t="n">
-        <v>0.1166585721223893</v>
+        <v>0.0745753220085867</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0260621206711886</v>
+        <v>0.0202942219071249</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.1319842947749926</v>
+        <v>-0.1251519756838905</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.1064828206854785</v>
+        <v>-0.1045151919637525</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.119855807406154</v>
+        <v>-0.1170948531660128</v>
       </c>
       <c r="I3" t="n">
-        <v>68.27253957329656</v>
+        <v>72.94932555596054</v>
       </c>
       <c r="J3" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K3" t="n">
         <v>49.36</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M3" t="n">
         <v>49.36</v>
       </c>
       <c r="N3" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O3" t="n">
-        <v>29.78723404255319</v>
+        <v>27.65957446808511</v>
       </c>
       <c r="P3" t="n">
-        <v>57.70144680851064</v>
+        <v>53.27591489361702</v>
       </c>
       <c r="Q3" t="b">
         <v>0</v>
@@ -909,25 +909,25 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>38100</v>
+        <v>37885</v>
       </c>
       <c r="D4" t="n">
-        <v>0.307705508838167</v>
+        <v>0.2594747340425531</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0709768095572733</v>
+        <v>0.0784230002846571</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.0057411273486429</v>
+        <v>-0.0192855293813098</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0197603467408711</v>
+        <v>0.0013512543388281</v>
       </c>
       <c r="H4" t="n">
-        <v>0.0063873600201955</v>
+        <v>-0.0112284068634321</v>
       </c>
       <c r="I4" t="n">
-        <v>91.82072829131651</v>
+        <v>87.63089005235602</v>
       </c>
       <c r="J4" t="n">
         <v>60</v>
@@ -937,7 +937,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M4" t="n">
@@ -947,16 +947,16 @@
         <v>60</v>
       </c>
       <c r="O4" t="n">
-        <v>57.44680851063831</v>
+        <v>55.31914893617022</v>
       </c>
       <c r="P4" t="n">
-        <v>56.88136170212766</v>
+        <v>56.45582978723404</v>
       </c>
       <c r="Q4" t="b">
         <v>0</v>
       </c>
       <c r="R4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S4" t="b">
         <v>0</v>
@@ -974,25 +974,25 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>333.1</v>
+        <v>354.55</v>
       </c>
       <c r="D5" t="n">
-        <v>0.1456577815993123</v>
+        <v>0.1877721943048576</v>
       </c>
       <c r="E5" t="n">
-        <v>0.007866868381240601</v>
+        <v>0.0877435189446234</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.156815592962916</v>
+        <v>-0.1092827534229368</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.1313141188734019</v>
+        <v>-0.0886459697027988</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.1446871055940775</v>
+        <v>-0.1012256309050591</v>
       </c>
       <c r="I5" t="n">
-        <v>84.88982161594964</v>
+        <v>90.36496350364968</v>
       </c>
       <c r="J5" t="n">
         <v>60</v>
@@ -1002,7 +1002,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M5" t="n">
@@ -1012,10 +1012,10 @@
         <v>60</v>
       </c>
       <c r="O5" t="n">
-        <v>23.40425531914894</v>
+        <v>29.78723404255319</v>
       </c>
       <c r="P5" t="n">
-        <v>49.12885106382979</v>
+        <v>50.40544680851064</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
@@ -1039,48 +1039,48 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>124.7</v>
+        <v>131.76</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1699033680457828</v>
+        <v>0.185638441464951</v>
       </c>
       <c r="E6" t="n">
-        <v>0.1558068403003059</v>
+        <v>0.2014224491656788</v>
       </c>
       <c r="F6" t="n">
-        <v>0.1764150943396227</v>
+        <v>0.235211399643761</v>
       </c>
       <c r="G6" t="n">
-        <v>0.2019165684291368</v>
+        <v>0.255848183363899</v>
       </c>
       <c r="H6" t="n">
-        <v>0.1885435817084613</v>
+        <v>0.2432685221616387</v>
       </c>
       <c r="I6" t="n">
-        <v>76.39060568603213</v>
+        <v>82.3102823102823</v>
       </c>
       <c r="J6" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="K6" t="n">
         <v>51.57</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M6" t="n">
         <v>51.57</v>
       </c>
       <c r="N6" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="O6" t="n">
-        <v>76.59574468085107</v>
+        <v>82.97872340425532</v>
       </c>
       <c r="P6" t="n">
-        <v>63.94714893617022</v>
+        <v>61.22374468085107</v>
       </c>
       <c r="Q6" t="b">
         <v>0</v>
@@ -1104,25 +1104,25 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2885.2</v>
+        <v>3024.4</v>
       </c>
       <c r="D7" t="n">
-        <v>0.1676244435451233</v>
+        <v>0.177450751382076</v>
       </c>
       <c r="E7" t="n">
-        <v>0.2385490448594118</v>
+        <v>0.3306348717497469</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.0644920722414967</v>
+        <v>-0.0356174866872867</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.0389905981519826</v>
+        <v>-0.0149807029671487</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.0523635848726582</v>
+        <v>-0.0275603641694089</v>
       </c>
       <c r="I7" t="n">
-        <v>90.46879046879052</v>
+        <v>93.96037699557606</v>
       </c>
       <c r="J7" t="n">
         <v>60</v>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M7" t="n">
@@ -1142,10 +1142,10 @@
         <v>60</v>
       </c>
       <c r="O7" t="n">
-        <v>40.42553191489361</v>
+        <v>51.06382978723404</v>
       </c>
       <c r="P7" t="n">
-        <v>51.57710638297873</v>
+        <v>53.70476595744681</v>
       </c>
       <c r="Q7" t="b">
         <v>0</v>
@@ -1169,25 +1169,25 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>581.3</v>
+        <v>588.45</v>
       </c>
       <c r="D8" t="n">
-        <v>0.198680276317146</v>
+        <v>0.189508793208005</v>
       </c>
       <c r="E8" t="n">
-        <v>0.3035093620361027</v>
+        <v>0.3239959500506244</v>
       </c>
       <c r="F8" t="n">
-        <v>0.4049546827794561</v>
+        <v>0.4020729092208721</v>
       </c>
       <c r="G8" t="n">
-        <v>0.4304561568689702</v>
+        <v>0.4227096929410101</v>
       </c>
       <c r="H8" t="n">
-        <v>0.4170831701482946</v>
+        <v>0.4101300317387498</v>
       </c>
       <c r="I8" t="n">
-        <v>77.82191327375034</v>
+        <v>79.17460317460311</v>
       </c>
       <c r="J8" t="n">
         <v>70</v>
@@ -1197,7 +1197,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M8" t="n">
@@ -1234,48 +1234,48 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>441.95</v>
+        <v>434</v>
       </c>
       <c r="D9" t="n">
-        <v>0.1062578222778471</v>
+        <v>0.0723993081294787</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.1276154757204896</v>
+        <v>-0.1354581673306772</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.0549556292098791</v>
+        <v>-0.0827433160731269</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.029454155120365</v>
+        <v>-0.0621065323529889</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.0428271418410406</v>
+        <v>-0.07468619355524909</v>
       </c>
       <c r="I9" t="n">
-        <v>71.46302250803853</v>
+        <v>69.07536907536905</v>
       </c>
       <c r="J9" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="K9" t="n">
         <v>53.44</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M9" t="n">
         <v>53.44</v>
       </c>
       <c r="N9" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="O9" t="n">
-        <v>46.80851063829788</v>
+        <v>40.42553191489361</v>
       </c>
       <c r="P9" t="n">
-        <v>58.73770212765958</v>
+        <v>53.46110638297873</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -1299,25 +1299,25 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>139665</v>
+        <v>137040</v>
       </c>
       <c r="D10" t="n">
-        <v>0.1175435087017402</v>
+        <v>0.073602569626699</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.0249240758194575</v>
+        <v>-0.0214923241699392</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.0610125050423557</v>
+        <v>-0.1054538333496524</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.0355110309528416</v>
+        <v>-0.0848170496295144</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.0488840176735172</v>
+        <v>-0.0973967108317747</v>
       </c>
       <c r="I10" t="n">
-        <v>74.00090826521344</v>
+        <v>74.27073837739289</v>
       </c>
       <c r="J10" t="n">
         <v>70</v>
@@ -1327,7 +1327,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M10" t="n">
@@ -1337,10 +1337,10 @@
         <v>70</v>
       </c>
       <c r="O10" t="n">
-        <v>42.5531914893617</v>
+        <v>31.91489361702128</v>
       </c>
       <c r="P10" t="n">
-        <v>56.27463829787234</v>
+        <v>54.14697872340425</v>
       </c>
       <c r="Q10" t="b">
         <v>0</v>
@@ -1376,10 +1376,10 @@
         <v>-0.0042030657656173</v>
       </c>
       <c r="G11" t="n">
-        <v>0.0212984083238967</v>
+        <v>0.0164337179545206</v>
       </c>
       <c r="H11" t="n">
-        <v>0.0079254216032211</v>
+        <v>0.0038540567522603</v>
       </c>
       <c r="I11" t="n">
         <v>27.6054590570719</v>
@@ -1392,7 +1392,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M11" t="n">
@@ -1429,48 +1429,48 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>438.15</v>
+        <v>442.8</v>
       </c>
       <c r="D12" t="n">
-        <v>0.1099430018999365</v>
+        <v>0.0662171923910426</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.0118403247631935</v>
+        <v>0.0273781902552203</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.1740810556079171</v>
+        <v>-0.1520490233626963</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.148579581518403</v>
+        <v>-0.1314122396425583</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.1619525682390785</v>
+        <v>-0.1439919008448186</v>
       </c>
       <c r="I12" t="n">
-        <v>53.78670788253476</v>
+        <v>58.70165745856355</v>
       </c>
       <c r="J12" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K12" t="n">
         <v>71.28</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M12" t="n">
         <v>71.28</v>
       </c>
       <c r="N12" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O12" t="n">
-        <v>17.02127659574468</v>
+        <v>23.40425531914894</v>
       </c>
       <c r="P12" t="n">
-        <v>55.91625531914894</v>
+        <v>65.19285106382979</v>
       </c>
       <c r="Q12" t="b">
         <v>1</v>
@@ -1494,25 +1494,25 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1803.9</v>
+        <v>1798.8</v>
       </c>
       <c r="D13" t="n">
-        <v>0.1476650973406286</v>
+        <v>0.1385530729793023</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.0297439759036144</v>
+        <v>-0.0426822778073443</v>
       </c>
       <c r="F13" t="n">
-        <v>0.0288011862666819</v>
+        <v>0.0161563665122583</v>
       </c>
       <c r="G13" t="n">
-        <v>0.054302660356196</v>
+        <v>0.0367931502323963</v>
       </c>
       <c r="H13" t="n">
-        <v>0.0409296736355204</v>
+        <v>0.024213489030136</v>
       </c>
       <c r="I13" t="n">
-        <v>68.67619639527658</v>
+        <v>65.44328985186823</v>
       </c>
       <c r="J13" t="n">
         <v>60</v>
@@ -1522,7 +1522,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M13" t="n">
@@ -1532,10 +1532,10 @@
         <v>60</v>
       </c>
       <c r="O13" t="n">
-        <v>61.70212765957447</v>
+        <v>63.82978723404256</v>
       </c>
       <c r="P13" t="n">
-        <v>59.8484255319149</v>
+        <v>60.27395744680852</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
@@ -1559,48 +1559,48 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>612.6</v>
+        <v>624.25</v>
       </c>
       <c r="D14" t="n">
-        <v>0.1727768737436583</v>
+        <v>0.1324263038548752</v>
       </c>
       <c r="E14" t="n">
-        <v>0.0672473867595819</v>
+        <v>0.0916324210894465</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.2875501540966447</v>
+        <v>-0.2638127248068872</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.2620486800071306</v>
+        <v>-0.2431759410867492</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.2754216667278062</v>
+        <v>-0.2557556022890095</v>
       </c>
       <c r="I14" t="n">
-        <v>71.01699798329011</v>
+        <v>81.04535896665664</v>
       </c>
       <c r="J14" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="K14" t="n">
         <v>54.64</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M14" t="n">
         <v>54.64</v>
       </c>
       <c r="N14" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="O14" t="n">
-        <v>2.127659574468085</v>
+        <v>4.25531914893617</v>
       </c>
       <c r="P14" t="n">
-        <v>50.28153191489362</v>
+        <v>46.70706382978724</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
@@ -1624,48 +1624,48 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>108.92</v>
+        <v>109.42</v>
       </c>
       <c r="D15" t="n">
-        <v>0.1734539969834088</v>
+        <v>0.1661515506767559</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.0137631293009778</v>
+        <v>0.0081076100976598</v>
       </c>
       <c r="F15" t="n">
-        <v>0.2253346833164584</v>
+        <v>0.1556822982678496</v>
       </c>
       <c r="G15" t="n">
-        <v>0.2508361574059725</v>
+        <v>0.1763190819879876</v>
       </c>
       <c r="H15" t="n">
-        <v>0.237463170685297</v>
+        <v>0.1637394207857273</v>
       </c>
       <c r="I15" t="n">
-        <v>79.73770491803278</v>
+        <v>81.86015831134566</v>
       </c>
       <c r="J15" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="K15" t="n">
         <v>51.91</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M15" t="n">
         <v>51.91</v>
       </c>
       <c r="N15" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="O15" t="n">
-        <v>82.97872340425532</v>
+        <v>74.46808510638297</v>
       </c>
       <c r="P15" t="n">
-        <v>65.35974468085107</v>
+        <v>59.65761702127659</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
@@ -1689,48 +1689,48 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>180.77</v>
+        <v>178.01</v>
       </c>
       <c r="D16" t="n">
-        <v>0.2187837108953614</v>
+        <v>0.1443908711025392</v>
       </c>
       <c r="E16" t="n">
-        <v>0.1949365415124273</v>
+        <v>0.2406607192640089</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.0296312201406407</v>
+        <v>-0.0899284253578732</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.0041297460511267</v>
+        <v>-0.0692916416377352</v>
       </c>
       <c r="H16" t="n">
-        <v>-0.0175027327718022</v>
+        <v>-0.0818713028399955</v>
       </c>
       <c r="I16" t="n">
-        <v>81.79035960214229</v>
+        <v>76.13307618129213</v>
       </c>
       <c r="J16" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K16" t="n">
         <v>52.61</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M16" t="n">
         <v>52.61</v>
       </c>
       <c r="N16" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O16" t="n">
-        <v>51.06382978723404</v>
+        <v>38.29787234042553</v>
       </c>
       <c r="P16" t="n">
-        <v>55.2567659574468</v>
+        <v>56.70357446808511</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>
@@ -1754,25 +1754,25 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>7653</v>
+        <v>7684.5</v>
       </c>
       <c r="D17" t="n">
-        <v>0.169021614603223</v>
+        <v>0.122972380534853</v>
       </c>
       <c r="E17" t="n">
-        <v>0.0327935222672064</v>
+        <v>0.0394994927291174</v>
       </c>
       <c r="F17" t="n">
-        <v>0.1394327402665078</v>
+        <v>0.1344947220786889</v>
       </c>
       <c r="G17" t="n">
-        <v>0.1649342143560219</v>
+        <v>0.1551315057988269</v>
       </c>
       <c r="H17" t="n">
-        <v>0.1515612276353464</v>
+        <v>0.1425518445965666</v>
       </c>
       <c r="I17" t="n">
-        <v>83.90183028286189</v>
+        <v>87.80075981426762</v>
       </c>
       <c r="J17" t="n">
         <v>60</v>
@@ -1782,7 +1782,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M17" t="n">
@@ -1792,10 +1792,10 @@
         <v>60</v>
       </c>
       <c r="O17" t="n">
-        <v>70.21276595744681</v>
+        <v>72.3404255319149</v>
       </c>
       <c r="P17" t="n">
-        <v>59.90255319148936</v>
+        <v>60.32808510638298</v>
       </c>
       <c r="Q17" t="b">
         <v>0</v>
@@ -1819,25 +1819,25 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>748.1</v>
+        <v>733.8</v>
       </c>
       <c r="D18" t="n">
-        <v>0.1359805633588946</v>
+        <v>0.0526466790991249</v>
       </c>
       <c r="E18" t="n">
-        <v>0.2627225926238501</v>
+        <v>0.253608951909114</v>
       </c>
       <c r="F18" t="n">
-        <v>0.1160674324929136</v>
+        <v>0.0866281652598845</v>
       </c>
       <c r="G18" t="n">
-        <v>0.1415689065824277</v>
+        <v>0.1072649489800225</v>
       </c>
       <c r="H18" t="n">
-        <v>0.1281959198617521</v>
+        <v>0.09468528777776231</v>
       </c>
       <c r="I18" t="n">
-        <v>78.78187670215402</v>
+        <v>73.33177788147458</v>
       </c>
       <c r="J18" t="n">
         <v>70</v>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M18" t="n">
@@ -1884,25 +1884,25 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2389.8</v>
+        <v>2399.1</v>
       </c>
       <c r="D19" t="n">
-        <v>0.08155322230267931</v>
+        <v>0.07073998036240289</v>
       </c>
       <c r="E19" t="n">
-        <v>-0.0341120362137254</v>
+        <v>-0.0155519080837095</v>
       </c>
       <c r="F19" t="n">
-        <v>-0.1503235440517669</v>
+        <v>-0.1708370774866939</v>
       </c>
       <c r="G19" t="n">
-        <v>-0.1248220699622528</v>
+        <v>-0.1502002937665559</v>
       </c>
       <c r="H19" t="n">
-        <v>-0.1381950566829284</v>
+        <v>-0.1627799549688162</v>
       </c>
       <c r="I19" t="n">
-        <v>65.99350046425253</v>
+        <v>66.72727272727266</v>
       </c>
       <c r="J19" t="n">
         <v>60</v>
@@ -1912,7 +1912,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M19" t="n">
@@ -1922,10 +1922,10 @@
         <v>60</v>
       </c>
       <c r="O19" t="n">
-        <v>25.53191489361702</v>
+        <v>21.27659574468085</v>
       </c>
       <c r="P19" t="n">
-        <v>49.61438297872341</v>
+        <v>48.76331914893618</v>
       </c>
       <c r="Q19" t="b">
         <v>0</v>
@@ -1949,25 +1949,25 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2267.8</v>
+        <v>2275.2</v>
       </c>
       <c r="D20" t="n">
-        <v>0.1661438782331465</v>
+        <v>0.1311524311424876</v>
       </c>
       <c r="E20" t="n">
-        <v>0.0712834805611979</v>
+        <v>0.0429999083157603</v>
       </c>
       <c r="F20" t="n">
-        <v>0.1548019146552604</v>
+        <v>0.1746605400382053</v>
       </c>
       <c r="G20" t="n">
-        <v>0.1803033887447744</v>
+        <v>0.1952973237583433</v>
       </c>
       <c r="H20" t="n">
-        <v>0.1669304020240989</v>
+        <v>0.182717662556083</v>
       </c>
       <c r="I20" t="n">
-        <v>83.63552903373879</v>
+        <v>83.51445086705199</v>
       </c>
       <c r="J20" t="n">
         <v>60</v>
@@ -1977,7 +1977,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M20" t="n">
@@ -1987,10 +1987,10 @@
         <v>60</v>
       </c>
       <c r="O20" t="n">
-        <v>72.3404255319149</v>
+        <v>78.72340425531915</v>
       </c>
       <c r="P20" t="n">
-        <v>58.09208510638298</v>
+        <v>59.36868085106384</v>
       </c>
       <c r="Q20" t="b">
         <v>0</v>
@@ -2014,25 +2014,25 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1016</v>
+        <v>1031.85</v>
       </c>
       <c r="D21" t="n">
-        <v>0.2226233453670276</v>
+        <v>0.1998255813953486</v>
       </c>
       <c r="E21" t="n">
-        <v>0.1477632173520107</v>
+        <v>0.1558754340763972</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.1813713641124807</v>
+        <v>-0.1999922468599783</v>
       </c>
       <c r="G21" t="n">
-        <v>-0.1558698900229667</v>
+        <v>-0.1793554631398403</v>
       </c>
       <c r="H21" t="n">
-        <v>-0.1692428767436422</v>
+        <v>-0.1919351243421005</v>
       </c>
       <c r="I21" t="n">
-        <v>89.69263381028085</v>
+        <v>89.97681010048954</v>
       </c>
       <c r="J21" t="n">
         <v>60</v>
@@ -2042,7 +2042,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M21" t="n">
@@ -2052,10 +2052,10 @@
         <v>60</v>
       </c>
       <c r="O21" t="n">
-        <v>14.8936170212766</v>
+        <v>12.76595744680851</v>
       </c>
       <c r="P21" t="n">
-        <v>46.35072340425532</v>
+        <v>45.9251914893617</v>
       </c>
       <c r="Q21" t="b">
         <v>0</v>
@@ -2079,25 +2079,25 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>450.65</v>
+        <v>457.2</v>
       </c>
       <c r="D22" t="n">
-        <v>0.2662264681090194</v>
+        <v>0.2295280354981845</v>
       </c>
       <c r="E22" t="n">
-        <v>0.3238836662749706</v>
+        <v>0.3678384442782347</v>
       </c>
       <c r="F22" t="n">
-        <v>0.4383977018831788</v>
+        <v>0.4595371109337589</v>
       </c>
       <c r="G22" t="n">
-        <v>0.4638991759726929</v>
+        <v>0.4801738946538969</v>
       </c>
       <c r="H22" t="n">
-        <v>0.4505261892520174</v>
+        <v>0.4675942334516366</v>
       </c>
       <c r="I22" t="n">
-        <v>82.40574506283662</v>
+        <v>88.76353790613715</v>
       </c>
       <c r="J22" t="n">
         <v>60</v>
@@ -2107,7 +2107,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M22" t="n">
@@ -2144,25 +2144,25 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>393.55</v>
+        <v>394.15</v>
       </c>
       <c r="D23" t="n">
-        <v>0.198933739527799</v>
+        <v>0.1831007053879634</v>
       </c>
       <c r="E23" t="n">
-        <v>0.0314506617743415</v>
+        <v>0.0744173367861522</v>
       </c>
       <c r="F23" t="n">
-        <v>-0.0078154544308584</v>
+        <v>-0.0111640742599098</v>
       </c>
       <c r="G23" t="n">
-        <v>0.0176860196586556</v>
+        <v>0.0094727094602281</v>
       </c>
       <c r="H23" t="n">
-        <v>0.0043130329379801</v>
+        <v>-0.0031069517420321</v>
       </c>
       <c r="I23" t="n">
-        <v>80.76545632973502</v>
+        <v>80.36072144288575</v>
       </c>
       <c r="J23" t="n">
         <v>60</v>
@@ -2172,7 +2172,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M23" t="n">
@@ -2182,16 +2182,16 @@
         <v>60</v>
       </c>
       <c r="O23" t="n">
-        <v>55.31914893617022</v>
+        <v>57.44680851063831</v>
       </c>
       <c r="P23" t="n">
-        <v>54.94382978723405</v>
+        <v>55.36936170212766</v>
       </c>
       <c r="Q23" t="b">
         <v>0</v>
       </c>
       <c r="R23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S23" t="b">
         <v>0</v>
@@ -2209,25 +2209,25 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>124.33</v>
+        <v>126.29</v>
       </c>
       <c r="D24" t="n">
-        <v>0.1057452863749555</v>
+        <v>0.0720713073005094</v>
       </c>
       <c r="E24" t="n">
-        <v>0.0627404051628344</v>
+        <v>0.0860853113175095</v>
       </c>
       <c r="F24" t="n">
-        <v>0.2319659135949265</v>
+        <v>0.2444816712652739</v>
       </c>
       <c r="G24" t="n">
-        <v>0.2574673876844406</v>
+        <v>0.265118454985412</v>
       </c>
       <c r="H24" t="n">
-        <v>0.2440944009637651</v>
+        <v>0.2525387937831517</v>
       </c>
       <c r="I24" t="n">
-        <v>57.90613718411552</v>
+        <v>69.90291262135922</v>
       </c>
       <c r="J24" t="n">
         <v>60</v>
@@ -2237,7 +2237,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M24" t="n">
@@ -2274,25 +2274,25 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>626</v>
+        <v>628.95</v>
       </c>
       <c r="D25" t="n">
-        <v>0.15775846125393</v>
+        <v>0.09917860887801461</v>
       </c>
       <c r="E25" t="n">
-        <v>0.1125921976361858</v>
+        <v>0.1385771180304129</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.08123578190357381</v>
+        <v>-0.0788664323374339</v>
       </c>
       <c r="G25" t="n">
-        <v>-0.0557343078140597</v>
+        <v>-0.0582296486172959</v>
       </c>
       <c r="H25" t="n">
-        <v>-0.0691072945347353</v>
+        <v>-0.0708093098195562</v>
       </c>
       <c r="I25" t="n">
-        <v>84.96767241379307</v>
+        <v>85.33893851812924</v>
       </c>
       <c r="J25" t="n">
         <v>60</v>
@@ -2302,7 +2302,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M25" t="n">
@@ -2312,10 +2312,10 @@
         <v>60</v>
       </c>
       <c r="O25" t="n">
-        <v>36.17021276595745</v>
+        <v>44.68085106382978</v>
       </c>
       <c r="P25" t="n">
-        <v>53.99804255319149</v>
+        <v>55.70017021276595</v>
       </c>
       <c r="Q25" t="b">
         <v>0</v>
@@ -2339,25 +2339,25 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>129.13</v>
+        <v>130.04</v>
       </c>
       <c r="D26" t="n">
-        <v>0.0753664223850765</v>
+        <v>0.0509981411137152</v>
       </c>
       <c r="E26" t="n">
-        <v>-0.06298526957405121</v>
+        <v>-0.0285372777528762</v>
       </c>
       <c r="F26" t="n">
-        <v>-0.2083742030407063</v>
+        <v>-0.2105390966488587</v>
       </c>
       <c r="G26" t="n">
-        <v>-0.1828727289511922</v>
+        <v>-0.1899023129287207</v>
       </c>
       <c r="H26" t="n">
-        <v>-0.1962457156718677</v>
+        <v>-0.202481974130981</v>
       </c>
       <c r="I26" t="n">
-        <v>58.41848067525539</v>
+        <v>56.70675300647543</v>
       </c>
       <c r="J26" t="n">
         <v>60</v>
@@ -2367,7 +2367,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M26" t="n">
@@ -2404,48 +2404,48 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>5506.4</v>
+        <v>5315.9</v>
       </c>
       <c r="D27" t="n">
-        <v>0.1452579034941763</v>
+        <v>0.0577852949955226</v>
       </c>
       <c r="E27" t="n">
-        <v>0.057804245509557</v>
+        <v>0.1093280467445743</v>
       </c>
       <c r="F27" t="n">
-        <v>0.0758890191481047</v>
+        <v>0.0018658122879757</v>
       </c>
       <c r="G27" t="n">
-        <v>0.1013904932376188</v>
+        <v>0.0225025960081137</v>
       </c>
       <c r="H27" t="n">
-        <v>0.08801750651694321</v>
+        <v>0.009922934805853399</v>
       </c>
       <c r="I27" t="n">
-        <v>76.29801920768305</v>
+        <v>67.66251912968258</v>
       </c>
       <c r="J27" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="K27" t="n">
         <v>57.69</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M27" t="n">
         <v>57.69</v>
       </c>
       <c r="N27" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="O27" t="n">
-        <v>65.95744680851064</v>
+        <v>61.70212765957447</v>
       </c>
       <c r="P27" t="n">
-        <v>64.26748936170213</v>
+        <v>59.4164255319149</v>
       </c>
       <c r="Q27" t="b">
         <v>0</v>
@@ -2469,25 +2469,25 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1774.8</v>
+        <v>1794.4</v>
       </c>
       <c r="D28" t="n">
-        <v>0.1988651715752498</v>
+        <v>0.1416210713831276</v>
       </c>
       <c r="E28" t="n">
-        <v>0.302988033184054</v>
+        <v>0.2868617326448652</v>
       </c>
       <c r="F28" t="n">
-        <v>0.3464835748425765</v>
+        <v>0.3775525871334255</v>
       </c>
       <c r="G28" t="n">
-        <v>0.3719850489320906</v>
+        <v>0.3981893708535635</v>
       </c>
       <c r="H28" t="n">
-        <v>0.358612062211415</v>
+        <v>0.3856097096513032</v>
       </c>
       <c r="I28" t="n">
-        <v>71.45562130177515</v>
+        <v>71.40147023950676</v>
       </c>
       <c r="J28" t="n">
         <v>70</v>
@@ -2497,7 +2497,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M28" t="n">
@@ -2534,25 +2534,25 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>544.45</v>
+        <v>541.45</v>
       </c>
       <c r="D29" t="n">
-        <v>0.1091983294285423</v>
+        <v>0.039052005373249</v>
       </c>
       <c r="E29" t="n">
-        <v>0.0154807423295719</v>
+        <v>0.0332029386508923</v>
       </c>
       <c r="F29" t="n">
-        <v>-0.0609692997585372</v>
+        <v>-0.0796362400135983</v>
       </c>
       <c r="G29" t="n">
-        <v>-0.0354678256690231</v>
+        <v>-0.0589994562934603</v>
       </c>
       <c r="H29" t="n">
-        <v>-0.0488408123896987</v>
+        <v>-0.0715791174957206</v>
       </c>
       <c r="I29" t="n">
-        <v>61.7260061919505</v>
+        <v>66.76433654248643</v>
       </c>
       <c r="J29" t="n">
         <v>80</v>
@@ -2562,7 +2562,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M29" t="n">
@@ -2572,10 +2572,10 @@
         <v>80</v>
       </c>
       <c r="O29" t="n">
-        <v>44.68085106382978</v>
+        <v>42.5531914893617</v>
       </c>
       <c r="P29" t="n">
-        <v>60.70417021276596</v>
+        <v>60.27863829787234</v>
       </c>
       <c r="Q29" t="b">
         <v>0</v>
@@ -2599,25 +2599,25 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>125.62</v>
+        <v>125.79</v>
       </c>
       <c r="D30" t="n">
-        <v>0.1159278671049126</v>
+        <v>0.1217228464419475</v>
       </c>
       <c r="E30" t="n">
-        <v>0.0289130968957327</v>
+        <v>0.0151723024776047</v>
       </c>
       <c r="F30" t="n">
-        <v>-0.0255216817934992</v>
+        <v>-0.0284986098239109</v>
       </c>
       <c r="G30" t="n">
-        <v>-2.020770398514227e-05</v>
+        <v>-0.007861826103772901</v>
       </c>
       <c r="H30" t="n">
-        <v>-0.0133931944246606</v>
+        <v>-0.0204414873060332</v>
       </c>
       <c r="I30" t="n">
-        <v>79.41760423560557</v>
+        <v>79.00776240296997</v>
       </c>
       <c r="J30" t="n">
         <v>70</v>
@@ -2627,7 +2627,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M30" t="n">
@@ -2664,48 +2664,48 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>40.01</v>
+        <v>41.29</v>
       </c>
       <c r="D31" t="n">
-        <v>0.1147952075787126</v>
+        <v>0.100773127166089</v>
       </c>
       <c r="E31" t="n">
-        <v>-0.08044127786715689</v>
+        <v>-0.0719262755675432</v>
       </c>
       <c r="F31" t="n">
-        <v>-0.1271815008726005</v>
+        <v>-0.0972890249234805</v>
       </c>
       <c r="G31" t="n">
-        <v>-0.1016800267830864</v>
+        <v>-0.07665224120334251</v>
       </c>
       <c r="H31" t="n">
-        <v>-0.1150530135037619</v>
+        <v>-0.0892319024056028</v>
       </c>
       <c r="I31" t="n">
-        <v>62.38030095759229</v>
+        <v>78.28418230563</v>
       </c>
       <c r="J31" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K31" t="n">
         <v>48.99</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M31" t="n">
         <v>48.99</v>
       </c>
       <c r="N31" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O31" t="n">
-        <v>31.91489361702128</v>
+        <v>34.04255319148936</v>
       </c>
       <c r="P31" t="n">
-        <v>57.97897872340426</v>
+        <v>54.40451063829788</v>
       </c>
       <c r="Q31" t="b">
         <v>0</v>
@@ -2729,25 +2729,25 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>754.25</v>
+        <v>763.95</v>
       </c>
       <c r="D32" t="n">
-        <v>0.1787919043525825</v>
+        <v>0.1447516295796809</v>
       </c>
       <c r="E32" t="n">
-        <v>0.0880698211194459</v>
+        <v>0.1227129105738848</v>
       </c>
       <c r="F32" t="n">
-        <v>-0.2768456375838926</v>
+        <v>-0.2652914021927293</v>
       </c>
       <c r="G32" t="n">
-        <v>-0.2513441634943785</v>
+        <v>-0.2446546184725913</v>
       </c>
       <c r="H32" t="n">
-        <v>-0.264717150215054</v>
+        <v>-0.2572342796748516</v>
       </c>
       <c r="I32" t="n">
-        <v>85.83929992044554</v>
+        <v>89.94263862332699</v>
       </c>
       <c r="J32" t="n">
         <v>60</v>
@@ -2757,7 +2757,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M32" t="n">
@@ -2767,10 +2767,10 @@
         <v>60</v>
       </c>
       <c r="O32" t="n">
-        <v>4.25531914893617</v>
+        <v>2.127659574468085</v>
       </c>
       <c r="P32" t="n">
-        <v>43.99506382978724</v>
+        <v>43.56953191489362</v>
       </c>
       <c r="Q32" t="b">
         <v>0</v>
@@ -2794,25 +2794,25 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>605.45</v>
+        <v>612.35</v>
       </c>
       <c r="D33" t="n">
-        <v>0.1850655705617538</v>
+        <v>0.1551594038860593</v>
       </c>
       <c r="E33" t="n">
-        <v>0.0545153705477663</v>
+        <v>0.06811442525728249</v>
       </c>
       <c r="F33" t="n">
-        <v>0.1565425023877746</v>
+        <v>0.1590952110543253</v>
       </c>
       <c r="G33" t="n">
-        <v>0.1820439764772887</v>
+        <v>0.1797319947744633</v>
       </c>
       <c r="H33" t="n">
-        <v>0.1686709897566132</v>
+        <v>0.167152333572203</v>
       </c>
       <c r="I33" t="n">
-        <v>82.1819914244879</v>
+        <v>89.7398843930636</v>
       </c>
       <c r="J33" t="n">
         <v>60</v>
@@ -2822,7 +2822,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M33" t="n">
@@ -2832,10 +2832,10 @@
         <v>60</v>
       </c>
       <c r="O33" t="n">
-        <v>74.46808510638297</v>
+        <v>76.59574468085107</v>
       </c>
       <c r="P33" t="n">
-        <v>58.8856170212766</v>
+        <v>59.31114893617022</v>
       </c>
       <c r="Q33" t="b">
         <v>0</v>
@@ -2871,10 +2871,10 @@
         <v>-0.2401052253975846</v>
       </c>
       <c r="G34" t="n">
-        <v>-0.2146037513080705</v>
+        <v>-0.2194684416774466</v>
       </c>
       <c r="H34" t="n">
-        <v>-0.227976738028746</v>
+        <v>-0.2320481028797069</v>
       </c>
       <c r="I34" t="n">
         <v>63.3225806451613</v>
@@ -2887,7 +2887,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M34" t="n">
@@ -2924,48 +2924,48 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>116.08</v>
+        <v>118.41</v>
       </c>
       <c r="D35" t="n">
-        <v>0.1267715006794798</v>
+        <v>0.09073323507737641</v>
       </c>
       <c r="E35" t="n">
-        <v>-0.00326292289198</v>
+        <v>0.0228921907394608</v>
       </c>
       <c r="F35" t="n">
-        <v>0.2375266524520256</v>
+        <v>0.2669591268992082</v>
       </c>
       <c r="G35" t="n">
-        <v>0.2630281265415397</v>
+        <v>0.2875959106193462</v>
       </c>
       <c r="H35" t="n">
-        <v>0.2496551398208641</v>
+        <v>0.2750162494170859</v>
       </c>
       <c r="I35" t="n">
-        <v>67.62656758012076</v>
+        <v>70.46610169491525</v>
       </c>
       <c r="J35" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K35" t="n">
         <v>49.07</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M35" t="n">
         <v>49.07</v>
       </c>
       <c r="N35" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O35" t="n">
         <v>87.2340425531915</v>
       </c>
       <c r="P35" t="n">
-        <v>69.07480851063831</v>
+        <v>65.07480851063831</v>
       </c>
       <c r="Q35" t="b">
         <v>0</v>
@@ -2989,25 +2989,25 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>488.7</v>
+        <v>486.85</v>
       </c>
       <c r="D36" t="n">
-        <v>0.0906047757197052</v>
+        <v>0.0642693190512624</v>
       </c>
       <c r="E36" t="n">
-        <v>-0.0418586413096755</v>
+        <v>-0.0438923802042419</v>
       </c>
       <c r="F36" t="n">
-        <v>0.072886937431394</v>
+        <v>0.06929497034922021</v>
       </c>
       <c r="G36" t="n">
-        <v>0.0983884115209081</v>
+        <v>0.0899317540693582</v>
       </c>
       <c r="H36" t="n">
-        <v>0.08501542480023259</v>
+        <v>0.0773520928670979</v>
       </c>
       <c r="I36" t="n">
-        <v>66.80522565320663</v>
+        <v>64.98237367802585</v>
       </c>
       <c r="J36" t="n">
         <v>80</v>
@@ -3017,7 +3017,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M36" t="n">
@@ -3027,10 +3027,10 @@
         <v>80</v>
       </c>
       <c r="O36" t="n">
-        <v>63.82978723404256</v>
+        <v>65.95744680851064</v>
       </c>
       <c r="P36" t="n">
-        <v>63.88595744680852</v>
+        <v>64.31148936170213</v>
       </c>
       <c r="Q36" t="b">
         <v>0</v>
@@ -3054,48 +3054,48 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2374.6</v>
+        <v>2547</v>
       </c>
       <c r="D37" t="n">
-        <v>0.1615143807474075</v>
+        <v>0.2037430880476392</v>
       </c>
       <c r="E37" t="n">
-        <v>0.3499715747583853</v>
+        <v>0.4817615917156319</v>
       </c>
       <c r="F37" t="n">
-        <v>0.6933609070812237</v>
+        <v>0.8181169248340352</v>
       </c>
       <c r="G37" t="n">
-        <v>0.7188623811707378</v>
+        <v>0.8387537085541732</v>
       </c>
       <c r="H37" t="n">
-        <v>0.7054893944500622</v>
+        <v>0.8261740473519129</v>
       </c>
       <c r="I37" t="n">
-        <v>73.33199356913184</v>
+        <v>80.89430894308947</v>
       </c>
       <c r="J37" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="K37" t="n">
         <v>48.59</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M37" t="n">
         <v>48.59</v>
       </c>
       <c r="N37" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="O37" t="n">
         <v>100</v>
       </c>
       <c r="P37" t="n">
-        <v>67.43600000000001</v>
+        <v>63.43600000000001</v>
       </c>
       <c r="Q37" t="b">
         <v>0</v>
@@ -3119,25 +3119,25 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>864.7</v>
+        <v>880.2</v>
       </c>
       <c r="D38" t="n">
-        <v>0.1584941050375135</v>
+        <v>0.1505882352941177</v>
       </c>
       <c r="E38" t="n">
-        <v>0.025558915969875</v>
+        <v>0.044933816109693</v>
       </c>
       <c r="F38" t="n">
-        <v>-0.1823167848699762</v>
+        <v>-0.1898757478140819</v>
       </c>
       <c r="G38" t="n">
-        <v>-0.1568153107804621</v>
+        <v>-0.1692389640939439</v>
       </c>
       <c r="H38" t="n">
-        <v>-0.1701882975011377</v>
+        <v>-0.1818186252962041</v>
       </c>
       <c r="I38" t="n">
-        <v>83.08605341246295</v>
+        <v>86.96767573114418</v>
       </c>
       <c r="J38" t="n">
         <v>60</v>
@@ -3147,7 +3147,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M38" t="n">
@@ -3157,10 +3157,10 @@
         <v>60</v>
       </c>
       <c r="O38" t="n">
-        <v>12.76595744680851</v>
+        <v>14.8936170212766</v>
       </c>
       <c r="P38" t="n">
-        <v>46.5011914893617</v>
+        <v>46.92672340425532</v>
       </c>
       <c r="Q38" t="b">
         <v>0</v>
@@ -3184,48 +3184,48 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>3586.8</v>
+        <v>3591.6</v>
       </c>
       <c r="D39" t="n">
-        <v>0.2208304969366916</v>
+        <v>0.2035789685332261</v>
       </c>
       <c r="E39" t="n">
-        <v>0.3096724723408919</v>
+        <v>0.3066065192083818</v>
       </c>
       <c r="F39" t="n">
-        <v>0.3102944399795426</v>
+        <v>0.3140641006878384</v>
       </c>
       <c r="G39" t="n">
-        <v>0.3357959140690567</v>
+        <v>0.3347008844079764</v>
       </c>
       <c r="H39" t="n">
-        <v>0.3224229273483812</v>
+        <v>0.3221212232057161</v>
       </c>
       <c r="I39" t="n">
-        <v>74.83197736116026</v>
+        <v>81.92144782441277</v>
       </c>
       <c r="J39" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="K39" t="n">
         <v>48.69</v>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M39" t="n">
         <v>48.69</v>
       </c>
       <c r="N39" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="O39" t="n">
         <v>89.36170212765957</v>
       </c>
       <c r="P39" t="n">
-        <v>65.34834042553192</v>
+        <v>61.34834042553192</v>
       </c>
       <c r="Q39" t="b">
         <v>0</v>
@@ -3249,25 +3249,25 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>217.4</v>
+        <v>216.28</v>
       </c>
       <c r="D40" t="n">
-        <v>0.2024336283185841</v>
+        <v>0.1906413432424993</v>
       </c>
       <c r="E40" t="n">
-        <v>0.1419266729698498</v>
+        <v>0.1553418803418804</v>
       </c>
       <c r="F40" t="n">
-        <v>-0.0504062199702978</v>
+        <v>-0.0579729082277102</v>
       </c>
       <c r="G40" t="n">
-        <v>-0.0249047458807837</v>
+        <v>-0.0373361245075722</v>
       </c>
       <c r="H40" t="n">
-        <v>-0.0382777326014592</v>
+        <v>-0.0499157857098325</v>
       </c>
       <c r="I40" t="n">
-        <v>87.51271617497457</v>
+        <v>84.57405986185725</v>
       </c>
       <c r="J40" t="n">
         <v>60</v>
@@ -3277,7 +3277,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M40" t="n">
@@ -3314,48 +3314,48 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>835.25</v>
+        <v>835.9</v>
       </c>
       <c r="D41" t="n">
-        <v>0.0481239804241435</v>
+        <v>0.0510499182698354</v>
       </c>
       <c r="E41" t="n">
-        <v>-0.0918234206806567</v>
+        <v>-0.1016657710908114</v>
       </c>
       <c r="F41" t="n">
-        <v>-0.1733471892319873</v>
+        <v>-0.184925162108137</v>
       </c>
       <c r="G41" t="n">
-        <v>-0.1478457151424732</v>
+        <v>-0.164288378387999</v>
       </c>
       <c r="H41" t="n">
-        <v>-0.1612187018631488</v>
+        <v>-0.1768680395902593</v>
       </c>
       <c r="I41" t="n">
-        <v>78.6235662148071</v>
+        <v>80.3886925795053</v>
       </c>
       <c r="J41" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="K41" t="n">
         <v>48.05</v>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M41" t="n">
         <v>48.05</v>
       </c>
       <c r="N41" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="O41" t="n">
-        <v>19.14893617021277</v>
+        <v>17.02127659574468</v>
       </c>
       <c r="P41" t="n">
-        <v>43.04978723404256</v>
+        <v>46.62425531914894</v>
       </c>
       <c r="Q41" t="b">
         <v>0</v>
@@ -3379,25 +3379,25 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>621.2</v>
+        <v>625.45</v>
       </c>
       <c r="D42" t="n">
-        <v>0.2161315583398591</v>
+        <v>0.1903130649919115</v>
       </c>
       <c r="E42" t="n">
-        <v>0.0310373443983402</v>
+        <v>0.0407687827606289</v>
       </c>
       <c r="F42" t="n">
-        <v>-0.1733315589859604</v>
+        <v>-0.1725757375314194</v>
       </c>
       <c r="G42" t="n">
-        <v>-0.1478300848964463</v>
+        <v>-0.1519389538112814</v>
       </c>
       <c r="H42" t="n">
-        <v>-0.1612030716171218</v>
+        <v>-0.1645186150135417</v>
       </c>
       <c r="I42" t="n">
-        <v>81.83457871682553</v>
+        <v>82.43174924165821</v>
       </c>
       <c r="J42" t="n">
         <v>60</v>
@@ -3407,7 +3407,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M42" t="n">
@@ -3417,10 +3417,10 @@
         <v>60</v>
       </c>
       <c r="O42" t="n">
-        <v>21.27659574468085</v>
+        <v>19.14893617021277</v>
       </c>
       <c r="P42" t="n">
-        <v>47.31931914893617</v>
+        <v>46.89378723404256</v>
       </c>
       <c r="Q42" t="b">
         <v>0</v>
@@ -3444,25 +3444,25 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>422.1</v>
+        <v>428.7</v>
       </c>
       <c r="D43" t="n">
-        <v>0.0547226386806598</v>
+        <v>0.06854436689930191</v>
       </c>
       <c r="E43" t="n">
-        <v>-0.0369609856262833</v>
+        <v>-0.0054518037350655</v>
       </c>
       <c r="F43" t="n">
-        <v>-0.0901056262125457</v>
+        <v>-0.09642744230161231</v>
       </c>
       <c r="G43" t="n">
-        <v>-0.0646041521230316</v>
+        <v>-0.0757906585814743</v>
       </c>
       <c r="H43" t="n">
-        <v>-0.07797713884370711</v>
+        <v>-0.08837031978373459</v>
       </c>
       <c r="I43" t="n">
-        <v>50.07342143906023</v>
+        <v>58.71886120996441</v>
       </c>
       <c r="J43" t="n">
         <v>80</v>
@@ -3472,7 +3472,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M43" t="n">
@@ -3482,10 +3482,10 @@
         <v>80</v>
       </c>
       <c r="O43" t="n">
-        <v>34.04255319148936</v>
+        <v>36.17021276595745</v>
       </c>
       <c r="P43" t="n">
-        <v>59.40051063829787</v>
+        <v>59.82604255319149</v>
       </c>
       <c r="Q43" t="b">
         <v>0</v>
@@ -3509,25 +3509,25 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>279.95</v>
+        <v>277.79</v>
       </c>
       <c r="D44" t="n">
-        <v>0.2475490196078431</v>
+        <v>0.2398571747377818</v>
       </c>
       <c r="E44" t="n">
-        <v>0.1827207435572455</v>
+        <v>0.1084996009577017</v>
       </c>
       <c r="F44" t="n">
-        <v>-0.0665221740580193</v>
+        <v>-0.06750587445451479</v>
       </c>
       <c r="G44" t="n">
-        <v>-0.0410206999685052</v>
+        <v>-0.0468690907343768</v>
       </c>
       <c r="H44" t="n">
-        <v>-0.0543936866891807</v>
+        <v>-0.0594487519366371</v>
       </c>
       <c r="I44" t="n">
-        <v>95.93781344032088</v>
+        <v>90.23003360041356</v>
       </c>
       <c r="J44" t="n">
         <v>60</v>
@@ -3537,7 +3537,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M44" t="n">
@@ -3547,10 +3547,10 @@
         <v>60</v>
       </c>
       <c r="O44" t="n">
-        <v>38.29787234042553</v>
+        <v>46.80851063829788</v>
       </c>
       <c r="P44" t="n">
-        <v>50.53957446808511</v>
+        <v>52.24170212765958</v>
       </c>
       <c r="Q44" t="b">
         <v>0</v>
@@ -3574,25 +3574,25 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>104.01</v>
+        <v>103.02</v>
       </c>
       <c r="D45" t="n">
-        <v>0.1269910066096</v>
+        <v>0.1098901098901099</v>
       </c>
       <c r="E45" t="n">
-        <v>-0.0950143565648655</v>
+        <v>-0.1070468926063968</v>
       </c>
       <c r="F45" t="n">
-        <v>-0.2476128472222222</v>
+        <v>-0.2490706319702602</v>
       </c>
       <c r="G45" t="n">
-        <v>-0.2221113731327081</v>
+        <v>-0.2284338482501222</v>
       </c>
       <c r="H45" t="n">
-        <v>-0.2354843598533836</v>
+        <v>-0.2410135094523825</v>
       </c>
       <c r="I45" t="n">
-        <v>87.52173913043481</v>
+        <v>81.56638013371538</v>
       </c>
       <c r="J45" t="n">
         <v>60</v>
@@ -3602,7 +3602,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M45" t="n">
@@ -3639,25 +3639,25 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>527.65</v>
+        <v>533.8</v>
       </c>
       <c r="D46" t="n">
-        <v>0.1099074463609592</v>
+        <v>0.0911692559280457</v>
       </c>
       <c r="E46" t="n">
-        <v>-0.0093870271285083</v>
+        <v>-0.0184793601176795</v>
       </c>
       <c r="F46" t="n">
-        <v>-0.1352126526264033</v>
+        <v>-0.1381982563771392</v>
       </c>
       <c r="G46" t="n">
-        <v>-0.1097111785368892</v>
+        <v>-0.1175614726570012</v>
       </c>
       <c r="H46" t="n">
-        <v>-0.1230841652575648</v>
+        <v>-0.1301411338592615</v>
       </c>
       <c r="I46" t="n">
-        <v>67.7721701514059</v>
+        <v>66.44144144144144</v>
       </c>
       <c r="J46" t="n">
         <v>80</v>
@@ -3667,7 +3667,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M46" t="n">
@@ -3677,10 +3677,10 @@
         <v>80</v>
       </c>
       <c r="O46" t="n">
-        <v>27.65957446808511</v>
+        <v>25.53191489361702</v>
       </c>
       <c r="P46" t="n">
-        <v>57.37591489361702</v>
+        <v>56.95038297872341</v>
       </c>
       <c r="Q46" t="b">
         <v>0</v>
@@ -3704,25 +3704,25 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>1045.9</v>
+        <v>1077.2</v>
       </c>
       <c r="D47" t="n">
-        <v>0.0638795646424577</v>
+        <v>0.049697914636523</v>
       </c>
       <c r="E47" t="n">
-        <v>0.3764558794498915</v>
+        <v>0.4410702341137125</v>
       </c>
       <c r="F47" t="n">
-        <v>0.193200616051566</v>
+        <v>0.2284883389405256</v>
       </c>
       <c r="G47" t="n">
-        <v>0.2187020901410801</v>
+        <v>0.2491251226606636</v>
       </c>
       <c r="H47" t="n">
-        <v>0.2053291034204045</v>
+        <v>0.2365454614584033</v>
       </c>
       <c r="I47" t="n">
-        <v>60.97423359037055</v>
+        <v>68.11058284909316</v>
       </c>
       <c r="J47" t="n">
         <v>80</v>
@@ -3732,7 +3732,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M47" t="n">
@@ -3769,25 +3769,25 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>15380</v>
+        <v>15184</v>
       </c>
       <c r="D48" t="n">
-        <v>0.1543946558582902</v>
+        <v>0.1510878629368508</v>
       </c>
       <c r="E48" t="n">
-        <v>0.1195224923569659</v>
+        <v>0.1024468162346621</v>
       </c>
       <c r="F48" t="n">
-        <v>0.1771909682357444</v>
+        <v>0.1190212985481613</v>
       </c>
       <c r="G48" t="n">
-        <v>0.2026924423252585</v>
+        <v>0.1396580822682993</v>
       </c>
       <c r="H48" t="n">
-        <v>0.1893194556045829</v>
+        <v>0.127078421066039</v>
       </c>
       <c r="I48" t="n">
-        <v>64.16690160699183</v>
+        <v>68.10293237582286</v>
       </c>
       <c r="J48" t="n">
         <v>80</v>
@@ -3797,7 +3797,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M48" t="n">
@@ -3807,10 +3807,10 @@
         <v>80</v>
       </c>
       <c r="O48" t="n">
-        <v>78.72340425531915</v>
+        <v>70.21276595744681</v>
       </c>
       <c r="P48" t="n">
-        <v>67.86068085106383</v>
+        <v>66.15855319148936</v>
       </c>
       <c r="Q48" t="b">
         <v>0</v>
@@ -3936,57 +3936,57 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>RICOAUTO</t>
+          <t>LUMAXTECH</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Castings</t>
+          <t>Lighting</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>116.08</v>
+        <v>1794.4</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1267715006794798</v>
+        <v>0.1416210713831276</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.00326292289198</v>
+        <v>0.2868617326448652</v>
       </c>
       <c r="F2" t="n">
-        <v>0.2375266524520256</v>
+        <v>0.3775525871334255</v>
       </c>
       <c r="G2" t="n">
-        <v>0.2630281265415397</v>
+        <v>0.3981893708535635</v>
       </c>
       <c r="H2" t="n">
-        <v>0.2496551398208641</v>
+        <v>0.3856097096513032</v>
       </c>
       <c r="I2" t="n">
-        <v>67.62656758012076</v>
+        <v>71.40147023950676</v>
       </c>
       <c r="J2" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K2" t="n">
-        <v>49.07</v>
+        <v>54.51</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M2" t="n">
-        <v>49.07</v>
+        <v>54.51</v>
       </c>
       <c r="N2" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O2" t="n">
-        <v>87.2340425531915</v>
+        <v>91.48936170212764</v>
       </c>
       <c r="P2" t="n">
-        <v>69.07480851063831</v>
+        <v>68.10187234042553</v>
       </c>
       <c r="Q2" t="b">
         <v>0</v>
@@ -4001,57 +4001,57 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>LUMAXTECH</t>
+          <t>WHEELS</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Lighting</t>
+          <t>Wheels</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1774.8</v>
+        <v>1077.2</v>
       </c>
       <c r="D3" t="n">
-        <v>0.1988651715752498</v>
+        <v>0.049697914636523</v>
       </c>
       <c r="E3" t="n">
-        <v>0.302988033184054</v>
+        <v>0.4410702341137125</v>
       </c>
       <c r="F3" t="n">
-        <v>0.3464835748425765</v>
+        <v>0.2284883389405256</v>
       </c>
       <c r="G3" t="n">
-        <v>0.3719850489320906</v>
+        <v>0.2491251226606636</v>
       </c>
       <c r="H3" t="n">
-        <v>0.358612062211415</v>
+        <v>0.2365454614584033</v>
       </c>
       <c r="I3" t="n">
-        <v>71.45562130177515</v>
+        <v>68.11058284909316</v>
       </c>
       <c r="J3" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K3" t="n">
-        <v>54.51</v>
+        <v>46.83</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M3" t="n">
-        <v>54.51</v>
+        <v>46.83</v>
       </c>
       <c r="N3" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O3" t="n">
-        <v>91.48936170212764</v>
+        <v>80.85106382978722</v>
       </c>
       <c r="P3" t="n">
-        <v>68.10187234042553</v>
+        <v>66.90221276595744</v>
       </c>
       <c r="Q3" t="b">
         <v>0</v>
@@ -4066,57 +4066,57 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ZFCVINDIA</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Brakes/Transmission</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>15380</v>
+        <v>588.45</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1543946558582902</v>
+        <v>0.189508793208005</v>
       </c>
       <c r="E4" t="n">
-        <v>0.1195224923569659</v>
+        <v>0.3239959500506244</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1771909682357444</v>
+        <v>0.4020729092208721</v>
       </c>
       <c r="G4" t="n">
-        <v>0.2026924423252585</v>
+        <v>0.4227096929410101</v>
       </c>
       <c r="H4" t="n">
-        <v>0.1893194556045829</v>
+        <v>0.4101300317387498</v>
       </c>
       <c r="I4" t="n">
-        <v>64.16690160699183</v>
+        <v>79.17460317460311</v>
       </c>
       <c r="J4" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K4" t="n">
-        <v>50.29</v>
+        <v>49.66</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M4" t="n">
-        <v>50.29</v>
+        <v>49.66</v>
       </c>
       <c r="N4" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O4" t="n">
-        <v>78.72340425531915</v>
+        <v>93.61702127659576</v>
       </c>
       <c r="P4" t="n">
-        <v>67.86068085106383</v>
+        <v>66.58740425531916</v>
       </c>
       <c r="Q4" t="b">
         <v>0</v>
@@ -4131,57 +4131,57 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SANSERA</t>
+          <t>ZFCVINDIA</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Forgings</t>
+          <t>Brakes/Transmission</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>2374.6</v>
+        <v>15184</v>
       </c>
       <c r="D5" t="n">
-        <v>0.1615143807474075</v>
+        <v>0.1510878629368508</v>
       </c>
       <c r="E5" t="n">
-        <v>0.3499715747583853</v>
+        <v>0.1024468162346621</v>
       </c>
       <c r="F5" t="n">
-        <v>0.6933609070812237</v>
+        <v>0.1190212985481613</v>
       </c>
       <c r="G5" t="n">
-        <v>0.7188623811707378</v>
+        <v>0.1396580822682993</v>
       </c>
       <c r="H5" t="n">
-        <v>0.7054893944500622</v>
+        <v>0.127078421066039</v>
       </c>
       <c r="I5" t="n">
-        <v>73.33199356913184</v>
+        <v>68.10293237582286</v>
       </c>
       <c r="J5" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K5" t="n">
-        <v>48.59</v>
+        <v>50.29</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M5" t="n">
-        <v>48.59</v>
+        <v>50.29</v>
       </c>
       <c r="N5" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O5" t="n">
-        <v>100</v>
+        <v>70.21276595744681</v>
       </c>
       <c r="P5" t="n">
-        <v>67.43600000000001</v>
+        <v>66.15855319148936</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
@@ -4196,57 +4196,57 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>WHEELS</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Wheels</t>
+          <t>Forgings</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1045.9</v>
+        <v>1903.2</v>
       </c>
       <c r="D6" t="n">
-        <v>0.0638795646424577</v>
+        <v>0.1137640449438202</v>
       </c>
       <c r="E6" t="n">
-        <v>0.3764558794498915</v>
+        <v>0.3791304347826087</v>
       </c>
       <c r="F6" t="n">
-        <v>0.193200616051566</v>
+        <v>0.5597443042124242</v>
       </c>
       <c r="G6" t="n">
-        <v>0.2187020901410801</v>
+        <v>0.5803810879325622</v>
       </c>
       <c r="H6" t="n">
-        <v>0.2053291034204045</v>
+        <v>0.5678014267303019</v>
       </c>
       <c r="I6" t="n">
-        <v>60.97423359037055</v>
+        <v>87.81195589088799</v>
       </c>
       <c r="J6" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K6" t="n">
-        <v>46.83</v>
+        <v>54.83</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M6" t="n">
-        <v>46.83</v>
+        <v>54.83</v>
       </c>
       <c r="N6" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O6" t="n">
-        <v>80.85106382978722</v>
+        <v>97.87234042553192</v>
       </c>
       <c r="P6" t="n">
-        <v>66.90221276595744</v>
+        <v>65.50646808510639</v>
       </c>
       <c r="Q6" t="b">
         <v>0</v>
@@ -4261,63 +4261,63 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>ASKAUTOLTD</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>581.3</v>
+        <v>442.8</v>
       </c>
       <c r="D7" t="n">
-        <v>0.198680276317146</v>
+        <v>0.0662171923910426</v>
       </c>
       <c r="E7" t="n">
-        <v>0.3035093620361027</v>
+        <v>0.0273781902552203</v>
       </c>
       <c r="F7" t="n">
-        <v>0.4049546827794561</v>
+        <v>-0.1520490233626963</v>
       </c>
       <c r="G7" t="n">
-        <v>0.4304561568689702</v>
+        <v>-0.1314122396425583</v>
       </c>
       <c r="H7" t="n">
-        <v>0.4170831701482946</v>
+        <v>-0.1439919008448186</v>
       </c>
       <c r="I7" t="n">
-        <v>77.82191327375034</v>
+        <v>58.70165745856355</v>
       </c>
       <c r="J7" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K7" t="n">
-        <v>49.66</v>
+        <v>71.28</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M7" t="n">
-        <v>49.66</v>
+        <v>71.28</v>
       </c>
       <c r="N7" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O7" t="n">
-        <v>93.61702127659576</v>
+        <v>23.40425531914894</v>
       </c>
       <c r="P7" t="n">
-        <v>66.58740425531916</v>
+        <v>65.19285106382979</v>
       </c>
       <c r="Q7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S7" t="b">
         <v>0</v>
@@ -4326,57 +4326,57 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>RICOAUTO</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Forgings</t>
+          <t>Castings</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1895.8</v>
+        <v>118.41</v>
       </c>
       <c r="D8" t="n">
-        <v>0.1499454082251607</v>
+        <v>0.09073323507737641</v>
       </c>
       <c r="E8" t="n">
-        <v>0.3598737536762069</v>
+        <v>0.0228921907394608</v>
       </c>
       <c r="F8" t="n">
-        <v>0.5544440800262382</v>
+        <v>0.2669591268992082</v>
       </c>
       <c r="G8" t="n">
-        <v>0.5799455541157523</v>
+        <v>0.2875959106193462</v>
       </c>
       <c r="H8" t="n">
-        <v>0.5665725673950768</v>
+        <v>0.2750162494170859</v>
       </c>
       <c r="I8" t="n">
-        <v>81.32231404958674</v>
+        <v>70.46610169491525</v>
       </c>
       <c r="J8" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K8" t="n">
-        <v>54.83</v>
+        <v>49.07</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M8" t="n">
-        <v>54.83</v>
+        <v>49.07</v>
       </c>
       <c r="N8" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O8" t="n">
-        <v>97.87234042553192</v>
+        <v>87.2340425531915</v>
       </c>
       <c r="P8" t="n">
-        <v>65.50646808510639</v>
+        <v>65.07480851063831</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
@@ -4391,57 +4391,57 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BHARATGEAR</t>
+          <t>GNA</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Gears</t>
+          <t>Axles</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>108.92</v>
+        <v>457.2</v>
       </c>
       <c r="D9" t="n">
-        <v>0.1734539969834088</v>
+        <v>0.2295280354981845</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.0137631293009778</v>
+        <v>0.3678384442782347</v>
       </c>
       <c r="F9" t="n">
-        <v>0.2253346833164584</v>
+        <v>0.4595371109337589</v>
       </c>
       <c r="G9" t="n">
-        <v>0.2508361574059725</v>
+        <v>0.4801738946538969</v>
       </c>
       <c r="H9" t="n">
-        <v>0.237463170685297</v>
+        <v>0.4675942334516366</v>
       </c>
       <c r="I9" t="n">
-        <v>79.73770491803278</v>
+        <v>88.76353790613715</v>
       </c>
       <c r="J9" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="K9" t="n">
-        <v>51.91</v>
+        <v>54.47</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M9" t="n">
-        <v>51.91</v>
+        <v>54.47</v>
       </c>
       <c r="N9" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="O9" t="n">
-        <v>82.97872340425532</v>
+        <v>95.74468085106383</v>
       </c>
       <c r="P9" t="n">
-        <v>65.35974468085107</v>
+        <v>64.93693617021276</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -4456,57 +4456,57 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SHRIPISTON</t>
+          <t>SANDHAR</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Engine/Parts</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>3586.8</v>
+        <v>486.85</v>
       </c>
       <c r="D10" t="n">
-        <v>0.2208304969366916</v>
+        <v>0.0642693190512624</v>
       </c>
       <c r="E10" t="n">
-        <v>0.3096724723408919</v>
+        <v>-0.0438923802042419</v>
       </c>
       <c r="F10" t="n">
-        <v>0.3102944399795426</v>
+        <v>0.06929497034922021</v>
       </c>
       <c r="G10" t="n">
-        <v>0.3357959140690567</v>
+        <v>0.0899317540693582</v>
       </c>
       <c r="H10" t="n">
-        <v>0.3224229273483812</v>
+        <v>0.0773520928670979</v>
       </c>
       <c r="I10" t="n">
-        <v>74.83197736116026</v>
+        <v>64.98237367802585</v>
       </c>
       <c r="J10" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K10" t="n">
-        <v>48.69</v>
+        <v>47.8</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M10" t="n">
-        <v>48.69</v>
+        <v>47.8</v>
       </c>
       <c r="N10" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O10" t="n">
-        <v>89.36170212765957</v>
+        <v>65.95744680851064</v>
       </c>
       <c r="P10" t="n">
-        <v>65.34834042553192</v>
+        <v>64.31148936170213</v>
       </c>
       <c r="Q10" t="b">
         <v>0</v>
@@ -4521,57 +4521,57 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>GNA</t>
+          <t>SANSERA</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Axles</t>
+          <t>Forgings</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>450.65</v>
+        <v>2547</v>
       </c>
       <c r="D11" t="n">
-        <v>0.2662264681090194</v>
+        <v>0.2037430880476392</v>
       </c>
       <c r="E11" t="n">
-        <v>0.3238836662749706</v>
+        <v>0.4817615917156319</v>
       </c>
       <c r="F11" t="n">
-        <v>0.4383977018831788</v>
+        <v>0.8181169248340352</v>
       </c>
       <c r="G11" t="n">
-        <v>0.4638991759726929</v>
+        <v>0.8387537085541732</v>
       </c>
       <c r="H11" t="n">
-        <v>0.4505261892520174</v>
+        <v>0.8261740473519129</v>
       </c>
       <c r="I11" t="n">
-        <v>82.40574506283662</v>
+        <v>80.89430894308947</v>
       </c>
       <c r="J11" t="n">
         <v>60</v>
       </c>
       <c r="K11" t="n">
-        <v>54.47</v>
+        <v>48.59</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M11" t="n">
-        <v>54.47</v>
+        <v>48.59</v>
       </c>
       <c r="N11" t="n">
         <v>60</v>
       </c>
       <c r="O11" t="n">
-        <v>95.74468085106383</v>
+        <v>100</v>
       </c>
       <c r="P11" t="n">
-        <v>64.93693617021276</v>
+        <v>63.43600000000001</v>
       </c>
       <c r="Q11" t="b">
         <v>0</v>
@@ -4586,57 +4586,57 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>LUMAXIND</t>
+          <t>DIVGIITTS</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Lighting</t>
+          <t>Transmission</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>5506.4</v>
+        <v>733.8</v>
       </c>
       <c r="D12" t="n">
-        <v>0.1452579034941763</v>
+        <v>0.0526466790991249</v>
       </c>
       <c r="E12" t="n">
-        <v>0.057804245509557</v>
+        <v>0.253608951909114</v>
       </c>
       <c r="F12" t="n">
-        <v>0.0758890191481047</v>
+        <v>0.0866281652598845</v>
       </c>
       <c r="G12" t="n">
-        <v>0.1013904932376188</v>
+        <v>0.1072649489800225</v>
       </c>
       <c r="H12" t="n">
-        <v>0.08801750651694321</v>
+        <v>0.09468528777776231</v>
       </c>
       <c r="I12" t="n">
-        <v>76.29801920768305</v>
+        <v>73.33177788147458</v>
       </c>
       <c r="J12" t="n">
         <v>70</v>
       </c>
       <c r="K12" t="n">
-        <v>57.69</v>
+        <v>49.92</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M12" t="n">
-        <v>57.69</v>
+        <v>49.92</v>
       </c>
       <c r="N12" t="n">
         <v>70</v>
       </c>
       <c r="O12" t="n">
-        <v>65.95744680851064</v>
+        <v>68.08510638297872</v>
       </c>
       <c r="P12" t="n">
-        <v>64.26748936170213</v>
+        <v>61.58502127659575</v>
       </c>
       <c r="Q12" t="b">
         <v>0</v>
@@ -4651,57 +4651,57 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MOTHERSON</t>
+          <t>SHRIPISTON</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Engine/Parts</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>124.7</v>
+        <v>3591.6</v>
       </c>
       <c r="D13" t="n">
-        <v>0.1699033680457828</v>
+        <v>0.2035789685332261</v>
       </c>
       <c r="E13" t="n">
-        <v>0.1558068403003059</v>
+        <v>0.3066065192083818</v>
       </c>
       <c r="F13" t="n">
-        <v>0.1764150943396227</v>
+        <v>0.3140641006878384</v>
       </c>
       <c r="G13" t="n">
-        <v>0.2019165684291368</v>
+        <v>0.3347008844079764</v>
       </c>
       <c r="H13" t="n">
-        <v>0.1885435817084613</v>
+        <v>0.3221212232057161</v>
       </c>
       <c r="I13" t="n">
-        <v>76.39060568603213</v>
+        <v>81.92144782441277</v>
       </c>
       <c r="J13" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="K13" t="n">
-        <v>51.57</v>
+        <v>48.69</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M13" t="n">
-        <v>51.57</v>
+        <v>48.69</v>
       </c>
       <c r="N13" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="O13" t="n">
-        <v>76.59574468085107</v>
+        <v>89.36170212765957</v>
       </c>
       <c r="P13" t="n">
-        <v>63.94714893617022</v>
+        <v>61.34834042553192</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
@@ -4716,57 +4716,57 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SANDHAR</t>
+          <t>MOTHERSON</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>488.7</v>
+        <v>131.76</v>
       </c>
       <c r="D14" t="n">
-        <v>0.0906047757197052</v>
+        <v>0.185638441464951</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.0418586413096755</v>
+        <v>0.2014224491656788</v>
       </c>
       <c r="F14" t="n">
-        <v>0.072886937431394</v>
+        <v>0.235211399643761</v>
       </c>
       <c r="G14" t="n">
-        <v>0.0983884115209081</v>
+        <v>0.255848183363899</v>
       </c>
       <c r="H14" t="n">
-        <v>0.08501542480023259</v>
+        <v>0.2432685221616387</v>
       </c>
       <c r="I14" t="n">
-        <v>66.80522565320663</v>
+        <v>82.3102823102823</v>
       </c>
       <c r="J14" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K14" t="n">
-        <v>47.8</v>
+        <v>51.57</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M14" t="n">
-        <v>47.8</v>
+        <v>51.57</v>
       </c>
       <c r="N14" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O14" t="n">
-        <v>63.82978723404256</v>
+        <v>82.97872340425532</v>
       </c>
       <c r="P14" t="n">
-        <v>63.88595744680852</v>
+        <v>61.22374468085107</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
@@ -4781,57 +4781,57 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>DIVGIITTS</t>
+          <t>JAMNAAUTO</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Transmission</t>
+          <t>Suspension</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>748.1</v>
+        <v>126.29</v>
       </c>
       <c r="D15" t="n">
-        <v>0.1359805633588946</v>
+        <v>0.0720713073005094</v>
       </c>
       <c r="E15" t="n">
-        <v>0.2627225926238501</v>
+        <v>0.0860853113175095</v>
       </c>
       <c r="F15" t="n">
-        <v>0.1160674324929136</v>
+        <v>0.2444816712652739</v>
       </c>
       <c r="G15" t="n">
-        <v>0.1415689065824277</v>
+        <v>0.265118454985412</v>
       </c>
       <c r="H15" t="n">
-        <v>0.1281959198617521</v>
+        <v>0.2525387937831517</v>
       </c>
       <c r="I15" t="n">
-        <v>78.78187670215402</v>
+        <v>69.90291262135922</v>
       </c>
       <c r="J15" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="K15" t="n">
-        <v>49.92</v>
+        <v>48.3</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M15" t="n">
-        <v>49.92</v>
+        <v>48.3</v>
       </c>
       <c r="N15" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="O15" t="n">
-        <v>68.08510638297872</v>
+        <v>85.1063829787234</v>
       </c>
       <c r="P15" t="n">
-        <v>61.58502127659575</v>
+        <v>60.34127659574468</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
@@ -4846,63 +4846,63 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>MINDACORP</t>
+          <t>CRAFTSMAN</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Castings</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>544.45</v>
+        <v>7684.5</v>
       </c>
       <c r="D16" t="n">
-        <v>0.1091983294285423</v>
+        <v>0.122972380534853</v>
       </c>
       <c r="E16" t="n">
-        <v>0.0154807423295719</v>
+        <v>0.0394994927291174</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.0609692997585372</v>
+        <v>0.1344947220786889</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.0354678256690231</v>
+        <v>0.1551315057988269</v>
       </c>
       <c r="H16" t="n">
-        <v>-0.0488408123896987</v>
+        <v>0.1425518445965666</v>
       </c>
       <c r="I16" t="n">
-        <v>61.7260061919505</v>
+        <v>87.80075981426762</v>
       </c>
       <c r="J16" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K16" t="n">
-        <v>49.42</v>
+        <v>54.65</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="M16" t="n">
-        <v>49.42</v>
+        <v>54.65</v>
       </c>
       <c r="N16" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O16" t="n">
-        <v>44.68085106382978</v>
+        <v>72.3404255319149</v>
       </c>
       <c r="P16" t="n">
-        <v>60.70417021276596</v>
+        <v>60.32808510638298</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>
       </c>
       <c r="R16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S16" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
chore: auto-refresh NSE data and pipeline outputs (2026-04-24)
</commit_message>
<xml_diff>
--- a/working-sector/output/auto_components_comprehensive_report.xlsx
+++ b/working-sector/output/auto_components_comprehensive_report.xlsx
@@ -435,7 +435,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
     </row>
@@ -447,7 +447,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
     </row>
@@ -779,48 +779,48 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1903.2</v>
+        <v>1856</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1137640449438202</v>
+        <v>0.0688165850849409</v>
       </c>
       <c r="E2" t="n">
-        <v>0.3791304347826087</v>
+        <v>0.3174332765474164</v>
       </c>
       <c r="F2" t="n">
-        <v>0.5597443042124242</v>
+        <v>0.5253122945430639</v>
       </c>
       <c r="G2" t="n">
-        <v>0.5803810879325622</v>
+        <v>0.5588247755404134</v>
       </c>
       <c r="H2" t="n">
-        <v>0.5678014267303019</v>
+        <v>0.5325283268469598</v>
       </c>
       <c r="I2" t="n">
-        <v>87.81195589088799</v>
+        <v>75.48103353490929</v>
       </c>
       <c r="J2" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K2" t="n">
         <v>54.83</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M2" t="n">
         <v>54.83</v>
       </c>
       <c r="N2" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O2" t="n">
         <v>97.87234042553192</v>
       </c>
       <c r="P2" t="n">
-        <v>65.50646808510639</v>
+        <v>69.50646808510639</v>
       </c>
       <c r="Q2" t="b">
         <v>0</v>
@@ -844,48 +844,48 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1151.3</v>
+        <v>1108.1</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0745753220085867</v>
+        <v>0.0188488414858403</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0202942219071249</v>
+        <v>-0.0229256679305176</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.1251519756838905</v>
+        <v>-0.1889775305569787</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.1045151919637525</v>
+        <v>-0.1554650495596292</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.1170948531660128</v>
+        <v>-0.1817614982530828</v>
       </c>
       <c r="I3" t="n">
-        <v>72.94932555596054</v>
+        <v>60.13582342954154</v>
       </c>
       <c r="J3" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K3" t="n">
         <v>49.36</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M3" t="n">
         <v>49.36</v>
       </c>
       <c r="N3" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O3" t="n">
-        <v>27.65957446808511</v>
+        <v>25.53191489361702</v>
       </c>
       <c r="P3" t="n">
-        <v>53.27591489361702</v>
+        <v>56.8503829787234</v>
       </c>
       <c r="Q3" t="b">
         <v>0</v>
@@ -909,48 +909,48 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>37885</v>
+        <v>36690</v>
       </c>
       <c r="D4" t="n">
-        <v>0.2594747340425531</v>
+        <v>0.2073050345508391</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0784230002846571</v>
+        <v>0.0404083368779242</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.0192855293813098</v>
+        <v>-0.0536497291720402</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0013512543388281</v>
+        <v>-0.0201372481746907</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.0112284068634321</v>
+        <v>-0.0464336968681443</v>
       </c>
       <c r="I4" t="n">
-        <v>87.63089005235602</v>
+        <v>71.50466045272969</v>
       </c>
       <c r="J4" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K4" t="n">
         <v>53.48</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M4" t="n">
         <v>53.48</v>
       </c>
       <c r="N4" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O4" t="n">
-        <v>55.31914893617022</v>
+        <v>51.06382978723404</v>
       </c>
       <c r="P4" t="n">
-        <v>56.45582978723404</v>
+        <v>59.6047659574468</v>
       </c>
       <c r="Q4" t="b">
         <v>0</v>
@@ -974,48 +974,48 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>354.55</v>
+        <v>342.8</v>
       </c>
       <c r="D5" t="n">
-        <v>0.1877721943048576</v>
+        <v>0.1160670682077162</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0877435189446234</v>
+        <v>0.0541205412054122</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.1092827534229368</v>
+        <v>-0.1490629266476356</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.0886459697027988</v>
+        <v>-0.1155504456502861</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.1012256309050591</v>
+        <v>-0.1418468943437397</v>
       </c>
       <c r="I5" t="n">
-        <v>90.36496350364968</v>
+        <v>77.56892230576443</v>
       </c>
       <c r="J5" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K5" t="n">
         <v>51.12</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M5" t="n">
         <v>51.12</v>
       </c>
       <c r="N5" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O5" t="n">
-        <v>29.78723404255319</v>
+        <v>31.91489361702128</v>
       </c>
       <c r="P5" t="n">
-        <v>50.40544680851064</v>
+        <v>54.83097872340426</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
@@ -1039,48 +1039,48 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>131.76</v>
+        <v>125.7</v>
       </c>
       <c r="D6" t="n">
-        <v>0.185638441464951</v>
+        <v>0.1111111111111111</v>
       </c>
       <c r="E6" t="n">
-        <v>0.2014224491656788</v>
+        <v>0.1595940959409594</v>
       </c>
       <c r="F6" t="n">
-        <v>0.235211399643761</v>
+        <v>0.2072608528620823</v>
       </c>
       <c r="G6" t="n">
-        <v>0.255848183363899</v>
+        <v>0.2407733338594317</v>
       </c>
       <c r="H6" t="n">
-        <v>0.2432685221616387</v>
+        <v>0.2144768851659781</v>
       </c>
       <c r="I6" t="n">
-        <v>82.3102823102823</v>
+        <v>70.17584451642759</v>
       </c>
       <c r="J6" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K6" t="n">
         <v>51.57</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M6" t="n">
         <v>51.57</v>
       </c>
       <c r="N6" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O6" t="n">
         <v>82.97872340425532</v>
       </c>
       <c r="P6" t="n">
-        <v>61.22374468085107</v>
+        <v>65.22374468085107</v>
       </c>
       <c r="Q6" t="b">
         <v>0</v>
@@ -1104,48 +1104,48 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>3024.4</v>
+        <v>2968.7</v>
       </c>
       <c r="D7" t="n">
-        <v>0.177450751382076</v>
+        <v>0.106732776617954</v>
       </c>
       <c r="E7" t="n">
-        <v>0.3306348717497469</v>
+        <v>0.3376137694872487</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.0356174866872867</v>
+        <v>-0.07758513547104159</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.0149807029671487</v>
+        <v>-0.0440726544736921</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.0275603641694089</v>
+        <v>-0.0703691031671457</v>
       </c>
       <c r="I7" t="n">
-        <v>93.96037699557606</v>
+        <v>78.16880841121491</v>
       </c>
       <c r="J7" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K7" t="n">
         <v>48.73</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M7" t="n">
         <v>48.73</v>
       </c>
       <c r="N7" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O7" t="n">
-        <v>51.06382978723404</v>
+        <v>44.68085106382978</v>
       </c>
       <c r="P7" t="n">
-        <v>53.70476595744681</v>
+        <v>56.42817021276596</v>
       </c>
       <c r="Q7" t="b">
         <v>0</v>
@@ -1169,48 +1169,48 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>588.45</v>
+        <v>564.85</v>
       </c>
       <c r="D8" t="n">
-        <v>0.189508793208005</v>
+        <v>0.1044090331410696</v>
       </c>
       <c r="E8" t="n">
-        <v>0.3239959500506244</v>
+        <v>0.2384345538259153</v>
       </c>
       <c r="F8" t="n">
-        <v>0.4020729092208721</v>
+        <v>0.3642072213500784</v>
       </c>
       <c r="G8" t="n">
-        <v>0.4227096929410101</v>
+        <v>0.3977197023474279</v>
       </c>
       <c r="H8" t="n">
-        <v>0.4101300317387498</v>
+        <v>0.3714232536539743</v>
       </c>
       <c r="I8" t="n">
-        <v>79.17460317460311</v>
+        <v>66.4784546805349</v>
       </c>
       <c r="J8" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K8" t="n">
         <v>49.66</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M8" t="n">
         <v>49.66</v>
       </c>
       <c r="N8" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O8" t="n">
-        <v>93.61702127659576</v>
+        <v>91.48936170212764</v>
       </c>
       <c r="P8" t="n">
-        <v>66.58740425531916</v>
+        <v>70.16187234042553</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
@@ -1234,48 +1234,48 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>434</v>
+        <v>423.85</v>
       </c>
       <c r="D9" t="n">
-        <v>0.0723993081294787</v>
+        <v>0.0100083402835697</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.1354581673306772</v>
+        <v>-0.1509415064102564</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.0827433160731269</v>
+        <v>-0.1142110762800417</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.0621065323529889</v>
+        <v>-0.0806985952826923</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.07468619355524909</v>
+        <v>-0.1069950439761459</v>
       </c>
       <c r="I9" t="n">
-        <v>69.07536907536905</v>
+        <v>58.8637919233402</v>
       </c>
       <c r="J9" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="K9" t="n">
         <v>53.44</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M9" t="n">
         <v>53.44</v>
       </c>
       <c r="N9" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="O9" t="n">
-        <v>40.42553191489361</v>
+        <v>38.29787234042553</v>
       </c>
       <c r="P9" t="n">
-        <v>53.46110638297873</v>
+        <v>45.03557446808512</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -1299,48 +1299,48 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>137040</v>
+        <v>132145</v>
       </c>
       <c r="D10" t="n">
-        <v>0.073602569626699</v>
+        <v>0.0167346310687082</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.0214923241699392</v>
+        <v>-0.0387706855791961</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.1054538333496524</v>
+        <v>-0.1403525891230809</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.0848170496295144</v>
+        <v>-0.1068401081257314</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.0973967108317747</v>
+        <v>-0.133136556819185</v>
       </c>
       <c r="I10" t="n">
-        <v>74.27073837739289</v>
+        <v>59.74025974025973</v>
       </c>
       <c r="J10" t="n">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="K10" t="n">
         <v>49.41</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M10" t="n">
         <v>49.41</v>
       </c>
       <c r="N10" t="n">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="O10" t="n">
-        <v>31.91489361702128</v>
+        <v>34.04255319148936</v>
       </c>
       <c r="P10" t="n">
-        <v>54.14697872340425</v>
+        <v>42.57251063829787</v>
       </c>
       <c r="Q10" t="b">
         <v>0</v>
@@ -1376,10 +1376,10 @@
         <v>-0.0042030657656173</v>
       </c>
       <c r="G11" t="n">
-        <v>0.0164337179545206</v>
+        <v>0.0293094152317321</v>
       </c>
       <c r="H11" t="n">
-        <v>0.0038540567522603</v>
+        <v>0.0030129665382785</v>
       </c>
       <c r="I11" t="n">
         <v>27.6054590570719</v>
@@ -1392,7 +1392,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M11" t="n">
@@ -1402,10 +1402,10 @@
         <v>20</v>
       </c>
       <c r="O11" t="n">
-        <v>59.57446808510638</v>
+        <v>61.70212765957447</v>
       </c>
       <c r="P11" t="n">
-        <v>23.91489361702128</v>
+        <v>24.3404255319149</v>
       </c>
       <c r="Q11" t="b">
         <v>0</v>
@@ -1429,48 +1429,48 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>442.8</v>
+        <v>428.65</v>
       </c>
       <c r="D12" t="n">
-        <v>0.0662171923910426</v>
+        <v>-0.0348981200045029</v>
       </c>
       <c r="E12" t="n">
-        <v>0.0273781902552203</v>
+        <v>0.0077583166803807</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.1520490233626963</v>
+        <v>-0.1658883051177272</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.1314122396425583</v>
+        <v>-0.1323758241203777</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.1439919008448186</v>
+        <v>-0.1586722728138313</v>
       </c>
       <c r="I12" t="n">
-        <v>58.70165745856355</v>
+        <v>43.95036194415717</v>
       </c>
       <c r="J12" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K12" t="n">
         <v>71.28</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M12" t="n">
         <v>71.28</v>
       </c>
       <c r="N12" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O12" t="n">
-        <v>23.40425531914894</v>
+        <v>29.78723404255319</v>
       </c>
       <c r="P12" t="n">
-        <v>65.19285106382979</v>
+        <v>58.46944680851064</v>
       </c>
       <c r="Q12" t="b">
         <v>1</v>
@@ -1494,25 +1494,25 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1798.8</v>
+        <v>1796.3</v>
       </c>
       <c r="D13" t="n">
-        <v>0.1385530729793023</v>
+        <v>0.0884028114396509</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.0426822778073443</v>
+        <v>-0.0737379466817924</v>
       </c>
       <c r="F13" t="n">
-        <v>0.0161563665122583</v>
+        <v>0.0287497852356681</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0367931502323963</v>
+        <v>0.0622622662330176</v>
       </c>
       <c r="H13" t="n">
-        <v>0.024213489030136</v>
+        <v>0.035965817539564</v>
       </c>
       <c r="I13" t="n">
-        <v>65.44328985186823</v>
+        <v>63.5140728476821</v>
       </c>
       <c r="J13" t="n">
         <v>60</v>
@@ -1522,7 +1522,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M13" t="n">
@@ -1532,10 +1532,10 @@
         <v>60</v>
       </c>
       <c r="O13" t="n">
-        <v>63.82978723404256</v>
+        <v>65.95744680851064</v>
       </c>
       <c r="P13" t="n">
-        <v>60.27395744680852</v>
+        <v>60.69948936170213</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
@@ -1559,48 +1559,48 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>624.25</v>
+        <v>606.8</v>
       </c>
       <c r="D14" t="n">
-        <v>0.1324263038548752</v>
+        <v>0.08212215782434221</v>
       </c>
       <c r="E14" t="n">
-        <v>0.0916324210894465</v>
+        <v>0.1049804242920877</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.2638127248068872</v>
+        <v>-0.2373531075221517</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.2431759410867492</v>
+        <v>-0.2038406265248022</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.2557556022890095</v>
+        <v>-0.2301370752182558</v>
       </c>
       <c r="I14" t="n">
-        <v>81.04535896665664</v>
+        <v>71.51162790697671</v>
       </c>
       <c r="J14" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K14" t="n">
         <v>54.64</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M14" t="n">
         <v>54.64</v>
       </c>
       <c r="N14" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O14" t="n">
-        <v>4.25531914893617</v>
+        <v>8.51063829787234</v>
       </c>
       <c r="P14" t="n">
-        <v>46.70706382978724</v>
+        <v>51.55812765957447</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
@@ -1624,48 +1624,48 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>109.42</v>
+        <v>108.47</v>
       </c>
       <c r="D15" t="n">
-        <v>0.1661515506767559</v>
+        <v>0.1333194023612998</v>
       </c>
       <c r="E15" t="n">
-        <v>0.0081076100976598</v>
+        <v>-0.0090443997807417</v>
       </c>
       <c r="F15" t="n">
-        <v>0.1556822982678496</v>
+        <v>0.132372899050005</v>
       </c>
       <c r="G15" t="n">
-        <v>0.1763190819879876</v>
+        <v>0.1658853800473545</v>
       </c>
       <c r="H15" t="n">
-        <v>0.1637394207857273</v>
+        <v>0.1395889313539009</v>
       </c>
       <c r="I15" t="n">
-        <v>81.86015831134566</v>
+        <v>76.72320461927102</v>
       </c>
       <c r="J15" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K15" t="n">
         <v>51.91</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M15" t="n">
         <v>51.91</v>
       </c>
       <c r="N15" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O15" t="n">
         <v>74.46808510638297</v>
       </c>
       <c r="P15" t="n">
-        <v>59.65761702127659</v>
+        <v>63.65761702127659</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
@@ -1689,48 +1689,48 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>178.01</v>
+        <v>171.18</v>
       </c>
       <c r="D16" t="n">
-        <v>0.1443908711025392</v>
+        <v>0.0783671412372433</v>
       </c>
       <c r="E16" t="n">
-        <v>0.2406607192640089</v>
+        <v>0.2236757452283939</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.0899284253578732</v>
+        <v>-0.206176961602671</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.0692916416377352</v>
+        <v>-0.1726644806053215</v>
       </c>
       <c r="H16" t="n">
-        <v>-0.0818713028399955</v>
+        <v>-0.1989609292987751</v>
       </c>
       <c r="I16" t="n">
-        <v>76.13307618129213</v>
+        <v>63.31140350877192</v>
       </c>
       <c r="J16" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="K16" t="n">
         <v>52.61</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M16" t="n">
         <v>52.61</v>
       </c>
       <c r="N16" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="O16" t="n">
-        <v>38.29787234042553</v>
+        <v>17.02127659574468</v>
       </c>
       <c r="P16" t="n">
-        <v>56.70357446808511</v>
+        <v>48.44825531914893</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>
@@ -1754,48 +1754,48 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>7684.5</v>
+        <v>7570</v>
       </c>
       <c r="D17" t="n">
-        <v>0.122972380534853</v>
+        <v>0.0739111930770322</v>
       </c>
       <c r="E17" t="n">
-        <v>0.0394994927291174</v>
+        <v>0.0516079738834478</v>
       </c>
       <c r="F17" t="n">
-        <v>0.1344947220786889</v>
+        <v>0.1321319075749645</v>
       </c>
       <c r="G17" t="n">
-        <v>0.1551315057988269</v>
+        <v>0.165644388572314</v>
       </c>
       <c r="H17" t="n">
-        <v>0.1425518445965666</v>
+        <v>0.1393479398788604</v>
       </c>
       <c r="I17" t="n">
-        <v>87.80075981426762</v>
+        <v>77.69582016157359</v>
       </c>
       <c r="J17" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K17" t="n">
         <v>54.65</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M17" t="n">
         <v>54.65</v>
       </c>
       <c r="N17" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O17" t="n">
         <v>72.3404255319149</v>
       </c>
       <c r="P17" t="n">
-        <v>60.32808510638298</v>
+        <v>64.32808510638299</v>
       </c>
       <c r="Q17" t="b">
         <v>0</v>
@@ -1819,25 +1819,25 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>733.8</v>
+        <v>752.5</v>
       </c>
       <c r="D18" t="n">
-        <v>0.0526466790991249</v>
+        <v>0.07862108507131089</v>
       </c>
       <c r="E18" t="n">
-        <v>0.253608951909114</v>
+        <v>0.2626898229717258</v>
       </c>
       <c r="F18" t="n">
-        <v>0.0866281652598845</v>
+        <v>0.1508755830848054</v>
       </c>
       <c r="G18" t="n">
-        <v>0.1072649489800225</v>
+        <v>0.1843880640821549</v>
       </c>
       <c r="H18" t="n">
-        <v>0.09468528777776231</v>
+        <v>0.1580916153887013</v>
       </c>
       <c r="I18" t="n">
-        <v>73.33177788147458</v>
+        <v>73.06209850107068</v>
       </c>
       <c r="J18" t="n">
         <v>70</v>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M18" t="n">
@@ -1857,10 +1857,10 @@
         <v>70</v>
       </c>
       <c r="O18" t="n">
-        <v>68.08510638297872</v>
+        <v>78.72340425531915</v>
       </c>
       <c r="P18" t="n">
-        <v>61.58502127659575</v>
+        <v>63.71268085106384</v>
       </c>
       <c r="Q18" t="b">
         <v>0</v>
@@ -1884,48 +1884,48 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2399.1</v>
+        <v>2318.6</v>
       </c>
       <c r="D19" t="n">
-        <v>0.07073998036240289</v>
+        <v>-0.0062149072050061</v>
       </c>
       <c r="E19" t="n">
-        <v>-0.0155519080837095</v>
+        <v>-0.0162918964785745</v>
       </c>
       <c r="F19" t="n">
-        <v>-0.1708370774866939</v>
+        <v>-0.2143002372077261</v>
       </c>
       <c r="G19" t="n">
-        <v>-0.1502002937665559</v>
+        <v>-0.1807877562103766</v>
       </c>
       <c r="H19" t="n">
-        <v>-0.1627799549688162</v>
+        <v>-0.2070842049038302</v>
       </c>
       <c r="I19" t="n">
-        <v>66.72727272727266</v>
+        <v>62.4946785866326</v>
       </c>
       <c r="J19" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="K19" t="n">
         <v>51.27</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M19" t="n">
         <v>51.27</v>
       </c>
       <c r="N19" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="O19" t="n">
-        <v>21.27659574468085</v>
+        <v>14.8936170212766</v>
       </c>
       <c r="P19" t="n">
-        <v>48.76331914893618</v>
+        <v>39.48672340425532</v>
       </c>
       <c r="Q19" t="b">
         <v>0</v>
@@ -1949,48 +1949,48 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2275.2</v>
+        <v>2175</v>
       </c>
       <c r="D20" t="n">
-        <v>0.1311524311424876</v>
+        <v>0.0438663851027067</v>
       </c>
       <c r="E20" t="n">
-        <v>0.0429999083157603</v>
+        <v>0.0137024608501119</v>
       </c>
       <c r="F20" t="n">
-        <v>0.1746605400382053</v>
+        <v>0.1344669309409556</v>
       </c>
       <c r="G20" t="n">
-        <v>0.1952973237583433</v>
+        <v>0.1679794119383051</v>
       </c>
       <c r="H20" t="n">
-        <v>0.182717662556083</v>
+        <v>0.1416829632448515</v>
       </c>
       <c r="I20" t="n">
-        <v>83.51445086705199</v>
+        <v>65.25526742301457</v>
       </c>
       <c r="J20" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K20" t="n">
         <v>49.06</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M20" t="n">
         <v>49.06</v>
       </c>
       <c r="N20" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O20" t="n">
-        <v>78.72340425531915</v>
+        <v>76.59574468085107</v>
       </c>
       <c r="P20" t="n">
-        <v>59.36868085106384</v>
+        <v>66.94314893617022</v>
       </c>
       <c r="Q20" t="b">
         <v>0</v>
@@ -2014,48 +2014,48 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1031.85</v>
+        <v>973</v>
       </c>
       <c r="D21" t="n">
-        <v>0.1998255813953486</v>
+        <v>0.1041134751773049</v>
       </c>
       <c r="E21" t="n">
-        <v>0.1558754340763972</v>
+        <v>0.0802709004107915</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.1999922468599783</v>
+        <v>-0.2584971803078799</v>
       </c>
       <c r="G21" t="n">
-        <v>-0.1793554631398403</v>
+        <v>-0.2249846993105304</v>
       </c>
       <c r="H21" t="n">
-        <v>-0.1919351243421005</v>
+        <v>-0.251281148003984</v>
       </c>
       <c r="I21" t="n">
-        <v>89.97681010048954</v>
+        <v>67.53058262492225</v>
       </c>
       <c r="J21" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K21" t="n">
         <v>48.43</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M21" t="n">
         <v>48.43</v>
       </c>
       <c r="N21" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O21" t="n">
-        <v>12.76595744680851</v>
+        <v>4.25531914893617</v>
       </c>
       <c r="P21" t="n">
-        <v>45.9251914893617</v>
+        <v>52.22306382978724</v>
       </c>
       <c r="Q21" t="b">
         <v>0</v>
@@ -2079,48 +2079,48 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>457.2</v>
+        <v>429.3</v>
       </c>
       <c r="D22" t="n">
-        <v>0.2295280354981845</v>
+        <v>0.08368042408178721</v>
       </c>
       <c r="E22" t="n">
-        <v>0.3678384442782347</v>
+        <v>0.2528819495111631</v>
       </c>
       <c r="F22" t="n">
-        <v>0.4595371109337589</v>
+        <v>0.3866279069767442</v>
       </c>
       <c r="G22" t="n">
-        <v>0.4801738946538969</v>
+        <v>0.4201403879740937</v>
       </c>
       <c r="H22" t="n">
-        <v>0.4675942334516366</v>
+        <v>0.3938439392806401</v>
       </c>
       <c r="I22" t="n">
-        <v>88.76353790613715</v>
+        <v>68.63583365720947</v>
       </c>
       <c r="J22" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K22" t="n">
         <v>54.47</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M22" t="n">
         <v>54.47</v>
       </c>
       <c r="N22" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O22" t="n">
         <v>95.74468085106383</v>
       </c>
       <c r="P22" t="n">
-        <v>64.93693617021276</v>
+        <v>72.93693617021276</v>
       </c>
       <c r="Q22" t="b">
         <v>0</v>
@@ -2144,48 +2144,48 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>394.15</v>
+        <v>381.6</v>
       </c>
       <c r="D23" t="n">
-        <v>0.1831007053879634</v>
+        <v>0.1385946591078624</v>
       </c>
       <c r="E23" t="n">
-        <v>0.0744173367861522</v>
+        <v>0.026634382566586</v>
       </c>
       <c r="F23" t="n">
-        <v>-0.0111640742599098</v>
+        <v>-0.0296249205340113</v>
       </c>
       <c r="G23" t="n">
-        <v>0.0094727094602281</v>
+        <v>0.0038875604633381</v>
       </c>
       <c r="H23" t="n">
-        <v>-0.0031069517420321</v>
+        <v>-0.0224088882301154</v>
       </c>
       <c r="I23" t="n">
-        <v>80.36072144288575</v>
+        <v>72.35002255299956</v>
       </c>
       <c r="J23" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K23" t="n">
         <v>49.7</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M23" t="n">
         <v>49.7</v>
       </c>
       <c r="N23" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O23" t="n">
         <v>57.44680851063831</v>
       </c>
       <c r="P23" t="n">
-        <v>55.36936170212766</v>
+        <v>59.36936170212766</v>
       </c>
       <c r="Q23" t="b">
         <v>0</v>
@@ -2209,25 +2209,25 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>126.29</v>
+        <v>122.99</v>
       </c>
       <c r="D24" t="n">
-        <v>0.0720713073005094</v>
+        <v>0.0125133777887544</v>
       </c>
       <c r="E24" t="n">
-        <v>0.0860853113175095</v>
+        <v>0.0563428669586876</v>
       </c>
       <c r="F24" t="n">
-        <v>0.2444816712652739</v>
+        <v>0.2539763458401305</v>
       </c>
       <c r="G24" t="n">
-        <v>0.265118454985412</v>
+        <v>0.28748882683748</v>
       </c>
       <c r="H24" t="n">
-        <v>0.2525387937831517</v>
+        <v>0.2611923781440264</v>
       </c>
       <c r="I24" t="n">
-        <v>69.90291262135922</v>
+        <v>61.40412155082081</v>
       </c>
       <c r="J24" t="n">
         <v>60</v>
@@ -2237,7 +2237,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M24" t="n">
@@ -2274,48 +2274,48 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>628.95</v>
+        <v>612.85</v>
       </c>
       <c r="D25" t="n">
-        <v>0.09917860887801461</v>
+        <v>0.0701999476119794</v>
       </c>
       <c r="E25" t="n">
-        <v>0.1385771180304129</v>
+        <v>0.1585066162570889</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.0788664323374339</v>
+        <v>-0.08386277001270639</v>
       </c>
       <c r="G25" t="n">
-        <v>-0.0582296486172959</v>
+        <v>-0.0503502890153569</v>
       </c>
       <c r="H25" t="n">
-        <v>-0.0708093098195562</v>
+        <v>-0.0766467377088105</v>
       </c>
       <c r="I25" t="n">
-        <v>85.33893851812924</v>
+        <v>73.61740707162284</v>
       </c>
       <c r="J25" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K25" t="n">
         <v>56.91</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M25" t="n">
         <v>56.91</v>
       </c>
       <c r="N25" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O25" t="n">
-        <v>44.68085106382978</v>
+        <v>42.5531914893617</v>
       </c>
       <c r="P25" t="n">
-        <v>55.70017021276595</v>
+        <v>59.27463829787234</v>
       </c>
       <c r="Q25" t="b">
         <v>0</v>
@@ -2339,48 +2339,48 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>130.04</v>
+        <v>128.99</v>
       </c>
       <c r="D26" t="n">
-        <v>0.0509981411137152</v>
+        <v>0.0250317863954228</v>
       </c>
       <c r="E26" t="n">
-        <v>-0.0285372777528762</v>
+        <v>-0.0130078812456958</v>
       </c>
       <c r="F26" t="n">
-        <v>-0.2105390966488587</v>
+        <v>-0.1955721858434673</v>
       </c>
       <c r="G26" t="n">
-        <v>-0.1899023129287207</v>
+        <v>-0.1620597048461178</v>
       </c>
       <c r="H26" t="n">
-        <v>-0.202481974130981</v>
+        <v>-0.1883561535395714</v>
       </c>
       <c r="I26" t="n">
-        <v>56.70675300647543</v>
+        <v>56.46532438478747</v>
       </c>
       <c r="J26" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="K26" t="n">
         <v>51.54</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M26" t="n">
         <v>51.54</v>
       </c>
       <c r="N26" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="O26" t="n">
-        <v>10.63829787234042</v>
+        <v>21.27659574468085</v>
       </c>
       <c r="P26" t="n">
-        <v>46.74365957446808</v>
+        <v>40.87131914893617</v>
       </c>
       <c r="Q26" t="b">
         <v>0</v>
@@ -2404,48 +2404,48 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>5315.9</v>
+        <v>5173.6</v>
       </c>
       <c r="D27" t="n">
-        <v>0.0577852949955226</v>
+        <v>0.0048752063707877</v>
       </c>
       <c r="E27" t="n">
-        <v>0.1093280467445743</v>
+        <v>0.117046313289431</v>
       </c>
       <c r="F27" t="n">
-        <v>0.0018658122879757</v>
+        <v>0.0109623839765511</v>
       </c>
       <c r="G27" t="n">
-        <v>0.0225025960081137</v>
+        <v>0.0444748649739006</v>
       </c>
       <c r="H27" t="n">
-        <v>0.009922934805853399</v>
+        <v>0.018178416280447</v>
       </c>
       <c r="I27" t="n">
-        <v>67.66251912968258</v>
+        <v>60.08005591206557</v>
       </c>
       <c r="J27" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="K27" t="n">
         <v>57.69</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M27" t="n">
         <v>57.69</v>
       </c>
       <c r="N27" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="O27" t="n">
-        <v>61.70212765957447</v>
+        <v>63.82978723404256</v>
       </c>
       <c r="P27" t="n">
-        <v>59.4164255319149</v>
+        <v>51.84195744680851</v>
       </c>
       <c r="Q27" t="b">
         <v>0</v>
@@ -2469,48 +2469,48 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1794.4</v>
+        <v>1727</v>
       </c>
       <c r="D28" t="n">
-        <v>0.1416210713831276</v>
+        <v>0.0638822152405593</v>
       </c>
       <c r="E28" t="n">
-        <v>0.2868617326448652</v>
+        <v>0.2536295005807201</v>
       </c>
       <c r="F28" t="n">
-        <v>0.3775525871334255</v>
+        <v>0.3721595423486414</v>
       </c>
       <c r="G28" t="n">
-        <v>0.3981893708535635</v>
+        <v>0.4056720233459909</v>
       </c>
       <c r="H28" t="n">
-        <v>0.3856097096513032</v>
+        <v>0.3793755746525373</v>
       </c>
       <c r="I28" t="n">
-        <v>71.40147023950676</v>
+        <v>57.3502722323049</v>
       </c>
       <c r="J28" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K28" t="n">
         <v>54.51</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M28" t="n">
         <v>54.51</v>
       </c>
       <c r="N28" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O28" t="n">
-        <v>91.48936170212764</v>
+        <v>93.61702127659576</v>
       </c>
       <c r="P28" t="n">
-        <v>68.10187234042553</v>
+        <v>72.52740425531915</v>
       </c>
       <c r="Q28" t="b">
         <v>0</v>
@@ -2534,48 +2534,48 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>541.45</v>
+        <v>527.6</v>
       </c>
       <c r="D29" t="n">
-        <v>0.039052005373249</v>
+        <v>-0.0300579097343506</v>
       </c>
       <c r="E29" t="n">
-        <v>0.0332029386508923</v>
+        <v>-0.0281819856327131</v>
       </c>
       <c r="F29" t="n">
-        <v>-0.0796362400135983</v>
+        <v>-0.1123075628838227</v>
       </c>
       <c r="G29" t="n">
-        <v>-0.0589994562934603</v>
+        <v>-0.0787950818864732</v>
       </c>
       <c r="H29" t="n">
-        <v>-0.0715791174957206</v>
+        <v>-0.1050915305799268</v>
       </c>
       <c r="I29" t="n">
-        <v>66.76433654248643</v>
+        <v>57.33067729083667</v>
       </c>
       <c r="J29" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K29" t="n">
         <v>49.42</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M29" t="n">
         <v>49.42</v>
       </c>
       <c r="N29" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O29" t="n">
-        <v>42.5531914893617</v>
+        <v>40.42553191489361</v>
       </c>
       <c r="P29" t="n">
-        <v>60.27863829787234</v>
+        <v>51.85310638297872</v>
       </c>
       <c r="Q29" t="b">
         <v>0</v>
@@ -2599,48 +2599,48 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>125.79</v>
+        <v>118.74</v>
       </c>
       <c r="D30" t="n">
-        <v>0.1217228464419475</v>
+        <v>0.0607468286582097</v>
       </c>
       <c r="E30" t="n">
-        <v>0.0151723024776047</v>
+        <v>-0.0266415279940979</v>
       </c>
       <c r="F30" t="n">
-        <v>-0.0284986098239109</v>
+        <v>-0.052051732396615</v>
       </c>
       <c r="G30" t="n">
-        <v>-0.007861826103772901</v>
+        <v>-0.0185392513992656</v>
       </c>
       <c r="H30" t="n">
-        <v>-0.0204414873060332</v>
+        <v>-0.0448357000927192</v>
       </c>
       <c r="I30" t="n">
-        <v>79.00776240296997</v>
+        <v>61.84588844163311</v>
       </c>
       <c r="J30" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K30" t="n">
         <v>52.38</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M30" t="n">
         <v>52.38</v>
       </c>
       <c r="N30" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O30" t="n">
         <v>53.19148936170212</v>
       </c>
       <c r="P30" t="n">
-        <v>59.59029787234042</v>
+        <v>63.59029787234042</v>
       </c>
       <c r="Q30" t="b">
         <v>0</v>
@@ -2664,48 +2664,48 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>41.29</v>
+        <v>39.9</v>
       </c>
       <c r="D31" t="n">
-        <v>0.100773127166089</v>
+        <v>0.0505529225908374</v>
       </c>
       <c r="E31" t="n">
-        <v>-0.0719262755675432</v>
+        <v>-0.07166123778501619</v>
       </c>
       <c r="F31" t="n">
-        <v>-0.0972890249234805</v>
+        <v>-0.1397153945666236</v>
       </c>
       <c r="G31" t="n">
-        <v>-0.07665224120334251</v>
+        <v>-0.1062029135692741</v>
       </c>
       <c r="H31" t="n">
-        <v>-0.0892319024056028</v>
+        <v>-0.1324993622627277</v>
       </c>
       <c r="I31" t="n">
-        <v>78.28418230563</v>
+        <v>68.38407494145198</v>
       </c>
       <c r="J31" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K31" t="n">
         <v>48.99</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M31" t="n">
         <v>48.99</v>
       </c>
       <c r="N31" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O31" t="n">
-        <v>34.04255319148936</v>
+        <v>36.17021276595745</v>
       </c>
       <c r="P31" t="n">
-        <v>54.40451063829788</v>
+        <v>58.8300425531915</v>
       </c>
       <c r="Q31" t="b">
         <v>0</v>
@@ -2729,48 +2729,48 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>763.95</v>
+        <v>723.25</v>
       </c>
       <c r="D32" t="n">
-        <v>0.1447516295796809</v>
+        <v>0.0534556842181925</v>
       </c>
       <c r="E32" t="n">
-        <v>0.1227129105738848</v>
+        <v>0.0729120308559561</v>
       </c>
       <c r="F32" t="n">
-        <v>-0.2652914021927293</v>
+        <v>-0.30215167888846</v>
       </c>
       <c r="G32" t="n">
-        <v>-0.2446546184725913</v>
+        <v>-0.2686391978911105</v>
       </c>
       <c r="H32" t="n">
-        <v>-0.2572342796748516</v>
+        <v>-0.2949356465845641</v>
       </c>
       <c r="I32" t="n">
-        <v>89.94263862332699</v>
+        <v>67.32402912621359</v>
       </c>
       <c r="J32" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K32" t="n">
         <v>47.86</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M32" t="n">
         <v>47.86</v>
       </c>
       <c r="N32" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O32" t="n">
         <v>2.127659574468085</v>
       </c>
       <c r="P32" t="n">
-        <v>43.56953191489362</v>
+        <v>51.56953191489362</v>
       </c>
       <c r="Q32" t="b">
         <v>0</v>
@@ -2794,48 +2794,48 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>612.35</v>
+        <v>594.65</v>
       </c>
       <c r="D33" t="n">
-        <v>0.1551594038860593</v>
+        <v>0.09320709624046319</v>
       </c>
       <c r="E33" t="n">
-        <v>0.06811442525728249</v>
+        <v>0.0226139294926912</v>
       </c>
       <c r="F33" t="n">
-        <v>0.1590952110543253</v>
+        <v>0.1291180100636095</v>
       </c>
       <c r="G33" t="n">
-        <v>0.1797319947744633</v>
+        <v>0.162630491060959</v>
       </c>
       <c r="H33" t="n">
-        <v>0.167152333572203</v>
+        <v>0.1363340423675054</v>
       </c>
       <c r="I33" t="n">
-        <v>89.7398843930636</v>
+        <v>73.09605817068504</v>
       </c>
       <c r="J33" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K33" t="n">
         <v>49.98</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M33" t="n">
         <v>49.98</v>
       </c>
       <c r="N33" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O33" t="n">
-        <v>76.59574468085107</v>
+        <v>70.21276595744681</v>
       </c>
       <c r="P33" t="n">
-        <v>59.31114893617022</v>
+        <v>62.03455319148937</v>
       </c>
       <c r="Q33" t="b">
         <v>0</v>
@@ -2871,10 +2871,10 @@
         <v>-0.2401052253975846</v>
       </c>
       <c r="G34" t="n">
-        <v>-0.2194684416774466</v>
+        <v>-0.2065927444002351</v>
       </c>
       <c r="H34" t="n">
-        <v>-0.2320481028797069</v>
+        <v>-0.2328891930936887</v>
       </c>
       <c r="I34" t="n">
         <v>63.3225806451613</v>
@@ -2887,7 +2887,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M34" t="n">
@@ -2897,10 +2897,10 @@
         <v>80</v>
       </c>
       <c r="O34" t="n">
-        <v>8.51063829787234</v>
+        <v>6.382978723404255</v>
       </c>
       <c r="P34" t="n">
-        <v>54.05412765957447</v>
+        <v>53.62859574468086</v>
       </c>
       <c r="Q34" t="b">
         <v>0</v>
@@ -2924,48 +2924,48 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>118.41</v>
+        <v>113.72</v>
       </c>
       <c r="D35" t="n">
-        <v>0.09073323507737641</v>
+        <v>0.0419644493311344</v>
       </c>
       <c r="E35" t="n">
-        <v>0.0228921907394608</v>
+        <v>-0.0166882836143537</v>
       </c>
       <c r="F35" t="n">
-        <v>0.2669591268992082</v>
+        <v>0.2714669051878353</v>
       </c>
       <c r="G35" t="n">
-        <v>0.2875959106193462</v>
+        <v>0.3049793861851848</v>
       </c>
       <c r="H35" t="n">
-        <v>0.2750162494170859</v>
+        <v>0.2786829374917312</v>
       </c>
       <c r="I35" t="n">
-        <v>70.46610169491525</v>
+        <v>56.86274509803921</v>
       </c>
       <c r="J35" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="K35" t="n">
         <v>49.07</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M35" t="n">
         <v>49.07</v>
       </c>
       <c r="N35" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="O35" t="n">
         <v>87.2340425531915</v>
       </c>
       <c r="P35" t="n">
-        <v>65.07480851063831</v>
+        <v>61.07480851063831</v>
       </c>
       <c r="Q35" t="b">
         <v>0</v>
@@ -2989,48 +2989,48 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>486.85</v>
+        <v>471.25</v>
       </c>
       <c r="D36" t="n">
-        <v>0.0642693190512624</v>
+        <v>0.0134408602150537</v>
       </c>
       <c r="E36" t="n">
-        <v>-0.0438923802042419</v>
+        <v>-0.049132364810331</v>
       </c>
       <c r="F36" t="n">
-        <v>0.06929497034922021</v>
+        <v>-0.0043312909359813</v>
       </c>
       <c r="G36" t="n">
-        <v>0.0899317540693582</v>
+        <v>0.0291811900613681</v>
       </c>
       <c r="H36" t="n">
-        <v>0.0773520928670979</v>
+        <v>0.0028847413679145</v>
       </c>
       <c r="I36" t="n">
-        <v>64.98237367802585</v>
+        <v>52.03380876914951</v>
       </c>
       <c r="J36" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="K36" t="n">
         <v>47.8</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M36" t="n">
         <v>47.8</v>
       </c>
       <c r="N36" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="O36" t="n">
-        <v>65.95744680851064</v>
+        <v>59.57446808510638</v>
       </c>
       <c r="P36" t="n">
-        <v>64.31148936170213</v>
+        <v>47.03489361702128</v>
       </c>
       <c r="Q36" t="b">
         <v>0</v>
@@ -3054,48 +3054,48 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2547</v>
+        <v>2530.7</v>
       </c>
       <c r="D37" t="n">
-        <v>0.2037430880476392</v>
+        <v>0.1592762253779203</v>
       </c>
       <c r="E37" t="n">
-        <v>0.4817615917156319</v>
+        <v>0.5236002408187836</v>
       </c>
       <c r="F37" t="n">
-        <v>0.8181169248340352</v>
+        <v>0.741227466629971</v>
       </c>
       <c r="G37" t="n">
-        <v>0.8387537085541732</v>
+        <v>0.7747399476273205</v>
       </c>
       <c r="H37" t="n">
-        <v>0.8261740473519129</v>
+        <v>0.7484434989338669</v>
       </c>
       <c r="I37" t="n">
-        <v>80.89430894308947</v>
+        <v>78.30092118730811</v>
       </c>
       <c r="J37" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K37" t="n">
         <v>48.59</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M37" t="n">
         <v>48.59</v>
       </c>
       <c r="N37" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O37" t="n">
         <v>100</v>
       </c>
       <c r="P37" t="n">
-        <v>63.43600000000001</v>
+        <v>67.43600000000001</v>
       </c>
       <c r="Q37" t="b">
         <v>0</v>
@@ -3119,48 +3119,48 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>880.2</v>
+        <v>845</v>
       </c>
       <c r="D38" t="n">
-        <v>0.1505882352941177</v>
+        <v>0.0626925737282273</v>
       </c>
       <c r="E38" t="n">
-        <v>0.044933816109693</v>
+        <v>0.0058925063984287</v>
       </c>
       <c r="F38" t="n">
-        <v>-0.1898757478140819</v>
+        <v>-0.2146110233293058</v>
       </c>
       <c r="G38" t="n">
-        <v>-0.1692389640939439</v>
+        <v>-0.1810985423319563</v>
       </c>
       <c r="H38" t="n">
-        <v>-0.1818186252962041</v>
+        <v>-0.2073949910254099</v>
       </c>
       <c r="I38" t="n">
-        <v>86.96767573114418</v>
+        <v>72.51077341800861</v>
       </c>
       <c r="J38" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K38" t="n">
         <v>49.87</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M38" t="n">
         <v>49.87</v>
       </c>
       <c r="N38" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O38" t="n">
-        <v>14.8936170212766</v>
+        <v>12.76595744680851</v>
       </c>
       <c r="P38" t="n">
-        <v>46.92672340425532</v>
+        <v>50.5011914893617</v>
       </c>
       <c r="Q38" t="b">
         <v>0</v>
@@ -3184,48 +3184,48 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>3591.6</v>
+        <v>3478.7</v>
       </c>
       <c r="D39" t="n">
-        <v>0.2035789685332261</v>
+        <v>0.1214016311530898</v>
       </c>
       <c r="E39" t="n">
-        <v>0.3066065192083818</v>
+        <v>0.2882642669333035</v>
       </c>
       <c r="F39" t="n">
-        <v>0.3140641006878384</v>
+        <v>0.2815723548482167</v>
       </c>
       <c r="G39" t="n">
-        <v>0.3347008844079764</v>
+        <v>0.3150848358455662</v>
       </c>
       <c r="H39" t="n">
-        <v>0.3221212232057161</v>
+        <v>0.2887883871521126</v>
       </c>
       <c r="I39" t="n">
-        <v>81.92144782441277</v>
+        <v>73.04347826086955</v>
       </c>
       <c r="J39" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K39" t="n">
         <v>48.69</v>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M39" t="n">
         <v>48.69</v>
       </c>
       <c r="N39" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O39" t="n">
         <v>89.36170212765957</v>
       </c>
       <c r="P39" t="n">
-        <v>61.34834042553192</v>
+        <v>65.34834042553192</v>
       </c>
       <c r="Q39" t="b">
         <v>0</v>
@@ -3249,48 +3249,48 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>216.28</v>
+        <v>207.89</v>
       </c>
       <c r="D40" t="n">
-        <v>0.1906413432424993</v>
+        <v>0.1187708535141534</v>
       </c>
       <c r="E40" t="n">
-        <v>0.1553418803418804</v>
+        <v>0.1576456175520657</v>
       </c>
       <c r="F40" t="n">
-        <v>-0.0579729082277102</v>
+        <v>-0.070134633448137</v>
       </c>
       <c r="G40" t="n">
-        <v>-0.0373361245075722</v>
+        <v>-0.0366221524507875</v>
       </c>
       <c r="H40" t="n">
-        <v>-0.0499157857098325</v>
+        <v>-0.0629186011442411</v>
       </c>
       <c r="I40" t="n">
-        <v>84.57405986185725</v>
+        <v>68.97590361445781</v>
       </c>
       <c r="J40" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K40" t="n">
         <v>45.44</v>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M40" t="n">
         <v>45.44</v>
       </c>
       <c r="N40" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O40" t="n">
         <v>48.93617021276596</v>
       </c>
       <c r="P40" t="n">
-        <v>51.9632340425532</v>
+        <v>59.9632340425532</v>
       </c>
       <c r="Q40" t="b">
         <v>0</v>
@@ -3314,25 +3314,25 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>835.9</v>
+        <v>801.55</v>
       </c>
       <c r="D41" t="n">
-        <v>0.0510499182698354</v>
+        <v>0.0031914893617019</v>
       </c>
       <c r="E41" t="n">
-        <v>-0.1016657710908114</v>
+        <v>-0.1196595277320153</v>
       </c>
       <c r="F41" t="n">
-        <v>-0.184925162108137</v>
+        <v>-0.2026758181637322</v>
       </c>
       <c r="G41" t="n">
-        <v>-0.164288378387999</v>
+        <v>-0.1691633371663827</v>
       </c>
       <c r="H41" t="n">
-        <v>-0.1768680395902593</v>
+        <v>-0.1954597858598363</v>
       </c>
       <c r="I41" t="n">
-        <v>80.3886925795053</v>
+        <v>61.06583072100312</v>
       </c>
       <c r="J41" t="n">
         <v>60</v>
@@ -3342,7 +3342,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M41" t="n">
@@ -3352,10 +3352,10 @@
         <v>60</v>
       </c>
       <c r="O41" t="n">
-        <v>17.02127659574468</v>
+        <v>19.14893617021277</v>
       </c>
       <c r="P41" t="n">
-        <v>46.62425531914894</v>
+        <v>47.04978723404256</v>
       </c>
       <c r="Q41" t="b">
         <v>0</v>
@@ -3379,48 +3379,48 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>625.45</v>
+        <v>617.55</v>
       </c>
       <c r="D42" t="n">
-        <v>0.1903130649919115</v>
+        <v>0.175054704595186</v>
       </c>
       <c r="E42" t="n">
-        <v>0.0407687827606289</v>
+        <v>0.0398215187742043</v>
       </c>
       <c r="F42" t="n">
-        <v>-0.1725757375314194</v>
+        <v>-0.1941671559992172</v>
       </c>
       <c r="G42" t="n">
-        <v>-0.1519389538112814</v>
+        <v>-0.1606546750018677</v>
       </c>
       <c r="H42" t="n">
-        <v>-0.1645186150135417</v>
+        <v>-0.1869511236953213</v>
       </c>
       <c r="I42" t="n">
-        <v>82.43174924165821</v>
+        <v>72.20066518847</v>
       </c>
       <c r="J42" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K42" t="n">
         <v>47.66</v>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M42" t="n">
         <v>47.66</v>
       </c>
       <c r="N42" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O42" t="n">
-        <v>19.14893617021277</v>
+        <v>23.40425531914894</v>
       </c>
       <c r="P42" t="n">
-        <v>46.89378723404256</v>
+        <v>51.74485106382978</v>
       </c>
       <c r="Q42" t="b">
         <v>0</v>
@@ -3444,48 +3444,48 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>428.7</v>
+        <v>417.25</v>
       </c>
       <c r="D43" t="n">
-        <v>0.06854436689930191</v>
+        <v>0.0165671823608235</v>
       </c>
       <c r="E43" t="n">
-        <v>-0.0054518037350655</v>
+        <v>0.0054216867469878</v>
       </c>
       <c r="F43" t="n">
-        <v>-0.09642744230161231</v>
+        <v>-0.0721592172559484</v>
       </c>
       <c r="G43" t="n">
-        <v>-0.0757906585814743</v>
+        <v>-0.0386467362585989</v>
       </c>
       <c r="H43" t="n">
-        <v>-0.08837031978373459</v>
+        <v>-0.06494318495205249</v>
       </c>
       <c r="I43" t="n">
-        <v>58.71886120996441</v>
+        <v>51.78323297823067</v>
       </c>
       <c r="J43" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="K43" t="n">
         <v>51.48</v>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M43" t="n">
         <v>51.48</v>
       </c>
       <c r="N43" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="O43" t="n">
-        <v>36.17021276595745</v>
+        <v>46.80851063829788</v>
       </c>
       <c r="P43" t="n">
-        <v>59.82604255319149</v>
+        <v>45.95370212765958</v>
       </c>
       <c r="Q43" t="b">
         <v>0</v>
@@ -3509,25 +3509,25 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>277.79</v>
+        <v>277.78</v>
       </c>
       <c r="D44" t="n">
-        <v>0.2398571747377818</v>
+        <v>0.1627459187944746</v>
       </c>
       <c r="E44" t="n">
-        <v>0.1084996009577017</v>
+        <v>0.1275827075299369</v>
       </c>
       <c r="F44" t="n">
-        <v>-0.06750587445451479</v>
+        <v>-0.0398202557898377</v>
       </c>
       <c r="G44" t="n">
-        <v>-0.0468690907343768</v>
+        <v>-0.0063077747924882</v>
       </c>
       <c r="H44" t="n">
-        <v>-0.0594487519366371</v>
+        <v>-0.0326042234859418</v>
       </c>
       <c r="I44" t="n">
-        <v>90.23003360041356</v>
+        <v>84.51015004413055</v>
       </c>
       <c r="J44" t="n">
         <v>60</v>
@@ -3537,7 +3537,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M44" t="n">
@@ -3547,10 +3547,10 @@
         <v>60</v>
       </c>
       <c r="O44" t="n">
-        <v>46.80851063829788</v>
+        <v>55.31914893617022</v>
       </c>
       <c r="P44" t="n">
-        <v>52.24170212765958</v>
+        <v>53.94382978723405</v>
       </c>
       <c r="Q44" t="b">
         <v>0</v>
@@ -3574,48 +3574,48 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>103.02</v>
+        <v>102.66</v>
       </c>
       <c r="D45" t="n">
-        <v>0.1098901098901099</v>
+        <v>0.1118812953536227</v>
       </c>
       <c r="E45" t="n">
-        <v>-0.1070468926063968</v>
+        <v>-0.06867458949469291</v>
       </c>
       <c r="F45" t="n">
-        <v>-0.2490706319702602</v>
+        <v>-0.2280622603203249</v>
       </c>
       <c r="G45" t="n">
-        <v>-0.2284338482501222</v>
+        <v>-0.1945497793229754</v>
       </c>
       <c r="H45" t="n">
-        <v>-0.2410135094523825</v>
+        <v>-0.220846228016429</v>
       </c>
       <c r="I45" t="n">
-        <v>81.56638013371538</v>
+        <v>73.73926036608142</v>
       </c>
       <c r="J45" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K45" t="n">
         <v>59.6</v>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M45" t="n">
         <v>59.6</v>
       </c>
       <c r="N45" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O45" t="n">
-        <v>6.382978723404255</v>
+        <v>10.63829787234042</v>
       </c>
       <c r="P45" t="n">
-        <v>49.11659574468086</v>
+        <v>53.96765957446809</v>
       </c>
       <c r="Q45" t="b">
         <v>0</v>
@@ -3639,48 +3639,48 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>533.8</v>
+        <v>512.25</v>
       </c>
       <c r="D46" t="n">
-        <v>0.0911692559280457</v>
+        <v>0.03820429671666</v>
       </c>
       <c r="E46" t="n">
-        <v>-0.0184793601176795</v>
+        <v>-0.0734376413131953</v>
       </c>
       <c r="F46" t="n">
-        <v>-0.1381982563771392</v>
+        <v>-0.1743230174081237</v>
       </c>
       <c r="G46" t="n">
-        <v>-0.1175614726570012</v>
+        <v>-0.1408105364107742</v>
       </c>
       <c r="H46" t="n">
-        <v>-0.1301411338592615</v>
+        <v>-0.1671069851042278</v>
       </c>
       <c r="I46" t="n">
-        <v>66.44144144144144</v>
+        <v>61.39438085327785</v>
       </c>
       <c r="J46" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K46" t="n">
         <v>49.61</v>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M46" t="n">
         <v>49.61</v>
       </c>
       <c r="N46" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O46" t="n">
-        <v>25.53191489361702</v>
+        <v>27.65957446808511</v>
       </c>
       <c r="P46" t="n">
-        <v>56.95038297872341</v>
+        <v>49.37591489361702</v>
       </c>
       <c r="Q46" t="b">
         <v>0</v>
@@ -3704,25 +3704,25 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>1077.2</v>
+        <v>1047.95</v>
       </c>
       <c r="D47" t="n">
-        <v>0.049697914636523</v>
+        <v>-0.0381809003717129</v>
       </c>
       <c r="E47" t="n">
-        <v>0.4410702341137125</v>
+        <v>0.4326042378673957</v>
       </c>
       <c r="F47" t="n">
-        <v>0.2284883389405256</v>
+        <v>0.1903788266030557</v>
       </c>
       <c r="G47" t="n">
-        <v>0.2491251226606636</v>
+        <v>0.2238913076004052</v>
       </c>
       <c r="H47" t="n">
-        <v>0.2365454614584033</v>
+        <v>0.1975948589069516</v>
       </c>
       <c r="I47" t="n">
-        <v>68.11058284909316</v>
+        <v>69.63096309630966</v>
       </c>
       <c r="J47" t="n">
         <v>80</v>
@@ -3732,7 +3732,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M47" t="n">
@@ -3769,25 +3769,25 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>15184</v>
+        <v>15002</v>
       </c>
       <c r="D48" t="n">
-        <v>0.1510878629368508</v>
+        <v>0.103737492642731</v>
       </c>
       <c r="E48" t="n">
-        <v>0.1024468162346621</v>
+        <v>0.1065870030242679</v>
       </c>
       <c r="F48" t="n">
-        <v>0.1190212985481613</v>
+        <v>0.1065053842749668</v>
       </c>
       <c r="G48" t="n">
-        <v>0.1396580822682993</v>
+        <v>0.1400178652723163</v>
       </c>
       <c r="H48" t="n">
-        <v>0.127078421066039</v>
+        <v>0.1137214165788627</v>
       </c>
       <c r="I48" t="n">
-        <v>68.10293237582286</v>
+        <v>68.91160553217077</v>
       </c>
       <c r="J48" t="n">
         <v>80</v>
@@ -3797,7 +3797,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M48" t="n">
@@ -3807,10 +3807,10 @@
         <v>80</v>
       </c>
       <c r="O48" t="n">
-        <v>70.21276595744681</v>
+        <v>68.08510638297872</v>
       </c>
       <c r="P48" t="n">
-        <v>66.15855319148936</v>
+        <v>65.73302127659575</v>
       </c>
       <c r="Q48" t="b">
         <v>0</v>
@@ -3936,57 +3936,57 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>LUMAXTECH</t>
+          <t>GNA</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Lighting</t>
+          <t>Axles</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1794.4</v>
+        <v>429.3</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1416210713831276</v>
+        <v>0.08368042408178721</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2868617326448652</v>
+        <v>0.2528819495111631</v>
       </c>
       <c r="F2" t="n">
-        <v>0.3775525871334255</v>
+        <v>0.3866279069767442</v>
       </c>
       <c r="G2" t="n">
-        <v>0.3981893708535635</v>
+        <v>0.4201403879740937</v>
       </c>
       <c r="H2" t="n">
-        <v>0.3856097096513032</v>
+        <v>0.3938439392806401</v>
       </c>
       <c r="I2" t="n">
-        <v>71.40147023950676</v>
+        <v>68.63583365720947</v>
       </c>
       <c r="J2" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K2" t="n">
-        <v>54.51</v>
+        <v>54.47</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M2" t="n">
-        <v>54.51</v>
+        <v>54.47</v>
       </c>
       <c r="N2" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O2" t="n">
-        <v>91.48936170212764</v>
+        <v>95.74468085106383</v>
       </c>
       <c r="P2" t="n">
-        <v>68.10187234042553</v>
+        <v>72.93693617021276</v>
       </c>
       <c r="Q2" t="b">
         <v>0</v>
@@ -4001,57 +4001,57 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>WHEELS</t>
+          <t>LUMAXTECH</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Wheels</t>
+          <t>Lighting</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1077.2</v>
+        <v>1727</v>
       </c>
       <c r="D3" t="n">
-        <v>0.049697914636523</v>
+        <v>0.0638822152405593</v>
       </c>
       <c r="E3" t="n">
-        <v>0.4410702341137125</v>
+        <v>0.2536295005807201</v>
       </c>
       <c r="F3" t="n">
-        <v>0.2284883389405256</v>
+        <v>0.3721595423486414</v>
       </c>
       <c r="G3" t="n">
-        <v>0.2491251226606636</v>
+        <v>0.4056720233459909</v>
       </c>
       <c r="H3" t="n">
-        <v>0.2365454614584033</v>
+        <v>0.3793755746525373</v>
       </c>
       <c r="I3" t="n">
-        <v>68.11058284909316</v>
+        <v>57.3502722323049</v>
       </c>
       <c r="J3" t="n">
         <v>80</v>
       </c>
       <c r="K3" t="n">
-        <v>46.83</v>
+        <v>54.51</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M3" t="n">
-        <v>46.83</v>
+        <v>54.51</v>
       </c>
       <c r="N3" t="n">
         <v>80</v>
       </c>
       <c r="O3" t="n">
-        <v>80.85106382978722</v>
+        <v>93.61702127659576</v>
       </c>
       <c r="P3" t="n">
-        <v>66.90221276595744</v>
+        <v>72.52740425531915</v>
       </c>
       <c r="Q3" t="b">
         <v>0</v>
@@ -4075,48 +4075,48 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>588.45</v>
+        <v>564.85</v>
       </c>
       <c r="D4" t="n">
-        <v>0.189508793208005</v>
+        <v>0.1044090331410696</v>
       </c>
       <c r="E4" t="n">
-        <v>0.3239959500506244</v>
+        <v>0.2384345538259153</v>
       </c>
       <c r="F4" t="n">
-        <v>0.4020729092208721</v>
+        <v>0.3642072213500784</v>
       </c>
       <c r="G4" t="n">
-        <v>0.4227096929410101</v>
+        <v>0.3977197023474279</v>
       </c>
       <c r="H4" t="n">
-        <v>0.4101300317387498</v>
+        <v>0.3714232536539743</v>
       </c>
       <c r="I4" t="n">
-        <v>79.17460317460311</v>
+        <v>66.4784546805349</v>
       </c>
       <c r="J4" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K4" t="n">
         <v>49.66</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M4" t="n">
         <v>49.66</v>
       </c>
       <c r="N4" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O4" t="n">
-        <v>93.61702127659576</v>
+        <v>91.48936170212764</v>
       </c>
       <c r="P4" t="n">
-        <v>66.58740425531916</v>
+        <v>70.16187234042553</v>
       </c>
       <c r="Q4" t="b">
         <v>0</v>
@@ -4131,57 +4131,57 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ZFCVINDIA</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Brakes/Transmission</t>
+          <t>Forgings</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>15184</v>
+        <v>1856</v>
       </c>
       <c r="D5" t="n">
-        <v>0.1510878629368508</v>
+        <v>0.0688165850849409</v>
       </c>
       <c r="E5" t="n">
-        <v>0.1024468162346621</v>
+        <v>0.3174332765474164</v>
       </c>
       <c r="F5" t="n">
-        <v>0.1190212985481613</v>
+        <v>0.5253122945430639</v>
       </c>
       <c r="G5" t="n">
-        <v>0.1396580822682993</v>
+        <v>0.5588247755404134</v>
       </c>
       <c r="H5" t="n">
-        <v>0.127078421066039</v>
+        <v>0.5325283268469598</v>
       </c>
       <c r="I5" t="n">
-        <v>68.10293237582286</v>
+        <v>75.48103353490929</v>
       </c>
       <c r="J5" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K5" t="n">
-        <v>50.29</v>
+        <v>54.83</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M5" t="n">
-        <v>50.29</v>
+        <v>54.83</v>
       </c>
       <c r="N5" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O5" t="n">
-        <v>70.21276595744681</v>
+        <v>97.87234042553192</v>
       </c>
       <c r="P5" t="n">
-        <v>66.15855319148936</v>
+        <v>69.50646808510639</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
@@ -4196,7 +4196,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>SANSERA</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -4205,48 +4205,48 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1903.2</v>
+        <v>2530.7</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1137640449438202</v>
+        <v>0.1592762253779203</v>
       </c>
       <c r="E6" t="n">
-        <v>0.3791304347826087</v>
+        <v>0.5236002408187836</v>
       </c>
       <c r="F6" t="n">
-        <v>0.5597443042124242</v>
+        <v>0.741227466629971</v>
       </c>
       <c r="G6" t="n">
-        <v>0.5803810879325622</v>
+        <v>0.7747399476273205</v>
       </c>
       <c r="H6" t="n">
-        <v>0.5678014267303019</v>
+        <v>0.7484434989338669</v>
       </c>
       <c r="I6" t="n">
-        <v>87.81195589088799</v>
+        <v>78.30092118730811</v>
       </c>
       <c r="J6" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K6" t="n">
-        <v>54.83</v>
+        <v>48.59</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M6" t="n">
-        <v>54.83</v>
+        <v>48.59</v>
       </c>
       <c r="N6" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O6" t="n">
-        <v>97.87234042553192</v>
+        <v>100</v>
       </c>
       <c r="P6" t="n">
-        <v>65.50646808510639</v>
+        <v>67.43600000000001</v>
       </c>
       <c r="Q6" t="b">
         <v>0</v>
@@ -4261,63 +4261,63 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ASKAUTOLTD</t>
+          <t>FIEMIND</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Lighting</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>442.8</v>
+        <v>2175</v>
       </c>
       <c r="D7" t="n">
-        <v>0.0662171923910426</v>
+        <v>0.0438663851027067</v>
       </c>
       <c r="E7" t="n">
-        <v>0.0273781902552203</v>
+        <v>0.0137024608501119</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.1520490233626963</v>
+        <v>0.1344669309409556</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.1314122396425583</v>
+        <v>0.1679794119383051</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.1439919008448186</v>
+        <v>0.1416829632448515</v>
       </c>
       <c r="I7" t="n">
-        <v>58.70165745856355</v>
+        <v>65.25526742301457</v>
       </c>
       <c r="J7" t="n">
         <v>80</v>
       </c>
       <c r="K7" t="n">
-        <v>71.28</v>
+        <v>49.06</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M7" t="n">
-        <v>71.28</v>
+        <v>49.06</v>
       </c>
       <c r="N7" t="n">
         <v>80</v>
       </c>
       <c r="O7" t="n">
-        <v>23.40425531914894</v>
+        <v>76.59574468085107</v>
       </c>
       <c r="P7" t="n">
-        <v>65.19285106382979</v>
+        <v>66.94314893617022</v>
       </c>
       <c r="Q7" t="b">
+        <v>0</v>
+      </c>
+      <c r="R7" t="b">
         <v>1</v>
-      </c>
-      <c r="R7" t="b">
-        <v>0</v>
       </c>
       <c r="S7" t="b">
         <v>0</v>
@@ -4326,57 +4326,57 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>RICOAUTO</t>
+          <t>WHEELS</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Castings</t>
+          <t>Wheels</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>118.41</v>
+        <v>1047.95</v>
       </c>
       <c r="D8" t="n">
-        <v>0.09073323507737641</v>
+        <v>-0.0381809003717129</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0228921907394608</v>
+        <v>0.4326042378673957</v>
       </c>
       <c r="F8" t="n">
-        <v>0.2669591268992082</v>
+        <v>0.1903788266030557</v>
       </c>
       <c r="G8" t="n">
-        <v>0.2875959106193462</v>
+        <v>0.2238913076004052</v>
       </c>
       <c r="H8" t="n">
-        <v>0.2750162494170859</v>
+        <v>0.1975948589069516</v>
       </c>
       <c r="I8" t="n">
-        <v>70.46610169491525</v>
+        <v>69.63096309630966</v>
       </c>
       <c r="J8" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K8" t="n">
-        <v>49.07</v>
+        <v>46.83</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M8" t="n">
-        <v>49.07</v>
+        <v>46.83</v>
       </c>
       <c r="N8" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O8" t="n">
-        <v>87.2340425531915</v>
+        <v>80.85106382978722</v>
       </c>
       <c r="P8" t="n">
-        <v>65.07480851063831</v>
+        <v>66.90221276595744</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
@@ -4391,57 +4391,57 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>GNA</t>
+          <t>ZFCVINDIA</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Axles</t>
+          <t>Brakes/Transmission</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>457.2</v>
+        <v>15002</v>
       </c>
       <c r="D9" t="n">
-        <v>0.2295280354981845</v>
+        <v>0.103737492642731</v>
       </c>
       <c r="E9" t="n">
-        <v>0.3678384442782347</v>
+        <v>0.1065870030242679</v>
       </c>
       <c r="F9" t="n">
-        <v>0.4595371109337589</v>
+        <v>0.1065053842749668</v>
       </c>
       <c r="G9" t="n">
-        <v>0.4801738946538969</v>
+        <v>0.1400178652723163</v>
       </c>
       <c r="H9" t="n">
-        <v>0.4675942334516366</v>
+        <v>0.1137214165788627</v>
       </c>
       <c r="I9" t="n">
-        <v>88.76353790613715</v>
+        <v>68.91160553217077</v>
       </c>
       <c r="J9" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K9" t="n">
-        <v>54.47</v>
+        <v>50.29</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M9" t="n">
-        <v>54.47</v>
+        <v>50.29</v>
       </c>
       <c r="N9" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O9" t="n">
-        <v>95.74468085106383</v>
+        <v>68.08510638297872</v>
       </c>
       <c r="P9" t="n">
-        <v>64.93693617021276</v>
+        <v>65.73302127659575</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -4456,57 +4456,57 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SANDHAR</t>
+          <t>SHRIPISTON</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Engine/Parts</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>486.85</v>
+        <v>3478.7</v>
       </c>
       <c r="D10" t="n">
-        <v>0.0642693190512624</v>
+        <v>0.1214016311530898</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.0438923802042419</v>
+        <v>0.2882642669333035</v>
       </c>
       <c r="F10" t="n">
-        <v>0.06929497034922021</v>
+        <v>0.2815723548482167</v>
       </c>
       <c r="G10" t="n">
-        <v>0.0899317540693582</v>
+        <v>0.3150848358455662</v>
       </c>
       <c r="H10" t="n">
-        <v>0.0773520928670979</v>
+        <v>0.2887883871521126</v>
       </c>
       <c r="I10" t="n">
-        <v>64.98237367802585</v>
+        <v>73.04347826086955</v>
       </c>
       <c r="J10" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K10" t="n">
-        <v>47.8</v>
+        <v>48.69</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M10" t="n">
-        <v>47.8</v>
+        <v>48.69</v>
       </c>
       <c r="N10" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O10" t="n">
-        <v>65.95744680851064</v>
+        <v>89.36170212765957</v>
       </c>
       <c r="P10" t="n">
-        <v>64.31148936170213</v>
+        <v>65.34834042553192</v>
       </c>
       <c r="Q10" t="b">
         <v>0</v>
@@ -4521,57 +4521,57 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SANSERA</t>
+          <t>MOTHERSON</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Forgings</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>2547</v>
+        <v>125.7</v>
       </c>
       <c r="D11" t="n">
-        <v>0.2037430880476392</v>
+        <v>0.1111111111111111</v>
       </c>
       <c r="E11" t="n">
-        <v>0.4817615917156319</v>
+        <v>0.1595940959409594</v>
       </c>
       <c r="F11" t="n">
-        <v>0.8181169248340352</v>
+        <v>0.2072608528620823</v>
       </c>
       <c r="G11" t="n">
-        <v>0.8387537085541732</v>
+        <v>0.2407733338594317</v>
       </c>
       <c r="H11" t="n">
-        <v>0.8261740473519129</v>
+        <v>0.2144768851659781</v>
       </c>
       <c r="I11" t="n">
-        <v>80.89430894308947</v>
+        <v>70.17584451642759</v>
       </c>
       <c r="J11" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K11" t="n">
-        <v>48.59</v>
+        <v>51.57</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M11" t="n">
-        <v>48.59</v>
+        <v>51.57</v>
       </c>
       <c r="N11" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O11" t="n">
-        <v>100</v>
+        <v>82.97872340425532</v>
       </c>
       <c r="P11" t="n">
-        <v>63.43600000000001</v>
+        <v>65.22374468085107</v>
       </c>
       <c r="Q11" t="b">
         <v>0</v>
@@ -4586,57 +4586,57 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>DIVGIITTS</t>
+          <t>CRAFTSMAN</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Transmission</t>
+          <t>Castings</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>733.8</v>
+        <v>7570</v>
       </c>
       <c r="D12" t="n">
-        <v>0.0526466790991249</v>
+        <v>0.0739111930770322</v>
       </c>
       <c r="E12" t="n">
-        <v>0.253608951909114</v>
+        <v>0.0516079738834478</v>
       </c>
       <c r="F12" t="n">
-        <v>0.0866281652598845</v>
+        <v>0.1321319075749645</v>
       </c>
       <c r="G12" t="n">
-        <v>0.1072649489800225</v>
+        <v>0.165644388572314</v>
       </c>
       <c r="H12" t="n">
-        <v>0.09468528777776231</v>
+        <v>0.1393479398788604</v>
       </c>
       <c r="I12" t="n">
-        <v>73.33177788147458</v>
+        <v>77.69582016157359</v>
       </c>
       <c r="J12" t="n">
         <v>70</v>
       </c>
       <c r="K12" t="n">
-        <v>49.92</v>
+        <v>54.65</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M12" t="n">
-        <v>49.92</v>
+        <v>54.65</v>
       </c>
       <c r="N12" t="n">
         <v>70</v>
       </c>
       <c r="O12" t="n">
-        <v>68.08510638297872</v>
+        <v>72.3404255319149</v>
       </c>
       <c r="P12" t="n">
-        <v>61.58502127659575</v>
+        <v>64.32808510638299</v>
       </c>
       <c r="Q12" t="b">
         <v>0</v>
@@ -4651,57 +4651,57 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>SHRIPISTON</t>
+          <t>DIVGIITTS</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Engine/Parts</t>
+          <t>Transmission</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>3591.6</v>
+        <v>752.5</v>
       </c>
       <c r="D13" t="n">
-        <v>0.2035789685332261</v>
+        <v>0.07862108507131089</v>
       </c>
       <c r="E13" t="n">
-        <v>0.3066065192083818</v>
+        <v>0.2626898229717258</v>
       </c>
       <c r="F13" t="n">
-        <v>0.3140641006878384</v>
+        <v>0.1508755830848054</v>
       </c>
       <c r="G13" t="n">
-        <v>0.3347008844079764</v>
+        <v>0.1843880640821549</v>
       </c>
       <c r="H13" t="n">
-        <v>0.3221212232057161</v>
+        <v>0.1580916153887013</v>
       </c>
       <c r="I13" t="n">
-        <v>81.92144782441277</v>
+        <v>73.06209850107068</v>
       </c>
       <c r="J13" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K13" t="n">
-        <v>48.69</v>
+        <v>49.92</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M13" t="n">
-        <v>48.69</v>
+        <v>49.92</v>
       </c>
       <c r="N13" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O13" t="n">
-        <v>89.36170212765957</v>
+        <v>78.72340425531915</v>
       </c>
       <c r="P13" t="n">
-        <v>61.34834042553192</v>
+        <v>63.71268085106384</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
@@ -4716,57 +4716,57 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>MOTHERSON</t>
+          <t>BHARATGEAR</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Gears</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>131.76</v>
+        <v>108.47</v>
       </c>
       <c r="D14" t="n">
-        <v>0.185638441464951</v>
+        <v>0.1333194023612998</v>
       </c>
       <c r="E14" t="n">
-        <v>0.2014224491656788</v>
+        <v>-0.0090443997807417</v>
       </c>
       <c r="F14" t="n">
-        <v>0.235211399643761</v>
+        <v>0.132372899050005</v>
       </c>
       <c r="G14" t="n">
-        <v>0.255848183363899</v>
+        <v>0.1658853800473545</v>
       </c>
       <c r="H14" t="n">
-        <v>0.2432685221616387</v>
+        <v>0.1395889313539009</v>
       </c>
       <c r="I14" t="n">
-        <v>82.3102823102823</v>
+        <v>76.72320461927102</v>
       </c>
       <c r="J14" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K14" t="n">
-        <v>51.57</v>
+        <v>51.91</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M14" t="n">
-        <v>51.57</v>
+        <v>51.91</v>
       </c>
       <c r="N14" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O14" t="n">
-        <v>82.97872340425532</v>
+        <v>74.46808510638297</v>
       </c>
       <c r="P14" t="n">
-        <v>61.22374468085107</v>
+        <v>63.65761702127659</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
@@ -4781,63 +4781,63 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>JAMNAAUTO</t>
+          <t>MENONBE</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Suspension</t>
+          <t>Bearings</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>126.29</v>
+        <v>118.74</v>
       </c>
       <c r="D15" t="n">
-        <v>0.0720713073005094</v>
+        <v>0.0607468286582097</v>
       </c>
       <c r="E15" t="n">
-        <v>0.0860853113175095</v>
+        <v>-0.0266415279940979</v>
       </c>
       <c r="F15" t="n">
-        <v>0.2444816712652739</v>
+        <v>-0.052051732396615</v>
       </c>
       <c r="G15" t="n">
-        <v>0.265118454985412</v>
+        <v>-0.0185392513992656</v>
       </c>
       <c r="H15" t="n">
-        <v>0.2525387937831517</v>
+        <v>-0.0448357000927192</v>
       </c>
       <c r="I15" t="n">
-        <v>69.90291262135922</v>
+        <v>61.84588844163311</v>
       </c>
       <c r="J15" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K15" t="n">
-        <v>48.3</v>
+        <v>52.38</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M15" t="n">
-        <v>48.3</v>
+        <v>52.38</v>
       </c>
       <c r="N15" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O15" t="n">
-        <v>85.1063829787234</v>
+        <v>53.19148936170212</v>
       </c>
       <c r="P15" t="n">
-        <v>60.34127659574468</v>
+        <v>63.59029787234042</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
       </c>
       <c r="R15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S15" t="b">
         <v>0</v>
@@ -4846,57 +4846,57 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CRAFTSMAN</t>
+          <t>PRICOLLTD</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Castings</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>7684.5</v>
+        <v>594.65</v>
       </c>
       <c r="D16" t="n">
-        <v>0.122972380534853</v>
+        <v>0.09320709624046319</v>
       </c>
       <c r="E16" t="n">
-        <v>0.0394994927291174</v>
+        <v>0.0226139294926912</v>
       </c>
       <c r="F16" t="n">
-        <v>0.1344947220786889</v>
+        <v>0.1291180100636095</v>
       </c>
       <c r="G16" t="n">
-        <v>0.1551315057988269</v>
+        <v>0.162630491060959</v>
       </c>
       <c r="H16" t="n">
-        <v>0.1425518445965666</v>
+        <v>0.1363340423675054</v>
       </c>
       <c r="I16" t="n">
-        <v>87.80075981426762</v>
+        <v>73.09605817068504</v>
       </c>
       <c r="J16" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K16" t="n">
-        <v>54.65</v>
+        <v>49.98</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="M16" t="n">
-        <v>54.65</v>
+        <v>49.98</v>
       </c>
       <c r="N16" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O16" t="n">
-        <v>72.3404255319149</v>
+        <v>70.21276595744681</v>
       </c>
       <c r="P16" t="n">
-        <v>60.32808510638298</v>
+        <v>62.03455319148937</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
chore: auto-refresh NSE data and pipeline outputs (2026-04-27)
</commit_message>
<xml_diff>
--- a/working-sector/output/auto_components_comprehensive_report.xlsx
+++ b/working-sector/output/auto_components_comprehensive_report.xlsx
@@ -435,7 +435,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
     </row>
@@ -447,7 +447,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
     </row>
@@ -779,25 +779,25 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1856</v>
+        <v>1901.1</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0688165850849409</v>
+        <v>0.1020230711263114</v>
       </c>
       <c r="E2" t="n">
-        <v>0.3174332765474164</v>
+        <v>0.3402185407120197</v>
       </c>
       <c r="F2" t="n">
-        <v>0.5253122945430639</v>
+        <v>0.5962216624685137</v>
       </c>
       <c r="G2" t="n">
-        <v>0.5588247755404134</v>
+        <v>0.6229506906413951</v>
       </c>
       <c r="H2" t="n">
-        <v>0.5325283268469598</v>
+        <v>0.6008840229575163</v>
       </c>
       <c r="I2" t="n">
-        <v>75.48103353490929</v>
+        <v>78.14796668299851</v>
       </c>
       <c r="J2" t="n">
         <v>70</v>
@@ -807,7 +807,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M2" t="n">
@@ -844,25 +844,25 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1108.1</v>
+        <v>1130.9</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0188488414858403</v>
+        <v>0.0783827596071327</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.0229256679305176</v>
+        <v>-0.0123144104803493</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.1889775305569787</v>
+        <v>-0.1376391642519444</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.1554650495596292</v>
+        <v>-0.110910136079063</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.1817614982530828</v>
+        <v>-0.1329768037629418</v>
       </c>
       <c r="I3" t="n">
-        <v>60.13582342954154</v>
+        <v>68.85980020668271</v>
       </c>
       <c r="J3" t="n">
         <v>80</v>
@@ -872,7 +872,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M3" t="n">
@@ -882,10 +882,10 @@
         <v>80</v>
       </c>
       <c r="O3" t="n">
-        <v>25.53191489361702</v>
+        <v>29.78723404255319</v>
       </c>
       <c r="P3" t="n">
-        <v>56.8503829787234</v>
+        <v>57.70144680851064</v>
       </c>
       <c r="Q3" t="b">
         <v>0</v>
@@ -909,25 +909,25 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>36690</v>
+        <v>37225</v>
       </c>
       <c r="D4" t="n">
-        <v>0.2073050345508391</v>
+        <v>0.2569643761607294</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0404083368779242</v>
+        <v>0.0542339280657038</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.0536497291720402</v>
+        <v>-0.029335071707953</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.0201372481746907</v>
+        <v>-0.0026060435350716</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.0464336968681443</v>
+        <v>-0.0246727112189504</v>
       </c>
       <c r="I4" t="n">
-        <v>71.50466045272969</v>
+        <v>73.53673723536737</v>
       </c>
       <c r="J4" t="n">
         <v>70</v>
@@ -937,7 +937,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M4" t="n">
@@ -947,10 +947,10 @@
         <v>70</v>
       </c>
       <c r="O4" t="n">
-        <v>51.06382978723404</v>
+        <v>53.19148936170212</v>
       </c>
       <c r="P4" t="n">
-        <v>59.6047659574468</v>
+        <v>60.03029787234042</v>
       </c>
       <c r="Q4" t="b">
         <v>0</v>
@@ -974,48 +974,48 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>342.8</v>
+        <v>352.35</v>
       </c>
       <c r="D5" t="n">
-        <v>0.1160670682077162</v>
+        <v>0.1711816519860396</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0541205412054122</v>
+        <v>0.09002320185614859</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.1490629266476356</v>
+        <v>-0.1154763399020961</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.1155504456502861</v>
+        <v>-0.0887473117292148</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.1418468943437397</v>
+        <v>-0.1108139794130935</v>
       </c>
       <c r="I5" t="n">
-        <v>77.56892230576443</v>
+        <v>81.37813211845105</v>
       </c>
       <c r="J5" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="K5" t="n">
         <v>51.12</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M5" t="n">
         <v>51.12</v>
       </c>
       <c r="N5" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="O5" t="n">
-        <v>31.91489361702128</v>
+        <v>36.17021276595745</v>
       </c>
       <c r="P5" t="n">
-        <v>54.83097872340426</v>
+        <v>51.68204255319149</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
@@ -1039,25 +1039,25 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>125.7</v>
+        <v>127.93</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.169592247211556</v>
       </c>
       <c r="E6" t="n">
-        <v>0.1595940959409594</v>
+        <v>0.1664994984954864</v>
       </c>
       <c r="F6" t="n">
-        <v>0.2072608528620823</v>
+        <v>0.2586580086580088</v>
       </c>
       <c r="G6" t="n">
-        <v>0.2407733338594317</v>
+        <v>0.2853870368308902</v>
       </c>
       <c r="H6" t="n">
-        <v>0.2144768851659781</v>
+        <v>0.2633203691470114</v>
       </c>
       <c r="I6" t="n">
-        <v>70.17584451642759</v>
+        <v>71.52639717252046</v>
       </c>
       <c r="J6" t="n">
         <v>70</v>
@@ -1067,7 +1067,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M6" t="n">
@@ -1104,25 +1104,25 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2968.7</v>
+        <v>2994.4</v>
       </c>
       <c r="D7" t="n">
-        <v>0.106732776617954</v>
+        <v>0.1668160386548727</v>
       </c>
       <c r="E7" t="n">
-        <v>0.3376137694872487</v>
+        <v>0.3677431142374274</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.07758513547104159</v>
+        <v>-0.0470371077588949</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.0440726544736921</v>
+        <v>-0.0203080795860135</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.0703691031671457</v>
+        <v>-0.0423747472698923</v>
       </c>
       <c r="I7" t="n">
-        <v>78.16880841121491</v>
+        <v>78.80034032898465</v>
       </c>
       <c r="J7" t="n">
         <v>70</v>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M7" t="n">
@@ -1169,25 +1169,25 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>564.85</v>
+        <v>588.65</v>
       </c>
       <c r="D8" t="n">
-        <v>0.1044090331410696</v>
+        <v>0.204398976982097</v>
       </c>
       <c r="E8" t="n">
-        <v>0.2384345538259153</v>
+        <v>0.2067445674456745</v>
       </c>
       <c r="F8" t="n">
-        <v>0.3642072213500784</v>
+        <v>0.4525601480567549</v>
       </c>
       <c r="G8" t="n">
-        <v>0.3977197023474279</v>
+        <v>0.4792891762296363</v>
       </c>
       <c r="H8" t="n">
-        <v>0.3714232536539743</v>
+        <v>0.4572225085457575</v>
       </c>
       <c r="I8" t="n">
-        <v>66.4784546805349</v>
+        <v>69.7262479871175</v>
       </c>
       <c r="J8" t="n">
         <v>80</v>
@@ -1197,7 +1197,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M8" t="n">
@@ -1207,10 +1207,10 @@
         <v>80</v>
       </c>
       <c r="O8" t="n">
-        <v>91.48936170212764</v>
+        <v>95.74468085106383</v>
       </c>
       <c r="P8" t="n">
-        <v>70.16187234042553</v>
+        <v>71.01293617021277</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
@@ -1234,25 +1234,25 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>423.85</v>
+        <v>428.55</v>
       </c>
       <c r="D9" t="n">
-        <v>0.0100083402835697</v>
+        <v>0.0390350345496424</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.1509415064102564</v>
+        <v>-0.1546503599960548</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.1142110762800417</v>
+        <v>-0.1198398028342574</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.0806985952826923</v>
+        <v>-0.093110774661376</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.1069950439761459</v>
+        <v>-0.1151774423452548</v>
       </c>
       <c r="I9" t="n">
-        <v>58.8637919233402</v>
+        <v>60.35620052770448</v>
       </c>
       <c r="J9" t="n">
         <v>40</v>
@@ -1262,7 +1262,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M9" t="n">
@@ -1272,10 +1272,10 @@
         <v>40</v>
       </c>
       <c r="O9" t="n">
-        <v>38.29787234042553</v>
+        <v>34.04255319148936</v>
       </c>
       <c r="P9" t="n">
-        <v>45.03557446808512</v>
+        <v>44.18451063829788</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -1299,25 +1299,25 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>132145</v>
+        <v>132205</v>
       </c>
       <c r="D10" t="n">
-        <v>0.0167346310687082</v>
+        <v>0.0202971252170558</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.0387706855791961</v>
+        <v>-0.0265444370812164</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.1403525891230809</v>
+        <v>-0.1482185426196766</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.1068401081257314</v>
+        <v>-0.1214895144467952</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.133136556819185</v>
+        <v>-0.143556182130674</v>
       </c>
       <c r="I10" t="n">
-        <v>59.74025974025973</v>
+        <v>59.63232477977786</v>
       </c>
       <c r="J10" t="n">
         <v>40</v>
@@ -1327,7 +1327,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M10" t="n">
@@ -1337,10 +1337,10 @@
         <v>40</v>
       </c>
       <c r="O10" t="n">
-        <v>34.04255319148936</v>
+        <v>25.53191489361702</v>
       </c>
       <c r="P10" t="n">
-        <v>42.57251063829787</v>
+        <v>40.8703829787234</v>
       </c>
       <c r="Q10" t="b">
         <v>0</v>
@@ -1376,10 +1376,10 @@
         <v>-0.0042030657656173</v>
       </c>
       <c r="G11" t="n">
-        <v>0.0293094152317321</v>
+        <v>0.022525962407264</v>
       </c>
       <c r="H11" t="n">
-        <v>0.0030129665382785</v>
+        <v>0.0004592947233852</v>
       </c>
       <c r="I11" t="n">
         <v>27.6054590570719</v>
@@ -1392,7 +1392,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M11" t="n">
@@ -1402,10 +1402,10 @@
         <v>20</v>
       </c>
       <c r="O11" t="n">
-        <v>61.70212765957447</v>
+        <v>55.31914893617022</v>
       </c>
       <c r="P11" t="n">
-        <v>24.3404255319149</v>
+        <v>23.06382978723404</v>
       </c>
       <c r="Q11" t="b">
         <v>0</v>
@@ -1429,25 +1429,25 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>428.65</v>
+        <v>435.55</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.0348981200045029</v>
+        <v>-0.0072934472934472</v>
       </c>
       <c r="E12" t="n">
-        <v>0.0077583166803807</v>
+        <v>0.0133783154955793</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.1658883051177272</v>
+        <v>-0.1268918512578931</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.1323758241203777</v>
+        <v>-0.1001628230850117</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.1586722728138313</v>
+        <v>-0.1222294907688905</v>
       </c>
       <c r="I12" t="n">
-        <v>43.95036194415717</v>
+        <v>52.22634508348798</v>
       </c>
       <c r="J12" t="n">
         <v>60</v>
@@ -1457,7 +1457,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M12" t="n">
@@ -1467,10 +1467,10 @@
         <v>60</v>
       </c>
       <c r="O12" t="n">
-        <v>29.78723404255319</v>
+        <v>31.91489361702128</v>
       </c>
       <c r="P12" t="n">
-        <v>58.46944680851064</v>
+        <v>58.89497872340426</v>
       </c>
       <c r="Q12" t="b">
         <v>1</v>
@@ -1494,48 +1494,48 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1796.3</v>
+        <v>1877.9</v>
       </c>
       <c r="D13" t="n">
-        <v>0.0884028114396509</v>
+        <v>0.1844960262394348</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.0737379466817924</v>
+        <v>-0.0340020576131686</v>
       </c>
       <c r="F13" t="n">
-        <v>0.0287497852356681</v>
+        <v>0.0899645945789076</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0622622662330176</v>
+        <v>0.1166936227517889</v>
       </c>
       <c r="H13" t="n">
-        <v>0.035965817539564</v>
+        <v>0.09462695506791011</v>
       </c>
       <c r="I13" t="n">
-        <v>63.5140728476821</v>
+        <v>69.02985074626865</v>
       </c>
       <c r="J13" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K13" t="n">
         <v>58.77</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M13" t="n">
         <v>58.77</v>
       </c>
       <c r="N13" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O13" t="n">
         <v>65.95744680851064</v>
       </c>
       <c r="P13" t="n">
-        <v>60.69948936170213</v>
+        <v>68.69948936170213</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
@@ -1559,25 +1559,25 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>606.8</v>
+        <v>624.55</v>
       </c>
       <c r="D14" t="n">
-        <v>0.08212215782434221</v>
+        <v>0.1747390200319758</v>
       </c>
       <c r="E14" t="n">
-        <v>0.1049804242920877</v>
+        <v>0.1261269383339343</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.2373531075221517</v>
+        <v>-0.2362113244466186</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.2038406265248022</v>
+        <v>-0.2094822962737372</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.2301370752182558</v>
+        <v>-0.231548963957616</v>
       </c>
       <c r="I14" t="n">
-        <v>71.51162790697671</v>
+        <v>73.77575595397374</v>
       </c>
       <c r="J14" t="n">
         <v>70</v>
@@ -1587,7 +1587,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M14" t="n">
@@ -1624,25 +1624,25 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>108.47</v>
+        <v>109.75</v>
       </c>
       <c r="D15" t="n">
-        <v>0.1333194023612998</v>
+        <v>0.2274913320657645</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.0090443997807417</v>
+        <v>0.0238828248903815</v>
       </c>
       <c r="F15" t="n">
-        <v>0.132372899050005</v>
+        <v>0.1909929462832338</v>
       </c>
       <c r="G15" t="n">
-        <v>0.1658853800473545</v>
+        <v>0.2177219744561151</v>
       </c>
       <c r="H15" t="n">
-        <v>0.1395889313539009</v>
+        <v>0.1956553067722364</v>
       </c>
       <c r="I15" t="n">
-        <v>76.72320461927102</v>
+        <v>76.79856115107913</v>
       </c>
       <c r="J15" t="n">
         <v>70</v>
@@ -1652,7 +1652,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M15" t="n">
@@ -1662,10 +1662,10 @@
         <v>70</v>
       </c>
       <c r="O15" t="n">
-        <v>74.46808510638297</v>
+        <v>80.85106382978722</v>
       </c>
       <c r="P15" t="n">
-        <v>63.65761702127659</v>
+        <v>64.93421276595744</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
@@ -1689,48 +1689,48 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>171.18</v>
+        <v>177.08</v>
       </c>
       <c r="D16" t="n">
-        <v>0.0783671412372433</v>
+        <v>0.1817150483817151</v>
       </c>
       <c r="E16" t="n">
-        <v>0.2236757452283939</v>
+        <v>0.3086018326928763</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.206176961602671</v>
+        <v>-0.1525245273988991</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.1726644806053215</v>
+        <v>-0.1257954992260177</v>
       </c>
       <c r="H16" t="n">
-        <v>-0.1989609292987751</v>
+        <v>-0.1478621669098965</v>
       </c>
       <c r="I16" t="n">
-        <v>63.31140350877192</v>
+        <v>64.79377104377103</v>
       </c>
       <c r="J16" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K16" t="n">
         <v>52.61</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M16" t="n">
         <v>52.61</v>
       </c>
       <c r="N16" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O16" t="n">
-        <v>17.02127659574468</v>
+        <v>23.40425531914894</v>
       </c>
       <c r="P16" t="n">
-        <v>48.44825531914893</v>
+        <v>57.72485106382978</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>
@@ -1754,48 +1754,48 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>7570</v>
+        <v>7633</v>
       </c>
       <c r="D17" t="n">
-        <v>0.0739111930770322</v>
+        <v>0.1023974581166955</v>
       </c>
       <c r="E17" t="n">
-        <v>0.0516079738834478</v>
+        <v>0.0082557294762564</v>
       </c>
       <c r="F17" t="n">
-        <v>0.1321319075749645</v>
+        <v>0.1505878806150136</v>
       </c>
       <c r="G17" t="n">
-        <v>0.165644388572314</v>
+        <v>0.1773169087878949</v>
       </c>
       <c r="H17" t="n">
-        <v>0.1393479398788604</v>
+        <v>0.1552502411040162</v>
       </c>
       <c r="I17" t="n">
-        <v>77.69582016157359</v>
+        <v>80.64849948258021</v>
       </c>
       <c r="J17" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="K17" t="n">
         <v>54.65</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M17" t="n">
         <v>54.65</v>
       </c>
       <c r="N17" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="O17" t="n">
-        <v>72.3404255319149</v>
+        <v>74.46808510638297</v>
       </c>
       <c r="P17" t="n">
-        <v>64.32808510638299</v>
+        <v>60.7536170212766</v>
       </c>
       <c r="Q17" t="b">
         <v>0</v>
@@ -1819,25 +1819,25 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>752.5</v>
+        <v>743.8</v>
       </c>
       <c r="D18" t="n">
-        <v>0.07862108507131089</v>
+        <v>0.1023341978510559</v>
       </c>
       <c r="E18" t="n">
-        <v>0.2626898229717258</v>
+        <v>0.2479865771812079</v>
       </c>
       <c r="F18" t="n">
-        <v>0.1508755830848054</v>
+        <v>0.1549689440993789</v>
       </c>
       <c r="G18" t="n">
-        <v>0.1843880640821549</v>
+        <v>0.1816979722722602</v>
       </c>
       <c r="H18" t="n">
-        <v>0.1580916153887013</v>
+        <v>0.1596313045883814</v>
       </c>
       <c r="I18" t="n">
-        <v>73.06209850107068</v>
+        <v>71.23173277661793</v>
       </c>
       <c r="J18" t="n">
         <v>70</v>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M18" t="n">
@@ -1857,10 +1857,10 @@
         <v>70</v>
       </c>
       <c r="O18" t="n">
-        <v>78.72340425531915</v>
+        <v>76.59574468085107</v>
       </c>
       <c r="P18" t="n">
-        <v>63.71268085106384</v>
+        <v>63.28714893617022</v>
       </c>
       <c r="Q18" t="b">
         <v>0</v>
@@ -1884,48 +1884,48 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2318.6</v>
+        <v>2368</v>
       </c>
       <c r="D19" t="n">
-        <v>-0.0062149072050061</v>
+        <v>0.047787610619469</v>
       </c>
       <c r="E19" t="n">
-        <v>-0.0162918964785745</v>
+        <v>0.0145237993230795</v>
       </c>
       <c r="F19" t="n">
-        <v>-0.2143002372077261</v>
+        <v>-0.1893464790661052</v>
       </c>
       <c r="G19" t="n">
-        <v>-0.1807877562103766</v>
+        <v>-0.1626174508932238</v>
       </c>
       <c r="H19" t="n">
-        <v>-0.2070842049038302</v>
+        <v>-0.1846841185771026</v>
       </c>
       <c r="I19" t="n">
-        <v>62.4946785866326</v>
+        <v>64.95624502784406</v>
       </c>
       <c r="J19" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K19" t="n">
         <v>51.27</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M19" t="n">
         <v>51.27</v>
       </c>
       <c r="N19" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O19" t="n">
         <v>14.8936170212766</v>
       </c>
       <c r="P19" t="n">
-        <v>39.48672340425532</v>
+        <v>47.48672340425532</v>
       </c>
       <c r="Q19" t="b">
         <v>0</v>
@@ -1949,25 +1949,25 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2175</v>
+        <v>2211.4</v>
       </c>
       <c r="D20" t="n">
-        <v>0.0438663851027067</v>
+        <v>0.1247647627282437</v>
       </c>
       <c r="E20" t="n">
-        <v>0.0137024608501119</v>
+        <v>0.0466183917838043</v>
       </c>
       <c r="F20" t="n">
-        <v>0.1344669309409556</v>
+        <v>0.1594400461385205</v>
       </c>
       <c r="G20" t="n">
-        <v>0.1679794119383051</v>
+        <v>0.1861690743114019</v>
       </c>
       <c r="H20" t="n">
-        <v>0.1416829632448515</v>
+        <v>0.1641024066275231</v>
       </c>
       <c r="I20" t="n">
-        <v>65.25526742301457</v>
+        <v>67.23347344287353</v>
       </c>
       <c r="J20" t="n">
         <v>80</v>
@@ -1977,7 +1977,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M20" t="n">
@@ -1987,10 +1987,10 @@
         <v>80</v>
       </c>
       <c r="O20" t="n">
-        <v>76.59574468085107</v>
+        <v>78.72340425531915</v>
       </c>
       <c r="P20" t="n">
-        <v>66.94314893617022</v>
+        <v>67.36868085106383</v>
       </c>
       <c r="Q20" t="b">
         <v>0</v>
@@ -2014,48 +2014,48 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>973</v>
+        <v>1013.5</v>
       </c>
       <c r="D21" t="n">
-        <v>0.1041134751773049</v>
+        <v>0.2313206171789574</v>
       </c>
       <c r="E21" t="n">
-        <v>0.0802709004107915</v>
+        <v>0.1435179961638271</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.2584971803078799</v>
+        <v>-0.2300387449669527</v>
       </c>
       <c r="G21" t="n">
-        <v>-0.2249846993105304</v>
+        <v>-0.2033097167940714</v>
       </c>
       <c r="H21" t="n">
-        <v>-0.251281148003984</v>
+        <v>-0.2253763844779501</v>
       </c>
       <c r="I21" t="n">
-        <v>67.53058262492225</v>
+        <v>72.1004810261892</v>
       </c>
       <c r="J21" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K21" t="n">
         <v>48.43</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M21" t="n">
         <v>48.43</v>
       </c>
       <c r="N21" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O21" t="n">
-        <v>4.25531914893617</v>
+        <v>10.63829787234042</v>
       </c>
       <c r="P21" t="n">
-        <v>52.22306382978724</v>
+        <v>49.49965957446808</v>
       </c>
       <c r="Q21" t="b">
         <v>0</v>
@@ -2079,48 +2079,48 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>429.3</v>
+        <v>440.6</v>
       </c>
       <c r="D22" t="n">
-        <v>0.08368042408178721</v>
+        <v>0.1660711922720656</v>
       </c>
       <c r="E22" t="n">
-        <v>0.2528819495111631</v>
+        <v>0.2943595769682727</v>
       </c>
       <c r="F22" t="n">
-        <v>0.3866279069767442</v>
+        <v>0.4187731444211882</v>
       </c>
       <c r="G22" t="n">
-        <v>0.4201403879740937</v>
+        <v>0.4455021725940695</v>
       </c>
       <c r="H22" t="n">
-        <v>0.3938439392806401</v>
+        <v>0.4234355049101908</v>
       </c>
       <c r="I22" t="n">
-        <v>68.63583365720947</v>
+        <v>72.01735357917572</v>
       </c>
       <c r="J22" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K22" t="n">
         <v>54.47</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M22" t="n">
         <v>54.47</v>
       </c>
       <c r="N22" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O22" t="n">
-        <v>95.74468085106383</v>
+        <v>93.61702127659576</v>
       </c>
       <c r="P22" t="n">
-        <v>72.93693617021276</v>
+        <v>68.51140425531915</v>
       </c>
       <c r="Q22" t="b">
         <v>0</v>
@@ -2144,25 +2144,25 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>381.6</v>
+        <v>392.5</v>
       </c>
       <c r="D23" t="n">
-        <v>0.1385946591078624</v>
+        <v>0.2176205987280906</v>
       </c>
       <c r="E23" t="n">
-        <v>0.026634382566586</v>
+        <v>0.0839547086440208</v>
       </c>
       <c r="F23" t="n">
-        <v>-0.0296249205340113</v>
+        <v>0.0064102564102563</v>
       </c>
       <c r="G23" t="n">
-        <v>0.0038875604633381</v>
+        <v>0.0331392845831377</v>
       </c>
       <c r="H23" t="n">
-        <v>-0.0224088882301154</v>
+        <v>0.0110726168992589</v>
       </c>
       <c r="I23" t="n">
-        <v>72.35002255299956</v>
+        <v>72.49887842081651</v>
       </c>
       <c r="J23" t="n">
         <v>70</v>
@@ -2172,7 +2172,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M23" t="n">
@@ -2191,7 +2191,7 @@
         <v>0</v>
       </c>
       <c r="R23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S23" t="b">
         <v>0</v>
@@ -2209,25 +2209,25 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>122.99</v>
+        <v>124.51</v>
       </c>
       <c r="D24" t="n">
-        <v>0.0125133777887544</v>
+        <v>0.06765563368204409</v>
       </c>
       <c r="E24" t="n">
-        <v>0.0563428669586876</v>
+        <v>0.07447359337245429</v>
       </c>
       <c r="F24" t="n">
-        <v>0.2539763458401305</v>
+        <v>0.2842702423929861</v>
       </c>
       <c r="G24" t="n">
-        <v>0.28748882683748</v>
+        <v>0.3109992705658675</v>
       </c>
       <c r="H24" t="n">
-        <v>0.2611923781440264</v>
+        <v>0.2889326028819887</v>
       </c>
       <c r="I24" t="n">
-        <v>61.40412155082081</v>
+        <v>66.99403717993687</v>
       </c>
       <c r="J24" t="n">
         <v>60</v>
@@ -2237,7 +2237,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M24" t="n">
@@ -2274,25 +2274,25 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>612.85</v>
+        <v>628.75</v>
       </c>
       <c r="D25" t="n">
-        <v>0.0701999476119794</v>
+        <v>0.1501875057166377</v>
       </c>
       <c r="E25" t="n">
-        <v>0.1585066162570889</v>
+        <v>0.1697674418604651</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.08386277001270639</v>
+        <v>-0.0459028831562974</v>
       </c>
       <c r="G25" t="n">
-        <v>-0.0503502890153569</v>
+        <v>-0.019173854983416</v>
       </c>
       <c r="H25" t="n">
-        <v>-0.0766467377088105</v>
+        <v>-0.0412405226672948</v>
       </c>
       <c r="I25" t="n">
-        <v>73.61740707162284</v>
+        <v>77.18600953895069</v>
       </c>
       <c r="J25" t="n">
         <v>70</v>
@@ -2302,7 +2302,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M25" t="n">
@@ -2312,10 +2312,10 @@
         <v>70</v>
       </c>
       <c r="O25" t="n">
-        <v>42.5531914893617</v>
+        <v>46.80851063829788</v>
       </c>
       <c r="P25" t="n">
-        <v>59.27463829787234</v>
+        <v>60.12570212765957</v>
       </c>
       <c r="Q25" t="b">
         <v>0</v>
@@ -2339,48 +2339,48 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>128.99</v>
+        <v>129.73</v>
       </c>
       <c r="D26" t="n">
-        <v>0.0250317863954228</v>
+        <v>0.0737460685316999</v>
       </c>
       <c r="E26" t="n">
-        <v>-0.0130078812456958</v>
+        <v>-0.0237055990367248</v>
       </c>
       <c r="F26" t="n">
-        <v>-0.1955721858434673</v>
+        <v>-0.1785601215728488</v>
       </c>
       <c r="G26" t="n">
-        <v>-0.1620597048461178</v>
+        <v>-0.1518310933999674</v>
       </c>
       <c r="H26" t="n">
-        <v>-0.1883561535395714</v>
+        <v>-0.1738977610838462</v>
       </c>
       <c r="I26" t="n">
-        <v>56.46532438478747</v>
+        <v>55.16129032258062</v>
       </c>
       <c r="J26" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="K26" t="n">
         <v>51.54</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M26" t="n">
         <v>51.54</v>
       </c>
       <c r="N26" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O26" t="n">
         <v>21.27659574468085</v>
       </c>
       <c r="P26" t="n">
-        <v>40.87131914893617</v>
+        <v>48.87131914893617</v>
       </c>
       <c r="Q26" t="b">
         <v>0</v>
@@ -2404,25 +2404,25 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>5173.6</v>
+        <v>5051.3</v>
       </c>
       <c r="D27" t="n">
-        <v>0.0048752063707877</v>
+        <v>0.0351024590163935</v>
       </c>
       <c r="E27" t="n">
-        <v>0.117046313289431</v>
+        <v>0.07543112625079849</v>
       </c>
       <c r="F27" t="n">
-        <v>0.0109623839765511</v>
+        <v>0.0140118438221419</v>
       </c>
       <c r="G27" t="n">
-        <v>0.0444748649739006</v>
+        <v>0.0407408719950233</v>
       </c>
       <c r="H27" t="n">
-        <v>0.018178416280447</v>
+        <v>0.0186742043111445</v>
       </c>
       <c r="I27" t="n">
-        <v>60.08005591206557</v>
+        <v>57.66205256418075</v>
       </c>
       <c r="J27" t="n">
         <v>40</v>
@@ -2432,7 +2432,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M27" t="n">
@@ -2442,10 +2442,10 @@
         <v>40</v>
       </c>
       <c r="O27" t="n">
-        <v>63.82978723404256</v>
+        <v>59.57446808510638</v>
       </c>
       <c r="P27" t="n">
-        <v>51.84195744680851</v>
+        <v>50.99089361702128</v>
       </c>
       <c r="Q27" t="b">
         <v>0</v>
@@ -2469,25 +2469,25 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1727</v>
+        <v>1747.6</v>
       </c>
       <c r="D28" t="n">
-        <v>0.0638822152405593</v>
+        <v>0.0862754848334161</v>
       </c>
       <c r="E28" t="n">
-        <v>0.2536295005807201</v>
+        <v>0.2897416974169742</v>
       </c>
       <c r="F28" t="n">
-        <v>0.3721595423486414</v>
+        <v>0.4163222303266065</v>
       </c>
       <c r="G28" t="n">
-        <v>0.4056720233459909</v>
+        <v>0.4430512584994879</v>
       </c>
       <c r="H28" t="n">
-        <v>0.3793755746525373</v>
+        <v>0.4209845908156091</v>
       </c>
       <c r="I28" t="n">
-        <v>57.3502722323049</v>
+        <v>63.05350553505533</v>
       </c>
       <c r="J28" t="n">
         <v>80</v>
@@ -2497,7 +2497,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M28" t="n">
@@ -2507,10 +2507,10 @@
         <v>80</v>
       </c>
       <c r="O28" t="n">
-        <v>93.61702127659576</v>
+        <v>91.48936170212764</v>
       </c>
       <c r="P28" t="n">
-        <v>72.52740425531915</v>
+        <v>72.10187234042553</v>
       </c>
       <c r="Q28" t="b">
         <v>0</v>
@@ -2534,25 +2534,25 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>527.6</v>
+        <v>526.8</v>
       </c>
       <c r="D29" t="n">
-        <v>-0.0300579097343506</v>
+        <v>-0.003593720446378</v>
       </c>
       <c r="E29" t="n">
-        <v>-0.0281819856327131</v>
+        <v>-0.023992589161649</v>
       </c>
       <c r="F29" t="n">
-        <v>-0.1123075628838227</v>
+        <v>-0.0950785879927854</v>
       </c>
       <c r="G29" t="n">
-        <v>-0.0787950818864732</v>
+        <v>-0.06834955981990409</v>
       </c>
       <c r="H29" t="n">
-        <v>-0.1050915305799268</v>
+        <v>-0.0904162275037828</v>
       </c>
       <c r="I29" t="n">
-        <v>57.33067729083667</v>
+        <v>58.8307440719542</v>
       </c>
       <c r="J29" t="n">
         <v>60</v>
@@ -2562,7 +2562,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M29" t="n">
@@ -2599,25 +2599,25 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>118.74</v>
+        <v>120.4</v>
       </c>
       <c r="D30" t="n">
-        <v>0.0607468286582097</v>
+        <v>0.1023622047244094</v>
       </c>
       <c r="E30" t="n">
-        <v>-0.0266415279940979</v>
+        <v>-0.0264413358130508</v>
       </c>
       <c r="F30" t="n">
-        <v>-0.052051732396615</v>
+        <v>-0.0313757039420755</v>
       </c>
       <c r="G30" t="n">
-        <v>-0.0185392513992656</v>
+        <v>-0.0046466757691941</v>
       </c>
       <c r="H30" t="n">
-        <v>-0.0448357000927192</v>
+        <v>-0.0267133434530729</v>
       </c>
       <c r="I30" t="n">
-        <v>61.84588844163311</v>
+        <v>64.09405255878286</v>
       </c>
       <c r="J30" t="n">
         <v>80</v>
@@ -2627,7 +2627,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M30" t="n">
@@ -2637,10 +2637,10 @@
         <v>80</v>
       </c>
       <c r="O30" t="n">
-        <v>53.19148936170212</v>
+        <v>51.06382978723404</v>
       </c>
       <c r="P30" t="n">
-        <v>63.59029787234042</v>
+        <v>63.1647659574468</v>
       </c>
       <c r="Q30" t="b">
         <v>0</v>
@@ -2664,48 +2664,48 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>39.9</v>
+        <v>41.1</v>
       </c>
       <c r="D31" t="n">
-        <v>0.0505529225908374</v>
+        <v>0.0844327176781003</v>
       </c>
       <c r="E31" t="n">
-        <v>-0.07166123778501619</v>
+        <v>-0.0272189349112426</v>
       </c>
       <c r="F31" t="n">
-        <v>-0.1397153945666236</v>
+        <v>-0.1014429383471797</v>
       </c>
       <c r="G31" t="n">
-        <v>-0.1062029135692741</v>
+        <v>-0.0747139101742984</v>
       </c>
       <c r="H31" t="n">
-        <v>-0.1324993622627277</v>
+        <v>-0.09678057785817711</v>
       </c>
       <c r="I31" t="n">
-        <v>68.38407494145198</v>
+        <v>71.54899894625922</v>
       </c>
       <c r="J31" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K31" t="n">
         <v>48.99</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M31" t="n">
         <v>48.99</v>
       </c>
       <c r="N31" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O31" t="n">
-        <v>36.17021276595745</v>
+        <v>38.29787234042553</v>
       </c>
       <c r="P31" t="n">
-        <v>58.8300425531915</v>
+        <v>55.25557446808512</v>
       </c>
       <c r="Q31" t="b">
         <v>0</v>
@@ -2729,25 +2729,25 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>723.25</v>
+        <v>737.6</v>
       </c>
       <c r="D32" t="n">
-        <v>0.0534556842181925</v>
+        <v>0.1297289018226375</v>
       </c>
       <c r="E32" t="n">
-        <v>0.0729120308559561</v>
+        <v>0.1285189718482251</v>
       </c>
       <c r="F32" t="n">
-        <v>-0.30215167888846</v>
+        <v>-0.2801795647506587</v>
       </c>
       <c r="G32" t="n">
-        <v>-0.2686391978911105</v>
+        <v>-0.2534505365777774</v>
       </c>
       <c r="H32" t="n">
-        <v>-0.2949356465845641</v>
+        <v>-0.2755172042616561</v>
       </c>
       <c r="I32" t="n">
-        <v>67.32402912621359</v>
+        <v>69.67905405405405</v>
       </c>
       <c r="J32" t="n">
         <v>80</v>
@@ -2757,7 +2757,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M32" t="n">
@@ -2794,25 +2794,25 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>594.65</v>
+        <v>600</v>
       </c>
       <c r="D33" t="n">
-        <v>0.09320709624046319</v>
+        <v>0.142204454597373</v>
       </c>
       <c r="E33" t="n">
-        <v>0.0226139294926912</v>
+        <v>0.0527239231511535</v>
       </c>
       <c r="F33" t="n">
-        <v>0.1291180100636095</v>
+        <v>0.1427483096847921</v>
       </c>
       <c r="G33" t="n">
-        <v>0.162630491060959</v>
+        <v>0.1694773378576735</v>
       </c>
       <c r="H33" t="n">
-        <v>0.1363340423675054</v>
+        <v>0.1474106701737947</v>
       </c>
       <c r="I33" t="n">
-        <v>73.09605817068504</v>
+        <v>73.20884146341464</v>
       </c>
       <c r="J33" t="n">
         <v>70</v>
@@ -2822,7 +2822,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M33" t="n">
@@ -2871,10 +2871,10 @@
         <v>-0.2401052253975846</v>
       </c>
       <c r="G34" t="n">
-        <v>-0.2065927444002351</v>
+        <v>-0.2133761972247032</v>
       </c>
       <c r="H34" t="n">
-        <v>-0.2328891930936887</v>
+        <v>-0.235442864908582</v>
       </c>
       <c r="I34" t="n">
         <v>63.3225806451613</v>
@@ -2887,7 +2887,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M34" t="n">
@@ -2924,48 +2924,48 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>113.72</v>
+        <v>116.42</v>
       </c>
       <c r="D35" t="n">
-        <v>0.0419644493311344</v>
+        <v>0.1079177769318615</v>
       </c>
       <c r="E35" t="n">
-        <v>-0.0166882836143537</v>
+        <v>0.009713790112749299</v>
       </c>
       <c r="F35" t="n">
-        <v>0.2714669051878353</v>
+        <v>0.2892580287929125</v>
       </c>
       <c r="G35" t="n">
-        <v>0.3049793861851848</v>
+        <v>0.3159870569657939</v>
       </c>
       <c r="H35" t="n">
-        <v>0.2786829374917312</v>
+        <v>0.2939203892819151</v>
       </c>
       <c r="I35" t="n">
-        <v>56.86274509803921</v>
+        <v>64.76702508960574</v>
       </c>
       <c r="J35" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K35" t="n">
         <v>49.07</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M35" t="n">
         <v>49.07</v>
       </c>
       <c r="N35" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O35" t="n">
         <v>87.2340425531915</v>
       </c>
       <c r="P35" t="n">
-        <v>61.07480851063831</v>
+        <v>69.07480851063831</v>
       </c>
       <c r="Q35" t="b">
         <v>0</v>
@@ -2989,48 +2989,48 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>471.25</v>
+        <v>504.4</v>
       </c>
       <c r="D36" t="n">
-        <v>0.0134408602150537</v>
+        <v>0.0901231899719039</v>
       </c>
       <c r="E36" t="n">
-        <v>-0.049132364810331</v>
+        <v>0.0303339801858848</v>
       </c>
       <c r="F36" t="n">
-        <v>-0.0043312909359813</v>
+        <v>0.053797137783349</v>
       </c>
       <c r="G36" t="n">
-        <v>0.0291811900613681</v>
+        <v>0.0805261659562304</v>
       </c>
       <c r="H36" t="n">
-        <v>0.0028847413679145</v>
+        <v>0.0584594982723516</v>
       </c>
       <c r="I36" t="n">
-        <v>52.03380876914951</v>
+        <v>62.96900489396409</v>
       </c>
       <c r="J36" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="K36" t="n">
         <v>47.8</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M36" t="n">
         <v>47.8</v>
       </c>
       <c r="N36" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="O36" t="n">
-        <v>59.57446808510638</v>
+        <v>63.82978723404256</v>
       </c>
       <c r="P36" t="n">
-        <v>47.03489361702128</v>
+        <v>63.88595744680852</v>
       </c>
       <c r="Q36" t="b">
         <v>0</v>
@@ -3054,48 +3054,48 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2530.7</v>
+        <v>2602.4</v>
       </c>
       <c r="D37" t="n">
-        <v>0.1592762253779203</v>
+        <v>0.2052612078547611</v>
       </c>
       <c r="E37" t="n">
-        <v>0.5236002408187836</v>
+        <v>0.5805648344974188</v>
       </c>
       <c r="F37" t="n">
-        <v>0.741227466629971</v>
+        <v>0.8089809537049912</v>
       </c>
       <c r="G37" t="n">
-        <v>0.7747399476273205</v>
+        <v>0.8357099818778726</v>
       </c>
       <c r="H37" t="n">
-        <v>0.7484434989338669</v>
+        <v>0.8136433141939938</v>
       </c>
       <c r="I37" t="n">
-        <v>78.30092118730811</v>
+        <v>80.17632914774248</v>
       </c>
       <c r="J37" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="K37" t="n">
         <v>48.59</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M37" t="n">
         <v>48.59</v>
       </c>
       <c r="N37" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="O37" t="n">
         <v>100</v>
       </c>
       <c r="P37" t="n">
-        <v>67.43600000000001</v>
+        <v>63.43600000000001</v>
       </c>
       <c r="Q37" t="b">
         <v>0</v>
@@ -3119,25 +3119,25 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>845</v>
+        <v>872.45</v>
       </c>
       <c r="D38" t="n">
-        <v>0.0626925737282273</v>
+        <v>0.1523576806234314</v>
       </c>
       <c r="E38" t="n">
-        <v>0.0058925063984287</v>
+        <v>0.0612455905607589</v>
       </c>
       <c r="F38" t="n">
-        <v>-0.2146110233293058</v>
+        <v>-0.1818735933983496</v>
       </c>
       <c r="G38" t="n">
-        <v>-0.1810985423319563</v>
+        <v>-0.1551445652254682</v>
       </c>
       <c r="H38" t="n">
-        <v>-0.2073949910254099</v>
+        <v>-0.177211232909347</v>
       </c>
       <c r="I38" t="n">
-        <v>72.51077341800861</v>
+        <v>74.07486631016043</v>
       </c>
       <c r="J38" t="n">
         <v>70</v>
@@ -3147,7 +3147,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M38" t="n">
@@ -3157,10 +3157,10 @@
         <v>70</v>
       </c>
       <c r="O38" t="n">
-        <v>12.76595744680851</v>
+        <v>19.14893617021277</v>
       </c>
       <c r="P38" t="n">
-        <v>50.5011914893617</v>
+        <v>51.77778723404256</v>
       </c>
       <c r="Q38" t="b">
         <v>0</v>
@@ -3184,25 +3184,25 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>3478.7</v>
+        <v>3569.2</v>
       </c>
       <c r="D39" t="n">
-        <v>0.1214016311530898</v>
+        <v>0.1765946925993076</v>
       </c>
       <c r="E39" t="n">
-        <v>0.2882642669333035</v>
+        <v>0.3250176337379813</v>
       </c>
       <c r="F39" t="n">
-        <v>0.2815723548482167</v>
+        <v>0.3059641419685326</v>
       </c>
       <c r="G39" t="n">
-        <v>0.3150848358455662</v>
+        <v>0.332693170141414</v>
       </c>
       <c r="H39" t="n">
-        <v>0.2887883871521126</v>
+        <v>0.3106265024575352</v>
       </c>
       <c r="I39" t="n">
-        <v>73.04347826086955</v>
+        <v>74.81996315525035</v>
       </c>
       <c r="J39" t="n">
         <v>70</v>
@@ -3212,7 +3212,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M39" t="n">
@@ -3249,25 +3249,25 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>207.89</v>
+        <v>210.31</v>
       </c>
       <c r="D40" t="n">
-        <v>0.1187708535141534</v>
+        <v>0.1751131474548808</v>
       </c>
       <c r="E40" t="n">
-        <v>0.1576456175520657</v>
+        <v>0.08799793067770301</v>
       </c>
       <c r="F40" t="n">
-        <v>-0.070134633448137</v>
+        <v>-0.0424786013476596</v>
       </c>
       <c r="G40" t="n">
-        <v>-0.0366221524507875</v>
+        <v>-0.0157495731747783</v>
       </c>
       <c r="H40" t="n">
-        <v>-0.0629186011442411</v>
+        <v>-0.037816240858657</v>
       </c>
       <c r="I40" t="n">
-        <v>68.97590361445781</v>
+        <v>69.93954554930163</v>
       </c>
       <c r="J40" t="n">
         <v>80</v>
@@ -3277,7 +3277,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M40" t="n">
@@ -3314,48 +3314,48 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>801.55</v>
+        <v>818.6</v>
       </c>
       <c r="D41" t="n">
-        <v>0.0031914893617019</v>
+        <v>0.0733626171900609</v>
       </c>
       <c r="E41" t="n">
-        <v>-0.1196595277320153</v>
+        <v>-0.09781231057475059</v>
       </c>
       <c r="F41" t="n">
-        <v>-0.2026758181637322</v>
+        <v>-0.1846207480452214</v>
       </c>
       <c r="G41" t="n">
-        <v>-0.1691633371663827</v>
+        <v>-0.15789171987234</v>
       </c>
       <c r="H41" t="n">
-        <v>-0.1954597858598363</v>
+        <v>-0.1799583875562188</v>
       </c>
       <c r="I41" t="n">
-        <v>61.06583072100312</v>
+        <v>71.37511693171189</v>
       </c>
       <c r="J41" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="K41" t="n">
         <v>48.05</v>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M41" t="n">
         <v>48.05</v>
       </c>
       <c r="N41" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="O41" t="n">
-        <v>19.14893617021277</v>
+        <v>17.02127659574468</v>
       </c>
       <c r="P41" t="n">
-        <v>47.04978723404256</v>
+        <v>42.62425531914894</v>
       </c>
       <c r="Q41" t="b">
         <v>0</v>
@@ -3379,48 +3379,48 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>617.55</v>
+        <v>605.3</v>
       </c>
       <c r="D42" t="n">
-        <v>0.175054704595186</v>
+        <v>0.2203629032258063</v>
       </c>
       <c r="E42" t="n">
-        <v>0.0398215187742043</v>
+        <v>0.0427217915590008</v>
       </c>
       <c r="F42" t="n">
-        <v>-0.1941671559992172</v>
+        <v>-0.216490842016698</v>
       </c>
       <c r="G42" t="n">
-        <v>-0.1606546750018677</v>
+        <v>-0.1897618138438166</v>
       </c>
       <c r="H42" t="n">
-        <v>-0.1869511236953213</v>
+        <v>-0.2118284815276954</v>
       </c>
       <c r="I42" t="n">
-        <v>72.20066518847</v>
+        <v>69.42963752665241</v>
       </c>
       <c r="J42" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K42" t="n">
         <v>47.66</v>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M42" t="n">
         <v>47.66</v>
       </c>
       <c r="N42" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O42" t="n">
-        <v>23.40425531914894</v>
+        <v>12.76595744680851</v>
       </c>
       <c r="P42" t="n">
-        <v>51.74485106382978</v>
+        <v>53.6171914893617</v>
       </c>
       <c r="Q42" t="b">
         <v>0</v>
@@ -3444,48 +3444,48 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>417.25</v>
+        <v>424.25</v>
       </c>
       <c r="D43" t="n">
-        <v>0.0165671823608235</v>
+        <v>0.0236457956327662</v>
       </c>
       <c r="E43" t="n">
-        <v>0.0054216867469878</v>
+        <v>0.0319873510094865</v>
       </c>
       <c r="F43" t="n">
-        <v>-0.0721592172559484</v>
+        <v>-0.0553328879982186</v>
       </c>
       <c r="G43" t="n">
-        <v>-0.0386467362585989</v>
+        <v>-0.0286038598253373</v>
       </c>
       <c r="H43" t="n">
-        <v>-0.06494318495205249</v>
+        <v>-0.050670527509216</v>
       </c>
       <c r="I43" t="n">
-        <v>51.78323297823067</v>
+        <v>52.74625510667272</v>
       </c>
       <c r="J43" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="K43" t="n">
         <v>51.48</v>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M43" t="n">
         <v>51.48</v>
       </c>
       <c r="N43" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="O43" t="n">
-        <v>46.80851063829788</v>
+        <v>42.5531914893617</v>
       </c>
       <c r="P43" t="n">
-        <v>45.95370212765958</v>
+        <v>61.10263829787234</v>
       </c>
       <c r="Q43" t="b">
         <v>0</v>
@@ -3509,25 +3509,25 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>277.78</v>
+        <v>295.37</v>
       </c>
       <c r="D44" t="n">
-        <v>0.1627459187944746</v>
+        <v>0.2676824034334764</v>
       </c>
       <c r="E44" t="n">
-        <v>0.1275827075299369</v>
+        <v>0.2481301500105641</v>
       </c>
       <c r="F44" t="n">
-        <v>-0.0398202557898377</v>
+        <v>0.0342086834733892</v>
       </c>
       <c r="G44" t="n">
-        <v>-0.0063077747924882</v>
+        <v>0.0609377116462706</v>
       </c>
       <c r="H44" t="n">
-        <v>-0.0326042234859418</v>
+        <v>0.0388710439623918</v>
       </c>
       <c r="I44" t="n">
-        <v>84.51015004413055</v>
+        <v>88.34080717488784</v>
       </c>
       <c r="J44" t="n">
         <v>60</v>
@@ -3537,7 +3537,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M44" t="n">
@@ -3547,16 +3547,16 @@
         <v>60</v>
       </c>
       <c r="O44" t="n">
-        <v>55.31914893617022</v>
+        <v>61.70212765957447</v>
       </c>
       <c r="P44" t="n">
-        <v>53.94382978723405</v>
+        <v>55.2204255319149</v>
       </c>
       <c r="Q44" t="b">
         <v>0</v>
       </c>
       <c r="R44" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S44" t="b">
         <v>0</v>
@@ -3574,48 +3574,48 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>102.66</v>
+        <v>100.61</v>
       </c>
       <c r="D45" t="n">
-        <v>0.1118812953536227</v>
+        <v>0.1624494511842866</v>
       </c>
       <c r="E45" t="n">
-        <v>-0.06867458949469291</v>
+        <v>-0.0592800374006545</v>
       </c>
       <c r="F45" t="n">
-        <v>-0.2280622603203249</v>
+        <v>-0.2425656854626214</v>
       </c>
       <c r="G45" t="n">
-        <v>-0.1945497793229754</v>
+        <v>-0.2158366572897401</v>
       </c>
       <c r="H45" t="n">
-        <v>-0.220846228016429</v>
+        <v>-0.2379033249736188</v>
       </c>
       <c r="I45" t="n">
-        <v>73.73926036608142</v>
+        <v>66.9818181818182</v>
       </c>
       <c r="J45" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K45" t="n">
         <v>59.6</v>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M45" t="n">
         <v>59.6</v>
       </c>
       <c r="N45" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O45" t="n">
-        <v>10.63829787234042</v>
+        <v>4.25531914893617</v>
       </c>
       <c r="P45" t="n">
-        <v>53.96765957446809</v>
+        <v>56.69106382978724</v>
       </c>
       <c r="Q45" t="b">
         <v>0</v>
@@ -3639,48 +3639,48 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>512.25</v>
+        <v>521.35</v>
       </c>
       <c r="D46" t="n">
-        <v>0.03820429671666</v>
+        <v>0.0692165709598031</v>
       </c>
       <c r="E46" t="n">
-        <v>-0.0734376413131953</v>
+        <v>-0.0542403628117913</v>
       </c>
       <c r="F46" t="n">
-        <v>-0.1743230174081237</v>
+        <v>-0.1471454277768689</v>
       </c>
       <c r="G46" t="n">
-        <v>-0.1408105364107742</v>
+        <v>-0.1204163996039875</v>
       </c>
       <c r="H46" t="n">
-        <v>-0.1671069851042278</v>
+        <v>-0.1424830672878663</v>
       </c>
       <c r="I46" t="n">
-        <v>61.39438085327785</v>
+        <v>66.39455782312928</v>
       </c>
       <c r="J46" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K46" t="n">
         <v>49.61</v>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M46" t="n">
         <v>49.61</v>
       </c>
       <c r="N46" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O46" t="n">
         <v>27.65957446808511</v>
       </c>
       <c r="P46" t="n">
-        <v>49.37591489361702</v>
+        <v>57.37591489361702</v>
       </c>
       <c r="Q46" t="b">
         <v>0</v>
@@ -3704,25 +3704,25 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>1047.95</v>
+        <v>1053</v>
       </c>
       <c r="D47" t="n">
-        <v>-0.0381809003717129</v>
+        <v>-0.0268921541447185</v>
       </c>
       <c r="E47" t="n">
-        <v>0.4326042378673957</v>
+        <v>0.4746866465933759</v>
       </c>
       <c r="F47" t="n">
-        <v>0.1903788266030557</v>
+        <v>0.1441299505622861</v>
       </c>
       <c r="G47" t="n">
-        <v>0.2238913076004052</v>
+        <v>0.1708589787351675</v>
       </c>
       <c r="H47" t="n">
-        <v>0.1975948589069516</v>
+        <v>0.1487923110512887</v>
       </c>
       <c r="I47" t="n">
-        <v>69.63096309630966</v>
+        <v>67.72527262291948</v>
       </c>
       <c r="J47" t="n">
         <v>80</v>
@@ -3732,7 +3732,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M47" t="n">
@@ -3742,10 +3742,10 @@
         <v>80</v>
       </c>
       <c r="O47" t="n">
-        <v>80.85106382978722</v>
+        <v>72.3404255319149</v>
       </c>
       <c r="P47" t="n">
-        <v>66.90221276595744</v>
+        <v>65.20008510638299</v>
       </c>
       <c r="Q47" t="b">
         <v>0</v>
@@ -3769,25 +3769,25 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>15002</v>
+        <v>14888</v>
       </c>
       <c r="D48" t="n">
-        <v>0.103737492642731</v>
+        <v>0.0884632256177804</v>
       </c>
       <c r="E48" t="n">
-        <v>0.1065870030242679</v>
+        <v>0.0604743927630173</v>
       </c>
       <c r="F48" t="n">
-        <v>0.1065053842749668</v>
+        <v>0.1223520542781757</v>
       </c>
       <c r="G48" t="n">
-        <v>0.1400178652723163</v>
+        <v>0.1490810824510571</v>
       </c>
       <c r="H48" t="n">
-        <v>0.1137214165788627</v>
+        <v>0.1270144147671783</v>
       </c>
       <c r="I48" t="n">
-        <v>68.91160553217077</v>
+        <v>68.5201793721973</v>
       </c>
       <c r="J48" t="n">
         <v>80</v>
@@ -3797,7 +3797,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M48" t="n">
@@ -3936,57 +3936,57 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>GNA</t>
+          <t>LUMAXTECH</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Axles</t>
+          <t>Lighting</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>429.3</v>
+        <v>1747.6</v>
       </c>
       <c r="D2" t="n">
-        <v>0.08368042408178721</v>
+        <v>0.0862754848334161</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2528819495111631</v>
+        <v>0.2897416974169742</v>
       </c>
       <c r="F2" t="n">
-        <v>0.3866279069767442</v>
+        <v>0.4163222303266065</v>
       </c>
       <c r="G2" t="n">
-        <v>0.4201403879740937</v>
+        <v>0.4430512584994879</v>
       </c>
       <c r="H2" t="n">
-        <v>0.3938439392806401</v>
+        <v>0.4209845908156091</v>
       </c>
       <c r="I2" t="n">
-        <v>68.63583365720947</v>
+        <v>63.05350553505533</v>
       </c>
       <c r="J2" t="n">
         <v>80</v>
       </c>
       <c r="K2" t="n">
-        <v>54.47</v>
+        <v>54.51</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M2" t="n">
-        <v>54.47</v>
+        <v>54.51</v>
       </c>
       <c r="N2" t="n">
         <v>80</v>
       </c>
       <c r="O2" t="n">
-        <v>95.74468085106383</v>
+        <v>91.48936170212764</v>
       </c>
       <c r="P2" t="n">
-        <v>72.93693617021276</v>
+        <v>72.10187234042553</v>
       </c>
       <c r="Q2" t="b">
         <v>0</v>
@@ -4001,57 +4001,57 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>LUMAXTECH</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Lighting</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1727</v>
+        <v>588.65</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0638822152405593</v>
+        <v>0.204398976982097</v>
       </c>
       <c r="E3" t="n">
-        <v>0.2536295005807201</v>
+        <v>0.2067445674456745</v>
       </c>
       <c r="F3" t="n">
-        <v>0.3721595423486414</v>
+        <v>0.4525601480567549</v>
       </c>
       <c r="G3" t="n">
-        <v>0.4056720233459909</v>
+        <v>0.4792891762296363</v>
       </c>
       <c r="H3" t="n">
-        <v>0.3793755746525373</v>
+        <v>0.4572225085457575</v>
       </c>
       <c r="I3" t="n">
-        <v>57.3502722323049</v>
+        <v>69.7262479871175</v>
       </c>
       <c r="J3" t="n">
         <v>80</v>
       </c>
       <c r="K3" t="n">
-        <v>54.51</v>
+        <v>49.66</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M3" t="n">
-        <v>54.51</v>
+        <v>49.66</v>
       </c>
       <c r="N3" t="n">
         <v>80</v>
       </c>
       <c r="O3" t="n">
-        <v>93.61702127659576</v>
+        <v>95.74468085106383</v>
       </c>
       <c r="P3" t="n">
-        <v>72.52740425531915</v>
+        <v>71.01293617021277</v>
       </c>
       <c r="Q3" t="b">
         <v>0</v>
@@ -4066,57 +4066,57 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Forgings</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>564.85</v>
+        <v>1901.1</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1044090331410696</v>
+        <v>0.1020230711263114</v>
       </c>
       <c r="E4" t="n">
-        <v>0.2384345538259153</v>
+        <v>0.3402185407120197</v>
       </c>
       <c r="F4" t="n">
-        <v>0.3642072213500784</v>
+        <v>0.5962216624685137</v>
       </c>
       <c r="G4" t="n">
-        <v>0.3977197023474279</v>
+        <v>0.6229506906413951</v>
       </c>
       <c r="H4" t="n">
-        <v>0.3714232536539743</v>
+        <v>0.6008840229575163</v>
       </c>
       <c r="I4" t="n">
-        <v>66.4784546805349</v>
+        <v>78.14796668299851</v>
       </c>
       <c r="J4" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K4" t="n">
-        <v>49.66</v>
+        <v>54.83</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M4" t="n">
-        <v>49.66</v>
+        <v>54.83</v>
       </c>
       <c r="N4" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O4" t="n">
-        <v>91.48936170212764</v>
+        <v>97.87234042553192</v>
       </c>
       <c r="P4" t="n">
-        <v>70.16187234042553</v>
+        <v>69.50646808510639</v>
       </c>
       <c r="Q4" t="b">
         <v>0</v>
@@ -4131,57 +4131,57 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>RICOAUTO</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Forgings</t>
+          <t>Castings</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1856</v>
+        <v>116.42</v>
       </c>
       <c r="D5" t="n">
-        <v>0.0688165850849409</v>
+        <v>0.1079177769318615</v>
       </c>
       <c r="E5" t="n">
-        <v>0.3174332765474164</v>
+        <v>0.009713790112749299</v>
       </c>
       <c r="F5" t="n">
-        <v>0.5253122945430639</v>
+        <v>0.2892580287929125</v>
       </c>
       <c r="G5" t="n">
-        <v>0.5588247755404134</v>
+        <v>0.3159870569657939</v>
       </c>
       <c r="H5" t="n">
-        <v>0.5325283268469598</v>
+        <v>0.2939203892819151</v>
       </c>
       <c r="I5" t="n">
-        <v>75.48103353490929</v>
+        <v>64.76702508960574</v>
       </c>
       <c r="J5" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K5" t="n">
-        <v>54.83</v>
+        <v>49.07</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M5" t="n">
-        <v>54.83</v>
+        <v>49.07</v>
       </c>
       <c r="N5" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O5" t="n">
-        <v>97.87234042553192</v>
+        <v>87.2340425531915</v>
       </c>
       <c r="P5" t="n">
-        <v>69.50646808510639</v>
+        <v>69.07480851063831</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
@@ -4196,57 +4196,57 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SANSERA</t>
+          <t>AUTOAXLES</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Forgings</t>
+          <t>Axles</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>2530.7</v>
+        <v>1877.9</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1592762253779203</v>
+        <v>0.1844960262394348</v>
       </c>
       <c r="E6" t="n">
-        <v>0.5236002408187836</v>
+        <v>-0.0340020576131686</v>
       </c>
       <c r="F6" t="n">
-        <v>0.741227466629971</v>
+        <v>0.0899645945789076</v>
       </c>
       <c r="G6" t="n">
-        <v>0.7747399476273205</v>
+        <v>0.1166936227517889</v>
       </c>
       <c r="H6" t="n">
-        <v>0.7484434989338669</v>
+        <v>0.09462695506791011</v>
       </c>
       <c r="I6" t="n">
-        <v>78.30092118730811</v>
+        <v>69.02985074626865</v>
       </c>
       <c r="J6" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K6" t="n">
-        <v>48.59</v>
+        <v>58.77</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M6" t="n">
-        <v>48.59</v>
+        <v>58.77</v>
       </c>
       <c r="N6" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O6" t="n">
-        <v>100</v>
+        <v>65.95744680851064</v>
       </c>
       <c r="P6" t="n">
-        <v>67.43600000000001</v>
+        <v>68.69948936170213</v>
       </c>
       <c r="Q6" t="b">
         <v>0</v>
@@ -4261,57 +4261,57 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>FIEMIND</t>
+          <t>GNA</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Lighting</t>
+          <t>Axles</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2175</v>
+        <v>440.6</v>
       </c>
       <c r="D7" t="n">
-        <v>0.0438663851027067</v>
+        <v>0.1660711922720656</v>
       </c>
       <c r="E7" t="n">
-        <v>0.0137024608501119</v>
+        <v>0.2943595769682727</v>
       </c>
       <c r="F7" t="n">
-        <v>0.1344669309409556</v>
+        <v>0.4187731444211882</v>
       </c>
       <c r="G7" t="n">
-        <v>0.1679794119383051</v>
+        <v>0.4455021725940695</v>
       </c>
       <c r="H7" t="n">
-        <v>0.1416829632448515</v>
+        <v>0.4234355049101908</v>
       </c>
       <c r="I7" t="n">
-        <v>65.25526742301457</v>
+        <v>72.01735357917572</v>
       </c>
       <c r="J7" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K7" t="n">
-        <v>49.06</v>
+        <v>54.47</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M7" t="n">
-        <v>49.06</v>
+        <v>54.47</v>
       </c>
       <c r="N7" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="O7" t="n">
-        <v>76.59574468085107</v>
+        <v>93.61702127659576</v>
       </c>
       <c r="P7" t="n">
-        <v>66.94314893617022</v>
+        <v>68.51140425531915</v>
       </c>
       <c r="Q7" t="b">
         <v>0</v>
@@ -4326,57 +4326,57 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>WHEELS</t>
+          <t>FIEMIND</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Wheels</t>
+          <t>Lighting</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1047.95</v>
+        <v>2211.4</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.0381809003717129</v>
+        <v>0.1247647627282437</v>
       </c>
       <c r="E8" t="n">
-        <v>0.4326042378673957</v>
+        <v>0.0466183917838043</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1903788266030557</v>
+        <v>0.1594400461385205</v>
       </c>
       <c r="G8" t="n">
-        <v>0.2238913076004052</v>
+        <v>0.1861690743114019</v>
       </c>
       <c r="H8" t="n">
-        <v>0.1975948589069516</v>
+        <v>0.1641024066275231</v>
       </c>
       <c r="I8" t="n">
-        <v>69.63096309630966</v>
+        <v>67.23347344287353</v>
       </c>
       <c r="J8" t="n">
         <v>80</v>
       </c>
       <c r="K8" t="n">
-        <v>46.83</v>
+        <v>49.06</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M8" t="n">
-        <v>46.83</v>
+        <v>49.06</v>
       </c>
       <c r="N8" t="n">
         <v>80</v>
       </c>
       <c r="O8" t="n">
-        <v>80.85106382978722</v>
+        <v>78.72340425531915</v>
       </c>
       <c r="P8" t="n">
-        <v>66.90221276595744</v>
+        <v>67.36868085106383</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
@@ -4400,25 +4400,25 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>15002</v>
+        <v>14888</v>
       </c>
       <c r="D9" t="n">
-        <v>0.103737492642731</v>
+        <v>0.0884632256177804</v>
       </c>
       <c r="E9" t="n">
-        <v>0.1065870030242679</v>
+        <v>0.0604743927630173</v>
       </c>
       <c r="F9" t="n">
-        <v>0.1065053842749668</v>
+        <v>0.1223520542781757</v>
       </c>
       <c r="G9" t="n">
-        <v>0.1400178652723163</v>
+        <v>0.1490810824510571</v>
       </c>
       <c r="H9" t="n">
-        <v>0.1137214165788627</v>
+        <v>0.1270144147671783</v>
       </c>
       <c r="I9" t="n">
-        <v>68.91160553217077</v>
+        <v>68.5201793721973</v>
       </c>
       <c r="J9" t="n">
         <v>80</v>
@@ -4428,7 +4428,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M9" t="n">
@@ -4465,25 +4465,25 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>3478.7</v>
+        <v>3569.2</v>
       </c>
       <c r="D10" t="n">
-        <v>0.1214016311530898</v>
+        <v>0.1765946925993076</v>
       </c>
       <c r="E10" t="n">
-        <v>0.2882642669333035</v>
+        <v>0.3250176337379813</v>
       </c>
       <c r="F10" t="n">
-        <v>0.2815723548482167</v>
+        <v>0.3059641419685326</v>
       </c>
       <c r="G10" t="n">
-        <v>0.3150848358455662</v>
+        <v>0.332693170141414</v>
       </c>
       <c r="H10" t="n">
-        <v>0.2887883871521126</v>
+        <v>0.3106265024575352</v>
       </c>
       <c r="I10" t="n">
-        <v>73.04347826086955</v>
+        <v>74.81996315525035</v>
       </c>
       <c r="J10" t="n">
         <v>70</v>
@@ -4493,7 +4493,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M10" t="n">
@@ -4530,25 +4530,25 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>125.7</v>
+        <v>127.93</v>
       </c>
       <c r="D11" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.169592247211556</v>
       </c>
       <c r="E11" t="n">
-        <v>0.1595940959409594</v>
+        <v>0.1664994984954864</v>
       </c>
       <c r="F11" t="n">
-        <v>0.2072608528620823</v>
+        <v>0.2586580086580088</v>
       </c>
       <c r="G11" t="n">
-        <v>0.2407733338594317</v>
+        <v>0.2853870368308902</v>
       </c>
       <c r="H11" t="n">
-        <v>0.2144768851659781</v>
+        <v>0.2633203691470114</v>
       </c>
       <c r="I11" t="n">
-        <v>70.17584451642759</v>
+        <v>71.52639717252046</v>
       </c>
       <c r="J11" t="n">
         <v>70</v>
@@ -4558,7 +4558,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M11" t="n">
@@ -4586,57 +4586,57 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CRAFTSMAN</t>
+          <t>WHEELS</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Castings</t>
+          <t>Wheels</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>7570</v>
+        <v>1053</v>
       </c>
       <c r="D12" t="n">
-        <v>0.0739111930770322</v>
+        <v>-0.0268921541447185</v>
       </c>
       <c r="E12" t="n">
-        <v>0.0516079738834478</v>
+        <v>0.4746866465933759</v>
       </c>
       <c r="F12" t="n">
-        <v>0.1321319075749645</v>
+        <v>0.1441299505622861</v>
       </c>
       <c r="G12" t="n">
-        <v>0.165644388572314</v>
+        <v>0.1708589787351675</v>
       </c>
       <c r="H12" t="n">
-        <v>0.1393479398788604</v>
+        <v>0.1487923110512887</v>
       </c>
       <c r="I12" t="n">
-        <v>77.69582016157359</v>
+        <v>67.72527262291948</v>
       </c>
       <c r="J12" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K12" t="n">
-        <v>54.65</v>
+        <v>46.83</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M12" t="n">
-        <v>54.65</v>
+        <v>46.83</v>
       </c>
       <c r="N12" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O12" t="n">
         <v>72.3404255319149</v>
       </c>
       <c r="P12" t="n">
-        <v>64.32808510638299</v>
+        <v>65.20008510638299</v>
       </c>
       <c r="Q12" t="b">
         <v>0</v>
@@ -4651,57 +4651,57 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>DIVGIITTS</t>
+          <t>BHARATGEAR</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Transmission</t>
+          <t>Gears</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>752.5</v>
+        <v>109.75</v>
       </c>
       <c r="D13" t="n">
-        <v>0.07862108507131089</v>
+        <v>0.2274913320657645</v>
       </c>
       <c r="E13" t="n">
-        <v>0.2626898229717258</v>
+        <v>0.0238828248903815</v>
       </c>
       <c r="F13" t="n">
-        <v>0.1508755830848054</v>
+        <v>0.1909929462832338</v>
       </c>
       <c r="G13" t="n">
-        <v>0.1843880640821549</v>
+        <v>0.2177219744561151</v>
       </c>
       <c r="H13" t="n">
-        <v>0.1580916153887013</v>
+        <v>0.1956553067722364</v>
       </c>
       <c r="I13" t="n">
-        <v>73.06209850107068</v>
+        <v>76.79856115107913</v>
       </c>
       <c r="J13" t="n">
         <v>70</v>
       </c>
       <c r="K13" t="n">
-        <v>49.92</v>
+        <v>51.91</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M13" t="n">
-        <v>49.92</v>
+        <v>51.91</v>
       </c>
       <c r="N13" t="n">
         <v>70</v>
       </c>
       <c r="O13" t="n">
-        <v>78.72340425531915</v>
+        <v>80.85106382978722</v>
       </c>
       <c r="P13" t="n">
-        <v>63.71268085106384</v>
+        <v>64.93421276595744</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
@@ -4716,57 +4716,57 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>BHARATGEAR</t>
+          <t>SANDHAR</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Gears</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>108.47</v>
+        <v>504.4</v>
       </c>
       <c r="D14" t="n">
-        <v>0.1333194023612998</v>
+        <v>0.0901231899719039</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.0090443997807417</v>
+        <v>0.0303339801858848</v>
       </c>
       <c r="F14" t="n">
-        <v>0.132372899050005</v>
+        <v>0.053797137783349</v>
       </c>
       <c r="G14" t="n">
-        <v>0.1658853800473545</v>
+        <v>0.0805261659562304</v>
       </c>
       <c r="H14" t="n">
-        <v>0.1395889313539009</v>
+        <v>0.0584594982723516</v>
       </c>
       <c r="I14" t="n">
-        <v>76.72320461927102</v>
+        <v>62.96900489396409</v>
       </c>
       <c r="J14" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K14" t="n">
-        <v>51.91</v>
+        <v>47.8</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M14" t="n">
-        <v>51.91</v>
+        <v>47.8</v>
       </c>
       <c r="N14" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O14" t="n">
-        <v>74.46808510638297</v>
+        <v>63.82978723404256</v>
       </c>
       <c r="P14" t="n">
-        <v>63.65761702127659</v>
+        <v>63.88595744680852</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
@@ -4781,63 +4781,63 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>MENONBE</t>
+          <t>SANSERA</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Bearings</t>
+          <t>Forgings</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>118.74</v>
+        <v>2602.4</v>
       </c>
       <c r="D15" t="n">
-        <v>0.0607468286582097</v>
+        <v>0.2052612078547611</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.0266415279940979</v>
+        <v>0.5805648344974188</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.052051732396615</v>
+        <v>0.8089809537049912</v>
       </c>
       <c r="G15" t="n">
-        <v>-0.0185392513992656</v>
+        <v>0.8357099818778726</v>
       </c>
       <c r="H15" t="n">
-        <v>-0.0448357000927192</v>
+        <v>0.8136433141939938</v>
       </c>
       <c r="I15" t="n">
-        <v>61.84588844163311</v>
+        <v>80.17632914774248</v>
       </c>
       <c r="J15" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K15" t="n">
-        <v>52.38</v>
+        <v>48.59</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M15" t="n">
-        <v>52.38</v>
+        <v>48.59</v>
       </c>
       <c r="N15" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O15" t="n">
-        <v>53.19148936170212</v>
+        <v>100</v>
       </c>
       <c r="P15" t="n">
-        <v>63.59029787234042</v>
+        <v>63.43600000000001</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
       </c>
       <c r="R15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S15" t="b">
         <v>0</v>
@@ -4846,57 +4846,57 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>PRICOLLTD</t>
+          <t>DIVGIITTS</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Transmission</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>594.65</v>
+        <v>743.8</v>
       </c>
       <c r="D16" t="n">
-        <v>0.09320709624046319</v>
+        <v>0.1023341978510559</v>
       </c>
       <c r="E16" t="n">
-        <v>0.0226139294926912</v>
+        <v>0.2479865771812079</v>
       </c>
       <c r="F16" t="n">
-        <v>0.1291180100636095</v>
+        <v>0.1549689440993789</v>
       </c>
       <c r="G16" t="n">
-        <v>0.162630491060959</v>
+        <v>0.1816979722722602</v>
       </c>
       <c r="H16" t="n">
-        <v>0.1363340423675054</v>
+        <v>0.1596313045883814</v>
       </c>
       <c r="I16" t="n">
-        <v>73.09605817068504</v>
+        <v>71.23173277661793</v>
       </c>
       <c r="J16" t="n">
         <v>70</v>
       </c>
       <c r="K16" t="n">
-        <v>49.98</v>
+        <v>49.92</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="M16" t="n">
-        <v>49.98</v>
+        <v>49.92</v>
       </c>
       <c r="N16" t="n">
         <v>70</v>
       </c>
       <c r="O16" t="n">
-        <v>70.21276595744681</v>
+        <v>76.59574468085107</v>
       </c>
       <c r="P16" t="n">
-        <v>62.03455319148937</v>
+        <v>63.28714893617022</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
chore: auto-refresh NSE data and pipeline outputs (2026-04-28)
</commit_message>
<xml_diff>
--- a/working-sector/output/auto_components_comprehensive_report.xlsx
+++ b/working-sector/output/auto_components_comprehensive_report.xlsx
@@ -435,7 +435,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -447,7 +447,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -779,48 +779,48 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1901.1</v>
+        <v>1894.8</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1020230711263114</v>
+        <v>0.1314940881404513</v>
       </c>
       <c r="E2" t="n">
-        <v>0.3402185407120197</v>
+        <v>0.2986087314097732</v>
       </c>
       <c r="F2" t="n">
-        <v>0.5962216624685137</v>
+        <v>0.5668568593401142</v>
       </c>
       <c r="G2" t="n">
-        <v>0.6229506906413951</v>
+        <v>0.6028433431494672</v>
       </c>
       <c r="H2" t="n">
-        <v>0.6008840229575163</v>
+        <v>0.578238803694088</v>
       </c>
       <c r="I2" t="n">
-        <v>78.14796668299851</v>
+        <v>68.62680683311432</v>
       </c>
       <c r="J2" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K2" t="n">
         <v>54.83</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="M2" t="n">
         <v>54.83</v>
       </c>
       <c r="N2" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O2" t="n">
         <v>97.87234042553192</v>
       </c>
       <c r="P2" t="n">
-        <v>69.50646808510639</v>
+        <v>73.50646808510639</v>
       </c>
       <c r="Q2" t="b">
         <v>0</v>
@@ -844,25 +844,25 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1130.9</v>
+        <v>1129.7</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0783827596071327</v>
+        <v>0.09509499806126399</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.0123144104803493</v>
+        <v>-0.0164548145568517</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.1376391642519444</v>
+        <v>-0.1034126984126984</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.110910136079063</v>
+        <v>-0.0674262146033454</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.1329768037629418</v>
+        <v>-0.0920307540587246</v>
       </c>
       <c r="I3" t="n">
-        <v>68.85980020668271</v>
+        <v>58.86843286933091</v>
       </c>
       <c r="J3" t="n">
         <v>80</v>
@@ -872,7 +872,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="M3" t="n">
@@ -882,10 +882,10 @@
         <v>80</v>
       </c>
       <c r="O3" t="n">
-        <v>29.78723404255319</v>
+        <v>38.29787234042553</v>
       </c>
       <c r="P3" t="n">
-        <v>57.70144680851064</v>
+        <v>59.40357446808511</v>
       </c>
       <c r="Q3" t="b">
         <v>0</v>
@@ -909,48 +909,48 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>37225</v>
+        <v>37320</v>
       </c>
       <c r="D4" t="n">
-        <v>0.2569643761607294</v>
+        <v>0.2983127500434859</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0542339280657038</v>
+        <v>0.0313665883653446</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.029335071707953</v>
+        <v>-0.0297673209411153</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.0026060435350716</v>
+        <v>0.0062191628682376</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.0246727112189504</v>
+        <v>-0.0183853765871415</v>
       </c>
       <c r="I4" t="n">
-        <v>73.53673723536737</v>
+        <v>62.28926353149956</v>
       </c>
       <c r="J4" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K4" t="n">
         <v>53.48</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="M4" t="n">
         <v>53.48</v>
       </c>
       <c r="N4" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O4" t="n">
-        <v>53.19148936170212</v>
+        <v>48.93617021276596</v>
       </c>
       <c r="P4" t="n">
-        <v>60.03029787234042</v>
+        <v>63.17923404255319</v>
       </c>
       <c r="Q4" t="b">
         <v>0</v>
@@ -974,48 +974,48 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>352.35</v>
+        <v>356.25</v>
       </c>
       <c r="D5" t="n">
-        <v>0.1711816519860396</v>
+        <v>0.2374088225078152</v>
       </c>
       <c r="E5" t="n">
-        <v>0.09002320185614859</v>
+        <v>0.1092947220924802</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.1154763399020961</v>
+        <v>-0.1039989939637827</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.0887473117292148</v>
+        <v>-0.0680125101544297</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.1108139794130935</v>
+        <v>-0.0926170496098089</v>
       </c>
       <c r="I5" t="n">
-        <v>81.37813211845105</v>
+        <v>78.14171122994655</v>
       </c>
       <c r="J5" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K5" t="n">
         <v>51.12</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="M5" t="n">
         <v>51.12</v>
       </c>
       <c r="N5" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O5" t="n">
         <v>36.17021276595745</v>
       </c>
       <c r="P5" t="n">
-        <v>51.68204255319149</v>
+        <v>55.68204255319149</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
@@ -1039,48 +1039,48 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>127.93</v>
+        <v>125.22</v>
       </c>
       <c r="D6" t="n">
-        <v>0.169592247211556</v>
+        <v>0.1916634944803958</v>
       </c>
       <c r="E6" t="n">
-        <v>0.1664994984954864</v>
+        <v>0.1237548236561068</v>
       </c>
       <c r="F6" t="n">
-        <v>0.2586580086580088</v>
+        <v>0.2105568445475638</v>
       </c>
       <c r="G6" t="n">
-        <v>0.2853870368308902</v>
+        <v>0.2465433283569168</v>
       </c>
       <c r="H6" t="n">
-        <v>0.2633203691470114</v>
+        <v>0.2219387889015376</v>
       </c>
       <c r="I6" t="n">
-        <v>71.52639717252046</v>
+        <v>59.27956147220047</v>
       </c>
       <c r="J6" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K6" t="n">
         <v>51.57</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="M6" t="n">
         <v>51.57</v>
       </c>
       <c r="N6" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O6" t="n">
         <v>82.97872340425532</v>
       </c>
       <c r="P6" t="n">
-        <v>65.22374468085107</v>
+        <v>69.22374468085107</v>
       </c>
       <c r="Q6" t="b">
         <v>0</v>
@@ -1104,25 +1104,25 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2994.4</v>
+        <v>3001</v>
       </c>
       <c r="D7" t="n">
-        <v>0.1668160386548727</v>
+        <v>0.1921503197870733</v>
       </c>
       <c r="E7" t="n">
-        <v>0.3677431142374274</v>
+        <v>0.3158240890954533</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.0470371077588949</v>
+        <v>-0.0597192630655469</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.0203080795860135</v>
+        <v>-0.0237327792561939</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.0423747472698923</v>
+        <v>-0.0483373187115732</v>
       </c>
       <c r="I7" t="n">
-        <v>78.80034032898465</v>
+        <v>73.90469540932096</v>
       </c>
       <c r="J7" t="n">
         <v>70</v>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="M7" t="n">
@@ -1169,25 +1169,25 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>588.65</v>
+        <v>598.8</v>
       </c>
       <c r="D8" t="n">
-        <v>0.204398976982097</v>
+        <v>0.243613707165109</v>
       </c>
       <c r="E8" t="n">
-        <v>0.2067445674456745</v>
+        <v>0.211900425015179</v>
       </c>
       <c r="F8" t="n">
-        <v>0.4525601480567549</v>
+        <v>0.3943415997205728</v>
       </c>
       <c r="G8" t="n">
-        <v>0.4792891762296363</v>
+        <v>0.4303280835299258</v>
       </c>
       <c r="H8" t="n">
-        <v>0.4572225085457575</v>
+        <v>0.4057235440745466</v>
       </c>
       <c r="I8" t="n">
-        <v>69.7262479871175</v>
+        <v>68.2967959527824</v>
       </c>
       <c r="J8" t="n">
         <v>80</v>
@@ -1197,7 +1197,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="M8" t="n">
@@ -1207,10 +1207,10 @@
         <v>80</v>
       </c>
       <c r="O8" t="n">
-        <v>95.74468085106383</v>
+        <v>93.61702127659576</v>
       </c>
       <c r="P8" t="n">
-        <v>71.01293617021277</v>
+        <v>70.58740425531916</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
@@ -1234,48 +1234,48 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>428.55</v>
+        <v>423.65</v>
       </c>
       <c r="D9" t="n">
-        <v>0.0390350345496424</v>
+        <v>0.0275284986660198</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.1546503599960548</v>
+        <v>-0.1543912175648703</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.1198398028342574</v>
+        <v>-0.1262246055481077</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.093110774661376</v>
+        <v>-0.0902381217387547</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.1151774423452548</v>
+        <v>-0.114842661194134</v>
       </c>
       <c r="I9" t="n">
-        <v>60.35620052770448</v>
+        <v>39.16449086161877</v>
       </c>
       <c r="J9" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K9" t="n">
         <v>53.44</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="M9" t="n">
         <v>53.44</v>
       </c>
       <c r="N9" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O9" t="n">
-        <v>34.04255319148936</v>
+        <v>31.91489361702128</v>
       </c>
       <c r="P9" t="n">
-        <v>44.18451063829788</v>
+        <v>39.75897872340426</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -1299,25 +1299,25 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>132205</v>
+        <v>130120</v>
       </c>
       <c r="D10" t="n">
-        <v>0.0202971252170558</v>
+        <v>0.01264640647496</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.0265444370812164</v>
+        <v>-0.03568384777856</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.1482185426196766</v>
+        <v>-0.1677912442838413</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.1214895144467952</v>
+        <v>-0.1318047604744883</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.143556182130674</v>
+        <v>-0.1564092999298675</v>
       </c>
       <c r="I10" t="n">
-        <v>59.63232477977786</v>
+        <v>43.43637992831541</v>
       </c>
       <c r="J10" t="n">
         <v>40</v>
@@ -1327,7 +1327,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="M10" t="n">
@@ -1337,10 +1337,10 @@
         <v>40</v>
       </c>
       <c r="O10" t="n">
-        <v>25.53191489361702</v>
+        <v>23.40425531914894</v>
       </c>
       <c r="P10" t="n">
-        <v>40.8703829787234</v>
+        <v>40.44485106382978</v>
       </c>
       <c r="Q10" t="b">
         <v>0</v>
@@ -1376,10 +1376,10 @@
         <v>-0.0042030657656173</v>
       </c>
       <c r="G11" t="n">
-        <v>0.022525962407264</v>
+        <v>0.0317834180437356</v>
       </c>
       <c r="H11" t="n">
-        <v>0.0004592947233852</v>
+        <v>0.0071788785883564</v>
       </c>
       <c r="I11" t="n">
         <v>27.6054590570719</v>
@@ -1392,7 +1392,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="M11" t="n">
@@ -1402,10 +1402,10 @@
         <v>20</v>
       </c>
       <c r="O11" t="n">
-        <v>55.31914893617022</v>
+        <v>57.44680851063831</v>
       </c>
       <c r="P11" t="n">
-        <v>23.06382978723404</v>
+        <v>23.48936170212766</v>
       </c>
       <c r="Q11" t="b">
         <v>0</v>
@@ -1429,48 +1429,48 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>435.55</v>
+        <v>449</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.0072934472934472</v>
+        <v>0.0095559302979202</v>
       </c>
       <c r="E12" t="n">
-        <v>0.0133783154955793</v>
+        <v>0.0511529907526631</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.1268918512578931</v>
+        <v>-0.0821749795584627</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.1001628230850117</v>
+        <v>-0.0461884957491097</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.1222294907688905</v>
+        <v>-0.0707930352044889</v>
       </c>
       <c r="I12" t="n">
-        <v>52.22634508348798</v>
+        <v>57.08333333333333</v>
       </c>
       <c r="J12" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K12" t="n">
         <v>71.28</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="M12" t="n">
         <v>71.28</v>
       </c>
       <c r="N12" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="O12" t="n">
-        <v>31.91489361702128</v>
+        <v>40.42553191489361</v>
       </c>
       <c r="P12" t="n">
-        <v>58.89497872340426</v>
+        <v>68.59710638297872</v>
       </c>
       <c r="Q12" t="b">
         <v>1</v>
@@ -1494,25 +1494,25 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1877.9</v>
+        <v>1883.7</v>
       </c>
       <c r="D13" t="n">
-        <v>0.1844960262394348</v>
+        <v>0.2175683536940083</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.0340020576131686</v>
+        <v>-0.0154191929751201</v>
       </c>
       <c r="F13" t="n">
-        <v>0.0899645945789076</v>
+        <v>0.09225327612199941</v>
       </c>
       <c r="G13" t="n">
-        <v>0.1166936227517889</v>
+        <v>0.1282397599313524</v>
       </c>
       <c r="H13" t="n">
-        <v>0.09462695506791011</v>
+        <v>0.1036352204759731</v>
       </c>
       <c r="I13" t="n">
-        <v>69.02985074626865</v>
+        <v>66.42912172573189</v>
       </c>
       <c r="J13" t="n">
         <v>80</v>
@@ -1522,7 +1522,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="M13" t="n">
@@ -1559,48 +1559,48 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>624.55</v>
+        <v>625.6</v>
       </c>
       <c r="D14" t="n">
-        <v>0.1747390200319758</v>
+        <v>0.2404084465153166</v>
       </c>
       <c r="E14" t="n">
-        <v>0.1261269383339343</v>
+        <v>0.0873381420005214</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.2362113244466186</v>
+        <v>-0.223965763195435</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.2094822962737372</v>
+        <v>-0.187979279386082</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.231548963957616</v>
+        <v>-0.2125838188414612</v>
       </c>
       <c r="I14" t="n">
-        <v>73.77575595397374</v>
+        <v>67.26786907147627</v>
       </c>
       <c r="J14" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K14" t="n">
         <v>54.64</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="M14" t="n">
         <v>54.64</v>
       </c>
       <c r="N14" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O14" t="n">
-        <v>8.51063829787234</v>
+        <v>6.382978723404255</v>
       </c>
       <c r="P14" t="n">
-        <v>51.55812765957447</v>
+        <v>55.13259574468086</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
@@ -1624,48 +1624,48 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>109.75</v>
+        <v>107.36</v>
       </c>
       <c r="D15" t="n">
-        <v>0.2274913320657645</v>
+        <v>0.2451867316167941</v>
       </c>
       <c r="E15" t="n">
-        <v>0.0238828248903815</v>
+        <v>